<commit_message>
chore: update CATAPULT data 2026-06-18
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -1321,10 +1321,10 @@
         <v>142.3</v>
       </c>
       <c r="F9">
-        <v>8256.340000000002</v>
+        <v>8256.34</v>
       </c>
       <c r="G9">
-        <v>58.02066057624737</v>
+        <v>58.02066057624736</v>
       </c>
       <c r="H9">
         <v>499.06</v>
@@ -1354,10 +1354,10 @@
         <v>33.84</v>
       </c>
       <c r="Q9">
-        <v>871.5351299999999</v>
+        <v>871.53513</v>
       </c>
       <c r="R9">
-        <v>6.124631974701334</v>
+        <v>6.124631974701335</v>
       </c>
       <c r="S9">
         <v>1096.84001</v>
@@ -2751,10 +2751,10 @@
         <v>114.4713333333333</v>
       </c>
       <c r="F22">
-        <v>8536.459999999997</v>
+        <v>8536.459999999999</v>
       </c>
       <c r="G22">
-        <v>74.57290617155967</v>
+        <v>74.57290617155968</v>
       </c>
       <c r="H22">
         <v>176.52</v>
@@ -2977,7 +2977,7 @@
         <v>62.29918508342559</v>
       </c>
       <c r="H24">
-        <v>84.63999999999999</v>
+        <v>84.64</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>0.6773277138322418</v>
+        <v>0.6773277138322419</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -3004,10 +3004,10 @@
         <v>33.984</v>
       </c>
       <c r="Q24">
-        <v>965.6688100000001</v>
+        <v>965.66881</v>
       </c>
       <c r="R24">
-        <v>7.727720314229699</v>
+        <v>7.727720314229698</v>
       </c>
       <c r="S24">
         <v>1013.94</v>
@@ -3191,10 +3191,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F26">
-        <v>9359.540000000001</v>
+        <v>9359.539999999999</v>
       </c>
       <c r="G26">
-        <v>74.89928911532871</v>
+        <v>74.8992891153287</v>
       </c>
       <c r="H26">
         <v>180.97</v>
@@ -3266,7 +3266,7 @@
         <v>0</v>
       </c>
       <c r="AE26">
-        <v>801.2445000000001</v>
+        <v>801.2445</v>
       </c>
       <c r="AF26">
         <v>0</v>
@@ -3316,7 +3316,7 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>1.858649985995706</v>
+        <v>1.858649985995705</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -3444,10 +3444,10 @@
         <v>33.84</v>
       </c>
       <c r="Q28">
-        <v>945.4113000000001</v>
+        <v>945.4113</v>
       </c>
       <c r="R28">
-        <v>7.565610520559639</v>
+        <v>7.565610520559638</v>
       </c>
       <c r="S28">
         <v>1575.19001</v>
@@ -3747,7 +3747,7 @@
         <v>74.94482307907758</v>
       </c>
       <c r="H31">
-        <v>337.4999999999999</v>
+        <v>337.5</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -4110,7 +4110,7 @@
         <v>6.844402790188991</v>
       </c>
       <c r="S34">
-        <v>898.6499899999999</v>
+        <v>898.64999</v>
       </c>
       <c r="T34">
         <v>21</v>
@@ -4181,10 +4181,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F35">
-        <v>8757.950000000001</v>
+        <v>8757.949999999999</v>
       </c>
       <c r="G35">
-        <v>70.08509276178029</v>
+        <v>70.08509276178027</v>
       </c>
       <c r="H35">
         <v>203.09</v>
@@ -4366,7 +4366,7 @@
         <v>0</v>
       </c>
       <c r="AE36">
-        <v>762.7650000000001</v>
+        <v>762.765</v>
       </c>
       <c r="AF36">
         <v>0</v>
@@ -4401,10 +4401,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F37">
-        <v>8234.929999999998</v>
+        <v>8234.93</v>
       </c>
       <c r="G37">
-        <v>65.89964922576256</v>
+        <v>65.89964922576257</v>
       </c>
       <c r="H37">
         <v>42.54</v>
@@ -4434,10 +4434,10 @@
         <v>32.004</v>
       </c>
       <c r="Q37">
-        <v>847.99138</v>
+        <v>847.9913799999999</v>
       </c>
       <c r="R37">
-        <v>6.78601208370567</v>
+        <v>6.786012083705669</v>
       </c>
       <c r="S37">
         <v>1039.69</v>
@@ -4476,7 +4476,7 @@
         <v>0</v>
       </c>
       <c r="AE37">
-        <v>690.5905999999999</v>
+        <v>690.5906</v>
       </c>
       <c r="AF37">
         <v>0</v>
@@ -4657,7 +4657,7 @@
         <v>3.75311</v>
       </c>
       <c r="R39">
-        <v>0.08257667766776676</v>
+        <v>0.08257667766776677</v>
       </c>
       <c r="S39">
         <v>0</v>
@@ -4731,10 +4731,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F40">
-        <v>8274.099999999999</v>
+        <v>8274.1</v>
       </c>
       <c r="G40">
-        <v>66.21310535230803</v>
+        <v>66.21310535230805</v>
       </c>
       <c r="H40">
         <v>297.8200000000001</v>
@@ -4856,7 +4856,7 @@
         <v>0</v>
       </c>
       <c r="K41">
-        <v>0.3757152193339291</v>
+        <v>0.375715219333929</v>
       </c>
       <c r="L41">
         <v>0</v>
@@ -4951,7 +4951,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F42">
-        <v>7142.569999999999</v>
+        <v>7142.57</v>
       </c>
       <c r="G42">
         <v>93.52463631483153</v>
@@ -4966,7 +4966,7 @@
         <v>0</v>
       </c>
       <c r="K42">
-        <v>2.101059302614867</v>
+        <v>2.101059302614866</v>
       </c>
       <c r="L42">
         <v>0</v>
@@ -5094,13 +5094,13 @@
         <v>32.4</v>
       </c>
       <c r="Q43">
-        <v>806.5637</v>
+        <v>806.5636999999999</v>
       </c>
       <c r="R43">
         <v>10.56112529625119</v>
       </c>
       <c r="S43">
-        <v>911.0899999999999</v>
+        <v>911.09</v>
       </c>
       <c r="T43">
         <v>9</v>
@@ -5281,7 +5281,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F45">
-        <v>7078.56</v>
+        <v>7078.559999999999</v>
       </c>
       <c r="G45">
         <v>92.68649094551596</v>
@@ -5320,7 +5320,7 @@
         <v>8.81651228869597</v>
       </c>
       <c r="S45">
-        <v>830.0500099999999</v>
+        <v>830.05001</v>
       </c>
       <c r="T45">
         <v>28</v>
@@ -5356,7 +5356,7 @@
         <v>0</v>
       </c>
       <c r="AE45">
-        <v>664.0912000000001</v>
+        <v>664.0912</v>
       </c>
       <c r="AF45">
         <v>0</v>
@@ -5611,10 +5611,10 @@
         <v>76.37083333333334</v>
       </c>
       <c r="F48">
-        <v>6636.860000000001</v>
+        <v>6636.86</v>
       </c>
       <c r="G48">
-        <v>86.90307163511376</v>
+        <v>86.90307163511375</v>
       </c>
       <c r="H48">
         <v>201.92</v>
@@ -5650,7 +5650,7 @@
         <v>10.01454228817721</v>
       </c>
       <c r="S48">
-        <v>940.6600000000001</v>
+        <v>940.66</v>
       </c>
       <c r="T48">
         <v>11</v>
@@ -5686,7 +5686,7 @@
         <v>0</v>
       </c>
       <c r="AE48">
-        <v>553.3290000000001</v>
+        <v>553.329</v>
       </c>
       <c r="AF48">
         <v>0</v>
@@ -5864,10 +5864,10 @@
         <v>34.92</v>
       </c>
       <c r="Q50">
-        <v>675.5848699999999</v>
+        <v>675.58487</v>
       </c>
       <c r="R50">
-        <v>8.846091710204133</v>
+        <v>8.846091710204135</v>
       </c>
       <c r="S50">
         <v>952.77999</v>
@@ -6016,7 +6016,7 @@
         <v>0</v>
       </c>
       <c r="AE51">
-        <v>630.7519299999999</v>
+        <v>630.75193</v>
       </c>
       <c r="AF51">
         <v>0</v>
@@ -6051,10 +6051,10 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F52">
-        <v>6693.129999999999</v>
+        <v>6693.13</v>
       </c>
       <c r="G52">
-        <v>87.63967998323969</v>
+        <v>87.6396799832397</v>
       </c>
       <c r="H52">
         <v>16.96</v>
@@ -6304,13 +6304,13 @@
         <v>33.012</v>
       </c>
       <c r="Q54">
-        <v>685.1758299999999</v>
+        <v>685.17583</v>
       </c>
       <c r="R54">
-        <v>8.971675505100102</v>
+        <v>8.971675505100103</v>
       </c>
       <c r="S54">
-        <v>843.77997</v>
+        <v>843.7799699999999</v>
       </c>
       <c r="T54">
         <v>17</v>
@@ -6355,7 +6355,7 @@
         <v>3</v>
       </c>
       <c r="AH54">
-        <v>2055.527489999999</v>
+        <v>2055.52749</v>
       </c>
     </row>
     <row r="55">
@@ -6491,7 +6491,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F56">
-        <v>6802.68</v>
+        <v>6802.679999999999</v>
       </c>
       <c r="G56">
         <v>89.07412499508975</v>
@@ -6530,7 +6530,7 @@
         <v>8.080355370494035</v>
       </c>
       <c r="S56">
-        <v>862.5100000000001</v>
+        <v>862.51</v>
       </c>
       <c r="T56">
         <v>10</v>
@@ -6634,13 +6634,13 @@
         <v>36</v>
       </c>
       <c r="Q57">
-        <v>618.2029799999999</v>
+        <v>618.20298</v>
       </c>
       <c r="R57">
-        <v>8.094734650587263</v>
+        <v>8.094734650587265</v>
       </c>
       <c r="S57">
-        <v>742.09999</v>
+        <v>742.0999899999999</v>
       </c>
       <c r="T57">
         <v>12</v>
@@ -6676,7 +6676,7 @@
         <v>0</v>
       </c>
       <c r="AE57">
-        <v>509.4404000000001</v>
+        <v>509.4404</v>
       </c>
       <c r="AF57">
         <v>0</v>
@@ -6855,7 +6855,7 @@
         <v>6.301423002309469</v>
       </c>
       <c r="S59">
-        <v>900.0399500000001</v>
+        <v>900.03995</v>
       </c>
       <c r="T59">
         <v>20</v>
@@ -7374,10 +7374,10 @@
         <v>32.004</v>
       </c>
       <c r="Q64">
-        <v>671.0377699999999</v>
+        <v>671.03777</v>
       </c>
       <c r="R64">
-        <v>6.19896323325635</v>
+        <v>6.198963233256351</v>
       </c>
       <c r="S64">
         <v>862.40997</v>
@@ -7626,7 +7626,7 @@
         <v>0</v>
       </c>
       <c r="AE66">
-        <v>584.6215999999999</v>
+        <v>584.6216000000001</v>
       </c>
       <c r="AF66">
         <v>0</v>
@@ -7656,10 +7656,10 @@
         <v>108.25</v>
       </c>
       <c r="F67">
-        <v>5820.460000000001</v>
+        <v>5820.46</v>
       </c>
       <c r="G67">
-        <v>53.76868360277137</v>
+        <v>53.76868360277136</v>
       </c>
       <c r="H67">
         <v>25.29</v>
@@ -8076,10 +8076,10 @@
         <v>108.25</v>
       </c>
       <c r="F71">
-        <v>6131.409999999999</v>
+        <v>6131.41</v>
       </c>
       <c r="G71">
-        <v>56.64120092378752</v>
+        <v>56.64120092378753</v>
       </c>
       <c r="H71">
         <v>57.77</v>
@@ -8109,10 +8109,10 @@
         <v>34.992</v>
       </c>
       <c r="Q71">
-        <v>678.6408300000001</v>
+        <v>678.6408299999999</v>
       </c>
       <c r="R71">
-        <v>6.26919935334873</v>
+        <v>6.269199353348729</v>
       </c>
       <c r="S71">
         <v>981.28002</v>
@@ -8256,7 +8256,7 @@
         <v>0</v>
       </c>
       <c r="AE72">
-        <v>507.1950000000001</v>
+        <v>507.195</v>
       </c>
       <c r="AF72">
         <v>0</v>
@@ -8325,7 +8325,7 @@
         <v>5.857015889145496</v>
       </c>
       <c r="S73">
-        <v>790.5800099999999</v>
+        <v>790.58001</v>
       </c>
       <c r="T73">
         <v>33</v>
@@ -8496,10 +8496,10 @@
         <v>108.25</v>
       </c>
       <c r="F75">
-        <v>5283.150000000001</v>
+        <v>5283.15</v>
       </c>
       <c r="G75">
-        <v>48.80508083140878</v>
+        <v>48.80508083140877</v>
       </c>
       <c r="H75">
         <v>30.94</v>
@@ -8535,7 +8535,7 @@
         <v>5.961701524249423</v>
       </c>
       <c r="S75">
-        <v>806.9200000000001</v>
+        <v>806.92</v>
       </c>
       <c r="T75">
         <v>42</v>
@@ -8640,7 +8640,7 @@
         <v>5.930582817551963</v>
       </c>
       <c r="S76">
-        <v>598.8199999999999</v>
+        <v>598.8200000000001</v>
       </c>
       <c r="T76">
         <v>28</v>
@@ -8676,7 +8676,7 @@
         <v>0</v>
       </c>
       <c r="AE76">
-        <v>484.7602499999999</v>
+        <v>484.76025</v>
       </c>
       <c r="AF76">
         <v>0</v>
@@ -8744,7 +8744,7 @@
         <v>32.364</v>
       </c>
       <c r="Q77">
-        <v>758.4063100000001</v>
+        <v>758.40631</v>
       </c>
       <c r="R77">
         <v>11.09411010637131</v>
@@ -9261,10 +9261,10 @@
         <v>71.20933333333333</v>
       </c>
       <c r="F82">
-        <v>7086.919999999999</v>
+        <v>7086.92</v>
       </c>
       <c r="G82">
-        <v>99.52234725785009</v>
+        <v>99.5223472578501</v>
       </c>
       <c r="H82">
         <v>246.93</v>
@@ -9410,7 +9410,7 @@
         <v>7.952642350253712</v>
       </c>
       <c r="S83">
-        <v>931.2800099999999</v>
+        <v>931.2800100000001</v>
       </c>
       <c r="T83">
         <v>15</v>
@@ -9446,7 +9446,7 @@
         <v>0</v>
       </c>
       <c r="AE83">
-        <v>558.38181</v>
+        <v>558.3818100000001</v>
       </c>
       <c r="AF83">
         <v>0</v>
@@ -9481,10 +9481,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F84">
-        <v>6362.629999999999</v>
+        <v>6362.63</v>
       </c>
       <c r="G84">
-        <v>93.07374800995692</v>
+        <v>93.07374800995693</v>
       </c>
       <c r="H84">
         <v>345.63</v>
@@ -9701,10 +9701,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F86">
-        <v>6656.71</v>
+        <v>6656.709999999999</v>
       </c>
       <c r="G86">
-        <v>97.3756055460337</v>
+        <v>97.37560554603368</v>
       </c>
       <c r="H86">
         <v>144.12</v>
@@ -9776,7 +9776,7 @@
         <v>0</v>
       </c>
       <c r="AE86">
-        <v>621.0583999999999</v>
+        <v>621.0584</v>
       </c>
       <c r="AF86">
         <v>0</v>
@@ -9921,7 +9921,7 @@
         <v>68.7235</v>
       </c>
       <c r="F88">
-        <v>7172.649999999999</v>
+        <v>7172.65</v>
       </c>
       <c r="G88">
         <v>104.3696843146813</v>
@@ -10070,7 +10070,7 @@
         <v>8.221425422162724</v>
       </c>
       <c r="S89">
-        <v>925.6099999999999</v>
+        <v>925.61</v>
       </c>
       <c r="T89">
         <v>14</v>
@@ -10364,7 +10364,7 @@
         <v>13609.36</v>
       </c>
       <c r="G92">
-        <v>75.02431100445061</v>
+        <v>75.02431100445058</v>
       </c>
       <c r="H92">
         <v>783.59</v>
@@ -10376,7 +10376,7 @@
         <v>0</v>
       </c>
       <c r="K92">
-        <v>4.319696140007865</v>
+        <v>4.319696140007864</v>
       </c>
       <c r="L92">
         <v>0</v>
@@ -10397,7 +10397,7 @@
         <v>1367.31024</v>
       </c>
       <c r="R92">
-        <v>7.537570369608122</v>
+        <v>7.53757036960812</v>
       </c>
       <c r="S92">
         <v>2768.85995</v>
@@ -10474,7 +10474,7 @@
         <v>13532.14</v>
       </c>
       <c r="G93">
-        <v>74.59862035509136</v>
+        <v>74.59862035509134</v>
       </c>
       <c r="H93">
         <v>905.78</v>
@@ -10486,7 +10486,7 @@
         <v>0</v>
       </c>
       <c r="K93">
-        <v>4.99329288237002</v>
+        <v>4.993292882370019</v>
       </c>
       <c r="L93">
         <v>0</v>
@@ -10584,10 +10584,10 @@
         <v>12701.11</v>
       </c>
       <c r="G94">
-        <v>70.01740175450848</v>
+        <v>70.01740175450847</v>
       </c>
       <c r="H94">
-        <v>368.9400000000001</v>
+        <v>368.94</v>
       </c>
       <c r="I94">
         <v>0</v>
@@ -10617,7 +10617,7 @@
         <v>1622.4067</v>
       </c>
       <c r="R94">
-        <v>8.943840477179263</v>
+        <v>8.943840477179261</v>
       </c>
       <c r="S94">
         <v>1981.77002</v>
@@ -10694,10 +10694,10 @@
         <v>14057.61</v>
       </c>
       <c r="G95">
-        <v>77.49537852031798</v>
+        <v>77.49537852031797</v>
       </c>
       <c r="H95">
-        <v>717.6199999999999</v>
+        <v>717.62</v>
       </c>
       <c r="I95">
         <v>0</v>
@@ -10727,7 +10727,7 @@
         <v>1301.95454</v>
       </c>
       <c r="R95">
-        <v>7.177284040000148</v>
+        <v>7.177284040000147</v>
       </c>
       <c r="S95">
         <v>2534.90994</v>
@@ -10775,7 +10775,7 @@
         <v>3</v>
       </c>
       <c r="AH95">
-        <v>3905.863620000001</v>
+        <v>3905.86362</v>
       </c>
     </row>
     <row r="96">
@@ -10804,7 +10804,7 @@
         <v>13466.34</v>
       </c>
       <c r="G96">
-        <v>74.23588473313023</v>
+        <v>74.23588473313021</v>
       </c>
       <c r="H96">
         <v>1259.67</v>
@@ -10816,7 +10816,7 @@
         <v>0</v>
       </c>
       <c r="K96">
-        <v>6.944182080786773</v>
+        <v>6.944182080786772</v>
       </c>
       <c r="L96">
         <v>0</v>
@@ -10837,7 +10837,7 @@
         <v>1361.55609</v>
       </c>
       <c r="R96">
-        <v>7.505849470229586</v>
+        <v>7.505849470229585</v>
       </c>
       <c r="S96">
         <v>3031.29993</v>
@@ -10914,10 +10914,10 @@
         <v>11839.12</v>
       </c>
       <c r="G97">
-        <v>65.26550997982353</v>
+        <v>65.26550997982351</v>
       </c>
       <c r="H97">
-        <v>580.6799999999998</v>
+        <v>580.6799999999999</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -10947,7 +10947,7 @@
         <v>1362.04584</v>
       </c>
       <c r="R97">
-        <v>7.508549314771463</v>
+        <v>7.508549314771462</v>
       </c>
       <c r="S97">
         <v>2197.63005</v>
@@ -10986,7 +10986,7 @@
         <v>0</v>
       </c>
       <c r="AE97">
-        <v>846.5939999999999</v>
+        <v>846.5940000000001</v>
       </c>
       <c r="AF97">
         <v>0</v>
@@ -11134,7 +11134,7 @@
         <v>13587.06</v>
       </c>
       <c r="G99">
-        <v>74.90137780734219</v>
+        <v>74.90137780734217</v>
       </c>
       <c r="H99">
         <v>610.51</v>
@@ -11167,7 +11167,7 @@
         <v>1448.92289</v>
       </c>
       <c r="R99">
-        <v>7.987476378082978</v>
+        <v>7.987476378082977</v>
       </c>
       <c r="S99">
         <v>2588.26003</v>
@@ -11244,10 +11244,10 @@
         <v>13570.48</v>
       </c>
       <c r="G100">
-        <v>74.80997725092706</v>
+        <v>74.80997725092705</v>
       </c>
       <c r="H100">
-        <v>420.2499999999999</v>
+        <v>420.25</v>
       </c>
       <c r="I100">
         <v>0</v>
@@ -11277,7 +11277,7 @@
         <v>1254.50062</v>
       </c>
       <c r="R100">
-        <v>6.915684842649184</v>
+        <v>6.915684842649182</v>
       </c>
       <c r="S100">
         <v>2110.94003</v>
@@ -11464,7 +11464,7 @@
         <v>11738.1</v>
       </c>
       <c r="G102">
-        <v>64.70861708422302</v>
+        <v>64.70861708422301</v>
       </c>
       <c r="H102">
         <v>228.83</v>
@@ -11497,7 +11497,7 @@
         <v>1103.19668</v>
       </c>
       <c r="R102">
-        <v>6.081591700079751</v>
+        <v>6.08159170007975</v>
       </c>
       <c r="S102">
         <v>1850.74</v>
@@ -11574,7 +11574,7 @@
         <v>14309.53</v>
       </c>
       <c r="G103">
-        <v>78.88413775868344</v>
+        <v>78.88413775868342</v>
       </c>
       <c r="H103">
         <v>1603.26</v>
@@ -11607,7 +11607,7 @@
         <v>1351.15255</v>
       </c>
       <c r="R103">
-        <v>7.448497881285855</v>
+        <v>7.448497881285856</v>
       </c>
       <c r="S103">
         <v>3616.20992</v>
@@ -11655,7 +11655,7 @@
         <v>3</v>
       </c>
       <c r="AH103">
-        <v>4053.457649999999</v>
+        <v>4053.45765</v>
       </c>
     </row>
     <row r="104">
@@ -11684,7 +11684,7 @@
         <v>12247.15</v>
       </c>
       <c r="G104">
-        <v>67.51485672494204</v>
+        <v>67.51485672494202</v>
       </c>
       <c r="H104">
         <v>385.08</v>
@@ -11794,7 +11794,7 @@
         <v>13585.76</v>
       </c>
       <c r="G105">
-        <v>74.89421129809371</v>
+        <v>74.89421129809369</v>
       </c>
       <c r="H105">
         <v>1185.27</v>
@@ -11806,7 +11806,7 @@
         <v>0</v>
       </c>
       <c r="K105">
-        <v>6.534037243797295</v>
+        <v>6.534037243797294</v>
       </c>
       <c r="L105">
         <v>0</v>
@@ -11827,7 +11827,7 @@
         <v>1300.14625</v>
       </c>
       <c r="R105">
-        <v>7.167315480762517</v>
+        <v>7.167315480762516</v>
       </c>
       <c r="S105">
         <v>2929.39002</v>
@@ -11904,7 +11904,7 @@
         <v>12266.49</v>
       </c>
       <c r="G106">
-        <v>67.62147233176162</v>
+        <v>67.62147233176159</v>
       </c>
       <c r="H106">
         <v>463.29</v>
@@ -11916,7 +11916,7 @@
         <v>0</v>
       </c>
       <c r="K106">
-        <v>2.553978515172787</v>
+        <v>2.553978515172786</v>
       </c>
       <c r="L106">
         <v>0</v>
@@ -11937,7 +11937,7 @@
         <v>1240.70238</v>
       </c>
       <c r="R106">
-        <v>6.839619292977924</v>
+        <v>6.839619292977923</v>
       </c>
       <c r="S106">
         <v>2345.96002</v>
@@ -12014,7 +12014,7 @@
         <v>12956.01</v>
       </c>
       <c r="G107">
-        <v>71.42258883715118</v>
+        <v>71.42258883715117</v>
       </c>
       <c r="H107">
         <v>550.62</v>
@@ -12047,7 +12047,7 @@
         <v>1367.91901</v>
       </c>
       <c r="R107">
-        <v>7.540926335635192</v>
+        <v>7.540926335635191</v>
       </c>
       <c r="S107">
         <v>2087.11996</v>
@@ -12234,10 +12234,10 @@
         <v>18303.41</v>
       </c>
       <c r="G109">
-        <v>79.93284853654792</v>
+        <v>79.93284853654791</v>
       </c>
       <c r="H109">
-        <v>472.7499999999999</v>
+        <v>472.75</v>
       </c>
       <c r="I109">
         <v>0</v>
@@ -12267,7 +12267,7 @@
         <v>1772.41724</v>
       </c>
       <c r="R109">
-        <v>7.740325916781971</v>
+        <v>7.74032591678197</v>
       </c>
       <c r="S109">
         <v>2454.89998</v>
@@ -12356,7 +12356,7 @@
         <v>0</v>
       </c>
       <c r="K110">
-        <v>1.783742591394335</v>
+        <v>1.783742591394336</v>
       </c>
       <c r="L110">
         <v>0</v>
@@ -12564,7 +12564,7 @@
         <v>19147.53</v>
       </c>
       <c r="G112">
-        <v>85.15633651543349</v>
+        <v>85.15633651543351</v>
       </c>
       <c r="H112">
         <v>370.36</v>
@@ -12597,7 +12597,7 @@
         <v>1718.72645</v>
       </c>
       <c r="R112">
-        <v>7.643829149460865</v>
+        <v>7.643829149460866</v>
       </c>
       <c r="S112">
         <v>1940.40001</v>
@@ -12645,7 +12645,7 @@
         <v>3</v>
       </c>
       <c r="AH112">
-        <v>5156.179349999999</v>
+        <v>5156.17935</v>
       </c>
     </row>
     <row r="113">
@@ -12784,7 +12784,7 @@
         <v>16065.62</v>
       </c>
       <c r="G114">
-        <v>70.16019256006037</v>
+        <v>70.16019256006038</v>
       </c>
       <c r="H114">
         <v>375.7</v>
@@ -12817,7 +12817,7 @@
         <v>1707.62189</v>
       </c>
       <c r="R114">
-        <v>7.457358049186664</v>
+        <v>7.457358049186663</v>
       </c>
       <c r="S114">
         <v>2101.00999</v>
@@ -12865,7 +12865,7 @@
         <v>3</v>
       </c>
       <c r="AH114">
-        <v>5122.86567</v>
+        <v>5122.865669999999</v>
       </c>
     </row>
     <row r="115">
@@ -12894,7 +12894,7 @@
         <v>17963.75</v>
       </c>
       <c r="G115">
-        <v>79.89161735634409</v>
+        <v>79.89161735634407</v>
       </c>
       <c r="H115">
         <v>370.21</v>
@@ -12927,7 +12927,7 @@
         <v>1698.34145</v>
       </c>
       <c r="R115">
-        <v>7.553169313969441</v>
+        <v>7.553169313969442</v>
       </c>
       <c r="S115">
         <v>1988.68005</v>
@@ -12975,7 +12975,7 @@
         <v>3</v>
       </c>
       <c r="AH115">
-        <v>5095.02435</v>
+        <v>5095.024350000001</v>
       </c>
     </row>
     <row r="116">
@@ -13004,7 +13004,7 @@
         <v>16860.45</v>
       </c>
       <c r="G116">
-        <v>74.74106193604921</v>
+        <v>74.74106193604919</v>
       </c>
       <c r="H116">
         <v>198.18</v>
@@ -13016,7 +13016,7 @@
         <v>0</v>
       </c>
       <c r="K116">
-        <v>0.8785165078326039</v>
+        <v>0.878516507832604</v>
       </c>
       <c r="L116">
         <v>0</v>
@@ -13037,7 +13037,7 @@
         <v>1727.96753</v>
       </c>
       <c r="R116">
-        <v>7.659945504610609</v>
+        <v>7.659945504610608</v>
       </c>
       <c r="S116">
         <v>2211.12</v>
@@ -13085,7 +13085,7 @@
         <v>3</v>
       </c>
       <c r="AH116">
-        <v>5183.902590000001</v>
+        <v>5183.90259</v>
       </c>
     </row>
     <row r="117">
@@ -13114,10 +13114,10 @@
         <v>18388.95</v>
       </c>
       <c r="G117">
-        <v>81.78264321118603</v>
+        <v>81.78264321118604</v>
       </c>
       <c r="H117">
-        <v>270.9999999999999</v>
+        <v>271</v>
       </c>
       <c r="I117">
         <v>0</v>
@@ -13147,7 +13147,7 @@
         <v>1735.53757</v>
       </c>
       <c r="R117">
-        <v>7.718594583536246</v>
+        <v>7.718594583536245</v>
       </c>
       <c r="S117">
         <v>1729.52995</v>
@@ -13195,7 +13195,7 @@
         <v>3</v>
       </c>
       <c r="AH117">
-        <v>5206.61271</v>
+        <v>5206.612709999999</v>
       </c>
     </row>
     <row r="118">
@@ -13257,7 +13257,7 @@
         <v>1527.87451</v>
       </c>
       <c r="R118">
-        <v>6.772948728083817</v>
+        <v>6.772948728083818</v>
       </c>
       <c r="S118">
         <v>1992.10995</v>
@@ -13305,7 +13305,7 @@
         <v>3</v>
       </c>
       <c r="AH118">
-        <v>4583.62353</v>
+        <v>4583.623530000001</v>
       </c>
     </row>
     <row r="119">
@@ -13346,7 +13346,7 @@
         <v>0</v>
       </c>
       <c r="K119">
-        <v>4.8997186563169</v>
+        <v>4.899718656316899</v>
       </c>
       <c r="L119">
         <v>0</v>
@@ -13370,7 +13370,7 @@
         <v>6.606615921757134</v>
       </c>
       <c r="S119">
-        <v>3415.690039999999</v>
+        <v>3415.69004</v>
       </c>
       <c r="T119">
         <v>77</v>
@@ -13444,7 +13444,7 @@
         <v>18290.91</v>
       </c>
       <c r="G120">
-        <v>74.02184932102797</v>
+        <v>74.021849321028</v>
       </c>
       <c r="H120">
         <v>113.2</v>
@@ -13477,7 +13477,7 @@
         <v>1736.55142</v>
       </c>
       <c r="R120">
-        <v>7.027684655900511</v>
+        <v>7.02768465590051</v>
       </c>
       <c r="S120">
         <v>1459.61002</v>
@@ -13525,7 +13525,7 @@
         <v>3</v>
       </c>
       <c r="AH120">
-        <v>5209.654260000001</v>
+        <v>5209.65426</v>
       </c>
     </row>
     <row r="121">
@@ -13697,10 +13697,10 @@
         <v>1747.75452</v>
       </c>
       <c r="R122">
-        <v>7.052093914697219</v>
+        <v>7.052093914697221</v>
       </c>
       <c r="S122">
-        <v>2673.450039999999</v>
+        <v>2673.45004</v>
       </c>
       <c r="T122">
         <v>69</v>
@@ -13956,7 +13956,7 @@
         <v>0</v>
       </c>
       <c r="AE124">
-        <v>822.8863999999999</v>
+        <v>822.8864</v>
       </c>
       <c r="AF124">
         <v>0</v>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-19
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH124"/>
+  <dimension ref="A1:AH156"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -13968,6 +13968,3526 @@
         <v>2942.50395</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B125" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E125">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F125">
+        <v>5866.37</v>
+      </c>
+      <c r="G125">
+        <v>63.88722608327902</v>
+      </c>
+      <c r="H125">
+        <v>101.63</v>
+      </c>
+      <c r="I125">
+        <v>0</v>
+      </c>
+      <c r="J125">
+        <v>0</v>
+      </c>
+      <c r="K125">
+        <v>1.10679326173488</v>
+      </c>
+      <c r="L125">
+        <v>0</v>
+      </c>
+      <c r="M125">
+        <v>0</v>
+      </c>
+      <c r="N125">
+        <v>25.53717</v>
+      </c>
+      <c r="O125">
+        <v>78.90609936967002</v>
+      </c>
+      <c r="P125">
+        <v>32.364</v>
+      </c>
+      <c r="Q125">
+        <v>582.29178</v>
+      </c>
+      <c r="R125">
+        <v>6.341401342788637</v>
+      </c>
+      <c r="S125">
+        <v>881.17</v>
+      </c>
+      <c r="T125">
+        <v>6</v>
+      </c>
+      <c r="U125">
+        <v>9</v>
+      </c>
+      <c r="V125">
+        <v>15</v>
+      </c>
+      <c r="W125">
+        <v>59</v>
+      </c>
+      <c r="X125">
+        <v>6</v>
+      </c>
+      <c r="Y125">
+        <v>36</v>
+      </c>
+      <c r="Z125">
+        <v>9</v>
+      </c>
+      <c r="AA125">
+        <v>7</v>
+      </c>
+      <c r="AB125">
+        <v>3.57844</v>
+      </c>
+      <c r="AC125">
+        <v>-2.29354</v>
+      </c>
+      <c r="AD125">
+        <v>0</v>
+      </c>
+      <c r="AE125">
+        <v>469.4830000000001</v>
+      </c>
+      <c r="AF125">
+        <v>0</v>
+      </c>
+      <c r="AG125">
+        <v>3</v>
+      </c>
+      <c r="AH125">
+        <v>1746.87534</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B126" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E126">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F126">
+        <v>6505.129999999999</v>
+      </c>
+      <c r="G126">
+        <v>70.84358999025307</v>
+      </c>
+      <c r="H126">
+        <v>205.73</v>
+      </c>
+      <c r="I126">
+        <v>0</v>
+      </c>
+      <c r="J126">
+        <v>0</v>
+      </c>
+      <c r="K126">
+        <v>2.240485857883665</v>
+      </c>
+      <c r="L126">
+        <v>0</v>
+      </c>
+      <c r="M126">
+        <v>0</v>
+      </c>
+      <c r="N126">
+        <v>28.06244</v>
+      </c>
+      <c r="O126">
+        <v>86.61246913580247</v>
+      </c>
+      <c r="P126">
+        <v>32.4</v>
+      </c>
+      <c r="Q126">
+        <v>742.99425</v>
+      </c>
+      <c r="R126">
+        <v>8.091518541845526</v>
+      </c>
+      <c r="S126">
+        <v>1255.76</v>
+      </c>
+      <c r="T126">
+        <v>31</v>
+      </c>
+      <c r="U126">
+        <v>16</v>
+      </c>
+      <c r="V126">
+        <v>47</v>
+      </c>
+      <c r="W126">
+        <v>118</v>
+      </c>
+      <c r="X126">
+        <v>31</v>
+      </c>
+      <c r="Y126">
+        <v>61</v>
+      </c>
+      <c r="Z126">
+        <v>16</v>
+      </c>
+      <c r="AA126">
+        <v>12</v>
+      </c>
+      <c r="AB126">
+        <v>3.90055</v>
+      </c>
+      <c r="AC126">
+        <v>-2.25977</v>
+      </c>
+      <c r="AD126">
+        <v>0</v>
+      </c>
+      <c r="AE126">
+        <v>540.6233</v>
+      </c>
+      <c r="AF126">
+        <v>0</v>
+      </c>
+      <c r="AG126">
+        <v>3</v>
+      </c>
+      <c r="AH126">
+        <v>2228.98275</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B127" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E127">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F127">
+        <v>5290.24</v>
+      </c>
+      <c r="G127">
+        <v>57.61292910518873</v>
+      </c>
+      <c r="H127">
+        <v>81.05</v>
+      </c>
+      <c r="I127">
+        <v>0</v>
+      </c>
+      <c r="J127">
+        <v>0</v>
+      </c>
+      <c r="K127">
+        <v>0.882668443014976</v>
+      </c>
+      <c r="L127">
+        <v>0</v>
+      </c>
+      <c r="M127">
+        <v>0</v>
+      </c>
+      <c r="N127">
+        <v>25.43687</v>
+      </c>
+      <c r="O127">
+        <v>74.84954684557438</v>
+      </c>
+      <c r="P127">
+        <v>33.984</v>
+      </c>
+      <c r="Q127">
+        <v>662.60838</v>
+      </c>
+      <c r="R127">
+        <v>7.216082752662254</v>
+      </c>
+      <c r="S127">
+        <v>571.95001</v>
+      </c>
+      <c r="T127">
+        <v>9</v>
+      </c>
+      <c r="U127">
+        <v>15</v>
+      </c>
+      <c r="V127">
+        <v>24</v>
+      </c>
+      <c r="W127">
+        <v>57</v>
+      </c>
+      <c r="X127">
+        <v>9</v>
+      </c>
+      <c r="Y127">
+        <v>38</v>
+      </c>
+      <c r="Z127">
+        <v>15</v>
+      </c>
+      <c r="AA127">
+        <v>11</v>
+      </c>
+      <c r="AB127">
+        <v>3.87292</v>
+      </c>
+      <c r="AC127">
+        <v>-2.60968</v>
+      </c>
+      <c r="AD127">
+        <v>0</v>
+      </c>
+      <c r="AE127">
+        <v>485.6536</v>
+      </c>
+      <c r="AF127">
+        <v>0</v>
+      </c>
+      <c r="AG127">
+        <v>3</v>
+      </c>
+      <c r="AH127">
+        <v>1987.82514</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Dagoberto Espinoza</t>
+        </is>
+      </c>
+      <c r="B128" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E128">
+        <v>113.163</v>
+      </c>
+      <c r="F128">
+        <v>7157.05</v>
+      </c>
+      <c r="G128">
+        <v>63.24549543578732</v>
+      </c>
+      <c r="H128">
+        <v>225.97</v>
+      </c>
+      <c r="I128">
+        <v>0</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>1.996854095419881</v>
+      </c>
+      <c r="L128">
+        <v>0</v>
+      </c>
+      <c r="M128">
+        <v>0</v>
+      </c>
+      <c r="N128">
+        <v>29.28217</v>
+      </c>
+      <c r="O128">
+        <v>82.3272885739991</v>
+      </c>
+      <c r="P128">
+        <v>35.568</v>
+      </c>
+      <c r="Q128">
+        <v>628.97713</v>
+      </c>
+      <c r="R128">
+        <v>5.558151781059181</v>
+      </c>
+      <c r="S128">
+        <v>1047.82999</v>
+      </c>
+      <c r="T128">
+        <v>37</v>
+      </c>
+      <c r="U128">
+        <v>15</v>
+      </c>
+      <c r="V128">
+        <v>52</v>
+      </c>
+      <c r="W128">
+        <v>111</v>
+      </c>
+      <c r="X128">
+        <v>37</v>
+      </c>
+      <c r="Y128">
+        <v>70</v>
+      </c>
+      <c r="Z128">
+        <v>15</v>
+      </c>
+      <c r="AA128">
+        <v>14</v>
+      </c>
+      <c r="AB128">
+        <v>5.05473</v>
+      </c>
+      <c r="AC128">
+        <v>-2.10859</v>
+      </c>
+      <c r="AD128">
+        <v>0</v>
+      </c>
+      <c r="AE128">
+        <v>677.4304</v>
+      </c>
+      <c r="AF128">
+        <v>0</v>
+      </c>
+      <c r="AG128">
+        <v>3</v>
+      </c>
+      <c r="AH128">
+        <v>1886.93139</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B129" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E129">
+        <v>113.163</v>
+      </c>
+      <c r="F129">
+        <v>6408.839999999999</v>
+      </c>
+      <c r="G129">
+        <v>56.63370536306036</v>
+      </c>
+      <c r="H129">
+        <v>286.85</v>
+      </c>
+      <c r="I129">
+        <v>0</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>2.534839125862693</v>
+      </c>
+      <c r="L129">
+        <v>0</v>
+      </c>
+      <c r="M129">
+        <v>0</v>
+      </c>
+      <c r="N129">
+        <v>26.30469</v>
+      </c>
+      <c r="O129">
+        <v>73.06858333333334</v>
+      </c>
+      <c r="P129">
+        <v>36</v>
+      </c>
+      <c r="Q129">
+        <v>613.2202</v>
+      </c>
+      <c r="R129">
+        <v>5.418910774723187</v>
+      </c>
+      <c r="S129">
+        <v>1023.20001</v>
+      </c>
+      <c r="T129">
+        <v>27</v>
+      </c>
+      <c r="U129">
+        <v>15</v>
+      </c>
+      <c r="V129">
+        <v>42</v>
+      </c>
+      <c r="W129">
+        <v>95</v>
+      </c>
+      <c r="X129">
+        <v>27</v>
+      </c>
+      <c r="Y129">
+        <v>51</v>
+      </c>
+      <c r="Z129">
+        <v>15</v>
+      </c>
+      <c r="AA129">
+        <v>16</v>
+      </c>
+      <c r="AB129">
+        <v>3.78909</v>
+      </c>
+      <c r="AC129">
+        <v>-2.2518</v>
+      </c>
+      <c r="AD129">
+        <v>0</v>
+      </c>
+      <c r="AE129">
+        <v>524.8838000000001</v>
+      </c>
+      <c r="AF129">
+        <v>0</v>
+      </c>
+      <c r="AG129">
+        <v>3</v>
+      </c>
+      <c r="AH129">
+        <v>1839.6606</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B130" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E130">
+        <v>60.53416666666667</v>
+      </c>
+      <c r="F130">
+        <v>2959.6</v>
+      </c>
+      <c r="G130">
+        <v>48.8913974201897</v>
+      </c>
+      <c r="H130">
+        <v>0</v>
+      </c>
+      <c r="I130">
+        <v>0</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>0</v>
+      </c>
+      <c r="L130">
+        <v>0</v>
+      </c>
+      <c r="M130">
+        <v>0</v>
+      </c>
+      <c r="N130">
+        <v>19.13209</v>
+      </c>
+      <c r="O130">
+        <v>59.78030871141108</v>
+      </c>
+      <c r="P130">
+        <v>32.004</v>
+      </c>
+      <c r="Q130">
+        <v>350.61662</v>
+      </c>
+      <c r="R130">
+        <v>5.792045043432772</v>
+      </c>
+      <c r="S130">
+        <v>212.02</v>
+      </c>
+      <c r="T130">
+        <v>8</v>
+      </c>
+      <c r="U130">
+        <v>1</v>
+      </c>
+      <c r="V130">
+        <v>9</v>
+      </c>
+      <c r="W130">
+        <v>33</v>
+      </c>
+      <c r="X130">
+        <v>8</v>
+      </c>
+      <c r="Y130">
+        <v>15</v>
+      </c>
+      <c r="Z130">
+        <v>1</v>
+      </c>
+      <c r="AA130">
+        <v>6</v>
+      </c>
+      <c r="AB130">
+        <v>3.60801</v>
+      </c>
+      <c r="AC130">
+        <v>-2.65044</v>
+      </c>
+      <c r="AD130">
+        <v>0</v>
+      </c>
+      <c r="AE130">
+        <v>199.6728</v>
+      </c>
+      <c r="AF130">
+        <v>0</v>
+      </c>
+      <c r="AG130">
+        <v>3</v>
+      </c>
+      <c r="AH130">
+        <v>1051.84986</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B131" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E131">
+        <v>113.1631666666667</v>
+      </c>
+      <c r="F131">
+        <v>6269.6</v>
+      </c>
+      <c r="G131">
+        <v>55.40318625465589</v>
+      </c>
+      <c r="H131">
+        <v>211.59</v>
+      </c>
+      <c r="I131">
+        <v>0</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>1.869778004916205</v>
+      </c>
+      <c r="L131">
+        <v>0</v>
+      </c>
+      <c r="M131">
+        <v>0</v>
+      </c>
+      <c r="N131">
+        <v>26.01866</v>
+      </c>
+      <c r="O131">
+        <v>76.88729314420803</v>
+      </c>
+      <c r="P131">
+        <v>33.84</v>
+      </c>
+      <c r="Q131">
+        <v>619.42111</v>
+      </c>
+      <c r="R131">
+        <v>5.473698980380837</v>
+      </c>
+      <c r="S131">
+        <v>780.15</v>
+      </c>
+      <c r="T131">
+        <v>18</v>
+      </c>
+      <c r="U131">
+        <v>11</v>
+      </c>
+      <c r="V131">
+        <v>29</v>
+      </c>
+      <c r="W131">
+        <v>78</v>
+      </c>
+      <c r="X131">
+        <v>18</v>
+      </c>
+      <c r="Y131">
+        <v>54</v>
+      </c>
+      <c r="Z131">
+        <v>11</v>
+      </c>
+      <c r="AA131">
+        <v>12</v>
+      </c>
+      <c r="AB131">
+        <v>4.42553</v>
+      </c>
+      <c r="AC131">
+        <v>-2.25918</v>
+      </c>
+      <c r="AD131">
+        <v>0</v>
+      </c>
+      <c r="AE131">
+        <v>510.5212</v>
+      </c>
+      <c r="AF131">
+        <v>0</v>
+      </c>
+      <c r="AG131">
+        <v>3</v>
+      </c>
+      <c r="AH131">
+        <v>1858.26333</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B132" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E132">
+        <v>113.163</v>
+      </c>
+      <c r="F132">
+        <v>6279.68</v>
+      </c>
+      <c r="G132">
+        <v>55.49234290359924</v>
+      </c>
+      <c r="H132">
+        <v>144.11</v>
+      </c>
+      <c r="I132">
+        <v>0</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>1.27347277820489</v>
+      </c>
+      <c r="L132">
+        <v>0</v>
+      </c>
+      <c r="M132">
+        <v>0</v>
+      </c>
+      <c r="N132">
+        <v>24.40203</v>
+      </c>
+      <c r="O132">
+        <v>72.41818019943021</v>
+      </c>
+      <c r="P132">
+        <v>33.696</v>
+      </c>
+      <c r="Q132">
+        <v>647.28536</v>
+      </c>
+      <c r="R132">
+        <v>5.719938142325672</v>
+      </c>
+      <c r="S132">
+        <v>882.44998</v>
+      </c>
+      <c r="T132">
+        <v>20</v>
+      </c>
+      <c r="U132">
+        <v>6</v>
+      </c>
+      <c r="V132">
+        <v>26</v>
+      </c>
+      <c r="W132">
+        <v>113</v>
+      </c>
+      <c r="X132">
+        <v>20</v>
+      </c>
+      <c r="Y132">
+        <v>55</v>
+      </c>
+      <c r="Z132">
+        <v>6</v>
+      </c>
+      <c r="AA132">
+        <v>22</v>
+      </c>
+      <c r="AB132">
+        <v>3.90635</v>
+      </c>
+      <c r="AC132">
+        <v>-3.04921</v>
+      </c>
+      <c r="AD132">
+        <v>0</v>
+      </c>
+      <c r="AE132">
+        <v>590.4456</v>
+      </c>
+      <c r="AF132">
+        <v>0</v>
+      </c>
+      <c r="AG132">
+        <v>3</v>
+      </c>
+      <c r="AH132">
+        <v>1941.85608</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B133" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E133">
+        <v>113.163</v>
+      </c>
+      <c r="F133">
+        <v>6758.219999999999</v>
+      </c>
+      <c r="G133">
+        <v>59.72111025688608</v>
+      </c>
+      <c r="H133">
+        <v>242.25</v>
+      </c>
+      <c r="I133">
+        <v>0</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>2.140717372285994</v>
+      </c>
+      <c r="L133">
+        <v>0</v>
+      </c>
+      <c r="M133">
+        <v>0</v>
+      </c>
+      <c r="N133">
+        <v>28.03068</v>
+      </c>
+      <c r="O133">
+        <v>80.10596707818931</v>
+      </c>
+      <c r="P133">
+        <v>34.992</v>
+      </c>
+      <c r="Q133">
+        <v>630.8665599999999</v>
+      </c>
+      <c r="R133">
+        <v>5.574848316145737</v>
+      </c>
+      <c r="S133">
+        <v>831.40002</v>
+      </c>
+      <c r="T133">
+        <v>27</v>
+      </c>
+      <c r="U133">
+        <v>18</v>
+      </c>
+      <c r="V133">
+        <v>45</v>
+      </c>
+      <c r="W133">
+        <v>86</v>
+      </c>
+      <c r="X133">
+        <v>27</v>
+      </c>
+      <c r="Y133">
+        <v>52</v>
+      </c>
+      <c r="Z133">
+        <v>18</v>
+      </c>
+      <c r="AA133">
+        <v>11</v>
+      </c>
+      <c r="AB133">
+        <v>3.88186</v>
+      </c>
+      <c r="AC133">
+        <v>-3.58043</v>
+      </c>
+      <c r="AD133">
+        <v>0</v>
+      </c>
+      <c r="AE133">
+        <v>541.85907</v>
+      </c>
+      <c r="AF133">
+        <v>0</v>
+      </c>
+      <c r="AG133">
+        <v>3</v>
+      </c>
+      <c r="AH133">
+        <v>1892.59968</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B134" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E134">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F134">
+        <v>5702.19</v>
+      </c>
+      <c r="G134">
+        <v>62.09923712616368</v>
+      </c>
+      <c r="H134">
+        <v>82.16999999999999</v>
+      </c>
+      <c r="I134">
+        <v>0</v>
+      </c>
+      <c r="J134">
+        <v>0</v>
+      </c>
+      <c r="K134">
+        <v>0.8948657120609571</v>
+      </c>
+      <c r="L134">
+        <v>0</v>
+      </c>
+      <c r="M134">
+        <v>0</v>
+      </c>
+      <c r="N134">
+        <v>24.89188</v>
+      </c>
+      <c r="O134">
+        <v>71.28258877434135</v>
+      </c>
+      <c r="P134">
+        <v>34.92</v>
+      </c>
+      <c r="Q134">
+        <v>465.95186</v>
+      </c>
+      <c r="R134">
+        <v>5.074410891870847</v>
+      </c>
+      <c r="S134">
+        <v>678.81001</v>
+      </c>
+      <c r="T134">
+        <v>22</v>
+      </c>
+      <c r="U134">
+        <v>5</v>
+      </c>
+      <c r="V134">
+        <v>27</v>
+      </c>
+      <c r="W134">
+        <v>77</v>
+      </c>
+      <c r="X134">
+        <v>22</v>
+      </c>
+      <c r="Y134">
+        <v>40</v>
+      </c>
+      <c r="Z134">
+        <v>5</v>
+      </c>
+      <c r="AA134">
+        <v>9</v>
+      </c>
+      <c r="AB134">
+        <v>4.10547</v>
+      </c>
+      <c r="AC134">
+        <v>-2.40479</v>
+      </c>
+      <c r="AD134">
+        <v>0</v>
+      </c>
+      <c r="AE134">
+        <v>528.1104</v>
+      </c>
+      <c r="AF134">
+        <v>0</v>
+      </c>
+      <c r="AG134">
+        <v>3</v>
+      </c>
+      <c r="AH134">
+        <v>1397.85558</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B135" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E135">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F135">
+        <v>5959.490000000001</v>
+      </c>
+      <c r="G135">
+        <v>64.90134188110204</v>
+      </c>
+      <c r="H135">
+        <v>238.23</v>
+      </c>
+      <c r="I135">
+        <v>0</v>
+      </c>
+      <c r="J135">
+        <v>0</v>
+      </c>
+      <c r="K135">
+        <v>2.59442446859294</v>
+      </c>
+      <c r="L135">
+        <v>0</v>
+      </c>
+      <c r="M135">
+        <v>0</v>
+      </c>
+      <c r="N135">
+        <v>25.41771</v>
+      </c>
+      <c r="O135">
+        <v>72.63863168724281</v>
+      </c>
+      <c r="P135">
+        <v>34.992</v>
+      </c>
+      <c r="Q135">
+        <v>504.51436</v>
+      </c>
+      <c r="R135">
+        <v>5.49437266650089</v>
+      </c>
+      <c r="S135">
+        <v>1015.70998</v>
+      </c>
+      <c r="T135">
+        <v>22</v>
+      </c>
+      <c r="U135">
+        <v>22</v>
+      </c>
+      <c r="V135">
+        <v>44</v>
+      </c>
+      <c r="W135">
+        <v>92</v>
+      </c>
+      <c r="X135">
+        <v>22</v>
+      </c>
+      <c r="Y135">
+        <v>58</v>
+      </c>
+      <c r="Z135">
+        <v>22</v>
+      </c>
+      <c r="AA135">
+        <v>7</v>
+      </c>
+      <c r="AB135">
+        <v>4.12258</v>
+      </c>
+      <c r="AC135">
+        <v>-2.41991</v>
+      </c>
+      <c r="AD135">
+        <v>0</v>
+      </c>
+      <c r="AE135">
+        <v>500.63307</v>
+      </c>
+      <c r="AF135">
+        <v>0</v>
+      </c>
+      <c r="AG135">
+        <v>3</v>
+      </c>
+      <c r="AH135">
+        <v>1513.54308</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B136" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E136">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F136">
+        <v>5319.16</v>
+      </c>
+      <c r="G136">
+        <v>57.92788001662603</v>
+      </c>
+      <c r="H136">
+        <v>47.73999999999999</v>
+      </c>
+      <c r="I136">
+        <v>0</v>
+      </c>
+      <c r="J136">
+        <v>0</v>
+      </c>
+      <c r="K136">
+        <v>0.519908593084947</v>
+      </c>
+      <c r="L136">
+        <v>0</v>
+      </c>
+      <c r="M136">
+        <v>0</v>
+      </c>
+      <c r="N136">
+        <v>23.71702</v>
+      </c>
+      <c r="O136">
+        <v>69.78878295668551</v>
+      </c>
+      <c r="P136">
+        <v>33.984</v>
+      </c>
+      <c r="Q136">
+        <v>527.20625</v>
+      </c>
+      <c r="R136">
+        <v>5.741496851761434</v>
+      </c>
+      <c r="S136">
+        <v>527.57001</v>
+      </c>
+      <c r="T136">
+        <v>11</v>
+      </c>
+      <c r="U136">
+        <v>11</v>
+      </c>
+      <c r="V136">
+        <v>22</v>
+      </c>
+      <c r="W136">
+        <v>43</v>
+      </c>
+      <c r="X136">
+        <v>11</v>
+      </c>
+      <c r="Y136">
+        <v>37</v>
+      </c>
+      <c r="Z136">
+        <v>11</v>
+      </c>
+      <c r="AA136">
+        <v>17</v>
+      </c>
+      <c r="AB136">
+        <v>4.03017</v>
+      </c>
+      <c r="AC136">
+        <v>-2.70483</v>
+      </c>
+      <c r="AD136">
+        <v>0</v>
+      </c>
+      <c r="AE136">
+        <v>485.7496</v>
+      </c>
+      <c r="AF136">
+        <v>0</v>
+      </c>
+      <c r="AG136">
+        <v>3</v>
+      </c>
+      <c r="AH136">
+        <v>1581.61875</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B137" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E137">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F137">
+        <v>5793.08</v>
+      </c>
+      <c r="G137">
+        <v>63.08906729008263</v>
+      </c>
+      <c r="H137">
+        <v>128.42</v>
+      </c>
+      <c r="I137">
+        <v>0</v>
+      </c>
+      <c r="J137">
+        <v>0</v>
+      </c>
+      <c r="K137">
+        <v>1.398547581147233</v>
+      </c>
+      <c r="L137">
+        <v>0</v>
+      </c>
+      <c r="M137">
+        <v>0</v>
+      </c>
+      <c r="N137">
+        <v>27.06962</v>
+      </c>
+      <c r="O137">
+        <v>77.35945358939188</v>
+      </c>
+      <c r="P137">
+        <v>34.992</v>
+      </c>
+      <c r="Q137">
+        <v>565.3764200000001</v>
+      </c>
+      <c r="R137">
+        <v>6.157185988387184</v>
+      </c>
+      <c r="S137">
+        <v>916.58998</v>
+      </c>
+      <c r="T137">
+        <v>7</v>
+      </c>
+      <c r="U137">
+        <v>15</v>
+      </c>
+      <c r="V137">
+        <v>22</v>
+      </c>
+      <c r="W137">
+        <v>86</v>
+      </c>
+      <c r="X137">
+        <v>7</v>
+      </c>
+      <c r="Y137">
+        <v>58</v>
+      </c>
+      <c r="Z137">
+        <v>15</v>
+      </c>
+      <c r="AA137">
+        <v>19</v>
+      </c>
+      <c r="AB137">
+        <v>3.68433</v>
+      </c>
+      <c r="AC137">
+        <v>-3.08386</v>
+      </c>
+      <c r="AD137">
+        <v>0</v>
+      </c>
+      <c r="AE137">
+        <v>543.8056</v>
+      </c>
+      <c r="AF137">
+        <v>0</v>
+      </c>
+      <c r="AG137">
+        <v>3</v>
+      </c>
+      <c r="AH137">
+        <v>1696.12926</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B138" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E138">
+        <v>91.82383333333334</v>
+      </c>
+      <c r="F138">
+        <v>5327.23</v>
+      </c>
+      <c r="G138">
+        <v>58.01576569626985</v>
+      </c>
+      <c r="H138">
+        <v>69.39</v>
+      </c>
+      <c r="I138">
+        <v>0</v>
+      </c>
+      <c r="J138">
+        <v>0</v>
+      </c>
+      <c r="K138">
+        <v>0.7556861599112793</v>
+      </c>
+      <c r="L138">
+        <v>0</v>
+      </c>
+      <c r="M138">
+        <v>0</v>
+      </c>
+      <c r="N138">
+        <v>23.28645</v>
+      </c>
+      <c r="O138">
+        <v>70.53934932751727</v>
+      </c>
+      <c r="P138">
+        <v>33.012</v>
+      </c>
+      <c r="Q138">
+        <v>552.48181</v>
+      </c>
+      <c r="R138">
+        <v>6.016758285339862</v>
+      </c>
+      <c r="S138">
+        <v>705.61</v>
+      </c>
+      <c r="T138">
+        <v>10</v>
+      </c>
+      <c r="U138">
+        <v>15</v>
+      </c>
+      <c r="V138">
+        <v>25</v>
+      </c>
+      <c r="W138">
+        <v>77</v>
+      </c>
+      <c r="X138">
+        <v>10</v>
+      </c>
+      <c r="Y138">
+        <v>57</v>
+      </c>
+      <c r="Z138">
+        <v>15</v>
+      </c>
+      <c r="AA138">
+        <v>8</v>
+      </c>
+      <c r="AB138">
+        <v>3.85905</v>
+      </c>
+      <c r="AC138">
+        <v>-2.34054</v>
+      </c>
+      <c r="AD138">
+        <v>0</v>
+      </c>
+      <c r="AE138">
+        <v>462.03075</v>
+      </c>
+      <c r="AF138">
+        <v>0</v>
+      </c>
+      <c r="AG138">
+        <v>3</v>
+      </c>
+      <c r="AH138">
+        <v>1657.44543</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B139" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E139">
+        <v>113.163</v>
+      </c>
+      <c r="F139">
+        <v>6046.12</v>
+      </c>
+      <c r="G139">
+        <v>53.42841741558637</v>
+      </c>
+      <c r="H139">
+        <v>73.61999999999999</v>
+      </c>
+      <c r="I139">
+        <v>0</v>
+      </c>
+      <c r="J139">
+        <v>0</v>
+      </c>
+      <c r="K139">
+        <v>0.6505659977201028</v>
+      </c>
+      <c r="L139">
+        <v>0</v>
+      </c>
+      <c r="M139">
+        <v>0</v>
+      </c>
+      <c r="N139">
+        <v>25.79919</v>
+      </c>
+      <c r="O139">
+        <v>80.61239220097488</v>
+      </c>
+      <c r="P139">
+        <v>32.004</v>
+      </c>
+      <c r="Q139">
+        <v>609.1166899999999</v>
+      </c>
+      <c r="R139">
+        <v>5.382648833982839</v>
+      </c>
+      <c r="S139">
+        <v>719.31999</v>
+      </c>
+      <c r="T139">
+        <v>15</v>
+      </c>
+      <c r="U139">
+        <v>5</v>
+      </c>
+      <c r="V139">
+        <v>20</v>
+      </c>
+      <c r="W139">
+        <v>96</v>
+      </c>
+      <c r="X139">
+        <v>15</v>
+      </c>
+      <c r="Y139">
+        <v>46</v>
+      </c>
+      <c r="Z139">
+        <v>5</v>
+      </c>
+      <c r="AA139">
+        <v>21</v>
+      </c>
+      <c r="AB139">
+        <v>3.96358</v>
+      </c>
+      <c r="AC139">
+        <v>-2.29472</v>
+      </c>
+      <c r="AD139">
+        <v>0</v>
+      </c>
+      <c r="AE139">
+        <v>489.3574</v>
+      </c>
+      <c r="AF139">
+        <v>0</v>
+      </c>
+      <c r="AG139">
+        <v>3</v>
+      </c>
+      <c r="AH139">
+        <v>1827.35007</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B140" s="2">
+        <v>46191</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Sesión 6 18 jun PM</t>
+        </is>
+      </c>
+      <c r="E140">
+        <v>60.53416666666667</v>
+      </c>
+      <c r="F140">
+        <v>2502.35</v>
+      </c>
+      <c r="G140">
+        <v>41.33781197946063</v>
+      </c>
+      <c r="H140">
+        <v>0</v>
+      </c>
+      <c r="I140">
+        <v>0</v>
+      </c>
+      <c r="J140">
+        <v>0</v>
+      </c>
+      <c r="K140">
+        <v>0</v>
+      </c>
+      <c r="L140">
+        <v>0</v>
+      </c>
+      <c r="M140">
+        <v>0</v>
+      </c>
+      <c r="N140">
+        <v>18.82284</v>
+      </c>
+      <c r="O140">
+        <v>52.28566666666666</v>
+      </c>
+      <c r="P140">
+        <v>36</v>
+      </c>
+      <c r="Q140">
+        <v>273.71852</v>
+      </c>
+      <c r="R140">
+        <v>4.521719469720956</v>
+      </c>
+      <c r="S140">
+        <v>166.83</v>
+      </c>
+      <c r="T140">
+        <v>4</v>
+      </c>
+      <c r="U140">
+        <v>0</v>
+      </c>
+      <c r="V140">
+        <v>4</v>
+      </c>
+      <c r="W140">
+        <v>33</v>
+      </c>
+      <c r="X140">
+        <v>4</v>
+      </c>
+      <c r="Y140">
+        <v>10</v>
+      </c>
+      <c r="Z140">
+        <v>0</v>
+      </c>
+      <c r="AA140">
+        <v>7</v>
+      </c>
+      <c r="AB140">
+        <v>4.04672</v>
+      </c>
+      <c r="AC140">
+        <v>-2.44381</v>
+      </c>
+      <c r="AD140">
+        <v>0</v>
+      </c>
+      <c r="AE140">
+        <v>195.9433</v>
+      </c>
+      <c r="AF140">
+        <v>0</v>
+      </c>
+      <c r="AG140">
+        <v>3</v>
+      </c>
+      <c r="AH140">
+        <v>821.15556</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B141" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E141">
+        <v>101</v>
+      </c>
+      <c r="F141">
+        <v>4422.52</v>
+      </c>
+      <c r="G141">
+        <v>43.78732673267326</v>
+      </c>
+      <c r="H141">
+        <v>57.31</v>
+      </c>
+      <c r="I141">
+        <v>0</v>
+      </c>
+      <c r="J141">
+        <v>0</v>
+      </c>
+      <c r="K141">
+        <v>0.5674257425742575</v>
+      </c>
+      <c r="L141">
+        <v>0</v>
+      </c>
+      <c r="M141">
+        <v>0</v>
+      </c>
+      <c r="N141">
+        <v>24.22245</v>
+      </c>
+      <c r="O141">
+        <v>74.84380793474232</v>
+      </c>
+      <c r="P141">
+        <v>32.364</v>
+      </c>
+      <c r="Q141">
+        <v>515.62801</v>
+      </c>
+      <c r="R141">
+        <v>5.105227821782178</v>
+      </c>
+      <c r="S141">
+        <v>493.04</v>
+      </c>
+      <c r="T141">
+        <v>12</v>
+      </c>
+      <c r="U141">
+        <v>14</v>
+      </c>
+      <c r="V141">
+        <v>26</v>
+      </c>
+      <c r="W141">
+        <v>79</v>
+      </c>
+      <c r="X141">
+        <v>12</v>
+      </c>
+      <c r="Y141">
+        <v>61</v>
+      </c>
+      <c r="Z141">
+        <v>14</v>
+      </c>
+      <c r="AA141">
+        <v>39</v>
+      </c>
+      <c r="AB141">
+        <v>3.73904</v>
+      </c>
+      <c r="AC141">
+        <v>-1.17353</v>
+      </c>
+      <c r="AD141">
+        <v>0</v>
+      </c>
+      <c r="AE141">
+        <v>368.27</v>
+      </c>
+      <c r="AF141">
+        <v>0</v>
+      </c>
+      <c r="AG141">
+        <v>3</v>
+      </c>
+      <c r="AH141">
+        <v>1546.88403</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B142" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E142">
+        <v>101</v>
+      </c>
+      <c r="F142">
+        <v>4400.25</v>
+      </c>
+      <c r="G142">
+        <v>43.56683168316832</v>
+      </c>
+      <c r="H142">
+        <v>79.13000000000001</v>
+      </c>
+      <c r="I142">
+        <v>0</v>
+      </c>
+      <c r="J142">
+        <v>0</v>
+      </c>
+      <c r="K142">
+        <v>0.7834653465346536</v>
+      </c>
+      <c r="L142">
+        <v>0</v>
+      </c>
+      <c r="M142">
+        <v>0</v>
+      </c>
+      <c r="N142">
+        <v>28.46455</v>
+      </c>
+      <c r="O142">
+        <v>87.85354938271604</v>
+      </c>
+      <c r="P142">
+        <v>32.4</v>
+      </c>
+      <c r="Q142">
+        <v>598.2261699999999</v>
+      </c>
+      <c r="R142">
+        <v>5.923031386138613</v>
+      </c>
+      <c r="S142">
+        <v>617.22999</v>
+      </c>
+      <c r="T142">
+        <v>32</v>
+      </c>
+      <c r="U142">
+        <v>28</v>
+      </c>
+      <c r="V142">
+        <v>60</v>
+      </c>
+      <c r="W142">
+        <v>110</v>
+      </c>
+      <c r="X142">
+        <v>32</v>
+      </c>
+      <c r="Y142">
+        <v>93</v>
+      </c>
+      <c r="Z142">
+        <v>28</v>
+      </c>
+      <c r="AA142">
+        <v>24</v>
+      </c>
+      <c r="AB142">
+        <v>3.89857</v>
+      </c>
+      <c r="AC142">
+        <v>-1.03831</v>
+      </c>
+      <c r="AD142">
+        <v>0</v>
+      </c>
+      <c r="AE142">
+        <v>371.9037</v>
+      </c>
+      <c r="AF142">
+        <v>0</v>
+      </c>
+      <c r="AG142">
+        <v>3</v>
+      </c>
+      <c r="AH142">
+        <v>1794.67851</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B143" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E143">
+        <v>101</v>
+      </c>
+      <c r="F143">
+        <v>4227.74</v>
+      </c>
+      <c r="G143">
+        <v>41.85881188118812</v>
+      </c>
+      <c r="H143">
+        <v>87.95999999999999</v>
+      </c>
+      <c r="I143">
+        <v>0</v>
+      </c>
+      <c r="J143">
+        <v>0</v>
+      </c>
+      <c r="K143">
+        <v>0.8708910891089108</v>
+      </c>
+      <c r="L143">
+        <v>0</v>
+      </c>
+      <c r="M143">
+        <v>0</v>
+      </c>
+      <c r="N143">
+        <v>27.58086</v>
+      </c>
+      <c r="O143">
+        <v>81.15836864406779</v>
+      </c>
+      <c r="P143">
+        <v>33.984</v>
+      </c>
+      <c r="Q143">
+        <v>591.91333</v>
+      </c>
+      <c r="R143">
+        <v>5.86052801980198</v>
+      </c>
+      <c r="S143">
+        <v>437.77</v>
+      </c>
+      <c r="T143">
+        <v>15</v>
+      </c>
+      <c r="U143">
+        <v>9</v>
+      </c>
+      <c r="V143">
+        <v>24</v>
+      </c>
+      <c r="W143">
+        <v>66</v>
+      </c>
+      <c r="X143">
+        <v>15</v>
+      </c>
+      <c r="Y143">
+        <v>60</v>
+      </c>
+      <c r="Z143">
+        <v>9</v>
+      </c>
+      <c r="AA143">
+        <v>14</v>
+      </c>
+      <c r="AB143">
+        <v>4.06104</v>
+      </c>
+      <c r="AC143">
+        <v>-1.34036</v>
+      </c>
+      <c r="AD143">
+        <v>0</v>
+      </c>
+      <c r="AE143">
+        <v>390.016</v>
+      </c>
+      <c r="AF143">
+        <v>0</v>
+      </c>
+      <c r="AG143">
+        <v>3</v>
+      </c>
+      <c r="AH143">
+        <v>1775.73999</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Dagoberto Espinoza</t>
+        </is>
+      </c>
+      <c r="B144" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E144">
+        <v>101</v>
+      </c>
+      <c r="F144">
+        <v>5713.3</v>
+      </c>
+      <c r="G144">
+        <v>56.56732673267327</v>
+      </c>
+      <c r="H144">
+        <v>72</v>
+      </c>
+      <c r="I144">
+        <v>0</v>
+      </c>
+      <c r="J144">
+        <v>0</v>
+      </c>
+      <c r="K144">
+        <v>0.7128712871287128</v>
+      </c>
+      <c r="L144">
+        <v>0</v>
+      </c>
+      <c r="M144">
+        <v>0</v>
+      </c>
+      <c r="N144">
+        <v>27.68428</v>
+      </c>
+      <c r="O144">
+        <v>77.83479532163744</v>
+      </c>
+      <c r="P144">
+        <v>35.568</v>
+      </c>
+      <c r="Q144">
+        <v>609.02973</v>
+      </c>
+      <c r="R144">
+        <v>6.029997326732673</v>
+      </c>
+      <c r="S144">
+        <v>779.60998</v>
+      </c>
+      <c r="T144">
+        <v>44</v>
+      </c>
+      <c r="U144">
+        <v>51</v>
+      </c>
+      <c r="V144">
+        <v>95</v>
+      </c>
+      <c r="W144">
+        <v>137</v>
+      </c>
+      <c r="X144">
+        <v>44</v>
+      </c>
+      <c r="Y144">
+        <v>124</v>
+      </c>
+      <c r="Z144">
+        <v>51</v>
+      </c>
+      <c r="AA144">
+        <v>38</v>
+      </c>
+      <c r="AB144">
+        <v>4.27888</v>
+      </c>
+      <c r="AC144">
+        <v>-1.21086</v>
+      </c>
+      <c r="AD144">
+        <v>0</v>
+      </c>
+      <c r="AE144">
+        <v>567.1967999999999</v>
+      </c>
+      <c r="AF144">
+        <v>0</v>
+      </c>
+      <c r="AG144">
+        <v>3</v>
+      </c>
+      <c r="AH144">
+        <v>1827.08919</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B145" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E145">
+        <v>101</v>
+      </c>
+      <c r="F145">
+        <v>4515.04</v>
+      </c>
+      <c r="G145">
+        <v>44.70336633663366</v>
+      </c>
+      <c r="H145">
+        <v>113.31</v>
+      </c>
+      <c r="I145">
+        <v>0</v>
+      </c>
+      <c r="J145">
+        <v>0</v>
+      </c>
+      <c r="K145">
+        <v>1.121881188118812</v>
+      </c>
+      <c r="L145">
+        <v>0</v>
+      </c>
+      <c r="M145">
+        <v>0</v>
+      </c>
+      <c r="N145">
+        <v>28.88958</v>
+      </c>
+      <c r="O145">
+        <v>80.24883333333332</v>
+      </c>
+      <c r="P145">
+        <v>36</v>
+      </c>
+      <c r="Q145">
+        <v>495.78647</v>
+      </c>
+      <c r="R145">
+        <v>4.90877693069307</v>
+      </c>
+      <c r="S145">
+        <v>584.14</v>
+      </c>
+      <c r="T145">
+        <v>29</v>
+      </c>
+      <c r="U145">
+        <v>31</v>
+      </c>
+      <c r="V145">
+        <v>60</v>
+      </c>
+      <c r="W145">
+        <v>88</v>
+      </c>
+      <c r="X145">
+        <v>29</v>
+      </c>
+      <c r="Y145">
+        <v>81</v>
+      </c>
+      <c r="Z145">
+        <v>31</v>
+      </c>
+      <c r="AA145">
+        <v>28</v>
+      </c>
+      <c r="AB145">
+        <v>4.38661</v>
+      </c>
+      <c r="AC145">
+        <v>-1.10536</v>
+      </c>
+      <c r="AD145">
+        <v>0</v>
+      </c>
+      <c r="AE145">
+        <v>382.5689</v>
+      </c>
+      <c r="AF145">
+        <v>0</v>
+      </c>
+      <c r="AG145">
+        <v>3</v>
+      </c>
+      <c r="AH145">
+        <v>1487.35941</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B146" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E146">
+        <v>101</v>
+      </c>
+      <c r="F146">
+        <v>4108.09</v>
+      </c>
+      <c r="G146">
+        <v>40.67415841584159</v>
+      </c>
+      <c r="H146">
+        <v>16.26</v>
+      </c>
+      <c r="I146">
+        <v>0</v>
+      </c>
+      <c r="J146">
+        <v>0</v>
+      </c>
+      <c r="K146">
+        <v>0.160990099009901</v>
+      </c>
+      <c r="L146">
+        <v>0</v>
+      </c>
+      <c r="M146">
+        <v>0</v>
+      </c>
+      <c r="N146">
+        <v>22.67776</v>
+      </c>
+      <c r="O146">
+        <v>70.85914260717411</v>
+      </c>
+      <c r="P146">
+        <v>32.004</v>
+      </c>
+      <c r="Q146">
+        <v>514.32473</v>
+      </c>
+      <c r="R146">
+        <v>5.092324059405941</v>
+      </c>
+      <c r="S146">
+        <v>334.19</v>
+      </c>
+      <c r="T146">
+        <v>15</v>
+      </c>
+      <c r="U146">
+        <v>28</v>
+      </c>
+      <c r="V146">
+        <v>43</v>
+      </c>
+      <c r="W146">
+        <v>71</v>
+      </c>
+      <c r="X146">
+        <v>15</v>
+      </c>
+      <c r="Y146">
+        <v>65</v>
+      </c>
+      <c r="Z146">
+        <v>28</v>
+      </c>
+      <c r="AA146">
+        <v>67</v>
+      </c>
+      <c r="AB146">
+        <v>4.24167</v>
+      </c>
+      <c r="AC146">
+        <v>-1.95064</v>
+      </c>
+      <c r="AD146">
+        <v>0</v>
+      </c>
+      <c r="AE146">
+        <v>281.9346</v>
+      </c>
+      <c r="AF146">
+        <v>0</v>
+      </c>
+      <c r="AG146">
+        <v>3</v>
+      </c>
+      <c r="AH146">
+        <v>1542.97419</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B147" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E147">
+        <v>101</v>
+      </c>
+      <c r="F147">
+        <v>5114.7</v>
+      </c>
+      <c r="G147">
+        <v>50.64059405940594</v>
+      </c>
+      <c r="H147">
+        <v>150.17</v>
+      </c>
+      <c r="I147">
+        <v>0</v>
+      </c>
+      <c r="J147">
+        <v>0</v>
+      </c>
+      <c r="K147">
+        <v>1.486831683168317</v>
+      </c>
+      <c r="L147">
+        <v>15.06</v>
+      </c>
+      <c r="M147">
+        <v>1</v>
+      </c>
+      <c r="N147">
+        <v>30.46936</v>
+      </c>
+      <c r="O147">
+        <v>90.03947990543735</v>
+      </c>
+      <c r="P147">
+        <v>33.84</v>
+      </c>
+      <c r="Q147">
+        <v>593.20456</v>
+      </c>
+      <c r="R147">
+        <v>5.873312475247525</v>
+      </c>
+      <c r="S147">
+        <v>769.60998</v>
+      </c>
+      <c r="T147">
+        <v>45</v>
+      </c>
+      <c r="U147">
+        <v>45</v>
+      </c>
+      <c r="V147">
+        <v>90</v>
+      </c>
+      <c r="W147">
+        <v>115</v>
+      </c>
+      <c r="X147">
+        <v>45</v>
+      </c>
+      <c r="Y147">
+        <v>100</v>
+      </c>
+      <c r="Z147">
+        <v>45</v>
+      </c>
+      <c r="AA147">
+        <v>59</v>
+      </c>
+      <c r="AB147">
+        <v>4.26681</v>
+      </c>
+      <c r="AC147">
+        <v>-1.4227</v>
+      </c>
+      <c r="AD147">
+        <v>0</v>
+      </c>
+      <c r="AE147">
+        <v>444.3383</v>
+      </c>
+      <c r="AF147">
+        <v>0</v>
+      </c>
+      <c r="AG147">
+        <v>3</v>
+      </c>
+      <c r="AH147">
+        <v>1779.61368</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B148" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E148">
+        <v>101</v>
+      </c>
+      <c r="F148">
+        <v>5114.150000000001</v>
+      </c>
+      <c r="G148">
+        <v>50.63514851485149</v>
+      </c>
+      <c r="H148">
+        <v>59.50000000000001</v>
+      </c>
+      <c r="I148">
+        <v>0</v>
+      </c>
+      <c r="J148">
+        <v>0</v>
+      </c>
+      <c r="K148">
+        <v>0.5891089108910892</v>
+      </c>
+      <c r="L148">
+        <v>0</v>
+      </c>
+      <c r="M148">
+        <v>0</v>
+      </c>
+      <c r="N148">
+        <v>24.76522</v>
+      </c>
+      <c r="O148">
+        <v>73.4960232668566</v>
+      </c>
+      <c r="P148">
+        <v>33.696</v>
+      </c>
+      <c r="Q148">
+        <v>589.86017</v>
+      </c>
+      <c r="R148">
+        <v>5.840199702970297</v>
+      </c>
+      <c r="S148">
+        <v>655.76</v>
+      </c>
+      <c r="T148">
+        <v>36</v>
+      </c>
+      <c r="U148">
+        <v>41</v>
+      </c>
+      <c r="V148">
+        <v>77</v>
+      </c>
+      <c r="W148">
+        <v>128</v>
+      </c>
+      <c r="X148">
+        <v>36</v>
+      </c>
+      <c r="Y148">
+        <v>116</v>
+      </c>
+      <c r="Z148">
+        <v>41</v>
+      </c>
+      <c r="AA148">
+        <v>43</v>
+      </c>
+      <c r="AB148">
+        <v>4.23286</v>
+      </c>
+      <c r="AC148">
+        <v>-1.50173</v>
+      </c>
+      <c r="AD148">
+        <v>0</v>
+      </c>
+      <c r="AE148">
+        <v>499.608</v>
+      </c>
+      <c r="AF148">
+        <v>0</v>
+      </c>
+      <c r="AG148">
+        <v>3</v>
+      </c>
+      <c r="AH148">
+        <v>1769.58051</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B149" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E149">
+        <v>101</v>
+      </c>
+      <c r="F149">
+        <v>4655.98</v>
+      </c>
+      <c r="G149">
+        <v>46.09881188118811</v>
+      </c>
+      <c r="H149">
+        <v>84.10000000000001</v>
+      </c>
+      <c r="I149">
+        <v>0</v>
+      </c>
+      <c r="J149">
+        <v>0</v>
+      </c>
+      <c r="K149">
+        <v>0.8326732673267327</v>
+      </c>
+      <c r="L149">
+        <v>0</v>
+      </c>
+      <c r="M149">
+        <v>0</v>
+      </c>
+      <c r="N149">
+        <v>25.52001</v>
+      </c>
+      <c r="O149">
+        <v>72.93098422496571</v>
+      </c>
+      <c r="P149">
+        <v>34.992</v>
+      </c>
+      <c r="Q149">
+        <v>503.99442</v>
+      </c>
+      <c r="R149">
+        <v>4.990043762376238</v>
+      </c>
+      <c r="S149">
+        <v>613.22</v>
+      </c>
+      <c r="T149">
+        <v>30</v>
+      </c>
+      <c r="U149">
+        <v>34</v>
+      </c>
+      <c r="V149">
+        <v>64</v>
+      </c>
+      <c r="W149">
+        <v>101</v>
+      </c>
+      <c r="X149">
+        <v>30</v>
+      </c>
+      <c r="Y149">
+        <v>91</v>
+      </c>
+      <c r="Z149">
+        <v>34</v>
+      </c>
+      <c r="AA149">
+        <v>27</v>
+      </c>
+      <c r="AB149">
+        <v>4.44872</v>
+      </c>
+      <c r="AC149">
+        <v>-0.87904</v>
+      </c>
+      <c r="AD149">
+        <v>0</v>
+      </c>
+      <c r="AE149">
+        <v>386.11641</v>
+      </c>
+      <c r="AF149">
+        <v>0</v>
+      </c>
+      <c r="AG149">
+        <v>3</v>
+      </c>
+      <c r="AH149">
+        <v>1511.98326</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B150" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E150">
+        <v>101</v>
+      </c>
+      <c r="F150">
+        <v>4824.73</v>
+      </c>
+      <c r="G150">
+        <v>47.76960396039603</v>
+      </c>
+      <c r="H150">
+        <v>57.88</v>
+      </c>
+      <c r="I150">
+        <v>0</v>
+      </c>
+      <c r="J150">
+        <v>0</v>
+      </c>
+      <c r="K150">
+        <v>0.5730693069306931</v>
+      </c>
+      <c r="L150">
+        <v>0</v>
+      </c>
+      <c r="M150">
+        <v>0</v>
+      </c>
+      <c r="N150">
+        <v>23.05072</v>
+      </c>
+      <c r="O150">
+        <v>66.01008018327606</v>
+      </c>
+      <c r="P150">
+        <v>34.92</v>
+      </c>
+      <c r="Q150">
+        <v>461.31373</v>
+      </c>
+      <c r="R150">
+        <v>4.567462673267326</v>
+      </c>
+      <c r="S150">
+        <v>482.92</v>
+      </c>
+      <c r="T150">
+        <v>24</v>
+      </c>
+      <c r="U150">
+        <v>14</v>
+      </c>
+      <c r="V150">
+        <v>38</v>
+      </c>
+      <c r="W150">
+        <v>72</v>
+      </c>
+      <c r="X150">
+        <v>24</v>
+      </c>
+      <c r="Y150">
+        <v>67</v>
+      </c>
+      <c r="Z150">
+        <v>14</v>
+      </c>
+      <c r="AA150">
+        <v>24</v>
+      </c>
+      <c r="AB150">
+        <v>3.81153</v>
+      </c>
+      <c r="AC150">
+        <v>-1.5841</v>
+      </c>
+      <c r="AD150">
+        <v>0</v>
+      </c>
+      <c r="AE150">
+        <v>446.0504</v>
+      </c>
+      <c r="AF150">
+        <v>0</v>
+      </c>
+      <c r="AG150">
+        <v>3</v>
+      </c>
+      <c r="AH150">
+        <v>1383.94119</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B151" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E151">
+        <v>101</v>
+      </c>
+      <c r="F151">
+        <v>4728.51</v>
+      </c>
+      <c r="G151">
+        <v>46.81693069306931</v>
+      </c>
+      <c r="H151">
+        <v>93.34</v>
+      </c>
+      <c r="I151">
+        <v>0</v>
+      </c>
+      <c r="J151">
+        <v>0</v>
+      </c>
+      <c r="K151">
+        <v>0.9241584158415842</v>
+      </c>
+      <c r="L151">
+        <v>0</v>
+      </c>
+      <c r="M151">
+        <v>0</v>
+      </c>
+      <c r="N151">
+        <v>26.12775</v>
+      </c>
+      <c r="O151">
+        <v>74.66778120713306</v>
+      </c>
+      <c r="P151">
+        <v>34.992</v>
+      </c>
+      <c r="Q151">
+        <v>500.97208</v>
+      </c>
+      <c r="R151">
+        <v>4.960119603960396</v>
+      </c>
+      <c r="S151">
+        <v>654.3700100000001</v>
+      </c>
+      <c r="T151">
+        <v>25</v>
+      </c>
+      <c r="U151">
+        <v>23</v>
+      </c>
+      <c r="V151">
+        <v>48</v>
+      </c>
+      <c r="W151">
+        <v>101</v>
+      </c>
+      <c r="X151">
+        <v>25</v>
+      </c>
+      <c r="Y151">
+        <v>83</v>
+      </c>
+      <c r="Z151">
+        <v>23</v>
+      </c>
+      <c r="AA151">
+        <v>54</v>
+      </c>
+      <c r="AB151">
+        <v>3.91968</v>
+      </c>
+      <c r="AC151">
+        <v>-1.71894</v>
+      </c>
+      <c r="AD151">
+        <v>0</v>
+      </c>
+      <c r="AE151">
+        <v>410.61714</v>
+      </c>
+      <c r="AF151">
+        <v>0</v>
+      </c>
+      <c r="AG151">
+        <v>3</v>
+      </c>
+      <c r="AH151">
+        <v>1502.91624</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B152" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E152">
+        <v>101</v>
+      </c>
+      <c r="F152">
+        <v>4161.61</v>
+      </c>
+      <c r="G152">
+        <v>41.20405940594059</v>
+      </c>
+      <c r="H152">
+        <v>52.45</v>
+      </c>
+      <c r="I152">
+        <v>0</v>
+      </c>
+      <c r="J152">
+        <v>0</v>
+      </c>
+      <c r="K152">
+        <v>0.5193069306930693</v>
+      </c>
+      <c r="L152">
+        <v>0</v>
+      </c>
+      <c r="M152">
+        <v>0</v>
+      </c>
+      <c r="N152">
+        <v>24.8696</v>
+      </c>
+      <c r="O152">
+        <v>73.18032015065913</v>
+      </c>
+      <c r="P152">
+        <v>33.984</v>
+      </c>
+      <c r="Q152">
+        <v>502.61805</v>
+      </c>
+      <c r="R152">
+        <v>4.976416336633664</v>
+      </c>
+      <c r="S152">
+        <v>378.56</v>
+      </c>
+      <c r="T152">
+        <v>11</v>
+      </c>
+      <c r="U152">
+        <v>15</v>
+      </c>
+      <c r="V152">
+        <v>26</v>
+      </c>
+      <c r="W152">
+        <v>61</v>
+      </c>
+      <c r="X152">
+        <v>11</v>
+      </c>
+      <c r="Y152">
+        <v>54</v>
+      </c>
+      <c r="Z152">
+        <v>15</v>
+      </c>
+      <c r="AA152">
+        <v>47</v>
+      </c>
+      <c r="AB152">
+        <v>3.43314</v>
+      </c>
+      <c r="AC152">
+        <v>-1.06918</v>
+      </c>
+      <c r="AD152">
+        <v>0</v>
+      </c>
+      <c r="AE152">
+        <v>391.4728</v>
+      </c>
+      <c r="AF152">
+        <v>0</v>
+      </c>
+      <c r="AG152">
+        <v>3</v>
+      </c>
+      <c r="AH152">
+        <v>1507.85415</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B153" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E153">
+        <v>101</v>
+      </c>
+      <c r="F153">
+        <v>4725.58</v>
+      </c>
+      <c r="G153">
+        <v>46.78792079207921</v>
+      </c>
+      <c r="H153">
+        <v>89.11999999999999</v>
+      </c>
+      <c r="I153">
+        <v>0</v>
+      </c>
+      <c r="J153">
+        <v>0</v>
+      </c>
+      <c r="K153">
+        <v>0.8823762376237623</v>
+      </c>
+      <c r="L153">
+        <v>0</v>
+      </c>
+      <c r="M153">
+        <v>0</v>
+      </c>
+      <c r="N153">
+        <v>26.27495</v>
+      </c>
+      <c r="O153">
+        <v>75.08844878829447</v>
+      </c>
+      <c r="P153">
+        <v>34.992</v>
+      </c>
+      <c r="Q153">
+        <v>577.27973</v>
+      </c>
+      <c r="R153">
+        <v>5.715640891089109</v>
+      </c>
+      <c r="S153">
+        <v>737.05999</v>
+      </c>
+      <c r="T153">
+        <v>31</v>
+      </c>
+      <c r="U153">
+        <v>24</v>
+      </c>
+      <c r="V153">
+        <v>55</v>
+      </c>
+      <c r="W153">
+        <v>119</v>
+      </c>
+      <c r="X153">
+        <v>31</v>
+      </c>
+      <c r="Y153">
+        <v>100</v>
+      </c>
+      <c r="Z153">
+        <v>24</v>
+      </c>
+      <c r="AA153">
+        <v>42</v>
+      </c>
+      <c r="AB153">
+        <v>4.15186</v>
+      </c>
+      <c r="AC153">
+        <v>-1.76996</v>
+      </c>
+      <c r="AD153">
+        <v>0</v>
+      </c>
+      <c r="AE153">
+        <v>463.0488</v>
+      </c>
+      <c r="AF153">
+        <v>0</v>
+      </c>
+      <c r="AG153">
+        <v>3</v>
+      </c>
+      <c r="AH153">
+        <v>1731.83919</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B154" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E154">
+        <v>101</v>
+      </c>
+      <c r="F154">
+        <v>4539.28</v>
+      </c>
+      <c r="G154">
+        <v>44.94336633663366</v>
+      </c>
+      <c r="H154">
+        <v>79.96000000000001</v>
+      </c>
+      <c r="I154">
+        <v>0</v>
+      </c>
+      <c r="J154">
+        <v>0</v>
+      </c>
+      <c r="K154">
+        <v>0.7916831683168317</v>
+      </c>
+      <c r="L154">
+        <v>0</v>
+      </c>
+      <c r="M154">
+        <v>0</v>
+      </c>
+      <c r="N154">
+        <v>25.44352</v>
+      </c>
+      <c r="O154">
+        <v>77.0735490124803</v>
+      </c>
+      <c r="P154">
+        <v>33.012</v>
+      </c>
+      <c r="Q154">
+        <v>558.07949</v>
+      </c>
+      <c r="R154">
+        <v>5.525539504950495</v>
+      </c>
+      <c r="S154">
+        <v>563.31998</v>
+      </c>
+      <c r="T154">
+        <v>18</v>
+      </c>
+      <c r="U154">
+        <v>21</v>
+      </c>
+      <c r="V154">
+        <v>39</v>
+      </c>
+      <c r="W154">
+        <v>80</v>
+      </c>
+      <c r="X154">
+        <v>18</v>
+      </c>
+      <c r="Y154">
+        <v>81</v>
+      </c>
+      <c r="Z154">
+        <v>21</v>
+      </c>
+      <c r="AA154">
+        <v>47</v>
+      </c>
+      <c r="AB154">
+        <v>3.83709</v>
+      </c>
+      <c r="AC154">
+        <v>-0.946</v>
+      </c>
+      <c r="AD154">
+        <v>0</v>
+      </c>
+      <c r="AE154">
+        <v>412.5015</v>
+      </c>
+      <c r="AF154">
+        <v>0</v>
+      </c>
+      <c r="AG154">
+        <v>3</v>
+      </c>
+      <c r="AH154">
+        <v>1674.23847</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B155" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E155">
+        <v>68.21666666666667</v>
+      </c>
+      <c r="F155">
+        <v>0</v>
+      </c>
+      <c r="G155">
+        <v>0</v>
+      </c>
+      <c r="H155">
+        <v>0</v>
+      </c>
+      <c r="I155">
+        <v>0</v>
+      </c>
+      <c r="J155">
+        <v>0</v>
+      </c>
+      <c r="K155">
+        <v>0</v>
+      </c>
+      <c r="L155">
+        <v>0</v>
+      </c>
+      <c r="M155">
+        <v>0</v>
+      </c>
+      <c r="N155">
+        <v>0</v>
+      </c>
+      <c r="O155">
+        <v>0</v>
+      </c>
+      <c r="P155">
+        <v>32.004</v>
+      </c>
+      <c r="Q155">
+        <v>5.37834</v>
+      </c>
+      <c r="R155">
+        <v>0.07884202296603958</v>
+      </c>
+      <c r="S155">
+        <v>0</v>
+      </c>
+      <c r="T155">
+        <v>0</v>
+      </c>
+      <c r="U155">
+        <v>0</v>
+      </c>
+      <c r="V155">
+        <v>0</v>
+      </c>
+      <c r="W155">
+        <v>0</v>
+      </c>
+      <c r="X155">
+        <v>0</v>
+      </c>
+      <c r="Y155">
+        <v>0</v>
+      </c>
+      <c r="Z155">
+        <v>0</v>
+      </c>
+      <c r="AA155">
+        <v>0</v>
+      </c>
+      <c r="AB155">
+        <v>0</v>
+      </c>
+      <c r="AC155">
+        <v>0</v>
+      </c>
+      <c r="AD155">
+        <v>0</v>
+      </c>
+      <c r="AE155">
+        <v>0</v>
+      </c>
+      <c r="AF155">
+        <v>0</v>
+      </c>
+      <c r="AG155">
+        <v>3</v>
+      </c>
+      <c r="AH155">
+        <v>16.13502</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B156" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E156">
+        <v>101</v>
+      </c>
+      <c r="F156">
+        <v>5267.559999999999</v>
+      </c>
+      <c r="G156">
+        <v>52.15405940594059</v>
+      </c>
+      <c r="H156">
+        <v>0</v>
+      </c>
+      <c r="I156">
+        <v>0</v>
+      </c>
+      <c r="J156">
+        <v>0</v>
+      </c>
+      <c r="K156">
+        <v>0</v>
+      </c>
+      <c r="L156">
+        <v>0</v>
+      </c>
+      <c r="M156">
+        <v>0</v>
+      </c>
+      <c r="N156">
+        <v>20.17957</v>
+      </c>
+      <c r="O156">
+        <v>56.05436111111111</v>
+      </c>
+      <c r="P156">
+        <v>36</v>
+      </c>
+      <c r="Q156">
+        <v>578.58226</v>
+      </c>
+      <c r="R156">
+        <v>5.728537227722772</v>
+      </c>
+      <c r="S156">
+        <v>345.91999</v>
+      </c>
+      <c r="T156">
+        <v>20</v>
+      </c>
+      <c r="U156">
+        <v>26</v>
+      </c>
+      <c r="V156">
+        <v>46</v>
+      </c>
+      <c r="W156">
+        <v>70</v>
+      </c>
+      <c r="X156">
+        <v>20</v>
+      </c>
+      <c r="Y156">
+        <v>65</v>
+      </c>
+      <c r="Z156">
+        <v>26</v>
+      </c>
+      <c r="AA156">
+        <v>67</v>
+      </c>
+      <c r="AB156">
+        <v>4.44842</v>
+      </c>
+      <c r="AC156">
+        <v>-1.44525</v>
+      </c>
+      <c r="AD156">
+        <v>0</v>
+      </c>
+      <c r="AE156">
+        <v>417.1209</v>
+      </c>
+      <c r="AF156">
+        <v>0</v>
+      </c>
+      <c r="AG156">
+        <v>3</v>
+      </c>
+      <c r="AH156">
+        <v>1735.74678</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-20
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH156"/>
+  <dimension ref="A1:AH158"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -15744,20 +15744,20 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E141">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F141">
-        <v>4422.52</v>
+        <v>17288.56</v>
       </c>
       <c r="G141">
-        <v>43.78732673267326</v>
+        <v>55.98173722982272</v>
       </c>
       <c r="H141">
-        <v>57.31</v>
+        <v>1693.79</v>
       </c>
       <c r="I141">
         <v>0</v>
@@ -15766,7 +15766,7 @@
         <v>0</v>
       </c>
       <c r="K141">
-        <v>0.5674257425742575</v>
+        <v>5.484627216060876</v>
       </c>
       <c r="L141">
         <v>0</v>
@@ -15775,49 +15775,49 @@
         <v>0</v>
       </c>
       <c r="N141">
-        <v>24.22245</v>
+        <v>28.53449</v>
       </c>
       <c r="O141">
-        <v>74.84380793474232</v>
+        <v>88.16737733283897</v>
       </c>
       <c r="P141">
         <v>32.364</v>
       </c>
       <c r="Q141">
-        <v>515.62801</v>
+        <v>1792.5641</v>
       </c>
       <c r="R141">
-        <v>5.105227821782178</v>
+        <v>5.804465635877925</v>
       </c>
       <c r="S141">
-        <v>493.04</v>
+        <v>2785.42003</v>
       </c>
       <c r="T141">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="U141">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="V141">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="W141">
-        <v>79</v>
+        <v>170</v>
       </c>
       <c r="X141">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="Y141">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="Z141">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="AA141">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="AB141">
-        <v>3.73904</v>
+        <v>3.96949</v>
       </c>
       <c r="AC141">
         <v>-1.17353</v>
@@ -15826,7 +15826,7 @@
         <v>0</v>
       </c>
       <c r="AE141">
-        <v>368.27</v>
+        <v>1363.8751</v>
       </c>
       <c r="AF141">
         <v>0</v>
@@ -15835,7 +15835,7 @@
         <v>3</v>
       </c>
       <c r="AH141">
-        <v>1546.88403</v>
+        <v>5377.692300000001</v>
       </c>
     </row>
     <row r="142">
@@ -15854,29 +15854,29 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E142">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F142">
-        <v>4400.25</v>
+        <v>17287.79</v>
       </c>
       <c r="G142">
-        <v>43.56683168316832</v>
+        <v>55.97924390836235</v>
       </c>
       <c r="H142">
-        <v>79.13000000000001</v>
+        <v>1844.95</v>
       </c>
       <c r="I142">
-        <v>0</v>
+        <v>8.030000000000001</v>
       </c>
       <c r="J142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K142">
-        <v>0.7834653465346536</v>
+        <v>5.97409536145066</v>
       </c>
       <c r="L142">
         <v>0</v>
@@ -15885,49 +15885,49 @@
         <v>0</v>
       </c>
       <c r="N142">
-        <v>28.46455</v>
+        <v>29.69156</v>
       </c>
       <c r="O142">
-        <v>87.85354938271604</v>
+        <v>91.64061728395062</v>
       </c>
       <c r="P142">
         <v>32.4</v>
       </c>
       <c r="Q142">
-        <v>598.2261699999999</v>
+        <v>2036.37995</v>
       </c>
       <c r="R142">
-        <v>5.923031386138613</v>
+        <v>6.593960819234194</v>
       </c>
       <c r="S142">
-        <v>617.22999</v>
+        <v>3140.64003</v>
       </c>
       <c r="T142">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U142">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="V142">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="W142">
-        <v>110</v>
+        <v>244</v>
       </c>
       <c r="X142">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="Y142">
-        <v>93</v>
+        <v>177</v>
       </c>
       <c r="Z142">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="AA142">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="AB142">
-        <v>3.89857</v>
+        <v>4.37114</v>
       </c>
       <c r="AC142">
         <v>-1.03831</v>
@@ -15936,7 +15936,7 @@
         <v>0</v>
       </c>
       <c r="AE142">
-        <v>371.9037</v>
+        <v>1392.6304</v>
       </c>
       <c r="AF142">
         <v>0</v>
@@ -15945,7 +15945,7 @@
         <v>3</v>
       </c>
       <c r="AH142">
-        <v>1794.67851</v>
+        <v>6109.13985</v>
       </c>
     </row>
     <row r="143">
@@ -15964,20 +15964,20 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E143">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F143">
-        <v>4227.74</v>
+        <v>16298.97</v>
       </c>
       <c r="G143">
-        <v>41.85881188118812</v>
+        <v>52.77736582206752</v>
       </c>
       <c r="H143">
-        <v>87.95999999999999</v>
+        <v>1011.57</v>
       </c>
       <c r="I143">
         <v>0</v>
@@ -15986,7 +15986,7 @@
         <v>0</v>
       </c>
       <c r="K143">
-        <v>0.8708910891089108</v>
+        <v>3.275544402169514</v>
       </c>
       <c r="L143">
         <v>0</v>
@@ -16004,37 +16004,37 @@
         <v>33.984</v>
       </c>
       <c r="Q143">
-        <v>591.91333</v>
+        <v>2036.07937</v>
       </c>
       <c r="R143">
-        <v>5.86052801980198</v>
+        <v>6.592987517202299</v>
       </c>
       <c r="S143">
-        <v>437.77</v>
+        <v>2179.37</v>
       </c>
       <c r="T143">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="U143">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="V143">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="W143">
-        <v>66</v>
+        <v>153</v>
       </c>
       <c r="X143">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="Y143">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="Z143">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="AA143">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AB143">
         <v>4.06104</v>
@@ -16046,7 +16046,7 @@
         <v>0</v>
       </c>
       <c r="AE143">
-        <v>390.016</v>
+        <v>1465.9648</v>
       </c>
       <c r="AF143">
         <v>0</v>
@@ -16055,13 +16055,13 @@
         <v>3</v>
       </c>
       <c r="AH143">
-        <v>1775.73999</v>
+        <v>6108.23811</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Dagoberto Espinoza</t>
+          <t>Dago Espinoza</t>
         </is>
       </c>
       <c r="B144" s="2">
@@ -16074,20 +16074,20 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada</t>
         </is>
       </c>
       <c r="E144">
-        <v>101</v>
+        <v>90.24583333333334</v>
       </c>
       <c r="F144">
-        <v>5713.3</v>
+        <v>8524.480000000001</v>
       </c>
       <c r="G144">
-        <v>56.56732673267327</v>
+        <v>94.45843298397895</v>
       </c>
       <c r="H144">
-        <v>72</v>
+        <v>1312.66</v>
       </c>
       <c r="I144">
         <v>0</v>
@@ -16096,7 +16096,7 @@
         <v>0</v>
       </c>
       <c r="K144">
-        <v>0.7128712871287128</v>
+        <v>14.54538067316127</v>
       </c>
       <c r="L144">
         <v>0</v>
@@ -16105,58 +16105,58 @@
         <v>0</v>
       </c>
       <c r="N144">
-        <v>27.68428</v>
+        <v>27.80303</v>
       </c>
       <c r="O144">
-        <v>77.83479532163744</v>
+        <v>78.16866284300495</v>
       </c>
       <c r="P144">
         <v>35.568</v>
       </c>
       <c r="Q144">
-        <v>609.02973</v>
+        <v>757.64877</v>
       </c>
       <c r="R144">
-        <v>6.029997326732673</v>
+        <v>8.395387820305647</v>
       </c>
       <c r="S144">
-        <v>779.60998</v>
+        <v>1626.56</v>
       </c>
       <c r="T144">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="U144">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="V144">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="W144">
-        <v>137</v>
+        <v>76</v>
       </c>
       <c r="X144">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="Y144">
-        <v>124</v>
+        <v>67</v>
       </c>
       <c r="Z144">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="AA144">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="AB144">
-        <v>4.27888</v>
+        <v>4.08188</v>
       </c>
       <c r="AC144">
-        <v>-1.21086</v>
+        <v>-1.39581</v>
       </c>
       <c r="AD144">
         <v>0</v>
       </c>
       <c r="AE144">
-        <v>567.1967999999999</v>
+        <v>759.8976</v>
       </c>
       <c r="AF144">
         <v>0</v>
@@ -16165,13 +16165,13 @@
         <v>3</v>
       </c>
       <c r="AH144">
-        <v>1827.08919</v>
+        <v>2272.94631</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Emilio Lara</t>
+          <t>Dagoberto Espinoza</t>
         </is>
       </c>
       <c r="B145" s="2">
@@ -16184,20 +16184,20 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E145">
-        <v>101</v>
+        <v>218.5791666666667</v>
       </c>
       <c r="F145">
-        <v>4515.04</v>
+        <v>10589</v>
       </c>
       <c r="G145">
-        <v>44.70336633663366</v>
+        <v>48.44469013896567</v>
       </c>
       <c r="H145">
-        <v>113.31</v>
+        <v>313.96</v>
       </c>
       <c r="I145">
         <v>0</v>
@@ -16206,7 +16206,7 @@
         <v>0</v>
       </c>
       <c r="K145">
-        <v>1.121881188118812</v>
+        <v>1.436367448864828</v>
       </c>
       <c r="L145">
         <v>0</v>
@@ -16215,58 +16215,58 @@
         <v>0</v>
       </c>
       <c r="N145">
-        <v>28.88958</v>
+        <v>27.94266</v>
       </c>
       <c r="O145">
-        <v>80.24883333333332</v>
+        <v>78.56123481781377</v>
       </c>
       <c r="P145">
-        <v>36</v>
+        <v>35.568</v>
       </c>
       <c r="Q145">
-        <v>495.78647</v>
+        <v>1045.92922</v>
       </c>
       <c r="R145">
-        <v>4.90877693069307</v>
+        <v>4.785127676852398</v>
       </c>
       <c r="S145">
-        <v>584.14</v>
+        <v>1514.84</v>
       </c>
       <c r="T145">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="U145">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="V145">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="W145">
-        <v>88</v>
+        <v>202</v>
       </c>
       <c r="X145">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="Y145">
-        <v>81</v>
+        <v>178</v>
       </c>
       <c r="Z145">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="AA145">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="AB145">
-        <v>4.38661</v>
+        <v>4.48386</v>
       </c>
       <c r="AC145">
-        <v>-1.10536</v>
+        <v>-1.21086</v>
       </c>
       <c r="AD145">
         <v>0</v>
       </c>
       <c r="AE145">
-        <v>382.5689</v>
+        <v>1034.252</v>
       </c>
       <c r="AF145">
         <v>0</v>
@@ -16275,13 +16275,13 @@
         <v>3</v>
       </c>
       <c r="AH145">
-        <v>1487.35941</v>
+        <v>3137.78766</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Erick Sánchez</t>
+          <t>Emilio Lara</t>
         </is>
       </c>
       <c r="B146" s="2">
@@ -16294,20 +16294,20 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E146">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F146">
-        <v>4108.09</v>
+        <v>17405.03</v>
       </c>
       <c r="G146">
-        <v>40.67415841584159</v>
+        <v>56.35887638630292</v>
       </c>
       <c r="H146">
-        <v>16.26</v>
+        <v>2977.8</v>
       </c>
       <c r="I146">
         <v>0</v>
@@ -16316,67 +16316,67 @@
         <v>0</v>
       </c>
       <c r="K146">
-        <v>0.160990099009901</v>
+        <v>9.642354084028172</v>
       </c>
       <c r="L146">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="M146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N146">
-        <v>22.67776</v>
+        <v>30.53683</v>
       </c>
       <c r="O146">
-        <v>70.85914260717411</v>
+        <v>84.82452777777777</v>
       </c>
       <c r="P146">
-        <v>32.004</v>
+        <v>36</v>
       </c>
       <c r="Q146">
-        <v>514.32473</v>
+        <v>1693.66433</v>
       </c>
       <c r="R146">
-        <v>5.092324059405941</v>
+        <v>5.484220286570064</v>
       </c>
       <c r="S146">
-        <v>334.19</v>
+        <v>3890.10999</v>
       </c>
       <c r="T146">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="U146">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="V146">
-        <v>43</v>
+        <v>125</v>
       </c>
       <c r="W146">
-        <v>71</v>
+        <v>215</v>
       </c>
       <c r="X146">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="Y146">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="Z146">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="AA146">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="AB146">
-        <v>4.24167</v>
+        <v>4.37683</v>
       </c>
       <c r="AC146">
-        <v>-1.95064</v>
+        <v>-1.10536</v>
       </c>
       <c r="AD146">
         <v>0</v>
       </c>
       <c r="AE146">
-        <v>281.9346</v>
+        <v>1409.0601</v>
       </c>
       <c r="AF146">
         <v>0</v>
@@ -16385,13 +16385,13 @@
         <v>3</v>
       </c>
       <c r="AH146">
-        <v>1542.97419</v>
+        <v>5080.992990000001</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Franco Rossano</t>
+          <t>Erick Sánchez</t>
         </is>
       </c>
       <c r="B147" s="2">
@@ -16404,89 +16404,89 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E147">
+        <v>308.825</v>
+      </c>
+      <c r="F147">
+        <v>16821.63</v>
+      </c>
+      <c r="G147">
+        <v>54.46978062009228</v>
+      </c>
+      <c r="H147">
+        <v>1234.07</v>
+      </c>
+      <c r="I147">
+        <v>0</v>
+      </c>
+      <c r="J147">
+        <v>0</v>
+      </c>
+      <c r="K147">
+        <v>3.996017161823039</v>
+      </c>
+      <c r="L147">
+        <v>0</v>
+      </c>
+      <c r="M147">
+        <v>0</v>
+      </c>
+      <c r="N147">
+        <v>28.7556</v>
+      </c>
+      <c r="O147">
+        <v>89.85001874765656</v>
+      </c>
+      <c r="P147">
+        <v>32.004</v>
+      </c>
+      <c r="Q147">
+        <v>1874.89228</v>
+      </c>
+      <c r="R147">
+        <v>6.071050854043553</v>
+      </c>
+      <c r="S147">
+        <v>2658.29997</v>
+      </c>
+      <c r="T147">
+        <v>47</v>
+      </c>
+      <c r="U147">
+        <v>54</v>
+      </c>
+      <c r="V147">
         <v>101</v>
       </c>
-      <c r="F147">
-        <v>5114.7</v>
-      </c>
-      <c r="G147">
-        <v>50.64059405940594</v>
-      </c>
-      <c r="H147">
-        <v>150.17</v>
-      </c>
-      <c r="I147">
-        <v>0</v>
-      </c>
-      <c r="J147">
-        <v>0</v>
-      </c>
-      <c r="K147">
-        <v>1.486831683168317</v>
-      </c>
-      <c r="L147">
-        <v>15.06</v>
-      </c>
-      <c r="M147">
-        <v>1</v>
-      </c>
-      <c r="N147">
-        <v>30.46936</v>
-      </c>
-      <c r="O147">
-        <v>90.03947990543735</v>
-      </c>
-      <c r="P147">
-        <v>33.84</v>
-      </c>
-      <c r="Q147">
-        <v>593.20456</v>
-      </c>
-      <c r="R147">
-        <v>5.873312475247525</v>
-      </c>
-      <c r="S147">
-        <v>769.60998</v>
-      </c>
-      <c r="T147">
-        <v>45</v>
-      </c>
-      <c r="U147">
-        <v>45</v>
-      </c>
-      <c r="V147">
-        <v>90</v>
-      </c>
       <c r="W147">
-        <v>115</v>
+        <v>177</v>
       </c>
       <c r="X147">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Y147">
-        <v>100</v>
+        <v>162</v>
       </c>
       <c r="Z147">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="AA147">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="AB147">
-        <v>4.26681</v>
+        <v>4.43851</v>
       </c>
       <c r="AC147">
-        <v>-1.4227</v>
+        <v>-1.90419</v>
       </c>
       <c r="AD147">
         <v>0</v>
       </c>
       <c r="AE147">
-        <v>444.3383</v>
+        <v>1145.235</v>
       </c>
       <c r="AF147">
         <v>0</v>
@@ -16495,13 +16495,13 @@
         <v>3</v>
       </c>
       <c r="AH147">
-        <v>1779.61368</v>
+        <v>5624.67684</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Henry Martín</t>
+          <t>Franco Rossano</t>
         </is>
       </c>
       <c r="B148" s="2">
@@ -16514,20 +16514,20 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E148">
-        <v>101</v>
+        <v>307.5123333333333</v>
       </c>
       <c r="F148">
-        <v>5114.150000000001</v>
+        <v>18002.72</v>
       </c>
       <c r="G148">
-        <v>50.63514851485149</v>
+        <v>58.54308282486232</v>
       </c>
       <c r="H148">
-        <v>59.50000000000001</v>
+        <v>1789.95</v>
       </c>
       <c r="I148">
         <v>0</v>
@@ -16536,67 +16536,67 @@
         <v>0</v>
       </c>
       <c r="K148">
-        <v>0.5891089108910892</v>
+        <v>5.820742149095375</v>
       </c>
       <c r="L148">
-        <v>0</v>
+        <v>15.06</v>
       </c>
       <c r="M148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N148">
-        <v>24.76522</v>
+        <v>30.46936</v>
       </c>
       <c r="O148">
-        <v>73.4960232668566</v>
+        <v>90.03947990543735</v>
       </c>
       <c r="P148">
-        <v>33.696</v>
+        <v>33.84</v>
       </c>
       <c r="Q148">
-        <v>589.86017</v>
+        <v>1845.8524</v>
       </c>
       <c r="R148">
-        <v>5.840199702970297</v>
+        <v>6.002531280588205</v>
       </c>
       <c r="S148">
-        <v>655.76</v>
+        <v>3176.92003</v>
       </c>
       <c r="T148">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="U148">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="V148">
-        <v>77</v>
+        <v>128</v>
       </c>
       <c r="W148">
-        <v>128</v>
+        <v>218</v>
       </c>
       <c r="X148">
-        <v>36</v>
+        <v>67</v>
       </c>
       <c r="Y148">
-        <v>116</v>
+        <v>174</v>
       </c>
       <c r="Z148">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="AA148">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="AB148">
-        <v>4.23286</v>
+        <v>4.26681</v>
       </c>
       <c r="AC148">
-        <v>-1.50173</v>
+        <v>-1.4227</v>
       </c>
       <c r="AD148">
         <v>0</v>
       </c>
       <c r="AE148">
-        <v>499.608</v>
+        <v>1457.6611</v>
       </c>
       <c r="AF148">
         <v>0</v>
@@ -16605,13 +16605,13 @@
         <v>3</v>
       </c>
       <c r="AH148">
-        <v>1769.58051</v>
+        <v>5537.5572</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Isaías Violante</t>
+          <t>Henry Martín</t>
         </is>
       </c>
       <c r="B149" s="2">
@@ -16624,20 +16624,20 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E149">
-        <v>101</v>
+        <v>307.5123333333333</v>
       </c>
       <c r="F149">
-        <v>4655.98</v>
+        <v>18391.61</v>
       </c>
       <c r="G149">
-        <v>46.09881188118811</v>
+        <v>59.80771502931591</v>
       </c>
       <c r="H149">
-        <v>84.10000000000001</v>
+        <v>1796.91</v>
       </c>
       <c r="I149">
         <v>0</v>
@@ -16646,7 +16646,7 @@
         <v>0</v>
       </c>
       <c r="K149">
-        <v>0.8326732673267327</v>
+        <v>5.84337538765383</v>
       </c>
       <c r="L149">
         <v>0</v>
@@ -16655,58 +16655,58 @@
         <v>0</v>
       </c>
       <c r="N149">
-        <v>25.52001</v>
+        <v>27.22911</v>
       </c>
       <c r="O149">
-        <v>72.93098422496571</v>
+        <v>80.80813746438747</v>
       </c>
       <c r="P149">
-        <v>34.992</v>
+        <v>33.696</v>
       </c>
       <c r="Q149">
-        <v>503.99442</v>
+        <v>1864.99843</v>
       </c>
       <c r="R149">
-        <v>4.990043762376238</v>
+        <v>6.064792295593564</v>
       </c>
       <c r="S149">
-        <v>613.22</v>
+        <v>3199.09003</v>
       </c>
       <c r="T149">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="U149">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="V149">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="W149">
-        <v>101</v>
+        <v>223</v>
       </c>
       <c r="X149">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="Y149">
-        <v>91</v>
+        <v>207</v>
       </c>
       <c r="Z149">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="AA149">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="AB149">
-        <v>4.44872</v>
+        <v>4.23286</v>
       </c>
       <c r="AC149">
-        <v>-0.87904</v>
+        <v>-1.50173</v>
       </c>
       <c r="AD149">
         <v>0</v>
       </c>
       <c r="AE149">
-        <v>386.11641</v>
+        <v>1702.7184</v>
       </c>
       <c r="AF149">
         <v>0</v>
@@ -16715,13 +16715,13 @@
         <v>3</v>
       </c>
       <c r="AH149">
-        <v>1511.98326</v>
+        <v>5594.99529</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>José Raúl Zúñiga</t>
+          <t>Isaías Violante</t>
         </is>
       </c>
       <c r="B150" s="2">
@@ -16734,89 +16734,89 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E150">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F150">
-        <v>4824.73</v>
+        <v>17985.02</v>
       </c>
       <c r="G150">
-        <v>47.76960396039603</v>
+        <v>58.23693030033191</v>
       </c>
       <c r="H150">
-        <v>57.88</v>
+        <v>1388.6</v>
       </c>
       <c r="I150">
-        <v>0</v>
+        <v>6.92</v>
       </c>
       <c r="J150">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K150">
-        <v>0.5730693069306931</v>
+        <v>4.496397636201733</v>
       </c>
       <c r="L150">
-        <v>0</v>
+        <v>30.24</v>
       </c>
       <c r="M150">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N150">
-        <v>23.05072</v>
+        <v>32.15074</v>
       </c>
       <c r="O150">
-        <v>66.01008018327606</v>
+        <v>91.88025834476451</v>
       </c>
       <c r="P150">
-        <v>34.92</v>
+        <v>34.992</v>
       </c>
       <c r="Q150">
-        <v>461.31373</v>
+        <v>1741.63772</v>
       </c>
       <c r="R150">
-        <v>4.567462673267326</v>
+        <v>5.639561952562131</v>
       </c>
       <c r="S150">
-        <v>482.92</v>
+        <v>2810.82001</v>
       </c>
       <c r="T150">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="U150">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="V150">
-        <v>38</v>
+        <v>133</v>
       </c>
       <c r="W150">
-        <v>72</v>
+        <v>209</v>
       </c>
       <c r="X150">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="Y150">
-        <v>67</v>
+        <v>186</v>
       </c>
       <c r="Z150">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="AA150">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="AB150">
-        <v>3.81153</v>
+        <v>4.64199</v>
       </c>
       <c r="AC150">
-        <v>-1.5841</v>
+        <v>-0.87904</v>
       </c>
       <c r="AD150">
         <v>0</v>
       </c>
       <c r="AE150">
-        <v>446.0504</v>
+        <v>1427.37885</v>
       </c>
       <c r="AF150">
         <v>0</v>
@@ -16825,13 +16825,13 @@
         <v>3</v>
       </c>
       <c r="AH150">
-        <v>1383.94119</v>
+        <v>5224.91316</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Kevin Álvarez</t>
+          <t>José Raúl Zúñiga</t>
         </is>
       </c>
       <c r="B151" s="2">
@@ -16844,20 +16844,20 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E151">
-        <v>101</v>
+        <v>307.5123333333333</v>
       </c>
       <c r="F151">
-        <v>4728.51</v>
+        <v>18445.82</v>
       </c>
       <c r="G151">
-        <v>46.81693069306931</v>
+        <v>59.98400064170869</v>
       </c>
       <c r="H151">
-        <v>93.34</v>
+        <v>1528.79</v>
       </c>
       <c r="I151">
         <v>0</v>
@@ -16866,7 +16866,7 @@
         <v>0</v>
       </c>
       <c r="K151">
-        <v>0.9241584158415842</v>
+        <v>4.971475398818693</v>
       </c>
       <c r="L151">
         <v>0</v>
@@ -16875,58 +16875,58 @@
         <v>0</v>
       </c>
       <c r="N151">
-        <v>26.12775</v>
+        <v>28.03511</v>
       </c>
       <c r="O151">
-        <v>74.66778120713306</v>
+        <v>80.28382016036655</v>
       </c>
       <c r="P151">
-        <v>34.992</v>
+        <v>34.92</v>
       </c>
       <c r="Q151">
-        <v>500.97208</v>
+        <v>1518.91438</v>
       </c>
       <c r="R151">
-        <v>4.960119603960396</v>
+        <v>4.939360849483545</v>
       </c>
       <c r="S151">
-        <v>654.3700100000001</v>
+        <v>2837.21004</v>
       </c>
       <c r="T151">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="U151">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="V151">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="W151">
-        <v>101</v>
+        <v>158</v>
       </c>
       <c r="X151">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="Y151">
-        <v>83</v>
+        <v>147</v>
       </c>
       <c r="Z151">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AA151">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="AB151">
-        <v>3.91968</v>
+        <v>3.81153</v>
       </c>
       <c r="AC151">
-        <v>-1.71894</v>
+        <v>-1.5841</v>
       </c>
       <c r="AD151">
         <v>0</v>
       </c>
       <c r="AE151">
-        <v>410.61714</v>
+        <v>1666.1376</v>
       </c>
       <c r="AF151">
         <v>0</v>
@@ -16935,13 +16935,13 @@
         <v>3</v>
       </c>
       <c r="AH151">
-        <v>1502.91624</v>
+        <v>4556.74314</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Miguel Vázquez</t>
+          <t>Kevin Álvarez</t>
         </is>
       </c>
       <c r="B152" s="2">
@@ -16954,20 +16954,20 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E152">
-        <v>101</v>
+        <v>308.825</v>
       </c>
       <c r="F152">
-        <v>4161.61</v>
+        <v>18063.59</v>
       </c>
       <c r="G152">
-        <v>41.20405940594059</v>
+        <v>58.49134623168462</v>
       </c>
       <c r="H152">
-        <v>52.45</v>
+        <v>2111.72</v>
       </c>
       <c r="I152">
         <v>0</v>
@@ -16976,7 +16976,7 @@
         <v>0</v>
       </c>
       <c r="K152">
-        <v>0.5193069306930693</v>
+        <v>6.837917914676598</v>
       </c>
       <c r="L152">
         <v>0</v>
@@ -16985,58 +16985,58 @@
         <v>0</v>
       </c>
       <c r="N152">
-        <v>24.8696</v>
+        <v>28.09404</v>
       </c>
       <c r="O152">
-        <v>73.18032015065913</v>
+        <v>80.28703703703705</v>
       </c>
       <c r="P152">
-        <v>33.984</v>
+        <v>34.992</v>
       </c>
       <c r="Q152">
-        <v>502.61805</v>
+        <v>1643.06226</v>
       </c>
       <c r="R152">
-        <v>4.976416336633664</v>
+        <v>5.320366744920263</v>
       </c>
       <c r="S152">
-        <v>378.56</v>
+        <v>3515.66006</v>
       </c>
       <c r="T152">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="U152">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="V152">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="W152">
-        <v>61</v>
+        <v>238</v>
       </c>
       <c r="X152">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="Y152">
+        <v>204</v>
+      </c>
+      <c r="Z152">
         <v>54</v>
       </c>
-      <c r="Z152">
-        <v>15</v>
-      </c>
       <c r="AA152">
-        <v>47</v>
+        <v>85</v>
       </c>
       <c r="AB152">
-        <v>3.43314</v>
+        <v>4.33431</v>
       </c>
       <c r="AC152">
-        <v>-1.06918</v>
+        <v>-1.71894</v>
       </c>
       <c r="AD152">
         <v>0</v>
       </c>
       <c r="AE152">
-        <v>391.4728</v>
+        <v>1503.75018</v>
       </c>
       <c r="AF152">
         <v>0</v>
@@ -17045,13 +17045,13 @@
         <v>3</v>
       </c>
       <c r="AH152">
-        <v>1507.85415</v>
+        <v>4929.18678</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Pato Salas</t>
+          <t>Luis Ángel Malagón</t>
         </is>
       </c>
       <c r="B153" s="2">
@@ -17064,20 +17064,20 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada</t>
         </is>
       </c>
       <c r="E153">
-        <v>101</v>
+        <v>34.15133333333333</v>
       </c>
       <c r="F153">
-        <v>4725.58</v>
+        <v>3408.52</v>
       </c>
       <c r="G153">
-        <v>46.78792079207921</v>
+        <v>99.80635211899975</v>
       </c>
       <c r="H153">
-        <v>89.11999999999999</v>
+        <v>0</v>
       </c>
       <c r="I153">
         <v>0</v>
@@ -17086,7 +17086,7 @@
         <v>0</v>
       </c>
       <c r="K153">
-        <v>0.8823762376237623</v>
+        <v>0</v>
       </c>
       <c r="L153">
         <v>0</v>
@@ -17095,58 +17095,58 @@
         <v>0</v>
       </c>
       <c r="N153">
-        <v>26.27495</v>
+        <v>16.98063</v>
       </c>
       <c r="O153">
-        <v>75.08844878829447</v>
+        <v>56.62474989995999</v>
       </c>
       <c r="P153">
-        <v>34.992</v>
+        <v>29.988</v>
       </c>
       <c r="Q153">
-        <v>577.27973</v>
+        <v>242.84204</v>
       </c>
       <c r="R153">
-        <v>5.715640891089109</v>
+        <v>7.11076307416011</v>
       </c>
       <c r="S153">
-        <v>737.05999</v>
+        <v>12.15</v>
       </c>
       <c r="T153">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="U153">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="V153">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="W153">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="X153">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="Y153">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="Z153">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AA153">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="AB153">
-        <v>4.15186</v>
+        <v>1.68668</v>
       </c>
       <c r="AC153">
-        <v>-1.76996</v>
+        <v>-1.42075</v>
       </c>
       <c r="AD153">
         <v>0</v>
       </c>
       <c r="AE153">
-        <v>463.0488</v>
+        <v>274.30026</v>
       </c>
       <c r="AF153">
         <v>0</v>
@@ -17155,13 +17155,13 @@
         <v>3</v>
       </c>
       <c r="AH153">
-        <v>1731.83919</v>
+        <v>728.52612</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Ramón Juárez</t>
+          <t>Miguel Vázquez</t>
         </is>
       </c>
       <c r="B154" s="2">
@@ -17174,20 +17174,20 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E154">
-        <v>101</v>
+        <v>307.5123333333333</v>
       </c>
       <c r="F154">
-        <v>4539.28</v>
+        <v>16062.82</v>
       </c>
       <c r="G154">
-        <v>44.94336633663366</v>
+        <v>52.23471795711175</v>
       </c>
       <c r="H154">
-        <v>79.96000000000001</v>
+        <v>1969.79</v>
       </c>
       <c r="I154">
         <v>0</v>
@@ -17196,7 +17196,7 @@
         <v>0</v>
       </c>
       <c r="K154">
-        <v>0.7916831683168317</v>
+        <v>6.405564221272427</v>
       </c>
       <c r="L154">
         <v>0</v>
@@ -17205,58 +17205,58 @@
         <v>0</v>
       </c>
       <c r="N154">
-        <v>25.44352</v>
+        <v>28.31333</v>
       </c>
       <c r="O154">
-        <v>77.0735490124803</v>
+        <v>83.31370645009416</v>
       </c>
       <c r="P154">
-        <v>33.012</v>
+        <v>33.984</v>
       </c>
       <c r="Q154">
-        <v>558.07949</v>
+        <v>1632.26711</v>
       </c>
       <c r="R154">
-        <v>5.525539504950495</v>
+        <v>5.307972829274057</v>
       </c>
       <c r="S154">
-        <v>563.31998</v>
+        <v>2698.55997</v>
       </c>
       <c r="T154">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="U154">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="V154">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="W154">
-        <v>80</v>
+        <v>134</v>
       </c>
       <c r="X154">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="Y154">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="Z154">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="AA154">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="AB154">
-        <v>3.83709</v>
+        <v>4.00059</v>
       </c>
       <c r="AC154">
-        <v>-0.946</v>
+        <v>-1.06918</v>
       </c>
       <c r="AD154">
         <v>0</v>
       </c>
       <c r="AE154">
-        <v>412.5015</v>
+        <v>1451.2184</v>
       </c>
       <c r="AF154">
         <v>0</v>
@@ -17265,13 +17265,13 @@
         <v>3</v>
       </c>
       <c r="AH154">
-        <v>1674.23847</v>
+        <v>4896.80133</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Raphael Veiga</t>
+          <t>Pato Salas</t>
         </is>
       </c>
       <c r="B155" s="2">
@@ -17284,20 +17284,20 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E155">
-        <v>68.21666666666667</v>
+        <v>218.5791666666667</v>
       </c>
       <c r="F155">
-        <v>0</v>
+        <v>7924.96</v>
       </c>
       <c r="G155">
-        <v>0</v>
+        <v>36.25670333021979</v>
       </c>
       <c r="H155">
-        <v>0</v>
+        <v>167.65</v>
       </c>
       <c r="I155">
         <v>0</v>
@@ -17306,7 +17306,7 @@
         <v>0</v>
       </c>
       <c r="K155">
-        <v>0</v>
+        <v>0.7669989896871843</v>
       </c>
       <c r="L155">
         <v>0</v>
@@ -17315,58 +17315,58 @@
         <v>0</v>
       </c>
       <c r="N155">
-        <v>0</v>
+        <v>26.27495</v>
       </c>
       <c r="O155">
-        <v>0</v>
+        <v>75.08844878829447</v>
       </c>
       <c r="P155">
-        <v>32.004</v>
+        <v>34.992</v>
       </c>
       <c r="Q155">
-        <v>5.37834</v>
+        <v>901.53407</v>
       </c>
       <c r="R155">
-        <v>0.07884202296603958</v>
+        <v>4.124519659162393</v>
       </c>
       <c r="S155">
-        <v>0</v>
+        <v>1133.02999</v>
       </c>
       <c r="T155">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="U155">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="V155">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="W155">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="X155">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="Y155">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="Z155">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="AA155">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="AB155">
-        <v>0</v>
+        <v>4.15186</v>
       </c>
       <c r="AC155">
-        <v>0</v>
+        <v>-1.76996</v>
       </c>
       <c r="AD155">
         <v>0</v>
       </c>
       <c r="AE155">
-        <v>0</v>
+        <v>763.7616</v>
       </c>
       <c r="AF155">
         <v>0</v>
@@ -17375,13 +17375,13 @@
         <v>3</v>
       </c>
       <c r="AH155">
-        <v>16.13502</v>
+        <v>2704.60221</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Thiago Espinosa</t>
+          <t>Ramón Juárez</t>
         </is>
       </c>
       <c r="B156" s="2">
@@ -17394,20 +17394,20 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Sesion 7 19 de junio AM</t>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
         </is>
       </c>
       <c r="E156">
-        <v>101</v>
+        <v>307.5123333333333</v>
       </c>
       <c r="F156">
-        <v>5267.559999999999</v>
+        <v>17028.45</v>
       </c>
       <c r="G156">
-        <v>52.15405940594059</v>
+        <v>55.37485217395076</v>
       </c>
       <c r="H156">
-        <v>0</v>
+        <v>1723.01</v>
       </c>
       <c r="I156">
         <v>0</v>
@@ -17416,7 +17416,7 @@
         <v>0</v>
       </c>
       <c r="K156">
-        <v>0</v>
+        <v>5.603059823074847</v>
       </c>
       <c r="L156">
         <v>0</v>
@@ -17425,58 +17425,58 @@
         <v>0</v>
       </c>
       <c r="N156">
-        <v>20.17957</v>
+        <v>27.77737</v>
       </c>
       <c r="O156">
-        <v>56.05436111111111</v>
+        <v>84.14325093905248</v>
       </c>
       <c r="P156">
-        <v>36</v>
+        <v>33.012</v>
       </c>
       <c r="Q156">
-        <v>578.58226</v>
+        <v>1789.01184</v>
       </c>
       <c r="R156">
-        <v>5.728537227722772</v>
+        <v>5.817691344628996</v>
       </c>
       <c r="S156">
-        <v>345.91999</v>
+        <v>3031.64001</v>
       </c>
       <c r="T156">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="U156">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="V156">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="W156">
-        <v>70</v>
+        <v>191</v>
       </c>
       <c r="X156">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="Y156">
-        <v>65</v>
+        <v>172</v>
       </c>
       <c r="Z156">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="AA156">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="AB156">
-        <v>4.44842</v>
+        <v>3.9815</v>
       </c>
       <c r="AC156">
-        <v>-1.44525</v>
+        <v>-0.946</v>
       </c>
       <c r="AD156">
         <v>0</v>
       </c>
       <c r="AE156">
-        <v>417.1209</v>
+        <v>1450.2345</v>
       </c>
       <c r="AF156">
         <v>0</v>
@@ -17485,7 +17485,227 @@
         <v>3</v>
       </c>
       <c r="AH156">
-        <v>1735.74678</v>
+        <v>5367.035519999999</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B157" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E157">
+        <v>307.5123333333333</v>
+      </c>
+      <c r="F157">
+        <v>13456.19</v>
+      </c>
+      <c r="G157">
+        <v>43.75821240774083</v>
+      </c>
+      <c r="H157">
+        <v>1575.82</v>
+      </c>
+      <c r="I157">
+        <v>0</v>
+      </c>
+      <c r="J157">
+        <v>0</v>
+      </c>
+      <c r="K157">
+        <v>5.124412354192842</v>
+      </c>
+      <c r="L157">
+        <v>0</v>
+      </c>
+      <c r="M157">
+        <v>0</v>
+      </c>
+      <c r="N157">
+        <v>28.10987</v>
+      </c>
+      <c r="O157">
+        <v>87.83236470441196</v>
+      </c>
+      <c r="P157">
+        <v>32.004</v>
+      </c>
+      <c r="Q157">
+        <v>1315.3738</v>
+      </c>
+      <c r="R157">
+        <v>4.277466811629236</v>
+      </c>
+      <c r="S157">
+        <v>2309.59997</v>
+      </c>
+      <c r="T157">
+        <v>20</v>
+      </c>
+      <c r="U157">
+        <v>13</v>
+      </c>
+      <c r="V157">
+        <v>33</v>
+      </c>
+      <c r="W157">
+        <v>105</v>
+      </c>
+      <c r="X157">
+        <v>20</v>
+      </c>
+      <c r="Y157">
+        <v>75</v>
+      </c>
+      <c r="Z157">
+        <v>13</v>
+      </c>
+      <c r="AA157">
+        <v>17</v>
+      </c>
+      <c r="AB157">
+        <v>3.99959</v>
+      </c>
+      <c r="AC157">
+        <v>0</v>
+      </c>
+      <c r="AD157">
+        <v>0</v>
+      </c>
+      <c r="AE157">
+        <v>1053.5784</v>
+      </c>
+      <c r="AF157">
+        <v>0</v>
+      </c>
+      <c r="AG157">
+        <v>3</v>
+      </c>
+      <c r="AH157">
+        <v>3946.1214</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B158" s="2">
+        <v>46192</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Sesión 9 Pretemporada | Sesión 8 Pretemporada | Sesion 7 19 de junio AM</t>
+        </is>
+      </c>
+      <c r="E158">
+        <v>262.1916666666667</v>
+      </c>
+      <c r="F158">
+        <v>16085.98</v>
+      </c>
+      <c r="G158">
+        <v>61.35198804945492</v>
+      </c>
+      <c r="H158">
+        <v>1298.26</v>
+      </c>
+      <c r="I158">
+        <v>0</v>
+      </c>
+      <c r="J158">
+        <v>0</v>
+      </c>
+      <c r="K158">
+        <v>4.951568509042367</v>
+      </c>
+      <c r="L158">
+        <v>0</v>
+      </c>
+      <c r="M158">
+        <v>0</v>
+      </c>
+      <c r="N158">
+        <v>28.65134</v>
+      </c>
+      <c r="O158">
+        <v>79.58705555555557</v>
+      </c>
+      <c r="P158">
+        <v>36</v>
+      </c>
+      <c r="Q158">
+        <v>1742.3385</v>
+      </c>
+      <c r="R158">
+        <v>6.645285573530814</v>
+      </c>
+      <c r="S158">
+        <v>2375.87999</v>
+      </c>
+      <c r="T158">
+        <v>56</v>
+      </c>
+      <c r="U158">
+        <v>40</v>
+      </c>
+      <c r="V158">
+        <v>96</v>
+      </c>
+      <c r="W158">
+        <v>152</v>
+      </c>
+      <c r="X158">
+        <v>56</v>
+      </c>
+      <c r="Y158">
+        <v>129</v>
+      </c>
+      <c r="Z158">
+        <v>40</v>
+      </c>
+      <c r="AA158">
+        <v>87</v>
+      </c>
+      <c r="AB158">
+        <v>4.72956</v>
+      </c>
+      <c r="AC158">
+        <v>-1.44525</v>
+      </c>
+      <c r="AD158">
+        <v>0</v>
+      </c>
+      <c r="AE158">
+        <v>1269.6768</v>
+      </c>
+      <c r="AF158">
+        <v>0</v>
+      </c>
+      <c r="AG158">
+        <v>3</v>
+      </c>
+      <c r="AH158">
+        <v>5227.0155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-21
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH158"/>
+  <dimension ref="A1:AH188"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -17708,6 +17708,3306 @@
         <v>5227.0155</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B159" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E159">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F159">
+        <v>5627.25</v>
+      </c>
+      <c r="G159">
+        <v>53.24641735754197</v>
+      </c>
+      <c r="H159">
+        <v>82.81999999999999</v>
+      </c>
+      <c r="I159">
+        <v>0</v>
+      </c>
+      <c r="J159">
+        <v>0</v>
+      </c>
+      <c r="K159">
+        <v>0.7836631188505264</v>
+      </c>
+      <c r="L159">
+        <v>0</v>
+      </c>
+      <c r="M159">
+        <v>0</v>
+      </c>
+      <c r="N159">
+        <v>24.28968</v>
+      </c>
+      <c r="O159">
+        <v>75.05153874675567</v>
+      </c>
+      <c r="P159">
+        <v>32.364</v>
+      </c>
+      <c r="Q159">
+        <v>540.26575</v>
+      </c>
+      <c r="R159">
+        <v>5.11212681300554</v>
+      </c>
+      <c r="S159">
+        <v>707.78</v>
+      </c>
+      <c r="T159">
+        <v>21</v>
+      </c>
+      <c r="U159">
+        <v>10</v>
+      </c>
+      <c r="V159">
+        <v>31</v>
+      </c>
+      <c r="W159">
+        <v>55</v>
+      </c>
+      <c r="X159">
+        <v>21</v>
+      </c>
+      <c r="Y159">
+        <v>36</v>
+      </c>
+      <c r="Z159">
+        <v>10</v>
+      </c>
+      <c r="AA159">
+        <v>5</v>
+      </c>
+      <c r="AB159">
+        <v>4.09971</v>
+      </c>
+      <c r="AC159">
+        <v>-1.02264</v>
+      </c>
+      <c r="AD159">
+        <v>0</v>
+      </c>
+      <c r="AE159">
+        <v>448.2919</v>
+      </c>
+      <c r="AF159">
+        <v>0</v>
+      </c>
+      <c r="AG159">
+        <v>3</v>
+      </c>
+      <c r="AH159">
+        <v>1620.79725</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B160" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E160">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F160">
+        <v>5776.589999999999</v>
+      </c>
+      <c r="G160">
+        <v>54.65950900411449</v>
+      </c>
+      <c r="H160">
+        <v>214.72</v>
+      </c>
+      <c r="I160">
+        <v>0</v>
+      </c>
+      <c r="J160">
+        <v>0</v>
+      </c>
+      <c r="K160">
+        <v>2.031733215160409</v>
+      </c>
+      <c r="L160">
+        <v>0</v>
+      </c>
+      <c r="M160">
+        <v>0</v>
+      </c>
+      <c r="N160">
+        <v>27.25904</v>
+      </c>
+      <c r="O160">
+        <v>84.13283950617284</v>
+      </c>
+      <c r="P160">
+        <v>32.4</v>
+      </c>
+      <c r="Q160">
+        <v>624.10414</v>
+      </c>
+      <c r="R160">
+        <v>5.905426187393451</v>
+      </c>
+      <c r="S160">
+        <v>894.6499899999999</v>
+      </c>
+      <c r="T160">
+        <v>12</v>
+      </c>
+      <c r="U160">
+        <v>11</v>
+      </c>
+      <c r="V160">
+        <v>23</v>
+      </c>
+      <c r="W160">
+        <v>58</v>
+      </c>
+      <c r="X160">
+        <v>12</v>
+      </c>
+      <c r="Y160">
+        <v>51</v>
+      </c>
+      <c r="Z160">
+        <v>11</v>
+      </c>
+      <c r="AA160">
+        <v>7</v>
+      </c>
+      <c r="AB160">
+        <v>3.838</v>
+      </c>
+      <c r="AC160">
+        <v>-1.11552</v>
+      </c>
+      <c r="AD160">
+        <v>0</v>
+      </c>
+      <c r="AE160">
+        <v>465.7408</v>
+      </c>
+      <c r="AF160">
+        <v>0</v>
+      </c>
+      <c r="AG160">
+        <v>3</v>
+      </c>
+      <c r="AH160">
+        <v>1872.31242</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B161" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E161">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F161">
+        <v>6234.639999999999</v>
+      </c>
+      <c r="G161">
+        <v>58.99369025972285</v>
+      </c>
+      <c r="H161">
+        <v>202.11</v>
+      </c>
+      <c r="I161">
+        <v>0</v>
+      </c>
+      <c r="J161">
+        <v>0</v>
+      </c>
+      <c r="K161">
+        <v>1.912414307545037</v>
+      </c>
+      <c r="L161">
+        <v>0</v>
+      </c>
+      <c r="M161">
+        <v>0</v>
+      </c>
+      <c r="N161">
+        <v>28.07638</v>
+      </c>
+      <c r="O161">
+        <v>78.93719073324337</v>
+      </c>
+      <c r="P161">
+        <v>35.568</v>
+      </c>
+      <c r="Q161">
+        <v>544.02559</v>
+      </c>
+      <c r="R161">
+        <v>5.147703339699321</v>
+      </c>
+      <c r="S161">
+        <v>856.53998</v>
+      </c>
+      <c r="T161">
+        <v>22</v>
+      </c>
+      <c r="U161">
+        <v>19</v>
+      </c>
+      <c r="V161">
+        <v>41</v>
+      </c>
+      <c r="W161">
+        <v>71</v>
+      </c>
+      <c r="X161">
+        <v>22</v>
+      </c>
+      <c r="Y161">
+        <v>56</v>
+      </c>
+      <c r="Z161">
+        <v>19</v>
+      </c>
+      <c r="AA161">
+        <v>8</v>
+      </c>
+      <c r="AB161">
+        <v>4.48433</v>
+      </c>
+      <c r="AC161">
+        <v>-1.1022</v>
+      </c>
+      <c r="AD161">
+        <v>0</v>
+      </c>
+      <c r="AE161">
+        <v>579.1864</v>
+      </c>
+      <c r="AF161">
+        <v>0</v>
+      </c>
+      <c r="AG161">
+        <v>3</v>
+      </c>
+      <c r="AH161">
+        <v>1632.07677</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B162" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E162">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F162">
+        <v>5867.84</v>
+      </c>
+      <c r="G162">
+        <v>55.52293884708855</v>
+      </c>
+      <c r="H162">
+        <v>283.8</v>
+      </c>
+      <c r="I162">
+        <v>0</v>
+      </c>
+      <c r="J162">
+        <v>0</v>
+      </c>
+      <c r="K162">
+        <v>2.685385089709967</v>
+      </c>
+      <c r="L162">
+        <v>0</v>
+      </c>
+      <c r="M162">
+        <v>0</v>
+      </c>
+      <c r="N162">
+        <v>28.08328</v>
+      </c>
+      <c r="O162">
+        <v>78.00911111111111</v>
+      </c>
+      <c r="P162">
+        <v>36</v>
+      </c>
+      <c r="Q162">
+        <v>535.13336</v>
+      </c>
+      <c r="R162">
+        <v>5.063562882136702</v>
+      </c>
+      <c r="S162">
+        <v>865.5700300000001</v>
+      </c>
+      <c r="T162">
+        <v>6</v>
+      </c>
+      <c r="U162">
+        <v>14</v>
+      </c>
+      <c r="V162">
+        <v>20</v>
+      </c>
+      <c r="W162">
+        <v>59</v>
+      </c>
+      <c r="X162">
+        <v>6</v>
+      </c>
+      <c r="Y162">
+        <v>48</v>
+      </c>
+      <c r="Z162">
+        <v>14</v>
+      </c>
+      <c r="AA162">
+        <v>15</v>
+      </c>
+      <c r="AB162">
+        <v>3.94378</v>
+      </c>
+      <c r="AC162">
+        <v>-1.93264</v>
+      </c>
+      <c r="AD162">
+        <v>0</v>
+      </c>
+      <c r="AE162">
+        <v>472.5658</v>
+      </c>
+      <c r="AF162">
+        <v>0</v>
+      </c>
+      <c r="AG162">
+        <v>3</v>
+      </c>
+      <c r="AH162">
+        <v>1605.40008</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B163" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E163">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F163">
+        <v>5287.57</v>
+      </c>
+      <c r="G163">
+        <v>50.03228202536197</v>
+      </c>
+      <c r="H163">
+        <v>199.18</v>
+      </c>
+      <c r="I163">
+        <v>0</v>
+      </c>
+      <c r="J163">
+        <v>0</v>
+      </c>
+      <c r="K163">
+        <v>1.884689930121322</v>
+      </c>
+      <c r="L163">
+        <v>0</v>
+      </c>
+      <c r="M163">
+        <v>0</v>
+      </c>
+      <c r="N163">
+        <v>28.69927</v>
+      </c>
+      <c r="O163">
+        <v>89.67400949881265</v>
+      </c>
+      <c r="P163">
+        <v>32.004</v>
+      </c>
+      <c r="Q163">
+        <v>551.10511</v>
+      </c>
+      <c r="R163">
+        <v>5.214691491391722</v>
+      </c>
+      <c r="S163">
+        <v>716.8499899999999</v>
+      </c>
+      <c r="T163">
+        <v>11</v>
+      </c>
+      <c r="U163">
+        <v>12</v>
+      </c>
+      <c r="V163">
+        <v>23</v>
+      </c>
+      <c r="W163">
+        <v>54</v>
+      </c>
+      <c r="X163">
+        <v>11</v>
+      </c>
+      <c r="Y163">
+        <v>44</v>
+      </c>
+      <c r="Z163">
+        <v>12</v>
+      </c>
+      <c r="AA163">
+        <v>4</v>
+      </c>
+      <c r="AB163">
+        <v>4.15343</v>
+      </c>
+      <c r="AC163">
+        <v>-1.1497</v>
+      </c>
+      <c r="AD163">
+        <v>0</v>
+      </c>
+      <c r="AE163">
+        <v>361.2402</v>
+      </c>
+      <c r="AF163">
+        <v>0</v>
+      </c>
+      <c r="AG163">
+        <v>3</v>
+      </c>
+      <c r="AH163">
+        <v>1653.31533</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B164" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E164">
+        <v>68.14366666666666</v>
+      </c>
+      <c r="F164">
+        <v>4623.15</v>
+      </c>
+      <c r="G164">
+        <v>67.84416257808257</v>
+      </c>
+      <c r="H164">
+        <v>239.04</v>
+      </c>
+      <c r="I164">
+        <v>0</v>
+      </c>
+      <c r="J164">
+        <v>0</v>
+      </c>
+      <c r="K164">
+        <v>3.507882855339944</v>
+      </c>
+      <c r="L164">
+        <v>0</v>
+      </c>
+      <c r="M164">
+        <v>0</v>
+      </c>
+      <c r="N164">
+        <v>29.46997</v>
+      </c>
+      <c r="O164">
+        <v>87.08619976359337</v>
+      </c>
+      <c r="P164">
+        <v>33.84</v>
+      </c>
+      <c r="Q164">
+        <v>427.0470299999999</v>
+      </c>
+      <c r="R164">
+        <v>6.266863098062426</v>
+      </c>
+      <c r="S164">
+        <v>721.78998</v>
+      </c>
+      <c r="T164">
+        <v>19</v>
+      </c>
+      <c r="U164">
+        <v>18</v>
+      </c>
+      <c r="V164">
+        <v>37</v>
+      </c>
+      <c r="W164">
+        <v>61</v>
+      </c>
+      <c r="X164">
+        <v>19</v>
+      </c>
+      <c r="Y164">
+        <v>48</v>
+      </c>
+      <c r="Z164">
+        <v>18</v>
+      </c>
+      <c r="AA164">
+        <v>10</v>
+      </c>
+      <c r="AB164">
+        <v>4.63556</v>
+      </c>
+      <c r="AC164">
+        <v>-3.69561</v>
+      </c>
+      <c r="AD164">
+        <v>0</v>
+      </c>
+      <c r="AE164">
+        <v>387.8049</v>
+      </c>
+      <c r="AF164">
+        <v>0</v>
+      </c>
+      <c r="AG164">
+        <v>3</v>
+      </c>
+      <c r="AH164">
+        <v>1281.14109</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B165" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E165">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F165">
+        <v>5024.37</v>
+      </c>
+      <c r="G165">
+        <v>47.54181917965492</v>
+      </c>
+      <c r="H165">
+        <v>125.63</v>
+      </c>
+      <c r="I165">
+        <v>0</v>
+      </c>
+      <c r="J165">
+        <v>0</v>
+      </c>
+      <c r="K165">
+        <v>1.188741821072104</v>
+      </c>
+      <c r="L165">
+        <v>0</v>
+      </c>
+      <c r="M165">
+        <v>0</v>
+      </c>
+      <c r="N165">
+        <v>25.77041</v>
+      </c>
+      <c r="O165">
+        <v>76.47913698955365</v>
+      </c>
+      <c r="P165">
+        <v>33.696</v>
+      </c>
+      <c r="Q165">
+        <v>467.84831</v>
+      </c>
+      <c r="R165">
+        <v>4.426895263988746</v>
+      </c>
+      <c r="S165">
+        <v>604.1600100000001</v>
+      </c>
+      <c r="T165">
+        <v>14</v>
+      </c>
+      <c r="U165">
+        <v>6</v>
+      </c>
+      <c r="V165">
+        <v>20</v>
+      </c>
+      <c r="W165">
+        <v>50</v>
+      </c>
+      <c r="X165">
+        <v>14</v>
+      </c>
+      <c r="Y165">
+        <v>52</v>
+      </c>
+      <c r="Z165">
+        <v>6</v>
+      </c>
+      <c r="AA165">
+        <v>5</v>
+      </c>
+      <c r="AB165">
+        <v>3.84533</v>
+      </c>
+      <c r="AC165">
+        <v>-1.60047</v>
+      </c>
+      <c r="AD165">
+        <v>0</v>
+      </c>
+      <c r="AE165">
+        <v>453.7904</v>
+      </c>
+      <c r="AF165">
+        <v>0</v>
+      </c>
+      <c r="AG165">
+        <v>3</v>
+      </c>
+      <c r="AH165">
+        <v>1403.54493</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B166" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E166">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F166">
+        <v>5265.5</v>
+      </c>
+      <c r="G166">
+        <v>49.82345028142294</v>
+      </c>
+      <c r="H166">
+        <v>224.31</v>
+      </c>
+      <c r="I166">
+        <v>0</v>
+      </c>
+      <c r="J166">
+        <v>0</v>
+      </c>
+      <c r="K166">
+        <v>2.12247614331516</v>
+      </c>
+      <c r="L166">
+        <v>7.119999999999999</v>
+      </c>
+      <c r="M166">
+        <v>1</v>
+      </c>
+      <c r="N166">
+        <v>30.70942</v>
+      </c>
+      <c r="O166">
+        <v>87.76125971650664</v>
+      </c>
+      <c r="P166">
+        <v>34.992</v>
+      </c>
+      <c r="Q166">
+        <v>424.64807</v>
+      </c>
+      <c r="R166">
+        <v>4.018124015335145</v>
+      </c>
+      <c r="S166">
+        <v>625.8</v>
+      </c>
+      <c r="T166">
+        <v>13</v>
+      </c>
+      <c r="U166">
+        <v>12</v>
+      </c>
+      <c r="V166">
+        <v>25</v>
+      </c>
+      <c r="W166">
+        <v>45</v>
+      </c>
+      <c r="X166">
+        <v>13</v>
+      </c>
+      <c r="Y166">
+        <v>41</v>
+      </c>
+      <c r="Z166">
+        <v>12</v>
+      </c>
+      <c r="AA166">
+        <v>6</v>
+      </c>
+      <c r="AB166">
+        <v>4.30512</v>
+      </c>
+      <c r="AC166">
+        <v>-0.82209</v>
+      </c>
+      <c r="AD166">
+        <v>0</v>
+      </c>
+      <c r="AE166">
+        <v>410.96745</v>
+      </c>
+      <c r="AF166">
+        <v>0</v>
+      </c>
+      <c r="AG166">
+        <v>3</v>
+      </c>
+      <c r="AH166">
+        <v>1273.94421</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B167" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E167">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F167">
+        <v>5938.690000000001</v>
+      </c>
+      <c r="G167">
+        <v>56.19333889503059</v>
+      </c>
+      <c r="H167">
+        <v>250.12</v>
+      </c>
+      <c r="I167">
+        <v>0</v>
+      </c>
+      <c r="J167">
+        <v>0</v>
+      </c>
+      <c r="K167">
+        <v>2.366696683010066</v>
+      </c>
+      <c r="L167">
+        <v>0</v>
+      </c>
+      <c r="M167">
+        <v>0</v>
+      </c>
+      <c r="N167">
+        <v>27.50342</v>
+      </c>
+      <c r="O167">
+        <v>78.76122565864833</v>
+      </c>
+      <c r="P167">
+        <v>34.92</v>
+      </c>
+      <c r="Q167">
+        <v>467.10749</v>
+      </c>
+      <c r="R167">
+        <v>4.419885443755628</v>
+      </c>
+      <c r="S167">
+        <v>746.18999</v>
+      </c>
+      <c r="T167">
+        <v>23</v>
+      </c>
+      <c r="U167">
+        <v>5</v>
+      </c>
+      <c r="V167">
+        <v>28</v>
+      </c>
+      <c r="W167">
+        <v>62</v>
+      </c>
+      <c r="X167">
+        <v>23</v>
+      </c>
+      <c r="Y167">
+        <v>43</v>
+      </c>
+      <c r="Z167">
+        <v>5</v>
+      </c>
+      <c r="AA167">
+        <v>3</v>
+      </c>
+      <c r="AB167">
+        <v>4.18847</v>
+      </c>
+      <c r="AC167">
+        <v>-1.42119</v>
+      </c>
+      <c r="AD167">
+        <v>0</v>
+      </c>
+      <c r="AE167">
+        <v>542.5672</v>
+      </c>
+      <c r="AF167">
+        <v>0</v>
+      </c>
+      <c r="AG167">
+        <v>3</v>
+      </c>
+      <c r="AH167">
+        <v>1401.32247</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B168" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E168">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F168">
+        <v>5472.22</v>
+      </c>
+      <c r="G168">
+        <v>51.77948553774726</v>
+      </c>
+      <c r="H168">
+        <v>153.22</v>
+      </c>
+      <c r="I168">
+        <v>0</v>
+      </c>
+      <c r="J168">
+        <v>0</v>
+      </c>
+      <c r="K168">
+        <v>1.449805156608038</v>
+      </c>
+      <c r="L168">
+        <v>0</v>
+      </c>
+      <c r="M168">
+        <v>0</v>
+      </c>
+      <c r="N168">
+        <v>27.73444</v>
+      </c>
+      <c r="O168">
+        <v>79.25937357110196</v>
+      </c>
+      <c r="P168">
+        <v>34.992</v>
+      </c>
+      <c r="Q168">
+        <v>435.50507</v>
+      </c>
+      <c r="R168">
+        <v>4.120855607720561</v>
+      </c>
+      <c r="S168">
+        <v>656.07001</v>
+      </c>
+      <c r="T168">
+        <v>11</v>
+      </c>
+      <c r="U168">
+        <v>9</v>
+      </c>
+      <c r="V168">
+        <v>20</v>
+      </c>
+      <c r="W168">
+        <v>55</v>
+      </c>
+      <c r="X168">
+        <v>11</v>
+      </c>
+      <c r="Y168">
+        <v>45</v>
+      </c>
+      <c r="Z168">
+        <v>9</v>
+      </c>
+      <c r="AA168">
+        <v>8</v>
+      </c>
+      <c r="AB168">
+        <v>4.65456</v>
+      </c>
+      <c r="AC168">
+        <v>-1.2058</v>
+      </c>
+      <c r="AD168">
+        <v>0</v>
+      </c>
+      <c r="AE168">
+        <v>440.4690900000001</v>
+      </c>
+      <c r="AF168">
+        <v>0</v>
+      </c>
+      <c r="AG168">
+        <v>3</v>
+      </c>
+      <c r="AH168">
+        <v>1306.51521</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Luis Ángel Malagón</t>
+        </is>
+      </c>
+      <c r="B169" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E169">
+        <v>37.5395</v>
+      </c>
+      <c r="F169">
+        <v>947.63</v>
+      </c>
+      <c r="G169">
+        <v>25.24354346754752</v>
+      </c>
+      <c r="H169">
+        <v>0</v>
+      </c>
+      <c r="I169">
+        <v>0</v>
+      </c>
+      <c r="J169">
+        <v>0</v>
+      </c>
+      <c r="K169">
+        <v>0</v>
+      </c>
+      <c r="L169">
+        <v>0</v>
+      </c>
+      <c r="M169">
+        <v>0</v>
+      </c>
+      <c r="N169">
+        <v>12.55742</v>
+      </c>
+      <c r="O169">
+        <v>41.87481659330399</v>
+      </c>
+      <c r="P169">
+        <v>29.988</v>
+      </c>
+      <c r="Q169">
+        <v>89.83387999999999</v>
+      </c>
+      <c r="R169">
+        <v>2.393049454574515</v>
+      </c>
+      <c r="S169">
+        <v>0</v>
+      </c>
+      <c r="T169">
+        <v>0</v>
+      </c>
+      <c r="U169">
+        <v>0</v>
+      </c>
+      <c r="V169">
+        <v>0</v>
+      </c>
+      <c r="W169">
+        <v>0</v>
+      </c>
+      <c r="X169">
+        <v>0</v>
+      </c>
+      <c r="Y169">
+        <v>0</v>
+      </c>
+      <c r="Z169">
+        <v>0</v>
+      </c>
+      <c r="AA169">
+        <v>0</v>
+      </c>
+      <c r="AB169">
+        <v>1.25924</v>
+      </c>
+      <c r="AC169">
+        <v>-1.22384</v>
+      </c>
+      <c r="AD169">
+        <v>0</v>
+      </c>
+      <c r="AE169">
+        <v>77.15916</v>
+      </c>
+      <c r="AF169">
+        <v>0</v>
+      </c>
+      <c r="AG169">
+        <v>3</v>
+      </c>
+      <c r="AH169">
+        <v>269.50164</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B170" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E170">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F170">
+        <v>4613.469999999999</v>
+      </c>
+      <c r="G170">
+        <v>43.65378276893671</v>
+      </c>
+      <c r="H170">
+        <v>29.61</v>
+      </c>
+      <c r="I170">
+        <v>0</v>
+      </c>
+      <c r="J170">
+        <v>0</v>
+      </c>
+      <c r="K170">
+        <v>0.280177070142044</v>
+      </c>
+      <c r="L170">
+        <v>0</v>
+      </c>
+      <c r="M170">
+        <v>0</v>
+      </c>
+      <c r="N170">
+        <v>22.36652</v>
+      </c>
+      <c r="O170">
+        <v>65.81485404896422</v>
+      </c>
+      <c r="P170">
+        <v>33.984</v>
+      </c>
+      <c r="Q170">
+        <v>436.54252</v>
+      </c>
+      <c r="R170">
+        <v>4.130672213644873</v>
+      </c>
+      <c r="S170">
+        <v>272.29999</v>
+      </c>
+      <c r="T170">
+        <v>7</v>
+      </c>
+      <c r="U170">
+        <v>5</v>
+      </c>
+      <c r="V170">
+        <v>12</v>
+      </c>
+      <c r="W170">
+        <v>24</v>
+      </c>
+      <c r="X170">
+        <v>7</v>
+      </c>
+      <c r="Y170">
+        <v>24</v>
+      </c>
+      <c r="Z170">
+        <v>5</v>
+      </c>
+      <c r="AA170">
+        <v>5</v>
+      </c>
+      <c r="AB170">
+        <v>4.21023</v>
+      </c>
+      <c r="AC170">
+        <v>-0.82694</v>
+      </c>
+      <c r="AD170">
+        <v>0</v>
+      </c>
+      <c r="AE170">
+        <v>406.048</v>
+      </c>
+      <c r="AF170">
+        <v>0</v>
+      </c>
+      <c r="AG170">
+        <v>3</v>
+      </c>
+      <c r="AH170">
+        <v>1309.62756</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B171" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E171">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F171">
+        <v>4747.48</v>
+      </c>
+      <c r="G171">
+        <v>44.92181820188961</v>
+      </c>
+      <c r="H171">
+        <v>38.28</v>
+      </c>
+      <c r="I171">
+        <v>0</v>
+      </c>
+      <c r="J171">
+        <v>0</v>
+      </c>
+      <c r="K171">
+        <v>0.3622147330306467</v>
+      </c>
+      <c r="L171">
+        <v>0</v>
+      </c>
+      <c r="M171">
+        <v>0</v>
+      </c>
+      <c r="N171">
+        <v>24.53837</v>
+      </c>
+      <c r="O171">
+        <v>74.33166727250696</v>
+      </c>
+      <c r="P171">
+        <v>33.012</v>
+      </c>
+      <c r="Q171">
+        <v>440.98581</v>
+      </c>
+      <c r="R171">
+        <v>4.172715711584469</v>
+      </c>
+      <c r="S171">
+        <v>431.37999</v>
+      </c>
+      <c r="T171">
+        <v>8</v>
+      </c>
+      <c r="U171">
+        <v>9</v>
+      </c>
+      <c r="V171">
+        <v>17</v>
+      </c>
+      <c r="W171">
+        <v>44</v>
+      </c>
+      <c r="X171">
+        <v>8</v>
+      </c>
+      <c r="Y171">
+        <v>35</v>
+      </c>
+      <c r="Z171">
+        <v>9</v>
+      </c>
+      <c r="AA171">
+        <v>13</v>
+      </c>
+      <c r="AB171">
+        <v>3.46219</v>
+      </c>
+      <c r="AC171">
+        <v>-1.00065</v>
+      </c>
+      <c r="AD171">
+        <v>0</v>
+      </c>
+      <c r="AE171">
+        <v>395.90325</v>
+      </c>
+      <c r="AF171">
+        <v>0</v>
+      </c>
+      <c r="AG171">
+        <v>3</v>
+      </c>
+      <c r="AH171">
+        <v>1322.95743</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B172" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E172">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F172">
+        <v>5150.190000000001</v>
+      </c>
+      <c r="G172">
+        <v>48.73235882724938</v>
+      </c>
+      <c r="H172">
+        <v>57.84</v>
+      </c>
+      <c r="I172">
+        <v>0</v>
+      </c>
+      <c r="J172">
+        <v>0</v>
+      </c>
+      <c r="K172">
+        <v>0.5472962423848642</v>
+      </c>
+      <c r="L172">
+        <v>0</v>
+      </c>
+      <c r="M172">
+        <v>0</v>
+      </c>
+      <c r="N172">
+        <v>26.73995</v>
+      </c>
+      <c r="O172">
+        <v>83.55189976252969</v>
+      </c>
+      <c r="P172">
+        <v>32.004</v>
+      </c>
+      <c r="Q172">
+        <v>464.15392</v>
+      </c>
+      <c r="R172">
+        <v>4.391938041220692</v>
+      </c>
+      <c r="S172">
+        <v>486.08001</v>
+      </c>
+      <c r="T172">
+        <v>8</v>
+      </c>
+      <c r="U172">
+        <v>6</v>
+      </c>
+      <c r="V172">
+        <v>14</v>
+      </c>
+      <c r="W172">
+        <v>44</v>
+      </c>
+      <c r="X172">
+        <v>8</v>
+      </c>
+      <c r="Y172">
+        <v>36</v>
+      </c>
+      <c r="Z172">
+        <v>6</v>
+      </c>
+      <c r="AA172">
+        <v>7</v>
+      </c>
+      <c r="AB172">
+        <v>3.83922</v>
+      </c>
+      <c r="AC172">
+        <v>-1.13204</v>
+      </c>
+      <c r="AD172">
+        <v>0</v>
+      </c>
+      <c r="AE172">
+        <v>405.4883</v>
+      </c>
+      <c r="AF172">
+        <v>0</v>
+      </c>
+      <c r="AG172">
+        <v>3</v>
+      </c>
+      <c r="AH172">
+        <v>1392.46176</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B173" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E173">
+        <v>105.6831666666667</v>
+      </c>
+      <c r="F173">
+        <v>2972.92</v>
+      </c>
+      <c r="G173">
+        <v>28.13049697287016</v>
+      </c>
+      <c r="H173">
+        <v>30.82</v>
+      </c>
+      <c r="I173">
+        <v>0</v>
+      </c>
+      <c r="J173">
+        <v>0</v>
+      </c>
+      <c r="K173">
+        <v>0.2916263864160013</v>
+      </c>
+      <c r="L173">
+        <v>0</v>
+      </c>
+      <c r="M173">
+        <v>0</v>
+      </c>
+      <c r="N173">
+        <v>24.64282</v>
+      </c>
+      <c r="O173">
+        <v>68.45227777777778</v>
+      </c>
+      <c r="P173">
+        <v>36</v>
+      </c>
+      <c r="Q173">
+        <v>334.48109</v>
+      </c>
+      <c r="R173">
+        <v>3.16494197278343</v>
+      </c>
+      <c r="S173">
+        <v>235.40999</v>
+      </c>
+      <c r="T173">
+        <v>1</v>
+      </c>
+      <c r="U173">
+        <v>6</v>
+      </c>
+      <c r="V173">
+        <v>7</v>
+      </c>
+      <c r="W173">
+        <v>23</v>
+      </c>
+      <c r="X173">
+        <v>1</v>
+      </c>
+      <c r="Y173">
+        <v>19</v>
+      </c>
+      <c r="Z173">
+        <v>6</v>
+      </c>
+      <c r="AA173">
+        <v>12</v>
+      </c>
+      <c r="AB173">
+        <v>3.11706</v>
+      </c>
+      <c r="AC173">
+        <v>0</v>
+      </c>
+      <c r="AD173">
+        <v>0</v>
+      </c>
+      <c r="AE173">
+        <v>230.3392</v>
+      </c>
+      <c r="AF173">
+        <v>0</v>
+      </c>
+      <c r="AG173">
+        <v>3</v>
+      </c>
+      <c r="AH173">
+        <v>1003.44327</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B174" s="2">
+        <v>46193</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Sesión 10 pretemporada</t>
+        </is>
+      </c>
+      <c r="E174">
+        <v>37.5395</v>
+      </c>
+      <c r="F174">
+        <v>838</v>
+      </c>
+      <c r="G174">
+        <v>22.32315294556401</v>
+      </c>
+      <c r="H174">
+        <v>0</v>
+      </c>
+      <c r="I174">
+        <v>0</v>
+      </c>
+      <c r="J174">
+        <v>0</v>
+      </c>
+      <c r="K174">
+        <v>0</v>
+      </c>
+      <c r="L174">
+        <v>0</v>
+      </c>
+      <c r="M174">
+        <v>0</v>
+      </c>
+      <c r="N174">
+        <v>9.45923</v>
+      </c>
+      <c r="O174">
+        <v>27.83436322975518</v>
+      </c>
+      <c r="P174">
+        <v>33.984</v>
+      </c>
+      <c r="Q174">
+        <v>91.35905</v>
+      </c>
+      <c r="R174">
+        <v>2.433677859321515</v>
+      </c>
+      <c r="S174">
+        <v>0</v>
+      </c>
+      <c r="T174">
+        <v>0</v>
+      </c>
+      <c r="U174">
+        <v>0</v>
+      </c>
+      <c r="V174">
+        <v>0</v>
+      </c>
+      <c r="W174">
+        <v>0</v>
+      </c>
+      <c r="X174">
+        <v>0</v>
+      </c>
+      <c r="Y174">
+        <v>0</v>
+      </c>
+      <c r="Z174">
+        <v>0</v>
+      </c>
+      <c r="AA174">
+        <v>0</v>
+      </c>
+      <c r="AB174">
+        <v>1.21581</v>
+      </c>
+      <c r="AC174">
+        <v>-1.24056</v>
+      </c>
+      <c r="AD174">
+        <v>0</v>
+      </c>
+      <c r="AE174">
+        <v>58.3919</v>
+      </c>
+      <c r="AF174">
+        <v>0</v>
+      </c>
+      <c r="AG174">
+        <v>3</v>
+      </c>
+      <c r="AH174">
+        <v>274.07715</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B175" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E175">
+        <v>66.039</v>
+      </c>
+      <c r="F175">
+        <v>7934.62</v>
+      </c>
+      <c r="G175">
+        <v>120.1505171186723</v>
+      </c>
+      <c r="H175">
+        <v>169.87</v>
+      </c>
+      <c r="I175">
+        <v>0</v>
+      </c>
+      <c r="J175">
+        <v>0</v>
+      </c>
+      <c r="K175">
+        <v>2.572267902300156</v>
+      </c>
+      <c r="L175">
+        <v>0</v>
+      </c>
+      <c r="M175">
+        <v>0</v>
+      </c>
+      <c r="N175">
+        <v>26.31018</v>
+      </c>
+      <c r="O175">
+        <v>81.29458657767891</v>
+      </c>
+      <c r="P175">
+        <v>32.364</v>
+      </c>
+      <c r="Q175">
+        <v>765.6454200000001</v>
+      </c>
+      <c r="R175">
+        <v>11.59383727797211</v>
+      </c>
+      <c r="S175">
+        <v>1018.09998</v>
+      </c>
+      <c r="T175">
+        <v>7</v>
+      </c>
+      <c r="U175">
+        <v>15</v>
+      </c>
+      <c r="V175">
+        <v>22</v>
+      </c>
+      <c r="W175">
+        <v>55</v>
+      </c>
+      <c r="X175">
+        <v>7</v>
+      </c>
+      <c r="Y175">
+        <v>50</v>
+      </c>
+      <c r="Z175">
+        <v>15</v>
+      </c>
+      <c r="AA175">
+        <v>11</v>
+      </c>
+      <c r="AB175">
+        <v>3.95879</v>
+      </c>
+      <c r="AC175">
+        <v>-4.31425</v>
+      </c>
+      <c r="AD175">
+        <v>0</v>
+      </c>
+      <c r="AE175">
+        <v>636.9258</v>
+      </c>
+      <c r="AF175">
+        <v>0</v>
+      </c>
+      <c r="AG175">
+        <v>3</v>
+      </c>
+      <c r="AH175">
+        <v>2296.93626</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B176" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E176">
+        <v>66.039</v>
+      </c>
+      <c r="F176">
+        <v>6331.5</v>
+      </c>
+      <c r="G176">
+        <v>95.87516467541907</v>
+      </c>
+      <c r="H176">
+        <v>444.79</v>
+      </c>
+      <c r="I176">
+        <v>0</v>
+      </c>
+      <c r="J176">
+        <v>0</v>
+      </c>
+      <c r="K176">
+        <v>6.73526249640364</v>
+      </c>
+      <c r="L176">
+        <v>8.85</v>
+      </c>
+      <c r="M176">
+        <v>1</v>
+      </c>
+      <c r="N176">
+        <v>30.25315</v>
+      </c>
+      <c r="O176">
+        <v>89.02174552730698</v>
+      </c>
+      <c r="P176">
+        <v>33.984</v>
+      </c>
+      <c r="Q176">
+        <v>679.71973</v>
+      </c>
+      <c r="R176">
+        <v>10.29270173685247</v>
+      </c>
+      <c r="S176">
+        <v>951.1200200000001</v>
+      </c>
+      <c r="T176">
+        <v>20</v>
+      </c>
+      <c r="U176">
+        <v>18</v>
+      </c>
+      <c r="V176">
+        <v>38</v>
+      </c>
+      <c r="W176">
+        <v>71</v>
+      </c>
+      <c r="X176">
+        <v>20</v>
+      </c>
+      <c r="Y176">
+        <v>59</v>
+      </c>
+      <c r="Z176">
+        <v>18</v>
+      </c>
+      <c r="AA176">
+        <v>14</v>
+      </c>
+      <c r="AB176">
+        <v>4.22058</v>
+      </c>
+      <c r="AC176">
+        <v>-4.94665</v>
+      </c>
+      <c r="AD176">
+        <v>0</v>
+      </c>
+      <c r="AE176">
+        <v>598.424</v>
+      </c>
+      <c r="AF176">
+        <v>0</v>
+      </c>
+      <c r="AG176">
+        <v>3</v>
+      </c>
+      <c r="AH176">
+        <v>2039.15919</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B177" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E177">
+        <v>66.336</v>
+      </c>
+      <c r="F177">
+        <v>7586.370000000001</v>
+      </c>
+      <c r="G177">
+        <v>114.3627894356006</v>
+      </c>
+      <c r="H177">
+        <v>476.17</v>
+      </c>
+      <c r="I177">
+        <v>0</v>
+      </c>
+      <c r="J177">
+        <v>0</v>
+      </c>
+      <c r="K177">
+        <v>7.178153642064641</v>
+      </c>
+      <c r="L177">
+        <v>0</v>
+      </c>
+      <c r="M177">
+        <v>0</v>
+      </c>
+      <c r="N177">
+        <v>29.09188</v>
+      </c>
+      <c r="O177">
+        <v>81.79228520017993</v>
+      </c>
+      <c r="P177">
+        <v>35.568</v>
+      </c>
+      <c r="Q177">
+        <v>656.3118899999999</v>
+      </c>
+      <c r="R177">
+        <v>9.893751356729377</v>
+      </c>
+      <c r="S177">
+        <v>1193.69</v>
+      </c>
+      <c r="T177">
+        <v>30</v>
+      </c>
+      <c r="U177">
+        <v>25</v>
+      </c>
+      <c r="V177">
+        <v>55</v>
+      </c>
+      <c r="W177">
+        <v>80</v>
+      </c>
+      <c r="X177">
+        <v>30</v>
+      </c>
+      <c r="Y177">
+        <v>67</v>
+      </c>
+      <c r="Z177">
+        <v>25</v>
+      </c>
+      <c r="AA177">
+        <v>15</v>
+      </c>
+      <c r="AB177">
+        <v>4.85114</v>
+      </c>
+      <c r="AC177">
+        <v>-5.47612</v>
+      </c>
+      <c r="AD177">
+        <v>0</v>
+      </c>
+      <c r="AE177">
+        <v>716.3887999999999</v>
+      </c>
+      <c r="AF177">
+        <v>0</v>
+      </c>
+      <c r="AG177">
+        <v>3</v>
+      </c>
+      <c r="AH177">
+        <v>1968.93567</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B178" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E178">
+        <v>62.65833333333333</v>
+      </c>
+      <c r="F178">
+        <v>6945.650000000001</v>
+      </c>
+      <c r="G178">
+        <v>110.8495810613114</v>
+      </c>
+      <c r="H178">
+        <v>492.3800000000001</v>
+      </c>
+      <c r="I178">
+        <v>0</v>
+      </c>
+      <c r="J178">
+        <v>0</v>
+      </c>
+      <c r="K178">
+        <v>7.858172629339009</v>
+      </c>
+      <c r="L178">
+        <v>51.94</v>
+      </c>
+      <c r="M178">
+        <v>3</v>
+      </c>
+      <c r="N178">
+        <v>31.24134</v>
+      </c>
+      <c r="O178">
+        <v>86.78149999999999</v>
+      </c>
+      <c r="P178">
+        <v>36</v>
+      </c>
+      <c r="Q178">
+        <v>588.49854</v>
+      </c>
+      <c r="R178">
+        <v>9.392183109456045</v>
+      </c>
+      <c r="S178">
+        <v>1246.72003</v>
+      </c>
+      <c r="T178">
+        <v>16</v>
+      </c>
+      <c r="U178">
+        <v>36</v>
+      </c>
+      <c r="V178">
+        <v>52</v>
+      </c>
+      <c r="W178">
+        <v>75</v>
+      </c>
+      <c r="X178">
+        <v>16</v>
+      </c>
+      <c r="Y178">
+        <v>65</v>
+      </c>
+      <c r="Z178">
+        <v>36</v>
+      </c>
+      <c r="AA178">
+        <v>35</v>
+      </c>
+      <c r="AB178">
+        <v>3.98883</v>
+      </c>
+      <c r="AC178">
+        <v>-4.79059</v>
+      </c>
+      <c r="AD178">
+        <v>0</v>
+      </c>
+      <c r="AE178">
+        <v>582.0269</v>
+      </c>
+      <c r="AF178">
+        <v>0</v>
+      </c>
+      <c r="AG178">
+        <v>3</v>
+      </c>
+      <c r="AH178">
+        <v>1765.49562</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B179" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E179">
+        <v>66.039</v>
+      </c>
+      <c r="F179">
+        <v>7272.85</v>
+      </c>
+      <c r="G179">
+        <v>110.1296203758385</v>
+      </c>
+      <c r="H179">
+        <v>145.95</v>
+      </c>
+      <c r="I179">
+        <v>0</v>
+      </c>
+      <c r="J179">
+        <v>0</v>
+      </c>
+      <c r="K179">
+        <v>2.210057693181302</v>
+      </c>
+      <c r="L179">
+        <v>0</v>
+      </c>
+      <c r="M179">
+        <v>0</v>
+      </c>
+      <c r="N179">
+        <v>28.54741</v>
+      </c>
+      <c r="O179">
+        <v>89.19950631171105</v>
+      </c>
+      <c r="P179">
+        <v>32.004</v>
+      </c>
+      <c r="Q179">
+        <v>772.85559</v>
+      </c>
+      <c r="R179">
+        <v>11.70301776223141</v>
+      </c>
+      <c r="S179">
+        <v>882.98996</v>
+      </c>
+      <c r="T179">
+        <v>9</v>
+      </c>
+      <c r="U179">
+        <v>15</v>
+      </c>
+      <c r="V179">
+        <v>24</v>
+      </c>
+      <c r="W179">
+        <v>51</v>
+      </c>
+      <c r="X179">
+        <v>9</v>
+      </c>
+      <c r="Y179">
+        <v>52</v>
+      </c>
+      <c r="Z179">
+        <v>15</v>
+      </c>
+      <c r="AA179">
+        <v>13</v>
+      </c>
+      <c r="AB179">
+        <v>4.51957</v>
+      </c>
+      <c r="AC179">
+        <v>-3.3094</v>
+      </c>
+      <c r="AD179">
+        <v>0</v>
+      </c>
+      <c r="AE179">
+        <v>503.1006</v>
+      </c>
+      <c r="AF179">
+        <v>0</v>
+      </c>
+      <c r="AG179">
+        <v>3</v>
+      </c>
+      <c r="AH179">
+        <v>2318.56677</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B180" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E180">
+        <v>66.336</v>
+      </c>
+      <c r="F180">
+        <v>6566.07</v>
+      </c>
+      <c r="G180">
+        <v>98.982000723589</v>
+      </c>
+      <c r="H180">
+        <v>386.0700000000001</v>
+      </c>
+      <c r="I180">
+        <v>0</v>
+      </c>
+      <c r="J180">
+        <v>0</v>
+      </c>
+      <c r="K180">
+        <v>5.819916787264835</v>
+      </c>
+      <c r="L180">
+        <v>0</v>
+      </c>
+      <c r="M180">
+        <v>0</v>
+      </c>
+      <c r="N180">
+        <v>29.60927</v>
+      </c>
+      <c r="O180">
+        <v>87.4978427895981</v>
+      </c>
+      <c r="P180">
+        <v>33.84</v>
+      </c>
+      <c r="Q180">
+        <v>590.09851</v>
+      </c>
+      <c r="R180">
+        <v>8.895599825132658</v>
+      </c>
+      <c r="S180">
+        <v>1173.37</v>
+      </c>
+      <c r="T180">
+        <v>32</v>
+      </c>
+      <c r="U180">
+        <v>26</v>
+      </c>
+      <c r="V180">
+        <v>58</v>
+      </c>
+      <c r="W180">
+        <v>89</v>
+      </c>
+      <c r="X180">
+        <v>32</v>
+      </c>
+      <c r="Y180">
+        <v>81</v>
+      </c>
+      <c r="Z180">
+        <v>26</v>
+      </c>
+      <c r="AA180">
+        <v>11</v>
+      </c>
+      <c r="AB180">
+        <v>4.42626</v>
+      </c>
+      <c r="AC180">
+        <v>-4.53224</v>
+      </c>
+      <c r="AD180">
+        <v>0</v>
+      </c>
+      <c r="AE180">
+        <v>557.7957</v>
+      </c>
+      <c r="AF180">
+        <v>0</v>
+      </c>
+      <c r="AG180">
+        <v>3</v>
+      </c>
+      <c r="AH180">
+        <v>1770.29553</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B181" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E181">
+        <v>66.039</v>
+      </c>
+      <c r="F181">
+        <v>6851.150000000001</v>
+      </c>
+      <c r="G181">
+        <v>103.7439997577189</v>
+      </c>
+      <c r="H181">
+        <v>302.15</v>
+      </c>
+      <c r="I181">
+        <v>0</v>
+      </c>
+      <c r="J181">
+        <v>0</v>
+      </c>
+      <c r="K181">
+        <v>4.575326700888868</v>
+      </c>
+      <c r="L181">
+        <v>0</v>
+      </c>
+      <c r="M181">
+        <v>0</v>
+      </c>
+      <c r="N181">
+        <v>28.08073</v>
+      </c>
+      <c r="O181">
+        <v>83.3354997625831</v>
+      </c>
+      <c r="P181">
+        <v>33.696</v>
+      </c>
+      <c r="Q181">
+        <v>602.7659</v>
+      </c>
+      <c r="R181">
+        <v>9.127423189327518</v>
+      </c>
+      <c r="S181">
+        <v>1097.44</v>
+      </c>
+      <c r="T181">
+        <v>18</v>
+      </c>
+      <c r="U181">
+        <v>18</v>
+      </c>
+      <c r="V181">
+        <v>36</v>
+      </c>
+      <c r="W181">
+        <v>86</v>
+      </c>
+      <c r="X181">
+        <v>18</v>
+      </c>
+      <c r="Y181">
+        <v>88</v>
+      </c>
+      <c r="Z181">
+        <v>18</v>
+      </c>
+      <c r="AA181">
+        <v>22</v>
+      </c>
+      <c r="AB181">
+        <v>3.81304</v>
+      </c>
+      <c r="AC181">
+        <v>-4.67614</v>
+      </c>
+      <c r="AD181">
+        <v>0</v>
+      </c>
+      <c r="AE181">
+        <v>648.5992</v>
+      </c>
+      <c r="AF181">
+        <v>0</v>
+      </c>
+      <c r="AG181">
+        <v>3</v>
+      </c>
+      <c r="AH181">
+        <v>1808.2977</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B182" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E182">
+        <v>66.039</v>
+      </c>
+      <c r="F182">
+        <v>7301.500000000001</v>
+      </c>
+      <c r="G182">
+        <v>110.5634549281485</v>
+      </c>
+      <c r="H182">
+        <v>239.6</v>
+      </c>
+      <c r="I182">
+        <v>0</v>
+      </c>
+      <c r="J182">
+        <v>0</v>
+      </c>
+      <c r="K182">
+        <v>3.628159118096882</v>
+      </c>
+      <c r="L182">
+        <v>13.34</v>
+      </c>
+      <c r="M182">
+        <v>1</v>
+      </c>
+      <c r="N182">
+        <v>30.83442</v>
+      </c>
+      <c r="O182">
+        <v>88.11848422496573</v>
+      </c>
+      <c r="P182">
+        <v>34.992</v>
+      </c>
+      <c r="Q182">
+        <v>617.01031</v>
+      </c>
+      <c r="R182">
+        <v>9.343120125986159</v>
+      </c>
+      <c r="S182">
+        <v>980.50003</v>
+      </c>
+      <c r="T182">
+        <v>17</v>
+      </c>
+      <c r="U182">
+        <v>21</v>
+      </c>
+      <c r="V182">
+        <v>38</v>
+      </c>
+      <c r="W182">
+        <v>70</v>
+      </c>
+      <c r="X182">
+        <v>17</v>
+      </c>
+      <c r="Y182">
+        <v>61</v>
+      </c>
+      <c r="Z182">
+        <v>21</v>
+      </c>
+      <c r="AA182">
+        <v>9</v>
+      </c>
+      <c r="AB182">
+        <v>4.23212</v>
+      </c>
+      <c r="AC182">
+        <v>-4.16708</v>
+      </c>
+      <c r="AD182">
+        <v>0</v>
+      </c>
+      <c r="AE182">
+        <v>584.24784</v>
+      </c>
+      <c r="AF182">
+        <v>0</v>
+      </c>
+      <c r="AG182">
+        <v>3</v>
+      </c>
+      <c r="AH182">
+        <v>1851.03093</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B183" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E183">
+        <v>62.65833333333333</v>
+      </c>
+      <c r="F183">
+        <v>6731.18</v>
+      </c>
+      <c r="G183">
+        <v>107.4267322782285</v>
+      </c>
+      <c r="H183">
+        <v>364.2300000000001</v>
+      </c>
+      <c r="I183">
+        <v>21.92</v>
+      </c>
+      <c r="J183">
+        <v>1</v>
+      </c>
+      <c r="K183">
+        <v>5.812953850246044</v>
+      </c>
+      <c r="L183">
+        <v>36.48</v>
+      </c>
+      <c r="M183">
+        <v>1</v>
+      </c>
+      <c r="N183">
+        <v>32.65497</v>
+      </c>
+      <c r="O183">
+        <v>93.51365979381443</v>
+      </c>
+      <c r="P183">
+        <v>34.92</v>
+      </c>
+      <c r="Q183">
+        <v>461.79134</v>
+      </c>
+      <c r="R183">
+        <v>7.369990796648491</v>
+      </c>
+      <c r="S183">
+        <v>928.44001</v>
+      </c>
+      <c r="T183">
+        <v>10</v>
+      </c>
+      <c r="U183">
+        <v>7</v>
+      </c>
+      <c r="V183">
+        <v>17</v>
+      </c>
+      <c r="W183">
+        <v>57</v>
+      </c>
+      <c r="X183">
+        <v>10</v>
+      </c>
+      <c r="Y183">
+        <v>44</v>
+      </c>
+      <c r="Z183">
+        <v>7</v>
+      </c>
+      <c r="AA183">
+        <v>13</v>
+      </c>
+      <c r="AB183">
+        <v>4.55477</v>
+      </c>
+      <c r="AC183">
+        <v>-4.0488</v>
+      </c>
+      <c r="AD183">
+        <v>0</v>
+      </c>
+      <c r="AE183">
+        <v>615.3768</v>
+      </c>
+      <c r="AF183">
+        <v>0</v>
+      </c>
+      <c r="AG183">
+        <v>3</v>
+      </c>
+      <c r="AH183">
+        <v>1385.37402</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B184" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E184">
+        <v>66.039</v>
+      </c>
+      <c r="F184">
+        <v>7220.47</v>
+      </c>
+      <c r="G184">
+        <v>109.3364527021911</v>
+      </c>
+      <c r="H184">
+        <v>341.57</v>
+      </c>
+      <c r="I184">
+        <v>0</v>
+      </c>
+      <c r="J184">
+        <v>0</v>
+      </c>
+      <c r="K184">
+        <v>5.172246702705976</v>
+      </c>
+      <c r="L184">
+        <v>0</v>
+      </c>
+      <c r="M184">
+        <v>0</v>
+      </c>
+      <c r="N184">
+        <v>28.78636</v>
+      </c>
+      <c r="O184">
+        <v>82.26554641060814</v>
+      </c>
+      <c r="P184">
+        <v>34.992</v>
+      </c>
+      <c r="Q184">
+        <v>571.88004</v>
+      </c>
+      <c r="R184">
+        <v>8.659731976559305</v>
+      </c>
+      <c r="S184">
+        <v>1311.41004</v>
+      </c>
+      <c r="T184">
+        <v>24</v>
+      </c>
+      <c r="U184">
+        <v>25</v>
+      </c>
+      <c r="V184">
+        <v>49</v>
+      </c>
+      <c r="W184">
+        <v>89</v>
+      </c>
+      <c r="X184">
+        <v>24</v>
+      </c>
+      <c r="Y184">
+        <v>86</v>
+      </c>
+      <c r="Z184">
+        <v>25</v>
+      </c>
+      <c r="AA184">
+        <v>15</v>
+      </c>
+      <c r="AB184">
+        <v>4.29975</v>
+      </c>
+      <c r="AC184">
+        <v>-5.11404</v>
+      </c>
+      <c r="AD184">
+        <v>0</v>
+      </c>
+      <c r="AE184">
+        <v>614.60653</v>
+      </c>
+      <c r="AF184">
+        <v>0</v>
+      </c>
+      <c r="AG184">
+        <v>3</v>
+      </c>
+      <c r="AH184">
+        <v>1715.64012</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B185" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E185">
+        <v>66.039</v>
+      </c>
+      <c r="F185">
+        <v>6397.8</v>
+      </c>
+      <c r="G185">
+        <v>96.87911688547676</v>
+      </c>
+      <c r="H185">
+        <v>210.56</v>
+      </c>
+      <c r="I185">
+        <v>11</v>
+      </c>
+      <c r="J185">
+        <v>1</v>
+      </c>
+      <c r="K185">
+        <v>3.18841896455125</v>
+      </c>
+      <c r="L185">
+        <v>16.95</v>
+      </c>
+      <c r="M185">
+        <v>1</v>
+      </c>
+      <c r="N185">
+        <v>31.63049</v>
+      </c>
+      <c r="O185">
+        <v>93.07465277777777</v>
+      </c>
+      <c r="P185">
+        <v>33.984</v>
+      </c>
+      <c r="Q185">
+        <v>571.2796599999999</v>
+      </c>
+      <c r="R185">
+        <v>8.650640682021228</v>
+      </c>
+      <c r="S185">
+        <v>714.15002</v>
+      </c>
+      <c r="T185">
+        <v>7</v>
+      </c>
+      <c r="U185">
+        <v>15</v>
+      </c>
+      <c r="V185">
+        <v>22</v>
+      </c>
+      <c r="W185">
+        <v>50</v>
+      </c>
+      <c r="X185">
+        <v>7</v>
+      </c>
+      <c r="Y185">
+        <v>54</v>
+      </c>
+      <c r="Z185">
+        <v>15</v>
+      </c>
+      <c r="AA185">
+        <v>14</v>
+      </c>
+      <c r="AB185">
+        <v>3.65081</v>
+      </c>
+      <c r="AC185">
+        <v>-4.60349</v>
+      </c>
+      <c r="AD185">
+        <v>0</v>
+      </c>
+      <c r="AE185">
+        <v>588.7872</v>
+      </c>
+      <c r="AF185">
+        <v>0</v>
+      </c>
+      <c r="AG185">
+        <v>3</v>
+      </c>
+      <c r="AH185">
+        <v>1713.83898</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B186" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E186">
+        <v>66.039</v>
+      </c>
+      <c r="F186">
+        <v>6317.47</v>
+      </c>
+      <c r="G186">
+        <v>95.66271445660898</v>
+      </c>
+      <c r="H186">
+        <v>243.8</v>
+      </c>
+      <c r="I186">
+        <v>0</v>
+      </c>
+      <c r="J186">
+        <v>0</v>
+      </c>
+      <c r="K186">
+        <v>3.691757900634473</v>
+      </c>
+      <c r="L186">
+        <v>0</v>
+      </c>
+      <c r="M186">
+        <v>0</v>
+      </c>
+      <c r="N186">
+        <v>29.5884</v>
+      </c>
+      <c r="O186">
+        <v>89.62922573609596</v>
+      </c>
+      <c r="P186">
+        <v>33.012</v>
+      </c>
+      <c r="Q186">
+        <v>588.98489</v>
+      </c>
+      <c r="R186">
+        <v>8.918743318342191</v>
+      </c>
+      <c r="S186">
+        <v>880.22</v>
+      </c>
+      <c r="T186">
+        <v>16</v>
+      </c>
+      <c r="U186">
+        <v>20</v>
+      </c>
+      <c r="V186">
+        <v>36</v>
+      </c>
+      <c r="W186">
+        <v>64</v>
+      </c>
+      <c r="X186">
+        <v>16</v>
+      </c>
+      <c r="Y186">
+        <v>64</v>
+      </c>
+      <c r="Z186">
+        <v>20</v>
+      </c>
+      <c r="AA186">
+        <v>14</v>
+      </c>
+      <c r="AB186">
+        <v>4.0474</v>
+      </c>
+      <c r="AC186">
+        <v>-4.40888</v>
+      </c>
+      <c r="AD186">
+        <v>0</v>
+      </c>
+      <c r="AE186">
+        <v>553.7505</v>
+      </c>
+      <c r="AF186">
+        <v>0</v>
+      </c>
+      <c r="AG186">
+        <v>3</v>
+      </c>
+      <c r="AH186">
+        <v>1766.95467</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B187" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E187">
+        <v>66.039</v>
+      </c>
+      <c r="F187">
+        <v>7275.8</v>
+      </c>
+      <c r="G187">
+        <v>110.1742909492875</v>
+      </c>
+      <c r="H187">
+        <v>230.04</v>
+      </c>
+      <c r="I187">
+        <v>0</v>
+      </c>
+      <c r="J187">
+        <v>0</v>
+      </c>
+      <c r="K187">
+        <v>3.483396174987507</v>
+      </c>
+      <c r="L187">
+        <v>0</v>
+      </c>
+      <c r="M187">
+        <v>0</v>
+      </c>
+      <c r="N187">
+        <v>27.5621</v>
+      </c>
+      <c r="O187">
+        <v>86.12079740032496</v>
+      </c>
+      <c r="P187">
+        <v>32.004</v>
+      </c>
+      <c r="Q187">
+        <v>663.59942</v>
+      </c>
+      <c r="R187">
+        <v>10.04859885825043</v>
+      </c>
+      <c r="S187">
+        <v>910.73001</v>
+      </c>
+      <c r="T187">
+        <v>12</v>
+      </c>
+      <c r="U187">
+        <v>9</v>
+      </c>
+      <c r="V187">
+        <v>21</v>
+      </c>
+      <c r="W187">
+        <v>64</v>
+      </c>
+      <c r="X187">
+        <v>12</v>
+      </c>
+      <c r="Y187">
+        <v>52</v>
+      </c>
+      <c r="Z187">
+        <v>9</v>
+      </c>
+      <c r="AA187">
+        <v>9</v>
+      </c>
+      <c r="AB187">
+        <v>3.84877</v>
+      </c>
+      <c r="AC187">
+        <v>-3.93934</v>
+      </c>
+      <c r="AD187">
+        <v>0</v>
+      </c>
+      <c r="AE187">
+        <v>584.7156</v>
+      </c>
+      <c r="AF187">
+        <v>0</v>
+      </c>
+      <c r="AG187">
+        <v>3</v>
+      </c>
+      <c r="AH187">
+        <v>1990.79826</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B188" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Futbol </t>
+        </is>
+      </c>
+      <c r="E188">
+        <v>62.65833333333333</v>
+      </c>
+      <c r="F188">
+        <v>6568.75</v>
+      </c>
+      <c r="G188">
+        <v>104.8344194706743</v>
+      </c>
+      <c r="H188">
+        <v>498.7</v>
+      </c>
+      <c r="I188">
+        <v>0</v>
+      </c>
+      <c r="J188">
+        <v>0</v>
+      </c>
+      <c r="K188">
+        <v>7.959037105998138</v>
+      </c>
+      <c r="L188">
+        <v>16.84</v>
+      </c>
+      <c r="M188">
+        <v>1</v>
+      </c>
+      <c r="N188">
+        <v>31.69526</v>
+      </c>
+      <c r="O188">
+        <v>88.04238888888889</v>
+      </c>
+      <c r="P188">
+        <v>36</v>
+      </c>
+      <c r="Q188">
+        <v>586.50848</v>
+      </c>
+      <c r="R188">
+        <v>9.360422609389547</v>
+      </c>
+      <c r="S188">
+        <v>1100.04001</v>
+      </c>
+      <c r="T188">
+        <v>18</v>
+      </c>
+      <c r="U188">
+        <v>27</v>
+      </c>
+      <c r="V188">
+        <v>45</v>
+      </c>
+      <c r="W188">
+        <v>66</v>
+      </c>
+      <c r="X188">
+        <v>18</v>
+      </c>
+      <c r="Y188">
+        <v>70</v>
+      </c>
+      <c r="Z188">
+        <v>27</v>
+      </c>
+      <c r="AA188">
+        <v>20</v>
+      </c>
+      <c r="AB188">
+        <v>3.95816</v>
+      </c>
+      <c r="AC188">
+        <v>-4.7201</v>
+      </c>
+      <c r="AD188">
+        <v>0</v>
+      </c>
+      <c r="AE188">
+        <v>540.8501</v>
+      </c>
+      <c r="AF188">
+        <v>0</v>
+      </c>
+      <c r="AG188">
+        <v>3</v>
+      </c>
+      <c r="AH188">
+        <v>1759.52544</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-22
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH188"/>
+  <dimension ref="A1:AH204"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -19484,7 +19484,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E175">
@@ -19594,7 +19594,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E176">
@@ -19704,7 +19704,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E177">
@@ -19814,7 +19814,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E178">
@@ -19924,7 +19924,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E179">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E180">
@@ -20144,7 +20144,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E181">
@@ -20254,7 +20254,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E182">
@@ -20364,7 +20364,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E183">
@@ -20474,7 +20474,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E184">
@@ -20584,7 +20584,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E185">
@@ -20694,7 +20694,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E186">
@@ -20804,7 +20804,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E187">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Futbol </t>
+          <t>Sesión 11 Futbol</t>
         </is>
       </c>
       <c r="E188">
@@ -21006,6 +21006,1766 @@
       </c>
       <c r="AH188">
         <v>1759.52544</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B189" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E189">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F189">
+        <v>5195.11</v>
+      </c>
+      <c r="G189">
+        <v>48.4543136950101</v>
+      </c>
+      <c r="H189">
+        <v>45.89</v>
+      </c>
+      <c r="I189">
+        <v>0</v>
+      </c>
+      <c r="J189">
+        <v>0</v>
+      </c>
+      <c r="K189">
+        <v>0.4280118140836313</v>
+      </c>
+      <c r="L189">
+        <v>0</v>
+      </c>
+      <c r="M189">
+        <v>0</v>
+      </c>
+      <c r="N189">
+        <v>23.02415</v>
+      </c>
+      <c r="O189">
+        <v>71.14123717711037</v>
+      </c>
+      <c r="P189">
+        <v>32.364</v>
+      </c>
+      <c r="Q189">
+        <v>583.91674</v>
+      </c>
+      <c r="R189">
+        <v>5.446137789522773</v>
+      </c>
+      <c r="S189">
+        <v>1072.94997</v>
+      </c>
+      <c r="T189">
+        <v>26</v>
+      </c>
+      <c r="U189">
+        <v>35</v>
+      </c>
+      <c r="V189">
+        <v>61</v>
+      </c>
+      <c r="W189">
+        <v>101</v>
+      </c>
+      <c r="X189">
+        <v>26</v>
+      </c>
+      <c r="Y189">
+        <v>106</v>
+      </c>
+      <c r="Z189">
+        <v>35</v>
+      </c>
+      <c r="AA189">
+        <v>92</v>
+      </c>
+      <c r="AB189">
+        <v>4.03344</v>
+      </c>
+      <c r="AC189">
+        <v>-3.17966</v>
+      </c>
+      <c r="AD189">
+        <v>0</v>
+      </c>
+      <c r="AE189">
+        <v>435.3636</v>
+      </c>
+      <c r="AF189">
+        <v>0</v>
+      </c>
+      <c r="AG189">
+        <v>3</v>
+      </c>
+      <c r="AH189">
+        <v>1751.75022</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B190" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E190">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F190">
+        <v>5495.650000000001</v>
+      </c>
+      <c r="G190">
+        <v>51.25742266438676</v>
+      </c>
+      <c r="H190">
+        <v>125.76</v>
+      </c>
+      <c r="I190">
+        <v>0</v>
+      </c>
+      <c r="J190">
+        <v>0</v>
+      </c>
+      <c r="K190">
+        <v>1.172951966423131</v>
+      </c>
+      <c r="L190">
+        <v>0</v>
+      </c>
+      <c r="M190">
+        <v>0</v>
+      </c>
+      <c r="N190">
+        <v>23.85232</v>
+      </c>
+      <c r="O190">
+        <v>73.61827160493827</v>
+      </c>
+      <c r="P190">
+        <v>32.4</v>
+      </c>
+      <c r="Q190">
+        <v>692.9135699999999</v>
+      </c>
+      <c r="R190">
+        <v>6.462741209389087</v>
+      </c>
+      <c r="S190">
+        <v>1269.02001</v>
+      </c>
+      <c r="T190">
+        <v>49</v>
+      </c>
+      <c r="U190">
+        <v>62</v>
+      </c>
+      <c r="V190">
+        <v>111</v>
+      </c>
+      <c r="W190">
+        <v>116</v>
+      </c>
+      <c r="X190">
+        <v>49</v>
+      </c>
+      <c r="Y190">
+        <v>117</v>
+      </c>
+      <c r="Z190">
+        <v>62</v>
+      </c>
+      <c r="AA190">
+        <v>30</v>
+      </c>
+      <c r="AB190">
+        <v>4.04281</v>
+      </c>
+      <c r="AC190">
+        <v>-3.33386</v>
+      </c>
+      <c r="AD190">
+        <v>0</v>
+      </c>
+      <c r="AE190">
+        <v>481.6434</v>
+      </c>
+      <c r="AF190">
+        <v>0</v>
+      </c>
+      <c r="AG190">
+        <v>3</v>
+      </c>
+      <c r="AH190">
+        <v>2078.74071</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B191" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E191">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F191">
+        <v>4651.41</v>
+      </c>
+      <c r="G191">
+        <v>43.38327374475361</v>
+      </c>
+      <c r="H191">
+        <v>40.74999999999999</v>
+      </c>
+      <c r="I191">
+        <v>0</v>
+      </c>
+      <c r="J191">
+        <v>0</v>
+      </c>
+      <c r="K191">
+        <v>0.3800715062956629</v>
+      </c>
+      <c r="L191">
+        <v>0</v>
+      </c>
+      <c r="M191">
+        <v>0</v>
+      </c>
+      <c r="N191">
+        <v>23.48263</v>
+      </c>
+      <c r="O191">
+        <v>69.09907603578154</v>
+      </c>
+      <c r="P191">
+        <v>33.984</v>
+      </c>
+      <c r="Q191">
+        <v>634.18938</v>
+      </c>
+      <c r="R191">
+        <v>5.91502608425307</v>
+      </c>
+      <c r="S191">
+        <v>865.99002</v>
+      </c>
+      <c r="T191">
+        <v>36</v>
+      </c>
+      <c r="U191">
+        <v>34</v>
+      </c>
+      <c r="V191">
+        <v>70</v>
+      </c>
+      <c r="W191">
+        <v>90</v>
+      </c>
+      <c r="X191">
+        <v>36</v>
+      </c>
+      <c r="Y191">
+        <v>83</v>
+      </c>
+      <c r="Z191">
+        <v>34</v>
+      </c>
+      <c r="AA191">
+        <v>18</v>
+      </c>
+      <c r="AB191">
+        <v>4.19102</v>
+      </c>
+      <c r="AC191">
+        <v>-3.26787</v>
+      </c>
+      <c r="AD191">
+        <v>0</v>
+      </c>
+      <c r="AE191">
+        <v>448.1776</v>
+      </c>
+      <c r="AF191">
+        <v>0</v>
+      </c>
+      <c r="AG191">
+        <v>3</v>
+      </c>
+      <c r="AH191">
+        <v>1902.56814</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B192" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E192">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F192">
+        <v>5713.14</v>
+      </c>
+      <c r="G192">
+        <v>53.28593191357065</v>
+      </c>
+      <c r="H192">
+        <v>212.13</v>
+      </c>
+      <c r="I192">
+        <v>0</v>
+      </c>
+      <c r="J192">
+        <v>0</v>
+      </c>
+      <c r="K192">
+        <v>1.978517021607337</v>
+      </c>
+      <c r="L192">
+        <v>0</v>
+      </c>
+      <c r="M192">
+        <v>0</v>
+      </c>
+      <c r="N192">
+        <v>25.38063</v>
+      </c>
+      <c r="O192">
+        <v>71.35804655870446</v>
+      </c>
+      <c r="P192">
+        <v>35.568</v>
+      </c>
+      <c r="Q192">
+        <v>551.8525500000001</v>
+      </c>
+      <c r="R192">
+        <v>5.147078035131354</v>
+      </c>
+      <c r="S192">
+        <v>1246.49002</v>
+      </c>
+      <c r="T192">
+        <v>52</v>
+      </c>
+      <c r="U192">
+        <v>44</v>
+      </c>
+      <c r="V192">
+        <v>96</v>
+      </c>
+      <c r="W192">
+        <v>114</v>
+      </c>
+      <c r="X192">
+        <v>52</v>
+      </c>
+      <c r="Y192">
+        <v>100</v>
+      </c>
+      <c r="Z192">
+        <v>44</v>
+      </c>
+      <c r="AA192">
+        <v>10</v>
+      </c>
+      <c r="AB192">
+        <v>4.44502</v>
+      </c>
+      <c r="AC192">
+        <v>-3.52053</v>
+      </c>
+      <c r="AD192">
+        <v>0</v>
+      </c>
+      <c r="AE192">
+        <v>563.0312</v>
+      </c>
+      <c r="AF192">
+        <v>0</v>
+      </c>
+      <c r="AG192">
+        <v>3</v>
+      </c>
+      <c r="AH192">
+        <v>1655.55765</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B193" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E193">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F193">
+        <v>4908.21</v>
+      </c>
+      <c r="G193">
+        <v>45.77842375252604</v>
+      </c>
+      <c r="H193">
+        <v>70.10999999999999</v>
+      </c>
+      <c r="I193">
+        <v>0</v>
+      </c>
+      <c r="J193">
+        <v>0</v>
+      </c>
+      <c r="K193">
+        <v>0.6539095289911393</v>
+      </c>
+      <c r="L193">
+        <v>0</v>
+      </c>
+      <c r="M193">
+        <v>0</v>
+      </c>
+      <c r="N193">
+        <v>24.03125</v>
+      </c>
+      <c r="O193">
+        <v>66.75347222222221</v>
+      </c>
+      <c r="P193">
+        <v>36</v>
+      </c>
+      <c r="Q193">
+        <v>550.08794</v>
+      </c>
+      <c r="R193">
+        <v>5.130619679776154</v>
+      </c>
+      <c r="S193">
+        <v>1076.36</v>
+      </c>
+      <c r="T193">
+        <v>35</v>
+      </c>
+      <c r="U193">
+        <v>49</v>
+      </c>
+      <c r="V193">
+        <v>84</v>
+      </c>
+      <c r="W193">
+        <v>109</v>
+      </c>
+      <c r="X193">
+        <v>35</v>
+      </c>
+      <c r="Y193">
+        <v>110</v>
+      </c>
+      <c r="Z193">
+        <v>49</v>
+      </c>
+      <c r="AA193">
+        <v>28</v>
+      </c>
+      <c r="AB193">
+        <v>4.20634</v>
+      </c>
+      <c r="AC193">
+        <v>-2.69485</v>
+      </c>
+      <c r="AD193">
+        <v>0</v>
+      </c>
+      <c r="AE193">
+        <v>426.9895</v>
+      </c>
+      <c r="AF193">
+        <v>0</v>
+      </c>
+      <c r="AG193">
+        <v>3</v>
+      </c>
+      <c r="AH193">
+        <v>1650.26382</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B194" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E194">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F194">
+        <v>4594.64</v>
+      </c>
+      <c r="G194">
+        <v>42.85378517021608</v>
+      </c>
+      <c r="H194">
+        <v>52.35</v>
+      </c>
+      <c r="I194">
+        <v>0</v>
+      </c>
+      <c r="J194">
+        <v>0</v>
+      </c>
+      <c r="K194">
+        <v>0.48826364060314</v>
+      </c>
+      <c r="L194">
+        <v>0</v>
+      </c>
+      <c r="M194">
+        <v>0</v>
+      </c>
+      <c r="N194">
+        <v>23.2906</v>
+      </c>
+      <c r="O194">
+        <v>72.7740282464692</v>
+      </c>
+      <c r="P194">
+        <v>32.004</v>
+      </c>
+      <c r="Q194">
+        <v>529.2741599999999</v>
+      </c>
+      <c r="R194">
+        <v>4.936491465879061</v>
+      </c>
+      <c r="S194">
+        <v>852.39001</v>
+      </c>
+      <c r="T194">
+        <v>26</v>
+      </c>
+      <c r="U194">
+        <v>43</v>
+      </c>
+      <c r="V194">
+        <v>69</v>
+      </c>
+      <c r="W194">
+        <v>77</v>
+      </c>
+      <c r="X194">
+        <v>26</v>
+      </c>
+      <c r="Y194">
+        <v>94</v>
+      </c>
+      <c r="Z194">
+        <v>43</v>
+      </c>
+      <c r="AA194">
+        <v>15</v>
+      </c>
+      <c r="AB194">
+        <v>4.18355</v>
+      </c>
+      <c r="AC194">
+        <v>-2.8917</v>
+      </c>
+      <c r="AD194">
+        <v>0</v>
+      </c>
+      <c r="AE194">
+        <v>333.8274</v>
+      </c>
+      <c r="AF194">
+        <v>0</v>
+      </c>
+      <c r="AG194">
+        <v>3</v>
+      </c>
+      <c r="AH194">
+        <v>1587.82248</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B195" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E195">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F195">
+        <v>5620.669999999999</v>
+      </c>
+      <c r="G195">
+        <v>52.42347271879371</v>
+      </c>
+      <c r="H195">
+        <v>333.89</v>
+      </c>
+      <c r="I195">
+        <v>0</v>
+      </c>
+      <c r="J195">
+        <v>0</v>
+      </c>
+      <c r="K195">
+        <v>3.114161355510649</v>
+      </c>
+      <c r="L195">
+        <v>0</v>
+      </c>
+      <c r="M195">
+        <v>0</v>
+      </c>
+      <c r="N195">
+        <v>26.27477</v>
+      </c>
+      <c r="O195">
+        <v>77.64411938534278</v>
+      </c>
+      <c r="P195">
+        <v>33.84</v>
+      </c>
+      <c r="Q195">
+        <v>584.37918</v>
+      </c>
+      <c r="R195">
+        <v>5.45045092491839</v>
+      </c>
+      <c r="S195">
+        <v>1262.66999</v>
+      </c>
+      <c r="T195">
+        <v>42</v>
+      </c>
+      <c r="U195">
+        <v>54</v>
+      </c>
+      <c r="V195">
+        <v>96</v>
+      </c>
+      <c r="W195">
+        <v>113</v>
+      </c>
+      <c r="X195">
+        <v>42</v>
+      </c>
+      <c r="Y195">
+        <v>96</v>
+      </c>
+      <c r="Z195">
+        <v>54</v>
+      </c>
+      <c r="AA195">
+        <v>25</v>
+      </c>
+      <c r="AB195">
+        <v>4.22005</v>
+      </c>
+      <c r="AC195">
+        <v>-3.58805</v>
+      </c>
+      <c r="AD195">
+        <v>0</v>
+      </c>
+      <c r="AE195">
+        <v>488.9521</v>
+      </c>
+      <c r="AF195">
+        <v>0</v>
+      </c>
+      <c r="AG195">
+        <v>3</v>
+      </c>
+      <c r="AH195">
+        <v>1753.13754</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B196" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E196">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F196">
+        <v>4946.24</v>
+      </c>
+      <c r="G196">
+        <v>46.13312606870822</v>
+      </c>
+      <c r="H196">
+        <v>75.11</v>
+      </c>
+      <c r="I196">
+        <v>0</v>
+      </c>
+      <c r="J196">
+        <v>0</v>
+      </c>
+      <c r="K196">
+        <v>0.700544069640914</v>
+      </c>
+      <c r="L196">
+        <v>0</v>
+      </c>
+      <c r="M196">
+        <v>0</v>
+      </c>
+      <c r="N196">
+        <v>23.6058</v>
+      </c>
+      <c r="O196">
+        <v>70.05519943019944</v>
+      </c>
+      <c r="P196">
+        <v>33.696</v>
+      </c>
+      <c r="Q196">
+        <v>576.6306499999999</v>
+      </c>
+      <c r="R196">
+        <v>5.378181097466189</v>
+      </c>
+      <c r="S196">
+        <v>1002.41</v>
+      </c>
+      <c r="T196">
+        <v>38</v>
+      </c>
+      <c r="U196">
+        <v>38</v>
+      </c>
+      <c r="V196">
+        <v>76</v>
+      </c>
+      <c r="W196">
+        <v>105</v>
+      </c>
+      <c r="X196">
+        <v>38</v>
+      </c>
+      <c r="Y196">
+        <v>96</v>
+      </c>
+      <c r="Z196">
+        <v>38</v>
+      </c>
+      <c r="AA196">
+        <v>63</v>
+      </c>
+      <c r="AB196">
+        <v>4.19611</v>
+      </c>
+      <c r="AC196">
+        <v>-3.5654</v>
+      </c>
+      <c r="AD196">
+        <v>0</v>
+      </c>
+      <c r="AE196">
+        <v>485.1904</v>
+      </c>
+      <c r="AF196">
+        <v>0</v>
+      </c>
+      <c r="AG196">
+        <v>3</v>
+      </c>
+      <c r="AH196">
+        <v>1729.89195</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B197" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E197">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F197">
+        <v>5316.98</v>
+      </c>
+      <c r="G197">
+        <v>49.59098398880771</v>
+      </c>
+      <c r="H197">
+        <v>75.72000000000001</v>
+      </c>
+      <c r="I197">
+        <v>0</v>
+      </c>
+      <c r="J197">
+        <v>0</v>
+      </c>
+      <c r="K197">
+        <v>0.7062334836001867</v>
+      </c>
+      <c r="L197">
+        <v>0</v>
+      </c>
+      <c r="M197">
+        <v>0</v>
+      </c>
+      <c r="N197">
+        <v>23.60841</v>
+      </c>
+      <c r="O197">
+        <v>67.46802126200274</v>
+      </c>
+      <c r="P197">
+        <v>34.992</v>
+      </c>
+      <c r="Q197">
+        <v>540.59011</v>
+      </c>
+      <c r="R197">
+        <v>5.042034291932224</v>
+      </c>
+      <c r="S197">
+        <v>957.1699600000001</v>
+      </c>
+      <c r="T197">
+        <v>43</v>
+      </c>
+      <c r="U197">
+        <v>34</v>
+      </c>
+      <c r="V197">
+        <v>77</v>
+      </c>
+      <c r="W197">
+        <v>97</v>
+      </c>
+      <c r="X197">
+        <v>43</v>
+      </c>
+      <c r="Y197">
+        <v>93</v>
+      </c>
+      <c r="Z197">
+        <v>34</v>
+      </c>
+      <c r="AA197">
+        <v>25</v>
+      </c>
+      <c r="AB197">
+        <v>3.94086</v>
+      </c>
+      <c r="AC197">
+        <v>-3.06322</v>
+      </c>
+      <c r="AD197">
+        <v>0</v>
+      </c>
+      <c r="AE197">
+        <v>438.60471</v>
+      </c>
+      <c r="AF197">
+        <v>0</v>
+      </c>
+      <c r="AG197">
+        <v>3</v>
+      </c>
+      <c r="AH197">
+        <v>1621.77033</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B198" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E198">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F198">
+        <v>5539.53</v>
+      </c>
+      <c r="G198">
+        <v>51.66668739312917</v>
+      </c>
+      <c r="H198">
+        <v>76.3</v>
+      </c>
+      <c r="I198">
+        <v>0</v>
+      </c>
+      <c r="J198">
+        <v>0</v>
+      </c>
+      <c r="K198">
+        <v>0.7116430903155604</v>
+      </c>
+      <c r="L198">
+        <v>0</v>
+      </c>
+      <c r="M198">
+        <v>0</v>
+      </c>
+      <c r="N198">
+        <v>23.61024</v>
+      </c>
+      <c r="O198">
+        <v>67.61237113402062</v>
+      </c>
+      <c r="P198">
+        <v>34.92</v>
+      </c>
+      <c r="Q198">
+        <v>611.42886</v>
+      </c>
+      <c r="R198">
+        <v>5.702740805223068</v>
+      </c>
+      <c r="S198">
+        <v>1141.11002</v>
+      </c>
+      <c r="T198">
+        <v>49</v>
+      </c>
+      <c r="U198">
+        <v>31</v>
+      </c>
+      <c r="V198">
+        <v>80</v>
+      </c>
+      <c r="W198">
+        <v>110</v>
+      </c>
+      <c r="X198">
+        <v>49</v>
+      </c>
+      <c r="Y198">
+        <v>103</v>
+      </c>
+      <c r="Z198">
+        <v>31</v>
+      </c>
+      <c r="AA198">
+        <v>10</v>
+      </c>
+      <c r="AB198">
+        <v>3.79987</v>
+      </c>
+      <c r="AC198">
+        <v>-3.07619</v>
+      </c>
+      <c r="AD198">
+        <v>0</v>
+      </c>
+      <c r="AE198">
+        <v>538.6208</v>
+      </c>
+      <c r="AF198">
+        <v>0</v>
+      </c>
+      <c r="AG198">
+        <v>3</v>
+      </c>
+      <c r="AH198">
+        <v>1834.28658</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B199" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E199">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F199">
+        <v>5258.72</v>
+      </c>
+      <c r="G199">
+        <v>49.04759832115653</v>
+      </c>
+      <c r="H199">
+        <v>142.3</v>
+      </c>
+      <c r="I199">
+        <v>0</v>
+      </c>
+      <c r="J199">
+        <v>0</v>
+      </c>
+      <c r="K199">
+        <v>1.327219026892585</v>
+      </c>
+      <c r="L199">
+        <v>0</v>
+      </c>
+      <c r="M199">
+        <v>0</v>
+      </c>
+      <c r="N199">
+        <v>23.5701</v>
+      </c>
+      <c r="O199">
+        <v>67.35853909465021</v>
+      </c>
+      <c r="P199">
+        <v>34.992</v>
+      </c>
+      <c r="Q199">
+        <v>495.11263</v>
+      </c>
+      <c r="R199">
+        <v>4.617870013990362</v>
+      </c>
+      <c r="S199">
+        <v>1194.50999</v>
+      </c>
+      <c r="T199">
+        <v>36</v>
+      </c>
+      <c r="U199">
+        <v>56</v>
+      </c>
+      <c r="V199">
+        <v>92</v>
+      </c>
+      <c r="W199">
+        <v>101</v>
+      </c>
+      <c r="X199">
+        <v>36</v>
+      </c>
+      <c r="Y199">
+        <v>111</v>
+      </c>
+      <c r="Z199">
+        <v>56</v>
+      </c>
+      <c r="AA199">
+        <v>19</v>
+      </c>
+      <c r="AB199">
+        <v>4.11382</v>
+      </c>
+      <c r="AC199">
+        <v>-2.8103</v>
+      </c>
+      <c r="AD199">
+        <v>0</v>
+      </c>
+      <c r="AE199">
+        <v>464.78943</v>
+      </c>
+      <c r="AF199">
+        <v>0</v>
+      </c>
+      <c r="AG199">
+        <v>3</v>
+      </c>
+      <c r="AH199">
+        <v>1485.33789</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B200" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E200">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F200">
+        <v>4522.42</v>
+      </c>
+      <c r="G200">
+        <v>42.18019586507073</v>
+      </c>
+      <c r="H200">
+        <v>42.38</v>
+      </c>
+      <c r="I200">
+        <v>0</v>
+      </c>
+      <c r="J200">
+        <v>0</v>
+      </c>
+      <c r="K200">
+        <v>0.3952743665474895</v>
+      </c>
+      <c r="L200">
+        <v>0</v>
+      </c>
+      <c r="M200">
+        <v>0</v>
+      </c>
+      <c r="N200">
+        <v>22.91071</v>
+      </c>
+      <c r="O200">
+        <v>67.41616643126177</v>
+      </c>
+      <c r="P200">
+        <v>33.984</v>
+      </c>
+      <c r="Q200">
+        <v>576.23023</v>
+      </c>
+      <c r="R200">
+        <v>5.374446416912793</v>
+      </c>
+      <c r="S200">
+        <v>922.84999</v>
+      </c>
+      <c r="T200">
+        <v>29</v>
+      </c>
+      <c r="U200">
+        <v>47</v>
+      </c>
+      <c r="V200">
+        <v>76</v>
+      </c>
+      <c r="W200">
+        <v>99</v>
+      </c>
+      <c r="X200">
+        <v>29</v>
+      </c>
+      <c r="Y200">
+        <v>103</v>
+      </c>
+      <c r="Z200">
+        <v>47</v>
+      </c>
+      <c r="AA200">
+        <v>63</v>
+      </c>
+      <c r="AB200">
+        <v>4.06863</v>
+      </c>
+      <c r="AC200">
+        <v>-3.19859</v>
+      </c>
+      <c r="AD200">
+        <v>0</v>
+      </c>
+      <c r="AE200">
+        <v>446.6696</v>
+      </c>
+      <c r="AF200">
+        <v>0</v>
+      </c>
+      <c r="AG200">
+        <v>3</v>
+      </c>
+      <c r="AH200">
+        <v>1728.69069</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B201" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E201">
+        <v>53.16666666666666</v>
+      </c>
+      <c r="F201">
+        <v>1627.37</v>
+      </c>
+      <c r="G201">
+        <v>30.60884012539185</v>
+      </c>
+      <c r="H201">
+        <v>0</v>
+      </c>
+      <c r="I201">
+        <v>0</v>
+      </c>
+      <c r="J201">
+        <v>0</v>
+      </c>
+      <c r="K201">
+        <v>0</v>
+      </c>
+      <c r="L201">
+        <v>0</v>
+      </c>
+      <c r="M201">
+        <v>0</v>
+      </c>
+      <c r="N201">
+        <v>20.46638</v>
+      </c>
+      <c r="O201">
+        <v>58.48874028349338</v>
+      </c>
+      <c r="P201">
+        <v>34.992</v>
+      </c>
+      <c r="Q201">
+        <v>199.70353</v>
+      </c>
+      <c r="R201">
+        <v>3.756179247648903</v>
+      </c>
+      <c r="S201">
+        <v>237.38</v>
+      </c>
+      <c r="T201">
+        <v>15</v>
+      </c>
+      <c r="U201">
+        <v>15</v>
+      </c>
+      <c r="V201">
+        <v>30</v>
+      </c>
+      <c r="W201">
+        <v>34</v>
+      </c>
+      <c r="X201">
+        <v>15</v>
+      </c>
+      <c r="Y201">
+        <v>26</v>
+      </c>
+      <c r="Z201">
+        <v>15</v>
+      </c>
+      <c r="AA201">
+        <v>8</v>
+      </c>
+      <c r="AB201">
+        <v>3.84602</v>
+      </c>
+      <c r="AC201">
+        <v>-3.40874</v>
+      </c>
+      <c r="AD201">
+        <v>0</v>
+      </c>
+      <c r="AE201">
+        <v>155.3864</v>
+      </c>
+      <c r="AF201">
+        <v>0</v>
+      </c>
+      <c r="AG201">
+        <v>3</v>
+      </c>
+      <c r="AH201">
+        <v>599.11059</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B202" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E202">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F202">
+        <v>4722.580000000001</v>
+      </c>
+      <c r="G202">
+        <v>44.04706979636251</v>
+      </c>
+      <c r="H202">
+        <v>34.44</v>
+      </c>
+      <c r="I202">
+        <v>0</v>
+      </c>
+      <c r="J202">
+        <v>0</v>
+      </c>
+      <c r="K202">
+        <v>0.3212187159956474</v>
+      </c>
+      <c r="L202">
+        <v>0</v>
+      </c>
+      <c r="M202">
+        <v>0</v>
+      </c>
+      <c r="N202">
+        <v>22.47953</v>
+      </c>
+      <c r="O202">
+        <v>68.09502605113292</v>
+      </c>
+      <c r="P202">
+        <v>33.012</v>
+      </c>
+      <c r="Q202">
+        <v>566.0236600000001</v>
+      </c>
+      <c r="R202">
+        <v>5.27925067620084</v>
+      </c>
+      <c r="S202">
+        <v>1034.10001</v>
+      </c>
+      <c r="T202">
+        <v>29</v>
+      </c>
+      <c r="U202">
+        <v>38</v>
+      </c>
+      <c r="V202">
+        <v>67</v>
+      </c>
+      <c r="W202">
+        <v>101</v>
+      </c>
+      <c r="X202">
+        <v>29</v>
+      </c>
+      <c r="Y202">
+        <v>98</v>
+      </c>
+      <c r="Z202">
+        <v>38</v>
+      </c>
+      <c r="AA202">
+        <v>33</v>
+      </c>
+      <c r="AB202">
+        <v>3.74724</v>
+      </c>
+      <c r="AC202">
+        <v>-2.7822</v>
+      </c>
+      <c r="AD202">
+        <v>0</v>
+      </c>
+      <c r="AE202">
+        <v>427.2645000000001</v>
+      </c>
+      <c r="AF202">
+        <v>0</v>
+      </c>
+      <c r="AG202">
+        <v>3</v>
+      </c>
+      <c r="AH202">
+        <v>1698.07098</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B203" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E203">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F203">
+        <v>3992.16</v>
+      </c>
+      <c r="G203">
+        <v>37.23450956008084</v>
+      </c>
+      <c r="H203">
+        <v>12.56</v>
+      </c>
+      <c r="I203">
+        <v>0</v>
+      </c>
+      <c r="J203">
+        <v>0</v>
+      </c>
+      <c r="K203">
+        <v>0.1171459661122338</v>
+      </c>
+      <c r="L203">
+        <v>0</v>
+      </c>
+      <c r="M203">
+        <v>0</v>
+      </c>
+      <c r="N203">
+        <v>22.64702</v>
+      </c>
+      <c r="O203">
+        <v>70.76309211348583</v>
+      </c>
+      <c r="P203">
+        <v>32.004</v>
+      </c>
+      <c r="Q203">
+        <v>430.24447</v>
+      </c>
+      <c r="R203">
+        <v>4.012850645111145</v>
+      </c>
+      <c r="S203">
+        <v>634.30999</v>
+      </c>
+      <c r="T203">
+        <v>20</v>
+      </c>
+      <c r="U203">
+        <v>15</v>
+      </c>
+      <c r="V203">
+        <v>35</v>
+      </c>
+      <c r="W203">
+        <v>81</v>
+      </c>
+      <c r="X203">
+        <v>20</v>
+      </c>
+      <c r="Y203">
+        <v>71</v>
+      </c>
+      <c r="Z203">
+        <v>15</v>
+      </c>
+      <c r="AA203">
+        <v>43</v>
+      </c>
+      <c r="AB203">
+        <v>3.87551</v>
+      </c>
+      <c r="AC203">
+        <v>-2.89696</v>
+      </c>
+      <c r="AD203">
+        <v>0</v>
+      </c>
+      <c r="AE203">
+        <v>328.8747</v>
+      </c>
+      <c r="AF203">
+        <v>0</v>
+      </c>
+      <c r="AG203">
+        <v>3</v>
+      </c>
+      <c r="AH203">
+        <v>1290.73341</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B204" s="2">
+        <v>46195</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Sesion 12</t>
+        </is>
+      </c>
+      <c r="E204">
+        <v>107.2166666666667</v>
+      </c>
+      <c r="F204">
+        <v>5479.57</v>
+      </c>
+      <c r="G204">
+        <v>51.10744598165708</v>
+      </c>
+      <c r="H204">
+        <v>71.47</v>
+      </c>
+      <c r="I204">
+        <v>0</v>
+      </c>
+      <c r="J204">
+        <v>0</v>
+      </c>
+      <c r="K204">
+        <v>0.6665941240478781</v>
+      </c>
+      <c r="L204">
+        <v>0</v>
+      </c>
+      <c r="M204">
+        <v>0</v>
+      </c>
+      <c r="N204">
+        <v>22.69942</v>
+      </c>
+      <c r="O204">
+        <v>63.05394444444444</v>
+      </c>
+      <c r="P204">
+        <v>36</v>
+      </c>
+      <c r="Q204">
+        <v>603.79105</v>
+      </c>
+      <c r="R204">
+        <v>5.631503653039018</v>
+      </c>
+      <c r="S204">
+        <v>982.3600100000001</v>
+      </c>
+      <c r="T204">
+        <v>38</v>
+      </c>
+      <c r="U204">
+        <v>40</v>
+      </c>
+      <c r="V204">
+        <v>78</v>
+      </c>
+      <c r="W204">
+        <v>96</v>
+      </c>
+      <c r="X204">
+        <v>38</v>
+      </c>
+      <c r="Y204">
+        <v>104</v>
+      </c>
+      <c r="Z204">
+        <v>40</v>
+      </c>
+      <c r="AA204">
+        <v>41</v>
+      </c>
+      <c r="AB204">
+        <v>4.3104</v>
+      </c>
+      <c r="AC204">
+        <v>-3.65595</v>
+      </c>
+      <c r="AD204">
+        <v>0</v>
+      </c>
+      <c r="AE204">
+        <v>458.3915</v>
+      </c>
+      <c r="AF204">
+        <v>0</v>
+      </c>
+      <c r="AG204">
+        <v>3</v>
+      </c>
+      <c r="AH204">
+        <v>1811.37315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-23
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -1347,10 +1347,10 @@
         <v>142.3</v>
       </c>
       <c r="F9">
-        <v>8256.340000000002</v>
+        <v>8256.34</v>
       </c>
       <c r="G9">
-        <v>58.02066057624737</v>
+        <v>58.02066057624736</v>
       </c>
       <c r="H9">
         <v>499.06</v>
@@ -1383,10 +1383,10 @@
         <v>33.84</v>
       </c>
       <c r="R9">
-        <v>871.5351299999999</v>
+        <v>871.53513</v>
       </c>
       <c r="S9">
-        <v>6.124631974701334</v>
+        <v>6.124631974701335</v>
       </c>
       <c r="T9">
         <v>1096.84001</v>
@@ -2816,10 +2816,10 @@
         <v>114.4713333333333</v>
       </c>
       <c r="F22">
-        <v>8536.459999999997</v>
+        <v>8536.459999999999</v>
       </c>
       <c r="G22">
-        <v>74.57290617155967</v>
+        <v>74.57290617155968</v>
       </c>
       <c r="H22">
         <v>176.52</v>
@@ -3048,7 +3048,7 @@
         <v>62.29918508342559</v>
       </c>
       <c r="H24">
-        <v>84.63999999999999</v>
+        <v>84.64</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -3057,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>0.6773277138322418</v>
+        <v>0.6773277138322419</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -3078,10 +3078,10 @@
         <v>33.984</v>
       </c>
       <c r="R24">
-        <v>965.6688100000001</v>
+        <v>965.66881</v>
       </c>
       <c r="S24">
-        <v>7.727720314229699</v>
+        <v>7.727720314229698</v>
       </c>
       <c r="T24">
         <v>1013.94</v>
@@ -3268,10 +3268,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F26">
-        <v>9359.540000000001</v>
+        <v>9359.539999999999</v>
       </c>
       <c r="G26">
-        <v>74.89928911532871</v>
+        <v>74.8992891153287</v>
       </c>
       <c r="H26">
         <v>180.97</v>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="AF26">
-        <v>801.2445000000001</v>
+        <v>801.2445</v>
       </c>
       <c r="AG26">
         <v>0</v>
@@ -3396,7 +3396,7 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>1.858649985995706</v>
+        <v>1.858649985995705</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -3530,10 +3530,10 @@
         <v>33.84</v>
       </c>
       <c r="R28">
-        <v>945.4113000000001</v>
+        <v>945.4113</v>
       </c>
       <c r="S28">
-        <v>7.565610520559639</v>
+        <v>7.565610520559638</v>
       </c>
       <c r="T28">
         <v>1575.19001</v>
@@ -3839,7 +3839,7 @@
         <v>74.94482307907758</v>
       </c>
       <c r="H31">
-        <v>337.4999999999999</v>
+        <v>337.5</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -4214,7 +4214,7 @@
         <v>6.844402790188991</v>
       </c>
       <c r="T34">
-        <v>898.6499899999999</v>
+        <v>898.64999</v>
       </c>
       <c r="U34">
         <v>21</v>
@@ -4285,10 +4285,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F35">
-        <v>8757.950000000001</v>
+        <v>8757.949999999999</v>
       </c>
       <c r="G35">
-        <v>70.08509276178029</v>
+        <v>70.08509276178027</v>
       </c>
       <c r="H35">
         <v>203.09</v>
@@ -4476,7 +4476,7 @@
         <v>0</v>
       </c>
       <c r="AF36">
-        <v>762.7650000000001</v>
+        <v>762.765</v>
       </c>
       <c r="AG36">
         <v>0</v>
@@ -4511,10 +4511,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F37">
-        <v>8234.929999999998</v>
+        <v>8234.93</v>
       </c>
       <c r="G37">
-        <v>65.89964922576256</v>
+        <v>65.89964922576257</v>
       </c>
       <c r="H37">
         <v>42.54</v>
@@ -4547,10 +4547,10 @@
         <v>32.004</v>
       </c>
       <c r="R37">
-        <v>847.99138</v>
+        <v>847.9913799999999</v>
       </c>
       <c r="S37">
-        <v>6.78601208370567</v>
+        <v>6.786012083705669</v>
       </c>
       <c r="T37">
         <v>1039.69</v>
@@ -4589,7 +4589,7 @@
         <v>0</v>
       </c>
       <c r="AF37">
-        <v>690.5905999999999</v>
+        <v>690.5906</v>
       </c>
       <c r="AG37">
         <v>0</v>
@@ -4776,7 +4776,7 @@
         <v>3.75311</v>
       </c>
       <c r="S39">
-        <v>0.08257667766776676</v>
+        <v>0.08257667766776677</v>
       </c>
       <c r="T39">
         <v>0</v>
@@ -4850,10 +4850,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F40">
-        <v>8274.099999999999</v>
+        <v>8274.1</v>
       </c>
       <c r="G40">
-        <v>66.21310535230803</v>
+        <v>66.21310535230805</v>
       </c>
       <c r="H40">
         <v>297.8200000000001</v>
@@ -4978,7 +4978,7 @@
         <v>0</v>
       </c>
       <c r="K41">
-        <v>0.3757152193339291</v>
+        <v>0.375715219333929</v>
       </c>
       <c r="L41">
         <v>0</v>
@@ -5076,7 +5076,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F42">
-        <v>7142.569999999999</v>
+        <v>7142.57</v>
       </c>
       <c r="G42">
         <v>93.52463631483153</v>
@@ -5091,7 +5091,7 @@
         <v>0</v>
       </c>
       <c r="K42">
-        <v>2.101059302614867</v>
+        <v>2.101059302614866</v>
       </c>
       <c r="L42">
         <v>0</v>
@@ -5225,13 +5225,13 @@
         <v>32.4</v>
       </c>
       <c r="R43">
-        <v>806.5637</v>
+        <v>806.5636999999999</v>
       </c>
       <c r="S43">
         <v>10.56112529625119</v>
       </c>
       <c r="T43">
-        <v>911.0899999999999</v>
+        <v>911.09</v>
       </c>
       <c r="U43">
         <v>9</v>
@@ -5415,7 +5415,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F45">
-        <v>7078.56</v>
+        <v>7078.559999999999</v>
       </c>
       <c r="G45">
         <v>92.68649094551596</v>
@@ -5457,7 +5457,7 @@
         <v>8.81651228869597</v>
       </c>
       <c r="T45">
-        <v>830.0500099999999</v>
+        <v>830.05001</v>
       </c>
       <c r="U45">
         <v>28</v>
@@ -5493,7 +5493,7 @@
         <v>0</v>
       </c>
       <c r="AF45">
-        <v>664.0912000000001</v>
+        <v>664.0912</v>
       </c>
       <c r="AG45">
         <v>0</v>
@@ -5754,10 +5754,10 @@
         <v>76.37083333333334</v>
       </c>
       <c r="F48">
-        <v>6636.860000000001</v>
+        <v>6636.86</v>
       </c>
       <c r="G48">
-        <v>86.90307163511376</v>
+        <v>86.90307163511375</v>
       </c>
       <c r="H48">
         <v>201.92</v>
@@ -5796,7 +5796,7 @@
         <v>10.01454228817721</v>
       </c>
       <c r="T48">
-        <v>940.6600000000001</v>
+        <v>940.66</v>
       </c>
       <c r="U48">
         <v>11</v>
@@ -5832,7 +5832,7 @@
         <v>0</v>
       </c>
       <c r="AF48">
-        <v>553.3290000000001</v>
+        <v>553.329</v>
       </c>
       <c r="AG48">
         <v>0</v>
@@ -6016,10 +6016,10 @@
         <v>34.92</v>
       </c>
       <c r="R50">
-        <v>675.5848699999999</v>
+        <v>675.58487</v>
       </c>
       <c r="S50">
-        <v>8.846091710204133</v>
+        <v>8.846091710204135</v>
       </c>
       <c r="T50">
         <v>952.77999</v>
@@ -6171,7 +6171,7 @@
         <v>0</v>
       </c>
       <c r="AF51">
-        <v>630.7519299999999</v>
+        <v>630.75193</v>
       </c>
       <c r="AG51">
         <v>0</v>
@@ -6206,10 +6206,10 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F52">
-        <v>6693.129999999999</v>
+        <v>6693.13</v>
       </c>
       <c r="G52">
-        <v>87.63967998323969</v>
+        <v>87.6396799832397</v>
       </c>
       <c r="H52">
         <v>16.96</v>
@@ -6468,13 +6468,13 @@
         <v>33.012</v>
       </c>
       <c r="R54">
-        <v>685.1758299999999</v>
+        <v>685.17583</v>
       </c>
       <c r="S54">
-        <v>8.971675505100102</v>
+        <v>8.971675505100103</v>
       </c>
       <c r="T54">
-        <v>843.77997</v>
+        <v>843.7799699999999</v>
       </c>
       <c r="U54">
         <v>17</v>
@@ -6519,7 +6519,7 @@
         <v>3</v>
       </c>
       <c r="AI54">
-        <v>2055.527489999999</v>
+        <v>2055.52749</v>
       </c>
     </row>
     <row r="55">
@@ -6658,7 +6658,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F56">
-        <v>6802.68</v>
+        <v>6802.679999999999</v>
       </c>
       <c r="G56">
         <v>89.07412499508975</v>
@@ -6700,7 +6700,7 @@
         <v>8.080355370494035</v>
       </c>
       <c r="T56">
-        <v>862.5100000000001</v>
+        <v>862.51</v>
       </c>
       <c r="U56">
         <v>10</v>
@@ -6807,13 +6807,13 @@
         <v>36</v>
       </c>
       <c r="R57">
-        <v>618.2029799999999</v>
+        <v>618.20298</v>
       </c>
       <c r="S57">
-        <v>8.094734650587263</v>
+        <v>8.094734650587265</v>
       </c>
       <c r="T57">
-        <v>742.09999</v>
+        <v>742.0999899999999</v>
       </c>
       <c r="U57">
         <v>12</v>
@@ -6849,7 +6849,7 @@
         <v>0</v>
       </c>
       <c r="AF57">
-        <v>509.4404000000001</v>
+        <v>509.4404</v>
       </c>
       <c r="AG57">
         <v>0</v>
@@ -7034,7 +7034,7 @@
         <v>6.301423002309469</v>
       </c>
       <c r="T59">
-        <v>900.0399500000001</v>
+        <v>900.03995</v>
       </c>
       <c r="U59">
         <v>20</v>
@@ -7568,10 +7568,10 @@
         <v>32.004</v>
       </c>
       <c r="R64">
-        <v>671.0377699999999</v>
+        <v>671.03777</v>
       </c>
       <c r="S64">
-        <v>6.19896323325635</v>
+        <v>6.198963233256351</v>
       </c>
       <c r="T64">
         <v>862.40997</v>
@@ -7826,7 +7826,7 @@
         <v>0</v>
       </c>
       <c r="AF66">
-        <v>584.6215999999999</v>
+        <v>584.6216000000001</v>
       </c>
       <c r="AG66">
         <v>0</v>
@@ -7856,10 +7856,10 @@
         <v>108.25</v>
       </c>
       <c r="F67">
-        <v>5820.460000000001</v>
+        <v>5820.46</v>
       </c>
       <c r="G67">
-        <v>53.76868360277137</v>
+        <v>53.76868360277136</v>
       </c>
       <c r="H67">
         <v>25.29</v>
@@ -8288,10 +8288,10 @@
         <v>108.25</v>
       </c>
       <c r="F71">
-        <v>6131.409999999999</v>
+        <v>6131.41</v>
       </c>
       <c r="G71">
-        <v>56.64120092378752</v>
+        <v>56.64120092378753</v>
       </c>
       <c r="H71">
         <v>57.77</v>
@@ -8324,10 +8324,10 @@
         <v>34.992</v>
       </c>
       <c r="R71">
-        <v>678.6408300000001</v>
+        <v>678.6408299999999</v>
       </c>
       <c r="S71">
-        <v>6.26919935334873</v>
+        <v>6.269199353348729</v>
       </c>
       <c r="T71">
         <v>981.28002</v>
@@ -8474,7 +8474,7 @@
         <v>0</v>
       </c>
       <c r="AF72">
-        <v>507.1950000000001</v>
+        <v>507.195</v>
       </c>
       <c r="AG72">
         <v>0</v>
@@ -8546,7 +8546,7 @@
         <v>5.857015889145496</v>
       </c>
       <c r="T73">
-        <v>790.5800099999999</v>
+        <v>790.58001</v>
       </c>
       <c r="U73">
         <v>33</v>
@@ -8720,10 +8720,10 @@
         <v>108.25</v>
       </c>
       <c r="F75">
-        <v>5283.150000000001</v>
+        <v>5283.15</v>
       </c>
       <c r="G75">
-        <v>48.80508083140878</v>
+        <v>48.80508083140877</v>
       </c>
       <c r="H75">
         <v>30.94</v>
@@ -8762,7 +8762,7 @@
         <v>5.961701524249423</v>
       </c>
       <c r="T75">
-        <v>806.9200000000001</v>
+        <v>806.92</v>
       </c>
       <c r="U75">
         <v>42</v>
@@ -8870,7 +8870,7 @@
         <v>5.930582817551963</v>
       </c>
       <c r="T76">
-        <v>598.8199999999999</v>
+        <v>598.8200000000001</v>
       </c>
       <c r="U76">
         <v>28</v>
@@ -8906,7 +8906,7 @@
         <v>0</v>
       </c>
       <c r="AF76">
-        <v>484.7602499999999</v>
+        <v>484.76025</v>
       </c>
       <c r="AG76">
         <v>0</v>
@@ -8977,7 +8977,7 @@
         <v>32.364</v>
       </c>
       <c r="R77">
-        <v>758.4063100000001</v>
+        <v>758.40631</v>
       </c>
       <c r="S77">
         <v>11.09411010637131</v>
@@ -9506,10 +9506,10 @@
         <v>71.20933333333333</v>
       </c>
       <c r="F82">
-        <v>7086.919999999999</v>
+        <v>7086.92</v>
       </c>
       <c r="G82">
-        <v>99.52234725785009</v>
+        <v>99.5223472578501</v>
       </c>
       <c r="H82">
         <v>246.93</v>
@@ -9661,7 +9661,7 @@
         <v>7.952642350253712</v>
       </c>
       <c r="T83">
-        <v>931.2800099999999</v>
+        <v>931.2800100000001</v>
       </c>
       <c r="U83">
         <v>15</v>
@@ -9697,7 +9697,7 @@
         <v>0</v>
       </c>
       <c r="AF83">
-        <v>558.38181</v>
+        <v>558.3818100000001</v>
       </c>
       <c r="AG83">
         <v>0</v>
@@ -9732,10 +9732,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F84">
-        <v>6362.629999999999</v>
+        <v>6362.63</v>
       </c>
       <c r="G84">
-        <v>93.07374800995692</v>
+        <v>93.07374800995693</v>
       </c>
       <c r="H84">
         <v>345.63</v>
@@ -9958,10 +9958,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F86">
-        <v>6656.71</v>
+        <v>6656.709999999999</v>
       </c>
       <c r="G86">
-        <v>97.3756055460337</v>
+        <v>97.37560554603368</v>
       </c>
       <c r="H86">
         <v>144.12</v>
@@ -10036,7 +10036,7 @@
         <v>0</v>
       </c>
       <c r="AF86">
-        <v>621.0583999999999</v>
+        <v>621.0584</v>
       </c>
       <c r="AG86">
         <v>0</v>
@@ -10184,7 +10184,7 @@
         <v>68.7235</v>
       </c>
       <c r="F88">
-        <v>7172.649999999999</v>
+        <v>7172.65</v>
       </c>
       <c r="G88">
         <v>104.3696843146813</v>
@@ -10339,7 +10339,7 @@
         <v>8.221425422162724</v>
       </c>
       <c r="T89">
-        <v>925.6099999999999</v>
+        <v>925.61</v>
       </c>
       <c r="U89">
         <v>14</v>
@@ -10639,7 +10639,7 @@
         <v>13609.36</v>
       </c>
       <c r="G92">
-        <v>75.02431100445061</v>
+        <v>75.02431100445058</v>
       </c>
       <c r="H92">
         <v>783.59</v>
@@ -10651,7 +10651,7 @@
         <v>0</v>
       </c>
       <c r="K92">
-        <v>4.319696140007865</v>
+        <v>4.319696140007864</v>
       </c>
       <c r="L92">
         <v>0</v>
@@ -10675,7 +10675,7 @@
         <v>1367.31024</v>
       </c>
       <c r="S92">
-        <v>7.537570369608122</v>
+        <v>7.53757036960812</v>
       </c>
       <c r="T92">
         <v>2768.85995</v>
@@ -10752,7 +10752,7 @@
         <v>13532.14</v>
       </c>
       <c r="G93">
-        <v>74.59862035509136</v>
+        <v>74.59862035509134</v>
       </c>
       <c r="H93">
         <v>905.78</v>
@@ -10764,7 +10764,7 @@
         <v>0</v>
       </c>
       <c r="K93">
-        <v>4.99329288237002</v>
+        <v>4.993292882370019</v>
       </c>
       <c r="L93">
         <v>0</v>
@@ -10865,10 +10865,10 @@
         <v>12701.11</v>
       </c>
       <c r="G94">
-        <v>70.01740175450848</v>
+        <v>70.01740175450847</v>
       </c>
       <c r="H94">
-        <v>368.9400000000001</v>
+        <v>368.94</v>
       </c>
       <c r="I94">
         <v>0</v>
@@ -10901,7 +10901,7 @@
         <v>1622.4067</v>
       </c>
       <c r="S94">
-        <v>8.943840477179263</v>
+        <v>8.943840477179261</v>
       </c>
       <c r="T94">
         <v>1981.77002</v>
@@ -10978,10 +10978,10 @@
         <v>14057.61</v>
       </c>
       <c r="G95">
-        <v>77.49537852031798</v>
+        <v>77.49537852031797</v>
       </c>
       <c r="H95">
-        <v>717.6199999999999</v>
+        <v>717.62</v>
       </c>
       <c r="I95">
         <v>0</v>
@@ -11014,7 +11014,7 @@
         <v>1301.95454</v>
       </c>
       <c r="S95">
-        <v>7.177284040000148</v>
+        <v>7.177284040000147</v>
       </c>
       <c r="T95">
         <v>2534.90994</v>
@@ -11062,7 +11062,7 @@
         <v>3</v>
       </c>
       <c r="AI95">
-        <v>3905.863620000001</v>
+        <v>3905.86362</v>
       </c>
     </row>
     <row r="96">
@@ -11091,7 +11091,7 @@
         <v>13466.34</v>
       </c>
       <c r="G96">
-        <v>74.23588473313023</v>
+        <v>74.23588473313021</v>
       </c>
       <c r="H96">
         <v>1259.67</v>
@@ -11103,7 +11103,7 @@
         <v>0</v>
       </c>
       <c r="K96">
-        <v>6.944182080786773</v>
+        <v>6.944182080786772</v>
       </c>
       <c r="L96">
         <v>0</v>
@@ -11127,7 +11127,7 @@
         <v>1361.55609</v>
       </c>
       <c r="S96">
-        <v>7.505849470229586</v>
+        <v>7.505849470229585</v>
       </c>
       <c r="T96">
         <v>3031.29993</v>
@@ -11204,10 +11204,10 @@
         <v>11839.12</v>
       </c>
       <c r="G97">
-        <v>65.26550997982353</v>
+        <v>65.26550997982351</v>
       </c>
       <c r="H97">
-        <v>580.6799999999998</v>
+        <v>580.6799999999999</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -11240,7 +11240,7 @@
         <v>1362.04584</v>
       </c>
       <c r="S97">
-        <v>7.508549314771463</v>
+        <v>7.508549314771462</v>
       </c>
       <c r="T97">
         <v>2197.63005</v>
@@ -11279,7 +11279,7 @@
         <v>0</v>
       </c>
       <c r="AF97">
-        <v>846.5939999999999</v>
+        <v>846.5940000000001</v>
       </c>
       <c r="AG97">
         <v>0</v>
@@ -11430,7 +11430,7 @@
         <v>13587.06</v>
       </c>
       <c r="G99">
-        <v>74.90137780734219</v>
+        <v>74.90137780734217</v>
       </c>
       <c r="H99">
         <v>610.51</v>
@@ -11466,7 +11466,7 @@
         <v>1448.92289</v>
       </c>
       <c r="S99">
-        <v>7.987476378082978</v>
+        <v>7.987476378082977</v>
       </c>
       <c r="T99">
         <v>2588.26003</v>
@@ -11543,10 +11543,10 @@
         <v>13570.48</v>
       </c>
       <c r="G100">
-        <v>74.80997725092706</v>
+        <v>74.80997725092705</v>
       </c>
       <c r="H100">
-        <v>420.2499999999999</v>
+        <v>420.25</v>
       </c>
       <c r="I100">
         <v>0</v>
@@ -11579,7 +11579,7 @@
         <v>1254.50062</v>
       </c>
       <c r="S100">
-        <v>6.915684842649184</v>
+        <v>6.915684842649182</v>
       </c>
       <c r="T100">
         <v>2110.94003</v>
@@ -11769,7 +11769,7 @@
         <v>11738.1</v>
       </c>
       <c r="G102">
-        <v>64.70861708422302</v>
+        <v>64.70861708422301</v>
       </c>
       <c r="H102">
         <v>228.83</v>
@@ -11805,7 +11805,7 @@
         <v>1103.19668</v>
       </c>
       <c r="S102">
-        <v>6.081591700079751</v>
+        <v>6.08159170007975</v>
       </c>
       <c r="T102">
         <v>1850.74</v>
@@ -11882,7 +11882,7 @@
         <v>14309.53</v>
       </c>
       <c r="G103">
-        <v>78.88413775868344</v>
+        <v>78.88413775868342</v>
       </c>
       <c r="H103">
         <v>1603.26</v>
@@ -11918,7 +11918,7 @@
         <v>1351.15255</v>
       </c>
       <c r="S103">
-        <v>7.448497881285855</v>
+        <v>7.448497881285856</v>
       </c>
       <c r="T103">
         <v>3616.20992</v>
@@ -11966,7 +11966,7 @@
         <v>3</v>
       </c>
       <c r="AI103">
-        <v>4053.457649999999</v>
+        <v>4053.45765</v>
       </c>
     </row>
     <row r="104">
@@ -11995,7 +11995,7 @@
         <v>12247.15</v>
       </c>
       <c r="G104">
-        <v>67.51485672494204</v>
+        <v>67.51485672494202</v>
       </c>
       <c r="H104">
         <v>385.08</v>
@@ -12108,7 +12108,7 @@
         <v>13585.76</v>
       </c>
       <c r="G105">
-        <v>74.89421129809371</v>
+        <v>74.89421129809369</v>
       </c>
       <c r="H105">
         <v>1185.27</v>
@@ -12120,7 +12120,7 @@
         <v>0</v>
       </c>
       <c r="K105">
-        <v>6.534037243797295</v>
+        <v>6.534037243797294</v>
       </c>
       <c r="L105">
         <v>0</v>
@@ -12144,7 +12144,7 @@
         <v>1300.14625</v>
       </c>
       <c r="S105">
-        <v>7.167315480762517</v>
+        <v>7.167315480762516</v>
       </c>
       <c r="T105">
         <v>2929.39002</v>
@@ -12221,7 +12221,7 @@
         <v>12266.49</v>
       </c>
       <c r="G106">
-        <v>67.62147233176162</v>
+        <v>67.62147233176159</v>
       </c>
       <c r="H106">
         <v>463.29</v>
@@ -12233,7 +12233,7 @@
         <v>0</v>
       </c>
       <c r="K106">
-        <v>2.553978515172787</v>
+        <v>2.553978515172786</v>
       </c>
       <c r="L106">
         <v>0</v>
@@ -12257,7 +12257,7 @@
         <v>1240.70238</v>
       </c>
       <c r="S106">
-        <v>6.839619292977924</v>
+        <v>6.839619292977923</v>
       </c>
       <c r="T106">
         <v>2345.96002</v>
@@ -12334,7 +12334,7 @@
         <v>12956.01</v>
       </c>
       <c r="G107">
-        <v>71.42258883715118</v>
+        <v>71.42258883715117</v>
       </c>
       <c r="H107">
         <v>550.62</v>
@@ -12370,7 +12370,7 @@
         <v>1367.91901</v>
       </c>
       <c r="S107">
-        <v>7.540926335635192</v>
+        <v>7.540926335635191</v>
       </c>
       <c r="T107">
         <v>2087.11996</v>
@@ -12560,10 +12560,10 @@
         <v>18303.41</v>
       </c>
       <c r="G109">
-        <v>79.93284853654792</v>
+        <v>79.93284853654791</v>
       </c>
       <c r="H109">
-        <v>472.7499999999999</v>
+        <v>472.75</v>
       </c>
       <c r="I109">
         <v>0</v>
@@ -12596,7 +12596,7 @@
         <v>1772.41724</v>
       </c>
       <c r="S109">
-        <v>7.740325916781971</v>
+        <v>7.74032591678197</v>
       </c>
       <c r="T109">
         <v>2454.89998</v>
@@ -12685,7 +12685,7 @@
         <v>0</v>
       </c>
       <c r="K110">
-        <v>1.783742591394335</v>
+        <v>1.783742591394336</v>
       </c>
       <c r="L110">
         <v>0</v>
@@ -12899,7 +12899,7 @@
         <v>19147.53</v>
       </c>
       <c r="G112">
-        <v>85.15633651543349</v>
+        <v>85.15633651543351</v>
       </c>
       <c r="H112">
         <v>370.36</v>
@@ -12935,7 +12935,7 @@
         <v>1718.72645</v>
       </c>
       <c r="S112">
-        <v>7.643829149460865</v>
+        <v>7.643829149460866</v>
       </c>
       <c r="T112">
         <v>1940.40001</v>
@@ -12983,7 +12983,7 @@
         <v>3</v>
       </c>
       <c r="AI112">
-        <v>5156.179349999999</v>
+        <v>5156.17935</v>
       </c>
     </row>
     <row r="113">
@@ -13125,7 +13125,7 @@
         <v>16065.62</v>
       </c>
       <c r="G114">
-        <v>70.16019256006037</v>
+        <v>70.16019256006038</v>
       </c>
       <c r="H114">
         <v>375.7</v>
@@ -13161,7 +13161,7 @@
         <v>1707.62189</v>
       </c>
       <c r="S114">
-        <v>7.457358049186664</v>
+        <v>7.457358049186663</v>
       </c>
       <c r="T114">
         <v>2101.00999</v>
@@ -13209,7 +13209,7 @@
         <v>3</v>
       </c>
       <c r="AI114">
-        <v>5122.86567</v>
+        <v>5122.865669999999</v>
       </c>
     </row>
     <row r="115">
@@ -13238,7 +13238,7 @@
         <v>17963.75</v>
       </c>
       <c r="G115">
-        <v>79.89161735634409</v>
+        <v>79.89161735634407</v>
       </c>
       <c r="H115">
         <v>370.21</v>
@@ -13274,7 +13274,7 @@
         <v>1698.34145</v>
       </c>
       <c r="S115">
-        <v>7.553169313969441</v>
+        <v>7.553169313969442</v>
       </c>
       <c r="T115">
         <v>1988.68005</v>
@@ -13322,7 +13322,7 @@
         <v>3</v>
       </c>
       <c r="AI115">
-        <v>5095.02435</v>
+        <v>5095.024350000001</v>
       </c>
     </row>
     <row r="116">
@@ -13351,7 +13351,7 @@
         <v>16860.45</v>
       </c>
       <c r="G116">
-        <v>74.74106193604921</v>
+        <v>74.74106193604919</v>
       </c>
       <c r="H116">
         <v>198.18</v>
@@ -13363,7 +13363,7 @@
         <v>0</v>
       </c>
       <c r="K116">
-        <v>0.8785165078326039</v>
+        <v>0.878516507832604</v>
       </c>
       <c r="L116">
         <v>0</v>
@@ -13387,7 +13387,7 @@
         <v>1727.96753</v>
       </c>
       <c r="S116">
-        <v>7.659945504610609</v>
+        <v>7.659945504610608</v>
       </c>
       <c r="T116">
         <v>2211.12</v>
@@ -13435,7 +13435,7 @@
         <v>3</v>
       </c>
       <c r="AI116">
-        <v>5183.902590000001</v>
+        <v>5183.90259</v>
       </c>
     </row>
     <row r="117">
@@ -13464,10 +13464,10 @@
         <v>18388.95</v>
       </c>
       <c r="G117">
-        <v>81.78264321118603</v>
+        <v>81.78264321118604</v>
       </c>
       <c r="H117">
-        <v>270.9999999999999</v>
+        <v>271</v>
       </c>
       <c r="I117">
         <v>0</v>
@@ -13500,7 +13500,7 @@
         <v>1735.53757</v>
       </c>
       <c r="S117">
-        <v>7.718594583536246</v>
+        <v>7.718594583536245</v>
       </c>
       <c r="T117">
         <v>1729.52995</v>
@@ -13548,7 +13548,7 @@
         <v>3</v>
       </c>
       <c r="AI117">
-        <v>5206.61271</v>
+        <v>5206.612709999999</v>
       </c>
     </row>
     <row r="118">
@@ -13613,7 +13613,7 @@
         <v>1527.87451</v>
       </c>
       <c r="S118">
-        <v>6.772948728083817</v>
+        <v>6.772948728083818</v>
       </c>
       <c r="T118">
         <v>1992.10995</v>
@@ -13661,7 +13661,7 @@
         <v>3</v>
       </c>
       <c r="AI118">
-        <v>4583.62353</v>
+        <v>4583.623530000001</v>
       </c>
     </row>
     <row r="119">
@@ -13702,7 +13702,7 @@
         <v>0</v>
       </c>
       <c r="K119">
-        <v>4.8997186563169</v>
+        <v>4.899718656316899</v>
       </c>
       <c r="L119">
         <v>0</v>
@@ -13729,7 +13729,7 @@
         <v>6.606615921757134</v>
       </c>
       <c r="T119">
-        <v>3415.690039999999</v>
+        <v>3415.69004</v>
       </c>
       <c r="U119">
         <v>77</v>
@@ -13803,7 +13803,7 @@
         <v>18290.91</v>
       </c>
       <c r="G120">
-        <v>74.02184932102797</v>
+        <v>74.021849321028</v>
       </c>
       <c r="H120">
         <v>113.2</v>
@@ -13839,7 +13839,7 @@
         <v>1736.55142</v>
       </c>
       <c r="S120">
-        <v>7.027684655900511</v>
+        <v>7.02768465590051</v>
       </c>
       <c r="T120">
         <v>1459.61002</v>
@@ -13887,7 +13887,7 @@
         <v>3</v>
       </c>
       <c r="AI120">
-        <v>5209.654260000001</v>
+        <v>5209.65426</v>
       </c>
     </row>
     <row r="121">
@@ -14065,10 +14065,10 @@
         <v>1747.75452</v>
       </c>
       <c r="S122">
-        <v>7.052093914697219</v>
+        <v>7.052093914697221</v>
       </c>
       <c r="T122">
-        <v>2673.450039999999</v>
+        <v>2673.45004</v>
       </c>
       <c r="U122">
         <v>69</v>
@@ -14330,7 +14330,7 @@
         <v>0</v>
       </c>
       <c r="AF124">
-        <v>822.8863999999999</v>
+        <v>822.8864</v>
       </c>
       <c r="AG124">
         <v>0</v>
@@ -14591,10 +14591,10 @@
         <v>91.82383333333334</v>
       </c>
       <c r="F127">
-        <v>5290.240000000001</v>
+        <v>5290.24</v>
       </c>
       <c r="G127">
-        <v>57.61292910518874</v>
+        <v>57.61292910518873</v>
       </c>
       <c r="H127">
         <v>81.05</v>
@@ -14627,10 +14627,10 @@
         <v>33.984</v>
       </c>
       <c r="R127">
-        <v>662.6083799999999</v>
+        <v>662.60838</v>
       </c>
       <c r="S127">
-        <v>7.216082752662252</v>
+        <v>7.216082752662254</v>
       </c>
       <c r="T127">
         <v>571.95001</v>
@@ -14707,7 +14707,7 @@
         <v>7157.05</v>
       </c>
       <c r="G128">
-        <v>63.24549543578731</v>
+        <v>63.24549543578732</v>
       </c>
       <c r="H128">
         <v>225.97</v>
@@ -14743,7 +14743,7 @@
         <v>628.97713</v>
       </c>
       <c r="S128">
-        <v>5.55815178105918</v>
+        <v>5.558151781059181</v>
       </c>
       <c r="T128">
         <v>1047.82999</v>
@@ -14820,7 +14820,7 @@
         <v>6408.839999999999</v>
       </c>
       <c r="G129">
-        <v>56.63370536306035</v>
+        <v>56.63370536306036</v>
       </c>
       <c r="H129">
         <v>286.85</v>
@@ -14856,7 +14856,7 @@
         <v>613.2202</v>
       </c>
       <c r="S129">
-        <v>5.418910774723186</v>
+        <v>5.418910774723187</v>
       </c>
       <c r="T129">
         <v>1023.20001</v>
@@ -15043,10 +15043,10 @@
         <v>113.1631666666667</v>
       </c>
       <c r="F131">
-        <v>6269.599999999999</v>
+        <v>6269.6</v>
       </c>
       <c r="G131">
-        <v>55.40318625465588</v>
+        <v>55.40318625465589</v>
       </c>
       <c r="H131">
         <v>211.59</v>
@@ -15085,7 +15085,7 @@
         <v>5.473698980380837</v>
       </c>
       <c r="T131">
-        <v>780.1500000000001</v>
+        <v>780.15</v>
       </c>
       <c r="U131">
         <v>18</v>
@@ -15156,7 +15156,7 @@
         <v>113.163</v>
       </c>
       <c r="F132">
-        <v>6279.680000000001</v>
+        <v>6279.68</v>
       </c>
       <c r="G132">
         <v>55.49234290359924</v>
@@ -15195,7 +15195,7 @@
         <v>647.28536</v>
       </c>
       <c r="S132">
-        <v>5.719938142325671</v>
+        <v>5.719938142325672</v>
       </c>
       <c r="T132">
         <v>882.44998</v>
@@ -15272,7 +15272,7 @@
         <v>6758.219999999999</v>
       </c>
       <c r="G133">
-        <v>59.72111025688607</v>
+        <v>59.72111025688608</v>
       </c>
       <c r="H133">
         <v>242.25</v>
@@ -15308,7 +15308,7 @@
         <v>630.8665599999999</v>
       </c>
       <c r="S133">
-        <v>5.574848316145736</v>
+        <v>5.574848316145737</v>
       </c>
       <c r="T133">
         <v>831.40002</v>
@@ -15424,7 +15424,7 @@
         <v>5.074410891870847</v>
       </c>
       <c r="T134">
-        <v>678.8100099999999</v>
+        <v>678.81001</v>
       </c>
       <c r="U134">
         <v>22</v>
@@ -15950,7 +15950,7 @@
         <v>6046.12</v>
       </c>
       <c r="G139">
-        <v>53.42841741558636</v>
+        <v>53.42841741558637</v>
       </c>
       <c r="H139">
         <v>73.61999999999999</v>
@@ -15962,7 +15962,7 @@
         <v>0</v>
       </c>
       <c r="K139">
-        <v>0.6505659977201027</v>
+        <v>0.6505659977201028</v>
       </c>
       <c r="L139">
         <v>0</v>
@@ -15986,7 +15986,7 @@
         <v>609.1166899999999</v>
       </c>
       <c r="S139">
-        <v>5.382648833982838</v>
+        <v>5.382648833982839</v>
       </c>
       <c r="T139">
         <v>719.31999</v>
@@ -16176,7 +16176,7 @@
         <v>17288.56</v>
       </c>
       <c r="G141">
-        <v>55.98173722982271</v>
+        <v>55.98173722982272</v>
       </c>
       <c r="H141">
         <v>1693.79</v>
@@ -16212,10 +16212,10 @@
         <v>1792.5641</v>
       </c>
       <c r="S141">
-        <v>5.804465635877924</v>
+        <v>5.804465635877925</v>
       </c>
       <c r="T141">
-        <v>2785.420029999999</v>
+        <v>2785.42003</v>
       </c>
       <c r="U141">
         <v>33</v>
@@ -16260,7 +16260,7 @@
         <v>3</v>
       </c>
       <c r="AI141">
-        <v>5377.6923</v>
+        <v>5377.692300000001</v>
       </c>
     </row>
     <row r="142">
@@ -16289,7 +16289,7 @@
         <v>17287.79</v>
       </c>
       <c r="G142">
-        <v>55.97924390836233</v>
+        <v>55.97924390836235</v>
       </c>
       <c r="H142">
         <v>1844.95</v>
@@ -16402,7 +16402,7 @@
         <v>16298.97</v>
       </c>
       <c r="G143">
-        <v>52.77736582206753</v>
+        <v>52.77736582206752</v>
       </c>
       <c r="H143">
         <v>1011.57</v>
@@ -16438,7 +16438,7 @@
         <v>2036.07937</v>
       </c>
       <c r="S143">
-        <v>6.5929875172023</v>
+        <v>6.592987517202299</v>
       </c>
       <c r="T143">
         <v>2179.37</v>
@@ -16486,7 +16486,7 @@
         <v>3</v>
       </c>
       <c r="AI143">
-        <v>6108.238110000001</v>
+        <v>6108.23811</v>
       </c>
     </row>
     <row r="144">
@@ -16744,7 +16744,7 @@
         <v>56.35887638630292</v>
       </c>
       <c r="H146">
-        <v>2977.800000000001</v>
+        <v>2977.8</v>
       </c>
       <c r="I146">
         <v>0</v>
@@ -16753,7 +16753,7 @@
         <v>0</v>
       </c>
       <c r="K146">
-        <v>9.642354084028174</v>
+        <v>9.642354084028172</v>
       </c>
       <c r="L146">
         <v>25.15</v>
@@ -16780,7 +16780,7 @@
         <v>5.484220286570064</v>
       </c>
       <c r="T146">
-        <v>3890.109990000001</v>
+        <v>3890.10999</v>
       </c>
       <c r="U146">
         <v>72</v>
@@ -16967,7 +16967,7 @@
         <v>18002.72</v>
       </c>
       <c r="G148">
-        <v>58.5430828248623</v>
+        <v>58.54308282486232</v>
       </c>
       <c r="H148">
         <v>1789.95</v>
@@ -16979,7 +16979,7 @@
         <v>0</v>
       </c>
       <c r="K148">
-        <v>5.820742149095374</v>
+        <v>5.820742149095375</v>
       </c>
       <c r="L148">
         <v>15.06</v>
@@ -17003,7 +17003,7 @@
         <v>1845.8524</v>
       </c>
       <c r="S148">
-        <v>6.002531280588203</v>
+        <v>6.002531280588205</v>
       </c>
       <c r="T148">
         <v>3176.92003</v>
@@ -17051,7 +17051,7 @@
         <v>3</v>
       </c>
       <c r="AI148">
-        <v>5537.557199999999</v>
+        <v>5537.5572</v>
       </c>
     </row>
     <row r="149">
@@ -17080,7 +17080,7 @@
         <v>18391.61</v>
       </c>
       <c r="G149">
-        <v>59.80771502931589</v>
+        <v>59.80771502931591</v>
       </c>
       <c r="H149">
         <v>1796.91</v>
@@ -17092,7 +17092,7 @@
         <v>0</v>
       </c>
       <c r="K149">
-        <v>5.843375387653829</v>
+        <v>5.84337538765383</v>
       </c>
       <c r="L149">
         <v>0</v>
@@ -17318,7 +17318,7 @@
         <v>0</v>
       </c>
       <c r="K151">
-        <v>4.971475398818692</v>
+        <v>4.971475398818693</v>
       </c>
       <c r="L151">
         <v>0</v>
@@ -17342,7 +17342,7 @@
         <v>1518.91438</v>
       </c>
       <c r="S151">
-        <v>4.939360849483544</v>
+        <v>4.939360849483545</v>
       </c>
       <c r="T151">
         <v>2837.21004</v>
@@ -17422,7 +17422,7 @@
         <v>58.49134623168462</v>
       </c>
       <c r="H152">
-        <v>2111.720000000001</v>
+        <v>2111.72</v>
       </c>
       <c r="I152">
         <v>0</v>
@@ -17431,7 +17431,7 @@
         <v>0</v>
       </c>
       <c r="K152">
-        <v>6.837917914676599</v>
+        <v>6.837917914676598</v>
       </c>
       <c r="L152">
         <v>0</v>
@@ -17455,10 +17455,10 @@
         <v>1643.06226</v>
       </c>
       <c r="S152">
-        <v>5.320366744920261</v>
+        <v>5.320366744920263</v>
       </c>
       <c r="T152">
-        <v>3515.660060000001</v>
+        <v>3515.66006</v>
       </c>
       <c r="U152">
         <v>64</v>
@@ -17503,7 +17503,7 @@
         <v>3</v>
       </c>
       <c r="AI152">
-        <v>4929.186779999999</v>
+        <v>4929.18678</v>
       </c>
     </row>
     <row r="153">
@@ -17645,7 +17645,7 @@
         <v>16062.82</v>
       </c>
       <c r="G154">
-        <v>52.23471795711174</v>
+        <v>52.23471795711175</v>
       </c>
       <c r="H154">
         <v>1969.79</v>
@@ -17657,7 +17657,7 @@
         <v>0</v>
       </c>
       <c r="K154">
-        <v>6.405564221272426</v>
+        <v>6.405564221272427</v>
       </c>
       <c r="L154">
         <v>0</v>
@@ -17681,7 +17681,7 @@
         <v>1632.26711</v>
       </c>
       <c r="S154">
-        <v>5.307972829274056</v>
+        <v>5.307972829274057</v>
       </c>
       <c r="T154">
         <v>2698.55997</v>
@@ -17755,7 +17755,7 @@
         <v>218.5791666666667</v>
       </c>
       <c r="F155">
-        <v>7924.959999999999</v>
+        <v>7924.96</v>
       </c>
       <c r="G155">
         <v>36.25670333021979</v>
@@ -17833,7 +17833,7 @@
         <v>0</v>
       </c>
       <c r="AF155">
-        <v>763.7615999999999</v>
+        <v>763.7616</v>
       </c>
       <c r="AG155">
         <v>0</v>
@@ -17907,7 +17907,7 @@
         <v>1789.01184</v>
       </c>
       <c r="S156">
-        <v>5.817691344628995</v>
+        <v>5.817691344628996</v>
       </c>
       <c r="T156">
         <v>3031.64001</v>
@@ -17996,7 +17996,7 @@
         <v>0</v>
       </c>
       <c r="K157">
-        <v>5.12441235419284</v>
+        <v>5.124412354192842</v>
       </c>
       <c r="L157">
         <v>0</v>
@@ -18068,7 +18068,7 @@
         <v>3</v>
       </c>
       <c r="AI157">
-        <v>3946.121400000001</v>
+        <v>3946.1214</v>
       </c>
     </row>
     <row r="158">
@@ -18097,7 +18097,7 @@
         <v>16085.98</v>
       </c>
       <c r="G158">
-        <v>61.3519880494549</v>
+        <v>61.35198804945492</v>
       </c>
       <c r="H158">
         <v>1298.26</v>
@@ -18285,7 +18285,7 @@
         <v>0</v>
       </c>
       <c r="AF159">
-        <v>448.2918999999999</v>
+        <v>448.2919</v>
       </c>
       <c r="AG159">
         <v>0</v>
@@ -18659,10 +18659,10 @@
         <v>105.6831666666667</v>
       </c>
       <c r="F163">
-        <v>5287.570000000001</v>
+        <v>5287.57</v>
       </c>
       <c r="G163">
-        <v>50.03228202536198</v>
+        <v>50.03228202536197</v>
       </c>
       <c r="H163">
         <v>199.18</v>
@@ -18998,10 +18998,10 @@
         <v>105.6831666666667</v>
       </c>
       <c r="F166">
-        <v>5265.499999999999</v>
+        <v>5265.5</v>
       </c>
       <c r="G166">
-        <v>49.82345028142292</v>
+        <v>49.82345028142294</v>
       </c>
       <c r="H166">
         <v>224.31</v>
@@ -19489,7 +19489,7 @@
         <v>436.54252</v>
       </c>
       <c r="S170">
-        <v>4.130672213644872</v>
+        <v>4.130672213644873</v>
       </c>
       <c r="T170">
         <v>272.29999</v>
@@ -19715,7 +19715,7 @@
         <v>464.15392</v>
       </c>
       <c r="S172">
-        <v>4.391938041220693</v>
+        <v>4.391938041220692</v>
       </c>
       <c r="T172">
         <v>486.08001</v>
@@ -19792,7 +19792,7 @@
         <v>2972.92</v>
       </c>
       <c r="G173">
-        <v>28.13049697287017</v>
+        <v>28.13049697287016</v>
       </c>
       <c r="H173">
         <v>30.82</v>
@@ -21590,20 +21590,20 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E189">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F189">
-        <v>5195.110000000001</v>
+        <v>10456.34</v>
       </c>
       <c r="G189">
-        <v>48.45431369501011</v>
+        <v>48.69944964952999</v>
       </c>
       <c r="H189">
-        <v>45.89</v>
+        <v>104.03</v>
       </c>
       <c r="I189">
         <v>0</v>
@@ -21612,70 +21612,70 @@
         <v>0</v>
       </c>
       <c r="K189">
-        <v>0.4280118140836313</v>
+        <v>0.4845102346557787</v>
       </c>
       <c r="L189">
         <v>0</v>
       </c>
       <c r="M189">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N189">
         <v>0</v>
       </c>
       <c r="O189">
-        <v>23.02415</v>
+        <v>26.51126</v>
       </c>
       <c r="P189">
-        <v>71.14123717711037</v>
+        <v>81.91589420343593</v>
       </c>
       <c r="Q189">
         <v>32.364</v>
       </c>
       <c r="R189">
-        <v>583.91674</v>
+        <v>1056.91405</v>
       </c>
       <c r="S189">
-        <v>5.446137789522773</v>
+        <v>4.922480768782941</v>
       </c>
       <c r="T189">
-        <v>1072.94997</v>
+        <v>1567.55997</v>
       </c>
       <c r="U189">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="V189">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="W189">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="X189">
-        <v>101</v>
+        <v>147</v>
       </c>
       <c r="Y189">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="Z189">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="AA189">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="AB189">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="AC189">
         <v>4.03344</v>
       </c>
       <c r="AD189">
-        <v>-3.17966</v>
+        <v>-1.46059</v>
       </c>
       <c r="AE189">
         <v>0</v>
       </c>
       <c r="AF189">
-        <v>435.3636</v>
+        <v>847.581</v>
       </c>
       <c r="AG189">
         <v>0</v>
@@ -21684,7 +21684,7 @@
         <v>3</v>
       </c>
       <c r="AI189">
-        <v>1751.75022</v>
+        <v>3170.74215</v>
       </c>
     </row>
     <row r="190">
@@ -21703,20 +21703,20 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E190">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F190">
-        <v>5495.650000000001</v>
+        <v>11093.82</v>
       </c>
       <c r="G190">
-        <v>51.25742266438676</v>
+        <v>51.66845459414564</v>
       </c>
       <c r="H190">
-        <v>125.76</v>
+        <v>190.83</v>
       </c>
       <c r="I190">
         <v>0</v>
@@ -21725,70 +21725,70 @@
         <v>0</v>
       </c>
       <c r="K190">
-        <v>1.172951966423131</v>
+        <v>0.8887733161526699</v>
       </c>
       <c r="L190">
         <v>0</v>
       </c>
       <c r="M190">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N190">
         <v>0</v>
       </c>
       <c r="O190">
-        <v>23.85232</v>
+        <v>27.01389</v>
       </c>
       <c r="P190">
-        <v>73.61827160493827</v>
+        <v>83.37620370370371</v>
       </c>
       <c r="Q190">
         <v>32.4</v>
       </c>
       <c r="R190">
-        <v>692.91357</v>
+        <v>1312.96965</v>
       </c>
       <c r="S190">
-        <v>6.462741209389088</v>
+        <v>6.115036366600169</v>
       </c>
       <c r="T190">
-        <v>1269.02001</v>
+        <v>1912.92002</v>
       </c>
       <c r="U190">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="V190">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="W190">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="X190">
-        <v>116</v>
+        <v>191</v>
       </c>
       <c r="Y190">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="Z190">
-        <v>117</v>
+        <v>160</v>
       </c>
       <c r="AA190">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="AB190">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="AC190">
-        <v>4.04281</v>
+        <v>4.05143</v>
       </c>
       <c r="AD190">
-        <v>-3.33386</v>
+        <v>-1.27618</v>
       </c>
       <c r="AE190">
         <v>0</v>
       </c>
       <c r="AF190">
-        <v>481.6434</v>
+        <v>934.2787999999999</v>
       </c>
       <c r="AG190">
         <v>0</v>
@@ -21797,7 +21797,7 @@
         <v>3</v>
       </c>
       <c r="AI190">
-        <v>2078.74071</v>
+        <v>3938.90895</v>
       </c>
     </row>
     <row r="191">
@@ -21816,20 +21816,20 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E191">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F191">
-        <v>4651.41</v>
+        <v>9885.26</v>
       </c>
       <c r="G191">
-        <v>43.38327374475361</v>
+        <v>46.03969664744191</v>
       </c>
       <c r="H191">
-        <v>40.74999999999999</v>
+        <v>118.61</v>
       </c>
       <c r="I191">
         <v>0</v>
@@ -21838,70 +21838,70 @@
         <v>0</v>
       </c>
       <c r="K191">
-        <v>0.3800715062956629</v>
+        <v>0.5524152545662012</v>
       </c>
       <c r="L191">
         <v>0</v>
       </c>
       <c r="M191">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N191">
         <v>0</v>
       </c>
       <c r="O191">
-        <v>23.48263</v>
+        <v>25.87651</v>
       </c>
       <c r="P191">
-        <v>69.09907603578154</v>
+        <v>76.14321445386064</v>
       </c>
       <c r="Q191">
         <v>33.984</v>
       </c>
       <c r="R191">
-        <v>634.18938</v>
+        <v>1224.11294</v>
       </c>
       <c r="S191">
-        <v>5.91502608425307</v>
+        <v>5.701194345905749</v>
       </c>
       <c r="T191">
-        <v>865.99002</v>
+        <v>1277.86002</v>
       </c>
       <c r="U191">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="V191">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="W191">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="X191">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="Y191">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="Z191">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="AA191">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="AB191">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="AC191">
         <v>4.19102</v>
       </c>
       <c r="AD191">
-        <v>-3.26787</v>
+        <v>-1.23637</v>
       </c>
       <c r="AE191">
         <v>0</v>
       </c>
       <c r="AF191">
-        <v>448.1776</v>
+        <v>919.9072</v>
       </c>
       <c r="AG191">
         <v>0</v>
@@ -21910,7 +21910,7 @@
         <v>3</v>
       </c>
       <c r="AI191">
-        <v>1902.56814</v>
+        <v>3672.33882</v>
       </c>
     </row>
     <row r="192">
@@ -21929,20 +21929,20 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E192">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F192">
-        <v>5713.139999999999</v>
+        <v>12163.65</v>
       </c>
       <c r="G192">
-        <v>53.28593191357064</v>
+        <v>56.65109022177027</v>
       </c>
       <c r="H192">
-        <v>212.13</v>
+        <v>361.6100000000001</v>
       </c>
       <c r="I192">
         <v>0</v>
@@ -21951,70 +21951,70 @@
         <v>0</v>
       </c>
       <c r="K192">
-        <v>1.978517021607337</v>
+        <v>1.684165586406577</v>
       </c>
       <c r="L192">
         <v>0</v>
       </c>
       <c r="M192">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N192">
         <v>0</v>
       </c>
       <c r="O192">
-        <v>25.38063</v>
+        <v>28.72615</v>
       </c>
       <c r="P192">
-        <v>71.35804655870446</v>
+        <v>80.76402946468737</v>
       </c>
       <c r="Q192">
         <v>35.568</v>
       </c>
       <c r="R192">
-        <v>551.8525500000001</v>
+        <v>1141.34858</v>
       </c>
       <c r="S192">
-        <v>5.147078035131354</v>
+        <v>5.315726889549551</v>
       </c>
       <c r="T192">
-        <v>1246.49002</v>
+        <v>1981.19004</v>
       </c>
       <c r="U192">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="V192">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="W192">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="X192">
-        <v>114</v>
+        <v>192</v>
       </c>
       <c r="Y192">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="Z192">
-        <v>100</v>
+        <v>161</v>
       </c>
       <c r="AA192">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="AB192">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="AC192">
-        <v>4.44502</v>
+        <v>4.46698</v>
       </c>
       <c r="AD192">
-        <v>-3.52053</v>
+        <v>-1.10449</v>
       </c>
       <c r="AE192">
         <v>0</v>
       </c>
       <c r="AF192">
-        <v>563.0312</v>
+        <v>1162.4072</v>
       </c>
       <c r="AG192">
         <v>0</v>
@@ -22023,7 +22023,7 @@
         <v>3</v>
       </c>
       <c r="AI192">
-        <v>1655.55765</v>
+        <v>3424.04574</v>
       </c>
     </row>
     <row r="193">
@@ -22042,20 +22042,20 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E193">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F193">
-        <v>4908.21</v>
+        <v>10724.31</v>
       </c>
       <c r="G193">
-        <v>45.77842375252604</v>
+        <v>49.94749547843232</v>
       </c>
       <c r="H193">
-        <v>70.10999999999999</v>
+        <v>254.13</v>
       </c>
       <c r="I193">
         <v>0</v>
@@ -22064,70 +22064,70 @@
         <v>0</v>
       </c>
       <c r="K193">
-        <v>0.6539095289911393</v>
+        <v>1.183587291483928</v>
       </c>
       <c r="L193">
         <v>0</v>
       </c>
       <c r="M193">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N193">
         <v>0</v>
       </c>
       <c r="O193">
-        <v>24.03125</v>
+        <v>27.47896</v>
       </c>
       <c r="P193">
-        <v>66.75347222222221</v>
+        <v>76.33044444444444</v>
       </c>
       <c r="Q193">
         <v>36</v>
       </c>
       <c r="R193">
-        <v>550.08794</v>
+        <v>1095.76894</v>
       </c>
       <c r="S193">
-        <v>5.130619679776154</v>
+        <v>5.103443874343111</v>
       </c>
       <c r="T193">
-        <v>1076.36</v>
+        <v>1877.14</v>
       </c>
       <c r="U193">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="V193">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="W193">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="X193">
-        <v>109</v>
+        <v>189</v>
       </c>
       <c r="Y193">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="Z193">
-        <v>110</v>
+        <v>168</v>
       </c>
       <c r="AA193">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="AB193">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="AC193">
         <v>4.20634</v>
       </c>
       <c r="AD193">
-        <v>-2.69485</v>
+        <v>-2.16614</v>
       </c>
       <c r="AE193">
         <v>0</v>
       </c>
       <c r="AF193">
-        <v>426.9895</v>
+        <v>905.9435</v>
       </c>
       <c r="AG193">
         <v>0</v>
@@ -22136,7 +22136,7 @@
         <v>3</v>
       </c>
       <c r="AI193">
-        <v>1650.26382</v>
+        <v>3287.30682</v>
       </c>
     </row>
     <row r="194">
@@ -22155,20 +22155,20 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E194">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F194">
-        <v>4594.64</v>
+        <v>9824.199999999999</v>
       </c>
       <c r="G194">
-        <v>42.85378517021608</v>
+        <v>45.75531526776219</v>
       </c>
       <c r="H194">
-        <v>52.35</v>
+        <v>196.96</v>
       </c>
       <c r="I194">
         <v>0</v>
@@ -22177,7 +22177,7 @@
         <v>0</v>
       </c>
       <c r="K194">
-        <v>0.48826364060314</v>
+        <v>0.9173232319311946</v>
       </c>
       <c r="L194">
         <v>0</v>
@@ -22189,58 +22189,58 @@
         <v>0</v>
       </c>
       <c r="O194">
-        <v>23.2906</v>
+        <v>24.12588</v>
       </c>
       <c r="P194">
-        <v>72.7740282464692</v>
+        <v>75.38395200599925</v>
       </c>
       <c r="Q194">
         <v>32.004</v>
       </c>
       <c r="R194">
-        <v>529.2741599999999</v>
+        <v>1063.36103</v>
       </c>
       <c r="S194">
-        <v>4.936491465879061</v>
+        <v>4.952506989994333</v>
       </c>
       <c r="T194">
-        <v>852.3900100000001</v>
+        <v>1460.52001</v>
       </c>
       <c r="U194">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="V194">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="W194">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="X194">
-        <v>77</v>
+        <v>130</v>
       </c>
       <c r="Y194">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="Z194">
-        <v>94</v>
+        <v>141</v>
       </c>
       <c r="AA194">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="AB194">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AC194">
         <v>4.18355</v>
       </c>
       <c r="AD194">
-        <v>-2.8917</v>
+        <v>-1.49791</v>
       </c>
       <c r="AE194">
         <v>0</v>
       </c>
       <c r="AF194">
-        <v>333.8274</v>
+        <v>697.2546</v>
       </c>
       <c r="AG194">
         <v>0</v>
@@ -22249,7 +22249,7 @@
         <v>3</v>
       </c>
       <c r="AI194">
-        <v>1587.82248</v>
+        <v>3190.08309</v>
       </c>
     </row>
     <row r="195">
@@ -22268,20 +22268,20 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E195">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F195">
-        <v>5620.669999999999</v>
+        <v>11322.65</v>
       </c>
       <c r="G195">
-        <v>52.42347271879371</v>
+        <v>52.73420944367252</v>
       </c>
       <c r="H195">
-        <v>333.89</v>
+        <v>463.88</v>
       </c>
       <c r="I195">
         <v>0</v>
@@ -22290,7 +22290,7 @@
         <v>0</v>
       </c>
       <c r="K195">
-        <v>3.114161355510649</v>
+        <v>2.160478781621865</v>
       </c>
       <c r="L195">
         <v>0</v>
@@ -22311,49 +22311,49 @@
         <v>33.84</v>
       </c>
       <c r="R195">
-        <v>584.37918</v>
+        <v>1120.93282</v>
       </c>
       <c r="S195">
-        <v>5.45045092491839</v>
+        <v>5.220642349817973</v>
       </c>
       <c r="T195">
-        <v>1262.66999</v>
+        <v>1943.71999</v>
       </c>
       <c r="U195">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="V195">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="W195">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="X195">
-        <v>113</v>
+        <v>186</v>
       </c>
       <c r="Y195">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="Z195">
-        <v>96</v>
+        <v>153</v>
       </c>
       <c r="AA195">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="AB195">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="AC195">
         <v>4.22005</v>
       </c>
       <c r="AD195">
-        <v>-3.58805</v>
+        <v>-1.28486</v>
       </c>
       <c r="AE195">
         <v>0</v>
       </c>
       <c r="AF195">
-        <v>488.9521</v>
+        <v>954.4661</v>
       </c>
       <c r="AG195">
         <v>0</v>
@@ -22362,7 +22362,7 @@
         <v>3</v>
       </c>
       <c r="AI195">
-        <v>1753.13754</v>
+        <v>3362.79846</v>
       </c>
     </row>
     <row r="196">
@@ -22381,20 +22381,20 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E196">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F196">
-        <v>4946.24</v>
+        <v>10779.14</v>
       </c>
       <c r="G196">
-        <v>46.13312606870822</v>
+        <v>50.20286120145622</v>
       </c>
       <c r="H196">
-        <v>75.11</v>
+        <v>140.26</v>
       </c>
       <c r="I196">
         <v>0</v>
@@ -22403,7 +22403,7 @@
         <v>0</v>
       </c>
       <c r="K196">
-        <v>0.700544069640914</v>
+        <v>0.6532481545017736</v>
       </c>
       <c r="L196">
         <v>0</v>
@@ -22415,58 +22415,58 @@
         <v>0</v>
       </c>
       <c r="O196">
-        <v>23.6058</v>
+        <v>23.8992</v>
       </c>
       <c r="P196">
-        <v>70.05519943019944</v>
+        <v>70.92592592592594</v>
       </c>
       <c r="Q196">
         <v>33.696</v>
       </c>
       <c r="R196">
-        <v>576.6306499999999</v>
+        <v>1109.06043</v>
       </c>
       <c r="S196">
-        <v>5.378181097466189</v>
+        <v>5.165347776475429</v>
       </c>
       <c r="T196">
-        <v>1002.41</v>
+        <v>1670.01001</v>
       </c>
       <c r="U196">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="V196">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="W196">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="X196">
-        <v>105</v>
+        <v>168</v>
       </c>
       <c r="Y196">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="Z196">
-        <v>96</v>
+        <v>150</v>
       </c>
       <c r="AA196">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="AB196">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="AC196">
         <v>4.19611</v>
       </c>
       <c r="AD196">
-        <v>-3.5654</v>
+        <v>-1.60527</v>
       </c>
       <c r="AE196">
         <v>0</v>
       </c>
       <c r="AF196">
-        <v>485.1904</v>
+        <v>1027.1288</v>
       </c>
       <c r="AG196">
         <v>0</v>
@@ -22475,7 +22475,7 @@
         <v>3</v>
       </c>
       <c r="AI196">
-        <v>1729.89195</v>
+        <v>3327.18129</v>
       </c>
     </row>
     <row r="197">
@@ -22494,20 +22494,20 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E197">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F197">
-        <v>5316.98</v>
+        <v>11185.45</v>
       </c>
       <c r="G197">
-        <v>49.59098398880771</v>
+        <v>52.09521296001614</v>
       </c>
       <c r="H197">
-        <v>75.72000000000001</v>
+        <v>216.68</v>
       </c>
       <c r="I197">
         <v>0</v>
@@ -22516,70 +22516,70 @@
         <v>0</v>
       </c>
       <c r="K197">
-        <v>0.7062334836001867</v>
+        <v>1.009167332934866</v>
       </c>
       <c r="L197">
         <v>0</v>
       </c>
       <c r="M197">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N197">
         <v>0</v>
       </c>
       <c r="O197">
-        <v>23.60841</v>
+        <v>25.52795</v>
       </c>
       <c r="P197">
-        <v>67.46802126200274</v>
+        <v>72.95367512574303</v>
       </c>
       <c r="Q197">
         <v>34.992</v>
       </c>
       <c r="R197">
-        <v>540.59011</v>
+        <v>1046.27767</v>
       </c>
       <c r="S197">
-        <v>5.042034291932224</v>
+        <v>4.87294279925792</v>
       </c>
       <c r="T197">
-        <v>957.1699599999999</v>
+        <v>1464.97997</v>
       </c>
       <c r="U197">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="V197">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="W197">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="X197">
-        <v>97</v>
+        <v>148</v>
       </c>
       <c r="Y197">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="Z197">
-        <v>93</v>
+        <v>132</v>
       </c>
       <c r="AA197">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="AB197">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="AC197">
-        <v>3.94086</v>
+        <v>3.9913</v>
       </c>
       <c r="AD197">
-        <v>-3.06322</v>
+        <v>-0.9593</v>
       </c>
       <c r="AE197">
         <v>0</v>
       </c>
       <c r="AF197">
-        <v>438.60471</v>
+        <v>894.97623</v>
       </c>
       <c r="AG197">
         <v>0</v>
@@ -22588,7 +22588,7 @@
         <v>3</v>
       </c>
       <c r="AI197">
-        <v>1621.77033</v>
+        <v>3138.83301</v>
       </c>
     </row>
     <row r="198">
@@ -22607,20 +22607,20 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E198">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F198">
-        <v>5539.53</v>
+        <v>10768.12</v>
       </c>
       <c r="G198">
-        <v>51.66668739312917</v>
+        <v>50.15153655677769</v>
       </c>
       <c r="H198">
-        <v>76.3</v>
+        <v>216.32</v>
       </c>
       <c r="I198">
         <v>0</v>
@@ -22629,70 +22629,70 @@
         <v>0</v>
       </c>
       <c r="K198">
-        <v>0.7116430903155604</v>
+        <v>1.007490665776584</v>
       </c>
       <c r="L198">
         <v>0</v>
       </c>
       <c r="M198">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N198">
         <v>0</v>
       </c>
       <c r="O198">
-        <v>23.61024</v>
+        <v>26.55438</v>
       </c>
       <c r="P198">
-        <v>67.61237113402062</v>
+        <v>76.043470790378</v>
       </c>
       <c r="Q198">
         <v>34.92</v>
       </c>
       <c r="R198">
-        <v>611.42886</v>
+        <v>996.65897</v>
       </c>
       <c r="S198">
-        <v>5.702740805223068</v>
+        <v>4.641848230572784</v>
       </c>
       <c r="T198">
-        <v>1141.11002</v>
+        <v>1665.76002</v>
       </c>
       <c r="U198">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="V198">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W198">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="X198">
-        <v>110</v>
+        <v>162</v>
       </c>
       <c r="Y198">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="Z198">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="AA198">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="AB198">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="AC198">
-        <v>3.79987</v>
+        <v>3.88242</v>
       </c>
       <c r="AD198">
-        <v>-3.07619</v>
+        <v>-0.9626</v>
       </c>
       <c r="AE198">
         <v>0</v>
       </c>
       <c r="AF198">
-        <v>538.6207999999999</v>
+        <v>1012.1784</v>
       </c>
       <c r="AG198">
         <v>0</v>
@@ -22701,7 +22701,7 @@
         <v>3</v>
       </c>
       <c r="AI198">
-        <v>1834.28658</v>
+        <v>2989.97691</v>
       </c>
     </row>
     <row r="199">
@@ -22720,20 +22720,20 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E199">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F199">
-        <v>5258.72</v>
+        <v>10937.69</v>
       </c>
       <c r="G199">
-        <v>49.04759832115653</v>
+        <v>50.94129336241627</v>
       </c>
       <c r="H199">
-        <v>142.3</v>
+        <v>219.64</v>
       </c>
       <c r="I199">
         <v>0</v>
@@ -22742,70 +22742,70 @@
         <v>0</v>
       </c>
       <c r="K199">
-        <v>1.327219026892585</v>
+        <v>1.022953262902963</v>
       </c>
       <c r="L199">
         <v>0</v>
       </c>
       <c r="M199">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N199">
         <v>0</v>
       </c>
       <c r="O199">
-        <v>23.5701</v>
+        <v>26.66008</v>
       </c>
       <c r="P199">
-        <v>67.35853909465021</v>
+        <v>76.18907178783722</v>
       </c>
       <c r="Q199">
         <v>34.992</v>
       </c>
       <c r="R199">
-        <v>495.11263</v>
+        <v>930.4163699999999</v>
       </c>
       <c r="S199">
-        <v>4.617870013990362</v>
+        <v>4.333329364186079</v>
       </c>
       <c r="T199">
-        <v>1194.50999</v>
+        <v>1836.82999</v>
       </c>
       <c r="U199">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="V199">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="W199">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="X199">
-        <v>101</v>
+        <v>161</v>
       </c>
       <c r="Y199">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="Z199">
-        <v>111</v>
+        <v>168</v>
       </c>
       <c r="AA199">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="AB199">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="AC199">
         <v>4.11382</v>
       </c>
       <c r="AD199">
-        <v>-2.8103</v>
+        <v>-1.6686</v>
       </c>
       <c r="AE199">
         <v>0</v>
       </c>
       <c r="AF199">
-        <v>464.7894299999999</v>
+        <v>931.70318</v>
       </c>
       <c r="AG199">
         <v>0</v>
@@ -22814,7 +22814,7 @@
         <v>3</v>
       </c>
       <c r="AI199">
-        <v>1485.33789</v>
+        <v>2791.24911</v>
       </c>
     </row>
     <row r="200">
@@ -22833,20 +22833,20 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E200">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F200">
-        <v>4522.42</v>
+        <v>9357.35</v>
       </c>
       <c r="G200">
-        <v>42.18019586507073</v>
+        <v>43.5810039820845</v>
       </c>
       <c r="H200">
-        <v>42.38</v>
+        <v>105.98</v>
       </c>
       <c r="I200">
         <v>0</v>
@@ -22855,70 +22855,70 @@
         <v>0</v>
       </c>
       <c r="K200">
-        <v>0.3952743665474895</v>
+        <v>0.4935921817631396</v>
       </c>
       <c r="L200">
         <v>0</v>
       </c>
       <c r="M200">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N200">
         <v>0</v>
       </c>
       <c r="O200">
-        <v>22.91071</v>
+        <v>26.22896</v>
       </c>
       <c r="P200">
-        <v>67.41616643126177</v>
+        <v>77.18032015065913</v>
       </c>
       <c r="Q200">
         <v>33.984</v>
       </c>
       <c r="R200">
-        <v>576.23023</v>
+        <v>1064.56136</v>
       </c>
       <c r="S200">
-        <v>5.374446416912793</v>
+        <v>4.958097417466835</v>
       </c>
       <c r="T200">
-        <v>922.84999</v>
+        <v>1280.04999</v>
       </c>
       <c r="U200">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="V200">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="W200">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="X200">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="Y200">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="Z200">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="AA200">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="AB200">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="AC200">
         <v>4.06863</v>
       </c>
       <c r="AD200">
-        <v>-3.19859</v>
+        <v>-1.6363</v>
       </c>
       <c r="AE200">
         <v>0</v>
       </c>
       <c r="AF200">
-        <v>446.6696000000001</v>
+        <v>887.1184</v>
       </c>
       <c r="AG200">
         <v>0</v>
@@ -22927,7 +22927,7 @@
         <v>3</v>
       </c>
       <c r="AI200">
-        <v>1728.69069</v>
+        <v>3193.68408</v>
       </c>
     </row>
     <row r="201">
@@ -22946,20 +22946,20 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E201">
-        <v>53.16666666666666</v>
+        <v>160.7518333333333</v>
       </c>
       <c r="F201">
-        <v>1627.37</v>
+        <v>6211.17</v>
       </c>
       <c r="G201">
-        <v>30.60884012539185</v>
+        <v>38.63825295927159</v>
       </c>
       <c r="H201">
-        <v>0</v>
+        <v>42.98</v>
       </c>
       <c r="I201">
         <v>0</v>
@@ -22968,70 +22968,70 @@
         <v>0</v>
       </c>
       <c r="K201">
-        <v>0</v>
+        <v>0.2673686458734011</v>
       </c>
       <c r="L201">
         <v>0</v>
       </c>
       <c r="M201">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N201">
         <v>0</v>
       </c>
       <c r="O201">
-        <v>20.46638</v>
+        <v>25.29827</v>
       </c>
       <c r="P201">
-        <v>58.48874028349338</v>
+        <v>72.29729652491999</v>
       </c>
       <c r="Q201">
         <v>34.992</v>
       </c>
       <c r="R201">
-        <v>199.70353</v>
+        <v>698.01602</v>
       </c>
       <c r="S201">
-        <v>3.756179247648903</v>
+        <v>4.34219632539183</v>
       </c>
       <c r="T201">
-        <v>237.38</v>
+        <v>569.87</v>
       </c>
       <c r="U201">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="V201">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="W201">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="X201">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="Y201">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Z201">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="AA201">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="AB201">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="AC201">
         <v>3.84602</v>
       </c>
       <c r="AD201">
-        <v>-3.40874</v>
+        <v>-1.1701</v>
       </c>
       <c r="AE201">
         <v>0</v>
       </c>
       <c r="AF201">
-        <v>155.3864</v>
+        <v>566.0584</v>
       </c>
       <c r="AG201">
         <v>0</v>
@@ -23040,7 +23040,7 @@
         <v>3</v>
       </c>
       <c r="AI201">
-        <v>599.11059</v>
+        <v>2094.04806</v>
       </c>
     </row>
     <row r="202">
@@ -23059,20 +23059,20 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E202">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F202">
-        <v>4722.580000000001</v>
+        <v>9841.369999999999</v>
       </c>
       <c r="G202">
-        <v>44.04706979636251</v>
+        <v>45.83528297639469</v>
       </c>
       <c r="H202">
-        <v>34.44</v>
+        <v>40.99</v>
       </c>
       <c r="I202">
         <v>0</v>
@@ -23081,7 +23081,7 @@
         <v>0</v>
       </c>
       <c r="K202">
-        <v>0.3212187159956474</v>
+        <v>0.190907185605502</v>
       </c>
       <c r="L202">
         <v>0</v>
@@ -23093,58 +23093,58 @@
         <v>0</v>
       </c>
       <c r="O202">
-        <v>22.47953</v>
+        <v>23.44121</v>
       </c>
       <c r="P202">
-        <v>68.09502605113292</v>
+        <v>71.00814855204169</v>
       </c>
       <c r="Q202">
         <v>33.012</v>
       </c>
       <c r="R202">
-        <v>566.0236600000001</v>
+        <v>1055.07972</v>
       </c>
       <c r="S202">
-        <v>5.27925067620084</v>
+        <v>4.913937544148354</v>
       </c>
       <c r="T202">
-        <v>1034.10001</v>
+        <v>1563.62</v>
       </c>
       <c r="U202">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="V202">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="W202">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="X202">
-        <v>101</v>
+        <v>169</v>
       </c>
       <c r="Y202">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="Z202">
-        <v>98</v>
+        <v>150</v>
       </c>
       <c r="AA202">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="AB202">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="AC202">
         <v>3.74724</v>
       </c>
       <c r="AD202">
-        <v>-2.7822</v>
+        <v>-2.62863</v>
       </c>
       <c r="AE202">
         <v>0</v>
       </c>
       <c r="AF202">
-        <v>427.2645000000001</v>
+        <v>870.8505</v>
       </c>
       <c r="AG202">
         <v>0</v>
@@ -23153,7 +23153,7 @@
         <v>3</v>
       </c>
       <c r="AI202">
-        <v>1698.07098</v>
+        <v>3165.23916</v>
       </c>
     </row>
     <row r="203">
@@ -23172,20 +23172,20 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E203">
-        <v>107.2166666666667</v>
+        <v>214.7116666666667</v>
       </c>
       <c r="F203">
-        <v>3992.16</v>
+        <v>9636.360000000001</v>
       </c>
       <c r="G203">
-        <v>37.23450956008084</v>
+        <v>44.88046760384081</v>
       </c>
       <c r="H203">
-        <v>12.56</v>
+        <v>63.37</v>
       </c>
       <c r="I203">
         <v>0</v>
@@ -23194,70 +23194,70 @@
         <v>0</v>
       </c>
       <c r="K203">
-        <v>0.1171459661122338</v>
+        <v>0.2951399939453686</v>
       </c>
       <c r="L203">
         <v>0</v>
       </c>
       <c r="M203">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N203">
         <v>0</v>
       </c>
       <c r="O203">
-        <v>22.64702</v>
+        <v>28.23078</v>
       </c>
       <c r="P203">
-        <v>70.76309211348583</v>
+        <v>88.21016122984628</v>
       </c>
       <c r="Q203">
         <v>32.004</v>
       </c>
       <c r="R203">
-        <v>430.24447</v>
+        <v>949.93412</v>
       </c>
       <c r="S203">
-        <v>4.012850645111145</v>
+        <v>4.42423150426541</v>
       </c>
       <c r="T203">
-        <v>634.30999</v>
+        <v>1149.02999</v>
       </c>
       <c r="U203">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="V203">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="W203">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="X203">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="Y203">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="Z203">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="AA203">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="AB203">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="AC203">
         <v>3.87551</v>
       </c>
       <c r="AD203">
-        <v>-2.89696</v>
+        <v>-2.27001</v>
       </c>
       <c r="AE203">
         <v>0</v>
       </c>
       <c r="AF203">
-        <v>328.8747</v>
+        <v>777.8134</v>
       </c>
       <c r="AG203">
         <v>0</v>
@@ -23266,7 +23266,7 @@
         <v>3</v>
       </c>
       <c r="AI203">
-        <v>1290.73341</v>
+        <v>2849.80236</v>
       </c>
     </row>
     <row r="204">
@@ -23285,20 +23285,20 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Sesion 12</t>
+          <t>Sesión 13 Pretemporada | Sesion 12</t>
         </is>
       </c>
       <c r="E204">
-        <v>107.2166666666667</v>
+        <v>214.8018333333333</v>
       </c>
       <c r="F204">
-        <v>5479.57</v>
+        <v>10435.25</v>
       </c>
       <c r="G204">
-        <v>51.10744598165708</v>
+        <v>48.58082372046793</v>
       </c>
       <c r="H204">
-        <v>71.47</v>
+        <v>170</v>
       </c>
       <c r="I204">
         <v>0</v>
@@ -23307,70 +23307,70 @@
         <v>0</v>
       </c>
       <c r="K204">
-        <v>0.6665941240478781</v>
+        <v>0.7914271371054404</v>
       </c>
       <c r="L204">
         <v>0</v>
       </c>
       <c r="M204">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N204">
         <v>0</v>
       </c>
       <c r="O204">
-        <v>22.69942</v>
+        <v>27.8967</v>
       </c>
       <c r="P204">
-        <v>63.05394444444444</v>
+        <v>77.49083333333333</v>
       </c>
       <c r="Q204">
         <v>36</v>
       </c>
       <c r="R204">
-        <v>603.7910499999999</v>
+        <v>1134.47696</v>
       </c>
       <c r="S204">
-        <v>5.631503653039017</v>
+        <v>5.281505015087549</v>
       </c>
       <c r="T204">
-        <v>982.3600100000001</v>
+        <v>1415.07001</v>
       </c>
       <c r="U204">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="V204">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="W204">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="X204">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="Y204">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="Z204">
-        <v>104</v>
+        <v>146</v>
       </c>
       <c r="AA204">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="AB204">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="AC204">
-        <v>4.3104</v>
+        <v>4.50221</v>
       </c>
       <c r="AD204">
-        <v>-3.65595</v>
+        <v>-1.24555</v>
       </c>
       <c r="AE204">
         <v>0</v>
       </c>
       <c r="AF204">
-        <v>458.3915</v>
+        <v>856.6558</v>
       </c>
       <c r="AG204">
         <v>0</v>
@@ -23379,7 +23379,7 @@
         <v>3</v>
       </c>
       <c r="AI204">
-        <v>1811.37315</v>
+        <v>3403.43088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-26
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI254"/>
+  <dimension ref="A1:AI270"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -27240,20 +27240,20 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E239">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F239">
-        <v>3723.75</v>
+        <v>10463.67</v>
       </c>
       <c r="G239">
-        <v>39.00317367213767</v>
+        <v>54.09007025107393</v>
       </c>
       <c r="H239">
-        <v>227.84</v>
+        <v>276.78</v>
       </c>
       <c r="I239">
         <v>0</v>
@@ -27262,7 +27262,7 @@
         <v>0</v>
       </c>
       <c r="K239">
-        <v>2.386433860882134</v>
+        <v>1.430764697672255</v>
       </c>
       <c r="L239">
         <v>0</v>
@@ -27283,49 +27283,49 @@
         <v>32.364</v>
       </c>
       <c r="R239">
-        <v>411.43036</v>
+        <v>1067.75903</v>
       </c>
       <c r="S239">
-        <v>4.309389670378013</v>
+        <v>5.519589297437567</v>
       </c>
       <c r="T239">
-        <v>629.00001</v>
+        <v>1399.06003</v>
       </c>
       <c r="U239">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="V239">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="W239">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="X239">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="Y239">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="Z239">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="AA239">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="AB239">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="AC239">
         <v>3.82345</v>
       </c>
       <c r="AD239">
-        <v>-2.65168</v>
+        <v>-1.75601</v>
       </c>
       <c r="AE239">
         <v>0</v>
       </c>
       <c r="AF239">
-        <v>305.1503</v>
+        <v>835.87</v>
       </c>
       <c r="AG239">
         <v>0</v>
@@ -27334,7 +27334,7 @@
         <v>3</v>
       </c>
       <c r="AI239">
-        <v>1234.29108</v>
+        <v>3203.27709</v>
       </c>
     </row>
     <row r="240">
@@ -27353,20 +27353,20 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E240">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F240">
-        <v>3794.6</v>
+        <v>10654.48</v>
       </c>
       <c r="G240">
-        <v>39.74526829574854</v>
+        <v>55.07642841265656</v>
       </c>
       <c r="H240">
-        <v>217.57</v>
+        <v>399.7</v>
       </c>
       <c r="I240">
         <v>0</v>
@@ -27375,70 +27375,70 @@
         <v>0</v>
       </c>
       <c r="K240">
-        <v>2.27886418149634</v>
+        <v>2.066177648889371</v>
       </c>
       <c r="L240">
         <v>0</v>
       </c>
       <c r="M240">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N240">
         <v>0</v>
       </c>
       <c r="O240">
-        <v>26.81207</v>
+        <v>28.49867</v>
       </c>
       <c r="P240">
-        <v>82.7533024691358</v>
+        <v>87.95885802469137</v>
       </c>
       <c r="Q240">
         <v>32.4</v>
       </c>
       <c r="R240">
-        <v>470.69794</v>
+        <v>1245.04387</v>
       </c>
       <c r="S240">
-        <v>4.930168110355807</v>
+        <v>6.436031563874716</v>
       </c>
       <c r="T240">
-        <v>623.48999</v>
+        <v>1709.89998</v>
       </c>
       <c r="U240">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="V240">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="W240">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="X240">
-        <v>64</v>
+        <v>171</v>
       </c>
       <c r="Y240">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="Z240">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="AA240">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="AB240">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="AC240">
         <v>4.19474</v>
       </c>
       <c r="AD240">
-        <v>-2.70678</v>
+        <v>-2.6867</v>
       </c>
       <c r="AE240">
         <v>0</v>
       </c>
       <c r="AF240">
-        <v>316.0906</v>
+        <v>875.8582</v>
       </c>
       <c r="AG240">
         <v>0</v>
@@ -27447,7 +27447,7 @@
         <v>3</v>
       </c>
       <c r="AI240">
-        <v>1412.09382</v>
+        <v>3735.13161</v>
       </c>
     </row>
     <row r="241">
@@ -27466,20 +27466,20 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E241">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F241">
-        <v>4311.83</v>
+        <v>11095.95</v>
       </c>
       <c r="G241">
-        <v>45.16282090224461</v>
+        <v>57.35852860443838</v>
       </c>
       <c r="H241">
-        <v>233.75</v>
+        <v>356.89</v>
       </c>
       <c r="I241">
         <v>0</v>
@@ -27488,70 +27488,70 @@
         <v>0</v>
       </c>
       <c r="K241">
-        <v>2.448336178814952</v>
+        <v>1.844879012039349</v>
       </c>
       <c r="L241">
         <v>0</v>
       </c>
       <c r="M241">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N241">
         <v>0</v>
       </c>
       <c r="O241">
-        <v>25.96879</v>
+        <v>26.86718</v>
       </c>
       <c r="P241">
-        <v>76.41475400188324</v>
+        <v>79.05832156308851</v>
       </c>
       <c r="Q241">
         <v>33.984</v>
       </c>
       <c r="R241">
-        <v>516.91335</v>
+        <v>1302.75219</v>
       </c>
       <c r="S241">
-        <v>5.414235961999728</v>
+        <v>6.734344400849835</v>
       </c>
       <c r="T241">
-        <v>636.08001</v>
+        <v>1489.50999</v>
       </c>
       <c r="U241">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="V241">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="W241">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="X241">
-        <v>51</v>
+        <v>130</v>
       </c>
       <c r="Y241">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="Z241">
-        <v>52</v>
+        <v>111</v>
       </c>
       <c r="AA241">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="AB241">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AC241">
-        <v>3.8399</v>
+        <v>4.11278</v>
       </c>
       <c r="AD241">
-        <v>-3.02688</v>
+        <v>-1.90368</v>
       </c>
       <c r="AE241">
         <v>0</v>
       </c>
       <c r="AF241">
-        <v>404.244</v>
+        <v>1034.3792</v>
       </c>
       <c r="AG241">
         <v>0</v>
@@ -27560,7 +27560,7 @@
         <v>3</v>
       </c>
       <c r="AI241">
-        <v>1550.74005</v>
+        <v>3908.25657</v>
       </c>
     </row>
     <row r="242">
@@ -27579,20 +27579,20 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E242">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F242">
-        <v>4651.7</v>
+        <v>11865.87</v>
       </c>
       <c r="G242">
-        <v>48.72267552082788</v>
+        <v>61.33849231580415</v>
       </c>
       <c r="H242">
-        <v>254.1</v>
+        <v>516.95</v>
       </c>
       <c r="I242">
         <v>0</v>
@@ -27601,13 +27601,13 @@
         <v>0</v>
       </c>
       <c r="K242">
-        <v>2.661485446147078</v>
+        <v>2.672280549395448</v>
       </c>
       <c r="L242">
         <v>0</v>
       </c>
       <c r="M242">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="N242">
         <v>0</v>
@@ -27622,40 +27622,40 @@
         <v>35.568</v>
       </c>
       <c r="R242">
-        <v>463.09491</v>
+        <v>1082.09471</v>
       </c>
       <c r="S242">
-        <v>4.850532716055849</v>
+        <v>5.593695030731614</v>
       </c>
       <c r="T242">
-        <v>761.03</v>
+        <v>1675.04</v>
       </c>
       <c r="U242">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="V242">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="W242">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="X242">
-        <v>91</v>
+        <v>165</v>
       </c>
       <c r="Y242">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="Z242">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="AA242">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="AB242">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="AC242">
-        <v>4.09731</v>
+        <v>4.33347</v>
       </c>
       <c r="AD242">
         <v>-2.38461</v>
@@ -27664,7 +27664,7 @@
         <v>0</v>
       </c>
       <c r="AF242">
-        <v>443.46</v>
+        <v>1101.7896</v>
       </c>
       <c r="AG242">
         <v>0</v>
@@ -27673,7 +27673,7 @@
         <v>3</v>
       </c>
       <c r="AI242">
-        <v>1389.28473</v>
+        <v>3246.28413</v>
       </c>
     </row>
     <row r="243">
@@ -27692,20 +27692,20 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E243">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F243">
-        <v>4366.24</v>
+        <v>10937.15</v>
       </c>
       <c r="G243">
-        <v>45.73272024551444</v>
+        <v>56.53764041168473</v>
       </c>
       <c r="H243">
-        <v>153.98</v>
+        <v>400.26</v>
       </c>
       <c r="I243">
         <v>0</v>
@@ -27714,58 +27714,58 @@
         <v>0</v>
       </c>
       <c r="K243">
-        <v>1.612811999203964</v>
+        <v>2.069072468712684</v>
       </c>
       <c r="L243">
         <v>0</v>
       </c>
       <c r="M243">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N243">
         <v>0</v>
       </c>
       <c r="O243">
-        <v>24.75218</v>
+        <v>28.36836</v>
       </c>
       <c r="P243">
-        <v>68.75605555555555</v>
+        <v>78.801</v>
       </c>
       <c r="Q243">
         <v>36</v>
       </c>
       <c r="R243">
-        <v>418.41357</v>
+        <v>1021.10342</v>
       </c>
       <c r="S243">
-        <v>4.38253296743582</v>
+        <v>5.278411467621957</v>
       </c>
       <c r="T243">
-        <v>638.70998</v>
+        <v>1591.66</v>
       </c>
       <c r="U243">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="V243">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="W243">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="X243">
-        <v>70</v>
+        <v>146</v>
       </c>
       <c r="Y243">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="Z243">
-        <v>51</v>
+        <v>95</v>
       </c>
       <c r="AA243">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="AB243">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="AC243">
         <v>4.10414</v>
@@ -27777,7 +27777,7 @@
         <v>0</v>
       </c>
       <c r="AF243">
-        <v>355.9437</v>
+        <v>883.9285</v>
       </c>
       <c r="AG243">
         <v>0</v>
@@ -27786,7 +27786,7 @@
         <v>3</v>
       </c>
       <c r="AI243">
-        <v>1255.24071</v>
+        <v>3063.31026</v>
       </c>
     </row>
     <row r="244">
@@ -27805,80 +27805,80 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E244">
-        <v>95.473</v>
+        <v>164.1861666666667</v>
       </c>
       <c r="F244">
-        <v>3376.9</v>
+        <v>8594.390000000001</v>
       </c>
       <c r="G244">
-        <v>35.37020937856776</v>
+        <v>52.34539653665504</v>
       </c>
       <c r="H244">
-        <v>230.91</v>
+        <v>473.04</v>
       </c>
       <c r="I244">
-        <v>0</v>
+        <v>0.78</v>
       </c>
       <c r="J244">
         <v>0</v>
       </c>
       <c r="K244">
-        <v>2.418589548877693</v>
+        <v>2.881119704563011</v>
       </c>
       <c r="L244">
         <v>0</v>
       </c>
       <c r="M244">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N244">
         <v>0</v>
       </c>
       <c r="O244">
-        <v>26.83137</v>
+        <v>28.80893</v>
       </c>
       <c r="P244">
-        <v>83.8375515560555</v>
+        <v>90.01665416822898</v>
       </c>
       <c r="Q244">
         <v>32.004</v>
       </c>
       <c r="R244">
-        <v>372.85363</v>
+        <v>921.2788399999999</v>
       </c>
       <c r="S244">
-        <v>3.905330617033088</v>
+        <v>5.611184295875515</v>
       </c>
       <c r="T244">
-        <v>550.51001</v>
+        <v>1400.84002</v>
       </c>
       <c r="U244">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="V244">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="W244">
-        <v>26</v>
+        <v>69</v>
       </c>
       <c r="X244">
-        <v>51</v>
+        <v>123</v>
       </c>
       <c r="Y244">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="Z244">
-        <v>45</v>
+        <v>108</v>
       </c>
       <c r="AA244">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="AB244">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="AC244">
         <v>3.87615</v>
@@ -27890,7 +27890,7 @@
         <v>0</v>
       </c>
       <c r="AF244">
-        <v>241.3482</v>
+        <v>610.2534000000001</v>
       </c>
       <c r="AG244">
         <v>0</v>
@@ -27899,7 +27899,7 @@
         <v>3</v>
       </c>
       <c r="AI244">
-        <v>1118.56089</v>
+        <v>2763.83652</v>
       </c>
     </row>
     <row r="245">
@@ -27918,20 +27918,20 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E245">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F245">
-        <v>4522.5</v>
+        <v>10954.77</v>
       </c>
       <c r="G245">
-        <v>47.36941334199198</v>
+        <v>56.62872384969682</v>
       </c>
       <c r="H245">
-        <v>274.47</v>
+        <v>481.67</v>
       </c>
       <c r="I245">
         <v>0</v>
@@ -27940,13 +27940,13 @@
         <v>0</v>
       </c>
       <c r="K245">
-        <v>2.87484419678862</v>
+        <v>2.489906900526754</v>
       </c>
       <c r="L245">
         <v>0</v>
       </c>
       <c r="M245">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N245">
         <v>0</v>
@@ -27961,49 +27961,49 @@
         <v>33.84</v>
       </c>
       <c r="R245">
-        <v>446.78263</v>
+        <v>1043.98915</v>
       </c>
       <c r="S245">
-        <v>4.679675196128748</v>
+        <v>5.396715154898706</v>
       </c>
       <c r="T245">
-        <v>782.79999</v>
+        <v>1512.10998</v>
       </c>
       <c r="U245">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="V245">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="W245">
+        <v>69</v>
+      </c>
+      <c r="X245">
+        <v>149</v>
+      </c>
+      <c r="Y245">
         <v>40</v>
       </c>
-      <c r="X245">
-        <v>78</v>
-      </c>
-      <c r="Y245">
-        <v>21</v>
-      </c>
       <c r="Z245">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="AA245">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="AB245">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="AC245">
-        <v>3.94111</v>
+        <v>4.23566</v>
       </c>
       <c r="AD245">
-        <v>-3.05641</v>
+        <v>-2.00598</v>
       </c>
       <c r="AE245">
         <v>0</v>
       </c>
       <c r="AF245">
-        <v>379.5036</v>
+        <v>892.4446999999999</v>
       </c>
       <c r="AG245">
         <v>0</v>
@@ -28012,7 +28012,7 @@
         <v>3</v>
       </c>
       <c r="AI245">
-        <v>1340.34789</v>
+        <v>3131.96745</v>
       </c>
     </row>
     <row r="246">
@@ -28031,20 +28031,20 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E246">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F246">
-        <v>3767.91</v>
+        <v>9852.299999999999</v>
       </c>
       <c r="G246">
-        <v>39.46571281933112</v>
+        <v>50.92970240218352</v>
       </c>
       <c r="H246">
-        <v>276.6</v>
+        <v>402.09</v>
       </c>
       <c r="I246">
         <v>0</v>
@@ -28053,13 +28053,13 @@
         <v>0</v>
       </c>
       <c r="K246">
-        <v>2.897154169241566</v>
+        <v>2.07853232634958</v>
       </c>
       <c r="L246">
         <v>0</v>
       </c>
       <c r="M246">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N246">
         <v>0</v>
@@ -28074,40 +28074,40 @@
         <v>33.696</v>
       </c>
       <c r="R246">
-        <v>386.3225</v>
+        <v>975.53298</v>
       </c>
       <c r="S246">
-        <v>4.046405790118672</v>
+        <v>5.042843229998604</v>
       </c>
       <c r="T246">
-        <v>711.1200100000001</v>
+        <v>1503.77001</v>
       </c>
       <c r="U246">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="V246">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="W246">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="X246">
-        <v>78</v>
+        <v>173</v>
       </c>
       <c r="Y246">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="Z246">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="AA246">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="AB246">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="AC246">
-        <v>3.83384</v>
+        <v>3.88935</v>
       </c>
       <c r="AD246">
         <v>-1.29731</v>
@@ -28116,7 +28116,7 @@
         <v>0</v>
       </c>
       <c r="AF246">
-        <v>367.4944</v>
+        <v>927.2848</v>
       </c>
       <c r="AG246">
         <v>0</v>
@@ -28125,7 +28125,7 @@
         <v>3</v>
       </c>
       <c r="AI246">
-        <v>1158.9675</v>
+        <v>2926.59894</v>
       </c>
     </row>
     <row r="247">
@@ -28144,83 +28144,83 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E247">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F247">
-        <v>4018</v>
+        <v>10445.02</v>
       </c>
       <c r="G247">
-        <v>42.08519686194003</v>
+        <v>53.99366241231539</v>
       </c>
       <c r="H247">
-        <v>270.75</v>
+        <v>508.25</v>
       </c>
       <c r="I247">
-        <v>0</v>
+        <v>10.42</v>
       </c>
       <c r="J247">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K247">
-        <v>2.835880301236999</v>
+        <v>2.627307455711841</v>
       </c>
       <c r="L247">
-        <v>0</v>
+        <v>18.82</v>
       </c>
       <c r="M247">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N247">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O247">
-        <v>28.48308</v>
+        <v>31.6363</v>
       </c>
       <c r="P247">
-        <v>81.3988340192044</v>
+        <v>90.41009373571103</v>
       </c>
       <c r="Q247">
         <v>34.992</v>
       </c>
       <c r="R247">
-        <v>370.35445</v>
+        <v>965.5452300000001</v>
       </c>
       <c r="S247">
-        <v>3.879153792171609</v>
+        <v>4.991213343051657</v>
       </c>
       <c r="T247">
-        <v>615.25001</v>
+        <v>1438.51001</v>
       </c>
       <c r="U247">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="V247">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="W247">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="X247">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="Y247">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="Z247">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="AA247">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="AB247">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="AC247">
-        <v>4.06416</v>
+        <v>4.96087</v>
       </c>
       <c r="AD247">
         <v>-1.93607</v>
@@ -28229,7 +28229,7 @@
         <v>0</v>
       </c>
       <c r="AF247">
-        <v>330.14775</v>
+        <v>836.67399</v>
       </c>
       <c r="AG247">
         <v>0</v>
@@ -28238,7 +28238,7 @@
         <v>3</v>
       </c>
       <c r="AI247">
-        <v>1111.06335</v>
+        <v>2896.63569</v>
       </c>
     </row>
     <row r="248">
@@ -28257,92 +28257,92 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E248">
-        <v>62.47116666666667</v>
+        <v>160.4471666666667</v>
       </c>
       <c r="F248">
-        <v>3270.62</v>
+        <v>9967.84</v>
       </c>
       <c r="G248">
-        <v>52.35407267886252</v>
+        <v>62.12537252657417</v>
       </c>
       <c r="H248">
-        <v>225.95</v>
+        <v>355.8</v>
       </c>
       <c r="I248">
-        <v>0</v>
+        <v>2.54</v>
       </c>
       <c r="J248">
         <v>0</v>
       </c>
       <c r="K248">
-        <v>3.616868582039181</v>
+        <v>2.217552403023633</v>
       </c>
       <c r="L248">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="M248">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N248">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O248">
-        <v>27.59293</v>
+        <v>31.41848</v>
       </c>
       <c r="P248">
-        <v>79.01755441008018</v>
+        <v>89.97273768613974</v>
       </c>
       <c r="Q248">
         <v>34.92</v>
       </c>
       <c r="R248">
-        <v>302.41782</v>
+        <v>846.21602</v>
       </c>
       <c r="S248">
-        <v>4.840918397020492</v>
+        <v>5.274110086082334</v>
       </c>
       <c r="T248">
-        <v>546.25001</v>
+        <v>1271.98002</v>
       </c>
       <c r="U248">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="V248">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="W248">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="X248">
-        <v>65</v>
+        <v>140</v>
       </c>
       <c r="Y248">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Z248">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="AA248">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AB248">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="AC248">
         <v>4.12922</v>
       </c>
       <c r="AD248">
-        <v>-2.87777</v>
+        <v>-2.54951</v>
       </c>
       <c r="AE248">
         <v>0</v>
       </c>
       <c r="AF248">
-        <v>314.5504</v>
+        <v>922.9656</v>
       </c>
       <c r="AG248">
         <v>0</v>
@@ -28351,7 +28351,7 @@
         <v>3</v>
       </c>
       <c r="AI248">
-        <v>907.25346</v>
+        <v>2538.64806</v>
       </c>
     </row>
     <row r="249">
@@ -28370,20 +28370,20 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E249">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F249">
-        <v>4344.08</v>
+        <v>11789.95</v>
       </c>
       <c r="G249">
-        <v>45.50061273868005</v>
+        <v>60.94603745690078</v>
       </c>
       <c r="H249">
-        <v>256.16</v>
+        <v>495.97</v>
       </c>
       <c r="I249">
         <v>0</v>
@@ -28392,61 +28392,61 @@
         <v>0</v>
       </c>
       <c r="K249">
-        <v>2.683062227017063</v>
+        <v>2.563828192443486</v>
       </c>
       <c r="L249">
-        <v>0</v>
+        <v>11.6</v>
       </c>
       <c r="M249">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N249">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O249">
-        <v>26.65835</v>
+        <v>30.47778</v>
       </c>
       <c r="P249">
-        <v>76.18412780064014</v>
+        <v>87.09927983539096</v>
       </c>
       <c r="Q249">
         <v>34.992</v>
       </c>
       <c r="R249">
-        <v>363.86491</v>
+        <v>981.08146</v>
       </c>
       <c r="S249">
-        <v>3.811181276381804</v>
+        <v>5.071525104807985</v>
       </c>
       <c r="T249">
-        <v>705.18999</v>
+        <v>1867.54003</v>
       </c>
       <c r="U249">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="V249">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="W249">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="X249">
-        <v>66</v>
+        <v>183</v>
       </c>
       <c r="Y249">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="Z249">
-        <v>62</v>
+        <v>154</v>
       </c>
       <c r="AA249">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="AB249">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="AC249">
-        <v>3.74742</v>
+        <v>4.44991</v>
       </c>
       <c r="AD249">
         <v>-2.86719</v>
@@ -28455,7 +28455,7 @@
         <v>0</v>
       </c>
       <c r="AF249">
-        <v>369.19503</v>
+        <v>995.8168899999999</v>
       </c>
       <c r="AG249">
         <v>0</v>
@@ -28464,7 +28464,7 @@
         <v>3</v>
       </c>
       <c r="AI249">
-        <v>1091.59473</v>
+        <v>2943.24438</v>
       </c>
     </row>
     <row r="250">
@@ -28483,20 +28483,20 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E250">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F250">
-        <v>3929.75</v>
+        <v>10364.86</v>
       </c>
       <c r="G250">
-        <v>41.16085175913609</v>
+        <v>53.57928963189264</v>
       </c>
       <c r="H250">
-        <v>162.93</v>
+        <v>276.83</v>
       </c>
       <c r="I250">
         <v>0</v>
@@ -28505,13 +28505,13 @@
         <v>0</v>
       </c>
       <c r="K250">
-        <v>1.706555780168215</v>
+        <v>1.431023163727907</v>
       </c>
       <c r="L250">
         <v>0</v>
       </c>
       <c r="M250">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N250">
         <v>0</v>
@@ -28526,49 +28526,49 @@
         <v>33.984</v>
       </c>
       <c r="R250">
-        <v>393.15299</v>
+        <v>1036.23388</v>
       </c>
       <c r="S250">
-        <v>4.117949472625768</v>
+        <v>5.35662567395024</v>
       </c>
       <c r="T250">
-        <v>568.54</v>
+        <v>1269.53</v>
       </c>
       <c r="U250">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V250">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="W250">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="X250">
-        <v>57</v>
+        <v>121</v>
       </c>
       <c r="Y250">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Z250">
-        <v>53</v>
+        <v>121</v>
       </c>
       <c r="AA250">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="AB250">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="AC250">
         <v>3.5879</v>
       </c>
       <c r="AD250">
-        <v>-2.37494</v>
+        <v>-2.18503</v>
       </c>
       <c r="AE250">
         <v>0</v>
       </c>
       <c r="AF250">
-        <v>369.5488</v>
+        <v>963.3439999999999</v>
       </c>
       <c r="AG250">
         <v>0</v>
@@ -28577,7 +28577,7 @@
         <v>3</v>
       </c>
       <c r="AI250">
-        <v>1179.45897</v>
+        <v>3108.70164</v>
       </c>
     </row>
     <row r="251">
@@ -28596,20 +28596,20 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E251">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F251">
-        <v>3752.03</v>
+        <v>10479.97</v>
       </c>
       <c r="G251">
-        <v>39.29938307165377</v>
+        <v>54.17433018521677</v>
       </c>
       <c r="H251">
-        <v>371.34</v>
+        <v>427.2400000000001</v>
       </c>
       <c r="I251">
         <v>0</v>
@@ -28618,7 +28618,7 @@
         <v>0</v>
       </c>
       <c r="K251">
-        <v>3.889476605951421</v>
+        <v>2.208540752342995</v>
       </c>
       <c r="L251">
         <v>0</v>
@@ -28639,37 +28639,37 @@
         <v>34.992</v>
       </c>
       <c r="R251">
-        <v>387.32896</v>
+        <v>974.56976</v>
       </c>
       <c r="S251">
-        <v>4.05694761869848</v>
+        <v>5.037864036516084</v>
       </c>
       <c r="T251">
-        <v>768.2800100000001</v>
+        <v>1552.66001</v>
       </c>
       <c r="U251">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="V251">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="W251">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="X251">
-        <v>69</v>
+        <v>150</v>
       </c>
       <c r="Y251">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="Z251">
-        <v>72</v>
+        <v>134</v>
       </c>
       <c r="AA251">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AB251">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AC251">
         <v>4.2024</v>
@@ -28681,7 +28681,7 @@
         <v>0</v>
       </c>
       <c r="AF251">
-        <v>369.3928</v>
+        <v>986.0328</v>
       </c>
       <c r="AG251">
         <v>0</v>
@@ -28690,7 +28690,7 @@
         <v>3</v>
       </c>
       <c r="AI251">
-        <v>1161.98688</v>
+        <v>2923.70928</v>
       </c>
     </row>
     <row r="252">
@@ -28709,20 +28709,20 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E252">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F252">
-        <v>4277.02</v>
+        <v>10871.58</v>
       </c>
       <c r="G252">
-        <v>44.79821520220377</v>
+        <v>56.1986880263015</v>
       </c>
       <c r="H252">
-        <v>357.07</v>
+        <v>428.52</v>
       </c>
       <c r="I252">
         <v>0</v>
@@ -28731,13 +28731,13 @@
         <v>0</v>
       </c>
       <c r="K252">
-        <v>3.740010264682161</v>
+        <v>2.215157483367709</v>
       </c>
       <c r="L252">
         <v>0</v>
       </c>
       <c r="M252">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N252">
         <v>0</v>
@@ -28752,49 +28752,49 @@
         <v>33.012</v>
       </c>
       <c r="R252">
-        <v>445.1698</v>
+        <v>1090.1221</v>
       </c>
       <c r="S252">
-        <v>4.662782147832371</v>
+        <v>5.635191187341366</v>
       </c>
       <c r="T252">
-        <v>797.0999999999999</v>
+        <v>1554.22998</v>
       </c>
       <c r="U252">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="V252">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="W252">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="X252">
-        <v>90</v>
+        <v>164</v>
       </c>
       <c r="Y252">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="Z252">
-        <v>68</v>
+        <v>136</v>
       </c>
       <c r="AA252">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="AB252">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="AC252">
         <v>3.99062</v>
       </c>
       <c r="AD252">
-        <v>-2.95586</v>
+        <v>-2.40647</v>
       </c>
       <c r="AE252">
         <v>0</v>
       </c>
       <c r="AF252">
-        <v>385.77525</v>
+        <v>952.36725</v>
       </c>
       <c r="AG252">
         <v>0</v>
@@ -28803,7 +28803,7 @@
         <v>3</v>
       </c>
       <c r="AI252">
-        <v>1335.5094</v>
+        <v>3270.3663</v>
       </c>
     </row>
     <row r="253">
@@ -28822,20 +28822,20 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E253">
-        <v>95.473</v>
+        <v>193.449</v>
       </c>
       <c r="F253">
-        <v>3620</v>
+        <v>9809.210000000001</v>
       </c>
       <c r="G253">
-        <v>37.91647900453531</v>
+        <v>50.70695635542184</v>
       </c>
       <c r="H253">
-        <v>208.83</v>
+        <v>342.78</v>
       </c>
       <c r="I253">
         <v>0</v>
@@ -28844,61 +28844,61 @@
         <v>0</v>
       </c>
       <c r="K253">
-        <v>2.187319975280969</v>
+        <v>1.771939891134097</v>
       </c>
       <c r="L253">
         <v>0</v>
       </c>
       <c r="M253">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N253">
         <v>0</v>
       </c>
       <c r="O253">
-        <v>27.66138</v>
+        <v>27.83737</v>
       </c>
       <c r="P253">
-        <v>86.43100862392203</v>
+        <v>86.98090863642045</v>
       </c>
       <c r="Q253">
         <v>32.004</v>
       </c>
       <c r="R253">
-        <v>377.17898</v>
+        <v>955.33079</v>
       </c>
       <c r="S253">
-        <v>3.950635048652498</v>
+        <v>4.93841162270159</v>
       </c>
       <c r="T253">
-        <v>575.8100000000001</v>
+        <v>1305.80998</v>
       </c>
       <c r="U253">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="V253">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="W253">
+        <v>47</v>
+      </c>
+      <c r="X253">
+        <v>135</v>
+      </c>
+      <c r="Y253">
+        <v>29</v>
+      </c>
+      <c r="Z253">
+        <v>96</v>
+      </c>
+      <c r="AA253">
+        <v>18</v>
+      </c>
+      <c r="AB253">
         <v>23</v>
       </c>
-      <c r="X253">
-        <v>62</v>
-      </c>
-      <c r="Y253">
-        <v>13</v>
-      </c>
-      <c r="Z253">
-        <v>52</v>
-      </c>
-      <c r="AA253">
-        <v>10</v>
-      </c>
-      <c r="AB253">
-        <v>12</v>
-      </c>
       <c r="AC253">
-        <v>3.87193</v>
+        <v>4.289</v>
       </c>
       <c r="AD253">
         <v>-1.51904</v>
@@ -28907,7 +28907,7 @@
         <v>0</v>
       </c>
       <c r="AF253">
-        <v>300.1733</v>
+        <v>794.7975</v>
       </c>
       <c r="AG253">
         <v>0</v>
@@ -28916,7 +28916,7 @@
         <v>3</v>
       </c>
       <c r="AI253">
-        <v>1131.53694</v>
+        <v>2865.99237</v>
       </c>
     </row>
     <row r="254">
@@ -28935,20 +28935,20 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Sesión 17 Pretemporada</t>
+          <t>Sesión 18 pretemporada  | Sesión 17 Pretemporada</t>
         </is>
       </c>
       <c r="E254">
-        <v>62.47116666666667</v>
+        <v>134.957</v>
       </c>
       <c r="F254">
-        <v>3454.25</v>
+        <v>7720.4</v>
       </c>
       <c r="G254">
-        <v>55.29350873869812</v>
+        <v>57.20636943619078</v>
       </c>
       <c r="H254">
-        <v>272.38</v>
+        <v>397.6300000000001</v>
       </c>
       <c r="I254">
         <v>0</v>
@@ -28957,70 +28957,70 @@
         <v>0</v>
       </c>
       <c r="K254">
-        <v>4.360091455524815</v>
+        <v>2.94634587312996</v>
       </c>
       <c r="L254">
         <v>0</v>
       </c>
       <c r="M254">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N254">
         <v>0</v>
       </c>
       <c r="O254">
-        <v>28.48521</v>
+        <v>29.07256</v>
       </c>
       <c r="P254">
-        <v>79.12558333333332</v>
+        <v>80.75711111111112</v>
       </c>
       <c r="Q254">
         <v>36</v>
       </c>
       <c r="R254">
-        <v>390.02639</v>
+        <v>853.2602400000001</v>
       </c>
       <c r="S254">
-        <v>6.243302483545742</v>
+        <v>6.322460042828458</v>
       </c>
       <c r="T254">
-        <v>672.0700000000001</v>
+        <v>1224.52</v>
       </c>
       <c r="U254">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="V254">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="W254">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="X254">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="Y254">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="Z254">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="AA254">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="AB254">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="AC254">
         <v>4.23547</v>
       </c>
       <c r="AD254">
-        <v>-3.30771</v>
+        <v>-2.82998</v>
       </c>
       <c r="AE254">
         <v>0</v>
       </c>
       <c r="AF254">
-        <v>295.2901000000001</v>
+        <v>640.7737000000001</v>
       </c>
       <c r="AG254">
         <v>0</v>
@@ -29029,7 +29029,1815 @@
         <v>3</v>
       </c>
       <c r="AI254">
-        <v>1170.07917</v>
+        <v>2559.78072</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B255" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E255">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F255">
+        <v>3129.73</v>
+      </c>
+      <c r="G255">
+        <v>24.86198290756714</v>
+      </c>
+      <c r="H255">
+        <v>120.42</v>
+      </c>
+      <c r="I255">
+        <v>0</v>
+      </c>
+      <c r="J255">
+        <v>0</v>
+      </c>
+      <c r="K255">
+        <v>0.9565936939382104</v>
+      </c>
+      <c r="L255">
+        <v>0</v>
+      </c>
+      <c r="M255">
+        <v>3</v>
+      </c>
+      <c r="N255">
+        <v>0</v>
+      </c>
+      <c r="O255">
+        <v>25.86529</v>
+      </c>
+      <c r="P255">
+        <v>79.91994191076506</v>
+      </c>
+      <c r="Q255">
+        <v>32.364</v>
+      </c>
+      <c r="R255">
+        <v>340.78178</v>
+      </c>
+      <c r="S255">
+        <v>2.707105977055627</v>
+      </c>
+      <c r="T255">
+        <v>323.87</v>
+      </c>
+      <c r="U255">
+        <v>13</v>
+      </c>
+      <c r="V255">
+        <v>3</v>
+      </c>
+      <c r="W255">
+        <v>16</v>
+      </c>
+      <c r="X255">
+        <v>31</v>
+      </c>
+      <c r="Y255">
+        <v>13</v>
+      </c>
+      <c r="Z255">
+        <v>10</v>
+      </c>
+      <c r="AA255">
+        <v>3</v>
+      </c>
+      <c r="AB255">
+        <v>4</v>
+      </c>
+      <c r="AC255">
+        <v>4.14879</v>
+      </c>
+      <c r="AD255">
+        <v>-0.82957</v>
+      </c>
+      <c r="AE255">
+        <v>0</v>
+      </c>
+      <c r="AF255">
+        <v>238.9541</v>
+      </c>
+      <c r="AG255">
+        <v>0</v>
+      </c>
+      <c r="AH255">
+        <v>3</v>
+      </c>
+      <c r="AI255">
+        <v>1022.34534</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B256" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E256">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F256">
+        <v>3304.06</v>
+      </c>
+      <c r="G256">
+        <v>26.24682744057037</v>
+      </c>
+      <c r="H256">
+        <v>160.22</v>
+      </c>
+      <c r="I256">
+        <v>0</v>
+      </c>
+      <c r="J256">
+        <v>0</v>
+      </c>
+      <c r="K256">
+        <v>1.272757362919615</v>
+      </c>
+      <c r="L256">
+        <v>0</v>
+      </c>
+      <c r="M256">
+        <v>2</v>
+      </c>
+      <c r="N256">
+        <v>0</v>
+      </c>
+      <c r="O256">
+        <v>26.93891</v>
+      </c>
+      <c r="P256">
+        <v>83.14478395061728</v>
+      </c>
+      <c r="Q256">
+        <v>32.4</v>
+      </c>
+      <c r="R256">
+        <v>397.55399</v>
+      </c>
+      <c r="S256">
+        <v>3.158093670768762</v>
+      </c>
+      <c r="T256">
+        <v>490.43999</v>
+      </c>
+      <c r="U256">
+        <v>17</v>
+      </c>
+      <c r="V256">
+        <v>7</v>
+      </c>
+      <c r="W256">
+        <v>24</v>
+      </c>
+      <c r="X256">
+        <v>42</v>
+      </c>
+      <c r="Y256">
+        <v>17</v>
+      </c>
+      <c r="Z256">
+        <v>24</v>
+      </c>
+      <c r="AA256">
+        <v>7</v>
+      </c>
+      <c r="AB256">
+        <v>1</v>
+      </c>
+      <c r="AC256">
+        <v>4.24135</v>
+      </c>
+      <c r="AD256">
+        <v>-1.67768</v>
+      </c>
+      <c r="AE256">
+        <v>0</v>
+      </c>
+      <c r="AF256">
+        <v>265.1873</v>
+      </c>
+      <c r="AG256">
+        <v>0</v>
+      </c>
+      <c r="AH256">
+        <v>3</v>
+      </c>
+      <c r="AI256">
+        <v>1192.66197</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B257" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E257">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F257">
+        <v>3982.18</v>
+      </c>
+      <c r="G257">
+        <v>31.63368440563746</v>
+      </c>
+      <c r="H257">
+        <v>106.95</v>
+      </c>
+      <c r="I257">
+        <v>0</v>
+      </c>
+      <c r="J257">
+        <v>0</v>
+      </c>
+      <c r="K257">
+        <v>0.8495905627527952</v>
+      </c>
+      <c r="L257">
+        <v>0</v>
+      </c>
+      <c r="M257">
+        <v>4</v>
+      </c>
+      <c r="N257">
+        <v>0</v>
+      </c>
+      <c r="O257">
+        <v>26.69925</v>
+      </c>
+      <c r="P257">
+        <v>78.564177259887</v>
+      </c>
+      <c r="Q257">
+        <v>33.984</v>
+      </c>
+      <c r="R257">
+        <v>545.07885</v>
+      </c>
+      <c r="S257">
+        <v>4.330003243722734</v>
+      </c>
+      <c r="T257">
+        <v>544.55002</v>
+      </c>
+      <c r="U257">
+        <v>24</v>
+      </c>
+      <c r="V257">
+        <v>11</v>
+      </c>
+      <c r="W257">
+        <v>35</v>
+      </c>
+      <c r="X257">
+        <v>42</v>
+      </c>
+      <c r="Y257">
+        <v>24</v>
+      </c>
+      <c r="Z257">
+        <v>36</v>
+      </c>
+      <c r="AA257">
+        <v>11</v>
+      </c>
+      <c r="AB257">
+        <v>21</v>
+      </c>
+      <c r="AC257">
+        <v>4.66577</v>
+      </c>
+      <c r="AD257">
+        <v>-1.70509</v>
+      </c>
+      <c r="AE257">
+        <v>0</v>
+      </c>
+      <c r="AF257">
+        <v>369.6376</v>
+      </c>
+      <c r="AG257">
+        <v>0</v>
+      </c>
+      <c r="AH257">
+        <v>3</v>
+      </c>
+      <c r="AI257">
+        <v>1635.23655</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B258" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E258">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F258">
+        <v>4154.79</v>
+      </c>
+      <c r="G258">
+        <v>33.00486558410179</v>
+      </c>
+      <c r="H258">
+        <v>214.32</v>
+      </c>
+      <c r="I258">
+        <v>0</v>
+      </c>
+      <c r="J258">
+        <v>0</v>
+      </c>
+      <c r="K258">
+        <v>1.70251752603253</v>
+      </c>
+      <c r="L258">
+        <v>0</v>
+      </c>
+      <c r="M258">
+        <v>5</v>
+      </c>
+      <c r="N258">
+        <v>0</v>
+      </c>
+      <c r="O258">
+        <v>28.56173</v>
+      </c>
+      <c r="P258">
+        <v>80.30176000899687</v>
+      </c>
+      <c r="Q258">
+        <v>35.568</v>
+      </c>
+      <c r="R258">
+        <v>454.78602</v>
+      </c>
+      <c r="S258">
+        <v>3.612734087554034</v>
+      </c>
+      <c r="T258">
+        <v>638.68001</v>
+      </c>
+      <c r="U258">
+        <v>30</v>
+      </c>
+      <c r="V258">
+        <v>15</v>
+      </c>
+      <c r="W258">
+        <v>45</v>
+      </c>
+      <c r="X258">
+        <v>68</v>
+      </c>
+      <c r="Y258">
+        <v>30</v>
+      </c>
+      <c r="Z258">
+        <v>48</v>
+      </c>
+      <c r="AA258">
+        <v>15</v>
+      </c>
+      <c r="AB258">
+        <v>12</v>
+      </c>
+      <c r="AC258">
+        <v>5.22356</v>
+      </c>
+      <c r="AD258">
+        <v>-2.10787</v>
+      </c>
+      <c r="AE258">
+        <v>0</v>
+      </c>
+      <c r="AF258">
+        <v>398.912</v>
+      </c>
+      <c r="AG258">
+        <v>0</v>
+      </c>
+      <c r="AH258">
+        <v>3</v>
+      </c>
+      <c r="AI258">
+        <v>1364.35806</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B259" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E259">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F259">
+        <v>3652.16</v>
+      </c>
+      <c r="G259">
+        <v>29.01206797254089</v>
+      </c>
+      <c r="H259">
+        <v>163.04</v>
+      </c>
+      <c r="I259">
+        <v>0</v>
+      </c>
+      <c r="J259">
+        <v>0</v>
+      </c>
+      <c r="K259">
+        <v>1.29515890931478</v>
+      </c>
+      <c r="L259">
+        <v>0</v>
+      </c>
+      <c r="M259">
+        <v>3</v>
+      </c>
+      <c r="N259">
+        <v>0</v>
+      </c>
+      <c r="O259">
+        <v>27.86056</v>
+      </c>
+      <c r="P259">
+        <v>77.39044444444444</v>
+      </c>
+      <c r="Q259">
+        <v>36</v>
+      </c>
+      <c r="R259">
+        <v>395.84695</v>
+      </c>
+      <c r="S259">
+        <v>3.144533268017556</v>
+      </c>
+      <c r="T259">
+        <v>549.24999</v>
+      </c>
+      <c r="U259">
+        <v>24</v>
+      </c>
+      <c r="V259">
+        <v>14</v>
+      </c>
+      <c r="W259">
+        <v>38</v>
+      </c>
+      <c r="X259">
+        <v>59</v>
+      </c>
+      <c r="Y259">
+        <v>24</v>
+      </c>
+      <c r="Z259">
+        <v>38</v>
+      </c>
+      <c r="AA259">
+        <v>14</v>
+      </c>
+      <c r="AB259">
+        <v>6</v>
+      </c>
+      <c r="AC259">
+        <v>4.74092</v>
+      </c>
+      <c r="AD259">
+        <v>-0.38961</v>
+      </c>
+      <c r="AE259">
+        <v>0</v>
+      </c>
+      <c r="AF259">
+        <v>303.4038</v>
+      </c>
+      <c r="AG259">
+        <v>0</v>
+      </c>
+      <c r="AH259">
+        <v>3</v>
+      </c>
+      <c r="AI259">
+        <v>1187.54085</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B260" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E260">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F260">
+        <v>3669.98</v>
+      </c>
+      <c r="G260">
+        <v>29.15362668061247</v>
+      </c>
+      <c r="H260">
+        <v>230.79</v>
+      </c>
+      <c r="I260">
+        <v>0</v>
+      </c>
+      <c r="J260">
+        <v>0</v>
+      </c>
+      <c r="K260">
+        <v>1.833352089553227</v>
+      </c>
+      <c r="L260">
+        <v>0</v>
+      </c>
+      <c r="M260">
+        <v>2</v>
+      </c>
+      <c r="N260">
+        <v>0</v>
+      </c>
+      <c r="O260">
+        <v>26.24445</v>
+      </c>
+      <c r="P260">
+        <v>82.00365579302587</v>
+      </c>
+      <c r="Q260">
+        <v>32.004</v>
+      </c>
+      <c r="R260">
+        <v>439.91511</v>
+      </c>
+      <c r="S260">
+        <v>3.494602392411013</v>
+      </c>
+      <c r="T260">
+        <v>509.79999</v>
+      </c>
+      <c r="U260">
+        <v>22</v>
+      </c>
+      <c r="V260">
+        <v>2</v>
+      </c>
+      <c r="W260">
+        <v>24</v>
+      </c>
+      <c r="X260">
+        <v>41</v>
+      </c>
+      <c r="Y260">
+        <v>22</v>
+      </c>
+      <c r="Z260">
+        <v>28</v>
+      </c>
+      <c r="AA260">
+        <v>2</v>
+      </c>
+      <c r="AB260">
+        <v>7</v>
+      </c>
+      <c r="AC260">
+        <v>4.19666</v>
+      </c>
+      <c r="AD260">
+        <v>-2.31307</v>
+      </c>
+      <c r="AE260">
+        <v>0</v>
+      </c>
+      <c r="AF260">
+        <v>253.188</v>
+      </c>
+      <c r="AG260">
+        <v>0</v>
+      </c>
+      <c r="AH260">
+        <v>3</v>
+      </c>
+      <c r="AI260">
+        <v>1319.74533</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B261" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E261">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F261">
+        <v>3776.98</v>
+      </c>
+      <c r="G261">
+        <v>30.00361443390418</v>
+      </c>
+      <c r="H261">
+        <v>250.01</v>
+      </c>
+      <c r="I261">
+        <v>0</v>
+      </c>
+      <c r="J261">
+        <v>0</v>
+      </c>
+      <c r="K261">
+        <v>1.986032132714599</v>
+      </c>
+      <c r="L261">
+        <v>0</v>
+      </c>
+      <c r="M261">
+        <v>2</v>
+      </c>
+      <c r="N261">
+        <v>0</v>
+      </c>
+      <c r="O261">
+        <v>29.20258</v>
+      </c>
+      <c r="P261">
+        <v>86.29604018912529</v>
+      </c>
+      <c r="Q261">
+        <v>33.84</v>
+      </c>
+      <c r="R261">
+        <v>417.41229</v>
+      </c>
+      <c r="S261">
+        <v>3.315844248350004</v>
+      </c>
+      <c r="T261">
+        <v>590.62001</v>
+      </c>
+      <c r="U261">
+        <v>17</v>
+      </c>
+      <c r="V261">
+        <v>9</v>
+      </c>
+      <c r="W261">
+        <v>26</v>
+      </c>
+      <c r="X261">
+        <v>54</v>
+      </c>
+      <c r="Y261">
+        <v>17</v>
+      </c>
+      <c r="Z261">
+        <v>30</v>
+      </c>
+      <c r="AA261">
+        <v>9</v>
+      </c>
+      <c r="AB261">
+        <v>11</v>
+      </c>
+      <c r="AC261">
+        <v>4.78498</v>
+      </c>
+      <c r="AD261">
+        <v>-1.91507</v>
+      </c>
+      <c r="AE261">
+        <v>0</v>
+      </c>
+      <c r="AF261">
+        <v>311.0198</v>
+      </c>
+      <c r="AG261">
+        <v>0</v>
+      </c>
+      <c r="AH261">
+        <v>3</v>
+      </c>
+      <c r="AI261">
+        <v>1252.23687</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B262" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E262">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F262">
+        <v>3252.27</v>
+      </c>
+      <c r="G262">
+        <v>25.83541748035562</v>
+      </c>
+      <c r="H262">
+        <v>78.46000000000001</v>
+      </c>
+      <c r="I262">
+        <v>0</v>
+      </c>
+      <c r="J262">
+        <v>0</v>
+      </c>
+      <c r="K262">
+        <v>0.6232713936754027</v>
+      </c>
+      <c r="L262">
+        <v>0</v>
+      </c>
+      <c r="M262">
+        <v>0</v>
+      </c>
+      <c r="N262">
+        <v>0</v>
+      </c>
+      <c r="O262">
+        <v>24.9593</v>
+      </c>
+      <c r="P262">
+        <v>74.07199667616334</v>
+      </c>
+      <c r="Q262">
+        <v>33.696</v>
+      </c>
+      <c r="R262">
+        <v>385.52693</v>
+      </c>
+      <c r="S262">
+        <v>3.062552981907971</v>
+      </c>
+      <c r="T262">
+        <v>373.85</v>
+      </c>
+      <c r="U262">
+        <v>18</v>
+      </c>
+      <c r="V262">
+        <v>8</v>
+      </c>
+      <c r="W262">
+        <v>26</v>
+      </c>
+      <c r="X262">
+        <v>35</v>
+      </c>
+      <c r="Y262">
+        <v>18</v>
+      </c>
+      <c r="Z262">
+        <v>25</v>
+      </c>
+      <c r="AA262">
+        <v>8</v>
+      </c>
+      <c r="AB262">
+        <v>10</v>
+      </c>
+      <c r="AC262">
+        <v>4.58185</v>
+      </c>
+      <c r="AD262">
+        <v>-2.01177</v>
+      </c>
+      <c r="AE262">
+        <v>0</v>
+      </c>
+      <c r="AF262">
+        <v>300.0584</v>
+      </c>
+      <c r="AG262">
+        <v>0</v>
+      </c>
+      <c r="AH262">
+        <v>3</v>
+      </c>
+      <c r="AI262">
+        <v>1156.58079</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B263" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E263">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F263">
+        <v>4355.15</v>
+      </c>
+      <c r="G263">
+        <v>34.59648751166747</v>
+      </c>
+      <c r="H263">
+        <v>183</v>
+      </c>
+      <c r="I263">
+        <v>0</v>
+      </c>
+      <c r="J263">
+        <v>0</v>
+      </c>
+      <c r="K263">
+        <v>1.453717372452188</v>
+      </c>
+      <c r="L263">
+        <v>0</v>
+      </c>
+      <c r="M263">
+        <v>3</v>
+      </c>
+      <c r="N263">
+        <v>0</v>
+      </c>
+      <c r="O263">
+        <v>28.86292</v>
+      </c>
+      <c r="P263">
+        <v>82.48433927754915</v>
+      </c>
+      <c r="Q263">
+        <v>34.992</v>
+      </c>
+      <c r="R263">
+        <v>460.57711</v>
+      </c>
+      <c r="S263">
+        <v>3.658737410714877</v>
+      </c>
+      <c r="T263">
+        <v>535.8499899999999</v>
+      </c>
+      <c r="U263">
+        <v>23</v>
+      </c>
+      <c r="V263">
+        <v>12</v>
+      </c>
+      <c r="W263">
+        <v>35</v>
+      </c>
+      <c r="X263">
+        <v>49</v>
+      </c>
+      <c r="Y263">
+        <v>23</v>
+      </c>
+      <c r="Z263">
+        <v>36</v>
+      </c>
+      <c r="AA263">
+        <v>12</v>
+      </c>
+      <c r="AB263">
+        <v>13</v>
+      </c>
+      <c r="AC263">
+        <v>4.67681</v>
+      </c>
+      <c r="AD263">
+        <v>-2.52243</v>
+      </c>
+      <c r="AE263">
+        <v>0</v>
+      </c>
+      <c r="AF263">
+        <v>344.63016</v>
+      </c>
+      <c r="AG263">
+        <v>0</v>
+      </c>
+      <c r="AH263">
+        <v>3</v>
+      </c>
+      <c r="AI263">
+        <v>1381.73133</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B264" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E264">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F264">
+        <v>3681.97</v>
+      </c>
+      <c r="G264">
+        <v>29.24887297184581</v>
+      </c>
+      <c r="H264">
+        <v>126.42</v>
+      </c>
+      <c r="I264">
+        <v>0</v>
+      </c>
+      <c r="J264">
+        <v>0</v>
+      </c>
+      <c r="K264">
+        <v>1.004256558608774</v>
+      </c>
+      <c r="L264">
+        <v>0</v>
+      </c>
+      <c r="M264">
+        <v>2</v>
+      </c>
+      <c r="N264">
+        <v>0</v>
+      </c>
+      <c r="O264">
+        <v>27.01013</v>
+      </c>
+      <c r="P264">
+        <v>77.34859679266896</v>
+      </c>
+      <c r="Q264">
+        <v>34.92</v>
+      </c>
+      <c r="R264">
+        <v>356.23206</v>
+      </c>
+      <c r="S264">
+        <v>2.829840077849346</v>
+      </c>
+      <c r="T264">
+        <v>500.4099899999999</v>
+      </c>
+      <c r="U264">
+        <v>18</v>
+      </c>
+      <c r="V264">
+        <v>4</v>
+      </c>
+      <c r="W264">
+        <v>22</v>
+      </c>
+      <c r="X264">
+        <v>42</v>
+      </c>
+      <c r="Y264">
+        <v>18</v>
+      </c>
+      <c r="Z264">
+        <v>38</v>
+      </c>
+      <c r="AA264">
+        <v>4</v>
+      </c>
+      <c r="AB264">
+        <v>11</v>
+      </c>
+      <c r="AC264">
+        <v>4.1026</v>
+      </c>
+      <c r="AD264">
+        <v>-1.75943</v>
+      </c>
+      <c r="AE264">
+        <v>0</v>
+      </c>
+      <c r="AF264">
+        <v>341.7104</v>
+      </c>
+      <c r="AG264">
+        <v>0</v>
+      </c>
+      <c r="AH264">
+        <v>3</v>
+      </c>
+      <c r="AI264">
+        <v>1068.69618</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B265" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E265">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F265">
+        <v>3905.06</v>
+      </c>
+      <c r="G265">
+        <v>31.02105771840515</v>
+      </c>
+      <c r="H265">
+        <v>175.17</v>
+      </c>
+      <c r="I265">
+        <v>0</v>
+      </c>
+      <c r="J265">
+        <v>0</v>
+      </c>
+      <c r="K265">
+        <v>1.391517334057103</v>
+      </c>
+      <c r="L265">
+        <v>0</v>
+      </c>
+      <c r="M265">
+        <v>6</v>
+      </c>
+      <c r="N265">
+        <v>0</v>
+      </c>
+      <c r="O265">
+        <v>27.29209</v>
+      </c>
+      <c r="P265">
+        <v>77.995227480567</v>
+      </c>
+      <c r="Q265">
+        <v>34.992</v>
+      </c>
+      <c r="R265">
+        <v>405.41803</v>
+      </c>
+      <c r="S265">
+        <v>3.220564116482745</v>
+      </c>
+      <c r="T265">
+        <v>611.54</v>
+      </c>
+      <c r="U265">
+        <v>22</v>
+      </c>
+      <c r="V265">
+        <v>18</v>
+      </c>
+      <c r="W265">
+        <v>40</v>
+      </c>
+      <c r="X265">
+        <v>62</v>
+      </c>
+      <c r="Y265">
+        <v>22</v>
+      </c>
+      <c r="Z265">
+        <v>55</v>
+      </c>
+      <c r="AA265">
+        <v>18</v>
+      </c>
+      <c r="AB265">
+        <v>14</v>
+      </c>
+      <c r="AC265">
+        <v>4.39602</v>
+      </c>
+      <c r="AD265">
+        <v>-2.13</v>
+      </c>
+      <c r="AE265">
+        <v>0</v>
+      </c>
+      <c r="AF265">
+        <v>331.45214</v>
+      </c>
+      <c r="AG265">
+        <v>0</v>
+      </c>
+      <c r="AH265">
+        <v>3</v>
+      </c>
+      <c r="AI265">
+        <v>1216.25409</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B266" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E266">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F266">
+        <v>3648.27</v>
+      </c>
+      <c r="G266">
+        <v>28.98116654861281</v>
+      </c>
+      <c r="H266">
+        <v>98.56</v>
+      </c>
+      <c r="I266">
+        <v>0</v>
+      </c>
+      <c r="J266">
+        <v>0</v>
+      </c>
+      <c r="K266">
+        <v>0.7829419903217906</v>
+      </c>
+      <c r="L266">
+        <v>0</v>
+      </c>
+      <c r="M266">
+        <v>1</v>
+      </c>
+      <c r="N266">
+        <v>0</v>
+      </c>
+      <c r="O266">
+        <v>25.95667</v>
+      </c>
+      <c r="P266">
+        <v>76.37909016007532</v>
+      </c>
+      <c r="Q266">
+        <v>33.984</v>
+      </c>
+      <c r="R266">
+        <v>412.89287</v>
+      </c>
+      <c r="S266">
+        <v>3.279942831041764</v>
+      </c>
+      <c r="T266">
+        <v>580.55999</v>
+      </c>
+      <c r="U266">
+        <v>22</v>
+      </c>
+      <c r="V266">
+        <v>20</v>
+      </c>
+      <c r="W266">
+        <v>42</v>
+      </c>
+      <c r="X266">
+        <v>53</v>
+      </c>
+      <c r="Y266">
+        <v>22</v>
+      </c>
+      <c r="Z266">
+        <v>51</v>
+      </c>
+      <c r="AA266">
+        <v>20</v>
+      </c>
+      <c r="AB266">
+        <v>26</v>
+      </c>
+      <c r="AC266">
+        <v>4.21691</v>
+      </c>
+      <c r="AD266">
+        <v>-1.96182</v>
+      </c>
+      <c r="AE266">
+        <v>0</v>
+      </c>
+      <c r="AF266">
+        <v>349.82</v>
+      </c>
+      <c r="AG266">
+        <v>0</v>
+      </c>
+      <c r="AH266">
+        <v>3</v>
+      </c>
+      <c r="AI266">
+        <v>1238.67861</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B267" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E267">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F267">
+        <v>3684.24</v>
+      </c>
+      <c r="G267">
+        <v>29.26690542231284</v>
+      </c>
+      <c r="H267">
+        <v>112.86</v>
+      </c>
+      <c r="I267">
+        <v>0</v>
+      </c>
+      <c r="J267">
+        <v>0</v>
+      </c>
+      <c r="K267">
+        <v>0.8965384844533003</v>
+      </c>
+      <c r="L267">
+        <v>0</v>
+      </c>
+      <c r="M267">
+        <v>1</v>
+      </c>
+      <c r="N267">
+        <v>0</v>
+      </c>
+      <c r="O267">
+        <v>25.95829</v>
+      </c>
+      <c r="P267">
+        <v>74.18349908550526</v>
+      </c>
+      <c r="Q267">
+        <v>34.992</v>
+      </c>
+      <c r="R267">
+        <v>381.80891</v>
+      </c>
+      <c r="S267">
+        <v>3.033017734557562</v>
+      </c>
+      <c r="T267">
+        <v>502.87001</v>
+      </c>
+      <c r="U267">
+        <v>22</v>
+      </c>
+      <c r="V267">
+        <v>20</v>
+      </c>
+      <c r="W267">
+        <v>42</v>
+      </c>
+      <c r="X267">
+        <v>41</v>
+      </c>
+      <c r="Y267">
+        <v>22</v>
+      </c>
+      <c r="Z267">
+        <v>41</v>
+      </c>
+      <c r="AA267">
+        <v>20</v>
+      </c>
+      <c r="AB267">
+        <v>13</v>
+      </c>
+      <c r="AC267">
+        <v>4.46884</v>
+      </c>
+      <c r="AD267">
+        <v>-1.63427</v>
+      </c>
+      <c r="AE267">
+        <v>0</v>
+      </c>
+      <c r="AF267">
+        <v>345.1224</v>
+      </c>
+      <c r="AG267">
+        <v>0</v>
+      </c>
+      <c r="AH267">
+        <v>3</v>
+      </c>
+      <c r="AI267">
+        <v>1145.42673</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B268" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E268">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F268">
+        <v>3692.78</v>
+      </c>
+      <c r="G268">
+        <v>29.33474556636061</v>
+      </c>
+      <c r="H268">
+        <v>67.02</v>
+      </c>
+      <c r="I268">
+        <v>0</v>
+      </c>
+      <c r="J268">
+        <v>0</v>
+      </c>
+      <c r="K268">
+        <v>0.5323941983701947</v>
+      </c>
+      <c r="L268">
+        <v>0</v>
+      </c>
+      <c r="M268">
+        <v>0</v>
+      </c>
+      <c r="N268">
+        <v>0</v>
+      </c>
+      <c r="O268">
+        <v>22.94909</v>
+      </c>
+      <c r="P268">
+        <v>69.51741790863929</v>
+      </c>
+      <c r="Q268">
+        <v>33.012</v>
+      </c>
+      <c r="R268">
+        <v>415.28049</v>
+      </c>
+      <c r="S268">
+        <v>3.298909632532553</v>
+      </c>
+      <c r="T268">
+        <v>571.7800099999999</v>
+      </c>
+      <c r="U268">
+        <v>22</v>
+      </c>
+      <c r="V268">
+        <v>20</v>
+      </c>
+      <c r="W268">
+        <v>42</v>
+      </c>
+      <c r="X268">
+        <v>64</v>
+      </c>
+      <c r="Y268">
+        <v>22</v>
+      </c>
+      <c r="Z268">
+        <v>61</v>
+      </c>
+      <c r="AA268">
+        <v>20</v>
+      </c>
+      <c r="AB268">
+        <v>13</v>
+      </c>
+      <c r="AC268">
+        <v>4.26797</v>
+      </c>
+      <c r="AD268">
+        <v>-1.06657</v>
+      </c>
+      <c r="AE268">
+        <v>0</v>
+      </c>
+      <c r="AF268">
+        <v>337.31025</v>
+      </c>
+      <c r="AG268">
+        <v>0</v>
+      </c>
+      <c r="AH268">
+        <v>3</v>
+      </c>
+      <c r="AI268">
+        <v>1245.84147</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B269" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E269">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F269">
+        <v>3387.06</v>
+      </c>
+      <c r="G269">
+        <v>26.90616373517983</v>
+      </c>
+      <c r="H269">
+        <v>145.99</v>
+      </c>
+      <c r="I269">
+        <v>0</v>
+      </c>
+      <c r="J269">
+        <v>0</v>
+      </c>
+      <c r="K269">
+        <v>1.159716935542595</v>
+      </c>
+      <c r="L269">
+        <v>0</v>
+      </c>
+      <c r="M269">
+        <v>2</v>
+      </c>
+      <c r="N269">
+        <v>0</v>
+      </c>
+      <c r="O269">
+        <v>26.5755</v>
+      </c>
+      <c r="P269">
+        <v>83.03805774278217</v>
+      </c>
+      <c r="Q269">
+        <v>32.004</v>
+      </c>
+      <c r="R269">
+        <v>348.63988</v>
+      </c>
+      <c r="S269">
+        <v>2.769529236533586</v>
+      </c>
+      <c r="T269">
+        <v>466.12999</v>
+      </c>
+      <c r="U269">
+        <v>16</v>
+      </c>
+      <c r="V269">
+        <v>9</v>
+      </c>
+      <c r="W269">
+        <v>25</v>
+      </c>
+      <c r="X269">
+        <v>36</v>
+      </c>
+      <c r="Y269">
+        <v>16</v>
+      </c>
+      <c r="Z269">
+        <v>25</v>
+      </c>
+      <c r="AA269">
+        <v>9</v>
+      </c>
+      <c r="AB269">
+        <v>13</v>
+      </c>
+      <c r="AC269">
+        <v>4.44805</v>
+      </c>
+      <c r="AD269">
+        <v>-1.26914</v>
+      </c>
+      <c r="AE269">
+        <v>0</v>
+      </c>
+      <c r="AF269">
+        <v>273.462</v>
+      </c>
+      <c r="AG269">
+        <v>0</v>
+      </c>
+      <c r="AH269">
+        <v>3</v>
+      </c>
+      <c r="AI269">
+        <v>1045.91964</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B270" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 19 pretemporada </t>
+        </is>
+      </c>
+      <c r="E270">
+        <v>125.8841666666667</v>
+      </c>
+      <c r="F270">
+        <v>3060.18</v>
+      </c>
+      <c r="G270">
+        <v>24.30949086792752</v>
+      </c>
+      <c r="H270">
+        <v>175.09</v>
+      </c>
+      <c r="I270">
+        <v>0</v>
+      </c>
+      <c r="J270">
+        <v>0</v>
+      </c>
+      <c r="K270">
+        <v>1.390881829194829</v>
+      </c>
+      <c r="L270">
+        <v>0</v>
+      </c>
+      <c r="M270">
+        <v>5</v>
+      </c>
+      <c r="N270">
+        <v>0</v>
+      </c>
+      <c r="O270">
+        <v>27.47299</v>
+      </c>
+      <c r="P270">
+        <v>76.31386111111111</v>
+      </c>
+      <c r="Q270">
+        <v>36</v>
+      </c>
+      <c r="R270">
+        <v>374.32809</v>
+      </c>
+      <c r="S270">
+        <v>2.973591516010088</v>
+      </c>
+      <c r="T270">
+        <v>435.74001</v>
+      </c>
+      <c r="U270">
+        <v>24</v>
+      </c>
+      <c r="V270">
+        <v>8</v>
+      </c>
+      <c r="W270">
+        <v>32</v>
+      </c>
+      <c r="X270">
+        <v>40</v>
+      </c>
+      <c r="Y270">
+        <v>24</v>
+      </c>
+      <c r="Z270">
+        <v>24</v>
+      </c>
+      <c r="AA270">
+        <v>8</v>
+      </c>
+      <c r="AB270">
+        <v>22</v>
+      </c>
+      <c r="AC270">
+        <v>4.38131</v>
+      </c>
+      <c r="AD270">
+        <v>-1.95372</v>
+      </c>
+      <c r="AE270">
+        <v>0</v>
+      </c>
+      <c r="AF270">
+        <v>244.7158</v>
+      </c>
+      <c r="AG270">
+        <v>0</v>
+      </c>
+      <c r="AH270">
+        <v>3</v>
+      </c>
+      <c r="AI270">
+        <v>1122.98427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-28
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI269"/>
+  <dimension ref="A1:AI283"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -30727,6 +30727,1588 @@
         <v>1122.98427</v>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B270" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E270">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F270">
+        <v>10564</v>
+      </c>
+      <c r="G270">
+        <v>113.634163394826</v>
+      </c>
+      <c r="H270">
+        <v>232.7</v>
+      </c>
+      <c r="I270">
+        <v>0</v>
+      </c>
+      <c r="J270">
+        <v>0</v>
+      </c>
+      <c r="K270">
+        <v>2.503092561716775</v>
+      </c>
+      <c r="L270">
+        <v>0</v>
+      </c>
+      <c r="M270">
+        <v>3</v>
+      </c>
+      <c r="N270">
+        <v>0</v>
+      </c>
+      <c r="O270">
+        <v>26.97144</v>
+      </c>
+      <c r="P270">
+        <v>83.33778272154247</v>
+      </c>
+      <c r="Q270">
+        <v>32.364</v>
+      </c>
+      <c r="R270">
+        <v>1038.10101</v>
+      </c>
+      <c r="S270">
+        <v>11.16657892755338</v>
+      </c>
+      <c r="T270">
+        <v>1268.59002</v>
+      </c>
+      <c r="U270">
+        <v>9</v>
+      </c>
+      <c r="V270">
+        <v>10</v>
+      </c>
+      <c r="W270">
+        <v>19</v>
+      </c>
+      <c r="X270">
+        <v>72</v>
+      </c>
+      <c r="Y270">
+        <v>9</v>
+      </c>
+      <c r="Z270">
+        <v>51</v>
+      </c>
+      <c r="AA270">
+        <v>10</v>
+      </c>
+      <c r="AB270">
+        <v>15</v>
+      </c>
+      <c r="AC270">
+        <v>4.32614</v>
+      </c>
+      <c r="AD270">
+        <v>-4.824</v>
+      </c>
+      <c r="AE270">
+        <v>0</v>
+      </c>
+      <c r="AF270">
+        <v>838.8407999999999</v>
+      </c>
+      <c r="AG270">
+        <v>0</v>
+      </c>
+      <c r="AH270">
+        <v>3</v>
+      </c>
+      <c r="AI270">
+        <v>3114.30303</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B271" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E271">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F271">
+        <v>9389.990000000002</v>
+      </c>
+      <c r="G271">
+        <v>101.0056472866133</v>
+      </c>
+      <c r="H271">
+        <v>508.8899999999999</v>
+      </c>
+      <c r="I271">
+        <v>26.91</v>
+      </c>
+      <c r="J271">
+        <v>2</v>
+      </c>
+      <c r="K271">
+        <v>5.473995589738073</v>
+      </c>
+      <c r="L271">
+        <v>9.969999999999999</v>
+      </c>
+      <c r="M271">
+        <v>8</v>
+      </c>
+      <c r="N271">
+        <v>1</v>
+      </c>
+      <c r="O271">
+        <v>30.19985</v>
+      </c>
+      <c r="P271">
+        <v>93.20941358024693</v>
+      </c>
+      <c r="Q271">
+        <v>32.4</v>
+      </c>
+      <c r="R271">
+        <v>992.7741699999999</v>
+      </c>
+      <c r="S271">
+        <v>10.67901005754854</v>
+      </c>
+      <c r="T271">
+        <v>1836.95001</v>
+      </c>
+      <c r="U271">
+        <v>25</v>
+      </c>
+      <c r="V271">
+        <v>32</v>
+      </c>
+      <c r="W271">
+        <v>57</v>
+      </c>
+      <c r="X271">
+        <v>133</v>
+      </c>
+      <c r="Y271">
+        <v>25</v>
+      </c>
+      <c r="Z271">
+        <v>111</v>
+      </c>
+      <c r="AA271">
+        <v>32</v>
+      </c>
+      <c r="AB271">
+        <v>19</v>
+      </c>
+      <c r="AC271">
+        <v>3.97611</v>
+      </c>
+      <c r="AD271">
+        <v>-4.17912</v>
+      </c>
+      <c r="AE271">
+        <v>0</v>
+      </c>
+      <c r="AF271">
+        <v>784.8273999999999</v>
+      </c>
+      <c r="AG271">
+        <v>0</v>
+      </c>
+      <c r="AH271">
+        <v>3</v>
+      </c>
+      <c r="AI271">
+        <v>2978.32251</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B272" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E272">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F272">
+        <v>8470.700000000001</v>
+      </c>
+      <c r="G272">
+        <v>91.11708707578123</v>
+      </c>
+      <c r="H272">
+        <v>626.5400000000001</v>
+      </c>
+      <c r="I272">
+        <v>8.58</v>
+      </c>
+      <c r="J272">
+        <v>1</v>
+      </c>
+      <c r="K272">
+        <v>6.73952562792449</v>
+      </c>
+      <c r="L272">
+        <v>22.26</v>
+      </c>
+      <c r="M272">
+        <v>15</v>
+      </c>
+      <c r="N272">
+        <v>2</v>
+      </c>
+      <c r="O272">
+        <v>30.91465</v>
+      </c>
+      <c r="P272">
+        <v>90.9682497645951</v>
+      </c>
+      <c r="Q272">
+        <v>33.984</v>
+      </c>
+      <c r="R272">
+        <v>899.93463</v>
+      </c>
+      <c r="S272">
+        <v>9.680359597698059</v>
+      </c>
+      <c r="T272">
+        <v>1309.57</v>
+      </c>
+      <c r="U272">
+        <v>27</v>
+      </c>
+      <c r="V272">
+        <v>20</v>
+      </c>
+      <c r="W272">
+        <v>47</v>
+      </c>
+      <c r="X272">
+        <v>76</v>
+      </c>
+      <c r="Y272">
+        <v>27</v>
+      </c>
+      <c r="Z272">
+        <v>75</v>
+      </c>
+      <c r="AA272">
+        <v>20</v>
+      </c>
+      <c r="AB272">
+        <v>20</v>
+      </c>
+      <c r="AC272">
+        <v>4.0919</v>
+      </c>
+      <c r="AD272">
+        <v>-4.95388</v>
+      </c>
+      <c r="AE272">
+        <v>0</v>
+      </c>
+      <c r="AF272">
+        <v>798.7096000000001</v>
+      </c>
+      <c r="AG272">
+        <v>0</v>
+      </c>
+      <c r="AH272">
+        <v>3</v>
+      </c>
+      <c r="AI272">
+        <v>2699.80389</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B273" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E273">
+        <v>135.0218333333333</v>
+      </c>
+      <c r="F273">
+        <v>11070.29</v>
+      </c>
+      <c r="G273">
+        <v>81.98888821684396</v>
+      </c>
+      <c r="H273">
+        <v>865.48</v>
+      </c>
+      <c r="I273">
+        <v>28.79</v>
+      </c>
+      <c r="J273">
+        <v>3</v>
+      </c>
+      <c r="K273">
+        <v>6.409926295870669</v>
+      </c>
+      <c r="L273">
+        <v>64.57000000000001</v>
+      </c>
+      <c r="M273">
+        <v>21</v>
+      </c>
+      <c r="N273">
+        <v>4</v>
+      </c>
+      <c r="O273">
+        <v>34.29679</v>
+      </c>
+      <c r="P273">
+        <v>96.42597278452543</v>
+      </c>
+      <c r="Q273">
+        <v>35.568</v>
+      </c>
+      <c r="R273">
+        <v>891.0671599999999</v>
+      </c>
+      <c r="S273">
+        <v>6.599430166232375</v>
+      </c>
+      <c r="T273">
+        <v>1669.22</v>
+      </c>
+      <c r="U273">
+        <v>32</v>
+      </c>
+      <c r="V273">
+        <v>23</v>
+      </c>
+      <c r="W273">
+        <v>55</v>
+      </c>
+      <c r="X273">
+        <v>99</v>
+      </c>
+      <c r="Y273">
+        <v>32</v>
+      </c>
+      <c r="Z273">
+        <v>74</v>
+      </c>
+      <c r="AA273">
+        <v>23</v>
+      </c>
+      <c r="AB273">
+        <v>12</v>
+      </c>
+      <c r="AC273">
+        <v>4.51253</v>
+      </c>
+      <c r="AD273">
+        <v>-3.97387</v>
+      </c>
+      <c r="AE273">
+        <v>0</v>
+      </c>
+      <c r="AF273">
+        <v>1023.0488</v>
+      </c>
+      <c r="AG273">
+        <v>0</v>
+      </c>
+      <c r="AH273">
+        <v>3</v>
+      </c>
+      <c r="AI273">
+        <v>2673.20148</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B274" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E274">
+        <v>135.0218333333333</v>
+      </c>
+      <c r="F274">
+        <v>11437.95</v>
+      </c>
+      <c r="G274">
+        <v>84.71185524316439</v>
+      </c>
+      <c r="H274">
+        <v>561.1800000000001</v>
+      </c>
+      <c r="I274">
+        <v>0</v>
+      </c>
+      <c r="J274">
+        <v>0</v>
+      </c>
+      <c r="K274">
+        <v>4.15621671063075</v>
+      </c>
+      <c r="L274">
+        <v>35.72</v>
+      </c>
+      <c r="M274">
+        <v>12</v>
+      </c>
+      <c r="N274">
+        <v>1</v>
+      </c>
+      <c r="O274">
+        <v>30.89641</v>
+      </c>
+      <c r="P274">
+        <v>85.82336111111111</v>
+      </c>
+      <c r="Q274">
+        <v>36</v>
+      </c>
+      <c r="R274">
+        <v>1026.42478</v>
+      </c>
+      <c r="S274">
+        <v>7.601917072670965</v>
+      </c>
+      <c r="T274">
+        <v>1445.64997</v>
+      </c>
+      <c r="U274">
+        <v>26</v>
+      </c>
+      <c r="V274">
+        <v>29</v>
+      </c>
+      <c r="W274">
+        <v>55</v>
+      </c>
+      <c r="X274">
+        <v>122</v>
+      </c>
+      <c r="Y274">
+        <v>26</v>
+      </c>
+      <c r="Z274">
+        <v>93</v>
+      </c>
+      <c r="AA274">
+        <v>29</v>
+      </c>
+      <c r="AB274">
+        <v>30</v>
+      </c>
+      <c r="AC274">
+        <v>4.02164</v>
+      </c>
+      <c r="AD274">
+        <v>-3.98067</v>
+      </c>
+      <c r="AE274">
+        <v>0</v>
+      </c>
+      <c r="AF274">
+        <v>922.3998</v>
+      </c>
+      <c r="AG274">
+        <v>0</v>
+      </c>
+      <c r="AH274">
+        <v>3</v>
+      </c>
+      <c r="AI274">
+        <v>3079.27434</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B275" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E275">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F275">
+        <v>9261.099999999999</v>
+      </c>
+      <c r="G275">
+        <v>99.61921153122142</v>
+      </c>
+      <c r="H275">
+        <v>454.99</v>
+      </c>
+      <c r="I275">
+        <v>0</v>
+      </c>
+      <c r="J275">
+        <v>0</v>
+      </c>
+      <c r="K275">
+        <v>4.894207497445276</v>
+      </c>
+      <c r="L275">
+        <v>0</v>
+      </c>
+      <c r="M275">
+        <v>8</v>
+      </c>
+      <c r="N275">
+        <v>0</v>
+      </c>
+      <c r="O275">
+        <v>27.78112</v>
+      </c>
+      <c r="P275">
+        <v>86.80514935633047</v>
+      </c>
+      <c r="Q275">
+        <v>32.004</v>
+      </c>
+      <c r="R275">
+        <v>911.78638</v>
+      </c>
+      <c r="S275">
+        <v>9.807845748399936</v>
+      </c>
+      <c r="T275">
+        <v>1459.15002</v>
+      </c>
+      <c r="U275">
+        <v>25</v>
+      </c>
+      <c r="V275">
+        <v>39</v>
+      </c>
+      <c r="W275">
+        <v>64</v>
+      </c>
+      <c r="X275">
+        <v>98</v>
+      </c>
+      <c r="Y275">
+        <v>25</v>
+      </c>
+      <c r="Z275">
+        <v>103</v>
+      </c>
+      <c r="AA275">
+        <v>39</v>
+      </c>
+      <c r="AB275">
+        <v>16</v>
+      </c>
+      <c r="AC275">
+        <v>3.89903</v>
+      </c>
+      <c r="AD275">
+        <v>-5.45512</v>
+      </c>
+      <c r="AE275">
+        <v>0</v>
+      </c>
+      <c r="AF275">
+        <v>656.58</v>
+      </c>
+      <c r="AG275">
+        <v>0</v>
+      </c>
+      <c r="AH275">
+        <v>3</v>
+      </c>
+      <c r="AI275">
+        <v>2735.35914</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B276" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E276">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F276">
+        <v>7897.9</v>
+      </c>
+      <c r="G276">
+        <v>84.95562846232454</v>
+      </c>
+      <c r="H276">
+        <v>364.76</v>
+      </c>
+      <c r="I276">
+        <v>0</v>
+      </c>
+      <c r="J276">
+        <v>0</v>
+      </c>
+      <c r="K276">
+        <v>3.923627171516162</v>
+      </c>
+      <c r="L276">
+        <v>0</v>
+      </c>
+      <c r="M276">
+        <v>6</v>
+      </c>
+      <c r="N276">
+        <v>0</v>
+      </c>
+      <c r="O276">
+        <v>27.17256</v>
+      </c>
+      <c r="P276">
+        <v>80.64031339031339</v>
+      </c>
+      <c r="Q276">
+        <v>33.696</v>
+      </c>
+      <c r="R276">
+        <v>719.60437</v>
+      </c>
+      <c r="S276">
+        <v>7.74059452482117</v>
+      </c>
+      <c r="T276">
+        <v>1247.73001</v>
+      </c>
+      <c r="U276">
+        <v>21</v>
+      </c>
+      <c r="V276">
+        <v>34</v>
+      </c>
+      <c r="W276">
+        <v>55</v>
+      </c>
+      <c r="X276">
+        <v>97</v>
+      </c>
+      <c r="Y276">
+        <v>21</v>
+      </c>
+      <c r="Z276">
+        <v>89</v>
+      </c>
+      <c r="AA276">
+        <v>34</v>
+      </c>
+      <c r="AB276">
+        <v>16</v>
+      </c>
+      <c r="AC276">
+        <v>4.71996</v>
+      </c>
+      <c r="AD276">
+        <v>-4.20412</v>
+      </c>
+      <c r="AE276">
+        <v>0</v>
+      </c>
+      <c r="AF276">
+        <v>749.7311999999999</v>
+      </c>
+      <c r="AG276">
+        <v>0</v>
+      </c>
+      <c r="AH276">
+        <v>3</v>
+      </c>
+      <c r="AI276">
+        <v>2158.81311</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B277" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E277">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F277">
+        <v>8693.450000000001</v>
+      </c>
+      <c r="G277">
+        <v>93.51315011025656</v>
+      </c>
+      <c r="H277">
+        <v>595.5999999999999</v>
+      </c>
+      <c r="I277">
+        <v>0</v>
+      </c>
+      <c r="J277">
+        <v>0</v>
+      </c>
+      <c r="K277">
+        <v>6.406712203517452</v>
+      </c>
+      <c r="L277">
+        <v>4.08</v>
+      </c>
+      <c r="M277">
+        <v>10</v>
+      </c>
+      <c r="N277">
+        <v>0</v>
+      </c>
+      <c r="O277">
+        <v>29.99264</v>
+      </c>
+      <c r="P277">
+        <v>85.71284865112027</v>
+      </c>
+      <c r="Q277">
+        <v>34.992</v>
+      </c>
+      <c r="R277">
+        <v>705.8837599999999</v>
+      </c>
+      <c r="S277">
+        <v>7.59300553971925</v>
+      </c>
+      <c r="T277">
+        <v>1447.40998</v>
+      </c>
+      <c r="U277">
+        <v>27</v>
+      </c>
+      <c r="V277">
+        <v>16</v>
+      </c>
+      <c r="W277">
+        <v>43</v>
+      </c>
+      <c r="X277">
+        <v>94</v>
+      </c>
+      <c r="Y277">
+        <v>27</v>
+      </c>
+      <c r="Z277">
+        <v>81</v>
+      </c>
+      <c r="AA277">
+        <v>16</v>
+      </c>
+      <c r="AB277">
+        <v>10</v>
+      </c>
+      <c r="AC277">
+        <v>4.46449</v>
+      </c>
+      <c r="AD277">
+        <v>-4.76258</v>
+      </c>
+      <c r="AE277">
+        <v>0</v>
+      </c>
+      <c r="AF277">
+        <v>704.08497</v>
+      </c>
+      <c r="AG277">
+        <v>0</v>
+      </c>
+      <c r="AH277">
+        <v>3</v>
+      </c>
+      <c r="AI277">
+        <v>2117.65128</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B278" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E278">
+        <v>90.5025</v>
+      </c>
+      <c r="F278">
+        <v>7620.969999999999</v>
+      </c>
+      <c r="G278">
+        <v>84.2072870915168</v>
+      </c>
+      <c r="H278">
+        <v>421.41</v>
+      </c>
+      <c r="I278">
+        <v>10.51</v>
+      </c>
+      <c r="J278">
+        <v>1</v>
+      </c>
+      <c r="K278">
+        <v>4.6563354603464</v>
+      </c>
+      <c r="L278">
+        <v>17.51</v>
+      </c>
+      <c r="M278">
+        <v>12</v>
+      </c>
+      <c r="N278">
+        <v>1</v>
+      </c>
+      <c r="O278">
+        <v>32.52348</v>
+      </c>
+      <c r="P278">
+        <v>93.13711340206184</v>
+      </c>
+      <c r="Q278">
+        <v>34.92</v>
+      </c>
+      <c r="R278">
+        <v>584.2881199999999</v>
+      </c>
+      <c r="S278">
+        <v>6.456043976685726</v>
+      </c>
+      <c r="T278">
+        <v>1060.80997</v>
+      </c>
+      <c r="U278">
+        <v>20</v>
+      </c>
+      <c r="V278">
+        <v>10</v>
+      </c>
+      <c r="W278">
+        <v>30</v>
+      </c>
+      <c r="X278">
+        <v>69</v>
+      </c>
+      <c r="Y278">
+        <v>20</v>
+      </c>
+      <c r="Z278">
+        <v>52</v>
+      </c>
+      <c r="AA278">
+        <v>10</v>
+      </c>
+      <c r="AB278">
+        <v>14</v>
+      </c>
+      <c r="AC278">
+        <v>4.35688</v>
+      </c>
+      <c r="AD278">
+        <v>-3.46881</v>
+      </c>
+      <c r="AE278">
+        <v>0</v>
+      </c>
+      <c r="AF278">
+        <v>696.2592</v>
+      </c>
+      <c r="AG278">
+        <v>0</v>
+      </c>
+      <c r="AH278">
+        <v>3</v>
+      </c>
+      <c r="AI278">
+        <v>1752.86436</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B279" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E279">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F279">
+        <v>8937.02</v>
+      </c>
+      <c r="G279">
+        <v>96.13316839670846</v>
+      </c>
+      <c r="H279">
+        <v>820.0700000000001</v>
+      </c>
+      <c r="I279">
+        <v>19.12</v>
+      </c>
+      <c r="J279">
+        <v>1</v>
+      </c>
+      <c r="K279">
+        <v>8.821276824611415</v>
+      </c>
+      <c r="L279">
+        <v>51.92</v>
+      </c>
+      <c r="M279">
+        <v>23</v>
+      </c>
+      <c r="N279">
+        <v>4</v>
+      </c>
+      <c r="O279">
+        <v>32.03853</v>
+      </c>
+      <c r="P279">
+        <v>91.55958504801099</v>
+      </c>
+      <c r="Q279">
+        <v>34.992</v>
+      </c>
+      <c r="R279">
+        <v>697.11337</v>
+      </c>
+      <c r="S279">
+        <v>7.498664766309902</v>
+      </c>
+      <c r="T279">
+        <v>1829.59002</v>
+      </c>
+      <c r="U279">
+        <v>42</v>
+      </c>
+      <c r="V279">
+        <v>36</v>
+      </c>
+      <c r="W279">
+        <v>78</v>
+      </c>
+      <c r="X279">
+        <v>106</v>
+      </c>
+      <c r="Y279">
+        <v>42</v>
+      </c>
+      <c r="Z279">
+        <v>103</v>
+      </c>
+      <c r="AA279">
+        <v>36</v>
+      </c>
+      <c r="AB279">
+        <v>14</v>
+      </c>
+      <c r="AC279">
+        <v>4.41862</v>
+      </c>
+      <c r="AD279">
+        <v>-4.9661</v>
+      </c>
+      <c r="AE279">
+        <v>0</v>
+      </c>
+      <c r="AF279">
+        <v>767.5852600000001</v>
+      </c>
+      <c r="AG279">
+        <v>0</v>
+      </c>
+      <c r="AH279">
+        <v>3</v>
+      </c>
+      <c r="AI279">
+        <v>2091.34011</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B280" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E280">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F280">
+        <v>8896.809999999999</v>
+      </c>
+      <c r="G280">
+        <v>95.70064002581617</v>
+      </c>
+      <c r="H280">
+        <v>381.72</v>
+      </c>
+      <c r="I280">
+        <v>0</v>
+      </c>
+      <c r="J280">
+        <v>0</v>
+      </c>
+      <c r="K280">
+        <v>4.10606142096488</v>
+      </c>
+      <c r="L280">
+        <v>0</v>
+      </c>
+      <c r="M280">
+        <v>6</v>
+      </c>
+      <c r="N280">
+        <v>0</v>
+      </c>
+      <c r="O280">
+        <v>28.75241</v>
+      </c>
+      <c r="P280">
+        <v>84.60572622410545</v>
+      </c>
+      <c r="Q280">
+        <v>33.984</v>
+      </c>
+      <c r="R280">
+        <v>806.22091</v>
+      </c>
+      <c r="S280">
+        <v>8.672305814016029</v>
+      </c>
+      <c r="T280">
+        <v>1267.27997</v>
+      </c>
+      <c r="U280">
+        <v>25</v>
+      </c>
+      <c r="V280">
+        <v>33</v>
+      </c>
+      <c r="W280">
+        <v>58</v>
+      </c>
+      <c r="X280">
+        <v>82</v>
+      </c>
+      <c r="Y280">
+        <v>25</v>
+      </c>
+      <c r="Z280">
+        <v>100</v>
+      </c>
+      <c r="AA280">
+        <v>33</v>
+      </c>
+      <c r="AB280">
+        <v>21</v>
+      </c>
+      <c r="AC280">
+        <v>4.20668</v>
+      </c>
+      <c r="AD280">
+        <v>-5.08979</v>
+      </c>
+      <c r="AE280">
+        <v>0</v>
+      </c>
+      <c r="AF280">
+        <v>835.1888000000001</v>
+      </c>
+      <c r="AG280">
+        <v>0</v>
+      </c>
+      <c r="AH280">
+        <v>3</v>
+      </c>
+      <c r="AI280">
+        <v>2418.66273</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B281" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E281">
+        <v>135.0218333333333</v>
+      </c>
+      <c r="F281">
+        <v>8081.759999999999</v>
+      </c>
+      <c r="G281">
+        <v>59.85520860206559</v>
+      </c>
+      <c r="H281">
+        <v>254.47</v>
+      </c>
+      <c r="I281">
+        <v>0</v>
+      </c>
+      <c r="J281">
+        <v>0</v>
+      </c>
+      <c r="K281">
+        <v>1.88465816022347</v>
+      </c>
+      <c r="L281">
+        <v>0</v>
+      </c>
+      <c r="M281">
+        <v>1</v>
+      </c>
+      <c r="N281">
+        <v>0</v>
+      </c>
+      <c r="O281">
+        <v>26.81674</v>
+      </c>
+      <c r="P281">
+        <v>76.63677411979882</v>
+      </c>
+      <c r="Q281">
+        <v>34.992</v>
+      </c>
+      <c r="R281">
+        <v>760.56808</v>
+      </c>
+      <c r="S281">
+        <v>5.632926625446996</v>
+      </c>
+      <c r="T281">
+        <v>1158.87</v>
+      </c>
+      <c r="U281">
+        <v>26</v>
+      </c>
+      <c r="V281">
+        <v>28</v>
+      </c>
+      <c r="W281">
+        <v>54</v>
+      </c>
+      <c r="X281">
+        <v>106</v>
+      </c>
+      <c r="Y281">
+        <v>26</v>
+      </c>
+      <c r="Z281">
+        <v>98</v>
+      </c>
+      <c r="AA281">
+        <v>28</v>
+      </c>
+      <c r="AB281">
+        <v>38</v>
+      </c>
+      <c r="AC281">
+        <v>4.36804</v>
+      </c>
+      <c r="AD281">
+        <v>-3.75893</v>
+      </c>
+      <c r="AE281">
+        <v>0</v>
+      </c>
+      <c r="AF281">
+        <v>763.8088</v>
+      </c>
+      <c r="AG281">
+        <v>0</v>
+      </c>
+      <c r="AH281">
+        <v>3</v>
+      </c>
+      <c r="AI281">
+        <v>2281.70424</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B282" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E282">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F282">
+        <v>7718.290000000001</v>
+      </c>
+      <c r="G282">
+        <v>83.02361103641157</v>
+      </c>
+      <c r="H282">
+        <v>303.74</v>
+      </c>
+      <c r="I282">
+        <v>0</v>
+      </c>
+      <c r="J282">
+        <v>0</v>
+      </c>
+      <c r="K282">
+        <v>3.267251116011403</v>
+      </c>
+      <c r="L282">
+        <v>0</v>
+      </c>
+      <c r="M282">
+        <v>7</v>
+      </c>
+      <c r="N282">
+        <v>0</v>
+      </c>
+      <c r="O282">
+        <v>28.93019</v>
+      </c>
+      <c r="P282">
+        <v>87.635375015146</v>
+      </c>
+      <c r="Q282">
+        <v>33.012</v>
+      </c>
+      <c r="R282">
+        <v>667.0199</v>
+      </c>
+      <c r="S282">
+        <v>7.174957241972787</v>
+      </c>
+      <c r="T282">
+        <v>1068.40998</v>
+      </c>
+      <c r="U282">
+        <v>15</v>
+      </c>
+      <c r="V282">
+        <v>14</v>
+      </c>
+      <c r="W282">
+        <v>29</v>
+      </c>
+      <c r="X282">
+        <v>82</v>
+      </c>
+      <c r="Y282">
+        <v>15</v>
+      </c>
+      <c r="Z282">
+        <v>70</v>
+      </c>
+      <c r="AA282">
+        <v>14</v>
+      </c>
+      <c r="AB282">
+        <v>11</v>
+      </c>
+      <c r="AC282">
+        <v>3.91521</v>
+      </c>
+      <c r="AD282">
+        <v>-3.28479</v>
+      </c>
+      <c r="AE282">
+        <v>0</v>
+      </c>
+      <c r="AF282">
+        <v>670.7062500000001</v>
+      </c>
+      <c r="AG282">
+        <v>0</v>
+      </c>
+      <c r="AH282">
+        <v>3</v>
+      </c>
+      <c r="AI282">
+        <v>2001.0597</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B283" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sesión 21 amistoso </t>
+        </is>
+      </c>
+      <c r="E283">
+        <v>92.96499999999999</v>
+      </c>
+      <c r="F283">
+        <v>9516.349999999999</v>
+      </c>
+      <c r="G283">
+        <v>102.3648684988974</v>
+      </c>
+      <c r="H283">
+        <v>433.87</v>
+      </c>
+      <c r="I283">
+        <v>38</v>
+      </c>
+      <c r="J283">
+        <v>3</v>
+      </c>
+      <c r="K283">
+        <v>4.667025224546873</v>
+      </c>
+      <c r="L283">
+        <v>26.87</v>
+      </c>
+      <c r="M283">
+        <v>9</v>
+      </c>
+      <c r="N283">
+        <v>1</v>
+      </c>
+      <c r="O283">
+        <v>30.58076</v>
+      </c>
+      <c r="P283">
+        <v>95.55293088363955</v>
+      </c>
+      <c r="Q283">
+        <v>32.004</v>
+      </c>
+      <c r="R283">
+        <v>824.8252600000001</v>
+      </c>
+      <c r="S283">
+        <v>8.872427902974239</v>
+      </c>
+      <c r="T283">
+        <v>1387.40003</v>
+      </c>
+      <c r="U283">
+        <v>20</v>
+      </c>
+      <c r="V283">
+        <v>27</v>
+      </c>
+      <c r="W283">
+        <v>47</v>
+      </c>
+      <c r="X283">
+        <v>97</v>
+      </c>
+      <c r="Y283">
+        <v>20</v>
+      </c>
+      <c r="Z283">
+        <v>91</v>
+      </c>
+      <c r="AA283">
+        <v>27</v>
+      </c>
+      <c r="AB283">
+        <v>17</v>
+      </c>
+      <c r="AC283">
+        <v>3.86013</v>
+      </c>
+      <c r="AD283">
+        <v>-4.13401</v>
+      </c>
+      <c r="AE283">
+        <v>0</v>
+      </c>
+      <c r="AF283">
+        <v>778.9558</v>
+      </c>
+      <c r="AG283">
+        <v>0</v>
+      </c>
+      <c r="AH283">
+        <v>3</v>
+      </c>
+      <c r="AI283">
+        <v>2474.47578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-29
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI283"/>
+  <dimension ref="A1:AI298"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -32309,6 +32309,1701 @@
         <v>2474.47578</v>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B284" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E284">
+        <v>278.45</v>
+      </c>
+      <c r="F284">
+        <v>15136.53</v>
+      </c>
+      <c r="G284">
+        <v>54.35995690429162</v>
+      </c>
+      <c r="H284">
+        <v>290.25</v>
+      </c>
+      <c r="I284">
+        <v>0</v>
+      </c>
+      <c r="J284">
+        <v>0</v>
+      </c>
+      <c r="K284">
+        <v>1.042377446579278</v>
+      </c>
+      <c r="L284">
+        <v>0</v>
+      </c>
+      <c r="M284">
+        <v>4</v>
+      </c>
+      <c r="N284">
+        <v>0</v>
+      </c>
+      <c r="O284">
+        <v>27.91498</v>
+      </c>
+      <c r="P284">
+        <v>86.25318254851069</v>
+      </c>
+      <c r="Q284">
+        <v>32.364</v>
+      </c>
+      <c r="R284">
+        <v>1657.89956</v>
+      </c>
+      <c r="S284">
+        <v>5.954029664212606</v>
+      </c>
+      <c r="T284">
+        <v>2328.35001</v>
+      </c>
+      <c r="U284">
+        <v>32</v>
+      </c>
+      <c r="V284">
+        <v>62</v>
+      </c>
+      <c r="W284">
+        <v>94</v>
+      </c>
+      <c r="X284">
+        <v>222</v>
+      </c>
+      <c r="Y284">
+        <v>32</v>
+      </c>
+      <c r="Z284">
+        <v>180</v>
+      </c>
+      <c r="AA284">
+        <v>62</v>
+      </c>
+      <c r="AB284">
+        <v>157</v>
+      </c>
+      <c r="AC284">
+        <v>4.08031</v>
+      </c>
+      <c r="AD284">
+        <v>-1.30718</v>
+      </c>
+      <c r="AE284">
+        <v>0</v>
+      </c>
+      <c r="AF284">
+        <v>1239.6132</v>
+      </c>
+      <c r="AG284">
+        <v>0</v>
+      </c>
+      <c r="AH284">
+        <v>3</v>
+      </c>
+      <c r="AI284">
+        <v>4973.69868</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B285" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E285">
+        <v>278.45</v>
+      </c>
+      <c r="F285">
+        <v>16233.79</v>
+      </c>
+      <c r="G285">
+        <v>58.30055665289998</v>
+      </c>
+      <c r="H285">
+        <v>264.75</v>
+      </c>
+      <c r="I285">
+        <v>0</v>
+      </c>
+      <c r="J285">
+        <v>0</v>
+      </c>
+      <c r="K285">
+        <v>0.9507990662596517</v>
+      </c>
+      <c r="L285">
+        <v>0</v>
+      </c>
+      <c r="M285">
+        <v>4</v>
+      </c>
+      <c r="N285">
+        <v>0</v>
+      </c>
+      <c r="O285">
+        <v>26.04827</v>
+      </c>
+      <c r="P285">
+        <v>80.3958950617284</v>
+      </c>
+      <c r="Q285">
+        <v>32.4</v>
+      </c>
+      <c r="R285">
+        <v>2013.25963</v>
+      </c>
+      <c r="S285">
+        <v>7.230237493266296</v>
+      </c>
+      <c r="T285">
+        <v>3086.46996</v>
+      </c>
+      <c r="U285">
+        <v>102</v>
+      </c>
+      <c r="V285">
+        <v>94</v>
+      </c>
+      <c r="W285">
+        <v>196</v>
+      </c>
+      <c r="X285">
+        <v>370</v>
+      </c>
+      <c r="Y285">
+        <v>102</v>
+      </c>
+      <c r="Z285">
+        <v>289</v>
+      </c>
+      <c r="AA285">
+        <v>94</v>
+      </c>
+      <c r="AB285">
+        <v>66</v>
+      </c>
+      <c r="AC285">
+        <v>4.32018</v>
+      </c>
+      <c r="AD285">
+        <v>-2.16682</v>
+      </c>
+      <c r="AE285">
+        <v>0</v>
+      </c>
+      <c r="AF285">
+        <v>1395.4332</v>
+      </c>
+      <c r="AG285">
+        <v>0</v>
+      </c>
+      <c r="AH285">
+        <v>3</v>
+      </c>
+      <c r="AI285">
+        <v>6039.77889</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B286" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E286">
+        <v>278.45</v>
+      </c>
+      <c r="F286">
+        <v>13490.93</v>
+      </c>
+      <c r="G286">
+        <v>48.45009876099839</v>
+      </c>
+      <c r="H286">
+        <v>213.87</v>
+      </c>
+      <c r="I286">
+        <v>0</v>
+      </c>
+      <c r="J286">
+        <v>0</v>
+      </c>
+      <c r="K286">
+        <v>0.7680732627042558</v>
+      </c>
+      <c r="L286">
+        <v>0</v>
+      </c>
+      <c r="M286">
+        <v>2</v>
+      </c>
+      <c r="N286">
+        <v>0</v>
+      </c>
+      <c r="O286">
+        <v>26.16713</v>
+      </c>
+      <c r="P286">
+        <v>76.99838159133709</v>
+      </c>
+      <c r="Q286">
+        <v>33.984</v>
+      </c>
+      <c r="R286">
+        <v>1748.62919</v>
+      </c>
+      <c r="S286">
+        <v>6.279867803914527</v>
+      </c>
+      <c r="T286">
+        <v>1772.23002</v>
+      </c>
+      <c r="U286">
+        <v>54</v>
+      </c>
+      <c r="V286">
+        <v>35</v>
+      </c>
+      <c r="W286">
+        <v>89</v>
+      </c>
+      <c r="X286">
+        <v>202</v>
+      </c>
+      <c r="Y286">
+        <v>54</v>
+      </c>
+      <c r="Z286">
+        <v>175</v>
+      </c>
+      <c r="AA286">
+        <v>35</v>
+      </c>
+      <c r="AB286">
+        <v>36</v>
+      </c>
+      <c r="AC286">
+        <v>4.47016</v>
+      </c>
+      <c r="AD286">
+        <v>-1.55112</v>
+      </c>
+      <c r="AE286">
+        <v>0</v>
+      </c>
+      <c r="AF286">
+        <v>1271.2608</v>
+      </c>
+      <c r="AG286">
+        <v>0</v>
+      </c>
+      <c r="AH286">
+        <v>3</v>
+      </c>
+      <c r="AI286">
+        <v>5245.887570000001</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B287" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E287">
+        <v>182.3833333333333</v>
+      </c>
+      <c r="F287">
+        <v>12326.39</v>
+      </c>
+      <c r="G287">
+        <v>67.58506808005117</v>
+      </c>
+      <c r="H287">
+        <v>426.76</v>
+      </c>
+      <c r="I287">
+        <v>0</v>
+      </c>
+      <c r="J287">
+        <v>0</v>
+      </c>
+      <c r="K287">
+        <v>2.339906789728594</v>
+      </c>
+      <c r="L287">
+        <v>2.23</v>
+      </c>
+      <c r="M287">
+        <v>10</v>
+      </c>
+      <c r="N287">
+        <v>0</v>
+      </c>
+      <c r="O287">
+        <v>30.24115</v>
+      </c>
+      <c r="P287">
+        <v>85.02347615834459</v>
+      </c>
+      <c r="Q287">
+        <v>35.568</v>
+      </c>
+      <c r="R287">
+        <v>1207.66266</v>
+      </c>
+      <c r="S287">
+        <v>6.621562606232295</v>
+      </c>
+      <c r="T287">
+        <v>2280.72002</v>
+      </c>
+      <c r="U287">
+        <v>79</v>
+      </c>
+      <c r="V287">
+        <v>56</v>
+      </c>
+      <c r="W287">
+        <v>135</v>
+      </c>
+      <c r="X287">
+        <v>220</v>
+      </c>
+      <c r="Y287">
+        <v>79</v>
+      </c>
+      <c r="Z287">
+        <v>174</v>
+      </c>
+      <c r="AA287">
+        <v>56</v>
+      </c>
+      <c r="AB287">
+        <v>32</v>
+      </c>
+      <c r="AC287">
+        <v>4.63916</v>
+      </c>
+      <c r="AD287">
+        <v>-1.68587</v>
+      </c>
+      <c r="AE287">
+        <v>0</v>
+      </c>
+      <c r="AF287">
+        <v>1199.38</v>
+      </c>
+      <c r="AG287">
+        <v>0</v>
+      </c>
+      <c r="AH287">
+        <v>3</v>
+      </c>
+      <c r="AI287">
+        <v>3622.98798</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B288" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E288">
+        <v>190.7833333333333</v>
+      </c>
+      <c r="F288">
+        <v>9135.68</v>
+      </c>
+      <c r="G288">
+        <v>47.88510526775575</v>
+      </c>
+      <c r="H288">
+        <v>126.37</v>
+      </c>
+      <c r="I288">
+        <v>0</v>
+      </c>
+      <c r="J288">
+        <v>0</v>
+      </c>
+      <c r="K288">
+        <v>0.6623744212457413</v>
+      </c>
+      <c r="L288">
+        <v>0</v>
+      </c>
+      <c r="M288">
+        <v>1</v>
+      </c>
+      <c r="N288">
+        <v>0</v>
+      </c>
+      <c r="O288">
+        <v>27.10994</v>
+      </c>
+      <c r="P288">
+        <v>75.30538888888888</v>
+      </c>
+      <c r="Q288">
+        <v>36</v>
+      </c>
+      <c r="R288">
+        <v>1063.48438</v>
+      </c>
+      <c r="S288">
+        <v>5.574304429108063</v>
+      </c>
+      <c r="T288">
+        <v>1248.97003</v>
+      </c>
+      <c r="U288">
+        <v>35</v>
+      </c>
+      <c r="V288">
+        <v>52</v>
+      </c>
+      <c r="W288">
+        <v>87</v>
+      </c>
+      <c r="X288">
+        <v>162</v>
+      </c>
+      <c r="Y288">
+        <v>35</v>
+      </c>
+      <c r="Z288">
+        <v>123</v>
+      </c>
+      <c r="AA288">
+        <v>52</v>
+      </c>
+      <c r="AB288">
+        <v>327</v>
+      </c>
+      <c r="AC288">
+        <v>3.91658</v>
+      </c>
+      <c r="AD288">
+        <v>-1.84711</v>
+      </c>
+      <c r="AE288">
+        <v>0</v>
+      </c>
+      <c r="AF288">
+        <v>768.6672</v>
+      </c>
+      <c r="AG288">
+        <v>0</v>
+      </c>
+      <c r="AH288">
+        <v>3</v>
+      </c>
+      <c r="AI288">
+        <v>3190.45314</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B289" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E289">
+        <v>278.45</v>
+      </c>
+      <c r="F289">
+        <v>13636.3</v>
+      </c>
+      <c r="G289">
+        <v>48.97216735500091</v>
+      </c>
+      <c r="H289">
+        <v>362.89</v>
+      </c>
+      <c r="I289">
+        <v>0</v>
+      </c>
+      <c r="J289">
+        <v>0</v>
+      </c>
+      <c r="K289">
+        <v>1.303250134674089</v>
+      </c>
+      <c r="L289">
+        <v>0</v>
+      </c>
+      <c r="M289">
+        <v>7</v>
+      </c>
+      <c r="N289">
+        <v>0</v>
+      </c>
+      <c r="O289">
+        <v>28.21624</v>
+      </c>
+      <c r="P289">
+        <v>88.1647294088239</v>
+      </c>
+      <c r="Q289">
+        <v>32.004</v>
+      </c>
+      <c r="R289">
+        <v>1607.11153</v>
+      </c>
+      <c r="S289">
+        <v>5.771634153348896</v>
+      </c>
+      <c r="T289">
+        <v>2200.42997</v>
+      </c>
+      <c r="U289">
+        <v>66</v>
+      </c>
+      <c r="V289">
+        <v>69</v>
+      </c>
+      <c r="W289">
+        <v>135</v>
+      </c>
+      <c r="X289">
+        <v>254</v>
+      </c>
+      <c r="Y289">
+        <v>66</v>
+      </c>
+      <c r="Z289">
+        <v>224</v>
+      </c>
+      <c r="AA289">
+        <v>69</v>
+      </c>
+      <c r="AB289">
+        <v>49</v>
+      </c>
+      <c r="AC289">
+        <v>4.29885</v>
+      </c>
+      <c r="AD289">
+        <v>-1.54091</v>
+      </c>
+      <c r="AE289">
+        <v>0</v>
+      </c>
+      <c r="AF289">
+        <v>982.3104000000001</v>
+      </c>
+      <c r="AG289">
+        <v>0</v>
+      </c>
+      <c r="AH289">
+        <v>3</v>
+      </c>
+      <c r="AI289">
+        <v>4821.334589999999</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B290" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E290">
+        <v>278.45</v>
+      </c>
+      <c r="F290">
+        <v>14757.29</v>
+      </c>
+      <c r="G290">
+        <v>52.997988866942</v>
+      </c>
+      <c r="H290">
+        <v>414.1</v>
+      </c>
+      <c r="I290">
+        <v>0</v>
+      </c>
+      <c r="J290">
+        <v>0</v>
+      </c>
+      <c r="K290">
+        <v>1.487161070210092</v>
+      </c>
+      <c r="L290">
+        <v>0</v>
+      </c>
+      <c r="M290">
+        <v>8</v>
+      </c>
+      <c r="N290">
+        <v>0</v>
+      </c>
+      <c r="O290">
+        <v>26.08549</v>
+      </c>
+      <c r="P290">
+        <v>77.08478132387707</v>
+      </c>
+      <c r="Q290">
+        <v>33.84</v>
+      </c>
+      <c r="R290">
+        <v>1626.78565</v>
+      </c>
+      <c r="S290">
+        <v>5.842289998204346</v>
+      </c>
+      <c r="T290">
+        <v>2533.60008</v>
+      </c>
+      <c r="U290">
+        <v>87</v>
+      </c>
+      <c r="V290">
+        <v>97</v>
+      </c>
+      <c r="W290">
+        <v>184</v>
+      </c>
+      <c r="X290">
+        <v>272</v>
+      </c>
+      <c r="Y290">
+        <v>87</v>
+      </c>
+      <c r="Z290">
+        <v>245</v>
+      </c>
+      <c r="AA290">
+        <v>97</v>
+      </c>
+      <c r="AB290">
+        <v>70</v>
+      </c>
+      <c r="AC290">
+        <v>4.41645</v>
+      </c>
+      <c r="AD290">
+        <v>-1.58803</v>
+      </c>
+      <c r="AE290">
+        <v>0</v>
+      </c>
+      <c r="AF290">
+        <v>1267.2415</v>
+      </c>
+      <c r="AG290">
+        <v>0</v>
+      </c>
+      <c r="AH290">
+        <v>3</v>
+      </c>
+      <c r="AI290">
+        <v>4880.35695</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B291" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E291">
+        <v>278.45</v>
+      </c>
+      <c r="F291">
+        <v>13381.19</v>
+      </c>
+      <c r="G291">
+        <v>48.0559885078111</v>
+      </c>
+      <c r="H291">
+        <v>168.13</v>
+      </c>
+      <c r="I291">
+        <v>0</v>
+      </c>
+      <c r="J291">
+        <v>0</v>
+      </c>
+      <c r="K291">
+        <v>0.6038067875740708</v>
+      </c>
+      <c r="L291">
+        <v>0</v>
+      </c>
+      <c r="M291">
+        <v>1</v>
+      </c>
+      <c r="N291">
+        <v>0</v>
+      </c>
+      <c r="O291">
+        <v>25.63968</v>
+      </c>
+      <c r="P291">
+        <v>76.0911680911681</v>
+      </c>
+      <c r="Q291">
+        <v>33.696</v>
+      </c>
+      <c r="R291">
+        <v>1440.77944</v>
+      </c>
+      <c r="S291">
+        <v>5.174284216196804</v>
+      </c>
+      <c r="T291">
+        <v>1901.09996</v>
+      </c>
+      <c r="U291">
+        <v>61</v>
+      </c>
+      <c r="V291">
+        <v>67</v>
+      </c>
+      <c r="W291">
+        <v>128</v>
+      </c>
+      <c r="X291">
+        <v>254</v>
+      </c>
+      <c r="Y291">
+        <v>61</v>
+      </c>
+      <c r="Z291">
+        <v>194</v>
+      </c>
+      <c r="AA291">
+        <v>67</v>
+      </c>
+      <c r="AB291">
+        <v>112</v>
+      </c>
+      <c r="AC291">
+        <v>4.5806</v>
+      </c>
+      <c r="AD291">
+        <v>-1.5989</v>
+      </c>
+      <c r="AE291">
+        <v>0</v>
+      </c>
+      <c r="AF291">
+        <v>1282.2672</v>
+      </c>
+      <c r="AG291">
+        <v>0</v>
+      </c>
+      <c r="AH291">
+        <v>3</v>
+      </c>
+      <c r="AI291">
+        <v>4322.33832</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B292" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E292">
+        <v>278.45</v>
+      </c>
+      <c r="F292">
+        <v>15101.73</v>
+      </c>
+      <c r="G292">
+        <v>54.23497934997307</v>
+      </c>
+      <c r="H292">
+        <v>372.13</v>
+      </c>
+      <c r="I292">
+        <v>0</v>
+      </c>
+      <c r="J292">
+        <v>0</v>
+      </c>
+      <c r="K292">
+        <v>1.336433830131083</v>
+      </c>
+      <c r="L292">
+        <v>0</v>
+      </c>
+      <c r="M292">
+        <v>6</v>
+      </c>
+      <c r="N292">
+        <v>0</v>
+      </c>
+      <c r="O292">
+        <v>26.33373</v>
+      </c>
+      <c r="P292">
+        <v>75.25643004115227</v>
+      </c>
+      <c r="Q292">
+        <v>34.992</v>
+      </c>
+      <c r="R292">
+        <v>1480.66133</v>
+      </c>
+      <c r="S292">
+        <v>5.317512407972706</v>
+      </c>
+      <c r="T292">
+        <v>2016.47996</v>
+      </c>
+      <c r="U292">
+        <v>61</v>
+      </c>
+      <c r="V292">
+        <v>67</v>
+      </c>
+      <c r="W292">
+        <v>128</v>
+      </c>
+      <c r="X292">
+        <v>229</v>
+      </c>
+      <c r="Y292">
+        <v>61</v>
+      </c>
+      <c r="Z292">
+        <v>182</v>
+      </c>
+      <c r="AA292">
+        <v>67</v>
+      </c>
+      <c r="AB292">
+        <v>90</v>
+      </c>
+      <c r="AC292">
+        <v>4.26246</v>
+      </c>
+      <c r="AD292">
+        <v>-1.23407</v>
+      </c>
+      <c r="AE292">
+        <v>0</v>
+      </c>
+      <c r="AF292">
+        <v>1228.98936</v>
+      </c>
+      <c r="AG292">
+        <v>0</v>
+      </c>
+      <c r="AH292">
+        <v>3</v>
+      </c>
+      <c r="AI292">
+        <v>4441.98399</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B293" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E293">
+        <v>278.45</v>
+      </c>
+      <c r="F293">
+        <v>14553.96</v>
+      </c>
+      <c r="G293">
+        <v>52.26776800143652</v>
+      </c>
+      <c r="H293">
+        <v>210.17</v>
+      </c>
+      <c r="I293">
+        <v>0</v>
+      </c>
+      <c r="J293">
+        <v>0</v>
+      </c>
+      <c r="K293">
+        <v>0.7547854192853295</v>
+      </c>
+      <c r="L293">
+        <v>0</v>
+      </c>
+      <c r="M293">
+        <v>0</v>
+      </c>
+      <c r="N293">
+        <v>0</v>
+      </c>
+      <c r="O293">
+        <v>25.12831</v>
+      </c>
+      <c r="P293">
+        <v>71.95965063001145</v>
+      </c>
+      <c r="Q293">
+        <v>34.92</v>
+      </c>
+      <c r="R293">
+        <v>1430.58387</v>
+      </c>
+      <c r="S293">
+        <v>5.137668773567966</v>
+      </c>
+      <c r="T293">
+        <v>2250.37004</v>
+      </c>
+      <c r="U293">
+        <v>78</v>
+      </c>
+      <c r="V293">
+        <v>63</v>
+      </c>
+      <c r="W293">
+        <v>141</v>
+      </c>
+      <c r="X293">
+        <v>269</v>
+      </c>
+      <c r="Y293">
+        <v>78</v>
+      </c>
+      <c r="Z293">
+        <v>235</v>
+      </c>
+      <c r="AA293">
+        <v>63</v>
+      </c>
+      <c r="AB293">
+        <v>84</v>
+      </c>
+      <c r="AC293">
+        <v>4.21585</v>
+      </c>
+      <c r="AD293">
+        <v>-1.54533</v>
+      </c>
+      <c r="AE293">
+        <v>0</v>
+      </c>
+      <c r="AF293">
+        <v>1403.2184</v>
+      </c>
+      <c r="AG293">
+        <v>0</v>
+      </c>
+      <c r="AH293">
+        <v>3</v>
+      </c>
+      <c r="AI293">
+        <v>4291.751609999999</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B294" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E294">
+        <v>278.45</v>
+      </c>
+      <c r="F294">
+        <v>15414.18</v>
+      </c>
+      <c r="G294">
+        <v>55.3570838570659</v>
+      </c>
+      <c r="H294">
+        <v>380.04</v>
+      </c>
+      <c r="I294">
+        <v>0</v>
+      </c>
+      <c r="J294">
+        <v>0</v>
+      </c>
+      <c r="K294">
+        <v>1.364841084575328</v>
+      </c>
+      <c r="L294">
+        <v>2.26</v>
+      </c>
+      <c r="M294">
+        <v>5</v>
+      </c>
+      <c r="N294">
+        <v>0</v>
+      </c>
+      <c r="O294">
+        <v>30.07799</v>
+      </c>
+      <c r="P294">
+        <v>85.95676154549612</v>
+      </c>
+      <c r="Q294">
+        <v>34.992</v>
+      </c>
+      <c r="R294">
+        <v>1512.00804</v>
+      </c>
+      <c r="S294">
+        <v>5.430088130723648</v>
+      </c>
+      <c r="T294">
+        <v>2822.51999</v>
+      </c>
+      <c r="U294">
+        <v>107</v>
+      </c>
+      <c r="V294">
+        <v>110</v>
+      </c>
+      <c r="W294">
+        <v>217</v>
+      </c>
+      <c r="X294">
+        <v>305</v>
+      </c>
+      <c r="Y294">
+        <v>107</v>
+      </c>
+      <c r="Z294">
+        <v>263</v>
+      </c>
+      <c r="AA294">
+        <v>110</v>
+      </c>
+      <c r="AB294">
+        <v>113</v>
+      </c>
+      <c r="AC294">
+        <v>4.75902</v>
+      </c>
+      <c r="AD294">
+        <v>-1.73813</v>
+      </c>
+      <c r="AE294">
+        <v>0</v>
+      </c>
+      <c r="AF294">
+        <v>1359.42919</v>
+      </c>
+      <c r="AG294">
+        <v>0</v>
+      </c>
+      <c r="AH294">
+        <v>3</v>
+      </c>
+      <c r="AI294">
+        <v>4536.02412</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B295" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E295">
+        <v>278.45</v>
+      </c>
+      <c r="F295">
+        <v>14041.96</v>
+      </c>
+      <c r="G295">
+        <v>50.42901777697971</v>
+      </c>
+      <c r="H295">
+        <v>318.3</v>
+      </c>
+      <c r="I295">
+        <v>0</v>
+      </c>
+      <c r="J295">
+        <v>0</v>
+      </c>
+      <c r="K295">
+        <v>1.143113664930867</v>
+      </c>
+      <c r="L295">
+        <v>0</v>
+      </c>
+      <c r="M295">
+        <v>3</v>
+      </c>
+      <c r="N295">
+        <v>0</v>
+      </c>
+      <c r="O295">
+        <v>26.28769</v>
+      </c>
+      <c r="P295">
+        <v>77.35313677024482</v>
+      </c>
+      <c r="Q295">
+        <v>33.984</v>
+      </c>
+      <c r="R295">
+        <v>1575.53174</v>
+      </c>
+      <c r="S295">
+        <v>5.658221368288741</v>
+      </c>
+      <c r="T295">
+        <v>2106.25996</v>
+      </c>
+      <c r="U295">
+        <v>54</v>
+      </c>
+      <c r="V295">
+        <v>72</v>
+      </c>
+      <c r="W295">
+        <v>126</v>
+      </c>
+      <c r="X295">
+        <v>209</v>
+      </c>
+      <c r="Y295">
+        <v>54</v>
+      </c>
+      <c r="Z295">
+        <v>219</v>
+      </c>
+      <c r="AA295">
+        <v>72</v>
+      </c>
+      <c r="AB295">
+        <v>190</v>
+      </c>
+      <c r="AC295">
+        <v>4.31611</v>
+      </c>
+      <c r="AD295">
+        <v>-2.01724</v>
+      </c>
+      <c r="AE295">
+        <v>0</v>
+      </c>
+      <c r="AF295">
+        <v>1351.5832</v>
+      </c>
+      <c r="AG295">
+        <v>0</v>
+      </c>
+      <c r="AH295">
+        <v>3</v>
+      </c>
+      <c r="AI295">
+        <v>4726.595219999999</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B296" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E296">
+        <v>278.45</v>
+      </c>
+      <c r="F296">
+        <v>14748.74</v>
+      </c>
+      <c r="G296">
+        <v>52.96728317471719</v>
+      </c>
+      <c r="H296">
+        <v>258.76</v>
+      </c>
+      <c r="I296">
+        <v>0</v>
+      </c>
+      <c r="J296">
+        <v>0</v>
+      </c>
+      <c r="K296">
+        <v>0.9292871251571198</v>
+      </c>
+      <c r="L296">
+        <v>0</v>
+      </c>
+      <c r="M296">
+        <v>1</v>
+      </c>
+      <c r="N296">
+        <v>0</v>
+      </c>
+      <c r="O296">
+        <v>25.26913</v>
+      </c>
+      <c r="P296">
+        <v>72.21402034750801</v>
+      </c>
+      <c r="Q296">
+        <v>34.992</v>
+      </c>
+      <c r="R296">
+        <v>1603.701</v>
+      </c>
+      <c r="S296">
+        <v>5.759385886155504</v>
+      </c>
+      <c r="T296">
+        <v>2382.35004</v>
+      </c>
+      <c r="U296">
+        <v>73</v>
+      </c>
+      <c r="V296">
+        <v>83</v>
+      </c>
+      <c r="W296">
+        <v>156</v>
+      </c>
+      <c r="X296">
+        <v>264</v>
+      </c>
+      <c r="Y296">
+        <v>73</v>
+      </c>
+      <c r="Z296">
+        <v>250</v>
+      </c>
+      <c r="AA296">
+        <v>83</v>
+      </c>
+      <c r="AB296">
+        <v>204</v>
+      </c>
+      <c r="AC296">
+        <v>4.0114</v>
+      </c>
+      <c r="AD296">
+        <v>-1.58858</v>
+      </c>
+      <c r="AE296">
+        <v>0</v>
+      </c>
+      <c r="AF296">
+        <v>1432.3232</v>
+      </c>
+      <c r="AG296">
+        <v>0</v>
+      </c>
+      <c r="AH296">
+        <v>3</v>
+      </c>
+      <c r="AI296">
+        <v>4811.103</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B297" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E297">
+        <v>278.45</v>
+      </c>
+      <c r="F297">
+        <v>13860.84</v>
+      </c>
+      <c r="G297">
+        <v>49.77855988507812</v>
+      </c>
+      <c r="H297">
+        <v>321.83</v>
+      </c>
+      <c r="I297">
+        <v>0</v>
+      </c>
+      <c r="J297">
+        <v>0</v>
+      </c>
+      <c r="K297">
+        <v>1.155790985814329</v>
+      </c>
+      <c r="L297">
+        <v>0</v>
+      </c>
+      <c r="M297">
+        <v>2</v>
+      </c>
+      <c r="N297">
+        <v>0</v>
+      </c>
+      <c r="O297">
+        <v>27.92416</v>
+      </c>
+      <c r="P297">
+        <v>84.58790742760208</v>
+      </c>
+      <c r="Q297">
+        <v>33.012</v>
+      </c>
+      <c r="R297">
+        <v>1534.60377</v>
+      </c>
+      <c r="S297">
+        <v>5.511236379960495</v>
+      </c>
+      <c r="T297">
+        <v>2308.75995</v>
+      </c>
+      <c r="U297">
+        <v>73</v>
+      </c>
+      <c r="V297">
+        <v>67</v>
+      </c>
+      <c r="W297">
+        <v>140</v>
+      </c>
+      <c r="X297">
+        <v>260</v>
+      </c>
+      <c r="Y297">
+        <v>73</v>
+      </c>
+      <c r="Z297">
+        <v>219</v>
+      </c>
+      <c r="AA297">
+        <v>67</v>
+      </c>
+      <c r="AB297">
+        <v>285</v>
+      </c>
+      <c r="AC297">
+        <v>4.58365</v>
+      </c>
+      <c r="AD297">
+        <v>-1.75198</v>
+      </c>
+      <c r="AE297">
+        <v>0</v>
+      </c>
+      <c r="AF297">
+        <v>1247.199</v>
+      </c>
+      <c r="AG297">
+        <v>0</v>
+      </c>
+      <c r="AH297">
+        <v>3</v>
+      </c>
+      <c r="AI297">
+        <v>4603.81131</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B298" s="2">
+        <v>46201</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Sesión 24 Pretemporada | Sesión 23 Pretemporada | Sesion 22 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E298">
+        <v>278.45</v>
+      </c>
+      <c r="F298">
+        <v>14725.61</v>
+      </c>
+      <c r="G298">
+        <v>52.88421619680373</v>
+      </c>
+      <c r="H298">
+        <v>156.04</v>
+      </c>
+      <c r="I298">
+        <v>0</v>
+      </c>
+      <c r="J298">
+        <v>0</v>
+      </c>
+      <c r="K298">
+        <v>0.5603878613754715</v>
+      </c>
+      <c r="L298">
+        <v>0</v>
+      </c>
+      <c r="M298">
+        <v>2</v>
+      </c>
+      <c r="N298">
+        <v>0</v>
+      </c>
+      <c r="O298">
+        <v>27.25827</v>
+      </c>
+      <c r="P298">
+        <v>85.17144731908512</v>
+      </c>
+      <c r="Q298">
+        <v>32.004</v>
+      </c>
+      <c r="R298">
+        <v>1565.06879</v>
+      </c>
+      <c r="S298">
+        <v>5.620645681450889</v>
+      </c>
+      <c r="T298">
+        <v>1926.41998</v>
+      </c>
+      <c r="U298">
+        <v>56</v>
+      </c>
+      <c r="V298">
+        <v>61</v>
+      </c>
+      <c r="W298">
+        <v>117</v>
+      </c>
+      <c r="X298">
+        <v>234</v>
+      </c>
+      <c r="Y298">
+        <v>56</v>
+      </c>
+      <c r="Z298">
+        <v>227</v>
+      </c>
+      <c r="AA298">
+        <v>61</v>
+      </c>
+      <c r="AB298">
+        <v>111</v>
+      </c>
+      <c r="AC298">
+        <v>4.07903</v>
+      </c>
+      <c r="AD298">
+        <v>-1.52172</v>
+      </c>
+      <c r="AE298">
+        <v>0</v>
+      </c>
+      <c r="AF298">
+        <v>1227.3695</v>
+      </c>
+      <c r="AG298">
+        <v>0</v>
+      </c>
+      <c r="AH298">
+        <v>3</v>
+      </c>
+      <c r="AI298">
+        <v>4695.20637</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-06-30
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI298"/>
+  <dimension ref="A1:AI313"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -34004,6 +34004,1701 @@
         <v>4695.20637</v>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B299" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E299">
+        <v>89.45</v>
+      </c>
+      <c r="F299">
+        <v>9230.719999999999</v>
+      </c>
+      <c r="G299">
+        <v>103.1941866964785</v>
+      </c>
+      <c r="H299">
+        <v>246.69</v>
+      </c>
+      <c r="I299">
+        <v>0</v>
+      </c>
+      <c r="J299">
+        <v>0</v>
+      </c>
+      <c r="K299">
+        <v>2.757853549468977</v>
+      </c>
+      <c r="L299">
+        <v>0</v>
+      </c>
+      <c r="M299">
+        <v>3</v>
+      </c>
+      <c r="N299">
+        <v>0</v>
+      </c>
+      <c r="O299">
+        <v>28.1236</v>
+      </c>
+      <c r="P299">
+        <v>86.89778766530713</v>
+      </c>
+      <c r="Q299">
+        <v>32.364</v>
+      </c>
+      <c r="R299">
+        <v>921.86371</v>
+      </c>
+      <c r="S299">
+        <v>10.30591067635551</v>
+      </c>
+      <c r="T299">
+        <v>1158.47003</v>
+      </c>
+      <c r="U299">
+        <v>8</v>
+      </c>
+      <c r="V299">
+        <v>10</v>
+      </c>
+      <c r="W299">
+        <v>18</v>
+      </c>
+      <c r="X299">
+        <v>75</v>
+      </c>
+      <c r="Y299">
+        <v>8</v>
+      </c>
+      <c r="Z299">
+        <v>49</v>
+      </c>
+      <c r="AA299">
+        <v>10</v>
+      </c>
+      <c r="AB299">
+        <v>11</v>
+      </c>
+      <c r="AC299">
+        <v>4.10311</v>
+      </c>
+      <c r="AD299">
+        <v>-2.0551</v>
+      </c>
+      <c r="AE299">
+        <v>0</v>
+      </c>
+      <c r="AF299">
+        <v>736.5953000000001</v>
+      </c>
+      <c r="AG299">
+        <v>0</v>
+      </c>
+      <c r="AH299">
+        <v>3</v>
+      </c>
+      <c r="AI299">
+        <v>2765.59113</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B300" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E300">
+        <v>89.45</v>
+      </c>
+      <c r="F300">
+        <v>8979.17</v>
+      </c>
+      <c r="G300">
+        <v>100.382001117943</v>
+      </c>
+      <c r="H300">
+        <v>457.19</v>
+      </c>
+      <c r="I300">
+        <v>0</v>
+      </c>
+      <c r="J300">
+        <v>0</v>
+      </c>
+      <c r="K300">
+        <v>5.111123532699832</v>
+      </c>
+      <c r="L300">
+        <v>0</v>
+      </c>
+      <c r="M300">
+        <v>6</v>
+      </c>
+      <c r="N300">
+        <v>0</v>
+      </c>
+      <c r="O300">
+        <v>26.91157</v>
+      </c>
+      <c r="P300">
+        <v>83.06040123456791</v>
+      </c>
+      <c r="Q300">
+        <v>32.4</v>
+      </c>
+      <c r="R300">
+        <v>1067.82102</v>
+      </c>
+      <c r="S300">
+        <v>11.93763018446059</v>
+      </c>
+      <c r="T300">
+        <v>1733.09002</v>
+      </c>
+      <c r="U300">
+        <v>30</v>
+      </c>
+      <c r="V300">
+        <v>30</v>
+      </c>
+      <c r="W300">
+        <v>60</v>
+      </c>
+      <c r="X300">
+        <v>116</v>
+      </c>
+      <c r="Y300">
+        <v>30</v>
+      </c>
+      <c r="Z300">
+        <v>98</v>
+      </c>
+      <c r="AA300">
+        <v>30</v>
+      </c>
+      <c r="AB300">
+        <v>16</v>
+      </c>
+      <c r="AC300">
+        <v>4.37763</v>
+      </c>
+      <c r="AD300">
+        <v>-3.47698</v>
+      </c>
+      <c r="AE300">
+        <v>0</v>
+      </c>
+      <c r="AF300">
+        <v>745.1486</v>
+      </c>
+      <c r="AG300">
+        <v>0</v>
+      </c>
+      <c r="AH300">
+        <v>3</v>
+      </c>
+      <c r="AI300">
+        <v>3203.46306</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B301" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E301">
+        <v>89.45</v>
+      </c>
+      <c r="F301">
+        <v>7451.75</v>
+      </c>
+      <c r="G301">
+        <v>83.30631637786473</v>
+      </c>
+      <c r="H301">
+        <v>501.08</v>
+      </c>
+      <c r="I301">
+        <v>8.44</v>
+      </c>
+      <c r="J301">
+        <v>1</v>
+      </c>
+      <c r="K301">
+        <v>5.601788708775852</v>
+      </c>
+      <c r="L301">
+        <v>13.43</v>
+      </c>
+      <c r="M301">
+        <v>13</v>
+      </c>
+      <c r="N301">
+        <v>1</v>
+      </c>
+      <c r="O301">
+        <v>31.36284</v>
+      </c>
+      <c r="P301">
+        <v>92.28707627118644</v>
+      </c>
+      <c r="Q301">
+        <v>33.984</v>
+      </c>
+      <c r="R301">
+        <v>865.9964</v>
+      </c>
+      <c r="S301">
+        <v>9.681346003353829</v>
+      </c>
+      <c r="T301">
+        <v>1135.14</v>
+      </c>
+      <c r="U301">
+        <v>11</v>
+      </c>
+      <c r="V301">
+        <v>15</v>
+      </c>
+      <c r="W301">
+        <v>26</v>
+      </c>
+      <c r="X301">
+        <v>69</v>
+      </c>
+      <c r="Y301">
+        <v>11</v>
+      </c>
+      <c r="Z301">
+        <v>64</v>
+      </c>
+      <c r="AA301">
+        <v>15</v>
+      </c>
+      <c r="AB301">
+        <v>9</v>
+      </c>
+      <c r="AC301">
+        <v>4.41787</v>
+      </c>
+      <c r="AD301">
+        <v>-2.57609</v>
+      </c>
+      <c r="AE301">
+        <v>0</v>
+      </c>
+      <c r="AF301">
+        <v>691.1544</v>
+      </c>
+      <c r="AG301">
+        <v>0</v>
+      </c>
+      <c r="AH301">
+        <v>3</v>
+      </c>
+      <c r="AI301">
+        <v>2597.9892</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B302" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E302">
+        <v>89.45</v>
+      </c>
+      <c r="F302">
+        <v>8697.93</v>
+      </c>
+      <c r="G302">
+        <v>97.23789826718837</v>
+      </c>
+      <c r="H302">
+        <v>619.0799999999999</v>
+      </c>
+      <c r="I302">
+        <v>6.899999999999999</v>
+      </c>
+      <c r="J302">
+        <v>1</v>
+      </c>
+      <c r="K302">
+        <v>6.92096143096702</v>
+      </c>
+      <c r="L302">
+        <v>26.25</v>
+      </c>
+      <c r="M302">
+        <v>14</v>
+      </c>
+      <c r="N302">
+        <v>2</v>
+      </c>
+      <c r="O302">
+        <v>32.5241</v>
+      </c>
+      <c r="P302">
+        <v>91.44202654071076</v>
+      </c>
+      <c r="Q302">
+        <v>35.568</v>
+      </c>
+      <c r="R302">
+        <v>785.44357</v>
+      </c>
+      <c r="S302">
+        <v>8.780811291224147</v>
+      </c>
+      <c r="T302">
+        <v>1397.44999</v>
+      </c>
+      <c r="U302">
+        <v>27</v>
+      </c>
+      <c r="V302">
+        <v>15</v>
+      </c>
+      <c r="W302">
+        <v>42</v>
+      </c>
+      <c r="X302">
+        <v>95</v>
+      </c>
+      <c r="Y302">
+        <v>27</v>
+      </c>
+      <c r="Z302">
+        <v>68</v>
+      </c>
+      <c r="AA302">
+        <v>15</v>
+      </c>
+      <c r="AB302">
+        <v>6</v>
+      </c>
+      <c r="AC302">
+        <v>4.39544</v>
+      </c>
+      <c r="AD302">
+        <v>-2.14203</v>
+      </c>
+      <c r="AE302">
+        <v>0</v>
+      </c>
+      <c r="AF302">
+        <v>814.328</v>
+      </c>
+      <c r="AG302">
+        <v>0</v>
+      </c>
+      <c r="AH302">
+        <v>3</v>
+      </c>
+      <c r="AI302">
+        <v>2356.33071</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B303" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E303">
+        <v>89.45</v>
+      </c>
+      <c r="F303">
+        <v>8386.75</v>
+      </c>
+      <c r="G303">
+        <v>93.75908328675237</v>
+      </c>
+      <c r="H303">
+        <v>616.9800000000001</v>
+      </c>
+      <c r="I303">
+        <v>0</v>
+      </c>
+      <c r="J303">
+        <v>0</v>
+      </c>
+      <c r="K303">
+        <v>6.897484628283959</v>
+      </c>
+      <c r="L303">
+        <v>56.62</v>
+      </c>
+      <c r="M303">
+        <v>15</v>
+      </c>
+      <c r="N303">
+        <v>2</v>
+      </c>
+      <c r="O303">
+        <v>31.8516</v>
+      </c>
+      <c r="P303">
+        <v>88.47666666666667</v>
+      </c>
+      <c r="Q303">
+        <v>36</v>
+      </c>
+      <c r="R303">
+        <v>770.3845</v>
+      </c>
+      <c r="S303">
+        <v>8.612459474566798</v>
+      </c>
+      <c r="T303">
+        <v>1352.66001</v>
+      </c>
+      <c r="U303">
+        <v>22</v>
+      </c>
+      <c r="V303">
+        <v>28</v>
+      </c>
+      <c r="W303">
+        <v>50</v>
+      </c>
+      <c r="X303">
+        <v>81</v>
+      </c>
+      <c r="Y303">
+        <v>22</v>
+      </c>
+      <c r="Z303">
+        <v>71</v>
+      </c>
+      <c r="AA303">
+        <v>28</v>
+      </c>
+      <c r="AB303">
+        <v>24</v>
+      </c>
+      <c r="AC303">
+        <v>4.0927</v>
+      </c>
+      <c r="AD303">
+        <v>-3.35756</v>
+      </c>
+      <c r="AE303">
+        <v>0</v>
+      </c>
+      <c r="AF303">
+        <v>688.1658</v>
+      </c>
+      <c r="AG303">
+        <v>0</v>
+      </c>
+      <c r="AH303">
+        <v>3</v>
+      </c>
+      <c r="AI303">
+        <v>2311.1535</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B304" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E304">
+        <v>89.45</v>
+      </c>
+      <c r="F304">
+        <v>8178.54</v>
+      </c>
+      <c r="G304">
+        <v>91.43141419787591</v>
+      </c>
+      <c r="H304">
+        <v>424.79</v>
+      </c>
+      <c r="I304">
+        <v>0</v>
+      </c>
+      <c r="J304">
+        <v>0</v>
+      </c>
+      <c r="K304">
+        <v>4.748910005589715</v>
+      </c>
+      <c r="L304">
+        <v>0</v>
+      </c>
+      <c r="M304">
+        <v>6</v>
+      </c>
+      <c r="N304">
+        <v>0</v>
+      </c>
+      <c r="O304">
+        <v>27.95949</v>
+      </c>
+      <c r="P304">
+        <v>87.3624859392576</v>
+      </c>
+      <c r="Q304">
+        <v>32.004</v>
+      </c>
+      <c r="R304">
+        <v>926.38633</v>
+      </c>
+      <c r="S304">
+        <v>10.35647098937954</v>
+      </c>
+      <c r="T304">
+        <v>1312.54</v>
+      </c>
+      <c r="U304">
+        <v>16</v>
+      </c>
+      <c r="V304">
+        <v>18</v>
+      </c>
+      <c r="W304">
+        <v>34</v>
+      </c>
+      <c r="X304">
+        <v>79</v>
+      </c>
+      <c r="Y304">
+        <v>16</v>
+      </c>
+      <c r="Z304">
+        <v>81</v>
+      </c>
+      <c r="AA304">
+        <v>18</v>
+      </c>
+      <c r="AB304">
+        <v>12</v>
+      </c>
+      <c r="AC304">
+        <v>4.06346</v>
+      </c>
+      <c r="AD304">
+        <v>-4.00854</v>
+      </c>
+      <c r="AE304">
+        <v>0</v>
+      </c>
+      <c r="AF304">
+        <v>572.8128</v>
+      </c>
+      <c r="AG304">
+        <v>0</v>
+      </c>
+      <c r="AH304">
+        <v>3</v>
+      </c>
+      <c r="AI304">
+        <v>2779.15899</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B305" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E305">
+        <v>89.45</v>
+      </c>
+      <c r="F305">
+        <v>4493.389999999999</v>
+      </c>
+      <c r="G305">
+        <v>50.23353828954723</v>
+      </c>
+      <c r="H305">
+        <v>190.68</v>
+      </c>
+      <c r="I305">
+        <v>0</v>
+      </c>
+      <c r="J305">
+        <v>0</v>
+      </c>
+      <c r="K305">
+        <v>2.131693683622135</v>
+      </c>
+      <c r="L305">
+        <v>9.979999999999999</v>
+      </c>
+      <c r="M305">
+        <v>4</v>
+      </c>
+      <c r="N305">
+        <v>1</v>
+      </c>
+      <c r="O305">
+        <v>30.20726</v>
+      </c>
+      <c r="P305">
+        <v>89.26495271867611</v>
+      </c>
+      <c r="Q305">
+        <v>33.84</v>
+      </c>
+      <c r="R305">
+        <v>469.54419</v>
+      </c>
+      <c r="S305">
+        <v>5.249236333147008</v>
+      </c>
+      <c r="T305">
+        <v>593.03999</v>
+      </c>
+      <c r="U305">
+        <v>13</v>
+      </c>
+      <c r="V305">
+        <v>20</v>
+      </c>
+      <c r="W305">
+        <v>33</v>
+      </c>
+      <c r="X305">
+        <v>51</v>
+      </c>
+      <c r="Y305">
+        <v>13</v>
+      </c>
+      <c r="Z305">
+        <v>44</v>
+      </c>
+      <c r="AA305">
+        <v>20</v>
+      </c>
+      <c r="AB305">
+        <v>9</v>
+      </c>
+      <c r="AC305">
+        <v>4.21237</v>
+      </c>
+      <c r="AD305">
+        <v>0</v>
+      </c>
+      <c r="AE305">
+        <v>0</v>
+      </c>
+      <c r="AF305">
+        <v>367.9144</v>
+      </c>
+      <c r="AG305">
+        <v>0</v>
+      </c>
+      <c r="AH305">
+        <v>3</v>
+      </c>
+      <c r="AI305">
+        <v>1408.63257</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B306" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E306">
+        <v>89.45</v>
+      </c>
+      <c r="F306">
+        <v>6122.920000000001</v>
+      </c>
+      <c r="G306">
+        <v>68.45075461151482</v>
+      </c>
+      <c r="H306">
+        <v>221.46</v>
+      </c>
+      <c r="I306">
+        <v>0</v>
+      </c>
+      <c r="J306">
+        <v>0</v>
+      </c>
+      <c r="K306">
+        <v>2.475796534376746</v>
+      </c>
+      <c r="L306">
+        <v>0</v>
+      </c>
+      <c r="M306">
+        <v>3</v>
+      </c>
+      <c r="N306">
+        <v>0</v>
+      </c>
+      <c r="O306">
+        <v>27.83365</v>
+      </c>
+      <c r="P306">
+        <v>82.60223765432099</v>
+      </c>
+      <c r="Q306">
+        <v>33.696</v>
+      </c>
+      <c r="R306">
+        <v>610.79884</v>
+      </c>
+      <c r="S306">
+        <v>6.828382783678033</v>
+      </c>
+      <c r="T306">
+        <v>951.67002</v>
+      </c>
+      <c r="U306">
+        <v>18</v>
+      </c>
+      <c r="V306">
+        <v>20</v>
+      </c>
+      <c r="W306">
+        <v>38</v>
+      </c>
+      <c r="X306">
+        <v>77</v>
+      </c>
+      <c r="Y306">
+        <v>18</v>
+      </c>
+      <c r="Z306">
+        <v>71</v>
+      </c>
+      <c r="AA306">
+        <v>20</v>
+      </c>
+      <c r="AB306">
+        <v>14</v>
+      </c>
+      <c r="AC306">
+        <v>4.06664</v>
+      </c>
+      <c r="AD306">
+        <v>-2.98604</v>
+      </c>
+      <c r="AE306">
+        <v>0</v>
+      </c>
+      <c r="AF306">
+        <v>579.396</v>
+      </c>
+      <c r="AG306">
+        <v>0</v>
+      </c>
+      <c r="AH306">
+        <v>3</v>
+      </c>
+      <c r="AI306">
+        <v>1832.39652</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B307" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E307">
+        <v>89.45</v>
+      </c>
+      <c r="F307">
+        <v>8483.41</v>
+      </c>
+      <c r="G307">
+        <v>94.83968697596423</v>
+      </c>
+      <c r="H307">
+        <v>507.09</v>
+      </c>
+      <c r="I307">
+        <v>5.92</v>
+      </c>
+      <c r="J307">
+        <v>0</v>
+      </c>
+      <c r="K307">
+        <v>5.668977082168809</v>
+      </c>
+      <c r="L307">
+        <v>41</v>
+      </c>
+      <c r="M307">
+        <v>13</v>
+      </c>
+      <c r="N307">
+        <v>3</v>
+      </c>
+      <c r="O307">
+        <v>31.64946</v>
+      </c>
+      <c r="P307">
+        <v>90.44770233196159</v>
+      </c>
+      <c r="Q307">
+        <v>34.992</v>
+      </c>
+      <c r="R307">
+        <v>739.26504</v>
+      </c>
+      <c r="S307">
+        <v>8.264561654555617</v>
+      </c>
+      <c r="T307">
+        <v>1135.34997</v>
+      </c>
+      <c r="U307">
+        <v>21</v>
+      </c>
+      <c r="V307">
+        <v>17</v>
+      </c>
+      <c r="W307">
+        <v>38</v>
+      </c>
+      <c r="X307">
+        <v>69</v>
+      </c>
+      <c r="Y307">
+        <v>21</v>
+      </c>
+      <c r="Z307">
+        <v>57</v>
+      </c>
+      <c r="AA307">
+        <v>17</v>
+      </c>
+      <c r="AB307">
+        <v>11</v>
+      </c>
+      <c r="AC307">
+        <v>3.82277</v>
+      </c>
+      <c r="AD307">
+        <v>-2.34778</v>
+      </c>
+      <c r="AE307">
+        <v>0</v>
+      </c>
+      <c r="AF307">
+        <v>674.14242</v>
+      </c>
+      <c r="AG307">
+        <v>0</v>
+      </c>
+      <c r="AH307">
+        <v>3</v>
+      </c>
+      <c r="AI307">
+        <v>2217.79512</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B308" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E308">
+        <v>89.45</v>
+      </c>
+      <c r="F308">
+        <v>6578.599999999999</v>
+      </c>
+      <c r="G308">
+        <v>73.54499720514254</v>
+      </c>
+      <c r="H308">
+        <v>335.5</v>
+      </c>
+      <c r="I308">
+        <v>6.850000000000001</v>
+      </c>
+      <c r="J308">
+        <v>0</v>
+      </c>
+      <c r="K308">
+        <v>3.750698714365567</v>
+      </c>
+      <c r="L308">
+        <v>15.93</v>
+      </c>
+      <c r="M308">
+        <v>9</v>
+      </c>
+      <c r="N308">
+        <v>1</v>
+      </c>
+      <c r="O308">
+        <v>31.43712</v>
+      </c>
+      <c r="P308">
+        <v>90.02611683848797</v>
+      </c>
+      <c r="Q308">
+        <v>34.92</v>
+      </c>
+      <c r="R308">
+        <v>512.94678</v>
+      </c>
+      <c r="S308">
+        <v>5.73445254332029</v>
+      </c>
+      <c r="T308">
+        <v>891.0699999999999</v>
+      </c>
+      <c r="U308">
+        <v>24</v>
+      </c>
+      <c r="V308">
+        <v>13</v>
+      </c>
+      <c r="W308">
+        <v>37</v>
+      </c>
+      <c r="X308">
+        <v>56</v>
+      </c>
+      <c r="Y308">
+        <v>24</v>
+      </c>
+      <c r="Z308">
+        <v>46</v>
+      </c>
+      <c r="AA308">
+        <v>13</v>
+      </c>
+      <c r="AB308">
+        <v>6</v>
+      </c>
+      <c r="AC308">
+        <v>4.61106</v>
+      </c>
+      <c r="AD308">
+        <v>-2.43599</v>
+      </c>
+      <c r="AE308">
+        <v>0</v>
+      </c>
+      <c r="AF308">
+        <v>610.0392000000001</v>
+      </c>
+      <c r="AG308">
+        <v>0</v>
+      </c>
+      <c r="AH308">
+        <v>3</v>
+      </c>
+      <c r="AI308">
+        <v>1538.84034</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B309" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E309">
+        <v>89.45</v>
+      </c>
+      <c r="F309">
+        <v>7871.570000000001</v>
+      </c>
+      <c r="G309">
+        <v>87.99966461710453</v>
+      </c>
+      <c r="H309">
+        <v>355.59</v>
+      </c>
+      <c r="I309">
+        <v>0</v>
+      </c>
+      <c r="J309">
+        <v>0</v>
+      </c>
+      <c r="K309">
+        <v>3.975293460033539</v>
+      </c>
+      <c r="L309">
+        <v>0</v>
+      </c>
+      <c r="M309">
+        <v>4</v>
+      </c>
+      <c r="N309">
+        <v>0</v>
+      </c>
+      <c r="O309">
+        <v>28.60437</v>
+      </c>
+      <c r="P309">
+        <v>81.7454561042524</v>
+      </c>
+      <c r="Q309">
+        <v>34.992</v>
+      </c>
+      <c r="R309">
+        <v>646.6133</v>
+      </c>
+      <c r="S309">
+        <v>7.228768026830632</v>
+      </c>
+      <c r="T309">
+        <v>1199.50999</v>
+      </c>
+      <c r="U309">
+        <v>16</v>
+      </c>
+      <c r="V309">
+        <v>31</v>
+      </c>
+      <c r="W309">
+        <v>47</v>
+      </c>
+      <c r="X309">
+        <v>77</v>
+      </c>
+      <c r="Y309">
+        <v>16</v>
+      </c>
+      <c r="Z309">
+        <v>86</v>
+      </c>
+      <c r="AA309">
+        <v>31</v>
+      </c>
+      <c r="AB309">
+        <v>19</v>
+      </c>
+      <c r="AC309">
+        <v>4.08383</v>
+      </c>
+      <c r="AD309">
+        <v>-4.20531</v>
+      </c>
+      <c r="AE309">
+        <v>0</v>
+      </c>
+      <c r="AF309">
+        <v>660.11114</v>
+      </c>
+      <c r="AG309">
+        <v>0</v>
+      </c>
+      <c r="AH309">
+        <v>3</v>
+      </c>
+      <c r="AI309">
+        <v>1939.8399</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B310" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E310">
+        <v>89.45</v>
+      </c>
+      <c r="F310">
+        <v>7573.82</v>
+      </c>
+      <c r="G310">
+        <v>84.67098937954164</v>
+      </c>
+      <c r="H310">
+        <v>216.84</v>
+      </c>
+      <c r="I310">
+        <v>0</v>
+      </c>
+      <c r="J310">
+        <v>0</v>
+      </c>
+      <c r="K310">
+        <v>2.424147568474008</v>
+      </c>
+      <c r="L310">
+        <v>0</v>
+      </c>
+      <c r="M310">
+        <v>3</v>
+      </c>
+      <c r="N310">
+        <v>0</v>
+      </c>
+      <c r="O310">
+        <v>27.99866</v>
+      </c>
+      <c r="P310">
+        <v>82.38777071563088</v>
+      </c>
+      <c r="Q310">
+        <v>33.984</v>
+      </c>
+      <c r="R310">
+        <v>743.91733</v>
+      </c>
+      <c r="S310">
+        <v>8.316571604248184</v>
+      </c>
+      <c r="T310">
+        <v>903.22998</v>
+      </c>
+      <c r="U310">
+        <v>9</v>
+      </c>
+      <c r="V310">
+        <v>18</v>
+      </c>
+      <c r="W310">
+        <v>27</v>
+      </c>
+      <c r="X310">
+        <v>50</v>
+      </c>
+      <c r="Y310">
+        <v>9</v>
+      </c>
+      <c r="Z310">
+        <v>57</v>
+      </c>
+      <c r="AA310">
+        <v>18</v>
+      </c>
+      <c r="AB310">
+        <v>19</v>
+      </c>
+      <c r="AC310">
+        <v>3.8918</v>
+      </c>
+      <c r="AD310">
+        <v>-2.7641</v>
+      </c>
+      <c r="AE310">
+        <v>0</v>
+      </c>
+      <c r="AF310">
+        <v>694.2008000000001</v>
+      </c>
+      <c r="AG310">
+        <v>0</v>
+      </c>
+      <c r="AH310">
+        <v>3</v>
+      </c>
+      <c r="AI310">
+        <v>2231.75199</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B311" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E311">
+        <v>89.45</v>
+      </c>
+      <c r="F311">
+        <v>8068.339999999999</v>
+      </c>
+      <c r="G311">
+        <v>90.19944102850754</v>
+      </c>
+      <c r="H311">
+        <v>97.41999999999999</v>
+      </c>
+      <c r="I311">
+        <v>0</v>
+      </c>
+      <c r="J311">
+        <v>0</v>
+      </c>
+      <c r="K311">
+        <v>1.089100055897149</v>
+      </c>
+      <c r="L311">
+        <v>0</v>
+      </c>
+      <c r="M311">
+        <v>2</v>
+      </c>
+      <c r="N311">
+        <v>0</v>
+      </c>
+      <c r="O311">
+        <v>26.37926</v>
+      </c>
+      <c r="P311">
+        <v>75.3865454961134</v>
+      </c>
+      <c r="Q311">
+        <v>34.992</v>
+      </c>
+      <c r="R311">
+        <v>719.70307</v>
+      </c>
+      <c r="S311">
+        <v>8.045869983230855</v>
+      </c>
+      <c r="T311">
+        <v>958.4100100000001</v>
+      </c>
+      <c r="U311">
+        <v>5</v>
+      </c>
+      <c r="V311">
+        <v>14</v>
+      </c>
+      <c r="W311">
+        <v>19</v>
+      </c>
+      <c r="X311">
+        <v>60</v>
+      </c>
+      <c r="Y311">
+        <v>5</v>
+      </c>
+      <c r="Z311">
+        <v>69</v>
+      </c>
+      <c r="AA311">
+        <v>14</v>
+      </c>
+      <c r="AB311">
+        <v>10</v>
+      </c>
+      <c r="AC311">
+        <v>3.14991</v>
+      </c>
+      <c r="AD311">
+        <v>-3.10475</v>
+      </c>
+      <c r="AE311">
+        <v>0</v>
+      </c>
+      <c r="AF311">
+        <v>737.124</v>
+      </c>
+      <c r="AG311">
+        <v>0</v>
+      </c>
+      <c r="AH311">
+        <v>3</v>
+      </c>
+      <c r="AI311">
+        <v>2159.10921</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B312" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E312">
+        <v>89.45</v>
+      </c>
+      <c r="F312">
+        <v>6995.38</v>
+      </c>
+      <c r="G312">
+        <v>78.20435997764113</v>
+      </c>
+      <c r="H312">
+        <v>225.43</v>
+      </c>
+      <c r="I312">
+        <v>0</v>
+      </c>
+      <c r="J312">
+        <v>0</v>
+      </c>
+      <c r="K312">
+        <v>2.520178870877585</v>
+      </c>
+      <c r="L312">
+        <v>0</v>
+      </c>
+      <c r="M312">
+        <v>2</v>
+      </c>
+      <c r="N312">
+        <v>0</v>
+      </c>
+      <c r="O312">
+        <v>26.778</v>
+      </c>
+      <c r="P312">
+        <v>81.11595783351508</v>
+      </c>
+      <c r="Q312">
+        <v>33.012</v>
+      </c>
+      <c r="R312">
+        <v>667.06282</v>
+      </c>
+      <c r="S312">
+        <v>7.457382001117943</v>
+      </c>
+      <c r="T312">
+        <v>788.37</v>
+      </c>
+      <c r="U312">
+        <v>13</v>
+      </c>
+      <c r="V312">
+        <v>11</v>
+      </c>
+      <c r="W312">
+        <v>24</v>
+      </c>
+      <c r="X312">
+        <v>50</v>
+      </c>
+      <c r="Y312">
+        <v>13</v>
+      </c>
+      <c r="Z312">
+        <v>46</v>
+      </c>
+      <c r="AA312">
+        <v>11</v>
+      </c>
+      <c r="AB312">
+        <v>10</v>
+      </c>
+      <c r="AC312">
+        <v>4.27284</v>
+      </c>
+      <c r="AD312">
+        <v>-2.00256</v>
+      </c>
+      <c r="AE312">
+        <v>0</v>
+      </c>
+      <c r="AF312">
+        <v>598.455</v>
+      </c>
+      <c r="AG312">
+        <v>0</v>
+      </c>
+      <c r="AH312">
+        <v>3</v>
+      </c>
+      <c r="AI312">
+        <v>2001.18846</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B313" s="2">
+        <v>46202</v>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Sesión 25 Pretemporada</t>
+        </is>
+      </c>
+      <c r="E313">
+        <v>89.45</v>
+      </c>
+      <c r="F313">
+        <v>7339.15</v>
+      </c>
+      <c r="G313">
+        <v>82.04751257685858</v>
+      </c>
+      <c r="H313">
+        <v>240.05</v>
+      </c>
+      <c r="I313">
+        <v>0</v>
+      </c>
+      <c r="J313">
+        <v>0</v>
+      </c>
+      <c r="K313">
+        <v>2.683622135271101</v>
+      </c>
+      <c r="L313">
+        <v>0</v>
+      </c>
+      <c r="M313">
+        <v>6</v>
+      </c>
+      <c r="N313">
+        <v>0</v>
+      </c>
+      <c r="O313">
+        <v>27.84367</v>
+      </c>
+      <c r="P313">
+        <v>87.00059367579053</v>
+      </c>
+      <c r="Q313">
+        <v>32.004</v>
+      </c>
+      <c r="R313">
+        <v>639.37168</v>
+      </c>
+      <c r="S313">
+        <v>7.147810844046953</v>
+      </c>
+      <c r="T313">
+        <v>843.13</v>
+      </c>
+      <c r="U313">
+        <v>9</v>
+      </c>
+      <c r="V313">
+        <v>8</v>
+      </c>
+      <c r="W313">
+        <v>17</v>
+      </c>
+      <c r="X313">
+        <v>63</v>
+      </c>
+      <c r="Y313">
+        <v>9</v>
+      </c>
+      <c r="Z313">
+        <v>53</v>
+      </c>
+      <c r="AA313">
+        <v>8</v>
+      </c>
+      <c r="AB313">
+        <v>12</v>
+      </c>
+      <c r="AC313">
+        <v>3.61773</v>
+      </c>
+      <c r="AD313">
+        <v>-2.40024</v>
+      </c>
+      <c r="AE313">
+        <v>0</v>
+      </c>
+      <c r="AF313">
+        <v>585.4548</v>
+      </c>
+      <c r="AG313">
+        <v>0</v>
+      </c>
+      <c r="AH313">
+        <v>3</v>
+      </c>
+      <c r="AI313">
+        <v>1918.11504</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-06
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI347"/>
+  <dimension ref="A1:AI362"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -39456,6 +39456,1696 @@
         <v>1026.84138</v>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B348" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E348">
+        <v>305.0515</v>
+      </c>
+      <c r="F348">
+        <v>21952.84</v>
+      </c>
+      <c r="G348">
+        <v>71.96437322878269</v>
+      </c>
+      <c r="H348">
+        <v>455.54</v>
+      </c>
+      <c r="I348">
+        <v>0</v>
+      </c>
+      <c r="J348">
+        <v>0</v>
+      </c>
+      <c r="K348">
+        <v>1.493321619464255</v>
+      </c>
+      <c r="L348">
+        <v>0</v>
+      </c>
+      <c r="M348">
+        <v>4</v>
+      </c>
+      <c r="N348">
+        <v>0</v>
+      </c>
+      <c r="O348">
+        <v>25.94925</v>
+      </c>
+      <c r="P348">
+        <v>80.1793659621802</v>
+      </c>
+      <c r="Q348">
+        <v>32.364</v>
+      </c>
+      <c r="R348">
+        <v>2162.76354</v>
+      </c>
+      <c r="S348">
+        <v>7.089830864624498</v>
+      </c>
+      <c r="T348">
+        <v>2903.72992</v>
+      </c>
+      <c r="U348">
+        <v>28</v>
+      </c>
+      <c r="V348">
+        <v>50</v>
+      </c>
+      <c r="W348">
+        <v>78</v>
+      </c>
+      <c r="X348">
+        <v>162</v>
+      </c>
+      <c r="Y348">
+        <v>28</v>
+      </c>
+      <c r="Z348">
+        <v>158</v>
+      </c>
+      <c r="AA348">
+        <v>50</v>
+      </c>
+      <c r="AB348">
+        <v>39</v>
+      </c>
+      <c r="AC348">
+        <v>4.13692</v>
+      </c>
+      <c r="AD348">
+        <v>0</v>
+      </c>
+      <c r="AE348">
+        <v>0</v>
+      </c>
+      <c r="AF348">
+        <v>1760.8458</v>
+      </c>
+      <c r="AG348">
+        <v>0</v>
+      </c>
+      <c r="AH348">
+        <v>3</v>
+      </c>
+      <c r="AI348">
+        <v>6488.29062</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B349" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E349">
+        <v>292.0328333333334</v>
+      </c>
+      <c r="F349">
+        <v>13778.48</v>
+      </c>
+      <c r="G349">
+        <v>47.18127014256958</v>
+      </c>
+      <c r="H349">
+        <v>527.3399999999999</v>
+      </c>
+      <c r="I349">
+        <v>0</v>
+      </c>
+      <c r="J349">
+        <v>0</v>
+      </c>
+      <c r="K349">
+        <v>1.805755859643635</v>
+      </c>
+      <c r="L349">
+        <v>0</v>
+      </c>
+      <c r="M349">
+        <v>2</v>
+      </c>
+      <c r="N349">
+        <v>0</v>
+      </c>
+      <c r="O349">
+        <v>26.69682</v>
+      </c>
+      <c r="P349">
+        <v>82.39759259259259</v>
+      </c>
+      <c r="Q349">
+        <v>32.4</v>
+      </c>
+      <c r="R349">
+        <v>1594.71751</v>
+      </c>
+      <c r="S349">
+        <v>5.46074731323019</v>
+      </c>
+      <c r="T349">
+        <v>2556.19006</v>
+      </c>
+      <c r="U349">
+        <v>16</v>
+      </c>
+      <c r="V349">
+        <v>50</v>
+      </c>
+      <c r="W349">
+        <v>66</v>
+      </c>
+      <c r="X349">
+        <v>165</v>
+      </c>
+      <c r="Y349">
+        <v>16</v>
+      </c>
+      <c r="Z349">
+        <v>184</v>
+      </c>
+      <c r="AA349">
+        <v>50</v>
+      </c>
+      <c r="AB349">
+        <v>34</v>
+      </c>
+      <c r="AC349">
+        <v>4.16344</v>
+      </c>
+      <c r="AD349">
+        <v>-4.85024</v>
+      </c>
+      <c r="AE349">
+        <v>0</v>
+      </c>
+      <c r="AF349">
+        <v>1152.0033</v>
+      </c>
+      <c r="AG349">
+        <v>0</v>
+      </c>
+      <c r="AH349">
+        <v>3</v>
+      </c>
+      <c r="AI349">
+        <v>4784.152529999999</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B350" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E350">
+        <v>275.8828333333333</v>
+      </c>
+      <c r="F350">
+        <v>17704.6</v>
+      </c>
+      <c r="G350">
+        <v>64.17434454360757</v>
+      </c>
+      <c r="H350">
+        <v>629.54</v>
+      </c>
+      <c r="I350">
+        <v>0</v>
+      </c>
+      <c r="J350">
+        <v>0</v>
+      </c>
+      <c r="K350">
+        <v>2.281910738677107</v>
+      </c>
+      <c r="L350">
+        <v>0</v>
+      </c>
+      <c r="M350">
+        <v>8</v>
+      </c>
+      <c r="N350">
+        <v>0</v>
+      </c>
+      <c r="O350">
+        <v>28.89668</v>
+      </c>
+      <c r="P350">
+        <v>85.0302495291902</v>
+      </c>
+      <c r="Q350">
+        <v>33.984</v>
+      </c>
+      <c r="R350">
+        <v>1980.91483</v>
+      </c>
+      <c r="S350">
+        <v>7.180275793407468</v>
+      </c>
+      <c r="T350">
+        <v>2395.58007</v>
+      </c>
+      <c r="U350">
+        <v>46</v>
+      </c>
+      <c r="V350">
+        <v>54</v>
+      </c>
+      <c r="W350">
+        <v>100</v>
+      </c>
+      <c r="X350">
+        <v>174</v>
+      </c>
+      <c r="Y350">
+        <v>46</v>
+      </c>
+      <c r="Z350">
+        <v>166</v>
+      </c>
+      <c r="AA350">
+        <v>54</v>
+      </c>
+      <c r="AB350">
+        <v>35</v>
+      </c>
+      <c r="AC350">
+        <v>4.15887</v>
+      </c>
+      <c r="AD350">
+        <v>-4.90985</v>
+      </c>
+      <c r="AE350">
+        <v>0</v>
+      </c>
+      <c r="AF350">
+        <v>1666.8336</v>
+      </c>
+      <c r="AG350">
+        <v>0</v>
+      </c>
+      <c r="AH350">
+        <v>3</v>
+      </c>
+      <c r="AI350">
+        <v>5942.744490000001</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B351" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E351">
+        <v>258.8775</v>
+      </c>
+      <c r="F351">
+        <v>10452.72</v>
+      </c>
+      <c r="G351">
+        <v>40.37708955007678</v>
+      </c>
+      <c r="H351">
+        <v>606.0599999999999</v>
+      </c>
+      <c r="I351">
+        <v>0</v>
+      </c>
+      <c r="J351">
+        <v>0</v>
+      </c>
+      <c r="K351">
+        <v>2.341107280470493</v>
+      </c>
+      <c r="L351">
+        <v>0</v>
+      </c>
+      <c r="M351">
+        <v>8</v>
+      </c>
+      <c r="N351">
+        <v>0</v>
+      </c>
+      <c r="O351">
+        <v>26.87032</v>
+      </c>
+      <c r="P351">
+        <v>75.5463337831759</v>
+      </c>
+      <c r="Q351">
+        <v>35.568</v>
+      </c>
+      <c r="R351">
+        <v>951.3793000000001</v>
+      </c>
+      <c r="S351">
+        <v>3.675017334453555</v>
+      </c>
+      <c r="T351">
+        <v>1698.65997</v>
+      </c>
+      <c r="U351">
+        <v>60</v>
+      </c>
+      <c r="V351">
+        <v>27</v>
+      </c>
+      <c r="W351">
+        <v>87</v>
+      </c>
+      <c r="X351">
+        <v>150</v>
+      </c>
+      <c r="Y351">
+        <v>60</v>
+      </c>
+      <c r="Z351">
+        <v>116</v>
+      </c>
+      <c r="AA351">
+        <v>27</v>
+      </c>
+      <c r="AB351">
+        <v>25</v>
+      </c>
+      <c r="AC351">
+        <v>5.10719</v>
+      </c>
+      <c r="AD351">
+        <v>-3.11132</v>
+      </c>
+      <c r="AE351">
+        <v>0</v>
+      </c>
+      <c r="AF351">
+        <v>999.456</v>
+      </c>
+      <c r="AG351">
+        <v>0</v>
+      </c>
+      <c r="AH351">
+        <v>3</v>
+      </c>
+      <c r="AI351">
+        <v>2854.1379</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B352" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E352">
+        <v>258.8775</v>
+      </c>
+      <c r="F352">
+        <v>9142.199999999999</v>
+      </c>
+      <c r="G352">
+        <v>35.31477243097603</v>
+      </c>
+      <c r="H352">
+        <v>1631.36</v>
+      </c>
+      <c r="I352">
+        <v>0</v>
+      </c>
+      <c r="J352">
+        <v>0</v>
+      </c>
+      <c r="K352">
+        <v>6.301667777230543</v>
+      </c>
+      <c r="L352">
+        <v>0</v>
+      </c>
+      <c r="M352">
+        <v>4</v>
+      </c>
+      <c r="N352">
+        <v>0</v>
+      </c>
+      <c r="O352">
+        <v>27.65056</v>
+      </c>
+      <c r="P352">
+        <v>76.8071111111111</v>
+      </c>
+      <c r="Q352">
+        <v>36</v>
+      </c>
+      <c r="R352">
+        <v>994.41335</v>
+      </c>
+      <c r="S352">
+        <v>3.841250591495978</v>
+      </c>
+      <c r="T352">
+        <v>2769.15</v>
+      </c>
+      <c r="U352">
+        <v>98</v>
+      </c>
+      <c r="V352">
+        <v>83</v>
+      </c>
+      <c r="W352">
+        <v>181</v>
+      </c>
+      <c r="X352">
+        <v>169</v>
+      </c>
+      <c r="Y352">
+        <v>98</v>
+      </c>
+      <c r="Z352">
+        <v>141</v>
+      </c>
+      <c r="AA352">
+        <v>83</v>
+      </c>
+      <c r="AB352">
+        <v>41</v>
+      </c>
+      <c r="AC352">
+        <v>4.89137</v>
+      </c>
+      <c r="AD352">
+        <v>-4.06575</v>
+      </c>
+      <c r="AE352">
+        <v>0</v>
+      </c>
+      <c r="AF352">
+        <v>825.0207</v>
+      </c>
+      <c r="AG352">
+        <v>0</v>
+      </c>
+      <c r="AH352">
+        <v>3</v>
+      </c>
+      <c r="AI352">
+        <v>2983.24005</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B353" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E353">
+        <v>261.5161666666667</v>
+      </c>
+      <c r="F353">
+        <v>17235.83</v>
+      </c>
+      <c r="G353">
+        <v>65.90732121723515</v>
+      </c>
+      <c r="H353">
+        <v>721.4300000000001</v>
+      </c>
+      <c r="I353">
+        <v>52.86</v>
+      </c>
+      <c r="J353">
+        <v>6</v>
+      </c>
+      <c r="K353">
+        <v>2.758643984406318</v>
+      </c>
+      <c r="L353">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="M353">
+        <v>24</v>
+      </c>
+      <c r="N353">
+        <v>2</v>
+      </c>
+      <c r="O353">
+        <v>30.1627</v>
+      </c>
+      <c r="P353">
+        <v>94.24665666791651</v>
+      </c>
+      <c r="Q353">
+        <v>32.004</v>
+      </c>
+      <c r="R353">
+        <v>1812.02643</v>
+      </c>
+      <c r="S353">
+        <v>6.928927007062024</v>
+      </c>
+      <c r="T353">
+        <v>2210.37</v>
+      </c>
+      <c r="U353">
+        <v>22</v>
+      </c>
+      <c r="V353">
+        <v>46</v>
+      </c>
+      <c r="W353">
+        <v>68</v>
+      </c>
+      <c r="X353">
+        <v>125</v>
+      </c>
+      <c r="Y353">
+        <v>22</v>
+      </c>
+      <c r="Z353">
+        <v>154</v>
+      </c>
+      <c r="AA353">
+        <v>46</v>
+      </c>
+      <c r="AB353">
+        <v>50</v>
+      </c>
+      <c r="AC353">
+        <v>4.29087</v>
+      </c>
+      <c r="AD353">
+        <v>-4.60895</v>
+      </c>
+      <c r="AE353">
+        <v>0</v>
+      </c>
+      <c r="AF353">
+        <v>1196.8308</v>
+      </c>
+      <c r="AG353">
+        <v>0</v>
+      </c>
+      <c r="AH353">
+        <v>3</v>
+      </c>
+      <c r="AI353">
+        <v>5436.079290000001</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B354" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E354">
+        <v>258.8775</v>
+      </c>
+      <c r="F354">
+        <v>7748.639999999999</v>
+      </c>
+      <c r="G354">
+        <v>29.93168583596488</v>
+      </c>
+      <c r="H354">
+        <v>303.83</v>
+      </c>
+      <c r="I354">
+        <v>0</v>
+      </c>
+      <c r="J354">
+        <v>0</v>
+      </c>
+      <c r="K354">
+        <v>1.173643904935732</v>
+      </c>
+      <c r="L354">
+        <v>0</v>
+      </c>
+      <c r="M354">
+        <v>0</v>
+      </c>
+      <c r="N354">
+        <v>0</v>
+      </c>
+      <c r="O354">
+        <v>24.22349</v>
+      </c>
+      <c r="P354">
+        <v>71.58241725768322</v>
+      </c>
+      <c r="Q354">
+        <v>33.84</v>
+      </c>
+      <c r="R354">
+        <v>796.68317</v>
+      </c>
+      <c r="S354">
+        <v>3.077452347152611</v>
+      </c>
+      <c r="T354">
+        <v>1227.64998</v>
+      </c>
+      <c r="U354">
+        <v>67</v>
+      </c>
+      <c r="V354">
+        <v>27</v>
+      </c>
+      <c r="W354">
+        <v>94</v>
+      </c>
+      <c r="X354">
+        <v>134</v>
+      </c>
+      <c r="Y354">
+        <v>67</v>
+      </c>
+      <c r="Z354">
+        <v>81</v>
+      </c>
+      <c r="AA354">
+        <v>27</v>
+      </c>
+      <c r="AB354">
+        <v>17</v>
+      </c>
+      <c r="AC354">
+        <v>4.11513</v>
+      </c>
+      <c r="AD354">
+        <v>-3.45031</v>
+      </c>
+      <c r="AE354">
+        <v>0</v>
+      </c>
+      <c r="AF354">
+        <v>643.2678</v>
+      </c>
+      <c r="AG354">
+        <v>0</v>
+      </c>
+      <c r="AH354">
+        <v>3</v>
+      </c>
+      <c r="AI354">
+        <v>2390.04951</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B355" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Activity 20260704223835 | Amistoso vs Tampico | Activity 20260704161350</t>
+        </is>
+      </c>
+      <c r="E355">
+        <v>359.1906666666666</v>
+      </c>
+      <c r="F355">
+        <v>7516.52</v>
+      </c>
+      <c r="G355">
+        <v>20.92626757191167</v>
+      </c>
+      <c r="H355">
+        <v>512.9299999999999</v>
+      </c>
+      <c r="I355">
+        <v>164.93</v>
+      </c>
+      <c r="J355">
+        <v>16</v>
+      </c>
+      <c r="K355">
+        <v>1.428015946962245</v>
+      </c>
+      <c r="L355">
+        <v>166.82</v>
+      </c>
+      <c r="M355">
+        <v>19</v>
+      </c>
+      <c r="N355">
+        <v>8</v>
+      </c>
+      <c r="O355">
+        <v>37.87989</v>
+      </c>
+      <c r="P355">
+        <v>112.4165776353276</v>
+      </c>
+      <c r="Q355">
+        <v>33.696</v>
+      </c>
+      <c r="R355">
+        <v>863.14681</v>
+      </c>
+      <c r="S355">
+        <v>2.40303240061917</v>
+      </c>
+      <c r="T355">
+        <v>1318</v>
+      </c>
+      <c r="U355">
+        <v>30</v>
+      </c>
+      <c r="V355">
+        <v>20</v>
+      </c>
+      <c r="W355">
+        <v>50</v>
+      </c>
+      <c r="X355">
+        <v>107</v>
+      </c>
+      <c r="Y355">
+        <v>30</v>
+      </c>
+      <c r="Z355">
+        <v>91</v>
+      </c>
+      <c r="AA355">
+        <v>20</v>
+      </c>
+      <c r="AB355">
+        <v>31</v>
+      </c>
+      <c r="AC355">
+        <v>9.967460000000001</v>
+      </c>
+      <c r="AD355">
+        <v>0</v>
+      </c>
+      <c r="AE355">
+        <v>0</v>
+      </c>
+      <c r="AF355">
+        <v>1125.2928</v>
+      </c>
+      <c r="AG355">
+        <v>0</v>
+      </c>
+      <c r="AH355">
+        <v>3</v>
+      </c>
+      <c r="AI355">
+        <v>2589.44043</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B356" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E356">
+        <v>292.0328333333334</v>
+      </c>
+      <c r="F356">
+        <v>18011.81</v>
+      </c>
+      <c r="G356">
+        <v>61.67734564092964</v>
+      </c>
+      <c r="H356">
+        <v>877.0899999999999</v>
+      </c>
+      <c r="I356">
+        <v>0</v>
+      </c>
+      <c r="J356">
+        <v>0</v>
+      </c>
+      <c r="K356">
+        <v>3.003395166182797</v>
+      </c>
+      <c r="L356">
+        <v>0</v>
+      </c>
+      <c r="M356">
+        <v>18</v>
+      </c>
+      <c r="N356">
+        <v>0</v>
+      </c>
+      <c r="O356">
+        <v>28.46</v>
+      </c>
+      <c r="P356">
+        <v>81.33287608596251</v>
+      </c>
+      <c r="Q356">
+        <v>34.992</v>
+      </c>
+      <c r="R356">
+        <v>1558.2008</v>
+      </c>
+      <c r="S356">
+        <v>5.335704147421779</v>
+      </c>
+      <c r="T356">
+        <v>2692.46005</v>
+      </c>
+      <c r="U356">
+        <v>40</v>
+      </c>
+      <c r="V356">
+        <v>44</v>
+      </c>
+      <c r="W356">
+        <v>84</v>
+      </c>
+      <c r="X356">
+        <v>168</v>
+      </c>
+      <c r="Y356">
+        <v>40</v>
+      </c>
+      <c r="Z356">
+        <v>144</v>
+      </c>
+      <c r="AA356">
+        <v>44</v>
+      </c>
+      <c r="AB356">
+        <v>25</v>
+      </c>
+      <c r="AC356">
+        <v>4.10329</v>
+      </c>
+      <c r="AD356">
+        <v>-4.20697</v>
+      </c>
+      <c r="AE356">
+        <v>0</v>
+      </c>
+      <c r="AF356">
+        <v>1453.43877</v>
+      </c>
+      <c r="AG356">
+        <v>0</v>
+      </c>
+      <c r="AH356">
+        <v>3</v>
+      </c>
+      <c r="AI356">
+        <v>4674.6024</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B357" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E357">
+        <v>245.8588333333333</v>
+      </c>
+      <c r="F357">
+        <v>7125.25</v>
+      </c>
+      <c r="G357">
+        <v>28.98106162547207</v>
+      </c>
+      <c r="H357">
+        <v>347.96</v>
+      </c>
+      <c r="I357">
+        <v>0</v>
+      </c>
+      <c r="J357">
+        <v>0</v>
+      </c>
+      <c r="K357">
+        <v>1.415283702775238</v>
+      </c>
+      <c r="L357">
+        <v>0</v>
+      </c>
+      <c r="M357">
+        <v>6</v>
+      </c>
+      <c r="N357">
+        <v>0</v>
+      </c>
+      <c r="O357">
+        <v>28.42518</v>
+      </c>
+      <c r="P357">
+        <v>81.40085910652921</v>
+      </c>
+      <c r="Q357">
+        <v>34.92</v>
+      </c>
+      <c r="R357">
+        <v>680.3570199999999</v>
+      </c>
+      <c r="S357">
+        <v>2.767266934345115</v>
+      </c>
+      <c r="T357">
+        <v>1064.00998</v>
+      </c>
+      <c r="U357">
+        <v>46</v>
+      </c>
+      <c r="V357">
+        <v>14</v>
+      </c>
+      <c r="W357">
+        <v>60</v>
+      </c>
+      <c r="X357">
+        <v>94</v>
+      </c>
+      <c r="Y357">
+        <v>46</v>
+      </c>
+      <c r="Z357">
+        <v>71</v>
+      </c>
+      <c r="AA357">
+        <v>14</v>
+      </c>
+      <c r="AB357">
+        <v>21</v>
+      </c>
+      <c r="AC357">
+        <v>3.92378</v>
+      </c>
+      <c r="AD357">
+        <v>-4.26226</v>
+      </c>
+      <c r="AE357">
+        <v>0</v>
+      </c>
+      <c r="AF357">
+        <v>671.5824</v>
+      </c>
+      <c r="AG357">
+        <v>0</v>
+      </c>
+      <c r="AH357">
+        <v>3</v>
+      </c>
+      <c r="AI357">
+        <v>2041.07106</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B358" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E358">
+        <v>292.0328333333334</v>
+      </c>
+      <c r="F358">
+        <v>15422.71</v>
+      </c>
+      <c r="G358">
+        <v>52.81156171366575</v>
+      </c>
+      <c r="H358">
+        <v>1283.57</v>
+      </c>
+      <c r="I358">
+        <v>10.12</v>
+      </c>
+      <c r="J358">
+        <v>0</v>
+      </c>
+      <c r="K358">
+        <v>4.395293451592487</v>
+      </c>
+      <c r="L358">
+        <v>30.12</v>
+      </c>
+      <c r="M358">
+        <v>36</v>
+      </c>
+      <c r="N358">
+        <v>2</v>
+      </c>
+      <c r="O358">
+        <v>31.46879</v>
+      </c>
+      <c r="P358">
+        <v>89.93138431641519</v>
+      </c>
+      <c r="Q358">
+        <v>34.992</v>
+      </c>
+      <c r="R358">
+        <v>1322.82834</v>
+      </c>
+      <c r="S358">
+        <v>4.529724705612439</v>
+      </c>
+      <c r="T358">
+        <v>3115.13007</v>
+      </c>
+      <c r="U358">
+        <v>65</v>
+      </c>
+      <c r="V358">
+        <v>82</v>
+      </c>
+      <c r="W358">
+        <v>147</v>
+      </c>
+      <c r="X358">
+        <v>181</v>
+      </c>
+      <c r="Y358">
+        <v>65</v>
+      </c>
+      <c r="Z358">
+        <v>182</v>
+      </c>
+      <c r="AA358">
+        <v>82</v>
+      </c>
+      <c r="AB358">
+        <v>37</v>
+      </c>
+      <c r="AC358">
+        <v>4.69417</v>
+      </c>
+      <c r="AD358">
+        <v>-5.24722</v>
+      </c>
+      <c r="AE358">
+        <v>0</v>
+      </c>
+      <c r="AF358">
+        <v>1373.25928</v>
+      </c>
+      <c r="AG358">
+        <v>0</v>
+      </c>
+      <c r="AH358">
+        <v>3</v>
+      </c>
+      <c r="AI358">
+        <v>3968.48502</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B359" s="2">
+        <v>46207</v>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Activity 20260704185730 | Activity 20260704161350</t>
+        </is>
+      </c>
+      <c r="E359">
+        <v>66.81666666666666</v>
+      </c>
+      <c r="F359">
+        <v>0</v>
+      </c>
+      <c r="G359">
+        <v>0</v>
+      </c>
+      <c r="H359">
+        <v>0</v>
+      </c>
+      <c r="I359">
+        <v>0</v>
+      </c>
+      <c r="J359">
+        <v>0</v>
+      </c>
+      <c r="K359">
+        <v>0</v>
+      </c>
+      <c r="L359">
+        <v>0</v>
+      </c>
+      <c r="M359">
+        <v>0</v>
+      </c>
+      <c r="N359">
+        <v>0</v>
+      </c>
+      <c r="O359">
+        <v>0.00401</v>
+      </c>
+      <c r="P359">
+        <v>0.01179967043314501</v>
+      </c>
+      <c r="Q359">
+        <v>33.984</v>
+      </c>
+      <c r="R359">
+        <v>9.305240000000001</v>
+      </c>
+      <c r="S359">
+        <v>0.1392652531803442</v>
+      </c>
+      <c r="T359">
+        <v>0</v>
+      </c>
+      <c r="U359">
+        <v>0</v>
+      </c>
+      <c r="V359">
+        <v>0</v>
+      </c>
+      <c r="W359">
+        <v>0</v>
+      </c>
+      <c r="X359">
+        <v>0</v>
+      </c>
+      <c r="Y359">
+        <v>0</v>
+      </c>
+      <c r="Z359">
+        <v>0</v>
+      </c>
+      <c r="AA359">
+        <v>0</v>
+      </c>
+      <c r="AB359">
+        <v>1</v>
+      </c>
+      <c r="AC359">
+        <v>0</v>
+      </c>
+      <c r="AD359">
+        <v>0</v>
+      </c>
+      <c r="AE359">
+        <v>0</v>
+      </c>
+      <c r="AF359">
+        <v>0</v>
+      </c>
+      <c r="AG359">
+        <v>0</v>
+      </c>
+      <c r="AH359">
+        <v>3</v>
+      </c>
+      <c r="AI359">
+        <v>27.91572</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B360" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E360">
+        <v>258.8775</v>
+      </c>
+      <c r="F360">
+        <v>11764.28</v>
+      </c>
+      <c r="G360">
+        <v>45.44342401328814</v>
+      </c>
+      <c r="H360">
+        <v>494.3</v>
+      </c>
+      <c r="I360">
+        <v>0</v>
+      </c>
+      <c r="J360">
+        <v>0</v>
+      </c>
+      <c r="K360">
+        <v>1.909397301812633</v>
+      </c>
+      <c r="L360">
+        <v>0</v>
+      </c>
+      <c r="M360">
+        <v>4</v>
+      </c>
+      <c r="N360">
+        <v>0</v>
+      </c>
+      <c r="O360">
+        <v>26.40669</v>
+      </c>
+      <c r="P360">
+        <v>75.46493484224966</v>
+      </c>
+      <c r="Q360">
+        <v>34.992</v>
+      </c>
+      <c r="R360">
+        <v>1119.21103</v>
+      </c>
+      <c r="S360">
+        <v>4.323322923004123</v>
+      </c>
+      <c r="T360">
+        <v>2038.59997</v>
+      </c>
+      <c r="U360">
+        <v>39</v>
+      </c>
+      <c r="V360">
+        <v>39</v>
+      </c>
+      <c r="W360">
+        <v>78</v>
+      </c>
+      <c r="X360">
+        <v>130</v>
+      </c>
+      <c r="Y360">
+        <v>39</v>
+      </c>
+      <c r="Z360">
+        <v>118</v>
+      </c>
+      <c r="AA360">
+        <v>39</v>
+      </c>
+      <c r="AB360">
+        <v>28</v>
+      </c>
+      <c r="AC360">
+        <v>3.83877</v>
+      </c>
+      <c r="AD360">
+        <v>-2.70335</v>
+      </c>
+      <c r="AE360">
+        <v>0</v>
+      </c>
+      <c r="AF360">
+        <v>1112.8176</v>
+      </c>
+      <c r="AG360">
+        <v>0</v>
+      </c>
+      <c r="AH360">
+        <v>3</v>
+      </c>
+      <c r="AI360">
+        <v>3357.63309</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B361" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Activity 20260704223835 | Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E361">
+        <v>450.1495</v>
+      </c>
+      <c r="F361">
+        <v>20173.03</v>
+      </c>
+      <c r="G361">
+        <v>44.81406732652152</v>
+      </c>
+      <c r="H361">
+        <v>669.1700000000001</v>
+      </c>
+      <c r="I361">
+        <v>40.56</v>
+      </c>
+      <c r="J361">
+        <v>4</v>
+      </c>
+      <c r="K361">
+        <v>1.486550579307541</v>
+      </c>
+      <c r="L361">
+        <v>37.48</v>
+      </c>
+      <c r="M361">
+        <v>10</v>
+      </c>
+      <c r="N361">
+        <v>3</v>
+      </c>
+      <c r="O361">
+        <v>266.83429</v>
+      </c>
+      <c r="P361">
+        <v>808.2948321822367</v>
+      </c>
+      <c r="Q361">
+        <v>33.012</v>
+      </c>
+      <c r="R361">
+        <v>1871.74762</v>
+      </c>
+      <c r="S361">
+        <v>4.158057756367606</v>
+      </c>
+      <c r="T361">
+        <v>3503.80995</v>
+      </c>
+      <c r="U361">
+        <v>41</v>
+      </c>
+      <c r="V361">
+        <v>66</v>
+      </c>
+      <c r="W361">
+        <v>107</v>
+      </c>
+      <c r="X361">
+        <v>209</v>
+      </c>
+      <c r="Y361">
+        <v>41</v>
+      </c>
+      <c r="Z361">
+        <v>189</v>
+      </c>
+      <c r="AA361">
+        <v>66</v>
+      </c>
+      <c r="AB361">
+        <v>28</v>
+      </c>
+      <c r="AC361">
+        <v>6.86781</v>
+      </c>
+      <c r="AD361">
+        <v>-4.259</v>
+      </c>
+      <c r="AE361">
+        <v>0</v>
+      </c>
+      <c r="AF361">
+        <v>1844.74575</v>
+      </c>
+      <c r="AG361">
+        <v>0</v>
+      </c>
+      <c r="AH361">
+        <v>3</v>
+      </c>
+      <c r="AI361">
+        <v>5615.24286</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B362" s="2">
+        <v>46207</v>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+        </is>
+      </c>
+      <c r="E362">
+        <v>292.0328333333334</v>
+      </c>
+      <c r="F362">
+        <v>13204.55</v>
+      </c>
+      <c r="G362">
+        <v>45.21597742719567</v>
+      </c>
+      <c r="H362">
+        <v>443.26</v>
+      </c>
+      <c r="I362">
+        <v>0</v>
+      </c>
+      <c r="J362">
+        <v>0</v>
+      </c>
+      <c r="K362">
+        <v>1.517843027924371</v>
+      </c>
+      <c r="L362">
+        <v>0</v>
+      </c>
+      <c r="M362">
+        <v>2</v>
+      </c>
+      <c r="N362">
+        <v>0</v>
+      </c>
+      <c r="O362">
+        <v>26.45102</v>
+      </c>
+      <c r="P362">
+        <v>82.6491063617048</v>
+      </c>
+      <c r="Q362">
+        <v>32.004</v>
+      </c>
+      <c r="R362">
+        <v>1221.18793</v>
+      </c>
+      <c r="S362">
+        <v>4.181680244858311</v>
+      </c>
+      <c r="T362">
+        <v>1907.04997</v>
+      </c>
+      <c r="U362">
+        <v>32</v>
+      </c>
+      <c r="V362">
+        <v>44</v>
+      </c>
+      <c r="W362">
+        <v>76</v>
+      </c>
+      <c r="X362">
+        <v>130</v>
+      </c>
+      <c r="Y362">
+        <v>32</v>
+      </c>
+      <c r="Z362">
+        <v>126</v>
+      </c>
+      <c r="AA362">
+        <v>44</v>
+      </c>
+      <c r="AB362">
+        <v>28</v>
+      </c>
+      <c r="AC362">
+        <v>3.98444</v>
+      </c>
+      <c r="AD362">
+        <v>-3.16343</v>
+      </c>
+      <c r="AE362">
+        <v>0</v>
+      </c>
+      <c r="AF362">
+        <v>1107.6352</v>
+      </c>
+      <c r="AG362">
+        <v>0</v>
+      </c>
+      <c r="AH362">
+        <v>3</v>
+      </c>
+      <c r="AI362">
+        <v>3663.56379</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-07
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI362"/>
+  <dimension ref="A1:AI378"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -35708,6 +35708,11 @@
       <c r="B314" s="2">
         <v>46205</v>
       </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D314" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -35816,6 +35821,11 @@
       <c r="B315" s="2">
         <v>46205</v>
       </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D315" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -35924,6 +35934,11 @@
       <c r="B316" s="2">
         <v>46205</v>
       </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D316" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36032,6 +36047,11 @@
       <c r="B317" s="2">
         <v>46205</v>
       </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D317" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36140,6 +36160,11 @@
       <c r="B318" s="2">
         <v>46205</v>
       </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D318" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36248,6 +36273,11 @@
       <c r="B319" s="2">
         <v>46205</v>
       </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D319" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36356,6 +36386,11 @@
       <c r="B320" s="2">
         <v>46205</v>
       </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D320" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36464,6 +36499,11 @@
       <c r="B321" s="2">
         <v>46205</v>
       </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D321" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36572,6 +36612,11 @@
       <c r="B322" s="2">
         <v>46205</v>
       </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D322" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36680,6 +36725,11 @@
       <c r="B323" s="2">
         <v>46205</v>
       </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D323" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36788,6 +36838,11 @@
       <c r="B324" s="2">
         <v>46205</v>
       </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D324" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -36896,6 +36951,11 @@
       <c r="B325" s="2">
         <v>46205</v>
       </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D325" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -37004,6 +37064,11 @@
       <c r="B326" s="2">
         <v>46205</v>
       </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D326" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -37112,6 +37177,11 @@
       <c r="B327" s="2">
         <v>46205</v>
       </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D327" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -37220,6 +37290,11 @@
       <c r="B328" s="2">
         <v>46205</v>
       </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D328" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -37328,6 +37403,11 @@
       <c r="B329" s="2">
         <v>46205</v>
       </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D329" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -37436,6 +37516,11 @@
       <c r="B330" s="2">
         <v>46205</v>
       </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D330" t="inlineStr">
         <is>
           <t>Sesión 26</t>
@@ -39472,20 +39557,20 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E348">
-        <v>305.0515</v>
+        <v>94.3995</v>
       </c>
       <c r="F348">
-        <v>21952.84</v>
+        <v>10800.15</v>
       </c>
       <c r="G348">
-        <v>71.96437322878269</v>
+        <v>114.4089746238062</v>
       </c>
       <c r="H348">
-        <v>455.54</v>
+        <v>227.77</v>
       </c>
       <c r="I348">
         <v>0</v>
@@ -39494,13 +39579,13 @@
         <v>0</v>
       </c>
       <c r="K348">
-        <v>1.493321619464255</v>
+        <v>2.412830576433138</v>
       </c>
       <c r="L348">
         <v>0</v>
       </c>
       <c r="M348">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N348">
         <v>0</v>
@@ -39515,49 +39600,49 @@
         <v>32.364</v>
       </c>
       <c r="R348">
-        <v>2162.76354</v>
+        <v>1050.34399</v>
       </c>
       <c r="S348">
-        <v>7.089830864624498</v>
+        <v>11.1265842509759</v>
       </c>
       <c r="T348">
-        <v>2903.72992</v>
+        <v>1451.52997</v>
       </c>
       <c r="U348">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="V348">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="W348">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="X348">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="Y348">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="Z348">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="AA348">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AB348">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="AC348">
         <v>4.13692</v>
       </c>
       <c r="AD348">
-        <v>0</v>
+        <v>-4.45073</v>
       </c>
       <c r="AE348">
         <v>0</v>
       </c>
       <c r="AF348">
-        <v>1760.8458</v>
+        <v>865.7558</v>
       </c>
       <c r="AG348">
         <v>0</v>
@@ -39566,7 +39651,7 @@
         <v>3</v>
       </c>
       <c r="AI348">
-        <v>6488.29062</v>
+        <v>3151.03197</v>
       </c>
     </row>
     <row r="349">
@@ -39585,20 +39670,20 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E349">
-        <v>292.0328333333334</v>
+        <v>94.3995</v>
       </c>
       <c r="F349">
-        <v>13778.48</v>
+        <v>6766.08</v>
       </c>
       <c r="G349">
-        <v>47.18127014256958</v>
+        <v>71.67495590548678</v>
       </c>
       <c r="H349">
-        <v>527.3399999999999</v>
+        <v>263.67</v>
       </c>
       <c r="I349">
         <v>0</v>
@@ -39607,13 +39692,13 @@
         <v>0</v>
       </c>
       <c r="K349">
-        <v>1.805755859643635</v>
+        <v>2.793129200896191</v>
       </c>
       <c r="L349">
         <v>0</v>
       </c>
       <c r="M349">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N349">
         <v>0</v>
@@ -39628,37 +39713,37 @@
         <v>32.4</v>
       </c>
       <c r="R349">
-        <v>1594.71751</v>
+        <v>772.6411099999999</v>
       </c>
       <c r="S349">
-        <v>5.46074731323019</v>
+        <v>8.184800872885978</v>
       </c>
       <c r="T349">
-        <v>2556.19006</v>
+        <v>1274.13</v>
       </c>
       <c r="U349">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="V349">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="W349">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="X349">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="Y349">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="Z349">
-        <v>184</v>
+        <v>92</v>
       </c>
       <c r="AA349">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AB349">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="AC349">
         <v>4.16344</v>
@@ -39670,7 +39755,7 @@
         <v>0</v>
       </c>
       <c r="AF349">
-        <v>1152.0033</v>
+        <v>560.4186</v>
       </c>
       <c r="AG349">
         <v>0</v>
@@ -39679,7 +39764,7 @@
         <v>3</v>
       </c>
       <c r="AI349">
-        <v>4784.152529999999</v>
+        <v>2317.92333</v>
       </c>
     </row>
     <row r="350">
@@ -39698,20 +39783,20 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E350">
-        <v>275.8828333333333</v>
+        <v>94.3995</v>
       </c>
       <c r="F350">
-        <v>17704.6</v>
+        <v>8661.750000000002</v>
       </c>
       <c r="G350">
-        <v>64.17434454360757</v>
+        <v>91.75631226860314</v>
       </c>
       <c r="H350">
-        <v>629.54</v>
+        <v>314.77</v>
       </c>
       <c r="I350">
         <v>0</v>
@@ -39720,13 +39805,13 @@
         <v>0</v>
       </c>
       <c r="K350">
-        <v>2.281910738677107</v>
+        <v>3.334445627360314</v>
       </c>
       <c r="L350">
         <v>0</v>
       </c>
       <c r="M350">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N350">
         <v>0</v>
@@ -39741,37 +39826,37 @@
         <v>33.984</v>
       </c>
       <c r="R350">
-        <v>1980.91483</v>
+        <v>950.71396</v>
       </c>
       <c r="S350">
-        <v>7.180275793407468</v>
+        <v>10.07117580071928</v>
       </c>
       <c r="T350">
-        <v>2395.58007</v>
+        <v>1197.42004</v>
       </c>
       <c r="U350">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="V350">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="W350">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="X350">
-        <v>174</v>
+        <v>87</v>
       </c>
       <c r="Y350">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="Z350">
-        <v>166</v>
+        <v>83</v>
       </c>
       <c r="AA350">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="AB350">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="AC350">
         <v>4.15887</v>
@@ -39783,7 +39868,7 @@
         <v>0</v>
       </c>
       <c r="AF350">
-        <v>1666.8336</v>
+        <v>809.8696</v>
       </c>
       <c r="AG350">
         <v>0</v>
@@ -39792,7 +39877,7 @@
         <v>3</v>
       </c>
       <c r="AI350">
-        <v>5942.744490000001</v>
+        <v>2852.14188</v>
       </c>
     </row>
     <row r="351">
@@ -39811,20 +39896,20 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E351">
-        <v>258.8775</v>
+        <v>60.18500000000001</v>
       </c>
       <c r="F351">
-        <v>10452.72</v>
+        <v>4184.29</v>
       </c>
       <c r="G351">
-        <v>40.37708955007678</v>
+        <v>69.52380161169725</v>
       </c>
       <c r="H351">
-        <v>606.0599999999999</v>
+        <v>211.54</v>
       </c>
       <c r="I351">
         <v>0</v>
@@ -39833,13 +39918,13 @@
         <v>0</v>
       </c>
       <c r="K351">
-        <v>2.341107280470493</v>
+        <v>3.514829276397773</v>
       </c>
       <c r="L351">
         <v>0</v>
       </c>
       <c r="M351">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N351">
         <v>0</v>
@@ -39854,37 +39939,37 @@
         <v>35.568</v>
       </c>
       <c r="R351">
-        <v>951.3793000000001</v>
+        <v>361.58097</v>
       </c>
       <c r="S351">
-        <v>3.675017334453555</v>
+        <v>6.007825371770373</v>
       </c>
       <c r="T351">
-        <v>1698.65997</v>
+        <v>661.87999</v>
       </c>
       <c r="U351">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="V351">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="W351">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="X351">
-        <v>150</v>
+        <v>59</v>
       </c>
       <c r="Y351">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="Z351">
-        <v>116</v>
+        <v>48</v>
       </c>
       <c r="AA351">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="AB351">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="AC351">
         <v>5.10719</v>
@@ -39896,7 +39981,7 @@
         <v>0</v>
       </c>
       <c r="AF351">
-        <v>999.456</v>
+        <v>396.44</v>
       </c>
       <c r="AG351">
         <v>0</v>
@@ -39905,7 +39990,7 @@
         <v>3</v>
       </c>
       <c r="AI351">
-        <v>2854.1379</v>
+        <v>1084.74291</v>
       </c>
     </row>
     <row r="352">
@@ -39924,20 +40009,20 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E352">
-        <v>258.8775</v>
+        <v>60.18500000000001</v>
       </c>
       <c r="F352">
-        <v>9142.199999999999</v>
+        <v>3438.47</v>
       </c>
       <c r="G352">
-        <v>35.31477243097603</v>
+        <v>57.13167732823793</v>
       </c>
       <c r="H352">
-        <v>1631.36</v>
+        <v>712.37</v>
       </c>
       <c r="I352">
         <v>0</v>
@@ -39946,58 +40031,58 @@
         <v>0</v>
       </c>
       <c r="K352">
-        <v>6.301667777230543</v>
+        <v>11.83633795796295</v>
       </c>
       <c r="L352">
         <v>0</v>
       </c>
       <c r="M352">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N352">
         <v>0</v>
       </c>
       <c r="O352">
-        <v>27.65056</v>
+        <v>24.56296</v>
       </c>
       <c r="P352">
-        <v>76.8071111111111</v>
+        <v>68.23044444444444</v>
       </c>
       <c r="Q352">
         <v>36</v>
       </c>
       <c r="R352">
-        <v>994.41335</v>
+        <v>355.14161</v>
       </c>
       <c r="S352">
-        <v>3.841250591495978</v>
+        <v>5.900832599484921</v>
       </c>
       <c r="T352">
-        <v>2769.15</v>
+        <v>1179.78</v>
       </c>
       <c r="U352">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="V352">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="W352">
-        <v>181</v>
+        <v>84</v>
       </c>
       <c r="X352">
-        <v>169</v>
+        <v>68</v>
       </c>
       <c r="Y352">
-        <v>98</v>
+        <v>45</v>
       </c>
       <c r="Z352">
-        <v>141</v>
+        <v>62</v>
       </c>
       <c r="AA352">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="AB352">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="AC352">
         <v>4.89137</v>
@@ -40009,7 +40094,7 @@
         <v>0</v>
       </c>
       <c r="AF352">
-        <v>825.0207</v>
+        <v>309.6366</v>
       </c>
       <c r="AG352">
         <v>0</v>
@@ -40018,7 +40103,7 @@
         <v>3</v>
       </c>
       <c r="AI352">
-        <v>2983.24005</v>
+        <v>1065.42483</v>
       </c>
     </row>
     <row r="353">
@@ -40037,38 +40122,38 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E353">
-        <v>261.5161666666667</v>
+        <v>94.3995</v>
       </c>
       <c r="F353">
-        <v>17235.83</v>
+        <v>8486.620000000001</v>
       </c>
       <c r="G353">
-        <v>65.90732121723515</v>
+        <v>89.90111176436316</v>
       </c>
       <c r="H353">
-        <v>721.4300000000001</v>
+        <v>354.86</v>
       </c>
       <c r="I353">
-        <v>52.86</v>
+        <v>26.43</v>
       </c>
       <c r="J353">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K353">
-        <v>2.758643984406318</v>
+        <v>3.759130080138136</v>
       </c>
       <c r="L353">
-        <v>9.539999999999999</v>
+        <v>4.77</v>
       </c>
       <c r="M353">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N353">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O353">
         <v>30.1627</v>
@@ -40080,37 +40165,37 @@
         <v>32.004</v>
       </c>
       <c r="R353">
-        <v>1812.02643</v>
+        <v>874.1758399999999</v>
       </c>
       <c r="S353">
-        <v>6.928927007062024</v>
+        <v>9.260386336792036</v>
       </c>
       <c r="T353">
-        <v>2210.37</v>
+        <v>1097.64002</v>
       </c>
       <c r="U353">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="V353">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="W353">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="X353">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="Y353">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="Z353">
-        <v>154</v>
+        <v>77</v>
       </c>
       <c r="AA353">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="AB353">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="AC353">
         <v>4.29087</v>
@@ -40122,7 +40207,7 @@
         <v>0</v>
       </c>
       <c r="AF353">
-        <v>1196.8308</v>
+        <v>585.9995999999999</v>
       </c>
       <c r="AG353">
         <v>0</v>
@@ -40131,7 +40216,7 @@
         <v>3</v>
       </c>
       <c r="AI353">
-        <v>5436.079290000001</v>
+        <v>2622.52752</v>
       </c>
     </row>
     <row r="354">
@@ -40150,20 +40235,20 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E354">
-        <v>258.8775</v>
+        <v>60.18500000000001</v>
       </c>
       <c r="F354">
-        <v>7748.639999999999</v>
+        <v>2837.02</v>
       </c>
       <c r="G354">
-        <v>29.93168583596488</v>
+        <v>47.13832350253384</v>
       </c>
       <c r="H354">
-        <v>303.83</v>
+        <v>104.18</v>
       </c>
       <c r="I354">
         <v>0</v>
@@ -40172,7 +40257,7 @@
         <v>0</v>
       </c>
       <c r="K354">
-        <v>1.173643904935732</v>
+        <v>1.730996095372601</v>
       </c>
       <c r="L354">
         <v>0</v>
@@ -40184,49 +40269,49 @@
         <v>0</v>
       </c>
       <c r="O354">
-        <v>24.22349</v>
+        <v>22.62191</v>
       </c>
       <c r="P354">
-        <v>71.58241725768322</v>
+        <v>66.8496158392435</v>
       </c>
       <c r="Q354">
         <v>33.84</v>
       </c>
       <c r="R354">
-        <v>796.68317</v>
+        <v>273.33804</v>
       </c>
       <c r="S354">
-        <v>3.077452347152611</v>
+        <v>4.541630638863503</v>
       </c>
       <c r="T354">
-        <v>1227.64998</v>
+        <v>464.12001</v>
       </c>
       <c r="U354">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="V354">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="W354">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="X354">
-        <v>134</v>
+        <v>52</v>
       </c>
       <c r="Y354">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="Z354">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="AA354">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="AB354">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="AC354">
-        <v>4.11513</v>
+        <v>3.84558</v>
       </c>
       <c r="AD354">
         <v>-3.45031</v>
@@ -40235,7 +40320,7 @@
         <v>0</v>
       </c>
       <c r="AF354">
-        <v>643.2678</v>
+        <v>235.9756</v>
       </c>
       <c r="AG354">
         <v>0</v>
@@ -40244,7 +40329,7 @@
         <v>3</v>
       </c>
       <c r="AI354">
-        <v>2390.04951</v>
+        <v>820.0141199999999</v>
       </c>
     </row>
     <row r="355">
@@ -40263,92 +40348,92 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>Activity 20260704223835 | Amistoso vs Tampico | Activity 20260704161350</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E355">
-        <v>359.1906666666666</v>
+        <v>94.3995</v>
       </c>
       <c r="F355">
-        <v>7516.52</v>
+        <v>4710.620000000001</v>
       </c>
       <c r="G355">
-        <v>20.92626757191167</v>
+        <v>49.90089989883422</v>
       </c>
       <c r="H355">
-        <v>512.9299999999999</v>
+        <v>130.05</v>
       </c>
       <c r="I355">
-        <v>164.93</v>
+        <v>0</v>
       </c>
       <c r="J355">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K355">
-        <v>1.428015946962245</v>
+        <v>1.377655601989417</v>
       </c>
       <c r="L355">
-        <v>166.82</v>
+        <v>0</v>
       </c>
       <c r="M355">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="N355">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O355">
-        <v>37.87989</v>
+        <v>27.62873</v>
       </c>
       <c r="P355">
-        <v>112.4165776353276</v>
+        <v>81.99409425451093</v>
       </c>
       <c r="Q355">
         <v>33.696</v>
       </c>
       <c r="R355">
-        <v>863.14681</v>
+        <v>481.60199</v>
       </c>
       <c r="S355">
-        <v>2.40303240061917</v>
+        <v>5.101743017706662</v>
       </c>
       <c r="T355">
-        <v>1318</v>
+        <v>510.82001</v>
       </c>
       <c r="U355">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="V355">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="W355">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="X355">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="Y355">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="Z355">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="AA355">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="AB355">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="AC355">
-        <v>9.967460000000001</v>
+        <v>3.84558</v>
       </c>
       <c r="AD355">
-        <v>0</v>
+        <v>-4.95532</v>
       </c>
       <c r="AE355">
         <v>0</v>
       </c>
       <c r="AF355">
-        <v>1125.2928</v>
+        <v>322.74</v>
       </c>
       <c r="AG355">
         <v>0</v>
@@ -40357,7 +40442,7 @@
         <v>3</v>
       </c>
       <c r="AI355">
-        <v>2589.44043</v>
+        <v>1444.80597</v>
       </c>
     </row>
     <row r="356">
@@ -40376,20 +40461,20 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E356">
-        <v>292.0328333333334</v>
+        <v>94.3995</v>
       </c>
       <c r="F356">
-        <v>18011.81</v>
+        <v>8847.27</v>
       </c>
       <c r="G356">
-        <v>61.67734564092964</v>
+        <v>93.72157691513196</v>
       </c>
       <c r="H356">
-        <v>877.0899999999999</v>
+        <v>438.5399999999999</v>
       </c>
       <c r="I356">
         <v>0</v>
@@ -40398,13 +40483,13 @@
         <v>0</v>
       </c>
       <c r="K356">
-        <v>3.003395166182797</v>
+        <v>4.645575453259815</v>
       </c>
       <c r="L356">
         <v>0</v>
       </c>
       <c r="M356">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="N356">
         <v>0</v>
@@ -40419,37 +40504,37 @@
         <v>34.992</v>
       </c>
       <c r="R356">
-        <v>1558.2008</v>
+        <v>747.5897199999999</v>
       </c>
       <c r="S356">
-        <v>5.335704147421779</v>
+        <v>7.919424573223374</v>
       </c>
       <c r="T356">
-        <v>2692.46005</v>
+        <v>1346.14999</v>
       </c>
       <c r="U356">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="V356">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="W356">
+        <v>42</v>
+      </c>
+      <c r="X356">
         <v>84</v>
       </c>
-      <c r="X356">
-        <v>168</v>
-      </c>
       <c r="Y356">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="Z356">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="AA356">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="AB356">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="AC356">
         <v>4.10329</v>
@@ -40461,7 +40546,7 @@
         <v>0</v>
       </c>
       <c r="AF356">
-        <v>1453.43877</v>
+        <v>707.4776999999999</v>
       </c>
       <c r="AG356">
         <v>0</v>
@@ -40470,7 +40555,7 @@
         <v>3</v>
       </c>
       <c r="AI356">
-        <v>4674.6024</v>
+        <v>2242.76916</v>
       </c>
     </row>
     <row r="357">
@@ -40489,20 +40574,20 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E357">
-        <v>245.8588333333333</v>
+        <v>48.2255</v>
       </c>
       <c r="F357">
-        <v>7125.25</v>
+        <v>2765.01</v>
       </c>
       <c r="G357">
-        <v>28.98106162547207</v>
+        <v>57.33501985464122</v>
       </c>
       <c r="H357">
-        <v>347.96</v>
+        <v>124.46</v>
       </c>
       <c r="I357">
         <v>0</v>
@@ -40511,13 +40596,13 @@
         <v>0</v>
       </c>
       <c r="K357">
-        <v>1.415283702775238</v>
+        <v>2.580792319416076</v>
       </c>
       <c r="L357">
         <v>0</v>
       </c>
       <c r="M357">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N357">
         <v>0</v>
@@ -40532,37 +40617,37 @@
         <v>34.92</v>
       </c>
       <c r="R357">
-        <v>680.3570199999999</v>
+        <v>249.18753</v>
       </c>
       <c r="S357">
-        <v>2.767266934345115</v>
+        <v>5.167132118899752</v>
       </c>
       <c r="T357">
-        <v>1064.00998</v>
+        <v>423.82999</v>
       </c>
       <c r="U357">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="V357">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="W357">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="X357">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="Y357">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="Z357">
-        <v>71</v>
+        <v>30</v>
       </c>
       <c r="AA357">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="AB357">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="AC357">
         <v>3.92378</v>
@@ -40574,7 +40659,7 @@
         <v>0</v>
       </c>
       <c r="AF357">
-        <v>671.5824</v>
+        <v>261.8984</v>
       </c>
       <c r="AG357">
         <v>0</v>
@@ -40583,7 +40668,7 @@
         <v>3</v>
       </c>
       <c r="AI357">
-        <v>2041.07106</v>
+        <v>747.56259</v>
       </c>
     </row>
     <row r="358">
@@ -40602,38 +40687,38 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E358">
-        <v>292.0328333333334</v>
+        <v>94.3995</v>
       </c>
       <c r="F358">
-        <v>15422.71</v>
+        <v>7543.74</v>
       </c>
       <c r="G358">
-        <v>52.81156171366575</v>
+        <v>79.91292326760205</v>
       </c>
       <c r="H358">
-        <v>1283.57</v>
+        <v>641.78</v>
       </c>
       <c r="I358">
-        <v>10.12</v>
+        <v>5.06</v>
       </c>
       <c r="J358">
         <v>0</v>
       </c>
       <c r="K358">
-        <v>4.395293451592487</v>
+        <v>6.79855295843728</v>
       </c>
       <c r="L358">
-        <v>30.12</v>
+        <v>15.06</v>
       </c>
       <c r="M358">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="N358">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O358">
         <v>31.46879</v>
@@ -40645,37 +40730,37 @@
         <v>34.992</v>
       </c>
       <c r="R358">
-        <v>1322.82834</v>
+        <v>631.34887</v>
       </c>
       <c r="S358">
-        <v>4.529724705612439</v>
+        <v>6.688053114688108</v>
       </c>
       <c r="T358">
-        <v>3115.13007</v>
+        <v>1550.51007</v>
       </c>
       <c r="U358">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="V358">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="W358">
-        <v>147</v>
+        <v>73</v>
       </c>
       <c r="X358">
-        <v>181</v>
+        <v>89</v>
       </c>
       <c r="Y358">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="Z358">
-        <v>182</v>
+        <v>91</v>
       </c>
       <c r="AA358">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="AB358">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="AC358">
         <v>4.69417</v>
@@ -40687,7 +40772,7 @@
         <v>0</v>
       </c>
       <c r="AF358">
-        <v>1373.25928</v>
+        <v>652.88618</v>
       </c>
       <c r="AG358">
         <v>0</v>
@@ -40696,7 +40781,7 @@
         <v>3</v>
       </c>
       <c r="AI358">
-        <v>3968.48502</v>
+        <v>1894.04661</v>
       </c>
     </row>
     <row r="359">
@@ -40708,19 +40793,24 @@
       <c r="B359" s="2">
         <v>46207</v>
       </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Activity 20260704185730 | Activity 20260704161350</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E359">
-        <v>66.81666666666666</v>
+        <v>94.3995</v>
       </c>
       <c r="F359">
-        <v>0</v>
+        <v>9301.27</v>
       </c>
       <c r="G359">
-        <v>0</v>
+        <v>98.53092442226918</v>
       </c>
       <c r="H359">
         <v>0</v>
@@ -40744,19 +40834,19 @@
         <v>0</v>
       </c>
       <c r="O359">
-        <v>0.00401</v>
+        <v>30.85394</v>
       </c>
       <c r="P359">
-        <v>0.01179967043314501</v>
+        <v>85.70538888888889</v>
       </c>
       <c r="Q359">
-        <v>33.984</v>
+        <v>36</v>
       </c>
       <c r="R359">
-        <v>9.305240000000001</v>
+        <v>892.79669</v>
       </c>
       <c r="S359">
-        <v>0.1392652531803442</v>
+        <v>9.457642148528329</v>
       </c>
       <c r="T359">
         <v>0</v>
@@ -40783,13 +40873,13 @@
         <v>0</v>
       </c>
       <c r="AB359">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC359">
-        <v>0</v>
+        <v>4.47009</v>
       </c>
       <c r="AD359">
-        <v>0</v>
+        <v>-4.259</v>
       </c>
       <c r="AE359">
         <v>0</v>
@@ -40804,7 +40894,7 @@
         <v>3</v>
       </c>
       <c r="AI359">
-        <v>27.91572</v>
+        <v>2678.39007</v>
       </c>
     </row>
     <row r="360">
@@ -40823,20 +40913,20 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E360">
-        <v>258.8775</v>
+        <v>60.18500000000001</v>
       </c>
       <c r="F360">
-        <v>11764.28</v>
+        <v>4868.29</v>
       </c>
       <c r="G360">
-        <v>45.44342401328814</v>
+        <v>80.88875965772201</v>
       </c>
       <c r="H360">
-        <v>494.3</v>
+        <v>158.53</v>
       </c>
       <c r="I360">
         <v>0</v>
@@ -40845,70 +40935,70 @@
         <v>0</v>
       </c>
       <c r="K360">
-        <v>1.909397301812633</v>
+        <v>2.634045027830854</v>
       </c>
       <c r="L360">
         <v>0</v>
       </c>
       <c r="M360">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N360">
         <v>0</v>
       </c>
       <c r="O360">
-        <v>26.40669</v>
+        <v>24.47792</v>
       </c>
       <c r="P360">
-        <v>75.46493484224966</v>
+        <v>69.95290352080477</v>
       </c>
       <c r="Q360">
         <v>34.992</v>
       </c>
       <c r="R360">
-        <v>1119.21103</v>
+        <v>443.73477</v>
       </c>
       <c r="S360">
-        <v>4.323322923004123</v>
+        <v>7.372846556450942</v>
       </c>
       <c r="T360">
-        <v>2038.59997</v>
+        <v>829.59998</v>
       </c>
       <c r="U360">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="V360">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="W360">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="X360">
-        <v>130</v>
+        <v>51</v>
       </c>
       <c r="Y360">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="Z360">
-        <v>118</v>
+        <v>48</v>
       </c>
       <c r="AA360">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="AB360">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="AC360">
-        <v>3.83877</v>
+        <v>3.82955</v>
       </c>
       <c r="AD360">
-        <v>-2.70335</v>
+        <v>-2.69074</v>
       </c>
       <c r="AE360">
         <v>0</v>
       </c>
       <c r="AF360">
-        <v>1112.8176</v>
+        <v>454.9639999999999</v>
       </c>
       <c r="AG360">
         <v>0</v>
@@ -40917,7 +41007,7 @@
         <v>3</v>
       </c>
       <c r="AI360">
-        <v>3357.63309</v>
+        <v>1331.20431</v>
       </c>
     </row>
     <row r="361">
@@ -40936,83 +41026,83 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>Activity 20260704223835 | Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E361">
-        <v>450.1495</v>
+        <v>94.3995</v>
       </c>
       <c r="F361">
-        <v>20173.03</v>
+        <v>9505.459999999999</v>
       </c>
       <c r="G361">
-        <v>44.81406732652152</v>
+        <v>100.6939655400717</v>
       </c>
       <c r="H361">
-        <v>669.1700000000001</v>
+        <v>301.55</v>
       </c>
       <c r="I361">
-        <v>40.56</v>
+        <v>10.02</v>
       </c>
       <c r="J361">
+        <v>1</v>
+      </c>
+      <c r="K361">
+        <v>3.194402512725173</v>
+      </c>
+      <c r="L361">
+        <v>10.02</v>
+      </c>
+      <c r="M361">
         <v>4</v>
       </c>
-      <c r="K361">
-        <v>1.486550579307541</v>
-      </c>
-      <c r="L361">
-        <v>37.48</v>
-      </c>
-      <c r="M361">
-        <v>10</v>
-      </c>
       <c r="N361">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O361">
-        <v>266.83429</v>
+        <v>30.85394</v>
       </c>
       <c r="P361">
-        <v>808.2948321822367</v>
+        <v>93.4628014055495</v>
       </c>
       <c r="Q361">
         <v>33.012</v>
       </c>
       <c r="R361">
-        <v>1871.74762</v>
+        <v>878.50073</v>
       </c>
       <c r="S361">
-        <v>4.158057756367606</v>
+        <v>9.306201092166802</v>
       </c>
       <c r="T361">
-        <v>3503.80995</v>
+        <v>1379.32996</v>
       </c>
       <c r="U361">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="V361">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="W361">
-        <v>107</v>
+        <v>50</v>
       </c>
       <c r="X361">
-        <v>209</v>
+        <v>103</v>
       </c>
       <c r="Y361">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="Z361">
-        <v>189</v>
+        <v>92</v>
       </c>
       <c r="AA361">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="AB361">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="AC361">
-        <v>6.86781</v>
+        <v>4.48906</v>
       </c>
       <c r="AD361">
         <v>-4.259</v>
@@ -41021,7 +41111,7 @@
         <v>0</v>
       </c>
       <c r="AF361">
-        <v>1844.74575</v>
+        <v>833.70975</v>
       </c>
       <c r="AG361">
         <v>0</v>
@@ -41030,7 +41120,7 @@
         <v>3</v>
       </c>
       <c r="AI361">
-        <v>5615.24286</v>
+        <v>2635.50219</v>
       </c>
     </row>
     <row r="362">
@@ -41049,20 +41139,20 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Amistoso vs Tampico | Activity 20260704185730</t>
+          <t>Amistoso vs Tampico</t>
         </is>
       </c>
       <c r="E362">
-        <v>292.0328333333334</v>
+        <v>94.3995</v>
       </c>
       <c r="F362">
-        <v>13204.55</v>
+        <v>6454.940000000001</v>
       </c>
       <c r="G362">
-        <v>45.21597742719567</v>
+        <v>68.37896387163067</v>
       </c>
       <c r="H362">
-        <v>443.26</v>
+        <v>221.63</v>
       </c>
       <c r="I362">
         <v>0</v>
@@ -41071,13 +41161,13 @@
         <v>0</v>
       </c>
       <c r="K362">
-        <v>1.517843027924371</v>
+        <v>2.347787859045864</v>
       </c>
       <c r="L362">
         <v>0</v>
       </c>
       <c r="M362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N362">
         <v>0</v>
@@ -41092,37 +41182,37 @@
         <v>32.004</v>
       </c>
       <c r="R362">
-        <v>1221.18793</v>
+        <v>582.8236400000001</v>
       </c>
       <c r="S362">
-        <v>4.181680244858311</v>
+        <v>6.174011938622557</v>
       </c>
       <c r="T362">
-        <v>1907.04997</v>
+        <v>953.19999</v>
       </c>
       <c r="U362">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="V362">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="W362">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="X362">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="Y362">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="Z362">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="AA362">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="AB362">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="AC362">
         <v>3.98444</v>
@@ -41134,7 +41224,7 @@
         <v>0</v>
       </c>
       <c r="AF362">
-        <v>1107.6352</v>
+        <v>526.1949000000001</v>
       </c>
       <c r="AG362">
         <v>0</v>
@@ -41143,7 +41233,1815 @@
         <v>3</v>
       </c>
       <c r="AI362">
-        <v>3663.56379</v>
+        <v>1748.47092</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B363" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E363">
+        <v>69.7</v>
+      </c>
+      <c r="F363">
+        <v>2877.2</v>
+      </c>
+      <c r="G363">
+        <v>41.27977044476327</v>
+      </c>
+      <c r="H363">
+        <v>0</v>
+      </c>
+      <c r="I363">
+        <v>0</v>
+      </c>
+      <c r="J363">
+        <v>0</v>
+      </c>
+      <c r="K363">
+        <v>0</v>
+      </c>
+      <c r="L363">
+        <v>0</v>
+      </c>
+      <c r="M363">
+        <v>0</v>
+      </c>
+      <c r="N363">
+        <v>0</v>
+      </c>
+      <c r="O363">
+        <v>19.03212</v>
+      </c>
+      <c r="P363">
+        <v>58.80645161290323</v>
+      </c>
+      <c r="Q363">
+        <v>32.364</v>
+      </c>
+      <c r="R363">
+        <v>318.02921</v>
+      </c>
+      <c r="S363">
+        <v>4.562829411764707</v>
+      </c>
+      <c r="T363">
+        <v>354.45999</v>
+      </c>
+      <c r="U363">
+        <v>11</v>
+      </c>
+      <c r="V363">
+        <v>16</v>
+      </c>
+      <c r="W363">
+        <v>27</v>
+      </c>
+      <c r="X363">
+        <v>63</v>
+      </c>
+      <c r="Y363">
+        <v>11</v>
+      </c>
+      <c r="Z363">
+        <v>60</v>
+      </c>
+      <c r="AA363">
+        <v>16</v>
+      </c>
+      <c r="AB363">
+        <v>35</v>
+      </c>
+      <c r="AC363">
+        <v>3.49302</v>
+      </c>
+      <c r="AD363">
+        <v>-2.83458</v>
+      </c>
+      <c r="AE363">
+        <v>0</v>
+      </c>
+      <c r="AF363">
+        <v>241.5084</v>
+      </c>
+      <c r="AG363">
+        <v>0</v>
+      </c>
+      <c r="AH363">
+        <v>3</v>
+      </c>
+      <c r="AI363">
+        <v>954.0876300000001</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B364" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E364">
+        <v>69.7</v>
+      </c>
+      <c r="F364">
+        <v>3258.73</v>
+      </c>
+      <c r="G364">
+        <v>46.75365853658536</v>
+      </c>
+      <c r="H364">
+        <v>0.95</v>
+      </c>
+      <c r="I364">
+        <v>0</v>
+      </c>
+      <c r="J364">
+        <v>0</v>
+      </c>
+      <c r="K364">
+        <v>0.01362984218077475</v>
+      </c>
+      <c r="L364">
+        <v>0</v>
+      </c>
+      <c r="M364">
+        <v>0</v>
+      </c>
+      <c r="N364">
+        <v>0</v>
+      </c>
+      <c r="O364">
+        <v>20.99707</v>
+      </c>
+      <c r="P364">
+        <v>64.80577160493827</v>
+      </c>
+      <c r="Q364">
+        <v>32.4</v>
+      </c>
+      <c r="R364">
+        <v>460.20196</v>
+      </c>
+      <c r="S364">
+        <v>6.602610616929698</v>
+      </c>
+      <c r="T364">
+        <v>562.02</v>
+      </c>
+      <c r="U364">
+        <v>36</v>
+      </c>
+      <c r="V364">
+        <v>28</v>
+      </c>
+      <c r="W364">
+        <v>64</v>
+      </c>
+      <c r="X364">
+        <v>106</v>
+      </c>
+      <c r="Y364">
+        <v>36</v>
+      </c>
+      <c r="Z364">
+        <v>78</v>
+      </c>
+      <c r="AA364">
+        <v>28</v>
+      </c>
+      <c r="AB364">
+        <v>34</v>
+      </c>
+      <c r="AC364">
+        <v>3.90562</v>
+      </c>
+      <c r="AD364">
+        <v>-3.18606</v>
+      </c>
+      <c r="AE364">
+        <v>0</v>
+      </c>
+      <c r="AF364">
+        <v>289.2974</v>
+      </c>
+      <c r="AG364">
+        <v>0</v>
+      </c>
+      <c r="AH364">
+        <v>3</v>
+      </c>
+      <c r="AI364">
+        <v>1380.60588</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B365" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E365">
+        <v>69.7</v>
+      </c>
+      <c r="F365">
+        <v>2776.56</v>
+      </c>
+      <c r="G365">
+        <v>39.83586800573888</v>
+      </c>
+      <c r="H365">
+        <v>17.52</v>
+      </c>
+      <c r="I365">
+        <v>0</v>
+      </c>
+      <c r="J365">
+        <v>0</v>
+      </c>
+      <c r="K365">
+        <v>0.2513629842180775</v>
+      </c>
+      <c r="L365">
+        <v>0</v>
+      </c>
+      <c r="M365">
+        <v>0</v>
+      </c>
+      <c r="N365">
+        <v>0</v>
+      </c>
+      <c r="O365">
+        <v>23.81896</v>
+      </c>
+      <c r="P365">
+        <v>70.08874764595103</v>
+      </c>
+      <c r="Q365">
+        <v>33.984</v>
+      </c>
+      <c r="R365">
+        <v>396.32672</v>
+      </c>
+      <c r="S365">
+        <v>5.68617962697274</v>
+      </c>
+      <c r="T365">
+        <v>245.6</v>
+      </c>
+      <c r="U365">
+        <v>8</v>
+      </c>
+      <c r="V365">
+        <v>3</v>
+      </c>
+      <c r="W365">
+        <v>11</v>
+      </c>
+      <c r="X365">
+        <v>45</v>
+      </c>
+      <c r="Y365">
+        <v>8</v>
+      </c>
+      <c r="Z365">
+        <v>45</v>
+      </c>
+      <c r="AA365">
+        <v>3</v>
+      </c>
+      <c r="AB365">
+        <v>14</v>
+      </c>
+      <c r="AC365">
+        <v>3.45041</v>
+      </c>
+      <c r="AD365">
+        <v>-2.77883</v>
+      </c>
+      <c r="AE365">
+        <v>0</v>
+      </c>
+      <c r="AF365">
+        <v>258.1776</v>
+      </c>
+      <c r="AG365">
+        <v>0</v>
+      </c>
+      <c r="AH365">
+        <v>3</v>
+      </c>
+      <c r="AI365">
+        <v>1188.98016</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B366" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E366">
+        <v>69.7</v>
+      </c>
+      <c r="F366">
+        <v>3262.38</v>
+      </c>
+      <c r="G366">
+        <v>46.80602582496412</v>
+      </c>
+      <c r="H366">
+        <v>0</v>
+      </c>
+      <c r="I366">
+        <v>0</v>
+      </c>
+      <c r="J366">
+        <v>0</v>
+      </c>
+      <c r="K366">
+        <v>0</v>
+      </c>
+      <c r="L366">
+        <v>0</v>
+      </c>
+      <c r="M366">
+        <v>0</v>
+      </c>
+      <c r="N366">
+        <v>0</v>
+      </c>
+      <c r="O366">
+        <v>20.2555</v>
+      </c>
+      <c r="P366">
+        <v>56.94866171839856</v>
+      </c>
+      <c r="Q366">
+        <v>35.568</v>
+      </c>
+      <c r="R366">
+        <v>377.15638</v>
+      </c>
+      <c r="S366">
+        <v>5.411138880918221</v>
+      </c>
+      <c r="T366">
+        <v>557.99</v>
+      </c>
+      <c r="U366">
+        <v>51</v>
+      </c>
+      <c r="V366">
+        <v>34</v>
+      </c>
+      <c r="W366">
+        <v>85</v>
+      </c>
+      <c r="X366">
+        <v>114</v>
+      </c>
+      <c r="Y366">
+        <v>51</v>
+      </c>
+      <c r="Z366">
+        <v>96</v>
+      </c>
+      <c r="AA366">
+        <v>34</v>
+      </c>
+      <c r="AB366">
+        <v>30</v>
+      </c>
+      <c r="AC366">
+        <v>4.27991</v>
+      </c>
+      <c r="AD366">
+        <v>-3.53589</v>
+      </c>
+      <c r="AE366">
+        <v>0</v>
+      </c>
+      <c r="AF366">
+        <v>342.752</v>
+      </c>
+      <c r="AG366">
+        <v>0</v>
+      </c>
+      <c r="AH366">
+        <v>3</v>
+      </c>
+      <c r="AI366">
+        <v>1131.46914</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B367" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E367">
+        <v>69.7</v>
+      </c>
+      <c r="F367">
+        <v>3533.39</v>
+      </c>
+      <c r="G367">
+        <v>50.69426111908177</v>
+      </c>
+      <c r="H367">
+        <v>22.95</v>
+      </c>
+      <c r="I367">
+        <v>0</v>
+      </c>
+      <c r="J367">
+        <v>0</v>
+      </c>
+      <c r="K367">
+        <v>0.3292682926829268</v>
+      </c>
+      <c r="L367">
+        <v>0</v>
+      </c>
+      <c r="M367">
+        <v>0</v>
+      </c>
+      <c r="N367">
+        <v>0</v>
+      </c>
+      <c r="O367">
+        <v>24.0091</v>
+      </c>
+      <c r="P367">
+        <v>66.69194444444445</v>
+      </c>
+      <c r="Q367">
+        <v>36</v>
+      </c>
+      <c r="R367">
+        <v>459.22363</v>
+      </c>
+      <c r="S367">
+        <v>6.588574318507891</v>
+      </c>
+      <c r="T367">
+        <v>631.57999</v>
+      </c>
+      <c r="U367">
+        <v>47</v>
+      </c>
+      <c r="V367">
+        <v>36</v>
+      </c>
+      <c r="W367">
+        <v>83</v>
+      </c>
+      <c r="X367">
+        <v>127</v>
+      </c>
+      <c r="Y367">
+        <v>47</v>
+      </c>
+      <c r="Z367">
+        <v>107</v>
+      </c>
+      <c r="AA367">
+        <v>36</v>
+      </c>
+      <c r="AB367">
+        <v>49</v>
+      </c>
+      <c r="AC367">
+        <v>4.22953</v>
+      </c>
+      <c r="AD367">
+        <v>-4.17897</v>
+      </c>
+      <c r="AE367">
+        <v>0</v>
+      </c>
+      <c r="AF367">
+        <v>322.147</v>
+      </c>
+      <c r="AG367">
+        <v>0</v>
+      </c>
+      <c r="AH367">
+        <v>3</v>
+      </c>
+      <c r="AI367">
+        <v>1377.67089</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B368" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E368">
+        <v>69.7</v>
+      </c>
+      <c r="F368">
+        <v>2570.85</v>
+      </c>
+      <c r="G368">
+        <v>36.8845050215208</v>
+      </c>
+      <c r="H368">
+        <v>13.81</v>
+      </c>
+      <c r="I368">
+        <v>0</v>
+      </c>
+      <c r="J368">
+        <v>0</v>
+      </c>
+      <c r="K368">
+        <v>0.1981348637015782</v>
+      </c>
+      <c r="L368">
+        <v>0</v>
+      </c>
+      <c r="M368">
+        <v>0</v>
+      </c>
+      <c r="N368">
+        <v>0</v>
+      </c>
+      <c r="O368">
+        <v>22.85205</v>
+      </c>
+      <c r="P368">
+        <v>71.40373078365204</v>
+      </c>
+      <c r="Q368">
+        <v>32.004</v>
+      </c>
+      <c r="R368">
+        <v>331.94508</v>
+      </c>
+      <c r="S368">
+        <v>4.762483213773314</v>
+      </c>
+      <c r="T368">
+        <v>392.06</v>
+      </c>
+      <c r="U368">
+        <v>22</v>
+      </c>
+      <c r="V368">
+        <v>20</v>
+      </c>
+      <c r="W368">
+        <v>42</v>
+      </c>
+      <c r="X368">
+        <v>66</v>
+      </c>
+      <c r="Y368">
+        <v>22</v>
+      </c>
+      <c r="Z368">
+        <v>63</v>
+      </c>
+      <c r="AA368">
+        <v>20</v>
+      </c>
+      <c r="AB368">
+        <v>14</v>
+      </c>
+      <c r="AC368">
+        <v>4.07591</v>
+      </c>
+      <c r="AD368">
+        <v>-2.80633</v>
+      </c>
+      <c r="AE368">
+        <v>0</v>
+      </c>
+      <c r="AF368">
+        <v>190.7094</v>
+      </c>
+      <c r="AG368">
+        <v>0</v>
+      </c>
+      <c r="AH368">
+        <v>3</v>
+      </c>
+      <c r="AI368">
+        <v>995.8352400000001</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B369" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E369">
+        <v>69.7</v>
+      </c>
+      <c r="F369">
+        <v>2764.9</v>
+      </c>
+      <c r="G369">
+        <v>39.66857962697274</v>
+      </c>
+      <c r="H369">
+        <v>26.07</v>
+      </c>
+      <c r="I369">
+        <v>0</v>
+      </c>
+      <c r="J369">
+        <v>0</v>
+      </c>
+      <c r="K369">
+        <v>0.3740315638450502</v>
+      </c>
+      <c r="L369">
+        <v>0</v>
+      </c>
+      <c r="M369">
+        <v>0</v>
+      </c>
+      <c r="N369">
+        <v>0</v>
+      </c>
+      <c r="O369">
+        <v>24.4573</v>
+      </c>
+      <c r="P369">
+        <v>72.27334515366429</v>
+      </c>
+      <c r="Q369">
+        <v>33.84</v>
+      </c>
+      <c r="R369">
+        <v>339.82262</v>
+      </c>
+      <c r="S369">
+        <v>4.87550387374462</v>
+      </c>
+      <c r="T369">
+        <v>433.2</v>
+      </c>
+      <c r="U369">
+        <v>15</v>
+      </c>
+      <c r="V369">
+        <v>27</v>
+      </c>
+      <c r="W369">
+        <v>42</v>
+      </c>
+      <c r="X369">
+        <v>75</v>
+      </c>
+      <c r="Y369">
+        <v>15</v>
+      </c>
+      <c r="Z369">
+        <v>82</v>
+      </c>
+      <c r="AA369">
+        <v>27</v>
+      </c>
+      <c r="AB369">
+        <v>36</v>
+      </c>
+      <c r="AC369">
+        <v>4.17768</v>
+      </c>
+      <c r="AD369">
+        <v>0</v>
+      </c>
+      <c r="AE369">
+        <v>0</v>
+      </c>
+      <c r="AF369">
+        <v>248.6722</v>
+      </c>
+      <c r="AG369">
+        <v>0</v>
+      </c>
+      <c r="AH369">
+        <v>3</v>
+      </c>
+      <c r="AI369">
+        <v>1019.46786</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B370" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E370">
+        <v>52.9</v>
+      </c>
+      <c r="F370">
+        <v>2378.3</v>
+      </c>
+      <c r="G370">
+        <v>44.95841209829867</v>
+      </c>
+      <c r="H370">
+        <v>0</v>
+      </c>
+      <c r="I370">
+        <v>0</v>
+      </c>
+      <c r="J370">
+        <v>0</v>
+      </c>
+      <c r="K370">
+        <v>0</v>
+      </c>
+      <c r="L370">
+        <v>0</v>
+      </c>
+      <c r="M370">
+        <v>0</v>
+      </c>
+      <c r="N370">
+        <v>0</v>
+      </c>
+      <c r="O370">
+        <v>20.82891</v>
+      </c>
+      <c r="P370">
+        <v>61.81419159544161</v>
+      </c>
+      <c r="Q370">
+        <v>33.696</v>
+      </c>
+      <c r="R370">
+        <v>319.44484</v>
+      </c>
+      <c r="S370">
+        <v>6.038654820415879</v>
+      </c>
+      <c r="T370">
+        <v>366.78001</v>
+      </c>
+      <c r="U370">
+        <v>29</v>
+      </c>
+      <c r="V370">
+        <v>27</v>
+      </c>
+      <c r="W370">
+        <v>56</v>
+      </c>
+      <c r="X370">
+        <v>68</v>
+      </c>
+      <c r="Y370">
+        <v>29</v>
+      </c>
+      <c r="Z370">
+        <v>66</v>
+      </c>
+      <c r="AA370">
+        <v>27</v>
+      </c>
+      <c r="AB370">
+        <v>27</v>
+      </c>
+      <c r="AC370">
+        <v>3.90287</v>
+      </c>
+      <c r="AD370">
+        <v>-3.8237</v>
+      </c>
+      <c r="AE370">
+        <v>0</v>
+      </c>
+      <c r="AF370">
+        <v>244.3544</v>
+      </c>
+      <c r="AG370">
+        <v>0</v>
+      </c>
+      <c r="AH370">
+        <v>3</v>
+      </c>
+      <c r="AI370">
+        <v>958.33452</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B371" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E371">
+        <v>52.9</v>
+      </c>
+      <c r="F371">
+        <v>2561.25</v>
+      </c>
+      <c r="G371">
+        <v>48.41682419659735</v>
+      </c>
+      <c r="H371">
+        <v>0</v>
+      </c>
+      <c r="I371">
+        <v>0</v>
+      </c>
+      <c r="J371">
+        <v>0</v>
+      </c>
+      <c r="K371">
+        <v>0</v>
+      </c>
+      <c r="L371">
+        <v>0</v>
+      </c>
+      <c r="M371">
+        <v>0</v>
+      </c>
+      <c r="N371">
+        <v>0</v>
+      </c>
+      <c r="O371">
+        <v>19.50083</v>
+      </c>
+      <c r="P371">
+        <v>55.72939529035209</v>
+      </c>
+      <c r="Q371">
+        <v>34.992</v>
+      </c>
+      <c r="R371">
+        <v>292.66553</v>
+      </c>
+      <c r="S371">
+        <v>5.532429678638941</v>
+      </c>
+      <c r="T371">
+        <v>344.53</v>
+      </c>
+      <c r="U371">
+        <v>19</v>
+      </c>
+      <c r="V371">
+        <v>10</v>
+      </c>
+      <c r="W371">
+        <v>29</v>
+      </c>
+      <c r="X371">
+        <v>82</v>
+      </c>
+      <c r="Y371">
+        <v>19</v>
+      </c>
+      <c r="Z371">
+        <v>75</v>
+      </c>
+      <c r="AA371">
+        <v>10</v>
+      </c>
+      <c r="AB371">
+        <v>22</v>
+      </c>
+      <c r="AC371">
+        <v>4.09066</v>
+      </c>
+      <c r="AD371">
+        <v>-2.87678</v>
+      </c>
+      <c r="AE371">
+        <v>0</v>
+      </c>
+      <c r="AF371">
+        <v>221.57142</v>
+      </c>
+      <c r="AG371">
+        <v>0</v>
+      </c>
+      <c r="AH371">
+        <v>3</v>
+      </c>
+      <c r="AI371">
+        <v>877.99659</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B372" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E372">
+        <v>52.9</v>
+      </c>
+      <c r="F372">
+        <v>2350.71</v>
+      </c>
+      <c r="G372">
+        <v>44.43686200378073</v>
+      </c>
+      <c r="H372">
+        <v>0</v>
+      </c>
+      <c r="I372">
+        <v>0</v>
+      </c>
+      <c r="J372">
+        <v>0</v>
+      </c>
+      <c r="K372">
+        <v>0</v>
+      </c>
+      <c r="L372">
+        <v>0</v>
+      </c>
+      <c r="M372">
+        <v>0</v>
+      </c>
+      <c r="N372">
+        <v>0</v>
+      </c>
+      <c r="O372">
+        <v>20.70838</v>
+      </c>
+      <c r="P372">
+        <v>59.30234822451317</v>
+      </c>
+      <c r="Q372">
+        <v>34.92</v>
+      </c>
+      <c r="R372">
+        <v>289.3408</v>
+      </c>
+      <c r="S372">
+        <v>5.469580340264651</v>
+      </c>
+      <c r="T372">
+        <v>322.50999</v>
+      </c>
+      <c r="U372">
+        <v>20</v>
+      </c>
+      <c r="V372">
+        <v>15</v>
+      </c>
+      <c r="W372">
+        <v>35</v>
+      </c>
+      <c r="X372">
+        <v>62</v>
+      </c>
+      <c r="Y372">
+        <v>20</v>
+      </c>
+      <c r="Z372">
+        <v>52</v>
+      </c>
+      <c r="AA372">
+        <v>15</v>
+      </c>
+      <c r="AB372">
+        <v>21</v>
+      </c>
+      <c r="AC372">
+        <v>4.20597</v>
+      </c>
+      <c r="AD372">
+        <v>-3.19234</v>
+      </c>
+      <c r="AE372">
+        <v>0</v>
+      </c>
+      <c r="AF372">
+        <v>233.7776</v>
+      </c>
+      <c r="AG372">
+        <v>0</v>
+      </c>
+      <c r="AH372">
+        <v>3</v>
+      </c>
+      <c r="AI372">
+        <v>868.0224000000001</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B373" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E373">
+        <v>69.7</v>
+      </c>
+      <c r="F373">
+        <v>2966.17</v>
+      </c>
+      <c r="G373">
+        <v>42.55624103299856</v>
+      </c>
+      <c r="H373">
+        <v>0</v>
+      </c>
+      <c r="I373">
+        <v>0</v>
+      </c>
+      <c r="J373">
+        <v>0</v>
+      </c>
+      <c r="K373">
+        <v>0</v>
+      </c>
+      <c r="L373">
+        <v>0</v>
+      </c>
+      <c r="M373">
+        <v>0</v>
+      </c>
+      <c r="N373">
+        <v>0</v>
+      </c>
+      <c r="O373">
+        <v>20.34281</v>
+      </c>
+      <c r="P373">
+        <v>58.13560242341107</v>
+      </c>
+      <c r="Q373">
+        <v>34.992</v>
+      </c>
+      <c r="R373">
+        <v>316.80447</v>
+      </c>
+      <c r="S373">
+        <v>4.545257819225252</v>
+      </c>
+      <c r="T373">
+        <v>444.77001</v>
+      </c>
+      <c r="U373">
+        <v>21</v>
+      </c>
+      <c r="V373">
+        <v>21</v>
+      </c>
+      <c r="W373">
+        <v>42</v>
+      </c>
+      <c r="X373">
+        <v>89</v>
+      </c>
+      <c r="Y373">
+        <v>21</v>
+      </c>
+      <c r="Z373">
+        <v>72</v>
+      </c>
+      <c r="AA373">
+        <v>21</v>
+      </c>
+      <c r="AB373">
+        <v>67</v>
+      </c>
+      <c r="AC373">
+        <v>3.85945</v>
+      </c>
+      <c r="AD373">
+        <v>-3.44306</v>
+      </c>
+      <c r="AE373">
+        <v>0</v>
+      </c>
+      <c r="AF373">
+        <v>269.5799</v>
+      </c>
+      <c r="AG373">
+        <v>0</v>
+      </c>
+      <c r="AH373">
+        <v>3</v>
+      </c>
+      <c r="AI373">
+        <v>950.4134100000001</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B374" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E374">
+        <v>69.7</v>
+      </c>
+      <c r="F374">
+        <v>2790.93</v>
+      </c>
+      <c r="G374">
+        <v>40.04203730272597</v>
+      </c>
+      <c r="H374">
+        <v>6.880000000000001</v>
+      </c>
+      <c r="I374">
+        <v>0</v>
+      </c>
+      <c r="J374">
+        <v>0</v>
+      </c>
+      <c r="K374">
+        <v>0.09870875179340029</v>
+      </c>
+      <c r="L374">
+        <v>0</v>
+      </c>
+      <c r="M374">
+        <v>0</v>
+      </c>
+      <c r="N374">
+        <v>0</v>
+      </c>
+      <c r="O374">
+        <v>21.13979</v>
+      </c>
+      <c r="P374">
+        <v>62.20512594161958</v>
+      </c>
+      <c r="Q374">
+        <v>33.984</v>
+      </c>
+      <c r="R374">
+        <v>385.37218</v>
+      </c>
+      <c r="S374">
+        <v>5.52901262553802</v>
+      </c>
+      <c r="T374">
+        <v>385.94</v>
+      </c>
+      <c r="U374">
+        <v>16</v>
+      </c>
+      <c r="V374">
+        <v>17</v>
+      </c>
+      <c r="W374">
+        <v>33</v>
+      </c>
+      <c r="X374">
+        <v>65</v>
+      </c>
+      <c r="Y374">
+        <v>16</v>
+      </c>
+      <c r="Z374">
+        <v>60</v>
+      </c>
+      <c r="AA374">
+        <v>17</v>
+      </c>
+      <c r="AB374">
+        <v>53</v>
+      </c>
+      <c r="AC374">
+        <v>3.92536</v>
+      </c>
+      <c r="AD374">
+        <v>-3.08303</v>
+      </c>
+      <c r="AE374">
+        <v>0</v>
+      </c>
+      <c r="AF374">
+        <v>275.612</v>
+      </c>
+      <c r="AG374">
+        <v>0</v>
+      </c>
+      <c r="AH374">
+        <v>3</v>
+      </c>
+      <c r="AI374">
+        <v>1156.11654</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B375" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E375">
+        <v>69.7</v>
+      </c>
+      <c r="F375">
+        <v>2546.24</v>
+      </c>
+      <c r="G375">
+        <v>36.53142037302726</v>
+      </c>
+      <c r="H375">
+        <v>0</v>
+      </c>
+      <c r="I375">
+        <v>0</v>
+      </c>
+      <c r="J375">
+        <v>0</v>
+      </c>
+      <c r="K375">
+        <v>0</v>
+      </c>
+      <c r="L375">
+        <v>0</v>
+      </c>
+      <c r="M375">
+        <v>0</v>
+      </c>
+      <c r="N375">
+        <v>0</v>
+      </c>
+      <c r="O375">
+        <v>19.95648</v>
+      </c>
+      <c r="P375">
+        <v>57.03155006858711</v>
+      </c>
+      <c r="Q375">
+        <v>34.992</v>
+      </c>
+      <c r="R375">
+        <v>326.65239</v>
+      </c>
+      <c r="S375">
+        <v>4.686547919655666</v>
+      </c>
+      <c r="T375">
+        <v>404.81</v>
+      </c>
+      <c r="U375">
+        <v>15</v>
+      </c>
+      <c r="V375">
+        <v>19</v>
+      </c>
+      <c r="W375">
+        <v>34</v>
+      </c>
+      <c r="X375">
+        <v>84</v>
+      </c>
+      <c r="Y375">
+        <v>15</v>
+      </c>
+      <c r="Z375">
+        <v>76</v>
+      </c>
+      <c r="AA375">
+        <v>19</v>
+      </c>
+      <c r="AB375">
+        <v>38</v>
+      </c>
+      <c r="AC375">
+        <v>3.89727</v>
+      </c>
+      <c r="AD375">
+        <v>0</v>
+      </c>
+      <c r="AE375">
+        <v>0</v>
+      </c>
+      <c r="AF375">
+        <v>255.6072</v>
+      </c>
+      <c r="AG375">
+        <v>0</v>
+      </c>
+      <c r="AH375">
+        <v>3</v>
+      </c>
+      <c r="AI375">
+        <v>979.9571699999999</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B376" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E376">
+        <v>69.7</v>
+      </c>
+      <c r="F376">
+        <v>2924.54</v>
+      </c>
+      <c r="G376">
+        <v>41.95896700143471</v>
+      </c>
+      <c r="H376">
+        <v>11.97</v>
+      </c>
+      <c r="I376">
+        <v>0</v>
+      </c>
+      <c r="J376">
+        <v>0</v>
+      </c>
+      <c r="K376">
+        <v>0.1717360114777618</v>
+      </c>
+      <c r="L376">
+        <v>0</v>
+      </c>
+      <c r="M376">
+        <v>0</v>
+      </c>
+      <c r="N376">
+        <v>0</v>
+      </c>
+      <c r="O376">
+        <v>23.11616</v>
+      </c>
+      <c r="P376">
+        <v>70.02350660365929</v>
+      </c>
+      <c r="Q376">
+        <v>33.012</v>
+      </c>
+      <c r="R376">
+        <v>345.55249</v>
+      </c>
+      <c r="S376">
+        <v>4.957711477761837</v>
+      </c>
+      <c r="T376">
+        <v>472.07</v>
+      </c>
+      <c r="U376">
+        <v>26</v>
+      </c>
+      <c r="V376">
+        <v>24</v>
+      </c>
+      <c r="W376">
+        <v>50</v>
+      </c>
+      <c r="X376">
+        <v>97</v>
+      </c>
+      <c r="Y376">
+        <v>26</v>
+      </c>
+      <c r="Z376">
+        <v>83</v>
+      </c>
+      <c r="AA376">
+        <v>24</v>
+      </c>
+      <c r="AB376">
+        <v>48</v>
+      </c>
+      <c r="AC376">
+        <v>3.98992</v>
+      </c>
+      <c r="AD376">
+        <v>-2.9731</v>
+      </c>
+      <c r="AE376">
+        <v>0</v>
+      </c>
+      <c r="AF376">
+        <v>273.2887500000001</v>
+      </c>
+      <c r="AG376">
+        <v>0</v>
+      </c>
+      <c r="AH376">
+        <v>3</v>
+      </c>
+      <c r="AI376">
+        <v>1036.65747</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B377" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E377">
+        <v>52.9</v>
+      </c>
+      <c r="F377">
+        <v>2345.74</v>
+      </c>
+      <c r="G377">
+        <v>44.34291115311909</v>
+      </c>
+      <c r="H377">
+        <v>5.53</v>
+      </c>
+      <c r="I377">
+        <v>0</v>
+      </c>
+      <c r="J377">
+        <v>0</v>
+      </c>
+      <c r="K377">
+        <v>0.1045368620037807</v>
+      </c>
+      <c r="L377">
+        <v>0</v>
+      </c>
+      <c r="M377">
+        <v>0</v>
+      </c>
+      <c r="N377">
+        <v>0</v>
+      </c>
+      <c r="O377">
+        <v>21.22046</v>
+      </c>
+      <c r="P377">
+        <v>66.30564929383827</v>
+      </c>
+      <c r="Q377">
+        <v>32.004</v>
+      </c>
+      <c r="R377">
+        <v>277.13314</v>
+      </c>
+      <c r="S377">
+        <v>5.238811720226844</v>
+      </c>
+      <c r="T377">
+        <v>253.59</v>
+      </c>
+      <c r="U377">
+        <v>15</v>
+      </c>
+      <c r="V377">
+        <v>13</v>
+      </c>
+      <c r="W377">
+        <v>28</v>
+      </c>
+      <c r="X377">
+        <v>48</v>
+      </c>
+      <c r="Y377">
+        <v>15</v>
+      </c>
+      <c r="Z377">
+        <v>44</v>
+      </c>
+      <c r="AA377">
+        <v>13</v>
+      </c>
+      <c r="AB377">
+        <v>23</v>
+      </c>
+      <c r="AC377">
+        <v>3.86956</v>
+      </c>
+      <c r="AD377">
+        <v>-3.21814</v>
+      </c>
+      <c r="AE377">
+        <v>0</v>
+      </c>
+      <c r="AF377">
+        <v>195.6073</v>
+      </c>
+      <c r="AG377">
+        <v>0</v>
+      </c>
+      <c r="AH377">
+        <v>3</v>
+      </c>
+      <c r="AI377">
+        <v>831.3994200000001</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B378" s="2">
+        <v>46209</v>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Sesión 28</t>
+        </is>
+      </c>
+      <c r="E378">
+        <v>69.7</v>
+      </c>
+      <c r="F378">
+        <v>2867.22</v>
+      </c>
+      <c r="G378">
+        <v>41.13658536585366</v>
+      </c>
+      <c r="H378">
+        <v>1.52</v>
+      </c>
+      <c r="I378">
+        <v>0</v>
+      </c>
+      <c r="J378">
+        <v>0</v>
+      </c>
+      <c r="K378">
+        <v>0.0218077474892396</v>
+      </c>
+      <c r="L378">
+        <v>0</v>
+      </c>
+      <c r="M378">
+        <v>0</v>
+      </c>
+      <c r="N378">
+        <v>0</v>
+      </c>
+      <c r="O378">
+        <v>21.14752</v>
+      </c>
+      <c r="P378">
+        <v>58.74311111111111</v>
+      </c>
+      <c r="Q378">
+        <v>36</v>
+      </c>
+      <c r="R378">
+        <v>368.31494</v>
+      </c>
+      <c r="S378">
+        <v>5.284288952654232</v>
+      </c>
+      <c r="T378">
+        <v>444.34</v>
+      </c>
+      <c r="U378">
+        <v>38</v>
+      </c>
+      <c r="V378">
+        <v>27</v>
+      </c>
+      <c r="W378">
+        <v>65</v>
+      </c>
+      <c r="X378">
+        <v>83</v>
+      </c>
+      <c r="Y378">
+        <v>38</v>
+      </c>
+      <c r="Z378">
+        <v>80</v>
+      </c>
+      <c r="AA378">
+        <v>27</v>
+      </c>
+      <c r="AB378">
+        <v>41</v>
+      </c>
+      <c r="AC378">
+        <v>4.35677</v>
+      </c>
+      <c r="AD378">
+        <v>-3.48271</v>
+      </c>
+      <c r="AE378">
+        <v>0</v>
+      </c>
+      <c r="AF378">
+        <v>256.7607</v>
+      </c>
+      <c r="AG378">
+        <v>0</v>
+      </c>
+      <c r="AH378">
+        <v>3</v>
+      </c>
+      <c r="AI378">
+        <v>1104.94482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-08
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI378"/>
+  <dimension ref="A1:AI402"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -41252,17 +41252,17 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E363">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F363">
-        <v>2877.2</v>
+        <v>5315.2</v>
       </c>
       <c r="G363">
-        <v>41.27977044476327</v>
+        <v>41.46021840873635</v>
       </c>
       <c r="H363">
         <v>0</v>
@@ -41295,37 +41295,37 @@
         <v>32.364</v>
       </c>
       <c r="R363">
-        <v>318.02921</v>
+        <v>597.84475</v>
       </c>
       <c r="S363">
-        <v>4.562829411764707</v>
+        <v>4.663375585023402</v>
       </c>
       <c r="T363">
-        <v>354.45999</v>
+        <v>646.17998</v>
       </c>
       <c r="U363">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="V363">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="W363">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="X363">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="Y363">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="Z363">
-        <v>60</v>
+        <v>115</v>
       </c>
       <c r="AA363">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="AB363">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="AC363">
         <v>3.49302</v>
@@ -41337,7 +41337,7 @@
         <v>0</v>
       </c>
       <c r="AF363">
-        <v>241.5084</v>
+        <v>447.0529</v>
       </c>
       <c r="AG363">
         <v>0</v>
@@ -41346,7 +41346,7 @@
         <v>3</v>
       </c>
       <c r="AI363">
-        <v>954.0876300000001</v>
+        <v>1793.53425</v>
       </c>
     </row>
     <row r="364">
@@ -41365,20 +41365,20 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E364">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F364">
-        <v>3258.73</v>
+        <v>5672.09</v>
       </c>
       <c r="G364">
-        <v>46.75365853658536</v>
+        <v>44.24407176287052</v>
       </c>
       <c r="H364">
-        <v>0.95</v>
+        <v>1.9</v>
       </c>
       <c r="I364">
         <v>0</v>
@@ -41387,7 +41387,7 @@
         <v>0</v>
       </c>
       <c r="K364">
-        <v>0.01362984218077475</v>
+        <v>0.01482059282371295</v>
       </c>
       <c r="L364">
         <v>0</v>
@@ -41408,37 +41408,37 @@
         <v>32.4</v>
       </c>
       <c r="R364">
-        <v>460.20196</v>
+        <v>838.4855799999999</v>
       </c>
       <c r="S364">
-        <v>6.602610616929698</v>
+        <v>6.540449141965679</v>
       </c>
       <c r="T364">
-        <v>562.02</v>
+        <v>1037.39</v>
       </c>
       <c r="U364">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="V364">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="W364">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="X364">
-        <v>106</v>
+        <v>206</v>
       </c>
       <c r="Y364">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="Z364">
-        <v>78</v>
+        <v>152</v>
       </c>
       <c r="AA364">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="AB364">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="AC364">
         <v>3.90562</v>
@@ -41450,7 +41450,7 @@
         <v>0</v>
       </c>
       <c r="AF364">
-        <v>289.2974</v>
+        <v>511.7238</v>
       </c>
       <c r="AG364">
         <v>0</v>
@@ -41459,7 +41459,7 @@
         <v>3</v>
       </c>
       <c r="AI364">
-        <v>1380.60588</v>
+        <v>2515.45674</v>
       </c>
     </row>
     <row r="365">
@@ -41478,17 +41478,17 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E365">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F365">
-        <v>2776.56</v>
+        <v>5096.36</v>
       </c>
       <c r="G365">
-        <v>39.83586800573888</v>
+        <v>39.75319812792512</v>
       </c>
       <c r="H365">
         <v>17.52</v>
@@ -41500,7 +41500,7 @@
         <v>0</v>
       </c>
       <c r="K365">
-        <v>0.2513629842180775</v>
+        <v>0.1366614664586583</v>
       </c>
       <c r="L365">
         <v>0</v>
@@ -41521,37 +41521,37 @@
         <v>33.984</v>
       </c>
       <c r="R365">
-        <v>396.32672</v>
+        <v>753.9197799999999</v>
       </c>
       <c r="S365">
-        <v>5.68617962697274</v>
+        <v>5.880809516380656</v>
       </c>
       <c r="T365">
-        <v>245.6</v>
+        <v>427.12</v>
       </c>
       <c r="U365">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="V365">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W365">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="X365">
+        <v>83</v>
+      </c>
+      <c r="Y365">
+        <v>13</v>
+      </c>
+      <c r="Z365">
+        <v>84</v>
+      </c>
+      <c r="AA365">
+        <v>6</v>
+      </c>
+      <c r="AB365">
         <v>45</v>
-      </c>
-      <c r="Y365">
-        <v>8</v>
-      </c>
-      <c r="Z365">
-        <v>45</v>
-      </c>
-      <c r="AA365">
-        <v>3</v>
-      </c>
-      <c r="AB365">
-        <v>14</v>
       </c>
       <c r="AC365">
         <v>3.45041</v>
@@ -41563,7 +41563,7 @@
         <v>0</v>
       </c>
       <c r="AF365">
-        <v>258.1776</v>
+        <v>472.4936</v>
       </c>
       <c r="AG365">
         <v>0</v>
@@ -41572,7 +41572,7 @@
         <v>3</v>
       </c>
       <c r="AI365">
-        <v>1188.98016</v>
+        <v>2261.75934</v>
       </c>
     </row>
     <row r="366">
@@ -41591,17 +41591,17 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E366">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F366">
-        <v>3262.38</v>
+        <v>6125.200000000001</v>
       </c>
       <c r="G366">
-        <v>46.80602582496412</v>
+        <v>47.77847113884556</v>
       </c>
       <c r="H366">
         <v>0</v>
@@ -41634,37 +41634,37 @@
         <v>35.568</v>
       </c>
       <c r="R366">
-        <v>377.15638</v>
+        <v>719.5448299999999</v>
       </c>
       <c r="S366">
-        <v>5.411138880918221</v>
+        <v>5.612674180967239</v>
       </c>
       <c r="T366">
-        <v>557.99</v>
+        <v>1045.68</v>
       </c>
       <c r="U366">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="V366">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="W366">
-        <v>85</v>
+        <v>155</v>
       </c>
       <c r="X366">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="Y366">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="Z366">
-        <v>96</v>
+        <v>179</v>
       </c>
       <c r="AA366">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="AB366">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="AC366">
         <v>4.27991</v>
@@ -41676,7 +41676,7 @@
         <v>0</v>
       </c>
       <c r="AF366">
-        <v>342.752</v>
+        <v>643.7375999999999</v>
       </c>
       <c r="AG366">
         <v>0</v>
@@ -41685,7 +41685,7 @@
         <v>3</v>
       </c>
       <c r="AI366">
-        <v>1131.46914</v>
+        <v>2158.63449</v>
       </c>
     </row>
     <row r="367">
@@ -41704,20 +41704,20 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E367">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F367">
-        <v>3533.39</v>
+        <v>6654.87</v>
       </c>
       <c r="G367">
-        <v>50.69426111908177</v>
+        <v>51.9100624024961</v>
       </c>
       <c r="H367">
-        <v>22.95</v>
+        <v>45.90000000000001</v>
       </c>
       <c r="I367">
         <v>0</v>
@@ -41726,7 +41726,7 @@
         <v>0</v>
       </c>
       <c r="K367">
-        <v>0.3292682926829268</v>
+        <v>0.358034321372855</v>
       </c>
       <c r="L367">
         <v>0</v>
@@ -41747,37 +41747,37 @@
         <v>36</v>
       </c>
       <c r="R367">
-        <v>459.22363</v>
+        <v>877.70944</v>
       </c>
       <c r="S367">
-        <v>6.588574318507891</v>
+        <v>6.846407488299532</v>
       </c>
       <c r="T367">
-        <v>631.57999</v>
+        <v>1183.53998</v>
       </c>
       <c r="U367">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="V367">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="W367">
-        <v>83</v>
+        <v>150</v>
       </c>
       <c r="X367">
-        <v>127</v>
+        <v>233</v>
       </c>
       <c r="Y367">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="Z367">
+        <v>200</v>
+      </c>
+      <c r="AA367">
+        <v>68</v>
+      </c>
+      <c r="AB367">
         <v>107</v>
-      </c>
-      <c r="AA367">
-        <v>36</v>
-      </c>
-      <c r="AB367">
-        <v>49</v>
       </c>
       <c r="AC367">
         <v>4.22953</v>
@@ -41789,7 +41789,7 @@
         <v>0</v>
       </c>
       <c r="AF367">
-        <v>322.147</v>
+        <v>606.1867</v>
       </c>
       <c r="AG367">
         <v>0</v>
@@ -41798,7 +41798,7 @@
         <v>3</v>
       </c>
       <c r="AI367">
-        <v>1377.67089</v>
+        <v>2633.12832</v>
       </c>
     </row>
     <row r="368">
@@ -41817,20 +41817,20 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E368">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F368">
-        <v>2570.85</v>
+        <v>4654.87</v>
       </c>
       <c r="G368">
-        <v>36.8845050215208</v>
+        <v>36.3094383775351</v>
       </c>
       <c r="H368">
-        <v>13.81</v>
+        <v>27.62</v>
       </c>
       <c r="I368">
         <v>0</v>
@@ -41839,7 +41839,7 @@
         <v>0</v>
       </c>
       <c r="K368">
-        <v>0.1981348637015782</v>
+        <v>0.2154446177847114</v>
       </c>
       <c r="L368">
         <v>0</v>
@@ -41860,37 +41860,37 @@
         <v>32.004</v>
       </c>
       <c r="R368">
-        <v>331.94508</v>
+        <v>625.58593</v>
       </c>
       <c r="S368">
-        <v>4.762483213773314</v>
+        <v>4.879765444617785</v>
       </c>
       <c r="T368">
-        <v>392.06</v>
+        <v>728</v>
       </c>
       <c r="U368">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="V368">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="W368">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="X368">
-        <v>66</v>
+        <v>128</v>
       </c>
       <c r="Y368">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="Z368">
-        <v>63</v>
+        <v>123</v>
       </c>
       <c r="AA368">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="AB368">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="AC368">
         <v>4.07591</v>
@@ -41902,7 +41902,7 @@
         <v>0</v>
       </c>
       <c r="AF368">
-        <v>190.7094</v>
+        <v>348.306</v>
       </c>
       <c r="AG368">
         <v>0</v>
@@ -41911,7 +41911,7 @@
         <v>3</v>
       </c>
       <c r="AI368">
-        <v>995.8352400000001</v>
+        <v>1876.75779</v>
       </c>
     </row>
     <row r="369">
@@ -41930,20 +41930,20 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E369">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F369">
-        <v>2764.9</v>
+        <v>5121.98</v>
       </c>
       <c r="G369">
-        <v>39.66857962697274</v>
+        <v>39.95304212168487</v>
       </c>
       <c r="H369">
-        <v>26.07</v>
+        <v>52.14</v>
       </c>
       <c r="I369">
         <v>0</v>
@@ -41952,7 +41952,7 @@
         <v>0</v>
       </c>
       <c r="K369">
-        <v>0.3740315638450502</v>
+        <v>0.4067082683307333</v>
       </c>
       <c r="L369">
         <v>0</v>
@@ -41973,37 +41973,37 @@
         <v>33.84</v>
       </c>
       <c r="R369">
-        <v>339.82262</v>
+        <v>639.7687099999999</v>
       </c>
       <c r="S369">
-        <v>4.87550387374462</v>
+        <v>4.990395553822153</v>
       </c>
       <c r="T369">
-        <v>433.2</v>
+        <v>802.01</v>
       </c>
       <c r="U369">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="V369">
+        <v>50</v>
+      </c>
+      <c r="W369">
+        <v>77</v>
+      </c>
+      <c r="X369">
+        <v>135</v>
+      </c>
+      <c r="Y369">
         <v>27</v>
       </c>
-      <c r="W369">
-        <v>42</v>
-      </c>
-      <c r="X369">
-        <v>75</v>
-      </c>
-      <c r="Y369">
-        <v>15</v>
-      </c>
       <c r="Z369">
-        <v>82</v>
+        <v>152</v>
       </c>
       <c r="AA369">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="AB369">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="AC369">
         <v>4.17768</v>
@@ -42015,7 +42015,7 @@
         <v>0</v>
       </c>
       <c r="AF369">
-        <v>248.6722</v>
+        <v>461.8348</v>
       </c>
       <c r="AG369">
         <v>0</v>
@@ -42024,7 +42024,7 @@
         <v>3</v>
       </c>
       <c r="AI369">
-        <v>1019.46786</v>
+        <v>1919.30613</v>
       </c>
     </row>
     <row r="370">
@@ -42043,17 +42043,17 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E370">
-        <v>52.9</v>
+        <v>111.4</v>
       </c>
       <c r="F370">
-        <v>2378.3</v>
+        <v>4883.93</v>
       </c>
       <c r="G370">
-        <v>44.95841209829867</v>
+        <v>43.84138240574507</v>
       </c>
       <c r="H370">
         <v>0</v>
@@ -42086,37 +42086,37 @@
         <v>33.696</v>
       </c>
       <c r="R370">
-        <v>319.44484</v>
+        <v>646.40248</v>
       </c>
       <c r="S370">
-        <v>6.038654820415879</v>
+        <v>5.802535727109515</v>
       </c>
       <c r="T370">
-        <v>366.78001</v>
+        <v>733.56002</v>
       </c>
       <c r="U370">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="V370">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="W370">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="X370">
-        <v>68</v>
+        <v>136</v>
       </c>
       <c r="Y370">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="Z370">
-        <v>66</v>
+        <v>132</v>
       </c>
       <c r="AA370">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="AB370">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="AC370">
         <v>3.90287</v>
@@ -42128,7 +42128,7 @@
         <v>0</v>
       </c>
       <c r="AF370">
-        <v>244.3544</v>
+        <v>499.148</v>
       </c>
       <c r="AG370">
         <v>0</v>
@@ -42137,7 +42137,7 @@
         <v>3</v>
       </c>
       <c r="AI370">
-        <v>958.33452</v>
+        <v>1939.20744</v>
       </c>
     </row>
     <row r="371">
@@ -42156,17 +42156,17 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E371">
-        <v>52.9</v>
+        <v>111.4</v>
       </c>
       <c r="F371">
-        <v>2561.25</v>
+        <v>5165.42</v>
       </c>
       <c r="G371">
-        <v>48.41682419659735</v>
+        <v>46.36822262118492</v>
       </c>
       <c r="H371">
         <v>0</v>
@@ -42199,37 +42199,37 @@
         <v>34.992</v>
       </c>
       <c r="R371">
-        <v>292.66553</v>
+        <v>595.6703699999999</v>
       </c>
       <c r="S371">
-        <v>5.532429678638941</v>
+        <v>5.34713078994614</v>
       </c>
       <c r="T371">
-        <v>344.53</v>
+        <v>689.0599999999999</v>
       </c>
       <c r="U371">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="V371">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="W371">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="X371">
-        <v>82</v>
+        <v>164</v>
       </c>
       <c r="Y371">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="Z371">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="AA371">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="AB371">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="AC371">
         <v>4.09066</v>
@@ -42241,7 +42241,7 @@
         <v>0</v>
       </c>
       <c r="AF371">
-        <v>221.57142</v>
+        <v>445.32324</v>
       </c>
       <c r="AG371">
         <v>0</v>
@@ -42250,7 +42250,7 @@
         <v>3</v>
       </c>
       <c r="AI371">
-        <v>877.99659</v>
+        <v>1787.01111</v>
       </c>
     </row>
     <row r="372">
@@ -42269,17 +42269,17 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E372">
-        <v>52.9</v>
+        <v>111.4</v>
       </c>
       <c r="F372">
-        <v>2350.71</v>
+        <v>4790.51</v>
       </c>
       <c r="G372">
-        <v>44.43686200378073</v>
+        <v>43.00278276481149</v>
       </c>
       <c r="H372">
         <v>0</v>
@@ -42312,37 +42312,37 @@
         <v>34.92</v>
       </c>
       <c r="R372">
-        <v>289.3408</v>
+        <v>594.2471399999999</v>
       </c>
       <c r="S372">
-        <v>5.469580340264651</v>
+        <v>5.334354937163375</v>
       </c>
       <c r="T372">
-        <v>322.50999</v>
+        <v>659.88998</v>
       </c>
       <c r="U372">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="V372">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="W372">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="X372">
-        <v>62</v>
+        <v>127</v>
       </c>
       <c r="Y372">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="Z372">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="AA372">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="AB372">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="AC372">
         <v>4.20597</v>
@@ -42354,7 +42354,7 @@
         <v>0</v>
       </c>
       <c r="AF372">
-        <v>233.7776</v>
+        <v>476.0064</v>
       </c>
       <c r="AG372">
         <v>0</v>
@@ -42363,7 +42363,7 @@
         <v>3</v>
       </c>
       <c r="AI372">
-        <v>868.0224000000001</v>
+        <v>1782.74142</v>
       </c>
     </row>
     <row r="373">
@@ -42382,17 +42382,17 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E373">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F373">
-        <v>2966.17</v>
+        <v>5449.63</v>
       </c>
       <c r="G373">
-        <v>42.55624103299856</v>
+        <v>42.50881435257411</v>
       </c>
       <c r="H373">
         <v>0</v>
@@ -42425,37 +42425,37 @@
         <v>34.992</v>
       </c>
       <c r="R373">
-        <v>316.80447</v>
+        <v>611.19537</v>
       </c>
       <c r="S373">
-        <v>4.545257819225252</v>
+        <v>4.767514586583464</v>
       </c>
       <c r="T373">
-        <v>444.77001</v>
+        <v>826.82002</v>
       </c>
       <c r="U373">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="V373">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="W373">
-        <v>42</v>
+        <v>81</v>
       </c>
       <c r="X373">
-        <v>89</v>
+        <v>170</v>
       </c>
       <c r="Y373">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="Z373">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="AA373">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="AB373">
-        <v>67</v>
+        <v>134</v>
       </c>
       <c r="AC373">
         <v>3.85945</v>
@@ -42467,7 +42467,7 @@
         <v>0</v>
       </c>
       <c r="AF373">
-        <v>269.5799</v>
+        <v>498.40935</v>
       </c>
       <c r="AG373">
         <v>0</v>
@@ -42476,7 +42476,7 @@
         <v>3</v>
       </c>
       <c r="AI373">
-        <v>950.4134100000001</v>
+        <v>1833.58611</v>
       </c>
     </row>
     <row r="374">
@@ -42495,20 +42495,20 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E374">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F374">
-        <v>2790.93</v>
+        <v>5078.179999999999</v>
       </c>
       <c r="G374">
-        <v>40.04203730272597</v>
+        <v>39.61138845553822</v>
       </c>
       <c r="H374">
-        <v>6.880000000000001</v>
+        <v>12.66</v>
       </c>
       <c r="I374">
         <v>0</v>
@@ -42517,7 +42517,7 @@
         <v>0</v>
       </c>
       <c r="K374">
-        <v>0.09870875179340029</v>
+        <v>0.09875195007800315</v>
       </c>
       <c r="L374">
         <v>0</v>
@@ -42538,37 +42538,37 @@
         <v>33.984</v>
       </c>
       <c r="R374">
-        <v>385.37218</v>
+        <v>728.5777400000001</v>
       </c>
       <c r="S374">
-        <v>5.52901262553802</v>
+        <v>5.683133697347895</v>
       </c>
       <c r="T374">
-        <v>385.94</v>
+        <v>704.62</v>
       </c>
       <c r="U374">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="V374">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="W374">
+        <v>61</v>
+      </c>
+      <c r="X374">
+        <v>121</v>
+      </c>
+      <c r="Y374">
+        <v>28</v>
+      </c>
+      <c r="Z374">
+        <v>110</v>
+      </c>
+      <c r="AA374">
         <v>33</v>
       </c>
-      <c r="X374">
-        <v>65</v>
-      </c>
-      <c r="Y374">
-        <v>16</v>
-      </c>
-      <c r="Z374">
-        <v>60</v>
-      </c>
-      <c r="AA374">
-        <v>17</v>
-      </c>
       <c r="AB374">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="AC374">
         <v>3.92536</v>
@@ -42580,7 +42580,7 @@
         <v>0</v>
       </c>
       <c r="AF374">
-        <v>275.612</v>
+        <v>501.4448</v>
       </c>
       <c r="AG374">
         <v>0</v>
@@ -42589,7 +42589,7 @@
         <v>3</v>
       </c>
       <c r="AI374">
-        <v>1156.11654</v>
+        <v>2185.73322</v>
       </c>
     </row>
     <row r="375">
@@ -42608,17 +42608,17 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E375">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F375">
-        <v>2546.24</v>
+        <v>5131.96</v>
       </c>
       <c r="G375">
-        <v>36.53142037302726</v>
+        <v>40.03088923556943</v>
       </c>
       <c r="H375">
         <v>0</v>
@@ -42651,37 +42651,37 @@
         <v>34.992</v>
       </c>
       <c r="R375">
-        <v>326.65239</v>
+        <v>660.59281</v>
       </c>
       <c r="S375">
-        <v>4.686547919655666</v>
+        <v>5.152830031201248</v>
       </c>
       <c r="T375">
-        <v>404.81</v>
+        <v>810.11</v>
       </c>
       <c r="U375">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="V375">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="W375">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="X375">
-        <v>84</v>
+        <v>168</v>
       </c>
       <c r="Y375">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="Z375">
-        <v>76</v>
+        <v>152</v>
       </c>
       <c r="AA375">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="AB375">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="AC375">
         <v>3.89727</v>
@@ -42693,7 +42693,7 @@
         <v>0</v>
       </c>
       <c r="AF375">
-        <v>255.6072</v>
+        <v>514.1976000000001</v>
       </c>
       <c r="AG375">
         <v>0</v>
@@ -42702,7 +42702,7 @@
         <v>3</v>
       </c>
       <c r="AI375">
-        <v>979.9571699999999</v>
+        <v>1981.77843</v>
       </c>
     </row>
     <row r="376">
@@ -42721,20 +42721,20 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E376">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F376">
-        <v>2924.54</v>
+        <v>5316.75</v>
       </c>
       <c r="G376">
-        <v>41.95896700143471</v>
+        <v>41.4723088923557</v>
       </c>
       <c r="H376">
-        <v>11.97</v>
+        <v>22.87</v>
       </c>
       <c r="I376">
         <v>0</v>
@@ -42743,7 +42743,7 @@
         <v>0</v>
       </c>
       <c r="K376">
-        <v>0.1717360114777618</v>
+        <v>0.178393135725429</v>
       </c>
       <c r="L376">
         <v>0</v>
@@ -42764,37 +42764,37 @@
         <v>33.012</v>
       </c>
       <c r="R376">
-        <v>345.55249</v>
+        <v>649.42518</v>
       </c>
       <c r="S376">
-        <v>4.957711477761837</v>
+        <v>5.065719032761311</v>
       </c>
       <c r="T376">
-        <v>472.07</v>
+        <v>860.37</v>
       </c>
       <c r="U376">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="V376">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="W376">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="X376">
-        <v>97</v>
+        <v>184</v>
       </c>
       <c r="Y376">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="Z376">
-        <v>83</v>
+        <v>157</v>
       </c>
       <c r="AA376">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="AB376">
-        <v>48</v>
+        <v>106</v>
       </c>
       <c r="AC376">
         <v>3.98992</v>
@@ -42806,7 +42806,7 @@
         <v>0</v>
       </c>
       <c r="AF376">
-        <v>273.2887500000001</v>
+        <v>497.73825</v>
       </c>
       <c r="AG376">
         <v>0</v>
@@ -42815,7 +42815,7 @@
         <v>3</v>
       </c>
       <c r="AI376">
-        <v>1036.65747</v>
+        <v>1948.27554</v>
       </c>
     </row>
     <row r="377">
@@ -42834,20 +42834,20 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E377">
-        <v>52.9</v>
+        <v>111.4</v>
       </c>
       <c r="F377">
-        <v>2345.74</v>
+        <v>4749.22</v>
       </c>
       <c r="G377">
-        <v>44.34291115311909</v>
+        <v>42.63213644524237</v>
       </c>
       <c r="H377">
-        <v>5.53</v>
+        <v>11.06</v>
       </c>
       <c r="I377">
         <v>0</v>
@@ -42856,7 +42856,7 @@
         <v>0</v>
       </c>
       <c r="K377">
-        <v>0.1045368620037807</v>
+        <v>0.09928186714542191</v>
       </c>
       <c r="L377">
         <v>0</v>
@@ -42877,37 +42877,37 @@
         <v>32.004</v>
       </c>
       <c r="R377">
-        <v>277.13314</v>
+        <v>561.6697300000001</v>
       </c>
       <c r="S377">
-        <v>5.238811720226844</v>
+        <v>5.041918581687613</v>
       </c>
       <c r="T377">
-        <v>253.59</v>
+        <v>507.18</v>
       </c>
       <c r="U377">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="V377">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="W377">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="X377">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="Y377">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="Z377">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="AA377">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="AB377">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="AC377">
         <v>3.86956</v>
@@ -42919,7 +42919,7 @@
         <v>0</v>
       </c>
       <c r="AF377">
-        <v>195.6073</v>
+        <v>394.9568</v>
       </c>
       <c r="AG377">
         <v>0</v>
@@ -42928,7 +42928,7 @@
         <v>3</v>
       </c>
       <c r="AI377">
-        <v>831.3994200000001</v>
+        <v>1685.00919</v>
       </c>
     </row>
     <row r="378">
@@ -42947,20 +42947,20 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>Sesión 28</t>
+          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
         </is>
       </c>
       <c r="E378">
-        <v>69.7</v>
+        <v>128.2</v>
       </c>
       <c r="F378">
-        <v>2867.22</v>
+        <v>5350.58</v>
       </c>
       <c r="G378">
-        <v>41.13658536585366</v>
+        <v>41.73619344773791</v>
       </c>
       <c r="H378">
-        <v>1.52</v>
+        <v>3.04</v>
       </c>
       <c r="I378">
         <v>0</v>
@@ -42969,7 +42969,7 @@
         <v>0</v>
       </c>
       <c r="K378">
-        <v>0.0218077474892396</v>
+        <v>0.02371294851794072</v>
       </c>
       <c r="L378">
         <v>0</v>
@@ -42990,37 +42990,37 @@
         <v>36</v>
       </c>
       <c r="R378">
-        <v>368.31494</v>
+        <v>699.7805</v>
       </c>
       <c r="S378">
-        <v>5.284288952654232</v>
+        <v>5.45850624024961</v>
       </c>
       <c r="T378">
-        <v>444.34</v>
+        <v>824.22</v>
       </c>
       <c r="U378">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="V378">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="W378">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="X378">
-        <v>83</v>
+        <v>150</v>
       </c>
       <c r="Y378">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="Z378">
-        <v>80</v>
+        <v>148</v>
       </c>
       <c r="AA378">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="AB378">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="AC378">
         <v>4.35677</v>
@@ -43032,7 +43032,7 @@
         <v>0</v>
       </c>
       <c r="AF378">
-        <v>256.7607</v>
+        <v>479.0751</v>
       </c>
       <c r="AG378">
         <v>0</v>
@@ -43041,7 +43041,2719 @@
         <v>3</v>
       </c>
       <c r="AI378">
-        <v>1104.94482</v>
+        <v>2099.3415</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B379" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E379">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F379">
+        <v>6609.96</v>
+      </c>
+      <c r="G379">
+        <v>58.81619457214889</v>
+      </c>
+      <c r="H379">
+        <v>0</v>
+      </c>
+      <c r="I379">
+        <v>0</v>
+      </c>
+      <c r="J379">
+        <v>0</v>
+      </c>
+      <c r="K379">
+        <v>0</v>
+      </c>
+      <c r="L379">
+        <v>0</v>
+      </c>
+      <c r="M379">
+        <v>0</v>
+      </c>
+      <c r="N379">
+        <v>0</v>
+      </c>
+      <c r="O379">
+        <v>29.03417</v>
+      </c>
+      <c r="P379">
+        <v>80.65047222222222</v>
+      </c>
+      <c r="Q379">
+        <v>36</v>
+      </c>
+      <c r="R379">
+        <v>674.0479799999999</v>
+      </c>
+      <c r="S379">
+        <v>5.997757496663206</v>
+      </c>
+      <c r="T379">
+        <v>0</v>
+      </c>
+      <c r="U379">
+        <v>0</v>
+      </c>
+      <c r="V379">
+        <v>0</v>
+      </c>
+      <c r="W379">
+        <v>0</v>
+      </c>
+      <c r="X379">
+        <v>0</v>
+      </c>
+      <c r="Y379">
+        <v>0</v>
+      </c>
+      <c r="Z379">
+        <v>0</v>
+      </c>
+      <c r="AA379">
+        <v>0</v>
+      </c>
+      <c r="AB379">
+        <v>0</v>
+      </c>
+      <c r="AC379">
+        <v>4.19117</v>
+      </c>
+      <c r="AD379">
+        <v>-3.47487</v>
+      </c>
+      <c r="AE379">
+        <v>0</v>
+      </c>
+      <c r="AF379">
+        <v>0</v>
+      </c>
+      <c r="AG379">
+        <v>0</v>
+      </c>
+      <c r="AH379">
+        <v>3</v>
+      </c>
+      <c r="AI379">
+        <v>2022.14394</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B380" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E380">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F380">
+        <v>6550.559999999999</v>
+      </c>
+      <c r="G380">
+        <v>58.28764644816847</v>
+      </c>
+      <c r="H380">
+        <v>252.68</v>
+      </c>
+      <c r="I380">
+        <v>0</v>
+      </c>
+      <c r="J380">
+        <v>0</v>
+      </c>
+      <c r="K380">
+        <v>2.248376093726828</v>
+      </c>
+      <c r="L380">
+        <v>0</v>
+      </c>
+      <c r="M380">
+        <v>4</v>
+      </c>
+      <c r="N380">
+        <v>0</v>
+      </c>
+      <c r="O380">
+        <v>28.20462</v>
+      </c>
+      <c r="P380">
+        <v>78.34616666666666</v>
+      </c>
+      <c r="Q380">
+        <v>36</v>
+      </c>
+      <c r="R380">
+        <v>556.95975</v>
+      </c>
+      <c r="S380">
+        <v>4.955892777695388</v>
+      </c>
+      <c r="T380">
+        <v>1156.36003</v>
+      </c>
+      <c r="U380">
+        <v>42</v>
+      </c>
+      <c r="V380">
+        <v>38</v>
+      </c>
+      <c r="W380">
+        <v>80</v>
+      </c>
+      <c r="X380">
+        <v>122</v>
+      </c>
+      <c r="Y380">
+        <v>42</v>
+      </c>
+      <c r="Z380">
+        <v>126</v>
+      </c>
+      <c r="AA380">
+        <v>38</v>
+      </c>
+      <c r="AB380">
+        <v>25</v>
+      </c>
+      <c r="AC380">
+        <v>4.33888</v>
+      </c>
+      <c r="AD380">
+        <v>-4.11128</v>
+      </c>
+      <c r="AE380">
+        <v>0</v>
+      </c>
+      <c r="AF380">
+        <v>1625.178</v>
+      </c>
+      <c r="AG380">
+        <v>0</v>
+      </c>
+      <c r="AH380">
+        <v>3</v>
+      </c>
+      <c r="AI380">
+        <v>1670.87925</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Alejandro Fernandez</t>
+        </is>
+      </c>
+      <c r="B381" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E381">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F381">
+        <v>7451.58</v>
+      </c>
+      <c r="G381">
+        <v>66.3050274358594</v>
+      </c>
+      <c r="H381">
+        <v>231.03</v>
+      </c>
+      <c r="I381">
+        <v>0</v>
+      </c>
+      <c r="J381">
+        <v>0</v>
+      </c>
+      <c r="K381">
+        <v>2.055731870087498</v>
+      </c>
+      <c r="L381">
+        <v>0</v>
+      </c>
+      <c r="M381">
+        <v>1</v>
+      </c>
+      <c r="N381">
+        <v>0</v>
+      </c>
+      <c r="O381">
+        <v>28.59527</v>
+      </c>
+      <c r="P381">
+        <v>79.43130555555555</v>
+      </c>
+      <c r="Q381">
+        <v>36</v>
+      </c>
+      <c r="R381">
+        <v>884.49452</v>
+      </c>
+      <c r="S381">
+        <v>7.870335340352958</v>
+      </c>
+      <c r="T381">
+        <v>1395.85</v>
+      </c>
+      <c r="U381">
+        <v>45</v>
+      </c>
+      <c r="V381">
+        <v>32</v>
+      </c>
+      <c r="W381">
+        <v>77</v>
+      </c>
+      <c r="X381">
+        <v>147</v>
+      </c>
+      <c r="Y381">
+        <v>45</v>
+      </c>
+      <c r="Z381">
+        <v>134</v>
+      </c>
+      <c r="AA381">
+        <v>32</v>
+      </c>
+      <c r="AB381">
+        <v>72</v>
+      </c>
+      <c r="AC381">
+        <v>4.48659</v>
+      </c>
+      <c r="AD381">
+        <v>-3.42707</v>
+      </c>
+      <c r="AE381">
+        <v>0</v>
+      </c>
+      <c r="AF381">
+        <v>1823.104</v>
+      </c>
+      <c r="AG381">
+        <v>0</v>
+      </c>
+      <c r="AH381">
+        <v>3</v>
+      </c>
+      <c r="AI381">
+        <v>2653.48356</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B382" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E382">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F382">
+        <v>6640.95</v>
+      </c>
+      <c r="G382">
+        <v>59.09194720450837</v>
+      </c>
+      <c r="H382">
+        <v>334.82</v>
+      </c>
+      <c r="I382">
+        <v>0</v>
+      </c>
+      <c r="J382">
+        <v>0</v>
+      </c>
+      <c r="K382">
+        <v>2.979267388402788</v>
+      </c>
+      <c r="L382">
+        <v>0</v>
+      </c>
+      <c r="M382">
+        <v>5</v>
+      </c>
+      <c r="N382">
+        <v>0</v>
+      </c>
+      <c r="O382">
+        <v>28.43461</v>
+      </c>
+      <c r="P382">
+        <v>87.76114197530865</v>
+      </c>
+      <c r="Q382">
+        <v>32.4</v>
+      </c>
+      <c r="R382">
+        <v>806.36786</v>
+      </c>
+      <c r="S382">
+        <v>7.175155212813287</v>
+      </c>
+      <c r="T382">
+        <v>1465.88004</v>
+      </c>
+      <c r="U382">
+        <v>46</v>
+      </c>
+      <c r="V382">
+        <v>26</v>
+      </c>
+      <c r="W382">
+        <v>72</v>
+      </c>
+      <c r="X382">
+        <v>145</v>
+      </c>
+      <c r="Y382">
+        <v>46</v>
+      </c>
+      <c r="Z382">
+        <v>118</v>
+      </c>
+      <c r="AA382">
+        <v>26</v>
+      </c>
+      <c r="AB382">
+        <v>16</v>
+      </c>
+      <c r="AC382">
+        <v>4.28824</v>
+      </c>
+      <c r="AD382">
+        <v>-3.01502</v>
+      </c>
+      <c r="AE382">
+        <v>0</v>
+      </c>
+      <c r="AF382">
+        <v>577.4607999999999</v>
+      </c>
+      <c r="AG382">
+        <v>0</v>
+      </c>
+      <c r="AH382">
+        <v>3</v>
+      </c>
+      <c r="AI382">
+        <v>2419.10358</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B383" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E383">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F383">
+        <v>5882.97</v>
+      </c>
+      <c r="G383">
+        <v>52.34735281032182</v>
+      </c>
+      <c r="H383">
+        <v>210.5</v>
+      </c>
+      <c r="I383">
+        <v>0</v>
+      </c>
+      <c r="J383">
+        <v>0</v>
+      </c>
+      <c r="K383">
+        <v>1.873053537001335</v>
+      </c>
+      <c r="L383">
+        <v>0</v>
+      </c>
+      <c r="M383">
+        <v>6</v>
+      </c>
+      <c r="N383">
+        <v>0</v>
+      </c>
+      <c r="O383">
+        <v>29.46053</v>
+      </c>
+      <c r="P383">
+        <v>86.68941266478342</v>
+      </c>
+      <c r="Q383">
+        <v>33.984</v>
+      </c>
+      <c r="R383">
+        <v>699.61224</v>
+      </c>
+      <c r="S383">
+        <v>6.225231262049533</v>
+      </c>
+      <c r="T383">
+        <v>928.94003</v>
+      </c>
+      <c r="U383">
+        <v>26</v>
+      </c>
+      <c r="V383">
+        <v>26</v>
+      </c>
+      <c r="W383">
+        <v>52</v>
+      </c>
+      <c r="X383">
+        <v>95</v>
+      </c>
+      <c r="Y383">
+        <v>26</v>
+      </c>
+      <c r="Z383">
+        <v>87</v>
+      </c>
+      <c r="AA383">
+        <v>26</v>
+      </c>
+      <c r="AB383">
+        <v>28</v>
+      </c>
+      <c r="AC383">
+        <v>4.3619</v>
+      </c>
+      <c r="AD383">
+        <v>-2.24475</v>
+      </c>
+      <c r="AE383">
+        <v>0</v>
+      </c>
+      <c r="AF383">
+        <v>560.884</v>
+      </c>
+      <c r="AG383">
+        <v>0</v>
+      </c>
+      <c r="AH383">
+        <v>3</v>
+      </c>
+      <c r="AI383">
+        <v>2098.83672</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B384" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E384">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F384">
+        <v>7073.309999999999</v>
+      </c>
+      <c r="G384">
+        <v>62.93913688269316</v>
+      </c>
+      <c r="H384">
+        <v>232.32</v>
+      </c>
+      <c r="I384">
+        <v>0</v>
+      </c>
+      <c r="J384">
+        <v>0</v>
+      </c>
+      <c r="K384">
+        <v>2.06721044045677</v>
+      </c>
+      <c r="L384">
+        <v>0</v>
+      </c>
+      <c r="M384">
+        <v>0</v>
+      </c>
+      <c r="N384">
+        <v>0</v>
+      </c>
+      <c r="O384">
+        <v>24.93721</v>
+      </c>
+      <c r="P384">
+        <v>70.11136414754836</v>
+      </c>
+      <c r="Q384">
+        <v>35.568</v>
+      </c>
+      <c r="R384">
+        <v>639.65775</v>
+      </c>
+      <c r="S384">
+        <v>5.6917492214148</v>
+      </c>
+      <c r="T384">
+        <v>1141.92001</v>
+      </c>
+      <c r="U384">
+        <v>50</v>
+      </c>
+      <c r="V384">
+        <v>32</v>
+      </c>
+      <c r="W384">
+        <v>82</v>
+      </c>
+      <c r="X384">
+        <v>142</v>
+      </c>
+      <c r="Y384">
+        <v>50</v>
+      </c>
+      <c r="Z384">
+        <v>102</v>
+      </c>
+      <c r="AA384">
+        <v>32</v>
+      </c>
+      <c r="AB384">
+        <v>28</v>
+      </c>
+      <c r="AC384">
+        <v>4.59245</v>
+      </c>
+      <c r="AD384">
+        <v>-4.02125</v>
+      </c>
+      <c r="AE384">
+        <v>0</v>
+      </c>
+      <c r="AF384">
+        <v>688.444</v>
+      </c>
+      <c r="AG384">
+        <v>0</v>
+      </c>
+      <c r="AH384">
+        <v>3</v>
+      </c>
+      <c r="AI384">
+        <v>1918.97325</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B385" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E385">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F385">
+        <v>7004.07</v>
+      </c>
+      <c r="G385">
+        <v>62.32303129170992</v>
+      </c>
+      <c r="H385">
+        <v>312.99</v>
+      </c>
+      <c r="I385">
+        <v>0</v>
+      </c>
+      <c r="J385">
+        <v>0</v>
+      </c>
+      <c r="K385">
+        <v>2.785021503781699</v>
+      </c>
+      <c r="L385">
+        <v>15.02</v>
+      </c>
+      <c r="M385">
+        <v>6</v>
+      </c>
+      <c r="N385">
+        <v>1</v>
+      </c>
+      <c r="O385">
+        <v>30.67104</v>
+      </c>
+      <c r="P385">
+        <v>85.19733333333333</v>
+      </c>
+      <c r="Q385">
+        <v>36</v>
+      </c>
+      <c r="R385">
+        <v>665.08218</v>
+      </c>
+      <c r="S385">
+        <v>5.917978763161797</v>
+      </c>
+      <c r="T385">
+        <v>1109.35</v>
+      </c>
+      <c r="U385">
+        <v>30</v>
+      </c>
+      <c r="V385">
+        <v>25</v>
+      </c>
+      <c r="W385">
+        <v>55</v>
+      </c>
+      <c r="X385">
+        <v>100</v>
+      </c>
+      <c r="Y385">
+        <v>30</v>
+      </c>
+      <c r="Z385">
+        <v>82</v>
+      </c>
+      <c r="AA385">
+        <v>25</v>
+      </c>
+      <c r="AB385">
+        <v>30</v>
+      </c>
+      <c r="AC385">
+        <v>4.07669</v>
+      </c>
+      <c r="AD385">
+        <v>-3.10266</v>
+      </c>
+      <c r="AE385">
+        <v>0</v>
+      </c>
+      <c r="AF385">
+        <v>1660.48</v>
+      </c>
+      <c r="AG385">
+        <v>0</v>
+      </c>
+      <c r="AH385">
+        <v>3</v>
+      </c>
+      <c r="AI385">
+        <v>1995.24654</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B386" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E386">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F386">
+        <v>6179.040000000001</v>
+      </c>
+      <c r="G386">
+        <v>54.98181818181818</v>
+      </c>
+      <c r="H386">
+        <v>138.56</v>
+      </c>
+      <c r="I386">
+        <v>0</v>
+      </c>
+      <c r="J386">
+        <v>0</v>
+      </c>
+      <c r="K386">
+        <v>1.23292303129171</v>
+      </c>
+      <c r="L386">
+        <v>0</v>
+      </c>
+      <c r="M386">
+        <v>2</v>
+      </c>
+      <c r="N386">
+        <v>0</v>
+      </c>
+      <c r="O386">
+        <v>27.13894</v>
+      </c>
+      <c r="P386">
+        <v>75.38594444444445</v>
+      </c>
+      <c r="Q386">
+        <v>36</v>
+      </c>
+      <c r="R386">
+        <v>581.3761</v>
+      </c>
+      <c r="S386">
+        <v>5.173152306095209</v>
+      </c>
+      <c r="T386">
+        <v>840.18997</v>
+      </c>
+      <c r="U386">
+        <v>34</v>
+      </c>
+      <c r="V386">
+        <v>21</v>
+      </c>
+      <c r="W386">
+        <v>55</v>
+      </c>
+      <c r="X386">
+        <v>97</v>
+      </c>
+      <c r="Y386">
+        <v>34</v>
+      </c>
+      <c r="Z386">
+        <v>67</v>
+      </c>
+      <c r="AA386">
+        <v>21</v>
+      </c>
+      <c r="AB386">
+        <v>13</v>
+      </c>
+      <c r="AC386">
+        <v>4.02625</v>
+      </c>
+      <c r="AD386">
+        <v>-3.22452</v>
+      </c>
+      <c r="AE386">
+        <v>0</v>
+      </c>
+      <c r="AF386">
+        <v>511.0259</v>
+      </c>
+      <c r="AG386">
+        <v>0</v>
+      </c>
+      <c r="AH386">
+        <v>3</v>
+      </c>
+      <c r="AI386">
+        <v>1744.1283</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B387" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E387">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F387">
+        <v>6322.6</v>
+      </c>
+      <c r="G387">
+        <v>56.25923179593653</v>
+      </c>
+      <c r="H387">
+        <v>155.29</v>
+      </c>
+      <c r="I387">
+        <v>0</v>
+      </c>
+      <c r="J387">
+        <v>0</v>
+      </c>
+      <c r="K387">
+        <v>1.381788521429631</v>
+      </c>
+      <c r="L387">
+        <v>0</v>
+      </c>
+      <c r="M387">
+        <v>1</v>
+      </c>
+      <c r="N387">
+        <v>0</v>
+      </c>
+      <c r="O387">
+        <v>25.77215</v>
+      </c>
+      <c r="P387">
+        <v>80.52790276215474</v>
+      </c>
+      <c r="Q387">
+        <v>32.004</v>
+      </c>
+      <c r="R387">
+        <v>676.50623</v>
+      </c>
+      <c r="S387">
+        <v>6.019631291709921</v>
+      </c>
+      <c r="T387">
+        <v>983.89002</v>
+      </c>
+      <c r="U387">
+        <v>22</v>
+      </c>
+      <c r="V387">
+        <v>26</v>
+      </c>
+      <c r="W387">
+        <v>48</v>
+      </c>
+      <c r="X387">
+        <v>97</v>
+      </c>
+      <c r="Y387">
+        <v>22</v>
+      </c>
+      <c r="Z387">
+        <v>99</v>
+      </c>
+      <c r="AA387">
+        <v>26</v>
+      </c>
+      <c r="AB387">
+        <v>15</v>
+      </c>
+      <c r="AC387">
+        <v>4.55742</v>
+      </c>
+      <c r="AD387">
+        <v>-3.78965</v>
+      </c>
+      <c r="AE387">
+        <v>0</v>
+      </c>
+      <c r="AF387">
+        <v>454.674</v>
+      </c>
+      <c r="AG387">
+        <v>0</v>
+      </c>
+      <c r="AH387">
+        <v>3</v>
+      </c>
+      <c r="AI387">
+        <v>2029.51869</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B388" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E388">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F388">
+        <v>6886.38</v>
+      </c>
+      <c r="G388">
+        <v>61.27581195313658</v>
+      </c>
+      <c r="H388">
+        <v>287.73</v>
+      </c>
+      <c r="I388">
+        <v>0</v>
+      </c>
+      <c r="J388">
+        <v>0</v>
+      </c>
+      <c r="K388">
+        <v>2.560255079341539</v>
+      </c>
+      <c r="L388">
+        <v>0</v>
+      </c>
+      <c r="M388">
+        <v>6</v>
+      </c>
+      <c r="N388">
+        <v>0</v>
+      </c>
+      <c r="O388">
+        <v>29.67884</v>
+      </c>
+      <c r="P388">
+        <v>87.70342789598108</v>
+      </c>
+      <c r="Q388">
+        <v>33.84</v>
+      </c>
+      <c r="R388">
+        <v>666.3904700000001</v>
+      </c>
+      <c r="S388">
+        <v>5.929620080083049</v>
+      </c>
+      <c r="T388">
+        <v>1098.49</v>
+      </c>
+      <c r="U388">
+        <v>45</v>
+      </c>
+      <c r="V388">
+        <v>24</v>
+      </c>
+      <c r="W388">
+        <v>69</v>
+      </c>
+      <c r="X388">
+        <v>124</v>
+      </c>
+      <c r="Y388">
+        <v>45</v>
+      </c>
+      <c r="Z388">
+        <v>97</v>
+      </c>
+      <c r="AA388">
+        <v>24</v>
+      </c>
+      <c r="AB388">
+        <v>30</v>
+      </c>
+      <c r="AC388">
+        <v>4.53657</v>
+      </c>
+      <c r="AD388">
+        <v>-3.81264</v>
+      </c>
+      <c r="AE388">
+        <v>0</v>
+      </c>
+      <c r="AF388">
+        <v>581.6426</v>
+      </c>
+      <c r="AG388">
+        <v>0</v>
+      </c>
+      <c r="AH388">
+        <v>3</v>
+      </c>
+      <c r="AI388">
+        <v>1999.17141</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Guillermo Cortes</t>
+        </is>
+      </c>
+      <c r="B389" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E389">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F389">
+        <v>5858.77</v>
+      </c>
+      <c r="G389">
+        <v>52.13201838944089</v>
+      </c>
+      <c r="H389">
+        <v>717.3800000000001</v>
+      </c>
+      <c r="I389">
+        <v>146.18</v>
+      </c>
+      <c r="J389">
+        <v>6</v>
+      </c>
+      <c r="K389">
+        <v>6.383330861634288</v>
+      </c>
+      <c r="L389">
+        <v>229.11</v>
+      </c>
+      <c r="M389">
+        <v>14</v>
+      </c>
+      <c r="N389">
+        <v>5</v>
+      </c>
+      <c r="O389">
+        <v>41.62648</v>
+      </c>
+      <c r="P389">
+        <v>115.6291111111111</v>
+      </c>
+      <c r="Q389">
+        <v>36</v>
+      </c>
+      <c r="R389">
+        <v>528.29197</v>
+      </c>
+      <c r="S389">
+        <v>4.700803529586238</v>
+      </c>
+      <c r="T389">
+        <v>1422.98001</v>
+      </c>
+      <c r="U389">
+        <v>45</v>
+      </c>
+      <c r="V389">
+        <v>62</v>
+      </c>
+      <c r="W389">
+        <v>107</v>
+      </c>
+      <c r="X389">
+        <v>100</v>
+      </c>
+      <c r="Y389">
+        <v>45</v>
+      </c>
+      <c r="Z389">
+        <v>115</v>
+      </c>
+      <c r="AA389">
+        <v>62</v>
+      </c>
+      <c r="AB389">
+        <v>27</v>
+      </c>
+      <c r="AC389">
+        <v>6.12231</v>
+      </c>
+      <c r="AD389">
+        <v>-3.50021</v>
+      </c>
+      <c r="AE389">
+        <v>0</v>
+      </c>
+      <c r="AF389">
+        <v>1480.312</v>
+      </c>
+      <c r="AG389">
+        <v>0</v>
+      </c>
+      <c r="AH389">
+        <v>3</v>
+      </c>
+      <c r="AI389">
+        <v>1584.87591</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B390" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E390">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F390">
+        <v>5622.170000000001</v>
+      </c>
+      <c r="G390">
+        <v>50.02672401008454</v>
+      </c>
+      <c r="H390">
+        <v>95.17</v>
+      </c>
+      <c r="I390">
+        <v>0</v>
+      </c>
+      <c r="J390">
+        <v>0</v>
+      </c>
+      <c r="K390">
+        <v>0.8468337535221711</v>
+      </c>
+      <c r="L390">
+        <v>0</v>
+      </c>
+      <c r="M390">
+        <v>1</v>
+      </c>
+      <c r="N390">
+        <v>0</v>
+      </c>
+      <c r="O390">
+        <v>27.69909</v>
+      </c>
+      <c r="P390">
+        <v>82.20290242165244</v>
+      </c>
+      <c r="Q390">
+        <v>33.696</v>
+      </c>
+      <c r="R390">
+        <v>560.54006</v>
+      </c>
+      <c r="S390">
+        <v>4.987750793415394</v>
+      </c>
+      <c r="T390">
+        <v>833.92002</v>
+      </c>
+      <c r="U390">
+        <v>21</v>
+      </c>
+      <c r="V390">
+        <v>28</v>
+      </c>
+      <c r="W390">
+        <v>49</v>
+      </c>
+      <c r="X390">
+        <v>111</v>
+      </c>
+      <c r="Y390">
+        <v>21</v>
+      </c>
+      <c r="Z390">
+        <v>88</v>
+      </c>
+      <c r="AA390">
+        <v>28</v>
+      </c>
+      <c r="AB390">
+        <v>29</v>
+      </c>
+      <c r="AC390">
+        <v>4.10527</v>
+      </c>
+      <c r="AD390">
+        <v>-2.55094</v>
+      </c>
+      <c r="AE390">
+        <v>0</v>
+      </c>
+      <c r="AF390">
+        <v>546.6384</v>
+      </c>
+      <c r="AG390">
+        <v>0</v>
+      </c>
+      <c r="AH390">
+        <v>3</v>
+      </c>
+      <c r="AI390">
+        <v>1681.62018</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B391" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E391">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F391">
+        <v>6903.41</v>
+      </c>
+      <c r="G391">
+        <v>61.4273468782441</v>
+      </c>
+      <c r="H391">
+        <v>253.15</v>
+      </c>
+      <c r="I391">
+        <v>0</v>
+      </c>
+      <c r="J391">
+        <v>0</v>
+      </c>
+      <c r="K391">
+        <v>2.252558208512532</v>
+      </c>
+      <c r="L391">
+        <v>0</v>
+      </c>
+      <c r="M391">
+        <v>3</v>
+      </c>
+      <c r="N391">
+        <v>0</v>
+      </c>
+      <c r="O391">
+        <v>26.32719</v>
+      </c>
+      <c r="P391">
+        <v>73.13108333333334</v>
+      </c>
+      <c r="Q391">
+        <v>36</v>
+      </c>
+      <c r="R391">
+        <v>869.80299</v>
+      </c>
+      <c r="S391">
+        <v>7.739608393889959</v>
+      </c>
+      <c r="T391">
+        <v>1162.08001</v>
+      </c>
+      <c r="U391">
+        <v>30</v>
+      </c>
+      <c r="V391">
+        <v>25</v>
+      </c>
+      <c r="W391">
+        <v>55</v>
+      </c>
+      <c r="X391">
+        <v>115</v>
+      </c>
+      <c r="Y391">
+        <v>30</v>
+      </c>
+      <c r="Z391">
+        <v>91</v>
+      </c>
+      <c r="AA391">
+        <v>25</v>
+      </c>
+      <c r="AB391">
+        <v>28</v>
+      </c>
+      <c r="AC391">
+        <v>3.98859</v>
+      </c>
+      <c r="AD391">
+        <v>-3.97648</v>
+      </c>
+      <c r="AE391">
+        <v>0</v>
+      </c>
+      <c r="AF391">
+        <v>1656.732</v>
+      </c>
+      <c r="AG391">
+        <v>0</v>
+      </c>
+      <c r="AH391">
+        <v>3</v>
+      </c>
+      <c r="AI391">
+        <v>2609.40897</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B392" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E392">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F392">
+        <v>7415.75</v>
+      </c>
+      <c r="G392">
+        <v>65.98620791932375</v>
+      </c>
+      <c r="H392">
+        <v>355.52</v>
+      </c>
+      <c r="I392">
+        <v>0</v>
+      </c>
+      <c r="J392">
+        <v>0</v>
+      </c>
+      <c r="K392">
+        <v>3.163458401305057</v>
+      </c>
+      <c r="L392">
+        <v>0</v>
+      </c>
+      <c r="M392">
+        <v>7</v>
+      </c>
+      <c r="N392">
+        <v>0</v>
+      </c>
+      <c r="O392">
+        <v>27.75329</v>
+      </c>
+      <c r="P392">
+        <v>79.3132430269776</v>
+      </c>
+      <c r="Q392">
+        <v>34.992</v>
+      </c>
+      <c r="R392">
+        <v>682.36867</v>
+      </c>
+      <c r="S392">
+        <v>6.071795966187156</v>
+      </c>
+      <c r="T392">
+        <v>1029.55</v>
+      </c>
+      <c r="U392">
+        <v>33</v>
+      </c>
+      <c r="V392">
+        <v>16</v>
+      </c>
+      <c r="W392">
+        <v>49</v>
+      </c>
+      <c r="X392">
+        <v>110</v>
+      </c>
+      <c r="Y392">
+        <v>33</v>
+      </c>
+      <c r="Z392">
+        <v>78</v>
+      </c>
+      <c r="AA392">
+        <v>16</v>
+      </c>
+      <c r="AB392">
+        <v>20</v>
+      </c>
+      <c r="AC392">
+        <v>4.15752</v>
+      </c>
+      <c r="AD392">
+        <v>-3.3995</v>
+      </c>
+      <c r="AE392">
+        <v>0</v>
+      </c>
+      <c r="AF392">
+        <v>601.56339</v>
+      </c>
+      <c r="AG392">
+        <v>0</v>
+      </c>
+      <c r="AH392">
+        <v>3</v>
+      </c>
+      <c r="AI392">
+        <v>2047.10601</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B393" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E393">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F393">
+        <v>6747.77</v>
+      </c>
+      <c r="G393">
+        <v>60.04244401601661</v>
+      </c>
+      <c r="H393">
+        <v>220.26</v>
+      </c>
+      <c r="I393">
+        <v>0</v>
+      </c>
+      <c r="J393">
+        <v>0</v>
+      </c>
+      <c r="K393">
+        <v>1.959899154678926</v>
+      </c>
+      <c r="L393">
+        <v>20.69</v>
+      </c>
+      <c r="M393">
+        <v>5</v>
+      </c>
+      <c r="N393">
+        <v>2</v>
+      </c>
+      <c r="O393">
+        <v>30.73734</v>
+      </c>
+      <c r="P393">
+        <v>88.02216494845361</v>
+      </c>
+      <c r="Q393">
+        <v>34.92</v>
+      </c>
+      <c r="R393">
+        <v>619.22077</v>
+      </c>
+      <c r="S393">
+        <v>5.509898591131543</v>
+      </c>
+      <c r="T393">
+        <v>906.13001</v>
+      </c>
+      <c r="U393">
+        <v>37</v>
+      </c>
+      <c r="V393">
+        <v>20</v>
+      </c>
+      <c r="W393">
+        <v>57</v>
+      </c>
+      <c r="X393">
+        <v>104</v>
+      </c>
+      <c r="Y393">
+        <v>37</v>
+      </c>
+      <c r="Z393">
+        <v>69</v>
+      </c>
+      <c r="AA393">
+        <v>20</v>
+      </c>
+      <c r="AB393">
+        <v>19</v>
+      </c>
+      <c r="AC393">
+        <v>4.65728</v>
+      </c>
+      <c r="AD393">
+        <v>-3.31796</v>
+      </c>
+      <c r="AE393">
+        <v>0</v>
+      </c>
+      <c r="AF393">
+        <v>640.568</v>
+      </c>
+      <c r="AG393">
+        <v>0</v>
+      </c>
+      <c r="AH393">
+        <v>3</v>
+      </c>
+      <c r="AI393">
+        <v>1857.66231</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B394" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E394">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F394">
+        <v>6981.27</v>
+      </c>
+      <c r="G394">
+        <v>62.12015423402047</v>
+      </c>
+      <c r="H394">
+        <v>0</v>
+      </c>
+      <c r="I394">
+        <v>0</v>
+      </c>
+      <c r="J394">
+        <v>0</v>
+      </c>
+      <c r="K394">
+        <v>0</v>
+      </c>
+      <c r="L394">
+        <v>0</v>
+      </c>
+      <c r="M394">
+        <v>0</v>
+      </c>
+      <c r="N394">
+        <v>0</v>
+      </c>
+      <c r="O394">
+        <v>26.79458</v>
+      </c>
+      <c r="P394">
+        <v>74.42938888888889</v>
+      </c>
+      <c r="Q394">
+        <v>36</v>
+      </c>
+      <c r="R394">
+        <v>699.5155599999999</v>
+      </c>
+      <c r="S394">
+        <v>6.224370992139996</v>
+      </c>
+      <c r="T394">
+        <v>0</v>
+      </c>
+      <c r="U394">
+        <v>0</v>
+      </c>
+      <c r="V394">
+        <v>0</v>
+      </c>
+      <c r="W394">
+        <v>0</v>
+      </c>
+      <c r="X394">
+        <v>0</v>
+      </c>
+      <c r="Y394">
+        <v>0</v>
+      </c>
+      <c r="Z394">
+        <v>0</v>
+      </c>
+      <c r="AA394">
+        <v>0</v>
+      </c>
+      <c r="AB394">
+        <v>0</v>
+      </c>
+      <c r="AC394">
+        <v>4.01195</v>
+      </c>
+      <c r="AD394">
+        <v>-4.31381</v>
+      </c>
+      <c r="AE394">
+        <v>0</v>
+      </c>
+      <c r="AF394">
+        <v>0</v>
+      </c>
+      <c r="AG394">
+        <v>0</v>
+      </c>
+      <c r="AH394">
+        <v>3</v>
+      </c>
+      <c r="AI394">
+        <v>2098.54668</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Luis Ángel Malagón</t>
+        </is>
+      </c>
+      <c r="B395" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>RTP</t>
+        </is>
+      </c>
+      <c r="E395">
+        <v>37.34033333333333</v>
+      </c>
+      <c r="F395">
+        <v>756.4</v>
+      </c>
+      <c r="G395">
+        <v>20.25691611394292</v>
+      </c>
+      <c r="H395">
+        <v>0</v>
+      </c>
+      <c r="I395">
+        <v>0</v>
+      </c>
+      <c r="J395">
+        <v>0</v>
+      </c>
+      <c r="K395">
+        <v>0</v>
+      </c>
+      <c r="L395">
+        <v>0</v>
+      </c>
+      <c r="M395">
+        <v>0</v>
+      </c>
+      <c r="N395">
+        <v>0</v>
+      </c>
+      <c r="O395">
+        <v>15.72703</v>
+      </c>
+      <c r="P395">
+        <v>52.44441109777244</v>
+      </c>
+      <c r="Q395">
+        <v>29.988</v>
+      </c>
+      <c r="R395">
+        <v>73.17626</v>
+      </c>
+      <c r="S395">
+        <v>1.95971094705457</v>
+      </c>
+      <c r="T395">
+        <v>24.51</v>
+      </c>
+      <c r="U395">
+        <v>1</v>
+      </c>
+      <c r="V395">
+        <v>1</v>
+      </c>
+      <c r="W395">
+        <v>2</v>
+      </c>
+      <c r="X395">
+        <v>5</v>
+      </c>
+      <c r="Y395">
+        <v>1</v>
+      </c>
+      <c r="Z395">
+        <v>5</v>
+      </c>
+      <c r="AA395">
+        <v>1</v>
+      </c>
+      <c r="AB395">
+        <v>7</v>
+      </c>
+      <c r="AC395">
+        <v>3.61843</v>
+      </c>
+      <c r="AD395">
+        <v>-3.07893</v>
+      </c>
+      <c r="AE395">
+        <v>0</v>
+      </c>
+      <c r="AF395">
+        <v>63.75954</v>
+      </c>
+      <c r="AG395">
+        <v>0</v>
+      </c>
+      <c r="AH395">
+        <v>3</v>
+      </c>
+      <c r="AI395">
+        <v>219.52878</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B396" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E396">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F396">
+        <v>6201.01</v>
+      </c>
+      <c r="G396">
+        <v>55.17730980275842</v>
+      </c>
+      <c r="H396">
+        <v>88.42</v>
+      </c>
+      <c r="I396">
+        <v>0</v>
+      </c>
+      <c r="J396">
+        <v>0</v>
+      </c>
+      <c r="K396">
+        <v>0.7867714667062138</v>
+      </c>
+      <c r="L396">
+        <v>0</v>
+      </c>
+      <c r="M396">
+        <v>1</v>
+      </c>
+      <c r="N396">
+        <v>0</v>
+      </c>
+      <c r="O396">
+        <v>25.78202</v>
+      </c>
+      <c r="P396">
+        <v>71.61672222222222</v>
+      </c>
+      <c r="Q396">
+        <v>36</v>
+      </c>
+      <c r="R396">
+        <v>707.42239</v>
+      </c>
+      <c r="S396">
+        <v>6.294726887142221</v>
+      </c>
+      <c r="T396">
+        <v>901.97</v>
+      </c>
+      <c r="U396">
+        <v>22</v>
+      </c>
+      <c r="V396">
+        <v>36</v>
+      </c>
+      <c r="W396">
+        <v>58</v>
+      </c>
+      <c r="X396">
+        <v>107</v>
+      </c>
+      <c r="Y396">
+        <v>22</v>
+      </c>
+      <c r="Z396">
+        <v>111</v>
+      </c>
+      <c r="AA396">
+        <v>36</v>
+      </c>
+      <c r="AB396">
+        <v>34</v>
+      </c>
+      <c r="AC396">
+        <v>3.83523</v>
+      </c>
+      <c r="AD396">
+        <v>-3.48341</v>
+      </c>
+      <c r="AE396">
+        <v>0</v>
+      </c>
+      <c r="AF396">
+        <v>1508.898</v>
+      </c>
+      <c r="AG396">
+        <v>0</v>
+      </c>
+      <c r="AH396">
+        <v>3</v>
+      </c>
+      <c r="AI396">
+        <v>2122.26717</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B397" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E397">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F397">
+        <v>6518.75</v>
+      </c>
+      <c r="G397">
+        <v>58.00459736022542</v>
+      </c>
+      <c r="H397">
+        <v>171.87</v>
+      </c>
+      <c r="I397">
+        <v>0</v>
+      </c>
+      <c r="J397">
+        <v>0</v>
+      </c>
+      <c r="K397">
+        <v>1.529319294082752</v>
+      </c>
+      <c r="L397">
+        <v>0</v>
+      </c>
+      <c r="M397">
+        <v>3</v>
+      </c>
+      <c r="N397">
+        <v>0</v>
+      </c>
+      <c r="O397">
+        <v>26.69193</v>
+      </c>
+      <c r="P397">
+        <v>78.5426377118644</v>
+      </c>
+      <c r="Q397">
+        <v>33.984</v>
+      </c>
+      <c r="R397">
+        <v>692.43371</v>
+      </c>
+      <c r="S397">
+        <v>6.161355865341836</v>
+      </c>
+      <c r="T397">
+        <v>972.58</v>
+      </c>
+      <c r="U397">
+        <v>20</v>
+      </c>
+      <c r="V397">
+        <v>29</v>
+      </c>
+      <c r="W397">
+        <v>49</v>
+      </c>
+      <c r="X397">
+        <v>90</v>
+      </c>
+      <c r="Y397">
+        <v>20</v>
+      </c>
+      <c r="Z397">
+        <v>86</v>
+      </c>
+      <c r="AA397">
+        <v>29</v>
+      </c>
+      <c r="AB397">
+        <v>32</v>
+      </c>
+      <c r="AC397">
+        <v>3.86911</v>
+      </c>
+      <c r="AD397">
+        <v>-2.84828</v>
+      </c>
+      <c r="AE397">
+        <v>0</v>
+      </c>
+      <c r="AF397">
+        <v>622.4264000000001</v>
+      </c>
+      <c r="AG397">
+        <v>0</v>
+      </c>
+      <c r="AH397">
+        <v>3</v>
+      </c>
+      <c r="AI397">
+        <v>2077.30113</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B398" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E398">
+        <v>72.15000000000001</v>
+      </c>
+      <c r="F398">
+        <v>3422.15</v>
+      </c>
+      <c r="G398">
+        <v>47.43104643104643</v>
+      </c>
+      <c r="H398">
+        <v>43.03000000000001</v>
+      </c>
+      <c r="I398">
+        <v>0</v>
+      </c>
+      <c r="J398">
+        <v>0</v>
+      </c>
+      <c r="K398">
+        <v>0.5963963963963964</v>
+      </c>
+      <c r="L398">
+        <v>0</v>
+      </c>
+      <c r="M398">
+        <v>0</v>
+      </c>
+      <c r="N398">
+        <v>0</v>
+      </c>
+      <c r="O398">
+        <v>23.2567</v>
+      </c>
+      <c r="P398">
+        <v>66.46290580704161</v>
+      </c>
+      <c r="Q398">
+        <v>34.992</v>
+      </c>
+      <c r="R398">
+        <v>337.82899</v>
+      </c>
+      <c r="S398">
+        <v>4.682314483714483</v>
+      </c>
+      <c r="T398">
+        <v>518.84</v>
+      </c>
+      <c r="U398">
+        <v>16</v>
+      </c>
+      <c r="V398">
+        <v>9</v>
+      </c>
+      <c r="W398">
+        <v>25</v>
+      </c>
+      <c r="X398">
+        <v>62</v>
+      </c>
+      <c r="Y398">
+        <v>16</v>
+      </c>
+      <c r="Z398">
+        <v>66</v>
+      </c>
+      <c r="AA398">
+        <v>9</v>
+      </c>
+      <c r="AB398">
+        <v>19</v>
+      </c>
+      <c r="AC398">
+        <v>3.94769</v>
+      </c>
+      <c r="AD398">
+        <v>-2.95672</v>
+      </c>
+      <c r="AE398">
+        <v>0</v>
+      </c>
+      <c r="AF398">
+        <v>336.128</v>
+      </c>
+      <c r="AG398">
+        <v>0</v>
+      </c>
+      <c r="AH398">
+        <v>3</v>
+      </c>
+      <c r="AI398">
+        <v>1013.48697</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B399" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E399">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F399">
+        <v>7006.26</v>
+      </c>
+      <c r="G399">
+        <v>62.34251816698799</v>
+      </c>
+      <c r="H399">
+        <v>182.53</v>
+      </c>
+      <c r="I399">
+        <v>0</v>
+      </c>
+      <c r="J399">
+        <v>0</v>
+      </c>
+      <c r="K399">
+        <v>1.624173216669138</v>
+      </c>
+      <c r="L399">
+        <v>0</v>
+      </c>
+      <c r="M399">
+        <v>4</v>
+      </c>
+      <c r="N399">
+        <v>0</v>
+      </c>
+      <c r="O399">
+        <v>27.40305</v>
+      </c>
+      <c r="P399">
+        <v>83.00936023264268</v>
+      </c>
+      <c r="Q399">
+        <v>33.012</v>
+      </c>
+      <c r="R399">
+        <v>708.1821</v>
+      </c>
+      <c r="S399">
+        <v>6.301486875278066</v>
+      </c>
+      <c r="T399">
+        <v>1140.66</v>
+      </c>
+      <c r="U399">
+        <v>29</v>
+      </c>
+      <c r="V399">
+        <v>32</v>
+      </c>
+      <c r="W399">
+        <v>61</v>
+      </c>
+      <c r="X399">
+        <v>143</v>
+      </c>
+      <c r="Y399">
+        <v>29</v>
+      </c>
+      <c r="Z399">
+        <v>115</v>
+      </c>
+      <c r="AA399">
+        <v>32</v>
+      </c>
+      <c r="AB399">
+        <v>40</v>
+      </c>
+      <c r="AC399">
+        <v>4.67771</v>
+      </c>
+      <c r="AD399">
+        <v>-2.90657</v>
+      </c>
+      <c r="AE399">
+        <v>0</v>
+      </c>
+      <c r="AF399">
+        <v>635.82375</v>
+      </c>
+      <c r="AG399">
+        <v>0</v>
+      </c>
+      <c r="AH399">
+        <v>3</v>
+      </c>
+      <c r="AI399">
+        <v>2124.5463</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B400" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E400">
+        <v>112.3833333333333</v>
+      </c>
+      <c r="F400">
+        <v>6399.84</v>
+      </c>
+      <c r="G400">
+        <v>56.94652231944238</v>
+      </c>
+      <c r="H400">
+        <v>149.91</v>
+      </c>
+      <c r="I400">
+        <v>0</v>
+      </c>
+      <c r="J400">
+        <v>0</v>
+      </c>
+      <c r="K400">
+        <v>1.333916654308172</v>
+      </c>
+      <c r="L400">
+        <v>0</v>
+      </c>
+      <c r="M400">
+        <v>2</v>
+      </c>
+      <c r="N400">
+        <v>0</v>
+      </c>
+      <c r="O400">
+        <v>27.30133</v>
+      </c>
+      <c r="P400">
+        <v>85.30599300087491</v>
+      </c>
+      <c r="Q400">
+        <v>32.004</v>
+      </c>
+      <c r="R400">
+        <v>605.31791</v>
+      </c>
+      <c r="S400">
+        <v>5.386189322260121</v>
+      </c>
+      <c r="T400">
+        <v>757.2</v>
+      </c>
+      <c r="U400">
+        <v>20</v>
+      </c>
+      <c r="V400">
+        <v>23</v>
+      </c>
+      <c r="W400">
+        <v>43</v>
+      </c>
+      <c r="X400">
+        <v>93</v>
+      </c>
+      <c r="Y400">
+        <v>20</v>
+      </c>
+      <c r="Z400">
+        <v>76</v>
+      </c>
+      <c r="AA400">
+        <v>23</v>
+      </c>
+      <c r="AB400">
+        <v>22</v>
+      </c>
+      <c r="AC400">
+        <v>4.36478</v>
+      </c>
+      <c r="AD400">
+        <v>-2.62083</v>
+      </c>
+      <c r="AE400">
+        <v>0</v>
+      </c>
+      <c r="AF400">
+        <v>531.7900000000001</v>
+      </c>
+      <c r="AG400">
+        <v>0</v>
+      </c>
+      <c r="AH400">
+        <v>3</v>
+      </c>
+      <c r="AI400">
+        <v>1815.95373</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B401" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Sesion 29</t>
+        </is>
+      </c>
+      <c r="E401">
+        <v>72.15000000000001</v>
+      </c>
+      <c r="F401">
+        <v>4211.299999999999</v>
+      </c>
+      <c r="G401">
+        <v>58.36867636867635</v>
+      </c>
+      <c r="H401">
+        <v>70.56000000000002</v>
+      </c>
+      <c r="I401">
+        <v>0</v>
+      </c>
+      <c r="J401">
+        <v>0</v>
+      </c>
+      <c r="K401">
+        <v>0.9779625779625781</v>
+      </c>
+      <c r="L401">
+        <v>0</v>
+      </c>
+      <c r="M401">
+        <v>1</v>
+      </c>
+      <c r="N401">
+        <v>0</v>
+      </c>
+      <c r="O401">
+        <v>25.36778</v>
+      </c>
+      <c r="P401">
+        <v>70.46605555555556</v>
+      </c>
+      <c r="Q401">
+        <v>36</v>
+      </c>
+      <c r="R401">
+        <v>474.61928</v>
+      </c>
+      <c r="S401">
+        <v>6.578229799029798</v>
+      </c>
+      <c r="T401">
+        <v>587.93001</v>
+      </c>
+      <c r="U401">
+        <v>19</v>
+      </c>
+      <c r="V401">
+        <v>25</v>
+      </c>
+      <c r="W401">
+        <v>44</v>
+      </c>
+      <c r="X401">
+        <v>76</v>
+      </c>
+      <c r="Y401">
+        <v>19</v>
+      </c>
+      <c r="Z401">
+        <v>71</v>
+      </c>
+      <c r="AA401">
+        <v>25</v>
+      </c>
+      <c r="AB401">
+        <v>27</v>
+      </c>
+      <c r="AC401">
+        <v>4.67091</v>
+      </c>
+      <c r="AD401">
+        <v>-4.03921</v>
+      </c>
+      <c r="AE401">
+        <v>0</v>
+      </c>
+      <c r="AF401">
+        <v>359.2715</v>
+      </c>
+      <c r="AG401">
+        <v>0</v>
+      </c>
+      <c r="AH401">
+        <v>3</v>
+      </c>
+      <c r="AI401">
+        <v>1423.85784</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B402" s="2">
+        <v>46210</v>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>RTP</t>
+        </is>
+      </c>
+      <c r="E402">
+        <v>41.676</v>
+      </c>
+      <c r="F402">
+        <v>3959.07</v>
+      </c>
+      <c r="G402">
+        <v>94.99640080621941</v>
+      </c>
+      <c r="H402">
+        <v>70.67</v>
+      </c>
+      <c r="I402">
+        <v>0</v>
+      </c>
+      <c r="J402">
+        <v>0</v>
+      </c>
+      <c r="K402">
+        <v>1.695700163163451</v>
+      </c>
+      <c r="L402">
+        <v>0</v>
+      </c>
+      <c r="M402">
+        <v>0</v>
+      </c>
+      <c r="N402">
+        <v>0</v>
+      </c>
+      <c r="O402">
+        <v>21.83875</v>
+      </c>
+      <c r="P402">
+        <v>64.26185852165725</v>
+      </c>
+      <c r="Q402">
+        <v>33.984</v>
+      </c>
+      <c r="R402">
+        <v>349.3541</v>
+      </c>
+      <c r="S402">
+        <v>8.382620692964776</v>
+      </c>
+      <c r="T402">
+        <v>302.62</v>
+      </c>
+      <c r="U402">
+        <v>0</v>
+      </c>
+      <c r="V402">
+        <v>0</v>
+      </c>
+      <c r="W402">
+        <v>0</v>
+      </c>
+      <c r="X402">
+        <v>1</v>
+      </c>
+      <c r="Y402">
+        <v>0</v>
+      </c>
+      <c r="Z402">
+        <v>0</v>
+      </c>
+      <c r="AA402">
+        <v>0</v>
+      </c>
+      <c r="AB402">
+        <v>0</v>
+      </c>
+      <c r="AC402">
+        <v>2.32284</v>
+      </c>
+      <c r="AD402">
+        <v>-1.89608</v>
+      </c>
+      <c r="AE402">
+        <v>0</v>
+      </c>
+      <c r="AF402">
+        <v>291.4002</v>
+      </c>
+      <c r="AG402">
+        <v>0</v>
+      </c>
+      <c r="AH402">
+        <v>3</v>
+      </c>
+      <c r="AI402">
+        <v>1048.0623</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-09
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI402"/>
+  <dimension ref="A1:AI421"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -45756,6 +45756,2153 @@
         <v>1048.0623</v>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B403" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E403">
+        <v>82.786</v>
+      </c>
+      <c r="F403">
+        <v>8967.089999999998</v>
+      </c>
+      <c r="G403">
+        <v>108.3165027903269</v>
+      </c>
+      <c r="H403">
+        <v>0</v>
+      </c>
+      <c r="I403">
+        <v>0</v>
+      </c>
+      <c r="J403">
+        <v>0</v>
+      </c>
+      <c r="K403">
+        <v>0</v>
+      </c>
+      <c r="L403">
+        <v>0</v>
+      </c>
+      <c r="M403">
+        <v>0</v>
+      </c>
+      <c r="N403">
+        <v>0</v>
+      </c>
+      <c r="O403">
+        <v>30.0385</v>
+      </c>
+      <c r="P403">
+        <v>83.44027777777777</v>
+      </c>
+      <c r="Q403">
+        <v>36</v>
+      </c>
+      <c r="R403">
+        <v>945.37673</v>
+      </c>
+      <c r="S403">
+        <v>11.41952419491218</v>
+      </c>
+      <c r="T403">
+        <v>0</v>
+      </c>
+      <c r="U403">
+        <v>0</v>
+      </c>
+      <c r="V403">
+        <v>0</v>
+      </c>
+      <c r="W403">
+        <v>0</v>
+      </c>
+      <c r="X403">
+        <v>0</v>
+      </c>
+      <c r="Y403">
+        <v>0</v>
+      </c>
+      <c r="Z403">
+        <v>0</v>
+      </c>
+      <c r="AA403">
+        <v>0</v>
+      </c>
+      <c r="AB403">
+        <v>0</v>
+      </c>
+      <c r="AC403">
+        <v>4.23209</v>
+      </c>
+      <c r="AD403">
+        <v>-3.74016</v>
+      </c>
+      <c r="AE403">
+        <v>0</v>
+      </c>
+      <c r="AF403">
+        <v>0</v>
+      </c>
+      <c r="AG403">
+        <v>0</v>
+      </c>
+      <c r="AH403">
+        <v>3</v>
+      </c>
+      <c r="AI403">
+        <v>2836.13019</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B404" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E404">
+        <v>82.786</v>
+      </c>
+      <c r="F404">
+        <v>7273.349999999999</v>
+      </c>
+      <c r="G404">
+        <v>87.85724639431787</v>
+      </c>
+      <c r="H404">
+        <v>190.78</v>
+      </c>
+      <c r="I404">
+        <v>0</v>
+      </c>
+      <c r="J404">
+        <v>0</v>
+      </c>
+      <c r="K404">
+        <v>2.304495929263402</v>
+      </c>
+      <c r="L404">
+        <v>0</v>
+      </c>
+      <c r="M404">
+        <v>3</v>
+      </c>
+      <c r="N404">
+        <v>0</v>
+      </c>
+      <c r="O404">
+        <v>29.68098</v>
+      </c>
+      <c r="P404">
+        <v>82.44716666666667</v>
+      </c>
+      <c r="Q404">
+        <v>36</v>
+      </c>
+      <c r="R404">
+        <v>576.26224</v>
+      </c>
+      <c r="S404">
+        <v>6.960865846882323</v>
+      </c>
+      <c r="T404">
+        <v>1137.07998</v>
+      </c>
+      <c r="U404">
+        <v>28</v>
+      </c>
+      <c r="V404">
+        <v>33</v>
+      </c>
+      <c r="W404">
+        <v>61</v>
+      </c>
+      <c r="X404">
+        <v>100</v>
+      </c>
+      <c r="Y404">
+        <v>28</v>
+      </c>
+      <c r="Z404">
+        <v>104</v>
+      </c>
+      <c r="AA404">
+        <v>33</v>
+      </c>
+      <c r="AB404">
+        <v>28</v>
+      </c>
+      <c r="AC404">
+        <v>4.02885</v>
+      </c>
+      <c r="AD404">
+        <v>-3.56639</v>
+      </c>
+      <c r="AE404">
+        <v>0</v>
+      </c>
+      <c r="AF404">
+        <v>1745.442</v>
+      </c>
+      <c r="AG404">
+        <v>0</v>
+      </c>
+      <c r="AH404">
+        <v>3</v>
+      </c>
+      <c r="AI404">
+        <v>1728.78672</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B405" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E405">
+        <v>82.786</v>
+      </c>
+      <c r="F405">
+        <v>8943.91</v>
+      </c>
+      <c r="G405">
+        <v>108.0365037566738</v>
+      </c>
+      <c r="H405">
+        <v>519.2</v>
+      </c>
+      <c r="I405">
+        <v>0</v>
+      </c>
+      <c r="J405">
+        <v>0</v>
+      </c>
+      <c r="K405">
+        <v>6.271591815041191</v>
+      </c>
+      <c r="L405">
+        <v>0</v>
+      </c>
+      <c r="M405">
+        <v>9</v>
+      </c>
+      <c r="N405">
+        <v>0</v>
+      </c>
+      <c r="O405">
+        <v>28.31543</v>
+      </c>
+      <c r="P405">
+        <v>87.3933024691358</v>
+      </c>
+      <c r="Q405">
+        <v>32.4</v>
+      </c>
+      <c r="R405">
+        <v>1000.33718</v>
+      </c>
+      <c r="S405">
+        <v>12.08340999685937</v>
+      </c>
+      <c r="T405">
+        <v>1821.31</v>
+      </c>
+      <c r="U405">
+        <v>24</v>
+      </c>
+      <c r="V405">
+        <v>33</v>
+      </c>
+      <c r="W405">
+        <v>57</v>
+      </c>
+      <c r="X405">
+        <v>112</v>
+      </c>
+      <c r="Y405">
+        <v>24</v>
+      </c>
+      <c r="Z405">
+        <v>105</v>
+      </c>
+      <c r="AA405">
+        <v>33</v>
+      </c>
+      <c r="AB405">
+        <v>9</v>
+      </c>
+      <c r="AC405">
+        <v>4.23609</v>
+      </c>
+      <c r="AD405">
+        <v>-4.10146</v>
+      </c>
+      <c r="AE405">
+        <v>0</v>
+      </c>
+      <c r="AF405">
+        <v>750.8256</v>
+      </c>
+      <c r="AG405">
+        <v>0</v>
+      </c>
+      <c r="AH405">
+        <v>3</v>
+      </c>
+      <c r="AI405">
+        <v>3001.01154</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B406" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E406">
+        <v>82.786</v>
+      </c>
+      <c r="F406">
+        <v>7010.91</v>
+      </c>
+      <c r="G406">
+        <v>84.6871451694731</v>
+      </c>
+      <c r="H406">
+        <v>522.86</v>
+      </c>
+      <c r="I406">
+        <v>17.41</v>
+      </c>
+      <c r="J406">
+        <v>1</v>
+      </c>
+      <c r="K406">
+        <v>6.31580218877588</v>
+      </c>
+      <c r="L406">
+        <v>31.39</v>
+      </c>
+      <c r="M406">
+        <v>16</v>
+      </c>
+      <c r="N406">
+        <v>2</v>
+      </c>
+      <c r="O406">
+        <v>32.35937</v>
+      </c>
+      <c r="P406">
+        <v>95.2194267890772</v>
+      </c>
+      <c r="Q406">
+        <v>33.984</v>
+      </c>
+      <c r="R406">
+        <v>747.39282</v>
+      </c>
+      <c r="S406">
+        <v>9.028009808421714</v>
+      </c>
+      <c r="T406">
+        <v>1069.29</v>
+      </c>
+      <c r="U406">
+        <v>18</v>
+      </c>
+      <c r="V406">
+        <v>17</v>
+      </c>
+      <c r="W406">
+        <v>35</v>
+      </c>
+      <c r="X406">
+        <v>64</v>
+      </c>
+      <c r="Y406">
+        <v>18</v>
+      </c>
+      <c r="Z406">
+        <v>60</v>
+      </c>
+      <c r="AA406">
+        <v>17</v>
+      </c>
+      <c r="AB406">
+        <v>9</v>
+      </c>
+      <c r="AC406">
+        <v>4.87381</v>
+      </c>
+      <c r="AD406">
+        <v>-2.54924</v>
+      </c>
+      <c r="AE406">
+        <v>0</v>
+      </c>
+      <c r="AF406">
+        <v>655.6184000000001</v>
+      </c>
+      <c r="AG406">
+        <v>0</v>
+      </c>
+      <c r="AH406">
+        <v>3</v>
+      </c>
+      <c r="AI406">
+        <v>2242.17846</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B407" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E407">
+        <v>82.786</v>
+      </c>
+      <c r="F407">
+        <v>7763.3</v>
+      </c>
+      <c r="G407">
+        <v>93.77551759959414</v>
+      </c>
+      <c r="H407">
+        <v>505.97</v>
+      </c>
+      <c r="I407">
+        <v>0</v>
+      </c>
+      <c r="J407">
+        <v>0</v>
+      </c>
+      <c r="K407">
+        <v>6.111782185393666</v>
+      </c>
+      <c r="L407">
+        <v>2.38</v>
+      </c>
+      <c r="M407">
+        <v>13</v>
+      </c>
+      <c r="N407">
+        <v>0</v>
+      </c>
+      <c r="O407">
+        <v>30.10512</v>
+      </c>
+      <c r="P407">
+        <v>84.64102564102565</v>
+      </c>
+      <c r="Q407">
+        <v>35.568</v>
+      </c>
+      <c r="R407">
+        <v>664.80654</v>
+      </c>
+      <c r="S407">
+        <v>8.030422293624527</v>
+      </c>
+      <c r="T407">
+        <v>1177.43997</v>
+      </c>
+      <c r="U407">
+        <v>26</v>
+      </c>
+      <c r="V407">
+        <v>25</v>
+      </c>
+      <c r="W407">
+        <v>51</v>
+      </c>
+      <c r="X407">
+        <v>84</v>
+      </c>
+      <c r="Y407">
+        <v>26</v>
+      </c>
+      <c r="Z407">
+        <v>66</v>
+      </c>
+      <c r="AA407">
+        <v>25</v>
+      </c>
+      <c r="AB407">
+        <v>12</v>
+      </c>
+      <c r="AC407">
+        <v>4.61956</v>
+      </c>
+      <c r="AD407">
+        <v>-3.35035</v>
+      </c>
+      <c r="AE407">
+        <v>0</v>
+      </c>
+      <c r="AF407">
+        <v>737.0215999999999</v>
+      </c>
+      <c r="AG407">
+        <v>0</v>
+      </c>
+      <c r="AH407">
+        <v>3</v>
+      </c>
+      <c r="AI407">
+        <v>1994.41962</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B408" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E408">
+        <v>82.786</v>
+      </c>
+      <c r="F408">
+        <v>8071.630000000001</v>
+      </c>
+      <c r="G408">
+        <v>97.49993960331459</v>
+      </c>
+      <c r="H408">
+        <v>358.8</v>
+      </c>
+      <c r="I408">
+        <v>0</v>
+      </c>
+      <c r="J408">
+        <v>0</v>
+      </c>
+      <c r="K408">
+        <v>4.334066146449883</v>
+      </c>
+      <c r="L408">
+        <v>0</v>
+      </c>
+      <c r="M408">
+        <v>5</v>
+      </c>
+      <c r="N408">
+        <v>0</v>
+      </c>
+      <c r="O408">
+        <v>29.28776</v>
+      </c>
+      <c r="P408">
+        <v>81.35488888888889</v>
+      </c>
+      <c r="Q408">
+        <v>36</v>
+      </c>
+      <c r="R408">
+        <v>770.25032</v>
+      </c>
+      <c r="S408">
+        <v>9.304113255864518</v>
+      </c>
+      <c r="T408">
+        <v>1153.19999</v>
+      </c>
+      <c r="U408">
+        <v>14</v>
+      </c>
+      <c r="V408">
+        <v>13</v>
+      </c>
+      <c r="W408">
+        <v>27</v>
+      </c>
+      <c r="X408">
+        <v>66</v>
+      </c>
+      <c r="Y408">
+        <v>14</v>
+      </c>
+      <c r="Z408">
+        <v>65</v>
+      </c>
+      <c r="AA408">
+        <v>13</v>
+      </c>
+      <c r="AB408">
+        <v>13</v>
+      </c>
+      <c r="AC408">
+        <v>3.80718</v>
+      </c>
+      <c r="AD408">
+        <v>-3.04569</v>
+      </c>
+      <c r="AE408">
+        <v>0</v>
+      </c>
+      <c r="AF408">
+        <v>1864.636</v>
+      </c>
+      <c r="AG408">
+        <v>0</v>
+      </c>
+      <c r="AH408">
+        <v>3</v>
+      </c>
+      <c r="AI408">
+        <v>2310.75096</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B409" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E409">
+        <v>82.786</v>
+      </c>
+      <c r="F409">
+        <v>7743.389999999999</v>
+      </c>
+      <c r="G409">
+        <v>93.53501799821225</v>
+      </c>
+      <c r="H409">
+        <v>536.05</v>
+      </c>
+      <c r="I409">
+        <v>16.1</v>
+      </c>
+      <c r="J409">
+        <v>1</v>
+      </c>
+      <c r="K409">
+        <v>6.475128644939965</v>
+      </c>
+      <c r="L409">
+        <v>58.09</v>
+      </c>
+      <c r="M409">
+        <v>19</v>
+      </c>
+      <c r="N409">
+        <v>2</v>
+      </c>
+      <c r="O409">
+        <v>32.71645</v>
+      </c>
+      <c r="P409">
+        <v>90.87902777777779</v>
+      </c>
+      <c r="Q409">
+        <v>36</v>
+      </c>
+      <c r="R409">
+        <v>694.23591</v>
+      </c>
+      <c r="S409">
+        <v>8.385909574082573</v>
+      </c>
+      <c r="T409">
+        <v>1364.99001</v>
+      </c>
+      <c r="U409">
+        <v>29</v>
+      </c>
+      <c r="V409">
+        <v>40</v>
+      </c>
+      <c r="W409">
+        <v>69</v>
+      </c>
+      <c r="X409">
+        <v>102</v>
+      </c>
+      <c r="Y409">
+        <v>29</v>
+      </c>
+      <c r="Z409">
+        <v>90</v>
+      </c>
+      <c r="AA409">
+        <v>40</v>
+      </c>
+      <c r="AB409">
+        <v>25</v>
+      </c>
+      <c r="AC409">
+        <v>4.5149</v>
+      </c>
+      <c r="AD409">
+        <v>-3.96735</v>
+      </c>
+      <c r="AE409">
+        <v>0</v>
+      </c>
+      <c r="AF409">
+        <v>649.4978</v>
+      </c>
+      <c r="AG409">
+        <v>0</v>
+      </c>
+      <c r="AH409">
+        <v>3</v>
+      </c>
+      <c r="AI409">
+        <v>2082.70773</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B410" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E410">
+        <v>82.786</v>
+      </c>
+      <c r="F410">
+        <v>7758.34</v>
+      </c>
+      <c r="G410">
+        <v>93.71560408764768</v>
+      </c>
+      <c r="H410">
+        <v>283.97</v>
+      </c>
+      <c r="I410">
+        <v>3.08</v>
+      </c>
+      <c r="J410">
+        <v>0</v>
+      </c>
+      <c r="K410">
+        <v>3.430169352305946</v>
+      </c>
+      <c r="L410">
+        <v>0</v>
+      </c>
+      <c r="M410">
+        <v>3</v>
+      </c>
+      <c r="N410">
+        <v>0</v>
+      </c>
+      <c r="O410">
+        <v>28.9273</v>
+      </c>
+      <c r="P410">
+        <v>90.38651418572678</v>
+      </c>
+      <c r="Q410">
+        <v>32.004</v>
+      </c>
+      <c r="R410">
+        <v>792.04194</v>
+      </c>
+      <c r="S410">
+        <v>9.567341579494117</v>
+      </c>
+      <c r="T410">
+        <v>1093.67999</v>
+      </c>
+      <c r="U410">
+        <v>9</v>
+      </c>
+      <c r="V410">
+        <v>16</v>
+      </c>
+      <c r="W410">
+        <v>25</v>
+      </c>
+      <c r="X410">
+        <v>65</v>
+      </c>
+      <c r="Y410">
+        <v>9</v>
+      </c>
+      <c r="Z410">
+        <v>70</v>
+      </c>
+      <c r="AA410">
+        <v>16</v>
+      </c>
+      <c r="AB410">
+        <v>16</v>
+      </c>
+      <c r="AC410">
+        <v>4.68737</v>
+      </c>
+      <c r="AD410">
+        <v>-3.87476</v>
+      </c>
+      <c r="AE410">
+        <v>0</v>
+      </c>
+      <c r="AF410">
+        <v>540.1314</v>
+      </c>
+      <c r="AG410">
+        <v>0</v>
+      </c>
+      <c r="AH410">
+        <v>3</v>
+      </c>
+      <c r="AI410">
+        <v>2376.12582</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B411" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E411">
+        <v>82.786</v>
+      </c>
+      <c r="F411">
+        <v>7516.170000000001</v>
+      </c>
+      <c r="G411">
+        <v>90.79035102553573</v>
+      </c>
+      <c r="H411">
+        <v>398.23</v>
+      </c>
+      <c r="I411">
+        <v>0</v>
+      </c>
+      <c r="J411">
+        <v>0</v>
+      </c>
+      <c r="K411">
+        <v>4.810354407750102</v>
+      </c>
+      <c r="L411">
+        <v>0</v>
+      </c>
+      <c r="M411">
+        <v>8</v>
+      </c>
+      <c r="N411">
+        <v>0</v>
+      </c>
+      <c r="O411">
+        <v>29.11733</v>
+      </c>
+      <c r="P411">
+        <v>86.04411938534278</v>
+      </c>
+      <c r="Q411">
+        <v>33.84</v>
+      </c>
+      <c r="R411">
+        <v>665.73258</v>
+      </c>
+      <c r="S411">
+        <v>8.041608242939628</v>
+      </c>
+      <c r="T411">
+        <v>1317.82001</v>
+      </c>
+      <c r="U411">
+        <v>27</v>
+      </c>
+      <c r="V411">
+        <v>24</v>
+      </c>
+      <c r="W411">
+        <v>51</v>
+      </c>
+      <c r="X411">
+        <v>111</v>
+      </c>
+      <c r="Y411">
+        <v>27</v>
+      </c>
+      <c r="Z411">
+        <v>83</v>
+      </c>
+      <c r="AA411">
+        <v>24</v>
+      </c>
+      <c r="AB411">
+        <v>21</v>
+      </c>
+      <c r="AC411">
+        <v>4.80876</v>
+      </c>
+      <c r="AD411">
+        <v>-3.59074</v>
+      </c>
+      <c r="AE411">
+        <v>0</v>
+      </c>
+      <c r="AF411">
+        <v>627.879</v>
+      </c>
+      <c r="AG411">
+        <v>0</v>
+      </c>
+      <c r="AH411">
+        <v>3</v>
+      </c>
+      <c r="AI411">
+        <v>1997.19774</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B412" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E412">
+        <v>82.786</v>
+      </c>
+      <c r="F412">
+        <v>7259.29</v>
+      </c>
+      <c r="G412">
+        <v>87.68741091488899</v>
+      </c>
+      <c r="H412">
+        <v>420.38</v>
+      </c>
+      <c r="I412">
+        <v>0</v>
+      </c>
+      <c r="J412">
+        <v>0</v>
+      </c>
+      <c r="K412">
+        <v>5.077911724204576</v>
+      </c>
+      <c r="L412">
+        <v>0</v>
+      </c>
+      <c r="M412">
+        <v>7</v>
+      </c>
+      <c r="N412">
+        <v>0</v>
+      </c>
+      <c r="O412">
+        <v>28.0647</v>
+      </c>
+      <c r="P412">
+        <v>83.28792735042735</v>
+      </c>
+      <c r="Q412">
+        <v>33.696</v>
+      </c>
+      <c r="R412">
+        <v>686.78451</v>
+      </c>
+      <c r="S412">
+        <v>8.295901601720097</v>
+      </c>
+      <c r="T412">
+        <v>1257.52001</v>
+      </c>
+      <c r="U412">
+        <v>30</v>
+      </c>
+      <c r="V412">
+        <v>32</v>
+      </c>
+      <c r="W412">
+        <v>62</v>
+      </c>
+      <c r="X412">
+        <v>102</v>
+      </c>
+      <c r="Y412">
+        <v>30</v>
+      </c>
+      <c r="Z412">
+        <v>91</v>
+      </c>
+      <c r="AA412">
+        <v>32</v>
+      </c>
+      <c r="AB412">
+        <v>15</v>
+      </c>
+      <c r="AC412">
+        <v>4.50056</v>
+      </c>
+      <c r="AD412">
+        <v>-3.76769</v>
+      </c>
+      <c r="AE412">
+        <v>0</v>
+      </c>
+      <c r="AF412">
+        <v>696.8096</v>
+      </c>
+      <c r="AG412">
+        <v>0</v>
+      </c>
+      <c r="AH412">
+        <v>3</v>
+      </c>
+      <c r="AI412">
+        <v>2060.35353</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B413" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E413">
+        <v>82.786</v>
+      </c>
+      <c r="F413">
+        <v>8497.16</v>
+      </c>
+      <c r="G413">
+        <v>102.6400599135119</v>
+      </c>
+      <c r="H413">
+        <v>139.61</v>
+      </c>
+      <c r="I413">
+        <v>0</v>
+      </c>
+      <c r="J413">
+        <v>0</v>
+      </c>
+      <c r="K413">
+        <v>1.686396250573768</v>
+      </c>
+      <c r="L413">
+        <v>5.649999999999999</v>
+      </c>
+      <c r="M413">
+        <v>2</v>
+      </c>
+      <c r="N413">
+        <v>1</v>
+      </c>
+      <c r="O413">
+        <v>30.17083</v>
+      </c>
+      <c r="P413">
+        <v>83.80786111111111</v>
+      </c>
+      <c r="Q413">
+        <v>36</v>
+      </c>
+      <c r="R413">
+        <v>934.37693</v>
+      </c>
+      <c r="S413">
+        <v>11.28665390283381</v>
+      </c>
+      <c r="T413">
+        <v>1026.41002</v>
+      </c>
+      <c r="U413">
+        <v>12</v>
+      </c>
+      <c r="V413">
+        <v>21</v>
+      </c>
+      <c r="W413">
+        <v>33</v>
+      </c>
+      <c r="X413">
+        <v>77</v>
+      </c>
+      <c r="Y413">
+        <v>12</v>
+      </c>
+      <c r="Z413">
+        <v>74</v>
+      </c>
+      <c r="AA413">
+        <v>21</v>
+      </c>
+      <c r="AB413">
+        <v>15</v>
+      </c>
+      <c r="AC413">
+        <v>3.91306</v>
+      </c>
+      <c r="AD413">
+        <v>-3.73288</v>
+      </c>
+      <c r="AE413">
+        <v>0</v>
+      </c>
+      <c r="AF413">
+        <v>1955.962</v>
+      </c>
+      <c r="AG413">
+        <v>0</v>
+      </c>
+      <c r="AH413">
+        <v>3</v>
+      </c>
+      <c r="AI413">
+        <v>2803.13079</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B414" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E414">
+        <v>82.786</v>
+      </c>
+      <c r="F414">
+        <v>7788.43</v>
+      </c>
+      <c r="G414">
+        <v>94.07907134056484</v>
+      </c>
+      <c r="H414">
+        <v>442.17</v>
+      </c>
+      <c r="I414">
+        <v>9.57</v>
+      </c>
+      <c r="J414">
+        <v>1</v>
+      </c>
+      <c r="K414">
+        <v>5.341120479308096</v>
+      </c>
+      <c r="L414">
+        <v>16.25</v>
+      </c>
+      <c r="M414">
+        <v>14</v>
+      </c>
+      <c r="N414">
+        <v>1</v>
+      </c>
+      <c r="O414">
+        <v>32.14973</v>
+      </c>
+      <c r="P414">
+        <v>91.87737197073616</v>
+      </c>
+      <c r="Q414">
+        <v>34.992</v>
+      </c>
+      <c r="R414">
+        <v>673.4404999999999</v>
+      </c>
+      <c r="S414">
+        <v>8.134714806851399</v>
+      </c>
+      <c r="T414">
+        <v>1188.03999</v>
+      </c>
+      <c r="U414">
+        <v>22</v>
+      </c>
+      <c r="V414">
+        <v>19</v>
+      </c>
+      <c r="W414">
+        <v>41</v>
+      </c>
+      <c r="X414">
+        <v>81</v>
+      </c>
+      <c r="Y414">
+        <v>22</v>
+      </c>
+      <c r="Z414">
+        <v>66</v>
+      </c>
+      <c r="AA414">
+        <v>19</v>
+      </c>
+      <c r="AB414">
+        <v>16</v>
+      </c>
+      <c r="AC414">
+        <v>4.32916</v>
+      </c>
+      <c r="AD414">
+        <v>-3.97201</v>
+      </c>
+      <c r="AE414">
+        <v>0</v>
+      </c>
+      <c r="AF414">
+        <v>632.2980600000001</v>
+      </c>
+      <c r="AG414">
+        <v>0</v>
+      </c>
+      <c r="AH414">
+        <v>3</v>
+      </c>
+      <c r="AI414">
+        <v>2020.3215</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B415" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E415">
+        <v>82.786</v>
+      </c>
+      <c r="F415">
+        <v>7014.670000000001</v>
+      </c>
+      <c r="G415">
+        <v>84.7325634769164</v>
+      </c>
+      <c r="H415">
+        <v>252.86</v>
+      </c>
+      <c r="I415">
+        <v>6.01</v>
+      </c>
+      <c r="J415">
+        <v>1</v>
+      </c>
+      <c r="K415">
+        <v>3.054381175561085</v>
+      </c>
+      <c r="L415">
+        <v>15.08</v>
+      </c>
+      <c r="M415">
+        <v>6</v>
+      </c>
+      <c r="N415">
+        <v>1</v>
+      </c>
+      <c r="O415">
+        <v>31.6505</v>
+      </c>
+      <c r="P415">
+        <v>90.63717067583048</v>
+      </c>
+      <c r="Q415">
+        <v>34.92</v>
+      </c>
+      <c r="R415">
+        <v>580.4557199999999</v>
+      </c>
+      <c r="S415">
+        <v>7.01152030536564</v>
+      </c>
+      <c r="T415">
+        <v>864.0800200000001</v>
+      </c>
+      <c r="U415">
+        <v>17</v>
+      </c>
+      <c r="V415">
+        <v>19</v>
+      </c>
+      <c r="W415">
+        <v>36</v>
+      </c>
+      <c r="X415">
+        <v>82</v>
+      </c>
+      <c r="Y415">
+        <v>17</v>
+      </c>
+      <c r="Z415">
+        <v>63</v>
+      </c>
+      <c r="AA415">
+        <v>19</v>
+      </c>
+      <c r="AB415">
+        <v>14</v>
+      </c>
+      <c r="AC415">
+        <v>4.9358</v>
+      </c>
+      <c r="AD415">
+        <v>-3.38437</v>
+      </c>
+      <c r="AE415">
+        <v>0</v>
+      </c>
+      <c r="AF415">
+        <v>657.3632</v>
+      </c>
+      <c r="AG415">
+        <v>0</v>
+      </c>
+      <c r="AH415">
+        <v>3</v>
+      </c>
+      <c r="AI415">
+        <v>1741.36716</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B416" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E416">
+        <v>82.786</v>
+      </c>
+      <c r="F416">
+        <v>7767.379999999999</v>
+      </c>
+      <c r="G416">
+        <v>93.82480129490493</v>
+      </c>
+      <c r="H416">
+        <v>339.54</v>
+      </c>
+      <c r="I416">
+        <v>0</v>
+      </c>
+      <c r="J416">
+        <v>0</v>
+      </c>
+      <c r="K416">
+        <v>4.101418114173894</v>
+      </c>
+      <c r="L416">
+        <v>0</v>
+      </c>
+      <c r="M416">
+        <v>5</v>
+      </c>
+      <c r="N416">
+        <v>0</v>
+      </c>
+      <c r="O416">
+        <v>28.80526</v>
+      </c>
+      <c r="P416">
+        <v>82.31955875628717</v>
+      </c>
+      <c r="Q416">
+        <v>34.992</v>
+      </c>
+      <c r="R416">
+        <v>624.69615</v>
+      </c>
+      <c r="S416">
+        <v>7.545915372164376</v>
+      </c>
+      <c r="T416">
+        <v>1262.95002</v>
+      </c>
+      <c r="U416">
+        <v>19</v>
+      </c>
+      <c r="V416">
+        <v>28</v>
+      </c>
+      <c r="W416">
+        <v>47</v>
+      </c>
+      <c r="X416">
+        <v>88</v>
+      </c>
+      <c r="Y416">
+        <v>19</v>
+      </c>
+      <c r="Z416">
+        <v>83</v>
+      </c>
+      <c r="AA416">
+        <v>28</v>
+      </c>
+      <c r="AB416">
+        <v>13</v>
+      </c>
+      <c r="AC416">
+        <v>4.30439</v>
+      </c>
+      <c r="AD416">
+        <v>-3.32813</v>
+      </c>
+      <c r="AE416">
+        <v>0</v>
+      </c>
+      <c r="AF416">
+        <v>652.4537899999999</v>
+      </c>
+      <c r="AG416">
+        <v>0</v>
+      </c>
+      <c r="AH416">
+        <v>3</v>
+      </c>
+      <c r="AI416">
+        <v>1874.08845</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B417" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E417">
+        <v>82.786</v>
+      </c>
+      <c r="F417">
+        <v>7873.41</v>
+      </c>
+      <c r="G417">
+        <v>95.10557340613147</v>
+      </c>
+      <c r="H417">
+        <v>287.23</v>
+      </c>
+      <c r="I417">
+        <v>0</v>
+      </c>
+      <c r="J417">
+        <v>0</v>
+      </c>
+      <c r="K417">
+        <v>3.469547991206242</v>
+      </c>
+      <c r="L417">
+        <v>0</v>
+      </c>
+      <c r="M417">
+        <v>3</v>
+      </c>
+      <c r="N417">
+        <v>0</v>
+      </c>
+      <c r="O417">
+        <v>26.06522</v>
+      </c>
+      <c r="P417">
+        <v>72.40338888888888</v>
+      </c>
+      <c r="Q417">
+        <v>36</v>
+      </c>
+      <c r="R417">
+        <v>814.24326</v>
+      </c>
+      <c r="S417">
+        <v>9.835518807527842</v>
+      </c>
+      <c r="T417">
+        <v>1073.38002</v>
+      </c>
+      <c r="U417">
+        <v>11</v>
+      </c>
+      <c r="V417">
+        <v>20</v>
+      </c>
+      <c r="W417">
+        <v>31</v>
+      </c>
+      <c r="X417">
+        <v>87</v>
+      </c>
+      <c r="Y417">
+        <v>11</v>
+      </c>
+      <c r="Z417">
+        <v>91</v>
+      </c>
+      <c r="AA417">
+        <v>20</v>
+      </c>
+      <c r="AB417">
+        <v>16</v>
+      </c>
+      <c r="AC417">
+        <v>3.40292</v>
+      </c>
+      <c r="AD417">
+        <v>-3.8247</v>
+      </c>
+      <c r="AE417">
+        <v>0</v>
+      </c>
+      <c r="AF417">
+        <v>1849.122</v>
+      </c>
+      <c r="AG417">
+        <v>0</v>
+      </c>
+      <c r="AH417">
+        <v>3</v>
+      </c>
+      <c r="AI417">
+        <v>2442.72978</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B418" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E418">
+        <v>82.786</v>
+      </c>
+      <c r="F418">
+        <v>6991.01</v>
+      </c>
+      <c r="G418">
+        <v>84.44676636146208</v>
+      </c>
+      <c r="H418">
+        <v>190.86</v>
+      </c>
+      <c r="I418">
+        <v>0</v>
+      </c>
+      <c r="J418">
+        <v>0</v>
+      </c>
+      <c r="K418">
+        <v>2.305462276230281</v>
+      </c>
+      <c r="L418">
+        <v>0</v>
+      </c>
+      <c r="M418">
+        <v>4</v>
+      </c>
+      <c r="N418">
+        <v>0</v>
+      </c>
+      <c r="O418">
+        <v>28.26051</v>
+      </c>
+      <c r="P418">
+        <v>83.15828036723163</v>
+      </c>
+      <c r="Q418">
+        <v>33.984</v>
+      </c>
+      <c r="R418">
+        <v>665.87757</v>
+      </c>
+      <c r="S418">
+        <v>8.043359626023724</v>
+      </c>
+      <c r="T418">
+        <v>928.80002</v>
+      </c>
+      <c r="U418">
+        <v>10</v>
+      </c>
+      <c r="V418">
+        <v>17</v>
+      </c>
+      <c r="W418">
+        <v>27</v>
+      </c>
+      <c r="X418">
+        <v>69</v>
+      </c>
+      <c r="Y418">
+        <v>10</v>
+      </c>
+      <c r="Z418">
+        <v>66</v>
+      </c>
+      <c r="AA418">
+        <v>17</v>
+      </c>
+      <c r="AB418">
+        <v>24</v>
+      </c>
+      <c r="AC418">
+        <v>3.6853</v>
+      </c>
+      <c r="AD418">
+        <v>-4.02804</v>
+      </c>
+      <c r="AE418">
+        <v>0</v>
+      </c>
+      <c r="AF418">
+        <v>652.3672</v>
+      </c>
+      <c r="AG418">
+        <v>0</v>
+      </c>
+      <c r="AH418">
+        <v>3</v>
+      </c>
+      <c r="AI418">
+        <v>1997.63271</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B419" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E419">
+        <v>82.786</v>
+      </c>
+      <c r="F419">
+        <v>6999.06</v>
+      </c>
+      <c r="G419">
+        <v>84.54400502500422</v>
+      </c>
+      <c r="H419">
+        <v>237.42</v>
+      </c>
+      <c r="I419">
+        <v>0</v>
+      </c>
+      <c r="J419">
+        <v>0</v>
+      </c>
+      <c r="K419">
+        <v>2.867876210953543</v>
+      </c>
+      <c r="L419">
+        <v>0</v>
+      </c>
+      <c r="M419">
+        <v>4</v>
+      </c>
+      <c r="N419">
+        <v>0</v>
+      </c>
+      <c r="O419">
+        <v>27.61028</v>
+      </c>
+      <c r="P419">
+        <v>83.63710166000243</v>
+      </c>
+      <c r="Q419">
+        <v>33.012</v>
+      </c>
+      <c r="R419">
+        <v>654.29008</v>
+      </c>
+      <c r="S419">
+        <v>7.903390428333293</v>
+      </c>
+      <c r="T419">
+        <v>1008.17</v>
+      </c>
+      <c r="U419">
+        <v>21</v>
+      </c>
+      <c r="V419">
+        <v>23</v>
+      </c>
+      <c r="W419">
+        <v>44</v>
+      </c>
+      <c r="X419">
+        <v>90</v>
+      </c>
+      <c r="Y419">
+        <v>21</v>
+      </c>
+      <c r="Z419">
+        <v>76</v>
+      </c>
+      <c r="AA419">
+        <v>23</v>
+      </c>
+      <c r="AB419">
+        <v>19</v>
+      </c>
+      <c r="AC419">
+        <v>4.8481</v>
+      </c>
+      <c r="AD419">
+        <v>-3.1952</v>
+      </c>
+      <c r="AE419">
+        <v>0</v>
+      </c>
+      <c r="AF419">
+        <v>619.77675</v>
+      </c>
+      <c r="AG419">
+        <v>0</v>
+      </c>
+      <c r="AH419">
+        <v>3</v>
+      </c>
+      <c r="AI419">
+        <v>1962.87024</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B420" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E420">
+        <v>82.786</v>
+      </c>
+      <c r="F420">
+        <v>7809.85</v>
+      </c>
+      <c r="G420">
+        <v>94.33781074094654</v>
+      </c>
+      <c r="H420">
+        <v>185.4</v>
+      </c>
+      <c r="I420">
+        <v>0</v>
+      </c>
+      <c r="J420">
+        <v>0</v>
+      </c>
+      <c r="K420">
+        <v>2.239509095740825</v>
+      </c>
+      <c r="L420">
+        <v>0</v>
+      </c>
+      <c r="M420">
+        <v>3</v>
+      </c>
+      <c r="N420">
+        <v>0</v>
+      </c>
+      <c r="O420">
+        <v>27.29713</v>
+      </c>
+      <c r="P420">
+        <v>85.29286964129484</v>
+      </c>
+      <c r="Q420">
+        <v>32.004</v>
+      </c>
+      <c r="R420">
+        <v>694.13471</v>
+      </c>
+      <c r="S420">
+        <v>8.384687145169474</v>
+      </c>
+      <c r="T420">
+        <v>974.62998</v>
+      </c>
+      <c r="U420">
+        <v>15</v>
+      </c>
+      <c r="V420">
+        <v>17</v>
+      </c>
+      <c r="W420">
+        <v>32</v>
+      </c>
+      <c r="X420">
+        <v>80</v>
+      </c>
+      <c r="Y420">
+        <v>15</v>
+      </c>
+      <c r="Z420">
+        <v>63</v>
+      </c>
+      <c r="AA420">
+        <v>17</v>
+      </c>
+      <c r="AB420">
+        <v>17</v>
+      </c>
+      <c r="AC420">
+        <v>4.27469</v>
+      </c>
+      <c r="AD420">
+        <v>-3.21629</v>
+      </c>
+      <c r="AE420">
+        <v>0</v>
+      </c>
+      <c r="AF420">
+        <v>633.3558</v>
+      </c>
+      <c r="AG420">
+        <v>0</v>
+      </c>
+      <c r="AH420">
+        <v>3</v>
+      </c>
+      <c r="AI420">
+        <v>2082.40413</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B421" s="2">
+        <v>46211</v>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Sesión 30</t>
+        </is>
+      </c>
+      <c r="E421">
+        <v>82.786</v>
+      </c>
+      <c r="F421">
+        <v>9508.84</v>
+      </c>
+      <c r="G421">
+        <v>114.8604836566569</v>
+      </c>
+      <c r="H421">
+        <v>248.76</v>
+      </c>
+      <c r="I421">
+        <v>0</v>
+      </c>
+      <c r="J421">
+        <v>0</v>
+      </c>
+      <c r="K421">
+        <v>3.004855893508564</v>
+      </c>
+      <c r="L421">
+        <v>19.21</v>
+      </c>
+      <c r="M421">
+        <v>5</v>
+      </c>
+      <c r="N421">
+        <v>1</v>
+      </c>
+      <c r="O421">
+        <v>31.76157</v>
+      </c>
+      <c r="P421">
+        <v>88.22658333333334</v>
+      </c>
+      <c r="Q421">
+        <v>36</v>
+      </c>
+      <c r="R421">
+        <v>947.21752</v>
+      </c>
+      <c r="S421">
+        <v>11.44175971782669</v>
+      </c>
+      <c r="T421">
+        <v>1400.37</v>
+      </c>
+      <c r="U421">
+        <v>18</v>
+      </c>
+      <c r="V421">
+        <v>28</v>
+      </c>
+      <c r="W421">
+        <v>46</v>
+      </c>
+      <c r="X421">
+        <v>102</v>
+      </c>
+      <c r="Y421">
+        <v>18</v>
+      </c>
+      <c r="Z421">
+        <v>119</v>
+      </c>
+      <c r="AA421">
+        <v>28</v>
+      </c>
+      <c r="AB421">
+        <v>16</v>
+      </c>
+      <c r="AC421">
+        <v>4.54711</v>
+      </c>
+      <c r="AD421">
+        <v>-4.96881</v>
+      </c>
+      <c r="AE421">
+        <v>0</v>
+      </c>
+      <c r="AF421">
+        <v>2243.716</v>
+      </c>
+      <c r="AG421">
+        <v>0</v>
+      </c>
+      <c r="AH421">
+        <v>3</v>
+      </c>
+      <c r="AI421">
+        <v>2841.65256</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-10
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI421"/>
+  <dimension ref="A1:AI441"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -47903,6 +47903,2266 @@
         <v>2841.65256</v>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B422" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E422">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F422">
+        <v>5580.96</v>
+      </c>
+      <c r="G422">
+        <v>45.23880032423669</v>
+      </c>
+      <c r="H422">
+        <v>61.11</v>
+      </c>
+      <c r="I422">
+        <v>0</v>
+      </c>
+      <c r="J422">
+        <v>0</v>
+      </c>
+      <c r="K422">
+        <v>0.4953526074034045</v>
+      </c>
+      <c r="L422">
+        <v>0</v>
+      </c>
+      <c r="M422">
+        <v>1</v>
+      </c>
+      <c r="N422">
+        <v>0</v>
+      </c>
+      <c r="O422">
+        <v>25.5592</v>
+      </c>
+      <c r="P422">
+        <v>78.97416882956372</v>
+      </c>
+      <c r="Q422">
+        <v>32.364</v>
+      </c>
+      <c r="R422">
+        <v>479.24548</v>
+      </c>
+      <c r="S422">
+        <v>3.884724236692786</v>
+      </c>
+      <c r="T422">
+        <v>523.58001</v>
+      </c>
+      <c r="U422">
+        <v>12</v>
+      </c>
+      <c r="V422">
+        <v>9</v>
+      </c>
+      <c r="W422">
+        <v>21</v>
+      </c>
+      <c r="X422">
+        <v>44</v>
+      </c>
+      <c r="Y422">
+        <v>12</v>
+      </c>
+      <c r="Z422">
+        <v>23</v>
+      </c>
+      <c r="AA422">
+        <v>9</v>
+      </c>
+      <c r="AB422">
+        <v>6</v>
+      </c>
+      <c r="AC422">
+        <v>3.78734</v>
+      </c>
+      <c r="AD422">
+        <v>-1.2089</v>
+      </c>
+      <c r="AE422">
+        <v>0</v>
+      </c>
+      <c r="AF422">
+        <v>438.5472</v>
+      </c>
+      <c r="AG422">
+        <v>0</v>
+      </c>
+      <c r="AH422">
+        <v>3</v>
+      </c>
+      <c r="AI422">
+        <v>1437.73644</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B423" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E423">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F423">
+        <v>5907.98</v>
+      </c>
+      <c r="G423">
+        <v>47.88959740610646</v>
+      </c>
+      <c r="H423">
+        <v>281.32</v>
+      </c>
+      <c r="I423">
+        <v>0</v>
+      </c>
+      <c r="J423">
+        <v>0</v>
+      </c>
+      <c r="K423">
+        <v>2.280356660362064</v>
+      </c>
+      <c r="L423">
+        <v>0</v>
+      </c>
+      <c r="M423">
+        <v>9</v>
+      </c>
+      <c r="N423">
+        <v>0</v>
+      </c>
+      <c r="O423">
+        <v>28.64146</v>
+      </c>
+      <c r="P423">
+        <v>79.55961111111111</v>
+      </c>
+      <c r="Q423">
+        <v>36</v>
+      </c>
+      <c r="R423">
+        <v>490.15112</v>
+      </c>
+      <c r="S423">
+        <v>3.973124452850581</v>
+      </c>
+      <c r="T423">
+        <v>862.80999</v>
+      </c>
+      <c r="U423">
+        <v>30</v>
+      </c>
+      <c r="V423">
+        <v>29</v>
+      </c>
+      <c r="W423">
+        <v>59</v>
+      </c>
+      <c r="X423">
+        <v>69</v>
+      </c>
+      <c r="Y423">
+        <v>30</v>
+      </c>
+      <c r="Z423">
+        <v>68</v>
+      </c>
+      <c r="AA423">
+        <v>29</v>
+      </c>
+      <c r="AB423">
+        <v>16</v>
+      </c>
+      <c r="AC423">
+        <v>4.71243</v>
+      </c>
+      <c r="AD423">
+        <v>-1.77719</v>
+      </c>
+      <c r="AE423">
+        <v>0</v>
+      </c>
+      <c r="AF423">
+        <v>1404.188</v>
+      </c>
+      <c r="AG423">
+        <v>0</v>
+      </c>
+      <c r="AH423">
+        <v>3</v>
+      </c>
+      <c r="AI423">
+        <v>1470.45336</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Alejandro Fernandez</t>
+        </is>
+      </c>
+      <c r="B424" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E424">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F424">
+        <v>6150.17</v>
+      </c>
+      <c r="G424">
+        <v>49.85276952175088</v>
+      </c>
+      <c r="H424">
+        <v>242.25</v>
+      </c>
+      <c r="I424">
+        <v>0</v>
+      </c>
+      <c r="J424">
+        <v>0</v>
+      </c>
+      <c r="K424">
+        <v>1.963658470683599</v>
+      </c>
+      <c r="L424">
+        <v>0</v>
+      </c>
+      <c r="M424">
+        <v>3</v>
+      </c>
+      <c r="N424">
+        <v>0</v>
+      </c>
+      <c r="O424">
+        <v>27.82173</v>
+      </c>
+      <c r="P424">
+        <v>77.28258333333333</v>
+      </c>
+      <c r="Q424">
+        <v>36</v>
+      </c>
+      <c r="R424">
+        <v>642.74341</v>
+      </c>
+      <c r="S424">
+        <v>5.210024939205621</v>
+      </c>
+      <c r="T424">
+        <v>1055.43003</v>
+      </c>
+      <c r="U424">
+        <v>46</v>
+      </c>
+      <c r="V424">
+        <v>22</v>
+      </c>
+      <c r="W424">
+        <v>68</v>
+      </c>
+      <c r="X424">
+        <v>101</v>
+      </c>
+      <c r="Y424">
+        <v>46</v>
+      </c>
+      <c r="Z424">
+        <v>74</v>
+      </c>
+      <c r="AA424">
+        <v>22</v>
+      </c>
+      <c r="AB424">
+        <v>28</v>
+      </c>
+      <c r="AC424">
+        <v>4.40108</v>
+      </c>
+      <c r="AD424">
+        <v>-2.17597</v>
+      </c>
+      <c r="AE424">
+        <v>0</v>
+      </c>
+      <c r="AF424">
+        <v>1476.812</v>
+      </c>
+      <c r="AG424">
+        <v>0</v>
+      </c>
+      <c r="AH424">
+        <v>3</v>
+      </c>
+      <c r="AI424">
+        <v>1928.23023</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B425" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E425">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F425">
+        <v>6197.879999999999</v>
+      </c>
+      <c r="G425">
+        <v>50.23950283707106</v>
+      </c>
+      <c r="H425">
+        <v>340.18</v>
+      </c>
+      <c r="I425">
+        <v>0</v>
+      </c>
+      <c r="J425">
+        <v>0</v>
+      </c>
+      <c r="K425">
+        <v>2.757470953796271</v>
+      </c>
+      <c r="L425">
+        <v>0</v>
+      </c>
+      <c r="M425">
+        <v>7</v>
+      </c>
+      <c r="N425">
+        <v>0</v>
+      </c>
+      <c r="O425">
+        <v>28.20053</v>
+      </c>
+      <c r="P425">
+        <v>87.03867283950618</v>
+      </c>
+      <c r="Q425">
+        <v>32.4</v>
+      </c>
+      <c r="R425">
+        <v>681.31408</v>
+      </c>
+      <c r="S425">
+        <v>5.522675601188868</v>
+      </c>
+      <c r="T425">
+        <v>1090.05002</v>
+      </c>
+      <c r="U425">
+        <v>43</v>
+      </c>
+      <c r="V425">
+        <v>15</v>
+      </c>
+      <c r="W425">
+        <v>58</v>
+      </c>
+      <c r="X425">
+        <v>88</v>
+      </c>
+      <c r="Y425">
+        <v>43</v>
+      </c>
+      <c r="Z425">
+        <v>61</v>
+      </c>
+      <c r="AA425">
+        <v>15</v>
+      </c>
+      <c r="AB425">
+        <v>17</v>
+      </c>
+      <c r="AC425">
+        <v>4.70311</v>
+      </c>
+      <c r="AD425">
+        <v>-1.75559</v>
+      </c>
+      <c r="AE425">
+        <v>0</v>
+      </c>
+      <c r="AF425">
+        <v>521.9263</v>
+      </c>
+      <c r="AG425">
+        <v>0</v>
+      </c>
+      <c r="AH425">
+        <v>3</v>
+      </c>
+      <c r="AI425">
+        <v>2043.94224</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B426" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E426">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F426">
+        <v>6193.6</v>
+      </c>
+      <c r="G426">
+        <v>50.20480951094299</v>
+      </c>
+      <c r="H426">
+        <v>311.51</v>
+      </c>
+      <c r="I426">
+        <v>0</v>
+      </c>
+      <c r="J426">
+        <v>0</v>
+      </c>
+      <c r="K426">
+        <v>2.525074304242097</v>
+      </c>
+      <c r="L426">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="M426">
+        <v>10</v>
+      </c>
+      <c r="N426">
+        <v>1</v>
+      </c>
+      <c r="O426">
+        <v>30.22088</v>
+      </c>
+      <c r="P426">
+        <v>84.96648672964463</v>
+      </c>
+      <c r="Q426">
+        <v>35.568</v>
+      </c>
+      <c r="R426">
+        <v>533.9412600000001</v>
+      </c>
+      <c r="S426">
+        <v>4.328083707106188</v>
+      </c>
+      <c r="T426">
+        <v>924.32999</v>
+      </c>
+      <c r="U426">
+        <v>36</v>
+      </c>
+      <c r="V426">
+        <v>14</v>
+      </c>
+      <c r="W426">
+        <v>50</v>
+      </c>
+      <c r="X426">
+        <v>79</v>
+      </c>
+      <c r="Y426">
+        <v>36</v>
+      </c>
+      <c r="Z426">
+        <v>52</v>
+      </c>
+      <c r="AA426">
+        <v>14</v>
+      </c>
+      <c r="AB426">
+        <v>13</v>
+      </c>
+      <c r="AC426">
+        <v>4.69057</v>
+      </c>
+      <c r="AD426">
+        <v>-1.56152</v>
+      </c>
+      <c r="AE426">
+        <v>0</v>
+      </c>
+      <c r="AF426">
+        <v>586.6712</v>
+      </c>
+      <c r="AG426">
+        <v>0</v>
+      </c>
+      <c r="AH426">
+        <v>3</v>
+      </c>
+      <c r="AI426">
+        <v>1601.82378</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B427" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E427">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F427">
+        <v>6282.73</v>
+      </c>
+      <c r="G427">
+        <v>50.9272899216428</v>
+      </c>
+      <c r="H427">
+        <v>291.07</v>
+      </c>
+      <c r="I427">
+        <v>0</v>
+      </c>
+      <c r="J427">
+        <v>0</v>
+      </c>
+      <c r="K427">
+        <v>2.359389354228587</v>
+      </c>
+      <c r="L427">
+        <v>0</v>
+      </c>
+      <c r="M427">
+        <v>5</v>
+      </c>
+      <c r="N427">
+        <v>0</v>
+      </c>
+      <c r="O427">
+        <v>29.24161</v>
+      </c>
+      <c r="P427">
+        <v>81.22669444444445</v>
+      </c>
+      <c r="Q427">
+        <v>36</v>
+      </c>
+      <c r="R427">
+        <v>645.53644</v>
+      </c>
+      <c r="S427">
+        <v>5.232665009456904</v>
+      </c>
+      <c r="T427">
+        <v>896.02001</v>
+      </c>
+      <c r="U427">
+        <v>27</v>
+      </c>
+      <c r="V427">
+        <v>13</v>
+      </c>
+      <c r="W427">
+        <v>40</v>
+      </c>
+      <c r="X427">
+        <v>76</v>
+      </c>
+      <c r="Y427">
+        <v>27</v>
+      </c>
+      <c r="Z427">
+        <v>44</v>
+      </c>
+      <c r="AA427">
+        <v>13</v>
+      </c>
+      <c r="AB427">
+        <v>5</v>
+      </c>
+      <c r="AC427">
+        <v>4.0966</v>
+      </c>
+      <c r="AD427">
+        <v>-1.56784</v>
+      </c>
+      <c r="AE427">
+        <v>0</v>
+      </c>
+      <c r="AF427">
+        <v>1447.478</v>
+      </c>
+      <c r="AG427">
+        <v>0</v>
+      </c>
+      <c r="AH427">
+        <v>3</v>
+      </c>
+      <c r="AI427">
+        <v>1936.60932</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B428" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E428">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F428">
+        <v>4768.24</v>
+      </c>
+      <c r="G428">
+        <v>38.65095920021616</v>
+      </c>
+      <c r="H428">
+        <v>181.63</v>
+      </c>
+      <c r="I428">
+        <v>0</v>
+      </c>
+      <c r="J428">
+        <v>0</v>
+      </c>
+      <c r="K428">
+        <v>1.47227776276682</v>
+      </c>
+      <c r="L428">
+        <v>0</v>
+      </c>
+      <c r="M428">
+        <v>3</v>
+      </c>
+      <c r="N428">
+        <v>0</v>
+      </c>
+      <c r="O428">
+        <v>26.58614</v>
+      </c>
+      <c r="P428">
+        <v>73.85038888888889</v>
+      </c>
+      <c r="Q428">
+        <v>36</v>
+      </c>
+      <c r="R428">
+        <v>426.80744</v>
+      </c>
+      <c r="S428">
+        <v>3.459665820048635</v>
+      </c>
+      <c r="T428">
+        <v>808.3</v>
+      </c>
+      <c r="U428">
+        <v>34</v>
+      </c>
+      <c r="V428">
+        <v>24</v>
+      </c>
+      <c r="W428">
+        <v>58</v>
+      </c>
+      <c r="X428">
+        <v>77</v>
+      </c>
+      <c r="Y428">
+        <v>34</v>
+      </c>
+      <c r="Z428">
+        <v>60</v>
+      </c>
+      <c r="AA428">
+        <v>24</v>
+      </c>
+      <c r="AB428">
+        <v>12</v>
+      </c>
+      <c r="AC428">
+        <v>4.4966</v>
+      </c>
+      <c r="AD428">
+        <v>0</v>
+      </c>
+      <c r="AE428">
+        <v>0</v>
+      </c>
+      <c r="AF428">
+        <v>408.1903</v>
+      </c>
+      <c r="AG428">
+        <v>0</v>
+      </c>
+      <c r="AH428">
+        <v>3</v>
+      </c>
+      <c r="AI428">
+        <v>1280.42232</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B429" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E429">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F429">
+        <v>5782.9</v>
+      </c>
+      <c r="G429">
+        <v>46.87570926776547</v>
+      </c>
+      <c r="H429">
+        <v>291.77</v>
+      </c>
+      <c r="I429">
+        <v>0</v>
+      </c>
+      <c r="J429">
+        <v>0</v>
+      </c>
+      <c r="K429">
+        <v>2.365063496352337</v>
+      </c>
+      <c r="L429">
+        <v>0</v>
+      </c>
+      <c r="M429">
+        <v>2</v>
+      </c>
+      <c r="N429">
+        <v>0</v>
+      </c>
+      <c r="O429">
+        <v>25.68151</v>
+      </c>
+      <c r="P429">
+        <v>80.2446881639795</v>
+      </c>
+      <c r="Q429">
+        <v>32.004</v>
+      </c>
+      <c r="R429">
+        <v>566.64255</v>
+      </c>
+      <c r="S429">
+        <v>4.593157660091867</v>
+      </c>
+      <c r="T429">
+        <v>826.8399900000001</v>
+      </c>
+      <c r="U429">
+        <v>21</v>
+      </c>
+      <c r="V429">
+        <v>18</v>
+      </c>
+      <c r="W429">
+        <v>39</v>
+      </c>
+      <c r="X429">
+        <v>63</v>
+      </c>
+      <c r="Y429">
+        <v>21</v>
+      </c>
+      <c r="Z429">
+        <v>55</v>
+      </c>
+      <c r="AA429">
+        <v>18</v>
+      </c>
+      <c r="AB429">
+        <v>20</v>
+      </c>
+      <c r="AC429">
+        <v>4.26801</v>
+      </c>
+      <c r="AD429">
+        <v>-1.67595</v>
+      </c>
+      <c r="AE429">
+        <v>0</v>
+      </c>
+      <c r="AF429">
+        <v>401.5782</v>
+      </c>
+      <c r="AG429">
+        <v>0</v>
+      </c>
+      <c r="AH429">
+        <v>3</v>
+      </c>
+      <c r="AI429">
+        <v>1699.92765</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B430" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E430">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F430">
+        <v>5823</v>
+      </c>
+      <c r="G430">
+        <v>47.20075655228317</v>
+      </c>
+      <c r="H430">
+        <v>219.36</v>
+      </c>
+      <c r="I430">
+        <v>0</v>
+      </c>
+      <c r="J430">
+        <v>0</v>
+      </c>
+      <c r="K430">
+        <v>1.778114023236963</v>
+      </c>
+      <c r="L430">
+        <v>1.6</v>
+      </c>
+      <c r="M430">
+        <v>4</v>
+      </c>
+      <c r="N430">
+        <v>0</v>
+      </c>
+      <c r="O430">
+        <v>29.98446</v>
+      </c>
+      <c r="P430">
+        <v>88.60656028368793</v>
+      </c>
+      <c r="Q430">
+        <v>33.84</v>
+      </c>
+      <c r="R430">
+        <v>537.22745</v>
+      </c>
+      <c r="S430">
+        <v>4.354721291542826</v>
+      </c>
+      <c r="T430">
+        <v>805.63001</v>
+      </c>
+      <c r="U430">
+        <v>36</v>
+      </c>
+      <c r="V430">
+        <v>17</v>
+      </c>
+      <c r="W430">
+        <v>53</v>
+      </c>
+      <c r="X430">
+        <v>84</v>
+      </c>
+      <c r="Y430">
+        <v>36</v>
+      </c>
+      <c r="Z430">
+        <v>52</v>
+      </c>
+      <c r="AA430">
+        <v>17</v>
+      </c>
+      <c r="AB430">
+        <v>22</v>
+      </c>
+      <c r="AC430">
+        <v>4.33037</v>
+      </c>
+      <c r="AD430">
+        <v>-1.34927</v>
+      </c>
+      <c r="AE430">
+        <v>0</v>
+      </c>
+      <c r="AF430">
+        <v>478.184</v>
+      </c>
+      <c r="AG430">
+        <v>0</v>
+      </c>
+      <c r="AH430">
+        <v>3</v>
+      </c>
+      <c r="AI430">
+        <v>1611.68235</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B431" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E431">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F431">
+        <v>5598.25</v>
+      </c>
+      <c r="G431">
+        <v>45.37895163469333</v>
+      </c>
+      <c r="H431">
+        <v>211.06</v>
+      </c>
+      <c r="I431">
+        <v>0</v>
+      </c>
+      <c r="J431">
+        <v>0</v>
+      </c>
+      <c r="K431">
+        <v>1.710834909483924</v>
+      </c>
+      <c r="L431">
+        <v>0</v>
+      </c>
+      <c r="M431">
+        <v>3</v>
+      </c>
+      <c r="N431">
+        <v>0</v>
+      </c>
+      <c r="O431">
+        <v>27.82254</v>
+      </c>
+      <c r="P431">
+        <v>82.56926638176638</v>
+      </c>
+      <c r="Q431">
+        <v>33.696</v>
+      </c>
+      <c r="R431">
+        <v>525.90128</v>
+      </c>
+      <c r="S431">
+        <v>4.262912293974602</v>
+      </c>
+      <c r="T431">
+        <v>813.8000000000001</v>
+      </c>
+      <c r="U431">
+        <v>33</v>
+      </c>
+      <c r="V431">
+        <v>17</v>
+      </c>
+      <c r="W431">
+        <v>50</v>
+      </c>
+      <c r="X431">
+        <v>68</v>
+      </c>
+      <c r="Y431">
+        <v>33</v>
+      </c>
+      <c r="Z431">
+        <v>62</v>
+      </c>
+      <c r="AA431">
+        <v>17</v>
+      </c>
+      <c r="AB431">
+        <v>15</v>
+      </c>
+      <c r="AC431">
+        <v>4.23886</v>
+      </c>
+      <c r="AD431">
+        <v>-1.74513</v>
+      </c>
+      <c r="AE431">
+        <v>0</v>
+      </c>
+      <c r="AF431">
+        <v>523.7848</v>
+      </c>
+      <c r="AG431">
+        <v>0</v>
+      </c>
+      <c r="AH431">
+        <v>3</v>
+      </c>
+      <c r="AI431">
+        <v>1577.70384</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B432" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E432">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F432">
+        <v>7134.95</v>
+      </c>
+      <c r="G432">
+        <v>57.83531477978925</v>
+      </c>
+      <c r="H432">
+        <v>411.93</v>
+      </c>
+      <c r="I432">
+        <v>0</v>
+      </c>
+      <c r="J432">
+        <v>0</v>
+      </c>
+      <c r="K432">
+        <v>3.339070521480681</v>
+      </c>
+      <c r="L432">
+        <v>8.84</v>
+      </c>
+      <c r="M432">
+        <v>11</v>
+      </c>
+      <c r="N432">
+        <v>1</v>
+      </c>
+      <c r="O432">
+        <v>30.46114</v>
+      </c>
+      <c r="P432">
+        <v>87.05172610882488</v>
+      </c>
+      <c r="Q432">
+        <v>34.992</v>
+      </c>
+      <c r="R432">
+        <v>629.63208</v>
+      </c>
+      <c r="S432">
+        <v>5.103745582275061</v>
+      </c>
+      <c r="T432">
+        <v>971.12999</v>
+      </c>
+      <c r="U432">
+        <v>33</v>
+      </c>
+      <c r="V432">
+        <v>13</v>
+      </c>
+      <c r="W432">
+        <v>46</v>
+      </c>
+      <c r="X432">
+        <v>79</v>
+      </c>
+      <c r="Y432">
+        <v>33</v>
+      </c>
+      <c r="Z432">
+        <v>52</v>
+      </c>
+      <c r="AA432">
+        <v>13</v>
+      </c>
+      <c r="AB432">
+        <v>15</v>
+      </c>
+      <c r="AC432">
+        <v>3.99508</v>
+      </c>
+      <c r="AD432">
+        <v>-1.14086</v>
+      </c>
+      <c r="AE432">
+        <v>0</v>
+      </c>
+      <c r="AF432">
+        <v>563.09727</v>
+      </c>
+      <c r="AG432">
+        <v>0</v>
+      </c>
+      <c r="AH432">
+        <v>3</v>
+      </c>
+      <c r="AI432">
+        <v>1888.89624</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B433" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E433">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F433">
+        <v>5655.05</v>
+      </c>
+      <c r="G433">
+        <v>45.83936773844907</v>
+      </c>
+      <c r="H433">
+        <v>149.9</v>
+      </c>
+      <c r="I433">
+        <v>0</v>
+      </c>
+      <c r="J433">
+        <v>0</v>
+      </c>
+      <c r="K433">
+        <v>1.215077006214536</v>
+      </c>
+      <c r="L433">
+        <v>0</v>
+      </c>
+      <c r="M433">
+        <v>2</v>
+      </c>
+      <c r="N433">
+        <v>0</v>
+      </c>
+      <c r="O433">
+        <v>27.81074</v>
+      </c>
+      <c r="P433">
+        <v>79.64129438717067</v>
+      </c>
+      <c r="Q433">
+        <v>34.92</v>
+      </c>
+      <c r="R433">
+        <v>510.10056</v>
+      </c>
+      <c r="S433">
+        <v>4.134832964063767</v>
+      </c>
+      <c r="T433">
+        <v>674.7700100000001</v>
+      </c>
+      <c r="U433">
+        <v>26</v>
+      </c>
+      <c r="V433">
+        <v>12</v>
+      </c>
+      <c r="W433">
+        <v>38</v>
+      </c>
+      <c r="X433">
+        <v>60</v>
+      </c>
+      <c r="Y433">
+        <v>26</v>
+      </c>
+      <c r="Z433">
+        <v>49</v>
+      </c>
+      <c r="AA433">
+        <v>12</v>
+      </c>
+      <c r="AB433">
+        <v>16</v>
+      </c>
+      <c r="AC433">
+        <v>4.2106</v>
+      </c>
+      <c r="AD433">
+        <v>-1.79571</v>
+      </c>
+      <c r="AE433">
+        <v>0</v>
+      </c>
+      <c r="AF433">
+        <v>518.4616</v>
+      </c>
+      <c r="AG433">
+        <v>0</v>
+      </c>
+      <c r="AH433">
+        <v>3</v>
+      </c>
+      <c r="AI433">
+        <v>1530.30168</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B434" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E434">
+        <v>85.93333333333334</v>
+      </c>
+      <c r="F434">
+        <v>3225.13</v>
+      </c>
+      <c r="G434">
+        <v>37.53060512024825</v>
+      </c>
+      <c r="H434">
+        <v>41.62</v>
+      </c>
+      <c r="I434">
+        <v>0</v>
+      </c>
+      <c r="J434">
+        <v>0</v>
+      </c>
+      <c r="K434">
+        <v>0.4843289371605896</v>
+      </c>
+      <c r="L434">
+        <v>0</v>
+      </c>
+      <c r="M434">
+        <v>1</v>
+      </c>
+      <c r="N434">
+        <v>0</v>
+      </c>
+      <c r="O434">
+        <v>26.21391</v>
+      </c>
+      <c r="P434">
+        <v>74.91400891632374</v>
+      </c>
+      <c r="Q434">
+        <v>34.992</v>
+      </c>
+      <c r="R434">
+        <v>296.05225</v>
+      </c>
+      <c r="S434">
+        <v>3.445138673390225</v>
+      </c>
+      <c r="T434">
+        <v>455.29001</v>
+      </c>
+      <c r="U434">
+        <v>27</v>
+      </c>
+      <c r="V434">
+        <v>11</v>
+      </c>
+      <c r="W434">
+        <v>38</v>
+      </c>
+      <c r="X434">
+        <v>57</v>
+      </c>
+      <c r="Y434">
+        <v>27</v>
+      </c>
+      <c r="Z434">
+        <v>40</v>
+      </c>
+      <c r="AA434">
+        <v>11</v>
+      </c>
+      <c r="AB434">
+        <v>23</v>
+      </c>
+      <c r="AC434">
+        <v>4.73041</v>
+      </c>
+      <c r="AD434">
+        <v>-1.8952</v>
+      </c>
+      <c r="AE434">
+        <v>0</v>
+      </c>
+      <c r="AF434">
+        <v>277.2621</v>
+      </c>
+      <c r="AG434">
+        <v>0</v>
+      </c>
+      <c r="AH434">
+        <v>3</v>
+      </c>
+      <c r="AI434">
+        <v>888.1567500000001</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B435" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E435">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F435">
+        <v>5665.110000000001</v>
+      </c>
+      <c r="G435">
+        <v>45.92091326668469</v>
+      </c>
+      <c r="H435">
+        <v>71.28999999999999</v>
+      </c>
+      <c r="I435">
+        <v>0</v>
+      </c>
+      <c r="J435">
+        <v>0</v>
+      </c>
+      <c r="K435">
+        <v>0.5778708457173737</v>
+      </c>
+      <c r="L435">
+        <v>0</v>
+      </c>
+      <c r="M435">
+        <v>1</v>
+      </c>
+      <c r="N435">
+        <v>0</v>
+      </c>
+      <c r="O435">
+        <v>26.40295</v>
+      </c>
+      <c r="P435">
+        <v>73.34152777777778</v>
+      </c>
+      <c r="Q435">
+        <v>36</v>
+      </c>
+      <c r="R435">
+        <v>572.25035</v>
+      </c>
+      <c r="S435">
+        <v>4.638614023236963</v>
+      </c>
+      <c r="T435">
+        <v>741.88</v>
+      </c>
+      <c r="U435">
+        <v>29</v>
+      </c>
+      <c r="V435">
+        <v>22</v>
+      </c>
+      <c r="W435">
+        <v>51</v>
+      </c>
+      <c r="X435">
+        <v>75</v>
+      </c>
+      <c r="Y435">
+        <v>29</v>
+      </c>
+      <c r="Z435">
+        <v>59</v>
+      </c>
+      <c r="AA435">
+        <v>22</v>
+      </c>
+      <c r="AB435">
+        <v>22</v>
+      </c>
+      <c r="AC435">
+        <v>4.28476</v>
+      </c>
+      <c r="AD435">
+        <v>-1.62042</v>
+      </c>
+      <c r="AE435">
+        <v>0</v>
+      </c>
+      <c r="AF435">
+        <v>1327.894</v>
+      </c>
+      <c r="AG435">
+        <v>0</v>
+      </c>
+      <c r="AH435">
+        <v>3</v>
+      </c>
+      <c r="AI435">
+        <v>1716.75105</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B436" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E436">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F436">
+        <v>5002.22</v>
+      </c>
+      <c r="G436">
+        <v>40.54758173466631</v>
+      </c>
+      <c r="H436">
+        <v>52.90000000000001</v>
+      </c>
+      <c r="I436">
+        <v>0</v>
+      </c>
+      <c r="J436">
+        <v>0</v>
+      </c>
+      <c r="K436">
+        <v>0.4288030262091327</v>
+      </c>
+      <c r="L436">
+        <v>0</v>
+      </c>
+      <c r="M436">
+        <v>1</v>
+      </c>
+      <c r="N436">
+        <v>0</v>
+      </c>
+      <c r="O436">
+        <v>25.60969</v>
+      </c>
+      <c r="P436">
+        <v>75.35808027306967</v>
+      </c>
+      <c r="Q436">
+        <v>33.984</v>
+      </c>
+      <c r="R436">
+        <v>515.9618400000001</v>
+      </c>
+      <c r="S436">
+        <v>4.182344015131046</v>
+      </c>
+      <c r="T436">
+        <v>540.5</v>
+      </c>
+      <c r="U436">
+        <v>17</v>
+      </c>
+      <c r="V436">
+        <v>11</v>
+      </c>
+      <c r="W436">
+        <v>28</v>
+      </c>
+      <c r="X436">
+        <v>56</v>
+      </c>
+      <c r="Y436">
+        <v>17</v>
+      </c>
+      <c r="Z436">
+        <v>43</v>
+      </c>
+      <c r="AA436">
+        <v>11</v>
+      </c>
+      <c r="AB436">
+        <v>16</v>
+      </c>
+      <c r="AC436">
+        <v>3.51474</v>
+      </c>
+      <c r="AD436">
+        <v>-0.94059</v>
+      </c>
+      <c r="AE436">
+        <v>0</v>
+      </c>
+      <c r="AF436">
+        <v>457.328</v>
+      </c>
+      <c r="AG436">
+        <v>0</v>
+      </c>
+      <c r="AH436">
+        <v>3</v>
+      </c>
+      <c r="AI436">
+        <v>1547.88552</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B437" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E437">
+        <v>85.93333333333334</v>
+      </c>
+      <c r="F437">
+        <v>4769.150000000001</v>
+      </c>
+      <c r="G437">
+        <v>55.49825446082234</v>
+      </c>
+      <c r="H437">
+        <v>144.47</v>
+      </c>
+      <c r="I437">
+        <v>0</v>
+      </c>
+      <c r="J437">
+        <v>0</v>
+      </c>
+      <c r="K437">
+        <v>1.681186966640807</v>
+      </c>
+      <c r="L437">
+        <v>0</v>
+      </c>
+      <c r="M437">
+        <v>0</v>
+      </c>
+      <c r="N437">
+        <v>0</v>
+      </c>
+      <c r="O437">
+        <v>24.98327</v>
+      </c>
+      <c r="P437">
+        <v>71.39709076360312</v>
+      </c>
+      <c r="Q437">
+        <v>34.992</v>
+      </c>
+      <c r="R437">
+        <v>433.02675</v>
+      </c>
+      <c r="S437">
+        <v>5.039101047323506</v>
+      </c>
+      <c r="T437">
+        <v>989.87999</v>
+      </c>
+      <c r="U437">
+        <v>33</v>
+      </c>
+      <c r="V437">
+        <v>20</v>
+      </c>
+      <c r="W437">
+        <v>53</v>
+      </c>
+      <c r="X437">
+        <v>92</v>
+      </c>
+      <c r="Y437">
+        <v>33</v>
+      </c>
+      <c r="Z437">
+        <v>62</v>
+      </c>
+      <c r="AA437">
+        <v>20</v>
+      </c>
+      <c r="AB437">
+        <v>11</v>
+      </c>
+      <c r="AC437">
+        <v>4.6514</v>
+      </c>
+      <c r="AD437">
+        <v>-2.61051</v>
+      </c>
+      <c r="AE437">
+        <v>0</v>
+      </c>
+      <c r="AF437">
+        <v>459.5616</v>
+      </c>
+      <c r="AG437">
+        <v>0</v>
+      </c>
+      <c r="AH437">
+        <v>3</v>
+      </c>
+      <c r="AI437">
+        <v>1299.08025</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B438" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E438">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F438">
+        <v>5505.39</v>
+      </c>
+      <c r="G438">
+        <v>44.62623615239125</v>
+      </c>
+      <c r="H438">
+        <v>96.39</v>
+      </c>
+      <c r="I438">
+        <v>0</v>
+      </c>
+      <c r="J438">
+        <v>0</v>
+      </c>
+      <c r="K438">
+        <v>0.7813293704404215</v>
+      </c>
+      <c r="L438">
+        <v>0</v>
+      </c>
+      <c r="M438">
+        <v>0</v>
+      </c>
+      <c r="N438">
+        <v>0</v>
+      </c>
+      <c r="O438">
+        <v>24.99156</v>
+      </c>
+      <c r="P438">
+        <v>75.70447110141767</v>
+      </c>
+      <c r="Q438">
+        <v>33.012</v>
+      </c>
+      <c r="R438">
+        <v>534.3320199999999</v>
+      </c>
+      <c r="S438">
+        <v>4.331251175358011</v>
+      </c>
+      <c r="T438">
+        <v>704.64001</v>
+      </c>
+      <c r="U438">
+        <v>30</v>
+      </c>
+      <c r="V438">
+        <v>16</v>
+      </c>
+      <c r="W438">
+        <v>46</v>
+      </c>
+      <c r="X438">
+        <v>78</v>
+      </c>
+      <c r="Y438">
+        <v>30</v>
+      </c>
+      <c r="Z438">
+        <v>53</v>
+      </c>
+      <c r="AA438">
+        <v>16</v>
+      </c>
+      <c r="AB438">
+        <v>25</v>
+      </c>
+      <c r="AC438">
+        <v>4.14873</v>
+      </c>
+      <c r="AD438">
+        <v>-1.26115</v>
+      </c>
+      <c r="AE438">
+        <v>0</v>
+      </c>
+      <c r="AF438">
+        <v>478.6935</v>
+      </c>
+      <c r="AG438">
+        <v>0</v>
+      </c>
+      <c r="AH438">
+        <v>3</v>
+      </c>
+      <c r="AI438">
+        <v>1602.99606</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B439" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E439">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F439">
+        <v>5641.58</v>
+      </c>
+      <c r="G439">
+        <v>45.73018103215347</v>
+      </c>
+      <c r="H439">
+        <v>125.81</v>
+      </c>
+      <c r="I439">
+        <v>0</v>
+      </c>
+      <c r="J439">
+        <v>0</v>
+      </c>
+      <c r="K439">
+        <v>1.019805457984329</v>
+      </c>
+      <c r="L439">
+        <v>0</v>
+      </c>
+      <c r="M439">
+        <v>2</v>
+      </c>
+      <c r="N439">
+        <v>0</v>
+      </c>
+      <c r="O439">
+        <v>28.04717</v>
+      </c>
+      <c r="P439">
+        <v>87.63645169353832</v>
+      </c>
+      <c r="Q439">
+        <v>32.004</v>
+      </c>
+      <c r="R439">
+        <v>455.97528</v>
+      </c>
+      <c r="S439">
+        <v>3.696097919481221</v>
+      </c>
+      <c r="T439">
+        <v>632.5599999999999</v>
+      </c>
+      <c r="U439">
+        <v>23</v>
+      </c>
+      <c r="V439">
+        <v>11</v>
+      </c>
+      <c r="W439">
+        <v>34</v>
+      </c>
+      <c r="X439">
+        <v>63</v>
+      </c>
+      <c r="Y439">
+        <v>23</v>
+      </c>
+      <c r="Z439">
+        <v>40</v>
+      </c>
+      <c r="AA439">
+        <v>11</v>
+      </c>
+      <c r="AB439">
+        <v>15</v>
+      </c>
+      <c r="AC439">
+        <v>4.19305</v>
+      </c>
+      <c r="AD439">
+        <v>-2.12339</v>
+      </c>
+      <c r="AE439">
+        <v>0</v>
+      </c>
+      <c r="AF439">
+        <v>448.6265</v>
+      </c>
+      <c r="AG439">
+        <v>0</v>
+      </c>
+      <c r="AH439">
+        <v>3</v>
+      </c>
+      <c r="AI439">
+        <v>1367.92584</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B440" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E440">
+        <v>123.3666666666667</v>
+      </c>
+      <c r="F440">
+        <v>6301.18</v>
+      </c>
+      <c r="G440">
+        <v>51.07684409619022</v>
+      </c>
+      <c r="H440">
+        <v>90.84</v>
+      </c>
+      <c r="I440">
+        <v>0</v>
+      </c>
+      <c r="J440">
+        <v>0</v>
+      </c>
+      <c r="K440">
+        <v>0.7363415293164011</v>
+      </c>
+      <c r="L440">
+        <v>0</v>
+      </c>
+      <c r="M440">
+        <v>2</v>
+      </c>
+      <c r="N440">
+        <v>0</v>
+      </c>
+      <c r="O440">
+        <v>28.90491</v>
+      </c>
+      <c r="P440">
+        <v>80.29141666666668</v>
+      </c>
+      <c r="Q440">
+        <v>36</v>
+      </c>
+      <c r="R440">
+        <v>630.8764200000001</v>
+      </c>
+      <c r="S440">
+        <v>5.113832099432586</v>
+      </c>
+      <c r="T440">
+        <v>643.67001</v>
+      </c>
+      <c r="U440">
+        <v>24</v>
+      </c>
+      <c r="V440">
+        <v>15</v>
+      </c>
+      <c r="W440">
+        <v>39</v>
+      </c>
+      <c r="X440">
+        <v>64</v>
+      </c>
+      <c r="Y440">
+        <v>24</v>
+      </c>
+      <c r="Z440">
+        <v>49</v>
+      </c>
+      <c r="AA440">
+        <v>15</v>
+      </c>
+      <c r="AB440">
+        <v>22</v>
+      </c>
+      <c r="AC440">
+        <v>4.38149</v>
+      </c>
+      <c r="AD440">
+        <v>-2.24125</v>
+      </c>
+      <c r="AE440">
+        <v>0</v>
+      </c>
+      <c r="AF440">
+        <v>1442.962</v>
+      </c>
+      <c r="AG440">
+        <v>0</v>
+      </c>
+      <c r="AH440">
+        <v>3</v>
+      </c>
+      <c r="AI440">
+        <v>1892.62926</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Thiago Espinosa</t>
+        </is>
+      </c>
+      <c r="B441" s="2">
+        <v>46212</v>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Sesion 31</t>
+        </is>
+      </c>
+      <c r="E441">
+        <v>85.93333333333334</v>
+      </c>
+      <c r="F441">
+        <v>3312.579999999999</v>
+      </c>
+      <c r="G441">
+        <v>38.54825446082233</v>
+      </c>
+      <c r="H441">
+        <v>86.41</v>
+      </c>
+      <c r="I441">
+        <v>0</v>
+      </c>
+      <c r="J441">
+        <v>0</v>
+      </c>
+      <c r="K441">
+        <v>1.005546935608999</v>
+      </c>
+      <c r="L441">
+        <v>0</v>
+      </c>
+      <c r="M441">
+        <v>1</v>
+      </c>
+      <c r="N441">
+        <v>0</v>
+      </c>
+      <c r="O441">
+        <v>27.63235</v>
+      </c>
+      <c r="P441">
+        <v>76.75652777777778</v>
+      </c>
+      <c r="Q441">
+        <v>36</v>
+      </c>
+      <c r="R441">
+        <v>370.86511</v>
+      </c>
+      <c r="S441">
+        <v>4.31573052754073</v>
+      </c>
+      <c r="T441">
+        <v>449.33999</v>
+      </c>
+      <c r="U441">
+        <v>32</v>
+      </c>
+      <c r="V441">
+        <v>18</v>
+      </c>
+      <c r="W441">
+        <v>50</v>
+      </c>
+      <c r="X441">
+        <v>57</v>
+      </c>
+      <c r="Y441">
+        <v>32</v>
+      </c>
+      <c r="Z441">
+        <v>44</v>
+      </c>
+      <c r="AA441">
+        <v>18</v>
+      </c>
+      <c r="AB441">
+        <v>22</v>
+      </c>
+      <c r="AC441">
+        <v>4.86662</v>
+      </c>
+      <c r="AD441">
+        <v>-1.63158</v>
+      </c>
+      <c r="AE441">
+        <v>0</v>
+      </c>
+      <c r="AF441">
+        <v>282.2232</v>
+      </c>
+      <c r="AG441">
+        <v>0</v>
+      </c>
+      <c r="AH441">
+        <v>3</v>
+      </c>
+      <c r="AI441">
+        <v>1112.59533</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-11
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI441"/>
+  <dimension ref="A1:AI458"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -41252,17 +41252,17 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E363">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F363">
-        <v>5315.2</v>
+        <v>2877.2</v>
       </c>
       <c r="G363">
-        <v>41.46021840873635</v>
+        <v>41.27977044476327</v>
       </c>
       <c r="H363">
         <v>0</v>
@@ -41295,37 +41295,37 @@
         <v>32.364</v>
       </c>
       <c r="R363">
-        <v>597.84475</v>
+        <v>318.02921</v>
       </c>
       <c r="S363">
-        <v>4.663375585023402</v>
+        <v>4.562829411764707</v>
       </c>
       <c r="T363">
-        <v>646.17998</v>
+        <v>354.45999</v>
       </c>
       <c r="U363">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="V363">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="W363">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="X363">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="Y363">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="Z363">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="AA363">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="AB363">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="AC363">
         <v>3.49302</v>
@@ -41337,7 +41337,7 @@
         <v>0</v>
       </c>
       <c r="AF363">
-        <v>447.0529</v>
+        <v>241.5084</v>
       </c>
       <c r="AG363">
         <v>0</v>
@@ -41346,7 +41346,7 @@
         <v>3</v>
       </c>
       <c r="AI363">
-        <v>1793.53425</v>
+        <v>954.0876300000001</v>
       </c>
     </row>
     <row r="364">
@@ -41365,20 +41365,20 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E364">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F364">
-        <v>5672.09</v>
+        <v>3258.73</v>
       </c>
       <c r="G364">
-        <v>44.24407176287052</v>
+        <v>46.75365853658536</v>
       </c>
       <c r="H364">
-        <v>1.9</v>
+        <v>0.95</v>
       </c>
       <c r="I364">
         <v>0</v>
@@ -41387,7 +41387,7 @@
         <v>0</v>
       </c>
       <c r="K364">
-        <v>0.01482059282371295</v>
+        <v>0.01362984218077475</v>
       </c>
       <c r="L364">
         <v>0</v>
@@ -41408,37 +41408,37 @@
         <v>32.4</v>
       </c>
       <c r="R364">
-        <v>838.4855799999999</v>
+        <v>460.20196</v>
       </c>
       <c r="S364">
-        <v>6.540449141965679</v>
+        <v>6.602610616929698</v>
       </c>
       <c r="T364">
-        <v>1037.39</v>
+        <v>562.02</v>
       </c>
       <c r="U364">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="V364">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="W364">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="X364">
-        <v>206</v>
+        <v>106</v>
       </c>
       <c r="Y364">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="Z364">
-        <v>152</v>
+        <v>78</v>
       </c>
       <c r="AA364">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="AB364">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="AC364">
         <v>3.90562</v>
@@ -41450,7 +41450,7 @@
         <v>0</v>
       </c>
       <c r="AF364">
-        <v>511.7238</v>
+        <v>289.2974</v>
       </c>
       <c r="AG364">
         <v>0</v>
@@ -41459,7 +41459,7 @@
         <v>3</v>
       </c>
       <c r="AI364">
-        <v>2515.45674</v>
+        <v>1380.60588</v>
       </c>
     </row>
     <row r="365">
@@ -41478,17 +41478,17 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E365">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F365">
-        <v>5096.36</v>
+        <v>2776.56</v>
       </c>
       <c r="G365">
-        <v>39.75319812792512</v>
+        <v>39.83586800573888</v>
       </c>
       <c r="H365">
         <v>17.52</v>
@@ -41500,7 +41500,7 @@
         <v>0</v>
       </c>
       <c r="K365">
-        <v>0.1366614664586583</v>
+        <v>0.2513629842180775</v>
       </c>
       <c r="L365">
         <v>0</v>
@@ -41521,37 +41521,37 @@
         <v>33.984</v>
       </c>
       <c r="R365">
-        <v>753.9197799999999</v>
+        <v>396.32672</v>
       </c>
       <c r="S365">
-        <v>5.880809516380656</v>
+        <v>5.68617962697274</v>
       </c>
       <c r="T365">
-        <v>427.12</v>
+        <v>245.6</v>
       </c>
       <c r="U365">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="V365">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="W365">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="X365">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="Y365">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="Z365">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="AA365">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AB365">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="AC365">
         <v>3.45041</v>
@@ -41563,7 +41563,7 @@
         <v>0</v>
       </c>
       <c r="AF365">
-        <v>472.4936</v>
+        <v>258.1776</v>
       </c>
       <c r="AG365">
         <v>0</v>
@@ -41572,7 +41572,7 @@
         <v>3</v>
       </c>
       <c r="AI365">
-        <v>2261.75934</v>
+        <v>1188.98016</v>
       </c>
     </row>
     <row r="366">
@@ -41591,17 +41591,17 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E366">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F366">
-        <v>6125.200000000001</v>
+        <v>3262.38</v>
       </c>
       <c r="G366">
-        <v>47.77847113884556</v>
+        <v>46.80602582496412</v>
       </c>
       <c r="H366">
         <v>0</v>
@@ -41634,37 +41634,37 @@
         <v>35.568</v>
       </c>
       <c r="R366">
-        <v>719.5448299999999</v>
+        <v>377.15638</v>
       </c>
       <c r="S366">
-        <v>5.612674180967239</v>
+        <v>5.411138880918221</v>
       </c>
       <c r="T366">
-        <v>1045.68</v>
+        <v>557.99</v>
       </c>
       <c r="U366">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="V366">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="W366">
-        <v>155</v>
+        <v>85</v>
       </c>
       <c r="X366">
-        <v>212</v>
+        <v>114</v>
       </c>
       <c r="Y366">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="Z366">
-        <v>179</v>
+        <v>96</v>
       </c>
       <c r="AA366">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="AB366">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="AC366">
         <v>4.27991</v>
@@ -41676,7 +41676,7 @@
         <v>0</v>
       </c>
       <c r="AF366">
-        <v>643.7375999999999</v>
+        <v>342.752</v>
       </c>
       <c r="AG366">
         <v>0</v>
@@ -41685,7 +41685,7 @@
         <v>3</v>
       </c>
       <c r="AI366">
-        <v>2158.63449</v>
+        <v>1131.46914</v>
       </c>
     </row>
     <row r="367">
@@ -41704,20 +41704,20 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E367">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F367">
-        <v>6654.87</v>
+        <v>3533.39</v>
       </c>
       <c r="G367">
-        <v>51.9100624024961</v>
+        <v>50.69426111908177</v>
       </c>
       <c r="H367">
-        <v>45.90000000000001</v>
+        <v>22.95</v>
       </c>
       <c r="I367">
         <v>0</v>
@@ -41726,7 +41726,7 @@
         <v>0</v>
       </c>
       <c r="K367">
-        <v>0.358034321372855</v>
+        <v>0.3292682926829268</v>
       </c>
       <c r="L367">
         <v>0</v>
@@ -41747,37 +41747,37 @@
         <v>36</v>
       </c>
       <c r="R367">
-        <v>877.70944</v>
+        <v>459.22363</v>
       </c>
       <c r="S367">
-        <v>6.846407488299532</v>
+        <v>6.588574318507891</v>
       </c>
       <c r="T367">
-        <v>1183.53998</v>
+        <v>631.57999</v>
       </c>
       <c r="U367">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="V367">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="W367">
-        <v>150</v>
+        <v>83</v>
       </c>
       <c r="X367">
-        <v>233</v>
+        <v>127</v>
       </c>
       <c r="Y367">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="Z367">
-        <v>200</v>
+        <v>107</v>
       </c>
       <c r="AA367">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="AB367">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="AC367">
         <v>4.22953</v>
@@ -41789,7 +41789,7 @@
         <v>0</v>
       </c>
       <c r="AF367">
-        <v>606.1867</v>
+        <v>322.147</v>
       </c>
       <c r="AG367">
         <v>0</v>
@@ -41798,7 +41798,7 @@
         <v>3</v>
       </c>
       <c r="AI367">
-        <v>2633.12832</v>
+        <v>1377.67089</v>
       </c>
     </row>
     <row r="368">
@@ -41817,20 +41817,20 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E368">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F368">
-        <v>4654.87</v>
+        <v>2570.85</v>
       </c>
       <c r="G368">
-        <v>36.3094383775351</v>
+        <v>36.8845050215208</v>
       </c>
       <c r="H368">
-        <v>27.62</v>
+        <v>13.81</v>
       </c>
       <c r="I368">
         <v>0</v>
@@ -41839,7 +41839,7 @@
         <v>0</v>
       </c>
       <c r="K368">
-        <v>0.2154446177847114</v>
+        <v>0.1981348637015782</v>
       </c>
       <c r="L368">
         <v>0</v>
@@ -41860,37 +41860,37 @@
         <v>32.004</v>
       </c>
       <c r="R368">
-        <v>625.58593</v>
+        <v>331.94508</v>
       </c>
       <c r="S368">
-        <v>4.879765444617785</v>
+        <v>4.762483213773314</v>
       </c>
       <c r="T368">
-        <v>728</v>
+        <v>392.06</v>
       </c>
       <c r="U368">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="V368">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="W368">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="X368">
-        <v>128</v>
+        <v>66</v>
       </c>
       <c r="Y368">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="Z368">
-        <v>123</v>
+        <v>63</v>
       </c>
       <c r="AA368">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="AB368">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="AC368">
         <v>4.07591</v>
@@ -41902,7 +41902,7 @@
         <v>0</v>
       </c>
       <c r="AF368">
-        <v>348.306</v>
+        <v>190.7094</v>
       </c>
       <c r="AG368">
         <v>0</v>
@@ -41911,7 +41911,7 @@
         <v>3</v>
       </c>
       <c r="AI368">
-        <v>1876.75779</v>
+        <v>995.8352400000001</v>
       </c>
     </row>
     <row r="369">
@@ -41930,20 +41930,20 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E369">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F369">
-        <v>5121.98</v>
+        <v>2764.9</v>
       </c>
       <c r="G369">
-        <v>39.95304212168487</v>
+        <v>39.66857962697274</v>
       </c>
       <c r="H369">
-        <v>52.14</v>
+        <v>26.07</v>
       </c>
       <c r="I369">
         <v>0</v>
@@ -41952,7 +41952,7 @@
         <v>0</v>
       </c>
       <c r="K369">
-        <v>0.4067082683307333</v>
+        <v>0.3740315638450502</v>
       </c>
       <c r="L369">
         <v>0</v>
@@ -41973,37 +41973,37 @@
         <v>33.84</v>
       </c>
       <c r="R369">
-        <v>639.7687099999999</v>
+        <v>339.82262</v>
       </c>
       <c r="S369">
-        <v>4.990395553822153</v>
+        <v>4.87550387374462</v>
       </c>
       <c r="T369">
-        <v>802.01</v>
+        <v>433.2</v>
       </c>
       <c r="U369">
+        <v>15</v>
+      </c>
+      <c r="V369">
         <v>27</v>
       </c>
-      <c r="V369">
-        <v>50</v>
-      </c>
       <c r="W369">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="X369">
-        <v>135</v>
+        <v>75</v>
       </c>
       <c r="Y369">
+        <v>15</v>
+      </c>
+      <c r="Z369">
+        <v>82</v>
+      </c>
+      <c r="AA369">
         <v>27</v>
       </c>
-      <c r="Z369">
-        <v>152</v>
-      </c>
-      <c r="AA369">
-        <v>50</v>
-      </c>
       <c r="AB369">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="AC369">
         <v>4.17768</v>
@@ -42015,7 +42015,7 @@
         <v>0</v>
       </c>
       <c r="AF369">
-        <v>461.8348</v>
+        <v>248.6722</v>
       </c>
       <c r="AG369">
         <v>0</v>
@@ -42024,7 +42024,7 @@
         <v>3</v>
       </c>
       <c r="AI369">
-        <v>1919.30613</v>
+        <v>1019.46786</v>
       </c>
     </row>
     <row r="370">
@@ -42043,17 +42043,17 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E370">
-        <v>111.4</v>
+        <v>52.9</v>
       </c>
       <c r="F370">
-        <v>4883.93</v>
+        <v>2378.3</v>
       </c>
       <c r="G370">
-        <v>43.84138240574507</v>
+        <v>44.95841209829867</v>
       </c>
       <c r="H370">
         <v>0</v>
@@ -42086,37 +42086,37 @@
         <v>33.696</v>
       </c>
       <c r="R370">
-        <v>646.40248</v>
+        <v>319.44484</v>
       </c>
       <c r="S370">
-        <v>5.802535727109515</v>
+        <v>6.038654820415879</v>
       </c>
       <c r="T370">
-        <v>733.56002</v>
+        <v>366.78001</v>
       </c>
       <c r="U370">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="V370">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="W370">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="X370">
-        <v>136</v>
+        <v>68</v>
       </c>
       <c r="Y370">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="Z370">
-        <v>132</v>
+        <v>66</v>
       </c>
       <c r="AA370">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="AB370">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="AC370">
         <v>3.90287</v>
@@ -42128,7 +42128,7 @@
         <v>0</v>
       </c>
       <c r="AF370">
-        <v>499.148</v>
+        <v>244.3544</v>
       </c>
       <c r="AG370">
         <v>0</v>
@@ -42137,7 +42137,7 @@
         <v>3</v>
       </c>
       <c r="AI370">
-        <v>1939.20744</v>
+        <v>958.33452</v>
       </c>
     </row>
     <row r="371">
@@ -42156,17 +42156,17 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E371">
-        <v>111.4</v>
+        <v>52.9</v>
       </c>
       <c r="F371">
-        <v>5165.42</v>
+        <v>2561.25</v>
       </c>
       <c r="G371">
-        <v>46.36822262118492</v>
+        <v>48.41682419659735</v>
       </c>
       <c r="H371">
         <v>0</v>
@@ -42199,37 +42199,37 @@
         <v>34.992</v>
       </c>
       <c r="R371">
-        <v>595.6703699999999</v>
+        <v>292.66553</v>
       </c>
       <c r="S371">
-        <v>5.34713078994614</v>
+        <v>5.532429678638941</v>
       </c>
       <c r="T371">
-        <v>689.0599999999999</v>
+        <v>344.53</v>
       </c>
       <c r="U371">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="V371">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="W371">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="X371">
-        <v>164</v>
+        <v>82</v>
       </c>
       <c r="Y371">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="Z371">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="AA371">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AB371">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="AC371">
         <v>4.09066</v>
@@ -42241,7 +42241,7 @@
         <v>0</v>
       </c>
       <c r="AF371">
-        <v>445.32324</v>
+        <v>221.57142</v>
       </c>
       <c r="AG371">
         <v>0</v>
@@ -42250,7 +42250,7 @@
         <v>3</v>
       </c>
       <c r="AI371">
-        <v>1787.01111</v>
+        <v>877.99659</v>
       </c>
     </row>
     <row r="372">
@@ -42269,17 +42269,17 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E372">
-        <v>111.4</v>
+        <v>52.9</v>
       </c>
       <c r="F372">
-        <v>4790.51</v>
+        <v>2350.71</v>
       </c>
       <c r="G372">
-        <v>43.00278276481149</v>
+        <v>44.43686200378073</v>
       </c>
       <c r="H372">
         <v>0</v>
@@ -42312,37 +42312,37 @@
         <v>34.92</v>
       </c>
       <c r="R372">
-        <v>594.2471399999999</v>
+        <v>289.3408</v>
       </c>
       <c r="S372">
-        <v>5.334354937163375</v>
+        <v>5.469580340264651</v>
       </c>
       <c r="T372">
-        <v>659.88998</v>
+        <v>322.50999</v>
       </c>
       <c r="U372">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="V372">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="W372">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="X372">
-        <v>127</v>
+        <v>62</v>
       </c>
       <c r="Y372">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="Z372">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="AA372">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="AB372">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="AC372">
         <v>4.20597</v>
@@ -42354,7 +42354,7 @@
         <v>0</v>
       </c>
       <c r="AF372">
-        <v>476.0064</v>
+        <v>233.7776</v>
       </c>
       <c r="AG372">
         <v>0</v>
@@ -42363,7 +42363,7 @@
         <v>3</v>
       </c>
       <c r="AI372">
-        <v>1782.74142</v>
+        <v>868.0224000000001</v>
       </c>
     </row>
     <row r="373">
@@ -42382,17 +42382,17 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E373">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F373">
-        <v>5449.63</v>
+        <v>2966.17</v>
       </c>
       <c r="G373">
-        <v>42.50881435257411</v>
+        <v>42.55624103299856</v>
       </c>
       <c r="H373">
         <v>0</v>
@@ -42425,37 +42425,37 @@
         <v>34.992</v>
       </c>
       <c r="R373">
-        <v>611.19537</v>
+        <v>316.80447</v>
       </c>
       <c r="S373">
-        <v>4.767514586583464</v>
+        <v>4.545257819225252</v>
       </c>
       <c r="T373">
-        <v>826.82002</v>
+        <v>444.77001</v>
       </c>
       <c r="U373">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="V373">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="W373">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="X373">
-        <v>170</v>
+        <v>89</v>
       </c>
       <c r="Y373">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="Z373">
-        <v>137</v>
+        <v>72</v>
       </c>
       <c r="AA373">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="AB373">
-        <v>134</v>
+        <v>67</v>
       </c>
       <c r="AC373">
         <v>3.85945</v>
@@ -42467,7 +42467,7 @@
         <v>0</v>
       </c>
       <c r="AF373">
-        <v>498.40935</v>
+        <v>269.5799</v>
       </c>
       <c r="AG373">
         <v>0</v>
@@ -42476,7 +42476,7 @@
         <v>3</v>
       </c>
       <c r="AI373">
-        <v>1833.58611</v>
+        <v>950.4134100000001</v>
       </c>
     </row>
     <row r="374">
@@ -42495,20 +42495,20 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E374">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F374">
-        <v>5078.179999999999</v>
+        <v>2790.93</v>
       </c>
       <c r="G374">
-        <v>39.61138845553822</v>
+        <v>40.04203730272597</v>
       </c>
       <c r="H374">
-        <v>12.66</v>
+        <v>6.880000000000001</v>
       </c>
       <c r="I374">
         <v>0</v>
@@ -42517,7 +42517,7 @@
         <v>0</v>
       </c>
       <c r="K374">
-        <v>0.09875195007800315</v>
+        <v>0.09870875179340029</v>
       </c>
       <c r="L374">
         <v>0</v>
@@ -42538,37 +42538,37 @@
         <v>33.984</v>
       </c>
       <c r="R374">
-        <v>728.5777400000001</v>
+        <v>385.37218</v>
       </c>
       <c r="S374">
-        <v>5.683133697347895</v>
+        <v>5.52901262553802</v>
       </c>
       <c r="T374">
-        <v>704.62</v>
+        <v>385.94</v>
       </c>
       <c r="U374">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="V374">
+        <v>17</v>
+      </c>
+      <c r="W374">
         <v>33</v>
       </c>
-      <c r="W374">
-        <v>61</v>
-      </c>
       <c r="X374">
-        <v>121</v>
+        <v>65</v>
       </c>
       <c r="Y374">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="Z374">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="AA374">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="AB374">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="AC374">
         <v>3.92536</v>
@@ -42580,7 +42580,7 @@
         <v>0</v>
       </c>
       <c r="AF374">
-        <v>501.4448</v>
+        <v>275.612</v>
       </c>
       <c r="AG374">
         <v>0</v>
@@ -42589,7 +42589,7 @@
         <v>3</v>
       </c>
       <c r="AI374">
-        <v>2185.73322</v>
+        <v>1156.11654</v>
       </c>
     </row>
     <row r="375">
@@ -42608,17 +42608,17 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E375">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F375">
-        <v>5131.96</v>
+        <v>2546.24</v>
       </c>
       <c r="G375">
-        <v>40.03088923556943</v>
+        <v>36.53142037302726</v>
       </c>
       <c r="H375">
         <v>0</v>
@@ -42651,37 +42651,37 @@
         <v>34.992</v>
       </c>
       <c r="R375">
-        <v>660.59281</v>
+        <v>326.65239</v>
       </c>
       <c r="S375">
-        <v>5.152830031201248</v>
+        <v>4.686547919655666</v>
       </c>
       <c r="T375">
-        <v>810.11</v>
+        <v>404.81</v>
       </c>
       <c r="U375">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="V375">
+        <v>19</v>
+      </c>
+      <c r="W375">
+        <v>34</v>
+      </c>
+      <c r="X375">
+        <v>84</v>
+      </c>
+      <c r="Y375">
+        <v>15</v>
+      </c>
+      <c r="Z375">
+        <v>76</v>
+      </c>
+      <c r="AA375">
+        <v>19</v>
+      </c>
+      <c r="AB375">
         <v>38</v>
-      </c>
-      <c r="W375">
-        <v>68</v>
-      </c>
-      <c r="X375">
-        <v>168</v>
-      </c>
-      <c r="Y375">
-        <v>30</v>
-      </c>
-      <c r="Z375">
-        <v>152</v>
-      </c>
-      <c r="AA375">
-        <v>38</v>
-      </c>
-      <c r="AB375">
-        <v>79</v>
       </c>
       <c r="AC375">
         <v>3.89727</v>
@@ -42693,7 +42693,7 @@
         <v>0</v>
       </c>
       <c r="AF375">
-        <v>514.1976000000001</v>
+        <v>255.6072</v>
       </c>
       <c r="AG375">
         <v>0</v>
@@ -42702,7 +42702,7 @@
         <v>3</v>
       </c>
       <c r="AI375">
-        <v>1981.77843</v>
+        <v>979.9571699999999</v>
       </c>
     </row>
     <row r="376">
@@ -42721,20 +42721,20 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E376">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F376">
-        <v>5316.75</v>
+        <v>2924.54</v>
       </c>
       <c r="G376">
-        <v>41.4723088923557</v>
+        <v>41.95896700143471</v>
       </c>
       <c r="H376">
-        <v>22.87</v>
+        <v>11.97</v>
       </c>
       <c r="I376">
         <v>0</v>
@@ -42743,7 +42743,7 @@
         <v>0</v>
       </c>
       <c r="K376">
-        <v>0.178393135725429</v>
+        <v>0.1717360114777618</v>
       </c>
       <c r="L376">
         <v>0</v>
@@ -42764,37 +42764,37 @@
         <v>33.012</v>
       </c>
       <c r="R376">
-        <v>649.42518</v>
+        <v>345.55249</v>
       </c>
       <c r="S376">
-        <v>5.065719032761311</v>
+        <v>4.957711477761837</v>
       </c>
       <c r="T376">
-        <v>860.37</v>
+        <v>472.07</v>
       </c>
       <c r="U376">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="V376">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="W376">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="X376">
-        <v>184</v>
+        <v>97</v>
       </c>
       <c r="Y376">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="Z376">
-        <v>157</v>
+        <v>83</v>
       </c>
       <c r="AA376">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="AB376">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="AC376">
         <v>3.98992</v>
@@ -42806,7 +42806,7 @@
         <v>0</v>
       </c>
       <c r="AF376">
-        <v>497.73825</v>
+        <v>273.2887500000001</v>
       </c>
       <c r="AG376">
         <v>0</v>
@@ -42815,7 +42815,7 @@
         <v>3</v>
       </c>
       <c r="AI376">
-        <v>1948.27554</v>
+        <v>1036.65747</v>
       </c>
     </row>
     <row r="377">
@@ -42834,20 +42834,20 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E377">
-        <v>111.4</v>
+        <v>52.9</v>
       </c>
       <c r="F377">
-        <v>4749.22</v>
+        <v>2345.74</v>
       </c>
       <c r="G377">
-        <v>42.63213644524237</v>
+        <v>44.34291115311909</v>
       </c>
       <c r="H377">
-        <v>11.06</v>
+        <v>5.53</v>
       </c>
       <c r="I377">
         <v>0</v>
@@ -42856,7 +42856,7 @@
         <v>0</v>
       </c>
       <c r="K377">
-        <v>0.09928186714542191</v>
+        <v>0.1045368620037807</v>
       </c>
       <c r="L377">
         <v>0</v>
@@ -42877,37 +42877,37 @@
         <v>32.004</v>
       </c>
       <c r="R377">
-        <v>561.6697300000001</v>
+        <v>277.13314</v>
       </c>
       <c r="S377">
-        <v>5.041918581687613</v>
+        <v>5.238811720226844</v>
       </c>
       <c r="T377">
-        <v>507.18</v>
+        <v>253.59</v>
       </c>
       <c r="U377">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="V377">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="W377">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="X377">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="Y377">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="Z377">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="AA377">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="AB377">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="AC377">
         <v>3.86956</v>
@@ -42919,7 +42919,7 @@
         <v>0</v>
       </c>
       <c r="AF377">
-        <v>394.9568</v>
+        <v>195.6073</v>
       </c>
       <c r="AG377">
         <v>0</v>
@@ -42928,7 +42928,7 @@
         <v>3</v>
       </c>
       <c r="AI377">
-        <v>1685.00919</v>
+        <v>831.3994200000001</v>
       </c>
     </row>
     <row r="378">
@@ -42947,20 +42947,20 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>Sesión 28 | 06 jul 10:27 a. m.</t>
+          <t>Sesión 28</t>
         </is>
       </c>
       <c r="E378">
-        <v>128.2</v>
+        <v>69.7</v>
       </c>
       <c r="F378">
-        <v>5350.58</v>
+        <v>2867.22</v>
       </c>
       <c r="G378">
-        <v>41.73619344773791</v>
+        <v>41.13658536585366</v>
       </c>
       <c r="H378">
-        <v>3.04</v>
+        <v>1.52</v>
       </c>
       <c r="I378">
         <v>0</v>
@@ -42969,7 +42969,7 @@
         <v>0</v>
       </c>
       <c r="K378">
-        <v>0.02371294851794072</v>
+        <v>0.0218077474892396</v>
       </c>
       <c r="L378">
         <v>0</v>
@@ -42990,37 +42990,37 @@
         <v>36</v>
       </c>
       <c r="R378">
-        <v>699.7805</v>
+        <v>368.31494</v>
       </c>
       <c r="S378">
-        <v>5.45850624024961</v>
+        <v>5.284288952654232</v>
       </c>
       <c r="T378">
-        <v>824.22</v>
+        <v>444.34</v>
       </c>
       <c r="U378">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="V378">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="W378">
-        <v>123</v>
+        <v>65</v>
       </c>
       <c r="X378">
-        <v>150</v>
+        <v>83</v>
       </c>
       <c r="Y378">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="Z378">
-        <v>148</v>
+        <v>80</v>
       </c>
       <c r="AA378">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="AB378">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="AC378">
         <v>4.35677</v>
@@ -43032,7 +43032,7 @@
         <v>0</v>
       </c>
       <c r="AF378">
-        <v>479.0751</v>
+        <v>256.7607</v>
       </c>
       <c r="AG378">
         <v>0</v>
@@ -43041,7 +43041,7 @@
         <v>3</v>
       </c>
       <c r="AI378">
-        <v>2099.3415</v>
+        <v>1104.94482</v>
       </c>
     </row>
     <row r="379">
@@ -50161,6 +50161,1927 @@
       </c>
       <c r="AI441">
         <v>1112.59533</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B442" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E442">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F442">
+        <v>2848.5</v>
+      </c>
+      <c r="G442">
+        <v>38.0561122244489</v>
+      </c>
+      <c r="H442">
+        <v>56.82</v>
+      </c>
+      <c r="I442">
+        <v>0</v>
+      </c>
+      <c r="J442">
+        <v>0</v>
+      </c>
+      <c r="K442">
+        <v>0.759118236472946</v>
+      </c>
+      <c r="L442">
+        <v>0</v>
+      </c>
+      <c r="M442">
+        <v>1</v>
+      </c>
+      <c r="N442">
+        <v>0</v>
+      </c>
+      <c r="O442">
+        <v>27.08687</v>
+      </c>
+      <c r="P442">
+        <v>83.69444444444446</v>
+      </c>
+      <c r="Q442">
+        <v>32.364</v>
+      </c>
+      <c r="R442">
+        <v>263.06908</v>
+      </c>
+      <c r="S442">
+        <v>3.514616967267869</v>
+      </c>
+      <c r="T442">
+        <v>264.34001</v>
+      </c>
+      <c r="U442">
+        <v>9</v>
+      </c>
+      <c r="V442">
+        <v>1</v>
+      </c>
+      <c r="W442">
+        <v>10</v>
+      </c>
+      <c r="X442">
+        <v>22</v>
+      </c>
+      <c r="Y442">
+        <v>9</v>
+      </c>
+      <c r="Z442">
+        <v>13</v>
+      </c>
+      <c r="AA442">
+        <v>1</v>
+      </c>
+      <c r="AB442">
+        <v>12</v>
+      </c>
+      <c r="AC442">
+        <v>4.15354</v>
+      </c>
+      <c r="AD442">
+        <v>-2.40276</v>
+      </c>
+      <c r="AE442">
+        <v>0</v>
+      </c>
+      <c r="AF442">
+        <v>218.5197</v>
+      </c>
+      <c r="AG442">
+        <v>0</v>
+      </c>
+      <c r="AH442">
+        <v>3</v>
+      </c>
+      <c r="AI442">
+        <v>789.20724</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B443" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E443">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F443">
+        <v>2703.25</v>
+      </c>
+      <c r="G443">
+        <v>36.11556446225784</v>
+      </c>
+      <c r="H443">
+        <v>11.9</v>
+      </c>
+      <c r="I443">
+        <v>0</v>
+      </c>
+      <c r="J443">
+        <v>0</v>
+      </c>
+      <c r="K443">
+        <v>0.1589846359385438</v>
+      </c>
+      <c r="L443">
+        <v>0</v>
+      </c>
+      <c r="M443">
+        <v>0</v>
+      </c>
+      <c r="N443">
+        <v>0</v>
+      </c>
+      <c r="O443">
+        <v>22.90987</v>
+      </c>
+      <c r="P443">
+        <v>63.63852777777779</v>
+      </c>
+      <c r="Q443">
+        <v>36</v>
+      </c>
+      <c r="R443">
+        <v>236.20478</v>
+      </c>
+      <c r="S443">
+        <v>3.155708483633935</v>
+      </c>
+      <c r="T443">
+        <v>178.58</v>
+      </c>
+      <c r="U443">
+        <v>8</v>
+      </c>
+      <c r="V443">
+        <v>9</v>
+      </c>
+      <c r="W443">
+        <v>17</v>
+      </c>
+      <c r="X443">
+        <v>22</v>
+      </c>
+      <c r="Y443">
+        <v>8</v>
+      </c>
+      <c r="Z443">
+        <v>20</v>
+      </c>
+      <c r="AA443">
+        <v>9</v>
+      </c>
+      <c r="AB443">
+        <v>19</v>
+      </c>
+      <c r="AC443">
+        <v>4.5943</v>
+      </c>
+      <c r="AD443">
+        <v>-3.16756</v>
+      </c>
+      <c r="AE443">
+        <v>0</v>
+      </c>
+      <c r="AF443">
+        <v>619.9399999999999</v>
+      </c>
+      <c r="AG443">
+        <v>0</v>
+      </c>
+      <c r="AH443">
+        <v>3</v>
+      </c>
+      <c r="AI443">
+        <v>708.6143400000001</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B444" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E444">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F444">
+        <v>2949.24</v>
+      </c>
+      <c r="G444">
+        <v>39.40200400801604</v>
+      </c>
+      <c r="H444">
+        <v>113.38</v>
+      </c>
+      <c r="I444">
+        <v>0</v>
+      </c>
+      <c r="J444">
+        <v>0</v>
+      </c>
+      <c r="K444">
+        <v>1.514762859051436</v>
+      </c>
+      <c r="L444">
+        <v>0</v>
+      </c>
+      <c r="M444">
+        <v>2</v>
+      </c>
+      <c r="N444">
+        <v>0</v>
+      </c>
+      <c r="O444">
+        <v>29.11992</v>
+      </c>
+      <c r="P444">
+        <v>89.8762962962963</v>
+      </c>
+      <c r="Q444">
+        <v>32.4</v>
+      </c>
+      <c r="R444">
+        <v>297.67398</v>
+      </c>
+      <c r="S444">
+        <v>3.976940280561122</v>
+      </c>
+      <c r="T444">
+        <v>407.24999</v>
+      </c>
+      <c r="U444">
+        <v>18</v>
+      </c>
+      <c r="V444">
+        <v>11</v>
+      </c>
+      <c r="W444">
+        <v>29</v>
+      </c>
+      <c r="X444">
+        <v>42</v>
+      </c>
+      <c r="Y444">
+        <v>18</v>
+      </c>
+      <c r="Z444">
+        <v>32</v>
+      </c>
+      <c r="AA444">
+        <v>11</v>
+      </c>
+      <c r="AB444">
+        <v>6</v>
+      </c>
+      <c r="AC444">
+        <v>4.14649</v>
+      </c>
+      <c r="AD444">
+        <v>-1.87846</v>
+      </c>
+      <c r="AE444">
+        <v>0</v>
+      </c>
+      <c r="AF444">
+        <v>239.3237</v>
+      </c>
+      <c r="AG444">
+        <v>0</v>
+      </c>
+      <c r="AH444">
+        <v>3</v>
+      </c>
+      <c r="AI444">
+        <v>893.0219399999999</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B445" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E445">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F445">
+        <v>2584.21</v>
+      </c>
+      <c r="G445">
+        <v>34.52518370073481</v>
+      </c>
+      <c r="H445">
+        <v>31.13</v>
+      </c>
+      <c r="I445">
+        <v>0</v>
+      </c>
+      <c r="J445">
+        <v>0</v>
+      </c>
+      <c r="K445">
+        <v>0.4158984635938544</v>
+      </c>
+      <c r="L445">
+        <v>0</v>
+      </c>
+      <c r="M445">
+        <v>1</v>
+      </c>
+      <c r="N445">
+        <v>0</v>
+      </c>
+      <c r="O445">
+        <v>26.18662</v>
+      </c>
+      <c r="P445">
+        <v>73.6241003148898</v>
+      </c>
+      <c r="Q445">
+        <v>35.568</v>
+      </c>
+      <c r="R445">
+        <v>253.5021</v>
+      </c>
+      <c r="S445">
+        <v>3.386801603206413</v>
+      </c>
+      <c r="T445">
+        <v>168.88</v>
+      </c>
+      <c r="U445">
+        <v>9</v>
+      </c>
+      <c r="V445">
+        <v>2</v>
+      </c>
+      <c r="W445">
+        <v>11</v>
+      </c>
+      <c r="X445">
+        <v>24</v>
+      </c>
+      <c r="Y445">
+        <v>9</v>
+      </c>
+      <c r="Z445">
+        <v>14</v>
+      </c>
+      <c r="AA445">
+        <v>2</v>
+      </c>
+      <c r="AB445">
+        <v>14</v>
+      </c>
+      <c r="AC445">
+        <v>4.89899</v>
+      </c>
+      <c r="AD445">
+        <v>-2.25433</v>
+      </c>
+      <c r="AE445">
+        <v>0</v>
+      </c>
+      <c r="AF445">
+        <v>231.4464</v>
+      </c>
+      <c r="AG445">
+        <v>0</v>
+      </c>
+      <c r="AH445">
+        <v>3</v>
+      </c>
+      <c r="AI445">
+        <v>760.5063</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B446" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E446">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F446">
+        <v>2883.05</v>
+      </c>
+      <c r="G446">
+        <v>38.51770207080829</v>
+      </c>
+      <c r="H446">
+        <v>27.81</v>
+      </c>
+      <c r="I446">
+        <v>0</v>
+      </c>
+      <c r="J446">
+        <v>0</v>
+      </c>
+      <c r="K446">
+        <v>0.3715430861723448</v>
+      </c>
+      <c r="L446">
+        <v>0</v>
+      </c>
+      <c r="M446">
+        <v>0</v>
+      </c>
+      <c r="N446">
+        <v>0</v>
+      </c>
+      <c r="O446">
+        <v>23.14376</v>
+      </c>
+      <c r="P446">
+        <v>64.28822222222223</v>
+      </c>
+      <c r="Q446">
+        <v>36</v>
+      </c>
+      <c r="R446">
+        <v>309.71679</v>
+      </c>
+      <c r="S446">
+        <v>4.137832865731463</v>
+      </c>
+      <c r="T446">
+        <v>172.13</v>
+      </c>
+      <c r="U446">
+        <v>7</v>
+      </c>
+      <c r="V446">
+        <v>1</v>
+      </c>
+      <c r="W446">
+        <v>8</v>
+      </c>
+      <c r="X446">
+        <v>14</v>
+      </c>
+      <c r="Y446">
+        <v>7</v>
+      </c>
+      <c r="Z446">
+        <v>11</v>
+      </c>
+      <c r="AA446">
+        <v>1</v>
+      </c>
+      <c r="AB446">
+        <v>17</v>
+      </c>
+      <c r="AC446">
+        <v>4.25649</v>
+      </c>
+      <c r="AD446">
+        <v>-2.36906</v>
+      </c>
+      <c r="AE446">
+        <v>0</v>
+      </c>
+      <c r="AF446">
+        <v>630.1420000000001</v>
+      </c>
+      <c r="AG446">
+        <v>0</v>
+      </c>
+      <c r="AH446">
+        <v>3</v>
+      </c>
+      <c r="AI446">
+        <v>929.1503700000001</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B447" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E447">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F447">
+        <v>2184.33</v>
+      </c>
+      <c r="G447">
+        <v>29.18276553106212</v>
+      </c>
+      <c r="H447">
+        <v>28.06</v>
+      </c>
+      <c r="I447">
+        <v>0</v>
+      </c>
+      <c r="J447">
+        <v>0</v>
+      </c>
+      <c r="K447">
+        <v>0.3748830995323982</v>
+      </c>
+      <c r="L447">
+        <v>0</v>
+      </c>
+      <c r="M447">
+        <v>0</v>
+      </c>
+      <c r="N447">
+        <v>0</v>
+      </c>
+      <c r="O447">
+        <v>23.98897</v>
+      </c>
+      <c r="P447">
+        <v>66.63602777777777</v>
+      </c>
+      <c r="Q447">
+        <v>36</v>
+      </c>
+      <c r="R447">
+        <v>221.19235</v>
+      </c>
+      <c r="S447">
+        <v>2.955141616566466</v>
+      </c>
+      <c r="T447">
+        <v>135.37</v>
+      </c>
+      <c r="U447">
+        <v>7</v>
+      </c>
+      <c r="V447">
+        <v>0</v>
+      </c>
+      <c r="W447">
+        <v>7</v>
+      </c>
+      <c r="X447">
+        <v>16</v>
+      </c>
+      <c r="Y447">
+        <v>7</v>
+      </c>
+      <c r="Z447">
+        <v>5</v>
+      </c>
+      <c r="AA447">
+        <v>0</v>
+      </c>
+      <c r="AB447">
+        <v>7</v>
+      </c>
+      <c r="AC447">
+        <v>4.04607</v>
+      </c>
+      <c r="AD447">
+        <v>-1.40888</v>
+      </c>
+      <c r="AE447">
+        <v>0</v>
+      </c>
+      <c r="AF447">
+        <v>165.0908</v>
+      </c>
+      <c r="AG447">
+        <v>0</v>
+      </c>
+      <c r="AH447">
+        <v>3</v>
+      </c>
+      <c r="AI447">
+        <v>663.5770499999999</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B448" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E448">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F448">
+        <v>3544.78</v>
+      </c>
+      <c r="G448">
+        <v>47.35845023380094</v>
+      </c>
+      <c r="H448">
+        <v>108.59</v>
+      </c>
+      <c r="I448">
+        <v>0</v>
+      </c>
+      <c r="J448">
+        <v>0</v>
+      </c>
+      <c r="K448">
+        <v>1.450768203072812</v>
+      </c>
+      <c r="L448">
+        <v>0</v>
+      </c>
+      <c r="M448">
+        <v>1</v>
+      </c>
+      <c r="N448">
+        <v>0</v>
+      </c>
+      <c r="O448">
+        <v>26.2262</v>
+      </c>
+      <c r="P448">
+        <v>81.94663167104113</v>
+      </c>
+      <c r="Q448">
+        <v>32.004</v>
+      </c>
+      <c r="R448">
+        <v>384.71614</v>
+      </c>
+      <c r="S448">
+        <v>5.139828189712759</v>
+      </c>
+      <c r="T448">
+        <v>416.29001</v>
+      </c>
+      <c r="U448">
+        <v>16</v>
+      </c>
+      <c r="V448">
+        <v>5</v>
+      </c>
+      <c r="W448">
+        <v>21</v>
+      </c>
+      <c r="X448">
+        <v>39</v>
+      </c>
+      <c r="Y448">
+        <v>16</v>
+      </c>
+      <c r="Z448">
+        <v>31</v>
+      </c>
+      <c r="AA448">
+        <v>5</v>
+      </c>
+      <c r="AB448">
+        <v>14</v>
+      </c>
+      <c r="AC448">
+        <v>4.75898</v>
+      </c>
+      <c r="AD448">
+        <v>-2.58658</v>
+      </c>
+      <c r="AE448">
+        <v>0</v>
+      </c>
+      <c r="AF448">
+        <v>246.24</v>
+      </c>
+      <c r="AG448">
+        <v>0</v>
+      </c>
+      <c r="AH448">
+        <v>3</v>
+      </c>
+      <c r="AI448">
+        <v>1154.14842</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B449" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E449">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F449">
+        <v>2910.92</v>
+      </c>
+      <c r="G449">
+        <v>38.89004676018705</v>
+      </c>
+      <c r="H449">
+        <v>118</v>
+      </c>
+      <c r="I449">
+        <v>0</v>
+      </c>
+      <c r="J449">
+        <v>0</v>
+      </c>
+      <c r="K449">
+        <v>1.576486305945224</v>
+      </c>
+      <c r="L449">
+        <v>0</v>
+      </c>
+      <c r="M449">
+        <v>0</v>
+      </c>
+      <c r="N449">
+        <v>0</v>
+      </c>
+      <c r="O449">
+        <v>24.96236</v>
+      </c>
+      <c r="P449">
+        <v>74.08107787274454</v>
+      </c>
+      <c r="Q449">
+        <v>33.696</v>
+      </c>
+      <c r="R449">
+        <v>304.11906</v>
+      </c>
+      <c r="S449">
+        <v>4.063046893787575</v>
+      </c>
+      <c r="T449">
+        <v>320.12</v>
+      </c>
+      <c r="U449">
+        <v>17</v>
+      </c>
+      <c r="V449">
+        <v>4</v>
+      </c>
+      <c r="W449">
+        <v>21</v>
+      </c>
+      <c r="X449">
+        <v>34</v>
+      </c>
+      <c r="Y449">
+        <v>17</v>
+      </c>
+      <c r="Z449">
+        <v>22</v>
+      </c>
+      <c r="AA449">
+        <v>4</v>
+      </c>
+      <c r="AB449">
+        <v>14</v>
+      </c>
+      <c r="AC449">
+        <v>4.34302</v>
+      </c>
+      <c r="AD449">
+        <v>-2.27254</v>
+      </c>
+      <c r="AE449">
+        <v>0</v>
+      </c>
+      <c r="AF449">
+        <v>264.6232</v>
+      </c>
+      <c r="AG449">
+        <v>0</v>
+      </c>
+      <c r="AH449">
+        <v>3</v>
+      </c>
+      <c r="AI449">
+        <v>912.35718</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B450" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E450">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F450">
+        <v>3696.55</v>
+      </c>
+      <c r="G450">
+        <v>49.38610554442219</v>
+      </c>
+      <c r="H450">
+        <v>109.1</v>
+      </c>
+      <c r="I450">
+        <v>0</v>
+      </c>
+      <c r="J450">
+        <v>0</v>
+      </c>
+      <c r="K450">
+        <v>1.457581830327321</v>
+      </c>
+      <c r="L450">
+        <v>0</v>
+      </c>
+      <c r="M450">
+        <v>3</v>
+      </c>
+      <c r="N450">
+        <v>0</v>
+      </c>
+      <c r="O450">
+        <v>28.70304</v>
+      </c>
+      <c r="P450">
+        <v>82.02743484224968</v>
+      </c>
+      <c r="Q450">
+        <v>34.992</v>
+      </c>
+      <c r="R450">
+        <v>337.34061</v>
+      </c>
+      <c r="S450">
+        <v>4.506888577154309</v>
+      </c>
+      <c r="T450">
+        <v>374.68001</v>
+      </c>
+      <c r="U450">
+        <v>20</v>
+      </c>
+      <c r="V450">
+        <v>6</v>
+      </c>
+      <c r="W450">
+        <v>26</v>
+      </c>
+      <c r="X450">
+        <v>38</v>
+      </c>
+      <c r="Y450">
+        <v>20</v>
+      </c>
+      <c r="Z450">
+        <v>28</v>
+      </c>
+      <c r="AA450">
+        <v>6</v>
+      </c>
+      <c r="AB450">
+        <v>22</v>
+      </c>
+      <c r="AC450">
+        <v>4.46686</v>
+      </c>
+      <c r="AD450">
+        <v>-2.57817</v>
+      </c>
+      <c r="AE450">
+        <v>0</v>
+      </c>
+      <c r="AF450">
+        <v>289.86831</v>
+      </c>
+      <c r="AG450">
+        <v>0</v>
+      </c>
+      <c r="AH450">
+        <v>3</v>
+      </c>
+      <c r="AI450">
+        <v>1012.02183</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B451" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E451">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F451">
+        <v>2949.07</v>
+      </c>
+      <c r="G451">
+        <v>39.3997327989312</v>
+      </c>
+      <c r="H451">
+        <v>26.45</v>
+      </c>
+      <c r="I451">
+        <v>0</v>
+      </c>
+      <c r="J451">
+        <v>0</v>
+      </c>
+      <c r="K451">
+        <v>0.353373413493654</v>
+      </c>
+      <c r="L451">
+        <v>0</v>
+      </c>
+      <c r="M451">
+        <v>0</v>
+      </c>
+      <c r="N451">
+        <v>0</v>
+      </c>
+      <c r="O451">
+        <v>23.7255</v>
+      </c>
+      <c r="P451">
+        <v>67.94243986254295</v>
+      </c>
+      <c r="Q451">
+        <v>34.92</v>
+      </c>
+      <c r="R451">
+        <v>274.03416</v>
+      </c>
+      <c r="S451">
+        <v>3.661111022044088</v>
+      </c>
+      <c r="T451">
+        <v>218.47999</v>
+      </c>
+      <c r="U451">
+        <v>12</v>
+      </c>
+      <c r="V451">
+        <v>0</v>
+      </c>
+      <c r="W451">
+        <v>12</v>
+      </c>
+      <c r="X451">
+        <v>33</v>
+      </c>
+      <c r="Y451">
+        <v>12</v>
+      </c>
+      <c r="Z451">
+        <v>11</v>
+      </c>
+      <c r="AA451">
+        <v>0</v>
+      </c>
+      <c r="AB451">
+        <v>14</v>
+      </c>
+      <c r="AC451">
+        <v>4.20298</v>
+      </c>
+      <c r="AD451">
+        <v>-2.34344</v>
+      </c>
+      <c r="AE451">
+        <v>0</v>
+      </c>
+      <c r="AF451">
+        <v>265.044</v>
+      </c>
+      <c r="AG451">
+        <v>0</v>
+      </c>
+      <c r="AH451">
+        <v>3</v>
+      </c>
+      <c r="AI451">
+        <v>822.10248</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B452" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E452">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F452">
+        <v>2982.89</v>
+      </c>
+      <c r="G452">
+        <v>39.85156980627923</v>
+      </c>
+      <c r="H452">
+        <v>62.05</v>
+      </c>
+      <c r="I452">
+        <v>0</v>
+      </c>
+      <c r="J452">
+        <v>0</v>
+      </c>
+      <c r="K452">
+        <v>0.828991315965264</v>
+      </c>
+      <c r="L452">
+        <v>0</v>
+      </c>
+      <c r="M452">
+        <v>0</v>
+      </c>
+      <c r="N452">
+        <v>0</v>
+      </c>
+      <c r="O452">
+        <v>23.99979</v>
+      </c>
+      <c r="P452">
+        <v>68.58650548696845</v>
+      </c>
+      <c r="Q452">
+        <v>34.992</v>
+      </c>
+      <c r="R452">
+        <v>255.89984</v>
+      </c>
+      <c r="S452">
+        <v>3.418835537742151</v>
+      </c>
+      <c r="T452">
+        <v>282.27</v>
+      </c>
+      <c r="U452">
+        <v>15</v>
+      </c>
+      <c r="V452">
+        <v>6</v>
+      </c>
+      <c r="W452">
+        <v>21</v>
+      </c>
+      <c r="X452">
+        <v>27</v>
+      </c>
+      <c r="Y452">
+        <v>15</v>
+      </c>
+      <c r="Z452">
+        <v>24</v>
+      </c>
+      <c r="AA452">
+        <v>6</v>
+      </c>
+      <c r="AB452">
+        <v>7</v>
+      </c>
+      <c r="AC452">
+        <v>4.64684</v>
+      </c>
+      <c r="AD452">
+        <v>-2.46422</v>
+      </c>
+      <c r="AE452">
+        <v>0</v>
+      </c>
+      <c r="AF452">
+        <v>244.72209</v>
+      </c>
+      <c r="AG452">
+        <v>0</v>
+      </c>
+      <c r="AH452">
+        <v>3</v>
+      </c>
+      <c r="AI452">
+        <v>767.6995199999999</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B453" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E453">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F453">
+        <v>2781.03</v>
+      </c>
+      <c r="G453">
+        <v>37.15470941883768</v>
+      </c>
+      <c r="H453">
+        <v>32.54</v>
+      </c>
+      <c r="I453">
+        <v>0</v>
+      </c>
+      <c r="J453">
+        <v>0</v>
+      </c>
+      <c r="K453">
+        <v>0.4347361389445558</v>
+      </c>
+      <c r="L453">
+        <v>0</v>
+      </c>
+      <c r="M453">
+        <v>0</v>
+      </c>
+      <c r="N453">
+        <v>0</v>
+      </c>
+      <c r="O453">
+        <v>23.42193</v>
+      </c>
+      <c r="P453">
+        <v>65.06091666666667</v>
+      </c>
+      <c r="Q453">
+        <v>36</v>
+      </c>
+      <c r="R453">
+        <v>291.69543</v>
+      </c>
+      <c r="S453">
+        <v>3.897066533066132</v>
+      </c>
+      <c r="T453">
+        <v>213.56</v>
+      </c>
+      <c r="U453">
+        <v>7</v>
+      </c>
+      <c r="V453">
+        <v>2</v>
+      </c>
+      <c r="W453">
+        <v>9</v>
+      </c>
+      <c r="X453">
+        <v>18</v>
+      </c>
+      <c r="Y453">
+        <v>7</v>
+      </c>
+      <c r="Z453">
+        <v>13</v>
+      </c>
+      <c r="AA453">
+        <v>2</v>
+      </c>
+      <c r="AB453">
+        <v>25</v>
+      </c>
+      <c r="AC453">
+        <v>4.31578</v>
+      </c>
+      <c r="AD453">
+        <v>-2.11012</v>
+      </c>
+      <c r="AE453">
+        <v>0</v>
+      </c>
+      <c r="AF453">
+        <v>615.09</v>
+      </c>
+      <c r="AG453">
+        <v>0</v>
+      </c>
+      <c r="AH453">
+        <v>3</v>
+      </c>
+      <c r="AI453">
+        <v>875.08629</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B454" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E454">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F454">
+        <v>2409.22</v>
+      </c>
+      <c r="G454">
+        <v>32.18730794923179</v>
+      </c>
+      <c r="H454">
+        <v>7.66</v>
+      </c>
+      <c r="I454">
+        <v>0</v>
+      </c>
+      <c r="J454">
+        <v>0</v>
+      </c>
+      <c r="K454">
+        <v>0.1023380093520374</v>
+      </c>
+      <c r="L454">
+        <v>0</v>
+      </c>
+      <c r="M454">
+        <v>0</v>
+      </c>
+      <c r="N454">
+        <v>0</v>
+      </c>
+      <c r="O454">
+        <v>21.90847</v>
+      </c>
+      <c r="P454">
+        <v>64.46701388888889</v>
+      </c>
+      <c r="Q454">
+        <v>33.984</v>
+      </c>
+      <c r="R454">
+        <v>253.74549</v>
+      </c>
+      <c r="S454">
+        <v>3.390053306613227</v>
+      </c>
+      <c r="T454">
+        <v>175.32</v>
+      </c>
+      <c r="U454">
+        <v>7</v>
+      </c>
+      <c r="V454">
+        <v>1</v>
+      </c>
+      <c r="W454">
+        <v>8</v>
+      </c>
+      <c r="X454">
+        <v>25</v>
+      </c>
+      <c r="Y454">
+        <v>7</v>
+      </c>
+      <c r="Z454">
+        <v>15</v>
+      </c>
+      <c r="AA454">
+        <v>1</v>
+      </c>
+      <c r="AB454">
+        <v>12</v>
+      </c>
+      <c r="AC454">
+        <v>3.92628</v>
+      </c>
+      <c r="AD454">
+        <v>-1.81452</v>
+      </c>
+      <c r="AE454">
+        <v>0</v>
+      </c>
+      <c r="AF454">
+        <v>210.696</v>
+      </c>
+      <c r="AG454">
+        <v>0</v>
+      </c>
+      <c r="AH454">
+        <v>3</v>
+      </c>
+      <c r="AI454">
+        <v>761.2364700000001</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B455" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E455">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F455">
+        <v>3007.65</v>
+      </c>
+      <c r="G455">
+        <v>40.18236472945893</v>
+      </c>
+      <c r="H455">
+        <v>47.23999999999999</v>
+      </c>
+      <c r="I455">
+        <v>0</v>
+      </c>
+      <c r="J455">
+        <v>0</v>
+      </c>
+      <c r="K455">
+        <v>0.631128924515698</v>
+      </c>
+      <c r="L455">
+        <v>0</v>
+      </c>
+      <c r="M455">
+        <v>0</v>
+      </c>
+      <c r="N455">
+        <v>0</v>
+      </c>
+      <c r="O455">
+        <v>24.75111</v>
+      </c>
+      <c r="P455">
+        <v>70.73362482853224</v>
+      </c>
+      <c r="Q455">
+        <v>34.992</v>
+      </c>
+      <c r="R455">
+        <v>370.68996</v>
+      </c>
+      <c r="S455">
+        <v>4.952437675350702</v>
+      </c>
+      <c r="T455">
+        <v>280.19001</v>
+      </c>
+      <c r="U455">
+        <v>16</v>
+      </c>
+      <c r="V455">
+        <v>6</v>
+      </c>
+      <c r="W455">
+        <v>22</v>
+      </c>
+      <c r="X455">
+        <v>36</v>
+      </c>
+      <c r="Y455">
+        <v>16</v>
+      </c>
+      <c r="Z455">
+        <v>24</v>
+      </c>
+      <c r="AA455">
+        <v>6</v>
+      </c>
+      <c r="AB455">
+        <v>10</v>
+      </c>
+      <c r="AC455">
+        <v>4.45444</v>
+      </c>
+      <c r="AD455">
+        <v>-2.10833</v>
+      </c>
+      <c r="AE455">
+        <v>0</v>
+      </c>
+      <c r="AF455">
+        <v>274.6312</v>
+      </c>
+      <c r="AG455">
+        <v>0</v>
+      </c>
+      <c r="AH455">
+        <v>3</v>
+      </c>
+      <c r="AI455">
+        <v>1112.06988</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B456" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E456">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F456">
+        <v>2667.51</v>
+      </c>
+      <c r="G456">
+        <v>35.63807615230461</v>
+      </c>
+      <c r="H456">
+        <v>26.4</v>
+      </c>
+      <c r="I456">
+        <v>0</v>
+      </c>
+      <c r="J456">
+        <v>0</v>
+      </c>
+      <c r="K456">
+        <v>0.3527054108216433</v>
+      </c>
+      <c r="L456">
+        <v>0</v>
+      </c>
+      <c r="M456">
+        <v>0</v>
+      </c>
+      <c r="N456">
+        <v>0</v>
+      </c>
+      <c r="O456">
+        <v>23.52185</v>
+      </c>
+      <c r="P456">
+        <v>71.25242336120199</v>
+      </c>
+      <c r="Q456">
+        <v>33.012</v>
+      </c>
+      <c r="R456">
+        <v>255.17558</v>
+      </c>
+      <c r="S456">
+        <v>3.409159385437542</v>
+      </c>
+      <c r="T456">
+        <v>182.32999</v>
+      </c>
+      <c r="U456">
+        <v>8</v>
+      </c>
+      <c r="V456">
+        <v>2</v>
+      </c>
+      <c r="W456">
+        <v>10</v>
+      </c>
+      <c r="X456">
+        <v>22</v>
+      </c>
+      <c r="Y456">
+        <v>8</v>
+      </c>
+      <c r="Z456">
+        <v>17</v>
+      </c>
+      <c r="AA456">
+        <v>2</v>
+      </c>
+      <c r="AB456">
+        <v>12</v>
+      </c>
+      <c r="AC456">
+        <v>4.00379</v>
+      </c>
+      <c r="AD456">
+        <v>-2.03831</v>
+      </c>
+      <c r="AE456">
+        <v>0</v>
+      </c>
+      <c r="AF456">
+        <v>211.96875</v>
+      </c>
+      <c r="AG456">
+        <v>0</v>
+      </c>
+      <c r="AH456">
+        <v>3</v>
+      </c>
+      <c r="AI456">
+        <v>765.52674</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B457" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E457">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F457">
+        <v>3261.61</v>
+      </c>
+      <c r="G457">
+        <v>43.57528390113561</v>
+      </c>
+      <c r="H457">
+        <v>87.42</v>
+      </c>
+      <c r="I457">
+        <v>0</v>
+      </c>
+      <c r="J457">
+        <v>0</v>
+      </c>
+      <c r="K457">
+        <v>1.167935871743487</v>
+      </c>
+      <c r="L457">
+        <v>0</v>
+      </c>
+      <c r="M457">
+        <v>1</v>
+      </c>
+      <c r="N457">
+        <v>0</v>
+      </c>
+      <c r="O457">
+        <v>25.32642</v>
+      </c>
+      <c r="P457">
+        <v>79.13517060367454</v>
+      </c>
+      <c r="Q457">
+        <v>32.004</v>
+      </c>
+      <c r="R457">
+        <v>293.5775</v>
+      </c>
+      <c r="S457">
+        <v>3.922211088844355</v>
+      </c>
+      <c r="T457">
+        <v>303.73</v>
+      </c>
+      <c r="U457">
+        <v>10</v>
+      </c>
+      <c r="V457">
+        <v>5</v>
+      </c>
+      <c r="W457">
+        <v>15</v>
+      </c>
+      <c r="X457">
+        <v>34</v>
+      </c>
+      <c r="Y457">
+        <v>10</v>
+      </c>
+      <c r="Z457">
+        <v>27</v>
+      </c>
+      <c r="AA457">
+        <v>5</v>
+      </c>
+      <c r="AB457">
+        <v>20</v>
+      </c>
+      <c r="AC457">
+        <v>3.79198</v>
+      </c>
+      <c r="AD457">
+        <v>-2.3954</v>
+      </c>
+      <c r="AE457">
+        <v>0</v>
+      </c>
+      <c r="AF457">
+        <v>259.6755</v>
+      </c>
+      <c r="AG457">
+        <v>0</v>
+      </c>
+      <c r="AH457">
+        <v>3</v>
+      </c>
+      <c r="AI457">
+        <v>880.7325</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B458" s="2">
+        <v>46213</v>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Sesión 32</t>
+        </is>
+      </c>
+      <c r="E458">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="F458">
+        <v>3473.46</v>
+      </c>
+      <c r="G458">
+        <v>46.4056112224449</v>
+      </c>
+      <c r="H458">
+        <v>37.39</v>
+      </c>
+      <c r="I458">
+        <v>0</v>
+      </c>
+      <c r="J458">
+        <v>0</v>
+      </c>
+      <c r="K458">
+        <v>0.4995323981295925</v>
+      </c>
+      <c r="L458">
+        <v>0</v>
+      </c>
+      <c r="M458">
+        <v>0</v>
+      </c>
+      <c r="N458">
+        <v>0</v>
+      </c>
+      <c r="O458">
+        <v>22.2783</v>
+      </c>
+      <c r="P458">
+        <v>61.88416666666667</v>
+      </c>
+      <c r="Q458">
+        <v>36</v>
+      </c>
+      <c r="R458">
+        <v>374.9798</v>
+      </c>
+      <c r="S458">
+        <v>5.009750167000669</v>
+      </c>
+      <c r="T458">
+        <v>296.53001</v>
+      </c>
+      <c r="U458">
+        <v>18</v>
+      </c>
+      <c r="V458">
+        <v>12</v>
+      </c>
+      <c r="W458">
+        <v>30</v>
+      </c>
+      <c r="X458">
+        <v>35</v>
+      </c>
+      <c r="Y458">
+        <v>18</v>
+      </c>
+      <c r="Z458">
+        <v>31</v>
+      </c>
+      <c r="AA458">
+        <v>12</v>
+      </c>
+      <c r="AB458">
+        <v>26</v>
+      </c>
+      <c r="AC458">
+        <v>4.47432</v>
+      </c>
+      <c r="AD458">
+        <v>-2.94184</v>
+      </c>
+      <c r="AE458">
+        <v>0</v>
+      </c>
+      <c r="AF458">
+        <v>787.044</v>
+      </c>
+      <c r="AG458">
+        <v>0</v>
+      </c>
+      <c r="AH458">
+        <v>3</v>
+      </c>
+      <c r="AI458">
+        <v>1124.9394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-12
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI458"/>
+  <dimension ref="A1:AI477"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -52084,6 +52084,2153 @@
         <v>1124.9394</v>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B459" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E459">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F459">
+        <v>7942.88</v>
+      </c>
+      <c r="G459">
+        <v>76.07478932976615</v>
+      </c>
+      <c r="H459">
+        <v>73.33</v>
+      </c>
+      <c r="I459">
+        <v>0</v>
+      </c>
+      <c r="J459">
+        <v>0</v>
+      </c>
+      <c r="K459">
+        <v>0.7023352111012318</v>
+      </c>
+      <c r="L459">
+        <v>0</v>
+      </c>
+      <c r="M459">
+        <v>0</v>
+      </c>
+      <c r="N459">
+        <v>0</v>
+      </c>
+      <c r="O459">
+        <v>25.3284</v>
+      </c>
+      <c r="P459">
+        <v>70.35666666666667</v>
+      </c>
+      <c r="Q459">
+        <v>36</v>
+      </c>
+      <c r="R459">
+        <v>892.81537</v>
+      </c>
+      <c r="S459">
+        <v>8.551147843493446</v>
+      </c>
+      <c r="T459">
+        <v>997.64001</v>
+      </c>
+      <c r="U459">
+        <v>24</v>
+      </c>
+      <c r="V459">
+        <v>25</v>
+      </c>
+      <c r="W459">
+        <v>49</v>
+      </c>
+      <c r="X459">
+        <v>132</v>
+      </c>
+      <c r="Y459">
+        <v>24</v>
+      </c>
+      <c r="Z459">
+        <v>100</v>
+      </c>
+      <c r="AA459">
+        <v>25</v>
+      </c>
+      <c r="AB459">
+        <v>61</v>
+      </c>
+      <c r="AC459">
+        <v>4.15071</v>
+      </c>
+      <c r="AD459">
+        <v>-2.27408</v>
+      </c>
+      <c r="AE459">
+        <v>0</v>
+      </c>
+      <c r="AF459">
+        <v>1895.784</v>
+      </c>
+      <c r="AG459">
+        <v>0</v>
+      </c>
+      <c r="AH459">
+        <v>3</v>
+      </c>
+      <c r="AI459">
+        <v>2678.44611</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B460" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E460">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F460">
+        <v>12980.37</v>
+      </c>
+      <c r="G460">
+        <v>109.3697795253476</v>
+      </c>
+      <c r="H460">
+        <v>439.7500000000001</v>
+      </c>
+      <c r="I460">
+        <v>0</v>
+      </c>
+      <c r="J460">
+        <v>0</v>
+      </c>
+      <c r="K460">
+        <v>3.705238028366803</v>
+      </c>
+      <c r="L460">
+        <v>0</v>
+      </c>
+      <c r="M460">
+        <v>1</v>
+      </c>
+      <c r="N460">
+        <v>0</v>
+      </c>
+      <c r="O460">
+        <v>25.62451</v>
+      </c>
+      <c r="P460">
+        <v>79.17596712396491</v>
+      </c>
+      <c r="Q460">
+        <v>32.364</v>
+      </c>
+      <c r="R460">
+        <v>1288.44986</v>
+      </c>
+      <c r="S460">
+        <v>10.85619879230445</v>
+      </c>
+      <c r="T460">
+        <v>1910.85997</v>
+      </c>
+      <c r="U460">
+        <v>11</v>
+      </c>
+      <c r="V460">
+        <v>20</v>
+      </c>
+      <c r="W460">
+        <v>31</v>
+      </c>
+      <c r="X460">
+        <v>115</v>
+      </c>
+      <c r="Y460">
+        <v>11</v>
+      </c>
+      <c r="Z460">
+        <v>99</v>
+      </c>
+      <c r="AA460">
+        <v>20</v>
+      </c>
+      <c r="AB460">
+        <v>23</v>
+      </c>
+      <c r="AC460">
+        <v>4.04226</v>
+      </c>
+      <c r="AD460">
+        <v>-3.03067</v>
+      </c>
+      <c r="AE460">
+        <v>0</v>
+      </c>
+      <c r="AF460">
+        <v>1041.2675</v>
+      </c>
+      <c r="AG460">
+        <v>0</v>
+      </c>
+      <c r="AH460">
+        <v>3</v>
+      </c>
+      <c r="AI460">
+        <v>3865.34958</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B461" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E461">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F461">
+        <v>8245.290000000001</v>
+      </c>
+      <c r="G461">
+        <v>78.97119177336528</v>
+      </c>
+      <c r="H461">
+        <v>64.61</v>
+      </c>
+      <c r="I461">
+        <v>0</v>
+      </c>
+      <c r="J461">
+        <v>0</v>
+      </c>
+      <c r="K461">
+        <v>0.6188173733703884</v>
+      </c>
+      <c r="L461">
+        <v>0</v>
+      </c>
+      <c r="M461">
+        <v>0</v>
+      </c>
+      <c r="N461">
+        <v>0</v>
+      </c>
+      <c r="O461">
+        <v>22.37046</v>
+      </c>
+      <c r="P461">
+        <v>62.14016666666667</v>
+      </c>
+      <c r="Q461">
+        <v>36</v>
+      </c>
+      <c r="R461">
+        <v>758.64987</v>
+      </c>
+      <c r="S461">
+        <v>7.266146414814837</v>
+      </c>
+      <c r="T461">
+        <v>1022.57999</v>
+      </c>
+      <c r="U461">
+        <v>30</v>
+      </c>
+      <c r="V461">
+        <v>29</v>
+      </c>
+      <c r="W461">
+        <v>59</v>
+      </c>
+      <c r="X461">
+        <v>146</v>
+      </c>
+      <c r="Y461">
+        <v>30</v>
+      </c>
+      <c r="Z461">
+        <v>124</v>
+      </c>
+      <c r="AA461">
+        <v>29</v>
+      </c>
+      <c r="AB461">
+        <v>53</v>
+      </c>
+      <c r="AC461">
+        <v>3.91401</v>
+      </c>
+      <c r="AD461">
+        <v>-2.29752</v>
+      </c>
+      <c r="AE461">
+        <v>0</v>
+      </c>
+      <c r="AF461">
+        <v>1965.396</v>
+      </c>
+      <c r="AG461">
+        <v>0</v>
+      </c>
+      <c r="AH461">
+        <v>3</v>
+      </c>
+      <c r="AI461">
+        <v>2275.94961</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B462" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E462">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F462">
+        <v>8814.34</v>
+      </c>
+      <c r="G462">
+        <v>74.26771520853812</v>
+      </c>
+      <c r="H462">
+        <v>630.7499999999999</v>
+      </c>
+      <c r="I462">
+        <v>0</v>
+      </c>
+      <c r="J462">
+        <v>0</v>
+      </c>
+      <c r="K462">
+        <v>5.314562561437999</v>
+      </c>
+      <c r="L462">
+        <v>0</v>
+      </c>
+      <c r="M462">
+        <v>6</v>
+      </c>
+      <c r="N462">
+        <v>0</v>
+      </c>
+      <c r="O462">
+        <v>27.87634</v>
+      </c>
+      <c r="P462">
+        <v>86.03808641975309</v>
+      </c>
+      <c r="Q462">
+        <v>32.4</v>
+      </c>
+      <c r="R462">
+        <v>1003.62671</v>
+      </c>
+      <c r="S462">
+        <v>8.456340766746242</v>
+      </c>
+      <c r="T462">
+        <v>2026.33995</v>
+      </c>
+      <c r="U462">
+        <v>40</v>
+      </c>
+      <c r="V462">
+        <v>34</v>
+      </c>
+      <c r="W462">
+        <v>74</v>
+      </c>
+      <c r="X462">
+        <v>150</v>
+      </c>
+      <c r="Y462">
+        <v>40</v>
+      </c>
+      <c r="Z462">
+        <v>133</v>
+      </c>
+      <c r="AA462">
+        <v>34</v>
+      </c>
+      <c r="AB462">
+        <v>15</v>
+      </c>
+      <c r="AC462">
+        <v>4.0885</v>
+      </c>
+      <c r="AD462">
+        <v>-4.01393</v>
+      </c>
+      <c r="AE462">
+        <v>0</v>
+      </c>
+      <c r="AF462">
+        <v>752.0296</v>
+      </c>
+      <c r="AG462">
+        <v>0</v>
+      </c>
+      <c r="AH462">
+        <v>3</v>
+      </c>
+      <c r="AI462">
+        <v>3010.88013</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B463" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E463">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F463">
+        <v>11041.99</v>
+      </c>
+      <c r="G463">
+        <v>93.03741047605673</v>
+      </c>
+      <c r="H463">
+        <v>575.87</v>
+      </c>
+      <c r="I463">
+        <v>0</v>
+      </c>
+      <c r="J463">
+        <v>0</v>
+      </c>
+      <c r="K463">
+        <v>4.85215559612414</v>
+      </c>
+      <c r="L463">
+        <v>0</v>
+      </c>
+      <c r="M463">
+        <v>13</v>
+      </c>
+      <c r="N463">
+        <v>0</v>
+      </c>
+      <c r="O463">
+        <v>29.52918</v>
+      </c>
+      <c r="P463">
+        <v>86.89141949152543</v>
+      </c>
+      <c r="Q463">
+        <v>33.984</v>
+      </c>
+      <c r="R463">
+        <v>1232.02074</v>
+      </c>
+      <c r="S463">
+        <v>10.38073927819126</v>
+      </c>
+      <c r="T463">
+        <v>1786.97001</v>
+      </c>
+      <c r="U463">
+        <v>30</v>
+      </c>
+      <c r="V463">
+        <v>37</v>
+      </c>
+      <c r="W463">
+        <v>67</v>
+      </c>
+      <c r="X463">
+        <v>130</v>
+      </c>
+      <c r="Y463">
+        <v>30</v>
+      </c>
+      <c r="Z463">
+        <v>135</v>
+      </c>
+      <c r="AA463">
+        <v>37</v>
+      </c>
+      <c r="AB463">
+        <v>23</v>
+      </c>
+      <c r="AC463">
+        <v>4.58103</v>
+      </c>
+      <c r="AD463">
+        <v>-3.19621</v>
+      </c>
+      <c r="AE463">
+        <v>0</v>
+      </c>
+      <c r="AF463">
+        <v>1047.504</v>
+      </c>
+      <c r="AG463">
+        <v>0</v>
+      </c>
+      <c r="AH463">
+        <v>3</v>
+      </c>
+      <c r="AI463">
+        <v>3696.06222</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B464" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E464">
+        <v>144.1088333333333</v>
+      </c>
+      <c r="F464">
+        <v>10557.06</v>
+      </c>
+      <c r="G464">
+        <v>73.25754956034386</v>
+      </c>
+      <c r="H464">
+        <v>393.02</v>
+      </c>
+      <c r="I464">
+        <v>0</v>
+      </c>
+      <c r="J464">
+        <v>0</v>
+      </c>
+      <c r="K464">
+        <v>2.727244339636825</v>
+      </c>
+      <c r="L464">
+        <v>17</v>
+      </c>
+      <c r="M464">
+        <v>13</v>
+      </c>
+      <c r="N464">
+        <v>2</v>
+      </c>
+      <c r="O464">
+        <v>31.36679</v>
+      </c>
+      <c r="P464">
+        <v>88.18823099415206</v>
+      </c>
+      <c r="Q464">
+        <v>35.568</v>
+      </c>
+      <c r="R464">
+        <v>974.85178</v>
+      </c>
+      <c r="S464">
+        <v>6.76469136173702</v>
+      </c>
+      <c r="T464">
+        <v>1286.53002</v>
+      </c>
+      <c r="U464">
+        <v>29</v>
+      </c>
+      <c r="V464">
+        <v>21</v>
+      </c>
+      <c r="W464">
+        <v>50</v>
+      </c>
+      <c r="X464">
+        <v>135</v>
+      </c>
+      <c r="Y464">
+        <v>29</v>
+      </c>
+      <c r="Z464">
+        <v>84</v>
+      </c>
+      <c r="AA464">
+        <v>21</v>
+      </c>
+      <c r="AB464">
+        <v>25</v>
+      </c>
+      <c r="AC464">
+        <v>4.24526</v>
+      </c>
+      <c r="AD464">
+        <v>-2.34237</v>
+      </c>
+      <c r="AE464">
+        <v>0</v>
+      </c>
+      <c r="AF464">
+        <v>984.1968000000001</v>
+      </c>
+      <c r="AG464">
+        <v>0</v>
+      </c>
+      <c r="AH464">
+        <v>3</v>
+      </c>
+      <c r="AI464">
+        <v>2924.55534</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B465" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E465">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F465">
+        <v>8401.360000000001</v>
+      </c>
+      <c r="G465">
+        <v>80.46598866954105</v>
+      </c>
+      <c r="H465">
+        <v>269.33</v>
+      </c>
+      <c r="I465">
+        <v>0</v>
+      </c>
+      <c r="J465">
+        <v>0</v>
+      </c>
+      <c r="K465">
+        <v>2.579571013308261</v>
+      </c>
+      <c r="L465">
+        <v>0</v>
+      </c>
+      <c r="M465">
+        <v>0</v>
+      </c>
+      <c r="N465">
+        <v>0</v>
+      </c>
+      <c r="O465">
+        <v>24.34747</v>
+      </c>
+      <c r="P465">
+        <v>67.63186111111111</v>
+      </c>
+      <c r="Q465">
+        <v>36</v>
+      </c>
+      <c r="R465">
+        <v>911.1489799999999</v>
+      </c>
+      <c r="S465">
+        <v>8.726742277553143</v>
+      </c>
+      <c r="T465">
+        <v>1145.07</v>
+      </c>
+      <c r="U465">
+        <v>10</v>
+      </c>
+      <c r="V465">
+        <v>11</v>
+      </c>
+      <c r="W465">
+        <v>21</v>
+      </c>
+      <c r="X465">
+        <v>100</v>
+      </c>
+      <c r="Y465">
+        <v>10</v>
+      </c>
+      <c r="Z465">
+        <v>87</v>
+      </c>
+      <c r="AA465">
+        <v>11</v>
+      </c>
+      <c r="AB465">
+        <v>25</v>
+      </c>
+      <c r="AC465">
+        <v>3.61633</v>
+      </c>
+      <c r="AD465">
+        <v>-1.89127</v>
+      </c>
+      <c r="AE465">
+        <v>0</v>
+      </c>
+      <c r="AF465">
+        <v>1939.15</v>
+      </c>
+      <c r="AG465">
+        <v>0</v>
+      </c>
+      <c r="AH465">
+        <v>3</v>
+      </c>
+      <c r="AI465">
+        <v>2733.44694</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B466" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E466">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F466">
+        <v>9166.880000000001</v>
+      </c>
+      <c r="G466">
+        <v>87.79793535987535</v>
+      </c>
+      <c r="H466">
+        <v>561.55</v>
+      </c>
+      <c r="I466">
+        <v>0</v>
+      </c>
+      <c r="J466">
+        <v>0</v>
+      </c>
+      <c r="K466">
+        <v>5.378376350659985</v>
+      </c>
+      <c r="L466">
+        <v>0</v>
+      </c>
+      <c r="M466">
+        <v>2</v>
+      </c>
+      <c r="N466">
+        <v>0</v>
+      </c>
+      <c r="O466">
+        <v>26.10913</v>
+      </c>
+      <c r="P466">
+        <v>72.52536111111111</v>
+      </c>
+      <c r="Q466">
+        <v>36</v>
+      </c>
+      <c r="R466">
+        <v>942.98865</v>
+      </c>
+      <c r="S466">
+        <v>9.031694157422821</v>
+      </c>
+      <c r="T466">
+        <v>1737.96997</v>
+      </c>
+      <c r="U466">
+        <v>45</v>
+      </c>
+      <c r="V466">
+        <v>42</v>
+      </c>
+      <c r="W466">
+        <v>87</v>
+      </c>
+      <c r="X466">
+        <v>164</v>
+      </c>
+      <c r="Y466">
+        <v>45</v>
+      </c>
+      <c r="Z466">
+        <v>127</v>
+      </c>
+      <c r="AA466">
+        <v>42</v>
+      </c>
+      <c r="AB466">
+        <v>68</v>
+      </c>
+      <c r="AC466">
+        <v>4.39973</v>
+      </c>
+      <c r="AD466">
+        <v>-2.28985</v>
+      </c>
+      <c r="AE466">
+        <v>0</v>
+      </c>
+      <c r="AF466">
+        <v>770.5243</v>
+      </c>
+      <c r="AG466">
+        <v>0</v>
+      </c>
+      <c r="AH466">
+        <v>3</v>
+      </c>
+      <c r="AI466">
+        <v>2828.96595</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B467" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E467">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F467">
+        <v>12147.03</v>
+      </c>
+      <c r="G467">
+        <v>102.3482376070776</v>
+      </c>
+      <c r="H467">
+        <v>679.13</v>
+      </c>
+      <c r="I467">
+        <v>24.19</v>
+      </c>
+      <c r="J467">
+        <v>2</v>
+      </c>
+      <c r="K467">
+        <v>5.722201937930066</v>
+      </c>
+      <c r="L467">
+        <v>6.54</v>
+      </c>
+      <c r="M467">
+        <v>13</v>
+      </c>
+      <c r="N467">
+        <v>1</v>
+      </c>
+      <c r="O467">
+        <v>30.36054</v>
+      </c>
+      <c r="P467">
+        <v>94.86482939632546</v>
+      </c>
+      <c r="Q467">
+        <v>32.004</v>
+      </c>
+      <c r="R467">
+        <v>1401.87338</v>
+      </c>
+      <c r="S467">
+        <v>11.81188074708608</v>
+      </c>
+      <c r="T467">
+        <v>2002.32997</v>
+      </c>
+      <c r="U467">
+        <v>24</v>
+      </c>
+      <c r="V467">
+        <v>37</v>
+      </c>
+      <c r="W467">
+        <v>61</v>
+      </c>
+      <c r="X467">
+        <v>121</v>
+      </c>
+      <c r="Y467">
+        <v>24</v>
+      </c>
+      <c r="Z467">
+        <v>133</v>
+      </c>
+      <c r="AA467">
+        <v>37</v>
+      </c>
+      <c r="AB467">
+        <v>27</v>
+      </c>
+      <c r="AC467">
+        <v>4.29716</v>
+      </c>
+      <c r="AD467">
+        <v>-3.4452</v>
+      </c>
+      <c r="AE467">
+        <v>0</v>
+      </c>
+      <c r="AF467">
+        <v>853.2570000000001</v>
+      </c>
+      <c r="AG467">
+        <v>0</v>
+      </c>
+      <c r="AH467">
+        <v>3</v>
+      </c>
+      <c r="AI467">
+        <v>4205.62014</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B468" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E468">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F468">
+        <v>11274.05</v>
+      </c>
+      <c r="G468">
+        <v>94.99269765482376</v>
+      </c>
+      <c r="H468">
+        <v>401.57</v>
+      </c>
+      <c r="I468">
+        <v>0</v>
+      </c>
+      <c r="J468">
+        <v>0</v>
+      </c>
+      <c r="K468">
+        <v>3.383541637410476</v>
+      </c>
+      <c r="L468">
+        <v>0</v>
+      </c>
+      <c r="M468">
+        <v>8</v>
+      </c>
+      <c r="N468">
+        <v>0</v>
+      </c>
+      <c r="O468">
+        <v>27.24657</v>
+      </c>
+      <c r="P468">
+        <v>80.8599537037037</v>
+      </c>
+      <c r="Q468">
+        <v>33.696</v>
+      </c>
+      <c r="R468">
+        <v>1266.27814</v>
+      </c>
+      <c r="S468">
+        <v>10.66938469316107</v>
+      </c>
+      <c r="T468">
+        <v>1777.72999</v>
+      </c>
+      <c r="U468">
+        <v>53</v>
+      </c>
+      <c r="V468">
+        <v>43</v>
+      </c>
+      <c r="W468">
+        <v>96</v>
+      </c>
+      <c r="X468">
+        <v>199</v>
+      </c>
+      <c r="Y468">
+        <v>53</v>
+      </c>
+      <c r="Z468">
+        <v>138</v>
+      </c>
+      <c r="AA468">
+        <v>43</v>
+      </c>
+      <c r="AB468">
+        <v>67</v>
+      </c>
+      <c r="AC468">
+        <v>4.56239</v>
+      </c>
+      <c r="AD468">
+        <v>-3.34035</v>
+      </c>
+      <c r="AE468">
+        <v>0</v>
+      </c>
+      <c r="AF468">
+        <v>1086.4512</v>
+      </c>
+      <c r="AG468">
+        <v>0</v>
+      </c>
+      <c r="AH468">
+        <v>3</v>
+      </c>
+      <c r="AI468">
+        <v>3798.83442</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B469" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E469">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F469">
+        <v>12573.11</v>
+      </c>
+      <c r="G469">
+        <v>105.9382951832608</v>
+      </c>
+      <c r="H469">
+        <v>593.35</v>
+      </c>
+      <c r="I469">
+        <v>0</v>
+      </c>
+      <c r="J469">
+        <v>0</v>
+      </c>
+      <c r="K469">
+        <v>4.999438281140289</v>
+      </c>
+      <c r="L469">
+        <v>0</v>
+      </c>
+      <c r="M469">
+        <v>12</v>
+      </c>
+      <c r="N469">
+        <v>0</v>
+      </c>
+      <c r="O469">
+        <v>29.69944</v>
+      </c>
+      <c r="P469">
+        <v>84.87494284407865</v>
+      </c>
+      <c r="Q469">
+        <v>34.992</v>
+      </c>
+      <c r="R469">
+        <v>1060.24183</v>
+      </c>
+      <c r="S469">
+        <v>8.933367476478022</v>
+      </c>
+      <c r="T469">
+        <v>1760.26001</v>
+      </c>
+      <c r="U469">
+        <v>27</v>
+      </c>
+      <c r="V469">
+        <v>37</v>
+      </c>
+      <c r="W469">
+        <v>64</v>
+      </c>
+      <c r="X469">
+        <v>115</v>
+      </c>
+      <c r="Y469">
+        <v>27</v>
+      </c>
+      <c r="Z469">
+        <v>112</v>
+      </c>
+      <c r="AA469">
+        <v>37</v>
+      </c>
+      <c r="AB469">
+        <v>19</v>
+      </c>
+      <c r="AC469">
+        <v>4.79161</v>
+      </c>
+      <c r="AD469">
+        <v>-3.49002</v>
+      </c>
+      <c r="AE469">
+        <v>0</v>
+      </c>
+      <c r="AF469">
+        <v>1005.56874</v>
+      </c>
+      <c r="AG469">
+        <v>0</v>
+      </c>
+      <c r="AH469">
+        <v>3</v>
+      </c>
+      <c r="AI469">
+        <v>3180.72549</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B470" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E470">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F470">
+        <v>7898.55</v>
+      </c>
+      <c r="G470">
+        <v>75.65020839552209</v>
+      </c>
+      <c r="H470">
+        <v>30.33</v>
+      </c>
+      <c r="I470">
+        <v>0</v>
+      </c>
+      <c r="J470">
+        <v>0</v>
+      </c>
+      <c r="K470">
+        <v>0.290492662657853</v>
+      </c>
+      <c r="L470">
+        <v>0</v>
+      </c>
+      <c r="M470">
+        <v>1</v>
+      </c>
+      <c r="N470">
+        <v>0</v>
+      </c>
+      <c r="O470">
+        <v>26.04056</v>
+      </c>
+      <c r="P470">
+        <v>74.57205040091638</v>
+      </c>
+      <c r="Q470">
+        <v>34.92</v>
+      </c>
+      <c r="R470">
+        <v>753.73544</v>
+      </c>
+      <c r="S470">
+        <v>7.219077313062591</v>
+      </c>
+      <c r="T470">
+        <v>868.2500200000001</v>
+      </c>
+      <c r="U470">
+        <v>29</v>
+      </c>
+      <c r="V470">
+        <v>11</v>
+      </c>
+      <c r="W470">
+        <v>40</v>
+      </c>
+      <c r="X470">
+        <v>150</v>
+      </c>
+      <c r="Y470">
+        <v>29</v>
+      </c>
+      <c r="Z470">
+        <v>90</v>
+      </c>
+      <c r="AA470">
+        <v>11</v>
+      </c>
+      <c r="AB470">
+        <v>17</v>
+      </c>
+      <c r="AC470">
+        <v>4.216</v>
+      </c>
+      <c r="AD470">
+        <v>-1.95547</v>
+      </c>
+      <c r="AE470">
+        <v>0</v>
+      </c>
+      <c r="AF470">
+        <v>738.1688</v>
+      </c>
+      <c r="AG470">
+        <v>0</v>
+      </c>
+      <c r="AH470">
+        <v>3</v>
+      </c>
+      <c r="AI470">
+        <v>2261.20632</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B471" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E471">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F471">
+        <v>12563.19</v>
+      </c>
+      <c r="G471">
+        <v>105.8547114169358</v>
+      </c>
+      <c r="H471">
+        <v>923.25</v>
+      </c>
+      <c r="I471">
+        <v>0</v>
+      </c>
+      <c r="J471">
+        <v>0</v>
+      </c>
+      <c r="K471">
+        <v>7.779104058418761</v>
+      </c>
+      <c r="L471">
+        <v>14.05</v>
+      </c>
+      <c r="M471">
+        <v>19</v>
+      </c>
+      <c r="N471">
+        <v>1</v>
+      </c>
+      <c r="O471">
+        <v>31.06503</v>
+      </c>
+      <c r="P471">
+        <v>88.77752057613169</v>
+      </c>
+      <c r="Q471">
+        <v>34.992</v>
+      </c>
+      <c r="R471">
+        <v>1031.73775</v>
+      </c>
+      <c r="S471">
+        <v>8.693198286757477</v>
+      </c>
+      <c r="T471">
+        <v>2432.64001</v>
+      </c>
+      <c r="U471">
+        <v>42</v>
+      </c>
+      <c r="V471">
+        <v>74</v>
+      </c>
+      <c r="W471">
+        <v>116</v>
+      </c>
+      <c r="X471">
+        <v>156</v>
+      </c>
+      <c r="Y471">
+        <v>42</v>
+      </c>
+      <c r="Z471">
+        <v>169</v>
+      </c>
+      <c r="AA471">
+        <v>74</v>
+      </c>
+      <c r="AB471">
+        <v>31</v>
+      </c>
+      <c r="AC471">
+        <v>4.84929</v>
+      </c>
+      <c r="AD471">
+        <v>-3.66417</v>
+      </c>
+      <c r="AE471">
+        <v>0</v>
+      </c>
+      <c r="AF471">
+        <v>1079.50956</v>
+      </c>
+      <c r="AG471">
+        <v>0</v>
+      </c>
+      <c r="AH471">
+        <v>3</v>
+      </c>
+      <c r="AI471">
+        <v>3095.21325</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B472" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E472">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F472">
+        <v>8535.220000000001</v>
+      </c>
+      <c r="G472">
+        <v>81.74806410057897</v>
+      </c>
+      <c r="H472">
+        <v>81.41000000000001</v>
+      </c>
+      <c r="I472">
+        <v>0</v>
+      </c>
+      <c r="J472">
+        <v>0</v>
+      </c>
+      <c r="K472">
+        <v>0.7797232992738482</v>
+      </c>
+      <c r="L472">
+        <v>0</v>
+      </c>
+      <c r="M472">
+        <v>0</v>
+      </c>
+      <c r="N472">
+        <v>0</v>
+      </c>
+      <c r="O472">
+        <v>22.43857</v>
+      </c>
+      <c r="P472">
+        <v>62.3293611111111</v>
+      </c>
+      <c r="Q472">
+        <v>36</v>
+      </c>
+      <c r="R472">
+        <v>961.49793</v>
+      </c>
+      <c r="S472">
+        <v>9.208971111958917</v>
+      </c>
+      <c r="T472">
+        <v>1062.57997</v>
+      </c>
+      <c r="U472">
+        <v>19</v>
+      </c>
+      <c r="V472">
+        <v>31</v>
+      </c>
+      <c r="W472">
+        <v>50</v>
+      </c>
+      <c r="X472">
+        <v>124</v>
+      </c>
+      <c r="Y472">
+        <v>19</v>
+      </c>
+      <c r="Z472">
+        <v>127</v>
+      </c>
+      <c r="AA472">
+        <v>31</v>
+      </c>
+      <c r="AB472">
+        <v>42</v>
+      </c>
+      <c r="AC472">
+        <v>4.30444</v>
+      </c>
+      <c r="AD472">
+        <v>-2.02548</v>
+      </c>
+      <c r="AE472">
+        <v>0</v>
+      </c>
+      <c r="AF472">
+        <v>2015.572</v>
+      </c>
+      <c r="AG472">
+        <v>0</v>
+      </c>
+      <c r="AH472">
+        <v>3</v>
+      </c>
+      <c r="AI472">
+        <v>2884.49379</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B473" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E473">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F473">
+        <v>11508.15</v>
+      </c>
+      <c r="G473">
+        <v>96.96517343069794</v>
+      </c>
+      <c r="H473">
+        <v>399.68</v>
+      </c>
+      <c r="I473">
+        <v>7.58</v>
+      </c>
+      <c r="J473">
+        <v>1</v>
+      </c>
+      <c r="K473">
+        <v>3.367616907737677</v>
+      </c>
+      <c r="L473">
+        <v>12.38</v>
+      </c>
+      <c r="M473">
+        <v>8</v>
+      </c>
+      <c r="N473">
+        <v>1</v>
+      </c>
+      <c r="O473">
+        <v>30.85562</v>
+      </c>
+      <c r="P473">
+        <v>90.79455037664782</v>
+      </c>
+      <c r="Q473">
+        <v>33.984</v>
+      </c>
+      <c r="R473">
+        <v>1148.67422</v>
+      </c>
+      <c r="S473">
+        <v>9.678479595562422</v>
+      </c>
+      <c r="T473">
+        <v>1610.31998</v>
+      </c>
+      <c r="U473">
+        <v>25</v>
+      </c>
+      <c r="V473">
+        <v>37</v>
+      </c>
+      <c r="W473">
+        <v>62</v>
+      </c>
+      <c r="X473">
+        <v>122</v>
+      </c>
+      <c r="Y473">
+        <v>25</v>
+      </c>
+      <c r="Z473">
+        <v>135</v>
+      </c>
+      <c r="AA473">
+        <v>37</v>
+      </c>
+      <c r="AB473">
+        <v>41</v>
+      </c>
+      <c r="AC473">
+        <v>4.34152</v>
+      </c>
+      <c r="AD473">
+        <v>-2.79458</v>
+      </c>
+      <c r="AE473">
+        <v>0</v>
+      </c>
+      <c r="AF473">
+        <v>1080.0624</v>
+      </c>
+      <c r="AG473">
+        <v>0</v>
+      </c>
+      <c r="AH473">
+        <v>3</v>
+      </c>
+      <c r="AI473">
+        <v>3446.022660000001</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B474" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E474">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F474">
+        <v>8115.679999999999</v>
+      </c>
+      <c r="G474">
+        <v>77.72982171048744</v>
+      </c>
+      <c r="H474">
+        <v>88.55</v>
+      </c>
+      <c r="I474">
+        <v>0</v>
+      </c>
+      <c r="J474">
+        <v>0</v>
+      </c>
+      <c r="K474">
+        <v>0.8481083177828184</v>
+      </c>
+      <c r="L474">
+        <v>0</v>
+      </c>
+      <c r="M474">
+        <v>0</v>
+      </c>
+      <c r="N474">
+        <v>0</v>
+      </c>
+      <c r="O474">
+        <v>24.55806</v>
+      </c>
+      <c r="P474">
+        <v>70.18192729766804</v>
+      </c>
+      <c r="Q474">
+        <v>34.992</v>
+      </c>
+      <c r="R474">
+        <v>779.8107699999999</v>
+      </c>
+      <c r="S474">
+        <v>7.468819879544034</v>
+      </c>
+      <c r="T474">
+        <v>1096.76</v>
+      </c>
+      <c r="U474">
+        <v>22</v>
+      </c>
+      <c r="V474">
+        <v>17</v>
+      </c>
+      <c r="W474">
+        <v>39</v>
+      </c>
+      <c r="X474">
+        <v>128</v>
+      </c>
+      <c r="Y474">
+        <v>22</v>
+      </c>
+      <c r="Z474">
+        <v>100</v>
+      </c>
+      <c r="AA474">
+        <v>17</v>
+      </c>
+      <c r="AB474">
+        <v>38</v>
+      </c>
+      <c r="AC474">
+        <v>3.60185</v>
+      </c>
+      <c r="AD474">
+        <v>-2.02401</v>
+      </c>
+      <c r="AE474">
+        <v>0</v>
+      </c>
+      <c r="AF474">
+        <v>764.7791999999999</v>
+      </c>
+      <c r="AG474">
+        <v>0</v>
+      </c>
+      <c r="AH474">
+        <v>3</v>
+      </c>
+      <c r="AI474">
+        <v>2339.43231</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B475" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E475">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F475">
+        <v>11277.12</v>
+      </c>
+      <c r="G475">
+        <v>95.01856480831344</v>
+      </c>
+      <c r="H475">
+        <v>586.1899999999999</v>
+      </c>
+      <c r="I475">
+        <v>14.18</v>
+      </c>
+      <c r="J475">
+        <v>1</v>
+      </c>
+      <c r="K475">
+        <v>4.939109675607358</v>
+      </c>
+      <c r="L475">
+        <v>14.18</v>
+      </c>
+      <c r="M475">
+        <v>11</v>
+      </c>
+      <c r="N475">
+        <v>1</v>
+      </c>
+      <c r="O475">
+        <v>30.54833</v>
+      </c>
+      <c r="P475">
+        <v>92.53704713437537</v>
+      </c>
+      <c r="Q475">
+        <v>33.012</v>
+      </c>
+      <c r="R475">
+        <v>1015.18162</v>
+      </c>
+      <c r="S475">
+        <v>8.553699929785141</v>
+      </c>
+      <c r="T475">
+        <v>1757.73005</v>
+      </c>
+      <c r="U475">
+        <v>26</v>
+      </c>
+      <c r="V475">
+        <v>32</v>
+      </c>
+      <c r="W475">
+        <v>58</v>
+      </c>
+      <c r="X475">
+        <v>147</v>
+      </c>
+      <c r="Y475">
+        <v>26</v>
+      </c>
+      <c r="Z475">
+        <v>120</v>
+      </c>
+      <c r="AA475">
+        <v>32</v>
+      </c>
+      <c r="AB475">
+        <v>30</v>
+      </c>
+      <c r="AC475">
+        <v>4.21731</v>
+      </c>
+      <c r="AD475">
+        <v>-2.79208</v>
+      </c>
+      <c r="AE475">
+        <v>0</v>
+      </c>
+      <c r="AF475">
+        <v>991.6515000000001</v>
+      </c>
+      <c r="AG475">
+        <v>0</v>
+      </c>
+      <c r="AH475">
+        <v>3</v>
+      </c>
+      <c r="AI475">
+        <v>3045.54486</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B476" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy</t>
+        </is>
+      </c>
+      <c r="E476">
+        <v>118.6833333333333</v>
+      </c>
+      <c r="F476">
+        <v>12579.97</v>
+      </c>
+      <c r="G476">
+        <v>105.996096053925</v>
+      </c>
+      <c r="H476">
+        <v>655.37</v>
+      </c>
+      <c r="I476">
+        <v>0</v>
+      </c>
+      <c r="J476">
+        <v>0</v>
+      </c>
+      <c r="K476">
+        <v>5.522005336329167</v>
+      </c>
+      <c r="L476">
+        <v>0</v>
+      </c>
+      <c r="M476">
+        <v>13</v>
+      </c>
+      <c r="N476">
+        <v>0</v>
+      </c>
+      <c r="O476">
+        <v>28.33243</v>
+      </c>
+      <c r="P476">
+        <v>88.52777777777779</v>
+      </c>
+      <c r="Q476">
+        <v>32.004</v>
+      </c>
+      <c r="R476">
+        <v>1159.66443</v>
+      </c>
+      <c r="S476">
+        <v>9.771080719000139</v>
+      </c>
+      <c r="T476">
+        <v>1902.56003</v>
+      </c>
+      <c r="U476">
+        <v>31</v>
+      </c>
+      <c r="V476">
+        <v>31</v>
+      </c>
+      <c r="W476">
+        <v>62</v>
+      </c>
+      <c r="X476">
+        <v>124</v>
+      </c>
+      <c r="Y476">
+        <v>31</v>
+      </c>
+      <c r="Z476">
+        <v>112</v>
+      </c>
+      <c r="AA476">
+        <v>31</v>
+      </c>
+      <c r="AB476">
+        <v>28</v>
+      </c>
+      <c r="AC476">
+        <v>4.40798</v>
+      </c>
+      <c r="AD476">
+        <v>-4.40101</v>
+      </c>
+      <c r="AE476">
+        <v>0</v>
+      </c>
+      <c r="AF476">
+        <v>1030.3678</v>
+      </c>
+      <c r="AG476">
+        <v>0</v>
+      </c>
+      <c r="AH476">
+        <v>3</v>
+      </c>
+      <c r="AI476">
+        <v>3478.993289999999</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B477" s="2">
+        <v>46214</v>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Amistoso vs Galaxy | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E477">
+        <v>104.4088333333333</v>
+      </c>
+      <c r="F477">
+        <v>9010.610000000001</v>
+      </c>
+      <c r="G477">
+        <v>86.30122291696264</v>
+      </c>
+      <c r="H477">
+        <v>15.35</v>
+      </c>
+      <c r="I477">
+        <v>0</v>
+      </c>
+      <c r="J477">
+        <v>0</v>
+      </c>
+      <c r="K477">
+        <v>0.1470182120606015</v>
+      </c>
+      <c r="L477">
+        <v>0</v>
+      </c>
+      <c r="M477">
+        <v>0</v>
+      </c>
+      <c r="N477">
+        <v>0</v>
+      </c>
+      <c r="O477">
+        <v>21.82094</v>
+      </c>
+      <c r="P477">
+        <v>60.61372222222222</v>
+      </c>
+      <c r="Q477">
+        <v>36</v>
+      </c>
+      <c r="R477">
+        <v>960.22336</v>
+      </c>
+      <c r="S477">
+        <v>9.19676361993637</v>
+      </c>
+      <c r="T477">
+        <v>1266.61</v>
+      </c>
+      <c r="U477">
+        <v>32</v>
+      </c>
+      <c r="V477">
+        <v>47</v>
+      </c>
+      <c r="W477">
+        <v>79</v>
+      </c>
+      <c r="X477">
+        <v>155</v>
+      </c>
+      <c r="Y477">
+        <v>32</v>
+      </c>
+      <c r="Z477">
+        <v>171</v>
+      </c>
+      <c r="AA477">
+        <v>47</v>
+      </c>
+      <c r="AB477">
+        <v>48</v>
+      </c>
+      <c r="AC477">
+        <v>3.89166</v>
+      </c>
+      <c r="AD477">
+        <v>-1.92672</v>
+      </c>
+      <c r="AE477">
+        <v>0</v>
+      </c>
+      <c r="AF477">
+        <v>2174.482</v>
+      </c>
+      <c r="AG477">
+        <v>0</v>
+      </c>
+      <c r="AH477">
+        <v>3</v>
+      </c>
+      <c r="AI477">
+        <v>2880.67008</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-14
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -1779,10 +1779,10 @@
         <v>142.3</v>
       </c>
       <c r="F13">
-        <v>8256.340000000002</v>
+        <v>8256.34</v>
       </c>
       <c r="G13">
-        <v>58.02066057624737</v>
+        <v>58.02066057624736</v>
       </c>
       <c r="H13">
         <v>499.06</v>
@@ -1815,10 +1815,10 @@
         <v>33.84</v>
       </c>
       <c r="R13">
-        <v>871.5351299999999</v>
+        <v>871.53513</v>
       </c>
       <c r="S13">
-        <v>6.124631974701334</v>
+        <v>6.124631974701335</v>
       </c>
       <c r="T13">
         <v>1096.84001</v>
@@ -3248,10 +3248,10 @@
         <v>114.4713333333333</v>
       </c>
       <c r="F26">
-        <v>8536.459999999997</v>
+        <v>8536.459999999999</v>
       </c>
       <c r="G26">
-        <v>74.57290617155967</v>
+        <v>74.57290617155968</v>
       </c>
       <c r="H26">
         <v>176.52</v>
@@ -3480,7 +3480,7 @@
         <v>62.29918508342559</v>
       </c>
       <c r="H28">
-        <v>84.63999999999999</v>
+        <v>84.64</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -3489,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="K28">
-        <v>0.6773277138322418</v>
+        <v>0.6773277138322419</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -3510,10 +3510,10 @@
         <v>33.984</v>
       </c>
       <c r="R28">
-        <v>965.6688100000001</v>
+        <v>965.66881</v>
       </c>
       <c r="S28">
-        <v>7.727720314229699</v>
+        <v>7.727720314229698</v>
       </c>
       <c r="T28">
         <v>1013.94</v>
@@ -3700,10 +3700,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F30">
-        <v>9359.540000000001</v>
+        <v>9359.539999999999</v>
       </c>
       <c r="G30">
-        <v>74.89928911532871</v>
+        <v>74.8992891153287</v>
       </c>
       <c r="H30">
         <v>180.97</v>
@@ -3778,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="AF30">
-        <v>801.2445000000001</v>
+        <v>801.2445</v>
       </c>
       <c r="AG30">
         <v>0</v>
@@ -3828,7 +3828,7 @@
         <v>0</v>
       </c>
       <c r="K31">
-        <v>1.858649985995706</v>
+        <v>1.858649985995705</v>
       </c>
       <c r="L31">
         <v>0</v>
@@ -3962,10 +3962,10 @@
         <v>33.84</v>
       </c>
       <c r="R32">
-        <v>945.4113000000001</v>
+        <v>945.4113</v>
       </c>
       <c r="S32">
-        <v>7.565610520559639</v>
+        <v>7.565610520559638</v>
       </c>
       <c r="T32">
         <v>1575.19001</v>
@@ -4271,7 +4271,7 @@
         <v>74.94482307907758</v>
       </c>
       <c r="H35">
-        <v>337.4999999999999</v>
+        <v>337.5</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -4646,7 +4646,7 @@
         <v>6.844402790188991</v>
       </c>
       <c r="T38">
-        <v>898.6499899999999</v>
+        <v>898.64999</v>
       </c>
       <c r="U38">
         <v>21</v>
@@ -4717,10 +4717,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F39">
-        <v>8757.950000000001</v>
+        <v>8757.949999999999</v>
       </c>
       <c r="G39">
-        <v>70.08509276178029</v>
+        <v>70.08509276178027</v>
       </c>
       <c r="H39">
         <v>203.09</v>
@@ -4908,7 +4908,7 @@
         <v>0</v>
       </c>
       <c r="AF40">
-        <v>762.7650000000001</v>
+        <v>762.765</v>
       </c>
       <c r="AG40">
         <v>0</v>
@@ -4943,10 +4943,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F41">
-        <v>8234.929999999998</v>
+        <v>8234.93</v>
       </c>
       <c r="G41">
-        <v>65.89964922576256</v>
+        <v>65.89964922576257</v>
       </c>
       <c r="H41">
         <v>42.54</v>
@@ -4979,10 +4979,10 @@
         <v>32.004</v>
       </c>
       <c r="R41">
-        <v>847.99138</v>
+        <v>847.9913799999999</v>
       </c>
       <c r="S41">
-        <v>6.78601208370567</v>
+        <v>6.786012083705669</v>
       </c>
       <c r="T41">
         <v>1039.69</v>
@@ -5021,7 +5021,7 @@
         <v>0</v>
       </c>
       <c r="AF41">
-        <v>690.5905999999999</v>
+        <v>690.5906</v>
       </c>
       <c r="AG41">
         <v>0</v>
@@ -5208,7 +5208,7 @@
         <v>3.75311</v>
       </c>
       <c r="S43">
-        <v>0.08257667766776676</v>
+        <v>0.08257667766776677</v>
       </c>
       <c r="T43">
         <v>0</v>
@@ -5282,10 +5282,10 @@
         <v>124.9616666666667</v>
       </c>
       <c r="F44">
-        <v>8274.099999999999</v>
+        <v>8274.1</v>
       </c>
       <c r="G44">
-        <v>66.21310535230803</v>
+        <v>66.21310535230805</v>
       </c>
       <c r="H44">
         <v>297.8200000000001</v>
@@ -5410,7 +5410,7 @@
         <v>0</v>
       </c>
       <c r="K45">
-        <v>0.3757152193339291</v>
+        <v>0.375715219333929</v>
       </c>
       <c r="L45">
         <v>0</v>
@@ -5508,7 +5508,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F46">
-        <v>7142.569999999999</v>
+        <v>7142.57</v>
       </c>
       <c r="G46">
         <v>93.52463631483153</v>
@@ -5523,7 +5523,7 @@
         <v>0</v>
       </c>
       <c r="K46">
-        <v>2.101059302614867</v>
+        <v>2.101059302614866</v>
       </c>
       <c r="L46">
         <v>0</v>
@@ -5657,13 +5657,13 @@
         <v>32.4</v>
       </c>
       <c r="R47">
-        <v>806.5637</v>
+        <v>806.5636999999999</v>
       </c>
       <c r="S47">
         <v>10.56112529625119</v>
       </c>
       <c r="T47">
-        <v>911.0899999999999</v>
+        <v>911.09</v>
       </c>
       <c r="U47">
         <v>9</v>
@@ -5847,7 +5847,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F49">
-        <v>7078.56</v>
+        <v>7078.559999999999</v>
       </c>
       <c r="G49">
         <v>92.68649094551596</v>
@@ -5889,7 +5889,7 @@
         <v>8.81651228869597</v>
       </c>
       <c r="T49">
-        <v>830.0500099999999</v>
+        <v>830.05001</v>
       </c>
       <c r="U49">
         <v>28</v>
@@ -5925,7 +5925,7 @@
         <v>0</v>
       </c>
       <c r="AF49">
-        <v>664.0912000000001</v>
+        <v>664.0912</v>
       </c>
       <c r="AG49">
         <v>0</v>
@@ -6186,10 +6186,10 @@
         <v>76.37083333333334</v>
       </c>
       <c r="F52">
-        <v>6636.860000000001</v>
+        <v>6636.86</v>
       </c>
       <c r="G52">
-        <v>86.90307163511376</v>
+        <v>86.90307163511375</v>
       </c>
       <c r="H52">
         <v>201.92</v>
@@ -6228,7 +6228,7 @@
         <v>10.01454228817721</v>
       </c>
       <c r="T52">
-        <v>940.6600000000001</v>
+        <v>940.66</v>
       </c>
       <c r="U52">
         <v>11</v>
@@ -6264,7 +6264,7 @@
         <v>0</v>
       </c>
       <c r="AF52">
-        <v>553.3290000000001</v>
+        <v>553.329</v>
       </c>
       <c r="AG52">
         <v>0</v>
@@ -6448,10 +6448,10 @@
         <v>34.92</v>
       </c>
       <c r="R54">
-        <v>675.5848699999999</v>
+        <v>675.58487</v>
       </c>
       <c r="S54">
-        <v>8.846091710204133</v>
+        <v>8.846091710204135</v>
       </c>
       <c r="T54">
         <v>952.77999</v>
@@ -6603,7 +6603,7 @@
         <v>0</v>
       </c>
       <c r="AF55">
-        <v>630.7519299999999</v>
+        <v>630.75193</v>
       </c>
       <c r="AG55">
         <v>0</v>
@@ -6638,10 +6638,10 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F56">
-        <v>6693.129999999999</v>
+        <v>6693.13</v>
       </c>
       <c r="G56">
-        <v>87.63967998323969</v>
+        <v>87.6396799832397</v>
       </c>
       <c r="H56">
         <v>16.96</v>
@@ -6900,13 +6900,13 @@
         <v>33.012</v>
       </c>
       <c r="R58">
-        <v>685.1758299999999</v>
+        <v>685.17583</v>
       </c>
       <c r="S58">
-        <v>8.971675505100102</v>
+        <v>8.971675505100103</v>
       </c>
       <c r="T58">
-        <v>843.77997</v>
+        <v>843.7799699999999</v>
       </c>
       <c r="U58">
         <v>17</v>
@@ -6951,7 +6951,7 @@
         <v>3</v>
       </c>
       <c r="AI58">
-        <v>2055.527489999999</v>
+        <v>2055.52749</v>
       </c>
     </row>
     <row r="59">
@@ -7090,7 +7090,7 @@
         <v>76.37100000000001</v>
       </c>
       <c r="F60">
-        <v>6802.68</v>
+        <v>6802.679999999999</v>
       </c>
       <c r="G60">
         <v>89.07412499508975</v>
@@ -7132,7 +7132,7 @@
         <v>8.080355370494035</v>
       </c>
       <c r="T60">
-        <v>862.5100000000001</v>
+        <v>862.51</v>
       </c>
       <c r="U60">
         <v>10</v>
@@ -7239,13 +7239,13 @@
         <v>36</v>
       </c>
       <c r="R61">
-        <v>618.2029799999999</v>
+        <v>618.20298</v>
       </c>
       <c r="S61">
-        <v>8.094734650587263</v>
+        <v>8.094734650587265</v>
       </c>
       <c r="T61">
-        <v>742.09999</v>
+        <v>742.0999899999999</v>
       </c>
       <c r="U61">
         <v>12</v>
@@ -7281,7 +7281,7 @@
         <v>0</v>
       </c>
       <c r="AF61">
-        <v>509.4404000000001</v>
+        <v>509.4404</v>
       </c>
       <c r="AG61">
         <v>0</v>
@@ -9301,7 +9301,7 @@
         <v>32.364</v>
       </c>
       <c r="R80">
-        <v>758.4063100000001</v>
+        <v>758.40631</v>
       </c>
       <c r="S80">
         <v>11.09411010637131</v>
@@ -9830,10 +9830,10 @@
         <v>71.20933333333333</v>
       </c>
       <c r="F85">
-        <v>7086.919999999999</v>
+        <v>7086.92</v>
       </c>
       <c r="G85">
-        <v>99.52234725785009</v>
+        <v>99.5223472578501</v>
       </c>
       <c r="H85">
         <v>246.93</v>
@@ -9985,7 +9985,7 @@
         <v>7.952642350253712</v>
       </c>
       <c r="T86">
-        <v>931.2800099999999</v>
+        <v>931.2800100000001</v>
       </c>
       <c r="U86">
         <v>15</v>
@@ -10021,7 +10021,7 @@
         <v>0</v>
       </c>
       <c r="AF86">
-        <v>558.38181</v>
+        <v>558.3818100000001</v>
       </c>
       <c r="AG86">
         <v>0</v>
@@ -10056,10 +10056,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F87">
-        <v>6362.629999999999</v>
+        <v>6362.63</v>
       </c>
       <c r="G87">
-        <v>93.07374800995692</v>
+        <v>93.07374800995693</v>
       </c>
       <c r="H87">
         <v>345.63</v>
@@ -10282,10 +10282,10 @@
         <v>68.36116666666666</v>
       </c>
       <c r="F89">
-        <v>6656.71</v>
+        <v>6656.709999999999</v>
       </c>
       <c r="G89">
-        <v>97.3756055460337</v>
+        <v>97.37560554603368</v>
       </c>
       <c r="H89">
         <v>144.12</v>
@@ -10360,7 +10360,7 @@
         <v>0</v>
       </c>
       <c r="AF89">
-        <v>621.0583999999999</v>
+        <v>621.0584</v>
       </c>
       <c r="AG89">
         <v>0</v>
@@ -10508,7 +10508,7 @@
         <v>68.7235</v>
       </c>
       <c r="F91">
-        <v>7172.649999999999</v>
+        <v>7172.65</v>
       </c>
       <c r="G91">
         <v>104.3696843146813</v>
@@ -10663,7 +10663,7 @@
         <v>8.221425422162724</v>
       </c>
       <c r="T92">
-        <v>925.6099999999999</v>
+        <v>925.61</v>
       </c>
       <c r="U92">
         <v>14</v>
@@ -10963,7 +10963,7 @@
         <v>13609.36</v>
       </c>
       <c r="G95">
-        <v>75.02431100445061</v>
+        <v>75.02431100445058</v>
       </c>
       <c r="H95">
         <v>783.59</v>
@@ -10975,7 +10975,7 @@
         <v>0</v>
       </c>
       <c r="K95">
-        <v>4.319696140007865</v>
+        <v>4.319696140007864</v>
       </c>
       <c r="L95">
         <v>0</v>
@@ -10999,7 +10999,7 @@
         <v>1367.31024</v>
       </c>
       <c r="S95">
-        <v>7.537570369608122</v>
+        <v>7.53757036960812</v>
       </c>
       <c r="T95">
         <v>2768.85995</v>
@@ -11076,7 +11076,7 @@
         <v>13532.14</v>
       </c>
       <c r="G96">
-        <v>74.59862035509136</v>
+        <v>74.59862035509134</v>
       </c>
       <c r="H96">
         <v>905.78</v>
@@ -11088,7 +11088,7 @@
         <v>0</v>
       </c>
       <c r="K96">
-        <v>4.99329288237002</v>
+        <v>4.993292882370019</v>
       </c>
       <c r="L96">
         <v>0</v>
@@ -11189,10 +11189,10 @@
         <v>12701.11</v>
       </c>
       <c r="G97">
-        <v>70.01740175450848</v>
+        <v>70.01740175450847</v>
       </c>
       <c r="H97">
-        <v>368.9400000000001</v>
+        <v>368.94</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -11225,7 +11225,7 @@
         <v>1622.4067</v>
       </c>
       <c r="S97">
-        <v>8.943840477179263</v>
+        <v>8.943840477179261</v>
       </c>
       <c r="T97">
         <v>1981.77002</v>
@@ -11302,10 +11302,10 @@
         <v>14057.61</v>
       </c>
       <c r="G98">
-        <v>77.49537852031798</v>
+        <v>77.49537852031797</v>
       </c>
       <c r="H98">
-        <v>717.6199999999999</v>
+        <v>717.62</v>
       </c>
       <c r="I98">
         <v>0</v>
@@ -11338,7 +11338,7 @@
         <v>1301.95454</v>
       </c>
       <c r="S98">
-        <v>7.177284040000148</v>
+        <v>7.177284040000147</v>
       </c>
       <c r="T98">
         <v>2534.90994</v>
@@ -11386,7 +11386,7 @@
         <v>3</v>
       </c>
       <c r="AI98">
-        <v>3905.863620000001</v>
+        <v>3905.86362</v>
       </c>
     </row>
     <row r="99">
@@ -11415,7 +11415,7 @@
         <v>13466.34</v>
       </c>
       <c r="G99">
-        <v>74.23588473313023</v>
+        <v>74.23588473313021</v>
       </c>
       <c r="H99">
         <v>1259.67</v>
@@ -11427,7 +11427,7 @@
         <v>0</v>
       </c>
       <c r="K99">
-        <v>6.944182080786773</v>
+        <v>6.944182080786772</v>
       </c>
       <c r="L99">
         <v>0</v>
@@ -11451,7 +11451,7 @@
         <v>1361.55609</v>
       </c>
       <c r="S99">
-        <v>7.505849470229586</v>
+        <v>7.505849470229585</v>
       </c>
       <c r="T99">
         <v>3031.29993</v>
@@ -11528,10 +11528,10 @@
         <v>11839.12</v>
       </c>
       <c r="G100">
-        <v>65.26550997982353</v>
+        <v>65.26550997982351</v>
       </c>
       <c r="H100">
-        <v>580.6799999999998</v>
+        <v>580.6799999999999</v>
       </c>
       <c r="I100">
         <v>0</v>
@@ -11564,7 +11564,7 @@
         <v>1362.04584</v>
       </c>
       <c r="S100">
-        <v>7.508549314771463</v>
+        <v>7.508549314771462</v>
       </c>
       <c r="T100">
         <v>2197.63005</v>
@@ -11603,7 +11603,7 @@
         <v>0</v>
       </c>
       <c r="AF100">
-        <v>846.5939999999999</v>
+        <v>846.5940000000001</v>
       </c>
       <c r="AG100">
         <v>0</v>
@@ -11754,7 +11754,7 @@
         <v>13587.06</v>
       </c>
       <c r="G102">
-        <v>74.90137780734219</v>
+        <v>74.90137780734217</v>
       </c>
       <c r="H102">
         <v>610.51</v>
@@ -11790,7 +11790,7 @@
         <v>1448.92289</v>
       </c>
       <c r="S102">
-        <v>7.987476378082978</v>
+        <v>7.987476378082977</v>
       </c>
       <c r="T102">
         <v>2588.26003</v>
@@ -11867,10 +11867,10 @@
         <v>13570.48</v>
       </c>
       <c r="G103">
-        <v>74.80997725092706</v>
+        <v>74.80997725092705</v>
       </c>
       <c r="H103">
-        <v>420.2499999999999</v>
+        <v>420.25</v>
       </c>
       <c r="I103">
         <v>0</v>
@@ -11903,7 +11903,7 @@
         <v>1254.50062</v>
       </c>
       <c r="S103">
-        <v>6.915684842649184</v>
+        <v>6.915684842649182</v>
       </c>
       <c r="T103">
         <v>2110.94003</v>
@@ -12093,7 +12093,7 @@
         <v>11738.1</v>
       </c>
       <c r="G105">
-        <v>64.70861708422302</v>
+        <v>64.70861708422301</v>
       </c>
       <c r="H105">
         <v>228.83</v>
@@ -12129,7 +12129,7 @@
         <v>1103.19668</v>
       </c>
       <c r="S105">
-        <v>6.081591700079751</v>
+        <v>6.08159170007975</v>
       </c>
       <c r="T105">
         <v>1850.74</v>
@@ -12206,7 +12206,7 @@
         <v>14309.53</v>
       </c>
       <c r="G106">
-        <v>78.88413775868344</v>
+        <v>78.88413775868342</v>
       </c>
       <c r="H106">
         <v>1603.26</v>
@@ -12242,7 +12242,7 @@
         <v>1351.15255</v>
       </c>
       <c r="S106">
-        <v>7.448497881285855</v>
+        <v>7.448497881285856</v>
       </c>
       <c r="T106">
         <v>3616.20992</v>
@@ -12290,7 +12290,7 @@
         <v>3</v>
       </c>
       <c r="AI106">
-        <v>4053.457649999999</v>
+        <v>4053.45765</v>
       </c>
     </row>
     <row r="107">
@@ -12319,7 +12319,7 @@
         <v>12247.15</v>
       </c>
       <c r="G107">
-        <v>67.51485672494204</v>
+        <v>67.51485672494202</v>
       </c>
       <c r="H107">
         <v>385.08</v>
@@ -12432,7 +12432,7 @@
         <v>13585.76</v>
       </c>
       <c r="G108">
-        <v>74.89421129809371</v>
+        <v>74.89421129809369</v>
       </c>
       <c r="H108">
         <v>1185.27</v>
@@ -12444,7 +12444,7 @@
         <v>0</v>
       </c>
       <c r="K108">
-        <v>6.534037243797295</v>
+        <v>6.534037243797294</v>
       </c>
       <c r="L108">
         <v>0</v>
@@ -12468,7 +12468,7 @@
         <v>1300.14625</v>
       </c>
       <c r="S108">
-        <v>7.167315480762517</v>
+        <v>7.167315480762516</v>
       </c>
       <c r="T108">
         <v>2929.39002</v>
@@ -12545,7 +12545,7 @@
         <v>12266.49</v>
       </c>
       <c r="G109">
-        <v>67.62147233176162</v>
+        <v>67.62147233176159</v>
       </c>
       <c r="H109">
         <v>463.29</v>
@@ -12557,7 +12557,7 @@
         <v>0</v>
       </c>
       <c r="K109">
-        <v>2.553978515172787</v>
+        <v>2.553978515172786</v>
       </c>
       <c r="L109">
         <v>0</v>
@@ -12581,7 +12581,7 @@
         <v>1240.70238</v>
       </c>
       <c r="S109">
-        <v>6.839619292977924</v>
+        <v>6.839619292977923</v>
       </c>
       <c r="T109">
         <v>2345.96002</v>
@@ -12658,7 +12658,7 @@
         <v>12956.01</v>
       </c>
       <c r="G110">
-        <v>71.42258883715118</v>
+        <v>71.42258883715117</v>
       </c>
       <c r="H110">
         <v>550.62</v>
@@ -12694,7 +12694,7 @@
         <v>1367.91901</v>
       </c>
       <c r="S110">
-        <v>7.540926335635192</v>
+        <v>7.540926335635191</v>
       </c>
       <c r="T110">
         <v>2087.11996</v>
@@ -12884,10 +12884,10 @@
         <v>18303.41</v>
       </c>
       <c r="G112">
-        <v>79.93284853654792</v>
+        <v>79.93284853654791</v>
       </c>
       <c r="H112">
-        <v>472.7499999999999</v>
+        <v>472.75</v>
       </c>
       <c r="I112">
         <v>0</v>
@@ -12920,7 +12920,7 @@
         <v>1772.41724</v>
       </c>
       <c r="S112">
-        <v>7.740325916781971</v>
+        <v>7.74032591678197</v>
       </c>
       <c r="T112">
         <v>2454.89998</v>
@@ -13009,7 +13009,7 @@
         <v>0</v>
       </c>
       <c r="K113">
-        <v>1.783742591394335</v>
+        <v>1.783742591394336</v>
       </c>
       <c r="L113">
         <v>0</v>
@@ -13223,7 +13223,7 @@
         <v>19147.53</v>
       </c>
       <c r="G115">
-        <v>85.15633651543349</v>
+        <v>85.15633651543351</v>
       </c>
       <c r="H115">
         <v>370.36</v>
@@ -13259,7 +13259,7 @@
         <v>1718.72645</v>
       </c>
       <c r="S115">
-        <v>7.643829149460865</v>
+        <v>7.643829149460866</v>
       </c>
       <c r="T115">
         <v>1940.40001</v>
@@ -13307,7 +13307,7 @@
         <v>3</v>
       </c>
       <c r="AI115">
-        <v>5156.179349999999</v>
+        <v>5156.17935</v>
       </c>
     </row>
     <row r="116">
@@ -13449,7 +13449,7 @@
         <v>16065.62</v>
       </c>
       <c r="G117">
-        <v>70.16019256006037</v>
+        <v>70.16019256006038</v>
       </c>
       <c r="H117">
         <v>375.7</v>
@@ -13485,7 +13485,7 @@
         <v>1707.62189</v>
       </c>
       <c r="S117">
-        <v>7.457358049186664</v>
+        <v>7.457358049186663</v>
       </c>
       <c r="T117">
         <v>2101.00999</v>
@@ -13533,7 +13533,7 @@
         <v>3</v>
       </c>
       <c r="AI117">
-        <v>5122.86567</v>
+        <v>5122.865669999999</v>
       </c>
     </row>
     <row r="118">
@@ -13562,7 +13562,7 @@
         <v>17963.75</v>
       </c>
       <c r="G118">
-        <v>79.89161735634409</v>
+        <v>79.89161735634407</v>
       </c>
       <c r="H118">
         <v>370.21</v>
@@ -13598,7 +13598,7 @@
         <v>1698.34145</v>
       </c>
       <c r="S118">
-        <v>7.553169313969441</v>
+        <v>7.553169313969442</v>
       </c>
       <c r="T118">
         <v>1988.68005</v>
@@ -13646,7 +13646,7 @@
         <v>3</v>
       </c>
       <c r="AI118">
-        <v>5095.02435</v>
+        <v>5095.024350000001</v>
       </c>
     </row>
     <row r="119">
@@ -13675,7 +13675,7 @@
         <v>16860.45</v>
       </c>
       <c r="G119">
-        <v>74.74106193604921</v>
+        <v>74.74106193604919</v>
       </c>
       <c r="H119">
         <v>198.18</v>
@@ -13687,7 +13687,7 @@
         <v>0</v>
       </c>
       <c r="K119">
-        <v>0.8785165078326039</v>
+        <v>0.878516507832604</v>
       </c>
       <c r="L119">
         <v>0</v>
@@ -13711,7 +13711,7 @@
         <v>1727.96753</v>
       </c>
       <c r="S119">
-        <v>7.659945504610609</v>
+        <v>7.659945504610608</v>
       </c>
       <c r="T119">
         <v>2211.12</v>
@@ -13759,7 +13759,7 @@
         <v>3</v>
       </c>
       <c r="AI119">
-        <v>5183.902590000001</v>
+        <v>5183.90259</v>
       </c>
     </row>
     <row r="120">
@@ -13788,10 +13788,10 @@
         <v>18388.95</v>
       </c>
       <c r="G120">
-        <v>81.78264321118603</v>
+        <v>81.78264321118604</v>
       </c>
       <c r="H120">
-        <v>270.9999999999999</v>
+        <v>271</v>
       </c>
       <c r="I120">
         <v>0</v>
@@ -13824,7 +13824,7 @@
         <v>1735.53757</v>
       </c>
       <c r="S120">
-        <v>7.718594583536246</v>
+        <v>7.718594583536245</v>
       </c>
       <c r="T120">
         <v>1729.52995</v>
@@ -13872,7 +13872,7 @@
         <v>3</v>
       </c>
       <c r="AI120">
-        <v>5206.61271</v>
+        <v>5206.612709999999</v>
       </c>
     </row>
     <row r="121">
@@ -13937,7 +13937,7 @@
         <v>1527.87451</v>
       </c>
       <c r="S121">
-        <v>6.772948728083817</v>
+        <v>6.772948728083818</v>
       </c>
       <c r="T121">
         <v>1992.10995</v>
@@ -13985,7 +13985,7 @@
         <v>3</v>
       </c>
       <c r="AI121">
-        <v>4583.62353</v>
+        <v>4583.623530000001</v>
       </c>
     </row>
     <row r="122">
@@ -14026,7 +14026,7 @@
         <v>0</v>
       </c>
       <c r="K122">
-        <v>4.8997186563169</v>
+        <v>4.899718656316899</v>
       </c>
       <c r="L122">
         <v>0</v>
@@ -14053,7 +14053,7 @@
         <v>6.606615921757134</v>
       </c>
       <c r="T122">
-        <v>3415.690039999999</v>
+        <v>3415.69004</v>
       </c>
       <c r="U122">
         <v>77</v>
@@ -14127,7 +14127,7 @@
         <v>18290.91</v>
       </c>
       <c r="G123">
-        <v>74.02184932102797</v>
+        <v>74.021849321028</v>
       </c>
       <c r="H123">
         <v>113.2</v>
@@ -14163,7 +14163,7 @@
         <v>1736.55142</v>
       </c>
       <c r="S123">
-        <v>7.027684655900511</v>
+        <v>7.02768465590051</v>
       </c>
       <c r="T123">
         <v>1459.61002</v>
@@ -14211,7 +14211,7 @@
         <v>3</v>
       </c>
       <c r="AI123">
-        <v>5209.654260000001</v>
+        <v>5209.65426</v>
       </c>
     </row>
     <row r="124">
@@ -14389,10 +14389,10 @@
         <v>1747.75452</v>
       </c>
       <c r="S125">
-        <v>7.052093914697219</v>
+        <v>7.052093914697221</v>
       </c>
       <c r="T125">
-        <v>2673.450039999999</v>
+        <v>2673.45004</v>
       </c>
       <c r="U125">
         <v>69</v>
@@ -14654,7 +14654,7 @@
         <v>0</v>
       </c>
       <c r="AF127">
-        <v>822.8863999999999</v>
+        <v>822.8864</v>
       </c>
       <c r="AG127">
         <v>0</v>
@@ -14915,10 +14915,10 @@
         <v>91.82383333333334</v>
       </c>
       <c r="F130">
-        <v>5290.240000000001</v>
+        <v>5290.24</v>
       </c>
       <c r="G130">
-        <v>57.61292910518874</v>
+        <v>57.61292910518873</v>
       </c>
       <c r="H130">
         <v>81.05</v>
@@ -14951,10 +14951,10 @@
         <v>33.984</v>
       </c>
       <c r="R130">
-        <v>662.6083799999999</v>
+        <v>662.60838</v>
       </c>
       <c r="S130">
-        <v>7.216082752662252</v>
+        <v>7.216082752662254</v>
       </c>
       <c r="T130">
         <v>571.95001</v>
@@ -15031,7 +15031,7 @@
         <v>7157.05</v>
       </c>
       <c r="G131">
-        <v>63.24549543578731</v>
+        <v>63.24549543578732</v>
       </c>
       <c r="H131">
         <v>225.97</v>
@@ -15067,7 +15067,7 @@
         <v>628.97713</v>
       </c>
       <c r="S131">
-        <v>5.55815178105918</v>
+        <v>5.558151781059181</v>
       </c>
       <c r="T131">
         <v>1047.82999</v>
@@ -15144,7 +15144,7 @@
         <v>6408.839999999999</v>
       </c>
       <c r="G132">
-        <v>56.63370536306035</v>
+        <v>56.63370536306036</v>
       </c>
       <c r="H132">
         <v>286.85</v>
@@ -15180,7 +15180,7 @@
         <v>613.2202</v>
       </c>
       <c r="S132">
-        <v>5.418910774723186</v>
+        <v>5.418910774723187</v>
       </c>
       <c r="T132">
         <v>1023.20001</v>
@@ -15367,10 +15367,10 @@
         <v>113.1631666666667</v>
       </c>
       <c r="F134">
-        <v>6269.599999999999</v>
+        <v>6269.6</v>
       </c>
       <c r="G134">
-        <v>55.40318625465588</v>
+        <v>55.40318625465589</v>
       </c>
       <c r="H134">
         <v>211.59</v>
@@ -15409,7 +15409,7 @@
         <v>5.473698980380837</v>
       </c>
       <c r="T134">
-        <v>780.1500000000001</v>
+        <v>780.15</v>
       </c>
       <c r="U134">
         <v>18</v>
@@ -15480,7 +15480,7 @@
         <v>113.163</v>
       </c>
       <c r="F135">
-        <v>6279.680000000001</v>
+        <v>6279.68</v>
       </c>
       <c r="G135">
         <v>55.49234290359924</v>
@@ -15519,7 +15519,7 @@
         <v>647.28536</v>
       </c>
       <c r="S135">
-        <v>5.719938142325671</v>
+        <v>5.719938142325672</v>
       </c>
       <c r="T135">
         <v>882.44998</v>
@@ -15596,7 +15596,7 @@
         <v>6758.219999999999</v>
       </c>
       <c r="G136">
-        <v>59.72111025688607</v>
+        <v>59.72111025688608</v>
       </c>
       <c r="H136">
         <v>242.25</v>
@@ -15632,7 +15632,7 @@
         <v>630.8665599999999</v>
       </c>
       <c r="S136">
-        <v>5.574848316145736</v>
+        <v>5.574848316145737</v>
       </c>
       <c r="T136">
         <v>831.40002</v>
@@ -15748,7 +15748,7 @@
         <v>5.074410891870847</v>
       </c>
       <c r="T137">
-        <v>678.8100099999999</v>
+        <v>678.81001</v>
       </c>
       <c r="U137">
         <v>22</v>
@@ -16274,7 +16274,7 @@
         <v>6046.12</v>
       </c>
       <c r="G142">
-        <v>53.42841741558636</v>
+        <v>53.42841741558637</v>
       </c>
       <c r="H142">
         <v>73.61999999999999</v>
@@ -16286,7 +16286,7 @@
         <v>0</v>
       </c>
       <c r="K142">
-        <v>0.6505659977201027</v>
+        <v>0.6505659977201028</v>
       </c>
       <c r="L142">
         <v>0</v>
@@ -16310,7 +16310,7 @@
         <v>609.1166899999999</v>
       </c>
       <c r="S142">
-        <v>5.382648833982838</v>
+        <v>5.382648833982839</v>
       </c>
       <c r="T142">
         <v>719.31999</v>
@@ -16500,7 +16500,7 @@
         <v>17288.56</v>
       </c>
       <c r="G144">
-        <v>55.98173722982271</v>
+        <v>55.98173722982272</v>
       </c>
       <c r="H144">
         <v>1693.79</v>
@@ -16536,10 +16536,10 @@
         <v>1792.5641</v>
       </c>
       <c r="S144">
-        <v>5.804465635877924</v>
+        <v>5.804465635877925</v>
       </c>
       <c r="T144">
-        <v>2785.420029999999</v>
+        <v>2785.42003</v>
       </c>
       <c r="U144">
         <v>33</v>
@@ -16584,7 +16584,7 @@
         <v>3</v>
       </c>
       <c r="AI144">
-        <v>5377.6923</v>
+        <v>5377.692300000001</v>
       </c>
     </row>
     <row r="145">
@@ -16613,7 +16613,7 @@
         <v>17287.79</v>
       </c>
       <c r="G145">
-        <v>55.97924390836233</v>
+        <v>55.97924390836235</v>
       </c>
       <c r="H145">
         <v>1844.95</v>
@@ -16726,7 +16726,7 @@
         <v>16298.97</v>
       </c>
       <c r="G146">
-        <v>52.77736582206753</v>
+        <v>52.77736582206752</v>
       </c>
       <c r="H146">
         <v>1011.57</v>
@@ -16762,7 +16762,7 @@
         <v>2036.07937</v>
       </c>
       <c r="S146">
-        <v>6.5929875172023</v>
+        <v>6.592987517202299</v>
       </c>
       <c r="T146">
         <v>2179.37</v>
@@ -16810,7 +16810,7 @@
         <v>3</v>
       </c>
       <c r="AI146">
-        <v>6108.238110000001</v>
+        <v>6108.23811</v>
       </c>
     </row>
     <row r="147">
@@ -17068,7 +17068,7 @@
         <v>56.35887638630292</v>
       </c>
       <c r="H149">
-        <v>2977.800000000001</v>
+        <v>2977.8</v>
       </c>
       <c r="I149">
         <v>0</v>
@@ -17077,7 +17077,7 @@
         <v>0</v>
       </c>
       <c r="K149">
-        <v>9.642354084028174</v>
+        <v>9.642354084028172</v>
       </c>
       <c r="L149">
         <v>25.15</v>
@@ -17104,7 +17104,7 @@
         <v>5.484220286570064</v>
       </c>
       <c r="T149">
-        <v>3890.109990000001</v>
+        <v>3890.10999</v>
       </c>
       <c r="U149">
         <v>72</v>
@@ -17291,7 +17291,7 @@
         <v>18002.72</v>
       </c>
       <c r="G151">
-        <v>58.5430828248623</v>
+        <v>58.54308282486232</v>
       </c>
       <c r="H151">
         <v>1789.95</v>
@@ -17303,7 +17303,7 @@
         <v>0</v>
       </c>
       <c r="K151">
-        <v>5.820742149095374</v>
+        <v>5.820742149095375</v>
       </c>
       <c r="L151">
         <v>15.06</v>
@@ -17327,7 +17327,7 @@
         <v>1845.8524</v>
       </c>
       <c r="S151">
-        <v>6.002531280588203</v>
+        <v>6.002531280588205</v>
       </c>
       <c r="T151">
         <v>3176.92003</v>
@@ -17375,7 +17375,7 @@
         <v>3</v>
       </c>
       <c r="AI151">
-        <v>5537.557199999999</v>
+        <v>5537.5572</v>
       </c>
     </row>
     <row r="152">
@@ -17404,7 +17404,7 @@
         <v>18391.61</v>
       </c>
       <c r="G152">
-        <v>59.80771502931589</v>
+        <v>59.80771502931591</v>
       </c>
       <c r="H152">
         <v>1796.91</v>
@@ -17416,7 +17416,7 @@
         <v>0</v>
       </c>
       <c r="K152">
-        <v>5.843375387653829</v>
+        <v>5.84337538765383</v>
       </c>
       <c r="L152">
         <v>0</v>
@@ -17642,7 +17642,7 @@
         <v>0</v>
       </c>
       <c r="K154">
-        <v>4.971475398818692</v>
+        <v>4.971475398818693</v>
       </c>
       <c r="L154">
         <v>0</v>
@@ -17666,7 +17666,7 @@
         <v>1518.91438</v>
       </c>
       <c r="S154">
-        <v>4.939360849483544</v>
+        <v>4.939360849483545</v>
       </c>
       <c r="T154">
         <v>2837.21004</v>
@@ -17746,7 +17746,7 @@
         <v>58.49134623168462</v>
       </c>
       <c r="H155">
-        <v>2111.720000000001</v>
+        <v>2111.72</v>
       </c>
       <c r="I155">
         <v>0</v>
@@ -17755,7 +17755,7 @@
         <v>0</v>
       </c>
       <c r="K155">
-        <v>6.837917914676599</v>
+        <v>6.837917914676598</v>
       </c>
       <c r="L155">
         <v>0</v>
@@ -17779,10 +17779,10 @@
         <v>1643.06226</v>
       </c>
       <c r="S155">
-        <v>5.320366744920261</v>
+        <v>5.320366744920263</v>
       </c>
       <c r="T155">
-        <v>3515.660060000001</v>
+        <v>3515.66006</v>
       </c>
       <c r="U155">
         <v>64</v>
@@ -17827,7 +17827,7 @@
         <v>3</v>
       </c>
       <c r="AI155">
-        <v>4929.186779999999</v>
+        <v>4929.18678</v>
       </c>
     </row>
     <row r="156">
@@ -17969,7 +17969,7 @@
         <v>16062.82</v>
       </c>
       <c r="G157">
-        <v>52.23471795711174</v>
+        <v>52.23471795711175</v>
       </c>
       <c r="H157">
         <v>1969.79</v>
@@ -17981,7 +17981,7 @@
         <v>0</v>
       </c>
       <c r="K157">
-        <v>6.405564221272426</v>
+        <v>6.405564221272427</v>
       </c>
       <c r="L157">
         <v>0</v>
@@ -18005,7 +18005,7 @@
         <v>1632.26711</v>
       </c>
       <c r="S157">
-        <v>5.307972829274056</v>
+        <v>5.307972829274057</v>
       </c>
       <c r="T157">
         <v>2698.55997</v>
@@ -18079,7 +18079,7 @@
         <v>218.5791666666667</v>
       </c>
       <c r="F158">
-        <v>7924.959999999999</v>
+        <v>7924.96</v>
       </c>
       <c r="G158">
         <v>36.25670333021979</v>
@@ -18157,7 +18157,7 @@
         <v>0</v>
       </c>
       <c r="AF158">
-        <v>763.7615999999999</v>
+        <v>763.7616</v>
       </c>
       <c r="AG158">
         <v>0</v>
@@ -18231,7 +18231,7 @@
         <v>1789.01184</v>
       </c>
       <c r="S159">
-        <v>5.817691344628995</v>
+        <v>5.817691344628996</v>
       </c>
       <c r="T159">
         <v>3031.64001</v>
@@ -18320,7 +18320,7 @@
         <v>0</v>
       </c>
       <c r="K160">
-        <v>5.12441235419284</v>
+        <v>5.124412354192842</v>
       </c>
       <c r="L160">
         <v>0</v>
@@ -18392,7 +18392,7 @@
         <v>3</v>
       </c>
       <c r="AI160">
-        <v>3946.121400000001</v>
+        <v>3946.1214</v>
       </c>
     </row>
     <row r="161">
@@ -18421,7 +18421,7 @@
         <v>16085.98</v>
       </c>
       <c r="G161">
-        <v>61.3519880494549</v>
+        <v>61.35198804945492</v>
       </c>
       <c r="H161">
         <v>1298.26</v>
@@ -18609,7 +18609,7 @@
         <v>0</v>
       </c>
       <c r="AF162">
-        <v>448.2918999999999</v>
+        <v>448.2919</v>
       </c>
       <c r="AG162">
         <v>0</v>
@@ -18983,10 +18983,10 @@
         <v>105.6831666666667</v>
       </c>
       <c r="F166">
-        <v>5287.570000000001</v>
+        <v>5287.57</v>
       </c>
       <c r="G166">
-        <v>50.03228202536198</v>
+        <v>50.03228202536197</v>
       </c>
       <c r="H166">
         <v>199.18</v>
@@ -19322,10 +19322,10 @@
         <v>105.6831666666667</v>
       </c>
       <c r="F169">
-        <v>5265.499999999999</v>
+        <v>5265.5</v>
       </c>
       <c r="G169">
-        <v>49.82345028142292</v>
+        <v>49.82345028142294</v>
       </c>
       <c r="H169">
         <v>224.31</v>
@@ -19813,7 +19813,7 @@
         <v>436.54252</v>
       </c>
       <c r="S173">
-        <v>4.130672213644872</v>
+        <v>4.130672213644873</v>
       </c>
       <c r="T173">
         <v>272.29999</v>
@@ -20039,7 +20039,7 @@
         <v>464.15392</v>
       </c>
       <c r="S175">
-        <v>4.391938041220693</v>
+        <v>4.391938041220692</v>
       </c>
       <c r="T175">
         <v>486.08001</v>
@@ -20116,7 +20116,7 @@
         <v>2972.92</v>
       </c>
       <c r="G176">
-        <v>28.13049697287017</v>
+        <v>28.13049697287016</v>
       </c>
       <c r="H176">
         <v>30.82</v>
@@ -22049,7 +22049,7 @@
         <v>0</v>
       </c>
       <c r="K193">
-        <v>0.4845102346557786</v>
+        <v>0.4845102346557787</v>
       </c>
       <c r="L193">
         <v>0</v>
@@ -22112,7 +22112,7 @@
         <v>0</v>
       </c>
       <c r="AF193">
-        <v>847.5809999999999</v>
+        <v>847.581</v>
       </c>
       <c r="AG193">
         <v>0</v>
@@ -22338,7 +22338,7 @@
         <v>0</v>
       </c>
       <c r="AF195">
-        <v>919.9071999999999</v>
+        <v>919.9072</v>
       </c>
       <c r="AG195">
         <v>0</v>
@@ -22599,7 +22599,7 @@
         <v>214.7116666666667</v>
       </c>
       <c r="F198">
-        <v>9824.200000000001</v>
+        <v>9824.199999999999</v>
       </c>
       <c r="G198">
         <v>45.75531526776219</v>
@@ -22614,7 +22614,7 @@
         <v>0</v>
       </c>
       <c r="K198">
-        <v>0.9173232319311947</v>
+        <v>0.9173232319311946</v>
       </c>
       <c r="L198">
         <v>0</v>
@@ -22718,7 +22718,7 @@
         <v>52.73420944367252</v>
       </c>
       <c r="H199">
-        <v>463.8800000000001</v>
+        <v>463.88</v>
       </c>
       <c r="I199">
         <v>0</v>
@@ -22790,7 +22790,7 @@
         <v>0</v>
       </c>
       <c r="AF199">
-        <v>954.4660999999999</v>
+        <v>954.4661</v>
       </c>
       <c r="AG199">
         <v>0</v>
@@ -23054,7 +23054,7 @@
         <v>10768.12</v>
       </c>
       <c r="G202">
-        <v>50.1515365567777</v>
+        <v>50.15153655677769</v>
       </c>
       <c r="H202">
         <v>216.32</v>
@@ -23242,7 +23242,7 @@
         <v>0</v>
       </c>
       <c r="AF203">
-        <v>931.7031800000001</v>
+        <v>931.70318</v>
       </c>
       <c r="AG203">
         <v>0</v>
@@ -23432,7 +23432,7 @@
         <v>4.34219632539183</v>
       </c>
       <c r="T205">
-        <v>569.8699999999999</v>
+        <v>569.87</v>
       </c>
       <c r="U205">
         <v>18</v>
@@ -23503,10 +23503,10 @@
         <v>214.7116666666667</v>
       </c>
       <c r="F206">
-        <v>9841.370000000001</v>
+        <v>9841.369999999999</v>
       </c>
       <c r="G206">
-        <v>45.8352829763947</v>
+        <v>45.83528297639469</v>
       </c>
       <c r="H206">
         <v>40.99</v>
@@ -23694,7 +23694,7 @@
         <v>0</v>
       </c>
       <c r="AF207">
-        <v>777.8133999999999</v>
+        <v>777.8134</v>
       </c>
       <c r="AG207">
         <v>0</v>
@@ -23807,7 +23807,7 @@
         <v>0</v>
       </c>
       <c r="AF208">
-        <v>856.6558000000001</v>
+        <v>856.6558</v>
       </c>
       <c r="AG208">
         <v>0</v>
@@ -23881,7 +23881,7 @@
         <v>524.71559</v>
       </c>
       <c r="S209">
-        <v>4.411042747257367</v>
+        <v>4.411042747257366</v>
       </c>
       <c r="T209">
         <v>441.52999</v>
@@ -23994,7 +23994,7 @@
         <v>743.73098</v>
       </c>
       <c r="S210">
-        <v>6.252204447059814</v>
+        <v>6.252204447059813</v>
       </c>
       <c r="T210">
         <v>804.3800200000001</v>
@@ -24033,7 +24033,7 @@
         <v>0</v>
       </c>
       <c r="AF210">
-        <v>474.9416000000001</v>
+        <v>474.9416</v>
       </c>
       <c r="AG210">
         <v>0</v>
@@ -24107,10 +24107,10 @@
         <v>696.7132300000001</v>
       </c>
       <c r="S211">
-        <v>5.856947837417512</v>
+        <v>5.856947837417511</v>
       </c>
       <c r="T211">
-        <v>582.8800000000001</v>
+        <v>582.88</v>
       </c>
       <c r="U211">
         <v>15</v>
@@ -24220,7 +24220,7 @@
         <v>564.84941</v>
       </c>
       <c r="S212">
-        <v>4.748429322012527</v>
+        <v>4.748429322012526</v>
       </c>
       <c r="T212">
         <v>709.40998</v>
@@ -24297,7 +24297,7 @@
         <v>5643.78</v>
       </c>
       <c r="G213">
-        <v>47.44466394855198</v>
+        <v>47.44466394855197</v>
       </c>
       <c r="H213">
         <v>155.62</v>
@@ -24333,7 +24333,7 @@
         <v>602.5131</v>
       </c>
       <c r="S213">
-        <v>5.065050649405238</v>
+        <v>5.065050649405237</v>
       </c>
       <c r="T213">
         <v>636.9700200000001</v>
@@ -24407,10 +24407,10 @@
         <v>118.955</v>
       </c>
       <c r="F214">
-        <v>5066.97</v>
+        <v>5066.969999999999</v>
       </c>
       <c r="G214">
-        <v>42.59568744483209</v>
+        <v>42.59568744483207</v>
       </c>
       <c r="H214">
         <v>114.87</v>
@@ -24422,7 +24422,7 @@
         <v>0</v>
       </c>
       <c r="K214">
-        <v>0.9656592829221136</v>
+        <v>0.9656592829221134</v>
       </c>
       <c r="L214">
         <v>0</v>
@@ -24446,7 +24446,7 @@
         <v>576.51539</v>
       </c>
       <c r="S214">
-        <v>4.846499852885546</v>
+        <v>4.846499852885545</v>
       </c>
       <c r="T214">
         <v>539.4400000000001</v>
@@ -24523,7 +24523,7 @@
         <v>5346.26</v>
       </c>
       <c r="G215">
-        <v>44.94355008196378</v>
+        <v>44.94355008196377</v>
       </c>
       <c r="H215">
         <v>122.36</v>
@@ -24535,7 +24535,7 @@
         <v>0</v>
       </c>
       <c r="K215">
-        <v>1.028624269681813</v>
+        <v>1.028624269681812</v>
       </c>
       <c r="L215">
         <v>0</v>
@@ -24559,7 +24559,7 @@
         <v>602.2756899999999</v>
       </c>
       <c r="S215">
-        <v>5.063054852675382</v>
+        <v>5.063054852675381</v>
       </c>
       <c r="T215">
         <v>636.9599999999999</v>
@@ -24648,7 +24648,7 @@
         <v>0</v>
       </c>
       <c r="K216">
-        <v>0.7863477785717289</v>
+        <v>0.7863477785717288</v>
       </c>
       <c r="L216">
         <v>0</v>
@@ -24669,7 +24669,7 @@
         <v>33.696</v>
       </c>
       <c r="R216">
-        <v>507.2115299999999</v>
+        <v>507.21153</v>
       </c>
       <c r="S216">
         <v>4.263894161657769</v>
@@ -24749,7 +24749,7 @@
         <v>5836.85</v>
       </c>
       <c r="G217">
-        <v>49.06771468202263</v>
+        <v>49.06771468202262</v>
       </c>
       <c r="H217">
         <v>184.94</v>
@@ -24782,7 +24782,7 @@
         <v>34.992</v>
       </c>
       <c r="R217">
-        <v>607.4305999999999</v>
+        <v>607.4306</v>
       </c>
       <c r="S217">
         <v>5.10638981127317</v>
@@ -24862,7 +24862,7 @@
         <v>5143.78</v>
       </c>
       <c r="G218">
-        <v>43.24139380437981</v>
+        <v>43.2413938043798</v>
       </c>
       <c r="H218">
         <v>137.44</v>
@@ -24898,7 +24898,7 @@
         <v>488.68669</v>
       </c>
       <c r="S218">
-        <v>4.108164347862638</v>
+        <v>4.108164347862637</v>
       </c>
       <c r="T218">
         <v>557.67002</v>
@@ -24975,7 +24975,7 @@
         <v>5281.13</v>
       </c>
       <c r="G219">
-        <v>44.39603211298391</v>
+        <v>44.3960321129839</v>
       </c>
       <c r="H219">
         <v>105.42</v>
@@ -24987,7 +24987,7 @@
         <v>0</v>
       </c>
       <c r="K219">
-        <v>0.8862174771972596</v>
+        <v>0.8862174771972595</v>
       </c>
       <c r="L219">
         <v>0</v>
@@ -25088,7 +25088,7 @@
         <v>5406.599999999999</v>
       </c>
       <c r="G220">
-        <v>45.45080072296247</v>
+        <v>45.45080072296246</v>
       </c>
       <c r="H220">
         <v>216.21</v>
@@ -25127,7 +25127,7 @@
         <v>5.227078390988189</v>
       </c>
       <c r="T220">
-        <v>639.3799899999999</v>
+        <v>639.37999</v>
       </c>
       <c r="U220">
         <v>14</v>
@@ -25201,7 +25201,7 @@
         <v>5644.610000000001</v>
       </c>
       <c r="G221">
-        <v>47.45164137699131</v>
+        <v>47.4516413769913</v>
       </c>
       <c r="H221">
         <v>233.03</v>
@@ -25237,10 +25237,10 @@
         <v>588.61037</v>
       </c>
       <c r="S221">
-        <v>4.948176789542265</v>
+        <v>4.948176789542264</v>
       </c>
       <c r="T221">
-        <v>767.3400200000001</v>
+        <v>767.34002</v>
       </c>
       <c r="U221">
         <v>26</v>
@@ -25314,7 +25314,7 @@
         <v>5131.67</v>
       </c>
       <c r="G222">
-        <v>43.13959060148797</v>
+        <v>43.13959060148796</v>
       </c>
       <c r="H222">
         <v>59.44</v>
@@ -25347,10 +25347,10 @@
         <v>33.012</v>
       </c>
       <c r="R222">
-        <v>604.64205</v>
+        <v>604.6420499999999</v>
       </c>
       <c r="S222">
-        <v>5.082947753352109</v>
+        <v>5.082947753352108</v>
       </c>
       <c r="T222">
         <v>532.51999</v>
@@ -25424,7 +25424,7 @@
         <v>118.955</v>
       </c>
       <c r="F223">
-        <v>5003.929999999999</v>
+        <v>5003.93</v>
       </c>
       <c r="G223">
         <v>42.06573914505486</v>
@@ -25463,7 +25463,7 @@
         <v>535.20877</v>
       </c>
       <c r="S223">
-        <v>4.499254087680216</v>
+        <v>4.499254087680215</v>
       </c>
       <c r="T223">
         <v>485.38999</v>
@@ -25540,7 +25540,7 @@
         <v>6277.34</v>
       </c>
       <c r="G224">
-        <v>52.77071161363542</v>
+        <v>52.77071161363541</v>
       </c>
       <c r="H224">
         <v>185.12</v>
@@ -25576,10 +25576,10 @@
         <v>684.08368</v>
       </c>
       <c r="S224">
-        <v>5.750777016518852</v>
+        <v>5.750777016518851</v>
       </c>
       <c r="T224">
-        <v>765.2100199999999</v>
+        <v>765.21002</v>
       </c>
       <c r="U224">
         <v>22</v>
@@ -25728,7 +25728,7 @@
         <v>0</v>
       </c>
       <c r="AF225">
-        <v>933.1609000000001</v>
+        <v>933.1609</v>
       </c>
       <c r="AG225">
         <v>0</v>
@@ -25778,7 +25778,7 @@
         <v>0</v>
       </c>
       <c r="K226">
-        <v>0.7638822854332321</v>
+        <v>0.7638822854332322</v>
       </c>
       <c r="L226">
         <v>0</v>
@@ -25879,7 +25879,7 @@
         <v>12485.47</v>
       </c>
       <c r="G227">
-        <v>61.40898434297894</v>
+        <v>61.40898434297893</v>
       </c>
       <c r="H227">
         <v>267.17</v>
@@ -26105,7 +26105,7 @@
         <v>14061.02</v>
       </c>
       <c r="G229">
-        <v>69.15822608410527</v>
+        <v>69.15822608410525</v>
       </c>
       <c r="H229">
         <v>441.39</v>
@@ -26218,7 +26218,7 @@
         <v>11744.62</v>
       </c>
       <c r="G230">
-        <v>59.84184325974086</v>
+        <v>59.84184325974085</v>
       </c>
       <c r="H230">
         <v>261.36</v>
@@ -26254,7 +26254,7 @@
         <v>1419.35561</v>
       </c>
       <c r="S230">
-        <v>7.231979914501607</v>
+        <v>7.231979914501608</v>
       </c>
       <c r="T230">
         <v>1697.14</v>
@@ -26456,7 +26456,7 @@
         <v>0</v>
       </c>
       <c r="K232">
-        <v>0.5488482662513321</v>
+        <v>0.548848266251332</v>
       </c>
       <c r="L232">
         <v>0</v>
@@ -26480,7 +26480,7 @@
         <v>1367.60503</v>
       </c>
       <c r="S232">
-        <v>6.726477727682598</v>
+        <v>6.726477727682597</v>
       </c>
       <c r="T232">
         <v>1770.56001</v>
@@ -26783,7 +26783,7 @@
         <v>13294.61</v>
       </c>
       <c r="G235">
-        <v>65.38868759734406</v>
+        <v>65.38868759734405</v>
       </c>
       <c r="H235">
         <v>277.9</v>
@@ -26932,7 +26932,7 @@
         <v>1378.64224</v>
       </c>
       <c r="S236">
-        <v>7.024534879573628</v>
+        <v>7.02453487957363</v>
       </c>
       <c r="T236">
         <v>1211.53001</v>
@@ -26980,7 +26980,7 @@
         <v>3</v>
       </c>
       <c r="AI236">
-        <v>4135.926719999999</v>
+        <v>4135.92672</v>
       </c>
     </row>
     <row r="237">
@@ -27497,7 +27497,7 @@
         <v>1067.75903</v>
       </c>
       <c r="S241">
-        <v>5.519589297437568</v>
+        <v>5.519589297437567</v>
       </c>
       <c r="T241">
         <v>1399.06003</v>
@@ -27574,7 +27574,7 @@
         <v>10654.48</v>
       </c>
       <c r="G242">
-        <v>55.07642841265657</v>
+        <v>55.07642841265656</v>
       </c>
       <c r="H242">
         <v>399.7</v>
@@ -27586,7 +27586,7 @@
         <v>0</v>
       </c>
       <c r="K242">
-        <v>2.066177648889372</v>
+        <v>2.066177648889371</v>
       </c>
       <c r="L242">
         <v>0</v>
@@ -27610,7 +27610,7 @@
         <v>1245.04387</v>
       </c>
       <c r="S242">
-        <v>6.436031563874717</v>
+        <v>6.436031563874716</v>
       </c>
       <c r="T242">
         <v>1709.89998</v>
@@ -27649,7 +27649,7 @@
         <v>0</v>
       </c>
       <c r="AF242">
-        <v>875.8581999999999</v>
+        <v>875.8582</v>
       </c>
       <c r="AG242">
         <v>0</v>
@@ -27687,7 +27687,7 @@
         <v>11095.95</v>
       </c>
       <c r="G243">
-        <v>57.35852860443839</v>
+        <v>57.35852860443838</v>
       </c>
       <c r="H243">
         <v>356.89</v>
@@ -27723,7 +27723,7 @@
         <v>1302.75219</v>
       </c>
       <c r="S243">
-        <v>6.734344400849837</v>
+        <v>6.734344400849835</v>
       </c>
       <c r="T243">
         <v>1489.50999</v>
@@ -27800,7 +27800,7 @@
         <v>11865.87</v>
       </c>
       <c r="G244">
-        <v>61.33849231580417</v>
+        <v>61.33849231580415</v>
       </c>
       <c r="H244">
         <v>516.95</v>
@@ -27836,7 +27836,7 @@
         <v>1082.09471</v>
       </c>
       <c r="S244">
-        <v>5.593695030731615</v>
+        <v>5.593695030731614</v>
       </c>
       <c r="T244">
         <v>1675.04</v>
@@ -27988,7 +27988,7 @@
         <v>0</v>
       </c>
       <c r="AF245">
-        <v>883.9284999999999</v>
+        <v>883.9285</v>
       </c>
       <c r="AG245">
         <v>0</v>
@@ -28023,7 +28023,7 @@
         <v>164.1861666666667</v>
       </c>
       <c r="F246">
-        <v>8594.389999999999</v>
+        <v>8594.390000000001</v>
       </c>
       <c r="G246">
         <v>52.34539653665504</v>
@@ -28038,7 +28038,7 @@
         <v>0</v>
       </c>
       <c r="K246">
-        <v>2.881119704563012</v>
+        <v>2.881119704563011</v>
       </c>
       <c r="L246">
         <v>0</v>
@@ -28062,7 +28062,7 @@
         <v>921.2788399999999</v>
       </c>
       <c r="S246">
-        <v>5.611184295875516</v>
+        <v>5.611184295875515</v>
       </c>
       <c r="T246">
         <v>1400.84002</v>
@@ -28139,7 +28139,7 @@
         <v>10954.77</v>
       </c>
       <c r="G247">
-        <v>56.62872384969683</v>
+        <v>56.62872384969682</v>
       </c>
       <c r="H247">
         <v>481.67</v>
@@ -28175,7 +28175,7 @@
         <v>1043.98915</v>
       </c>
       <c r="S247">
-        <v>5.396715154898707</v>
+        <v>5.396715154898706</v>
       </c>
       <c r="T247">
         <v>1512.10998</v>
@@ -28214,7 +28214,7 @@
         <v>0</v>
       </c>
       <c r="AF247">
-        <v>892.4447</v>
+        <v>892.4446999999999</v>
       </c>
       <c r="AG247">
         <v>0</v>
@@ -28264,7 +28264,7 @@
         <v>0</v>
       </c>
       <c r="K248">
-        <v>2.078532326349581</v>
+        <v>2.07853232634958</v>
       </c>
       <c r="L248">
         <v>0</v>
@@ -28288,7 +28288,7 @@
         <v>975.53298</v>
       </c>
       <c r="S248">
-        <v>5.042843229998605</v>
+        <v>5.042843229998604</v>
       </c>
       <c r="T248">
         <v>1503.77001</v>
@@ -28327,7 +28327,7 @@
         <v>0</v>
       </c>
       <c r="AF248">
-        <v>927.2848000000001</v>
+        <v>927.2848</v>
       </c>
       <c r="AG248">
         <v>0</v>
@@ -28377,7 +28377,7 @@
         <v>1</v>
       </c>
       <c r="K249">
-        <v>2.627307455711842</v>
+        <v>2.627307455711841</v>
       </c>
       <c r="L249">
         <v>18.82</v>
@@ -28440,7 +28440,7 @@
         <v>0</v>
       </c>
       <c r="AF249">
-        <v>836.6739900000001</v>
+        <v>836.67399</v>
       </c>
       <c r="AG249">
         <v>0</v>
@@ -28472,10 +28472,10 @@
         </is>
       </c>
       <c r="E250">
-        <v>160.4471666666666</v>
+        <v>160.4471666666667</v>
       </c>
       <c r="F250">
-        <v>9967.839999999998</v>
+        <v>9967.84</v>
       </c>
       <c r="G250">
         <v>62.12537252657417</v>
@@ -28511,10 +28511,10 @@
         <v>34.92</v>
       </c>
       <c r="R250">
-        <v>846.2160200000001</v>
+        <v>846.21602</v>
       </c>
       <c r="S250">
-        <v>5.274110086082335</v>
+        <v>5.274110086082334</v>
       </c>
       <c r="T250">
         <v>1271.98002</v>
@@ -28591,7 +28591,7 @@
         <v>11789.95</v>
       </c>
       <c r="G251">
-        <v>60.9460374569008</v>
+        <v>60.94603745690078</v>
       </c>
       <c r="H251">
         <v>495.97</v>
@@ -28627,7 +28627,7 @@
         <v>981.08146</v>
       </c>
       <c r="S251">
-        <v>5.071525104807986</v>
+        <v>5.071525104807985</v>
       </c>
       <c r="T251">
         <v>1867.54003</v>
@@ -28704,7 +28704,7 @@
         <v>10364.86</v>
       </c>
       <c r="G252">
-        <v>53.57928963189265</v>
+        <v>53.57928963189264</v>
       </c>
       <c r="H252">
         <v>276.83</v>
@@ -28716,7 +28716,7 @@
         <v>0</v>
       </c>
       <c r="K252">
-        <v>1.431023163727908</v>
+        <v>1.431023163727907</v>
       </c>
       <c r="L252">
         <v>0</v>
@@ -28740,7 +28740,7 @@
         <v>1036.23388</v>
       </c>
       <c r="S252">
-        <v>5.356625673950241</v>
+        <v>5.35662567395024</v>
       </c>
       <c r="T252">
         <v>1269.53</v>
@@ -28779,7 +28779,7 @@
         <v>0</v>
       </c>
       <c r="AF252">
-        <v>963.3440000000001</v>
+        <v>963.3439999999999</v>
       </c>
       <c r="AG252">
         <v>0</v>
@@ -28817,7 +28817,7 @@
         <v>10479.97</v>
       </c>
       <c r="G253">
-        <v>54.17433018521679</v>
+        <v>54.17433018521677</v>
       </c>
       <c r="H253">
         <v>427.2400000000001</v>
@@ -28892,7 +28892,7 @@
         <v>0</v>
       </c>
       <c r="AF253">
-        <v>986.0328000000001</v>
+        <v>986.0328</v>
       </c>
       <c r="AG253">
         <v>0</v>
@@ -28930,7 +28930,7 @@
         <v>10871.58</v>
       </c>
       <c r="G254">
-        <v>56.19868802630151</v>
+        <v>56.1986880263015</v>
       </c>
       <c r="H254">
         <v>428.52</v>
@@ -28942,7 +28942,7 @@
         <v>0</v>
       </c>
       <c r="K254">
-        <v>2.21515748336771</v>
+        <v>2.215157483367709</v>
       </c>
       <c r="L254">
         <v>0</v>
@@ -28966,7 +28966,7 @@
         <v>1090.1221</v>
       </c>
       <c r="S254">
-        <v>5.635191187341367</v>
+        <v>5.635191187341366</v>
       </c>
       <c r="T254">
         <v>1554.22998</v>
@@ -29040,7 +29040,7 @@
         <v>193.449</v>
       </c>
       <c r="F255">
-        <v>9809.209999999999</v>
+        <v>9809.210000000001</v>
       </c>
       <c r="G255">
         <v>50.70695635542184</v>
@@ -29076,7 +29076,7 @@
         <v>32.004</v>
       </c>
       <c r="R255">
-        <v>955.3307899999999</v>
+        <v>955.33079</v>
       </c>
       <c r="S255">
         <v>4.93841162270159</v>
@@ -29127,7 +29127,7 @@
         <v>3</v>
       </c>
       <c r="AI255">
-        <v>2865.992369999999</v>
+        <v>2865.99237</v>
       </c>
     </row>
     <row r="256">
@@ -29269,7 +29269,7 @@
         <v>8426.109999999999</v>
       </c>
       <c r="G257">
-        <v>35.52577545608244</v>
+        <v>35.52577545608243</v>
       </c>
       <c r="H257">
         <v>189.52</v>
@@ -29281,7 +29281,7 @@
         <v>0</v>
       </c>
       <c r="K257">
-        <v>0.7990454627861188</v>
+        <v>0.7990454627861187</v>
       </c>
       <c r="L257">
         <v>0</v>
@@ -29308,7 +29308,7 @@
         <v>3.505054746756724</v>
       </c>
       <c r="T257">
-        <v>814.4900099999998</v>
+        <v>814.49001</v>
       </c>
       <c r="U257">
         <v>22</v>
@@ -29382,7 +29382,7 @@
         <v>9683.720000000001</v>
       </c>
       <c r="G258">
-        <v>40.82805260073447</v>
+        <v>40.82805260073446</v>
       </c>
       <c r="H258">
         <v>403.72</v>
@@ -29531,7 +29531,7 @@
         <v>1207.27861</v>
       </c>
       <c r="S259">
-        <v>5.090072264875646</v>
+        <v>5.090072264875645</v>
       </c>
       <c r="T259">
         <v>1240.89999</v>
@@ -29570,7 +29570,7 @@
         <v>0</v>
       </c>
       <c r="AF259">
-        <v>894.8360000000001</v>
+        <v>894.8359999999999</v>
       </c>
       <c r="AG259">
         <v>0</v>
@@ -29608,10 +29608,10 @@
         <v>10462.28</v>
       </c>
       <c r="G260">
-        <v>44.1105812811205</v>
+        <v>44.11058128112049</v>
       </c>
       <c r="H260">
-        <v>431.0999999999999</v>
+        <v>431.1</v>
       </c>
       <c r="I260">
         <v>0</v>
@@ -29683,7 +29683,7 @@
         <v>0</v>
       </c>
       <c r="AF260">
-        <v>989.2775999999999</v>
+        <v>989.2776</v>
       </c>
       <c r="AG260">
         <v>0</v>
@@ -29754,7 +29754,7 @@
         <v>36</v>
       </c>
       <c r="R261">
-        <v>863.1482199999999</v>
+        <v>863.14822</v>
       </c>
       <c r="S261">
         <v>3.639165623168608</v>
@@ -29831,10 +29831,10 @@
         <v>237.183</v>
       </c>
       <c r="F262">
-        <v>8770.140000000001</v>
+        <v>8770.139999999999</v>
       </c>
       <c r="G262">
-        <v>36.97625883811236</v>
+        <v>36.97625883811234</v>
       </c>
       <c r="H262">
         <v>331.78</v>
@@ -29867,10 +29867,10 @@
         <v>32.004</v>
       </c>
       <c r="R262">
-        <v>954.08775</v>
+        <v>954.0877499999999</v>
       </c>
       <c r="S262">
-        <v>4.022580665562035</v>
+        <v>4.022580665562034</v>
       </c>
       <c r="T262">
         <v>1085.62999</v>
@@ -29959,7 +29959,7 @@
         <v>0</v>
       </c>
       <c r="K263">
-        <v>1.835376059835655</v>
+        <v>1.835376059835654</v>
       </c>
       <c r="L263">
         <v>0</v>
@@ -29980,7 +29980,7 @@
         <v>33.84</v>
       </c>
       <c r="R263">
-        <v>879.6897799999999</v>
+        <v>879.68978</v>
       </c>
       <c r="S263">
         <v>3.708907383750101</v>
@@ -30185,7 +30185,7 @@
         <v>0</v>
       </c>
       <c r="K265">
-        <v>1.898534043333629</v>
+        <v>1.898534043333628</v>
       </c>
       <c r="L265">
         <v>4.79</v>
@@ -30206,7 +30206,7 @@
         <v>34.992</v>
       </c>
       <c r="R265">
-        <v>983.5840699999999</v>
+        <v>983.58407</v>
       </c>
       <c r="S265">
         <v>4.146941686377185</v>
@@ -30396,10 +30396,10 @@
         <v>237.183</v>
       </c>
       <c r="F267">
-        <v>9114.310000000001</v>
+        <v>9114.309999999999</v>
       </c>
       <c r="G267">
-        <v>38.42733248167028</v>
+        <v>38.42733248167027</v>
       </c>
       <c r="H267">
         <v>379.81</v>
@@ -30432,7 +30432,7 @@
         <v>34.992</v>
       </c>
       <c r="R267">
-        <v>796.7861899999999</v>
+        <v>796.78619</v>
       </c>
       <c r="S267">
         <v>3.359373100095707</v>
@@ -30512,7 +30512,7 @@
         <v>8177.51</v>
       </c>
       <c r="G268">
-        <v>34.47763962847254</v>
+        <v>34.47763962847253</v>
       </c>
       <c r="H268">
         <v>137.61</v>
@@ -30524,7 +30524,7 @@
         <v>0</v>
       </c>
       <c r="K268">
-        <v>0.5801849205044208</v>
+        <v>0.5801849205044207</v>
       </c>
       <c r="L268">
         <v>0</v>
@@ -30545,13 +30545,13 @@
         <v>33.984</v>
       </c>
       <c r="R268">
-        <v>872.7103400000001</v>
+        <v>872.71034</v>
       </c>
       <c r="S268">
-        <v>3.679480991470722</v>
+        <v>3.679480991470721</v>
       </c>
       <c r="T268">
-        <v>912.10999</v>
+        <v>912.1099899999999</v>
       </c>
       <c r="U268">
         <v>38</v>
@@ -30637,7 +30637,7 @@
         <v>0</v>
       </c>
       <c r="K269">
-        <v>0.9455568063478414</v>
+        <v>0.9455568063478413</v>
       </c>
       <c r="L269">
         <v>0</v>
@@ -30658,7 +30658,7 @@
         <v>34.992</v>
       </c>
       <c r="R269">
-        <v>783.8301499999999</v>
+        <v>783.83015</v>
       </c>
       <c r="S269">
         <v>3.30474844318522</v>
@@ -30750,7 +30750,7 @@
         <v>0</v>
       </c>
       <c r="K270">
-        <v>0.3587946859597864</v>
+        <v>0.3587946859597863</v>
       </c>
       <c r="L270">
         <v>0</v>
@@ -30774,7 +30774,7 @@
         <v>784.45213</v>
       </c>
       <c r="S270">
-        <v>3.307370806508056</v>
+        <v>3.307370806508055</v>
       </c>
       <c r="T270">
         <v>819.97</v>
@@ -30851,7 +30851,7 @@
         <v>8220.539999999999</v>
       </c>
       <c r="G271">
-        <v>34.65906072526278</v>
+        <v>34.65906072526277</v>
       </c>
       <c r="H271">
         <v>231.06</v>
@@ -30863,7 +30863,7 @@
         <v>0</v>
       </c>
       <c r="K271">
-        <v>0.9741844904567359</v>
+        <v>0.9741844904567358</v>
       </c>
       <c r="L271">
         <v>0</v>
@@ -30884,10 +30884,10 @@
         <v>32.004</v>
       </c>
       <c r="R271">
-        <v>738.2151100000001</v>
+        <v>738.21511</v>
       </c>
       <c r="S271">
-        <v>3.112428420249344</v>
+        <v>3.112428420249343</v>
       </c>
       <c r="T271">
         <v>935.33</v>
@@ -31000,7 +31000,7 @@
         <v>374.32809</v>
       </c>
       <c r="S272">
-        <v>2.973591516010089</v>
+        <v>2.973591516010088</v>
       </c>
       <c r="T272">
         <v>435.74001</v>
@@ -31416,7 +31416,7 @@
         <v>11070.29</v>
       </c>
       <c r="G276">
-        <v>81.98888821684395</v>
+        <v>81.98888821684396</v>
       </c>
       <c r="H276">
         <v>865.48</v>
@@ -31428,7 +31428,7 @@
         <v>3</v>
       </c>
       <c r="K276">
-        <v>6.409926295870667</v>
+        <v>6.409926295870669</v>
       </c>
       <c r="L276">
         <v>64.57000000000001</v>
@@ -31452,7 +31452,7 @@
         <v>891.0671599999999</v>
       </c>
       <c r="S276">
-        <v>6.599430166232374</v>
+        <v>6.599430166232375</v>
       </c>
       <c r="T276">
         <v>1669.22</v>
@@ -31529,7 +31529,7 @@
         <v>11437.95</v>
       </c>
       <c r="G277">
-        <v>84.71185524316438</v>
+        <v>84.71185524316439</v>
       </c>
       <c r="H277">
         <v>561.1800000000001</v>
@@ -31541,7 +31541,7 @@
         <v>0</v>
       </c>
       <c r="K277">
-        <v>4.156216710630749</v>
+        <v>4.15621671063075</v>
       </c>
       <c r="L277">
         <v>35.72</v>
@@ -31565,7 +31565,7 @@
         <v>1026.42478</v>
       </c>
       <c r="S277">
-        <v>7.601917072670961</v>
+        <v>7.601917072670965</v>
       </c>
       <c r="T277">
         <v>1445.64997</v>
@@ -31604,7 +31604,7 @@
         <v>0</v>
       </c>
       <c r="AF277">
-        <v>922.3997999999999</v>
+        <v>922.3998</v>
       </c>
       <c r="AG277">
         <v>0</v>
@@ -31613,7 +31613,7 @@
         <v>3</v>
       </c>
       <c r="AI277">
-        <v>3079.274339999999</v>
+        <v>3079.27434</v>
       </c>
     </row>
     <row r="278">
@@ -32320,7 +32320,7 @@
         <v>8081.759999999999</v>
       </c>
       <c r="G284">
-        <v>59.85520860206558</v>
+        <v>59.85520860206559</v>
       </c>
       <c r="H284">
         <v>254.47</v>
@@ -32356,7 +32356,7 @@
         <v>760.56808</v>
       </c>
       <c r="S284">
-        <v>5.632926625446995</v>
+        <v>5.632926625446996</v>
       </c>
       <c r="T284">
         <v>1158.87</v>
@@ -32659,7 +32659,7 @@
         <v>15136.74</v>
       </c>
       <c r="G287">
-        <v>54.36071107918838</v>
+        <v>54.36071107918836</v>
       </c>
       <c r="H287">
         <v>290.25</v>
@@ -32772,7 +32772,7 @@
         <v>16233.9</v>
       </c>
       <c r="G288">
-        <v>58.30095169689353</v>
+        <v>58.30095169689351</v>
       </c>
       <c r="H288">
         <v>264.75</v>
@@ -32921,7 +32921,7 @@
         <v>1748.62919</v>
       </c>
       <c r="S289">
-        <v>6.279867803914526</v>
+        <v>6.279867803914527</v>
       </c>
       <c r="T289">
         <v>1772.23002</v>
@@ -32969,7 +32969,7 @@
         <v>3</v>
       </c>
       <c r="AI289">
-        <v>5245.88757</v>
+        <v>5245.887570000001</v>
       </c>
     </row>
     <row r="290">
@@ -33337,7 +33337,7 @@
         <v>14757.36</v>
       </c>
       <c r="G293">
-        <v>52.99824025857425</v>
+        <v>52.99824025857426</v>
       </c>
       <c r="H293">
         <v>414.1</v>
@@ -33349,7 +33349,7 @@
         <v>0</v>
       </c>
       <c r="K293">
-        <v>1.487161070210091</v>
+        <v>1.487161070210092</v>
       </c>
       <c r="L293">
         <v>0</v>
@@ -33566,7 +33566,7 @@
         <v>54.23584126414078</v>
       </c>
       <c r="H295">
-        <v>372.1299999999999</v>
+        <v>372.13</v>
       </c>
       <c r="I295">
         <v>0</v>
@@ -33599,7 +33599,7 @@
         <v>1480.68447</v>
       </c>
       <c r="S295">
-        <v>5.31759551086371</v>
+        <v>5.317595510863709</v>
       </c>
       <c r="T295">
         <v>2016.47996</v>
@@ -33789,7 +33789,7 @@
         <v>15414.18</v>
       </c>
       <c r="G297">
-        <v>55.35708385706591</v>
+        <v>55.3570838570659</v>
       </c>
       <c r="H297">
         <v>380.04</v>
@@ -33899,10 +33899,10 @@
         <v>278.45</v>
       </c>
       <c r="F298">
-        <v>14041.98000000001</v>
+        <v>14041.98</v>
       </c>
       <c r="G298">
-        <v>50.42908960316037</v>
+        <v>50.42908960316036</v>
       </c>
       <c r="H298">
         <v>318.3</v>
@@ -33938,7 +33938,7 @@
         <v>1575.53616</v>
       </c>
       <c r="S298">
-        <v>5.658237241874663</v>
+        <v>5.658237241874664</v>
       </c>
       <c r="T298">
         <v>2106.25996</v>
@@ -33986,7 +33986,7 @@
         <v>3</v>
       </c>
       <c r="AI298">
-        <v>4726.60848</v>
+        <v>4726.608480000001</v>
       </c>
     </row>
     <row r="299">
@@ -34128,7 +34128,7 @@
         <v>13860.97</v>
       </c>
       <c r="G300">
-        <v>49.7790267552523</v>
+        <v>49.77902675525229</v>
       </c>
       <c r="H300">
         <v>321.83</v>
@@ -34277,7 +34277,7 @@
         <v>1565.07067</v>
       </c>
       <c r="S301">
-        <v>5.620652433111869</v>
+        <v>5.62065243311187</v>
       </c>
       <c r="T301">
         <v>1926.41998</v>
@@ -34325,7 +34325,7 @@
         <v>3</v>
       </c>
       <c r="AI301">
-        <v>4695.212009999999</v>
+        <v>4695.21201</v>
       </c>
     </row>
     <row r="302">
@@ -34429,7 +34429,7 @@
         <v>0</v>
       </c>
       <c r="AF302">
-        <v>736.5953</v>
+        <v>736.5953000000001</v>
       </c>
       <c r="AG302">
         <v>0</v>
@@ -34577,7 +34577,7 @@
         <v>89.45</v>
       </c>
       <c r="F304">
-        <v>7451.750000000001</v>
+        <v>7451.75</v>
       </c>
       <c r="G304">
         <v>83.30631637786473</v>
@@ -34655,7 +34655,7 @@
         <v>0</v>
       </c>
       <c r="AF304">
-        <v>691.1543999999999</v>
+        <v>691.1544</v>
       </c>
       <c r="AG304">
         <v>0</v>
@@ -35029,7 +35029,7 @@
         <v>89.45</v>
       </c>
       <c r="F308">
-        <v>4493.39</v>
+        <v>4493.389999999999</v>
       </c>
       <c r="G308">
         <v>50.23353828954723</v>
@@ -35107,7 +35107,7 @@
         <v>0</v>
       </c>
       <c r="AF308">
-        <v>367.9143999999999</v>
+        <v>367.9144</v>
       </c>
       <c r="AG308">
         <v>0</v>
@@ -35142,10 +35142,10 @@
         <v>89.45</v>
       </c>
       <c r="F309">
-        <v>6122.92</v>
+        <v>6122.920000000001</v>
       </c>
       <c r="G309">
-        <v>68.45075461151481</v>
+        <v>68.45075461151482</v>
       </c>
       <c r="H309">
         <v>221.46</v>
@@ -35333,7 +35333,7 @@
         <v>0</v>
       </c>
       <c r="AF310">
-        <v>674.1424199999999</v>
+        <v>674.14242</v>
       </c>
       <c r="AG310">
         <v>0</v>
@@ -35487,7 +35487,7 @@
         <v>87.99966461710453</v>
       </c>
       <c r="H312">
-        <v>355.5900000000001</v>
+        <v>355.59</v>
       </c>
       <c r="I312">
         <v>0</v>
@@ -35820,10 +35820,10 @@
         <v>89.45</v>
       </c>
       <c r="F315">
-        <v>6995.380000000001</v>
+        <v>6995.38</v>
       </c>
       <c r="G315">
-        <v>78.20435997764115</v>
+        <v>78.20435997764113</v>
       </c>
       <c r="H315">
         <v>225.43</v>
@@ -36124,7 +36124,7 @@
         <v>0</v>
       </c>
       <c r="AF317">
-        <v>506.6347999999999</v>
+        <v>506.6348</v>
       </c>
       <c r="AG317">
         <v>0</v>
@@ -36287,7 +36287,7 @@
         <v>0</v>
       </c>
       <c r="K319">
-        <v>4.082123802278343</v>
+        <v>4.082123802278344</v>
       </c>
       <c r="L319">
         <v>0</v>
@@ -36388,7 +36388,7 @@
         <v>5271.27</v>
       </c>
       <c r="G320">
-        <v>52.42149857541357</v>
+        <v>52.42149857541359</v>
       </c>
       <c r="H320">
         <v>414.68</v>
@@ -36498,10 +36498,10 @@
         <v>100.5555</v>
       </c>
       <c r="F321">
-        <v>5103.339999999999</v>
+        <v>5103.34</v>
       </c>
       <c r="G321">
-        <v>50.7514755533014</v>
+        <v>50.75147555330142</v>
       </c>
       <c r="H321">
         <v>441.99</v>
@@ -36611,7 +36611,7 @@
         <v>100.5555</v>
       </c>
       <c r="F322">
-        <v>5283.149999999999</v>
+        <v>5283.15</v>
       </c>
       <c r="G322">
         <v>52.53964228709518</v>
@@ -36689,7 +36689,7 @@
         <v>0</v>
       </c>
       <c r="AF322">
-        <v>398.9658000000001</v>
+        <v>398.9658</v>
       </c>
       <c r="AG322">
         <v>0</v>
@@ -36730,7 +36730,7 @@
         <v>49.39381734465047</v>
       </c>
       <c r="H323">
-        <v>476.6699999999999</v>
+        <v>476.67</v>
       </c>
       <c r="I323">
         <v>0</v>
@@ -36739,7 +36739,7 @@
         <v>0</v>
       </c>
       <c r="K323">
-        <v>4.740367259871413</v>
+        <v>4.740367259871414</v>
       </c>
       <c r="L323">
         <v>0</v>
@@ -36950,10 +36950,10 @@
         <v>100.5555</v>
       </c>
       <c r="F325">
-        <v>6093.08</v>
+        <v>6093.080000000001</v>
       </c>
       <c r="G325">
-        <v>60.59419922331449</v>
+        <v>60.5941992233145</v>
       </c>
       <c r="H325">
         <v>652.0700000000001</v>
@@ -37141,7 +37141,7 @@
         <v>0</v>
       </c>
       <c r="AF326">
-        <v>535.5200000000001</v>
+        <v>535.52</v>
       </c>
       <c r="AG326">
         <v>0</v>
@@ -37325,7 +37325,7 @@
         <v>33.984</v>
       </c>
       <c r="R328">
-        <v>473.5408600000001</v>
+        <v>473.54086</v>
       </c>
       <c r="S328">
         <v>4.709248723341837</v>
@@ -37367,7 +37367,7 @@
         <v>0</v>
       </c>
       <c r="AF328">
-        <v>499.2312</v>
+        <v>499.2311999999999</v>
       </c>
       <c r="AG328">
         <v>0</v>
@@ -37402,10 +37402,10 @@
         <v>100.5555</v>
       </c>
       <c r="F329">
-        <v>4900.779999999999</v>
+        <v>4900.78</v>
       </c>
       <c r="G329">
-        <v>48.73706560058872</v>
+        <v>48.73706560058873</v>
       </c>
       <c r="H329">
         <v>357.56</v>
@@ -37438,7 +37438,7 @@
         <v>34.992</v>
       </c>
       <c r="R329">
-        <v>407.1949300000001</v>
+        <v>407.19493</v>
       </c>
       <c r="S329">
         <v>4.049454579809161</v>
@@ -37554,7 +37554,7 @@
         <v>456.16676</v>
       </c>
       <c r="S330">
-        <v>4.536467522910234</v>
+        <v>4.536467522910233</v>
       </c>
       <c r="T330">
         <v>1065.58</v>
@@ -37664,7 +37664,7 @@
         <v>32.004</v>
       </c>
       <c r="R331">
-        <v>470.2515099999999</v>
+        <v>470.25151</v>
       </c>
       <c r="S331">
         <v>4.676536937313225</v>
@@ -37741,13 +37741,13 @@
         <v>100.5555</v>
       </c>
       <c r="F332">
-        <v>4659.610000000001</v>
+        <v>4659.61</v>
       </c>
       <c r="G332">
-        <v>46.33868858491083</v>
+        <v>46.33868858491082</v>
       </c>
       <c r="H332">
-        <v>306.81</v>
+        <v>306.8099999999999</v>
       </c>
       <c r="I332">
         <v>0</v>
@@ -37756,7 +37756,7 @@
         <v>0</v>
       </c>
       <c r="K332">
-        <v>3.051150856989424</v>
+        <v>3.051150856989423</v>
       </c>
       <c r="L332">
         <v>0</v>
@@ -37777,7 +37777,7 @@
         <v>36</v>
       </c>
       <c r="R332">
-        <v>509.4021100000001</v>
+        <v>509.40211</v>
       </c>
       <c r="S332">
         <v>5.065880135845379</v>
@@ -38006,7 +38006,7 @@
         <v>383.3416</v>
       </c>
       <c r="S334">
-        <v>3.756133552164221</v>
+        <v>3.756133552164222</v>
       </c>
       <c r="T334">
         <v>600.4100100000001</v>
@@ -38122,7 +38122,7 @@
         <v>4.32010827229748</v>
       </c>
       <c r="T335">
-        <v>766.7199900000001</v>
+        <v>766.7199899999999</v>
       </c>
       <c r="U335">
         <v>31</v>
@@ -38193,7 +38193,7 @@
         <v>102.0575</v>
       </c>
       <c r="F336">
-        <v>4147.93</v>
+        <v>4147.929999999999</v>
       </c>
       <c r="G336">
         <v>40.64306885824168</v>
@@ -38306,10 +38306,10 @@
         <v>102.0575</v>
       </c>
       <c r="F337">
-        <v>4106.080000000001</v>
+        <v>4106.08</v>
       </c>
       <c r="G337">
-        <v>40.23300590353478</v>
+        <v>40.23300590353477</v>
       </c>
       <c r="H337">
         <v>117.12</v>
@@ -38949,7 +38949,7 @@
         <v>0</v>
       </c>
       <c r="AF342">
-        <v>398.9511</v>
+        <v>398.9510999999999</v>
       </c>
       <c r="AG342">
         <v>0</v>
@@ -39252,7 +39252,7 @@
         <v>3.458142615682336</v>
       </c>
       <c r="T345">
-        <v>415.9399999999999</v>
+        <v>415.94</v>
       </c>
       <c r="U345">
         <v>17</v>
@@ -39362,7 +39362,7 @@
         <v>289.84354</v>
       </c>
       <c r="S346">
-        <v>2.840002351615511</v>
+        <v>2.840002351615512</v>
       </c>
       <c r="T346">
         <v>443.60999</v>
@@ -39410,7 +39410,7 @@
         <v>3</v>
       </c>
       <c r="AI346">
-        <v>869.5306199999999</v>
+        <v>869.53062</v>
       </c>
     </row>
     <row r="347">
@@ -39698,10 +39698,10 @@
         <v>36</v>
       </c>
       <c r="R349">
-        <v>382.5288399999999</v>
+        <v>382.52884</v>
       </c>
       <c r="S349">
-        <v>3.74816980623668</v>
+        <v>3.748169806236681</v>
       </c>
       <c r="T349">
         <v>269.99</v>
@@ -41925,7 +41925,7 @@
         <v>3262.51</v>
       </c>
       <c r="G369">
-        <v>46.80789096126255</v>
+        <v>46.80789096126256</v>
       </c>
       <c r="H369">
         <v>0</v>
@@ -42187,7 +42187,7 @@
         <v>331.95494</v>
       </c>
       <c r="S371">
-        <v>4.762624677187947</v>
+        <v>4.762624677187948</v>
       </c>
       <c r="T371">
         <v>392.06</v>
@@ -42235,7 +42235,7 @@
         <v>3</v>
       </c>
       <c r="AI371">
-        <v>995.8648199999999</v>
+        <v>995.86482</v>
       </c>
     </row>
     <row r="372">
@@ -43281,7 +43281,7 @@
         <v>2867.36</v>
       </c>
       <c r="G381">
-        <v>41.13859397417503</v>
+        <v>41.13859397417504</v>
       </c>
       <c r="H381">
         <v>1.52</v>
@@ -43504,13 +43504,13 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F383">
-        <v>6550.56</v>
+        <v>6550.559999999999</v>
       </c>
       <c r="G383">
         <v>58.28764644816847</v>
       </c>
       <c r="H383">
-        <v>252.6799999999999</v>
+        <v>252.68</v>
       </c>
       <c r="I383">
         <v>0</v>
@@ -43519,7 +43519,7 @@
         <v>0</v>
       </c>
       <c r="K383">
-        <v>2.248376093726827</v>
+        <v>2.248376093726828</v>
       </c>
       <c r="L383">
         <v>0</v>
@@ -43617,7 +43617,7 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F384">
-        <v>7451.579999999999</v>
+        <v>7451.58</v>
       </c>
       <c r="G384">
         <v>66.3050274358594</v>
@@ -43766,10 +43766,10 @@
         <v>32.4</v>
       </c>
       <c r="R385">
-        <v>806.3678600000001</v>
+        <v>806.36786</v>
       </c>
       <c r="S385">
-        <v>7.175155212813288</v>
+        <v>7.175155212813287</v>
       </c>
       <c r="T385">
         <v>1465.88004</v>
@@ -43808,7 +43808,7 @@
         <v>0</v>
       </c>
       <c r="AF385">
-        <v>577.4608000000001</v>
+        <v>577.4607999999999</v>
       </c>
       <c r="AG385">
         <v>0</v>
@@ -44034,7 +44034,7 @@
         <v>0</v>
       </c>
       <c r="AF387">
-        <v>688.4440000000001</v>
+        <v>688.444</v>
       </c>
       <c r="AG387">
         <v>0</v>
@@ -44069,7 +44069,7 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F388">
-        <v>7004.070000000001</v>
+        <v>7004.07</v>
       </c>
       <c r="G388">
         <v>62.32303129170992</v>
@@ -44224,7 +44224,7 @@
         <v>5.173152306095209</v>
       </c>
       <c r="T389">
-        <v>840.1899699999999</v>
+        <v>840.18997</v>
       </c>
       <c r="U389">
         <v>34</v>
@@ -44408,10 +44408,10 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F391">
-        <v>6886.380000000001</v>
+        <v>6886.38</v>
       </c>
       <c r="G391">
-        <v>61.27581195313659</v>
+        <v>61.27581195313658</v>
       </c>
       <c r="H391">
         <v>287.73</v>
@@ -44486,7 +44486,7 @@
         <v>0</v>
       </c>
       <c r="AF391">
-        <v>581.6425999999999</v>
+        <v>581.6426</v>
       </c>
       <c r="AG391">
         <v>0</v>
@@ -44634,10 +44634,10 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F393">
-        <v>5622.17</v>
+        <v>5622.170000000001</v>
       </c>
       <c r="G393">
-        <v>50.02672401008453</v>
+        <v>50.02672401008454</v>
       </c>
       <c r="H393">
         <v>95.17</v>
@@ -44676,7 +44676,7 @@
         <v>4.987750793415394</v>
       </c>
       <c r="T393">
-        <v>833.9200199999999</v>
+        <v>833.92002</v>
       </c>
       <c r="U393">
         <v>21</v>
@@ -44747,10 +44747,10 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F394">
-        <v>6903.409999999999</v>
+        <v>6903.41</v>
       </c>
       <c r="G394">
-        <v>61.42734687824409</v>
+        <v>61.4273468782441</v>
       </c>
       <c r="H394">
         <v>253.15</v>
@@ -44762,7 +44762,7 @@
         <v>0</v>
       </c>
       <c r="K394">
-        <v>2.252558208512531</v>
+        <v>2.252558208512532</v>
       </c>
       <c r="L394">
         <v>0</v>
@@ -44783,10 +44783,10 @@
         <v>36</v>
       </c>
       <c r="R394">
-        <v>869.8029900000001</v>
+        <v>869.80299</v>
       </c>
       <c r="S394">
-        <v>7.739608393889961</v>
+        <v>7.739608393889959</v>
       </c>
       <c r="T394">
         <v>1162.08001</v>
@@ -44860,10 +44860,10 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F395">
-        <v>7415.749999999999</v>
+        <v>7415.75</v>
       </c>
       <c r="G395">
-        <v>65.98620791932373</v>
+        <v>65.98620791932375</v>
       </c>
       <c r="H395">
         <v>355.52</v>
@@ -45009,10 +45009,10 @@
         <v>34.92</v>
       </c>
       <c r="R396">
-        <v>619.2207700000001</v>
+        <v>619.22077</v>
       </c>
       <c r="S396">
-        <v>5.509898591131544</v>
+        <v>5.509898591131543</v>
       </c>
       <c r="T396">
         <v>906.13001</v>
@@ -45425,10 +45425,10 @@
         <v>112.3833333333333</v>
       </c>
       <c r="F400">
-        <v>6518.749999999999</v>
+        <v>6518.75</v>
       </c>
       <c r="G400">
-        <v>58.00459736022541</v>
+        <v>58.00459736022542</v>
       </c>
       <c r="H400">
         <v>171.87</v>
@@ -45440,7 +45440,7 @@
         <v>0</v>
       </c>
       <c r="K400">
-        <v>1.529319294082753</v>
+        <v>1.529319294082752</v>
       </c>
       <c r="L400">
         <v>0</v>
@@ -45467,7 +45467,7 @@
         <v>6.161355865341836</v>
       </c>
       <c r="T400">
-        <v>972.5799999999999</v>
+        <v>972.58</v>
       </c>
       <c r="U400">
         <v>20</v>
@@ -45580,7 +45580,7 @@
         <v>4.682314483714483</v>
       </c>
       <c r="T401">
-        <v>518.8399999999999</v>
+        <v>518.84</v>
       </c>
       <c r="U401">
         <v>16</v>
@@ -45779,7 +45779,7 @@
         <v>0</v>
       </c>
       <c r="K403">
-        <v>1.333916654308171</v>
+        <v>1.333916654308172</v>
       </c>
       <c r="L403">
         <v>0</v>
@@ -45842,7 +45842,7 @@
         <v>0</v>
       </c>
       <c r="AF403">
-        <v>531.79</v>
+        <v>531.7900000000001</v>
       </c>
       <c r="AG403">
         <v>0</v>
@@ -46103,7 +46103,7 @@
         <v>82.786</v>
       </c>
       <c r="F406">
-        <v>8967.09</v>
+        <v>8967.089999999998</v>
       </c>
       <c r="G406">
         <v>108.3165027903269</v>
@@ -46139,7 +46139,7 @@
         <v>36</v>
       </c>
       <c r="R406">
-        <v>945.3767300000001</v>
+        <v>945.37673</v>
       </c>
       <c r="S406">
         <v>11.41952419491218</v>
@@ -46520,7 +46520,7 @@
         <v>0</v>
       </c>
       <c r="AF409">
-        <v>655.6392000000001</v>
+        <v>655.6392</v>
       </c>
       <c r="AG409">
         <v>0</v>
@@ -46894,10 +46894,10 @@
         <v>82.786</v>
       </c>
       <c r="F413">
-        <v>7758.570000000001</v>
+        <v>7758.57</v>
       </c>
       <c r="G413">
-        <v>93.71838233517745</v>
+        <v>93.71838233517744</v>
       </c>
       <c r="H413">
         <v>283.97</v>
@@ -47022,7 +47022,7 @@
         <v>0</v>
       </c>
       <c r="K414">
-        <v>4.810354407750103</v>
+        <v>4.810354407750102</v>
       </c>
       <c r="L414">
         <v>0</v>
@@ -47248,7 +47248,7 @@
         <v>0</v>
       </c>
       <c r="K416">
-        <v>1.686396250573769</v>
+        <v>1.686396250573768</v>
       </c>
       <c r="L416">
         <v>5.649999999999999</v>
@@ -47361,7 +47361,7 @@
         <v>1</v>
       </c>
       <c r="K417">
-        <v>5.341120479308095</v>
+        <v>5.341120479308096</v>
       </c>
       <c r="L417">
         <v>16.25</v>
@@ -47459,7 +47459,7 @@
         <v>82.786</v>
       </c>
       <c r="F418">
-        <v>7014.859999999999</v>
+        <v>7014.86</v>
       </c>
       <c r="G418">
         <v>84.73485855096271</v>
@@ -47798,10 +47798,10 @@
         <v>82.786</v>
       </c>
       <c r="F421">
-        <v>6991.35</v>
+        <v>6991.349999999999</v>
       </c>
       <c r="G421">
-        <v>84.45087333607133</v>
+        <v>84.45087333607131</v>
       </c>
       <c r="H421">
         <v>190.86</v>
@@ -47813,7 +47813,7 @@
         <v>0</v>
       </c>
       <c r="K421">
-        <v>2.30546227623028</v>
+        <v>2.305462276230281</v>
       </c>
       <c r="L421">
         <v>0</v>
@@ -47834,10 +47834,10 @@
         <v>33.984</v>
       </c>
       <c r="R421">
-        <v>665.8988300000001</v>
+        <v>665.89883</v>
       </c>
       <c r="S421">
-        <v>8.043616432730174</v>
+        <v>8.043616432730172</v>
       </c>
       <c r="T421">
         <v>928.80002</v>
@@ -47989,7 +47989,7 @@
         <v>0</v>
       </c>
       <c r="AF422">
-        <v>619.7954999999999</v>
+        <v>619.7955000000001</v>
       </c>
       <c r="AG422">
         <v>0</v>
@@ -48039,7 +48039,7 @@
         <v>0</v>
       </c>
       <c r="K423">
-        <v>2.239509095740826</v>
+        <v>2.239509095740825</v>
       </c>
       <c r="L423">
         <v>0</v>
@@ -48066,7 +48066,7 @@
         <v>8.384923054622764</v>
       </c>
       <c r="T423">
-        <v>974.6299799999999</v>
+        <v>974.62998</v>
       </c>
       <c r="U423">
         <v>15</v>
@@ -48102,7 +48102,7 @@
         <v>0</v>
       </c>
       <c r="AF423">
-        <v>633.3970999999999</v>
+        <v>633.3971</v>
       </c>
       <c r="AG423">
         <v>0</v>
@@ -48250,10 +48250,10 @@
         <v>123.3666666666667</v>
       </c>
       <c r="F425">
-        <v>6150.009999999999</v>
+        <v>6150.01</v>
       </c>
       <c r="G425">
-        <v>49.85147257497973</v>
+        <v>49.85147257497974</v>
       </c>
       <c r="H425">
         <v>242.25</v>
@@ -48399,13 +48399,13 @@
         <v>32.364</v>
       </c>
       <c r="R426">
-        <v>479.2374699999999</v>
+        <v>479.23747</v>
       </c>
       <c r="S426">
         <v>3.884659308295055</v>
       </c>
       <c r="T426">
-        <v>523.5800099999999</v>
+        <v>523.58001</v>
       </c>
       <c r="U426">
         <v>12</v>
@@ -48512,10 +48512,10 @@
         <v>36</v>
       </c>
       <c r="R427">
-        <v>490.1332200000001</v>
+        <v>490.13322</v>
       </c>
       <c r="S427">
-        <v>3.97297935693056</v>
+        <v>3.972979356930559</v>
       </c>
       <c r="T427">
         <v>862.80999</v>
@@ -48589,10 +48589,10 @@
         <v>123.3666666666667</v>
       </c>
       <c r="F428">
-        <v>6197.799999999999</v>
+        <v>6197.8</v>
       </c>
       <c r="G428">
-        <v>50.23885436368549</v>
+        <v>50.2388543636855</v>
       </c>
       <c r="H428">
         <v>340.18</v>
@@ -48780,7 +48780,7 @@
         <v>0</v>
       </c>
       <c r="AF429">
-        <v>586.6687999999999</v>
+        <v>586.6688</v>
       </c>
       <c r="AG429">
         <v>0</v>
@@ -48857,7 +48857,7 @@
         <v>5.232585571467172</v>
       </c>
       <c r="T430">
-        <v>896.0200100000001</v>
+        <v>896.02001</v>
       </c>
       <c r="U430">
         <v>27</v>
@@ -49157,7 +49157,7 @@
         <v>5822.77</v>
       </c>
       <c r="G433">
-        <v>47.19889219129965</v>
+        <v>47.19889219129966</v>
       </c>
       <c r="H433">
         <v>219.36</v>
@@ -49196,7 +49196,7 @@
         <v>4.354627830316131</v>
       </c>
       <c r="T433">
-        <v>805.6300100000001</v>
+        <v>805.63001</v>
       </c>
       <c r="U433">
         <v>36</v>
@@ -49309,7 +49309,7 @@
         <v>4.262872331802216</v>
       </c>
       <c r="T434">
-        <v>813.8</v>
+        <v>813.8000000000001</v>
       </c>
       <c r="U434">
         <v>33</v>
@@ -49422,7 +49422,7 @@
         <v>5.103673601729263</v>
       </c>
       <c r="T435">
-        <v>971.1299899999999</v>
+        <v>971.12999</v>
       </c>
       <c r="U435">
         <v>33</v>
@@ -49493,10 +49493,10 @@
         <v>123.3666666666667</v>
       </c>
       <c r="F436">
-        <v>5654.819999999999</v>
+        <v>5654.82</v>
       </c>
       <c r="G436">
-        <v>45.83750337746554</v>
+        <v>45.83750337746555</v>
       </c>
       <c r="H436">
         <v>149.9</v>
@@ -49535,7 +49535,7 @@
         <v>4.134675628208592</v>
       </c>
       <c r="T436">
-        <v>674.77001</v>
+        <v>674.7700100000001</v>
       </c>
       <c r="U436">
         <v>26</v>
@@ -49719,10 +49719,10 @@
         <v>123.3666666666667</v>
       </c>
       <c r="F438">
-        <v>5664.949999999999</v>
+        <v>5664.95</v>
       </c>
       <c r="G438">
-        <v>45.91961631991353</v>
+        <v>45.91961631991354</v>
       </c>
       <c r="H438">
         <v>71.28999999999999</v>
@@ -49868,7 +49868,7 @@
         <v>33.984</v>
       </c>
       <c r="R439">
-        <v>515.9606199999999</v>
+        <v>515.9606200000001</v>
       </c>
       <c r="S439">
         <v>4.182334125911916</v>
@@ -49910,7 +49910,7 @@
         <v>0</v>
       </c>
       <c r="AF439">
-        <v>457.3272</v>
+        <v>457.3272000000001</v>
       </c>
       <c r="AG439">
         <v>0</v>
@@ -49987,7 +49987,7 @@
         <v>5.039024127230411</v>
       </c>
       <c r="T440">
-        <v>989.8799899999999</v>
+        <v>989.87999</v>
       </c>
       <c r="U440">
         <v>33</v>
@@ -50320,10 +50320,10 @@
         <v>36</v>
       </c>
       <c r="R443">
-        <v>630.8728900000001</v>
+        <v>630.87289</v>
       </c>
       <c r="S443">
-        <v>5.113803485544448</v>
+        <v>5.113803485544447</v>
       </c>
       <c r="T443">
         <v>643.67001</v>
@@ -51078,7 +51078,7 @@
         <v>2883.05</v>
       </c>
       <c r="G450">
-        <v>38.51770207080828</v>
+        <v>38.51770207080829</v>
       </c>
       <c r="H450">
         <v>27.81</v>
@@ -51227,7 +51227,7 @@
         <v>221.19235</v>
       </c>
       <c r="S451">
-        <v>2.955141616566467</v>
+        <v>2.955141616566466</v>
       </c>
       <c r="T451">
         <v>135.37</v>
@@ -51275,7 +51275,7 @@
         <v>3</v>
       </c>
       <c r="AI451">
-        <v>663.57705</v>
+        <v>663.5770499999999</v>
       </c>
     </row>
     <row r="452">
@@ -51414,7 +51414,7 @@
         <v>74.84999999999999</v>
       </c>
       <c r="F453">
-        <v>2910.920000000001</v>
+        <v>2910.92</v>
       </c>
       <c r="G453">
         <v>38.89004676018705</v>
@@ -51679,7 +51679,7 @@
         <v>274.03416</v>
       </c>
       <c r="S455">
-        <v>3.661111022044089</v>
+        <v>3.661111022044088</v>
       </c>
       <c r="T455">
         <v>218.47999</v>
@@ -51727,7 +51727,7 @@
         <v>3</v>
       </c>
       <c r="AI455">
-        <v>822.1024800000001</v>
+        <v>822.10248</v>
       </c>
     </row>
     <row r="456">
@@ -51982,7 +51982,7 @@
         <v>2409.22</v>
       </c>
       <c r="G458">
-        <v>32.1873079492318</v>
+        <v>32.18730794923179</v>
       </c>
       <c r="H458">
         <v>7.66</v>
@@ -52131,7 +52131,7 @@
         <v>370.68996</v>
       </c>
       <c r="S459">
-        <v>4.952437675350701</v>
+        <v>4.952437675350702</v>
       </c>
       <c r="T459">
         <v>280.19001</v>
@@ -52205,10 +52205,10 @@
         <v>74.84999999999999</v>
       </c>
       <c r="F460">
-        <v>2667.510000000001</v>
+        <v>2667.51</v>
       </c>
       <c r="G460">
-        <v>35.63807615230462</v>
+        <v>35.63807615230461</v>
       </c>
       <c r="H460">
         <v>26.4</v>
@@ -52547,7 +52547,7 @@
         <v>7942.88</v>
       </c>
       <c r="G463">
-        <v>76.07478932976616</v>
+        <v>76.07478932976615</v>
       </c>
       <c r="H463">
         <v>73.33</v>
@@ -52559,7 +52559,7 @@
         <v>0</v>
       </c>
       <c r="K463">
-        <v>0.7023352111012319</v>
+        <v>0.7023352111012318</v>
       </c>
       <c r="L463">
         <v>0</v>
@@ -52586,7 +52586,7 @@
         <v>8.551147843493446</v>
       </c>
       <c r="T463">
-        <v>997.6400100000001</v>
+        <v>997.64001</v>
       </c>
       <c r="U463">
         <v>24</v>
@@ -52663,7 +52663,7 @@
         <v>109.3697795253476</v>
       </c>
       <c r="H464">
-        <v>439.75</v>
+        <v>439.7500000000001</v>
       </c>
       <c r="I464">
         <v>0</v>
@@ -52672,7 +52672,7 @@
         <v>0</v>
       </c>
       <c r="K464">
-        <v>3.705238028366802</v>
+        <v>3.705238028366803</v>
       </c>
       <c r="L464">
         <v>0</v>
@@ -52744,7 +52744,7 @@
         <v>3</v>
       </c>
       <c r="AI464">
-        <v>3865.349580000001</v>
+        <v>3865.34958</v>
       </c>
     </row>
     <row r="465">
@@ -52773,7 +52773,7 @@
         <v>8245.290000000001</v>
       </c>
       <c r="G465">
-        <v>78.97119177336529</v>
+        <v>78.97119177336528</v>
       </c>
       <c r="H465">
         <v>64.61</v>
@@ -52785,7 +52785,7 @@
         <v>0</v>
       </c>
       <c r="K465">
-        <v>0.6188173733703886</v>
+        <v>0.6188173733703884</v>
       </c>
       <c r="L465">
         <v>0</v>
@@ -52809,7 +52809,7 @@
         <v>758.64987</v>
       </c>
       <c r="S465">
-        <v>7.266146414814838</v>
+        <v>7.266146414814837</v>
       </c>
       <c r="T465">
         <v>1022.57999</v>
@@ -52889,7 +52889,7 @@
         <v>74.26771520853812</v>
       </c>
       <c r="H466">
-        <v>630.75</v>
+        <v>630.7499999999999</v>
       </c>
       <c r="I466">
         <v>0</v>
@@ -52898,7 +52898,7 @@
         <v>0</v>
       </c>
       <c r="K466">
-        <v>5.314562561438001</v>
+        <v>5.314562561437999</v>
       </c>
       <c r="L466">
         <v>0</v>
@@ -53112,7 +53112,7 @@
         <v>10557.06</v>
       </c>
       <c r="G468">
-        <v>73.25754956034388</v>
+        <v>73.25754956034386</v>
       </c>
       <c r="H468">
         <v>393.02</v>
@@ -53124,7 +53124,7 @@
         <v>0</v>
       </c>
       <c r="K468">
-        <v>2.727244339636826</v>
+        <v>2.727244339636825</v>
       </c>
       <c r="L468">
         <v>17</v>
@@ -53148,7 +53148,7 @@
         <v>974.85178</v>
       </c>
       <c r="S468">
-        <v>6.764691361737022</v>
+        <v>6.76469136173702</v>
       </c>
       <c r="T468">
         <v>1286.53002</v>
@@ -53187,7 +53187,7 @@
         <v>0</v>
       </c>
       <c r="AF468">
-        <v>984.1967999999999</v>
+        <v>984.1968000000001</v>
       </c>
       <c r="AG468">
         <v>0</v>
@@ -53225,7 +53225,7 @@
         <v>8401.360000000001</v>
       </c>
       <c r="G469">
-        <v>80.46598866954106</v>
+        <v>80.46598866954105</v>
       </c>
       <c r="H469">
         <v>269.33</v>
@@ -53258,10 +53258,10 @@
         <v>36</v>
       </c>
       <c r="R469">
-        <v>911.1489800000001</v>
+        <v>911.1489799999999</v>
       </c>
       <c r="S469">
-        <v>8.726742277553145</v>
+        <v>8.726742277553143</v>
       </c>
       <c r="T469">
         <v>1145.07</v>
@@ -53335,13 +53335,13 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F470">
-        <v>9166.879999999999</v>
+        <v>9166.880000000001</v>
       </c>
       <c r="G470">
         <v>87.79793535987535</v>
       </c>
       <c r="H470">
-        <v>561.5500000000001</v>
+        <v>561.55</v>
       </c>
       <c r="I470">
         <v>0</v>
@@ -53350,7 +53350,7 @@
         <v>0</v>
       </c>
       <c r="K470">
-        <v>5.378376350659987</v>
+        <v>5.378376350659985</v>
       </c>
       <c r="L470">
         <v>0</v>
@@ -53374,7 +53374,7 @@
         <v>942.98865</v>
       </c>
       <c r="S470">
-        <v>9.031694157422823</v>
+        <v>9.031694157422821</v>
       </c>
       <c r="T470">
         <v>1737.96997</v>
@@ -53451,7 +53451,7 @@
         <v>12147.03</v>
       </c>
       <c r="G471">
-        <v>102.3482376070777</v>
+        <v>102.3482376070776</v>
       </c>
       <c r="H471">
         <v>679.13</v>
@@ -53713,7 +53713,7 @@
         <v>1060.24183</v>
       </c>
       <c r="S473">
-        <v>8.933367476478024</v>
+        <v>8.933367476478022</v>
       </c>
       <c r="T473">
         <v>1760.26001</v>
@@ -53761,7 +53761,7 @@
         <v>3</v>
       </c>
       <c r="AI473">
-        <v>3180.725490000001</v>
+        <v>3180.72549</v>
       </c>
     </row>
     <row r="474">
@@ -53826,10 +53826,10 @@
         <v>753.73544</v>
       </c>
       <c r="S474">
-        <v>7.219077313062592</v>
+        <v>7.219077313062591</v>
       </c>
       <c r="T474">
-        <v>868.2500199999999</v>
+        <v>868.2500200000001</v>
       </c>
       <c r="U474">
         <v>29</v>
@@ -53865,7 +53865,7 @@
         <v>0</v>
       </c>
       <c r="AF474">
-        <v>738.1687999999999</v>
+        <v>738.1688</v>
       </c>
       <c r="AG474">
         <v>0</v>
@@ -54013,7 +54013,7 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F476">
-        <v>8535.219999999999</v>
+        <v>8535.220000000001</v>
       </c>
       <c r="G476">
         <v>81.74806410057897</v>
@@ -54052,7 +54052,7 @@
         <v>961.49793</v>
       </c>
       <c r="S476">
-        <v>9.208971111958919</v>
+        <v>9.208971111958917</v>
       </c>
       <c r="T476">
         <v>1062.57997</v>
@@ -54242,7 +54242,7 @@
         <v>8115.679999999999</v>
       </c>
       <c r="G478">
-        <v>77.72982171048746</v>
+        <v>77.72982171048744</v>
       </c>
       <c r="H478">
         <v>88.55</v>
@@ -54254,7 +54254,7 @@
         <v>0</v>
       </c>
       <c r="K478">
-        <v>0.8481083177828185</v>
+        <v>0.8481083177828184</v>
       </c>
       <c r="L478">
         <v>0</v>
@@ -54275,10 +54275,10 @@
         <v>34.992</v>
       </c>
       <c r="R478">
-        <v>779.81077</v>
+        <v>779.8107699999999</v>
       </c>
       <c r="S478">
-        <v>7.468819879544037</v>
+        <v>7.468819879544034</v>
       </c>
       <c r="T478">
         <v>1096.76</v>
@@ -54391,7 +54391,7 @@
         <v>1015.18162</v>
       </c>
       <c r="S479">
-        <v>8.553699929785143</v>
+        <v>8.553699929785141</v>
       </c>
       <c r="T479">
         <v>1757.73005</v>
@@ -54504,7 +54504,7 @@
         <v>1159.66443</v>
       </c>
       <c r="S480">
-        <v>9.771080719000141</v>
+        <v>9.771080719000139</v>
       </c>
       <c r="T480">
         <v>1902.56003</v>
@@ -54552,7 +54552,7 @@
         <v>3</v>
       </c>
       <c r="AI480">
-        <v>3478.99329</v>
+        <v>3478.993289999999</v>
       </c>
     </row>
     <row r="481">
@@ -54614,7 +54614,7 @@
         <v>36</v>
       </c>
       <c r="R481">
-        <v>960.2233599999998</v>
+        <v>960.22336</v>
       </c>
       <c r="S481">
         <v>9.19676361993637</v>
@@ -54665,7 +54665,7 @@
         <v>3</v>
       </c>
       <c r="AI481">
-        <v>2880.670079999999</v>
+        <v>2880.67008</v>
       </c>
     </row>
     <row r="482">
@@ -54917,7 +54917,7 @@
         <v>117.7666666666667</v>
       </c>
       <c r="F484">
-        <v>6135.540000000001</v>
+        <v>6135.54</v>
       </c>
       <c r="G484">
         <v>52.09912255873196</v>
@@ -54953,13 +54953,13 @@
         <v>36</v>
       </c>
       <c r="R484">
-        <v>679.6586500000001</v>
+        <v>679.65865</v>
       </c>
       <c r="S484">
-        <v>5.771231106708181</v>
+        <v>5.771231106708179</v>
       </c>
       <c r="T484">
-        <v>796.9999800000001</v>
+        <v>796.9999799999999</v>
       </c>
       <c r="U484">
         <v>46</v>
@@ -55143,10 +55143,10 @@
         <v>117.7666666666667</v>
       </c>
       <c r="F486">
-        <v>6514.990000000001</v>
+        <v>6514.99</v>
       </c>
       <c r="G486">
-        <v>55.3211718086612</v>
+        <v>55.32117180866119</v>
       </c>
       <c r="H486">
         <v>23.79</v>
@@ -55185,7 +55185,7 @@
         <v>8.391884715539202</v>
       </c>
       <c r="T486">
-        <v>807.9900100000001</v>
+        <v>807.99001</v>
       </c>
       <c r="U486">
         <v>45</v>
@@ -55976,7 +55976,7 @@
         <v>6.328116105292952</v>
       </c>
       <c r="T493">
-        <v>532.19999</v>
+        <v>532.1999900000001</v>
       </c>
       <c r="U493">
         <v>29</v>
@@ -56160,7 +56160,7 @@
         <v>117.7666666666667</v>
       </c>
       <c r="F495">
-        <v>5161.339999999999</v>
+        <v>5161.34</v>
       </c>
       <c r="G495">
         <v>43.82683272006793</v>
@@ -56196,10 +56196,10 @@
         <v>36</v>
       </c>
       <c r="R495">
-        <v>807.4213899999999</v>
+        <v>807.42139</v>
       </c>
       <c r="S495">
-        <v>6.856111435041041</v>
+        <v>6.856111435041042</v>
       </c>
       <c r="T495">
         <v>382.29999</v>
@@ -56247,7 +56247,7 @@
         <v>3</v>
       </c>
       <c r="AI495">
-        <v>2422.264169999999</v>
+        <v>2422.26417</v>
       </c>
     </row>
     <row r="496">
@@ -56422,10 +56422,10 @@
         <v>33.012</v>
       </c>
       <c r="R497">
-        <v>813.6347699999999</v>
+        <v>813.63477</v>
       </c>
       <c r="S497">
-        <v>6.908871525615623</v>
+        <v>6.908871525615624</v>
       </c>
       <c r="T497">
         <v>499.65001</v>
@@ -56535,10 +56535,10 @@
         <v>34.92</v>
       </c>
       <c r="R498">
-        <v>660.7064300000001</v>
+        <v>660.70643</v>
       </c>
       <c r="S498">
-        <v>5.610300849136712</v>
+        <v>5.610300849136711</v>
       </c>
       <c r="T498">
         <v>635.0899900000001</v>
@@ -56761,10 +56761,10 @@
         <v>36</v>
       </c>
       <c r="R500">
-        <v>787.8786699999999</v>
+        <v>787.8786700000001</v>
       </c>
       <c r="S500">
-        <v>6.690167025191055</v>
+        <v>6.690167025191056</v>
       </c>
       <c r="T500">
         <v>892.57001</v>
@@ -56951,10 +56951,10 @@
         <v>117.7666666666667</v>
       </c>
       <c r="F502">
-        <v>4848.929999999999</v>
+        <v>4848.93</v>
       </c>
       <c r="G502">
-        <v>41.17404472120011</v>
+        <v>41.17404472120012</v>
       </c>
       <c r="H502">
         <v>0</v>
@@ -56987,13 +56987,13 @@
         <v>34.992</v>
       </c>
       <c r="R502">
-        <v>650.5084999999999</v>
+        <v>650.5085</v>
       </c>
       <c r="S502">
-        <v>5.52370648174356</v>
+        <v>5.523706481743561</v>
       </c>
       <c r="T502">
-        <v>692.0100100000001</v>
+        <v>692.01001</v>
       </c>
       <c r="U502">
         <v>50</v>
@@ -57558,7 +57558,7 @@
         <v>5.851755505236343</v>
       </c>
       <c r="T507">
-        <v>637.0600099999999</v>
+        <v>637.06001</v>
       </c>
       <c r="U507">
         <v>37</v>
@@ -57594,7 +57594,7 @@
         <v>0</v>
       </c>
       <c r="AF507">
-        <v>484.5953000000001</v>
+        <v>484.5953</v>
       </c>
       <c r="AG507">
         <v>0</v>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-15
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI508"/>
+  <dimension ref="A1:AI534"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -52544,10 +52544,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F463">
-        <v>7942.88</v>
+        <v>7942.790000000001</v>
       </c>
       <c r="G463">
-        <v>76.07478932976615</v>
+        <v>76.07392733373453</v>
       </c>
       <c r="H463">
         <v>73.33</v>
@@ -52580,10 +52580,10 @@
         <v>36</v>
       </c>
       <c r="R463">
-        <v>892.81537</v>
+        <v>892.812</v>
       </c>
       <c r="S463">
-        <v>8.551147843493446</v>
+        <v>8.551115566530928</v>
       </c>
       <c r="T463">
         <v>997.64001</v>
@@ -52622,7 +52622,7 @@
         <v>0</v>
       </c>
       <c r="AF463">
-        <v>1895.784</v>
+        <v>1895.764</v>
       </c>
       <c r="AG463">
         <v>0</v>
@@ -52631,7 +52631,7 @@
         <v>3</v>
       </c>
       <c r="AI463">
-        <v>2678.44611</v>
+        <v>2678.436</v>
       </c>
     </row>
     <row r="464">
@@ -52654,13 +52654,13 @@
         </is>
       </c>
       <c r="E464">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F464">
-        <v>12980.37</v>
+        <v>12980.42</v>
       </c>
       <c r="G464">
-        <v>109.3697795253476</v>
+        <v>109.3662076654974</v>
       </c>
       <c r="H464">
         <v>439.7500000000001</v>
@@ -52672,7 +52672,7 @@
         <v>0</v>
       </c>
       <c r="K464">
-        <v>3.705238028366803</v>
+        <v>3.705102748670881</v>
       </c>
       <c r="L464">
         <v>0</v>
@@ -52693,10 +52693,10 @@
         <v>32.364</v>
       </c>
       <c r="R464">
-        <v>1288.44986</v>
+        <v>1288.44267</v>
       </c>
       <c r="S464">
-        <v>10.85619879230445</v>
+        <v>10.8557418490548</v>
       </c>
       <c r="T464">
         <v>1910.85997</v>
@@ -52735,7 +52735,7 @@
         <v>0</v>
       </c>
       <c r="AF464">
-        <v>1041.2675</v>
+        <v>1041.2724</v>
       </c>
       <c r="AG464">
         <v>0</v>
@@ -52744,7 +52744,7 @@
         <v>3</v>
       </c>
       <c r="AI464">
-        <v>3865.34958</v>
+        <v>3865.32801</v>
       </c>
     </row>
     <row r="465">
@@ -52770,10 +52770,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F465">
-        <v>8245.290000000001</v>
+        <v>8245.18</v>
       </c>
       <c r="G465">
-        <v>78.97119177336528</v>
+        <v>78.97013822265995</v>
       </c>
       <c r="H465">
         <v>64.61</v>
@@ -52806,10 +52806,10 @@
         <v>36</v>
       </c>
       <c r="R465">
-        <v>758.64987</v>
+        <v>758.64167</v>
       </c>
       <c r="S465">
-        <v>7.266146414814837</v>
+        <v>7.266067877398623</v>
       </c>
       <c r="T465">
         <v>1022.57999</v>
@@ -52848,7 +52848,7 @@
         <v>0</v>
       </c>
       <c r="AF465">
-        <v>1965.396</v>
+        <v>1965.372</v>
       </c>
       <c r="AG465">
         <v>0</v>
@@ -52857,7 +52857,7 @@
         <v>3</v>
       </c>
       <c r="AI465">
-        <v>2275.94961</v>
+        <v>2275.92501</v>
       </c>
     </row>
     <row r="466">
@@ -52880,13 +52880,13 @@
         </is>
       </c>
       <c r="E466">
-        <v>118.6833333333333</v>
+        <v>83.94883333333334</v>
       </c>
       <c r="F466">
-        <v>8814.34</v>
+        <v>8814.199999999999</v>
       </c>
       <c r="G466">
-        <v>74.26771520853812</v>
+        <v>104.994907612375</v>
       </c>
       <c r="H466">
         <v>630.7499999999999</v>
@@ -52898,7 +52898,7 @@
         <v>0</v>
       </c>
       <c r="K466">
-        <v>5.314562561437999</v>
+        <v>7.51350525022186</v>
       </c>
       <c r="L466">
         <v>0</v>
@@ -52919,10 +52919,10 @@
         <v>32.4</v>
       </c>
       <c r="R466">
-        <v>1003.62671</v>
+        <v>1003.58479</v>
       </c>
       <c r="S466">
-        <v>8.456340766746242</v>
+        <v>11.95471991868063</v>
       </c>
       <c r="T466">
         <v>2026.33995</v>
@@ -52961,7 +52961,7 @@
         <v>0</v>
       </c>
       <c r="AF466">
-        <v>752.0296</v>
+        <v>752.0205</v>
       </c>
       <c r="AG466">
         <v>0</v>
@@ -52970,7 +52970,7 @@
         <v>3</v>
       </c>
       <c r="AI466">
-        <v>3010.88013</v>
+        <v>3010.754370000001</v>
       </c>
     </row>
     <row r="467">
@@ -52993,13 +52993,13 @@
         </is>
       </c>
       <c r="E467">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F467">
-        <v>11041.99</v>
+        <v>11041.83</v>
       </c>
       <c r="G467">
-        <v>93.03741047605673</v>
+        <v>93.03266556761024</v>
       </c>
       <c r="H467">
         <v>575.87</v>
@@ -53011,7 +53011,7 @@
         <v>0</v>
       </c>
       <c r="K467">
-        <v>4.85215559612414</v>
+        <v>4.851978442017283</v>
       </c>
       <c r="L467">
         <v>0</v>
@@ -53032,10 +53032,10 @@
         <v>33.984</v>
       </c>
       <c r="R467">
-        <v>1232.02074</v>
+        <v>1232.01593</v>
       </c>
       <c r="S467">
-        <v>10.38073927819126</v>
+        <v>10.38031974678638</v>
       </c>
       <c r="T467">
         <v>1786.97001</v>
@@ -53074,7 +53074,7 @@
         <v>0</v>
       </c>
       <c r="AF467">
-        <v>1047.504</v>
+        <v>1047.4944</v>
       </c>
       <c r="AG467">
         <v>0</v>
@@ -53083,7 +53083,7 @@
         <v>3</v>
       </c>
       <c r="AI467">
-        <v>3696.06222</v>
+        <v>3696.04779</v>
       </c>
     </row>
     <row r="468">
@@ -53106,13 +53106,13 @@
         </is>
       </c>
       <c r="E468">
-        <v>144.1088333333333</v>
+        <v>136.2401666666667</v>
       </c>
       <c r="F468">
-        <v>10557.06</v>
+        <v>10423.16</v>
       </c>
       <c r="G468">
-        <v>73.25754956034386</v>
+        <v>76.50577839868566</v>
       </c>
       <c r="H468">
         <v>393.02</v>
@@ -53124,7 +53124,7 @@
         <v>0</v>
       </c>
       <c r="K468">
-        <v>2.727244339636825</v>
+        <v>2.88475865536473</v>
       </c>
       <c r="L468">
         <v>17</v>
@@ -53145,10 +53145,10 @@
         <v>35.568</v>
       </c>
       <c r="R468">
-        <v>974.85178</v>
+        <v>953.3875800000001</v>
       </c>
       <c r="S468">
-        <v>6.76469136173702</v>
+        <v>6.997845079950726</v>
       </c>
       <c r="T468">
         <v>1286.53002</v>
@@ -53187,7 +53187,7 @@
         <v>0</v>
       </c>
       <c r="AF468">
-        <v>984.1968000000001</v>
+        <v>974.9488</v>
       </c>
       <c r="AG468">
         <v>0</v>
@@ -53196,7 +53196,7 @@
         <v>3</v>
       </c>
       <c r="AI468">
-        <v>2924.55534</v>
+        <v>2860.16274</v>
       </c>
     </row>
     <row r="469">
@@ -53222,10 +53222,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F469">
-        <v>8401.360000000001</v>
+        <v>8401.25</v>
       </c>
       <c r="G469">
-        <v>80.46598866954105</v>
+        <v>80.46493511883573</v>
       </c>
       <c r="H469">
         <v>269.33</v>
@@ -53258,10 +53258,10 @@
         <v>36</v>
       </c>
       <c r="R469">
-        <v>911.1489799999999</v>
+        <v>911.14175</v>
       </c>
       <c r="S469">
-        <v>8.726742277553143</v>
+        <v>8.726673030538603</v>
       </c>
       <c r="T469">
         <v>1145.07</v>
@@ -53300,7 +53300,7 @@
         <v>0</v>
       </c>
       <c r="AF469">
-        <v>1939.15</v>
+        <v>1939.126</v>
       </c>
       <c r="AG469">
         <v>0</v>
@@ -53309,7 +53309,7 @@
         <v>3</v>
       </c>
       <c r="AI469">
-        <v>2733.44694</v>
+        <v>2733.42525</v>
       </c>
     </row>
     <row r="470">
@@ -53335,10 +53335,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F470">
-        <v>9166.880000000001</v>
+        <v>9166.75</v>
       </c>
       <c r="G470">
-        <v>87.79793535987535</v>
+        <v>87.79669025449634</v>
       </c>
       <c r="H470">
         <v>561.55</v>
@@ -53371,10 +53371,10 @@
         <v>36</v>
       </c>
       <c r="R470">
-        <v>942.98865</v>
+        <v>942.98053</v>
       </c>
       <c r="S470">
-        <v>9.031694157422821</v>
+        <v>9.031616386225302</v>
       </c>
       <c r="T470">
         <v>1737.96997</v>
@@ -53413,7 +53413,7 @@
         <v>0</v>
       </c>
       <c r="AF470">
-        <v>770.5243</v>
+        <v>770.5145</v>
       </c>
       <c r="AG470">
         <v>0</v>
@@ -53422,7 +53422,7 @@
         <v>3</v>
       </c>
       <c r="AI470">
-        <v>2828.96595</v>
+        <v>2828.94159</v>
       </c>
     </row>
     <row r="471">
@@ -53445,13 +53445,13 @@
         </is>
       </c>
       <c r="E471">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F471">
-        <v>12147.03</v>
+        <v>12146.9</v>
       </c>
       <c r="G471">
-        <v>102.3482376070776</v>
+        <v>102.3434055209331</v>
       </c>
       <c r="H471">
         <v>679.13</v>
@@ -53463,7 +53463,7 @@
         <v>2</v>
       </c>
       <c r="K471">
-        <v>5.722201937930066</v>
+        <v>5.721993018089495</v>
       </c>
       <c r="L471">
         <v>6.54</v>
@@ -53484,10 +53484,10 @@
         <v>32.004</v>
       </c>
       <c r="R471">
-        <v>1401.87338</v>
+        <v>1401.84314</v>
       </c>
       <c r="S471">
-        <v>11.81188074708608</v>
+        <v>11.81119470430794</v>
       </c>
       <c r="T471">
         <v>2002.32997</v>
@@ -53526,7 +53526,7 @@
         <v>0</v>
       </c>
       <c r="AF471">
-        <v>853.2570000000001</v>
+        <v>853.2468</v>
       </c>
       <c r="AG471">
         <v>0</v>
@@ -53535,7 +53535,7 @@
         <v>3</v>
       </c>
       <c r="AI471">
-        <v>4205.62014</v>
+        <v>4205.52942</v>
       </c>
     </row>
     <row r="472">
@@ -53558,13 +53558,13 @@
         </is>
       </c>
       <c r="E472">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F472">
-        <v>11274.05</v>
+        <v>11274.12</v>
       </c>
       <c r="G472">
-        <v>94.99269765482376</v>
+        <v>94.98981921738569</v>
       </c>
       <c r="H472">
         <v>401.57</v>
@@ -53576,7 +53576,7 @@
         <v>0</v>
       </c>
       <c r="K472">
-        <v>3.383541637410476</v>
+        <v>3.383418102976159</v>
       </c>
       <c r="L472">
         <v>0</v>
@@ -53597,10 +53597,10 @@
         <v>33.696</v>
       </c>
       <c r="R472">
-        <v>1266.27814</v>
+        <v>1266.29706</v>
       </c>
       <c r="S472">
-        <v>10.66938469316107</v>
+        <v>10.66915455972679</v>
       </c>
       <c r="T472">
         <v>1777.72999</v>
@@ -53639,7 +53639,7 @@
         <v>0</v>
       </c>
       <c r="AF472">
-        <v>1086.4512</v>
+        <v>1086.4576</v>
       </c>
       <c r="AG472">
         <v>0</v>
@@ -53648,7 +53648,7 @@
         <v>3</v>
       </c>
       <c r="AI472">
-        <v>3798.83442</v>
+        <v>3798.89118</v>
       </c>
     </row>
     <row r="473">
@@ -53671,13 +53671,13 @@
         </is>
       </c>
       <c r="E473">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F473">
-        <v>12573.11</v>
+        <v>12573.24</v>
       </c>
       <c r="G473">
-        <v>105.9382951832608</v>
+        <v>105.9355226462733</v>
       </c>
       <c r="H473">
         <v>593.35</v>
@@ -53689,7 +53689,7 @@
         <v>0</v>
       </c>
       <c r="K473">
-        <v>4.999438281140289</v>
+        <v>4.999255749684747</v>
       </c>
       <c r="L473">
         <v>0</v>
@@ -53710,10 +53710,10 @@
         <v>34.992</v>
       </c>
       <c r="R473">
-        <v>1060.24183</v>
+        <v>1060.24579</v>
       </c>
       <c r="S473">
-        <v>8.933367476478022</v>
+        <v>8.933074680604275</v>
       </c>
       <c r="T473">
         <v>1760.26001</v>
@@ -53752,7 +53752,7 @@
         <v>0</v>
       </c>
       <c r="AF473">
-        <v>1005.56874</v>
+        <v>1005.5784</v>
       </c>
       <c r="AG473">
         <v>0</v>
@@ -53761,7 +53761,7 @@
         <v>3</v>
       </c>
       <c r="AI473">
-        <v>3180.72549</v>
+        <v>3180.73737</v>
       </c>
     </row>
     <row r="474">
@@ -53897,13 +53897,13 @@
         </is>
       </c>
       <c r="E475">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F475">
-        <v>12563.19</v>
+        <v>12563.24</v>
       </c>
       <c r="G475">
-        <v>105.8547114169358</v>
+        <v>105.8512678936031</v>
       </c>
       <c r="H475">
         <v>923.25</v>
@@ -53915,7 +53915,7 @@
         <v>0</v>
       </c>
       <c r="K475">
-        <v>7.779104058418761</v>
+        <v>7.778820040273771</v>
       </c>
       <c r="L475">
         <v>14.05</v>
@@ -53936,10 +53936,10 @@
         <v>34.992</v>
       </c>
       <c r="R475">
-        <v>1031.73775</v>
+        <v>1031.7324</v>
       </c>
       <c r="S475">
-        <v>8.693198286757477</v>
+        <v>8.692835818380454</v>
       </c>
       <c r="T475">
         <v>2432.64001</v>
@@ -53978,7 +53978,7 @@
         <v>0</v>
       </c>
       <c r="AF475">
-        <v>1079.50956</v>
+        <v>1079.51737</v>
       </c>
       <c r="AG475">
         <v>0</v>
@@ -53987,7 +53987,7 @@
         <v>3</v>
       </c>
       <c r="AI475">
-        <v>3095.21325</v>
+        <v>3095.1972</v>
       </c>
     </row>
     <row r="476">
@@ -54013,10 +54013,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F476">
-        <v>8535.220000000001</v>
+        <v>8535.130000000001</v>
       </c>
       <c r="G476">
-        <v>81.74806410057897</v>
+        <v>81.74720210454734</v>
       </c>
       <c r="H476">
         <v>81.41000000000001</v>
@@ -54049,10 +54049,10 @@
         <v>36</v>
       </c>
       <c r="R476">
-        <v>961.49793</v>
+        <v>961.49104</v>
       </c>
       <c r="S476">
-        <v>9.208971111958917</v>
+        <v>9.208905121373828</v>
       </c>
       <c r="T476">
         <v>1062.57997</v>
@@ -54091,7 +54091,7 @@
         <v>0</v>
       </c>
       <c r="AF476">
-        <v>2015.572</v>
+        <v>2015.548</v>
       </c>
       <c r="AG476">
         <v>0</v>
@@ -54100,7 +54100,7 @@
         <v>3</v>
       </c>
       <c r="AI476">
-        <v>2884.49379</v>
+        <v>2884.47312</v>
       </c>
     </row>
     <row r="477">
@@ -54123,13 +54123,13 @@
         </is>
       </c>
       <c r="E477">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F477">
-        <v>11508.15</v>
+        <v>11508.26</v>
       </c>
       <c r="G477">
-        <v>96.96517343069794</v>
+        <v>96.96255999640513</v>
       </c>
       <c r="H477">
         <v>399.68</v>
@@ -54141,7 +54141,7 @@
         <v>1</v>
       </c>
       <c r="K477">
-        <v>3.367616907737677</v>
+        <v>3.367493954721496</v>
       </c>
       <c r="L477">
         <v>12.38</v>
@@ -54162,10 +54162,10 @@
         <v>33.984</v>
       </c>
       <c r="R477">
-        <v>1148.67422</v>
+        <v>1148.66217</v>
       </c>
       <c r="S477">
-        <v>9.678479595562422</v>
+        <v>9.678024703493483</v>
       </c>
       <c r="T477">
         <v>1610.31998</v>
@@ -54204,7 +54204,7 @@
         <v>0</v>
       </c>
       <c r="AF477">
-        <v>1080.0624</v>
+        <v>1080.072</v>
       </c>
       <c r="AG477">
         <v>0</v>
@@ -54213,7 +54213,7 @@
         <v>3</v>
       </c>
       <c r="AI477">
-        <v>3446.022660000001</v>
+        <v>3445.98651</v>
       </c>
     </row>
     <row r="478">
@@ -54239,10 +54239,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F478">
-        <v>8115.679999999999</v>
+        <v>8115.590000000001</v>
       </c>
       <c r="G478">
-        <v>77.72982171048744</v>
+        <v>77.72895971445583</v>
       </c>
       <c r="H478">
         <v>88.55</v>
@@ -54275,10 +54275,10 @@
         <v>34.992</v>
       </c>
       <c r="R478">
-        <v>779.8107699999999</v>
+        <v>779.8064899999999</v>
       </c>
       <c r="S478">
-        <v>7.468819879544034</v>
+        <v>7.468778886843864</v>
       </c>
       <c r="T478">
         <v>1096.76</v>
@@ -54317,7 +54317,7 @@
         <v>0</v>
       </c>
       <c r="AF478">
-        <v>764.7791999999999</v>
+        <v>764.7744</v>
       </c>
       <c r="AG478">
         <v>0</v>
@@ -54326,7 +54326,7 @@
         <v>3</v>
       </c>
       <c r="AI478">
-        <v>2339.43231</v>
+        <v>2339.41947</v>
       </c>
     </row>
     <row r="479">
@@ -54349,13 +54349,13 @@
         </is>
       </c>
       <c r="E479">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F479">
         <v>11277.12</v>
       </c>
       <c r="G479">
-        <v>95.01856480831344</v>
+        <v>95.01509564318674</v>
       </c>
       <c r="H479">
         <v>586.1899999999999</v>
@@ -54367,7 +54367,7 @@
         <v>1</v>
       </c>
       <c r="K479">
-        <v>4.939109675607358</v>
+        <v>4.938929346772902</v>
       </c>
       <c r="L479">
         <v>14.18</v>
@@ -54388,10 +54388,10 @@
         <v>33.012</v>
       </c>
       <c r="R479">
-        <v>1015.18162</v>
+        <v>1015.18247</v>
       </c>
       <c r="S479">
-        <v>8.553699929785141</v>
+        <v>8.553394792494586</v>
       </c>
       <c r="T479">
         <v>1757.73005</v>
@@ -54439,7 +54439,7 @@
         <v>3</v>
       </c>
       <c r="AI479">
-        <v>3045.54486</v>
+        <v>3045.54741</v>
       </c>
     </row>
     <row r="480">
@@ -54462,13 +54462,13 @@
         </is>
       </c>
       <c r="E480">
-        <v>118.6833333333333</v>
+        <v>118.6876666666667</v>
       </c>
       <c r="F480">
-        <v>12579.97</v>
+        <v>12579.8</v>
       </c>
       <c r="G480">
-        <v>105.996096053925</v>
+        <v>105.9907937640249</v>
       </c>
       <c r="H480">
         <v>655.37</v>
@@ -54480,7 +54480,7 @@
         <v>0</v>
       </c>
       <c r="K480">
-        <v>5.522005336329167</v>
+        <v>5.521803725745163</v>
       </c>
       <c r="L480">
         <v>0</v>
@@ -54501,10 +54501,10 @@
         <v>32.004</v>
       </c>
       <c r="R480">
-        <v>1159.66443</v>
+        <v>1159.64936</v>
       </c>
       <c r="S480">
-        <v>9.771080719000139</v>
+        <v>9.770597001092503</v>
       </c>
       <c r="T480">
         <v>1902.56003</v>
@@ -54543,7 +54543,7 @@
         <v>0</v>
       </c>
       <c r="AF480">
-        <v>1030.3678</v>
+        <v>1030.3363</v>
       </c>
       <c r="AG480">
         <v>0</v>
@@ -54552,7 +54552,7 @@
         <v>3</v>
       </c>
       <c r="AI480">
-        <v>3478.993289999999</v>
+        <v>3478.94808</v>
       </c>
     </row>
     <row r="481">
@@ -54578,10 +54578,10 @@
         <v>104.4088333333333</v>
       </c>
       <c r="F481">
-        <v>9010.610000000001</v>
+        <v>9010.379999999999</v>
       </c>
       <c r="G481">
-        <v>86.30122291696264</v>
+        <v>86.29902003821513</v>
       </c>
       <c r="H481">
         <v>15.35</v>
@@ -54614,10 +54614,10 @@
         <v>36</v>
       </c>
       <c r="R481">
-        <v>960.22336</v>
+        <v>960.20241</v>
       </c>
       <c r="S481">
-        <v>9.19676361993637</v>
+        <v>9.196562966415675</v>
       </c>
       <c r="T481">
         <v>1266.61</v>
@@ -54656,7 +54656,7 @@
         <v>0</v>
       </c>
       <c r="AF481">
-        <v>2174.482</v>
+        <v>2174.454</v>
       </c>
       <c r="AG481">
         <v>0</v>
@@ -54665,7 +54665,7 @@
         <v>3</v>
       </c>
       <c r="AI481">
-        <v>2880.67008</v>
+        <v>2880.60723</v>
       </c>
     </row>
     <row r="482">
@@ -57717,6 +57717,2944 @@
       </c>
       <c r="AI508">
         <v>1518.87963</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B509" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E509">
+        <v>80.8095</v>
+      </c>
+      <c r="F509">
+        <v>5624.79</v>
+      </c>
+      <c r="G509">
+        <v>69.60555380246134</v>
+      </c>
+      <c r="H509">
+        <v>312.7</v>
+      </c>
+      <c r="I509">
+        <v>0</v>
+      </c>
+      <c r="J509">
+        <v>0</v>
+      </c>
+      <c r="K509">
+        <v>3.869594540245887</v>
+      </c>
+      <c r="L509">
+        <v>0</v>
+      </c>
+      <c r="M509">
+        <v>6</v>
+      </c>
+      <c r="N509">
+        <v>0</v>
+      </c>
+      <c r="O509">
+        <v>27.98504</v>
+      </c>
+      <c r="P509">
+        <v>77.73622222222222</v>
+      </c>
+      <c r="Q509">
+        <v>36</v>
+      </c>
+      <c r="R509">
+        <v>548.07789</v>
+      </c>
+      <c r="S509">
+        <v>6.782344773819911</v>
+      </c>
+      <c r="T509">
+        <v>1005.73</v>
+      </c>
+      <c r="U509">
+        <v>28</v>
+      </c>
+      <c r="V509">
+        <v>23</v>
+      </c>
+      <c r="W509">
+        <v>51</v>
+      </c>
+      <c r="X509">
+        <v>100</v>
+      </c>
+      <c r="Y509">
+        <v>28</v>
+      </c>
+      <c r="Z509">
+        <v>81</v>
+      </c>
+      <c r="AA509">
+        <v>23</v>
+      </c>
+      <c r="AB509">
+        <v>24</v>
+      </c>
+      <c r="AC509">
+        <v>4.60878</v>
+      </c>
+      <c r="AD509">
+        <v>-2.87264</v>
+      </c>
+      <c r="AE509">
+        <v>0</v>
+      </c>
+      <c r="AF509">
+        <v>1365.816</v>
+      </c>
+      <c r="AG509">
+        <v>0</v>
+      </c>
+      <c r="AH509">
+        <v>3</v>
+      </c>
+      <c r="AI509">
+        <v>1644.23367</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B510" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E510">
+        <v>80.8095</v>
+      </c>
+      <c r="F510">
+        <v>5972.27</v>
+      </c>
+      <c r="G510">
+        <v>73.90554328389607</v>
+      </c>
+      <c r="H510">
+        <v>182.39</v>
+      </c>
+      <c r="I510">
+        <v>0</v>
+      </c>
+      <c r="J510">
+        <v>0</v>
+      </c>
+      <c r="K510">
+        <v>2.257036610794523</v>
+      </c>
+      <c r="L510">
+        <v>0</v>
+      </c>
+      <c r="M510">
+        <v>1</v>
+      </c>
+      <c r="N510">
+        <v>0</v>
+      </c>
+      <c r="O510">
+        <v>25.34235</v>
+      </c>
+      <c r="P510">
+        <v>78.30413422321098</v>
+      </c>
+      <c r="Q510">
+        <v>32.364</v>
+      </c>
+      <c r="R510">
+        <v>559.8268399999999</v>
+      </c>
+      <c r="S510">
+        <v>6.927735476645691</v>
+      </c>
+      <c r="T510">
+        <v>962.3700200000001</v>
+      </c>
+      <c r="U510">
+        <v>15</v>
+      </c>
+      <c r="V510">
+        <v>9</v>
+      </c>
+      <c r="W510">
+        <v>24</v>
+      </c>
+      <c r="X510">
+        <v>72</v>
+      </c>
+      <c r="Y510">
+        <v>15</v>
+      </c>
+      <c r="Z510">
+        <v>47</v>
+      </c>
+      <c r="AA510">
+        <v>9</v>
+      </c>
+      <c r="AB510">
+        <v>4</v>
+      </c>
+      <c r="AC510">
+        <v>3.66981</v>
+      </c>
+      <c r="AD510">
+        <v>-2.77</v>
+      </c>
+      <c r="AE510">
+        <v>0</v>
+      </c>
+      <c r="AF510">
+        <v>478.7258</v>
+      </c>
+      <c r="AG510">
+        <v>0</v>
+      </c>
+      <c r="AH510">
+        <v>3</v>
+      </c>
+      <c r="AI510">
+        <v>1679.48052</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B511" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E511">
+        <v>135.7521666666667</v>
+      </c>
+      <c r="F511">
+        <v>7787.87</v>
+      </c>
+      <c r="G511">
+        <v>57.36829246433144</v>
+      </c>
+      <c r="H511">
+        <v>171.86</v>
+      </c>
+      <c r="I511">
+        <v>0</v>
+      </c>
+      <c r="J511">
+        <v>0</v>
+      </c>
+      <c r="K511">
+        <v>1.265983477243457</v>
+      </c>
+      <c r="L511">
+        <v>0</v>
+      </c>
+      <c r="M511">
+        <v>0</v>
+      </c>
+      <c r="N511">
+        <v>0</v>
+      </c>
+      <c r="O511">
+        <v>24.90096</v>
+      </c>
+      <c r="P511">
+        <v>69.16933333333334</v>
+      </c>
+      <c r="Q511">
+        <v>36</v>
+      </c>
+      <c r="R511">
+        <v>771.89678</v>
+      </c>
+      <c r="S511">
+        <v>5.686073371450179</v>
+      </c>
+      <c r="T511">
+        <v>1301.58</v>
+      </c>
+      <c r="U511">
+        <v>58</v>
+      </c>
+      <c r="V511">
+        <v>48</v>
+      </c>
+      <c r="W511">
+        <v>106</v>
+      </c>
+      <c r="X511">
+        <v>164</v>
+      </c>
+      <c r="Y511">
+        <v>58</v>
+      </c>
+      <c r="Z511">
+        <v>154</v>
+      </c>
+      <c r="AA511">
+        <v>48</v>
+      </c>
+      <c r="AB511">
+        <v>59</v>
+      </c>
+      <c r="AC511">
+        <v>4.56567</v>
+      </c>
+      <c r="AD511">
+        <v>-2.75104</v>
+      </c>
+      <c r="AE511">
+        <v>0</v>
+      </c>
+      <c r="AF511">
+        <v>1935.782</v>
+      </c>
+      <c r="AG511">
+        <v>0</v>
+      </c>
+      <c r="AH511">
+        <v>3</v>
+      </c>
+      <c r="AI511">
+        <v>2315.69034</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B512" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E512">
+        <v>80.8095</v>
+      </c>
+      <c r="F512">
+        <v>5944.639999999999</v>
+      </c>
+      <c r="G512">
+        <v>73.56362803878257</v>
+      </c>
+      <c r="H512">
+        <v>341.45</v>
+      </c>
+      <c r="I512">
+        <v>20.72</v>
+      </c>
+      <c r="J512">
+        <v>1</v>
+      </c>
+      <c r="K512">
+        <v>4.22536954194742</v>
+      </c>
+      <c r="L512">
+        <v>16.68</v>
+      </c>
+      <c r="M512">
+        <v>6</v>
+      </c>
+      <c r="N512">
+        <v>1</v>
+      </c>
+      <c r="O512">
+        <v>30.65669</v>
+      </c>
+      <c r="P512">
+        <v>94.61941358024693</v>
+      </c>
+      <c r="Q512">
+        <v>32.4</v>
+      </c>
+      <c r="R512">
+        <v>626.84111</v>
+      </c>
+      <c r="S512">
+        <v>7.757022503542281</v>
+      </c>
+      <c r="T512">
+        <v>1198.03002</v>
+      </c>
+      <c r="U512">
+        <v>22</v>
+      </c>
+      <c r="V512">
+        <v>17</v>
+      </c>
+      <c r="W512">
+        <v>39</v>
+      </c>
+      <c r="X512">
+        <v>107</v>
+      </c>
+      <c r="Y512">
+        <v>22</v>
+      </c>
+      <c r="Z512">
+        <v>51</v>
+      </c>
+      <c r="AA512">
+        <v>17</v>
+      </c>
+      <c r="AB512">
+        <v>5</v>
+      </c>
+      <c r="AC512">
+        <v>3.94083</v>
+      </c>
+      <c r="AD512">
+        <v>-2.6204</v>
+      </c>
+      <c r="AE512">
+        <v>0</v>
+      </c>
+      <c r="AF512">
+        <v>494.0355</v>
+      </c>
+      <c r="AG512">
+        <v>0</v>
+      </c>
+      <c r="AH512">
+        <v>3</v>
+      </c>
+      <c r="AI512">
+        <v>1880.52333</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Angel Coronel</t>
+        </is>
+      </c>
+      <c r="B513" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E513">
+        <v>80.8095</v>
+      </c>
+      <c r="F513">
+        <v>6578.85</v>
+      </c>
+      <c r="G513">
+        <v>81.41183895457837</v>
+      </c>
+      <c r="H513">
+        <v>387.74</v>
+      </c>
+      <c r="I513">
+        <v>0</v>
+      </c>
+      <c r="J513">
+        <v>0</v>
+      </c>
+      <c r="K513">
+        <v>4.798198231643556</v>
+      </c>
+      <c r="L513">
+        <v>0</v>
+      </c>
+      <c r="M513">
+        <v>4</v>
+      </c>
+      <c r="N513">
+        <v>0</v>
+      </c>
+      <c r="O513">
+        <v>27.62729</v>
+      </c>
+      <c r="P513">
+        <v>76.74247222222222</v>
+      </c>
+      <c r="Q513">
+        <v>36</v>
+      </c>
+      <c r="R513">
+        <v>659.55363</v>
+      </c>
+      <c r="S513">
+        <v>8.161832829060939</v>
+      </c>
+      <c r="T513">
+        <v>1057.72999</v>
+      </c>
+      <c r="U513">
+        <v>11</v>
+      </c>
+      <c r="V513">
+        <v>22</v>
+      </c>
+      <c r="W513">
+        <v>33</v>
+      </c>
+      <c r="X513">
+        <v>65</v>
+      </c>
+      <c r="Y513">
+        <v>11</v>
+      </c>
+      <c r="Z513">
+        <v>60</v>
+      </c>
+      <c r="AA513">
+        <v>22</v>
+      </c>
+      <c r="AB513">
+        <v>13</v>
+      </c>
+      <c r="AC513">
+        <v>3.53318</v>
+      </c>
+      <c r="AD513">
+        <v>-2.40006</v>
+      </c>
+      <c r="AE513">
+        <v>0</v>
+      </c>
+      <c r="AF513">
+        <v>1534.764</v>
+      </c>
+      <c r="AG513">
+        <v>0</v>
+      </c>
+      <c r="AH513">
+        <v>3</v>
+      </c>
+      <c r="AI513">
+        <v>1978.66089</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B514" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E514">
+        <v>122.5401666666667</v>
+      </c>
+      <c r="F514">
+        <v>8371.08</v>
+      </c>
+      <c r="G514">
+        <v>68.31294772734383</v>
+      </c>
+      <c r="H514">
+        <v>118.84</v>
+      </c>
+      <c r="I514">
+        <v>0</v>
+      </c>
+      <c r="J514">
+        <v>0</v>
+      </c>
+      <c r="K514">
+        <v>0.9698044586740947</v>
+      </c>
+      <c r="L514">
+        <v>0</v>
+      </c>
+      <c r="M514">
+        <v>1</v>
+      </c>
+      <c r="N514">
+        <v>0</v>
+      </c>
+      <c r="O514">
+        <v>25.37774</v>
+      </c>
+      <c r="P514">
+        <v>71.27777777777777</v>
+      </c>
+      <c r="Q514">
+        <v>35.604</v>
+      </c>
+      <c r="R514">
+        <v>801.68127</v>
+      </c>
+      <c r="S514">
+        <v>6.542191771133547</v>
+      </c>
+      <c r="T514">
+        <v>1246.04999</v>
+      </c>
+      <c r="U514">
+        <v>48</v>
+      </c>
+      <c r="V514">
+        <v>37</v>
+      </c>
+      <c r="W514">
+        <v>85</v>
+      </c>
+      <c r="X514">
+        <v>166</v>
+      </c>
+      <c r="Y514">
+        <v>48</v>
+      </c>
+      <c r="Z514">
+        <v>123</v>
+      </c>
+      <c r="AA514">
+        <v>37</v>
+      </c>
+      <c r="AB514">
+        <v>43</v>
+      </c>
+      <c r="AC514">
+        <v>4.56001</v>
+      </c>
+      <c r="AD514">
+        <v>-2.38391</v>
+      </c>
+      <c r="AE514">
+        <v>0</v>
+      </c>
+      <c r="AF514">
+        <v>712.8712399999999</v>
+      </c>
+      <c r="AG514">
+        <v>0</v>
+      </c>
+      <c r="AH514">
+        <v>3</v>
+      </c>
+      <c r="AI514">
+        <v>2405.04381</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B515" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E515">
+        <v>80.8095</v>
+      </c>
+      <c r="F515">
+        <v>5914.030000000001</v>
+      </c>
+      <c r="G515">
+        <v>73.18483594131879</v>
+      </c>
+      <c r="H515">
+        <v>262.44</v>
+      </c>
+      <c r="I515">
+        <v>0</v>
+      </c>
+      <c r="J515">
+        <v>0</v>
+      </c>
+      <c r="K515">
+        <v>3.247637963358268</v>
+      </c>
+      <c r="L515">
+        <v>0</v>
+      </c>
+      <c r="M515">
+        <v>6</v>
+      </c>
+      <c r="N515">
+        <v>0</v>
+      </c>
+      <c r="O515">
+        <v>29.49509</v>
+      </c>
+      <c r="P515">
+        <v>86.79110758003766</v>
+      </c>
+      <c r="Q515">
+        <v>33.984</v>
+      </c>
+      <c r="R515">
+        <v>705.13936</v>
+      </c>
+      <c r="S515">
+        <v>8.72594633056757</v>
+      </c>
+      <c r="T515">
+        <v>844.84999</v>
+      </c>
+      <c r="U515">
+        <v>19</v>
+      </c>
+      <c r="V515">
+        <v>21</v>
+      </c>
+      <c r="W515">
+        <v>40</v>
+      </c>
+      <c r="X515">
+        <v>72</v>
+      </c>
+      <c r="Y515">
+        <v>19</v>
+      </c>
+      <c r="Z515">
+        <v>64</v>
+      </c>
+      <c r="AA515">
+        <v>21</v>
+      </c>
+      <c r="AB515">
+        <v>9</v>
+      </c>
+      <c r="AC515">
+        <v>4.75597</v>
+      </c>
+      <c r="AD515">
+        <v>-2.41125</v>
+      </c>
+      <c r="AE515">
+        <v>0</v>
+      </c>
+      <c r="AF515">
+        <v>562.8416</v>
+      </c>
+      <c r="AG515">
+        <v>0</v>
+      </c>
+      <c r="AH515">
+        <v>3</v>
+      </c>
+      <c r="AI515">
+        <v>2115.41808</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B516" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E516">
+        <v>80.8095</v>
+      </c>
+      <c r="F516">
+        <v>6829.82</v>
+      </c>
+      <c r="G516">
+        <v>84.51753816073605</v>
+      </c>
+      <c r="H516">
+        <v>390.05</v>
+      </c>
+      <c r="I516">
+        <v>6.19</v>
+      </c>
+      <c r="J516">
+        <v>1</v>
+      </c>
+      <c r="K516">
+        <v>4.826783979606359</v>
+      </c>
+      <c r="L516">
+        <v>39.45</v>
+      </c>
+      <c r="M516">
+        <v>10</v>
+      </c>
+      <c r="N516">
+        <v>2</v>
+      </c>
+      <c r="O516">
+        <v>32.34409</v>
+      </c>
+      <c r="P516">
+        <v>90.93592555105714</v>
+      </c>
+      <c r="Q516">
+        <v>35.568</v>
+      </c>
+      <c r="R516">
+        <v>599.50933</v>
+      </c>
+      <c r="S516">
+        <v>7.418797666115989</v>
+      </c>
+      <c r="T516">
+        <v>1220.22</v>
+      </c>
+      <c r="U516">
+        <v>31</v>
+      </c>
+      <c r="V516">
+        <v>31</v>
+      </c>
+      <c r="W516">
+        <v>62</v>
+      </c>
+      <c r="X516">
+        <v>104</v>
+      </c>
+      <c r="Y516">
+        <v>31</v>
+      </c>
+      <c r="Z516">
+        <v>79</v>
+      </c>
+      <c r="AA516">
+        <v>31</v>
+      </c>
+      <c r="AB516">
+        <v>6</v>
+      </c>
+      <c r="AC516">
+        <v>4.6493</v>
+      </c>
+      <c r="AD516">
+        <v>-2.79759</v>
+      </c>
+      <c r="AE516">
+        <v>0</v>
+      </c>
+      <c r="AF516">
+        <v>665.3751999999999</v>
+      </c>
+      <c r="AG516">
+        <v>0</v>
+      </c>
+      <c r="AH516">
+        <v>3</v>
+      </c>
+      <c r="AI516">
+        <v>1798.52799</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B517" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E517">
+        <v>80.8095</v>
+      </c>
+      <c r="F517">
+        <v>6033.77</v>
+      </c>
+      <c r="G517">
+        <v>74.66659241797065</v>
+      </c>
+      <c r="H517">
+        <v>236.48</v>
+      </c>
+      <c r="I517">
+        <v>0</v>
+      </c>
+      <c r="J517">
+        <v>0</v>
+      </c>
+      <c r="K517">
+        <v>2.926388605300119</v>
+      </c>
+      <c r="L517">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="M517">
+        <v>4</v>
+      </c>
+      <c r="N517">
+        <v>1</v>
+      </c>
+      <c r="O517">
+        <v>31.09008</v>
+      </c>
+      <c r="P517">
+        <v>86.36133333333333</v>
+      </c>
+      <c r="Q517">
+        <v>36</v>
+      </c>
+      <c r="R517">
+        <v>591.54856</v>
+      </c>
+      <c r="S517">
+        <v>7.320284867497014</v>
+      </c>
+      <c r="T517">
+        <v>809.7500200000001</v>
+      </c>
+      <c r="U517">
+        <v>9</v>
+      </c>
+      <c r="V517">
+        <v>12</v>
+      </c>
+      <c r="W517">
+        <v>21</v>
+      </c>
+      <c r="X517">
+        <v>53</v>
+      </c>
+      <c r="Y517">
+        <v>9</v>
+      </c>
+      <c r="Z517">
+        <v>40</v>
+      </c>
+      <c r="AA517">
+        <v>12</v>
+      </c>
+      <c r="AB517">
+        <v>14</v>
+      </c>
+      <c r="AC517">
+        <v>4.04354</v>
+      </c>
+      <c r="AD517">
+        <v>-2.87983</v>
+      </c>
+      <c r="AE517">
+        <v>0</v>
+      </c>
+      <c r="AF517">
+        <v>1390.504</v>
+      </c>
+      <c r="AG517">
+        <v>0</v>
+      </c>
+      <c r="AH517">
+        <v>3</v>
+      </c>
+      <c r="AI517">
+        <v>1774.64568</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B518" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E518">
+        <v>88.64316666666667</v>
+      </c>
+      <c r="F518">
+        <v>6042.54</v>
+      </c>
+      <c r="G518">
+        <v>68.16701418985106</v>
+      </c>
+      <c r="H518">
+        <v>326.24</v>
+      </c>
+      <c r="I518">
+        <v>0</v>
+      </c>
+      <c r="J518">
+        <v>0</v>
+      </c>
+      <c r="K518">
+        <v>3.680373933692952</v>
+      </c>
+      <c r="L518">
+        <v>20.74</v>
+      </c>
+      <c r="M518">
+        <v>7</v>
+      </c>
+      <c r="N518">
+        <v>2</v>
+      </c>
+      <c r="O518">
+        <v>31.02748</v>
+      </c>
+      <c r="P518">
+        <v>86.18744444444445</v>
+      </c>
+      <c r="Q518">
+        <v>36</v>
+      </c>
+      <c r="R518">
+        <v>565.9136999999999</v>
+      </c>
+      <c r="S518">
+        <v>6.384177385359653</v>
+      </c>
+      <c r="T518">
+        <v>886.6</v>
+      </c>
+      <c r="U518">
+        <v>16</v>
+      </c>
+      <c r="V518">
+        <v>9</v>
+      </c>
+      <c r="W518">
+        <v>25</v>
+      </c>
+      <c r="X518">
+        <v>73</v>
+      </c>
+      <c r="Y518">
+        <v>16</v>
+      </c>
+      <c r="Z518">
+        <v>45</v>
+      </c>
+      <c r="AA518">
+        <v>9</v>
+      </c>
+      <c r="AB518">
+        <v>75</v>
+      </c>
+      <c r="AC518">
+        <v>4.07481</v>
+      </c>
+      <c r="AD518">
+        <v>-2.38567</v>
+      </c>
+      <c r="AE518">
+        <v>0</v>
+      </c>
+      <c r="AF518">
+        <v>485.5403</v>
+      </c>
+      <c r="AG518">
+        <v>0</v>
+      </c>
+      <c r="AH518">
+        <v>3</v>
+      </c>
+      <c r="AI518">
+        <v>1697.7411</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B519" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E519">
+        <v>80.8095</v>
+      </c>
+      <c r="F519">
+        <v>5387.91</v>
+      </c>
+      <c r="G519">
+        <v>66.67421528409407</v>
+      </c>
+      <c r="H519">
+        <v>240.42</v>
+      </c>
+      <c r="I519">
+        <v>0</v>
+      </c>
+      <c r="J519">
+        <v>0</v>
+      </c>
+      <c r="K519">
+        <v>2.975145249011565</v>
+      </c>
+      <c r="L519">
+        <v>0</v>
+      </c>
+      <c r="M519">
+        <v>5</v>
+      </c>
+      <c r="N519">
+        <v>0</v>
+      </c>
+      <c r="O519">
+        <v>27.00685</v>
+      </c>
+      <c r="P519">
+        <v>84.38585801774778</v>
+      </c>
+      <c r="Q519">
+        <v>32.004</v>
+      </c>
+      <c r="R519">
+        <v>568.05951</v>
+      </c>
+      <c r="S519">
+        <v>7.029612978672063</v>
+      </c>
+      <c r="T519">
+        <v>909.75999</v>
+      </c>
+      <c r="U519">
+        <v>15</v>
+      </c>
+      <c r="V519">
+        <v>19</v>
+      </c>
+      <c r="W519">
+        <v>34</v>
+      </c>
+      <c r="X519">
+        <v>73</v>
+      </c>
+      <c r="Y519">
+        <v>15</v>
+      </c>
+      <c r="Z519">
+        <v>66</v>
+      </c>
+      <c r="AA519">
+        <v>19</v>
+      </c>
+      <c r="AB519">
+        <v>13</v>
+      </c>
+      <c r="AC519">
+        <v>4.034</v>
+      </c>
+      <c r="AD519">
+        <v>-2.25451</v>
+      </c>
+      <c r="AE519">
+        <v>0</v>
+      </c>
+      <c r="AF519">
+        <v>382.2684</v>
+      </c>
+      <c r="AG519">
+        <v>0</v>
+      </c>
+      <c r="AH519">
+        <v>3</v>
+      </c>
+      <c r="AI519">
+        <v>1704.17853</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B520" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E520">
+        <v>80.8095</v>
+      </c>
+      <c r="F520">
+        <v>5343.4</v>
+      </c>
+      <c r="G520">
+        <v>66.12341370754676</v>
+      </c>
+      <c r="H520">
+        <v>154.45</v>
+      </c>
+      <c r="I520">
+        <v>0</v>
+      </c>
+      <c r="J520">
+        <v>0</v>
+      </c>
+      <c r="K520">
+        <v>1.911285183053973</v>
+      </c>
+      <c r="L520">
+        <v>0</v>
+      </c>
+      <c r="M520">
+        <v>1</v>
+      </c>
+      <c r="N520">
+        <v>0</v>
+      </c>
+      <c r="O520">
+        <v>28.30567</v>
+      </c>
+      <c r="P520">
+        <v>84.00305674264008</v>
+      </c>
+      <c r="Q520">
+        <v>33.696</v>
+      </c>
+      <c r="R520">
+        <v>506.43018</v>
+      </c>
+      <c r="S520">
+        <v>6.266963413955042</v>
+      </c>
+      <c r="T520">
+        <v>790.49</v>
+      </c>
+      <c r="U520">
+        <v>27</v>
+      </c>
+      <c r="V520">
+        <v>14</v>
+      </c>
+      <c r="W520">
+        <v>41</v>
+      </c>
+      <c r="X520">
+        <v>85</v>
+      </c>
+      <c r="Y520">
+        <v>27</v>
+      </c>
+      <c r="Z520">
+        <v>55</v>
+      </c>
+      <c r="AA520">
+        <v>14</v>
+      </c>
+      <c r="AB520">
+        <v>23</v>
+      </c>
+      <c r="AC520">
+        <v>4.3805</v>
+      </c>
+      <c r="AD520">
+        <v>-3.22218</v>
+      </c>
+      <c r="AE520">
+        <v>0</v>
+      </c>
+      <c r="AF520">
+        <v>500.0072</v>
+      </c>
+      <c r="AG520">
+        <v>0</v>
+      </c>
+      <c r="AH520">
+        <v>3</v>
+      </c>
+      <c r="AI520">
+        <v>1519.29054</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B521" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E521">
+        <v>142.3595</v>
+      </c>
+      <c r="F521">
+        <v>9077.709999999999</v>
+      </c>
+      <c r="G521">
+        <v>63.76609920658614</v>
+      </c>
+      <c r="H521">
+        <v>91.84999999999999</v>
+      </c>
+      <c r="I521">
+        <v>0</v>
+      </c>
+      <c r="J521">
+        <v>0</v>
+      </c>
+      <c r="K521">
+        <v>0.6451975456502727</v>
+      </c>
+      <c r="L521">
+        <v>0</v>
+      </c>
+      <c r="M521">
+        <v>1</v>
+      </c>
+      <c r="N521">
+        <v>0</v>
+      </c>
+      <c r="O521">
+        <v>27.46998</v>
+      </c>
+      <c r="P521">
+        <v>76.30550000000001</v>
+      </c>
+      <c r="Q521">
+        <v>36</v>
+      </c>
+      <c r="R521">
+        <v>1021.83311</v>
+      </c>
+      <c r="S521">
+        <v>7.177835760873002</v>
+      </c>
+      <c r="T521">
+        <v>636.65</v>
+      </c>
+      <c r="U521">
+        <v>31</v>
+      </c>
+      <c r="V521">
+        <v>32</v>
+      </c>
+      <c r="W521">
+        <v>63</v>
+      </c>
+      <c r="X521">
+        <v>92</v>
+      </c>
+      <c r="Y521">
+        <v>31</v>
+      </c>
+      <c r="Z521">
+        <v>91</v>
+      </c>
+      <c r="AA521">
+        <v>32</v>
+      </c>
+      <c r="AB521">
+        <v>25</v>
+      </c>
+      <c r="AC521">
+        <v>3.96446</v>
+      </c>
+      <c r="AD521">
+        <v>-2.64745</v>
+      </c>
+      <c r="AE521">
+        <v>0</v>
+      </c>
+      <c r="AF521">
+        <v>853.7380000000001</v>
+      </c>
+      <c r="AG521">
+        <v>0</v>
+      </c>
+      <c r="AH521">
+        <v>3</v>
+      </c>
+      <c r="AI521">
+        <v>3065.49933</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B522" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E522">
+        <v>80.8095</v>
+      </c>
+      <c r="F522">
+        <v>5573.88</v>
+      </c>
+      <c r="G522">
+        <v>68.9755536168396</v>
+      </c>
+      <c r="H522">
+        <v>228.46</v>
+      </c>
+      <c r="I522">
+        <v>0</v>
+      </c>
+      <c r="J522">
+        <v>0</v>
+      </c>
+      <c r="K522">
+        <v>2.827142848303727</v>
+      </c>
+      <c r="L522">
+        <v>0</v>
+      </c>
+      <c r="M522">
+        <v>3</v>
+      </c>
+      <c r="N522">
+        <v>0</v>
+      </c>
+      <c r="O522">
+        <v>28.54514</v>
+      </c>
+      <c r="P522">
+        <v>81.57618884316416</v>
+      </c>
+      <c r="Q522">
+        <v>34.992</v>
+      </c>
+      <c r="R522">
+        <v>511.23007</v>
+      </c>
+      <c r="S522">
+        <v>6.32636100953477</v>
+      </c>
+      <c r="T522">
+        <v>751.53999</v>
+      </c>
+      <c r="U522">
+        <v>20</v>
+      </c>
+      <c r="V522">
+        <v>16</v>
+      </c>
+      <c r="W522">
+        <v>36</v>
+      </c>
+      <c r="X522">
+        <v>65</v>
+      </c>
+      <c r="Y522">
+        <v>20</v>
+      </c>
+      <c r="Z522">
+        <v>47</v>
+      </c>
+      <c r="AA522">
+        <v>16</v>
+      </c>
+      <c r="AB522">
+        <v>7</v>
+      </c>
+      <c r="AC522">
+        <v>4.02959</v>
+      </c>
+      <c r="AD522">
+        <v>-2.3367</v>
+      </c>
+      <c r="AE522">
+        <v>0</v>
+      </c>
+      <c r="AF522">
+        <v>445.9539</v>
+      </c>
+      <c r="AG522">
+        <v>0</v>
+      </c>
+      <c r="AH522">
+        <v>3</v>
+      </c>
+      <c r="AI522">
+        <v>1533.69021</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B523" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E523">
+        <v>122.5401666666667</v>
+      </c>
+      <c r="F523">
+        <v>8833.18</v>
+      </c>
+      <c r="G523">
+        <v>72.08395614499192</v>
+      </c>
+      <c r="H523">
+        <v>71.50999999999999</v>
+      </c>
+      <c r="I523">
+        <v>0</v>
+      </c>
+      <c r="J523">
+        <v>0</v>
+      </c>
+      <c r="K523">
+        <v>0.58356375664578</v>
+      </c>
+      <c r="L523">
+        <v>0</v>
+      </c>
+      <c r="M523">
+        <v>0</v>
+      </c>
+      <c r="N523">
+        <v>0</v>
+      </c>
+      <c r="O523">
+        <v>23.12122</v>
+      </c>
+      <c r="P523">
+        <v>70.03883436326184</v>
+      </c>
+      <c r="Q523">
+        <v>33.012</v>
+      </c>
+      <c r="R523">
+        <v>987.2426499999999</v>
+      </c>
+      <c r="S523">
+        <v>8.056482024261433</v>
+      </c>
+      <c r="T523">
+        <v>1330.92002</v>
+      </c>
+      <c r="U523">
+        <v>34</v>
+      </c>
+      <c r="V523">
+        <v>40</v>
+      </c>
+      <c r="W523">
+        <v>74</v>
+      </c>
+      <c r="X523">
+        <v>165</v>
+      </c>
+      <c r="Y523">
+        <v>34</v>
+      </c>
+      <c r="Z523">
+        <v>143</v>
+      </c>
+      <c r="AA523">
+        <v>40</v>
+      </c>
+      <c r="AB523">
+        <v>39</v>
+      </c>
+      <c r="AC523">
+        <v>4.40797</v>
+      </c>
+      <c r="AD523">
+        <v>-2.56464</v>
+      </c>
+      <c r="AE523">
+        <v>0</v>
+      </c>
+      <c r="AF523">
+        <v>819.07644</v>
+      </c>
+      <c r="AG523">
+        <v>0</v>
+      </c>
+      <c r="AH523">
+        <v>3</v>
+      </c>
+      <c r="AI523">
+        <v>2961.72795</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B524" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E524">
+        <v>88.64316666666667</v>
+      </c>
+      <c r="F524">
+        <v>5886.24</v>
+      </c>
+      <c r="G524">
+        <v>66.40376490761649</v>
+      </c>
+      <c r="H524">
+        <v>204.89</v>
+      </c>
+      <c r="I524">
+        <v>0</v>
+      </c>
+      <c r="J524">
+        <v>0</v>
+      </c>
+      <c r="K524">
+        <v>2.31140208213079</v>
+      </c>
+      <c r="L524">
+        <v>0</v>
+      </c>
+      <c r="M524">
+        <v>4</v>
+      </c>
+      <c r="N524">
+        <v>0</v>
+      </c>
+      <c r="O524">
+        <v>29.39827</v>
+      </c>
+      <c r="P524">
+        <v>84.18748568155785</v>
+      </c>
+      <c r="Q524">
+        <v>34.92</v>
+      </c>
+      <c r="R524">
+        <v>498.07092</v>
+      </c>
+      <c r="S524">
+        <v>5.618830404298883</v>
+      </c>
+      <c r="T524">
+        <v>711.76</v>
+      </c>
+      <c r="U524">
+        <v>19</v>
+      </c>
+      <c r="V524">
+        <v>10</v>
+      </c>
+      <c r="W524">
+        <v>29</v>
+      </c>
+      <c r="X524">
+        <v>77</v>
+      </c>
+      <c r="Y524">
+        <v>19</v>
+      </c>
+      <c r="Z524">
+        <v>39</v>
+      </c>
+      <c r="AA524">
+        <v>10</v>
+      </c>
+      <c r="AB524">
+        <v>2</v>
+      </c>
+      <c r="AC524">
+        <v>4.36669</v>
+      </c>
+      <c r="AD524">
+        <v>-1.8905</v>
+      </c>
+      <c r="AE524">
+        <v>0</v>
+      </c>
+      <c r="AF524">
+        <v>548.1984</v>
+      </c>
+      <c r="AG524">
+        <v>0</v>
+      </c>
+      <c r="AH524">
+        <v>3</v>
+      </c>
+      <c r="AI524">
+        <v>1494.21276</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B525" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E525">
+        <v>80.8095</v>
+      </c>
+      <c r="F525">
+        <v>6493.490000000001</v>
+      </c>
+      <c r="G525">
+        <v>80.35552750604819</v>
+      </c>
+      <c r="H525">
+        <v>212.53</v>
+      </c>
+      <c r="I525">
+        <v>0</v>
+      </c>
+      <c r="J525">
+        <v>0</v>
+      </c>
+      <c r="K525">
+        <v>2.630012560404408</v>
+      </c>
+      <c r="L525">
+        <v>4.02</v>
+      </c>
+      <c r="M525">
+        <v>3</v>
+      </c>
+      <c r="N525">
+        <v>0</v>
+      </c>
+      <c r="O525">
+        <v>30.00988</v>
+      </c>
+      <c r="P525">
+        <v>85.76211705532694</v>
+      </c>
+      <c r="Q525">
+        <v>34.992</v>
+      </c>
+      <c r="R525">
+        <v>490.38143</v>
+      </c>
+      <c r="S525">
+        <v>6.068363620613913</v>
+      </c>
+      <c r="T525">
+        <v>874.47999</v>
+      </c>
+      <c r="U525">
+        <v>13</v>
+      </c>
+      <c r="V525">
+        <v>13</v>
+      </c>
+      <c r="W525">
+        <v>26</v>
+      </c>
+      <c r="X525">
+        <v>72</v>
+      </c>
+      <c r="Y525">
+        <v>13</v>
+      </c>
+      <c r="Z525">
+        <v>45</v>
+      </c>
+      <c r="AA525">
+        <v>13</v>
+      </c>
+      <c r="AB525">
+        <v>5</v>
+      </c>
+      <c r="AC525">
+        <v>3.95871</v>
+      </c>
+      <c r="AD525">
+        <v>-2.7955</v>
+      </c>
+      <c r="AE525">
+        <v>0</v>
+      </c>
+      <c r="AF525">
+        <v>534.73153</v>
+      </c>
+      <c r="AG525">
+        <v>0</v>
+      </c>
+      <c r="AH525">
+        <v>3</v>
+      </c>
+      <c r="AI525">
+        <v>1471.14429</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B526" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E526">
+        <v>88.64316666666667</v>
+      </c>
+      <c r="F526">
+        <v>4673.84</v>
+      </c>
+      <c r="G526">
+        <v>52.72645569596453</v>
+      </c>
+      <c r="H526">
+        <v>88.53</v>
+      </c>
+      <c r="I526">
+        <v>0</v>
+      </c>
+      <c r="J526">
+        <v>0</v>
+      </c>
+      <c r="K526">
+        <v>0.9987233458491818</v>
+      </c>
+      <c r="L526">
+        <v>0</v>
+      </c>
+      <c r="M526">
+        <v>1</v>
+      </c>
+      <c r="N526">
+        <v>0</v>
+      </c>
+      <c r="O526">
+        <v>25.49811</v>
+      </c>
+      <c r="P526">
+        <v>70.82808333333334</v>
+      </c>
+      <c r="Q526">
+        <v>36</v>
+      </c>
+      <c r="R526">
+        <v>513.44433</v>
+      </c>
+      <c r="S526">
+        <v>5.792260693153636</v>
+      </c>
+      <c r="T526">
+        <v>580.2</v>
+      </c>
+      <c r="U526">
+        <v>7</v>
+      </c>
+      <c r="V526">
+        <v>9</v>
+      </c>
+      <c r="W526">
+        <v>16</v>
+      </c>
+      <c r="X526">
+        <v>63</v>
+      </c>
+      <c r="Y526">
+        <v>7</v>
+      </c>
+      <c r="Z526">
+        <v>46</v>
+      </c>
+      <c r="AA526">
+        <v>9</v>
+      </c>
+      <c r="AB526">
+        <v>21</v>
+      </c>
+      <c r="AC526">
+        <v>4.18279</v>
+      </c>
+      <c r="AD526">
+        <v>-2.91075</v>
+      </c>
+      <c r="AE526">
+        <v>0</v>
+      </c>
+      <c r="AF526">
+        <v>1080.938</v>
+      </c>
+      <c r="AG526">
+        <v>0</v>
+      </c>
+      <c r="AH526">
+        <v>3</v>
+      </c>
+      <c r="AI526">
+        <v>1540.33299</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B527" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E527">
+        <v>88.64316666666667</v>
+      </c>
+      <c r="F527">
+        <v>5844.48</v>
+      </c>
+      <c r="G527">
+        <v>65.93266260418643</v>
+      </c>
+      <c r="H527">
+        <v>125.17</v>
+      </c>
+      <c r="I527">
+        <v>0</v>
+      </c>
+      <c r="J527">
+        <v>0</v>
+      </c>
+      <c r="K527">
+        <v>1.412065979893167</v>
+      </c>
+      <c r="L527">
+        <v>0</v>
+      </c>
+      <c r="M527">
+        <v>1</v>
+      </c>
+      <c r="N527">
+        <v>0</v>
+      </c>
+      <c r="O527">
+        <v>26.88245</v>
+      </c>
+      <c r="P527">
+        <v>79.10325447269302</v>
+      </c>
+      <c r="Q527">
+        <v>33.984</v>
+      </c>
+      <c r="R527">
+        <v>617.0817500000001</v>
+      </c>
+      <c r="S527">
+        <v>6.961413645345853</v>
+      </c>
+      <c r="T527">
+        <v>871.21</v>
+      </c>
+      <c r="U527">
+        <v>10</v>
+      </c>
+      <c r="V527">
+        <v>25</v>
+      </c>
+      <c r="W527">
+        <v>35</v>
+      </c>
+      <c r="X527">
+        <v>78</v>
+      </c>
+      <c r="Y527">
+        <v>10</v>
+      </c>
+      <c r="Z527">
+        <v>85</v>
+      </c>
+      <c r="AA527">
+        <v>25</v>
+      </c>
+      <c r="AB527">
+        <v>33</v>
+      </c>
+      <c r="AC527">
+        <v>3.82668</v>
+      </c>
+      <c r="AD527">
+        <v>-2.49811</v>
+      </c>
+      <c r="AE527">
+        <v>0</v>
+      </c>
+      <c r="AF527">
+        <v>555.9552</v>
+      </c>
+      <c r="AG527">
+        <v>0</v>
+      </c>
+      <c r="AH527">
+        <v>3</v>
+      </c>
+      <c r="AI527">
+        <v>1851.24525</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B528" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E528">
+        <v>80.8095</v>
+      </c>
+      <c r="F528">
+        <v>5555.86</v>
+      </c>
+      <c r="G528">
+        <v>68.75256003316441</v>
+      </c>
+      <c r="H528">
+        <v>185.93</v>
+      </c>
+      <c r="I528">
+        <v>0</v>
+      </c>
+      <c r="J528">
+        <v>0</v>
+      </c>
+      <c r="K528">
+        <v>2.300843341438816</v>
+      </c>
+      <c r="L528">
+        <v>0</v>
+      </c>
+      <c r="M528">
+        <v>3</v>
+      </c>
+      <c r="N528">
+        <v>0</v>
+      </c>
+      <c r="O528">
+        <v>27.83329</v>
+      </c>
+      <c r="P528">
+        <v>79.54186671239142</v>
+      </c>
+      <c r="Q528">
+        <v>34.992</v>
+      </c>
+      <c r="R528">
+        <v>485.10843</v>
+      </c>
+      <c r="S528">
+        <v>6.003111391606185</v>
+      </c>
+      <c r="T528">
+        <v>904.92002</v>
+      </c>
+      <c r="U528">
+        <v>16</v>
+      </c>
+      <c r="V528">
+        <v>21</v>
+      </c>
+      <c r="W528">
+        <v>37</v>
+      </c>
+      <c r="X528">
+        <v>78</v>
+      </c>
+      <c r="Y528">
+        <v>16</v>
+      </c>
+      <c r="Z528">
+        <v>76</v>
+      </c>
+      <c r="AA528">
+        <v>21</v>
+      </c>
+      <c r="AB528">
+        <v>25</v>
+      </c>
+      <c r="AC528">
+        <v>3.94496</v>
+      </c>
+      <c r="AD528">
+        <v>-2.50113</v>
+      </c>
+      <c r="AE528">
+        <v>0</v>
+      </c>
+      <c r="AF528">
+        <v>528.332</v>
+      </c>
+      <c r="AG528">
+        <v>0</v>
+      </c>
+      <c r="AH528">
+        <v>3</v>
+      </c>
+      <c r="AI528">
+        <v>1455.32529</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B529" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E529">
+        <v>88.64316666666667</v>
+      </c>
+      <c r="F529">
+        <v>5940.65</v>
+      </c>
+      <c r="G529">
+        <v>67.01757420669763</v>
+      </c>
+      <c r="H529">
+        <v>183.03</v>
+      </c>
+      <c r="I529">
+        <v>0</v>
+      </c>
+      <c r="J529">
+        <v>0</v>
+      </c>
+      <c r="K529">
+        <v>2.064795368697343</v>
+      </c>
+      <c r="L529">
+        <v>0</v>
+      </c>
+      <c r="M529">
+        <v>2</v>
+      </c>
+      <c r="N529">
+        <v>0</v>
+      </c>
+      <c r="O529">
+        <v>27.26166</v>
+      </c>
+      <c r="P529">
+        <v>82.58106143220647</v>
+      </c>
+      <c r="Q529">
+        <v>33.012</v>
+      </c>
+      <c r="R529">
+        <v>579.90972</v>
+      </c>
+      <c r="S529">
+        <v>6.542069082219159</v>
+      </c>
+      <c r="T529">
+        <v>1020.29</v>
+      </c>
+      <c r="U529">
+        <v>20</v>
+      </c>
+      <c r="V529">
+        <v>28</v>
+      </c>
+      <c r="W529">
+        <v>48</v>
+      </c>
+      <c r="X529">
+        <v>84</v>
+      </c>
+      <c r="Y529">
+        <v>20</v>
+      </c>
+      <c r="Z529">
+        <v>82</v>
+      </c>
+      <c r="AA529">
+        <v>28</v>
+      </c>
+      <c r="AB529">
+        <v>12</v>
+      </c>
+      <c r="AC529">
+        <v>5.15946</v>
+      </c>
+      <c r="AD529">
+        <v>-2.32423</v>
+      </c>
+      <c r="AE529">
+        <v>0</v>
+      </c>
+      <c r="AF529">
+        <v>534.92025</v>
+      </c>
+      <c r="AG529">
+        <v>0</v>
+      </c>
+      <c r="AH529">
+        <v>3</v>
+      </c>
+      <c r="AI529">
+        <v>1739.72916</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B530" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E530">
+        <v>80.8095</v>
+      </c>
+      <c r="F530">
+        <v>5322.94</v>
+      </c>
+      <c r="G530">
+        <v>65.87022565416194</v>
+      </c>
+      <c r="H530">
+        <v>52.32</v>
+      </c>
+      <c r="I530">
+        <v>0</v>
+      </c>
+      <c r="J530">
+        <v>0</v>
+      </c>
+      <c r="K530">
+        <v>0.6474486291834499</v>
+      </c>
+      <c r="L530">
+        <v>0</v>
+      </c>
+      <c r="M530">
+        <v>0</v>
+      </c>
+      <c r="N530">
+        <v>0</v>
+      </c>
+      <c r="O530">
+        <v>24.33107</v>
+      </c>
+      <c r="P530">
+        <v>76.0250906136733</v>
+      </c>
+      <c r="Q530">
+        <v>32.004</v>
+      </c>
+      <c r="R530">
+        <v>465.52312</v>
+      </c>
+      <c r="S530">
+        <v>5.76074743687314</v>
+      </c>
+      <c r="T530">
+        <v>612.84998</v>
+      </c>
+      <c r="U530">
+        <v>7</v>
+      </c>
+      <c r="V530">
+        <v>11</v>
+      </c>
+      <c r="W530">
+        <v>18</v>
+      </c>
+      <c r="X530">
+        <v>59</v>
+      </c>
+      <c r="Y530">
+        <v>7</v>
+      </c>
+      <c r="Z530">
+        <v>43</v>
+      </c>
+      <c r="AA530">
+        <v>11</v>
+      </c>
+      <c r="AB530">
+        <v>6</v>
+      </c>
+      <c r="AC530">
+        <v>3.85006</v>
+      </c>
+      <c r="AD530">
+        <v>-2.3784</v>
+      </c>
+      <c r="AE530">
+        <v>0</v>
+      </c>
+      <c r="AF530">
+        <v>427.007</v>
+      </c>
+      <c r="AG530">
+        <v>0</v>
+      </c>
+      <c r="AH530">
+        <v>3</v>
+      </c>
+      <c r="AI530">
+        <v>1396.56936</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B531" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E531">
+        <v>142.3595</v>
+      </c>
+      <c r="F531">
+        <v>10291.52</v>
+      </c>
+      <c r="G531">
+        <v>72.29247082210883</v>
+      </c>
+      <c r="H531">
+        <v>183.17</v>
+      </c>
+      <c r="I531">
+        <v>0</v>
+      </c>
+      <c r="J531">
+        <v>0</v>
+      </c>
+      <c r="K531">
+        <v>1.286672122338165</v>
+      </c>
+      <c r="L531">
+        <v>0</v>
+      </c>
+      <c r="M531">
+        <v>1</v>
+      </c>
+      <c r="N531">
+        <v>0</v>
+      </c>
+      <c r="O531">
+        <v>25.71285</v>
+      </c>
+      <c r="P531">
+        <v>71.42458333333333</v>
+      </c>
+      <c r="Q531">
+        <v>36</v>
+      </c>
+      <c r="R531">
+        <v>1065.90564</v>
+      </c>
+      <c r="S531">
+        <v>7.487421914238249</v>
+      </c>
+      <c r="T531">
+        <v>920.41</v>
+      </c>
+      <c r="U531">
+        <v>14</v>
+      </c>
+      <c r="V531">
+        <v>17</v>
+      </c>
+      <c r="W531">
+        <v>31</v>
+      </c>
+      <c r="X531">
+        <v>64</v>
+      </c>
+      <c r="Y531">
+        <v>14</v>
+      </c>
+      <c r="Z531">
+        <v>70</v>
+      </c>
+      <c r="AA531">
+        <v>17</v>
+      </c>
+      <c r="AB531">
+        <v>9</v>
+      </c>
+      <c r="AC531">
+        <v>4.48373</v>
+      </c>
+      <c r="AD531">
+        <v>-2.73142</v>
+      </c>
+      <c r="AE531">
+        <v>0</v>
+      </c>
+      <c r="AF531">
+        <v>1589.466</v>
+      </c>
+      <c r="AG531">
+        <v>0</v>
+      </c>
+      <c r="AH531">
+        <v>3</v>
+      </c>
+      <c r="AI531">
+        <v>3197.71692</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B532" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E532">
+        <v>80.8095</v>
+      </c>
+      <c r="F532">
+        <v>4259.56</v>
+      </c>
+      <c r="G532">
+        <v>52.71112926079236</v>
+      </c>
+      <c r="H532">
+        <v>116.29</v>
+      </c>
+      <c r="I532">
+        <v>0</v>
+      </c>
+      <c r="J532">
+        <v>0</v>
+      </c>
+      <c r="K532">
+        <v>1.439063476447695</v>
+      </c>
+      <c r="L532">
+        <v>0</v>
+      </c>
+      <c r="M532">
+        <v>1</v>
+      </c>
+      <c r="N532">
+        <v>0</v>
+      </c>
+      <c r="O532">
+        <v>25.28393</v>
+      </c>
+      <c r="P532">
+        <v>70.23313888888889</v>
+      </c>
+      <c r="Q532">
+        <v>36</v>
+      </c>
+      <c r="R532">
+        <v>489.74579</v>
+      </c>
+      <c r="S532">
+        <v>6.060497713758902</v>
+      </c>
+      <c r="T532">
+        <v>630.54999</v>
+      </c>
+      <c r="U532">
+        <v>15</v>
+      </c>
+      <c r="V532">
+        <v>9</v>
+      </c>
+      <c r="W532">
+        <v>24</v>
+      </c>
+      <c r="X532">
+        <v>70</v>
+      </c>
+      <c r="Y532">
+        <v>15</v>
+      </c>
+      <c r="Z532">
+        <v>40</v>
+      </c>
+      <c r="AA532">
+        <v>9</v>
+      </c>
+      <c r="AB532">
+        <v>9</v>
+      </c>
+      <c r="AC532">
+        <v>3.96219</v>
+      </c>
+      <c r="AD532">
+        <v>-2.60799</v>
+      </c>
+      <c r="AE532">
+        <v>0</v>
+      </c>
+      <c r="AF532">
+        <v>993.0839999999999</v>
+      </c>
+      <c r="AG532">
+        <v>0</v>
+      </c>
+      <c r="AH532">
+        <v>3</v>
+      </c>
+      <c r="AI532">
+        <v>1469.23737</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B533" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Sesión vespertina seleccionados | Sesión 34</t>
+        </is>
+      </c>
+      <c r="E533">
+        <v>122.5401666666667</v>
+      </c>
+      <c r="F533">
+        <v>8865.539999999999</v>
+      </c>
+      <c r="G533">
+        <v>72.34803282189105</v>
+      </c>
+      <c r="H533">
+        <v>332.96</v>
+      </c>
+      <c r="I533">
+        <v>0</v>
+      </c>
+      <c r="J533">
+        <v>0</v>
+      </c>
+      <c r="K533">
+        <v>2.71714988690783</v>
+      </c>
+      <c r="L533">
+        <v>0</v>
+      </c>
+      <c r="M533">
+        <v>4</v>
+      </c>
+      <c r="N533">
+        <v>0</v>
+      </c>
+      <c r="O533">
+        <v>28.16203</v>
+      </c>
+      <c r="P533">
+        <v>80.48133859167811</v>
+      </c>
+      <c r="Q533">
+        <v>34.992</v>
+      </c>
+      <c r="R533">
+        <v>955.8779</v>
+      </c>
+      <c r="S533">
+        <v>7.800527174083055</v>
+      </c>
+      <c r="T533">
+        <v>1773.2</v>
+      </c>
+      <c r="U533">
+        <v>61</v>
+      </c>
+      <c r="V533">
+        <v>53</v>
+      </c>
+      <c r="W533">
+        <v>114</v>
+      </c>
+      <c r="X533">
+        <v>206</v>
+      </c>
+      <c r="Y533">
+        <v>61</v>
+      </c>
+      <c r="Z533">
+        <v>183</v>
+      </c>
+      <c r="AA533">
+        <v>53</v>
+      </c>
+      <c r="AB533">
+        <v>62</v>
+      </c>
+      <c r="AC533">
+        <v>4.05959</v>
+      </c>
+      <c r="AD533">
+        <v>-2.81246</v>
+      </c>
+      <c r="AE533">
+        <v>0</v>
+      </c>
+      <c r="AF533">
+        <v>883.9808</v>
+      </c>
+      <c r="AG533">
+        <v>0</v>
+      </c>
+      <c r="AH533">
+        <v>3</v>
+      </c>
+      <c r="AI533">
+        <v>2867.6337</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B534" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Sesión 34</t>
+        </is>
+      </c>
+      <c r="E534">
+        <v>50.71066666666668</v>
+      </c>
+      <c r="F534">
+        <v>3941.83</v>
+      </c>
+      <c r="G534">
+        <v>77.73177240817184</v>
+      </c>
+      <c r="H534">
+        <v>0</v>
+      </c>
+      <c r="I534">
+        <v>0</v>
+      </c>
+      <c r="J534">
+        <v>0</v>
+      </c>
+      <c r="K534">
+        <v>0</v>
+      </c>
+      <c r="L534">
+        <v>0</v>
+      </c>
+      <c r="M534">
+        <v>0</v>
+      </c>
+      <c r="N534">
+        <v>0</v>
+      </c>
+      <c r="O534">
+        <v>20.70421</v>
+      </c>
+      <c r="P534">
+        <v>60.92340513182673</v>
+      </c>
+      <c r="Q534">
+        <v>33.984</v>
+      </c>
+      <c r="R534">
+        <v>411.45132</v>
+      </c>
+      <c r="S534">
+        <v>8.113703625798648</v>
+      </c>
+      <c r="T534">
+        <v>247.46</v>
+      </c>
+      <c r="U534">
+        <v>0</v>
+      </c>
+      <c r="V534">
+        <v>0</v>
+      </c>
+      <c r="W534">
+        <v>0</v>
+      </c>
+      <c r="X534">
+        <v>24</v>
+      </c>
+      <c r="Y534">
+        <v>0</v>
+      </c>
+      <c r="Z534">
+        <v>18</v>
+      </c>
+      <c r="AA534">
+        <v>0</v>
+      </c>
+      <c r="AB534">
+        <v>2</v>
+      </c>
+      <c r="AC534">
+        <v>2.936</v>
+      </c>
+      <c r="AD534">
+        <v>-2.36762</v>
+      </c>
+      <c r="AE534">
+        <v>0</v>
+      </c>
+      <c r="AF534">
+        <v>299.2542</v>
+      </c>
+      <c r="AG534">
+        <v>0</v>
+      </c>
+      <c r="AH534">
+        <v>3</v>
+      </c>
+      <c r="AI534">
+        <v>1234.35396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-16
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI534"/>
+  <dimension ref="A1:AI560"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -57742,10 +57742,10 @@
         <v>80.8095</v>
       </c>
       <c r="F509">
-        <v>5624.79</v>
+        <v>5624.97</v>
       </c>
       <c r="G509">
-        <v>69.60555380246134</v>
+        <v>69.60778126334156</v>
       </c>
       <c r="H509">
         <v>312.7</v>
@@ -57778,10 +57778,10 @@
         <v>36</v>
       </c>
       <c r="R509">
-        <v>548.07789</v>
+        <v>548.0933200000001</v>
       </c>
       <c r="S509">
-        <v>6.782344773819911</v>
+        <v>6.782535716716476</v>
       </c>
       <c r="T509">
         <v>1005.73</v>
@@ -57820,7 +57820,7 @@
         <v>0</v>
       </c>
       <c r="AF509">
-        <v>1365.816</v>
+        <v>1365.852</v>
       </c>
       <c r="AG509">
         <v>0</v>
@@ -57829,7 +57829,7 @@
         <v>3</v>
       </c>
       <c r="AI509">
-        <v>1644.23367</v>
+        <v>1644.27996</v>
       </c>
     </row>
     <row r="510">
@@ -57855,10 +57855,10 @@
         <v>80.8095</v>
       </c>
       <c r="F510">
-        <v>5972.27</v>
+        <v>5972.32</v>
       </c>
       <c r="G510">
-        <v>73.90554328389607</v>
+        <v>73.90616202302947</v>
       </c>
       <c r="H510">
         <v>182.39</v>
@@ -57891,10 +57891,10 @@
         <v>32.364</v>
       </c>
       <c r="R510">
-        <v>559.8268399999999</v>
+        <v>559.8287799999999</v>
       </c>
       <c r="S510">
-        <v>6.927735476645691</v>
+        <v>6.927759483724066</v>
       </c>
       <c r="T510">
         <v>962.3700200000001</v>
@@ -57933,7 +57933,7 @@
         <v>0</v>
       </c>
       <c r="AF510">
-        <v>478.7258</v>
+        <v>478.7272</v>
       </c>
       <c r="AG510">
         <v>0</v>
@@ -57942,7 +57942,7 @@
         <v>3</v>
       </c>
       <c r="AI510">
-        <v>1679.48052</v>
+        <v>1679.48634</v>
       </c>
     </row>
     <row r="511">
@@ -57968,10 +57968,10 @@
         <v>135.7521666666667</v>
       </c>
       <c r="F511">
-        <v>7787.87</v>
+        <v>7787.91</v>
       </c>
       <c r="G511">
-        <v>57.36829246433144</v>
+        <v>57.36858711892873</v>
       </c>
       <c r="H511">
         <v>171.86</v>
@@ -58004,10 +58004,10 @@
         <v>36</v>
       </c>
       <c r="R511">
-        <v>771.89678</v>
+        <v>771.90246</v>
       </c>
       <c r="S511">
-        <v>5.686073371450179</v>
+        <v>5.686115212402994</v>
       </c>
       <c r="T511">
         <v>1301.58</v>
@@ -58046,7 +58046,7 @@
         <v>0</v>
       </c>
       <c r="AF511">
-        <v>1935.782</v>
+        <v>1935.796</v>
       </c>
       <c r="AG511">
         <v>0</v>
@@ -58055,7 +58055,7 @@
         <v>3</v>
       </c>
       <c r="AI511">
-        <v>2315.69034</v>
+        <v>2315.70738</v>
       </c>
     </row>
     <row r="512">
@@ -58117,10 +58117,10 @@
         <v>32.4</v>
       </c>
       <c r="R512">
-        <v>626.84111</v>
+        <v>626.8431399999999</v>
       </c>
       <c r="S512">
-        <v>7.757022503542281</v>
+        <v>7.757047624351097</v>
       </c>
       <c r="T512">
         <v>1198.03002</v>
@@ -58168,7 +58168,7 @@
         <v>3</v>
       </c>
       <c r="AI512">
-        <v>1880.52333</v>
+        <v>1880.52942</v>
       </c>
     </row>
     <row r="513">
@@ -58194,10 +58194,10 @@
         <v>80.8095</v>
       </c>
       <c r="F513">
-        <v>6578.85</v>
+        <v>6578.929999999999</v>
       </c>
       <c r="G513">
-        <v>81.41183895457837</v>
+        <v>81.41282893719178</v>
       </c>
       <c r="H513">
         <v>387.74</v>
@@ -58230,10 +58230,10 @@
         <v>36</v>
       </c>
       <c r="R513">
-        <v>659.55363</v>
+        <v>659.5621599999999</v>
       </c>
       <c r="S513">
-        <v>8.161832829060939</v>
+        <v>8.161938385957097</v>
       </c>
       <c r="T513">
         <v>1057.72999</v>
@@ -58272,7 +58272,7 @@
         <v>0</v>
       </c>
       <c r="AF513">
-        <v>1534.764</v>
+        <v>1534.774</v>
       </c>
       <c r="AG513">
         <v>0</v>
@@ -58281,7 +58281,7 @@
         <v>3</v>
       </c>
       <c r="AI513">
-        <v>1978.66089</v>
+        <v>1978.68648</v>
       </c>
     </row>
     <row r="514">
@@ -58307,10 +58307,10 @@
         <v>122.5401666666667</v>
       </c>
       <c r="F514">
-        <v>8371.08</v>
+        <v>8371.18</v>
       </c>
       <c r="G514">
-        <v>68.31294772734383</v>
+        <v>68.31376378629592</v>
       </c>
       <c r="H514">
         <v>118.84</v>
@@ -58343,10 +58343,10 @@
         <v>35.604</v>
       </c>
       <c r="R514">
-        <v>801.68127</v>
+        <v>801.69874</v>
       </c>
       <c r="S514">
-        <v>6.542191771133547</v>
+        <v>6.542334336632479</v>
       </c>
       <c r="T514">
         <v>1246.04999</v>
@@ -58385,7 +58385,7 @@
         <v>0</v>
       </c>
       <c r="AF514">
-        <v>712.8712399999999</v>
+        <v>712.87763</v>
       </c>
       <c r="AG514">
         <v>0</v>
@@ -58394,7 +58394,7 @@
         <v>3</v>
       </c>
       <c r="AI514">
-        <v>2405.04381</v>
+        <v>2405.09622</v>
       </c>
     </row>
     <row r="515">
@@ -58420,10 +58420,10 @@
         <v>80.8095</v>
       </c>
       <c r="F515">
-        <v>5914.030000000001</v>
+        <v>5914.259999999999</v>
       </c>
       <c r="G515">
-        <v>73.18483594131879</v>
+        <v>73.18768214133239</v>
       </c>
       <c r="H515">
         <v>262.44</v>
@@ -58456,10 +58456,10 @@
         <v>33.984</v>
       </c>
       <c r="R515">
-        <v>705.13936</v>
+        <v>705.16873</v>
       </c>
       <c r="S515">
-        <v>8.72594633056757</v>
+        <v>8.726309777934524</v>
       </c>
       <c r="T515">
         <v>844.84999</v>
@@ -58498,7 +58498,7 @@
         <v>0</v>
       </c>
       <c r="AF515">
-        <v>562.8416</v>
+        <v>562.8616</v>
       </c>
       <c r="AG515">
         <v>0</v>
@@ -58507,7 +58507,7 @@
         <v>3</v>
       </c>
       <c r="AI515">
-        <v>2115.41808</v>
+        <v>2115.50619</v>
       </c>
     </row>
     <row r="516">
@@ -58533,10 +58533,10 @@
         <v>80.8095</v>
       </c>
       <c r="F516">
-        <v>6829.82</v>
+        <v>6829.85</v>
       </c>
       <c r="G516">
-        <v>84.51753816073605</v>
+        <v>84.5179094042161</v>
       </c>
       <c r="H516">
         <v>390.05</v>
@@ -58569,10 +58569,10 @@
         <v>35.568</v>
       </c>
       <c r="R516">
-        <v>599.50933</v>
+        <v>599.51222</v>
       </c>
       <c r="S516">
-        <v>7.418797666115989</v>
+        <v>7.418833429237899</v>
       </c>
       <c r="T516">
         <v>1220.22</v>
@@ -58611,7 +58611,7 @@
         <v>0</v>
       </c>
       <c r="AF516">
-        <v>665.3751999999999</v>
+        <v>665.3783999999999</v>
       </c>
       <c r="AG516">
         <v>0</v>
@@ -58620,7 +58620,7 @@
         <v>3</v>
       </c>
       <c r="AI516">
-        <v>1798.52799</v>
+        <v>1798.53666</v>
       </c>
     </row>
     <row r="517">
@@ -58646,10 +58646,10 @@
         <v>80.8095</v>
       </c>
       <c r="F517">
-        <v>6033.77</v>
+        <v>6033.889999999999</v>
       </c>
       <c r="G517">
-        <v>74.66659241797065</v>
+        <v>74.6680773918908</v>
       </c>
       <c r="H517">
         <v>236.48</v>
@@ -58682,10 +58682,10 @@
         <v>36</v>
       </c>
       <c r="R517">
-        <v>591.54856</v>
+        <v>591.556</v>
       </c>
       <c r="S517">
-        <v>7.320284867497014</v>
+        <v>7.320376935880065</v>
       </c>
       <c r="T517">
         <v>809.7500200000001</v>
@@ -58724,7 +58724,7 @@
         <v>0</v>
       </c>
       <c r="AF517">
-        <v>1390.504</v>
+        <v>1390.538</v>
       </c>
       <c r="AG517">
         <v>0</v>
@@ -58733,7 +58733,7 @@
         <v>3</v>
       </c>
       <c r="AI517">
-        <v>1774.64568</v>
+        <v>1774.668</v>
       </c>
     </row>
     <row r="518">
@@ -58759,10 +58759,10 @@
         <v>88.64316666666667</v>
       </c>
       <c r="F518">
-        <v>6042.54</v>
+        <v>6042.91</v>
       </c>
       <c r="G518">
-        <v>68.16701418985106</v>
+        <v>68.17118822845904</v>
       </c>
       <c r="H518">
         <v>326.24</v>
@@ -58795,10 +58795,10 @@
         <v>36</v>
       </c>
       <c r="R518">
-        <v>565.9136999999999</v>
+        <v>565.9345900000001</v>
       </c>
       <c r="S518">
-        <v>6.384177385359653</v>
+        <v>6.384413049323223</v>
       </c>
       <c r="T518">
         <v>886.6</v>
@@ -58837,7 +58837,7 @@
         <v>0</v>
       </c>
       <c r="AF518">
-        <v>485.5403</v>
+        <v>485.5571</v>
       </c>
       <c r="AG518">
         <v>0</v>
@@ -58846,7 +58846,7 @@
         <v>3</v>
       </c>
       <c r="AI518">
-        <v>1697.7411</v>
+        <v>1697.80377</v>
       </c>
     </row>
     <row r="519">
@@ -58872,10 +58872,10 @@
         <v>80.8095</v>
       </c>
       <c r="F519">
-        <v>5387.91</v>
+        <v>5387.93</v>
       </c>
       <c r="G519">
-        <v>66.67421528409407</v>
+        <v>66.67446277974743</v>
       </c>
       <c r="H519">
         <v>240.42</v>
@@ -58908,10 +58908,10 @@
         <v>32.004</v>
       </c>
       <c r="R519">
-        <v>568.05951</v>
+        <v>568.06345</v>
       </c>
       <c r="S519">
-        <v>7.029612978672063</v>
+        <v>7.029661735315774</v>
       </c>
       <c r="T519">
         <v>909.75999</v>
@@ -58950,7 +58950,7 @@
         <v>0</v>
       </c>
       <c r="AF519">
-        <v>382.2684</v>
+        <v>382.2726</v>
       </c>
       <c r="AG519">
         <v>0</v>
@@ -58959,7 +58959,7 @@
         <v>3</v>
       </c>
       <c r="AI519">
-        <v>1704.17853</v>
+        <v>1704.19035</v>
       </c>
     </row>
     <row r="520">
@@ -58985,10 +58985,10 @@
         <v>80.8095</v>
       </c>
       <c r="F520">
-        <v>5343.4</v>
+        <v>5343.429999999999</v>
       </c>
       <c r="G520">
-        <v>66.12341370754676</v>
+        <v>66.12378495102679</v>
       </c>
       <c r="H520">
         <v>154.45</v>
@@ -59021,10 +59021,10 @@
         <v>33.696</v>
       </c>
       <c r="R520">
-        <v>506.43018</v>
+        <v>506.45701</v>
       </c>
       <c r="S520">
-        <v>6.266963413955042</v>
+        <v>6.267295429374022</v>
       </c>
       <c r="T520">
         <v>790.49</v>
@@ -59063,7 +59063,7 @@
         <v>0</v>
       </c>
       <c r="AF520">
-        <v>500.0072</v>
+        <v>500.0088</v>
       </c>
       <c r="AG520">
         <v>0</v>
@@ -59072,7 +59072,7 @@
         <v>3</v>
       </c>
       <c r="AI520">
-        <v>1519.29054</v>
+        <v>1519.37103</v>
       </c>
     </row>
     <row r="521">
@@ -59211,10 +59211,10 @@
         <v>80.8095</v>
       </c>
       <c r="F522">
-        <v>5573.88</v>
+        <v>5574.030000000001</v>
       </c>
       <c r="G522">
-        <v>68.9755536168396</v>
+        <v>68.97740983423979</v>
       </c>
       <c r="H522">
         <v>228.46</v>
@@ -59247,10 +59247,10 @@
         <v>34.992</v>
       </c>
       <c r="R522">
-        <v>511.23007</v>
+        <v>511.23394</v>
       </c>
       <c r="S522">
-        <v>6.32636100953477</v>
+        <v>6.326408899943694</v>
       </c>
       <c r="T522">
         <v>751.53999</v>
@@ -59289,7 +59289,7 @@
         <v>0</v>
       </c>
       <c r="AF522">
-        <v>445.9539</v>
+        <v>445.96011</v>
       </c>
       <c r="AG522">
         <v>0</v>
@@ -59298,7 +59298,7 @@
         <v>3</v>
       </c>
       <c r="AI522">
-        <v>1533.69021</v>
+        <v>1533.70182</v>
       </c>
     </row>
     <row r="523">
@@ -59324,10 +59324,10 @@
         <v>122.5401666666667</v>
       </c>
       <c r="F523">
-        <v>8833.18</v>
+        <v>8833.85</v>
       </c>
       <c r="G523">
-        <v>72.08395614499192</v>
+        <v>72.08942373997098</v>
       </c>
       <c r="H523">
         <v>71.50999999999999</v>
@@ -59360,10 +59360,10 @@
         <v>33.012</v>
       </c>
       <c r="R523">
-        <v>987.2426499999999</v>
+        <v>987.3040099999999</v>
       </c>
       <c r="S523">
-        <v>8.056482024261433</v>
+        <v>8.05698275803444</v>
       </c>
       <c r="T523">
         <v>1330.92002</v>
@@ -59402,7 +59402,7 @@
         <v>0</v>
       </c>
       <c r="AF523">
-        <v>819.07644</v>
+        <v>819.09984</v>
       </c>
       <c r="AG523">
         <v>0</v>
@@ -59411,7 +59411,7 @@
         <v>3</v>
       </c>
       <c r="AI523">
-        <v>2961.72795</v>
+        <v>2961.91203</v>
       </c>
     </row>
     <row r="524">
@@ -59437,10 +59437,10 @@
         <v>88.64316666666667</v>
       </c>
       <c r="F524">
-        <v>5886.24</v>
+        <v>5886.309999999999</v>
       </c>
       <c r="G524">
-        <v>66.40376490761649</v>
+        <v>66.40455459059638</v>
       </c>
       <c r="H524">
         <v>204.89</v>
@@ -59473,10 +59473,10 @@
         <v>34.92</v>
       </c>
       <c r="R524">
-        <v>498.07092</v>
+        <v>498.07418</v>
       </c>
       <c r="S524">
-        <v>5.618830404298883</v>
+        <v>5.618867180963376</v>
       </c>
       <c r="T524">
         <v>711.76</v>
@@ -59515,7 +59515,7 @@
         <v>0</v>
       </c>
       <c r="AF524">
-        <v>548.1984</v>
+        <v>548.2024</v>
       </c>
       <c r="AG524">
         <v>0</v>
@@ -59524,7 +59524,7 @@
         <v>3</v>
       </c>
       <c r="AI524">
-        <v>1494.21276</v>
+        <v>1494.22254</v>
       </c>
     </row>
     <row r="525">
@@ -59550,10 +59550,10 @@
         <v>80.8095</v>
       </c>
       <c r="F525">
-        <v>6493.490000000001</v>
+        <v>6493.910000000001</v>
       </c>
       <c r="G525">
-        <v>80.35552750604819</v>
+        <v>80.3607249147687</v>
       </c>
       <c r="H525">
         <v>212.53</v>
@@ -59586,10 +59586,10 @@
         <v>34.992</v>
       </c>
       <c r="R525">
-        <v>490.38143</v>
+        <v>490.39939</v>
       </c>
       <c r="S525">
-        <v>6.068363620613913</v>
+        <v>6.068585871710628</v>
       </c>
       <c r="T525">
         <v>874.47999</v>
@@ -59628,7 +59628,7 @@
         <v>0</v>
       </c>
       <c r="AF525">
-        <v>534.73153</v>
+        <v>534.7386300000001</v>
       </c>
       <c r="AG525">
         <v>0</v>
@@ -59637,7 +59637,7 @@
         <v>3</v>
       </c>
       <c r="AI525">
-        <v>1471.14429</v>
+        <v>1471.19817</v>
       </c>
     </row>
     <row r="526">
@@ -59663,10 +59663,10 @@
         <v>88.64316666666667</v>
       </c>
       <c r="F526">
-        <v>4673.84</v>
+        <v>4673.91</v>
       </c>
       <c r="G526">
-        <v>52.72645569596453</v>
+        <v>52.72724537894442</v>
       </c>
       <c r="H526">
         <v>88.53</v>
@@ -59699,10 +59699,10 @@
         <v>36</v>
       </c>
       <c r="R526">
-        <v>513.44433</v>
+        <v>513.4507</v>
       </c>
       <c r="S526">
-        <v>5.792260693153636</v>
+        <v>5.792332554304806</v>
       </c>
       <c r="T526">
         <v>580.2</v>
@@ -59741,7 +59741,7 @@
         <v>0</v>
       </c>
       <c r="AF526">
-        <v>1080.938</v>
+        <v>1080.962</v>
       </c>
       <c r="AG526">
         <v>0</v>
@@ -59750,7 +59750,7 @@
         <v>3</v>
       </c>
       <c r="AI526">
-        <v>1540.33299</v>
+        <v>1540.3521</v>
       </c>
     </row>
     <row r="527">
@@ -59776,10 +59776,10 @@
         <v>88.64316666666667</v>
       </c>
       <c r="F527">
-        <v>5844.48</v>
+        <v>5844.56</v>
       </c>
       <c r="G527">
-        <v>65.93266260418643</v>
+        <v>65.93356509902061</v>
       </c>
       <c r="H527">
         <v>125.17</v>
@@ -59812,10 +59812,10 @@
         <v>33.984</v>
       </c>
       <c r="R527">
-        <v>617.0817500000001</v>
+        <v>617.10063</v>
       </c>
       <c r="S527">
-        <v>6.961413645345853</v>
+        <v>6.961626634126714</v>
       </c>
       <c r="T527">
         <v>871.21</v>
@@ -59854,7 +59854,7 @@
         <v>0</v>
       </c>
       <c r="AF527">
-        <v>555.9552</v>
+        <v>555.9599999999999</v>
       </c>
       <c r="AG527">
         <v>0</v>
@@ -59863,7 +59863,7 @@
         <v>3</v>
       </c>
       <c r="AI527">
-        <v>1851.24525</v>
+        <v>1851.30189</v>
       </c>
     </row>
     <row r="528">
@@ -59889,10 +59889,10 @@
         <v>80.8095</v>
       </c>
       <c r="F528">
-        <v>5555.86</v>
+        <v>5555.97</v>
       </c>
       <c r="G528">
-        <v>68.75256003316441</v>
+        <v>68.75392125925789</v>
       </c>
       <c r="H528">
         <v>185.93</v>
@@ -59925,10 +59925,10 @@
         <v>34.992</v>
       </c>
       <c r="R528">
-        <v>485.10843</v>
+        <v>485.11932</v>
       </c>
       <c r="S528">
-        <v>6.003111391606185</v>
+        <v>6.003246152989439</v>
       </c>
       <c r="T528">
         <v>904.92002</v>
@@ -59967,7 +59967,7 @@
         <v>0</v>
       </c>
       <c r="AF528">
-        <v>528.332</v>
+        <v>528.3384</v>
       </c>
       <c r="AG528">
         <v>0</v>
@@ -59976,7 +59976,7 @@
         <v>3</v>
       </c>
       <c r="AI528">
-        <v>1455.32529</v>
+        <v>1455.35796</v>
       </c>
     </row>
     <row r="529">
@@ -60002,10 +60002,10 @@
         <v>88.64316666666667</v>
       </c>
       <c r="F529">
-        <v>5940.65</v>
+        <v>5940.94</v>
       </c>
       <c r="G529">
-        <v>67.01757420669763</v>
+        <v>67.02084575047145</v>
       </c>
       <c r="H529">
         <v>183.03</v>
@@ -60038,10 +60038,10 @@
         <v>33.012</v>
       </c>
       <c r="R529">
-        <v>579.90972</v>
+        <v>579.9248</v>
       </c>
       <c r="S529">
-        <v>6.542069082219159</v>
+        <v>6.542239202495398</v>
       </c>
       <c r="T529">
         <v>1020.29</v>
@@ -60080,7 +60080,7 @@
         <v>0</v>
       </c>
       <c r="AF529">
-        <v>534.92025</v>
+        <v>534.93975</v>
       </c>
       <c r="AG529">
         <v>0</v>
@@ -60089,7 +60089,7 @@
         <v>3</v>
       </c>
       <c r="AI529">
-        <v>1739.72916</v>
+        <v>1739.7744</v>
       </c>
     </row>
     <row r="530">
@@ -60115,10 +60115,10 @@
         <v>80.8095</v>
       </c>
       <c r="F530">
-        <v>5322.94</v>
+        <v>5323.17</v>
       </c>
       <c r="G530">
-        <v>65.87022565416194</v>
+        <v>65.87307185417556</v>
       </c>
       <c r="H530">
         <v>52.32</v>
@@ -60151,10 +60151,10 @@
         <v>32.004</v>
       </c>
       <c r="R530">
-        <v>465.52312</v>
+        <v>465.53024</v>
       </c>
       <c r="S530">
-        <v>5.76074743687314</v>
+        <v>5.760835545325735</v>
       </c>
       <c r="T530">
         <v>612.84998</v>
@@ -60193,7 +60193,7 @@
         <v>0</v>
       </c>
       <c r="AF530">
-        <v>427.007</v>
+        <v>427.0161000000001</v>
       </c>
       <c r="AG530">
         <v>0</v>
@@ -60202,7 +60202,7 @@
         <v>3</v>
       </c>
       <c r="AI530">
-        <v>1396.56936</v>
+        <v>1396.59072</v>
       </c>
     </row>
     <row r="531">
@@ -60228,10 +60228,10 @@
         <v>142.3595</v>
       </c>
       <c r="F531">
-        <v>10291.52</v>
+        <v>10291.57</v>
       </c>
       <c r="G531">
-        <v>72.29247082210883</v>
+        <v>72.29282204559583</v>
       </c>
       <c r="H531">
         <v>183.17</v>
@@ -60264,10 +60264,10 @@
         <v>36</v>
       </c>
       <c r="R531">
-        <v>1065.90564</v>
+        <v>1065.91091</v>
       </c>
       <c r="S531">
-        <v>7.487421914238249</v>
+        <v>7.487458933193781</v>
       </c>
       <c r="T531">
         <v>920.41</v>
@@ -60306,7 +60306,7 @@
         <v>0</v>
       </c>
       <c r="AF531">
-        <v>1589.466</v>
+        <v>1589.474</v>
       </c>
       <c r="AG531">
         <v>0</v>
@@ -60315,7 +60315,7 @@
         <v>3</v>
       </c>
       <c r="AI531">
-        <v>3197.71692</v>
+        <v>3197.73273</v>
       </c>
     </row>
     <row r="532">
@@ -60377,10 +60377,10 @@
         <v>36</v>
       </c>
       <c r="R532">
-        <v>489.74579</v>
+        <v>489.74692</v>
       </c>
       <c r="S532">
-        <v>6.060497713758902</v>
+        <v>6.060511697263316</v>
       </c>
       <c r="T532">
         <v>630.54999</v>
@@ -60428,7 +60428,7 @@
         <v>3</v>
       </c>
       <c r="AI532">
-        <v>1469.23737</v>
+        <v>1469.24076</v>
       </c>
     </row>
     <row r="533">
@@ -60454,10 +60454,10 @@
         <v>122.5401666666667</v>
       </c>
       <c r="F533">
-        <v>8865.539999999999</v>
+        <v>8865.639999999999</v>
       </c>
       <c r="G533">
-        <v>72.34803282189105</v>
+        <v>72.34884888084315</v>
       </c>
       <c r="H533">
         <v>332.96</v>
@@ -60490,10 +60490,10 @@
         <v>34.992</v>
       </c>
       <c r="R533">
-        <v>955.8779</v>
+        <v>955.88334</v>
       </c>
       <c r="S533">
-        <v>7.800527174083055</v>
+        <v>7.80057156769005</v>
       </c>
       <c r="T533">
         <v>1773.2</v>
@@ -60532,7 +60532,7 @@
         <v>0</v>
       </c>
       <c r="AF533">
-        <v>883.9808</v>
+        <v>883.9888</v>
       </c>
       <c r="AG533">
         <v>0</v>
@@ -60541,7 +60541,7 @@
         <v>3</v>
       </c>
       <c r="AI533">
-        <v>2867.6337</v>
+        <v>2867.65002</v>
       </c>
     </row>
     <row r="534">
@@ -60567,10 +60567,10 @@
         <v>50.71066666666668</v>
       </c>
       <c r="F534">
-        <v>3941.83</v>
+        <v>3941.88</v>
       </c>
       <c r="G534">
-        <v>77.73177240817184</v>
+        <v>77.73275839402622</v>
       </c>
       <c r="H534">
         <v>0</v>
@@ -60603,10 +60603,10 @@
         <v>33.984</v>
       </c>
       <c r="R534">
-        <v>411.45132</v>
+        <v>411.46846</v>
       </c>
       <c r="S534">
-        <v>8.113703625798648</v>
+        <v>8.114041621749532</v>
       </c>
       <c r="T534">
         <v>247.46</v>
@@ -60645,7 +60645,7 @@
         <v>0</v>
       </c>
       <c r="AF534">
-        <v>299.2542</v>
+        <v>299.257</v>
       </c>
       <c r="AG534">
         <v>0</v>
@@ -60654,7 +60654,2945 @@
         <v>3</v>
       </c>
       <c r="AI534">
-        <v>1234.35396</v>
+        <v>1234.40538</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B535" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E535">
+        <v>43.44283333333333</v>
+      </c>
+      <c r="F535">
+        <v>3766.68</v>
+      </c>
+      <c r="G535">
+        <v>86.70428954526447</v>
+      </c>
+      <c r="H535">
+        <v>114.29</v>
+      </c>
+      <c r="I535">
+        <v>0</v>
+      </c>
+      <c r="J535">
+        <v>0</v>
+      </c>
+      <c r="K535">
+        <v>2.630813674675916</v>
+      </c>
+      <c r="L535">
+        <v>0</v>
+      </c>
+      <c r="M535">
+        <v>2</v>
+      </c>
+      <c r="N535">
+        <v>0</v>
+      </c>
+      <c r="O535">
+        <v>25.66809</v>
+      </c>
+      <c r="P535">
+        <v>71.30025000000001</v>
+      </c>
+      <c r="Q535">
+        <v>36</v>
+      </c>
+      <c r="R535">
+        <v>332.39163</v>
+      </c>
+      <c r="S535">
+        <v>7.651241977004263</v>
+      </c>
+      <c r="T535">
+        <v>544.6099899999999</v>
+      </c>
+      <c r="U535">
+        <v>7</v>
+      </c>
+      <c r="V535">
+        <v>15</v>
+      </c>
+      <c r="W535">
+        <v>22</v>
+      </c>
+      <c r="X535">
+        <v>46</v>
+      </c>
+      <c r="Y535">
+        <v>7</v>
+      </c>
+      <c r="Z535">
+        <v>40</v>
+      </c>
+      <c r="AA535">
+        <v>15</v>
+      </c>
+      <c r="AB535">
+        <v>9</v>
+      </c>
+      <c r="AC535">
+        <v>4.23109</v>
+      </c>
+      <c r="AD535">
+        <v>-4.84002</v>
+      </c>
+      <c r="AE535">
+        <v>0</v>
+      </c>
+      <c r="AF535">
+        <v>889.1840000000001</v>
+      </c>
+      <c r="AG535">
+        <v>0</v>
+      </c>
+      <c r="AH535">
+        <v>3</v>
+      </c>
+      <c r="AI535">
+        <v>997.1748899999999</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B536" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E536">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F536">
+        <v>7144.89</v>
+      </c>
+      <c r="G536">
+        <v>103.6635609839847</v>
+      </c>
+      <c r="H536">
+        <v>171.42</v>
+      </c>
+      <c r="I536">
+        <v>0</v>
+      </c>
+      <c r="J536">
+        <v>0</v>
+      </c>
+      <c r="K536">
+        <v>2.487093240606176</v>
+      </c>
+      <c r="L536">
+        <v>0</v>
+      </c>
+      <c r="M536">
+        <v>1</v>
+      </c>
+      <c r="N536">
+        <v>0</v>
+      </c>
+      <c r="O536">
+        <v>26.85911</v>
+      </c>
+      <c r="P536">
+        <v>82.99069954270178</v>
+      </c>
+      <c r="Q536">
+        <v>32.364</v>
+      </c>
+      <c r="R536">
+        <v>708.70748</v>
+      </c>
+      <c r="S536">
+        <v>10.2824733582723</v>
+      </c>
+      <c r="T536">
+        <v>900.32002</v>
+      </c>
+      <c r="U536">
+        <v>9</v>
+      </c>
+      <c r="V536">
+        <v>9</v>
+      </c>
+      <c r="W536">
+        <v>18</v>
+      </c>
+      <c r="X536">
+        <v>58</v>
+      </c>
+      <c r="Y536">
+        <v>9</v>
+      </c>
+      <c r="Z536">
+        <v>45</v>
+      </c>
+      <c r="AA536">
+        <v>9</v>
+      </c>
+      <c r="AB536">
+        <v>11</v>
+      </c>
+      <c r="AC536">
+        <v>4.09956</v>
+      </c>
+      <c r="AD536">
+        <v>-3.1408</v>
+      </c>
+      <c r="AE536">
+        <v>0</v>
+      </c>
+      <c r="AF536">
+        <v>565.8330999999999</v>
+      </c>
+      <c r="AG536">
+        <v>0</v>
+      </c>
+      <c r="AH536">
+        <v>3</v>
+      </c>
+      <c r="AI536">
+        <v>2126.12244</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B537" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E537">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F537">
+        <v>7536.22</v>
+      </c>
+      <c r="G537">
+        <v>101.0953464766564</v>
+      </c>
+      <c r="H537">
+        <v>249.68</v>
+      </c>
+      <c r="I537">
+        <v>0</v>
+      </c>
+      <c r="J537">
+        <v>0</v>
+      </c>
+      <c r="K537">
+        <v>3.349356322969813</v>
+      </c>
+      <c r="L537">
+        <v>0</v>
+      </c>
+      <c r="M537">
+        <v>3</v>
+      </c>
+      <c r="N537">
+        <v>0</v>
+      </c>
+      <c r="O537">
+        <v>29.50706</v>
+      </c>
+      <c r="P537">
+        <v>81.96405555555555</v>
+      </c>
+      <c r="Q537">
+        <v>36</v>
+      </c>
+      <c r="R537">
+        <v>611.89944</v>
+      </c>
+      <c r="S537">
+        <v>8.208383764761646</v>
+      </c>
+      <c r="T537">
+        <v>1193.35997</v>
+      </c>
+      <c r="U537">
+        <v>27</v>
+      </c>
+      <c r="V537">
+        <v>28</v>
+      </c>
+      <c r="W537">
+        <v>55</v>
+      </c>
+      <c r="X537">
+        <v>96</v>
+      </c>
+      <c r="Y537">
+        <v>27</v>
+      </c>
+      <c r="Z537">
+        <v>101</v>
+      </c>
+      <c r="AA537">
+        <v>28</v>
+      </c>
+      <c r="AB537">
+        <v>45</v>
+      </c>
+      <c r="AC537">
+        <v>4.34686</v>
+      </c>
+      <c r="AD537">
+        <v>-3.73913</v>
+      </c>
+      <c r="AE537">
+        <v>0</v>
+      </c>
+      <c r="AF537">
+        <v>1766.492</v>
+      </c>
+      <c r="AG537">
+        <v>0</v>
+      </c>
+      <c r="AH537">
+        <v>3</v>
+      </c>
+      <c r="AI537">
+        <v>1835.69832</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B538" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E538">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F538">
+        <v>6716.45</v>
+      </c>
+      <c r="G538">
+        <v>97.44742384709691</v>
+      </c>
+      <c r="H538">
+        <v>0</v>
+      </c>
+      <c r="I538">
+        <v>0</v>
+      </c>
+      <c r="J538">
+        <v>0</v>
+      </c>
+      <c r="K538">
+        <v>0</v>
+      </c>
+      <c r="L538">
+        <v>0</v>
+      </c>
+      <c r="M538">
+        <v>0</v>
+      </c>
+      <c r="N538">
+        <v>0</v>
+      </c>
+      <c r="O538">
+        <v>29.41863</v>
+      </c>
+      <c r="P538">
+        <v>81.71841666666667</v>
+      </c>
+      <c r="Q538">
+        <v>36</v>
+      </c>
+      <c r="R538">
+        <v>636.71669</v>
+      </c>
+      <c r="S538">
+        <v>9.23797559141371</v>
+      </c>
+      <c r="T538">
+        <v>0</v>
+      </c>
+      <c r="U538">
+        <v>0</v>
+      </c>
+      <c r="V538">
+        <v>0</v>
+      </c>
+      <c r="W538">
+        <v>0</v>
+      </c>
+      <c r="X538">
+        <v>0</v>
+      </c>
+      <c r="Y538">
+        <v>0</v>
+      </c>
+      <c r="Z538">
+        <v>0</v>
+      </c>
+      <c r="AA538">
+        <v>0</v>
+      </c>
+      <c r="AB538">
+        <v>0</v>
+      </c>
+      <c r="AC538">
+        <v>4.69053</v>
+      </c>
+      <c r="AD538">
+        <v>-3.59661</v>
+      </c>
+      <c r="AE538">
+        <v>0</v>
+      </c>
+      <c r="AF538">
+        <v>0</v>
+      </c>
+      <c r="AG538">
+        <v>0</v>
+      </c>
+      <c r="AH538">
+        <v>3</v>
+      </c>
+      <c r="AI538">
+        <v>1910.15007</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Angel Coronel</t>
+        </is>
+      </c>
+      <c r="B539" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E539">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F539">
+        <v>8142.46</v>
+      </c>
+      <c r="G539">
+        <v>109.2278111403748</v>
+      </c>
+      <c r="H539">
+        <v>358.14</v>
+      </c>
+      <c r="I539">
+        <v>0</v>
+      </c>
+      <c r="J539">
+        <v>0</v>
+      </c>
+      <c r="K539">
+        <v>4.804303402388692</v>
+      </c>
+      <c r="L539">
+        <v>0</v>
+      </c>
+      <c r="M539">
+        <v>7</v>
+      </c>
+      <c r="N539">
+        <v>0</v>
+      </c>
+      <c r="O539">
+        <v>29.54916</v>
+      </c>
+      <c r="P539">
+        <v>82.081</v>
+      </c>
+      <c r="Q539">
+        <v>36</v>
+      </c>
+      <c r="R539">
+        <v>877.53862</v>
+      </c>
+      <c r="S539">
+        <v>11.7718260395194</v>
+      </c>
+      <c r="T539">
+        <v>1385.48002</v>
+      </c>
+      <c r="U539">
+        <v>22</v>
+      </c>
+      <c r="V539">
+        <v>44</v>
+      </c>
+      <c r="W539">
+        <v>66</v>
+      </c>
+      <c r="X539">
+        <v>99</v>
+      </c>
+      <c r="Y539">
+        <v>22</v>
+      </c>
+      <c r="Z539">
+        <v>104</v>
+      </c>
+      <c r="AA539">
+        <v>44</v>
+      </c>
+      <c r="AB539">
+        <v>37</v>
+      </c>
+      <c r="AC539">
+        <v>4.45156</v>
+      </c>
+      <c r="AD539">
+        <v>-4.79103</v>
+      </c>
+      <c r="AE539">
+        <v>0</v>
+      </c>
+      <c r="AF539">
+        <v>1929.188</v>
+      </c>
+      <c r="AG539">
+        <v>0</v>
+      </c>
+      <c r="AH539">
+        <v>3</v>
+      </c>
+      <c r="AI539">
+        <v>2632.61586</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B540" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol | Trabajo Complementario Seleccionados</t>
+        </is>
+      </c>
+      <c r="E540">
+        <v>124.945</v>
+      </c>
+      <c r="F540">
+        <v>9130.73</v>
+      </c>
+      <c r="G540">
+        <v>73.0779943174997</v>
+      </c>
+      <c r="H540">
+        <v>448.55</v>
+      </c>
+      <c r="I540">
+        <v>12.49</v>
+      </c>
+      <c r="J540">
+        <v>1</v>
+      </c>
+      <c r="K540">
+        <v>3.589979591020049</v>
+      </c>
+      <c r="L540">
+        <v>50.55</v>
+      </c>
+      <c r="M540">
+        <v>9</v>
+      </c>
+      <c r="N540">
+        <v>3</v>
+      </c>
+      <c r="O540">
+        <v>32.97517</v>
+      </c>
+      <c r="P540">
+        <v>92.61647567689023</v>
+      </c>
+      <c r="Q540">
+        <v>35.604</v>
+      </c>
+      <c r="R540">
+        <v>796.78566</v>
+      </c>
+      <c r="S540">
+        <v>6.377091200128056</v>
+      </c>
+      <c r="T540">
+        <v>1495.4</v>
+      </c>
+      <c r="U540">
+        <v>83</v>
+      </c>
+      <c r="V540">
+        <v>69</v>
+      </c>
+      <c r="W540">
+        <v>152</v>
+      </c>
+      <c r="X540">
+        <v>186</v>
+      </c>
+      <c r="Y540">
+        <v>83</v>
+      </c>
+      <c r="Z540">
+        <v>164</v>
+      </c>
+      <c r="AA540">
+        <v>69</v>
+      </c>
+      <c r="AB540">
+        <v>41</v>
+      </c>
+      <c r="AC540">
+        <v>4.3304</v>
+      </c>
+      <c r="AD540">
+        <v>-1.45506</v>
+      </c>
+      <c r="AE540">
+        <v>0</v>
+      </c>
+      <c r="AF540">
+        <v>789.69963</v>
+      </c>
+      <c r="AG540">
+        <v>0</v>
+      </c>
+      <c r="AH540">
+        <v>3</v>
+      </c>
+      <c r="AI540">
+        <v>2390.35698</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B541" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E541">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F541">
+        <v>6053.4</v>
+      </c>
+      <c r="G541">
+        <v>87.82738433488173</v>
+      </c>
+      <c r="H541">
+        <v>308.44</v>
+      </c>
+      <c r="I541">
+        <v>22.36</v>
+      </c>
+      <c r="J541">
+        <v>1</v>
+      </c>
+      <c r="K541">
+        <v>4.475084815847445</v>
+      </c>
+      <c r="L541">
+        <v>24.76</v>
+      </c>
+      <c r="M541">
+        <v>10</v>
+      </c>
+      <c r="N541">
+        <v>1</v>
+      </c>
+      <c r="O541">
+        <v>32.02438</v>
+      </c>
+      <c r="P541">
+        <v>94.2336982109228</v>
+      </c>
+      <c r="Q541">
+        <v>33.984</v>
+      </c>
+      <c r="R541">
+        <v>670.05727</v>
+      </c>
+      <c r="S541">
+        <v>9.721706376362313</v>
+      </c>
+      <c r="T541">
+        <v>847.79002</v>
+      </c>
+      <c r="U541">
+        <v>13</v>
+      </c>
+      <c r="V541">
+        <v>22</v>
+      </c>
+      <c r="W541">
+        <v>35</v>
+      </c>
+      <c r="X541">
+        <v>59</v>
+      </c>
+      <c r="Y541">
+        <v>13</v>
+      </c>
+      <c r="Z541">
+        <v>61</v>
+      </c>
+      <c r="AA541">
+        <v>22</v>
+      </c>
+      <c r="AB541">
+        <v>8</v>
+      </c>
+      <c r="AC541">
+        <v>5.38509</v>
+      </c>
+      <c r="AD541">
+        <v>-3.03935</v>
+      </c>
+      <c r="AE541">
+        <v>0</v>
+      </c>
+      <c r="AF541">
+        <v>561.2528</v>
+      </c>
+      <c r="AG541">
+        <v>0</v>
+      </c>
+      <c r="AH541">
+        <v>3</v>
+      </c>
+      <c r="AI541">
+        <v>2010.17181</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B542" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E542">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F542">
+        <v>6713.45</v>
+      </c>
+      <c r="G542">
+        <v>97.4038975390709</v>
+      </c>
+      <c r="H542">
+        <v>334.22</v>
+      </c>
+      <c r="I542">
+        <v>8.040000000000001</v>
+      </c>
+      <c r="J542">
+        <v>1</v>
+      </c>
+      <c r="K542">
+        <v>4.849120889484286</v>
+      </c>
+      <c r="L542">
+        <v>20.99</v>
+      </c>
+      <c r="M542">
+        <v>8</v>
+      </c>
+      <c r="N542">
+        <v>1</v>
+      </c>
+      <c r="O542">
+        <v>32.34469</v>
+      </c>
+      <c r="P542">
+        <v>90.93761246063879</v>
+      </c>
+      <c r="Q542">
+        <v>35.568</v>
+      </c>
+      <c r="R542">
+        <v>591.8106300000001</v>
+      </c>
+      <c r="S542">
+        <v>8.586443924815558</v>
+      </c>
+      <c r="T542">
+        <v>974.05</v>
+      </c>
+      <c r="U542">
+        <v>23</v>
+      </c>
+      <c r="V542">
+        <v>20</v>
+      </c>
+      <c r="W542">
+        <v>43</v>
+      </c>
+      <c r="X542">
+        <v>84</v>
+      </c>
+      <c r="Y542">
+        <v>23</v>
+      </c>
+      <c r="Z542">
+        <v>63</v>
+      </c>
+      <c r="AA542">
+        <v>20</v>
+      </c>
+      <c r="AB542">
+        <v>6</v>
+      </c>
+      <c r="AC542">
+        <v>4.8735</v>
+      </c>
+      <c r="AD542">
+        <v>-3.77286</v>
+      </c>
+      <c r="AE542">
+        <v>0</v>
+      </c>
+      <c r="AF542">
+        <v>631.9536000000001</v>
+      </c>
+      <c r="AG542">
+        <v>0</v>
+      </c>
+      <c r="AH542">
+        <v>3</v>
+      </c>
+      <c r="AI542">
+        <v>1775.43189</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B543" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E543">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F543">
+        <v>7894.56</v>
+      </c>
+      <c r="G543">
+        <v>105.90233279824</v>
+      </c>
+      <c r="H543">
+        <v>432.36</v>
+      </c>
+      <c r="I543">
+        <v>3.54</v>
+      </c>
+      <c r="J543">
+        <v>0</v>
+      </c>
+      <c r="K543">
+        <v>5.799934715632923</v>
+      </c>
+      <c r="L543">
+        <v>19.6</v>
+      </c>
+      <c r="M543">
+        <v>9</v>
+      </c>
+      <c r="N543">
+        <v>1</v>
+      </c>
+      <c r="O543">
+        <v>32.53335</v>
+      </c>
+      <c r="P543">
+        <v>90.37041666666667</v>
+      </c>
+      <c r="Q543">
+        <v>36</v>
+      </c>
+      <c r="R543">
+        <v>759.4303</v>
+      </c>
+      <c r="S543">
+        <v>10.18745064546564</v>
+      </c>
+      <c r="T543">
+        <v>1261.26001</v>
+      </c>
+      <c r="U543">
+        <v>14</v>
+      </c>
+      <c r="V543">
+        <v>27</v>
+      </c>
+      <c r="W543">
+        <v>41</v>
+      </c>
+      <c r="X543">
+        <v>86</v>
+      </c>
+      <c r="Y543">
+        <v>14</v>
+      </c>
+      <c r="Z543">
+        <v>78</v>
+      </c>
+      <c r="AA543">
+        <v>27</v>
+      </c>
+      <c r="AB543">
+        <v>18</v>
+      </c>
+      <c r="AC543">
+        <v>6.87354</v>
+      </c>
+      <c r="AD543">
+        <v>-3.68831</v>
+      </c>
+      <c r="AE543">
+        <v>0</v>
+      </c>
+      <c r="AF543">
+        <v>1817.528</v>
+      </c>
+      <c r="AG543">
+        <v>0</v>
+      </c>
+      <c r="AH543">
+        <v>3</v>
+      </c>
+      <c r="AI543">
+        <v>2278.2909</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B544" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E544">
+        <v>31.10283333333333</v>
+      </c>
+      <c r="F544">
+        <v>3676.64</v>
+      </c>
+      <c r="G544">
+        <v>118.2091663674799</v>
+      </c>
+      <c r="H544">
+        <v>235.28</v>
+      </c>
+      <c r="I544">
+        <v>0</v>
+      </c>
+      <c r="J544">
+        <v>0</v>
+      </c>
+      <c r="K544">
+        <v>7.564584148282312</v>
+      </c>
+      <c r="L544">
+        <v>0</v>
+      </c>
+      <c r="M544">
+        <v>7</v>
+      </c>
+      <c r="N544">
+        <v>0</v>
+      </c>
+      <c r="O544">
+        <v>29.08462</v>
+      </c>
+      <c r="P544">
+        <v>80.7906111111111</v>
+      </c>
+      <c r="Q544">
+        <v>36</v>
+      </c>
+      <c r="R544">
+        <v>311.23013</v>
+      </c>
+      <c r="S544">
+        <v>10.0064880477127</v>
+      </c>
+      <c r="T544">
+        <v>608.38</v>
+      </c>
+      <c r="U544">
+        <v>12</v>
+      </c>
+      <c r="V544">
+        <v>15</v>
+      </c>
+      <c r="W544">
+        <v>27</v>
+      </c>
+      <c r="X544">
+        <v>41</v>
+      </c>
+      <c r="Y544">
+        <v>12</v>
+      </c>
+      <c r="Z544">
+        <v>38</v>
+      </c>
+      <c r="AA544">
+        <v>15</v>
+      </c>
+      <c r="AB544">
+        <v>12</v>
+      </c>
+      <c r="AC544">
+        <v>4.07838</v>
+      </c>
+      <c r="AD544">
+        <v>-6.35896</v>
+      </c>
+      <c r="AE544">
+        <v>0</v>
+      </c>
+      <c r="AF544">
+        <v>302.9635</v>
+      </c>
+      <c r="AG544">
+        <v>0</v>
+      </c>
+      <c r="AH544">
+        <v>3</v>
+      </c>
+      <c r="AI544">
+        <v>933.69039</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B545" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E545">
+        <v>80.51133333333334</v>
+      </c>
+      <c r="F545">
+        <v>6886.46</v>
+      </c>
+      <c r="G545">
+        <v>85.53404489637069</v>
+      </c>
+      <c r="H545">
+        <v>311.1</v>
+      </c>
+      <c r="I545">
+        <v>12.33</v>
+      </c>
+      <c r="J545">
+        <v>2</v>
+      </c>
+      <c r="K545">
+        <v>3.864052265933574</v>
+      </c>
+      <c r="L545">
+        <v>0</v>
+      </c>
+      <c r="M545">
+        <v>5</v>
+      </c>
+      <c r="N545">
+        <v>0</v>
+      </c>
+      <c r="O545">
+        <v>29.41066</v>
+      </c>
+      <c r="P545">
+        <v>91.89682539682539</v>
+      </c>
+      <c r="Q545">
+        <v>32.004</v>
+      </c>
+      <c r="R545">
+        <v>743.20861</v>
+      </c>
+      <c r="S545">
+        <v>9.23110547583363</v>
+      </c>
+      <c r="T545">
+        <v>1011.07002</v>
+      </c>
+      <c r="U545">
+        <v>28</v>
+      </c>
+      <c r="V545">
+        <v>28</v>
+      </c>
+      <c r="W545">
+        <v>56</v>
+      </c>
+      <c r="X545">
+        <v>74</v>
+      </c>
+      <c r="Y545">
+        <v>28</v>
+      </c>
+      <c r="Z545">
+        <v>79</v>
+      </c>
+      <c r="AA545">
+        <v>28</v>
+      </c>
+      <c r="AB545">
+        <v>9</v>
+      </c>
+      <c r="AC545">
+        <v>4.1412</v>
+      </c>
+      <c r="AD545">
+        <v>-3.57176</v>
+      </c>
+      <c r="AE545">
+        <v>0</v>
+      </c>
+      <c r="AF545">
+        <v>484.1130000000001</v>
+      </c>
+      <c r="AG545">
+        <v>0</v>
+      </c>
+      <c r="AH545">
+        <v>3</v>
+      </c>
+      <c r="AI545">
+        <v>2229.62583</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B546" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E546">
+        <v>68.645</v>
+      </c>
+      <c r="F546">
+        <v>6406.33</v>
+      </c>
+      <c r="G546">
+        <v>93.32551533250783</v>
+      </c>
+      <c r="H546">
+        <v>411.21</v>
+      </c>
+      <c r="I546">
+        <v>0</v>
+      </c>
+      <c r="J546">
+        <v>0</v>
+      </c>
+      <c r="K546">
+        <v>5.990385315754971</v>
+      </c>
+      <c r="L546">
+        <v>8.920000000000002</v>
+      </c>
+      <c r="M546">
+        <v>8</v>
+      </c>
+      <c r="N546">
+        <v>1</v>
+      </c>
+      <c r="O546">
+        <v>30.32931</v>
+      </c>
+      <c r="P546">
+        <v>89.62562056737588</v>
+      </c>
+      <c r="Q546">
+        <v>33.84</v>
+      </c>
+      <c r="R546">
+        <v>562.91481</v>
+      </c>
+      <c r="S546">
+        <v>8.200375992424794</v>
+      </c>
+      <c r="T546">
+        <v>1067.86999</v>
+      </c>
+      <c r="U546">
+        <v>34</v>
+      </c>
+      <c r="V546">
+        <v>27</v>
+      </c>
+      <c r="W546">
+        <v>61</v>
+      </c>
+      <c r="X546">
+        <v>87</v>
+      </c>
+      <c r="Y546">
+        <v>34</v>
+      </c>
+      <c r="Z546">
+        <v>80</v>
+      </c>
+      <c r="AA546">
+        <v>27</v>
+      </c>
+      <c r="AB546">
+        <v>15</v>
+      </c>
+      <c r="AC546">
+        <v>4.49615</v>
+      </c>
+      <c r="AD546">
+        <v>-2.01583</v>
+      </c>
+      <c r="AE546">
+        <v>0</v>
+      </c>
+      <c r="AF546">
+        <v>521.8927</v>
+      </c>
+      <c r="AG546">
+        <v>0</v>
+      </c>
+      <c r="AH546">
+        <v>3</v>
+      </c>
+      <c r="AI546">
+        <v>1688.74443</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Gio Valle</t>
+        </is>
+      </c>
+      <c r="B547" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E547">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F547">
+        <v>7265.03</v>
+      </c>
+      <c r="G547">
+        <v>97.45744219427019</v>
+      </c>
+      <c r="H547">
+        <v>210.41</v>
+      </c>
+      <c r="I547">
+        <v>0</v>
+      </c>
+      <c r="J547">
+        <v>0</v>
+      </c>
+      <c r="K547">
+        <v>2.822565139042287</v>
+      </c>
+      <c r="L547">
+        <v>0</v>
+      </c>
+      <c r="M547">
+        <v>3</v>
+      </c>
+      <c r="N547">
+        <v>0</v>
+      </c>
+      <c r="O547">
+        <v>25.7335</v>
+      </c>
+      <c r="P547">
+        <v>71.48194444444445</v>
+      </c>
+      <c r="Q547">
+        <v>36</v>
+      </c>
+      <c r="R547">
+        <v>661.05039</v>
+      </c>
+      <c r="S547">
+        <v>8.867723900785649</v>
+      </c>
+      <c r="T547">
+        <v>851.97</v>
+      </c>
+      <c r="U547">
+        <v>15</v>
+      </c>
+      <c r="V547">
+        <v>19</v>
+      </c>
+      <c r="W547">
+        <v>34</v>
+      </c>
+      <c r="X547">
+        <v>63</v>
+      </c>
+      <c r="Y547">
+        <v>15</v>
+      </c>
+      <c r="Z547">
+        <v>62</v>
+      </c>
+      <c r="AA547">
+        <v>19</v>
+      </c>
+      <c r="AB547">
+        <v>10</v>
+      </c>
+      <c r="AC547">
+        <v>4.08387</v>
+      </c>
+      <c r="AD547">
+        <v>-3.33119</v>
+      </c>
+      <c r="AE547">
+        <v>0</v>
+      </c>
+      <c r="AF547">
+        <v>1641.32</v>
+      </c>
+      <c r="AG547">
+        <v>0</v>
+      </c>
+      <c r="AH547">
+        <v>3</v>
+      </c>
+      <c r="AI547">
+        <v>1983.15117</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B548" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E548">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F548">
+        <v>5992.48</v>
+      </c>
+      <c r="G548">
+        <v>86.94351010656692</v>
+      </c>
+      <c r="H548">
+        <v>330.73</v>
+      </c>
+      <c r="I548">
+        <v>0</v>
+      </c>
+      <c r="J548">
+        <v>0</v>
+      </c>
+      <c r="K548">
+        <v>4.798485284480695</v>
+      </c>
+      <c r="L548">
+        <v>0</v>
+      </c>
+      <c r="M548">
+        <v>7</v>
+      </c>
+      <c r="N548">
+        <v>0</v>
+      </c>
+      <c r="O548">
+        <v>29.37443</v>
+      </c>
+      <c r="P548">
+        <v>87.17482787274454</v>
+      </c>
+      <c r="Q548">
+        <v>33.696</v>
+      </c>
+      <c r="R548">
+        <v>545.56281</v>
+      </c>
+      <c r="S548">
+        <v>7.915444971865078</v>
+      </c>
+      <c r="T548">
+        <v>1019.35002</v>
+      </c>
+      <c r="U548">
+        <v>24</v>
+      </c>
+      <c r="V548">
+        <v>22</v>
+      </c>
+      <c r="W548">
+        <v>46</v>
+      </c>
+      <c r="X548">
+        <v>87</v>
+      </c>
+      <c r="Y548">
+        <v>24</v>
+      </c>
+      <c r="Z548">
+        <v>77</v>
+      </c>
+      <c r="AA548">
+        <v>22</v>
+      </c>
+      <c r="AB548">
+        <v>15</v>
+      </c>
+      <c r="AC548">
+        <v>4.27466</v>
+      </c>
+      <c r="AD548">
+        <v>-4.1417</v>
+      </c>
+      <c r="AE548">
+        <v>0</v>
+      </c>
+      <c r="AF548">
+        <v>563.8112</v>
+      </c>
+      <c r="AG548">
+        <v>0</v>
+      </c>
+      <c r="AH548">
+        <v>3</v>
+      </c>
+      <c r="AI548">
+        <v>1636.68843</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B549" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E549">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F549">
+        <v>6498.12</v>
+      </c>
+      <c r="G549">
+        <v>94.27972423665737</v>
+      </c>
+      <c r="H549">
+        <v>301.83</v>
+      </c>
+      <c r="I549">
+        <v>0</v>
+      </c>
+      <c r="J549">
+        <v>0</v>
+      </c>
+      <c r="K549">
+        <v>4.379181850496805</v>
+      </c>
+      <c r="L549">
+        <v>4.029999999999999</v>
+      </c>
+      <c r="M549">
+        <v>4</v>
+      </c>
+      <c r="N549">
+        <v>0</v>
+      </c>
+      <c r="O549">
+        <v>30.06708</v>
+      </c>
+      <c r="P549">
+        <v>85.92558299039781</v>
+      </c>
+      <c r="Q549">
+        <v>34.992</v>
+      </c>
+      <c r="R549">
+        <v>524.68007</v>
+      </c>
+      <c r="S549">
+        <v>7.612462113976056</v>
+      </c>
+      <c r="T549">
+        <v>837.43998</v>
+      </c>
+      <c r="U549">
+        <v>13</v>
+      </c>
+      <c r="V549">
+        <v>21</v>
+      </c>
+      <c r="W549">
+        <v>34</v>
+      </c>
+      <c r="X549">
+        <v>47</v>
+      </c>
+      <c r="Y549">
+        <v>13</v>
+      </c>
+      <c r="Z549">
+        <v>53</v>
+      </c>
+      <c r="AA549">
+        <v>21</v>
+      </c>
+      <c r="AB549">
+        <v>6</v>
+      </c>
+      <c r="AC549">
+        <v>4.1683</v>
+      </c>
+      <c r="AD549">
+        <v>-3.86584</v>
+      </c>
+      <c r="AE549">
+        <v>0</v>
+      </c>
+      <c r="AF549">
+        <v>512.2118399999999</v>
+      </c>
+      <c r="AG549">
+        <v>0</v>
+      </c>
+      <c r="AH549">
+        <v>3</v>
+      </c>
+      <c r="AI549">
+        <v>1574.04021</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B550" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol | Trabajo Complementario Seleccionados</t>
+        </is>
+      </c>
+      <c r="E550">
+        <v>124.945</v>
+      </c>
+      <c r="F550">
+        <v>9798.82</v>
+      </c>
+      <c r="G550">
+        <v>78.42506702949298</v>
+      </c>
+      <c r="H550">
+        <v>283.91</v>
+      </c>
+      <c r="I550">
+        <v>0</v>
+      </c>
+      <c r="J550">
+        <v>0</v>
+      </c>
+      <c r="K550">
+        <v>2.27227980311337</v>
+      </c>
+      <c r="L550">
+        <v>0</v>
+      </c>
+      <c r="M550">
+        <v>4</v>
+      </c>
+      <c r="N550">
+        <v>0</v>
+      </c>
+      <c r="O550">
+        <v>29.39568</v>
+      </c>
+      <c r="P550">
+        <v>89.04543802253725</v>
+      </c>
+      <c r="Q550">
+        <v>33.012</v>
+      </c>
+      <c r="R550">
+        <v>998.68046</v>
+      </c>
+      <c r="S550">
+        <v>7.992960582656369</v>
+      </c>
+      <c r="T550">
+        <v>1570.35004</v>
+      </c>
+      <c r="U550">
+        <v>67</v>
+      </c>
+      <c r="V550">
+        <v>51</v>
+      </c>
+      <c r="W550">
+        <v>118</v>
+      </c>
+      <c r="X550">
+        <v>209</v>
+      </c>
+      <c r="Y550">
+        <v>67</v>
+      </c>
+      <c r="Z550">
+        <v>182</v>
+      </c>
+      <c r="AA550">
+        <v>51</v>
+      </c>
+      <c r="AB550">
+        <v>40</v>
+      </c>
+      <c r="AC550">
+        <v>4.39316</v>
+      </c>
+      <c r="AD550">
+        <v>-2.95208</v>
+      </c>
+      <c r="AE550">
+        <v>0</v>
+      </c>
+      <c r="AF550">
+        <v>918.00306</v>
+      </c>
+      <c r="AG550">
+        <v>0</v>
+      </c>
+      <c r="AH550">
+        <v>3</v>
+      </c>
+      <c r="AI550">
+        <v>2996.04138</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B551" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E551">
+        <v>68.645</v>
+      </c>
+      <c r="F551">
+        <v>6093.87</v>
+      </c>
+      <c r="G551">
+        <v>88.77369072765678</v>
+      </c>
+      <c r="H551">
+        <v>295.41</v>
+      </c>
+      <c r="I551">
+        <v>8.789999999999999</v>
+      </c>
+      <c r="J551">
+        <v>1</v>
+      </c>
+      <c r="K551">
+        <v>4.30344526185447</v>
+      </c>
+      <c r="L551">
+        <v>23.08</v>
+      </c>
+      <c r="M551">
+        <v>9</v>
+      </c>
+      <c r="N551">
+        <v>1</v>
+      </c>
+      <c r="O551">
+        <v>31.93313</v>
+      </c>
+      <c r="P551">
+        <v>91.44653493699884</v>
+      </c>
+      <c r="Q551">
+        <v>34.92</v>
+      </c>
+      <c r="R551">
+        <v>495.67495</v>
+      </c>
+      <c r="S551">
+        <v>7.22084565518246</v>
+      </c>
+      <c r="T551">
+        <v>931.97999</v>
+      </c>
+      <c r="U551">
+        <v>27</v>
+      </c>
+      <c r="V551">
+        <v>12</v>
+      </c>
+      <c r="W551">
+        <v>39</v>
+      </c>
+      <c r="X551">
+        <v>72</v>
+      </c>
+      <c r="Y551">
+        <v>27</v>
+      </c>
+      <c r="Z551">
+        <v>61</v>
+      </c>
+      <c r="AA551">
+        <v>12</v>
+      </c>
+      <c r="AB551">
+        <v>12</v>
+      </c>
+      <c r="AC551">
+        <v>4.4267</v>
+      </c>
+      <c r="AD551">
+        <v>-3.47653</v>
+      </c>
+      <c r="AE551">
+        <v>0</v>
+      </c>
+      <c r="AF551">
+        <v>565.8896</v>
+      </c>
+      <c r="AG551">
+        <v>0</v>
+      </c>
+      <c r="AH551">
+        <v>3</v>
+      </c>
+      <c r="AI551">
+        <v>1487.02485</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B552" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E552">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F552">
+        <v>6803.6</v>
+      </c>
+      <c r="G552">
+        <v>98.7118630952525</v>
+      </c>
+      <c r="H552">
+        <v>353.97</v>
+      </c>
+      <c r="I552">
+        <v>8.52</v>
+      </c>
+      <c r="J552">
+        <v>1</v>
+      </c>
+      <c r="K552">
+        <v>5.135669083988848</v>
+      </c>
+      <c r="L552">
+        <v>27.46</v>
+      </c>
+      <c r="M552">
+        <v>7</v>
+      </c>
+      <c r="N552">
+        <v>2</v>
+      </c>
+      <c r="O552">
+        <v>32.17878</v>
+      </c>
+      <c r="P552">
+        <v>91.96039094650207</v>
+      </c>
+      <c r="Q552">
+        <v>34.992</v>
+      </c>
+      <c r="R552">
+        <v>548.18448</v>
+      </c>
+      <c r="S552">
+        <v>7.953482177185927</v>
+      </c>
+      <c r="T552">
+        <v>1217.81001</v>
+      </c>
+      <c r="U552">
+        <v>24</v>
+      </c>
+      <c r="V552">
+        <v>33</v>
+      </c>
+      <c r="W552">
+        <v>57</v>
+      </c>
+      <c r="X552">
+        <v>76</v>
+      </c>
+      <c r="Y552">
+        <v>24</v>
+      </c>
+      <c r="Z552">
+        <v>81</v>
+      </c>
+      <c r="AA552">
+        <v>33</v>
+      </c>
+      <c r="AB552">
+        <v>14</v>
+      </c>
+      <c r="AC552">
+        <v>4.7357</v>
+      </c>
+      <c r="AD552">
+        <v>-3.02069</v>
+      </c>
+      <c r="AE552">
+        <v>0</v>
+      </c>
+      <c r="AF552">
+        <v>575.31087</v>
+      </c>
+      <c r="AG552">
+        <v>0</v>
+      </c>
+      <c r="AH552">
+        <v>3</v>
+      </c>
+      <c r="AI552">
+        <v>1644.55344</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B553" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E553">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F553">
+        <v>7582.14</v>
+      </c>
+      <c r="G553">
+        <v>101.7113447238158</v>
+      </c>
+      <c r="H553">
+        <v>189.73</v>
+      </c>
+      <c r="I553">
+        <v>0</v>
+      </c>
+      <c r="J553">
+        <v>0</v>
+      </c>
+      <c r="K553">
+        <v>2.545151294284935</v>
+      </c>
+      <c r="L553">
+        <v>0</v>
+      </c>
+      <c r="M553">
+        <v>1</v>
+      </c>
+      <c r="N553">
+        <v>0</v>
+      </c>
+      <c r="O553">
+        <v>27.88366</v>
+      </c>
+      <c r="P553">
+        <v>77.45461111111111</v>
+      </c>
+      <c r="Q553">
+        <v>36</v>
+      </c>
+      <c r="R553">
+        <v>806.30009</v>
+      </c>
+      <c r="S553">
+        <v>10.81618994173594</v>
+      </c>
+      <c r="T553">
+        <v>1040.26998</v>
+      </c>
+      <c r="U553">
+        <v>7</v>
+      </c>
+      <c r="V553">
+        <v>16</v>
+      </c>
+      <c r="W553">
+        <v>23</v>
+      </c>
+      <c r="X553">
+        <v>85</v>
+      </c>
+      <c r="Y553">
+        <v>7</v>
+      </c>
+      <c r="Z553">
+        <v>75</v>
+      </c>
+      <c r="AA553">
+        <v>16</v>
+      </c>
+      <c r="AB553">
+        <v>14</v>
+      </c>
+      <c r="AC553">
+        <v>3.82887</v>
+      </c>
+      <c r="AD553">
+        <v>-2.79687</v>
+      </c>
+      <c r="AE553">
+        <v>0</v>
+      </c>
+      <c r="AF553">
+        <v>1748.17</v>
+      </c>
+      <c r="AG553">
+        <v>0</v>
+      </c>
+      <c r="AH553">
+        <v>3</v>
+      </c>
+      <c r="AI553">
+        <v>2418.90027</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B554" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E554">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F554">
+        <v>6212.759999999999</v>
+      </c>
+      <c r="G554">
+        <v>90.13950181722335</v>
+      </c>
+      <c r="H554">
+        <v>207.21</v>
+      </c>
+      <c r="I554">
+        <v>0</v>
+      </c>
+      <c r="J554">
+        <v>0</v>
+      </c>
+      <c r="K554">
+        <v>3.006362095356468</v>
+      </c>
+      <c r="L554">
+        <v>0</v>
+      </c>
+      <c r="M554">
+        <v>3</v>
+      </c>
+      <c r="N554">
+        <v>0</v>
+      </c>
+      <c r="O554">
+        <v>28.54373</v>
+      </c>
+      <c r="P554">
+        <v>83.99167255178908</v>
+      </c>
+      <c r="Q554">
+        <v>33.984</v>
+      </c>
+      <c r="R554">
+        <v>575.81569</v>
+      </c>
+      <c r="S554">
+        <v>8.354377029716378</v>
+      </c>
+      <c r="T554">
+        <v>793</v>
+      </c>
+      <c r="U554">
+        <v>6</v>
+      </c>
+      <c r="V554">
+        <v>14</v>
+      </c>
+      <c r="W554">
+        <v>20</v>
+      </c>
+      <c r="X554">
+        <v>49</v>
+      </c>
+      <c r="Y554">
+        <v>6</v>
+      </c>
+      <c r="Z554">
+        <v>53</v>
+      </c>
+      <c r="AA554">
+        <v>14</v>
+      </c>
+      <c r="AB554">
+        <v>8</v>
+      </c>
+      <c r="AC554">
+        <v>3.93893</v>
+      </c>
+      <c r="AD554">
+        <v>-4.07</v>
+      </c>
+      <c r="AE554">
+        <v>0</v>
+      </c>
+      <c r="AF554">
+        <v>568.2576</v>
+      </c>
+      <c r="AG554">
+        <v>0</v>
+      </c>
+      <c r="AH554">
+        <v>3</v>
+      </c>
+      <c r="AI554">
+        <v>1727.44707</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B555" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E555">
+        <v>68.645</v>
+      </c>
+      <c r="F555">
+        <v>6264.820000000001</v>
+      </c>
+      <c r="G555">
+        <v>91.26403962415327</v>
+      </c>
+      <c r="H555">
+        <v>389.56</v>
+      </c>
+      <c r="I555">
+        <v>0</v>
+      </c>
+      <c r="J555">
+        <v>0</v>
+      </c>
+      <c r="K555">
+        <v>5.674994537111225</v>
+      </c>
+      <c r="L555">
+        <v>0</v>
+      </c>
+      <c r="M555">
+        <v>9</v>
+      </c>
+      <c r="N555">
+        <v>0</v>
+      </c>
+      <c r="O555">
+        <v>28.00912</v>
+      </c>
+      <c r="P555">
+        <v>80.04435299497028</v>
+      </c>
+      <c r="Q555">
+        <v>34.992</v>
+      </c>
+      <c r="R555">
+        <v>517.38684</v>
+      </c>
+      <c r="S555">
+        <v>7.53713802898973</v>
+      </c>
+      <c r="T555">
+        <v>1109.4</v>
+      </c>
+      <c r="U555">
+        <v>17</v>
+      </c>
+      <c r="V555">
+        <v>23</v>
+      </c>
+      <c r="W555">
+        <v>40</v>
+      </c>
+      <c r="X555">
+        <v>80</v>
+      </c>
+      <c r="Y555">
+        <v>17</v>
+      </c>
+      <c r="Z555">
+        <v>83</v>
+      </c>
+      <c r="AA555">
+        <v>23</v>
+      </c>
+      <c r="AB555">
+        <v>24</v>
+      </c>
+      <c r="AC555">
+        <v>3.96046</v>
+      </c>
+      <c r="AD555">
+        <v>-2.98367</v>
+      </c>
+      <c r="AE555">
+        <v>0</v>
+      </c>
+      <c r="AF555">
+        <v>586.4672</v>
+      </c>
+      <c r="AG555">
+        <v>0</v>
+      </c>
+      <c r="AH555">
+        <v>3</v>
+      </c>
+      <c r="AI555">
+        <v>1552.16052</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B556" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E556">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F556">
+        <v>6230.11</v>
+      </c>
+      <c r="G556">
+        <v>90.39122896530711</v>
+      </c>
+      <c r="H556">
+        <v>181.98</v>
+      </c>
+      <c r="I556">
+        <v>4.84</v>
+      </c>
+      <c r="J556">
+        <v>1</v>
+      </c>
+      <c r="K556">
+        <v>2.640305844857729</v>
+      </c>
+      <c r="L556">
+        <v>4.84</v>
+      </c>
+      <c r="M556">
+        <v>1</v>
+      </c>
+      <c r="N556">
+        <v>0</v>
+      </c>
+      <c r="O556">
+        <v>30.03339</v>
+      </c>
+      <c r="P556">
+        <v>90.9771901126863</v>
+      </c>
+      <c r="Q556">
+        <v>33.012</v>
+      </c>
+      <c r="R556">
+        <v>586.84867</v>
+      </c>
+      <c r="S556">
+        <v>8.514451991691312</v>
+      </c>
+      <c r="T556">
+        <v>891.5000200000001</v>
+      </c>
+      <c r="U556">
+        <v>10</v>
+      </c>
+      <c r="V556">
+        <v>22</v>
+      </c>
+      <c r="W556">
+        <v>32</v>
+      </c>
+      <c r="X556">
+        <v>66</v>
+      </c>
+      <c r="Y556">
+        <v>10</v>
+      </c>
+      <c r="Z556">
+        <v>64</v>
+      </c>
+      <c r="AA556">
+        <v>22</v>
+      </c>
+      <c r="AB556">
+        <v>20</v>
+      </c>
+      <c r="AC556">
+        <v>4.22281</v>
+      </c>
+      <c r="AD556">
+        <v>-3.75422</v>
+      </c>
+      <c r="AE556">
+        <v>0</v>
+      </c>
+      <c r="AF556">
+        <v>540.8579999999999</v>
+      </c>
+      <c r="AG556">
+        <v>0</v>
+      </c>
+      <c r="AH556">
+        <v>3</v>
+      </c>
+      <c r="AI556">
+        <v>1760.54601</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B557" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E557">
+        <v>68.92383333333333</v>
+      </c>
+      <c r="F557">
+        <v>6592.84</v>
+      </c>
+      <c r="G557">
+        <v>95.65399486873191</v>
+      </c>
+      <c r="H557">
+        <v>111.45</v>
+      </c>
+      <c r="I557">
+        <v>0</v>
+      </c>
+      <c r="J557">
+        <v>0</v>
+      </c>
+      <c r="K557">
+        <v>1.617002343166249</v>
+      </c>
+      <c r="L557">
+        <v>0</v>
+      </c>
+      <c r="M557">
+        <v>3</v>
+      </c>
+      <c r="N557">
+        <v>0</v>
+      </c>
+      <c r="O557">
+        <v>27.54689</v>
+      </c>
+      <c r="P557">
+        <v>86.07327209098864</v>
+      </c>
+      <c r="Q557">
+        <v>32.004</v>
+      </c>
+      <c r="R557">
+        <v>593.68001</v>
+      </c>
+      <c r="S557">
+        <v>8.613566328048112</v>
+      </c>
+      <c r="T557">
+        <v>822.30999</v>
+      </c>
+      <c r="U557">
+        <v>9</v>
+      </c>
+      <c r="V557">
+        <v>19</v>
+      </c>
+      <c r="W557">
+        <v>28</v>
+      </c>
+      <c r="X557">
+        <v>63</v>
+      </c>
+      <c r="Y557">
+        <v>9</v>
+      </c>
+      <c r="Z557">
+        <v>61</v>
+      </c>
+      <c r="AA557">
+        <v>19</v>
+      </c>
+      <c r="AB557">
+        <v>10</v>
+      </c>
+      <c r="AC557">
+        <v>4.19277</v>
+      </c>
+      <c r="AD557">
+        <v>-3.51066</v>
+      </c>
+      <c r="AE557">
+        <v>0</v>
+      </c>
+      <c r="AF557">
+        <v>529.9609</v>
+      </c>
+      <c r="AG557">
+        <v>0</v>
+      </c>
+      <c r="AH557">
+        <v>3</v>
+      </c>
+      <c r="AI557">
+        <v>1781.04003</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B558" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E558">
+        <v>74.54566666666666</v>
+      </c>
+      <c r="F558">
+        <v>9115.679999999998</v>
+      </c>
+      <c r="G558">
+        <v>122.2831642348985</v>
+      </c>
+      <c r="H558">
+        <v>237.14</v>
+      </c>
+      <c r="I558">
+        <v>0</v>
+      </c>
+      <c r="J558">
+        <v>0</v>
+      </c>
+      <c r="K558">
+        <v>3.181137289446737</v>
+      </c>
+      <c r="L558">
+        <v>0</v>
+      </c>
+      <c r="M558">
+        <v>5</v>
+      </c>
+      <c r="N558">
+        <v>0</v>
+      </c>
+      <c r="O558">
+        <v>27.68776</v>
+      </c>
+      <c r="P558">
+        <v>76.91044444444445</v>
+      </c>
+      <c r="Q558">
+        <v>36</v>
+      </c>
+      <c r="R558">
+        <v>990.1090300000001</v>
+      </c>
+      <c r="S558">
+        <v>13.28191260837876</v>
+      </c>
+      <c r="T558">
+        <v>1303.98999</v>
+      </c>
+      <c r="U558">
+        <v>13</v>
+      </c>
+      <c r="V558">
+        <v>24</v>
+      </c>
+      <c r="W558">
+        <v>37</v>
+      </c>
+      <c r="X558">
+        <v>88</v>
+      </c>
+      <c r="Y558">
+        <v>13</v>
+      </c>
+      <c r="Z558">
+        <v>99</v>
+      </c>
+      <c r="AA558">
+        <v>24</v>
+      </c>
+      <c r="AB558">
+        <v>25</v>
+      </c>
+      <c r="AC558">
+        <v>3.99845</v>
+      </c>
+      <c r="AD558">
+        <v>-2.92672</v>
+      </c>
+      <c r="AE558">
+        <v>0</v>
+      </c>
+      <c r="AF558">
+        <v>2104.014</v>
+      </c>
+      <c r="AG558">
+        <v>0</v>
+      </c>
+      <c r="AH558">
+        <v>3</v>
+      </c>
+      <c r="AI558">
+        <v>2970.32709</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B559" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol</t>
+        </is>
+      </c>
+      <c r="E559">
+        <v>68.645</v>
+      </c>
+      <c r="F559">
+        <v>7865.73</v>
+      </c>
+      <c r="G559">
+        <v>114.5856216767427</v>
+      </c>
+      <c r="H559">
+        <v>295.18</v>
+      </c>
+      <c r="I559">
+        <v>0</v>
+      </c>
+      <c r="J559">
+        <v>0</v>
+      </c>
+      <c r="K559">
+        <v>4.30009469007211</v>
+      </c>
+      <c r="L559">
+        <v>18.91</v>
+      </c>
+      <c r="M559">
+        <v>6</v>
+      </c>
+      <c r="N559">
+        <v>1</v>
+      </c>
+      <c r="O559">
+        <v>30.87018</v>
+      </c>
+      <c r="P559">
+        <v>85.7505</v>
+      </c>
+      <c r="Q559">
+        <v>36</v>
+      </c>
+      <c r="R559">
+        <v>819.7710400000001</v>
+      </c>
+      <c r="S559">
+        <v>11.94218136790735</v>
+      </c>
+      <c r="T559">
+        <v>1243.38</v>
+      </c>
+      <c r="U559">
+        <v>17</v>
+      </c>
+      <c r="V559">
+        <v>17</v>
+      </c>
+      <c r="W559">
+        <v>34</v>
+      </c>
+      <c r="X559">
+        <v>89</v>
+      </c>
+      <c r="Y559">
+        <v>17</v>
+      </c>
+      <c r="Z559">
+        <v>84</v>
+      </c>
+      <c r="AA559">
+        <v>17</v>
+      </c>
+      <c r="AB559">
+        <v>27</v>
+      </c>
+      <c r="AC559">
+        <v>3.75666</v>
+      </c>
+      <c r="AD559">
+        <v>-2.70669</v>
+      </c>
+      <c r="AE559">
+        <v>0</v>
+      </c>
+      <c r="AF559">
+        <v>1800.72</v>
+      </c>
+      <c r="AG559">
+        <v>0</v>
+      </c>
+      <c r="AH559">
+        <v>3</v>
+      </c>
+      <c r="AI559">
+        <v>2459.31312</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B560" s="2">
+        <v>46218</v>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Sesión 35 Futbol | Trabajo Complementario Seleccionados</t>
+        </is>
+      </c>
+      <c r="E560">
+        <v>124.945</v>
+      </c>
+      <c r="F560">
+        <v>9900.959999999999</v>
+      </c>
+      <c r="G560">
+        <v>79.24254672055704</v>
+      </c>
+      <c r="H560">
+        <v>19.61</v>
+      </c>
+      <c r="I560">
+        <v>0</v>
+      </c>
+      <c r="J560">
+        <v>0</v>
+      </c>
+      <c r="K560">
+        <v>0.1569490575853376</v>
+      </c>
+      <c r="L560">
+        <v>0</v>
+      </c>
+      <c r="M560">
+        <v>0</v>
+      </c>
+      <c r="N560">
+        <v>0</v>
+      </c>
+      <c r="O560">
+        <v>27.99556</v>
+      </c>
+      <c r="P560">
+        <v>77.76544444444444</v>
+      </c>
+      <c r="Q560">
+        <v>36</v>
+      </c>
+      <c r="R560">
+        <v>1031.92493</v>
+      </c>
+      <c r="S560">
+        <v>8.259033414702468</v>
+      </c>
+      <c r="T560">
+        <v>603.70001</v>
+      </c>
+      <c r="U560">
+        <v>65</v>
+      </c>
+      <c r="V560">
+        <v>53</v>
+      </c>
+      <c r="W560">
+        <v>118</v>
+      </c>
+      <c r="X560">
+        <v>125</v>
+      </c>
+      <c r="Y560">
+        <v>65</v>
+      </c>
+      <c r="Z560">
+        <v>114</v>
+      </c>
+      <c r="AA560">
+        <v>53</v>
+      </c>
+      <c r="AB560">
+        <v>22</v>
+      </c>
+      <c r="AC560">
+        <v>4.03883</v>
+      </c>
+      <c r="AD560">
+        <v>-2.48396</v>
+      </c>
+      <c r="AE560">
+        <v>0</v>
+      </c>
+      <c r="AF560">
+        <v>356.4288</v>
+      </c>
+      <c r="AG560">
+        <v>0</v>
+      </c>
+      <c r="AH560">
+        <v>3</v>
+      </c>
+      <c r="AI560">
+        <v>3095.774789999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-17
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI560"/>
+  <dimension ref="A1:AI581"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -63595,6 +63595,2379 @@
         <v>3095.774789999999</v>
       </c>
     </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B561" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E561">
+        <v>57.85166666666667</v>
+      </c>
+      <c r="F561">
+        <v>3619.45</v>
+      </c>
+      <c r="G561">
+        <v>62.56431678718562</v>
+      </c>
+      <c r="H561">
+        <v>0</v>
+      </c>
+      <c r="I561">
+        <v>0</v>
+      </c>
+      <c r="J561">
+        <v>0</v>
+      </c>
+      <c r="K561">
+        <v>0</v>
+      </c>
+      <c r="L561">
+        <v>0</v>
+      </c>
+      <c r="M561">
+        <v>0</v>
+      </c>
+      <c r="N561">
+        <v>0</v>
+      </c>
+      <c r="O561">
+        <v>19.07908</v>
+      </c>
+      <c r="P561">
+        <v>52.99744444444445</v>
+      </c>
+      <c r="Q561">
+        <v>36</v>
+      </c>
+      <c r="R561">
+        <v>426.10351</v>
+      </c>
+      <c r="S561">
+        <v>7.365449165970442</v>
+      </c>
+      <c r="T561">
+        <v>145.99001</v>
+      </c>
+      <c r="U561">
+        <v>1</v>
+      </c>
+      <c r="V561">
+        <v>3</v>
+      </c>
+      <c r="W561">
+        <v>4</v>
+      </c>
+      <c r="X561">
+        <v>26</v>
+      </c>
+      <c r="Y561">
+        <v>1</v>
+      </c>
+      <c r="Z561">
+        <v>23</v>
+      </c>
+      <c r="AA561">
+        <v>3</v>
+      </c>
+      <c r="AB561">
+        <v>28</v>
+      </c>
+      <c r="AC561">
+        <v>3.24924</v>
+      </c>
+      <c r="AD561">
+        <v>-1.4842</v>
+      </c>
+      <c r="AE561">
+        <v>0</v>
+      </c>
+      <c r="AF561">
+        <v>787.74</v>
+      </c>
+      <c r="AG561">
+        <v>0</v>
+      </c>
+      <c r="AH561">
+        <v>3</v>
+      </c>
+      <c r="AI561">
+        <v>1278.31053</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B562" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E562">
+        <v>109.1</v>
+      </c>
+      <c r="F562">
+        <v>5930.99</v>
+      </c>
+      <c r="G562">
+        <v>54.36287809349221</v>
+      </c>
+      <c r="H562">
+        <v>14.16</v>
+      </c>
+      <c r="I562">
+        <v>0</v>
+      </c>
+      <c r="J562">
+        <v>0</v>
+      </c>
+      <c r="K562">
+        <v>0.1297891842346471</v>
+      </c>
+      <c r="L562">
+        <v>0</v>
+      </c>
+      <c r="M562">
+        <v>0</v>
+      </c>
+      <c r="N562">
+        <v>0</v>
+      </c>
+      <c r="O562">
+        <v>23.00776</v>
+      </c>
+      <c r="P562">
+        <v>71.09059448770239</v>
+      </c>
+      <c r="Q562">
+        <v>32.364</v>
+      </c>
+      <c r="R562">
+        <v>520.34255</v>
+      </c>
+      <c r="S562">
+        <v>4.76940925756187</v>
+      </c>
+      <c r="T562">
+        <v>368.81999</v>
+      </c>
+      <c r="U562">
+        <v>0</v>
+      </c>
+      <c r="V562">
+        <v>4</v>
+      </c>
+      <c r="W562">
+        <v>4</v>
+      </c>
+      <c r="X562">
+        <v>25</v>
+      </c>
+      <c r="Y562">
+        <v>0</v>
+      </c>
+      <c r="Z562">
+        <v>24</v>
+      </c>
+      <c r="AA562">
+        <v>4</v>
+      </c>
+      <c r="AB562">
+        <v>3</v>
+      </c>
+      <c r="AC562">
+        <v>2.98685</v>
+      </c>
+      <c r="AD562">
+        <v>-1.0611</v>
+      </c>
+      <c r="AE562">
+        <v>0</v>
+      </c>
+      <c r="AF562">
+        <v>454.6192</v>
+      </c>
+      <c r="AG562">
+        <v>0</v>
+      </c>
+      <c r="AH562">
+        <v>3</v>
+      </c>
+      <c r="AI562">
+        <v>1561.02765</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B563" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E563">
+        <v>109.1</v>
+      </c>
+      <c r="F563">
+        <v>5329.31</v>
+      </c>
+      <c r="G563">
+        <v>48.84793767186068</v>
+      </c>
+      <c r="H563">
+        <v>81.97</v>
+      </c>
+      <c r="I563">
+        <v>0</v>
+      </c>
+      <c r="J563">
+        <v>0</v>
+      </c>
+      <c r="K563">
+        <v>0.7513290559120074</v>
+      </c>
+      <c r="L563">
+        <v>0</v>
+      </c>
+      <c r="M563">
+        <v>2</v>
+      </c>
+      <c r="N563">
+        <v>0</v>
+      </c>
+      <c r="O563">
+        <v>28.47501</v>
+      </c>
+      <c r="P563">
+        <v>79.09725</v>
+      </c>
+      <c r="Q563">
+        <v>36</v>
+      </c>
+      <c r="R563">
+        <v>475.71788</v>
+      </c>
+      <c r="S563">
+        <v>4.360383868010999</v>
+      </c>
+      <c r="T563">
+        <v>434.68001</v>
+      </c>
+      <c r="U563">
+        <v>11</v>
+      </c>
+      <c r="V563">
+        <v>21</v>
+      </c>
+      <c r="W563">
+        <v>32</v>
+      </c>
+      <c r="X563">
+        <v>51</v>
+      </c>
+      <c r="Y563">
+        <v>11</v>
+      </c>
+      <c r="Z563">
+        <v>57</v>
+      </c>
+      <c r="AA563">
+        <v>21</v>
+      </c>
+      <c r="AB563">
+        <v>27</v>
+      </c>
+      <c r="AC563">
+        <v>4.49735</v>
+      </c>
+      <c r="AD563">
+        <v>-1.72201</v>
+      </c>
+      <c r="AE563">
+        <v>0</v>
+      </c>
+      <c r="AF563">
+        <v>1223.156</v>
+      </c>
+      <c r="AG563">
+        <v>0</v>
+      </c>
+      <c r="AH563">
+        <v>3</v>
+      </c>
+      <c r="AI563">
+        <v>1427.15364</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B564" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E564">
+        <v>109.1</v>
+      </c>
+      <c r="F564">
+        <v>6400.55</v>
+      </c>
+      <c r="G564">
+        <v>58.66681943171403</v>
+      </c>
+      <c r="H564">
+        <v>106.2</v>
+      </c>
+      <c r="I564">
+        <v>0</v>
+      </c>
+      <c r="J564">
+        <v>0</v>
+      </c>
+      <c r="K564">
+        <v>0.9734188817598535</v>
+      </c>
+      <c r="L564">
+        <v>0</v>
+      </c>
+      <c r="M564">
+        <v>0</v>
+      </c>
+      <c r="N564">
+        <v>0</v>
+      </c>
+      <c r="O564">
+        <v>24.10305</v>
+      </c>
+      <c r="P564">
+        <v>74.39212962962964</v>
+      </c>
+      <c r="Q564">
+        <v>32.4</v>
+      </c>
+      <c r="R564">
+        <v>673.64475</v>
+      </c>
+      <c r="S564">
+        <v>6.174562328139323</v>
+      </c>
+      <c r="T564">
+        <v>599.7799799999999</v>
+      </c>
+      <c r="U564">
+        <v>16</v>
+      </c>
+      <c r="V564">
+        <v>8</v>
+      </c>
+      <c r="W564">
+        <v>24</v>
+      </c>
+      <c r="X564">
+        <v>52</v>
+      </c>
+      <c r="Y564">
+        <v>16</v>
+      </c>
+      <c r="Z564">
+        <v>44</v>
+      </c>
+      <c r="AA564">
+        <v>8</v>
+      </c>
+      <c r="AB564">
+        <v>10</v>
+      </c>
+      <c r="AC564">
+        <v>4.33268</v>
+      </c>
+      <c r="AD564">
+        <v>-1.4748</v>
+      </c>
+      <c r="AE564">
+        <v>0</v>
+      </c>
+      <c r="AF564">
+        <v>508.3407</v>
+      </c>
+      <c r="AG564">
+        <v>0</v>
+      </c>
+      <c r="AH564">
+        <v>3</v>
+      </c>
+      <c r="AI564">
+        <v>2020.93425</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B565" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Trabajo Compensatorio Seleccionados | Sesión 36</t>
+        </is>
+      </c>
+      <c r="E565">
+        <v>133.5635</v>
+      </c>
+      <c r="F565">
+        <v>8914.09</v>
+      </c>
+      <c r="G565">
+        <v>66.74046427354779</v>
+      </c>
+      <c r="H565">
+        <v>83.56</v>
+      </c>
+      <c r="I565">
+        <v>0</v>
+      </c>
+      <c r="J565">
+        <v>0</v>
+      </c>
+      <c r="K565">
+        <v>0.6256200234345461</v>
+      </c>
+      <c r="L565">
+        <v>0</v>
+      </c>
+      <c r="M565">
+        <v>0</v>
+      </c>
+      <c r="N565">
+        <v>0</v>
+      </c>
+      <c r="O565">
+        <v>24.43063</v>
+      </c>
+      <c r="P565">
+        <v>68.61765531962702</v>
+      </c>
+      <c r="Q565">
+        <v>35.604</v>
+      </c>
+      <c r="R565">
+        <v>906.86059</v>
+      </c>
+      <c r="S565">
+        <v>6.789733647291363</v>
+      </c>
+      <c r="T565">
+        <v>643.9899800000001</v>
+      </c>
+      <c r="U565">
+        <v>36</v>
+      </c>
+      <c r="V565">
+        <v>17</v>
+      </c>
+      <c r="W565">
+        <v>53</v>
+      </c>
+      <c r="X565">
+        <v>82</v>
+      </c>
+      <c r="Y565">
+        <v>36</v>
+      </c>
+      <c r="Z565">
+        <v>65</v>
+      </c>
+      <c r="AA565">
+        <v>17</v>
+      </c>
+      <c r="AB565">
+        <v>63</v>
+      </c>
+      <c r="AC565">
+        <v>4.18915</v>
+      </c>
+      <c r="AD565">
+        <v>-1.08856</v>
+      </c>
+      <c r="AE565">
+        <v>0</v>
+      </c>
+      <c r="AF565">
+        <v>435.62547</v>
+      </c>
+      <c r="AG565">
+        <v>0</v>
+      </c>
+      <c r="AH565">
+        <v>3</v>
+      </c>
+      <c r="AI565">
+        <v>2720.58177</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B566" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E566">
+        <v>109.1</v>
+      </c>
+      <c r="F566">
+        <v>6519.44</v>
+      </c>
+      <c r="G566">
+        <v>59.75655362053162</v>
+      </c>
+      <c r="H566">
+        <v>143.96</v>
+      </c>
+      <c r="I566">
+        <v>0</v>
+      </c>
+      <c r="J566">
+        <v>0</v>
+      </c>
+      <c r="K566">
+        <v>1.319523373052246</v>
+      </c>
+      <c r="L566">
+        <v>0</v>
+      </c>
+      <c r="M566">
+        <v>1</v>
+      </c>
+      <c r="N566">
+        <v>0</v>
+      </c>
+      <c r="O566">
+        <v>27.51977</v>
+      </c>
+      <c r="P566">
+        <v>80.97860758003766</v>
+      </c>
+      <c r="Q566">
+        <v>33.984</v>
+      </c>
+      <c r="R566">
+        <v>749.11592</v>
+      </c>
+      <c r="S566">
+        <v>6.866323739688359</v>
+      </c>
+      <c r="T566">
+        <v>671.4800300000001</v>
+      </c>
+      <c r="U566">
+        <v>15</v>
+      </c>
+      <c r="V566">
+        <v>11</v>
+      </c>
+      <c r="W566">
+        <v>26</v>
+      </c>
+      <c r="X566">
+        <v>54</v>
+      </c>
+      <c r="Y566">
+        <v>15</v>
+      </c>
+      <c r="Z566">
+        <v>54</v>
+      </c>
+      <c r="AA566">
+        <v>11</v>
+      </c>
+      <c r="AB566">
+        <v>9</v>
+      </c>
+      <c r="AC566">
+        <v>4.23477</v>
+      </c>
+      <c r="AD566">
+        <v>-1.7335</v>
+      </c>
+      <c r="AE566">
+        <v>0</v>
+      </c>
+      <c r="AF566">
+        <v>592.8904</v>
+      </c>
+      <c r="AG566">
+        <v>0</v>
+      </c>
+      <c r="AH566">
+        <v>3</v>
+      </c>
+      <c r="AI566">
+        <v>2247.34776</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B567" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E567">
+        <v>109.1</v>
+      </c>
+      <c r="F567">
+        <v>6270.360000000001</v>
+      </c>
+      <c r="G567">
+        <v>57.47351054078828</v>
+      </c>
+      <c r="H567">
+        <v>231.29</v>
+      </c>
+      <c r="I567">
+        <v>0</v>
+      </c>
+      <c r="J567">
+        <v>0</v>
+      </c>
+      <c r="K567">
+        <v>2.119981668194317</v>
+      </c>
+      <c r="L567">
+        <v>6.62</v>
+      </c>
+      <c r="M567">
+        <v>8</v>
+      </c>
+      <c r="N567">
+        <v>1</v>
+      </c>
+      <c r="O567">
+        <v>30.33459</v>
+      </c>
+      <c r="P567">
+        <v>85.28618421052632</v>
+      </c>
+      <c r="Q567">
+        <v>35.568</v>
+      </c>
+      <c r="R567">
+        <v>560.21913</v>
+      </c>
+      <c r="S567">
+        <v>5.134914115490376</v>
+      </c>
+      <c r="T567">
+        <v>701.28002</v>
+      </c>
+      <c r="U567">
+        <v>23</v>
+      </c>
+      <c r="V567">
+        <v>11</v>
+      </c>
+      <c r="W567">
+        <v>34</v>
+      </c>
+      <c r="X567">
+        <v>79</v>
+      </c>
+      <c r="Y567">
+        <v>23</v>
+      </c>
+      <c r="Z567">
+        <v>42</v>
+      </c>
+      <c r="AA567">
+        <v>11</v>
+      </c>
+      <c r="AB567">
+        <v>5</v>
+      </c>
+      <c r="AC567">
+        <v>4.81771</v>
+      </c>
+      <c r="AD567">
+        <v>-1.91828</v>
+      </c>
+      <c r="AE567">
+        <v>0</v>
+      </c>
+      <c r="AF567">
+        <v>576.884</v>
+      </c>
+      <c r="AG567">
+        <v>0</v>
+      </c>
+      <c r="AH567">
+        <v>3</v>
+      </c>
+      <c r="AI567">
+        <v>1680.65739</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B568" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E568">
+        <v>109.1</v>
+      </c>
+      <c r="F568">
+        <v>6003.08</v>
+      </c>
+      <c r="G568">
+        <v>55.02364802933089</v>
+      </c>
+      <c r="H568">
+        <v>144.87</v>
+      </c>
+      <c r="I568">
+        <v>0</v>
+      </c>
+      <c r="J568">
+        <v>0</v>
+      </c>
+      <c r="K568">
+        <v>1.327864344637947</v>
+      </c>
+      <c r="L568">
+        <v>0</v>
+      </c>
+      <c r="M568">
+        <v>3</v>
+      </c>
+      <c r="N568">
+        <v>0</v>
+      </c>
+      <c r="O568">
+        <v>27.91903</v>
+      </c>
+      <c r="P568">
+        <v>77.5528611111111</v>
+      </c>
+      <c r="Q568">
+        <v>36</v>
+      </c>
+      <c r="R568">
+        <v>596.4438700000001</v>
+      </c>
+      <c r="S568">
+        <v>5.466946562786435</v>
+      </c>
+      <c r="T568">
+        <v>521.1300100000001</v>
+      </c>
+      <c r="U568">
+        <v>9</v>
+      </c>
+      <c r="V568">
+        <v>9</v>
+      </c>
+      <c r="W568">
+        <v>18</v>
+      </c>
+      <c r="X568">
+        <v>51</v>
+      </c>
+      <c r="Y568">
+        <v>9</v>
+      </c>
+      <c r="Z568">
+        <v>36</v>
+      </c>
+      <c r="AA568">
+        <v>9</v>
+      </c>
+      <c r="AB568">
+        <v>13</v>
+      </c>
+      <c r="AC568">
+        <v>3.9627</v>
+      </c>
+      <c r="AD568">
+        <v>-1.66964</v>
+      </c>
+      <c r="AE568">
+        <v>0</v>
+      </c>
+      <c r="AF568">
+        <v>1344.698</v>
+      </c>
+      <c r="AG568">
+        <v>0</v>
+      </c>
+      <c r="AH568">
+        <v>3</v>
+      </c>
+      <c r="AI568">
+        <v>1789.33161</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B569" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Trabajo Compensatorio Seleccionados</t>
+        </is>
+      </c>
+      <c r="E569">
+        <v>75.71183333333333</v>
+      </c>
+      <c r="F569">
+        <v>5329.58</v>
+      </c>
+      <c r="G569">
+        <v>70.39295926880651</v>
+      </c>
+      <c r="H569">
+        <v>451.59</v>
+      </c>
+      <c r="I569">
+        <v>0</v>
+      </c>
+      <c r="J569">
+        <v>0</v>
+      </c>
+      <c r="K569">
+        <v>5.964589419091247</v>
+      </c>
+      <c r="L569">
+        <v>0</v>
+      </c>
+      <c r="M569">
+        <v>3</v>
+      </c>
+      <c r="N569">
+        <v>0</v>
+      </c>
+      <c r="O569">
+        <v>28.26205</v>
+      </c>
+      <c r="P569">
+        <v>78.50569444444444</v>
+      </c>
+      <c r="Q569">
+        <v>36</v>
+      </c>
+      <c r="R569">
+        <v>590.72986</v>
+      </c>
+      <c r="S569">
+        <v>7.802345208036614</v>
+      </c>
+      <c r="T569">
+        <v>1022.05001</v>
+      </c>
+      <c r="U569">
+        <v>38</v>
+      </c>
+      <c r="V569">
+        <v>42</v>
+      </c>
+      <c r="W569">
+        <v>80</v>
+      </c>
+      <c r="X569">
+        <v>102</v>
+      </c>
+      <c r="Y569">
+        <v>38</v>
+      </c>
+      <c r="Z569">
+        <v>88</v>
+      </c>
+      <c r="AA569">
+        <v>42</v>
+      </c>
+      <c r="AB569">
+        <v>79</v>
+      </c>
+      <c r="AC569">
+        <v>4.68853</v>
+      </c>
+      <c r="AD569">
+        <v>-2.40284</v>
+      </c>
+      <c r="AE569">
+        <v>0</v>
+      </c>
+      <c r="AF569">
+        <v>454.5121</v>
+      </c>
+      <c r="AG569">
+        <v>0</v>
+      </c>
+      <c r="AH569">
+        <v>3</v>
+      </c>
+      <c r="AI569">
+        <v>1772.18958</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B570" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E570">
+        <v>109.1</v>
+      </c>
+      <c r="F570">
+        <v>5730.83</v>
+      </c>
+      <c r="G570">
+        <v>52.52823098075161</v>
+      </c>
+      <c r="H570">
+        <v>177.62</v>
+      </c>
+      <c r="I570">
+        <v>0</v>
+      </c>
+      <c r="J570">
+        <v>0</v>
+      </c>
+      <c r="K570">
+        <v>1.628047662694776</v>
+      </c>
+      <c r="L570">
+        <v>0</v>
+      </c>
+      <c r="M570">
+        <v>4</v>
+      </c>
+      <c r="N570">
+        <v>0</v>
+      </c>
+      <c r="O570">
+        <v>28.13935</v>
+      </c>
+      <c r="P570">
+        <v>87.92447819022622</v>
+      </c>
+      <c r="Q570">
+        <v>32.004</v>
+      </c>
+      <c r="R570">
+        <v>562.41122</v>
+      </c>
+      <c r="S570">
+        <v>5.155006599450045</v>
+      </c>
+      <c r="T570">
+        <v>526.91999</v>
+      </c>
+      <c r="U570">
+        <v>8</v>
+      </c>
+      <c r="V570">
+        <v>7</v>
+      </c>
+      <c r="W570">
+        <v>15</v>
+      </c>
+      <c r="X570">
+        <v>29</v>
+      </c>
+      <c r="Y570">
+        <v>8</v>
+      </c>
+      <c r="Z570">
+        <v>36</v>
+      </c>
+      <c r="AA570">
+        <v>7</v>
+      </c>
+      <c r="AB570">
+        <v>8</v>
+      </c>
+      <c r="AC570">
+        <v>3.8637</v>
+      </c>
+      <c r="AD570">
+        <v>-1.80736</v>
+      </c>
+      <c r="AE570">
+        <v>0</v>
+      </c>
+      <c r="AF570">
+        <v>384.4548</v>
+      </c>
+      <c r="AG570">
+        <v>0</v>
+      </c>
+      <c r="AH570">
+        <v>3</v>
+      </c>
+      <c r="AI570">
+        <v>1687.23366</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B571" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E571">
+        <v>109.1</v>
+      </c>
+      <c r="F571">
+        <v>5205.849999999999</v>
+      </c>
+      <c r="G571">
+        <v>47.71631530705774</v>
+      </c>
+      <c r="H571">
+        <v>55.58000000000001</v>
+      </c>
+      <c r="I571">
+        <v>0</v>
+      </c>
+      <c r="J571">
+        <v>0</v>
+      </c>
+      <c r="K571">
+        <v>0.5094408799266729</v>
+      </c>
+      <c r="L571">
+        <v>0</v>
+      </c>
+      <c r="M571">
+        <v>1</v>
+      </c>
+      <c r="N571">
+        <v>0</v>
+      </c>
+      <c r="O571">
+        <v>25.65004</v>
+      </c>
+      <c r="P571">
+        <v>76.12191358024693</v>
+      </c>
+      <c r="Q571">
+        <v>33.696</v>
+      </c>
+      <c r="R571">
+        <v>477.91379</v>
+      </c>
+      <c r="S571">
+        <v>4.380511365719523</v>
+      </c>
+      <c r="T571">
+        <v>431.48001</v>
+      </c>
+      <c r="U571">
+        <v>12</v>
+      </c>
+      <c r="V571">
+        <v>11</v>
+      </c>
+      <c r="W571">
+        <v>23</v>
+      </c>
+      <c r="X571">
+        <v>53</v>
+      </c>
+      <c r="Y571">
+        <v>12</v>
+      </c>
+      <c r="Z571">
+        <v>53</v>
+      </c>
+      <c r="AA571">
+        <v>11</v>
+      </c>
+      <c r="AB571">
+        <v>9</v>
+      </c>
+      <c r="AC571">
+        <v>4.15782</v>
+      </c>
+      <c r="AD571">
+        <v>-2.21075</v>
+      </c>
+      <c r="AE571">
+        <v>0</v>
+      </c>
+      <c r="AF571">
+        <v>471.4504</v>
+      </c>
+      <c r="AG571">
+        <v>0</v>
+      </c>
+      <c r="AH571">
+        <v>3</v>
+      </c>
+      <c r="AI571">
+        <v>1433.74137</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B572" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E572">
+        <v>109.1</v>
+      </c>
+      <c r="F572">
+        <v>6678.85</v>
+      </c>
+      <c r="G572">
+        <v>61.21769019248396</v>
+      </c>
+      <c r="H572">
+        <v>215.33</v>
+      </c>
+      <c r="I572">
+        <v>0</v>
+      </c>
+      <c r="J572">
+        <v>0</v>
+      </c>
+      <c r="K572">
+        <v>1.973693858845096</v>
+      </c>
+      <c r="L572">
+        <v>0</v>
+      </c>
+      <c r="M572">
+        <v>3</v>
+      </c>
+      <c r="N572">
+        <v>0</v>
+      </c>
+      <c r="O572">
+        <v>28.96125</v>
+      </c>
+      <c r="P572">
+        <v>82.76534636488341</v>
+      </c>
+      <c r="Q572">
+        <v>34.992</v>
+      </c>
+      <c r="R572">
+        <v>626.70978</v>
+      </c>
+      <c r="S572">
+        <v>5.744360953253896</v>
+      </c>
+      <c r="T572">
+        <v>757.0200199999999</v>
+      </c>
+      <c r="U572">
+        <v>17</v>
+      </c>
+      <c r="V572">
+        <v>12</v>
+      </c>
+      <c r="W572">
+        <v>29</v>
+      </c>
+      <c r="X572">
+        <v>59</v>
+      </c>
+      <c r="Y572">
+        <v>17</v>
+      </c>
+      <c r="Z572">
+        <v>55</v>
+      </c>
+      <c r="AA572">
+        <v>12</v>
+      </c>
+      <c r="AB572">
+        <v>105</v>
+      </c>
+      <c r="AC572">
+        <v>4.52839</v>
+      </c>
+      <c r="AD572">
+        <v>-1.22979</v>
+      </c>
+      <c r="AE572">
+        <v>0</v>
+      </c>
+      <c r="AF572">
+        <v>521.36607</v>
+      </c>
+      <c r="AG572">
+        <v>0</v>
+      </c>
+      <c r="AH572">
+        <v>3</v>
+      </c>
+      <c r="AI572">
+        <v>1880.12934</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B573" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Trabajo Compensatorio Seleccionados | Sesión 36</t>
+        </is>
+      </c>
+      <c r="E573">
+        <v>133.5635</v>
+      </c>
+      <c r="F573">
+        <v>8876.82</v>
+      </c>
+      <c r="G573">
+        <v>66.46142097204699</v>
+      </c>
+      <c r="H573">
+        <v>120.61</v>
+      </c>
+      <c r="I573">
+        <v>0</v>
+      </c>
+      <c r="J573">
+        <v>0</v>
+      </c>
+      <c r="K573">
+        <v>0.903016168339404</v>
+      </c>
+      <c r="L573">
+        <v>0</v>
+      </c>
+      <c r="M573">
+        <v>0</v>
+      </c>
+      <c r="N573">
+        <v>0</v>
+      </c>
+      <c r="O573">
+        <v>22.80464</v>
+      </c>
+      <c r="P573">
+        <v>69.07984975160547</v>
+      </c>
+      <c r="Q573">
+        <v>33.012</v>
+      </c>
+      <c r="R573">
+        <v>1002.77152</v>
+      </c>
+      <c r="S573">
+        <v>7.507826015341017</v>
+      </c>
+      <c r="T573">
+        <v>778.7099900000001</v>
+      </c>
+      <c r="U573">
+        <v>34</v>
+      </c>
+      <c r="V573">
+        <v>26</v>
+      </c>
+      <c r="W573">
+        <v>60</v>
+      </c>
+      <c r="X573">
+        <v>84</v>
+      </c>
+      <c r="Y573">
+        <v>34</v>
+      </c>
+      <c r="Z573">
+        <v>78</v>
+      </c>
+      <c r="AA573">
+        <v>26</v>
+      </c>
+      <c r="AB573">
+        <v>31</v>
+      </c>
+      <c r="AC573">
+        <v>4.11861</v>
+      </c>
+      <c r="AD573">
+        <v>-1.26624</v>
+      </c>
+      <c r="AE573">
+        <v>0</v>
+      </c>
+      <c r="AF573">
+        <v>779.63964</v>
+      </c>
+      <c r="AG573">
+        <v>0</v>
+      </c>
+      <c r="AH573">
+        <v>3</v>
+      </c>
+      <c r="AI573">
+        <v>3008.31456</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B574" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E574">
+        <v>109.1</v>
+      </c>
+      <c r="F574">
+        <v>5788.33</v>
+      </c>
+      <c r="G574">
+        <v>53.05527039413382</v>
+      </c>
+      <c r="H574">
+        <v>142.08</v>
+      </c>
+      <c r="I574">
+        <v>0</v>
+      </c>
+      <c r="J574">
+        <v>0</v>
+      </c>
+      <c r="K574">
+        <v>1.302291475710357</v>
+      </c>
+      <c r="L574">
+        <v>0</v>
+      </c>
+      <c r="M574">
+        <v>2</v>
+      </c>
+      <c r="N574">
+        <v>0</v>
+      </c>
+      <c r="O574">
+        <v>26.70143</v>
+      </c>
+      <c r="P574">
+        <v>76.46457617411225</v>
+      </c>
+      <c r="Q574">
+        <v>34.92</v>
+      </c>
+      <c r="R574">
+        <v>555.78894</v>
+      </c>
+      <c r="S574">
+        <v>5.094307424381302</v>
+      </c>
+      <c r="T574">
+        <v>528.57999</v>
+      </c>
+      <c r="U574">
+        <v>11</v>
+      </c>
+      <c r="V574">
+        <v>6</v>
+      </c>
+      <c r="W574">
+        <v>17</v>
+      </c>
+      <c r="X574">
+        <v>60</v>
+      </c>
+      <c r="Y574">
+        <v>11</v>
+      </c>
+      <c r="Z574">
+        <v>33</v>
+      </c>
+      <c r="AA574">
+        <v>6</v>
+      </c>
+      <c r="AB574">
+        <v>110</v>
+      </c>
+      <c r="AC574">
+        <v>3.84773</v>
+      </c>
+      <c r="AD574">
+        <v>-1.45918</v>
+      </c>
+      <c r="AE574">
+        <v>0</v>
+      </c>
+      <c r="AF574">
+        <v>521.5592</v>
+      </c>
+      <c r="AG574">
+        <v>0</v>
+      </c>
+      <c r="AH574">
+        <v>3</v>
+      </c>
+      <c r="AI574">
+        <v>1667.36682</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B575" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E575">
+        <v>109.1</v>
+      </c>
+      <c r="F575">
+        <v>5962.120000000001</v>
+      </c>
+      <c r="G575">
+        <v>54.64821264894593</v>
+      </c>
+      <c r="H575">
+        <v>134.27</v>
+      </c>
+      <c r="I575">
+        <v>0</v>
+      </c>
+      <c r="J575">
+        <v>0</v>
+      </c>
+      <c r="K575">
+        <v>1.23070577451879</v>
+      </c>
+      <c r="L575">
+        <v>0</v>
+      </c>
+      <c r="M575">
+        <v>4</v>
+      </c>
+      <c r="N575">
+        <v>0</v>
+      </c>
+      <c r="O575">
+        <v>28.8415</v>
+      </c>
+      <c r="P575">
+        <v>82.42312528577961</v>
+      </c>
+      <c r="Q575">
+        <v>34.992</v>
+      </c>
+      <c r="R575">
+        <v>411.71096</v>
+      </c>
+      <c r="S575">
+        <v>3.773702658111824</v>
+      </c>
+      <c r="T575">
+        <v>432.59999</v>
+      </c>
+      <c r="U575">
+        <v>4</v>
+      </c>
+      <c r="V575">
+        <v>6</v>
+      </c>
+      <c r="W575">
+        <v>10</v>
+      </c>
+      <c r="X575">
+        <v>30</v>
+      </c>
+      <c r="Y575">
+        <v>4</v>
+      </c>
+      <c r="Z575">
+        <v>28</v>
+      </c>
+      <c r="AA575">
+        <v>6</v>
+      </c>
+      <c r="AB575">
+        <v>2</v>
+      </c>
+      <c r="AC575">
+        <v>3.57388</v>
+      </c>
+      <c r="AD575">
+        <v>-0.8908199999999999</v>
+      </c>
+      <c r="AE575">
+        <v>0</v>
+      </c>
+      <c r="AF575">
+        <v>469.36893</v>
+      </c>
+      <c r="AG575">
+        <v>0</v>
+      </c>
+      <c r="AH575">
+        <v>3</v>
+      </c>
+      <c r="AI575">
+        <v>1235.13288</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B576" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E576">
+        <v>109.1</v>
+      </c>
+      <c r="F576">
+        <v>5226.14</v>
+      </c>
+      <c r="G576">
+        <v>47.90229147571036</v>
+      </c>
+      <c r="H576">
+        <v>0</v>
+      </c>
+      <c r="I576">
+        <v>0</v>
+      </c>
+      <c r="J576">
+        <v>0</v>
+      </c>
+      <c r="K576">
+        <v>0</v>
+      </c>
+      <c r="L576">
+        <v>0</v>
+      </c>
+      <c r="M576">
+        <v>0</v>
+      </c>
+      <c r="N576">
+        <v>0</v>
+      </c>
+      <c r="O576">
+        <v>20.63789</v>
+      </c>
+      <c r="P576">
+        <v>57.32747222222222</v>
+      </c>
+      <c r="Q576">
+        <v>36</v>
+      </c>
+      <c r="R576">
+        <v>545.7596100000001</v>
+      </c>
+      <c r="S576">
+        <v>5.002379560036665</v>
+      </c>
+      <c r="T576">
+        <v>363.97999</v>
+      </c>
+      <c r="U576">
+        <v>2</v>
+      </c>
+      <c r="V576">
+        <v>9</v>
+      </c>
+      <c r="W576">
+        <v>11</v>
+      </c>
+      <c r="X576">
+        <v>44</v>
+      </c>
+      <c r="Y576">
+        <v>2</v>
+      </c>
+      <c r="Z576">
+        <v>44</v>
+      </c>
+      <c r="AA576">
+        <v>9</v>
+      </c>
+      <c r="AB576">
+        <v>15</v>
+      </c>
+      <c r="AC576">
+        <v>3.23536</v>
+      </c>
+      <c r="AD576">
+        <v>-1.40991</v>
+      </c>
+      <c r="AE576">
+        <v>0</v>
+      </c>
+      <c r="AF576">
+        <v>1174.336</v>
+      </c>
+      <c r="AG576">
+        <v>0</v>
+      </c>
+      <c r="AH576">
+        <v>3</v>
+      </c>
+      <c r="AI576">
+        <v>1637.27883</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B577" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E577">
+        <v>109.1</v>
+      </c>
+      <c r="F577">
+        <v>4985.83</v>
+      </c>
+      <c r="G577">
+        <v>45.69963336388634</v>
+      </c>
+      <c r="H577">
+        <v>56.91</v>
+      </c>
+      <c r="I577">
+        <v>0</v>
+      </c>
+      <c r="J577">
+        <v>0</v>
+      </c>
+      <c r="K577">
+        <v>0.5216315307057746</v>
+      </c>
+      <c r="L577">
+        <v>0</v>
+      </c>
+      <c r="M577">
+        <v>1</v>
+      </c>
+      <c r="N577">
+        <v>0</v>
+      </c>
+      <c r="O577">
+        <v>27.35971</v>
+      </c>
+      <c r="P577">
+        <v>80.50762123352165</v>
+      </c>
+      <c r="Q577">
+        <v>33.984</v>
+      </c>
+      <c r="R577">
+        <v>537.35465</v>
+      </c>
+      <c r="S577">
+        <v>4.92534051329056</v>
+      </c>
+      <c r="T577">
+        <v>316.11</v>
+      </c>
+      <c r="U577">
+        <v>4</v>
+      </c>
+      <c r="V577">
+        <v>7</v>
+      </c>
+      <c r="W577">
+        <v>11</v>
+      </c>
+      <c r="X577">
+        <v>22</v>
+      </c>
+      <c r="Y577">
+        <v>4</v>
+      </c>
+      <c r="Z577">
+        <v>27</v>
+      </c>
+      <c r="AA577">
+        <v>7</v>
+      </c>
+      <c r="AB577">
+        <v>12</v>
+      </c>
+      <c r="AC577">
+        <v>3.53005</v>
+      </c>
+      <c r="AD577">
+        <v>-1.47071</v>
+      </c>
+      <c r="AE577">
+        <v>0</v>
+      </c>
+      <c r="AF577">
+        <v>445.8632</v>
+      </c>
+      <c r="AG577">
+        <v>0</v>
+      </c>
+      <c r="AH577">
+        <v>3</v>
+      </c>
+      <c r="AI577">
+        <v>1612.06395</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B578" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E578">
+        <v>109.1</v>
+      </c>
+      <c r="F578">
+        <v>5693.67</v>
+      </c>
+      <c r="G578">
+        <v>52.18762603116407</v>
+      </c>
+      <c r="H578">
+        <v>71.52</v>
+      </c>
+      <c r="I578">
+        <v>0</v>
+      </c>
+      <c r="J578">
+        <v>0</v>
+      </c>
+      <c r="K578">
+        <v>0.6555453712190651</v>
+      </c>
+      <c r="L578">
+        <v>0</v>
+      </c>
+      <c r="M578">
+        <v>3</v>
+      </c>
+      <c r="N578">
+        <v>0</v>
+      </c>
+      <c r="O578">
+        <v>27.00535</v>
+      </c>
+      <c r="P578">
+        <v>84.38117110361205</v>
+      </c>
+      <c r="Q578">
+        <v>32.004</v>
+      </c>
+      <c r="R578">
+        <v>487.31969</v>
+      </c>
+      <c r="S578">
+        <v>4.46672493125573</v>
+      </c>
+      <c r="T578">
+        <v>402.99</v>
+      </c>
+      <c r="U578">
+        <v>6</v>
+      </c>
+      <c r="V578">
+        <v>5</v>
+      </c>
+      <c r="W578">
+        <v>11</v>
+      </c>
+      <c r="X578">
+        <v>33</v>
+      </c>
+      <c r="Y578">
+        <v>6</v>
+      </c>
+      <c r="Z578">
+        <v>32</v>
+      </c>
+      <c r="AA578">
+        <v>5</v>
+      </c>
+      <c r="AB578">
+        <v>11</v>
+      </c>
+      <c r="AC578">
+        <v>3.48666</v>
+      </c>
+      <c r="AD578">
+        <v>-2.27829</v>
+      </c>
+      <c r="AE578">
+        <v>0</v>
+      </c>
+      <c r="AF578">
+        <v>442.7703</v>
+      </c>
+      <c r="AG578">
+        <v>0</v>
+      </c>
+      <c r="AH578">
+        <v>3</v>
+      </c>
+      <c r="AI578">
+        <v>1461.95907</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B579" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E579">
+        <v>109.1</v>
+      </c>
+      <c r="F579">
+        <v>6763.51</v>
+      </c>
+      <c r="G579">
+        <v>61.99367552703942</v>
+      </c>
+      <c r="H579">
+        <v>82.62</v>
+      </c>
+      <c r="I579">
+        <v>0</v>
+      </c>
+      <c r="J579">
+        <v>0</v>
+      </c>
+      <c r="K579">
+        <v>0.7572868927589368</v>
+      </c>
+      <c r="L579">
+        <v>0</v>
+      </c>
+      <c r="M579">
+        <v>0</v>
+      </c>
+      <c r="N579">
+        <v>0</v>
+      </c>
+      <c r="O579">
+        <v>24.38704</v>
+      </c>
+      <c r="P579">
+        <v>67.74177777777778</v>
+      </c>
+      <c r="Q579">
+        <v>36</v>
+      </c>
+      <c r="R579">
+        <v>729.4684600000001</v>
+      </c>
+      <c r="S579">
+        <v>6.68623703024748</v>
+      </c>
+      <c r="T579">
+        <v>456.76</v>
+      </c>
+      <c r="U579">
+        <v>4</v>
+      </c>
+      <c r="V579">
+        <v>12</v>
+      </c>
+      <c r="W579">
+        <v>16</v>
+      </c>
+      <c r="X579">
+        <v>44</v>
+      </c>
+      <c r="Y579">
+        <v>4</v>
+      </c>
+      <c r="Z579">
+        <v>47</v>
+      </c>
+      <c r="AA579">
+        <v>12</v>
+      </c>
+      <c r="AB579">
+        <v>11</v>
+      </c>
+      <c r="AC579">
+        <v>3.399</v>
+      </c>
+      <c r="AD579">
+        <v>-1.74251</v>
+      </c>
+      <c r="AE579">
+        <v>0</v>
+      </c>
+      <c r="AF579">
+        <v>1516.986</v>
+      </c>
+      <c r="AG579">
+        <v>0</v>
+      </c>
+      <c r="AH579">
+        <v>3</v>
+      </c>
+      <c r="AI579">
+        <v>2188.40538</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B580" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Trabajo Compensatorio Seleccionados | Sesión 36</t>
+        </is>
+      </c>
+      <c r="E580">
+        <v>184.8118333333333</v>
+      </c>
+      <c r="F580">
+        <v>10253.04</v>
+      </c>
+      <c r="G580">
+        <v>55.47826573154137</v>
+      </c>
+      <c r="H580">
+        <v>292.63</v>
+      </c>
+      <c r="I580">
+        <v>0</v>
+      </c>
+      <c r="J580">
+        <v>0</v>
+      </c>
+      <c r="K580">
+        <v>1.583394281210348</v>
+      </c>
+      <c r="L580">
+        <v>0</v>
+      </c>
+      <c r="M580">
+        <v>4</v>
+      </c>
+      <c r="N580">
+        <v>0</v>
+      </c>
+      <c r="O580">
+        <v>26.2178</v>
+      </c>
+      <c r="P580">
+        <v>74.92512574302698</v>
+      </c>
+      <c r="Q580">
+        <v>34.992</v>
+      </c>
+      <c r="R580">
+        <v>1083.70235</v>
+      </c>
+      <c r="S580">
+        <v>5.863814726870845</v>
+      </c>
+      <c r="T580">
+        <v>1297.54</v>
+      </c>
+      <c r="U580">
+        <v>68</v>
+      </c>
+      <c r="V580">
+        <v>65</v>
+      </c>
+      <c r="W580">
+        <v>133</v>
+      </c>
+      <c r="X580">
+        <v>149</v>
+      </c>
+      <c r="Y580">
+        <v>68</v>
+      </c>
+      <c r="Z580">
+        <v>148</v>
+      </c>
+      <c r="AA580">
+        <v>65</v>
+      </c>
+      <c r="AB580">
+        <v>98</v>
+      </c>
+      <c r="AC580">
+        <v>4.47299</v>
+      </c>
+      <c r="AD580">
+        <v>-1.61063</v>
+      </c>
+      <c r="AE580">
+        <v>0</v>
+      </c>
+      <c r="AF580">
+        <v>980.4992</v>
+      </c>
+      <c r="AG580">
+        <v>0</v>
+      </c>
+      <c r="AH580">
+        <v>3</v>
+      </c>
+      <c r="AI580">
+        <v>3251.10705</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B581" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Sesión 36</t>
+        </is>
+      </c>
+      <c r="E581">
+        <v>76.84999999999999</v>
+      </c>
+      <c r="F581">
+        <v>5308.15</v>
+      </c>
+      <c r="G581">
+        <v>69.07156798959011</v>
+      </c>
+      <c r="H581">
+        <v>0</v>
+      </c>
+      <c r="I581">
+        <v>0</v>
+      </c>
+      <c r="J581">
+        <v>0</v>
+      </c>
+      <c r="K581">
+        <v>0</v>
+      </c>
+      <c r="L581">
+        <v>0</v>
+      </c>
+      <c r="M581">
+        <v>0</v>
+      </c>
+      <c r="N581">
+        <v>0</v>
+      </c>
+      <c r="O581">
+        <v>20.61211</v>
+      </c>
+      <c r="P581">
+        <v>60.65239524482109</v>
+      </c>
+      <c r="Q581">
+        <v>33.984</v>
+      </c>
+      <c r="R581">
+        <v>481.63669</v>
+      </c>
+      <c r="S581">
+        <v>6.267230839297333</v>
+      </c>
+      <c r="T581">
+        <v>383.76001</v>
+      </c>
+      <c r="U581">
+        <v>0</v>
+      </c>
+      <c r="V581">
+        <v>0</v>
+      </c>
+      <c r="W581">
+        <v>0</v>
+      </c>
+      <c r="X581">
+        <v>13</v>
+      </c>
+      <c r="Y581">
+        <v>0</v>
+      </c>
+      <c r="Z581">
+        <v>0</v>
+      </c>
+      <c r="AA581">
+        <v>0</v>
+      </c>
+      <c r="AB581">
+        <v>2</v>
+      </c>
+      <c r="AC581">
+        <v>2.55821</v>
+      </c>
+      <c r="AD581">
+        <v>-1.20019</v>
+      </c>
+      <c r="AE581">
+        <v>0</v>
+      </c>
+      <c r="AF581">
+        <v>394.0748</v>
+      </c>
+      <c r="AG581">
+        <v>0</v>
+      </c>
+      <c r="AH581">
+        <v>3</v>
+      </c>
+      <c r="AI581">
+        <v>1444.91007</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-18
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI581"/>
+  <dimension ref="A1:AI603"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -60680,10 +60680,10 @@
         <v>43.44283333333333</v>
       </c>
       <c r="F535">
-        <v>3766.68</v>
+        <v>3766.72</v>
       </c>
       <c r="G535">
-        <v>86.70428954526447</v>
+        <v>86.70521029552249</v>
       </c>
       <c r="H535">
         <v>114.29</v>
@@ -60716,10 +60716,10 @@
         <v>36</v>
       </c>
       <c r="R535">
-        <v>332.39163</v>
+        <v>332.39314</v>
       </c>
       <c r="S535">
-        <v>7.651241977004263</v>
+        <v>7.651276735326504</v>
       </c>
       <c r="T535">
         <v>544.6099899999999</v>
@@ -60758,7 +60758,7 @@
         <v>0</v>
       </c>
       <c r="AF535">
-        <v>889.1840000000001</v>
+        <v>889.1899999999999</v>
       </c>
       <c r="AG535">
         <v>0</v>
@@ -60767,7 +60767,7 @@
         <v>3</v>
       </c>
       <c r="AI535">
-        <v>997.1748899999999</v>
+        <v>997.1794200000001</v>
       </c>
     </row>
     <row r="536">
@@ -60793,10 +60793,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F536">
-        <v>7144.89</v>
+        <v>7144.92</v>
       </c>
       <c r="G536">
-        <v>103.6635609839847</v>
+        <v>103.663996247065</v>
       </c>
       <c r="H536">
         <v>171.42</v>
@@ -60829,10 +60829,10 @@
         <v>32.364</v>
       </c>
       <c r="R536">
-        <v>708.70748</v>
+        <v>708.70934</v>
       </c>
       <c r="S536">
-        <v>10.2824733582723</v>
+        <v>10.28250034458327</v>
       </c>
       <c r="T536">
         <v>900.32002</v>
@@ -60871,7 +60871,7 @@
         <v>0</v>
       </c>
       <c r="AF536">
-        <v>565.8330999999999</v>
+        <v>565.8352</v>
       </c>
       <c r="AG536">
         <v>0</v>
@@ -60880,7 +60880,7 @@
         <v>3</v>
       </c>
       <c r="AI536">
-        <v>2126.12244</v>
+        <v>2126.12802</v>
       </c>
     </row>
     <row r="537">
@@ -60942,10 +60942,10 @@
         <v>36</v>
       </c>
       <c r="R537">
-        <v>611.89944</v>
+        <v>611.90031</v>
       </c>
       <c r="S537">
-        <v>8.208383764761646</v>
+        <v>8.208395435460144</v>
       </c>
       <c r="T537">
         <v>1193.35997</v>
@@ -60993,7 +60993,7 @@
         <v>3</v>
       </c>
       <c r="AI537">
-        <v>1835.69832</v>
+        <v>1835.70093</v>
       </c>
     </row>
     <row r="538">
@@ -61132,10 +61132,10 @@
         <v>74.54566666666666</v>
       </c>
       <c r="F539">
-        <v>8142.46</v>
+        <v>8142.59</v>
       </c>
       <c r="G539">
-        <v>109.2278111403748</v>
+        <v>109.2295550378515</v>
       </c>
       <c r="H539">
         <v>358.14</v>
@@ -61168,10 +61168,10 @@
         <v>36</v>
       </c>
       <c r="R539">
-        <v>877.53862</v>
+        <v>877.54308</v>
       </c>
       <c r="S539">
-        <v>11.7718260395194</v>
+        <v>11.77188586861745</v>
       </c>
       <c r="T539">
         <v>1385.48002</v>
@@ -61210,7 +61210,7 @@
         <v>0</v>
       </c>
       <c r="AF539">
-        <v>1929.188</v>
+        <v>1929.212</v>
       </c>
       <c r="AG539">
         <v>0</v>
@@ -61219,7 +61219,7 @@
         <v>3</v>
       </c>
       <c r="AI539">
-        <v>2632.61586</v>
+        <v>2632.62924</v>
       </c>
     </row>
     <row r="540">
@@ -61245,10 +61245,10 @@
         <v>124.945</v>
       </c>
       <c r="F540">
-        <v>9130.73</v>
+        <v>9130.879999999999</v>
       </c>
       <c r="G540">
-        <v>73.0779943174997</v>
+        <v>73.07919484573212</v>
       </c>
       <c r="H540">
         <v>448.55</v>
@@ -61281,10 +61281,10 @@
         <v>35.604</v>
       </c>
       <c r="R540">
-        <v>796.78566</v>
+        <v>796.81598</v>
       </c>
       <c r="S540">
-        <v>6.377091200128056</v>
+        <v>6.377333866901437</v>
       </c>
       <c r="T540">
         <v>1495.4</v>
@@ -61323,7 +61323,7 @@
         <v>0</v>
       </c>
       <c r="AF540">
-        <v>789.69963</v>
+        <v>789.71028</v>
       </c>
       <c r="AG540">
         <v>0</v>
@@ -61332,7 +61332,7 @@
         <v>3</v>
       </c>
       <c r="AI540">
-        <v>2390.35698</v>
+        <v>2390.44794</v>
       </c>
     </row>
     <row r="541">
@@ -61358,10 +61358,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F541">
-        <v>6053.4</v>
+        <v>6053.57</v>
       </c>
       <c r="G541">
-        <v>87.82738433488173</v>
+        <v>87.82985082566988</v>
       </c>
       <c r="H541">
         <v>308.44</v>
@@ -61394,10 +61394,10 @@
         <v>33.984</v>
       </c>
       <c r="R541">
-        <v>670.05727</v>
+        <v>670.06494</v>
       </c>
       <c r="S541">
-        <v>9.721706376362313</v>
+        <v>9.721817658623166</v>
       </c>
       <c r="T541">
         <v>847.79002</v>
@@ -61436,7 +61436,7 @@
         <v>0</v>
       </c>
       <c r="AF541">
-        <v>561.2528</v>
+        <v>561.26</v>
       </c>
       <c r="AG541">
         <v>0</v>
@@ -61445,7 +61445,7 @@
         <v>3</v>
       </c>
       <c r="AI541">
-        <v>2010.17181</v>
+        <v>2010.19482</v>
       </c>
     </row>
     <row r="542">
@@ -61507,10 +61507,10 @@
         <v>35.568</v>
       </c>
       <c r="R542">
-        <v>591.8106300000001</v>
+        <v>591.8134600000001</v>
       </c>
       <c r="S542">
-        <v>8.586443924815558</v>
+        <v>8.586484984632795</v>
       </c>
       <c r="T542">
         <v>974.05</v>
@@ -61558,7 +61558,7 @@
         <v>3</v>
       </c>
       <c r="AI542">
-        <v>1775.43189</v>
+        <v>1775.44038</v>
       </c>
     </row>
     <row r="543">
@@ -61584,10 +61584,10 @@
         <v>74.54566666666666</v>
       </c>
       <c r="F543">
-        <v>7894.56</v>
+        <v>7894.66</v>
       </c>
       <c r="G543">
-        <v>105.90233279824</v>
+        <v>105.9036742578375</v>
       </c>
       <c r="H543">
         <v>432.36</v>
@@ -61620,10 +61620,10 @@
         <v>36</v>
       </c>
       <c r="R543">
-        <v>759.4303</v>
+        <v>759.43364</v>
       </c>
       <c r="S543">
-        <v>10.18745064546564</v>
+        <v>10.1874954502162</v>
       </c>
       <c r="T543">
         <v>1261.26001</v>
@@ -61662,7 +61662,7 @@
         <v>0</v>
       </c>
       <c r="AF543">
-        <v>1817.528</v>
+        <v>1817.548</v>
       </c>
       <c r="AG543">
         <v>0</v>
@@ -61671,7 +61671,7 @@
         <v>3</v>
       </c>
       <c r="AI543">
-        <v>2278.2909</v>
+        <v>2278.30092</v>
       </c>
     </row>
     <row r="544">
@@ -61733,10 +61733,10 @@
         <v>36</v>
       </c>
       <c r="R544">
-        <v>311.23013</v>
+        <v>311.2308</v>
       </c>
       <c r="S544">
-        <v>10.0064880477127</v>
+        <v>10.00650958915854</v>
       </c>
       <c r="T544">
         <v>608.38</v>
@@ -61784,7 +61784,7 @@
         <v>3</v>
       </c>
       <c r="AI544">
-        <v>933.69039</v>
+        <v>933.6923999999999</v>
       </c>
     </row>
     <row r="545">
@@ -61810,10 +61810,10 @@
         <v>80.51133333333334</v>
       </c>
       <c r="F545">
-        <v>6886.46</v>
+        <v>6886.61</v>
       </c>
       <c r="G545">
-        <v>85.53404489637069</v>
+        <v>85.53590798810933</v>
       </c>
       <c r="H545">
         <v>311.1</v>
@@ -61846,10 +61846,10 @@
         <v>32.004</v>
       </c>
       <c r="R545">
-        <v>743.20861</v>
+        <v>743.2203500000001</v>
       </c>
       <c r="S545">
-        <v>9.23110547583363</v>
+        <v>9.231251293813708</v>
       </c>
       <c r="T545">
         <v>1011.07002</v>
@@ -61888,7 +61888,7 @@
         <v>0</v>
       </c>
       <c r="AF545">
-        <v>484.1130000000001</v>
+        <v>484.1166</v>
       </c>
       <c r="AG545">
         <v>0</v>
@@ -61897,7 +61897,7 @@
         <v>3</v>
       </c>
       <c r="AI545">
-        <v>2229.62583</v>
+        <v>2229.66105</v>
       </c>
     </row>
     <row r="546">
@@ -61923,10 +61923,10 @@
         <v>68.645</v>
       </c>
       <c r="F546">
-        <v>6406.33</v>
+        <v>6406.49</v>
       </c>
       <c r="G546">
-        <v>93.32551533250783</v>
+        <v>93.32784616505208</v>
       </c>
       <c r="H546">
         <v>411.21</v>
@@ -61959,10 +61959,10 @@
         <v>33.84</v>
       </c>
       <c r="R546">
-        <v>562.91481</v>
+        <v>562.94258</v>
       </c>
       <c r="S546">
-        <v>8.200375992424794</v>
+        <v>8.200780537548257</v>
       </c>
       <c r="T546">
         <v>1067.86999</v>
@@ -62001,7 +62001,7 @@
         <v>0</v>
       </c>
       <c r="AF546">
-        <v>521.8927</v>
+        <v>521.9032</v>
       </c>
       <c r="AG546">
         <v>0</v>
@@ -62010,7 +62010,7 @@
         <v>3</v>
       </c>
       <c r="AI546">
-        <v>1688.74443</v>
+        <v>1688.82774</v>
       </c>
     </row>
     <row r="547">
@@ -62036,10 +62036,10 @@
         <v>74.54566666666666</v>
       </c>
       <c r="F547">
-        <v>7265.03</v>
+        <v>7265.18</v>
       </c>
       <c r="G547">
-        <v>97.45744219427019</v>
+        <v>97.4594543836664</v>
       </c>
       <c r="H547">
         <v>210.41</v>
@@ -62072,10 +62072,10 @@
         <v>36</v>
       </c>
       <c r="R547">
-        <v>661.05039</v>
+        <v>661.0550000000001</v>
       </c>
       <c r="S547">
-        <v>8.867723900785649</v>
+        <v>8.867785742073092</v>
       </c>
       <c r="T547">
         <v>851.97</v>
@@ -62114,7 +62114,7 @@
         <v>0</v>
       </c>
       <c r="AF547">
-        <v>1641.32</v>
+        <v>1641.348</v>
       </c>
       <c r="AG547">
         <v>0</v>
@@ -62123,7 +62123,7 @@
         <v>3</v>
       </c>
       <c r="AI547">
-        <v>1983.15117</v>
+        <v>1983.165</v>
       </c>
     </row>
     <row r="548">
@@ -62185,10 +62185,10 @@
         <v>33.696</v>
       </c>
       <c r="R548">
-        <v>545.56281</v>
+        <v>545.56549</v>
       </c>
       <c r="S548">
-        <v>7.915444971865078</v>
+        <v>7.915483855366914</v>
       </c>
       <c r="T548">
         <v>1019.35002</v>
@@ -62227,7 +62227,7 @@
         <v>0</v>
       </c>
       <c r="AF548">
-        <v>563.8112</v>
+        <v>563.8136</v>
       </c>
       <c r="AG548">
         <v>0</v>
@@ -62236,7 +62236,7 @@
         <v>3</v>
       </c>
       <c r="AI548">
-        <v>1636.68843</v>
+        <v>1636.69647</v>
       </c>
     </row>
     <row r="549">
@@ -62298,10 +62298,10 @@
         <v>34.992</v>
       </c>
       <c r="R549">
-        <v>524.68007</v>
+        <v>524.68205</v>
       </c>
       <c r="S549">
-        <v>7.612462113976056</v>
+        <v>7.612490841339353</v>
       </c>
       <c r="T549">
         <v>837.43998</v>
@@ -62349,7 +62349,7 @@
         <v>3</v>
       </c>
       <c r="AI549">
-        <v>1574.04021</v>
+        <v>1574.04615</v>
       </c>
     </row>
     <row r="550">
@@ -62375,10 +62375,10 @@
         <v>124.945</v>
       </c>
       <c r="F550">
-        <v>9798.82</v>
+        <v>9799.110000000001</v>
       </c>
       <c r="G550">
-        <v>78.42506702949298</v>
+        <v>78.42738805074234</v>
       </c>
       <c r="H550">
         <v>283.91</v>
@@ -62411,10 +62411,10 @@
         <v>33.012</v>
       </c>
       <c r="R550">
-        <v>998.68046</v>
+        <v>998.71034</v>
       </c>
       <c r="S550">
-        <v>7.992960582656369</v>
+        <v>7.993199727880268</v>
       </c>
       <c r="T550">
         <v>1570.35004</v>
@@ -62453,7 +62453,7 @@
         <v>0</v>
       </c>
       <c r="AF550">
-        <v>918.00306</v>
+        <v>918.04674</v>
       </c>
       <c r="AG550">
         <v>0</v>
@@ -62462,7 +62462,7 @@
         <v>3</v>
       </c>
       <c r="AI550">
-        <v>2996.04138</v>
+        <v>2996.13102</v>
       </c>
     </row>
     <row r="551">
@@ -62488,10 +62488,10 @@
         <v>68.645</v>
       </c>
       <c r="F551">
-        <v>6093.87</v>
+        <v>6093.98</v>
       </c>
       <c r="G551">
-        <v>88.77369072765678</v>
+        <v>88.77529317503097</v>
       </c>
       <c r="H551">
         <v>295.41</v>
@@ -62524,10 +62524,10 @@
         <v>34.92</v>
       </c>
       <c r="R551">
-        <v>495.67495</v>
+        <v>495.68954</v>
       </c>
       <c r="S551">
-        <v>7.22084565518246</v>
+        <v>7.221058197975089</v>
       </c>
       <c r="T551">
         <v>931.97999</v>
@@ -62566,7 +62566,7 @@
         <v>0</v>
       </c>
       <c r="AF551">
-        <v>565.8896</v>
+        <v>565.8952</v>
       </c>
       <c r="AG551">
         <v>0</v>
@@ -62575,7 +62575,7 @@
         <v>3</v>
       </c>
       <c r="AI551">
-        <v>1487.02485</v>
+        <v>1487.06862</v>
       </c>
     </row>
     <row r="552">
@@ -62601,10 +62601,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F552">
-        <v>6803.6</v>
+        <v>6803.690000000001</v>
       </c>
       <c r="G552">
-        <v>98.7118630952525</v>
+        <v>98.71316888449327</v>
       </c>
       <c r="H552">
         <v>353.97</v>
@@ -62637,10 +62637,10 @@
         <v>34.992</v>
       </c>
       <c r="R552">
-        <v>548.18448</v>
+        <v>548.18843</v>
       </c>
       <c r="S552">
-        <v>7.953482177185927</v>
+        <v>7.953539486824829</v>
       </c>
       <c r="T552">
         <v>1217.81001</v>
@@ -62679,7 +62679,7 @@
         <v>0</v>
       </c>
       <c r="AF552">
-        <v>575.31087</v>
+        <v>575.31726</v>
       </c>
       <c r="AG552">
         <v>0</v>
@@ -62688,7 +62688,7 @@
         <v>3</v>
       </c>
       <c r="AI552">
-        <v>1644.55344</v>
+        <v>1644.56529</v>
       </c>
     </row>
     <row r="553">
@@ -62714,10 +62714,10 @@
         <v>74.54566666666666</v>
       </c>
       <c r="F553">
-        <v>7582.14</v>
+        <v>7582.16</v>
       </c>
       <c r="G553">
-        <v>101.7113447238158</v>
+        <v>101.7116130157353</v>
       </c>
       <c r="H553">
         <v>189.73</v>
@@ -62750,10 +62750,10 @@
         <v>36</v>
       </c>
       <c r="R553">
-        <v>806.30009</v>
+        <v>806.3020200000001</v>
       </c>
       <c r="S553">
-        <v>10.81618994173594</v>
+        <v>10.81621583190617</v>
       </c>
       <c r="T553">
         <v>1040.26998</v>
@@ -62792,7 +62792,7 @@
         <v>0</v>
       </c>
       <c r="AF553">
-        <v>1748.17</v>
+        <v>1748.178</v>
       </c>
       <c r="AG553">
         <v>0</v>
@@ -62801,7 +62801,7 @@
         <v>3</v>
       </c>
       <c r="AI553">
-        <v>2418.90027</v>
+        <v>2418.90606</v>
       </c>
     </row>
     <row r="554">
@@ -62827,10 +62827,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F554">
-        <v>6212.759999999999</v>
+        <v>6212.81</v>
       </c>
       <c r="G554">
-        <v>90.13950181722335</v>
+        <v>90.14022725569046</v>
       </c>
       <c r="H554">
         <v>207.21</v>
@@ -62863,10 +62863,10 @@
         <v>33.984</v>
       </c>
       <c r="R554">
-        <v>575.81569</v>
+        <v>575.81708</v>
       </c>
       <c r="S554">
-        <v>8.354377029716378</v>
+        <v>8.354397196905763</v>
       </c>
       <c r="T554">
         <v>793</v>
@@ -62905,7 +62905,7 @@
         <v>0</v>
       </c>
       <c r="AF554">
-        <v>568.2576</v>
+        <v>568.2608</v>
       </c>
       <c r="AG554">
         <v>0</v>
@@ -62914,7 +62914,7 @@
         <v>3</v>
       </c>
       <c r="AI554">
-        <v>1727.44707</v>
+        <v>1727.45124</v>
       </c>
     </row>
     <row r="555">
@@ -62940,10 +62940,10 @@
         <v>68.645</v>
       </c>
       <c r="F555">
-        <v>6264.820000000001</v>
+        <v>6264.83</v>
       </c>
       <c r="G555">
-        <v>91.26403962415327</v>
+        <v>91.26418530118727</v>
       </c>
       <c r="H555">
         <v>389.56</v>
@@ -62976,10 +62976,10 @@
         <v>34.992</v>
       </c>
       <c r="R555">
-        <v>517.38684</v>
+        <v>517.38888</v>
       </c>
       <c r="S555">
-        <v>7.53713802898973</v>
+        <v>7.537167747104669</v>
       </c>
       <c r="T555">
         <v>1109.4</v>
@@ -63018,7 +63018,7 @@
         <v>0</v>
       </c>
       <c r="AF555">
-        <v>586.4672</v>
+        <v>586.468</v>
       </c>
       <c r="AG555">
         <v>0</v>
@@ -63027,7 +63027,7 @@
         <v>3</v>
       </c>
       <c r="AI555">
-        <v>1552.16052</v>
+        <v>1552.16664</v>
       </c>
     </row>
     <row r="556">
@@ -63053,10 +63053,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F556">
-        <v>6230.11</v>
+        <v>6230.22</v>
       </c>
       <c r="G556">
-        <v>90.39122896530711</v>
+        <v>90.39282492993473</v>
       </c>
       <c r="H556">
         <v>181.98</v>
@@ -63089,10 +63089,10 @@
         <v>33.012</v>
       </c>
       <c r="R556">
-        <v>586.84867</v>
+        <v>586.8526899999999</v>
       </c>
       <c r="S556">
-        <v>8.514451991691312</v>
+        <v>8.514510316944065</v>
       </c>
       <c r="T556">
         <v>891.5000200000001</v>
@@ -63131,7 +63131,7 @@
         <v>0</v>
       </c>
       <c r="AF556">
-        <v>540.8579999999999</v>
+        <v>540.867</v>
       </c>
       <c r="AG556">
         <v>0</v>
@@ -63140,7 +63140,7 @@
         <v>3</v>
       </c>
       <c r="AI556">
-        <v>1760.54601</v>
+        <v>1760.55807</v>
       </c>
     </row>
     <row r="557">
@@ -63166,10 +63166,10 @@
         <v>68.92383333333333</v>
       </c>
       <c r="F557">
-        <v>6592.84</v>
+        <v>6592.91</v>
       </c>
       <c r="G557">
-        <v>95.65399486873191</v>
+        <v>95.65501048258585</v>
       </c>
       <c r="H557">
         <v>111.45</v>
@@ -63202,10 +63202,10 @@
         <v>32.004</v>
       </c>
       <c r="R557">
-        <v>593.68001</v>
+        <v>593.68376</v>
       </c>
       <c r="S557">
-        <v>8.613566328048112</v>
+        <v>8.613620735933143</v>
       </c>
       <c r="T557">
         <v>822.30999</v>
@@ -63244,7 +63244,7 @@
         <v>0</v>
       </c>
       <c r="AF557">
-        <v>529.9609</v>
+        <v>529.9686</v>
       </c>
       <c r="AG557">
         <v>0</v>
@@ -63253,7 +63253,7 @@
         <v>3</v>
       </c>
       <c r="AI557">
-        <v>1781.04003</v>
+        <v>1781.05128</v>
       </c>
     </row>
     <row r="558">
@@ -63279,10 +63279,10 @@
         <v>74.54566666666666</v>
       </c>
       <c r="F558">
-        <v>9115.679999999998</v>
+        <v>9115.690000000001</v>
       </c>
       <c r="G558">
-        <v>122.2831642348985</v>
+        <v>122.2832983808583</v>
       </c>
       <c r="H558">
         <v>237.14</v>
@@ -63315,10 +63315,10 @@
         <v>36</v>
       </c>
       <c r="R558">
-        <v>990.1090300000001</v>
+        <v>990.11397</v>
       </c>
       <c r="S558">
-        <v>13.28191260837876</v>
+        <v>13.28197887648287</v>
       </c>
       <c r="T558">
         <v>1303.98999</v>
@@ -63357,7 +63357,7 @@
         <v>0</v>
       </c>
       <c r="AF558">
-        <v>2104.014</v>
+        <v>2104.022</v>
       </c>
       <c r="AG558">
         <v>0</v>
@@ -63366,7 +63366,7 @@
         <v>3</v>
       </c>
       <c r="AI558">
-        <v>2970.32709</v>
+        <v>2970.34191</v>
       </c>
     </row>
     <row r="559">
@@ -63392,10 +63392,10 @@
         <v>68.645</v>
       </c>
       <c r="F559">
-        <v>7865.73</v>
+        <v>7865.87</v>
       </c>
       <c r="G559">
-        <v>114.5856216767427</v>
+        <v>114.5876611552189</v>
       </c>
       <c r="H559">
         <v>295.18</v>
@@ -63428,10 +63428,10 @@
         <v>36</v>
       </c>
       <c r="R559">
-        <v>819.7710400000001</v>
+        <v>819.80733</v>
       </c>
       <c r="S559">
-        <v>11.94218136790735</v>
+        <v>11.94271002986379</v>
       </c>
       <c r="T559">
         <v>1243.38</v>
@@ -63470,7 +63470,7 @@
         <v>0</v>
       </c>
       <c r="AF559">
-        <v>1800.72</v>
+        <v>1800.74</v>
       </c>
       <c r="AG559">
         <v>0</v>
@@ -63479,7 +63479,7 @@
         <v>3</v>
       </c>
       <c r="AI559">
-        <v>2459.31312</v>
+        <v>2459.42199</v>
       </c>
     </row>
     <row r="560">
@@ -65966,6 +65966,2477 @@
       </c>
       <c r="AI581">
         <v>1444.91007</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B582" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E582">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F582">
+        <v>3948.34</v>
+      </c>
+      <c r="G582">
+        <v>38.0868810289389</v>
+      </c>
+      <c r="H582">
+        <v>50.62</v>
+      </c>
+      <c r="I582">
+        <v>0</v>
+      </c>
+      <c r="J582">
+        <v>0</v>
+      </c>
+      <c r="K582">
+        <v>0.4882958199356913</v>
+      </c>
+      <c r="L582">
+        <v>0</v>
+      </c>
+      <c r="M582">
+        <v>1</v>
+      </c>
+      <c r="N582">
+        <v>0</v>
+      </c>
+      <c r="O582">
+        <v>25.90446</v>
+      </c>
+      <c r="P582">
+        <v>80.040971449759</v>
+      </c>
+      <c r="Q582">
+        <v>32.364</v>
+      </c>
+      <c r="R582">
+        <v>336.53219</v>
+      </c>
+      <c r="S582">
+        <v>3.246291221864952</v>
+      </c>
+      <c r="T582">
+        <v>367.23001</v>
+      </c>
+      <c r="U582">
+        <v>7</v>
+      </c>
+      <c r="V582">
+        <v>3</v>
+      </c>
+      <c r="W582">
+        <v>10</v>
+      </c>
+      <c r="X582">
+        <v>40</v>
+      </c>
+      <c r="Y582">
+        <v>7</v>
+      </c>
+      <c r="Z582">
+        <v>20</v>
+      </c>
+      <c r="AA582">
+        <v>3</v>
+      </c>
+      <c r="AB582">
+        <v>15</v>
+      </c>
+      <c r="AC582">
+        <v>4.34631</v>
+      </c>
+      <c r="AD582">
+        <v>-1.73523</v>
+      </c>
+      <c r="AE582">
+        <v>0</v>
+      </c>
+      <c r="AF582">
+        <v>307.3168</v>
+      </c>
+      <c r="AG582">
+        <v>0</v>
+      </c>
+      <c r="AH582">
+        <v>3</v>
+      </c>
+      <c r="AI582">
+        <v>1009.59657</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B583" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E583">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F583">
+        <v>3423.79</v>
+      </c>
+      <c r="G583">
+        <v>33.02691318327974</v>
+      </c>
+      <c r="H583">
+        <v>4.83</v>
+      </c>
+      <c r="I583">
+        <v>0</v>
+      </c>
+      <c r="J583">
+        <v>0</v>
+      </c>
+      <c r="K583">
+        <v>0.04659163987138264</v>
+      </c>
+      <c r="L583">
+        <v>0</v>
+      </c>
+      <c r="M583">
+        <v>0</v>
+      </c>
+      <c r="N583">
+        <v>0</v>
+      </c>
+      <c r="O583">
+        <v>22.12002</v>
+      </c>
+      <c r="P583">
+        <v>61.44450000000001</v>
+      </c>
+      <c r="Q583">
+        <v>36</v>
+      </c>
+      <c r="R583">
+        <v>304.43663</v>
+      </c>
+      <c r="S583">
+        <v>2.936687749196141</v>
+      </c>
+      <c r="T583">
+        <v>304.29</v>
+      </c>
+      <c r="U583">
+        <v>18</v>
+      </c>
+      <c r="V583">
+        <v>13</v>
+      </c>
+      <c r="W583">
+        <v>31</v>
+      </c>
+      <c r="X583">
+        <v>47</v>
+      </c>
+      <c r="Y583">
+        <v>18</v>
+      </c>
+      <c r="Z583">
+        <v>50</v>
+      </c>
+      <c r="AA583">
+        <v>13</v>
+      </c>
+      <c r="AB583">
+        <v>24</v>
+      </c>
+      <c r="AC583">
+        <v>4.65709</v>
+      </c>
+      <c r="AD583">
+        <v>-4.03384</v>
+      </c>
+      <c r="AE583">
+        <v>0</v>
+      </c>
+      <c r="AF583">
+        <v>795.002</v>
+      </c>
+      <c r="AG583">
+        <v>0</v>
+      </c>
+      <c r="AH583">
+        <v>3</v>
+      </c>
+      <c r="AI583">
+        <v>913.30989</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B584" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E584">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F584">
+        <v>3322.55</v>
+      </c>
+      <c r="G584">
+        <v>32.05032154340836</v>
+      </c>
+      <c r="H584">
+        <v>22.43</v>
+      </c>
+      <c r="I584">
+        <v>0</v>
+      </c>
+      <c r="J584">
+        <v>0</v>
+      </c>
+      <c r="K584">
+        <v>0.2163665594855306</v>
+      </c>
+      <c r="L584">
+        <v>0</v>
+      </c>
+      <c r="M584">
+        <v>1</v>
+      </c>
+      <c r="N584">
+        <v>0</v>
+      </c>
+      <c r="O584">
+        <v>25.29335</v>
+      </c>
+      <c r="P584">
+        <v>78.0658950617284</v>
+      </c>
+      <c r="Q584">
+        <v>32.4</v>
+      </c>
+      <c r="R584">
+        <v>315.13766</v>
+      </c>
+      <c r="S584">
+        <v>3.039913118971061</v>
+      </c>
+      <c r="T584">
+        <v>305.34</v>
+      </c>
+      <c r="U584">
+        <v>7</v>
+      </c>
+      <c r="V584">
+        <v>8</v>
+      </c>
+      <c r="W584">
+        <v>15</v>
+      </c>
+      <c r="X584">
+        <v>39</v>
+      </c>
+      <c r="Y584">
+        <v>7</v>
+      </c>
+      <c r="Z584">
+        <v>29</v>
+      </c>
+      <c r="AA584">
+        <v>8</v>
+      </c>
+      <c r="AB584">
+        <v>5</v>
+      </c>
+      <c r="AC584">
+        <v>3.74738</v>
+      </c>
+      <c r="AD584">
+        <v>-2.6201</v>
+      </c>
+      <c r="AE584">
+        <v>0</v>
+      </c>
+      <c r="AF584">
+        <v>262.0247</v>
+      </c>
+      <c r="AG584">
+        <v>0</v>
+      </c>
+      <c r="AH584">
+        <v>3</v>
+      </c>
+      <c r="AI584">
+        <v>945.4129799999999</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B585" s="2">
+        <v>46220</v>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E585">
+        <v>76.1375</v>
+      </c>
+      <c r="F585">
+        <v>3666.1</v>
+      </c>
+      <c r="G585">
+        <v>48.15104252175341</v>
+      </c>
+      <c r="H585">
+        <v>111.52</v>
+      </c>
+      <c r="I585">
+        <v>0</v>
+      </c>
+      <c r="J585">
+        <v>0</v>
+      </c>
+      <c r="K585">
+        <v>1.464718437038253</v>
+      </c>
+      <c r="L585">
+        <v>0</v>
+      </c>
+      <c r="M585">
+        <v>0</v>
+      </c>
+      <c r="N585">
+        <v>0</v>
+      </c>
+      <c r="O585">
+        <v>24.14433</v>
+      </c>
+      <c r="P585">
+        <v>67.81353218739467</v>
+      </c>
+      <c r="Q585">
+        <v>35.604</v>
+      </c>
+      <c r="R585">
+        <v>382.53</v>
+      </c>
+      <c r="S585">
+        <v>5.024199638811361</v>
+      </c>
+      <c r="T585">
+        <v>496.91</v>
+      </c>
+      <c r="U585">
+        <v>28</v>
+      </c>
+      <c r="V585">
+        <v>11</v>
+      </c>
+      <c r="W585">
+        <v>39</v>
+      </c>
+      <c r="X585">
+        <v>76</v>
+      </c>
+      <c r="Y585">
+        <v>28</v>
+      </c>
+      <c r="Z585">
+        <v>63</v>
+      </c>
+      <c r="AA585">
+        <v>11</v>
+      </c>
+      <c r="AB585">
+        <v>66</v>
+      </c>
+      <c r="AC585">
+        <v>4.03486</v>
+      </c>
+      <c r="AD585">
+        <v>-3.93838</v>
+      </c>
+      <c r="AE585">
+        <v>0</v>
+      </c>
+      <c r="AF585">
+        <v>306.02633</v>
+      </c>
+      <c r="AG585">
+        <v>0</v>
+      </c>
+      <c r="AH585">
+        <v>3</v>
+      </c>
+      <c r="AI585">
+        <v>1147.59</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B586" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E586">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F586">
+        <v>4452.08</v>
+      </c>
+      <c r="G586">
+        <v>42.94610932475884</v>
+      </c>
+      <c r="H586">
+        <v>136.9</v>
+      </c>
+      <c r="I586">
+        <v>0</v>
+      </c>
+      <c r="J586">
+        <v>0</v>
+      </c>
+      <c r="K586">
+        <v>1.320578778135048</v>
+      </c>
+      <c r="L586">
+        <v>0</v>
+      </c>
+      <c r="M586">
+        <v>3</v>
+      </c>
+      <c r="N586">
+        <v>0</v>
+      </c>
+      <c r="O586">
+        <v>28.21802</v>
+      </c>
+      <c r="P586">
+        <v>83.03325094161957</v>
+      </c>
+      <c r="Q586">
+        <v>33.984</v>
+      </c>
+      <c r="R586">
+        <v>471.70333</v>
+      </c>
+      <c r="S586">
+        <v>4.550192893890675</v>
+      </c>
+      <c r="T586">
+        <v>534.3100000000001</v>
+      </c>
+      <c r="U586">
+        <v>18</v>
+      </c>
+      <c r="V586">
+        <v>13</v>
+      </c>
+      <c r="W586">
+        <v>31</v>
+      </c>
+      <c r="X586">
+        <v>60</v>
+      </c>
+      <c r="Y586">
+        <v>18</v>
+      </c>
+      <c r="Z586">
+        <v>54</v>
+      </c>
+      <c r="AA586">
+        <v>13</v>
+      </c>
+      <c r="AB586">
+        <v>5</v>
+      </c>
+      <c r="AC586">
+        <v>4.64362</v>
+      </c>
+      <c r="AD586">
+        <v>-2.78079</v>
+      </c>
+      <c r="AE586">
+        <v>0</v>
+      </c>
+      <c r="AF586">
+        <v>408.7984</v>
+      </c>
+      <c r="AG586">
+        <v>0</v>
+      </c>
+      <c r="AH586">
+        <v>3</v>
+      </c>
+      <c r="AI586">
+        <v>1415.10999</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B587" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E587">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F587">
+        <v>3883.96</v>
+      </c>
+      <c r="G587">
+        <v>37.46585209003215</v>
+      </c>
+      <c r="H587">
+        <v>72.52</v>
+      </c>
+      <c r="I587">
+        <v>0</v>
+      </c>
+      <c r="J587">
+        <v>0</v>
+      </c>
+      <c r="K587">
+        <v>0.6995498392282957</v>
+      </c>
+      <c r="L587">
+        <v>0</v>
+      </c>
+      <c r="M587">
+        <v>0</v>
+      </c>
+      <c r="N587">
+        <v>0</v>
+      </c>
+      <c r="O587">
+        <v>25.31427</v>
+      </c>
+      <c r="P587">
+        <v>71.17147435897436</v>
+      </c>
+      <c r="Q587">
+        <v>35.568</v>
+      </c>
+      <c r="R587">
+        <v>330.04551</v>
+      </c>
+      <c r="S587">
+        <v>3.183718745980707</v>
+      </c>
+      <c r="T587">
+        <v>417.17</v>
+      </c>
+      <c r="U587">
+        <v>24</v>
+      </c>
+      <c r="V587">
+        <v>11</v>
+      </c>
+      <c r="W587">
+        <v>35</v>
+      </c>
+      <c r="X587">
+        <v>54</v>
+      </c>
+      <c r="Y587">
+        <v>24</v>
+      </c>
+      <c r="Z587">
+        <v>34</v>
+      </c>
+      <c r="AA587">
+        <v>11</v>
+      </c>
+      <c r="AB587">
+        <v>7</v>
+      </c>
+      <c r="AC587">
+        <v>4.54087</v>
+      </c>
+      <c r="AD587">
+        <v>-3.79242</v>
+      </c>
+      <c r="AE587">
+        <v>0</v>
+      </c>
+      <c r="AF587">
+        <v>357.3144</v>
+      </c>
+      <c r="AG587">
+        <v>0</v>
+      </c>
+      <c r="AH587">
+        <v>3</v>
+      </c>
+      <c r="AI587">
+        <v>990.13653</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B588" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E588">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F588">
+        <v>4156.6</v>
+      </c>
+      <c r="G588">
+        <v>40.09581993569132</v>
+      </c>
+      <c r="H588">
+        <v>66.19</v>
+      </c>
+      <c r="I588">
+        <v>0</v>
+      </c>
+      <c r="J588">
+        <v>0</v>
+      </c>
+      <c r="K588">
+        <v>0.6384887459807074</v>
+      </c>
+      <c r="L588">
+        <v>0</v>
+      </c>
+      <c r="M588">
+        <v>0</v>
+      </c>
+      <c r="N588">
+        <v>0</v>
+      </c>
+      <c r="O588">
+        <v>24.97998</v>
+      </c>
+      <c r="P588">
+        <v>69.38883333333334</v>
+      </c>
+      <c r="Q588">
+        <v>36</v>
+      </c>
+      <c r="R588">
+        <v>408.70614</v>
+      </c>
+      <c r="S588">
+        <v>3.942502958199357</v>
+      </c>
+      <c r="T588">
+        <v>408.6</v>
+      </c>
+      <c r="U588">
+        <v>12</v>
+      </c>
+      <c r="V588">
+        <v>8</v>
+      </c>
+      <c r="W588">
+        <v>20</v>
+      </c>
+      <c r="X588">
+        <v>58</v>
+      </c>
+      <c r="Y588">
+        <v>12</v>
+      </c>
+      <c r="Z588">
+        <v>42</v>
+      </c>
+      <c r="AA588">
+        <v>8</v>
+      </c>
+      <c r="AB588">
+        <v>15</v>
+      </c>
+      <c r="AC588">
+        <v>4.29704</v>
+      </c>
+      <c r="AD588">
+        <v>-3.18858</v>
+      </c>
+      <c r="AE588">
+        <v>0</v>
+      </c>
+      <c r="AF588">
+        <v>940.0600000000001</v>
+      </c>
+      <c r="AG588">
+        <v>0</v>
+      </c>
+      <c r="AH588">
+        <v>3</v>
+      </c>
+      <c r="AI588">
+        <v>1226.11842</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B589" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E589">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F589">
+        <v>4217.03</v>
+      </c>
+      <c r="G589">
+        <v>40.67874598070739</v>
+      </c>
+      <c r="H589">
+        <v>102.27</v>
+      </c>
+      <c r="I589">
+        <v>0</v>
+      </c>
+      <c r="J589">
+        <v>0</v>
+      </c>
+      <c r="K589">
+        <v>0.9865273311897105</v>
+      </c>
+      <c r="L589">
+        <v>0</v>
+      </c>
+      <c r="M589">
+        <v>0</v>
+      </c>
+      <c r="N589">
+        <v>0</v>
+      </c>
+      <c r="O589">
+        <v>24.49583</v>
+      </c>
+      <c r="P589">
+        <v>76.53990126234221</v>
+      </c>
+      <c r="Q589">
+        <v>32.004</v>
+      </c>
+      <c r="R589">
+        <v>420.99053</v>
+      </c>
+      <c r="S589">
+        <v>4.061001897106109</v>
+      </c>
+      <c r="T589">
+        <v>470.13001</v>
+      </c>
+      <c r="U589">
+        <v>15</v>
+      </c>
+      <c r="V589">
+        <v>8</v>
+      </c>
+      <c r="W589">
+        <v>23</v>
+      </c>
+      <c r="X589">
+        <v>52</v>
+      </c>
+      <c r="Y589">
+        <v>15</v>
+      </c>
+      <c r="Z589">
+        <v>39</v>
+      </c>
+      <c r="AA589">
+        <v>8</v>
+      </c>
+      <c r="AB589">
+        <v>23</v>
+      </c>
+      <c r="AC589">
+        <v>3.7869</v>
+      </c>
+      <c r="AD589">
+        <v>-3.09491</v>
+      </c>
+      <c r="AE589">
+        <v>0</v>
+      </c>
+      <c r="AF589">
+        <v>288.8268</v>
+      </c>
+      <c r="AG589">
+        <v>0</v>
+      </c>
+      <c r="AH589">
+        <v>3</v>
+      </c>
+      <c r="AI589">
+        <v>1262.97159</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B590" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E590">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F590">
+        <v>3410.46</v>
+      </c>
+      <c r="G590">
+        <v>32.89832797427653</v>
+      </c>
+      <c r="H590">
+        <v>87.98</v>
+      </c>
+      <c r="I590">
+        <v>0</v>
+      </c>
+      <c r="J590">
+        <v>0</v>
+      </c>
+      <c r="K590">
+        <v>0.8486816720257234</v>
+      </c>
+      <c r="L590">
+        <v>0</v>
+      </c>
+      <c r="M590">
+        <v>1</v>
+      </c>
+      <c r="N590">
+        <v>0</v>
+      </c>
+      <c r="O590">
+        <v>25.75351</v>
+      </c>
+      <c r="P590">
+        <v>76.10375295508273</v>
+      </c>
+      <c r="Q590">
+        <v>33.84</v>
+      </c>
+      <c r="R590">
+        <v>302.58575</v>
+      </c>
+      <c r="S590">
+        <v>2.918833601286174</v>
+      </c>
+      <c r="T590">
+        <v>318.11</v>
+      </c>
+      <c r="U590">
+        <v>16</v>
+      </c>
+      <c r="V590">
+        <v>7</v>
+      </c>
+      <c r="W590">
+        <v>23</v>
+      </c>
+      <c r="X590">
+        <v>41</v>
+      </c>
+      <c r="Y590">
+        <v>16</v>
+      </c>
+      <c r="Z590">
+        <v>24</v>
+      </c>
+      <c r="AA590">
+        <v>7</v>
+      </c>
+      <c r="AB590">
+        <v>8</v>
+      </c>
+      <c r="AC590">
+        <v>4.56387</v>
+      </c>
+      <c r="AD590">
+        <v>-1.88538</v>
+      </c>
+      <c r="AE590">
+        <v>0</v>
+      </c>
+      <c r="AF590">
+        <v>266.4795</v>
+      </c>
+      <c r="AG590">
+        <v>0</v>
+      </c>
+      <c r="AH590">
+        <v>3</v>
+      </c>
+      <c r="AI590">
+        <v>907.7572500000001</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B591" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E591">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F591">
+        <v>3839.26</v>
+      </c>
+      <c r="G591">
+        <v>37.03466237942122</v>
+      </c>
+      <c r="H591">
+        <v>97.44</v>
+      </c>
+      <c r="I591">
+        <v>0</v>
+      </c>
+      <c r="J591">
+        <v>0</v>
+      </c>
+      <c r="K591">
+        <v>0.9399356913183279</v>
+      </c>
+      <c r="L591">
+        <v>0</v>
+      </c>
+      <c r="M591">
+        <v>1</v>
+      </c>
+      <c r="N591">
+        <v>0</v>
+      </c>
+      <c r="O591">
+        <v>26.86821</v>
+      </c>
+      <c r="P591">
+        <v>79.73709045584046</v>
+      </c>
+      <c r="Q591">
+        <v>33.696</v>
+      </c>
+      <c r="R591">
+        <v>379.66868</v>
+      </c>
+      <c r="S591">
+        <v>3.662398842443729</v>
+      </c>
+      <c r="T591">
+        <v>422.5</v>
+      </c>
+      <c r="U591">
+        <v>15</v>
+      </c>
+      <c r="V591">
+        <v>11</v>
+      </c>
+      <c r="W591">
+        <v>26</v>
+      </c>
+      <c r="X591">
+        <v>54</v>
+      </c>
+      <c r="Y591">
+        <v>15</v>
+      </c>
+      <c r="Z591">
+        <v>53</v>
+      </c>
+      <c r="AA591">
+        <v>11</v>
+      </c>
+      <c r="AB591">
+        <v>18</v>
+      </c>
+      <c r="AC591">
+        <v>3.92224</v>
+      </c>
+      <c r="AD591">
+        <v>-3.4981</v>
+      </c>
+      <c r="AE591">
+        <v>0</v>
+      </c>
+      <c r="AF591">
+        <v>352.6336</v>
+      </c>
+      <c r="AG591">
+        <v>0</v>
+      </c>
+      <c r="AH591">
+        <v>3</v>
+      </c>
+      <c r="AI591">
+        <v>1139.00604</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B592" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E592">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F592">
+        <v>4042.4</v>
+      </c>
+      <c r="G592">
+        <v>38.99421221864952</v>
+      </c>
+      <c r="H592">
+        <v>41.01</v>
+      </c>
+      <c r="I592">
+        <v>0</v>
+      </c>
+      <c r="J592">
+        <v>0</v>
+      </c>
+      <c r="K592">
+        <v>0.3955948553054662</v>
+      </c>
+      <c r="L592">
+        <v>0</v>
+      </c>
+      <c r="M592">
+        <v>0</v>
+      </c>
+      <c r="N592">
+        <v>0</v>
+      </c>
+      <c r="O592">
+        <v>24.38247</v>
+      </c>
+      <c r="P592">
+        <v>67.72908333333334</v>
+      </c>
+      <c r="Q592">
+        <v>36</v>
+      </c>
+      <c r="R592">
+        <v>448.37779</v>
+      </c>
+      <c r="S592">
+        <v>4.325187684887459</v>
+      </c>
+      <c r="T592">
+        <v>418.43</v>
+      </c>
+      <c r="U592">
+        <v>16</v>
+      </c>
+      <c r="V592">
+        <v>12</v>
+      </c>
+      <c r="W592">
+        <v>28</v>
+      </c>
+      <c r="X592">
+        <v>59</v>
+      </c>
+      <c r="Y592">
+        <v>16</v>
+      </c>
+      <c r="Z592">
+        <v>43</v>
+      </c>
+      <c r="AA592">
+        <v>12</v>
+      </c>
+      <c r="AB592">
+        <v>40</v>
+      </c>
+      <c r="AC592">
+        <v>4.36928</v>
+      </c>
+      <c r="AD592">
+        <v>-3.99207</v>
+      </c>
+      <c r="AE592">
+        <v>0</v>
+      </c>
+      <c r="AF592">
+        <v>934.596</v>
+      </c>
+      <c r="AG592">
+        <v>0</v>
+      </c>
+      <c r="AH592">
+        <v>3</v>
+      </c>
+      <c r="AI592">
+        <v>1345.13337</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B593" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E593">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F593">
+        <v>4960.25</v>
+      </c>
+      <c r="G593">
+        <v>47.84807073954984</v>
+      </c>
+      <c r="H593">
+        <v>330.46</v>
+      </c>
+      <c r="I593">
+        <v>0</v>
+      </c>
+      <c r="J593">
+        <v>0</v>
+      </c>
+      <c r="K593">
+        <v>3.187717041800643</v>
+      </c>
+      <c r="L593">
+        <v>28.81</v>
+      </c>
+      <c r="M593">
+        <v>11</v>
+      </c>
+      <c r="N593">
+        <v>3</v>
+      </c>
+      <c r="O593">
+        <v>30.62385</v>
+      </c>
+      <c r="P593">
+        <v>87.5167181069959</v>
+      </c>
+      <c r="Q593">
+        <v>34.992</v>
+      </c>
+      <c r="R593">
+        <v>446.86318</v>
+      </c>
+      <c r="S593">
+        <v>4.310577299035369</v>
+      </c>
+      <c r="T593">
+        <v>685.90999</v>
+      </c>
+      <c r="U593">
+        <v>27</v>
+      </c>
+      <c r="V593">
+        <v>14</v>
+      </c>
+      <c r="W593">
+        <v>41</v>
+      </c>
+      <c r="X593">
+        <v>61</v>
+      </c>
+      <c r="Y593">
+        <v>27</v>
+      </c>
+      <c r="Z593">
+        <v>45</v>
+      </c>
+      <c r="AA593">
+        <v>14</v>
+      </c>
+      <c r="AB593">
+        <v>21</v>
+      </c>
+      <c r="AC593">
+        <v>4.68901</v>
+      </c>
+      <c r="AD593">
+        <v>-2.47704</v>
+      </c>
+      <c r="AE593">
+        <v>0</v>
+      </c>
+      <c r="AF593">
+        <v>397.7505</v>
+      </c>
+      <c r="AG593">
+        <v>0</v>
+      </c>
+      <c r="AH593">
+        <v>3</v>
+      </c>
+      <c r="AI593">
+        <v>1340.58954</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B594" s="2">
+        <v>46220</v>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E594">
+        <v>76.1375</v>
+      </c>
+      <c r="F594">
+        <v>3920.3</v>
+      </c>
+      <c r="G594">
+        <v>51.48973895912001</v>
+      </c>
+      <c r="H594">
+        <v>35.25</v>
+      </c>
+      <c r="I594">
+        <v>0</v>
+      </c>
+      <c r="J594">
+        <v>0</v>
+      </c>
+      <c r="K594">
+        <v>0.4629781645050074</v>
+      </c>
+      <c r="L594">
+        <v>0</v>
+      </c>
+      <c r="M594">
+        <v>0</v>
+      </c>
+      <c r="N594">
+        <v>0</v>
+      </c>
+      <c r="O594">
+        <v>22.60483</v>
+      </c>
+      <c r="P594">
+        <v>68.47458499939417</v>
+      </c>
+      <c r="Q594">
+        <v>33.012</v>
+      </c>
+      <c r="R594">
+        <v>464.24896</v>
+      </c>
+      <c r="S594">
+        <v>6.097507273025776</v>
+      </c>
+      <c r="T594">
+        <v>505.81</v>
+      </c>
+      <c r="U594">
+        <v>16</v>
+      </c>
+      <c r="V594">
+        <v>6</v>
+      </c>
+      <c r="W594">
+        <v>22</v>
+      </c>
+      <c r="X594">
+        <v>72</v>
+      </c>
+      <c r="Y594">
+        <v>16</v>
+      </c>
+      <c r="Z594">
+        <v>56</v>
+      </c>
+      <c r="AA594">
+        <v>6</v>
+      </c>
+      <c r="AB594">
+        <v>68</v>
+      </c>
+      <c r="AC594">
+        <v>4.12946</v>
+      </c>
+      <c r="AD594">
+        <v>-3.33435</v>
+      </c>
+      <c r="AE594">
+        <v>0</v>
+      </c>
+      <c r="AF594">
+        <v>355.70574</v>
+      </c>
+      <c r="AG594">
+        <v>0</v>
+      </c>
+      <c r="AH594">
+        <v>3</v>
+      </c>
+      <c r="AI594">
+        <v>1392.74688</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B595" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E595">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F595">
+        <v>3499.86</v>
+      </c>
+      <c r="G595">
+        <v>33.76070739549839</v>
+      </c>
+      <c r="H595">
+        <v>0.5199999999999999</v>
+      </c>
+      <c r="I595">
+        <v>0</v>
+      </c>
+      <c r="J595">
+        <v>0</v>
+      </c>
+      <c r="K595">
+        <v>0.005016077170418005</v>
+      </c>
+      <c r="L595">
+        <v>0</v>
+      </c>
+      <c r="M595">
+        <v>0</v>
+      </c>
+      <c r="N595">
+        <v>0</v>
+      </c>
+      <c r="O595">
+        <v>20.89425</v>
+      </c>
+      <c r="P595">
+        <v>59.83462199312714</v>
+      </c>
+      <c r="Q595">
+        <v>34.92</v>
+      </c>
+      <c r="R595">
+        <v>313.40017</v>
+      </c>
+      <c r="S595">
+        <v>3.023152765273312</v>
+      </c>
+      <c r="T595">
+        <v>231.64</v>
+      </c>
+      <c r="U595">
+        <v>12</v>
+      </c>
+      <c r="V595">
+        <v>4</v>
+      </c>
+      <c r="W595">
+        <v>16</v>
+      </c>
+      <c r="X595">
+        <v>42</v>
+      </c>
+      <c r="Y595">
+        <v>12</v>
+      </c>
+      <c r="Z595">
+        <v>33</v>
+      </c>
+      <c r="AA595">
+        <v>4</v>
+      </c>
+      <c r="AB595">
+        <v>6</v>
+      </c>
+      <c r="AC595">
+        <v>3.86699</v>
+      </c>
+      <c r="AD595">
+        <v>-2.58413</v>
+      </c>
+      <c r="AE595">
+        <v>0</v>
+      </c>
+      <c r="AF595">
+        <v>308.8744</v>
+      </c>
+      <c r="AG595">
+        <v>0</v>
+      </c>
+      <c r="AH595">
+        <v>3</v>
+      </c>
+      <c r="AI595">
+        <v>940.20051</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B596" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E596">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F596">
+        <v>4138.98</v>
+      </c>
+      <c r="G596">
+        <v>39.92585209003216</v>
+      </c>
+      <c r="H596">
+        <v>115.67</v>
+      </c>
+      <c r="I596">
+        <v>0</v>
+      </c>
+      <c r="J596">
+        <v>0</v>
+      </c>
+      <c r="K596">
+        <v>1.115787781350482</v>
+      </c>
+      <c r="L596">
+        <v>4.069999999999999</v>
+      </c>
+      <c r="M596">
+        <v>2</v>
+      </c>
+      <c r="N596">
+        <v>0</v>
+      </c>
+      <c r="O596">
+        <v>30.13604</v>
+      </c>
+      <c r="P596">
+        <v>86.12265660722453</v>
+      </c>
+      <c r="Q596">
+        <v>34.992</v>
+      </c>
+      <c r="R596">
+        <v>326.86264</v>
+      </c>
+      <c r="S596">
+        <v>3.153015819935691</v>
+      </c>
+      <c r="T596">
+        <v>561.29</v>
+      </c>
+      <c r="U596">
+        <v>21</v>
+      </c>
+      <c r="V596">
+        <v>17</v>
+      </c>
+      <c r="W596">
+        <v>38</v>
+      </c>
+      <c r="X596">
+        <v>61</v>
+      </c>
+      <c r="Y596">
+        <v>21</v>
+      </c>
+      <c r="Z596">
+        <v>53</v>
+      </c>
+      <c r="AA596">
+        <v>17</v>
+      </c>
+      <c r="AB596">
+        <v>8</v>
+      </c>
+      <c r="AC596">
+        <v>4.75606</v>
+      </c>
+      <c r="AD596">
+        <v>-3.74333</v>
+      </c>
+      <c r="AE596">
+        <v>0</v>
+      </c>
+      <c r="AF596">
+        <v>348.33168</v>
+      </c>
+      <c r="AG596">
+        <v>0</v>
+      </c>
+      <c r="AH596">
+        <v>3</v>
+      </c>
+      <c r="AI596">
+        <v>980.5879199999999</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B597" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E597">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F597">
+        <v>3565.41</v>
+      </c>
+      <c r="G597">
+        <v>34.39302250803858</v>
+      </c>
+      <c r="H597">
+        <v>23.91</v>
+      </c>
+      <c r="I597">
+        <v>0</v>
+      </c>
+      <c r="J597">
+        <v>0</v>
+      </c>
+      <c r="K597">
+        <v>0.2306430868167202</v>
+      </c>
+      <c r="L597">
+        <v>0</v>
+      </c>
+      <c r="M597">
+        <v>0</v>
+      </c>
+      <c r="N597">
+        <v>0</v>
+      </c>
+      <c r="O597">
+        <v>22.5146</v>
+      </c>
+      <c r="P597">
+        <v>62.54055555555556</v>
+      </c>
+      <c r="Q597">
+        <v>36</v>
+      </c>
+      <c r="R597">
+        <v>334.20361</v>
+      </c>
+      <c r="S597">
+        <v>3.223829035369774</v>
+      </c>
+      <c r="T597">
+        <v>259.97</v>
+      </c>
+      <c r="U597">
+        <v>5</v>
+      </c>
+      <c r="V597">
+        <v>7</v>
+      </c>
+      <c r="W597">
+        <v>12</v>
+      </c>
+      <c r="X597">
+        <v>31</v>
+      </c>
+      <c r="Y597">
+        <v>5</v>
+      </c>
+      <c r="Z597">
+        <v>24</v>
+      </c>
+      <c r="AA597">
+        <v>7</v>
+      </c>
+      <c r="AB597">
+        <v>11</v>
+      </c>
+      <c r="AC597">
+        <v>3.4515</v>
+      </c>
+      <c r="AD597">
+        <v>-2.85479</v>
+      </c>
+      <c r="AE597">
+        <v>0</v>
+      </c>
+      <c r="AF597">
+        <v>779.9300000000001</v>
+      </c>
+      <c r="AG597">
+        <v>0</v>
+      </c>
+      <c r="AH597">
+        <v>3</v>
+      </c>
+      <c r="AI597">
+        <v>1002.61083</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B598" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E598">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F598">
+        <v>3247.65</v>
+      </c>
+      <c r="G598">
+        <v>31.32781350482315</v>
+      </c>
+      <c r="H598">
+        <v>16.52</v>
+      </c>
+      <c r="I598">
+        <v>0</v>
+      </c>
+      <c r="J598">
+        <v>0</v>
+      </c>
+      <c r="K598">
+        <v>0.1593569131832797</v>
+      </c>
+      <c r="L598">
+        <v>0</v>
+      </c>
+      <c r="M598">
+        <v>0</v>
+      </c>
+      <c r="N598">
+        <v>0</v>
+      </c>
+      <c r="O598">
+        <v>24.3178</v>
+      </c>
+      <c r="P598">
+        <v>71.55661487758944</v>
+      </c>
+      <c r="Q598">
+        <v>33.984</v>
+      </c>
+      <c r="R598">
+        <v>317.46633</v>
+      </c>
+      <c r="S598">
+        <v>3.06237617363344</v>
+      </c>
+      <c r="T598">
+        <v>283.43</v>
+      </c>
+      <c r="U598">
+        <v>12</v>
+      </c>
+      <c r="V598">
+        <v>10</v>
+      </c>
+      <c r="W598">
+        <v>22</v>
+      </c>
+      <c r="X598">
+        <v>46</v>
+      </c>
+      <c r="Y598">
+        <v>12</v>
+      </c>
+      <c r="Z598">
+        <v>34</v>
+      </c>
+      <c r="AA598">
+        <v>10</v>
+      </c>
+      <c r="AB598">
+        <v>15</v>
+      </c>
+      <c r="AC598">
+        <v>3.50442</v>
+      </c>
+      <c r="AD598">
+        <v>-2.97066</v>
+      </c>
+      <c r="AE598">
+        <v>0</v>
+      </c>
+      <c r="AF598">
+        <v>296.9456</v>
+      </c>
+      <c r="AG598">
+        <v>0</v>
+      </c>
+      <c r="AH598">
+        <v>3</v>
+      </c>
+      <c r="AI598">
+        <v>952.3989899999999</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B599" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E599">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F599">
+        <v>3028.86</v>
+      </c>
+      <c r="G599">
+        <v>29.21729903536977</v>
+      </c>
+      <c r="H599">
+        <v>0</v>
+      </c>
+      <c r="I599">
+        <v>0</v>
+      </c>
+      <c r="J599">
+        <v>0</v>
+      </c>
+      <c r="K599">
+        <v>0</v>
+      </c>
+      <c r="L599">
+        <v>0</v>
+      </c>
+      <c r="M599">
+        <v>0</v>
+      </c>
+      <c r="N599">
+        <v>0</v>
+      </c>
+      <c r="O599">
+        <v>20.49896</v>
+      </c>
+      <c r="P599">
+        <v>58.58184727937815</v>
+      </c>
+      <c r="Q599">
+        <v>34.992</v>
+      </c>
+      <c r="R599">
+        <v>241.98564</v>
+      </c>
+      <c r="S599">
+        <v>2.334266623794212</v>
+      </c>
+      <c r="T599">
+        <v>175.09</v>
+      </c>
+      <c r="U599">
+        <v>9</v>
+      </c>
+      <c r="V599">
+        <v>6</v>
+      </c>
+      <c r="W599">
+        <v>15</v>
+      </c>
+      <c r="X599">
+        <v>29</v>
+      </c>
+      <c r="Y599">
+        <v>9</v>
+      </c>
+      <c r="Z599">
+        <v>31</v>
+      </c>
+      <c r="AA599">
+        <v>6</v>
+      </c>
+      <c r="AB599">
+        <v>9</v>
+      </c>
+      <c r="AC599">
+        <v>4.22973</v>
+      </c>
+      <c r="AD599">
+        <v>-2.40235</v>
+      </c>
+      <c r="AE599">
+        <v>0</v>
+      </c>
+      <c r="AF599">
+        <v>271.8808</v>
+      </c>
+      <c r="AG599">
+        <v>0</v>
+      </c>
+      <c r="AH599">
+        <v>3</v>
+      </c>
+      <c r="AI599">
+        <v>725.95692</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B600" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E600">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F600">
+        <v>3871.74</v>
+      </c>
+      <c r="G600">
+        <v>37.34797427652732</v>
+      </c>
+      <c r="H600">
+        <v>50.12</v>
+      </c>
+      <c r="I600">
+        <v>0</v>
+      </c>
+      <c r="J600">
+        <v>0</v>
+      </c>
+      <c r="K600">
+        <v>0.4834726688102893</v>
+      </c>
+      <c r="L600">
+        <v>0</v>
+      </c>
+      <c r="M600">
+        <v>0</v>
+      </c>
+      <c r="N600">
+        <v>0</v>
+      </c>
+      <c r="O600">
+        <v>23.33112</v>
+      </c>
+      <c r="P600">
+        <v>70.67466375863322</v>
+      </c>
+      <c r="Q600">
+        <v>33.012</v>
+      </c>
+      <c r="R600">
+        <v>356.57046</v>
+      </c>
+      <c r="S600">
+        <v>3.439586430868167</v>
+      </c>
+      <c r="T600">
+        <v>367.07</v>
+      </c>
+      <c r="U600">
+        <v>11</v>
+      </c>
+      <c r="V600">
+        <v>6</v>
+      </c>
+      <c r="W600">
+        <v>17</v>
+      </c>
+      <c r="X600">
+        <v>50</v>
+      </c>
+      <c r="Y600">
+        <v>11</v>
+      </c>
+      <c r="Z600">
+        <v>39</v>
+      </c>
+      <c r="AA600">
+        <v>6</v>
+      </c>
+      <c r="AB600">
+        <v>12</v>
+      </c>
+      <c r="AC600">
+        <v>3.93683</v>
+      </c>
+      <c r="AD600">
+        <v>-2.98918</v>
+      </c>
+      <c r="AE600">
+        <v>0</v>
+      </c>
+      <c r="AF600">
+        <v>328.1535</v>
+      </c>
+      <c r="AG600">
+        <v>0</v>
+      </c>
+      <c r="AH600">
+        <v>3</v>
+      </c>
+      <c r="AI600">
+        <v>1069.71138</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B601" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E601">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F601">
+        <v>3979.67</v>
+      </c>
+      <c r="G601">
+        <v>38.38909967845659</v>
+      </c>
+      <c r="H601">
+        <v>54.43</v>
+      </c>
+      <c r="I601">
+        <v>0</v>
+      </c>
+      <c r="J601">
+        <v>0</v>
+      </c>
+      <c r="K601">
+        <v>0.525048231511254</v>
+      </c>
+      <c r="L601">
+        <v>0</v>
+      </c>
+      <c r="M601">
+        <v>1</v>
+      </c>
+      <c r="N601">
+        <v>0</v>
+      </c>
+      <c r="O601">
+        <v>25.6503</v>
+      </c>
+      <c r="P601">
+        <v>80.14716910386203</v>
+      </c>
+      <c r="Q601">
+        <v>32.004</v>
+      </c>
+      <c r="R601">
+        <v>311.8688</v>
+      </c>
+      <c r="S601">
+        <v>3.008380707395498</v>
+      </c>
+      <c r="T601">
+        <v>329.44</v>
+      </c>
+      <c r="U601">
+        <v>9</v>
+      </c>
+      <c r="V601">
+        <v>6</v>
+      </c>
+      <c r="W601">
+        <v>15</v>
+      </c>
+      <c r="X601">
+        <v>40</v>
+      </c>
+      <c r="Y601">
+        <v>9</v>
+      </c>
+      <c r="Z601">
+        <v>25</v>
+      </c>
+      <c r="AA601">
+        <v>6</v>
+      </c>
+      <c r="AB601">
+        <v>6</v>
+      </c>
+      <c r="AC601">
+        <v>4.08307</v>
+      </c>
+      <c r="AD601">
+        <v>-2.62219</v>
+      </c>
+      <c r="AE601">
+        <v>0</v>
+      </c>
+      <c r="AF601">
+        <v>310.6768</v>
+      </c>
+      <c r="AG601">
+        <v>0</v>
+      </c>
+      <c r="AH601">
+        <v>3</v>
+      </c>
+      <c r="AI601">
+        <v>935.6064000000001</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B602" s="2">
+        <v>46220</v>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Sesion 37</t>
+        </is>
+      </c>
+      <c r="E602">
+        <v>103.6666666666667</v>
+      </c>
+      <c r="F602">
+        <v>4156.559999999999</v>
+      </c>
+      <c r="G602">
+        <v>40.09543408360128</v>
+      </c>
+      <c r="H602">
+        <v>49.39</v>
+      </c>
+      <c r="I602">
+        <v>0</v>
+      </c>
+      <c r="J602">
+        <v>0</v>
+      </c>
+      <c r="K602">
+        <v>0.4764308681672025</v>
+      </c>
+      <c r="L602">
+        <v>0</v>
+      </c>
+      <c r="M602">
+        <v>0</v>
+      </c>
+      <c r="N602">
+        <v>0</v>
+      </c>
+      <c r="O602">
+        <v>24.84488</v>
+      </c>
+      <c r="P602">
+        <v>69.01355555555556</v>
+      </c>
+      <c r="Q602">
+        <v>36</v>
+      </c>
+      <c r="R602">
+        <v>392.5079</v>
+      </c>
+      <c r="S602">
+        <v>3.786249839228295</v>
+      </c>
+      <c r="T602">
+        <v>368.22</v>
+      </c>
+      <c r="U602">
+        <v>19</v>
+      </c>
+      <c r="V602">
+        <v>15</v>
+      </c>
+      <c r="W602">
+        <v>34</v>
+      </c>
+      <c r="X602">
+        <v>50</v>
+      </c>
+      <c r="Y602">
+        <v>19</v>
+      </c>
+      <c r="Z602">
+        <v>41</v>
+      </c>
+      <c r="AA602">
+        <v>15</v>
+      </c>
+      <c r="AB602">
+        <v>11</v>
+      </c>
+      <c r="AC602">
+        <v>4.08662</v>
+      </c>
+      <c r="AD602">
+        <v>-3.37051</v>
+      </c>
+      <c r="AE602">
+        <v>0</v>
+      </c>
+      <c r="AF602">
+        <v>947.602</v>
+      </c>
+      <c r="AG602">
+        <v>0</v>
+      </c>
+      <c r="AH602">
+        <v>3</v>
+      </c>
+      <c r="AI602">
+        <v>1177.5237</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B603" s="2">
+        <v>46220</v>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E603">
+        <v>76.1375</v>
+      </c>
+      <c r="F603">
+        <v>4046.36</v>
+      </c>
+      <c r="G603">
+        <v>53.14542768018388</v>
+      </c>
+      <c r="H603">
+        <v>127.21</v>
+      </c>
+      <c r="I603">
+        <v>0</v>
+      </c>
+      <c r="J603">
+        <v>0</v>
+      </c>
+      <c r="K603">
+        <v>1.670792973239205</v>
+      </c>
+      <c r="L603">
+        <v>0</v>
+      </c>
+      <c r="M603">
+        <v>0</v>
+      </c>
+      <c r="N603">
+        <v>0</v>
+      </c>
+      <c r="O603">
+        <v>24.85011</v>
+      </c>
+      <c r="P603">
+        <v>71.01654663923183</v>
+      </c>
+      <c r="Q603">
+        <v>34.992</v>
+      </c>
+      <c r="R603">
+        <v>477.18832</v>
+      </c>
+      <c r="S603">
+        <v>6.267454539484484</v>
+      </c>
+      <c r="T603">
+        <v>580.70001</v>
+      </c>
+      <c r="U603">
+        <v>30</v>
+      </c>
+      <c r="V603">
+        <v>9</v>
+      </c>
+      <c r="W603">
+        <v>39</v>
+      </c>
+      <c r="X603">
+        <v>88</v>
+      </c>
+      <c r="Y603">
+        <v>30</v>
+      </c>
+      <c r="Z603">
+        <v>61</v>
+      </c>
+      <c r="AA603">
+        <v>9</v>
+      </c>
+      <c r="AB603">
+        <v>48</v>
+      </c>
+      <c r="AC603">
+        <v>4.13149</v>
+      </c>
+      <c r="AD603">
+        <v>-3.9791</v>
+      </c>
+      <c r="AE603">
+        <v>0</v>
+      </c>
+      <c r="AF603">
+        <v>382.3952</v>
+      </c>
+      <c r="AG603">
+        <v>0</v>
+      </c>
+      <c r="AH603">
+        <v>3</v>
+      </c>
+      <c r="AI603">
+        <v>1431.56496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-19
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI603"/>
+  <dimension ref="A1:AI625"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -66316,6 +66316,11 @@
       <c r="B585" s="2">
         <v>46220</v>
       </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D585" t="inlineStr">
         <is>
           <t>Trabajo Seleccionados</t>
@@ -67328,6 +67333,11 @@
       <c r="B594" s="2">
         <v>46220</v>
       </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D594" t="inlineStr">
         <is>
           <t>Trabajo Seleccionados</t>
@@ -68340,6 +68350,11 @@
       <c r="B603" s="2">
         <v>46220</v>
       </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
       <c r="D603" t="inlineStr">
         <is>
           <t>Trabajo Seleccionados</t>
@@ -68437,6 +68452,2492 @@
       </c>
       <c r="AI603">
         <v>1431.56496</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B604" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E604">
+        <v>123.9633333333333</v>
+      </c>
+      <c r="F604">
+        <v>11934.76</v>
+      </c>
+      <c r="G604">
+        <v>96.27653338352738</v>
+      </c>
+      <c r="H604">
+        <v>636.22</v>
+      </c>
+      <c r="I604">
+        <v>0</v>
+      </c>
+      <c r="J604">
+        <v>0</v>
+      </c>
+      <c r="K604">
+        <v>5.132324074323052</v>
+      </c>
+      <c r="L604">
+        <v>0</v>
+      </c>
+      <c r="M604">
+        <v>9</v>
+      </c>
+      <c r="N604">
+        <v>0</v>
+      </c>
+      <c r="O604">
+        <v>29.0962</v>
+      </c>
+      <c r="P604">
+        <v>89.90297861821777</v>
+      </c>
+      <c r="Q604">
+        <v>32.364</v>
+      </c>
+      <c r="R604">
+        <v>1202.78533</v>
+      </c>
+      <c r="S604">
+        <v>9.702750786522895</v>
+      </c>
+      <c r="T604">
+        <v>1984.55002</v>
+      </c>
+      <c r="U604">
+        <v>31</v>
+      </c>
+      <c r="V604">
+        <v>33</v>
+      </c>
+      <c r="W604">
+        <v>64</v>
+      </c>
+      <c r="X604">
+        <v>118</v>
+      </c>
+      <c r="Y604">
+        <v>31</v>
+      </c>
+      <c r="Z604">
+        <v>112</v>
+      </c>
+      <c r="AA604">
+        <v>33</v>
+      </c>
+      <c r="AB604">
+        <v>42</v>
+      </c>
+      <c r="AC604">
+        <v>4.16505</v>
+      </c>
+      <c r="AD604">
+        <v>-3.83553</v>
+      </c>
+      <c r="AE604">
+        <v>0</v>
+      </c>
+      <c r="AF604">
+        <v>972.0284</v>
+      </c>
+      <c r="AG604">
+        <v>0</v>
+      </c>
+      <c r="AH604">
+        <v>3</v>
+      </c>
+      <c r="AI604">
+        <v>3608.35599</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B605" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E605">
+        <v>55.943</v>
+      </c>
+      <c r="F605">
+        <v>2595.27</v>
+      </c>
+      <c r="G605">
+        <v>46.39132688629498</v>
+      </c>
+      <c r="H605">
+        <v>24.64</v>
+      </c>
+      <c r="I605">
+        <v>0</v>
+      </c>
+      <c r="J605">
+        <v>0</v>
+      </c>
+      <c r="K605">
+        <v>0.4404483134619165</v>
+      </c>
+      <c r="L605">
+        <v>0</v>
+      </c>
+      <c r="M605">
+        <v>0</v>
+      </c>
+      <c r="N605">
+        <v>0</v>
+      </c>
+      <c r="O605">
+        <v>24.27484</v>
+      </c>
+      <c r="P605">
+        <v>67.43011111111112</v>
+      </c>
+      <c r="Q605">
+        <v>36</v>
+      </c>
+      <c r="R605">
+        <v>282.17018</v>
+      </c>
+      <c r="S605">
+        <v>5.043887170870351</v>
+      </c>
+      <c r="T605">
+        <v>195.59</v>
+      </c>
+      <c r="U605">
+        <v>6</v>
+      </c>
+      <c r="V605">
+        <v>4</v>
+      </c>
+      <c r="W605">
+        <v>10</v>
+      </c>
+      <c r="X605">
+        <v>30</v>
+      </c>
+      <c r="Y605">
+        <v>6</v>
+      </c>
+      <c r="Z605">
+        <v>19</v>
+      </c>
+      <c r="AA605">
+        <v>4</v>
+      </c>
+      <c r="AB605">
+        <v>15</v>
+      </c>
+      <c r="AC605">
+        <v>3.99352</v>
+      </c>
+      <c r="AD605">
+        <v>-2.45715</v>
+      </c>
+      <c r="AE605">
+        <v>0</v>
+      </c>
+      <c r="AF605">
+        <v>578.516</v>
+      </c>
+      <c r="AG605">
+        <v>0</v>
+      </c>
+      <c r="AH605">
+        <v>3</v>
+      </c>
+      <c r="AI605">
+        <v>846.51054</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B606" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E606">
+        <v>68.61016666666666</v>
+      </c>
+      <c r="F606">
+        <v>4435.42</v>
+      </c>
+      <c r="G606">
+        <v>64.64668744428062</v>
+      </c>
+      <c r="H606">
+        <v>246.04</v>
+      </c>
+      <c r="I606">
+        <v>25.02</v>
+      </c>
+      <c r="J606">
+        <v>2</v>
+      </c>
+      <c r="K606">
+        <v>3.586057459900258</v>
+      </c>
+      <c r="L606">
+        <v>8.9</v>
+      </c>
+      <c r="M606">
+        <v>5</v>
+      </c>
+      <c r="N606">
+        <v>1</v>
+      </c>
+      <c r="O606">
+        <v>30.51658</v>
+      </c>
+      <c r="P606">
+        <v>94.18697530864199</v>
+      </c>
+      <c r="Q606">
+        <v>32.4</v>
+      </c>
+      <c r="R606">
+        <v>473.45646</v>
+      </c>
+      <c r="S606">
+        <v>6.900674972853878</v>
+      </c>
+      <c r="T606">
+        <v>746.9499900000001</v>
+      </c>
+      <c r="U606">
+        <v>15</v>
+      </c>
+      <c r="V606">
+        <v>15</v>
+      </c>
+      <c r="W606">
+        <v>30</v>
+      </c>
+      <c r="X606">
+        <v>52</v>
+      </c>
+      <c r="Y606">
+        <v>15</v>
+      </c>
+      <c r="Z606">
+        <v>39</v>
+      </c>
+      <c r="AA606">
+        <v>15</v>
+      </c>
+      <c r="AB606">
+        <v>10</v>
+      </c>
+      <c r="AC606">
+        <v>3.68013</v>
+      </c>
+      <c r="AD606">
+        <v>-2.1465</v>
+      </c>
+      <c r="AE606">
+        <v>0</v>
+      </c>
+      <c r="AF606">
+        <v>360.3964</v>
+      </c>
+      <c r="AG606">
+        <v>0</v>
+      </c>
+      <c r="AH606">
+        <v>3</v>
+      </c>
+      <c r="AI606">
+        <v>1420.36938</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B607" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E607">
+        <v>104.4666666666667</v>
+      </c>
+      <c r="F607">
+        <v>8746.42</v>
+      </c>
+      <c r="G607">
+        <v>83.7245054243778</v>
+      </c>
+      <c r="H607">
+        <v>392.17</v>
+      </c>
+      <c r="I607">
+        <v>0</v>
+      </c>
+      <c r="J607">
+        <v>0</v>
+      </c>
+      <c r="K607">
+        <v>3.754020421186981</v>
+      </c>
+      <c r="L607">
+        <v>7.99</v>
+      </c>
+      <c r="M607">
+        <v>4</v>
+      </c>
+      <c r="N607">
+        <v>1</v>
+      </c>
+      <c r="O607">
+        <v>30.51072</v>
+      </c>
+      <c r="P607">
+        <v>85.69464105156725</v>
+      </c>
+      <c r="Q607">
+        <v>35.604</v>
+      </c>
+      <c r="R607">
+        <v>671.3025700000001</v>
+      </c>
+      <c r="S607">
+        <v>6.425997798340779</v>
+      </c>
+      <c r="T607">
+        <v>1234.90002</v>
+      </c>
+      <c r="U607">
+        <v>23</v>
+      </c>
+      <c r="V607">
+        <v>18</v>
+      </c>
+      <c r="W607">
+        <v>41</v>
+      </c>
+      <c r="X607">
+        <v>128</v>
+      </c>
+      <c r="Y607">
+        <v>23</v>
+      </c>
+      <c r="Z607">
+        <v>79</v>
+      </c>
+      <c r="AA607">
+        <v>18</v>
+      </c>
+      <c r="AB607">
+        <v>26</v>
+      </c>
+      <c r="AC607">
+        <v>4.38643</v>
+      </c>
+      <c r="AD607">
+        <v>-2.63833</v>
+      </c>
+      <c r="AE607">
+        <v>0</v>
+      </c>
+      <c r="AF607">
+        <v>718.0173199999999</v>
+      </c>
+      <c r="AG607">
+        <v>0</v>
+      </c>
+      <c r="AH607">
+        <v>3</v>
+      </c>
+      <c r="AI607">
+        <v>2013.90771</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B608" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E608">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F608">
+        <v>11062.66</v>
+      </c>
+      <c r="G608">
+        <v>82.07867815359961</v>
+      </c>
+      <c r="H608">
+        <v>505.48</v>
+      </c>
+      <c r="I608">
+        <v>19.81</v>
+      </c>
+      <c r="J608">
+        <v>1</v>
+      </c>
+      <c r="K608">
+        <v>3.750375608857321</v>
+      </c>
+      <c r="L608">
+        <v>28.65</v>
+      </c>
+      <c r="M608">
+        <v>8</v>
+      </c>
+      <c r="N608">
+        <v>2</v>
+      </c>
+      <c r="O608">
+        <v>31.65871</v>
+      </c>
+      <c r="P608">
+        <v>93.15769185499057</v>
+      </c>
+      <c r="Q608">
+        <v>33.984</v>
+      </c>
+      <c r="R608">
+        <v>1169.83893</v>
+      </c>
+      <c r="S608">
+        <v>8.679542987583575</v>
+      </c>
+      <c r="T608">
+        <v>1533.96</v>
+      </c>
+      <c r="U608">
+        <v>27</v>
+      </c>
+      <c r="V608">
+        <v>45</v>
+      </c>
+      <c r="W608">
+        <v>72</v>
+      </c>
+      <c r="X608">
+        <v>102</v>
+      </c>
+      <c r="Y608">
+        <v>27</v>
+      </c>
+      <c r="Z608">
+        <v>108</v>
+      </c>
+      <c r="AA608">
+        <v>45</v>
+      </c>
+      <c r="AB608">
+        <v>28</v>
+      </c>
+      <c r="AC608">
+        <v>4.96485</v>
+      </c>
+      <c r="AD608">
+        <v>-3.61949</v>
+      </c>
+      <c r="AE608">
+        <v>0</v>
+      </c>
+      <c r="AF608">
+        <v>1039.9472</v>
+      </c>
+      <c r="AG608">
+        <v>0</v>
+      </c>
+      <c r="AH608">
+        <v>3</v>
+      </c>
+      <c r="AI608">
+        <v>3509.51679</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B609" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E609">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F609">
+        <v>12420.63</v>
+      </c>
+      <c r="G609">
+        <v>92.15404723953766</v>
+      </c>
+      <c r="H609">
+        <v>854.61</v>
+      </c>
+      <c r="I609">
+        <v>0</v>
+      </c>
+      <c r="J609">
+        <v>0</v>
+      </c>
+      <c r="K609">
+        <v>6.340722677624346</v>
+      </c>
+      <c r="L609">
+        <v>19.4</v>
+      </c>
+      <c r="M609">
+        <v>17</v>
+      </c>
+      <c r="N609">
+        <v>1</v>
+      </c>
+      <c r="O609">
+        <v>31.58524</v>
+      </c>
+      <c r="P609">
+        <v>88.80240665766982</v>
+      </c>
+      <c r="Q609">
+        <v>35.568</v>
+      </c>
+      <c r="R609">
+        <v>1119.70534</v>
+      </c>
+      <c r="S609">
+        <v>8.307580114432406</v>
+      </c>
+      <c r="T609">
+        <v>2127.20997</v>
+      </c>
+      <c r="U609">
+        <v>56</v>
+      </c>
+      <c r="V609">
+        <v>49</v>
+      </c>
+      <c r="W609">
+        <v>105</v>
+      </c>
+      <c r="X609">
+        <v>182</v>
+      </c>
+      <c r="Y609">
+        <v>56</v>
+      </c>
+      <c r="Z609">
+        <v>132</v>
+      </c>
+      <c r="AA609">
+        <v>49</v>
+      </c>
+      <c r="AB609">
+        <v>23</v>
+      </c>
+      <c r="AC609">
+        <v>5.04787</v>
+      </c>
+      <c r="AD609">
+        <v>-4.47427</v>
+      </c>
+      <c r="AE609">
+        <v>0</v>
+      </c>
+      <c r="AF609">
+        <v>1180.4168</v>
+      </c>
+      <c r="AG609">
+        <v>0</v>
+      </c>
+      <c r="AH609">
+        <v>3</v>
+      </c>
+      <c r="AI609">
+        <v>3359.11602</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B610" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E610">
+        <v>104.4666666666667</v>
+      </c>
+      <c r="F610">
+        <v>10032.84</v>
+      </c>
+      <c r="G610">
+        <v>96.03867262284621</v>
+      </c>
+      <c r="H610">
+        <v>1023.49</v>
+      </c>
+      <c r="I610">
+        <v>0</v>
+      </c>
+      <c r="J610">
+        <v>0</v>
+      </c>
+      <c r="K610">
+        <v>9.79728781110402</v>
+      </c>
+      <c r="L610">
+        <v>0</v>
+      </c>
+      <c r="M610">
+        <v>17</v>
+      </c>
+      <c r="N610">
+        <v>0</v>
+      </c>
+      <c r="O610">
+        <v>29.45269</v>
+      </c>
+      <c r="P610">
+        <v>81.81302777777778</v>
+      </c>
+      <c r="Q610">
+        <v>36</v>
+      </c>
+      <c r="R610">
+        <v>881.3364800000001</v>
+      </c>
+      <c r="S610">
+        <v>8.436532992980217</v>
+      </c>
+      <c r="T610">
+        <v>1887.45002</v>
+      </c>
+      <c r="U610">
+        <v>29</v>
+      </c>
+      <c r="V610">
+        <v>28</v>
+      </c>
+      <c r="W610">
+        <v>57</v>
+      </c>
+      <c r="X610">
+        <v>113</v>
+      </c>
+      <c r="Y610">
+        <v>29</v>
+      </c>
+      <c r="Z610">
+        <v>77</v>
+      </c>
+      <c r="AA610">
+        <v>28</v>
+      </c>
+      <c r="AB610">
+        <v>21</v>
+      </c>
+      <c r="AC610">
+        <v>4.42128</v>
+      </c>
+      <c r="AD610">
+        <v>-2.66755</v>
+      </c>
+      <c r="AE610">
+        <v>0</v>
+      </c>
+      <c r="AF610">
+        <v>820.7416000000001</v>
+      </c>
+      <c r="AG610">
+        <v>0</v>
+      </c>
+      <c r="AH610">
+        <v>3</v>
+      </c>
+      <c r="AI610">
+        <v>2644.00944</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B611" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E611">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F611">
+        <v>12260.25</v>
+      </c>
+      <c r="G611">
+        <v>90.96411837954609</v>
+      </c>
+      <c r="H611">
+        <v>647.5300000000001</v>
+      </c>
+      <c r="I611">
+        <v>32.73999999999999</v>
+      </c>
+      <c r="J611">
+        <v>3</v>
+      </c>
+      <c r="K611">
+        <v>4.804306239620521</v>
+      </c>
+      <c r="L611">
+        <v>0</v>
+      </c>
+      <c r="M611">
+        <v>13</v>
+      </c>
+      <c r="N611">
+        <v>0</v>
+      </c>
+      <c r="O611">
+        <v>29.65815</v>
+      </c>
+      <c r="P611">
+        <v>92.67013498312711</v>
+      </c>
+      <c r="Q611">
+        <v>32.004</v>
+      </c>
+      <c r="R611">
+        <v>1288.35371</v>
+      </c>
+      <c r="S611">
+        <v>9.558855601734662</v>
+      </c>
+      <c r="T611">
+        <v>1853.59998</v>
+      </c>
+      <c r="U611">
+        <v>24</v>
+      </c>
+      <c r="V611">
+        <v>37</v>
+      </c>
+      <c r="W611">
+        <v>61</v>
+      </c>
+      <c r="X611">
+        <v>105</v>
+      </c>
+      <c r="Y611">
+        <v>24</v>
+      </c>
+      <c r="Z611">
+        <v>116</v>
+      </c>
+      <c r="AA611">
+        <v>37</v>
+      </c>
+      <c r="AB611">
+        <v>40</v>
+      </c>
+      <c r="AC611">
+        <v>4.29089</v>
+      </c>
+      <c r="AD611">
+        <v>-3.68214</v>
+      </c>
+      <c r="AE611">
+        <v>0</v>
+      </c>
+      <c r="AF611">
+        <v>852.8915999999999</v>
+      </c>
+      <c r="AG611">
+        <v>0</v>
+      </c>
+      <c r="AH611">
+        <v>3</v>
+      </c>
+      <c r="AI611">
+        <v>3865.06113</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B612" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E612">
+        <v>38.35783333333333</v>
+      </c>
+      <c r="F612">
+        <v>1760.45</v>
+      </c>
+      <c r="G612">
+        <v>45.89544943014682</v>
+      </c>
+      <c r="H612">
+        <v>0</v>
+      </c>
+      <c r="I612">
+        <v>0</v>
+      </c>
+      <c r="J612">
+        <v>0</v>
+      </c>
+      <c r="K612">
+        <v>0</v>
+      </c>
+      <c r="L612">
+        <v>0</v>
+      </c>
+      <c r="M612">
+        <v>0</v>
+      </c>
+      <c r="N612">
+        <v>0</v>
+      </c>
+      <c r="O612">
+        <v>19.34911</v>
+      </c>
+      <c r="P612">
+        <v>57.17822104018911</v>
+      </c>
+      <c r="Q612">
+        <v>33.84</v>
+      </c>
+      <c r="R612">
+        <v>211.63485</v>
+      </c>
+      <c r="S612">
+        <v>5.517382803164934</v>
+      </c>
+      <c r="T612">
+        <v>127.08</v>
+      </c>
+      <c r="U612">
+        <v>12</v>
+      </c>
+      <c r="V612">
+        <v>4</v>
+      </c>
+      <c r="W612">
+        <v>16</v>
+      </c>
+      <c r="X612">
+        <v>19</v>
+      </c>
+      <c r="Y612">
+        <v>12</v>
+      </c>
+      <c r="Z612">
+        <v>13</v>
+      </c>
+      <c r="AA612">
+        <v>4</v>
+      </c>
+      <c r="AB612">
+        <v>7</v>
+      </c>
+      <c r="AC612">
+        <v>3.87366</v>
+      </c>
+      <c r="AD612">
+        <v>-3.03735</v>
+      </c>
+      <c r="AE612">
+        <v>0</v>
+      </c>
+      <c r="AF612">
+        <v>137.9511</v>
+      </c>
+      <c r="AG612">
+        <v>0</v>
+      </c>
+      <c r="AH612">
+        <v>3</v>
+      </c>
+      <c r="AI612">
+        <v>634.90455</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B613" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E613">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F613">
+        <v>10533.85</v>
+      </c>
+      <c r="G613">
+        <v>78.1552071444205</v>
+      </c>
+      <c r="H613">
+        <v>467.37</v>
+      </c>
+      <c r="I613">
+        <v>0</v>
+      </c>
+      <c r="J613">
+        <v>0</v>
+      </c>
+      <c r="K613">
+        <v>3.467620970783504</v>
+      </c>
+      <c r="L613">
+        <v>0</v>
+      </c>
+      <c r="M613">
+        <v>5</v>
+      </c>
+      <c r="N613">
+        <v>0</v>
+      </c>
+      <c r="O613">
+        <v>27.26528</v>
+      </c>
+      <c r="P613">
+        <v>80.91547958214626</v>
+      </c>
+      <c r="Q613">
+        <v>33.696</v>
+      </c>
+      <c r="R613">
+        <v>1152.26028</v>
+      </c>
+      <c r="S613">
+        <v>8.549119350255413</v>
+      </c>
+      <c r="T613">
+        <v>1647.3</v>
+      </c>
+      <c r="U613">
+        <v>41</v>
+      </c>
+      <c r="V613">
+        <v>45</v>
+      </c>
+      <c r="W613">
+        <v>86</v>
+      </c>
+      <c r="X613">
+        <v>157</v>
+      </c>
+      <c r="Y613">
+        <v>41</v>
+      </c>
+      <c r="Z613">
+        <v>139</v>
+      </c>
+      <c r="AA613">
+        <v>45</v>
+      </c>
+      <c r="AB613">
+        <v>50</v>
+      </c>
+      <c r="AC613">
+        <v>4.31216</v>
+      </c>
+      <c r="AD613">
+        <v>-3.9919</v>
+      </c>
+      <c r="AE613">
+        <v>0</v>
+      </c>
+      <c r="AF613">
+        <v>1019.2528</v>
+      </c>
+      <c r="AG613">
+        <v>0</v>
+      </c>
+      <c r="AH613">
+        <v>3</v>
+      </c>
+      <c r="AI613">
+        <v>3456.78084</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B614" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E614">
+        <v>94.60316666666667</v>
+      </c>
+      <c r="F614">
+        <v>4047.920000000001</v>
+      </c>
+      <c r="G614">
+        <v>42.78841969701508</v>
+      </c>
+      <c r="H614">
+        <v>138.79</v>
+      </c>
+      <c r="I614">
+        <v>0</v>
+      </c>
+      <c r="J614">
+        <v>0</v>
+      </c>
+      <c r="K614">
+        <v>1.467075626432519</v>
+      </c>
+      <c r="L614">
+        <v>0</v>
+      </c>
+      <c r="M614">
+        <v>3</v>
+      </c>
+      <c r="N614">
+        <v>0</v>
+      </c>
+      <c r="O614">
+        <v>26.99518</v>
+      </c>
+      <c r="P614">
+        <v>74.98661111111112</v>
+      </c>
+      <c r="Q614">
+        <v>36</v>
+      </c>
+      <c r="R614">
+        <v>558.0625700000001</v>
+      </c>
+      <c r="S614">
+        <v>5.89898403682752</v>
+      </c>
+      <c r="T614">
+        <v>538.88999</v>
+      </c>
+      <c r="U614">
+        <v>14</v>
+      </c>
+      <c r="V614">
+        <v>11</v>
+      </c>
+      <c r="W614">
+        <v>25</v>
+      </c>
+      <c r="X614">
+        <v>50</v>
+      </c>
+      <c r="Y614">
+        <v>14</v>
+      </c>
+      <c r="Z614">
+        <v>41</v>
+      </c>
+      <c r="AA614">
+        <v>11</v>
+      </c>
+      <c r="AB614">
+        <v>308</v>
+      </c>
+      <c r="AC614">
+        <v>4.81753</v>
+      </c>
+      <c r="AD614">
+        <v>-2.84248</v>
+      </c>
+      <c r="AE614">
+        <v>0</v>
+      </c>
+      <c r="AF614">
+        <v>934.296</v>
+      </c>
+      <c r="AG614">
+        <v>0</v>
+      </c>
+      <c r="AH614">
+        <v>3</v>
+      </c>
+      <c r="AI614">
+        <v>1674.18771</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B615" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E615">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F615">
+        <v>12539.16</v>
+      </c>
+      <c r="G615">
+        <v>93.03347277747756</v>
+      </c>
+      <c r="H615">
+        <v>823.8299999999999</v>
+      </c>
+      <c r="I615">
+        <v>1.67</v>
+      </c>
+      <c r="J615">
+        <v>0</v>
+      </c>
+      <c r="K615">
+        <v>6.112352492373438</v>
+      </c>
+      <c r="L615">
+        <v>32.16</v>
+      </c>
+      <c r="M615">
+        <v>17</v>
+      </c>
+      <c r="N615">
+        <v>1</v>
+      </c>
+      <c r="O615">
+        <v>31.33482</v>
+      </c>
+      <c r="P615">
+        <v>89.5485253772291</v>
+      </c>
+      <c r="Q615">
+        <v>34.992</v>
+      </c>
+      <c r="R615">
+        <v>1089.53458</v>
+      </c>
+      <c r="S615">
+        <v>8.083730145284887</v>
+      </c>
+      <c r="T615">
+        <v>2021.42998</v>
+      </c>
+      <c r="U615">
+        <v>38</v>
+      </c>
+      <c r="V615">
+        <v>46</v>
+      </c>
+      <c r="W615">
+        <v>84</v>
+      </c>
+      <c r="X615">
+        <v>128</v>
+      </c>
+      <c r="Y615">
+        <v>38</v>
+      </c>
+      <c r="Z615">
+        <v>127</v>
+      </c>
+      <c r="AA615">
+        <v>46</v>
+      </c>
+      <c r="AB615">
+        <v>33</v>
+      </c>
+      <c r="AC615">
+        <v>4.36318</v>
+      </c>
+      <c r="AD615">
+        <v>-3.93302</v>
+      </c>
+      <c r="AE615">
+        <v>0</v>
+      </c>
+      <c r="AF615">
+        <v>1012.52532</v>
+      </c>
+      <c r="AG615">
+        <v>0</v>
+      </c>
+      <c r="AH615">
+        <v>3</v>
+      </c>
+      <c r="AI615">
+        <v>3268.60374</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B616" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E616">
+        <v>104.4666666666667</v>
+      </c>
+      <c r="F616">
+        <v>9040.17</v>
+      </c>
+      <c r="G616">
+        <v>86.53640714741545</v>
+      </c>
+      <c r="H616">
+        <v>185.04</v>
+      </c>
+      <c r="I616">
+        <v>0</v>
+      </c>
+      <c r="J616">
+        <v>0</v>
+      </c>
+      <c r="K616">
+        <v>1.771282705807275</v>
+      </c>
+      <c r="L616">
+        <v>0</v>
+      </c>
+      <c r="M616">
+        <v>0</v>
+      </c>
+      <c r="N616">
+        <v>0</v>
+      </c>
+      <c r="O616">
+        <v>24.92789</v>
+      </c>
+      <c r="P616">
+        <v>75.51160184175451</v>
+      </c>
+      <c r="Q616">
+        <v>33.012</v>
+      </c>
+      <c r="R616">
+        <v>868.54418</v>
+      </c>
+      <c r="S616">
+        <v>8.314079578813018</v>
+      </c>
+      <c r="T616">
+        <v>1032.09997</v>
+      </c>
+      <c r="U616">
+        <v>12</v>
+      </c>
+      <c r="V616">
+        <v>22</v>
+      </c>
+      <c r="W616">
+        <v>34</v>
+      </c>
+      <c r="X616">
+        <v>102</v>
+      </c>
+      <c r="Y616">
+        <v>12</v>
+      </c>
+      <c r="Z616">
+        <v>90</v>
+      </c>
+      <c r="AA616">
+        <v>22</v>
+      </c>
+      <c r="AB616">
+        <v>30</v>
+      </c>
+      <c r="AC616">
+        <v>3.95576</v>
+      </c>
+      <c r="AD616">
+        <v>-2.23206</v>
+      </c>
+      <c r="AE616">
+        <v>0</v>
+      </c>
+      <c r="AF616">
+        <v>813.51816</v>
+      </c>
+      <c r="AG616">
+        <v>0</v>
+      </c>
+      <c r="AH616">
+        <v>3</v>
+      </c>
+      <c r="AI616">
+        <v>2605.63254</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B617" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E617">
+        <v>38.35783333333333</v>
+      </c>
+      <c r="F617">
+        <v>2012.97</v>
+      </c>
+      <c r="G617">
+        <v>52.47872012235659</v>
+      </c>
+      <c r="H617">
+        <v>0</v>
+      </c>
+      <c r="I617">
+        <v>0</v>
+      </c>
+      <c r="J617">
+        <v>0</v>
+      </c>
+      <c r="K617">
+        <v>0</v>
+      </c>
+      <c r="L617">
+        <v>0</v>
+      </c>
+      <c r="M617">
+        <v>0</v>
+      </c>
+      <c r="N617">
+        <v>0</v>
+      </c>
+      <c r="O617">
+        <v>20.38388</v>
+      </c>
+      <c r="P617">
+        <v>58.37308132875143</v>
+      </c>
+      <c r="Q617">
+        <v>34.92</v>
+      </c>
+      <c r="R617">
+        <v>229.43171</v>
+      </c>
+      <c r="S617">
+        <v>5.981352179259344</v>
+      </c>
+      <c r="T617">
+        <v>119.91</v>
+      </c>
+      <c r="U617">
+        <v>6</v>
+      </c>
+      <c r="V617">
+        <v>3</v>
+      </c>
+      <c r="W617">
+        <v>9</v>
+      </c>
+      <c r="X617">
+        <v>17</v>
+      </c>
+      <c r="Y617">
+        <v>6</v>
+      </c>
+      <c r="Z617">
+        <v>9</v>
+      </c>
+      <c r="AA617">
+        <v>3</v>
+      </c>
+      <c r="AB617">
+        <v>3</v>
+      </c>
+      <c r="AC617">
+        <v>3.67796</v>
+      </c>
+      <c r="AD617">
+        <v>-2.47646</v>
+      </c>
+      <c r="AE617">
+        <v>0</v>
+      </c>
+      <c r="AF617">
+        <v>177.332</v>
+      </c>
+      <c r="AG617">
+        <v>0</v>
+      </c>
+      <c r="AH617">
+        <v>3</v>
+      </c>
+      <c r="AI617">
+        <v>688.29513</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B618" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E618">
+        <v>114.0725</v>
+      </c>
+      <c r="F618">
+        <v>10352.32</v>
+      </c>
+      <c r="G618">
+        <v>90.75210940410705</v>
+      </c>
+      <c r="H618">
+        <v>912.92</v>
+      </c>
+      <c r="I618">
+        <v>11.93</v>
+      </c>
+      <c r="J618">
+        <v>1</v>
+      </c>
+      <c r="K618">
+        <v>8.002980560608384</v>
+      </c>
+      <c r="L618">
+        <v>34.51</v>
+      </c>
+      <c r="M618">
+        <v>23</v>
+      </c>
+      <c r="N618">
+        <v>2</v>
+      </c>
+      <c r="O618">
+        <v>31.65133</v>
+      </c>
+      <c r="P618">
+        <v>90.45304641060815</v>
+      </c>
+      <c r="Q618">
+        <v>34.992</v>
+      </c>
+      <c r="R618">
+        <v>880.03355</v>
+      </c>
+      <c r="S618">
+        <v>7.71468627408008</v>
+      </c>
+      <c r="T618">
+        <v>1967.19999</v>
+      </c>
+      <c r="U618">
+        <v>37</v>
+      </c>
+      <c r="V618">
+        <v>50</v>
+      </c>
+      <c r="W618">
+        <v>87</v>
+      </c>
+      <c r="X618">
+        <v>129</v>
+      </c>
+      <c r="Y618">
+        <v>37</v>
+      </c>
+      <c r="Z618">
+        <v>128</v>
+      </c>
+      <c r="AA618">
+        <v>50</v>
+      </c>
+      <c r="AB618">
+        <v>34</v>
+      </c>
+      <c r="AC618">
+        <v>4.6265</v>
+      </c>
+      <c r="AD618">
+        <v>-4.14579</v>
+      </c>
+      <c r="AE618">
+        <v>0</v>
+      </c>
+      <c r="AF618">
+        <v>881.0844400000001</v>
+      </c>
+      <c r="AG618">
+        <v>0</v>
+      </c>
+      <c r="AH618">
+        <v>3</v>
+      </c>
+      <c r="AI618">
+        <v>2640.10065</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B619" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E619">
+        <v>38.35783333333333</v>
+      </c>
+      <c r="F619">
+        <v>1942.78</v>
+      </c>
+      <c r="G619">
+        <v>50.64884617222906</v>
+      </c>
+      <c r="H619">
+        <v>3.97</v>
+      </c>
+      <c r="I619">
+        <v>0</v>
+      </c>
+      <c r="J619">
+        <v>0</v>
+      </c>
+      <c r="K619">
+        <v>0.1034990679869822</v>
+      </c>
+      <c r="L619">
+        <v>0</v>
+      </c>
+      <c r="M619">
+        <v>0</v>
+      </c>
+      <c r="N619">
+        <v>0</v>
+      </c>
+      <c r="O619">
+        <v>21.50489</v>
+      </c>
+      <c r="P619">
+        <v>59.73580555555556</v>
+      </c>
+      <c r="Q619">
+        <v>36</v>
+      </c>
+      <c r="R619">
+        <v>256.40185</v>
+      </c>
+      <c r="S619">
+        <v>6.684471663762727</v>
+      </c>
+      <c r="T619">
+        <v>138.48</v>
+      </c>
+      <c r="U619">
+        <v>3</v>
+      </c>
+      <c r="V619">
+        <v>3</v>
+      </c>
+      <c r="W619">
+        <v>6</v>
+      </c>
+      <c r="X619">
+        <v>22</v>
+      </c>
+      <c r="Y619">
+        <v>3</v>
+      </c>
+      <c r="Z619">
+        <v>13</v>
+      </c>
+      <c r="AA619">
+        <v>3</v>
+      </c>
+      <c r="AB619">
+        <v>2</v>
+      </c>
+      <c r="AC619">
+        <v>3.67352</v>
+      </c>
+      <c r="AD619">
+        <v>-3.1004</v>
+      </c>
+      <c r="AE619">
+        <v>0</v>
+      </c>
+      <c r="AF619">
+        <v>444.682</v>
+      </c>
+      <c r="AG619">
+        <v>0</v>
+      </c>
+      <c r="AH619">
+        <v>3</v>
+      </c>
+      <c r="AI619">
+        <v>769.2055500000001</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B620" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E620">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F620">
+        <v>11391.64</v>
+      </c>
+      <c r="G620">
+        <v>84.51952362286026</v>
+      </c>
+      <c r="H620">
+        <v>425.99</v>
+      </c>
+      <c r="I620">
+        <v>0</v>
+      </c>
+      <c r="J620">
+        <v>0</v>
+      </c>
+      <c r="K620">
+        <v>3.160604782814611</v>
+      </c>
+      <c r="L620">
+        <v>0</v>
+      </c>
+      <c r="M620">
+        <v>10</v>
+      </c>
+      <c r="N620">
+        <v>0</v>
+      </c>
+      <c r="O620">
+        <v>29.36677</v>
+      </c>
+      <c r="P620">
+        <v>86.41351812617701</v>
+      </c>
+      <c r="Q620">
+        <v>33.984</v>
+      </c>
+      <c r="R620">
+        <v>1096.91899</v>
+      </c>
+      <c r="S620">
+        <v>8.138518289523635</v>
+      </c>
+      <c r="T620">
+        <v>1591.07</v>
+      </c>
+      <c r="U620">
+        <v>22</v>
+      </c>
+      <c r="V620">
+        <v>45</v>
+      </c>
+      <c r="W620">
+        <v>67</v>
+      </c>
+      <c r="X620">
+        <v>108</v>
+      </c>
+      <c r="Y620">
+        <v>22</v>
+      </c>
+      <c r="Z620">
+        <v>130</v>
+      </c>
+      <c r="AA620">
+        <v>45</v>
+      </c>
+      <c r="AB620">
+        <v>40</v>
+      </c>
+      <c r="AC620">
+        <v>3.90336</v>
+      </c>
+      <c r="AD620">
+        <v>-4.04098</v>
+      </c>
+      <c r="AE620">
+        <v>74.2</v>
+      </c>
+      <c r="AF620">
+        <v>1061.1992</v>
+      </c>
+      <c r="AG620">
+        <v>0</v>
+      </c>
+      <c r="AH620">
+        <v>3</v>
+      </c>
+      <c r="AI620">
+        <v>3290.75697</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B621" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E621">
+        <v>38.35783333333333</v>
+      </c>
+      <c r="F621">
+        <v>2173.77</v>
+      </c>
+      <c r="G621">
+        <v>56.67082343024241</v>
+      </c>
+      <c r="H621">
+        <v>4.41</v>
+      </c>
+      <c r="I621">
+        <v>0</v>
+      </c>
+      <c r="J621">
+        <v>0</v>
+      </c>
+      <c r="K621">
+        <v>0.1149699974364211</v>
+      </c>
+      <c r="L621">
+        <v>0</v>
+      </c>
+      <c r="M621">
+        <v>0</v>
+      </c>
+      <c r="N621">
+        <v>0</v>
+      </c>
+      <c r="O621">
+        <v>21.77638</v>
+      </c>
+      <c r="P621">
+        <v>62.23245313214449</v>
+      </c>
+      <c r="Q621">
+        <v>34.992</v>
+      </c>
+      <c r="R621">
+        <v>241.66652</v>
+      </c>
+      <c r="S621">
+        <v>6.300317275480454</v>
+      </c>
+      <c r="T621">
+        <v>159</v>
+      </c>
+      <c r="U621">
+        <v>7</v>
+      </c>
+      <c r="V621">
+        <v>4</v>
+      </c>
+      <c r="W621">
+        <v>11</v>
+      </c>
+      <c r="X621">
+        <v>23</v>
+      </c>
+      <c r="Y621">
+        <v>7</v>
+      </c>
+      <c r="Z621">
+        <v>16</v>
+      </c>
+      <c r="AA621">
+        <v>4</v>
+      </c>
+      <c r="AB621">
+        <v>4</v>
+      </c>
+      <c r="AC621">
+        <v>4.14587</v>
+      </c>
+      <c r="AD621">
+        <v>-2.88379</v>
+      </c>
+      <c r="AE621">
+        <v>0</v>
+      </c>
+      <c r="AF621">
+        <v>202.2376</v>
+      </c>
+      <c r="AG621">
+        <v>0</v>
+      </c>
+      <c r="AH621">
+        <v>3</v>
+      </c>
+      <c r="AI621">
+        <v>724.99956</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B622" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E622">
+        <v>134.7811666666667</v>
+      </c>
+      <c r="F622">
+        <v>11377.37</v>
+      </c>
+      <c r="G622">
+        <v>84.41364829655973</v>
+      </c>
+      <c r="H622">
+        <v>491.89</v>
+      </c>
+      <c r="I622">
+        <v>0</v>
+      </c>
+      <c r="J622">
+        <v>0</v>
+      </c>
+      <c r="K622">
+        <v>3.649545497825487</v>
+      </c>
+      <c r="L622">
+        <v>0</v>
+      </c>
+      <c r="M622">
+        <v>4</v>
+      </c>
+      <c r="N622">
+        <v>0</v>
+      </c>
+      <c r="O622">
+        <v>27.12986</v>
+      </c>
+      <c r="P622">
+        <v>82.18181267417908</v>
+      </c>
+      <c r="Q622">
+        <v>33.012</v>
+      </c>
+      <c r="R622">
+        <v>1063.97135</v>
+      </c>
+      <c r="S622">
+        <v>7.894065441882953</v>
+      </c>
+      <c r="T622">
+        <v>1629.74998</v>
+      </c>
+      <c r="U622">
+        <v>34</v>
+      </c>
+      <c r="V622">
+        <v>41</v>
+      </c>
+      <c r="W622">
+        <v>75</v>
+      </c>
+      <c r="X622">
+        <v>132</v>
+      </c>
+      <c r="Y622">
+        <v>34</v>
+      </c>
+      <c r="Z622">
+        <v>116</v>
+      </c>
+      <c r="AA622">
+        <v>41</v>
+      </c>
+      <c r="AB622">
+        <v>59</v>
+      </c>
+      <c r="AC622">
+        <v>4.29236</v>
+      </c>
+      <c r="AD622">
+        <v>-3.69383</v>
+      </c>
+      <c r="AE622">
+        <v>0</v>
+      </c>
+      <c r="AF622">
+        <v>993.0172500000001</v>
+      </c>
+      <c r="AG622">
+        <v>0</v>
+      </c>
+      <c r="AH622">
+        <v>3</v>
+      </c>
+      <c r="AI622">
+        <v>3191.91405</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B623" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E623">
+        <v>125.0045</v>
+      </c>
+      <c r="F623">
+        <v>11505.3</v>
+      </c>
+      <c r="G623">
+        <v>92.03908659288264</v>
+      </c>
+      <c r="H623">
+        <v>507.15</v>
+      </c>
+      <c r="I623">
+        <v>19.69</v>
+      </c>
+      <c r="J623">
+        <v>2</v>
+      </c>
+      <c r="K623">
+        <v>4.057053946057941</v>
+      </c>
+      <c r="L623">
+        <v>1.66</v>
+      </c>
+      <c r="M623">
+        <v>9</v>
+      </c>
+      <c r="N623">
+        <v>0</v>
+      </c>
+      <c r="O623">
+        <v>29.89055</v>
+      </c>
+      <c r="P623">
+        <v>93.39629421322336</v>
+      </c>
+      <c r="Q623">
+        <v>32.004</v>
+      </c>
+      <c r="R623">
+        <v>1042.4873</v>
+      </c>
+      <c r="S623">
+        <v>8.339598174465719</v>
+      </c>
+      <c r="T623">
+        <v>1776.4</v>
+      </c>
+      <c r="U623">
+        <v>18</v>
+      </c>
+      <c r="V623">
+        <v>28</v>
+      </c>
+      <c r="W623">
+        <v>46</v>
+      </c>
+      <c r="X623">
+        <v>138</v>
+      </c>
+      <c r="Y623">
+        <v>18</v>
+      </c>
+      <c r="Z623">
+        <v>102</v>
+      </c>
+      <c r="AA623">
+        <v>28</v>
+      </c>
+      <c r="AB623">
+        <v>29</v>
+      </c>
+      <c r="AC623">
+        <v>4.26276</v>
+      </c>
+      <c r="AD623">
+        <v>-4.42349</v>
+      </c>
+      <c r="AE623">
+        <v>0</v>
+      </c>
+      <c r="AF623">
+        <v>939.4286999999999</v>
+      </c>
+      <c r="AG623">
+        <v>0</v>
+      </c>
+      <c r="AH623">
+        <v>3</v>
+      </c>
+      <c r="AI623">
+        <v>3127.4619</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B624" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Partido vs Querétaro J1</t>
+        </is>
+      </c>
+      <c r="E624">
+        <v>38.35783333333333</v>
+      </c>
+      <c r="F624">
+        <v>1977.68</v>
+      </c>
+      <c r="G624">
+        <v>51.55869943992318</v>
+      </c>
+      <c r="H624">
+        <v>0</v>
+      </c>
+      <c r="I624">
+        <v>0</v>
+      </c>
+      <c r="J624">
+        <v>0</v>
+      </c>
+      <c r="K624">
+        <v>0</v>
+      </c>
+      <c r="L624">
+        <v>0</v>
+      </c>
+      <c r="M624">
+        <v>0</v>
+      </c>
+      <c r="N624">
+        <v>0</v>
+      </c>
+      <c r="O624">
+        <v>19.77327</v>
+      </c>
+      <c r="P624">
+        <v>54.92574999999999</v>
+      </c>
+      <c r="Q624">
+        <v>36</v>
+      </c>
+      <c r="R624">
+        <v>234.21619</v>
+      </c>
+      <c r="S624">
+        <v>6.106084980469005</v>
+      </c>
+      <c r="T624">
+        <v>124.19</v>
+      </c>
+      <c r="U624">
+        <v>5</v>
+      </c>
+      <c r="V624">
+        <v>4</v>
+      </c>
+      <c r="W624">
+        <v>9</v>
+      </c>
+      <c r="X624">
+        <v>21</v>
+      </c>
+      <c r="Y624">
+        <v>5</v>
+      </c>
+      <c r="Z624">
+        <v>20</v>
+      </c>
+      <c r="AA624">
+        <v>4</v>
+      </c>
+      <c r="AB624">
+        <v>3</v>
+      </c>
+      <c r="AC624">
+        <v>4.01925</v>
+      </c>
+      <c r="AD624">
+        <v>-3.00238</v>
+      </c>
+      <c r="AE624">
+        <v>0</v>
+      </c>
+      <c r="AF624">
+        <v>448.192</v>
+      </c>
+      <c r="AG624">
+        <v>0</v>
+      </c>
+      <c r="AH624">
+        <v>3</v>
+      </c>
+      <c r="AI624">
+        <v>702.6485700000001</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B625" s="2">
+        <v>46221</v>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E625">
+        <v>104.4666666666667</v>
+      </c>
+      <c r="F625">
+        <v>8747.59</v>
+      </c>
+      <c r="G625">
+        <v>83.73570516911296</v>
+      </c>
+      <c r="H625">
+        <v>293.03</v>
+      </c>
+      <c r="I625">
+        <v>0</v>
+      </c>
+      <c r="J625">
+        <v>0</v>
+      </c>
+      <c r="K625">
+        <v>2.805009572431397</v>
+      </c>
+      <c r="L625">
+        <v>0</v>
+      </c>
+      <c r="M625">
+        <v>4</v>
+      </c>
+      <c r="N625">
+        <v>0</v>
+      </c>
+      <c r="O625">
+        <v>28.00712</v>
+      </c>
+      <c r="P625">
+        <v>80.03863740283495</v>
+      </c>
+      <c r="Q625">
+        <v>34.992</v>
+      </c>
+      <c r="R625">
+        <v>852.92335</v>
+      </c>
+      <c r="S625">
+        <v>8.164550255264837</v>
+      </c>
+      <c r="T625">
+        <v>1296.66</v>
+      </c>
+      <c r="U625">
+        <v>32</v>
+      </c>
+      <c r="V625">
+        <v>42</v>
+      </c>
+      <c r="W625">
+        <v>74</v>
+      </c>
+      <c r="X625">
+        <v>162</v>
+      </c>
+      <c r="Y625">
+        <v>32</v>
+      </c>
+      <c r="Z625">
+        <v>126</v>
+      </c>
+      <c r="AA625">
+        <v>42</v>
+      </c>
+      <c r="AB625">
+        <v>55</v>
+      </c>
+      <c r="AC625">
+        <v>4.24346</v>
+      </c>
+      <c r="AD625">
+        <v>-4.07517</v>
+      </c>
+      <c r="AE625">
+        <v>0</v>
+      </c>
+      <c r="AF625">
+        <v>837.8408000000001</v>
+      </c>
+      <c r="AG625">
+        <v>0</v>
+      </c>
+      <c r="AH625">
+        <v>3</v>
+      </c>
+      <c r="AI625">
+        <v>2558.77005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-20
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -68587,13 +68587,13 @@
         </is>
       </c>
       <c r="E605">
-        <v>55.943</v>
+        <v>43.16583333333333</v>
       </c>
       <c r="F605">
-        <v>2595.27</v>
+        <v>2449.04</v>
       </c>
       <c r="G605">
-        <v>46.39132688629498</v>
+        <v>56.735612656615</v>
       </c>
       <c r="H605">
         <v>24.64</v>
@@ -68605,7 +68605,7 @@
         <v>0</v>
       </c>
       <c r="K605">
-        <v>0.4404483134619165</v>
+        <v>0.570821830537269</v>
       </c>
       <c r="L605">
         <v>0</v>
@@ -68626,13 +68626,13 @@
         <v>36</v>
       </c>
       <c r="R605">
-        <v>282.17018</v>
+        <v>249.93645</v>
       </c>
       <c r="S605">
-        <v>5.043887170870351</v>
+        <v>5.79014536960173</v>
       </c>
       <c r="T605">
-        <v>195.59</v>
+        <v>190.96</v>
       </c>
       <c r="U605">
         <v>6</v>
@@ -68644,7 +68644,7 @@
         <v>10</v>
       </c>
       <c r="X605">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Y605">
         <v>6</v>
@@ -68668,7 +68668,7 @@
         <v>0</v>
       </c>
       <c r="AF605">
-        <v>578.516</v>
+        <v>553.668</v>
       </c>
       <c r="AG605">
         <v>0</v>
@@ -68677,7 +68677,7 @@
         <v>3</v>
       </c>
       <c r="AI605">
-        <v>846.51054</v>
+        <v>749.80935</v>
       </c>
     </row>
     <row r="606">
@@ -68700,13 +68700,13 @@
         </is>
       </c>
       <c r="E606">
-        <v>68.61016666666666</v>
+        <v>62.62833333333333</v>
       </c>
       <c r="F606">
-        <v>4435.42</v>
+        <v>4254.17</v>
       </c>
       <c r="G606">
-        <v>64.64668744428062</v>
+        <v>67.92724272826463</v>
       </c>
       <c r="H606">
         <v>246.04</v>
@@ -68718,7 +68718,7 @@
         <v>2</v>
       </c>
       <c r="K606">
-        <v>3.586057459900258</v>
+        <v>3.928573329430237</v>
       </c>
       <c r="L606">
         <v>8.9</v>
@@ -68739,34 +68739,34 @@
         <v>32.4</v>
       </c>
       <c r="R606">
-        <v>473.45646</v>
+        <v>453.95698</v>
       </c>
       <c r="S606">
-        <v>6.900674972853878</v>
+        <v>7.248428240679139</v>
       </c>
       <c r="T606">
-        <v>746.9499900000001</v>
+        <v>708.38999</v>
       </c>
       <c r="U606">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V606">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W606">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="X606">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="Y606">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z606">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="AA606">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB606">
         <v>10</v>
@@ -68781,7 +68781,7 @@
         <v>0</v>
       </c>
       <c r="AF606">
-        <v>360.3964</v>
+        <v>345.0811</v>
       </c>
       <c r="AG606">
         <v>0</v>
@@ -68790,7 +68790,7 @@
         <v>3</v>
       </c>
       <c r="AI606">
-        <v>1420.36938</v>
+        <v>1361.87094</v>
       </c>
     </row>
     <row r="607">
@@ -69491,13 +69491,13 @@
         </is>
       </c>
       <c r="E613">
-        <v>134.7811666666667</v>
+        <v>130.3266666666667</v>
       </c>
       <c r="F613">
-        <v>10533.85</v>
+        <v>10491.18</v>
       </c>
       <c r="G613">
-        <v>78.1552071444205</v>
+        <v>80.49910481354544</v>
       </c>
       <c r="H613">
         <v>467.37</v>
@@ -69509,7 +69509,7 @@
         <v>0</v>
       </c>
       <c r="K613">
-        <v>3.467620970783504</v>
+        <v>3.586142513683564</v>
       </c>
       <c r="L613">
         <v>0</v>
@@ -69530,10 +69530,10 @@
         <v>33.696</v>
       </c>
       <c r="R613">
-        <v>1152.26028</v>
+        <v>1147.27872</v>
       </c>
       <c r="S613">
-        <v>8.549119350255413</v>
+        <v>8.80310031203642</v>
       </c>
       <c r="T613">
         <v>1647.3</v>
@@ -69572,7 +69572,7 @@
         <v>0</v>
       </c>
       <c r="AF613">
-        <v>1019.2528</v>
+        <v>1016.2848</v>
       </c>
       <c r="AG613">
         <v>0</v>
@@ -69581,7 +69581,7 @@
         <v>3</v>
       </c>
       <c r="AI613">
-        <v>3456.78084</v>
+        <v>3441.83616</v>
       </c>
     </row>
     <row r="614">
@@ -69604,13 +69604,13 @@
         </is>
       </c>
       <c r="E614">
-        <v>94.60316666666667</v>
+        <v>50.65283333333333</v>
       </c>
       <c r="F614">
-        <v>4047.920000000001</v>
+        <v>3275.15</v>
       </c>
       <c r="G614">
-        <v>42.78841969701508</v>
+        <v>64.65877196734635</v>
       </c>
       <c r="H614">
         <v>138.79</v>
@@ -69622,7 +69622,7 @@
         <v>0</v>
       </c>
       <c r="K614">
-        <v>1.467075626432519</v>
+        <v>2.740024414560554</v>
       </c>
       <c r="L614">
         <v>0</v>
@@ -69643,37 +69643,37 @@
         <v>36</v>
       </c>
       <c r="R614">
-        <v>558.0625700000001</v>
+        <v>441.20237</v>
       </c>
       <c r="S614">
-        <v>5.89898403682752</v>
+        <v>8.710319659643917</v>
       </c>
       <c r="T614">
-        <v>538.88999</v>
+        <v>404.94001</v>
       </c>
       <c r="U614">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="V614">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="W614">
+        <v>13</v>
+      </c>
+      <c r="X614">
+        <v>31</v>
+      </c>
+      <c r="Y614">
+        <v>8</v>
+      </c>
+      <c r="Z614">
         <v>25</v>
       </c>
-      <c r="X614">
-        <v>50</v>
-      </c>
-      <c r="Y614">
-        <v>14</v>
-      </c>
-      <c r="Z614">
-        <v>41</v>
-      </c>
       <c r="AA614">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="AB614">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="AC614">
         <v>4.81753</v>
@@ -69685,7 +69685,7 @@
         <v>0</v>
       </c>
       <c r="AF614">
-        <v>934.296</v>
+        <v>741.23</v>
       </c>
       <c r="AG614">
         <v>0</v>
@@ -69694,7 +69694,7 @@
         <v>3</v>
       </c>
       <c r="AI614">
-        <v>1674.18771</v>
+        <v>1323.60711</v>
       </c>
     </row>
     <row r="615">

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-23
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI676"/>
+  <dimension ref="A1:AI701"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -74014,10 +74014,10 @@
         <v>67.649</v>
       </c>
       <c r="F653">
-        <v>4048.39</v>
+        <v>4048.550000000001</v>
       </c>
       <c r="G653">
-        <v>59.84404795340656</v>
+        <v>59.84641310292836</v>
       </c>
       <c r="H653">
         <v>153.25</v>
@@ -74050,10 +74050,10 @@
         <v>36</v>
       </c>
       <c r="R653">
-        <v>416.70803</v>
+        <v>416.71587</v>
       </c>
       <c r="S653">
-        <v>6.159854986769945</v>
+        <v>6.159970879096512</v>
       </c>
       <c r="T653">
         <v>784.1500100000001</v>
@@ -74092,7 +74092,7 @@
         <v>0</v>
       </c>
       <c r="AF653">
-        <v>990.884</v>
+        <v>990.9159999999999</v>
       </c>
       <c r="AG653">
         <v>0</v>
@@ -74101,7 +74101,7 @@
         <v>3</v>
       </c>
       <c r="AI653">
-        <v>1250.12409</v>
+        <v>1250.14761</v>
       </c>
     </row>
     <row r="654">
@@ -74127,10 +74127,10 @@
         <v>122.5821666666667</v>
       </c>
       <c r="F654">
-        <v>6409.95</v>
+        <v>6410.25</v>
       </c>
       <c r="G654">
-        <v>52.29104831725115</v>
+        <v>52.29349565529515</v>
       </c>
       <c r="H654">
         <v>542.8</v>
@@ -74163,10 +74163,10 @@
         <v>32.364</v>
       </c>
       <c r="R654">
-        <v>669.5530200000001</v>
+        <v>669.56059</v>
       </c>
       <c r="S654">
-        <v>5.462075261083383</v>
+        <v>5.462137015580026</v>
       </c>
       <c r="T654">
         <v>1057.09999</v>
@@ -74205,7 +74205,7 @@
         <v>0</v>
       </c>
       <c r="AF654">
-        <v>525.5712</v>
+        <v>525.5922</v>
       </c>
       <c r="AG654">
         <v>0</v>
@@ -74214,7 +74214,7 @@
         <v>3</v>
       </c>
       <c r="AI654">
-        <v>2008.65906</v>
+        <v>2008.68177</v>
       </c>
     </row>
     <row r="655">
@@ -74240,10 +74240,10 @@
         <v>67.649</v>
       </c>
       <c r="F655">
-        <v>4040.63</v>
+        <v>4040.75</v>
       </c>
       <c r="G655">
-        <v>59.72933820159943</v>
+        <v>59.73111206374078</v>
       </c>
       <c r="H655">
         <v>150.4</v>
@@ -74276,10 +74276,10 @@
         <v>36</v>
       </c>
       <c r="R655">
-        <v>328.22033</v>
+        <v>328.22489</v>
       </c>
       <c r="S655">
-        <v>4.851813478395838</v>
+        <v>4.851880885157208</v>
       </c>
       <c r="T655">
         <v>778.41</v>
@@ -74318,7 +74318,7 @@
         <v>0</v>
       </c>
       <c r="AF655">
-        <v>1005.164</v>
+        <v>1005.194</v>
       </c>
       <c r="AG655">
         <v>0</v>
@@ -74327,7 +74327,7 @@
         <v>3</v>
       </c>
       <c r="AI655">
-        <v>984.66099</v>
+        <v>984.6746700000001</v>
       </c>
     </row>
     <row r="656">
@@ -74353,10 +74353,10 @@
         <v>67.649</v>
       </c>
       <c r="F656">
-        <v>4336.389999999999</v>
+        <v>4336.610000000001</v>
       </c>
       <c r="G656">
-        <v>64.10131709263995</v>
+        <v>64.10456917323243</v>
       </c>
       <c r="H656">
         <v>368.89</v>
@@ -74389,10 +74389,10 @@
         <v>32.4</v>
       </c>
       <c r="R656">
-        <v>447.5913</v>
+        <v>447.59845</v>
       </c>
       <c r="S656">
-        <v>6.616377182219989</v>
+        <v>6.616482874839243</v>
       </c>
       <c r="T656">
         <v>961.5700400000001</v>
@@ -74431,7 +74431,7 @@
         <v>0</v>
       </c>
       <c r="AF656">
-        <v>370.2538</v>
+        <v>370.2671</v>
       </c>
       <c r="AG656">
         <v>0</v>
@@ -74440,7 +74440,7 @@
         <v>3</v>
       </c>
       <c r="AI656">
-        <v>1342.7739</v>
+        <v>1342.79535</v>
       </c>
     </row>
     <row r="657">
@@ -74466,10 +74466,10 @@
         <v>130.8268333333333</v>
       </c>
       <c r="F657">
-        <v>7691.87</v>
+        <v>7691.98</v>
       </c>
       <c r="G657">
-        <v>58.79428404723292</v>
+        <v>58.79512485333667</v>
       </c>
       <c r="H657">
         <v>682.6</v>
@@ -74502,10 +74502,10 @@
         <v>35.604</v>
       </c>
       <c r="R657">
-        <v>728.7044100000001</v>
+        <v>728.7228</v>
       </c>
       <c r="S657">
-        <v>5.569991961384069</v>
+        <v>5.570132528877231</v>
       </c>
       <c r="T657">
         <v>1483.42</v>
@@ -74544,7 +74544,7 @@
         <v>0</v>
       </c>
       <c r="AF657">
-        <v>659.79732</v>
+        <v>659.80513</v>
       </c>
       <c r="AG657">
         <v>0</v>
@@ -74553,7 +74553,7 @@
         <v>3</v>
       </c>
       <c r="AI657">
-        <v>2186.11323</v>
+        <v>2186.1684</v>
       </c>
     </row>
     <row r="658">
@@ -74579,10 +74579,10 @@
         <v>67.649</v>
       </c>
       <c r="F658">
-        <v>4580.61</v>
+        <v>4580.96</v>
       </c>
       <c r="G658">
-        <v>67.71142219397181</v>
+        <v>67.71659595855076</v>
       </c>
       <c r="H658">
         <v>374.86</v>
@@ -74615,10 +74615,10 @@
         <v>33.984</v>
       </c>
       <c r="R658">
-        <v>531.98754</v>
+        <v>532.0191</v>
       </c>
       <c r="S658">
-        <v>7.86393797395379</v>
+        <v>7.864404499696965</v>
       </c>
       <c r="T658">
         <v>931.73002</v>
@@ -74657,7 +74657,7 @@
         <v>0</v>
       </c>
       <c r="AF658">
-        <v>443.3711999999999</v>
+        <v>443.4152</v>
       </c>
       <c r="AG658">
         <v>0</v>
@@ -74666,7 +74666,7 @@
         <v>3</v>
       </c>
       <c r="AI658">
-        <v>1595.96262</v>
+        <v>1596.0573</v>
       </c>
     </row>
     <row r="659">
@@ -74692,10 +74692,10 @@
         <v>67.649</v>
       </c>
       <c r="F659">
-        <v>4871.309999999999</v>
+        <v>4871.42</v>
       </c>
       <c r="G659">
-        <v>72.00860323138552</v>
+        <v>72.01022927168177</v>
       </c>
       <c r="H659">
         <v>345.73</v>
@@ -74728,10 +74728,10 @@
         <v>35.568</v>
       </c>
       <c r="R659">
-        <v>424.16783</v>
+        <v>424.1818</v>
       </c>
       <c r="S659">
-        <v>6.270127126786797</v>
+        <v>6.270333633904419</v>
       </c>
       <c r="T659">
         <v>946.5200100000001</v>
@@ -74770,7 +74770,7 @@
         <v>0</v>
       </c>
       <c r="AF659">
-        <v>475.6512</v>
+        <v>475.6616</v>
       </c>
       <c r="AG659">
         <v>0</v>
@@ -74779,7 +74779,7 @@
         <v>3</v>
       </c>
       <c r="AI659">
-        <v>1272.50349</v>
+        <v>1272.5454</v>
       </c>
     </row>
     <row r="660">
@@ -74805,10 +74805,10 @@
         <v>67.649</v>
       </c>
       <c r="F660">
-        <v>4661.74</v>
+        <v>4662.12</v>
       </c>
       <c r="G660">
-        <v>68.91070082336768</v>
+        <v>68.91631805348194</v>
       </c>
       <c r="H660">
         <v>339.34</v>
@@ -74841,10 +74841,10 @@
         <v>36</v>
       </c>
       <c r="R660">
-        <v>470.47241</v>
+        <v>470.49717</v>
       </c>
       <c r="S660">
-        <v>6.954609972061671</v>
+        <v>6.954975978950169</v>
       </c>
       <c r="T660">
         <v>929.08</v>
@@ -74883,7 +74883,7 @@
         <v>0</v>
       </c>
       <c r="AF660">
-        <v>1124.126</v>
+        <v>1124.204</v>
       </c>
       <c r="AG660">
         <v>0</v>
@@ -74892,7 +74892,7 @@
         <v>3</v>
       </c>
       <c r="AI660">
-        <v>1411.41723</v>
+        <v>1411.49151</v>
       </c>
     </row>
     <row r="661">
@@ -74918,10 +74918,10 @@
         <v>67.649</v>
       </c>
       <c r="F661">
-        <v>4968.26</v>
+        <v>4968.35</v>
       </c>
       <c r="G661">
-        <v>73.441736019749</v>
+        <v>73.44306641635501</v>
       </c>
       <c r="H661">
         <v>352.6399999999999</v>
@@ -74954,10 +74954,10 @@
         <v>36</v>
       </c>
       <c r="R661">
-        <v>447.25489</v>
+        <v>447.25901</v>
       </c>
       <c r="S661">
-        <v>6.611404307528566</v>
+        <v>6.611465210128753</v>
       </c>
       <c r="T661">
         <v>954.71001</v>
@@ -74996,7 +74996,7 @@
         <v>0</v>
       </c>
       <c r="AF661">
-        <v>413.5642</v>
+        <v>413.5726</v>
       </c>
       <c r="AG661">
         <v>0</v>
@@ -75005,7 +75005,7 @@
         <v>3</v>
       </c>
       <c r="AI661">
-        <v>1341.76467</v>
+        <v>1341.77703</v>
       </c>
     </row>
     <row r="662">
@@ -75031,10 +75031,10 @@
         <v>67.649</v>
       </c>
       <c r="F662">
-        <v>4578.64</v>
+        <v>4578.88</v>
       </c>
       <c r="G662">
-        <v>67.68230129048472</v>
+        <v>67.6858490147674</v>
       </c>
       <c r="H662">
         <v>264.34</v>
@@ -75067,10 +75067,10 @@
         <v>32.004</v>
       </c>
       <c r="R662">
-        <v>484.85566</v>
+        <v>484.87434</v>
       </c>
       <c r="S662">
-        <v>7.167225827432778</v>
+        <v>7.167501958639448</v>
       </c>
       <c r="T662">
         <v>869.39998</v>
@@ -75109,7 +75109,7 @@
         <v>0</v>
       </c>
       <c r="AF662">
-        <v>329.1864</v>
+        <v>329.2092</v>
       </c>
       <c r="AG662">
         <v>0</v>
@@ -75118,7 +75118,7 @@
         <v>3</v>
       </c>
       <c r="AI662">
-        <v>1454.56698</v>
+        <v>1454.62302</v>
       </c>
     </row>
     <row r="663">
@@ -75144,10 +75144,10 @@
         <v>67.649</v>
       </c>
       <c r="F663">
-        <v>4327.43</v>
+        <v>4327.52</v>
       </c>
       <c r="G663">
-        <v>63.96886871941936</v>
+        <v>63.97019911602536</v>
       </c>
       <c r="H663">
         <v>308.29</v>
@@ -75180,10 +75180,10 @@
         <v>33.84</v>
       </c>
       <c r="R663">
-        <v>423.9985</v>
+        <v>424.01584</v>
       </c>
       <c r="S663">
-        <v>6.26762405948351</v>
+        <v>6.267880382562935</v>
       </c>
       <c r="T663">
         <v>834.01</v>
@@ -75222,7 +75222,7 @@
         <v>0</v>
       </c>
       <c r="AF663">
-        <v>364.0868</v>
+        <v>364.0959</v>
       </c>
       <c r="AG663">
         <v>0</v>
@@ -75231,7 +75231,7 @@
         <v>3</v>
       </c>
       <c r="AI663">
-        <v>1271.9955</v>
+        <v>1272.04752</v>
       </c>
     </row>
     <row r="664">
@@ -75257,10 +75257,10 @@
         <v>67.649</v>
       </c>
       <c r="F664">
-        <v>4259.539999999999</v>
+        <v>4259.679999999999</v>
       </c>
       <c r="G664">
-        <v>62.96530621295214</v>
+        <v>62.96737571878371</v>
       </c>
       <c r="H664">
         <v>177.21</v>
@@ -75293,10 +75293,10 @@
         <v>33.696</v>
       </c>
       <c r="R664">
-        <v>407.409</v>
+        <v>407.41456</v>
       </c>
       <c r="S664">
-        <v>6.022395009534509</v>
+        <v>6.022477198480392</v>
       </c>
       <c r="T664">
         <v>861.0999999999999</v>
@@ -75335,7 +75335,7 @@
         <v>0</v>
       </c>
       <c r="AF664">
-        <v>421.9224</v>
+        <v>421.9344</v>
       </c>
       <c r="AG664">
         <v>0</v>
@@ -75344,7 +75344,7 @@
         <v>3</v>
       </c>
       <c r="AI664">
-        <v>1222.227</v>
+        <v>1222.24368</v>
       </c>
     </row>
     <row r="665">
@@ -75370,10 +75370,10 @@
         <v>67.649</v>
       </c>
       <c r="F665">
-        <v>4966.95</v>
+        <v>4967.12</v>
       </c>
       <c r="G665">
-        <v>73.42237135803929</v>
+        <v>73.4248843294062</v>
       </c>
       <c r="H665">
         <v>452.1199999999999</v>
@@ -75406,10 +75406,10 @@
         <v>36</v>
       </c>
       <c r="R665">
-        <v>542.59665</v>
+        <v>542.60815</v>
       </c>
       <c r="S665">
-        <v>8.020763795473695</v>
+        <v>8.020933790595574</v>
       </c>
       <c r="T665">
         <v>1108.60001</v>
@@ -75448,7 +75448,7 @@
         <v>0</v>
       </c>
       <c r="AF665">
-        <v>1217.064</v>
+        <v>1217.11</v>
       </c>
       <c r="AG665">
         <v>0</v>
@@ -75457,7 +75457,7 @@
         <v>3</v>
       </c>
       <c r="AI665">
-        <v>1627.78995</v>
+        <v>1627.82445</v>
       </c>
     </row>
     <row r="666">
@@ -75483,10 +75483,10 @@
         <v>67.649</v>
       </c>
       <c r="F666">
-        <v>5079.849999999999</v>
+        <v>5079.889999999999</v>
       </c>
       <c r="G666">
-        <v>75.09127998935682</v>
+        <v>75.09187127673727</v>
       </c>
       <c r="H666">
         <v>421.29</v>
@@ -75519,10 +75519,10 @@
         <v>34.992</v>
       </c>
       <c r="R666">
-        <v>473.36208</v>
+        <v>473.3663</v>
       </c>
       <c r="S666">
-        <v>6.997325607178229</v>
+        <v>6.997387987996866</v>
       </c>
       <c r="T666">
         <v>1005.88998</v>
@@ -75561,7 +75561,7 @@
         <v>0</v>
       </c>
       <c r="AF666">
-        <v>420.5343</v>
+        <v>420.53913</v>
       </c>
       <c r="AG666">
         <v>0</v>
@@ -75570,7 +75570,7 @@
         <v>3</v>
       </c>
       <c r="AI666">
-        <v>1420.08624</v>
+        <v>1420.0989</v>
       </c>
     </row>
     <row r="667">
@@ -75596,10 +75596,10 @@
         <v>130.8268333333333</v>
       </c>
       <c r="F667">
-        <v>8256.040000000001</v>
+        <v>8256.059999999999</v>
       </c>
       <c r="G667">
-        <v>63.10662567949237</v>
+        <v>63.1067785533294</v>
       </c>
       <c r="H667">
         <v>641.25</v>
@@ -75632,10 +75632,10 @@
         <v>33.012</v>
       </c>
       <c r="R667">
-        <v>968.4603999999999</v>
+        <v>968.46488</v>
       </c>
       <c r="S667">
-        <v>7.402612868664812</v>
+        <v>7.402647112404311</v>
       </c>
       <c r="T667">
         <v>1437.71001</v>
@@ -75674,7 +75674,7 @@
         <v>0</v>
       </c>
       <c r="AF667">
-        <v>769.8132000000001</v>
+        <v>769.81398</v>
       </c>
       <c r="AG667">
         <v>0</v>
@@ -75683,7 +75683,7 @@
         <v>3</v>
       </c>
       <c r="AI667">
-        <v>2905.3812</v>
+        <v>2905.39464</v>
       </c>
     </row>
     <row r="668">
@@ -75709,10 +75709,10 @@
         <v>67.649</v>
       </c>
       <c r="F668">
-        <v>4521.14</v>
+        <v>4521.3</v>
       </c>
       <c r="G668">
-        <v>66.83232568108916</v>
+        <v>66.83469083061095</v>
       </c>
       <c r="H668">
         <v>316.34</v>
@@ -75745,10 +75745,10 @@
         <v>34.992</v>
       </c>
       <c r="R668">
-        <v>369.40985</v>
+        <v>369.41493</v>
       </c>
       <c r="S668">
-        <v>5.460684562964714</v>
+        <v>5.460759656462032</v>
       </c>
       <c r="T668">
         <v>1023.48002</v>
@@ -75787,7 +75787,7 @@
         <v>0</v>
       </c>
       <c r="AF668">
-        <v>397.2947</v>
+        <v>397.30393</v>
       </c>
       <c r="AG668">
         <v>0</v>
@@ -75796,7 +75796,7 @@
         <v>3</v>
       </c>
       <c r="AI668">
-        <v>1108.22955</v>
+        <v>1108.24479</v>
       </c>
     </row>
     <row r="669">
@@ -75822,10 +75822,10 @@
         <v>56.21299999999999</v>
       </c>
       <c r="F669">
-        <v>3637.55</v>
+        <v>3637.79</v>
       </c>
       <c r="G669">
-        <v>64.71012043477488</v>
+        <v>64.71438990980735</v>
       </c>
       <c r="H669">
         <v>314.84</v>
@@ -75858,10 +75858,10 @@
         <v>36</v>
       </c>
       <c r="R669">
-        <v>361.55917</v>
+        <v>361.59006</v>
       </c>
       <c r="S669">
-        <v>6.431949371141907</v>
+        <v>6.432498888157544</v>
       </c>
       <c r="T669">
         <v>714.6900000000001</v>
@@ -75900,7 +75900,7 @@
         <v>0</v>
       </c>
       <c r="AF669">
-        <v>869.942</v>
+        <v>869.9899999999999</v>
       </c>
       <c r="AG669">
         <v>0</v>
@@ -75909,7 +75909,7 @@
         <v>3</v>
       </c>
       <c r="AI669">
-        <v>1084.67751</v>
+        <v>1084.77018</v>
       </c>
     </row>
     <row r="670">
@@ -75935,10 +75935,10 @@
         <v>67.649</v>
       </c>
       <c r="F670">
-        <v>3941.66</v>
+        <v>3941.86</v>
       </c>
       <c r="G670">
-        <v>58.26634540052329</v>
+        <v>58.26930183742554</v>
       </c>
       <c r="H670">
         <v>150.14</v>
@@ -75971,10 +75971,10 @@
         <v>33.984</v>
       </c>
       <c r="R670">
-        <v>411.33997</v>
+        <v>411.35098</v>
       </c>
       <c r="S670">
-        <v>6.080503333382607</v>
+        <v>6.080666085234076</v>
       </c>
       <c r="T670">
         <v>718.35998</v>
@@ -76013,7 +76013,7 @@
         <v>0</v>
       </c>
       <c r="AF670">
-        <v>380.9168</v>
+        <v>380.9304</v>
       </c>
       <c r="AG670">
         <v>0</v>
@@ -76022,7 +76022,7 @@
         <v>3</v>
       </c>
       <c r="AI670">
-        <v>1234.01991</v>
+        <v>1234.05294</v>
       </c>
     </row>
     <row r="671">
@@ -76048,10 +76048,10 @@
         <v>67.649</v>
       </c>
       <c r="F671">
-        <v>4017.67</v>
+        <v>4017.98</v>
       </c>
       <c r="G671">
-        <v>59.38993924522166</v>
+        <v>59.39452172242013</v>
       </c>
       <c r="H671">
         <v>198.14</v>
@@ -76084,10 +76084,10 @@
         <v>34.992</v>
       </c>
       <c r="R671">
-        <v>341.50385</v>
+        <v>341.52265</v>
       </c>
       <c r="S671">
-        <v>5.048172921994412</v>
+        <v>5.048450827063223</v>
       </c>
       <c r="T671">
         <v>824.9400000000001</v>
@@ -76126,7 +76126,7 @@
         <v>0</v>
       </c>
       <c r="AF671">
-        <v>395.3088</v>
+        <v>395.3304</v>
       </c>
       <c r="AG671">
         <v>0</v>
@@ -76135,7 +76135,7 @@
         <v>3</v>
       </c>
       <c r="AI671">
-        <v>1024.51155</v>
+        <v>1024.56795</v>
       </c>
     </row>
     <row r="672">
@@ -76161,10 +76161,10 @@
         <v>67.649</v>
       </c>
       <c r="F672">
-        <v>4063.56</v>
+        <v>4063.76</v>
       </c>
       <c r="G672">
-        <v>60.06829369244187</v>
+        <v>60.07125012934412</v>
       </c>
       <c r="H672">
         <v>99.45999999999999</v>
@@ -76197,10 +76197,10 @@
         <v>33.012</v>
       </c>
       <c r="R672">
-        <v>376.63674</v>
+        <v>376.6495</v>
       </c>
       <c r="S672">
-        <v>5.567513784387057</v>
+        <v>5.56770240506142</v>
       </c>
       <c r="T672">
         <v>696.5699999999999</v>
@@ -76239,7 +76239,7 @@
         <v>0</v>
       </c>
       <c r="AF672">
-        <v>361.79775</v>
+        <v>361.81275</v>
       </c>
       <c r="AG672">
         <v>0</v>
@@ -76248,13 +76248,13 @@
         <v>3</v>
       </c>
       <c r="AI672">
-        <v>1129.91022</v>
+        <v>1129.9485</v>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="inlineStr">
         <is>
-          <t>Ricardo Gonzalez</t>
+          <t>Raphael Veiga</t>
         </is>
       </c>
       <c r="B673" s="2">
@@ -76274,85 +76274,85 @@
         <v>67.649</v>
       </c>
       <c r="F673">
-        <v>5059.580000000001</v>
+        <v>4241.26</v>
       </c>
       <c r="G673">
-        <v>74.79164510931426</v>
+        <v>62.69508788008692</v>
       </c>
       <c r="H673">
-        <v>258.86</v>
+        <v>118.11</v>
       </c>
       <c r="I673">
-        <v>0</v>
+        <v>4.720000000000001</v>
       </c>
       <c r="J673">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K673">
-        <v>3.826516282576238</v>
+        <v>1.745923812621029</v>
       </c>
       <c r="L673">
         <v>0</v>
       </c>
       <c r="M673">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="N673">
         <v>0</v>
       </c>
       <c r="O673">
-        <v>29.28584</v>
+        <v>28.90342</v>
       </c>
       <c r="P673">
-        <v>81.34955555555555</v>
+        <v>90.31189851268591</v>
       </c>
       <c r="Q673">
-        <v>36</v>
+        <v>32.004</v>
       </c>
       <c r="R673">
-        <v>506.24914</v>
+        <v>362.97457</v>
       </c>
       <c r="S673">
-        <v>7.483468196130024</v>
+        <v>5.365557066623305</v>
       </c>
       <c r="T673">
-        <v>855.61001</v>
+        <v>699.34</v>
       </c>
       <c r="U673">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V673">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="W673">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="X673">
         <v>65</v>
       </c>
       <c r="Y673">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Z673">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AA673">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AB673">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="AC673">
-        <v>4.01974</v>
+        <v>4.04346</v>
       </c>
       <c r="AD673">
-        <v>-2.16456</v>
+        <v>-2.49083</v>
       </c>
       <c r="AE673">
         <v>0</v>
       </c>
       <c r="AF673">
-        <v>1198.778</v>
+        <v>355.7729</v>
       </c>
       <c r="AG673">
         <v>0</v>
@@ -76361,13 +76361,13 @@
         <v>3</v>
       </c>
       <c r="AI673">
-        <v>1518.74742</v>
+        <v>1088.92371</v>
       </c>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>Santiago Camarena</t>
+          <t>Ricardo Gonzalez</t>
         </is>
       </c>
       <c r="B674" s="2">
@@ -76387,13 +76387,13 @@
         <v>67.649</v>
       </c>
       <c r="F674">
-        <v>4985.41</v>
+        <v>5059.89</v>
       </c>
       <c r="G674">
-        <v>73.69525048411654</v>
+        <v>74.79622758651274</v>
       </c>
       <c r="H674">
-        <v>259.84</v>
+        <v>258.86</v>
       </c>
       <c r="I674">
         <v>0</v>
@@ -76402,70 +76402,70 @@
         <v>0</v>
       </c>
       <c r="K674">
-        <v>3.841002823397242</v>
+        <v>3.826516282576238</v>
       </c>
       <c r="L674">
         <v>0</v>
       </c>
       <c r="M674">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N674">
         <v>0</v>
       </c>
       <c r="O674">
-        <v>26.84098</v>
+        <v>29.28584</v>
       </c>
       <c r="P674">
-        <v>74.55827777777777</v>
+        <v>81.34955555555555</v>
       </c>
       <c r="Q674">
         <v>36</v>
       </c>
       <c r="R674">
-        <v>516.20298</v>
+        <v>506.30413</v>
       </c>
       <c r="S674">
-        <v>7.630607695605256</v>
+        <v>7.484281068456297</v>
       </c>
       <c r="T674">
-        <v>919.75997</v>
+        <v>855.61001</v>
       </c>
       <c r="U674">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="V674">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="W674">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="X674">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="Y674">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Z674">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="AA674">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="AB674">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="AC674">
-        <v>3.84027</v>
+        <v>4.01974</v>
       </c>
       <c r="AD674">
-        <v>-2.4507</v>
+        <v>-2.16456</v>
       </c>
       <c r="AE674">
         <v>0</v>
       </c>
       <c r="AF674">
-        <v>1162.218</v>
+        <v>1198.898</v>
       </c>
       <c r="AG674">
         <v>0</v>
@@ -76474,13 +76474,13 @@
         <v>3</v>
       </c>
       <c r="AI674">
-        <v>1548.60894</v>
+        <v>1518.91239</v>
       </c>
     </row>
     <row r="675">
       <c r="A675" t="inlineStr">
         <is>
-          <t>Sebastián Cáceres</t>
+          <t>Santiago Camarena</t>
         </is>
       </c>
       <c r="B675" s="2">
@@ -76488,97 +76488,97 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>MD-3</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>Vespertina seleccionados | Sesión 39</t>
+          <t>Sesión 39</t>
         </is>
       </c>
       <c r="E675">
-        <v>130.8268333333333</v>
+        <v>67.649</v>
       </c>
       <c r="F675">
-        <v>8139.74</v>
+        <v>4985.58</v>
       </c>
       <c r="G675">
-        <v>62.21766431708073</v>
+        <v>73.69776345548345</v>
       </c>
       <c r="H675">
-        <v>853.7099999999999</v>
+        <v>259.84</v>
       </c>
       <c r="I675">
-        <v>1.73</v>
+        <v>0</v>
       </c>
       <c r="J675">
         <v>0</v>
       </c>
       <c r="K675">
-        <v>6.525496171147356</v>
+        <v>3.841002823397242</v>
       </c>
       <c r="L675">
-        <v>27.36</v>
+        <v>0</v>
       </c>
       <c r="M675">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="N675">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O675">
-        <v>31.32208</v>
+        <v>26.84098</v>
       </c>
       <c r="P675">
-        <v>89.51211705532694</v>
+        <v>74.55827777777777</v>
       </c>
       <c r="Q675">
-        <v>34.992</v>
+        <v>36</v>
       </c>
       <c r="R675">
-        <v>897.02218</v>
+        <v>516.21361</v>
       </c>
       <c r="S675">
-        <v>6.856561128514666</v>
+        <v>7.630764830226611</v>
       </c>
       <c r="T675">
-        <v>1821.83001</v>
+        <v>919.75997</v>
       </c>
       <c r="U675">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="V675">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="W675">
-        <v>129</v>
+        <v>23</v>
       </c>
       <c r="X675">
-        <v>190</v>
+        <v>63</v>
       </c>
       <c r="Y675">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="Z675">
-        <v>153</v>
+        <v>36</v>
       </c>
       <c r="AA675">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="AB675">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="AC675">
-        <v>4.60516</v>
+        <v>3.84027</v>
       </c>
       <c r="AD675">
-        <v>-2.6402</v>
+        <v>-2.4507</v>
       </c>
       <c r="AE675">
         <v>0</v>
       </c>
       <c r="AF675">
-        <v>821.3448</v>
+        <v>1162.26</v>
       </c>
       <c r="AG675">
         <v>0</v>
@@ -76587,13 +76587,13 @@
         <v>3</v>
       </c>
       <c r="AI675">
-        <v>2691.06654</v>
+        <v>1548.64083</v>
       </c>
     </row>
     <row r="676">
       <c r="A676" t="inlineStr">
         <is>
-          <t>Víctor Dávila</t>
+          <t>Sebastián Cáceres</t>
         </is>
       </c>
       <c r="B676" s="2">
@@ -76613,94 +76613,2919 @@
         <v>130.8268333333333</v>
       </c>
       <c r="F676">
-        <v>7123.910000000001</v>
+        <v>8139.77</v>
       </c>
       <c r="G676">
-        <v>54.45297282285363</v>
+        <v>62.2178936278363</v>
       </c>
       <c r="H676">
+        <v>853.7099999999999</v>
+      </c>
+      <c r="I676">
+        <v>1.73</v>
+      </c>
+      <c r="J676">
+        <v>0</v>
+      </c>
+      <c r="K676">
+        <v>6.525496171147356</v>
+      </c>
+      <c r="L676">
+        <v>27.36</v>
+      </c>
+      <c r="M676">
+        <v>17</v>
+      </c>
+      <c r="N676">
+        <v>1</v>
+      </c>
+      <c r="O676">
+        <v>31.32208</v>
+      </c>
+      <c r="P676">
+        <v>89.51211705532694</v>
+      </c>
+      <c r="Q676">
+        <v>34.992</v>
+      </c>
+      <c r="R676">
+        <v>897.0345100000001</v>
+      </c>
+      <c r="S676">
+        <v>6.856655375235204</v>
+      </c>
+      <c r="T676">
+        <v>1821.83001</v>
+      </c>
+      <c r="U676">
+        <v>70</v>
+      </c>
+      <c r="V676">
+        <v>59</v>
+      </c>
+      <c r="W676">
+        <v>129</v>
+      </c>
+      <c r="X676">
+        <v>190</v>
+      </c>
+      <c r="Y676">
+        <v>70</v>
+      </c>
+      <c r="Z676">
+        <v>153</v>
+      </c>
+      <c r="AA676">
+        <v>59</v>
+      </c>
+      <c r="AB676">
+        <v>80</v>
+      </c>
+      <c r="AC676">
+        <v>4.60516</v>
+      </c>
+      <c r="AD676">
+        <v>-2.6402</v>
+      </c>
+      <c r="AE676">
+        <v>0</v>
+      </c>
+      <c r="AF676">
+        <v>821.3496</v>
+      </c>
+      <c r="AG676">
+        <v>0</v>
+      </c>
+      <c r="AH676">
+        <v>3</v>
+      </c>
+      <c r="AI676">
+        <v>2691.10353</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B677" s="2">
+        <v>46224</v>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Vespertina seleccionados | Sesión 39</t>
+        </is>
+      </c>
+      <c r="E677">
+        <v>130.8268333333333</v>
+      </c>
+      <c r="F677">
+        <v>7124.04</v>
+      </c>
+      <c r="G677">
+        <v>54.45396650279441</v>
+      </c>
+      <c r="H677">
         <v>436.26</v>
       </c>
-      <c r="I676">
-        <v>0</v>
-      </c>
-      <c r="J676">
-        <v>0</v>
-      </c>
-      <c r="K676">
+      <c r="I677">
+        <v>0</v>
+      </c>
+      <c r="J677">
+        <v>0</v>
+      </c>
+      <c r="K677">
         <v>3.334637007443682</v>
       </c>
-      <c r="L676">
-        <v>0</v>
-      </c>
-      <c r="M676">
+      <c r="L677">
+        <v>0</v>
+      </c>
+      <c r="M677">
         <v>1</v>
       </c>
-      <c r="N676">
-        <v>0</v>
-      </c>
-      <c r="O676">
+      <c r="N677">
+        <v>0</v>
+      </c>
+      <c r="O677">
         <v>25.13394</v>
       </c>
-      <c r="P676">
+      <c r="P677">
         <v>73.95815677966101</v>
       </c>
-      <c r="Q676">
+      <c r="Q677">
         <v>33.984</v>
       </c>
-      <c r="R676">
-        <v>766.5257</v>
-      </c>
-      <c r="S676">
-        <v>5.859086247597015</v>
-      </c>
-      <c r="T676">
+      <c r="R677">
+        <v>766.5307300000001</v>
+      </c>
+      <c r="S677">
+        <v>5.859124695367032</v>
+      </c>
+      <c r="T677">
         <v>1007.45001</v>
       </c>
-      <c r="U676">
+      <c r="U677">
         <v>21</v>
       </c>
-      <c r="V676">
+      <c r="V677">
         <v>14</v>
       </c>
-      <c r="W676">
+      <c r="W677">
         <v>35</v>
       </c>
-      <c r="X676">
+      <c r="X677">
         <v>71</v>
       </c>
-      <c r="Y676">
+      <c r="Y677">
         <v>21</v>
       </c>
-      <c r="Z676">
+      <c r="Z677">
         <v>46</v>
       </c>
-      <c r="AA676">
+      <c r="AA677">
         <v>14</v>
       </c>
-      <c r="AB676">
+      <c r="AB677">
         <v>24</v>
       </c>
-      <c r="AC676">
+      <c r="AC677">
         <v>3.73028</v>
       </c>
-      <c r="AD676">
+      <c r="AD677">
         <v>-1.38662</v>
       </c>
-      <c r="AE676">
-        <v>0</v>
-      </c>
-      <c r="AF676">
-        <v>574.4018</v>
-      </c>
-      <c r="AG676">
-        <v>0</v>
-      </c>
-      <c r="AH676">
-        <v>3</v>
-      </c>
-      <c r="AI676">
-        <v>2299.5771</v>
+      <c r="AE677">
+        <v>0</v>
+      </c>
+      <c r="AF677">
+        <v>574.4123</v>
+      </c>
+      <c r="AG677">
+        <v>0</v>
+      </c>
+      <c r="AH677">
+        <v>3</v>
+      </c>
+      <c r="AI677">
+        <v>2299.59219</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B678" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E678">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F678">
+        <v>4642.17</v>
+      </c>
+      <c r="G678">
+        <v>60.47471302052008</v>
+      </c>
+      <c r="H678">
+        <v>158.87</v>
+      </c>
+      <c r="I678">
+        <v>0</v>
+      </c>
+      <c r="J678">
+        <v>0</v>
+      </c>
+      <c r="K678">
+        <v>2.069639340560562</v>
+      </c>
+      <c r="L678">
+        <v>0</v>
+      </c>
+      <c r="M678">
+        <v>1</v>
+      </c>
+      <c r="N678">
+        <v>0</v>
+      </c>
+      <c r="O678">
+        <v>25.91282</v>
+      </c>
+      <c r="P678">
+        <v>71.98005555555555</v>
+      </c>
+      <c r="Q678">
+        <v>36</v>
+      </c>
+      <c r="R678">
+        <v>455.39061</v>
+      </c>
+      <c r="S678">
+        <v>5.932487705532021</v>
+      </c>
+      <c r="T678">
+        <v>727.19001</v>
+      </c>
+      <c r="U678">
+        <v>24</v>
+      </c>
+      <c r="V678">
+        <v>18</v>
+      </c>
+      <c r="W678">
+        <v>42</v>
+      </c>
+      <c r="X678">
+        <v>62</v>
+      </c>
+      <c r="Y678">
+        <v>24</v>
+      </c>
+      <c r="Z678">
+        <v>48</v>
+      </c>
+      <c r="AA678">
+        <v>18</v>
+      </c>
+      <c r="AB678">
+        <v>27</v>
+      </c>
+      <c r="AC678">
+        <v>4.36679</v>
+      </c>
+      <c r="AD678">
+        <v>-1.75109</v>
+      </c>
+      <c r="AE678">
+        <v>0</v>
+      </c>
+      <c r="AF678">
+        <v>1106.858</v>
+      </c>
+      <c r="AG678">
+        <v>0</v>
+      </c>
+      <c r="AH678">
+        <v>3</v>
+      </c>
+      <c r="AI678">
+        <v>1366.17183</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B679" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Sesión vespertina 22 de Julio | Sesión 40</t>
+        </is>
+      </c>
+      <c r="E679">
+        <v>106.1291666666667</v>
+      </c>
+      <c r="F679">
+        <v>4963.15</v>
+      </c>
+      <c r="G679">
+        <v>46.7651839346708</v>
+      </c>
+      <c r="H679">
+        <v>14.71</v>
+      </c>
+      <c r="I679">
+        <v>0</v>
+      </c>
+      <c r="J679">
+        <v>0</v>
+      </c>
+      <c r="K679">
+        <v>0.1386046876840328</v>
+      </c>
+      <c r="L679">
+        <v>0</v>
+      </c>
+      <c r="M679">
+        <v>0</v>
+      </c>
+      <c r="N679">
+        <v>0</v>
+      </c>
+      <c r="O679">
+        <v>25.04818</v>
+      </c>
+      <c r="P679">
+        <v>77.39519218885181</v>
+      </c>
+      <c r="Q679">
+        <v>32.364</v>
+      </c>
+      <c r="R679">
+        <v>524.91961</v>
+      </c>
+      <c r="S679">
+        <v>4.946044772486357</v>
+      </c>
+      <c r="T679">
+        <v>750.00999</v>
+      </c>
+      <c r="U679">
+        <v>14</v>
+      </c>
+      <c r="V679">
+        <v>17</v>
+      </c>
+      <c r="W679">
+        <v>31</v>
+      </c>
+      <c r="X679">
+        <v>64</v>
+      </c>
+      <c r="Y679">
+        <v>14</v>
+      </c>
+      <c r="Z679">
+        <v>76</v>
+      </c>
+      <c r="AA679">
+        <v>17</v>
+      </c>
+      <c r="AB679">
+        <v>24</v>
+      </c>
+      <c r="AC679">
+        <v>4.21239</v>
+      </c>
+      <c r="AD679">
+        <v>-1.28172</v>
+      </c>
+      <c r="AE679">
+        <v>0</v>
+      </c>
+      <c r="AF679">
+        <v>412.3819</v>
+      </c>
+      <c r="AG679">
+        <v>0</v>
+      </c>
+      <c r="AH679">
+        <v>3</v>
+      </c>
+      <c r="AI679">
+        <v>1574.75883</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B680" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E680">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F680">
+        <v>4439.579999999999</v>
+      </c>
+      <c r="G680">
+        <v>57.8355222733421</v>
+      </c>
+      <c r="H680">
+        <v>172.57</v>
+      </c>
+      <c r="I680">
+        <v>0</v>
+      </c>
+      <c r="J680">
+        <v>0</v>
+      </c>
+      <c r="K680">
+        <v>2.248112677034911</v>
+      </c>
+      <c r="L680">
+        <v>0</v>
+      </c>
+      <c r="M680">
+        <v>5</v>
+      </c>
+      <c r="N680">
+        <v>0</v>
+      </c>
+      <c r="O680">
+        <v>26.55816</v>
+      </c>
+      <c r="P680">
+        <v>73.77266666666667</v>
+      </c>
+      <c r="Q680">
+        <v>36</v>
+      </c>
+      <c r="R680">
+        <v>372.90336</v>
+      </c>
+      <c r="S680">
+        <v>4.857905608882848</v>
+      </c>
+      <c r="T680">
+        <v>614.6900000000001</v>
+      </c>
+      <c r="U680">
+        <v>10</v>
+      </c>
+      <c r="V680">
+        <v>18</v>
+      </c>
+      <c r="W680">
+        <v>28</v>
+      </c>
+      <c r="X680">
+        <v>49</v>
+      </c>
+      <c r="Y680">
+        <v>10</v>
+      </c>
+      <c r="Z680">
+        <v>31</v>
+      </c>
+      <c r="AA680">
+        <v>18</v>
+      </c>
+      <c r="AB680">
+        <v>15</v>
+      </c>
+      <c r="AC680">
+        <v>4.5442</v>
+      </c>
+      <c r="AD680">
+        <v>-1.99059</v>
+      </c>
+      <c r="AE680">
+        <v>0</v>
+      </c>
+      <c r="AF680">
+        <v>1028.72</v>
+      </c>
+      <c r="AG680">
+        <v>0</v>
+      </c>
+      <c r="AH680">
+        <v>3</v>
+      </c>
+      <c r="AI680">
+        <v>1118.71008</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B681" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E681">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F681">
+        <v>5058.01</v>
+      </c>
+      <c r="G681">
+        <v>65.89196500880425</v>
+      </c>
+      <c r="H681">
+        <v>144.22</v>
+      </c>
+      <c r="I681">
+        <v>0</v>
+      </c>
+      <c r="J681">
+        <v>0</v>
+      </c>
+      <c r="K681">
+        <v>1.878790115790548</v>
+      </c>
+      <c r="L681">
+        <v>0</v>
+      </c>
+      <c r="M681">
+        <v>3</v>
+      </c>
+      <c r="N681">
+        <v>0</v>
+      </c>
+      <c r="O681">
+        <v>28.17974</v>
+      </c>
+      <c r="P681">
+        <v>86.97450617283951</v>
+      </c>
+      <c r="Q681">
+        <v>32.4</v>
+      </c>
+      <c r="R681">
+        <v>502.83948</v>
+      </c>
+      <c r="S681">
+        <v>6.550616036980022</v>
+      </c>
+      <c r="T681">
+        <v>719.55</v>
+      </c>
+      <c r="U681">
+        <v>18</v>
+      </c>
+      <c r="V681">
+        <v>7</v>
+      </c>
+      <c r="W681">
+        <v>25</v>
+      </c>
+      <c r="X681">
+        <v>64</v>
+      </c>
+      <c r="Y681">
+        <v>18</v>
+      </c>
+      <c r="Z681">
+        <v>35</v>
+      </c>
+      <c r="AA681">
+        <v>7</v>
+      </c>
+      <c r="AB681">
+        <v>5</v>
+      </c>
+      <c r="AC681">
+        <v>4.29435</v>
+      </c>
+      <c r="AD681">
+        <v>-1.88372</v>
+      </c>
+      <c r="AE681">
+        <v>0</v>
+      </c>
+      <c r="AF681">
+        <v>410.9021</v>
+      </c>
+      <c r="AG681">
+        <v>0</v>
+      </c>
+      <c r="AH681">
+        <v>3</v>
+      </c>
+      <c r="AI681">
+        <v>1508.51844</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B682" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Sesión vespertina 22 de Julio | Sesión 40</t>
+        </is>
+      </c>
+      <c r="E682">
+        <v>91.16066666666666</v>
+      </c>
+      <c r="F682">
+        <v>5010.73</v>
+      </c>
+      <c r="G682">
+        <v>54.96592097468938</v>
+      </c>
+      <c r="H682">
+        <v>121.43</v>
+      </c>
+      <c r="I682">
+        <v>0</v>
+      </c>
+      <c r="J682">
+        <v>0</v>
+      </c>
+      <c r="K682">
+        <v>1.332043790816215</v>
+      </c>
+      <c r="L682">
+        <v>0</v>
+      </c>
+      <c r="M682">
+        <v>1</v>
+      </c>
+      <c r="N682">
+        <v>0</v>
+      </c>
+      <c r="O682">
+        <v>25.24001</v>
+      </c>
+      <c r="P682">
+        <v>70.89093922031233</v>
+      </c>
+      <c r="Q682">
+        <v>35.604</v>
+      </c>
+      <c r="R682">
+        <v>462.50969</v>
+      </c>
+      <c r="S682">
+        <v>5.073566340746375</v>
+      </c>
+      <c r="T682">
+        <v>971.72001</v>
+      </c>
+      <c r="U682">
+        <v>46</v>
+      </c>
+      <c r="V682">
+        <v>50</v>
+      </c>
+      <c r="W682">
+        <v>96</v>
+      </c>
+      <c r="X682">
+        <v>111</v>
+      </c>
+      <c r="Y682">
+        <v>46</v>
+      </c>
+      <c r="Z682">
+        <v>103</v>
+      </c>
+      <c r="AA682">
+        <v>50</v>
+      </c>
+      <c r="AB682">
+        <v>48</v>
+      </c>
+      <c r="AC682">
+        <v>4.64571</v>
+      </c>
+      <c r="AD682">
+        <v>-3.01431</v>
+      </c>
+      <c r="AE682">
+        <v>0</v>
+      </c>
+      <c r="AF682">
+        <v>446.09371</v>
+      </c>
+      <c r="AG682">
+        <v>0</v>
+      </c>
+      <c r="AH682">
+        <v>3</v>
+      </c>
+      <c r="AI682">
+        <v>1387.52907</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B683" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E683">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F683">
+        <v>5113.88</v>
+      </c>
+      <c r="G683">
+        <v>66.61979751309781</v>
+      </c>
+      <c r="H683">
+        <v>160.38</v>
+      </c>
+      <c r="I683">
+        <v>0</v>
+      </c>
+      <c r="J683">
+        <v>0</v>
+      </c>
+      <c r="K683">
+        <v>2.089310489325253</v>
+      </c>
+      <c r="L683">
+        <v>0</v>
+      </c>
+      <c r="M683">
+        <v>3</v>
+      </c>
+      <c r="N683">
+        <v>0</v>
+      </c>
+      <c r="O683">
+        <v>26.8469</v>
+      </c>
+      <c r="P683">
+        <v>78.99864642184558</v>
+      </c>
+      <c r="Q683">
+        <v>33.984</v>
+      </c>
+      <c r="R683">
+        <v>584.1535</v>
+      </c>
+      <c r="S683">
+        <v>7.609914172129065</v>
+      </c>
+      <c r="T683">
+        <v>733.15999</v>
+      </c>
+      <c r="U683">
+        <v>13</v>
+      </c>
+      <c r="V683">
+        <v>16</v>
+      </c>
+      <c r="W683">
+        <v>29</v>
+      </c>
+      <c r="X683">
+        <v>49</v>
+      </c>
+      <c r="Y683">
+        <v>13</v>
+      </c>
+      <c r="Z683">
+        <v>47</v>
+      </c>
+      <c r="AA683">
+        <v>16</v>
+      </c>
+      <c r="AB683">
+        <v>14</v>
+      </c>
+      <c r="AC683">
+        <v>4.26299</v>
+      </c>
+      <c r="AD683">
+        <v>-2.2676</v>
+      </c>
+      <c r="AE683">
+        <v>0</v>
+      </c>
+      <c r="AF683">
+        <v>476.6376</v>
+      </c>
+      <c r="AG683">
+        <v>0</v>
+      </c>
+      <c r="AH683">
+        <v>3</v>
+      </c>
+      <c r="AI683">
+        <v>1752.4605</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B684" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E684">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F684">
+        <v>5204.19</v>
+      </c>
+      <c r="G684">
+        <v>67.79628853623637</v>
+      </c>
+      <c r="H684">
+        <v>313.59</v>
+      </c>
+      <c r="I684">
+        <v>0</v>
+      </c>
+      <c r="J684">
+        <v>0</v>
+      </c>
+      <c r="K684">
+        <v>4.085215590145318</v>
+      </c>
+      <c r="L684">
+        <v>0</v>
+      </c>
+      <c r="M684">
+        <v>11</v>
+      </c>
+      <c r="N684">
+        <v>0</v>
+      </c>
+      <c r="O684">
+        <v>29.2171</v>
+      </c>
+      <c r="P684">
+        <v>82.14434322986955</v>
+      </c>
+      <c r="Q684">
+        <v>35.568</v>
+      </c>
+      <c r="R684">
+        <v>450.31588</v>
+      </c>
+      <c r="S684">
+        <v>5.866377924889213</v>
+      </c>
+      <c r="T684">
+        <v>768.02001</v>
+      </c>
+      <c r="U684">
+        <v>20</v>
+      </c>
+      <c r="V684">
+        <v>20</v>
+      </c>
+      <c r="W684">
+        <v>40</v>
+      </c>
+      <c r="X684">
+        <v>67</v>
+      </c>
+      <c r="Y684">
+        <v>20</v>
+      </c>
+      <c r="Z684">
+        <v>39</v>
+      </c>
+      <c r="AA684">
+        <v>20</v>
+      </c>
+      <c r="AB684">
+        <v>8</v>
+      </c>
+      <c r="AC684">
+        <v>4.64123</v>
+      </c>
+      <c r="AD684">
+        <v>-1.91389</v>
+      </c>
+      <c r="AE684">
+        <v>0</v>
+      </c>
+      <c r="AF684">
+        <v>494.9272</v>
+      </c>
+      <c r="AG684">
+        <v>0</v>
+      </c>
+      <c r="AH684">
+        <v>3</v>
+      </c>
+      <c r="AI684">
+        <v>1350.94764</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B685" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E685">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F685">
+        <v>5046.5</v>
+      </c>
+      <c r="G685">
+        <v>65.74202135166412</v>
+      </c>
+      <c r="H685">
+        <v>244.34</v>
+      </c>
+      <c r="I685">
+        <v>0</v>
+      </c>
+      <c r="J685">
+        <v>0</v>
+      </c>
+      <c r="K685">
+        <v>3.18307846964542</v>
+      </c>
+      <c r="L685">
+        <v>0</v>
+      </c>
+      <c r="M685">
+        <v>6</v>
+      </c>
+      <c r="N685">
+        <v>0</v>
+      </c>
+      <c r="O685">
+        <v>28.19754</v>
+      </c>
+      <c r="P685">
+        <v>78.3265</v>
+      </c>
+      <c r="Q685">
+        <v>36</v>
+      </c>
+      <c r="R685">
+        <v>481.6447</v>
+      </c>
+      <c r="S685">
+        <v>6.274506321473469</v>
+      </c>
+      <c r="T685">
+        <v>763.4899799999999</v>
+      </c>
+      <c r="U685">
+        <v>15</v>
+      </c>
+      <c r="V685">
+        <v>19</v>
+      </c>
+      <c r="W685">
+        <v>34</v>
+      </c>
+      <c r="X685">
+        <v>53</v>
+      </c>
+      <c r="Y685">
+        <v>15</v>
+      </c>
+      <c r="Z685">
+        <v>51</v>
+      </c>
+      <c r="AA685">
+        <v>19</v>
+      </c>
+      <c r="AB685">
+        <v>21</v>
+      </c>
+      <c r="AC685">
+        <v>3.93397</v>
+      </c>
+      <c r="AD685">
+        <v>-1.53562</v>
+      </c>
+      <c r="AE685">
+        <v>0</v>
+      </c>
+      <c r="AF685">
+        <v>1178.79</v>
+      </c>
+      <c r="AG685">
+        <v>0</v>
+      </c>
+      <c r="AH685">
+        <v>3</v>
+      </c>
+      <c r="AI685">
+        <v>1444.9341</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B686" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E686">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F686">
+        <v>4930.559999999999</v>
+      </c>
+      <c r="G686">
+        <v>64.2316418895593</v>
+      </c>
+      <c r="H686">
+        <v>187.91</v>
+      </c>
+      <c r="I686">
+        <v>0</v>
+      </c>
+      <c r="J686">
+        <v>0</v>
+      </c>
+      <c r="K686">
+        <v>2.447950704882831</v>
+      </c>
+      <c r="L686">
+        <v>0</v>
+      </c>
+      <c r="M686">
+        <v>4</v>
+      </c>
+      <c r="N686">
+        <v>0</v>
+      </c>
+      <c r="O686">
+        <v>28.25237</v>
+      </c>
+      <c r="P686">
+        <v>78.47880555555555</v>
+      </c>
+      <c r="Q686">
+        <v>36</v>
+      </c>
+      <c r="R686">
+        <v>466.73165</v>
+      </c>
+      <c r="S686">
+        <v>6.080230278370638</v>
+      </c>
+      <c r="T686">
+        <v>686.98001</v>
+      </c>
+      <c r="U686">
+        <v>13</v>
+      </c>
+      <c r="V686">
+        <v>21</v>
+      </c>
+      <c r="W686">
+        <v>34</v>
+      </c>
+      <c r="X686">
+        <v>53</v>
+      </c>
+      <c r="Y686">
+        <v>13</v>
+      </c>
+      <c r="Z686">
+        <v>46</v>
+      </c>
+      <c r="AA686">
+        <v>21</v>
+      </c>
+      <c r="AB686">
+        <v>16</v>
+      </c>
+      <c r="AC686">
+        <v>4.39234</v>
+      </c>
+      <c r="AD686">
+        <v>-2.26574</v>
+      </c>
+      <c r="AE686">
+        <v>0</v>
+      </c>
+      <c r="AF686">
+        <v>401.1483</v>
+      </c>
+      <c r="AG686">
+        <v>0</v>
+      </c>
+      <c r="AH686">
+        <v>3</v>
+      </c>
+      <c r="AI686">
+        <v>1400.19495</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B687" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E687">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F687">
+        <v>4735.53</v>
+      </c>
+      <c r="G687">
+        <v>61.69093715871316</v>
+      </c>
+      <c r="H687">
+        <v>294.67</v>
+      </c>
+      <c r="I687">
+        <v>0</v>
+      </c>
+      <c r="J687">
+        <v>0</v>
+      </c>
+      <c r="K687">
+        <v>3.838740004298992</v>
+      </c>
+      <c r="L687">
+        <v>0</v>
+      </c>
+      <c r="M687">
+        <v>5</v>
+      </c>
+      <c r="N687">
+        <v>0</v>
+      </c>
+      <c r="O687">
+        <v>28.71162</v>
+      </c>
+      <c r="P687">
+        <v>89.71259842519686</v>
+      </c>
+      <c r="Q687">
+        <v>32.004</v>
+      </c>
+      <c r="R687">
+        <v>484.80784</v>
+      </c>
+      <c r="S687">
+        <v>6.315713339687736</v>
+      </c>
+      <c r="T687">
+        <v>762.05</v>
+      </c>
+      <c r="U687">
+        <v>23</v>
+      </c>
+      <c r="V687">
+        <v>23</v>
+      </c>
+      <c r="W687">
+        <v>46</v>
+      </c>
+      <c r="X687">
+        <v>59</v>
+      </c>
+      <c r="Y687">
+        <v>23</v>
+      </c>
+      <c r="Z687">
+        <v>54</v>
+      </c>
+      <c r="AA687">
+        <v>23</v>
+      </c>
+      <c r="AB687">
+        <v>13</v>
+      </c>
+      <c r="AC687">
+        <v>4.0832</v>
+      </c>
+      <c r="AD687">
+        <v>-2.16507</v>
+      </c>
+      <c r="AE687">
+        <v>0</v>
+      </c>
+      <c r="AF687">
+        <v>340.4964</v>
+      </c>
+      <c r="AG687">
+        <v>0</v>
+      </c>
+      <c r="AH687">
+        <v>3</v>
+      </c>
+      <c r="AI687">
+        <v>1454.42352</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B688" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E688">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F688">
+        <v>4734.5</v>
+      </c>
+      <c r="G688">
+        <v>61.67751909035049</v>
+      </c>
+      <c r="H688">
+        <v>260.17</v>
+      </c>
+      <c r="I688">
+        <v>0</v>
+      </c>
+      <c r="J688">
+        <v>0</v>
+      </c>
+      <c r="K688">
+        <v>3.389299850403736</v>
+      </c>
+      <c r="L688">
+        <v>0</v>
+      </c>
+      <c r="M688">
+        <v>6</v>
+      </c>
+      <c r="N688">
+        <v>0</v>
+      </c>
+      <c r="O688">
+        <v>29.56963</v>
+      </c>
+      <c r="P688">
+        <v>87.38070330969266</v>
+      </c>
+      <c r="Q688">
+        <v>33.84</v>
+      </c>
+      <c r="R688">
+        <v>407.5571</v>
+      </c>
+      <c r="S688">
+        <v>5.309348572321868</v>
+      </c>
+      <c r="T688">
+        <v>700.59</v>
+      </c>
+      <c r="U688">
+        <v>21</v>
+      </c>
+      <c r="V688">
+        <v>11</v>
+      </c>
+      <c r="W688">
+        <v>32</v>
+      </c>
+      <c r="X688">
+        <v>67</v>
+      </c>
+      <c r="Y688">
+        <v>21</v>
+      </c>
+      <c r="Z688">
+        <v>52</v>
+      </c>
+      <c r="AA688">
+        <v>11</v>
+      </c>
+      <c r="AB688">
+        <v>10</v>
+      </c>
+      <c r="AC688">
+        <v>4.42661</v>
+      </c>
+      <c r="AD688">
+        <v>-1.89175</v>
+      </c>
+      <c r="AE688">
+        <v>0</v>
+      </c>
+      <c r="AF688">
+        <v>391.272</v>
+      </c>
+      <c r="AG688">
+        <v>0</v>
+      </c>
+      <c r="AH688">
+        <v>3</v>
+      </c>
+      <c r="AI688">
+        <v>1222.6713</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B689" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E689">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F689">
+        <v>4327.87</v>
+      </c>
+      <c r="G689">
+        <v>56.38024808228011</v>
+      </c>
+      <c r="H689">
+        <v>117.17</v>
+      </c>
+      <c r="I689">
+        <v>0</v>
+      </c>
+      <c r="J689">
+        <v>0</v>
+      </c>
+      <c r="K689">
+        <v>1.526402980634991</v>
+      </c>
+      <c r="L689">
+        <v>0</v>
+      </c>
+      <c r="M689">
+        <v>0</v>
+      </c>
+      <c r="N689">
+        <v>0</v>
+      </c>
+      <c r="O689">
+        <v>25.17154</v>
+      </c>
+      <c r="P689">
+        <v>74.70186372269706</v>
+      </c>
+      <c r="Q689">
+        <v>33.696</v>
+      </c>
+      <c r="R689">
+        <v>402.19368</v>
+      </c>
+      <c r="S689">
+        <v>5.23947795463477</v>
+      </c>
+      <c r="T689">
+        <v>673.64001</v>
+      </c>
+      <c r="U689">
+        <v>17</v>
+      </c>
+      <c r="V689">
+        <v>17</v>
+      </c>
+      <c r="W689">
+        <v>34</v>
+      </c>
+      <c r="X689">
+        <v>65</v>
+      </c>
+      <c r="Y689">
+        <v>17</v>
+      </c>
+      <c r="Z689">
+        <v>47</v>
+      </c>
+      <c r="AA689">
+        <v>17</v>
+      </c>
+      <c r="AB689">
+        <v>14</v>
+      </c>
+      <c r="AC689">
+        <v>4.18196</v>
+      </c>
+      <c r="AD689">
+        <v>-2.1571</v>
+      </c>
+      <c r="AE689">
+        <v>0</v>
+      </c>
+      <c r="AF689">
+        <v>408.3096</v>
+      </c>
+      <c r="AG689">
+        <v>0</v>
+      </c>
+      <c r="AH689">
+        <v>3</v>
+      </c>
+      <c r="AI689">
+        <v>1206.58104</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B690" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E690">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F690">
+        <v>5088.87</v>
+      </c>
+      <c r="G690">
+        <v>66.29398596965085</v>
+      </c>
+      <c r="H690">
+        <v>222.3</v>
+      </c>
+      <c r="I690">
+        <v>0</v>
+      </c>
+      <c r="J690">
+        <v>0</v>
+      </c>
+      <c r="K690">
+        <v>2.895957861185957</v>
+      </c>
+      <c r="L690">
+        <v>0</v>
+      </c>
+      <c r="M690">
+        <v>4</v>
+      </c>
+      <c r="N690">
+        <v>0</v>
+      </c>
+      <c r="O690">
+        <v>26.88172</v>
+      </c>
+      <c r="P690">
+        <v>74.67144444444445</v>
+      </c>
+      <c r="Q690">
+        <v>36</v>
+      </c>
+      <c r="R690">
+        <v>572.93773</v>
+      </c>
+      <c r="S690">
+        <v>7.463803523002867</v>
+      </c>
+      <c r="T690">
+        <v>842.5300100000001</v>
+      </c>
+      <c r="U690">
+        <v>25</v>
+      </c>
+      <c r="V690">
+        <v>20</v>
+      </c>
+      <c r="W690">
+        <v>45</v>
+      </c>
+      <c r="X690">
+        <v>59</v>
+      </c>
+      <c r="Y690">
+        <v>25</v>
+      </c>
+      <c r="Z690">
+        <v>58</v>
+      </c>
+      <c r="AA690">
+        <v>20</v>
+      </c>
+      <c r="AB690">
+        <v>18</v>
+      </c>
+      <c r="AC690">
+        <v>4.45689</v>
+      </c>
+      <c r="AD690">
+        <v>-1.79676</v>
+      </c>
+      <c r="AE690">
+        <v>0</v>
+      </c>
+      <c r="AF690">
+        <v>1219.522</v>
+      </c>
+      <c r="AG690">
+        <v>0</v>
+      </c>
+      <c r="AH690">
+        <v>3</v>
+      </c>
+      <c r="AI690">
+        <v>1718.81319</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B691" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E691">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F691">
+        <v>4937.26</v>
+      </c>
+      <c r="G691">
+        <v>64.31892447017086</v>
+      </c>
+      <c r="H691">
+        <v>200.49</v>
+      </c>
+      <c r="I691">
+        <v>0</v>
+      </c>
+      <c r="J691">
+        <v>0</v>
+      </c>
+      <c r="K691">
+        <v>2.61183352041913</v>
+      </c>
+      <c r="L691">
+        <v>0</v>
+      </c>
+      <c r="M691">
+        <v>4</v>
+      </c>
+      <c r="N691">
+        <v>0</v>
+      </c>
+      <c r="O691">
+        <v>28.01388</v>
+      </c>
+      <c r="P691">
+        <v>80.0579561042524</v>
+      </c>
+      <c r="Q691">
+        <v>34.992</v>
+      </c>
+      <c r="R691">
+        <v>405.95324</v>
+      </c>
+      <c r="S691">
+        <v>5.288454685793566</v>
+      </c>
+      <c r="T691">
+        <v>672.25999</v>
+      </c>
+      <c r="U691">
+        <v>18</v>
+      </c>
+      <c r="V691">
+        <v>12</v>
+      </c>
+      <c r="W691">
+        <v>30</v>
+      </c>
+      <c r="X691">
+        <v>45</v>
+      </c>
+      <c r="Y691">
+        <v>18</v>
+      </c>
+      <c r="Z691">
+        <v>45</v>
+      </c>
+      <c r="AA691">
+        <v>12</v>
+      </c>
+      <c r="AB691">
+        <v>10</v>
+      </c>
+      <c r="AC691">
+        <v>4.50822</v>
+      </c>
+      <c r="AD691">
+        <v>-1.87198</v>
+      </c>
+      <c r="AE691">
+        <v>0</v>
+      </c>
+      <c r="AF691">
+        <v>392.69211</v>
+      </c>
+      <c r="AG691">
+        <v>0</v>
+      </c>
+      <c r="AH691">
+        <v>3</v>
+      </c>
+      <c r="AI691">
+        <v>1217.85972</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B692" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Sesión vespertina 22 de Julio | Sesión 40</t>
+        </is>
+      </c>
+      <c r="E692">
+        <v>91.16066666666666</v>
+      </c>
+      <c r="F692">
+        <v>5019.24</v>
+      </c>
+      <c r="G692">
+        <v>55.05927263951558</v>
+      </c>
+      <c r="H692">
+        <v>48.48</v>
+      </c>
+      <c r="I692">
+        <v>0</v>
+      </c>
+      <c r="J692">
+        <v>0</v>
+      </c>
+      <c r="K692">
+        <v>0.5318083091391757</v>
+      </c>
+      <c r="L692">
+        <v>0</v>
+      </c>
+      <c r="M692">
+        <v>1</v>
+      </c>
+      <c r="N692">
+        <v>0</v>
+      </c>
+      <c r="O692">
+        <v>25.97433</v>
+      </c>
+      <c r="P692">
+        <v>78.6814794620138</v>
+      </c>
+      <c r="Q692">
+        <v>33.012</v>
+      </c>
+      <c r="R692">
+        <v>567.59174</v>
+      </c>
+      <c r="S692">
+        <v>6.226278950717049</v>
+      </c>
+      <c r="T692">
+        <v>981.01</v>
+      </c>
+      <c r="U692">
+        <v>32</v>
+      </c>
+      <c r="V692">
+        <v>55</v>
+      </c>
+      <c r="W692">
+        <v>87</v>
+      </c>
+      <c r="X692">
+        <v>115</v>
+      </c>
+      <c r="Y692">
+        <v>32</v>
+      </c>
+      <c r="Z692">
+        <v>119</v>
+      </c>
+      <c r="AA692">
+        <v>55</v>
+      </c>
+      <c r="AB692">
+        <v>48</v>
+      </c>
+      <c r="AC692">
+        <v>3.9098</v>
+      </c>
+      <c r="AD692">
+        <v>-2.59162</v>
+      </c>
+      <c r="AE692">
+        <v>0</v>
+      </c>
+      <c r="AF692">
+        <v>488.77764</v>
+      </c>
+      <c r="AG692">
+        <v>0</v>
+      </c>
+      <c r="AH692">
+        <v>3</v>
+      </c>
+      <c r="AI692">
+        <v>1702.77522</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B693" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E693">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F693">
+        <v>5201.02</v>
+      </c>
+      <c r="G693">
+        <v>67.75499215108135</v>
+      </c>
+      <c r="H693">
+        <v>364.36</v>
+      </c>
+      <c r="I693">
+        <v>0</v>
+      </c>
+      <c r="J693">
+        <v>0</v>
+      </c>
+      <c r="K693">
+        <v>4.746609115167411</v>
+      </c>
+      <c r="L693">
+        <v>7.38</v>
+      </c>
+      <c r="M693">
+        <v>8</v>
+      </c>
+      <c r="N693">
+        <v>1</v>
+      </c>
+      <c r="O693">
+        <v>30.56247</v>
+      </c>
+      <c r="P693">
+        <v>87.34130658436216</v>
+      </c>
+      <c r="Q693">
+        <v>34.992</v>
+      </c>
+      <c r="R693">
+        <v>422.50198</v>
+      </c>
+      <c r="S693">
+        <v>5.504039272818858</v>
+      </c>
+      <c r="T693">
+        <v>935.59001</v>
+      </c>
+      <c r="U693">
+        <v>18</v>
+      </c>
+      <c r="V693">
+        <v>20</v>
+      </c>
+      <c r="W693">
+        <v>38</v>
+      </c>
+      <c r="X693">
+        <v>67</v>
+      </c>
+      <c r="Y693">
+        <v>18</v>
+      </c>
+      <c r="Z693">
+        <v>52</v>
+      </c>
+      <c r="AA693">
+        <v>20</v>
+      </c>
+      <c r="AB693">
+        <v>15</v>
+      </c>
+      <c r="AC693">
+        <v>4.76255</v>
+      </c>
+      <c r="AD693">
+        <v>-2.13705</v>
+      </c>
+      <c r="AE693">
+        <v>0</v>
+      </c>
+      <c r="AF693">
+        <v>438.68628</v>
+      </c>
+      <c r="AG693">
+        <v>0</v>
+      </c>
+      <c r="AH693">
+        <v>3</v>
+      </c>
+      <c r="AI693">
+        <v>1267.50594</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B694" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E694">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F694">
+        <v>4514.809999999999</v>
+      </c>
+      <c r="G694">
+        <v>58.81556235385052</v>
+      </c>
+      <c r="H694">
+        <v>125.18</v>
+      </c>
+      <c r="I694">
+        <v>0</v>
+      </c>
+      <c r="J694">
+        <v>0</v>
+      </c>
+      <c r="K694">
+        <v>1.630751259843716</v>
+      </c>
+      <c r="L694">
+        <v>0</v>
+      </c>
+      <c r="M694">
+        <v>1</v>
+      </c>
+      <c r="N694">
+        <v>0</v>
+      </c>
+      <c r="O694">
+        <v>26.80534</v>
+      </c>
+      <c r="P694">
+        <v>74.45927777777777</v>
+      </c>
+      <c r="Q694">
+        <v>36</v>
+      </c>
+      <c r="R694">
+        <v>468.78382</v>
+      </c>
+      <c r="S694">
+        <v>6.106964411721919</v>
+      </c>
+      <c r="T694">
+        <v>585.5899900000001</v>
+      </c>
+      <c r="U694">
+        <v>8</v>
+      </c>
+      <c r="V694">
+        <v>13</v>
+      </c>
+      <c r="W694">
+        <v>21</v>
+      </c>
+      <c r="X694">
+        <v>60</v>
+      </c>
+      <c r="Y694">
+        <v>8</v>
+      </c>
+      <c r="Z694">
+        <v>49</v>
+      </c>
+      <c r="AA694">
+        <v>13</v>
+      </c>
+      <c r="AB694">
+        <v>13</v>
+      </c>
+      <c r="AC694">
+        <v>4.14445</v>
+      </c>
+      <c r="AD694">
+        <v>-1.4456</v>
+      </c>
+      <c r="AE694">
+        <v>0</v>
+      </c>
+      <c r="AF694">
+        <v>1049.368</v>
+      </c>
+      <c r="AG694">
+        <v>0</v>
+      </c>
+      <c r="AH694">
+        <v>3</v>
+      </c>
+      <c r="AI694">
+        <v>1406.35146</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B695" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E695">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F695">
+        <v>4141.459999999999</v>
+      </c>
+      <c r="G695">
+        <v>53.95183825365358</v>
+      </c>
+      <c r="H695">
+        <v>124.2</v>
+      </c>
+      <c r="I695">
+        <v>0</v>
+      </c>
+      <c r="J695">
+        <v>0</v>
+      </c>
+      <c r="K695">
+        <v>1.617984554022924</v>
+      </c>
+      <c r="L695">
+        <v>0</v>
+      </c>
+      <c r="M695">
+        <v>3</v>
+      </c>
+      <c r="N695">
+        <v>0</v>
+      </c>
+      <c r="O695">
+        <v>26.92116</v>
+      </c>
+      <c r="P695">
+        <v>79.21716101694915</v>
+      </c>
+      <c r="Q695">
+        <v>33.984</v>
+      </c>
+      <c r="R695">
+        <v>423.69926</v>
+      </c>
+      <c r="S695">
+        <v>5.519636539701632</v>
+      </c>
+      <c r="T695">
+        <v>502.74</v>
+      </c>
+      <c r="U695">
+        <v>7</v>
+      </c>
+      <c r="V695">
+        <v>19</v>
+      </c>
+      <c r="W695">
+        <v>26</v>
+      </c>
+      <c r="X695">
+        <v>40</v>
+      </c>
+      <c r="Y695">
+        <v>7</v>
+      </c>
+      <c r="Z695">
+        <v>41</v>
+      </c>
+      <c r="AA695">
+        <v>19</v>
+      </c>
+      <c r="AB695">
+        <v>20</v>
+      </c>
+      <c r="AC695">
+        <v>4.43106</v>
+      </c>
+      <c r="AD695">
+        <v>-2.041</v>
+      </c>
+      <c r="AE695">
+        <v>0</v>
+      </c>
+      <c r="AF695">
+        <v>387.9344</v>
+      </c>
+      <c r="AG695">
+        <v>0</v>
+      </c>
+      <c r="AH695">
+        <v>3</v>
+      </c>
+      <c r="AI695">
+        <v>1271.09778</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B696" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E696">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F696">
+        <v>4012.940000000001</v>
+      </c>
+      <c r="G696">
+        <v>52.27757597601249</v>
+      </c>
+      <c r="H696">
+        <v>188.5</v>
+      </c>
+      <c r="I696">
+        <v>0</v>
+      </c>
+      <c r="J696">
+        <v>0</v>
+      </c>
+      <c r="K696">
+        <v>2.455636782876981</v>
+      </c>
+      <c r="L696">
+        <v>0</v>
+      </c>
+      <c r="M696">
+        <v>3</v>
+      </c>
+      <c r="N696">
+        <v>0</v>
+      </c>
+      <c r="O696">
+        <v>26.53735</v>
+      </c>
+      <c r="P696">
+        <v>75.83833447645176</v>
+      </c>
+      <c r="Q696">
+        <v>34.992</v>
+      </c>
+      <c r="R696">
+        <v>324.56546</v>
+      </c>
+      <c r="S696">
+        <v>4.228195660622746</v>
+      </c>
+      <c r="T696">
+        <v>598.1</v>
+      </c>
+      <c r="U696">
+        <v>20</v>
+      </c>
+      <c r="V696">
+        <v>17</v>
+      </c>
+      <c r="W696">
+        <v>37</v>
+      </c>
+      <c r="X696">
+        <v>56</v>
+      </c>
+      <c r="Y696">
+        <v>20</v>
+      </c>
+      <c r="Z696">
+        <v>47</v>
+      </c>
+      <c r="AA696">
+        <v>17</v>
+      </c>
+      <c r="AB696">
+        <v>5</v>
+      </c>
+      <c r="AC696">
+        <v>4.13131</v>
+      </c>
+      <c r="AD696">
+        <v>-1.81766</v>
+      </c>
+      <c r="AE696">
+        <v>0</v>
+      </c>
+      <c r="AF696">
+        <v>380.6992</v>
+      </c>
+      <c r="AG696">
+        <v>0</v>
+      </c>
+      <c r="AH696">
+        <v>3</v>
+      </c>
+      <c r="AI696">
+        <v>973.6963800000001</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B697" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E697">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F697">
+        <v>4075.24</v>
+      </c>
+      <c r="G697">
+        <v>53.08917370319146</v>
+      </c>
+      <c r="H697">
+        <v>175.98</v>
+      </c>
+      <c r="I697">
+        <v>0</v>
+      </c>
+      <c r="J697">
+        <v>0</v>
+      </c>
+      <c r="K697">
+        <v>2.292535602390934</v>
+      </c>
+      <c r="L697">
+        <v>0</v>
+      </c>
+      <c r="M697">
+        <v>3</v>
+      </c>
+      <c r="N697">
+        <v>0</v>
+      </c>
+      <c r="O697">
+        <v>27.36774</v>
+      </c>
+      <c r="P697">
+        <v>82.90239912758996</v>
+      </c>
+      <c r="Q697">
+        <v>33.012</v>
+      </c>
+      <c r="R697">
+        <v>385.22441</v>
+      </c>
+      <c r="S697">
+        <v>5.018415017814765</v>
+      </c>
+      <c r="T697">
+        <v>583.5200199999999</v>
+      </c>
+      <c r="U697">
+        <v>14</v>
+      </c>
+      <c r="V697">
+        <v>12</v>
+      </c>
+      <c r="W697">
+        <v>26</v>
+      </c>
+      <c r="X697">
+        <v>52</v>
+      </c>
+      <c r="Y697">
+        <v>14</v>
+      </c>
+      <c r="Z697">
+        <v>37</v>
+      </c>
+      <c r="AA697">
+        <v>12</v>
+      </c>
+      <c r="AB697">
+        <v>8</v>
+      </c>
+      <c r="AC697">
+        <v>4.18914</v>
+      </c>
+      <c r="AD697">
+        <v>-2.20172</v>
+      </c>
+      <c r="AE697">
+        <v>0</v>
+      </c>
+      <c r="AF697">
+        <v>354.53475</v>
+      </c>
+      <c r="AG697">
+        <v>0</v>
+      </c>
+      <c r="AH697">
+        <v>3</v>
+      </c>
+      <c r="AI697">
+        <v>1155.67323</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B698" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E698">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F698">
+        <v>4490.31</v>
+      </c>
+      <c r="G698">
+        <v>58.49639470833071</v>
+      </c>
+      <c r="H698">
+        <v>151.15</v>
+      </c>
+      <c r="I698">
+        <v>0</v>
+      </c>
+      <c r="J698">
+        <v>0</v>
+      </c>
+      <c r="K698">
+        <v>1.969068964094725</v>
+      </c>
+      <c r="L698">
+        <v>0</v>
+      </c>
+      <c r="M698">
+        <v>6</v>
+      </c>
+      <c r="N698">
+        <v>0</v>
+      </c>
+      <c r="O698">
+        <v>28.68002</v>
+      </c>
+      <c r="P698">
+        <v>89.61386076740408</v>
+      </c>
+      <c r="Q698">
+        <v>32.004</v>
+      </c>
+      <c r="R698">
+        <v>388.41665</v>
+      </c>
+      <c r="S698">
+        <v>5.060001129028405</v>
+      </c>
+      <c r="T698">
+        <v>543.07999</v>
+      </c>
+      <c r="U698">
+        <v>8</v>
+      </c>
+      <c r="V698">
+        <v>14</v>
+      </c>
+      <c r="W698">
+        <v>22</v>
+      </c>
+      <c r="X698">
+        <v>32</v>
+      </c>
+      <c r="Y698">
+        <v>8</v>
+      </c>
+      <c r="Z698">
+        <v>39</v>
+      </c>
+      <c r="AA698">
+        <v>14</v>
+      </c>
+      <c r="AB698">
+        <v>6</v>
+      </c>
+      <c r="AC698">
+        <v>4.20332</v>
+      </c>
+      <c r="AD698">
+        <v>-2.09064</v>
+      </c>
+      <c r="AE698">
+        <v>0</v>
+      </c>
+      <c r="AF698">
+        <v>362.8471</v>
+      </c>
+      <c r="AG698">
+        <v>0</v>
+      </c>
+      <c r="AH698">
+        <v>3</v>
+      </c>
+      <c r="AI698">
+        <v>1165.24995</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B699" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E699">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F699">
+        <v>5338.45</v>
+      </c>
+      <c r="G699">
+        <v>69.54532723368499</v>
+      </c>
+      <c r="H699">
+        <v>74.84999999999999</v>
+      </c>
+      <c r="I699">
+        <v>0</v>
+      </c>
+      <c r="J699">
+        <v>0</v>
+      </c>
+      <c r="K699">
+        <v>0.9750897251901435</v>
+      </c>
+      <c r="L699">
+        <v>0</v>
+      </c>
+      <c r="M699">
+        <v>1</v>
+      </c>
+      <c r="N699">
+        <v>0</v>
+      </c>
+      <c r="O699">
+        <v>25.44296</v>
+      </c>
+      <c r="P699">
+        <v>70.67488888888889</v>
+      </c>
+      <c r="Q699">
+        <v>36</v>
+      </c>
+      <c r="R699">
+        <v>511.33966</v>
+      </c>
+      <c r="S699">
+        <v>6.661350014004294</v>
+      </c>
+      <c r="T699">
+        <v>542.70001</v>
+      </c>
+      <c r="U699">
+        <v>9</v>
+      </c>
+      <c r="V699">
+        <v>15</v>
+      </c>
+      <c r="W699">
+        <v>24</v>
+      </c>
+      <c r="X699">
+        <v>37</v>
+      </c>
+      <c r="Y699">
+        <v>9</v>
+      </c>
+      <c r="Z699">
+        <v>46</v>
+      </c>
+      <c r="AA699">
+        <v>15</v>
+      </c>
+      <c r="AB699">
+        <v>13</v>
+      </c>
+      <c r="AC699">
+        <v>4.42596</v>
+      </c>
+      <c r="AD699">
+        <v>-1.76968</v>
+      </c>
+      <c r="AE699">
+        <v>0</v>
+      </c>
+      <c r="AF699">
+        <v>1209.306</v>
+      </c>
+      <c r="AG699">
+        <v>0</v>
+      </c>
+      <c r="AH699">
+        <v>3</v>
+      </c>
+      <c r="AI699">
+        <v>1534.01898</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B700" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Sesión 40</t>
+        </is>
+      </c>
+      <c r="E700">
+        <v>76.76216666666667</v>
+      </c>
+      <c r="F700">
+        <v>5422.27</v>
+      </c>
+      <c r="G700">
+        <v>70.6372713988879</v>
+      </c>
+      <c r="H700">
+        <v>159.67</v>
+      </c>
+      <c r="I700">
+        <v>0</v>
+      </c>
+      <c r="J700">
+        <v>0</v>
+      </c>
+      <c r="K700">
+        <v>2.080061141230598</v>
+      </c>
+      <c r="L700">
+        <v>0</v>
+      </c>
+      <c r="M700">
+        <v>4</v>
+      </c>
+      <c r="N700">
+        <v>0</v>
+      </c>
+      <c r="O700">
+        <v>25.7063</v>
+      </c>
+      <c r="P700">
+        <v>71.40638888888888</v>
+      </c>
+      <c r="Q700">
+        <v>36</v>
+      </c>
+      <c r="R700">
+        <v>527.02124</v>
+      </c>
+      <c r="S700">
+        <v>6.865637890193303</v>
+      </c>
+      <c r="T700">
+        <v>723.26001</v>
+      </c>
+      <c r="U700">
+        <v>15</v>
+      </c>
+      <c r="V700">
+        <v>17</v>
+      </c>
+      <c r="W700">
+        <v>32</v>
+      </c>
+      <c r="X700">
+        <v>49</v>
+      </c>
+      <c r="Y700">
+        <v>15</v>
+      </c>
+      <c r="Z700">
+        <v>41</v>
+      </c>
+      <c r="AA700">
+        <v>17</v>
+      </c>
+      <c r="AB700">
+        <v>7</v>
+      </c>
+      <c r="AC700">
+        <v>4.67919</v>
+      </c>
+      <c r="AD700">
+        <v>-2.07731</v>
+      </c>
+      <c r="AE700">
+        <v>0</v>
+      </c>
+      <c r="AF700">
+        <v>1248.912</v>
+      </c>
+      <c r="AG700">
+        <v>0</v>
+      </c>
+      <c r="AH700">
+        <v>3</v>
+      </c>
+      <c r="AI700">
+        <v>1581.06372</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B701" s="2">
+        <v>46225</v>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Sesión vespertina 22 de Julio | Sesión 40</t>
+        </is>
+      </c>
+      <c r="E701">
+        <v>91.16066666666666</v>
+      </c>
+      <c r="F701">
+        <v>5294.52</v>
+      </c>
+      <c r="G701">
+        <v>58.0789960582415</v>
+      </c>
+      <c r="H701">
+        <v>128.82</v>
+      </c>
+      <c r="I701">
+        <v>0</v>
+      </c>
+      <c r="J701">
+        <v>0</v>
+      </c>
+      <c r="K701">
+        <v>1.41310945510125</v>
+      </c>
+      <c r="L701">
+        <v>0</v>
+      </c>
+      <c r="M701">
+        <v>2</v>
+      </c>
+      <c r="N701">
+        <v>0</v>
+      </c>
+      <c r="O701">
+        <v>26.43033</v>
+      </c>
+      <c r="P701">
+        <v>75.53249314128945</v>
+      </c>
+      <c r="Q701">
+        <v>34.992</v>
+      </c>
+      <c r="R701">
+        <v>614.43372</v>
+      </c>
+      <c r="S701">
+        <v>6.740118764671899</v>
+      </c>
+      <c r="T701">
+        <v>1143.04</v>
+      </c>
+      <c r="U701">
+        <v>57</v>
+      </c>
+      <c r="V701">
+        <v>66</v>
+      </c>
+      <c r="W701">
+        <v>123</v>
+      </c>
+      <c r="X701">
+        <v>140</v>
+      </c>
+      <c r="Y701">
+        <v>57</v>
+      </c>
+      <c r="Z701">
+        <v>137</v>
+      </c>
+      <c r="AA701">
+        <v>66</v>
+      </c>
+      <c r="AB701">
+        <v>54</v>
+      </c>
+      <c r="AC701">
+        <v>4.46656</v>
+      </c>
+      <c r="AD701">
+        <v>-3.48318</v>
+      </c>
+      <c r="AE701">
+        <v>0</v>
+      </c>
+      <c r="AF701">
+        <v>548.2144</v>
+      </c>
+      <c r="AG701">
+        <v>0</v>
+      </c>
+      <c r="AH701">
+        <v>3</v>
+      </c>
+      <c r="AI701">
+        <v>1843.30116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-24
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI701"/>
+  <dimension ref="A1:AI725"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -79528,6 +79528,2718 @@
         <v>1843.30116</v>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B702" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E702">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F702">
+        <v>2963.76</v>
+      </c>
+      <c r="G702">
+        <v>36.95184898885371</v>
+      </c>
+      <c r="H702">
+        <v>149.59</v>
+      </c>
+      <c r="I702">
+        <v>0</v>
+      </c>
+      <c r="J702">
+        <v>0</v>
+      </c>
+      <c r="K702">
+        <v>1.865072438470938</v>
+      </c>
+      <c r="L702">
+        <v>1.49</v>
+      </c>
+      <c r="M702">
+        <v>2</v>
+      </c>
+      <c r="N702">
+        <v>0</v>
+      </c>
+      <c r="O702">
+        <v>29.90848</v>
+      </c>
+      <c r="P702">
+        <v>83.07911111111112</v>
+      </c>
+      <c r="Q702">
+        <v>36</v>
+      </c>
+      <c r="R702">
+        <v>341.85928</v>
+      </c>
+      <c r="S702">
+        <v>4.262265665910282</v>
+      </c>
+      <c r="T702">
+        <v>422.15001</v>
+      </c>
+      <c r="U702">
+        <v>19</v>
+      </c>
+      <c r="V702">
+        <v>10</v>
+      </c>
+      <c r="W702">
+        <v>29</v>
+      </c>
+      <c r="X702">
+        <v>39</v>
+      </c>
+      <c r="Y702">
+        <v>19</v>
+      </c>
+      <c r="Z702">
+        <v>33</v>
+      </c>
+      <c r="AA702">
+        <v>10</v>
+      </c>
+      <c r="AB702">
+        <v>17</v>
+      </c>
+      <c r="AC702">
+        <v>4.73487</v>
+      </c>
+      <c r="AD702">
+        <v>-0.20299</v>
+      </c>
+      <c r="AE702">
+        <v>0</v>
+      </c>
+      <c r="AF702">
+        <v>683.3599999999999</v>
+      </c>
+      <c r="AG702">
+        <v>0</v>
+      </c>
+      <c r="AH702">
+        <v>3</v>
+      </c>
+      <c r="AI702">
+        <v>1025.57784</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B703" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Sesión AM Seleccionados</t>
+        </is>
+      </c>
+      <c r="E703">
+        <v>77.31700000000001</v>
+      </c>
+      <c r="F703">
+        <v>7539.240000000001</v>
+      </c>
+      <c r="G703">
+        <v>97.51076736034766</v>
+      </c>
+      <c r="H703">
+        <v>106.56</v>
+      </c>
+      <c r="I703">
+        <v>0</v>
+      </c>
+      <c r="J703">
+        <v>0</v>
+      </c>
+      <c r="K703">
+        <v>1.378222124500433</v>
+      </c>
+      <c r="L703">
+        <v>0</v>
+      </c>
+      <c r="M703">
+        <v>1</v>
+      </c>
+      <c r="N703">
+        <v>0</v>
+      </c>
+      <c r="O703">
+        <v>25.70888</v>
+      </c>
+      <c r="P703">
+        <v>79.43665801507849</v>
+      </c>
+      <c r="Q703">
+        <v>32.364</v>
+      </c>
+      <c r="R703">
+        <v>776.4910600000001</v>
+      </c>
+      <c r="S703">
+        <v>10.04295381352096</v>
+      </c>
+      <c r="T703">
+        <v>862.27</v>
+      </c>
+      <c r="U703">
+        <v>16</v>
+      </c>
+      <c r="V703">
+        <v>10</v>
+      </c>
+      <c r="W703">
+        <v>26</v>
+      </c>
+      <c r="X703">
+        <v>111</v>
+      </c>
+      <c r="Y703">
+        <v>16</v>
+      </c>
+      <c r="Z703">
+        <v>60</v>
+      </c>
+      <c r="AA703">
+        <v>10</v>
+      </c>
+      <c r="AB703">
+        <v>20</v>
+      </c>
+      <c r="AC703">
+        <v>3.70159</v>
+      </c>
+      <c r="AD703">
+        <v>-2.23486</v>
+      </c>
+      <c r="AE703">
+        <v>0</v>
+      </c>
+      <c r="AF703">
+        <v>618.3226</v>
+      </c>
+      <c r="AG703">
+        <v>0</v>
+      </c>
+      <c r="AH703">
+        <v>3</v>
+      </c>
+      <c r="AI703">
+        <v>2329.47318</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B704" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E704">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F704">
+        <v>2549.14</v>
+      </c>
+      <c r="G704">
+        <v>31.78241029349426</v>
+      </c>
+      <c r="H704">
+        <v>40.61</v>
+      </c>
+      <c r="I704">
+        <v>0</v>
+      </c>
+      <c r="J704">
+        <v>0</v>
+      </c>
+      <c r="K704">
+        <v>0.5063212228511583</v>
+      </c>
+      <c r="L704">
+        <v>0</v>
+      </c>
+      <c r="M704">
+        <v>1</v>
+      </c>
+      <c r="N704">
+        <v>0</v>
+      </c>
+      <c r="O704">
+        <v>25.88164</v>
+      </c>
+      <c r="P704">
+        <v>71.89344444444444</v>
+      </c>
+      <c r="Q704">
+        <v>36</v>
+      </c>
+      <c r="R704">
+        <v>243.61819</v>
+      </c>
+      <c r="S704">
+        <v>3.037406054409895</v>
+      </c>
+      <c r="T704">
+        <v>228.8</v>
+      </c>
+      <c r="U704">
+        <v>12</v>
+      </c>
+      <c r="V704">
+        <v>4</v>
+      </c>
+      <c r="W704">
+        <v>16</v>
+      </c>
+      <c r="X704">
+        <v>26</v>
+      </c>
+      <c r="Y704">
+        <v>12</v>
+      </c>
+      <c r="Z704">
+        <v>22</v>
+      </c>
+      <c r="AA704">
+        <v>4</v>
+      </c>
+      <c r="AB704">
+        <v>14</v>
+      </c>
+      <c r="AC704">
+        <v>4.83809</v>
+      </c>
+      <c r="AD704">
+        <v>0</v>
+      </c>
+      <c r="AE704">
+        <v>0</v>
+      </c>
+      <c r="AF704">
+        <v>566.2560000000001</v>
+      </c>
+      <c r="AG704">
+        <v>0</v>
+      </c>
+      <c r="AH704">
+        <v>3</v>
+      </c>
+      <c r="AI704">
+        <v>730.8545700000001</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B705" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E705">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F705">
+        <v>3265.5</v>
+      </c>
+      <c r="G705">
+        <v>40.71391167743062</v>
+      </c>
+      <c r="H705">
+        <v>96.52999999999999</v>
+      </c>
+      <c r="I705">
+        <v>0</v>
+      </c>
+      <c r="J705">
+        <v>0</v>
+      </c>
+      <c r="K705">
+        <v>1.203525920754058</v>
+      </c>
+      <c r="L705">
+        <v>0</v>
+      </c>
+      <c r="M705">
+        <v>1</v>
+      </c>
+      <c r="N705">
+        <v>0</v>
+      </c>
+      <c r="O705">
+        <v>25.21399</v>
+      </c>
+      <c r="P705">
+        <v>77.82095679012345</v>
+      </c>
+      <c r="Q705">
+        <v>32.4</v>
+      </c>
+      <c r="R705">
+        <v>360.49361</v>
+      </c>
+      <c r="S705">
+        <v>4.494596538912301</v>
+      </c>
+      <c r="T705">
+        <v>410.13001</v>
+      </c>
+      <c r="U705">
+        <v>14</v>
+      </c>
+      <c r="V705">
+        <v>8</v>
+      </c>
+      <c r="W705">
+        <v>22</v>
+      </c>
+      <c r="X705">
+        <v>37</v>
+      </c>
+      <c r="Y705">
+        <v>14</v>
+      </c>
+      <c r="Z705">
+        <v>28</v>
+      </c>
+      <c r="AA705">
+        <v>8</v>
+      </c>
+      <c r="AB705">
+        <v>6</v>
+      </c>
+      <c r="AC705">
+        <v>4.36484</v>
+      </c>
+      <c r="AD705">
+        <v>-0.56024</v>
+      </c>
+      <c r="AE705">
+        <v>0</v>
+      </c>
+      <c r="AF705">
+        <v>261.1322</v>
+      </c>
+      <c r="AG705">
+        <v>0</v>
+      </c>
+      <c r="AH705">
+        <v>3</v>
+      </c>
+      <c r="AI705">
+        <v>1081.48083</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B706" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Sesión AM Seleccionados</t>
+        </is>
+      </c>
+      <c r="E706">
+        <v>77.31700000000001</v>
+      </c>
+      <c r="F706">
+        <v>7162.740000000001</v>
+      </c>
+      <c r="G706">
+        <v>92.641204392307</v>
+      </c>
+      <c r="H706">
+        <v>73.86999999999999</v>
+      </c>
+      <c r="I706">
+        <v>0</v>
+      </c>
+      <c r="J706">
+        <v>0</v>
+      </c>
+      <c r="K706">
+        <v>0.9554173079659064</v>
+      </c>
+      <c r="L706">
+        <v>0</v>
+      </c>
+      <c r="M706">
+        <v>1</v>
+      </c>
+      <c r="N706">
+        <v>0</v>
+      </c>
+      <c r="O706">
+        <v>25.6321</v>
+      </c>
+      <c r="P706">
+        <v>71.99219188855184</v>
+      </c>
+      <c r="Q706">
+        <v>35.604</v>
+      </c>
+      <c r="R706">
+        <v>637.59048</v>
+      </c>
+      <c r="S706">
+        <v>8.246446189065793</v>
+      </c>
+      <c r="T706">
+        <v>922.3099999999999</v>
+      </c>
+      <c r="U706">
+        <v>26</v>
+      </c>
+      <c r="V706">
+        <v>18</v>
+      </c>
+      <c r="W706">
+        <v>44</v>
+      </c>
+      <c r="X706">
+        <v>123</v>
+      </c>
+      <c r="Y706">
+        <v>26</v>
+      </c>
+      <c r="Z706">
+        <v>83</v>
+      </c>
+      <c r="AA706">
+        <v>18</v>
+      </c>
+      <c r="AB706">
+        <v>26</v>
+      </c>
+      <c r="AC706">
+        <v>5.02576</v>
+      </c>
+      <c r="AD706">
+        <v>-2.24373</v>
+      </c>
+      <c r="AE706">
+        <v>0</v>
+      </c>
+      <c r="AF706">
+        <v>608.3457500000001</v>
+      </c>
+      <c r="AG706">
+        <v>0</v>
+      </c>
+      <c r="AH706">
+        <v>3</v>
+      </c>
+      <c r="AI706">
+        <v>1912.77144</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B707" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E707">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F707">
+        <v>3590.06</v>
+      </c>
+      <c r="G707">
+        <v>44.76049173378551</v>
+      </c>
+      <c r="H707">
+        <v>203.88</v>
+      </c>
+      <c r="I707">
+        <v>0</v>
+      </c>
+      <c r="J707">
+        <v>0</v>
+      </c>
+      <c r="K707">
+        <v>2.541954467246839</v>
+      </c>
+      <c r="L707">
+        <v>0</v>
+      </c>
+      <c r="M707">
+        <v>3</v>
+      </c>
+      <c r="N707">
+        <v>0</v>
+      </c>
+      <c r="O707">
+        <v>28.32644</v>
+      </c>
+      <c r="P707">
+        <v>83.35228342749529</v>
+      </c>
+      <c r="Q707">
+        <v>33.984</v>
+      </c>
+      <c r="R707">
+        <v>441.0741</v>
+      </c>
+      <c r="S707">
+        <v>5.499265640974492</v>
+      </c>
+      <c r="T707">
+        <v>538.38999</v>
+      </c>
+      <c r="U707">
+        <v>18</v>
+      </c>
+      <c r="V707">
+        <v>6</v>
+      </c>
+      <c r="W707">
+        <v>24</v>
+      </c>
+      <c r="X707">
+        <v>44</v>
+      </c>
+      <c r="Y707">
+        <v>18</v>
+      </c>
+      <c r="Z707">
+        <v>39</v>
+      </c>
+      <c r="AA707">
+        <v>6</v>
+      </c>
+      <c r="AB707">
+        <v>13</v>
+      </c>
+      <c r="AC707">
+        <v>4.48081</v>
+      </c>
+      <c r="AD707">
+        <v>0</v>
+      </c>
+      <c r="AE707">
+        <v>0</v>
+      </c>
+      <c r="AF707">
+        <v>329.116</v>
+      </c>
+      <c r="AG707">
+        <v>0</v>
+      </c>
+      <c r="AH707">
+        <v>3</v>
+      </c>
+      <c r="AI707">
+        <v>1323.2223</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B708" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E708">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F708">
+        <v>3000.43</v>
+      </c>
+      <c r="G708">
+        <v>37.40904670473532</v>
+      </c>
+      <c r="H708">
+        <v>94.19000000000001</v>
+      </c>
+      <c r="I708">
+        <v>0</v>
+      </c>
+      <c r="J708">
+        <v>0</v>
+      </c>
+      <c r="K708">
+        <v>1.174351046056405</v>
+      </c>
+      <c r="L708">
+        <v>0</v>
+      </c>
+      <c r="M708">
+        <v>1</v>
+      </c>
+      <c r="N708">
+        <v>0</v>
+      </c>
+      <c r="O708">
+        <v>29.0503</v>
+      </c>
+      <c r="P708">
+        <v>81.67538236617185</v>
+      </c>
+      <c r="Q708">
+        <v>35.568</v>
+      </c>
+      <c r="R708">
+        <v>274.19491</v>
+      </c>
+      <c r="S708">
+        <v>3.418633394010424</v>
+      </c>
+      <c r="T708">
+        <v>383.55001</v>
+      </c>
+      <c r="U708">
+        <v>25</v>
+      </c>
+      <c r="V708">
+        <v>7</v>
+      </c>
+      <c r="W708">
+        <v>32</v>
+      </c>
+      <c r="X708">
+        <v>45</v>
+      </c>
+      <c r="Y708">
+        <v>25</v>
+      </c>
+      <c r="Z708">
+        <v>31</v>
+      </c>
+      <c r="AA708">
+        <v>7</v>
+      </c>
+      <c r="AB708">
+        <v>7</v>
+      </c>
+      <c r="AC708">
+        <v>4.77666</v>
+      </c>
+      <c r="AD708">
+        <v>0</v>
+      </c>
+      <c r="AE708">
+        <v>0</v>
+      </c>
+      <c r="AF708">
+        <v>280.46</v>
+      </c>
+      <c r="AG708">
+        <v>0</v>
+      </c>
+      <c r="AH708">
+        <v>3</v>
+      </c>
+      <c r="AI708">
+        <v>822.58473</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B709" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E709">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F709">
+        <v>3115.03</v>
+      </c>
+      <c r="G709">
+        <v>38.83786749121013</v>
+      </c>
+      <c r="H709">
+        <v>74</v>
+      </c>
+      <c r="I709">
+        <v>0</v>
+      </c>
+      <c r="J709">
+        <v>0</v>
+      </c>
+      <c r="K709">
+        <v>0.9226242425753686</v>
+      </c>
+      <c r="L709">
+        <v>0</v>
+      </c>
+      <c r="M709">
+        <v>1</v>
+      </c>
+      <c r="N709">
+        <v>0</v>
+      </c>
+      <c r="O709">
+        <v>25.61625</v>
+      </c>
+      <c r="P709">
+        <v>71.15625</v>
+      </c>
+      <c r="Q709">
+        <v>36</v>
+      </c>
+      <c r="R709">
+        <v>295.1206</v>
+      </c>
+      <c r="S709">
+        <v>3.679532703289031</v>
+      </c>
+      <c r="T709">
+        <v>318.46999</v>
+      </c>
+      <c r="U709">
+        <v>11</v>
+      </c>
+      <c r="V709">
+        <v>2</v>
+      </c>
+      <c r="W709">
+        <v>13</v>
+      </c>
+      <c r="X709">
+        <v>31</v>
+      </c>
+      <c r="Y709">
+        <v>11</v>
+      </c>
+      <c r="Z709">
+        <v>20</v>
+      </c>
+      <c r="AA709">
+        <v>2</v>
+      </c>
+      <c r="AB709">
+        <v>10</v>
+      </c>
+      <c r="AC709">
+        <v>4.15333</v>
+      </c>
+      <c r="AD709">
+        <v>0</v>
+      </c>
+      <c r="AE709">
+        <v>0</v>
+      </c>
+      <c r="AF709">
+        <v>693.3480000000001</v>
+      </c>
+      <c r="AG709">
+        <v>0</v>
+      </c>
+      <c r="AH709">
+        <v>3</v>
+      </c>
+      <c r="AI709">
+        <v>885.3617999999999</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B710" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E710">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F710">
+        <v>3628.85</v>
+      </c>
+      <c r="G710">
+        <v>45.24412138742738</v>
+      </c>
+      <c r="H710">
+        <v>198.04</v>
+      </c>
+      <c r="I710">
+        <v>0</v>
+      </c>
+      <c r="J710">
+        <v>0</v>
+      </c>
+      <c r="K710">
+        <v>2.469141959454405</v>
+      </c>
+      <c r="L710">
+        <v>0</v>
+      </c>
+      <c r="M710">
+        <v>4</v>
+      </c>
+      <c r="N710">
+        <v>0</v>
+      </c>
+      <c r="O710">
+        <v>28.77386</v>
+      </c>
+      <c r="P710">
+        <v>79.92738888888888</v>
+      </c>
+      <c r="Q710">
+        <v>36</v>
+      </c>
+      <c r="R710">
+        <v>359.9031</v>
+      </c>
+      <c r="S710">
+        <v>4.487234122135502</v>
+      </c>
+      <c r="T710">
+        <v>453.30999</v>
+      </c>
+      <c r="U710">
+        <v>15</v>
+      </c>
+      <c r="V710">
+        <v>7</v>
+      </c>
+      <c r="W710">
+        <v>22</v>
+      </c>
+      <c r="X710">
+        <v>34</v>
+      </c>
+      <c r="Y710">
+        <v>15</v>
+      </c>
+      <c r="Z710">
+        <v>23</v>
+      </c>
+      <c r="AA710">
+        <v>7</v>
+      </c>
+      <c r="AB710">
+        <v>10</v>
+      </c>
+      <c r="AC710">
+        <v>4.2892</v>
+      </c>
+      <c r="AD710">
+        <v>0</v>
+      </c>
+      <c r="AE710">
+        <v>0</v>
+      </c>
+      <c r="AF710">
+        <v>288.1011</v>
+      </c>
+      <c r="AG710">
+        <v>0</v>
+      </c>
+      <c r="AH710">
+        <v>3</v>
+      </c>
+      <c r="AI710">
+        <v>1079.7093</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B711" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E711">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F711">
+        <v>3543.74</v>
+      </c>
+      <c r="G711">
+        <v>44.18297882951401</v>
+      </c>
+      <c r="H711">
+        <v>194.01</v>
+      </c>
+      <c r="I711">
+        <v>0</v>
+      </c>
+      <c r="J711">
+        <v>0</v>
+      </c>
+      <c r="K711">
+        <v>2.418896341919557</v>
+      </c>
+      <c r="L711">
+        <v>0</v>
+      </c>
+      <c r="M711">
+        <v>5</v>
+      </c>
+      <c r="N711">
+        <v>0</v>
+      </c>
+      <c r="O711">
+        <v>27.75937</v>
+      </c>
+      <c r="P711">
+        <v>86.73718910136233</v>
+      </c>
+      <c r="Q711">
+        <v>32.004</v>
+      </c>
+      <c r="R711">
+        <v>401.59325</v>
+      </c>
+      <c r="S711">
+        <v>5.007022541954468</v>
+      </c>
+      <c r="T711">
+        <v>535.77</v>
+      </c>
+      <c r="U711">
+        <v>20</v>
+      </c>
+      <c r="V711">
+        <v>11</v>
+      </c>
+      <c r="W711">
+        <v>31</v>
+      </c>
+      <c r="X711">
+        <v>48</v>
+      </c>
+      <c r="Y711">
+        <v>20</v>
+      </c>
+      <c r="Z711">
+        <v>42</v>
+      </c>
+      <c r="AA711">
+        <v>11</v>
+      </c>
+      <c r="AB711">
+        <v>11</v>
+      </c>
+      <c r="AC711">
+        <v>4.94633</v>
+      </c>
+      <c r="AD711">
+        <v>0</v>
+      </c>
+      <c r="AE711">
+        <v>0</v>
+      </c>
+      <c r="AF711">
+        <v>246.8706</v>
+      </c>
+      <c r="AG711">
+        <v>0</v>
+      </c>
+      <c r="AH711">
+        <v>3</v>
+      </c>
+      <c r="AI711">
+        <v>1204.77975</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B712" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E712">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F712">
+        <v>2728.05</v>
+      </c>
+      <c r="G712">
+        <v>34.01304141834776</v>
+      </c>
+      <c r="H712">
+        <v>78.09</v>
+      </c>
+      <c r="I712">
+        <v>0</v>
+      </c>
+      <c r="J712">
+        <v>0</v>
+      </c>
+      <c r="K712">
+        <v>0.9736179338204126</v>
+      </c>
+      <c r="L712">
+        <v>0</v>
+      </c>
+      <c r="M712">
+        <v>2</v>
+      </c>
+      <c r="N712">
+        <v>0</v>
+      </c>
+      <c r="O712">
+        <v>27.73173</v>
+      </c>
+      <c r="P712">
+        <v>81.94955673758864</v>
+      </c>
+      <c r="Q712">
+        <v>33.84</v>
+      </c>
+      <c r="R712">
+        <v>267.11839</v>
+      </c>
+      <c r="S712">
+        <v>3.330404084482458</v>
+      </c>
+      <c r="T712">
+        <v>305.02</v>
+      </c>
+      <c r="U712">
+        <v>13</v>
+      </c>
+      <c r="V712">
+        <v>6</v>
+      </c>
+      <c r="W712">
+        <v>19</v>
+      </c>
+      <c r="X712">
+        <v>25</v>
+      </c>
+      <c r="Y712">
+        <v>13</v>
+      </c>
+      <c r="Z712">
+        <v>25</v>
+      </c>
+      <c r="AA712">
+        <v>6</v>
+      </c>
+      <c r="AB712">
+        <v>3</v>
+      </c>
+      <c r="AC712">
+        <v>4.44957</v>
+      </c>
+      <c r="AD712">
+        <v>0</v>
+      </c>
+      <c r="AE712">
+        <v>0</v>
+      </c>
+      <c r="AF712">
+        <v>215.4495</v>
+      </c>
+      <c r="AG712">
+        <v>0</v>
+      </c>
+      <c r="AH712">
+        <v>3</v>
+      </c>
+      <c r="AI712">
+        <v>801.3551699999999</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B713" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E713">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F713">
+        <v>3126.47</v>
+      </c>
+      <c r="G713">
+        <v>38.98050021195422</v>
+      </c>
+      <c r="H713">
+        <v>105.06</v>
+      </c>
+      <c r="I713">
+        <v>0</v>
+      </c>
+      <c r="J713">
+        <v>0</v>
+      </c>
+      <c r="K713">
+        <v>1.309877066553625</v>
+      </c>
+      <c r="L713">
+        <v>0</v>
+      </c>
+      <c r="M713">
+        <v>0</v>
+      </c>
+      <c r="N713">
+        <v>0</v>
+      </c>
+      <c r="O713">
+        <v>23.51797</v>
+      </c>
+      <c r="P713">
+        <v>69.79454534662868</v>
+      </c>
+      <c r="Q713">
+        <v>33.696</v>
+      </c>
+      <c r="R713">
+        <v>333.59158</v>
+      </c>
+      <c r="S713">
+        <v>4.159184849013791</v>
+      </c>
+      <c r="T713">
+        <v>356.6</v>
+      </c>
+      <c r="U713">
+        <v>17</v>
+      </c>
+      <c r="V713">
+        <v>8</v>
+      </c>
+      <c r="W713">
+        <v>25</v>
+      </c>
+      <c r="X713">
+        <v>34</v>
+      </c>
+      <c r="Y713">
+        <v>17</v>
+      </c>
+      <c r="Z713">
+        <v>19</v>
+      </c>
+      <c r="AA713">
+        <v>8</v>
+      </c>
+      <c r="AB713">
+        <v>12</v>
+      </c>
+      <c r="AC713">
+        <v>4.51538</v>
+      </c>
+      <c r="AD713">
+        <v>0</v>
+      </c>
+      <c r="AE713">
+        <v>0</v>
+      </c>
+      <c r="AF713">
+        <v>280.7152</v>
+      </c>
+      <c r="AG713">
+        <v>0</v>
+      </c>
+      <c r="AH713">
+        <v>3</v>
+      </c>
+      <c r="AI713">
+        <v>1000.77474</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B714" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E714">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F714">
+        <v>3617.89</v>
+      </c>
+      <c r="G714">
+        <v>45.10747325636486</v>
+      </c>
+      <c r="H714">
+        <v>275.09</v>
+      </c>
+      <c r="I714">
+        <v>0</v>
+      </c>
+      <c r="J714">
+        <v>0</v>
+      </c>
+      <c r="K714">
+        <v>3.429793282298083</v>
+      </c>
+      <c r="L714">
+        <v>16.72</v>
+      </c>
+      <c r="M714">
+        <v>7</v>
+      </c>
+      <c r="N714">
+        <v>1</v>
+      </c>
+      <c r="O714">
+        <v>30.543</v>
+      </c>
+      <c r="P714">
+        <v>87.28566529492457</v>
+      </c>
+      <c r="Q714">
+        <v>34.992</v>
+      </c>
+      <c r="R714">
+        <v>322.61415</v>
+      </c>
+      <c r="S714">
+        <v>4.022319402538464</v>
+      </c>
+      <c r="T714">
+        <v>530.09001</v>
+      </c>
+      <c r="U714">
+        <v>20</v>
+      </c>
+      <c r="V714">
+        <v>11</v>
+      </c>
+      <c r="W714">
+        <v>31</v>
+      </c>
+      <c r="X714">
+        <v>39</v>
+      </c>
+      <c r="Y714">
+        <v>20</v>
+      </c>
+      <c r="Z714">
+        <v>34</v>
+      </c>
+      <c r="AA714">
+        <v>11</v>
+      </c>
+      <c r="AB714">
+        <v>6</v>
+      </c>
+      <c r="AC714">
+        <v>4.65197</v>
+      </c>
+      <c r="AD714">
+        <v>-0.23782</v>
+      </c>
+      <c r="AE714">
+        <v>0</v>
+      </c>
+      <c r="AF714">
+        <v>287.95632</v>
+      </c>
+      <c r="AG714">
+        <v>0</v>
+      </c>
+      <c r="AH714">
+        <v>3</v>
+      </c>
+      <c r="AI714">
+        <v>967.84245</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B715" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Sesión AM Seleccionados</t>
+        </is>
+      </c>
+      <c r="E715">
+        <v>77.31700000000001</v>
+      </c>
+      <c r="F715">
+        <v>7708.71</v>
+      </c>
+      <c r="G715">
+        <v>99.7026527154442</v>
+      </c>
+      <c r="H715">
+        <v>84.55</v>
+      </c>
+      <c r="I715">
+        <v>0</v>
+      </c>
+      <c r="J715">
+        <v>0</v>
+      </c>
+      <c r="K715">
+        <v>1.093549930804351</v>
+      </c>
+      <c r="L715">
+        <v>0</v>
+      </c>
+      <c r="M715">
+        <v>0</v>
+      </c>
+      <c r="N715">
+        <v>0</v>
+      </c>
+      <c r="O715">
+        <v>23.13447</v>
+      </c>
+      <c r="P715">
+        <v>70.07897128316975</v>
+      </c>
+      <c r="Q715">
+        <v>33.012</v>
+      </c>
+      <c r="R715">
+        <v>867.40355</v>
+      </c>
+      <c r="S715">
+        <v>11.21879470232937</v>
+      </c>
+      <c r="T715">
+        <v>1064.57001</v>
+      </c>
+      <c r="U715">
+        <v>20</v>
+      </c>
+      <c r="V715">
+        <v>25</v>
+      </c>
+      <c r="W715">
+        <v>45</v>
+      </c>
+      <c r="X715">
+        <v>131</v>
+      </c>
+      <c r="Y715">
+        <v>20</v>
+      </c>
+      <c r="Z715">
+        <v>118</v>
+      </c>
+      <c r="AA715">
+        <v>25</v>
+      </c>
+      <c r="AB715">
+        <v>33</v>
+      </c>
+      <c r="AC715">
+        <v>4.09001</v>
+      </c>
+      <c r="AD715">
+        <v>-2.1134</v>
+      </c>
+      <c r="AE715">
+        <v>0</v>
+      </c>
+      <c r="AF715">
+        <v>729.43494</v>
+      </c>
+      <c r="AG715">
+        <v>0</v>
+      </c>
+      <c r="AH715">
+        <v>3</v>
+      </c>
+      <c r="AI715">
+        <v>2602.21065</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B716" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E716">
+        <v>64.45333333333333</v>
+      </c>
+      <c r="F716">
+        <v>2962.26</v>
+      </c>
+      <c r="G716">
+        <v>45.95976417045924</v>
+      </c>
+      <c r="H716">
+        <v>0</v>
+      </c>
+      <c r="I716">
+        <v>0</v>
+      </c>
+      <c r="J716">
+        <v>0</v>
+      </c>
+      <c r="K716">
+        <v>0</v>
+      </c>
+      <c r="L716">
+        <v>0</v>
+      </c>
+      <c r="M716">
+        <v>0</v>
+      </c>
+      <c r="N716">
+        <v>0</v>
+      </c>
+      <c r="O716">
+        <v>17.19064</v>
+      </c>
+      <c r="P716">
+        <v>49.22863688430698</v>
+      </c>
+      <c r="Q716">
+        <v>34.92</v>
+      </c>
+      <c r="R716">
+        <v>347.36789</v>
+      </c>
+      <c r="S716">
+        <v>5.389448024410426</v>
+      </c>
+      <c r="T716">
+        <v>203.36</v>
+      </c>
+      <c r="U716">
+        <v>0</v>
+      </c>
+      <c r="V716">
+        <v>0</v>
+      </c>
+      <c r="W716">
+        <v>0</v>
+      </c>
+      <c r="X716">
+        <v>23</v>
+      </c>
+      <c r="Y716">
+        <v>0</v>
+      </c>
+      <c r="Z716">
+        <v>8</v>
+      </c>
+      <c r="AA716">
+        <v>0</v>
+      </c>
+      <c r="AB716">
+        <v>9</v>
+      </c>
+      <c r="AC716">
+        <v>2.93702</v>
+      </c>
+      <c r="AD716">
+        <v>-0.2193</v>
+      </c>
+      <c r="AE716">
+        <v>0</v>
+      </c>
+      <c r="AF716">
+        <v>262.1424</v>
+      </c>
+      <c r="AG716">
+        <v>0</v>
+      </c>
+      <c r="AH716">
+        <v>3</v>
+      </c>
+      <c r="AI716">
+        <v>1042.10367</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B717" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E717">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F717">
+        <v>3425.19</v>
+      </c>
+      <c r="G717">
+        <v>42.70490985711793</v>
+      </c>
+      <c r="H717">
+        <v>161.5</v>
+      </c>
+      <c r="I717">
+        <v>0</v>
+      </c>
+      <c r="J717">
+        <v>0</v>
+      </c>
+      <c r="K717">
+        <v>2.013565069944892</v>
+      </c>
+      <c r="L717">
+        <v>0</v>
+      </c>
+      <c r="M717">
+        <v>3</v>
+      </c>
+      <c r="N717">
+        <v>0</v>
+      </c>
+      <c r="O717">
+        <v>26.67096</v>
+      </c>
+      <c r="P717">
+        <v>76.22016460905351</v>
+      </c>
+      <c r="Q717">
+        <v>34.992</v>
+      </c>
+      <c r="R717">
+        <v>292.27294</v>
+      </c>
+      <c r="S717">
+        <v>3.644028376929407</v>
+      </c>
+      <c r="T717">
+        <v>491.53999</v>
+      </c>
+      <c r="U717">
+        <v>15</v>
+      </c>
+      <c r="V717">
+        <v>9</v>
+      </c>
+      <c r="W717">
+        <v>24</v>
+      </c>
+      <c r="X717">
+        <v>43</v>
+      </c>
+      <c r="Y717">
+        <v>15</v>
+      </c>
+      <c r="Z717">
+        <v>37</v>
+      </c>
+      <c r="AA717">
+        <v>9</v>
+      </c>
+      <c r="AB717">
+        <v>13</v>
+      </c>
+      <c r="AC717">
+        <v>4.62978</v>
+      </c>
+      <c r="AD717">
+        <v>0</v>
+      </c>
+      <c r="AE717">
+        <v>0</v>
+      </c>
+      <c r="AF717">
+        <v>282.722</v>
+      </c>
+      <c r="AG717">
+        <v>0</v>
+      </c>
+      <c r="AH717">
+        <v>3</v>
+      </c>
+      <c r="AI717">
+        <v>876.81882</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B718" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E718">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F718">
+        <v>2558.19</v>
+      </c>
+      <c r="G718">
+        <v>31.89524474478219</v>
+      </c>
+      <c r="H718">
+        <v>75.89</v>
+      </c>
+      <c r="I718">
+        <v>0</v>
+      </c>
+      <c r="J718">
+        <v>0</v>
+      </c>
+      <c r="K718">
+        <v>0.9461885644465503</v>
+      </c>
+      <c r="L718">
+        <v>0</v>
+      </c>
+      <c r="M718">
+        <v>1</v>
+      </c>
+      <c r="N718">
+        <v>0</v>
+      </c>
+      <c r="O718">
+        <v>29.50418</v>
+      </c>
+      <c r="P718">
+        <v>86.81785546139361</v>
+      </c>
+      <c r="Q718">
+        <v>33.984</v>
+      </c>
+      <c r="R718">
+        <v>256.27215</v>
+      </c>
+      <c r="S718">
+        <v>3.195174301174476</v>
+      </c>
+      <c r="T718">
+        <v>313.21</v>
+      </c>
+      <c r="U718">
+        <v>11</v>
+      </c>
+      <c r="V718">
+        <v>3</v>
+      </c>
+      <c r="W718">
+        <v>14</v>
+      </c>
+      <c r="X718">
+        <v>27</v>
+      </c>
+      <c r="Y718">
+        <v>11</v>
+      </c>
+      <c r="Z718">
+        <v>29</v>
+      </c>
+      <c r="AA718">
+        <v>3</v>
+      </c>
+      <c r="AB718">
+        <v>6</v>
+      </c>
+      <c r="AC718">
+        <v>4.3263</v>
+      </c>
+      <c r="AD718">
+        <v>0</v>
+      </c>
+      <c r="AE718">
+        <v>0</v>
+      </c>
+      <c r="AF718">
+        <v>233.2816</v>
+      </c>
+      <c r="AG718">
+        <v>0</v>
+      </c>
+      <c r="AH718">
+        <v>3</v>
+      </c>
+      <c r="AI718">
+        <v>768.81645</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B719" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E719">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F719">
+        <v>2623.37</v>
+      </c>
+      <c r="G719">
+        <v>32.70790215195871</v>
+      </c>
+      <c r="H719">
+        <v>42.91</v>
+      </c>
+      <c r="I719">
+        <v>0</v>
+      </c>
+      <c r="J719">
+        <v>0</v>
+      </c>
+      <c r="K719">
+        <v>0.5349973817420144</v>
+      </c>
+      <c r="L719">
+        <v>0</v>
+      </c>
+      <c r="M719">
+        <v>0</v>
+      </c>
+      <c r="N719">
+        <v>0</v>
+      </c>
+      <c r="O719">
+        <v>23.81939</v>
+      </c>
+      <c r="P719">
+        <v>68.07095907636031</v>
+      </c>
+      <c r="Q719">
+        <v>34.992</v>
+      </c>
+      <c r="R719">
+        <v>232.98958</v>
+      </c>
+      <c r="S719">
+        <v>2.904889659127746</v>
+      </c>
+      <c r="T719">
+        <v>248.06</v>
+      </c>
+      <c r="U719">
+        <v>10</v>
+      </c>
+      <c r="V719">
+        <v>7</v>
+      </c>
+      <c r="W719">
+        <v>17</v>
+      </c>
+      <c r="X719">
+        <v>28</v>
+      </c>
+      <c r="Y719">
+        <v>10</v>
+      </c>
+      <c r="Z719">
+        <v>29</v>
+      </c>
+      <c r="AA719">
+        <v>7</v>
+      </c>
+      <c r="AB719">
+        <v>8</v>
+      </c>
+      <c r="AC719">
+        <v>4.42053</v>
+      </c>
+      <c r="AD719">
+        <v>-0.67915</v>
+      </c>
+      <c r="AE719">
+        <v>0</v>
+      </c>
+      <c r="AF719">
+        <v>238.8696</v>
+      </c>
+      <c r="AG719">
+        <v>0</v>
+      </c>
+      <c r="AH719">
+        <v>3</v>
+      </c>
+      <c r="AI719">
+        <v>698.96874</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B720" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E720">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F720">
+        <v>2716.23</v>
+      </c>
+      <c r="G720">
+        <v>33.8656708974391</v>
+      </c>
+      <c r="H720">
+        <v>13.88</v>
+      </c>
+      <c r="I720">
+        <v>0</v>
+      </c>
+      <c r="J720">
+        <v>0</v>
+      </c>
+      <c r="K720">
+        <v>0.1730543849587313</v>
+      </c>
+      <c r="L720">
+        <v>0</v>
+      </c>
+      <c r="M720">
+        <v>0</v>
+      </c>
+      <c r="N720">
+        <v>0</v>
+      </c>
+      <c r="O720">
+        <v>21.52502</v>
+      </c>
+      <c r="P720">
+        <v>65.20362292499698</v>
+      </c>
+      <c r="Q720">
+        <v>33.012</v>
+      </c>
+      <c r="R720">
+        <v>258.10877</v>
+      </c>
+      <c r="S720">
+        <v>3.218073086801486</v>
+      </c>
+      <c r="T720">
+        <v>254.87</v>
+      </c>
+      <c r="U720">
+        <v>11</v>
+      </c>
+      <c r="V720">
+        <v>7</v>
+      </c>
+      <c r="W720">
+        <v>18</v>
+      </c>
+      <c r="X720">
+        <v>30</v>
+      </c>
+      <c r="Y720">
+        <v>11</v>
+      </c>
+      <c r="Z720">
+        <v>29</v>
+      </c>
+      <c r="AA720">
+        <v>7</v>
+      </c>
+      <c r="AB720">
+        <v>12</v>
+      </c>
+      <c r="AC720">
+        <v>4.19352</v>
+      </c>
+      <c r="AD720">
+        <v>0</v>
+      </c>
+      <c r="AE720">
+        <v>0</v>
+      </c>
+      <c r="AF720">
+        <v>226.42125</v>
+      </c>
+      <c r="AG720">
+        <v>0</v>
+      </c>
+      <c r="AH720">
+        <v>3</v>
+      </c>
+      <c r="AI720">
+        <v>774.3263099999999</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B721" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E721">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F721">
+        <v>3315.27</v>
+      </c>
+      <c r="G721">
+        <v>41.33443882003841</v>
+      </c>
+      <c r="H721">
+        <v>93.25999999999999</v>
+      </c>
+      <c r="I721">
+        <v>0</v>
+      </c>
+      <c r="J721">
+        <v>0</v>
+      </c>
+      <c r="K721">
+        <v>1.162755903548363</v>
+      </c>
+      <c r="L721">
+        <v>0</v>
+      </c>
+      <c r="M721">
+        <v>2</v>
+      </c>
+      <c r="N721">
+        <v>0</v>
+      </c>
+      <c r="O721">
+        <v>26.59908</v>
+      </c>
+      <c r="P721">
+        <v>83.11173603299589</v>
+      </c>
+      <c r="Q721">
+        <v>32.004</v>
+      </c>
+      <c r="R721">
+        <v>312.32832</v>
+      </c>
+      <c r="S721">
+        <v>3.894076752362666</v>
+      </c>
+      <c r="T721">
+        <v>394.33</v>
+      </c>
+      <c r="U721">
+        <v>12</v>
+      </c>
+      <c r="V721">
+        <v>8</v>
+      </c>
+      <c r="W721">
+        <v>20</v>
+      </c>
+      <c r="X721">
+        <v>34</v>
+      </c>
+      <c r="Y721">
+        <v>12</v>
+      </c>
+      <c r="Z721">
+        <v>28</v>
+      </c>
+      <c r="AA721">
+        <v>8</v>
+      </c>
+      <c r="AB721">
+        <v>10</v>
+      </c>
+      <c r="AC721">
+        <v>4.23796</v>
+      </c>
+      <c r="AD721">
+        <v>-0.49102</v>
+      </c>
+      <c r="AE721">
+        <v>0</v>
+      </c>
+      <c r="AF721">
+        <v>262.01</v>
+      </c>
+      <c r="AG721">
+        <v>0</v>
+      </c>
+      <c r="AH721">
+        <v>3</v>
+      </c>
+      <c r="AI721">
+        <v>936.9849599999999</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B722" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E722">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F722">
+        <v>3139.46</v>
+      </c>
+      <c r="G722">
+        <v>39.14245817021171</v>
+      </c>
+      <c r="H722">
+        <v>47.73</v>
+      </c>
+      <c r="I722">
+        <v>0</v>
+      </c>
+      <c r="J722">
+        <v>0</v>
+      </c>
+      <c r="K722">
+        <v>0.5950926364611127</v>
+      </c>
+      <c r="L722">
+        <v>0</v>
+      </c>
+      <c r="M722">
+        <v>1</v>
+      </c>
+      <c r="N722">
+        <v>0</v>
+      </c>
+      <c r="O722">
+        <v>26.54431</v>
+      </c>
+      <c r="P722">
+        <v>73.73419444444444</v>
+      </c>
+      <c r="Q722">
+        <v>36</v>
+      </c>
+      <c r="R722">
+        <v>291.51144</v>
+      </c>
+      <c r="S722">
+        <v>3.6345340747575</v>
+      </c>
+      <c r="T722">
+        <v>285.19</v>
+      </c>
+      <c r="U722">
+        <v>8</v>
+      </c>
+      <c r="V722">
+        <v>5</v>
+      </c>
+      <c r="W722">
+        <v>13</v>
+      </c>
+      <c r="X722">
+        <v>24</v>
+      </c>
+      <c r="Y722">
+        <v>8</v>
+      </c>
+      <c r="Z722">
+        <v>16</v>
+      </c>
+      <c r="AA722">
+        <v>5</v>
+      </c>
+      <c r="AB722">
+        <v>7</v>
+      </c>
+      <c r="AC722">
+        <v>4.41111</v>
+      </c>
+      <c r="AD722">
+        <v>-0.5471</v>
+      </c>
+      <c r="AE722">
+        <v>0</v>
+      </c>
+      <c r="AF722">
+        <v>695.0740000000001</v>
+      </c>
+      <c r="AG722">
+        <v>0</v>
+      </c>
+      <c r="AH722">
+        <v>3</v>
+      </c>
+      <c r="AI722">
+        <v>874.53432</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B723" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E723">
+        <v>80.20599999999999</v>
+      </c>
+      <c r="F723">
+        <v>3304.75</v>
+      </c>
+      <c r="G723">
+        <v>41.20327656285067</v>
+      </c>
+      <c r="H723">
+        <v>97.27</v>
+      </c>
+      <c r="I723">
+        <v>0</v>
+      </c>
+      <c r="J723">
+        <v>0</v>
+      </c>
+      <c r="K723">
+        <v>1.212752163179812</v>
+      </c>
+      <c r="L723">
+        <v>0</v>
+      </c>
+      <c r="M723">
+        <v>0</v>
+      </c>
+      <c r="N723">
+        <v>0</v>
+      </c>
+      <c r="O723">
+        <v>24.81287</v>
+      </c>
+      <c r="P723">
+        <v>68.92463888888889</v>
+      </c>
+      <c r="Q723">
+        <v>36</v>
+      </c>
+      <c r="R723">
+        <v>350.20731</v>
+      </c>
+      <c r="S723">
+        <v>4.366348028825774</v>
+      </c>
+      <c r="T723">
+        <v>442.39999</v>
+      </c>
+      <c r="U723">
+        <v>12</v>
+      </c>
+      <c r="V723">
+        <v>5</v>
+      </c>
+      <c r="W723">
+        <v>17</v>
+      </c>
+      <c r="X723">
+        <v>38</v>
+      </c>
+      <c r="Y723">
+        <v>12</v>
+      </c>
+      <c r="Z723">
+        <v>28</v>
+      </c>
+      <c r="AA723">
+        <v>5</v>
+      </c>
+      <c r="AB723">
+        <v>5</v>
+      </c>
+      <c r="AC723">
+        <v>4.33057</v>
+      </c>
+      <c r="AD723">
+        <v>0</v>
+      </c>
+      <c r="AE723">
+        <v>0</v>
+      </c>
+      <c r="AF723">
+        <v>744.6</v>
+      </c>
+      <c r="AG723">
+        <v>0</v>
+      </c>
+      <c r="AH723">
+        <v>3</v>
+      </c>
+      <c r="AI723">
+        <v>1050.62193</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B724" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Sesión 41 | Sesión AM Seleccionados</t>
+        </is>
+      </c>
+      <c r="E724">
+        <v>157.523</v>
+      </c>
+      <c r="F724">
+        <v>10492.15</v>
+      </c>
+      <c r="G724">
+        <v>66.60709864591202</v>
+      </c>
+      <c r="H724">
+        <v>236.68</v>
+      </c>
+      <c r="I724">
+        <v>0</v>
+      </c>
+      <c r="J724">
+        <v>0</v>
+      </c>
+      <c r="K724">
+        <v>1.502510744462713</v>
+      </c>
+      <c r="L724">
+        <v>0</v>
+      </c>
+      <c r="M724">
+        <v>6</v>
+      </c>
+      <c r="N724">
+        <v>0</v>
+      </c>
+      <c r="O724">
+        <v>27.49122</v>
+      </c>
+      <c r="P724">
+        <v>78.56430041152264</v>
+      </c>
+      <c r="Q724">
+        <v>34.992</v>
+      </c>
+      <c r="R724">
+        <v>1036.21628</v>
+      </c>
+      <c r="S724">
+        <v>6.578190359503058</v>
+      </c>
+      <c r="T724">
+        <v>1565.33</v>
+      </c>
+      <c r="U724">
+        <v>49</v>
+      </c>
+      <c r="V724">
+        <v>56</v>
+      </c>
+      <c r="W724">
+        <v>105</v>
+      </c>
+      <c r="X724">
+        <v>198</v>
+      </c>
+      <c r="Y724">
+        <v>49</v>
+      </c>
+      <c r="Z724">
+        <v>165</v>
+      </c>
+      <c r="AA724">
+        <v>56</v>
+      </c>
+      <c r="AB724">
+        <v>71</v>
+      </c>
+      <c r="AC724">
+        <v>4.20472</v>
+      </c>
+      <c r="AD724">
+        <v>0</v>
+      </c>
+      <c r="AE724">
+        <v>0</v>
+      </c>
+      <c r="AF724">
+        <v>1017.236</v>
+      </c>
+      <c r="AG724">
+        <v>0</v>
+      </c>
+      <c r="AH724">
+        <v>3</v>
+      </c>
+      <c r="AI724">
+        <v>3108.64884</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B725" s="2">
+        <v>46226</v>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Sesión 41</t>
+        </is>
+      </c>
+      <c r="E725">
+        <v>54.47666666666667</v>
+      </c>
+      <c r="F725">
+        <v>2041.36</v>
+      </c>
+      <c r="G725">
+        <v>37.47218992840972</v>
+      </c>
+      <c r="H725">
+        <v>0</v>
+      </c>
+      <c r="I725">
+        <v>0</v>
+      </c>
+      <c r="J725">
+        <v>0</v>
+      </c>
+      <c r="K725">
+        <v>0</v>
+      </c>
+      <c r="L725">
+        <v>0</v>
+      </c>
+      <c r="M725">
+        <v>0</v>
+      </c>
+      <c r="N725">
+        <v>0</v>
+      </c>
+      <c r="O725">
+        <v>20.76617</v>
+      </c>
+      <c r="P725">
+        <v>61.10572622410545</v>
+      </c>
+      <c r="Q725">
+        <v>33.984</v>
+      </c>
+      <c r="R725">
+        <v>257.85999</v>
+      </c>
+      <c r="S725">
+        <v>4.733402496481673</v>
+      </c>
+      <c r="T725">
+        <v>190.44</v>
+      </c>
+      <c r="U725">
+        <v>8</v>
+      </c>
+      <c r="V725">
+        <v>2</v>
+      </c>
+      <c r="W725">
+        <v>10</v>
+      </c>
+      <c r="X725">
+        <v>16</v>
+      </c>
+      <c r="Y725">
+        <v>8</v>
+      </c>
+      <c r="Z725">
+        <v>12</v>
+      </c>
+      <c r="AA725">
+        <v>2</v>
+      </c>
+      <c r="AB725">
+        <v>6</v>
+      </c>
+      <c r="AC725">
+        <v>4.08681</v>
+      </c>
+      <c r="AD725">
+        <v>0</v>
+      </c>
+      <c r="AE725">
+        <v>0</v>
+      </c>
+      <c r="AF725">
+        <v>159.3697</v>
+      </c>
+      <c r="AG725">
+        <v>0</v>
+      </c>
+      <c r="AH725">
+        <v>3</v>
+      </c>
+      <c r="AI725">
+        <v>773.57997</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-25
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI725"/>
+  <dimension ref="A1:AI749"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -79664,10 +79664,10 @@
         <v>77.31700000000001</v>
       </c>
       <c r="F703">
-        <v>7539.240000000001</v>
+        <v>7539.96</v>
       </c>
       <c r="G703">
-        <v>97.51076736034766</v>
+        <v>97.52007967199968</v>
       </c>
       <c r="H703">
         <v>106.56</v>
@@ -79700,10 +79700,10 @@
         <v>32.364</v>
       </c>
       <c r="R703">
-        <v>776.4910600000001</v>
+        <v>776.52268</v>
       </c>
       <c r="S703">
-        <v>10.04295381352096</v>
+        <v>10.04336277920768</v>
       </c>
       <c r="T703">
         <v>862.27</v>
@@ -79742,7 +79742,7 @@
         <v>0</v>
       </c>
       <c r="AF703">
-        <v>618.3226</v>
+        <v>618.366</v>
       </c>
       <c r="AG703">
         <v>0</v>
@@ -79751,7 +79751,7 @@
         <v>3</v>
       </c>
       <c r="AI703">
-        <v>2329.47318</v>
+        <v>2329.56804</v>
       </c>
     </row>
     <row r="704">
@@ -80003,10 +80003,10 @@
         <v>77.31700000000001</v>
       </c>
       <c r="F706">
-        <v>7162.740000000001</v>
+        <v>7163.47</v>
       </c>
       <c r="G706">
-        <v>92.641204392307</v>
+        <v>92.65064604162086</v>
       </c>
       <c r="H706">
         <v>73.86999999999999</v>
@@ -80039,10 +80039,10 @@
         <v>35.604</v>
       </c>
       <c r="R706">
-        <v>637.59048</v>
+        <v>637.66094</v>
       </c>
       <c r="S706">
-        <v>8.246446189065793</v>
+        <v>8.247357502231074</v>
       </c>
       <c r="T706">
         <v>922.3099999999999</v>
@@ -80081,7 +80081,7 @@
         <v>0</v>
       </c>
       <c r="AF706">
-        <v>608.3457500000001</v>
+        <v>608.38551</v>
       </c>
       <c r="AG706">
         <v>0</v>
@@ -80090,7 +80090,7 @@
         <v>3</v>
       </c>
       <c r="AI706">
-        <v>1912.77144</v>
+        <v>1912.98282</v>
       </c>
     </row>
     <row r="707">
@@ -81020,10 +81020,10 @@
         <v>77.31700000000001</v>
       </c>
       <c r="F715">
-        <v>7708.71</v>
+        <v>7709.120000000001</v>
       </c>
       <c r="G715">
-        <v>99.7026527154442</v>
+        <v>99.70795555957939</v>
       </c>
       <c r="H715">
         <v>84.55</v>
@@ -81056,10 +81056,10 @@
         <v>33.012</v>
       </c>
       <c r="R715">
-        <v>867.40355</v>
+        <v>867.42583</v>
       </c>
       <c r="S715">
-        <v>11.21879470232937</v>
+        <v>11.21908286663994</v>
       </c>
       <c r="T715">
         <v>1064.57001</v>
@@ -81098,7 +81098,7 @@
         <v>0</v>
       </c>
       <c r="AF715">
-        <v>729.43494</v>
+        <v>729.47004</v>
       </c>
       <c r="AG715">
         <v>0</v>
@@ -81107,7 +81107,7 @@
         <v>3</v>
       </c>
       <c r="AI715">
-        <v>2602.21065</v>
+        <v>2602.27749</v>
       </c>
     </row>
     <row r="716">
@@ -82037,10 +82037,10 @@
         <v>157.523</v>
       </c>
       <c r="F724">
-        <v>10492.15</v>
+        <v>10492.65</v>
       </c>
       <c r="G724">
-        <v>66.60709864591202</v>
+        <v>66.61027278556148</v>
       </c>
       <c r="H724">
         <v>236.68</v>
@@ -82073,10 +82073,10 @@
         <v>34.992</v>
       </c>
       <c r="R724">
-        <v>1036.21628</v>
+        <v>1036.24269</v>
       </c>
       <c r="S724">
-        <v>6.578190359503058</v>
+        <v>6.578358017559341</v>
       </c>
       <c r="T724">
         <v>1565.33</v>
@@ -82115,7 +82115,7 @@
         <v>0</v>
       </c>
       <c r="AF724">
-        <v>1017.236</v>
+        <v>1017.2736</v>
       </c>
       <c r="AG724">
         <v>0</v>
@@ -82124,7 +82124,7 @@
         <v>3</v>
       </c>
       <c r="AI724">
-        <v>3108.64884</v>
+        <v>3108.72807</v>
       </c>
     </row>
     <row r="725">
@@ -82238,6 +82238,2718 @@
       </c>
       <c r="AI725">
         <v>773.57997</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B726" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E726">
+        <v>35.84849999999999</v>
+      </c>
+      <c r="F726">
+        <v>1791.67</v>
+      </c>
+      <c r="G726">
+        <v>49.97893914668676</v>
+      </c>
+      <c r="H726">
+        <v>0</v>
+      </c>
+      <c r="I726">
+        <v>0</v>
+      </c>
+      <c r="J726">
+        <v>0</v>
+      </c>
+      <c r="K726">
+        <v>0</v>
+      </c>
+      <c r="L726">
+        <v>0</v>
+      </c>
+      <c r="M726">
+        <v>0</v>
+      </c>
+      <c r="N726">
+        <v>0</v>
+      </c>
+      <c r="O726">
+        <v>16.9268</v>
+      </c>
+      <c r="P726">
+        <v>47.01888888888889</v>
+      </c>
+      <c r="Q726">
+        <v>36</v>
+      </c>
+      <c r="R726">
+        <v>282.46651</v>
+      </c>
+      <c r="S726">
+        <v>7.879451302007058</v>
+      </c>
+      <c r="T726">
+        <v>102.58</v>
+      </c>
+      <c r="U726">
+        <v>2</v>
+      </c>
+      <c r="V726">
+        <v>1</v>
+      </c>
+      <c r="W726">
+        <v>3</v>
+      </c>
+      <c r="X726">
+        <v>21</v>
+      </c>
+      <c r="Y726">
+        <v>2</v>
+      </c>
+      <c r="Z726">
+        <v>14</v>
+      </c>
+      <c r="AA726">
+        <v>1</v>
+      </c>
+      <c r="AB726">
+        <v>22</v>
+      </c>
+      <c r="AC726">
+        <v>3.44243</v>
+      </c>
+      <c r="AD726">
+        <v>-2.51814</v>
+      </c>
+      <c r="AE726">
+        <v>0</v>
+      </c>
+      <c r="AF726">
+        <v>371.886</v>
+      </c>
+      <c r="AG726">
+        <v>0</v>
+      </c>
+      <c r="AH726">
+        <v>3</v>
+      </c>
+      <c r="AI726">
+        <v>847.3995299999999</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B727" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E727">
+        <v>87.08333333333333</v>
+      </c>
+      <c r="F727">
+        <v>4994.379999999999</v>
+      </c>
+      <c r="G727">
+        <v>57.35173205741626</v>
+      </c>
+      <c r="H727">
+        <v>35.08</v>
+      </c>
+      <c r="I727">
+        <v>0</v>
+      </c>
+      <c r="J727">
+        <v>0</v>
+      </c>
+      <c r="K727">
+        <v>0.4028325358851675</v>
+      </c>
+      <c r="L727">
+        <v>0</v>
+      </c>
+      <c r="M727">
+        <v>0</v>
+      </c>
+      <c r="N727">
+        <v>0</v>
+      </c>
+      <c r="O727">
+        <v>24.00329</v>
+      </c>
+      <c r="P727">
+        <v>74.16663576813744</v>
+      </c>
+      <c r="Q727">
+        <v>32.364</v>
+      </c>
+      <c r="R727">
+        <v>484.86057</v>
+      </c>
+      <c r="S727">
+        <v>5.567776880382775</v>
+      </c>
+      <c r="T727">
+        <v>411.48999</v>
+      </c>
+      <c r="U727">
+        <v>4</v>
+      </c>
+      <c r="V727">
+        <v>4</v>
+      </c>
+      <c r="W727">
+        <v>8</v>
+      </c>
+      <c r="X727">
+        <v>36</v>
+      </c>
+      <c r="Y727">
+        <v>4</v>
+      </c>
+      <c r="Z727">
+        <v>22</v>
+      </c>
+      <c r="AA727">
+        <v>4</v>
+      </c>
+      <c r="AB727">
+        <v>10</v>
+      </c>
+      <c r="AC727">
+        <v>3.17198</v>
+      </c>
+      <c r="AD727">
+        <v>-3.56587</v>
+      </c>
+      <c r="AE727">
+        <v>0</v>
+      </c>
+      <c r="AF727">
+        <v>387.0601</v>
+      </c>
+      <c r="AG727">
+        <v>0</v>
+      </c>
+      <c r="AH727">
+        <v>3</v>
+      </c>
+      <c r="AI727">
+        <v>1454.58171</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B728" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E728">
+        <v>58.16966666666667</v>
+      </c>
+      <c r="F728">
+        <v>4544.870000000001</v>
+      </c>
+      <c r="G728">
+        <v>78.1312711665301</v>
+      </c>
+      <c r="H728">
+        <v>120.05</v>
+      </c>
+      <c r="I728">
+        <v>0</v>
+      </c>
+      <c r="J728">
+        <v>0</v>
+      </c>
+      <c r="K728">
+        <v>2.063790406225467</v>
+      </c>
+      <c r="L728">
+        <v>0</v>
+      </c>
+      <c r="M728">
+        <v>1</v>
+      </c>
+      <c r="N728">
+        <v>0</v>
+      </c>
+      <c r="O728">
+        <v>25.35495</v>
+      </c>
+      <c r="P728">
+        <v>70.43041666666666</v>
+      </c>
+      <c r="Q728">
+        <v>36</v>
+      </c>
+      <c r="R728">
+        <v>418.40874</v>
+      </c>
+      <c r="S728">
+        <v>7.192902486404712</v>
+      </c>
+      <c r="T728">
+        <v>535.87</v>
+      </c>
+      <c r="U728">
+        <v>13</v>
+      </c>
+      <c r="V728">
+        <v>11</v>
+      </c>
+      <c r="W728">
+        <v>24</v>
+      </c>
+      <c r="X728">
+        <v>46</v>
+      </c>
+      <c r="Y728">
+        <v>13</v>
+      </c>
+      <c r="Z728">
+        <v>46</v>
+      </c>
+      <c r="AA728">
+        <v>11</v>
+      </c>
+      <c r="AB728">
+        <v>22</v>
+      </c>
+      <c r="AC728">
+        <v>4.22152</v>
+      </c>
+      <c r="AD728">
+        <v>-2.67092</v>
+      </c>
+      <c r="AE728">
+        <v>0</v>
+      </c>
+      <c r="AF728">
+        <v>1024.366</v>
+      </c>
+      <c r="AG728">
+        <v>0</v>
+      </c>
+      <c r="AH728">
+        <v>3</v>
+      </c>
+      <c r="AI728">
+        <v>1255.22622</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B729" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E729">
+        <v>61.83683333333333</v>
+      </c>
+      <c r="F729">
+        <v>5010.27</v>
+      </c>
+      <c r="G729">
+        <v>81.02403907056475</v>
+      </c>
+      <c r="H729">
+        <v>190.94</v>
+      </c>
+      <c r="I729">
+        <v>0</v>
+      </c>
+      <c r="J729">
+        <v>0</v>
+      </c>
+      <c r="K729">
+        <v>3.087803655318702</v>
+      </c>
+      <c r="L729">
+        <v>0</v>
+      </c>
+      <c r="M729">
+        <v>2</v>
+      </c>
+      <c r="N729">
+        <v>0</v>
+      </c>
+      <c r="O729">
+        <v>26.81726</v>
+      </c>
+      <c r="P729">
+        <v>82.76932098765432</v>
+      </c>
+      <c r="Q729">
+        <v>32.4</v>
+      </c>
+      <c r="R729">
+        <v>554.04684</v>
+      </c>
+      <c r="S729">
+        <v>8.959819093797925</v>
+      </c>
+      <c r="T729">
+        <v>834.08</v>
+      </c>
+      <c r="U729">
+        <v>16</v>
+      </c>
+      <c r="V729">
+        <v>15</v>
+      </c>
+      <c r="W729">
+        <v>31</v>
+      </c>
+      <c r="X729">
+        <v>46</v>
+      </c>
+      <c r="Y729">
+        <v>16</v>
+      </c>
+      <c r="Z729">
+        <v>54</v>
+      </c>
+      <c r="AA729">
+        <v>15</v>
+      </c>
+      <c r="AB729">
+        <v>9</v>
+      </c>
+      <c r="AC729">
+        <v>4.14843</v>
+      </c>
+      <c r="AD729">
+        <v>-2.50076</v>
+      </c>
+      <c r="AE729">
+        <v>0</v>
+      </c>
+      <c r="AF729">
+        <v>400.2299</v>
+      </c>
+      <c r="AG729">
+        <v>0</v>
+      </c>
+      <c r="AH729">
+        <v>3</v>
+      </c>
+      <c r="AI729">
+        <v>1662.14052</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B730" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E730">
+        <v>65.426</v>
+      </c>
+      <c r="F730">
+        <v>3867.47</v>
+      </c>
+      <c r="G730">
+        <v>59.11212667746767</v>
+      </c>
+      <c r="H730">
+        <v>99.14</v>
+      </c>
+      <c r="I730">
+        <v>0</v>
+      </c>
+      <c r="J730">
+        <v>0</v>
+      </c>
+      <c r="K730">
+        <v>1.515299727936906</v>
+      </c>
+      <c r="L730">
+        <v>0</v>
+      </c>
+      <c r="M730">
+        <v>0</v>
+      </c>
+      <c r="N730">
+        <v>0</v>
+      </c>
+      <c r="O730">
+        <v>24.34918</v>
+      </c>
+      <c r="P730">
+        <v>68.38888888888889</v>
+      </c>
+      <c r="Q730">
+        <v>35.604</v>
+      </c>
+      <c r="R730">
+        <v>362.73352</v>
+      </c>
+      <c r="S730">
+        <v>5.544179989606579</v>
+      </c>
+      <c r="T730">
+        <v>453.84</v>
+      </c>
+      <c r="U730">
+        <v>13</v>
+      </c>
+      <c r="V730">
+        <v>10</v>
+      </c>
+      <c r="W730">
+        <v>23</v>
+      </c>
+      <c r="X730">
+        <v>59</v>
+      </c>
+      <c r="Y730">
+        <v>13</v>
+      </c>
+      <c r="Z730">
+        <v>35</v>
+      </c>
+      <c r="AA730">
+        <v>10</v>
+      </c>
+      <c r="AB730">
+        <v>10</v>
+      </c>
+      <c r="AC730">
+        <v>3.62272</v>
+      </c>
+      <c r="AD730">
+        <v>-4.45041</v>
+      </c>
+      <c r="AE730">
+        <v>0</v>
+      </c>
+      <c r="AF730">
+        <v>319.98635</v>
+      </c>
+      <c r="AG730">
+        <v>0</v>
+      </c>
+      <c r="AH730">
+        <v>3</v>
+      </c>
+      <c r="AI730">
+        <v>1088.20056</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B731" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E731">
+        <v>111.3361666666667</v>
+      </c>
+      <c r="F731">
+        <v>10421.52</v>
+      </c>
+      <c r="G731">
+        <v>93.60408492598242</v>
+      </c>
+      <c r="H731">
+        <v>457.09</v>
+      </c>
+      <c r="I731">
+        <v>0</v>
+      </c>
+      <c r="J731">
+        <v>0</v>
+      </c>
+      <c r="K731">
+        <v>4.105494321252303</v>
+      </c>
+      <c r="L731">
+        <v>2.79</v>
+      </c>
+      <c r="M731">
+        <v>9</v>
+      </c>
+      <c r="N731">
+        <v>0</v>
+      </c>
+      <c r="O731">
+        <v>30.12249</v>
+      </c>
+      <c r="P731">
+        <v>88.63727048022598</v>
+      </c>
+      <c r="Q731">
+        <v>33.984</v>
+      </c>
+      <c r="R731">
+        <v>1146.02652</v>
+      </c>
+      <c r="S731">
+        <v>10.29338941973034</v>
+      </c>
+      <c r="T731">
+        <v>1611.66999</v>
+      </c>
+      <c r="U731">
+        <v>26</v>
+      </c>
+      <c r="V731">
+        <v>34</v>
+      </c>
+      <c r="W731">
+        <v>60</v>
+      </c>
+      <c r="X731">
+        <v>109</v>
+      </c>
+      <c r="Y731">
+        <v>26</v>
+      </c>
+      <c r="Z731">
+        <v>124</v>
+      </c>
+      <c r="AA731">
+        <v>34</v>
+      </c>
+      <c r="AB731">
+        <v>27</v>
+      </c>
+      <c r="AC731">
+        <v>4.35346</v>
+      </c>
+      <c r="AD731">
+        <v>-4.50694</v>
+      </c>
+      <c r="AE731">
+        <v>0</v>
+      </c>
+      <c r="AF731">
+        <v>963.6856</v>
+      </c>
+      <c r="AG731">
+        <v>0</v>
+      </c>
+      <c r="AH731">
+        <v>3</v>
+      </c>
+      <c r="AI731">
+        <v>3438.07956</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B732" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E732">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F732">
+        <v>12983.1</v>
+      </c>
+      <c r="G732">
+        <v>104.6440493541909</v>
+      </c>
+      <c r="H732">
+        <v>678.3000000000001</v>
+      </c>
+      <c r="I732">
+        <v>0</v>
+      </c>
+      <c r="J732">
+        <v>0</v>
+      </c>
+      <c r="K732">
+        <v>5.467111758897927</v>
+      </c>
+      <c r="L732">
+        <v>9.600000000000001</v>
+      </c>
+      <c r="M732">
+        <v>18</v>
+      </c>
+      <c r="N732">
+        <v>2</v>
+      </c>
+      <c r="O732">
+        <v>30.41558</v>
+      </c>
+      <c r="P732">
+        <v>85.51388888888889</v>
+      </c>
+      <c r="Q732">
+        <v>35.568</v>
+      </c>
+      <c r="R732">
+        <v>1168.75786</v>
+      </c>
+      <c r="S732">
+        <v>9.42021205913368</v>
+      </c>
+      <c r="T732">
+        <v>1968.71002</v>
+      </c>
+      <c r="U732">
+        <v>58</v>
+      </c>
+      <c r="V732">
+        <v>43</v>
+      </c>
+      <c r="W732">
+        <v>101</v>
+      </c>
+      <c r="X732">
+        <v>170</v>
+      </c>
+      <c r="Y732">
+        <v>58</v>
+      </c>
+      <c r="Z732">
+        <v>118</v>
+      </c>
+      <c r="AA732">
+        <v>43</v>
+      </c>
+      <c r="AB732">
+        <v>29</v>
+      </c>
+      <c r="AC732">
+        <v>4.66124</v>
+      </c>
+      <c r="AD732">
+        <v>-4.43348</v>
+      </c>
+      <c r="AE732">
+        <v>0</v>
+      </c>
+      <c r="AF732">
+        <v>1216.6792</v>
+      </c>
+      <c r="AG732">
+        <v>0</v>
+      </c>
+      <c r="AH732">
+        <v>3</v>
+      </c>
+      <c r="AI732">
+        <v>3506.27358</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B733" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E733">
+        <v>35.84849999999999</v>
+      </c>
+      <c r="F733">
+        <v>2252.86</v>
+      </c>
+      <c r="G733">
+        <v>62.84391257653738</v>
+      </c>
+      <c r="H733">
+        <v>0.36</v>
+      </c>
+      <c r="I733">
+        <v>0</v>
+      </c>
+      <c r="J733">
+        <v>0</v>
+      </c>
+      <c r="K733">
+        <v>0.01004226118247626</v>
+      </c>
+      <c r="L733">
+        <v>0</v>
+      </c>
+      <c r="M733">
+        <v>0</v>
+      </c>
+      <c r="N733">
+        <v>0</v>
+      </c>
+      <c r="O733">
+        <v>20.8862</v>
+      </c>
+      <c r="P733">
+        <v>58.01722222222222</v>
+      </c>
+      <c r="Q733">
+        <v>36</v>
+      </c>
+      <c r="R733">
+        <v>252.12381</v>
+      </c>
+      <c r="S733">
+        <v>7.033036528725052</v>
+      </c>
+      <c r="T733">
+        <v>111.04</v>
+      </c>
+      <c r="U733">
+        <v>9</v>
+      </c>
+      <c r="V733">
+        <v>9</v>
+      </c>
+      <c r="W733">
+        <v>18</v>
+      </c>
+      <c r="X733">
+        <v>15</v>
+      </c>
+      <c r="Y733">
+        <v>9</v>
+      </c>
+      <c r="Z733">
+        <v>16</v>
+      </c>
+      <c r="AA733">
+        <v>9</v>
+      </c>
+      <c r="AB733">
+        <v>17</v>
+      </c>
+      <c r="AC733">
+        <v>4.26224</v>
+      </c>
+      <c r="AD733">
+        <v>-3.56867</v>
+      </c>
+      <c r="AE733">
+        <v>0</v>
+      </c>
+      <c r="AF733">
+        <v>486.298</v>
+      </c>
+      <c r="AG733">
+        <v>0</v>
+      </c>
+      <c r="AH733">
+        <v>3</v>
+      </c>
+      <c r="AI733">
+        <v>756.3714299999999</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B734" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E734">
+        <v>35.84849999999999</v>
+      </c>
+      <c r="F734">
+        <v>2020.42</v>
+      </c>
+      <c r="G734">
+        <v>56.35995927305189</v>
+      </c>
+      <c r="H734">
+        <v>12.45</v>
+      </c>
+      <c r="I734">
+        <v>0</v>
+      </c>
+      <c r="J734">
+        <v>0</v>
+      </c>
+      <c r="K734">
+        <v>0.3472948658939705</v>
+      </c>
+      <c r="L734">
+        <v>0</v>
+      </c>
+      <c r="M734">
+        <v>0</v>
+      </c>
+      <c r="N734">
+        <v>0</v>
+      </c>
+      <c r="O734">
+        <v>22.05491</v>
+      </c>
+      <c r="P734">
+        <v>61.26363888888888</v>
+      </c>
+      <c r="Q734">
+        <v>36</v>
+      </c>
+      <c r="R734">
+        <v>245.83282</v>
+      </c>
+      <c r="S734">
+        <v>6.85754829351298</v>
+      </c>
+      <c r="T734">
+        <v>179.09</v>
+      </c>
+      <c r="U734">
+        <v>10</v>
+      </c>
+      <c r="V734">
+        <v>6</v>
+      </c>
+      <c r="W734">
+        <v>16</v>
+      </c>
+      <c r="X734">
+        <v>28</v>
+      </c>
+      <c r="Y734">
+        <v>10</v>
+      </c>
+      <c r="Z734">
+        <v>22</v>
+      </c>
+      <c r="AA734">
+        <v>6</v>
+      </c>
+      <c r="AB734">
+        <v>15</v>
+      </c>
+      <c r="AC734">
+        <v>4.42572</v>
+      </c>
+      <c r="AD734">
+        <v>-2.59389</v>
+      </c>
+      <c r="AE734">
+        <v>0</v>
+      </c>
+      <c r="AF734">
+        <v>158.8832</v>
+      </c>
+      <c r="AG734">
+        <v>0</v>
+      </c>
+      <c r="AH734">
+        <v>3</v>
+      </c>
+      <c r="AI734">
+        <v>737.49846</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B735" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E735">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F735">
+        <v>12964.61</v>
+      </c>
+      <c r="G735">
+        <v>104.4950195791326</v>
+      </c>
+      <c r="H735">
+        <v>526.2</v>
+      </c>
+      <c r="I735">
+        <v>6.96</v>
+      </c>
+      <c r="J735">
+        <v>1</v>
+      </c>
+      <c r="K735">
+        <v>4.241182673643062</v>
+      </c>
+      <c r="L735">
+        <v>0</v>
+      </c>
+      <c r="M735">
+        <v>12</v>
+      </c>
+      <c r="N735">
+        <v>0</v>
+      </c>
+      <c r="O735">
+        <v>29.62714</v>
+      </c>
+      <c r="P735">
+        <v>92.5732408448944</v>
+      </c>
+      <c r="Q735">
+        <v>32.004</v>
+      </c>
+      <c r="R735">
+        <v>1367.69791</v>
+      </c>
+      <c r="S735">
+        <v>11.02367289751013</v>
+      </c>
+      <c r="T735">
+        <v>1785.51</v>
+      </c>
+      <c r="U735">
+        <v>18</v>
+      </c>
+      <c r="V735">
+        <v>40</v>
+      </c>
+      <c r="W735">
+        <v>58</v>
+      </c>
+      <c r="X735">
+        <v>113</v>
+      </c>
+      <c r="Y735">
+        <v>18</v>
+      </c>
+      <c r="Z735">
+        <v>109</v>
+      </c>
+      <c r="AA735">
+        <v>40</v>
+      </c>
+      <c r="AB735">
+        <v>36</v>
+      </c>
+      <c r="AC735">
+        <v>4.20831</v>
+      </c>
+      <c r="AD735">
+        <v>-3.66839</v>
+      </c>
+      <c r="AE735">
+        <v>0</v>
+      </c>
+      <c r="AF735">
+        <v>889.1952</v>
+      </c>
+      <c r="AG735">
+        <v>0</v>
+      </c>
+      <c r="AH735">
+        <v>3</v>
+      </c>
+      <c r="AI735">
+        <v>4103.093730000001</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B736" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E736">
+        <v>49.63833333333334</v>
+      </c>
+      <c r="F736">
+        <v>3498.09</v>
+      </c>
+      <c r="G736">
+        <v>70.47154416949266</v>
+      </c>
+      <c r="H736">
+        <v>139.06</v>
+      </c>
+      <c r="I736">
+        <v>0</v>
+      </c>
+      <c r="J736">
+        <v>0</v>
+      </c>
+      <c r="K736">
+        <v>2.801463922371823</v>
+      </c>
+      <c r="L736">
+        <v>0</v>
+      </c>
+      <c r="M736">
+        <v>3</v>
+      </c>
+      <c r="N736">
+        <v>0</v>
+      </c>
+      <c r="O736">
+        <v>28.85395</v>
+      </c>
+      <c r="P736">
+        <v>85.2658096926714</v>
+      </c>
+      <c r="Q736">
+        <v>33.84</v>
+      </c>
+      <c r="R736">
+        <v>337.23323</v>
+      </c>
+      <c r="S736">
+        <v>6.793806466776348</v>
+      </c>
+      <c r="T736">
+        <v>444.45</v>
+      </c>
+      <c r="U736">
+        <v>11</v>
+      </c>
+      <c r="V736">
+        <v>10</v>
+      </c>
+      <c r="W736">
+        <v>21</v>
+      </c>
+      <c r="X736">
+        <v>40</v>
+      </c>
+      <c r="Y736">
+        <v>11</v>
+      </c>
+      <c r="Z736">
+        <v>36</v>
+      </c>
+      <c r="AA736">
+        <v>10</v>
+      </c>
+      <c r="AB736">
+        <v>11</v>
+      </c>
+      <c r="AC736">
+        <v>4.09142</v>
+      </c>
+      <c r="AD736">
+        <v>-3.24544</v>
+      </c>
+      <c r="AE736">
+        <v>0</v>
+      </c>
+      <c r="AF736">
+        <v>270.0439</v>
+      </c>
+      <c r="AG736">
+        <v>0</v>
+      </c>
+      <c r="AH736">
+        <v>3</v>
+      </c>
+      <c r="AI736">
+        <v>1011.69969</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B737" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E737">
+        <v>104.1058333333333</v>
+      </c>
+      <c r="F737">
+        <v>9744.99</v>
+      </c>
+      <c r="G737">
+        <v>93.60657023701842</v>
+      </c>
+      <c r="H737">
+        <v>540.23</v>
+      </c>
+      <c r="I737">
+        <v>0</v>
+      </c>
+      <c r="J737">
+        <v>0</v>
+      </c>
+      <c r="K737">
+        <v>5.189238515292931</v>
+      </c>
+      <c r="L737">
+        <v>0</v>
+      </c>
+      <c r="M737">
+        <v>11</v>
+      </c>
+      <c r="N737">
+        <v>0</v>
+      </c>
+      <c r="O737">
+        <v>27.6149</v>
+      </c>
+      <c r="P737">
+        <v>81.95305080721748</v>
+      </c>
+      <c r="Q737">
+        <v>33.696</v>
+      </c>
+      <c r="R737">
+        <v>1078.48381</v>
+      </c>
+      <c r="S737">
+        <v>10.35949452080015</v>
+      </c>
+      <c r="T737">
+        <v>1540.25998</v>
+      </c>
+      <c r="U737">
+        <v>38</v>
+      </c>
+      <c r="V737">
+        <v>43</v>
+      </c>
+      <c r="W737">
+        <v>81</v>
+      </c>
+      <c r="X737">
+        <v>132</v>
+      </c>
+      <c r="Y737">
+        <v>38</v>
+      </c>
+      <c r="Z737">
+        <v>123</v>
+      </c>
+      <c r="AA737">
+        <v>43</v>
+      </c>
+      <c r="AB737">
+        <v>50</v>
+      </c>
+      <c r="AC737">
+        <v>4.17203</v>
+      </c>
+      <c r="AD737">
+        <v>-3.62004</v>
+      </c>
+      <c r="AE737">
+        <v>0</v>
+      </c>
+      <c r="AF737">
+        <v>917.4295999999999</v>
+      </c>
+      <c r="AG737">
+        <v>0</v>
+      </c>
+      <c r="AH737">
+        <v>3</v>
+      </c>
+      <c r="AI737">
+        <v>3235.45143</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B738" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E738">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F738">
+        <v>12912.42</v>
+      </c>
+      <c r="G738">
+        <v>104.0743671204906</v>
+      </c>
+      <c r="H738">
+        <v>444.93</v>
+      </c>
+      <c r="I738">
+        <v>0</v>
+      </c>
+      <c r="J738">
+        <v>0</v>
+      </c>
+      <c r="K738">
+        <v>3.586144825131143</v>
+      </c>
+      <c r="L738">
+        <v>0</v>
+      </c>
+      <c r="M738">
+        <v>8</v>
+      </c>
+      <c r="N738">
+        <v>0</v>
+      </c>
+      <c r="O738">
+        <v>29.84331</v>
+      </c>
+      <c r="P738">
+        <v>82.89808333333333</v>
+      </c>
+      <c r="Q738">
+        <v>36</v>
+      </c>
+      <c r="R738">
+        <v>1317.96321</v>
+      </c>
+      <c r="S738">
+        <v>10.62281020667235</v>
+      </c>
+      <c r="T738">
+        <v>1755.37006</v>
+      </c>
+      <c r="U738">
+        <v>21</v>
+      </c>
+      <c r="V738">
+        <v>32</v>
+      </c>
+      <c r="W738">
+        <v>53</v>
+      </c>
+      <c r="X738">
+        <v>113</v>
+      </c>
+      <c r="Y738">
+        <v>21</v>
+      </c>
+      <c r="Z738">
+        <v>110</v>
+      </c>
+      <c r="AA738">
+        <v>32</v>
+      </c>
+      <c r="AB738">
+        <v>1121</v>
+      </c>
+      <c r="AC738">
+        <v>4.46712</v>
+      </c>
+      <c r="AD738">
+        <v>-4.00686</v>
+      </c>
+      <c r="AE738">
+        <v>0</v>
+      </c>
+      <c r="AF738">
+        <v>2944.776</v>
+      </c>
+      <c r="AG738">
+        <v>0</v>
+      </c>
+      <c r="AH738">
+        <v>3</v>
+      </c>
+      <c r="AI738">
+        <v>3953.889630000001</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B739" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E739">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F739">
+        <v>12172.96</v>
+      </c>
+      <c r="G739">
+        <v>98.1143045209997</v>
+      </c>
+      <c r="H739">
+        <v>571.11</v>
+      </c>
+      <c r="I739">
+        <v>50.03</v>
+      </c>
+      <c r="J739">
+        <v>3</v>
+      </c>
+      <c r="K739">
+        <v>4.603158184614764</v>
+      </c>
+      <c r="L739">
+        <v>89.39</v>
+      </c>
+      <c r="M739">
+        <v>13</v>
+      </c>
+      <c r="N739">
+        <v>5</v>
+      </c>
+      <c r="O739">
+        <v>33.06524</v>
+      </c>
+      <c r="P739">
+        <v>94.49371284865113</v>
+      </c>
+      <c r="Q739">
+        <v>34.992</v>
+      </c>
+      <c r="R739">
+        <v>990.5006100000001</v>
+      </c>
+      <c r="S739">
+        <v>7.983455008295104</v>
+      </c>
+      <c r="T739">
+        <v>1556.35001</v>
+      </c>
+      <c r="U739">
+        <v>31</v>
+      </c>
+      <c r="V739">
+        <v>43</v>
+      </c>
+      <c r="W739">
+        <v>74</v>
+      </c>
+      <c r="X739">
+        <v>112</v>
+      </c>
+      <c r="Y739">
+        <v>31</v>
+      </c>
+      <c r="Z739">
+        <v>109</v>
+      </c>
+      <c r="AA739">
+        <v>43</v>
+      </c>
+      <c r="AB739">
+        <v>18</v>
+      </c>
+      <c r="AC739">
+        <v>4.2825</v>
+      </c>
+      <c r="AD739">
+        <v>-4.29323</v>
+      </c>
+      <c r="AE739">
+        <v>0</v>
+      </c>
+      <c r="AF739">
+        <v>958.7025599999999</v>
+      </c>
+      <c r="AG739">
+        <v>0</v>
+      </c>
+      <c r="AH739">
+        <v>3</v>
+      </c>
+      <c r="AI739">
+        <v>2971.50183</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B740" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E740">
+        <v>77.68116666666667</v>
+      </c>
+      <c r="F740">
+        <v>3943.57</v>
+      </c>
+      <c r="G740">
+        <v>50.76610160763977</v>
+      </c>
+      <c r="H740">
+        <v>19.62</v>
+      </c>
+      <c r="I740">
+        <v>0</v>
+      </c>
+      <c r="J740">
+        <v>0</v>
+      </c>
+      <c r="K740">
+        <v>0.2525708719616723</v>
+      </c>
+      <c r="L740">
+        <v>0</v>
+      </c>
+      <c r="M740">
+        <v>0</v>
+      </c>
+      <c r="N740">
+        <v>0</v>
+      </c>
+      <c r="O740">
+        <v>23.8133</v>
+      </c>
+      <c r="P740">
+        <v>72.13528413910095</v>
+      </c>
+      <c r="Q740">
+        <v>33.012</v>
+      </c>
+      <c r="R740">
+        <v>475.86758</v>
+      </c>
+      <c r="S740">
+        <v>6.125906708404225</v>
+      </c>
+      <c r="T740">
+        <v>469.07999</v>
+      </c>
+      <c r="U740">
+        <v>4</v>
+      </c>
+      <c r="V740">
+        <v>11</v>
+      </c>
+      <c r="W740">
+        <v>15</v>
+      </c>
+      <c r="X740">
+        <v>49</v>
+      </c>
+      <c r="Y740">
+        <v>4</v>
+      </c>
+      <c r="Z740">
+        <v>45</v>
+      </c>
+      <c r="AA740">
+        <v>11</v>
+      </c>
+      <c r="AB740">
+        <v>19</v>
+      </c>
+      <c r="AC740">
+        <v>4.38788</v>
+      </c>
+      <c r="AD740">
+        <v>-4.59682</v>
+      </c>
+      <c r="AE740">
+        <v>0</v>
+      </c>
+      <c r="AF740">
+        <v>347.2599</v>
+      </c>
+      <c r="AG740">
+        <v>0</v>
+      </c>
+      <c r="AH740">
+        <v>3</v>
+      </c>
+      <c r="AI740">
+        <v>1427.60274</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B741" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E741">
+        <v>101.429</v>
+      </c>
+      <c r="F741">
+        <v>10306.68</v>
+      </c>
+      <c r="G741">
+        <v>101.6147255715821</v>
+      </c>
+      <c r="H741">
+        <v>704.37</v>
+      </c>
+      <c r="I741">
+        <v>13.22</v>
+      </c>
+      <c r="J741">
+        <v>1</v>
+      </c>
+      <c r="K741">
+        <v>6.944463614942472</v>
+      </c>
+      <c r="L741">
+        <v>18.93</v>
+      </c>
+      <c r="M741">
+        <v>15</v>
+      </c>
+      <c r="N741">
+        <v>1</v>
+      </c>
+      <c r="O741">
+        <v>32.57084</v>
+      </c>
+      <c r="P741">
+        <v>93.08081847279378</v>
+      </c>
+      <c r="Q741">
+        <v>34.992</v>
+      </c>
+      <c r="R741">
+        <v>893.56303</v>
+      </c>
+      <c r="S741">
+        <v>8.809739127862841</v>
+      </c>
+      <c r="T741">
+        <v>1935.21997</v>
+      </c>
+      <c r="U741">
+        <v>34</v>
+      </c>
+      <c r="V741">
+        <v>44</v>
+      </c>
+      <c r="W741">
+        <v>78</v>
+      </c>
+      <c r="X741">
+        <v>134</v>
+      </c>
+      <c r="Y741">
+        <v>34</v>
+      </c>
+      <c r="Z741">
+        <v>128</v>
+      </c>
+      <c r="AA741">
+        <v>44</v>
+      </c>
+      <c r="AB741">
+        <v>42</v>
+      </c>
+      <c r="AC741">
+        <v>4.54577</v>
+      </c>
+      <c r="AD741">
+        <v>-3.81186</v>
+      </c>
+      <c r="AE741">
+        <v>0</v>
+      </c>
+      <c r="AF741">
+        <v>858.39639</v>
+      </c>
+      <c r="AG741">
+        <v>0</v>
+      </c>
+      <c r="AH741">
+        <v>3</v>
+      </c>
+      <c r="AI741">
+        <v>2680.68909</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B742" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E742">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F742">
+        <v>11785.18</v>
+      </c>
+      <c r="G742">
+        <v>94.98878985512113</v>
+      </c>
+      <c r="H742">
+        <v>242.7</v>
+      </c>
+      <c r="I742">
+        <v>0</v>
+      </c>
+      <c r="J742">
+        <v>0</v>
+      </c>
+      <c r="K742">
+        <v>1.956166923020089</v>
+      </c>
+      <c r="L742">
+        <v>0</v>
+      </c>
+      <c r="M742">
+        <v>5</v>
+      </c>
+      <c r="N742">
+        <v>0</v>
+      </c>
+      <c r="O742">
+        <v>28.40544</v>
+      </c>
+      <c r="P742">
+        <v>83.58474576271185</v>
+      </c>
+      <c r="Q742">
+        <v>33.984</v>
+      </c>
+      <c r="R742">
+        <v>1151.15269</v>
+      </c>
+      <c r="S742">
+        <v>9.278314031823648</v>
+      </c>
+      <c r="T742">
+        <v>1277.85</v>
+      </c>
+      <c r="U742">
+        <v>16</v>
+      </c>
+      <c r="V742">
+        <v>30</v>
+      </c>
+      <c r="W742">
+        <v>46</v>
+      </c>
+      <c r="X742">
+        <v>103</v>
+      </c>
+      <c r="Y742">
+        <v>16</v>
+      </c>
+      <c r="Z742">
+        <v>111</v>
+      </c>
+      <c r="AA742">
+        <v>30</v>
+      </c>
+      <c r="AB742">
+        <v>28</v>
+      </c>
+      <c r="AC742">
+        <v>4.20526</v>
+      </c>
+      <c r="AD742">
+        <v>-4.1982</v>
+      </c>
+      <c r="AE742">
+        <v>0</v>
+      </c>
+      <c r="AF742">
+        <v>1077.332</v>
+      </c>
+      <c r="AG742">
+        <v>0</v>
+      </c>
+      <c r="AH742">
+        <v>3</v>
+      </c>
+      <c r="AI742">
+        <v>3453.458070000001</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B743" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E743">
+        <v>60.72083333333333</v>
+      </c>
+      <c r="F743">
+        <v>4737.18</v>
+      </c>
+      <c r="G743">
+        <v>78.01572771563852</v>
+      </c>
+      <c r="H743">
+        <v>102.53</v>
+      </c>
+      <c r="I743">
+        <v>0</v>
+      </c>
+      <c r="J743">
+        <v>0</v>
+      </c>
+      <c r="K743">
+        <v>1.688547313525012</v>
+      </c>
+      <c r="L743">
+        <v>0</v>
+      </c>
+      <c r="M743">
+        <v>0</v>
+      </c>
+      <c r="N743">
+        <v>0</v>
+      </c>
+      <c r="O743">
+        <v>24.80818</v>
+      </c>
+      <c r="P743">
+        <v>70.89671925011432</v>
+      </c>
+      <c r="Q743">
+        <v>34.992</v>
+      </c>
+      <c r="R743">
+        <v>443.83258</v>
+      </c>
+      <c r="S743">
+        <v>7.309395402456598</v>
+      </c>
+      <c r="T743">
+        <v>486.31999</v>
+      </c>
+      <c r="U743">
+        <v>7</v>
+      </c>
+      <c r="V743">
+        <v>13</v>
+      </c>
+      <c r="W743">
+        <v>20</v>
+      </c>
+      <c r="X743">
+        <v>45</v>
+      </c>
+      <c r="Y743">
+        <v>7</v>
+      </c>
+      <c r="Z743">
+        <v>47</v>
+      </c>
+      <c r="AA743">
+        <v>13</v>
+      </c>
+      <c r="AB743">
+        <v>12</v>
+      </c>
+      <c r="AC743">
+        <v>4.09967</v>
+      </c>
+      <c r="AD743">
+        <v>-2.22592</v>
+      </c>
+      <c r="AE743">
+        <v>0</v>
+      </c>
+      <c r="AF743">
+        <v>425.2848</v>
+      </c>
+      <c r="AG743">
+        <v>0</v>
+      </c>
+      <c r="AH743">
+        <v>3</v>
+      </c>
+      <c r="AI743">
+        <v>1331.49774</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B744" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E744">
+        <v>124.0691666666667</v>
+      </c>
+      <c r="F744">
+        <v>11760.9</v>
+      </c>
+      <c r="G744">
+        <v>94.79309256261628</v>
+      </c>
+      <c r="H744">
+        <v>440.83</v>
+      </c>
+      <c r="I744">
+        <v>0</v>
+      </c>
+      <c r="J744">
+        <v>0</v>
+      </c>
+      <c r="K744">
+        <v>3.553098741965167</v>
+      </c>
+      <c r="L744">
+        <v>0</v>
+      </c>
+      <c r="M744">
+        <v>7</v>
+      </c>
+      <c r="N744">
+        <v>0</v>
+      </c>
+      <c r="O744">
+        <v>28.99734</v>
+      </c>
+      <c r="P744">
+        <v>87.83878589603781</v>
+      </c>
+      <c r="Q744">
+        <v>33.012</v>
+      </c>
+      <c r="R744">
+        <v>1066.74312</v>
+      </c>
+      <c r="S744">
+        <v>8.597971185427484</v>
+      </c>
+      <c r="T744">
+        <v>1509.04001</v>
+      </c>
+      <c r="U744">
+        <v>37</v>
+      </c>
+      <c r="V744">
+        <v>31</v>
+      </c>
+      <c r="W744">
+        <v>68</v>
+      </c>
+      <c r="X744">
+        <v>139</v>
+      </c>
+      <c r="Y744">
+        <v>37</v>
+      </c>
+      <c r="Z744">
+        <v>103</v>
+      </c>
+      <c r="AA744">
+        <v>31</v>
+      </c>
+      <c r="AB744">
+        <v>40</v>
+      </c>
+      <c r="AC744">
+        <v>4.23452</v>
+      </c>
+      <c r="AD744">
+        <v>-4.18301</v>
+      </c>
+      <c r="AE744">
+        <v>0</v>
+      </c>
+      <c r="AF744">
+        <v>1009.43625</v>
+      </c>
+      <c r="AG744">
+        <v>0</v>
+      </c>
+      <c r="AH744">
+        <v>3</v>
+      </c>
+      <c r="AI744">
+        <v>3200.22936</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B745" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E745">
+        <v>99.67516666666667</v>
+      </c>
+      <c r="F745">
+        <v>10576.98</v>
+      </c>
+      <c r="G745">
+        <v>106.1144952520772</v>
+      </c>
+      <c r="H745">
+        <v>501.88</v>
+      </c>
+      <c r="I745">
+        <v>0</v>
+      </c>
+      <c r="J745">
+        <v>0</v>
+      </c>
+      <c r="K745">
+        <v>5.035155864633618</v>
+      </c>
+      <c r="L745">
+        <v>0</v>
+      </c>
+      <c r="M745">
+        <v>8</v>
+      </c>
+      <c r="N745">
+        <v>0</v>
+      </c>
+      <c r="O745">
+        <v>27.32674</v>
+      </c>
+      <c r="P745">
+        <v>85.38538932633422</v>
+      </c>
+      <c r="Q745">
+        <v>32.004</v>
+      </c>
+      <c r="R745">
+        <v>970.0047900000001</v>
+      </c>
+      <c r="S745">
+        <v>9.731659574183473</v>
+      </c>
+      <c r="T745">
+        <v>1622.24999</v>
+      </c>
+      <c r="U745">
+        <v>24</v>
+      </c>
+      <c r="V745">
+        <v>25</v>
+      </c>
+      <c r="W745">
+        <v>49</v>
+      </c>
+      <c r="X745">
+        <v>112</v>
+      </c>
+      <c r="Y745">
+        <v>24</v>
+      </c>
+      <c r="Z745">
+        <v>96</v>
+      </c>
+      <c r="AA745">
+        <v>25</v>
+      </c>
+      <c r="AB745">
+        <v>25</v>
+      </c>
+      <c r="AC745">
+        <v>4.22655</v>
+      </c>
+      <c r="AD745">
+        <v>-3.84498</v>
+      </c>
+      <c r="AE745">
+        <v>0</v>
+      </c>
+      <c r="AF745">
+        <v>849.3303</v>
+      </c>
+      <c r="AG745">
+        <v>0</v>
+      </c>
+      <c r="AH745">
+        <v>3</v>
+      </c>
+      <c r="AI745">
+        <v>2910.01437</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B746" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E746">
+        <v>35.84849999999999</v>
+      </c>
+      <c r="F746">
+        <v>2056.4</v>
+      </c>
+      <c r="G746">
+        <v>57.36362748790048</v>
+      </c>
+      <c r="H746">
+        <v>0</v>
+      </c>
+      <c r="I746">
+        <v>0</v>
+      </c>
+      <c r="J746">
+        <v>0</v>
+      </c>
+      <c r="K746">
+        <v>0</v>
+      </c>
+      <c r="L746">
+        <v>0</v>
+      </c>
+      <c r="M746">
+        <v>0</v>
+      </c>
+      <c r="N746">
+        <v>0</v>
+      </c>
+      <c r="O746">
+        <v>18.1685</v>
+      </c>
+      <c r="P746">
+        <v>50.46805555555556</v>
+      </c>
+      <c r="Q746">
+        <v>36</v>
+      </c>
+      <c r="R746">
+        <v>234.57263</v>
+      </c>
+      <c r="S746">
+        <v>6.543443379778792</v>
+      </c>
+      <c r="T746">
+        <v>99.98</v>
+      </c>
+      <c r="U746">
+        <v>6</v>
+      </c>
+      <c r="V746">
+        <v>6</v>
+      </c>
+      <c r="W746">
+        <v>12</v>
+      </c>
+      <c r="X746">
+        <v>15</v>
+      </c>
+      <c r="Y746">
+        <v>6</v>
+      </c>
+      <c r="Z746">
+        <v>15</v>
+      </c>
+      <c r="AA746">
+        <v>6</v>
+      </c>
+      <c r="AB746">
+        <v>7</v>
+      </c>
+      <c r="AC746">
+        <v>3.76097</v>
+      </c>
+      <c r="AD746">
+        <v>-3.18913</v>
+      </c>
+      <c r="AE746">
+        <v>0</v>
+      </c>
+      <c r="AF746">
+        <v>443.1700000000001</v>
+      </c>
+      <c r="AG746">
+        <v>0</v>
+      </c>
+      <c r="AH746">
+        <v>3</v>
+      </c>
+      <c r="AI746">
+        <v>703.71789</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B747" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Partido vs Atlante J2</t>
+        </is>
+      </c>
+      <c r="E747">
+        <v>35.84849999999999</v>
+      </c>
+      <c r="F747">
+        <v>2110.38</v>
+      </c>
+      <c r="G747">
+        <v>58.8694087618729</v>
+      </c>
+      <c r="H747">
+        <v>0</v>
+      </c>
+      <c r="I747">
+        <v>0</v>
+      </c>
+      <c r="J747">
+        <v>0</v>
+      </c>
+      <c r="K747">
+        <v>0</v>
+      </c>
+      <c r="L747">
+        <v>0</v>
+      </c>
+      <c r="M747">
+        <v>0</v>
+      </c>
+      <c r="N747">
+        <v>0</v>
+      </c>
+      <c r="O747">
+        <v>20.82447</v>
+      </c>
+      <c r="P747">
+        <v>57.84575000000001</v>
+      </c>
+      <c r="Q747">
+        <v>36</v>
+      </c>
+      <c r="R747">
+        <v>288.4156</v>
+      </c>
+      <c r="S747">
+        <v>8.045402178612775</v>
+      </c>
+      <c r="T747">
+        <v>128.91</v>
+      </c>
+      <c r="U747">
+        <v>9</v>
+      </c>
+      <c r="V747">
+        <v>4</v>
+      </c>
+      <c r="W747">
+        <v>13</v>
+      </c>
+      <c r="X747">
+        <v>18</v>
+      </c>
+      <c r="Y747">
+        <v>9</v>
+      </c>
+      <c r="Z747">
+        <v>19</v>
+      </c>
+      <c r="AA747">
+        <v>4</v>
+      </c>
+      <c r="AB747">
+        <v>8</v>
+      </c>
+      <c r="AC747">
+        <v>3.66353</v>
+      </c>
+      <c r="AD747">
+        <v>-2.70126</v>
+      </c>
+      <c r="AE747">
+        <v>0</v>
+      </c>
+      <c r="AF747">
+        <v>451.444</v>
+      </c>
+      <c r="AG747">
+        <v>0</v>
+      </c>
+      <c r="AH747">
+        <v>3</v>
+      </c>
+      <c r="AI747">
+        <v>865.2468000000001</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B748" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E748">
+        <v>64.64783333333334</v>
+      </c>
+      <c r="F748">
+        <v>3682.43</v>
+      </c>
+      <c r="G748">
+        <v>56.96138308321753</v>
+      </c>
+      <c r="H748">
+        <v>66.26000000000001</v>
+      </c>
+      <c r="I748">
+        <v>0</v>
+      </c>
+      <c r="J748">
+        <v>0</v>
+      </c>
+      <c r="K748">
+        <v>1.024937675147659</v>
+      </c>
+      <c r="L748">
+        <v>0</v>
+      </c>
+      <c r="M748">
+        <v>0</v>
+      </c>
+      <c r="N748">
+        <v>0</v>
+      </c>
+      <c r="O748">
+        <v>22.69943</v>
+      </c>
+      <c r="P748">
+        <v>64.8703417924097</v>
+      </c>
+      <c r="Q748">
+        <v>34.992</v>
+      </c>
+      <c r="R748">
+        <v>409.37338</v>
+      </c>
+      <c r="S748">
+        <v>6.332360403932072</v>
+      </c>
+      <c r="T748">
+        <v>389.73001</v>
+      </c>
+      <c r="U748">
+        <v>3</v>
+      </c>
+      <c r="V748">
+        <v>10</v>
+      </c>
+      <c r="W748">
+        <v>13</v>
+      </c>
+      <c r="X748">
+        <v>45</v>
+      </c>
+      <c r="Y748">
+        <v>3</v>
+      </c>
+      <c r="Z748">
+        <v>32</v>
+      </c>
+      <c r="AA748">
+        <v>10</v>
+      </c>
+      <c r="AB748">
+        <v>10</v>
+      </c>
+      <c r="AC748">
+        <v>3.38188</v>
+      </c>
+      <c r="AD748">
+        <v>-4.39091</v>
+      </c>
+      <c r="AE748">
+        <v>0</v>
+      </c>
+      <c r="AF748">
+        <v>333.8848</v>
+      </c>
+      <c r="AG748">
+        <v>0</v>
+      </c>
+      <c r="AH748">
+        <v>3</v>
+      </c>
+      <c r="AI748">
+        <v>1228.12014</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B749" s="2">
+        <v>46227</v>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Trabajo Seleccionados</t>
+        </is>
+      </c>
+      <c r="E749">
+        <v>65.49066666666667</v>
+      </c>
+      <c r="F749">
+        <v>4296.21</v>
+      </c>
+      <c r="G749">
+        <v>65.6003399975569</v>
+      </c>
+      <c r="H749">
+        <v>311.61</v>
+      </c>
+      <c r="I749">
+        <v>0</v>
+      </c>
+      <c r="J749">
+        <v>0</v>
+      </c>
+      <c r="K749">
+        <v>4.758082576652144</v>
+      </c>
+      <c r="L749">
+        <v>0</v>
+      </c>
+      <c r="M749">
+        <v>1</v>
+      </c>
+      <c r="N749">
+        <v>0</v>
+      </c>
+      <c r="O749">
+        <v>26.47499</v>
+      </c>
+      <c r="P749">
+        <v>77.90427848399246</v>
+      </c>
+      <c r="Q749">
+        <v>33.984</v>
+      </c>
+      <c r="R749">
+        <v>416.21472</v>
+      </c>
+      <c r="S749">
+        <v>6.355328800032574</v>
+      </c>
+      <c r="T749">
+        <v>555.57001</v>
+      </c>
+      <c r="U749">
+        <v>3</v>
+      </c>
+      <c r="V749">
+        <v>7</v>
+      </c>
+      <c r="W749">
+        <v>10</v>
+      </c>
+      <c r="X749">
+        <v>22</v>
+      </c>
+      <c r="Y749">
+        <v>3</v>
+      </c>
+      <c r="Z749">
+        <v>13</v>
+      </c>
+      <c r="AA749">
+        <v>7</v>
+      </c>
+      <c r="AB749">
+        <v>5</v>
+      </c>
+      <c r="AC749">
+        <v>3.61179</v>
+      </c>
+      <c r="AD749">
+        <v>-3.59819</v>
+      </c>
+      <c r="AE749">
+        <v>0</v>
+      </c>
+      <c r="AF749">
+        <v>328.3931</v>
+      </c>
+      <c r="AG749">
+        <v>0</v>
+      </c>
+      <c r="AH749">
+        <v>3</v>
+      </c>
+      <c r="AI749">
+        <v>1248.64416</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-26
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI749"/>
+  <dimension ref="A1:AI760"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -84952,6 +84952,1249 @@
         <v>1248.64416</v>
       </c>
     </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B750" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E750">
+        <v>68.739</v>
+      </c>
+      <c r="F750">
+        <v>6739.330000000001</v>
+      </c>
+      <c r="G750">
+        <v>98.04230495061029</v>
+      </c>
+      <c r="H750">
+        <v>327.06</v>
+      </c>
+      <c r="I750">
+        <v>0</v>
+      </c>
+      <c r="J750">
+        <v>0</v>
+      </c>
+      <c r="K750">
+        <v>4.757997643259285</v>
+      </c>
+      <c r="L750">
+        <v>0</v>
+      </c>
+      <c r="M750">
+        <v>7</v>
+      </c>
+      <c r="N750">
+        <v>0</v>
+      </c>
+      <c r="O750">
+        <v>29.4587</v>
+      </c>
+      <c r="P750">
+        <v>81.82972222222222</v>
+      </c>
+      <c r="Q750">
+        <v>36</v>
+      </c>
+      <c r="R750">
+        <v>642.56616</v>
+      </c>
+      <c r="S750">
+        <v>9.347912538733469</v>
+      </c>
+      <c r="T750">
+        <v>1212.17999</v>
+      </c>
+      <c r="U750">
+        <v>24</v>
+      </c>
+      <c r="V750">
+        <v>34</v>
+      </c>
+      <c r="W750">
+        <v>58</v>
+      </c>
+      <c r="X750">
+        <v>105</v>
+      </c>
+      <c r="Y750">
+        <v>24</v>
+      </c>
+      <c r="Z750">
+        <v>98</v>
+      </c>
+      <c r="AA750">
+        <v>34</v>
+      </c>
+      <c r="AB750">
+        <v>34</v>
+      </c>
+      <c r="AC750">
+        <v>4.47679</v>
+      </c>
+      <c r="AD750">
+        <v>-3.97017</v>
+      </c>
+      <c r="AE750">
+        <v>0</v>
+      </c>
+      <c r="AF750">
+        <v>1642.756</v>
+      </c>
+      <c r="AG750">
+        <v>0</v>
+      </c>
+      <c r="AH750">
+        <v>3</v>
+      </c>
+      <c r="AI750">
+        <v>1927.69848</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B751" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E751">
+        <v>113.225</v>
+      </c>
+      <c r="F751">
+        <v>11660.11</v>
+      </c>
+      <c r="G751">
+        <v>102.9817619783617</v>
+      </c>
+      <c r="H751">
+        <v>246.99</v>
+      </c>
+      <c r="I751">
+        <v>0</v>
+      </c>
+      <c r="J751">
+        <v>0</v>
+      </c>
+      <c r="K751">
+        <v>2.181408699492162</v>
+      </c>
+      <c r="L751">
+        <v>0</v>
+      </c>
+      <c r="M751">
+        <v>1</v>
+      </c>
+      <c r="N751">
+        <v>0</v>
+      </c>
+      <c r="O751">
+        <v>25.80106</v>
+      </c>
+      <c r="P751">
+        <v>79.7214806575207</v>
+      </c>
+      <c r="Q751">
+        <v>32.364</v>
+      </c>
+      <c r="R751">
+        <v>1068.70931</v>
+      </c>
+      <c r="S751">
+        <v>9.43881042172665</v>
+      </c>
+      <c r="T751">
+        <v>1357.45996</v>
+      </c>
+      <c r="U751">
+        <v>13</v>
+      </c>
+      <c r="V751">
+        <v>18</v>
+      </c>
+      <c r="W751">
+        <v>31</v>
+      </c>
+      <c r="X751">
+        <v>99</v>
+      </c>
+      <c r="Y751">
+        <v>13</v>
+      </c>
+      <c r="Z751">
+        <v>75</v>
+      </c>
+      <c r="AA751">
+        <v>18</v>
+      </c>
+      <c r="AB751">
+        <v>20</v>
+      </c>
+      <c r="AC751">
+        <v>3.66642</v>
+      </c>
+      <c r="AD751">
+        <v>-2.60398</v>
+      </c>
+      <c r="AE751">
+        <v>0</v>
+      </c>
+      <c r="AF751">
+        <v>935.9336000000001</v>
+      </c>
+      <c r="AG751">
+        <v>0</v>
+      </c>
+      <c r="AH751">
+        <v>3</v>
+      </c>
+      <c r="AI751">
+        <v>3206.12793</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B752" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E752">
+        <v>89.83133333333333</v>
+      </c>
+      <c r="F752">
+        <v>8585.139999999999</v>
+      </c>
+      <c r="G752">
+        <v>95.5695488582306</v>
+      </c>
+      <c r="H752">
+        <v>386.7</v>
+      </c>
+      <c r="I752">
+        <v>0</v>
+      </c>
+      <c r="J752">
+        <v>0</v>
+      </c>
+      <c r="K752">
+        <v>4.304734057158972</v>
+      </c>
+      <c r="L752">
+        <v>0</v>
+      </c>
+      <c r="M752">
+        <v>7</v>
+      </c>
+      <c r="N752">
+        <v>0</v>
+      </c>
+      <c r="O752">
+        <v>29.59941</v>
+      </c>
+      <c r="P752">
+        <v>82.22058333333334</v>
+      </c>
+      <c r="Q752">
+        <v>36</v>
+      </c>
+      <c r="R752">
+        <v>665.06375</v>
+      </c>
+      <c r="S752">
+        <v>7.403471876924904</v>
+      </c>
+      <c r="T752">
+        <v>1284.44</v>
+      </c>
+      <c r="U752">
+        <v>23</v>
+      </c>
+      <c r="V752">
+        <v>50</v>
+      </c>
+      <c r="W752">
+        <v>73</v>
+      </c>
+      <c r="X752">
+        <v>118</v>
+      </c>
+      <c r="Y752">
+        <v>23</v>
+      </c>
+      <c r="Z752">
+        <v>121</v>
+      </c>
+      <c r="AA752">
+        <v>50</v>
+      </c>
+      <c r="AB752">
+        <v>35</v>
+      </c>
+      <c r="AC752">
+        <v>4.40291</v>
+      </c>
+      <c r="AD752">
+        <v>-4.11242</v>
+      </c>
+      <c r="AE752">
+        <v>0</v>
+      </c>
+      <c r="AF752">
+        <v>2049.368</v>
+      </c>
+      <c r="AG752">
+        <v>0</v>
+      </c>
+      <c r="AH752">
+        <v>3</v>
+      </c>
+      <c r="AI752">
+        <v>1995.19125</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B753" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E753">
+        <v>113.225</v>
+      </c>
+      <c r="F753">
+        <v>12168.54</v>
+      </c>
+      <c r="G753">
+        <v>107.4722013689556</v>
+      </c>
+      <c r="H753">
+        <v>541.09</v>
+      </c>
+      <c r="I753">
+        <v>15.26</v>
+      </c>
+      <c r="J753">
+        <v>1</v>
+      </c>
+      <c r="K753">
+        <v>4.77889158754692</v>
+      </c>
+      <c r="L753">
+        <v>4.11</v>
+      </c>
+      <c r="M753">
+        <v>8</v>
+      </c>
+      <c r="N753">
+        <v>0</v>
+      </c>
+      <c r="O753">
+        <v>29.96021</v>
+      </c>
+      <c r="P753">
+        <v>92.46978395061728</v>
+      </c>
+      <c r="Q753">
+        <v>32.4</v>
+      </c>
+      <c r="R753">
+        <v>1246.19375</v>
+      </c>
+      <c r="S753">
+        <v>11.00634797968647</v>
+      </c>
+      <c r="T753">
+        <v>2076.52996</v>
+      </c>
+      <c r="U753">
+        <v>32</v>
+      </c>
+      <c r="V753">
+        <v>31</v>
+      </c>
+      <c r="W753">
+        <v>63</v>
+      </c>
+      <c r="X753">
+        <v>167</v>
+      </c>
+      <c r="Y753">
+        <v>32</v>
+      </c>
+      <c r="Z753">
+        <v>113</v>
+      </c>
+      <c r="AA753">
+        <v>31</v>
+      </c>
+      <c r="AB753">
+        <v>14</v>
+      </c>
+      <c r="AC753">
+        <v>4.51413</v>
+      </c>
+      <c r="AD753">
+        <v>-3.8598</v>
+      </c>
+      <c r="AE753">
+        <v>0</v>
+      </c>
+      <c r="AF753">
+        <v>1010.2253</v>
+      </c>
+      <c r="AG753">
+        <v>0</v>
+      </c>
+      <c r="AH753">
+        <v>3</v>
+      </c>
+      <c r="AI753">
+        <v>3738.58125</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B754" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E754">
+        <v>113.225</v>
+      </c>
+      <c r="F754">
+        <v>10391.86</v>
+      </c>
+      <c r="G754">
+        <v>91.78061382203576</v>
+      </c>
+      <c r="H754">
+        <v>474.3099999999999</v>
+      </c>
+      <c r="I754">
+        <v>0</v>
+      </c>
+      <c r="J754">
+        <v>0</v>
+      </c>
+      <c r="K754">
+        <v>4.189092514903952</v>
+      </c>
+      <c r="L754">
+        <v>20.65</v>
+      </c>
+      <c r="M754">
+        <v>11</v>
+      </c>
+      <c r="N754">
+        <v>1</v>
+      </c>
+      <c r="O754">
+        <v>31.74266</v>
+      </c>
+      <c r="P754">
+        <v>88.17405555555555</v>
+      </c>
+      <c r="Q754">
+        <v>36</v>
+      </c>
+      <c r="R754">
+        <v>950.1618100000001</v>
+      </c>
+      <c r="S754">
+        <v>8.391802252152795</v>
+      </c>
+      <c r="T754">
+        <v>1353.28996</v>
+      </c>
+      <c r="U754">
+        <v>28</v>
+      </c>
+      <c r="V754">
+        <v>43</v>
+      </c>
+      <c r="W754">
+        <v>71</v>
+      </c>
+      <c r="X754">
+        <v>106</v>
+      </c>
+      <c r="Y754">
+        <v>28</v>
+      </c>
+      <c r="Z754">
+        <v>104</v>
+      </c>
+      <c r="AA754">
+        <v>43</v>
+      </c>
+      <c r="AB754">
+        <v>29</v>
+      </c>
+      <c r="AC754">
+        <v>4.1367</v>
+      </c>
+      <c r="AD754">
+        <v>-3.73585</v>
+      </c>
+      <c r="AE754">
+        <v>0</v>
+      </c>
+      <c r="AF754">
+        <v>2445.84</v>
+      </c>
+      <c r="AG754">
+        <v>0</v>
+      </c>
+      <c r="AH754">
+        <v>3</v>
+      </c>
+      <c r="AI754">
+        <v>2850.48543</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B755" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E755">
+        <v>113.225</v>
+      </c>
+      <c r="F755">
+        <v>10249.45</v>
+      </c>
+      <c r="G755">
+        <v>90.52285272687128</v>
+      </c>
+      <c r="H755">
+        <v>339.77</v>
+      </c>
+      <c r="I755">
+        <v>0</v>
+      </c>
+      <c r="J755">
+        <v>0</v>
+      </c>
+      <c r="K755">
+        <v>3.000839037315081</v>
+      </c>
+      <c r="L755">
+        <v>18.16</v>
+      </c>
+      <c r="M755">
+        <v>7</v>
+      </c>
+      <c r="N755">
+        <v>2</v>
+      </c>
+      <c r="O755">
+        <v>31.14383</v>
+      </c>
+      <c r="P755">
+        <v>86.51063888888889</v>
+      </c>
+      <c r="Q755">
+        <v>36</v>
+      </c>
+      <c r="R755">
+        <v>845.32965</v>
+      </c>
+      <c r="S755">
+        <v>7.465927577831751</v>
+      </c>
+      <c r="T755">
+        <v>1177.66</v>
+      </c>
+      <c r="U755">
+        <v>31</v>
+      </c>
+      <c r="V755">
+        <v>32</v>
+      </c>
+      <c r="W755">
+        <v>63</v>
+      </c>
+      <c r="X755">
+        <v>110</v>
+      </c>
+      <c r="Y755">
+        <v>31</v>
+      </c>
+      <c r="Z755">
+        <v>86</v>
+      </c>
+      <c r="AA755">
+        <v>32</v>
+      </c>
+      <c r="AB755">
+        <v>22</v>
+      </c>
+      <c r="AC755">
+        <v>5.04734</v>
+      </c>
+      <c r="AD755">
+        <v>-4.14116</v>
+      </c>
+      <c r="AE755">
+        <v>0</v>
+      </c>
+      <c r="AF755">
+        <v>837.3064000000001</v>
+      </c>
+      <c r="AG755">
+        <v>0</v>
+      </c>
+      <c r="AH755">
+        <v>3</v>
+      </c>
+      <c r="AI755">
+        <v>2535.98895</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B756" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E756">
+        <v>113.225</v>
+      </c>
+      <c r="F756">
+        <v>10471.48</v>
+      </c>
+      <c r="G756">
+        <v>92.4838154117907</v>
+      </c>
+      <c r="H756">
+        <v>638.42</v>
+      </c>
+      <c r="I756">
+        <v>0</v>
+      </c>
+      <c r="J756">
+        <v>0</v>
+      </c>
+      <c r="K756">
+        <v>5.638507396776331</v>
+      </c>
+      <c r="L756">
+        <v>12.61</v>
+      </c>
+      <c r="M756">
+        <v>20</v>
+      </c>
+      <c r="N756">
+        <v>1</v>
+      </c>
+      <c r="O756">
+        <v>31.01347</v>
+      </c>
+      <c r="P756">
+        <v>91.64736997635934</v>
+      </c>
+      <c r="Q756">
+        <v>33.84</v>
+      </c>
+      <c r="R756">
+        <v>890.09898</v>
+      </c>
+      <c r="S756">
+        <v>7.861329035107087</v>
+      </c>
+      <c r="T756">
+        <v>1644.05002</v>
+      </c>
+      <c r="U756">
+        <v>47</v>
+      </c>
+      <c r="V756">
+        <v>52</v>
+      </c>
+      <c r="W756">
+        <v>99</v>
+      </c>
+      <c r="X756">
+        <v>150</v>
+      </c>
+      <c r="Y756">
+        <v>47</v>
+      </c>
+      <c r="Z756">
+        <v>141</v>
+      </c>
+      <c r="AA756">
+        <v>52</v>
+      </c>
+      <c r="AB756">
+        <v>32</v>
+      </c>
+      <c r="AC756">
+        <v>4.79902</v>
+      </c>
+      <c r="AD756">
+        <v>-4.87801</v>
+      </c>
+      <c r="AE756">
+        <v>0</v>
+      </c>
+      <c r="AF756">
+        <v>885.8332</v>
+      </c>
+      <c r="AG756">
+        <v>0</v>
+      </c>
+      <c r="AH756">
+        <v>3</v>
+      </c>
+      <c r="AI756">
+        <v>2670.29694</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B757" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E757">
+        <v>113.225</v>
+      </c>
+      <c r="F757">
+        <v>11234.54</v>
+      </c>
+      <c r="G757">
+        <v>99.22313976595275</v>
+      </c>
+      <c r="H757">
+        <v>262.89</v>
+      </c>
+      <c r="I757">
+        <v>0</v>
+      </c>
+      <c r="J757">
+        <v>0</v>
+      </c>
+      <c r="K757">
+        <v>2.32183705012144</v>
+      </c>
+      <c r="L757">
+        <v>0</v>
+      </c>
+      <c r="M757">
+        <v>4</v>
+      </c>
+      <c r="N757">
+        <v>0</v>
+      </c>
+      <c r="O757">
+        <v>27.62977</v>
+      </c>
+      <c r="P757">
+        <v>83.69614079728584</v>
+      </c>
+      <c r="Q757">
+        <v>33.012</v>
+      </c>
+      <c r="R757">
+        <v>1058.55971</v>
+      </c>
+      <c r="S757">
+        <v>9.349169441377787</v>
+      </c>
+      <c r="T757">
+        <v>1337.55995</v>
+      </c>
+      <c r="U757">
+        <v>16</v>
+      </c>
+      <c r="V757">
+        <v>41</v>
+      </c>
+      <c r="W757">
+        <v>57</v>
+      </c>
+      <c r="X757">
+        <v>132</v>
+      </c>
+      <c r="Y757">
+        <v>16</v>
+      </c>
+      <c r="Z757">
+        <v>108</v>
+      </c>
+      <c r="AA757">
+        <v>41</v>
+      </c>
+      <c r="AB757">
+        <v>35</v>
+      </c>
+      <c r="AC757">
+        <v>4.05221</v>
+      </c>
+      <c r="AD757">
+        <v>-3.97879</v>
+      </c>
+      <c r="AE757">
+        <v>0</v>
+      </c>
+      <c r="AF757">
+        <v>1022.66736</v>
+      </c>
+      <c r="AG757">
+        <v>0</v>
+      </c>
+      <c r="AH757">
+        <v>3</v>
+      </c>
+      <c r="AI757">
+        <v>3175.67913</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B758" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E758">
+        <v>67.94366666666666</v>
+      </c>
+      <c r="F758">
+        <v>5114.66</v>
+      </c>
+      <c r="G758">
+        <v>75.27795085144066</v>
+      </c>
+      <c r="H758">
+        <v>98.04000000000001</v>
+      </c>
+      <c r="I758">
+        <v>0</v>
+      </c>
+      <c r="J758">
+        <v>0</v>
+      </c>
+      <c r="K758">
+        <v>1.442960099297948</v>
+      </c>
+      <c r="L758">
+        <v>0</v>
+      </c>
+      <c r="M758">
+        <v>0</v>
+      </c>
+      <c r="N758">
+        <v>0</v>
+      </c>
+      <c r="O758">
+        <v>22.19239</v>
+      </c>
+      <c r="P758">
+        <v>63.55209049255441</v>
+      </c>
+      <c r="Q758">
+        <v>34.92</v>
+      </c>
+      <c r="R758">
+        <v>543.1098</v>
+      </c>
+      <c r="S758">
+        <v>7.993530915317101</v>
+      </c>
+      <c r="T758">
+        <v>672.52002</v>
+      </c>
+      <c r="U758">
+        <v>20</v>
+      </c>
+      <c r="V758">
+        <v>7</v>
+      </c>
+      <c r="W758">
+        <v>27</v>
+      </c>
+      <c r="X758">
+        <v>72</v>
+      </c>
+      <c r="Y758">
+        <v>20</v>
+      </c>
+      <c r="Z758">
+        <v>44</v>
+      </c>
+      <c r="AA758">
+        <v>7</v>
+      </c>
+      <c r="AB758">
+        <v>3</v>
+      </c>
+      <c r="AC758">
+        <v>3.5955</v>
+      </c>
+      <c r="AD758">
+        <v>-3.24963</v>
+      </c>
+      <c r="AE758">
+        <v>0</v>
+      </c>
+      <c r="AF758">
+        <v>467.8592</v>
+      </c>
+      <c r="AG758">
+        <v>0</v>
+      </c>
+      <c r="AH758">
+        <v>3</v>
+      </c>
+      <c r="AI758">
+        <v>1629.3294</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B759" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E759">
+        <v>113.225</v>
+      </c>
+      <c r="F759">
+        <v>10117.27</v>
+      </c>
+      <c r="G759">
+        <v>89.35544270258336</v>
+      </c>
+      <c r="H759">
+        <v>330.05</v>
+      </c>
+      <c r="I759">
+        <v>0</v>
+      </c>
+      <c r="J759">
+        <v>0</v>
+      </c>
+      <c r="K759">
+        <v>2.914992272024729</v>
+      </c>
+      <c r="L759">
+        <v>0</v>
+      </c>
+      <c r="M759">
+        <v>2</v>
+      </c>
+      <c r="N759">
+        <v>0</v>
+      </c>
+      <c r="O759">
+        <v>25.37637</v>
+      </c>
+      <c r="P759">
+        <v>72.52049039780523</v>
+      </c>
+      <c r="Q759">
+        <v>34.992</v>
+      </c>
+      <c r="R759">
+        <v>798.78984</v>
+      </c>
+      <c r="S759">
+        <v>7.054889291234269</v>
+      </c>
+      <c r="T759">
+        <v>1423.44002</v>
+      </c>
+      <c r="U759">
+        <v>26</v>
+      </c>
+      <c r="V759">
+        <v>34</v>
+      </c>
+      <c r="W759">
+        <v>60</v>
+      </c>
+      <c r="X759">
+        <v>122</v>
+      </c>
+      <c r="Y759">
+        <v>26</v>
+      </c>
+      <c r="Z759">
+        <v>119</v>
+      </c>
+      <c r="AA759">
+        <v>34</v>
+      </c>
+      <c r="AB759">
+        <v>25</v>
+      </c>
+      <c r="AC759">
+        <v>4.15405</v>
+      </c>
+      <c r="AD759">
+        <v>-3.90237</v>
+      </c>
+      <c r="AE759">
+        <v>0</v>
+      </c>
+      <c r="AF759">
+        <v>955.2088000000001</v>
+      </c>
+      <c r="AG759">
+        <v>0</v>
+      </c>
+      <c r="AH759">
+        <v>3</v>
+      </c>
+      <c r="AI759">
+        <v>2396.36952</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B760" s="2">
+        <v>46228</v>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Amistoso vs Zacatepec</t>
+        </is>
+      </c>
+      <c r="E760">
+        <v>70.4965</v>
+      </c>
+      <c r="F760">
+        <v>8310.07</v>
+      </c>
+      <c r="G760">
+        <v>117.8791854914783</v>
+      </c>
+      <c r="H760">
+        <v>116.63</v>
+      </c>
+      <c r="I760">
+        <v>0</v>
+      </c>
+      <c r="J760">
+        <v>0</v>
+      </c>
+      <c r="K760">
+        <v>1.654408374883859</v>
+      </c>
+      <c r="L760">
+        <v>0</v>
+      </c>
+      <c r="M760">
+        <v>0</v>
+      </c>
+      <c r="N760">
+        <v>0</v>
+      </c>
+      <c r="O760">
+        <v>24.02553</v>
+      </c>
+      <c r="P760">
+        <v>66.73758333333333</v>
+      </c>
+      <c r="Q760">
+        <v>36</v>
+      </c>
+      <c r="R760">
+        <v>787.8290400000001</v>
+      </c>
+      <c r="S760">
+        <v>11.1754348088203</v>
+      </c>
+      <c r="T760">
+        <v>863.37999</v>
+      </c>
+      <c r="U760">
+        <v>13</v>
+      </c>
+      <c r="V760">
+        <v>25</v>
+      </c>
+      <c r="W760">
+        <v>38</v>
+      </c>
+      <c r="X760">
+        <v>78</v>
+      </c>
+      <c r="Y760">
+        <v>13</v>
+      </c>
+      <c r="Z760">
+        <v>93</v>
+      </c>
+      <c r="AA760">
+        <v>25</v>
+      </c>
+      <c r="AB760">
+        <v>17</v>
+      </c>
+      <c r="AC760">
+        <v>4.6731</v>
+      </c>
+      <c r="AD760">
+        <v>-4.44976</v>
+      </c>
+      <c r="AE760">
+        <v>0</v>
+      </c>
+      <c r="AF760">
+        <v>1937.816</v>
+      </c>
+      <c r="AG760">
+        <v>0</v>
+      </c>
+      <c r="AH760">
+        <v>3</v>
+      </c>
+      <c r="AI760">
+        <v>2363.48712</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-28
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI760"/>
+  <dimension ref="A1:AI785"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -84975,10 +84975,10 @@
         <v>68.739</v>
       </c>
       <c r="F750">
-        <v>6739.330000000001</v>
+        <v>6739.37</v>
       </c>
       <c r="G750">
-        <v>98.04230495061029</v>
+        <v>98.0428868618979</v>
       </c>
       <c r="H750">
         <v>327.06</v>
@@ -85011,10 +85011,10 @@
         <v>36</v>
       </c>
       <c r="R750">
-        <v>642.56616</v>
+        <v>642.56674</v>
       </c>
       <c r="S750">
-        <v>9.347912538733469</v>
+        <v>9.34792097644714</v>
       </c>
       <c r="T750">
         <v>1212.17999</v>
@@ -85053,7 +85053,7 @@
         <v>0</v>
       </c>
       <c r="AF750">
-        <v>1642.756</v>
+        <v>1642.762</v>
       </c>
       <c r="AG750">
         <v>0</v>
@@ -85062,7 +85062,7 @@
         <v>3</v>
       </c>
       <c r="AI750">
-        <v>1927.69848</v>
+        <v>1927.70022</v>
       </c>
     </row>
     <row r="751">
@@ -85088,10 +85088,10 @@
         <v>113.225</v>
       </c>
       <c r="F751">
-        <v>11660.11</v>
+        <v>11660.28</v>
       </c>
       <c r="G751">
-        <v>102.9817619783617</v>
+        <v>102.9832634135571</v>
       </c>
       <c r="H751">
         <v>246.99</v>
@@ -85124,10 +85124,10 @@
         <v>32.364</v>
       </c>
       <c r="R751">
-        <v>1068.70931</v>
+        <v>1068.72058</v>
       </c>
       <c r="S751">
-        <v>9.43881042172665</v>
+        <v>9.438909958048134</v>
       </c>
       <c r="T751">
         <v>1357.45996</v>
@@ -85166,7 +85166,7 @@
         <v>0</v>
       </c>
       <c r="AF751">
-        <v>935.9336000000001</v>
+        <v>935.9469</v>
       </c>
       <c r="AG751">
         <v>0</v>
@@ -85175,7 +85175,7 @@
         <v>3</v>
       </c>
       <c r="AI751">
-        <v>3206.12793</v>
+        <v>3206.16174</v>
       </c>
     </row>
     <row r="752">
@@ -85201,10 +85201,10 @@
         <v>89.83133333333333</v>
       </c>
       <c r="F752">
-        <v>8585.139999999999</v>
+        <v>8585.389999999999</v>
       </c>
       <c r="G752">
-        <v>95.5695488582306</v>
+        <v>95.57233185154399</v>
       </c>
       <c r="H752">
         <v>386.7</v>
@@ -85237,10 +85237,10 @@
         <v>36</v>
       </c>
       <c r="R752">
-        <v>665.06375</v>
+        <v>665.0877399999999</v>
       </c>
       <c r="S752">
-        <v>7.403471876924904</v>
+        <v>7.403738932963257</v>
       </c>
       <c r="T752">
         <v>1284.44</v>
@@ -85279,7 +85279,7 @@
         <v>0</v>
       </c>
       <c r="AF752">
-        <v>2049.368</v>
+        <v>2049.462</v>
       </c>
       <c r="AG752">
         <v>0</v>
@@ -85288,7 +85288,7 @@
         <v>3</v>
       </c>
       <c r="AI752">
-        <v>1995.19125</v>
+        <v>1995.26322</v>
       </c>
     </row>
     <row r="753">
@@ -85314,10 +85314,10 @@
         <v>113.225</v>
       </c>
       <c r="F753">
-        <v>12168.54</v>
+        <v>12168.9</v>
       </c>
       <c r="G753">
-        <v>107.4722013689556</v>
+        <v>107.4753808787812</v>
       </c>
       <c r="H753">
         <v>541.09</v>
@@ -85350,10 +85350,10 @@
         <v>32.4</v>
       </c>
       <c r="R753">
-        <v>1246.19375</v>
+        <v>1246.21982</v>
       </c>
       <c r="S753">
-        <v>11.00634797968647</v>
+        <v>11.00657822918967</v>
       </c>
       <c r="T753">
         <v>2076.52996</v>
@@ -85392,7 +85392,7 @@
         <v>0</v>
       </c>
       <c r="AF753">
-        <v>1010.2253</v>
+        <v>1010.2561</v>
       </c>
       <c r="AG753">
         <v>0</v>
@@ -85401,7 +85401,7 @@
         <v>3</v>
       </c>
       <c r="AI753">
-        <v>3738.58125</v>
+        <v>3738.65946</v>
       </c>
     </row>
     <row r="754">
@@ -85427,10 +85427,10 @@
         <v>113.225</v>
       </c>
       <c r="F754">
-        <v>10391.86</v>
+        <v>10391.96</v>
       </c>
       <c r="G754">
-        <v>91.78061382203576</v>
+        <v>91.78149701920954</v>
       </c>
       <c r="H754">
         <v>474.3099999999999</v>
@@ -85463,10 +85463,10 @@
         <v>36</v>
       </c>
       <c r="R754">
-        <v>950.1618100000001</v>
+        <v>950.1679399999999</v>
       </c>
       <c r="S754">
-        <v>8.391802252152795</v>
+        <v>8.391856392139545</v>
       </c>
       <c r="T754">
         <v>1353.28996</v>
@@ -85505,7 +85505,7 @@
         <v>0</v>
       </c>
       <c r="AF754">
-        <v>2445.84</v>
+        <v>2445.86</v>
       </c>
       <c r="AG754">
         <v>0</v>
@@ -85514,7 +85514,7 @@
         <v>3</v>
       </c>
       <c r="AI754">
-        <v>2850.48543</v>
+        <v>2850.50382</v>
       </c>
     </row>
     <row r="755">
@@ -85540,10 +85540,10 @@
         <v>113.225</v>
       </c>
       <c r="F755">
-        <v>10249.45</v>
+        <v>10249.72</v>
       </c>
       <c r="G755">
-        <v>90.52285272687128</v>
+        <v>90.52523735924045</v>
       </c>
       <c r="H755">
         <v>339.77</v>
@@ -85576,10 +85576,10 @@
         <v>36</v>
       </c>
       <c r="R755">
-        <v>845.32965</v>
+        <v>845.3459</v>
       </c>
       <c r="S755">
-        <v>7.465927577831751</v>
+        <v>7.466071097372489</v>
       </c>
       <c r="T755">
         <v>1177.66</v>
@@ -85618,7 +85618,7 @@
         <v>0</v>
       </c>
       <c r="AF755">
-        <v>837.3064000000001</v>
+        <v>837.3344</v>
       </c>
       <c r="AG755">
         <v>0</v>
@@ -85627,7 +85627,7 @@
         <v>3</v>
       </c>
       <c r="AI755">
-        <v>2535.98895</v>
+        <v>2536.0377</v>
       </c>
     </row>
     <row r="756">
@@ -85653,10 +85653,10 @@
         <v>113.225</v>
       </c>
       <c r="F756">
-        <v>10471.48</v>
+        <v>10471.69</v>
       </c>
       <c r="G756">
-        <v>92.4838154117907</v>
+        <v>92.48567012585561</v>
       </c>
       <c r="H756">
         <v>638.42</v>
@@ -85689,10 +85689,10 @@
         <v>33.84</v>
       </c>
       <c r="R756">
-        <v>890.09898</v>
+        <v>890.11186</v>
       </c>
       <c r="S756">
-        <v>7.861329035107087</v>
+        <v>7.86144279090307</v>
       </c>
       <c r="T756">
         <v>1644.05002</v>
@@ -85731,7 +85731,7 @@
         <v>0</v>
       </c>
       <c r="AF756">
-        <v>885.8332</v>
+        <v>885.8479</v>
       </c>
       <c r="AG756">
         <v>0</v>
@@ -85740,7 +85740,7 @@
         <v>3</v>
       </c>
       <c r="AI756">
-        <v>2670.29694</v>
+        <v>2670.33558</v>
       </c>
     </row>
     <row r="757">
@@ -85766,10 +85766,10 @@
         <v>113.225</v>
       </c>
       <c r="F757">
-        <v>11234.54</v>
+        <v>11234.64</v>
       </c>
       <c r="G757">
-        <v>99.22313976595275</v>
+        <v>99.22402296312653</v>
       </c>
       <c r="H757">
         <v>262.89</v>
@@ -85802,10 +85802,10 @@
         <v>33.012</v>
       </c>
       <c r="R757">
-        <v>1058.55971</v>
+        <v>1058.57025</v>
       </c>
       <c r="S757">
-        <v>9.349169441377787</v>
+        <v>9.349262530359903</v>
       </c>
       <c r="T757">
         <v>1337.55995</v>
@@ -85844,7 +85844,7 @@
         <v>0</v>
       </c>
       <c r="AF757">
-        <v>1022.66736</v>
+        <v>1022.68062</v>
       </c>
       <c r="AG757">
         <v>0</v>
@@ -85853,7 +85853,7 @@
         <v>3</v>
       </c>
       <c r="AI757">
-        <v>3175.67913</v>
+        <v>3175.71075</v>
       </c>
     </row>
     <row r="758">
@@ -85879,10 +85879,10 @@
         <v>67.94366666666666</v>
       </c>
       <c r="F758">
-        <v>5114.66</v>
+        <v>5114.72</v>
       </c>
       <c r="G758">
-        <v>75.27795085144066</v>
+        <v>75.27883393595677</v>
       </c>
       <c r="H758">
         <v>98.04000000000001</v>
@@ -85915,10 +85915,10 @@
         <v>34.92</v>
       </c>
       <c r="R758">
-        <v>543.1098</v>
+        <v>543.1134</v>
       </c>
       <c r="S758">
-        <v>7.993530915317101</v>
+        <v>7.993583900388067</v>
       </c>
       <c r="T758">
         <v>672.52002</v>
@@ -85957,7 +85957,7 @@
         <v>0</v>
       </c>
       <c r="AF758">
-        <v>467.8592</v>
+        <v>467.8632</v>
       </c>
       <c r="AG758">
         <v>0</v>
@@ -85966,7 +85966,7 @@
         <v>3</v>
       </c>
       <c r="AI758">
-        <v>1629.3294</v>
+        <v>1629.3402</v>
       </c>
     </row>
     <row r="759">
@@ -85992,10 +85992,10 @@
         <v>113.225</v>
       </c>
       <c r="F759">
-        <v>10117.27</v>
+        <v>10117.33</v>
       </c>
       <c r="G759">
-        <v>89.35544270258336</v>
+        <v>89.35597262088761</v>
       </c>
       <c r="H759">
         <v>330.05</v>
@@ -86028,10 +86028,10 @@
         <v>34.992</v>
       </c>
       <c r="R759">
-        <v>798.78984</v>
+        <v>798.79537</v>
       </c>
       <c r="S759">
-        <v>7.054889291234269</v>
+        <v>7.054938132037978</v>
       </c>
       <c r="T759">
         <v>1423.44002</v>
@@ -86070,7 +86070,7 @@
         <v>0</v>
       </c>
       <c r="AF759">
-        <v>955.2088000000001</v>
+        <v>955.2152</v>
       </c>
       <c r="AG759">
         <v>0</v>
@@ -86079,7 +86079,7 @@
         <v>3</v>
       </c>
       <c r="AI759">
-        <v>2396.36952</v>
+        <v>2396.38611</v>
       </c>
     </row>
     <row r="760">
@@ -86105,10 +86105,10 @@
         <v>70.4965</v>
       </c>
       <c r="F760">
-        <v>8310.07</v>
+        <v>8310.17</v>
       </c>
       <c r="G760">
-        <v>117.8791854914783</v>
+        <v>117.8806040016171</v>
       </c>
       <c r="H760">
         <v>116.63</v>
@@ -86141,10 +86141,10 @@
         <v>36</v>
       </c>
       <c r="R760">
-        <v>787.8290400000001</v>
+        <v>787.8429</v>
       </c>
       <c r="S760">
-        <v>11.1754348088203</v>
+        <v>11.17563141432553</v>
       </c>
       <c r="T760">
         <v>863.37999</v>
@@ -86183,7 +86183,7 @@
         <v>0</v>
       </c>
       <c r="AF760">
-        <v>1937.816</v>
+        <v>1937.848</v>
       </c>
       <c r="AG760">
         <v>0</v>
@@ -86192,7 +86192,2832 @@
         <v>3</v>
       </c>
       <c r="AI760">
-        <v>2363.48712</v>
+        <v>2363.5287</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B761" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E761">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F761">
+        <v>7318.84</v>
+      </c>
+      <c r="G761">
+        <v>67.29080918070569</v>
+      </c>
+      <c r="H761">
+        <v>29.18</v>
+      </c>
+      <c r="I761">
+        <v>0</v>
+      </c>
+      <c r="J761">
+        <v>0</v>
+      </c>
+      <c r="K761">
+        <v>0.2682864787169814</v>
+      </c>
+      <c r="L761">
+        <v>0</v>
+      </c>
+      <c r="M761">
+        <v>1</v>
+      </c>
+      <c r="N761">
+        <v>0</v>
+      </c>
+      <c r="O761">
+        <v>25.58876</v>
+      </c>
+      <c r="P761">
+        <v>71.07988888888889</v>
+      </c>
+      <c r="Q761">
+        <v>36</v>
+      </c>
+      <c r="R761">
+        <v>849.05231</v>
+      </c>
+      <c r="S761">
+        <v>7.806348680480428</v>
+      </c>
+      <c r="T761">
+        <v>903.3599800000001</v>
+      </c>
+      <c r="U761">
+        <v>26</v>
+      </c>
+      <c r="V761">
+        <v>22</v>
+      </c>
+      <c r="W761">
+        <v>48</v>
+      </c>
+      <c r="X761">
+        <v>121</v>
+      </c>
+      <c r="Y761">
+        <v>26</v>
+      </c>
+      <c r="Z761">
+        <v>109</v>
+      </c>
+      <c r="AA761">
+        <v>22</v>
+      </c>
+      <c r="AB761">
+        <v>57</v>
+      </c>
+      <c r="AC761">
+        <v>4.34271</v>
+      </c>
+      <c r="AD761">
+        <v>-2.12432</v>
+      </c>
+      <c r="AE761">
+        <v>0</v>
+      </c>
+      <c r="AF761">
+        <v>1732.338</v>
+      </c>
+      <c r="AG761">
+        <v>0</v>
+      </c>
+      <c r="AH761">
+        <v>3</v>
+      </c>
+      <c r="AI761">
+        <v>2547.15693</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B762" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E762">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F762">
+        <v>7032.9</v>
+      </c>
+      <c r="G762">
+        <v>64.66182234985121</v>
+      </c>
+      <c r="H762">
+        <v>65.52</v>
+      </c>
+      <c r="I762">
+        <v>0</v>
+      </c>
+      <c r="J762">
+        <v>0</v>
+      </c>
+      <c r="K762">
+        <v>0.6024033613960459</v>
+      </c>
+      <c r="L762">
+        <v>0</v>
+      </c>
+      <c r="M762">
+        <v>0</v>
+      </c>
+      <c r="N762">
+        <v>0</v>
+      </c>
+      <c r="O762">
+        <v>24.24476</v>
+      </c>
+      <c r="P762">
+        <v>74.91274255345446</v>
+      </c>
+      <c r="Q762">
+        <v>32.364</v>
+      </c>
+      <c r="R762">
+        <v>747.36132</v>
+      </c>
+      <c r="S762">
+        <v>6.871382346541299</v>
+      </c>
+      <c r="T762">
+        <v>718.58</v>
+      </c>
+      <c r="U762">
+        <v>20</v>
+      </c>
+      <c r="V762">
+        <v>13</v>
+      </c>
+      <c r="W762">
+        <v>33</v>
+      </c>
+      <c r="X762">
+        <v>84</v>
+      </c>
+      <c r="Y762">
+        <v>20</v>
+      </c>
+      <c r="Z762">
+        <v>70</v>
+      </c>
+      <c r="AA762">
+        <v>13</v>
+      </c>
+      <c r="AB762">
+        <v>37</v>
+      </c>
+      <c r="AC762">
+        <v>4.12516</v>
+      </c>
+      <c r="AD762">
+        <v>-2.17103</v>
+      </c>
+      <c r="AE762">
+        <v>0</v>
+      </c>
+      <c r="AF762">
+        <v>565.0519</v>
+      </c>
+      <c r="AG762">
+        <v>0</v>
+      </c>
+      <c r="AH762">
+        <v>3</v>
+      </c>
+      <c r="AI762">
+        <v>2242.08396</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B763" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E763">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F763">
+        <v>8279.41</v>
+      </c>
+      <c r="G763">
+        <v>76.122472746887</v>
+      </c>
+      <c r="H763">
+        <v>64.83</v>
+      </c>
+      <c r="I763">
+        <v>0</v>
+      </c>
+      <c r="J763">
+        <v>0</v>
+      </c>
+      <c r="K763">
+        <v>0.5960593699527725</v>
+      </c>
+      <c r="L763">
+        <v>0</v>
+      </c>
+      <c r="M763">
+        <v>0</v>
+      </c>
+      <c r="N763">
+        <v>0</v>
+      </c>
+      <c r="O763">
+        <v>23.81626</v>
+      </c>
+      <c r="P763">
+        <v>66.15627777777777</v>
+      </c>
+      <c r="Q763">
+        <v>36</v>
+      </c>
+      <c r="R763">
+        <v>781.30817</v>
+      </c>
+      <c r="S763">
+        <v>7.183496152231277</v>
+      </c>
+      <c r="T763">
+        <v>940.9100099999999</v>
+      </c>
+      <c r="U763">
+        <v>21</v>
+      </c>
+      <c r="V763">
+        <v>30</v>
+      </c>
+      <c r="W763">
+        <v>51</v>
+      </c>
+      <c r="X763">
+        <v>127</v>
+      </c>
+      <c r="Y763">
+        <v>21</v>
+      </c>
+      <c r="Z763">
+        <v>111</v>
+      </c>
+      <c r="AA763">
+        <v>30</v>
+      </c>
+      <c r="AB763">
+        <v>53</v>
+      </c>
+      <c r="AC763">
+        <v>4.37552</v>
+      </c>
+      <c r="AD763">
+        <v>-2.42966</v>
+      </c>
+      <c r="AE763">
+        <v>0</v>
+      </c>
+      <c r="AF763">
+        <v>1954.78</v>
+      </c>
+      <c r="AG763">
+        <v>0</v>
+      </c>
+      <c r="AH763">
+        <v>3</v>
+      </c>
+      <c r="AI763">
+        <v>2343.92451</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B764" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E764">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F764">
+        <v>7679.98</v>
+      </c>
+      <c r="G764">
+        <v>70.61119913697199</v>
+      </c>
+      <c r="H764">
+        <v>65.08</v>
+      </c>
+      <c r="I764">
+        <v>0</v>
+      </c>
+      <c r="J764">
+        <v>0</v>
+      </c>
+      <c r="K764">
+        <v>0.598357917577147</v>
+      </c>
+      <c r="L764">
+        <v>0</v>
+      </c>
+      <c r="M764">
+        <v>0</v>
+      </c>
+      <c r="N764">
+        <v>0</v>
+      </c>
+      <c r="O764">
+        <v>24.93194</v>
+      </c>
+      <c r="P764">
+        <v>76.95043209876545</v>
+      </c>
+      <c r="Q764">
+        <v>32.4</v>
+      </c>
+      <c r="R764">
+        <v>930.8503499999999</v>
+      </c>
+      <c r="S764">
+        <v>8.55841544256236</v>
+      </c>
+      <c r="T764">
+        <v>783.96998</v>
+      </c>
+      <c r="U764">
+        <v>28</v>
+      </c>
+      <c r="V764">
+        <v>26</v>
+      </c>
+      <c r="W764">
+        <v>54</v>
+      </c>
+      <c r="X764">
+        <v>109</v>
+      </c>
+      <c r="Y764">
+        <v>28</v>
+      </c>
+      <c r="Z764">
+        <v>79</v>
+      </c>
+      <c r="AA764">
+        <v>26</v>
+      </c>
+      <c r="AB764">
+        <v>18</v>
+      </c>
+      <c r="AC764">
+        <v>4.12032</v>
+      </c>
+      <c r="AD764">
+        <v>-2.39904</v>
+      </c>
+      <c r="AE764">
+        <v>0</v>
+      </c>
+      <c r="AF764">
+        <v>629.1732999999999</v>
+      </c>
+      <c r="AG764">
+        <v>0</v>
+      </c>
+      <c r="AH764">
+        <v>3</v>
+      </c>
+      <c r="AI764">
+        <v>2792.55105</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B765" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E765">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F765">
+        <v>6686.42</v>
+      </c>
+      <c r="G765">
+        <v>61.47621922627822</v>
+      </c>
+      <c r="H765">
+        <v>72.89</v>
+      </c>
+      <c r="I765">
+        <v>0</v>
+      </c>
+      <c r="J765">
+        <v>0</v>
+      </c>
+      <c r="K765">
+        <v>0.6701645453626036</v>
+      </c>
+      <c r="L765">
+        <v>0</v>
+      </c>
+      <c r="M765">
+        <v>2</v>
+      </c>
+      <c r="N765">
+        <v>0</v>
+      </c>
+      <c r="O765">
+        <v>26.10517</v>
+      </c>
+      <c r="P765">
+        <v>76.81606049905838</v>
+      </c>
+      <c r="Q765">
+        <v>33.984</v>
+      </c>
+      <c r="R765">
+        <v>889.52423</v>
+      </c>
+      <c r="S765">
+        <v>8.178455222759913</v>
+      </c>
+      <c r="T765">
+        <v>606.26</v>
+      </c>
+      <c r="U765">
+        <v>16</v>
+      </c>
+      <c r="V765">
+        <v>18</v>
+      </c>
+      <c r="W765">
+        <v>34</v>
+      </c>
+      <c r="X765">
+        <v>75</v>
+      </c>
+      <c r="Y765">
+        <v>16</v>
+      </c>
+      <c r="Z765">
+        <v>87</v>
+      </c>
+      <c r="AA765">
+        <v>18</v>
+      </c>
+      <c r="AB765">
+        <v>29</v>
+      </c>
+      <c r="AC765">
+        <v>4.02232</v>
+      </c>
+      <c r="AD765">
+        <v>-2.49496</v>
+      </c>
+      <c r="AE765">
+        <v>0</v>
+      </c>
+      <c r="AF765">
+        <v>625.0384</v>
+      </c>
+      <c r="AG765">
+        <v>0</v>
+      </c>
+      <c r="AH765">
+        <v>3</v>
+      </c>
+      <c r="AI765">
+        <v>2668.57269</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B766" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E766">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F766">
+        <v>7524.65</v>
+      </c>
+      <c r="G766">
+        <v>69.18306552699568</v>
+      </c>
+      <c r="H766">
+        <v>188.68</v>
+      </c>
+      <c r="I766">
+        <v>0</v>
+      </c>
+      <c r="J766">
+        <v>0</v>
+      </c>
+      <c r="K766">
+        <v>1.734759863067856</v>
+      </c>
+      <c r="L766">
+        <v>0</v>
+      </c>
+      <c r="M766">
+        <v>5</v>
+      </c>
+      <c r="N766">
+        <v>0</v>
+      </c>
+      <c r="O766">
+        <v>28.63343</v>
+      </c>
+      <c r="P766">
+        <v>80.50334570400361</v>
+      </c>
+      <c r="Q766">
+        <v>35.568</v>
+      </c>
+      <c r="R766">
+        <v>757.71576</v>
+      </c>
+      <c r="S766">
+        <v>6.966583040396209</v>
+      </c>
+      <c r="T766">
+        <v>827.38999</v>
+      </c>
+      <c r="U766">
+        <v>29</v>
+      </c>
+      <c r="V766">
+        <v>22</v>
+      </c>
+      <c r="W766">
+        <v>51</v>
+      </c>
+      <c r="X766">
+        <v>91</v>
+      </c>
+      <c r="Y766">
+        <v>29</v>
+      </c>
+      <c r="Z766">
+        <v>73</v>
+      </c>
+      <c r="AA766">
+        <v>22</v>
+      </c>
+      <c r="AB766">
+        <v>24</v>
+      </c>
+      <c r="AC766">
+        <v>4.5411</v>
+      </c>
+      <c r="AD766">
+        <v>-1.83023</v>
+      </c>
+      <c r="AE766">
+        <v>0</v>
+      </c>
+      <c r="AF766">
+        <v>707.9608000000001</v>
+      </c>
+      <c r="AG766">
+        <v>0</v>
+      </c>
+      <c r="AH766">
+        <v>3</v>
+      </c>
+      <c r="AI766">
+        <v>2273.14728</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B767" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E767">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F767">
+        <v>8296.060000000001</v>
+      </c>
+      <c r="G767">
+        <v>76.27555601867036</v>
+      </c>
+      <c r="H767">
+        <v>69.87</v>
+      </c>
+      <c r="I767">
+        <v>0</v>
+      </c>
+      <c r="J767">
+        <v>0</v>
+      </c>
+      <c r="K767">
+        <v>0.6423980900601607</v>
+      </c>
+      <c r="L767">
+        <v>0</v>
+      </c>
+      <c r="M767">
+        <v>0</v>
+      </c>
+      <c r="N767">
+        <v>0</v>
+      </c>
+      <c r="O767">
+        <v>24.36051</v>
+      </c>
+      <c r="P767">
+        <v>67.66808333333334</v>
+      </c>
+      <c r="Q767">
+        <v>36</v>
+      </c>
+      <c r="R767">
+        <v>871.19006</v>
+      </c>
+      <c r="S767">
+        <v>8.009887371166407</v>
+      </c>
+      <c r="T767">
+        <v>781.3399900000001</v>
+      </c>
+      <c r="U767">
+        <v>17</v>
+      </c>
+      <c r="V767">
+        <v>17</v>
+      </c>
+      <c r="W767">
+        <v>34</v>
+      </c>
+      <c r="X767">
+        <v>98</v>
+      </c>
+      <c r="Y767">
+        <v>17</v>
+      </c>
+      <c r="Z767">
+        <v>96</v>
+      </c>
+      <c r="AA767">
+        <v>17</v>
+      </c>
+      <c r="AB767">
+        <v>49</v>
+      </c>
+      <c r="AC767">
+        <v>3.89178</v>
+      </c>
+      <c r="AD767">
+        <v>-2.26845</v>
+      </c>
+      <c r="AE767">
+        <v>0</v>
+      </c>
+      <c r="AF767">
+        <v>1919.196</v>
+      </c>
+      <c r="AG767">
+        <v>0</v>
+      </c>
+      <c r="AH767">
+        <v>3</v>
+      </c>
+      <c r="AI767">
+        <v>2613.57018</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B768" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E768">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F768">
+        <v>8034.78</v>
+      </c>
+      <c r="G768">
+        <v>73.87329792548415</v>
+      </c>
+      <c r="H768">
+        <v>192.21</v>
+      </c>
+      <c r="I768">
+        <v>0</v>
+      </c>
+      <c r="J768">
+        <v>0</v>
+      </c>
+      <c r="K768">
+        <v>1.767215355524023</v>
+      </c>
+      <c r="L768">
+        <v>0</v>
+      </c>
+      <c r="M768">
+        <v>1</v>
+      </c>
+      <c r="N768">
+        <v>0</v>
+      </c>
+      <c r="O768">
+        <v>28.20667</v>
+      </c>
+      <c r="P768">
+        <v>78.35186111111111</v>
+      </c>
+      <c r="Q768">
+        <v>36</v>
+      </c>
+      <c r="R768">
+        <v>890.1092199999999</v>
+      </c>
+      <c r="S768">
+        <v>8.183833732259043</v>
+      </c>
+      <c r="T768">
+        <v>1078.08001</v>
+      </c>
+      <c r="U768">
+        <v>33</v>
+      </c>
+      <c r="V768">
+        <v>38</v>
+      </c>
+      <c r="W768">
+        <v>71</v>
+      </c>
+      <c r="X768">
+        <v>111</v>
+      </c>
+      <c r="Y768">
+        <v>33</v>
+      </c>
+      <c r="Z768">
+        <v>108</v>
+      </c>
+      <c r="AA768">
+        <v>38</v>
+      </c>
+      <c r="AB768">
+        <v>35</v>
+      </c>
+      <c r="AC768">
+        <v>4.44006</v>
+      </c>
+      <c r="AD768">
+        <v>-2.77074</v>
+      </c>
+      <c r="AE768">
+        <v>0</v>
+      </c>
+      <c r="AF768">
+        <v>665.7546</v>
+      </c>
+      <c r="AG768">
+        <v>0</v>
+      </c>
+      <c r="AH768">
+        <v>3</v>
+      </c>
+      <c r="AI768">
+        <v>2670.32766</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B769" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E769">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F769">
+        <v>6573.449999999999</v>
+      </c>
+      <c r="G769">
+        <v>60.43755152577591</v>
+      </c>
+      <c r="H769">
+        <v>77.36000000000001</v>
+      </c>
+      <c r="I769">
+        <v>0</v>
+      </c>
+      <c r="J769">
+        <v>0</v>
+      </c>
+      <c r="K769">
+        <v>0.7112625768864183</v>
+      </c>
+      <c r="L769">
+        <v>0</v>
+      </c>
+      <c r="M769">
+        <v>0</v>
+      </c>
+      <c r="N769">
+        <v>0</v>
+      </c>
+      <c r="O769">
+        <v>25.15747</v>
+      </c>
+      <c r="P769">
+        <v>78.60726784151981</v>
+      </c>
+      <c r="Q769">
+        <v>32.004</v>
+      </c>
+      <c r="R769">
+        <v>814.15786</v>
+      </c>
+      <c r="S769">
+        <v>7.485522459875021</v>
+      </c>
+      <c r="T769">
+        <v>694.93998</v>
+      </c>
+      <c r="U769">
+        <v>24</v>
+      </c>
+      <c r="V769">
+        <v>27</v>
+      </c>
+      <c r="W769">
+        <v>51</v>
+      </c>
+      <c r="X769">
+        <v>90</v>
+      </c>
+      <c r="Y769">
+        <v>24</v>
+      </c>
+      <c r="Z769">
+        <v>87</v>
+      </c>
+      <c r="AA769">
+        <v>27</v>
+      </c>
+      <c r="AB769">
+        <v>32</v>
+      </c>
+      <c r="AC769">
+        <v>4.01364</v>
+      </c>
+      <c r="AD769">
+        <v>-1.88018</v>
+      </c>
+      <c r="AE769">
+        <v>0</v>
+      </c>
+      <c r="AF769">
+        <v>462.3924000000001</v>
+      </c>
+      <c r="AG769">
+        <v>0</v>
+      </c>
+      <c r="AH769">
+        <v>3</v>
+      </c>
+      <c r="AI769">
+        <v>2442.47358</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B770" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E770">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F770">
+        <v>7617.879999999999</v>
+      </c>
+      <c r="G770">
+        <v>70.04023990707738</v>
+      </c>
+      <c r="H770">
+        <v>202.99</v>
+      </c>
+      <c r="I770">
+        <v>0</v>
+      </c>
+      <c r="J770">
+        <v>0</v>
+      </c>
+      <c r="K770">
+        <v>1.866328729087048</v>
+      </c>
+      <c r="L770">
+        <v>0</v>
+      </c>
+      <c r="M770">
+        <v>2</v>
+      </c>
+      <c r="N770">
+        <v>0</v>
+      </c>
+      <c r="O770">
+        <v>28.01666</v>
+      </c>
+      <c r="P770">
+        <v>82.79154846335697</v>
+      </c>
+      <c r="Q770">
+        <v>33.84</v>
+      </c>
+      <c r="R770">
+        <v>814.71582</v>
+      </c>
+      <c r="S770">
+        <v>7.490652450405005</v>
+      </c>
+      <c r="T770">
+        <v>924.36001</v>
+      </c>
+      <c r="U770">
+        <v>38</v>
+      </c>
+      <c r="V770">
+        <v>36</v>
+      </c>
+      <c r="W770">
+        <v>74</v>
+      </c>
+      <c r="X770">
+        <v>123</v>
+      </c>
+      <c r="Y770">
+        <v>38</v>
+      </c>
+      <c r="Z770">
+        <v>111</v>
+      </c>
+      <c r="AA770">
+        <v>36</v>
+      </c>
+      <c r="AB770">
+        <v>48</v>
+      </c>
+      <c r="AC770">
+        <v>4.55306</v>
+      </c>
+      <c r="AD770">
+        <v>-1.83618</v>
+      </c>
+      <c r="AE770">
+        <v>0</v>
+      </c>
+      <c r="AF770">
+        <v>634.0684</v>
+      </c>
+      <c r="AG770">
+        <v>0</v>
+      </c>
+      <c r="AH770">
+        <v>3</v>
+      </c>
+      <c r="AI770">
+        <v>2444.14746</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B771" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E771">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F771">
+        <v>6946.619999999999</v>
+      </c>
+      <c r="G771">
+        <v>63.86854759372711</v>
+      </c>
+      <c r="H771">
+        <v>29.86</v>
+      </c>
+      <c r="I771">
+        <v>0</v>
+      </c>
+      <c r="J771">
+        <v>0</v>
+      </c>
+      <c r="K771">
+        <v>0.2745385282552798</v>
+      </c>
+      <c r="L771">
+        <v>0</v>
+      </c>
+      <c r="M771">
+        <v>0</v>
+      </c>
+      <c r="N771">
+        <v>0</v>
+      </c>
+      <c r="O771">
+        <v>22.90865</v>
+      </c>
+      <c r="P771">
+        <v>67.98625949667617</v>
+      </c>
+      <c r="Q771">
+        <v>33.696</v>
+      </c>
+      <c r="R771">
+        <v>786.56354</v>
+      </c>
+      <c r="S771">
+        <v>7.231815025146111</v>
+      </c>
+      <c r="T771">
+        <v>688.54</v>
+      </c>
+      <c r="U771">
+        <v>27</v>
+      </c>
+      <c r="V771">
+        <v>23</v>
+      </c>
+      <c r="W771">
+        <v>50</v>
+      </c>
+      <c r="X771">
+        <v>101</v>
+      </c>
+      <c r="Y771">
+        <v>27</v>
+      </c>
+      <c r="Z771">
+        <v>92</v>
+      </c>
+      <c r="AA771">
+        <v>23</v>
+      </c>
+      <c r="AB771">
+        <v>28</v>
+      </c>
+      <c r="AC771">
+        <v>4.10928</v>
+      </c>
+      <c r="AD771">
+        <v>-2.50047</v>
+      </c>
+      <c r="AE771">
+        <v>0</v>
+      </c>
+      <c r="AF771">
+        <v>649.8856000000001</v>
+      </c>
+      <c r="AG771">
+        <v>0</v>
+      </c>
+      <c r="AH771">
+        <v>3</v>
+      </c>
+      <c r="AI771">
+        <v>2359.69062</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B772" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E772">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F772">
+        <v>7358.84</v>
+      </c>
+      <c r="G772">
+        <v>67.6585768006056</v>
+      </c>
+      <c r="H772">
+        <v>110.61</v>
+      </c>
+      <c r="I772">
+        <v>0</v>
+      </c>
+      <c r="J772">
+        <v>0</v>
+      </c>
+      <c r="K772">
+        <v>1.016969410928215</v>
+      </c>
+      <c r="L772">
+        <v>0</v>
+      </c>
+      <c r="M772">
+        <v>2</v>
+      </c>
+      <c r="N772">
+        <v>0</v>
+      </c>
+      <c r="O772">
+        <v>27.60416</v>
+      </c>
+      <c r="P772">
+        <v>76.67822222222223</v>
+      </c>
+      <c r="Q772">
+        <v>36</v>
+      </c>
+      <c r="R772">
+        <v>931.58859</v>
+      </c>
+      <c r="S772">
+        <v>8.565202961755233</v>
+      </c>
+      <c r="T772">
+        <v>747.41998</v>
+      </c>
+      <c r="U772">
+        <v>18</v>
+      </c>
+      <c r="V772">
+        <v>23</v>
+      </c>
+      <c r="W772">
+        <v>41</v>
+      </c>
+      <c r="X772">
+        <v>87</v>
+      </c>
+      <c r="Y772">
+        <v>18</v>
+      </c>
+      <c r="Z772">
+        <v>74</v>
+      </c>
+      <c r="AA772">
+        <v>23</v>
+      </c>
+      <c r="AB772">
+        <v>39</v>
+      </c>
+      <c r="AC772">
+        <v>3.99711</v>
+      </c>
+      <c r="AD772">
+        <v>-2.4602</v>
+      </c>
+      <c r="AE772">
+        <v>0</v>
+      </c>
+      <c r="AF772">
+        <v>1706.154</v>
+      </c>
+      <c r="AG772">
+        <v>0</v>
+      </c>
+      <c r="AH772">
+        <v>3</v>
+      </c>
+      <c r="AI772">
+        <v>2794.76577</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B773" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E773">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F773">
+        <v>6445.15</v>
+      </c>
+      <c r="G773">
+        <v>59.25793688494696</v>
+      </c>
+      <c r="H773">
+        <v>165.19</v>
+      </c>
+      <c r="I773">
+        <v>0</v>
+      </c>
+      <c r="J773">
+        <v>0</v>
+      </c>
+      <c r="K773">
+        <v>1.518788328281637</v>
+      </c>
+      <c r="L773">
+        <v>0</v>
+      </c>
+      <c r="M773">
+        <v>5</v>
+      </c>
+      <c r="N773">
+        <v>0</v>
+      </c>
+      <c r="O773">
+        <v>26.96002</v>
+      </c>
+      <c r="P773">
+        <v>77.04623914037495</v>
+      </c>
+      <c r="Q773">
+        <v>34.992</v>
+      </c>
+      <c r="R773">
+        <v>631.40715</v>
+      </c>
+      <c r="S773">
+        <v>5.805277618582072</v>
+      </c>
+      <c r="T773">
+        <v>684.11001</v>
+      </c>
+      <c r="U773">
+        <v>22</v>
+      </c>
+      <c r="V773">
+        <v>29</v>
+      </c>
+      <c r="W773">
+        <v>51</v>
+      </c>
+      <c r="X773">
+        <v>79</v>
+      </c>
+      <c r="Y773">
+        <v>22</v>
+      </c>
+      <c r="Z773">
+        <v>84</v>
+      </c>
+      <c r="AA773">
+        <v>29</v>
+      </c>
+      <c r="AB773">
+        <v>21</v>
+      </c>
+      <c r="AC773">
+        <v>4.55315</v>
+      </c>
+      <c r="AD773">
+        <v>-2.47202</v>
+      </c>
+      <c r="AE773">
+        <v>0</v>
+      </c>
+      <c r="AF773">
+        <v>516.67269</v>
+      </c>
+      <c r="AG773">
+        <v>0</v>
+      </c>
+      <c r="AH773">
+        <v>3</v>
+      </c>
+      <c r="AI773">
+        <v>1894.22145</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B774" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Sesión 42 | Trabajo Especial</t>
+        </is>
+      </c>
+      <c r="E774">
+        <v>126.9276666666667</v>
+      </c>
+      <c r="F774">
+        <v>7425.18</v>
+      </c>
+      <c r="G774">
+        <v>58.49930275248633</v>
+      </c>
+      <c r="H774">
+        <v>136.17</v>
+      </c>
+      <c r="I774">
+        <v>0</v>
+      </c>
+      <c r="J774">
+        <v>0</v>
+      </c>
+      <c r="K774">
+        <v>1.072815750703157</v>
+      </c>
+      <c r="L774">
+        <v>0</v>
+      </c>
+      <c r="M774">
+        <v>3</v>
+      </c>
+      <c r="N774">
+        <v>0</v>
+      </c>
+      <c r="O774">
+        <v>25.30575</v>
+      </c>
+      <c r="P774">
+        <v>72.46778350515464</v>
+      </c>
+      <c r="Q774">
+        <v>34.92</v>
+      </c>
+      <c r="R774">
+        <v>799.74793</v>
+      </c>
+      <c r="S774">
+        <v>6.300816449263754</v>
+      </c>
+      <c r="T774">
+        <v>686.6299799999999</v>
+      </c>
+      <c r="U774">
+        <v>32</v>
+      </c>
+      <c r="V774">
+        <v>18</v>
+      </c>
+      <c r="W774">
+        <v>50</v>
+      </c>
+      <c r="X774">
+        <v>90</v>
+      </c>
+      <c r="Y774">
+        <v>32</v>
+      </c>
+      <c r="Z774">
+        <v>74</v>
+      </c>
+      <c r="AA774">
+        <v>18</v>
+      </c>
+      <c r="AB774">
+        <v>15</v>
+      </c>
+      <c r="AC774">
+        <v>4.42305</v>
+      </c>
+      <c r="AD774">
+        <v>-2.28933</v>
+      </c>
+      <c r="AE774">
+        <v>0</v>
+      </c>
+      <c r="AF774">
+        <v>674.0672</v>
+      </c>
+      <c r="AG774">
+        <v>0</v>
+      </c>
+      <c r="AH774">
+        <v>3</v>
+      </c>
+      <c r="AI774">
+        <v>2399.24379</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B775" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E775">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F775">
+        <v>7039.77</v>
+      </c>
+      <c r="G775">
+        <v>64.72498643856902</v>
+      </c>
+      <c r="H775">
+        <v>68.12</v>
+      </c>
+      <c r="I775">
+        <v>0</v>
+      </c>
+      <c r="J775">
+        <v>0</v>
+      </c>
+      <c r="K775">
+        <v>0.6263082566895398</v>
+      </c>
+      <c r="L775">
+        <v>0</v>
+      </c>
+      <c r="M775">
+        <v>2</v>
+      </c>
+      <c r="N775">
+        <v>0</v>
+      </c>
+      <c r="O775">
+        <v>26.05668</v>
+      </c>
+      <c r="P775">
+        <v>74.46467764060357</v>
+      </c>
+      <c r="Q775">
+        <v>34.992</v>
+      </c>
+      <c r="R775">
+        <v>671.62211</v>
+      </c>
+      <c r="S775">
+        <v>6.175021621671321</v>
+      </c>
+      <c r="T775">
+        <v>827.5</v>
+      </c>
+      <c r="U775">
+        <v>27</v>
+      </c>
+      <c r="V775">
+        <v>28</v>
+      </c>
+      <c r="W775">
+        <v>55</v>
+      </c>
+      <c r="X775">
+        <v>119</v>
+      </c>
+      <c r="Y775">
+        <v>27</v>
+      </c>
+      <c r="Z775">
+        <v>97</v>
+      </c>
+      <c r="AA775">
+        <v>28</v>
+      </c>
+      <c r="AB775">
+        <v>68</v>
+      </c>
+      <c r="AC775">
+        <v>4.10382</v>
+      </c>
+      <c r="AD775">
+        <v>-2.46489</v>
+      </c>
+      <c r="AE775">
+        <v>0</v>
+      </c>
+      <c r="AF775">
+        <v>594.99988</v>
+      </c>
+      <c r="AG775">
+        <v>0</v>
+      </c>
+      <c r="AH775">
+        <v>3</v>
+      </c>
+      <c r="AI775">
+        <v>2014.86633</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B776" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E776">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F776">
+        <v>7697.5</v>
+      </c>
+      <c r="G776">
+        <v>70.77228135448814</v>
+      </c>
+      <c r="H776">
+        <v>54.61</v>
+      </c>
+      <c r="I776">
+        <v>0</v>
+      </c>
+      <c r="J776">
+        <v>0</v>
+      </c>
+      <c r="K776">
+        <v>0.5020947430683466</v>
+      </c>
+      <c r="L776">
+        <v>0</v>
+      </c>
+      <c r="M776">
+        <v>0</v>
+      </c>
+      <c r="N776">
+        <v>0</v>
+      </c>
+      <c r="O776">
+        <v>24.53683</v>
+      </c>
+      <c r="P776">
+        <v>68.1578611111111</v>
+      </c>
+      <c r="Q776">
+        <v>36</v>
+      </c>
+      <c r="R776">
+        <v>899.72492</v>
+      </c>
+      <c r="S776">
+        <v>8.272242309825831</v>
+      </c>
+      <c r="T776">
+        <v>809.26003</v>
+      </c>
+      <c r="U776">
+        <v>22</v>
+      </c>
+      <c r="V776">
+        <v>28</v>
+      </c>
+      <c r="W776">
+        <v>50</v>
+      </c>
+      <c r="X776">
+        <v>93</v>
+      </c>
+      <c r="Y776">
+        <v>22</v>
+      </c>
+      <c r="Z776">
+        <v>83</v>
+      </c>
+      <c r="AA776">
+        <v>28</v>
+      </c>
+      <c r="AB776">
+        <v>33</v>
+      </c>
+      <c r="AC776">
+        <v>3.9333</v>
+      </c>
+      <c r="AD776">
+        <v>-2.14844</v>
+      </c>
+      <c r="AE776">
+        <v>0</v>
+      </c>
+      <c r="AF776">
+        <v>1803.476</v>
+      </c>
+      <c r="AG776">
+        <v>0</v>
+      </c>
+      <c r="AH776">
+        <v>3</v>
+      </c>
+      <c r="AI776">
+        <v>2699.17476</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B777" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E777">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F777">
+        <v>6973.5</v>
+      </c>
+      <c r="G777">
+        <v>64.11568743429986</v>
+      </c>
+      <c r="H777">
+        <v>63.22</v>
+      </c>
+      <c r="I777">
+        <v>0</v>
+      </c>
+      <c r="J777">
+        <v>0</v>
+      </c>
+      <c r="K777">
+        <v>0.5812567232518013</v>
+      </c>
+      <c r="L777">
+        <v>0</v>
+      </c>
+      <c r="M777">
+        <v>1</v>
+      </c>
+      <c r="N777">
+        <v>0</v>
+      </c>
+      <c r="O777">
+        <v>25.57689</v>
+      </c>
+      <c r="P777">
+        <v>75.26156426553672</v>
+      </c>
+      <c r="Q777">
+        <v>33.984</v>
+      </c>
+      <c r="R777">
+        <v>765.57813</v>
+      </c>
+      <c r="S777">
+        <v>7.038871167938019</v>
+      </c>
+      <c r="T777">
+        <v>723.81999</v>
+      </c>
+      <c r="U777">
+        <v>11</v>
+      </c>
+      <c r="V777">
+        <v>23</v>
+      </c>
+      <c r="W777">
+        <v>34</v>
+      </c>
+      <c r="X777">
+        <v>82</v>
+      </c>
+      <c r="Y777">
+        <v>11</v>
+      </c>
+      <c r="Z777">
+        <v>91</v>
+      </c>
+      <c r="AA777">
+        <v>23</v>
+      </c>
+      <c r="AB777">
+        <v>38</v>
+      </c>
+      <c r="AC777">
+        <v>3.89758</v>
+      </c>
+      <c r="AD777">
+        <v>-2.03744</v>
+      </c>
+      <c r="AE777">
+        <v>0</v>
+      </c>
+      <c r="AF777">
+        <v>649.2</v>
+      </c>
+      <c r="AG777">
+        <v>0</v>
+      </c>
+      <c r="AH777">
+        <v>3</v>
+      </c>
+      <c r="AI777">
+        <v>2296.73439</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B778" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Trabajo Especial</t>
+        </is>
+      </c>
+      <c r="E778">
+        <v>55.13333333333333</v>
+      </c>
+      <c r="F778">
+        <v>4199.830000000001</v>
+      </c>
+      <c r="G778">
+        <v>76.17587666263604</v>
+      </c>
+      <c r="H778">
+        <v>25.98</v>
+      </c>
+      <c r="I778">
+        <v>0</v>
+      </c>
+      <c r="J778">
+        <v>0</v>
+      </c>
+      <c r="K778">
+        <v>0.4712212817412334</v>
+      </c>
+      <c r="L778">
+        <v>0</v>
+      </c>
+      <c r="M778">
+        <v>0</v>
+      </c>
+      <c r="N778">
+        <v>0</v>
+      </c>
+      <c r="O778">
+        <v>21.66302</v>
+      </c>
+      <c r="P778">
+        <v>60.17505555555556</v>
+      </c>
+      <c r="Q778">
+        <v>36</v>
+      </c>
+      <c r="R778">
+        <v>482.39267</v>
+      </c>
+      <c r="S778">
+        <v>8.749564752116083</v>
+      </c>
+      <c r="T778">
+        <v>478.26001</v>
+      </c>
+      <c r="U778">
+        <v>9</v>
+      </c>
+      <c r="V778">
+        <v>15</v>
+      </c>
+      <c r="W778">
+        <v>24</v>
+      </c>
+      <c r="X778">
+        <v>47</v>
+      </c>
+      <c r="Y778">
+        <v>9</v>
+      </c>
+      <c r="Z778">
+        <v>55</v>
+      </c>
+      <c r="AA778">
+        <v>15</v>
+      </c>
+      <c r="AB778">
+        <v>6</v>
+      </c>
+      <c r="AC778">
+        <v>3.74841</v>
+      </c>
+      <c r="AD778">
+        <v>-3.90109</v>
+      </c>
+      <c r="AE778">
+        <v>0</v>
+      </c>
+      <c r="AF778">
+        <v>930.1560000000001</v>
+      </c>
+      <c r="AG778">
+        <v>0</v>
+      </c>
+      <c r="AH778">
+        <v>3</v>
+      </c>
+      <c r="AI778">
+        <v>1447.17801</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B779" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E779">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F779">
+        <v>7577.369999999999</v>
+      </c>
+      <c r="G779">
+        <v>69.66778325002375</v>
+      </c>
+      <c r="H779">
+        <v>35.31</v>
+      </c>
+      <c r="I779">
+        <v>0</v>
+      </c>
+      <c r="J779">
+        <v>0</v>
+      </c>
+      <c r="K779">
+        <v>0.324646866466642</v>
+      </c>
+      <c r="L779">
+        <v>0</v>
+      </c>
+      <c r="M779">
+        <v>0</v>
+      </c>
+      <c r="N779">
+        <v>0</v>
+      </c>
+      <c r="O779">
+        <v>23.32681</v>
+      </c>
+      <c r="P779">
+        <v>66.66326588934614</v>
+      </c>
+      <c r="Q779">
+        <v>34.992</v>
+      </c>
+      <c r="R779">
+        <v>763.44659</v>
+      </c>
+      <c r="S779">
+        <v>7.019273383124983</v>
+      </c>
+      <c r="T779">
+        <v>817.3299999999999</v>
+      </c>
+      <c r="U779">
+        <v>19</v>
+      </c>
+      <c r="V779">
+        <v>29</v>
+      </c>
+      <c r="W779">
+        <v>48</v>
+      </c>
+      <c r="X779">
+        <v>109</v>
+      </c>
+      <c r="Y779">
+        <v>19</v>
+      </c>
+      <c r="Z779">
+        <v>110</v>
+      </c>
+      <c r="AA779">
+        <v>29</v>
+      </c>
+      <c r="AB779">
+        <v>33</v>
+      </c>
+      <c r="AC779">
+        <v>3.7834</v>
+      </c>
+      <c r="AD779">
+        <v>-2.22534</v>
+      </c>
+      <c r="AE779">
+        <v>0</v>
+      </c>
+      <c r="AF779">
+        <v>714.056</v>
+      </c>
+      <c r="AG779">
+        <v>0</v>
+      </c>
+      <c r="AH779">
+        <v>3</v>
+      </c>
+      <c r="AI779">
+        <v>2290.33977</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B780" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E780">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F780">
+        <v>6818.27</v>
+      </c>
+      <c r="G780">
+        <v>62.68847324337329</v>
+      </c>
+      <c r="H780">
+        <v>67.19</v>
+      </c>
+      <c r="I780">
+        <v>0</v>
+      </c>
+      <c r="J780">
+        <v>0</v>
+      </c>
+      <c r="K780">
+        <v>0.617757659526867</v>
+      </c>
+      <c r="L780">
+        <v>0</v>
+      </c>
+      <c r="M780">
+        <v>2</v>
+      </c>
+      <c r="N780">
+        <v>0</v>
+      </c>
+      <c r="O780">
+        <v>28.24684</v>
+      </c>
+      <c r="P780">
+        <v>85.5653701684236</v>
+      </c>
+      <c r="Q780">
+        <v>33.012</v>
+      </c>
+      <c r="R780">
+        <v>731.84006</v>
+      </c>
+      <c r="S780">
+        <v>6.728676925340109</v>
+      </c>
+      <c r="T780">
+        <v>684.40002</v>
+      </c>
+      <c r="U780">
+        <v>20</v>
+      </c>
+      <c r="V780">
+        <v>19</v>
+      </c>
+      <c r="W780">
+        <v>39</v>
+      </c>
+      <c r="X780">
+        <v>105</v>
+      </c>
+      <c r="Y780">
+        <v>20</v>
+      </c>
+      <c r="Z780">
+        <v>86</v>
+      </c>
+      <c r="AA780">
+        <v>19</v>
+      </c>
+      <c r="AB780">
+        <v>42</v>
+      </c>
+      <c r="AC780">
+        <v>3.99279</v>
+      </c>
+      <c r="AD780">
+        <v>-1.76116</v>
+      </c>
+      <c r="AE780">
+        <v>0</v>
+      </c>
+      <c r="AF780">
+        <v>587.6745</v>
+      </c>
+      <c r="AG780">
+        <v>0</v>
+      </c>
+      <c r="AH780">
+        <v>3</v>
+      </c>
+      <c r="AI780">
+        <v>2195.52018</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B781" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E781">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F781">
+        <v>6806.549999999999</v>
+      </c>
+      <c r="G781">
+        <v>62.58071733074262</v>
+      </c>
+      <c r="H781">
+        <v>26.5</v>
+      </c>
+      <c r="I781">
+        <v>0</v>
+      </c>
+      <c r="J781">
+        <v>0</v>
+      </c>
+      <c r="K781">
+        <v>0.2436460481836877</v>
+      </c>
+      <c r="L781">
+        <v>0</v>
+      </c>
+      <c r="M781">
+        <v>0</v>
+      </c>
+      <c r="N781">
+        <v>0</v>
+      </c>
+      <c r="O781">
+        <v>23.01525</v>
+      </c>
+      <c r="P781">
+        <v>71.91366704161982</v>
+      </c>
+      <c r="Q781">
+        <v>32.004</v>
+      </c>
+      <c r="R781">
+        <v>720.69672</v>
+      </c>
+      <c r="S781">
+        <v>6.626222934601723</v>
+      </c>
+      <c r="T781">
+        <v>564.72999</v>
+      </c>
+      <c r="U781">
+        <v>16</v>
+      </c>
+      <c r="V781">
+        <v>15</v>
+      </c>
+      <c r="W781">
+        <v>31</v>
+      </c>
+      <c r="X781">
+        <v>83</v>
+      </c>
+      <c r="Y781">
+        <v>16</v>
+      </c>
+      <c r="Z781">
+        <v>67</v>
+      </c>
+      <c r="AA781">
+        <v>15</v>
+      </c>
+      <c r="AB781">
+        <v>38</v>
+      </c>
+      <c r="AC781">
+        <v>4.1734</v>
+      </c>
+      <c r="AD781">
+        <v>-2.07198</v>
+      </c>
+      <c r="AE781">
+        <v>0</v>
+      </c>
+      <c r="AF781">
+        <v>547.4056</v>
+      </c>
+      <c r="AG781">
+        <v>0</v>
+      </c>
+      <c r="AH781">
+        <v>3</v>
+      </c>
+      <c r="AI781">
+        <v>2162.09016</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B782" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E782">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F782">
+        <v>8414.51</v>
+      </c>
+      <c r="G782">
+        <v>77.36460788309894</v>
+      </c>
+      <c r="H782">
+        <v>40.94</v>
+      </c>
+      <c r="I782">
+        <v>0</v>
+      </c>
+      <c r="J782">
+        <v>0</v>
+      </c>
+      <c r="K782">
+        <v>0.3764101589675537</v>
+      </c>
+      <c r="L782">
+        <v>0</v>
+      </c>
+      <c r="M782">
+        <v>0</v>
+      </c>
+      <c r="N782">
+        <v>0</v>
+      </c>
+      <c r="O782">
+        <v>24.88649</v>
+      </c>
+      <c r="P782">
+        <v>69.12913888888889</v>
+      </c>
+      <c r="Q782">
+        <v>36</v>
+      </c>
+      <c r="R782">
+        <v>955.7971500000001</v>
+      </c>
+      <c r="S782">
+        <v>8.787781074065336</v>
+      </c>
+      <c r="T782">
+        <v>918.66002</v>
+      </c>
+      <c r="U782">
+        <v>32</v>
+      </c>
+      <c r="V782">
+        <v>46</v>
+      </c>
+      <c r="W782">
+        <v>78</v>
+      </c>
+      <c r="X782">
+        <v>121</v>
+      </c>
+      <c r="Y782">
+        <v>32</v>
+      </c>
+      <c r="Z782">
+        <v>138</v>
+      </c>
+      <c r="AA782">
+        <v>46</v>
+      </c>
+      <c r="AB782">
+        <v>39</v>
+      </c>
+      <c r="AC782">
+        <v>4.41309</v>
+      </c>
+      <c r="AD782">
+        <v>-2.30917</v>
+      </c>
+      <c r="AE782">
+        <v>0</v>
+      </c>
+      <c r="AF782">
+        <v>2001.41</v>
+      </c>
+      <c r="AG782">
+        <v>0</v>
+      </c>
+      <c r="AH782">
+        <v>3</v>
+      </c>
+      <c r="AI782">
+        <v>2867.39145</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B783" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E783">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F783">
+        <v>8064.029999999999</v>
+      </c>
+      <c r="G783">
+        <v>74.14222799753595</v>
+      </c>
+      <c r="H783">
+        <v>27.38</v>
+      </c>
+      <c r="I783">
+        <v>0</v>
+      </c>
+      <c r="J783">
+        <v>0</v>
+      </c>
+      <c r="K783">
+        <v>0.2517369358214857</v>
+      </c>
+      <c r="L783">
+        <v>0</v>
+      </c>
+      <c r="M783">
+        <v>0</v>
+      </c>
+      <c r="N783">
+        <v>0</v>
+      </c>
+      <c r="O783">
+        <v>23.50203</v>
+      </c>
+      <c r="P783">
+        <v>65.28341666666667</v>
+      </c>
+      <c r="Q783">
+        <v>36</v>
+      </c>
+      <c r="R783">
+        <v>921.29556</v>
+      </c>
+      <c r="S783">
+        <v>8.470566883138774</v>
+      </c>
+      <c r="T783">
+        <v>825.04002</v>
+      </c>
+      <c r="U783">
+        <v>22</v>
+      </c>
+      <c r="V783">
+        <v>25</v>
+      </c>
+      <c r="W783">
+        <v>47</v>
+      </c>
+      <c r="X783">
+        <v>114</v>
+      </c>
+      <c r="Y783">
+        <v>22</v>
+      </c>
+      <c r="Z783">
+        <v>101</v>
+      </c>
+      <c r="AA783">
+        <v>25</v>
+      </c>
+      <c r="AB783">
+        <v>46</v>
+      </c>
+      <c r="AC783">
+        <v>3.91553</v>
+      </c>
+      <c r="AD783">
+        <v>-2.00661</v>
+      </c>
+      <c r="AE783">
+        <v>0</v>
+      </c>
+      <c r="AF783">
+        <v>1882.86</v>
+      </c>
+      <c r="AG783">
+        <v>0</v>
+      </c>
+      <c r="AH783">
+        <v>3</v>
+      </c>
+      <c r="AI783">
+        <v>2763.88668</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B784" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E784">
+        <v>108.7643333333333</v>
+      </c>
+      <c r="F784">
+        <v>7273.61</v>
+      </c>
+      <c r="G784">
+        <v>66.87495594450387</v>
+      </c>
+      <c r="H784">
+        <v>52.05</v>
+      </c>
+      <c r="I784">
+        <v>0</v>
+      </c>
+      <c r="J784">
+        <v>0</v>
+      </c>
+      <c r="K784">
+        <v>0.4785576153947526</v>
+      </c>
+      <c r="L784">
+        <v>0</v>
+      </c>
+      <c r="M784">
+        <v>1</v>
+      </c>
+      <c r="N784">
+        <v>0</v>
+      </c>
+      <c r="O784">
+        <v>25.63495</v>
+      </c>
+      <c r="P784">
+        <v>73.25945930498399</v>
+      </c>
+      <c r="Q784">
+        <v>34.992</v>
+      </c>
+      <c r="R784">
+        <v>786.8002899999999</v>
+      </c>
+      <c r="S784">
+        <v>7.233991749746393</v>
+      </c>
+      <c r="T784">
+        <v>794.1700000000001</v>
+      </c>
+      <c r="U784">
+        <v>21</v>
+      </c>
+      <c r="V784">
+        <v>29</v>
+      </c>
+      <c r="W784">
+        <v>50</v>
+      </c>
+      <c r="X784">
+        <v>122</v>
+      </c>
+      <c r="Y784">
+        <v>21</v>
+      </c>
+      <c r="Z784">
+        <v>113</v>
+      </c>
+      <c r="AA784">
+        <v>29</v>
+      </c>
+      <c r="AB784">
+        <v>59</v>
+      </c>
+      <c r="AC784">
+        <v>4.44767</v>
+      </c>
+      <c r="AD784">
+        <v>-2.36564</v>
+      </c>
+      <c r="AE784">
+        <v>0</v>
+      </c>
+      <c r="AF784">
+        <v>689.8752000000001</v>
+      </c>
+      <c r="AG784">
+        <v>0</v>
+      </c>
+      <c r="AH784">
+        <v>3</v>
+      </c>
+      <c r="AI784">
+        <v>2360.400869999999</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B785" s="2">
+        <v>46230</v>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>MD+3</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Sesión 42</t>
+        </is>
+      </c>
+      <c r="E785">
+        <v>84.79616666666668</v>
+      </c>
+      <c r="F785">
+        <v>3300</v>
+      </c>
+      <c r="G785">
+        <v>38.91685355273528</v>
+      </c>
+      <c r="H785">
+        <v>1.6</v>
+      </c>
+      <c r="I785">
+        <v>0</v>
+      </c>
+      <c r="J785">
+        <v>0</v>
+      </c>
+      <c r="K785">
+        <v>0.01886877748011408</v>
+      </c>
+      <c r="L785">
+        <v>0</v>
+      </c>
+      <c r="M785">
+        <v>0</v>
+      </c>
+      <c r="N785">
+        <v>0</v>
+      </c>
+      <c r="O785">
+        <v>20.98318</v>
+      </c>
+      <c r="P785">
+        <v>61.74429143126176</v>
+      </c>
+      <c r="Q785">
+        <v>33.984</v>
+      </c>
+      <c r="R785">
+        <v>328.50216</v>
+      </c>
+      <c r="S785">
+        <v>3.874021349235519</v>
+      </c>
+      <c r="T785">
+        <v>180.75</v>
+      </c>
+      <c r="U785">
+        <v>20</v>
+      </c>
+      <c r="V785">
+        <v>24</v>
+      </c>
+      <c r="W785">
+        <v>44</v>
+      </c>
+      <c r="X785">
+        <v>26</v>
+      </c>
+      <c r="Y785">
+        <v>20</v>
+      </c>
+      <c r="Z785">
+        <v>25</v>
+      </c>
+      <c r="AA785">
+        <v>24</v>
+      </c>
+      <c r="AB785">
+        <v>0</v>
+      </c>
+      <c r="AC785">
+        <v>4.26622</v>
+      </c>
+      <c r="AD785">
+        <v>-1.84411</v>
+      </c>
+      <c r="AE785">
+        <v>0</v>
+      </c>
+      <c r="AF785">
+        <v>262.8073</v>
+      </c>
+      <c r="AG785">
+        <v>0</v>
+      </c>
+      <c r="AH785">
+        <v>3</v>
+      </c>
+      <c r="AI785">
+        <v>985.50648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-29
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI785"/>
+  <dimension ref="A1:AI808"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -89020,6 +89020,2605 @@
         <v>985.50648</v>
       </c>
     </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B786" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E786">
+        <v>118.65</v>
+      </c>
+      <c r="F786">
+        <v>6118.83</v>
+      </c>
+      <c r="G786">
+        <v>51.57041719342604</v>
+      </c>
+      <c r="H786">
+        <v>73.29000000000001</v>
+      </c>
+      <c r="I786">
+        <v>0</v>
+      </c>
+      <c r="J786">
+        <v>0</v>
+      </c>
+      <c r="K786">
+        <v>0.6176991150442478</v>
+      </c>
+      <c r="L786">
+        <v>0</v>
+      </c>
+      <c r="M786">
+        <v>1</v>
+      </c>
+      <c r="N786">
+        <v>0</v>
+      </c>
+      <c r="O786">
+        <v>28.1575</v>
+      </c>
+      <c r="P786">
+        <v>78.21527777777777</v>
+      </c>
+      <c r="Q786">
+        <v>36</v>
+      </c>
+      <c r="R786">
+        <v>747.78557</v>
+      </c>
+      <c r="S786">
+        <v>6.302448967551622</v>
+      </c>
+      <c r="T786">
+        <v>896.1800000000001</v>
+      </c>
+      <c r="U786">
+        <v>26</v>
+      </c>
+      <c r="V786">
+        <v>21</v>
+      </c>
+      <c r="W786">
+        <v>47</v>
+      </c>
+      <c r="X786">
+        <v>115</v>
+      </c>
+      <c r="Y786">
+        <v>26</v>
+      </c>
+      <c r="Z786">
+        <v>58</v>
+      </c>
+      <c r="AA786">
+        <v>21</v>
+      </c>
+      <c r="AB786">
+        <v>37</v>
+      </c>
+      <c r="AC786">
+        <v>4.03402</v>
+      </c>
+      <c r="AD786">
+        <v>-3.03258</v>
+      </c>
+      <c r="AE786">
+        <v>0</v>
+      </c>
+      <c r="AF786">
+        <v>1441.414</v>
+      </c>
+      <c r="AG786">
+        <v>0</v>
+      </c>
+      <c r="AH786">
+        <v>3</v>
+      </c>
+      <c r="AI786">
+        <v>2243.35671</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B787" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E787">
+        <v>118.65</v>
+      </c>
+      <c r="F787">
+        <v>6399.42</v>
+      </c>
+      <c r="G787">
+        <v>53.93527180783818</v>
+      </c>
+      <c r="H787">
+        <v>119.71</v>
+      </c>
+      <c r="I787">
+        <v>0</v>
+      </c>
+      <c r="J787">
+        <v>0</v>
+      </c>
+      <c r="K787">
+        <v>1.008933839022335</v>
+      </c>
+      <c r="L787">
+        <v>0</v>
+      </c>
+      <c r="M787">
+        <v>1</v>
+      </c>
+      <c r="N787">
+        <v>0</v>
+      </c>
+      <c r="O787">
+        <v>25.47772</v>
+      </c>
+      <c r="P787">
+        <v>78.72240761339762</v>
+      </c>
+      <c r="Q787">
+        <v>32.364</v>
+      </c>
+      <c r="R787">
+        <v>637.51325</v>
+      </c>
+      <c r="S787">
+        <v>5.373057311420143</v>
+      </c>
+      <c r="T787">
+        <v>785.27</v>
+      </c>
+      <c r="U787">
+        <v>13</v>
+      </c>
+      <c r="V787">
+        <v>7</v>
+      </c>
+      <c r="W787">
+        <v>20</v>
+      </c>
+      <c r="X787">
+        <v>66</v>
+      </c>
+      <c r="Y787">
+        <v>13</v>
+      </c>
+      <c r="Z787">
+        <v>36</v>
+      </c>
+      <c r="AA787">
+        <v>7</v>
+      </c>
+      <c r="AB787">
+        <v>12</v>
+      </c>
+      <c r="AC787">
+        <v>3.83508</v>
+      </c>
+      <c r="AD787">
+        <v>-1.70485</v>
+      </c>
+      <c r="AE787">
+        <v>0</v>
+      </c>
+      <c r="AF787">
+        <v>505.3181</v>
+      </c>
+      <c r="AG787">
+        <v>0</v>
+      </c>
+      <c r="AH787">
+        <v>3</v>
+      </c>
+      <c r="AI787">
+        <v>1912.53975</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B788" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E788">
+        <v>118.65</v>
+      </c>
+      <c r="F788">
+        <v>6479.39</v>
+      </c>
+      <c r="G788">
+        <v>54.60927096502318</v>
+      </c>
+      <c r="H788">
+        <v>95.08</v>
+      </c>
+      <c r="I788">
+        <v>0</v>
+      </c>
+      <c r="J788">
+        <v>0</v>
+      </c>
+      <c r="K788">
+        <v>0.8013485040033712</v>
+      </c>
+      <c r="L788">
+        <v>0</v>
+      </c>
+      <c r="M788">
+        <v>1</v>
+      </c>
+      <c r="N788">
+        <v>0</v>
+      </c>
+      <c r="O788">
+        <v>26.57668</v>
+      </c>
+      <c r="P788">
+        <v>73.82411111111111</v>
+      </c>
+      <c r="Q788">
+        <v>36</v>
+      </c>
+      <c r="R788">
+        <v>557.13176</v>
+      </c>
+      <c r="S788">
+        <v>4.695590054782975</v>
+      </c>
+      <c r="T788">
+        <v>956.82999</v>
+      </c>
+      <c r="U788">
+        <v>18</v>
+      </c>
+      <c r="V788">
+        <v>24</v>
+      </c>
+      <c r="W788">
+        <v>42</v>
+      </c>
+      <c r="X788">
+        <v>112</v>
+      </c>
+      <c r="Y788">
+        <v>18</v>
+      </c>
+      <c r="Z788">
+        <v>74</v>
+      </c>
+      <c r="AA788">
+        <v>24</v>
+      </c>
+      <c r="AB788">
+        <v>30</v>
+      </c>
+      <c r="AC788">
+        <v>3.97601</v>
+      </c>
+      <c r="AD788">
+        <v>-3.3222</v>
+      </c>
+      <c r="AE788">
+        <v>0</v>
+      </c>
+      <c r="AF788">
+        <v>1528.378</v>
+      </c>
+      <c r="AG788">
+        <v>0</v>
+      </c>
+      <c r="AH788">
+        <v>3</v>
+      </c>
+      <c r="AI788">
+        <v>1671.39528</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B789" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E789">
+        <v>118.65</v>
+      </c>
+      <c r="F789">
+        <v>6796.14</v>
+      </c>
+      <c r="G789">
+        <v>57.27888748419722</v>
+      </c>
+      <c r="H789">
+        <v>223.63</v>
+      </c>
+      <c r="I789">
+        <v>0</v>
+      </c>
+      <c r="J789">
+        <v>0</v>
+      </c>
+      <c r="K789">
+        <v>1.884787189211968</v>
+      </c>
+      <c r="L789">
+        <v>0</v>
+      </c>
+      <c r="M789">
+        <v>2</v>
+      </c>
+      <c r="N789">
+        <v>0</v>
+      </c>
+      <c r="O789">
+        <v>28.45995</v>
+      </c>
+      <c r="P789">
+        <v>87.83935185185186</v>
+      </c>
+      <c r="Q789">
+        <v>32.4</v>
+      </c>
+      <c r="R789">
+        <v>739.22964</v>
+      </c>
+      <c r="S789">
+        <v>6.230338305941846</v>
+      </c>
+      <c r="T789">
+        <v>1111.17002</v>
+      </c>
+      <c r="U789">
+        <v>31</v>
+      </c>
+      <c r="V789">
+        <v>11</v>
+      </c>
+      <c r="W789">
+        <v>42</v>
+      </c>
+      <c r="X789">
+        <v>109</v>
+      </c>
+      <c r="Y789">
+        <v>31</v>
+      </c>
+      <c r="Z789">
+        <v>66</v>
+      </c>
+      <c r="AA789">
+        <v>11</v>
+      </c>
+      <c r="AB789">
+        <v>9</v>
+      </c>
+      <c r="AC789">
+        <v>4.29189</v>
+      </c>
+      <c r="AD789">
+        <v>-3.54219</v>
+      </c>
+      <c r="AE789">
+        <v>0</v>
+      </c>
+      <c r="AF789">
+        <v>562.7755</v>
+      </c>
+      <c r="AG789">
+        <v>0</v>
+      </c>
+      <c r="AH789">
+        <v>3</v>
+      </c>
+      <c r="AI789">
+        <v>2217.68892</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B790" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E790">
+        <v>118.65</v>
+      </c>
+      <c r="F790">
+        <v>6207.72</v>
+      </c>
+      <c r="G790">
+        <v>52.31959544879899</v>
+      </c>
+      <c r="H790">
+        <v>234.28</v>
+      </c>
+      <c r="I790">
+        <v>0</v>
+      </c>
+      <c r="J790">
+        <v>0</v>
+      </c>
+      <c r="K790">
+        <v>1.974546986936367</v>
+      </c>
+      <c r="L790">
+        <v>0</v>
+      </c>
+      <c r="M790">
+        <v>4</v>
+      </c>
+      <c r="N790">
+        <v>0</v>
+      </c>
+      <c r="O790">
+        <v>28.09471</v>
+      </c>
+      <c r="P790">
+        <v>82.67040371939736</v>
+      </c>
+      <c r="Q790">
+        <v>33.984</v>
+      </c>
+      <c r="R790">
+        <v>721.42895</v>
+      </c>
+      <c r="S790">
+        <v>6.080311420143278</v>
+      </c>
+      <c r="T790">
+        <v>941.4100100000001</v>
+      </c>
+      <c r="U790">
+        <v>23</v>
+      </c>
+      <c r="V790">
+        <v>17</v>
+      </c>
+      <c r="W790">
+        <v>40</v>
+      </c>
+      <c r="X790">
+        <v>83</v>
+      </c>
+      <c r="Y790">
+        <v>23</v>
+      </c>
+      <c r="Z790">
+        <v>62</v>
+      </c>
+      <c r="AA790">
+        <v>17</v>
+      </c>
+      <c r="AB790">
+        <v>15</v>
+      </c>
+      <c r="AC790">
+        <v>4.12033</v>
+      </c>
+      <c r="AD790">
+        <v>-2.83657</v>
+      </c>
+      <c r="AE790">
+        <v>0</v>
+      </c>
+      <c r="AF790">
+        <v>576.5088000000001</v>
+      </c>
+      <c r="AG790">
+        <v>0</v>
+      </c>
+      <c r="AH790">
+        <v>3</v>
+      </c>
+      <c r="AI790">
+        <v>2164.28685</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B791" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E791">
+        <v>118.65</v>
+      </c>
+      <c r="F791">
+        <v>7213.89</v>
+      </c>
+      <c r="G791">
+        <v>60.79974715549937</v>
+      </c>
+      <c r="H791">
+        <v>270.14</v>
+      </c>
+      <c r="I791">
+        <v>18.96</v>
+      </c>
+      <c r="J791">
+        <v>1</v>
+      </c>
+      <c r="K791">
+        <v>2.276780446691951</v>
+      </c>
+      <c r="L791">
+        <v>29.91</v>
+      </c>
+      <c r="M791">
+        <v>7</v>
+      </c>
+      <c r="N791">
+        <v>1</v>
+      </c>
+      <c r="O791">
+        <v>33.46765</v>
+      </c>
+      <c r="P791">
+        <v>94.09483243364822</v>
+      </c>
+      <c r="Q791">
+        <v>35.568</v>
+      </c>
+      <c r="R791">
+        <v>648.74715</v>
+      </c>
+      <c r="S791">
+        <v>5.467738305941846</v>
+      </c>
+      <c r="T791">
+        <v>1147.37999</v>
+      </c>
+      <c r="U791">
+        <v>43</v>
+      </c>
+      <c r="V791">
+        <v>23</v>
+      </c>
+      <c r="W791">
+        <v>66</v>
+      </c>
+      <c r="X791">
+        <v>121</v>
+      </c>
+      <c r="Y791">
+        <v>43</v>
+      </c>
+      <c r="Z791">
+        <v>85</v>
+      </c>
+      <c r="AA791">
+        <v>23</v>
+      </c>
+      <c r="AB791">
+        <v>20</v>
+      </c>
+      <c r="AC791">
+        <v>4.44059</v>
+      </c>
+      <c r="AD791">
+        <v>-3.33409</v>
+      </c>
+      <c r="AE791">
+        <v>0</v>
+      </c>
+      <c r="AF791">
+        <v>691.968</v>
+      </c>
+      <c r="AG791">
+        <v>0</v>
+      </c>
+      <c r="AH791">
+        <v>3</v>
+      </c>
+      <c r="AI791">
+        <v>1946.24145</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B792" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E792">
+        <v>118.65</v>
+      </c>
+      <c r="F792">
+        <v>6856.48</v>
+      </c>
+      <c r="G792">
+        <v>57.78744205646861</v>
+      </c>
+      <c r="H792">
+        <v>214.77</v>
+      </c>
+      <c r="I792">
+        <v>0</v>
+      </c>
+      <c r="J792">
+        <v>0</v>
+      </c>
+      <c r="K792">
+        <v>1.810113780025284</v>
+      </c>
+      <c r="L792">
+        <v>0</v>
+      </c>
+      <c r="M792">
+        <v>3</v>
+      </c>
+      <c r="N792">
+        <v>0</v>
+      </c>
+      <c r="O792">
+        <v>26.19209</v>
+      </c>
+      <c r="P792">
+        <v>72.75580555555555</v>
+      </c>
+      <c r="Q792">
+        <v>36</v>
+      </c>
+      <c r="R792">
+        <v>731.93467</v>
+      </c>
+      <c r="S792">
+        <v>6.168855204382638</v>
+      </c>
+      <c r="T792">
+        <v>897.0900300000001</v>
+      </c>
+      <c r="U792">
+        <v>19</v>
+      </c>
+      <c r="V792">
+        <v>16</v>
+      </c>
+      <c r="W792">
+        <v>35</v>
+      </c>
+      <c r="X792">
+        <v>88</v>
+      </c>
+      <c r="Y792">
+        <v>19</v>
+      </c>
+      <c r="Z792">
+        <v>68</v>
+      </c>
+      <c r="AA792">
+        <v>16</v>
+      </c>
+      <c r="AB792">
+        <v>15</v>
+      </c>
+      <c r="AC792">
+        <v>4.16732</v>
+      </c>
+      <c r="AD792">
+        <v>-2.57342</v>
+      </c>
+      <c r="AE792">
+        <v>0</v>
+      </c>
+      <c r="AF792">
+        <v>1584.002</v>
+      </c>
+      <c r="AG792">
+        <v>0</v>
+      </c>
+      <c r="AH792">
+        <v>3</v>
+      </c>
+      <c r="AI792">
+        <v>2195.80401</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B793" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E793">
+        <v>118.65</v>
+      </c>
+      <c r="F793">
+        <v>6250.77</v>
+      </c>
+      <c r="G793">
+        <v>52.68242730720607</v>
+      </c>
+      <c r="H793">
+        <v>265.96</v>
+      </c>
+      <c r="I793">
+        <v>0</v>
+      </c>
+      <c r="J793">
+        <v>0</v>
+      </c>
+      <c r="K793">
+        <v>2.241550779603877</v>
+      </c>
+      <c r="L793">
+        <v>0</v>
+      </c>
+      <c r="M793">
+        <v>5</v>
+      </c>
+      <c r="N793">
+        <v>0</v>
+      </c>
+      <c r="O793">
+        <v>28.73222</v>
+      </c>
+      <c r="P793">
+        <v>79.81172222222223</v>
+      </c>
+      <c r="Q793">
+        <v>36</v>
+      </c>
+      <c r="R793">
+        <v>605.9688599999999</v>
+      </c>
+      <c r="S793">
+        <v>5.107196460176991</v>
+      </c>
+      <c r="T793">
+        <v>983.22001</v>
+      </c>
+      <c r="U793">
+        <v>21</v>
+      </c>
+      <c r="V793">
+        <v>23</v>
+      </c>
+      <c r="W793">
+        <v>44</v>
+      </c>
+      <c r="X793">
+        <v>88</v>
+      </c>
+      <c r="Y793">
+        <v>21</v>
+      </c>
+      <c r="Z793">
+        <v>52</v>
+      </c>
+      <c r="AA793">
+        <v>23</v>
+      </c>
+      <c r="AB793">
+        <v>24</v>
+      </c>
+      <c r="AC793">
+        <v>4.24301</v>
+      </c>
+      <c r="AD793">
+        <v>-3.12866</v>
+      </c>
+      <c r="AE793">
+        <v>0</v>
+      </c>
+      <c r="AF793">
+        <v>525.6642999999999</v>
+      </c>
+      <c r="AG793">
+        <v>0</v>
+      </c>
+      <c r="AH793">
+        <v>3</v>
+      </c>
+      <c r="AI793">
+        <v>1817.90658</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B794" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E794">
+        <v>118.65</v>
+      </c>
+      <c r="F794">
+        <v>5500.2</v>
+      </c>
+      <c r="G794">
+        <v>46.35651074589127</v>
+      </c>
+      <c r="H794">
+        <v>145.32</v>
+      </c>
+      <c r="I794">
+        <v>0</v>
+      </c>
+      <c r="J794">
+        <v>0</v>
+      </c>
+      <c r="K794">
+        <v>1.224778761061947</v>
+      </c>
+      <c r="L794">
+        <v>0</v>
+      </c>
+      <c r="M794">
+        <v>3</v>
+      </c>
+      <c r="N794">
+        <v>0</v>
+      </c>
+      <c r="O794">
+        <v>27.87504</v>
+      </c>
+      <c r="P794">
+        <v>87.09861267341581</v>
+      </c>
+      <c r="Q794">
+        <v>32.004</v>
+      </c>
+      <c r="R794">
+        <v>572.28257</v>
+      </c>
+      <c r="S794">
+        <v>4.823283354403708</v>
+      </c>
+      <c r="T794">
+        <v>708.2600199999999</v>
+      </c>
+      <c r="U794">
+        <v>18</v>
+      </c>
+      <c r="V794">
+        <v>19</v>
+      </c>
+      <c r="W794">
+        <v>37</v>
+      </c>
+      <c r="X794">
+        <v>78</v>
+      </c>
+      <c r="Y794">
+        <v>18</v>
+      </c>
+      <c r="Z794">
+        <v>52</v>
+      </c>
+      <c r="AA794">
+        <v>19</v>
+      </c>
+      <c r="AB794">
+        <v>13</v>
+      </c>
+      <c r="AC794">
+        <v>3.84655</v>
+      </c>
+      <c r="AD794">
+        <v>-2.24325</v>
+      </c>
+      <c r="AE794">
+        <v>0</v>
+      </c>
+      <c r="AF794">
+        <v>383.016</v>
+      </c>
+      <c r="AG794">
+        <v>0</v>
+      </c>
+      <c r="AH794">
+        <v>3</v>
+      </c>
+      <c r="AI794">
+        <v>1716.84771</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B795" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E795">
+        <v>118.65</v>
+      </c>
+      <c r="F795">
+        <v>6761.639999999999</v>
+      </c>
+      <c r="G795">
+        <v>56.98811630847028</v>
+      </c>
+      <c r="H795">
+        <v>267.01</v>
+      </c>
+      <c r="I795">
+        <v>0</v>
+      </c>
+      <c r="J795">
+        <v>0</v>
+      </c>
+      <c r="K795">
+        <v>2.250400337126001</v>
+      </c>
+      <c r="L795">
+        <v>12.51</v>
+      </c>
+      <c r="M795">
+        <v>6</v>
+      </c>
+      <c r="N795">
+        <v>1</v>
+      </c>
+      <c r="O795">
+        <v>31.85856</v>
+      </c>
+      <c r="P795">
+        <v>94.14468085106382</v>
+      </c>
+      <c r="Q795">
+        <v>33.84</v>
+      </c>
+      <c r="R795">
+        <v>601.9235600000001</v>
+      </c>
+      <c r="S795">
+        <v>5.073102064896755</v>
+      </c>
+      <c r="T795">
+        <v>1025.31997</v>
+      </c>
+      <c r="U795">
+        <v>37</v>
+      </c>
+      <c r="V795">
+        <v>27</v>
+      </c>
+      <c r="W795">
+        <v>64</v>
+      </c>
+      <c r="X795">
+        <v>119</v>
+      </c>
+      <c r="Y795">
+        <v>37</v>
+      </c>
+      <c r="Z795">
+        <v>80</v>
+      </c>
+      <c r="AA795">
+        <v>27</v>
+      </c>
+      <c r="AB795">
+        <v>15</v>
+      </c>
+      <c r="AC795">
+        <v>4.47172</v>
+      </c>
+      <c r="AD795">
+        <v>-3.06801</v>
+      </c>
+      <c r="AE795">
+        <v>0</v>
+      </c>
+      <c r="AF795">
+        <v>569.0076</v>
+      </c>
+      <c r="AG795">
+        <v>0</v>
+      </c>
+      <c r="AH795">
+        <v>3</v>
+      </c>
+      <c r="AI795">
+        <v>1805.77068</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B796" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E796">
+        <v>118.65</v>
+      </c>
+      <c r="F796">
+        <v>6242.5</v>
+      </c>
+      <c r="G796">
+        <v>52.61272650653181</v>
+      </c>
+      <c r="H796">
+        <v>191.18</v>
+      </c>
+      <c r="I796">
+        <v>0</v>
+      </c>
+      <c r="J796">
+        <v>0</v>
+      </c>
+      <c r="K796">
+        <v>1.611293721028234</v>
+      </c>
+      <c r="L796">
+        <v>0</v>
+      </c>
+      <c r="M796">
+        <v>2</v>
+      </c>
+      <c r="N796">
+        <v>0</v>
+      </c>
+      <c r="O796">
+        <v>29.27355</v>
+      </c>
+      <c r="P796">
+        <v>86.87544515669516</v>
+      </c>
+      <c r="Q796">
+        <v>33.696</v>
+      </c>
+      <c r="R796">
+        <v>608.77491</v>
+      </c>
+      <c r="S796">
+        <v>5.130846270543615</v>
+      </c>
+      <c r="T796">
+        <v>969.35</v>
+      </c>
+      <c r="U796">
+        <v>24</v>
+      </c>
+      <c r="V796">
+        <v>20</v>
+      </c>
+      <c r="W796">
+        <v>44</v>
+      </c>
+      <c r="X796">
+        <v>99</v>
+      </c>
+      <c r="Y796">
+        <v>24</v>
+      </c>
+      <c r="Z796">
+        <v>61</v>
+      </c>
+      <c r="AA796">
+        <v>20</v>
+      </c>
+      <c r="AB796">
+        <v>20</v>
+      </c>
+      <c r="AC796">
+        <v>4.43342</v>
+      </c>
+      <c r="AD796">
+        <v>-3.01518</v>
+      </c>
+      <c r="AE796">
+        <v>0</v>
+      </c>
+      <c r="AF796">
+        <v>586.832</v>
+      </c>
+      <c r="AG796">
+        <v>0</v>
+      </c>
+      <c r="AH796">
+        <v>3</v>
+      </c>
+      <c r="AI796">
+        <v>1826.32473</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B797" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E797">
+        <v>118.65</v>
+      </c>
+      <c r="F797">
+        <v>6592.83</v>
+      </c>
+      <c r="G797">
+        <v>55.5653603034134</v>
+      </c>
+      <c r="H797">
+        <v>173.85</v>
+      </c>
+      <c r="I797">
+        <v>0</v>
+      </c>
+      <c r="J797">
+        <v>0</v>
+      </c>
+      <c r="K797">
+        <v>1.465233881163085</v>
+      </c>
+      <c r="L797">
+        <v>0</v>
+      </c>
+      <c r="M797">
+        <v>2</v>
+      </c>
+      <c r="N797">
+        <v>0</v>
+      </c>
+      <c r="O797">
+        <v>29.56999</v>
+      </c>
+      <c r="P797">
+        <v>82.13886111111111</v>
+      </c>
+      <c r="Q797">
+        <v>36</v>
+      </c>
+      <c r="R797">
+        <v>740.09196</v>
+      </c>
+      <c r="S797">
+        <v>6.237606068268015</v>
+      </c>
+      <c r="T797">
+        <v>903.4100100000001</v>
+      </c>
+      <c r="U797">
+        <v>15</v>
+      </c>
+      <c r="V797">
+        <v>16</v>
+      </c>
+      <c r="W797">
+        <v>31</v>
+      </c>
+      <c r="X797">
+        <v>85</v>
+      </c>
+      <c r="Y797">
+        <v>15</v>
+      </c>
+      <c r="Z797">
+        <v>56</v>
+      </c>
+      <c r="AA797">
+        <v>16</v>
+      </c>
+      <c r="AB797">
+        <v>11</v>
+      </c>
+      <c r="AC797">
+        <v>4.63988</v>
+      </c>
+      <c r="AD797">
+        <v>-3.56886</v>
+      </c>
+      <c r="AE797">
+        <v>0</v>
+      </c>
+      <c r="AF797">
+        <v>1535.658</v>
+      </c>
+      <c r="AG797">
+        <v>0</v>
+      </c>
+      <c r="AH797">
+        <v>3</v>
+      </c>
+      <c r="AI797">
+        <v>2220.27588</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B798" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E798">
+        <v>118.65</v>
+      </c>
+      <c r="F798">
+        <v>6841.440000000001</v>
+      </c>
+      <c r="G798">
+        <v>57.66068268015171</v>
+      </c>
+      <c r="H798">
+        <v>427.12</v>
+      </c>
+      <c r="I798">
+        <v>0</v>
+      </c>
+      <c r="J798">
+        <v>0</v>
+      </c>
+      <c r="K798">
+        <v>3.599831436999578</v>
+      </c>
+      <c r="L798">
+        <v>7.52</v>
+      </c>
+      <c r="M798">
+        <v>10</v>
+      </c>
+      <c r="N798">
+        <v>1</v>
+      </c>
+      <c r="O798">
+        <v>30.96764</v>
+      </c>
+      <c r="P798">
+        <v>88.49919981710106</v>
+      </c>
+      <c r="Q798">
+        <v>34.992</v>
+      </c>
+      <c r="R798">
+        <v>640.59874</v>
+      </c>
+      <c r="S798">
+        <v>5.399062284028656</v>
+      </c>
+      <c r="T798">
+        <v>1018.69</v>
+      </c>
+      <c r="U798">
+        <v>20</v>
+      </c>
+      <c r="V798">
+        <v>22</v>
+      </c>
+      <c r="W798">
+        <v>42</v>
+      </c>
+      <c r="X798">
+        <v>91</v>
+      </c>
+      <c r="Y798">
+        <v>20</v>
+      </c>
+      <c r="Z798">
+        <v>66</v>
+      </c>
+      <c r="AA798">
+        <v>22</v>
+      </c>
+      <c r="AB798">
+        <v>16</v>
+      </c>
+      <c r="AC798">
+        <v>4.15462</v>
+      </c>
+      <c r="AD798">
+        <v>-3.06876</v>
+      </c>
+      <c r="AE798">
+        <v>0</v>
+      </c>
+      <c r="AF798">
+        <v>551.04297</v>
+      </c>
+      <c r="AG798">
+        <v>0</v>
+      </c>
+      <c r="AH798">
+        <v>3</v>
+      </c>
+      <c r="AI798">
+        <v>1921.79622</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B799" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E799">
+        <v>118.65</v>
+      </c>
+      <c r="F799">
+        <v>4698.259999999999</v>
+      </c>
+      <c r="G799">
+        <v>39.59764011799409</v>
+      </c>
+      <c r="H799">
+        <v>68.34999999999999</v>
+      </c>
+      <c r="I799">
+        <v>0</v>
+      </c>
+      <c r="J799">
+        <v>0</v>
+      </c>
+      <c r="K799">
+        <v>0.57606405394016</v>
+      </c>
+      <c r="L799">
+        <v>0</v>
+      </c>
+      <c r="M799">
+        <v>2</v>
+      </c>
+      <c r="N799">
+        <v>0</v>
+      </c>
+      <c r="O799">
+        <v>26.90309</v>
+      </c>
+      <c r="P799">
+        <v>77.04206758304696</v>
+      </c>
+      <c r="Q799">
+        <v>34.92</v>
+      </c>
+      <c r="R799">
+        <v>473.70672</v>
+      </c>
+      <c r="S799">
+        <v>3.992471302149178</v>
+      </c>
+      <c r="T799">
+        <v>623.56001</v>
+      </c>
+      <c r="U799">
+        <v>11</v>
+      </c>
+      <c r="V799">
+        <v>4</v>
+      </c>
+      <c r="W799">
+        <v>15</v>
+      </c>
+      <c r="X799">
+        <v>70</v>
+      </c>
+      <c r="Y799">
+        <v>11</v>
+      </c>
+      <c r="Z799">
+        <v>36</v>
+      </c>
+      <c r="AA799">
+        <v>4</v>
+      </c>
+      <c r="AB799">
+        <v>9</v>
+      </c>
+      <c r="AC799">
+        <v>3.62553</v>
+      </c>
+      <c r="AD799">
+        <v>0</v>
+      </c>
+      <c r="AE799">
+        <v>0</v>
+      </c>
+      <c r="AF799">
+        <v>430.1096</v>
+      </c>
+      <c r="AG799">
+        <v>0</v>
+      </c>
+      <c r="AH799">
+        <v>3</v>
+      </c>
+      <c r="AI799">
+        <v>1421.12016</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B800" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E800">
+        <v>118.65</v>
+      </c>
+      <c r="F800">
+        <v>5926.55</v>
+      </c>
+      <c r="G800">
+        <v>49.94985250737463</v>
+      </c>
+      <c r="H800">
+        <v>70.54000000000001</v>
+      </c>
+      <c r="I800">
+        <v>0</v>
+      </c>
+      <c r="J800">
+        <v>0</v>
+      </c>
+      <c r="K800">
+        <v>0.5945217024863043</v>
+      </c>
+      <c r="L800">
+        <v>0</v>
+      </c>
+      <c r="M800">
+        <v>0</v>
+      </c>
+      <c r="N800">
+        <v>0</v>
+      </c>
+      <c r="O800">
+        <v>22.98077</v>
+      </c>
+      <c r="P800">
+        <v>65.6743541380887</v>
+      </c>
+      <c r="Q800">
+        <v>34.992</v>
+      </c>
+      <c r="R800">
+        <v>487.14912</v>
+      </c>
+      <c r="S800">
+        <v>4.105765865992415</v>
+      </c>
+      <c r="T800">
+        <v>741.3000099999999</v>
+      </c>
+      <c r="U800">
+        <v>17</v>
+      </c>
+      <c r="V800">
+        <v>22</v>
+      </c>
+      <c r="W800">
+        <v>39</v>
+      </c>
+      <c r="X800">
+        <v>73</v>
+      </c>
+      <c r="Y800">
+        <v>17</v>
+      </c>
+      <c r="Z800">
+        <v>63</v>
+      </c>
+      <c r="AA800">
+        <v>22</v>
+      </c>
+      <c r="AB800">
+        <v>15</v>
+      </c>
+      <c r="AC800">
+        <v>3.82778</v>
+      </c>
+      <c r="AD800">
+        <v>-2.22425</v>
+      </c>
+      <c r="AE800">
+        <v>0</v>
+      </c>
+      <c r="AF800">
+        <v>493.36267</v>
+      </c>
+      <c r="AG800">
+        <v>0</v>
+      </c>
+      <c r="AH800">
+        <v>3</v>
+      </c>
+      <c r="AI800">
+        <v>1461.44736</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B801" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E801">
+        <v>118.65</v>
+      </c>
+      <c r="F801">
+        <v>6173.45</v>
+      </c>
+      <c r="G801">
+        <v>52.0307627475769</v>
+      </c>
+      <c r="H801">
+        <v>24.45</v>
+      </c>
+      <c r="I801">
+        <v>0</v>
+      </c>
+      <c r="J801">
+        <v>0</v>
+      </c>
+      <c r="K801">
+        <v>0.2060682680151706</v>
+      </c>
+      <c r="L801">
+        <v>0</v>
+      </c>
+      <c r="M801">
+        <v>0</v>
+      </c>
+      <c r="N801">
+        <v>0</v>
+      </c>
+      <c r="O801">
+        <v>22.87676</v>
+      </c>
+      <c r="P801">
+        <v>63.54655555555556</v>
+      </c>
+      <c r="Q801">
+        <v>36</v>
+      </c>
+      <c r="R801">
+        <v>713.9470699999999</v>
+      </c>
+      <c r="S801">
+        <v>6.017253013063632</v>
+      </c>
+      <c r="T801">
+        <v>702.06001</v>
+      </c>
+      <c r="U801">
+        <v>13</v>
+      </c>
+      <c r="V801">
+        <v>22</v>
+      </c>
+      <c r="W801">
+        <v>35</v>
+      </c>
+      <c r="X801">
+        <v>80</v>
+      </c>
+      <c r="Y801">
+        <v>13</v>
+      </c>
+      <c r="Z801">
+        <v>59</v>
+      </c>
+      <c r="AA801">
+        <v>22</v>
+      </c>
+      <c r="AB801">
+        <v>50</v>
+      </c>
+      <c r="AC801">
+        <v>3.50635</v>
+      </c>
+      <c r="AD801">
+        <v>-2.5599</v>
+      </c>
+      <c r="AE801">
+        <v>0</v>
+      </c>
+      <c r="AF801">
+        <v>1428.136</v>
+      </c>
+      <c r="AG801">
+        <v>0</v>
+      </c>
+      <c r="AH801">
+        <v>3</v>
+      </c>
+      <c r="AI801">
+        <v>2141.84121</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B802" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E802">
+        <v>118.65</v>
+      </c>
+      <c r="F802">
+        <v>5224.320000000001</v>
+      </c>
+      <c r="G802">
+        <v>44.03135271807839</v>
+      </c>
+      <c r="H802">
+        <v>110.46</v>
+      </c>
+      <c r="I802">
+        <v>0</v>
+      </c>
+      <c r="J802">
+        <v>0</v>
+      </c>
+      <c r="K802">
+        <v>0.9309734513274337</v>
+      </c>
+      <c r="L802">
+        <v>0</v>
+      </c>
+      <c r="M802">
+        <v>1</v>
+      </c>
+      <c r="N802">
+        <v>0</v>
+      </c>
+      <c r="O802">
+        <v>25.63547</v>
+      </c>
+      <c r="P802">
+        <v>75.43393950094162</v>
+      </c>
+      <c r="Q802">
+        <v>33.984</v>
+      </c>
+      <c r="R802">
+        <v>560.27561</v>
+      </c>
+      <c r="S802">
+        <v>4.722086894226718</v>
+      </c>
+      <c r="T802">
+        <v>744.52999</v>
+      </c>
+      <c r="U802">
+        <v>17</v>
+      </c>
+      <c r="V802">
+        <v>13</v>
+      </c>
+      <c r="W802">
+        <v>30</v>
+      </c>
+      <c r="X802">
+        <v>73</v>
+      </c>
+      <c r="Y802">
+        <v>17</v>
+      </c>
+      <c r="Z802">
+        <v>57</v>
+      </c>
+      <c r="AA802">
+        <v>13</v>
+      </c>
+      <c r="AB802">
+        <v>27</v>
+      </c>
+      <c r="AC802">
+        <v>3.9345</v>
+      </c>
+      <c r="AD802">
+        <v>-2.79654</v>
+      </c>
+      <c r="AE802">
+        <v>0</v>
+      </c>
+      <c r="AF802">
+        <v>486.4872</v>
+      </c>
+      <c r="AG802">
+        <v>0</v>
+      </c>
+      <c r="AH802">
+        <v>3</v>
+      </c>
+      <c r="AI802">
+        <v>1680.82683</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B803" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E803">
+        <v>118.65</v>
+      </c>
+      <c r="F803">
+        <v>6561.84</v>
+      </c>
+      <c r="G803">
+        <v>55.30417193426043</v>
+      </c>
+      <c r="H803">
+        <v>69.98</v>
+      </c>
+      <c r="I803">
+        <v>0</v>
+      </c>
+      <c r="J803">
+        <v>0</v>
+      </c>
+      <c r="K803">
+        <v>0.5898019384745049</v>
+      </c>
+      <c r="L803">
+        <v>0</v>
+      </c>
+      <c r="M803">
+        <v>0</v>
+      </c>
+      <c r="N803">
+        <v>0</v>
+      </c>
+      <c r="O803">
+        <v>23.7983</v>
+      </c>
+      <c r="P803">
+        <v>68.0106881572931</v>
+      </c>
+      <c r="Q803">
+        <v>34.992</v>
+      </c>
+      <c r="R803">
+        <v>597.26566</v>
+      </c>
+      <c r="S803">
+        <v>5.033844584913611</v>
+      </c>
+      <c r="T803">
+        <v>942.09998</v>
+      </c>
+      <c r="U803">
+        <v>20</v>
+      </c>
+      <c r="V803">
+        <v>23</v>
+      </c>
+      <c r="W803">
+        <v>43</v>
+      </c>
+      <c r="X803">
+        <v>121</v>
+      </c>
+      <c r="Y803">
+        <v>20</v>
+      </c>
+      <c r="Z803">
+        <v>83</v>
+      </c>
+      <c r="AA803">
+        <v>23</v>
+      </c>
+      <c r="AB803">
+        <v>29</v>
+      </c>
+      <c r="AC803">
+        <v>4.19698</v>
+      </c>
+      <c r="AD803">
+        <v>-2.56077</v>
+      </c>
+      <c r="AE803">
+        <v>0</v>
+      </c>
+      <c r="AF803">
+        <v>622.9968</v>
+      </c>
+      <c r="AG803">
+        <v>0</v>
+      </c>
+      <c r="AH803">
+        <v>3</v>
+      </c>
+      <c r="AI803">
+        <v>1791.79698</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B804" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E804">
+        <v>118.65</v>
+      </c>
+      <c r="F804">
+        <v>5788.2</v>
+      </c>
+      <c r="G804">
+        <v>48.78381795195954</v>
+      </c>
+      <c r="H804">
+        <v>146.54</v>
+      </c>
+      <c r="I804">
+        <v>0</v>
+      </c>
+      <c r="J804">
+        <v>0</v>
+      </c>
+      <c r="K804">
+        <v>1.235061104087653</v>
+      </c>
+      <c r="L804">
+        <v>0</v>
+      </c>
+      <c r="M804">
+        <v>2</v>
+      </c>
+      <c r="N804">
+        <v>0</v>
+      </c>
+      <c r="O804">
+        <v>27.04692</v>
+      </c>
+      <c r="P804">
+        <v>81.93057070156307</v>
+      </c>
+      <c r="Q804">
+        <v>33.012</v>
+      </c>
+      <c r="R804">
+        <v>556.60513</v>
+      </c>
+      <c r="S804">
+        <v>4.691151538137379</v>
+      </c>
+      <c r="T804">
+        <v>736.9</v>
+      </c>
+      <c r="U804">
+        <v>21</v>
+      </c>
+      <c r="V804">
+        <v>20</v>
+      </c>
+      <c r="W804">
+        <v>41</v>
+      </c>
+      <c r="X804">
+        <v>74</v>
+      </c>
+      <c r="Y804">
+        <v>21</v>
+      </c>
+      <c r="Z804">
+        <v>61</v>
+      </c>
+      <c r="AA804">
+        <v>20</v>
+      </c>
+      <c r="AB804">
+        <v>23</v>
+      </c>
+      <c r="AC804">
+        <v>3.99931</v>
+      </c>
+      <c r="AD804">
+        <v>-3.43734</v>
+      </c>
+      <c r="AE804">
+        <v>0</v>
+      </c>
+      <c r="AF804">
+        <v>502.59225</v>
+      </c>
+      <c r="AG804">
+        <v>0</v>
+      </c>
+      <c r="AH804">
+        <v>3</v>
+      </c>
+      <c r="AI804">
+        <v>1669.81539</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B805" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E805">
+        <v>118.65</v>
+      </c>
+      <c r="F805">
+        <v>5966.52</v>
+      </c>
+      <c r="G805">
+        <v>50.28672566371682</v>
+      </c>
+      <c r="H805">
+        <v>153.51</v>
+      </c>
+      <c r="I805">
+        <v>0</v>
+      </c>
+      <c r="J805">
+        <v>0</v>
+      </c>
+      <c r="K805">
+        <v>1.293805309734513</v>
+      </c>
+      <c r="L805">
+        <v>0</v>
+      </c>
+      <c r="M805">
+        <v>2</v>
+      </c>
+      <c r="N805">
+        <v>0</v>
+      </c>
+      <c r="O805">
+        <v>26.55039</v>
+      </c>
+      <c r="P805">
+        <v>82.95959880014999</v>
+      </c>
+      <c r="Q805">
+        <v>32.004</v>
+      </c>
+      <c r="R805">
+        <v>542.35117</v>
+      </c>
+      <c r="S805">
+        <v>4.571017024863043</v>
+      </c>
+      <c r="T805">
+        <v>817.7499799999999</v>
+      </c>
+      <c r="U805">
+        <v>24</v>
+      </c>
+      <c r="V805">
+        <v>12</v>
+      </c>
+      <c r="W805">
+        <v>36</v>
+      </c>
+      <c r="X805">
+        <v>93</v>
+      </c>
+      <c r="Y805">
+        <v>24</v>
+      </c>
+      <c r="Z805">
+        <v>64</v>
+      </c>
+      <c r="AA805">
+        <v>12</v>
+      </c>
+      <c r="AB805">
+        <v>23</v>
+      </c>
+      <c r="AC805">
+        <v>3.88851</v>
+      </c>
+      <c r="AD805">
+        <v>-2.5354</v>
+      </c>
+      <c r="AE805">
+        <v>0</v>
+      </c>
+      <c r="AF805">
+        <v>489.5667</v>
+      </c>
+      <c r="AG805">
+        <v>0</v>
+      </c>
+      <c r="AH805">
+        <v>3</v>
+      </c>
+      <c r="AI805">
+        <v>1627.05351</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B806" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E806">
+        <v>118.65</v>
+      </c>
+      <c r="F806">
+        <v>7312.99</v>
+      </c>
+      <c r="G806">
+        <v>61.63497682258744</v>
+      </c>
+      <c r="H806">
+        <v>87.67999999999999</v>
+      </c>
+      <c r="I806">
+        <v>0</v>
+      </c>
+      <c r="J806">
+        <v>0</v>
+      </c>
+      <c r="K806">
+        <v>0.7389801938474504</v>
+      </c>
+      <c r="L806">
+        <v>0</v>
+      </c>
+      <c r="M806">
+        <v>1</v>
+      </c>
+      <c r="N806">
+        <v>0</v>
+      </c>
+      <c r="O806">
+        <v>25.32491</v>
+      </c>
+      <c r="P806">
+        <v>70.34697222222222</v>
+      </c>
+      <c r="Q806">
+        <v>36</v>
+      </c>
+      <c r="R806">
+        <v>700.83866</v>
+      </c>
+      <c r="S806">
+        <v>5.906773367045933</v>
+      </c>
+      <c r="T806">
+        <v>901.71998</v>
+      </c>
+      <c r="U806">
+        <v>19</v>
+      </c>
+      <c r="V806">
+        <v>14</v>
+      </c>
+      <c r="W806">
+        <v>33</v>
+      </c>
+      <c r="X806">
+        <v>95</v>
+      </c>
+      <c r="Y806">
+        <v>19</v>
+      </c>
+      <c r="Z806">
+        <v>77</v>
+      </c>
+      <c r="AA806">
+        <v>14</v>
+      </c>
+      <c r="AB806">
+        <v>20</v>
+      </c>
+      <c r="AC806">
+        <v>4.20331</v>
+      </c>
+      <c r="AD806">
+        <v>-2.98445</v>
+      </c>
+      <c r="AE806">
+        <v>0</v>
+      </c>
+      <c r="AF806">
+        <v>1695.032</v>
+      </c>
+      <c r="AG806">
+        <v>0</v>
+      </c>
+      <c r="AH806">
+        <v>3</v>
+      </c>
+      <c r="AI806">
+        <v>2102.51598</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B807" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E807">
+        <v>118.65</v>
+      </c>
+      <c r="F807">
+        <v>6512.77</v>
+      </c>
+      <c r="G807">
+        <v>54.8906026127265</v>
+      </c>
+      <c r="H807">
+        <v>196.4</v>
+      </c>
+      <c r="I807">
+        <v>0</v>
+      </c>
+      <c r="J807">
+        <v>0</v>
+      </c>
+      <c r="K807">
+        <v>1.655288664138222</v>
+      </c>
+      <c r="L807">
+        <v>0</v>
+      </c>
+      <c r="M807">
+        <v>3</v>
+      </c>
+      <c r="N807">
+        <v>0</v>
+      </c>
+      <c r="O807">
+        <v>27.05579</v>
+      </c>
+      <c r="P807">
+        <v>77.31993026977595</v>
+      </c>
+      <c r="Q807">
+        <v>34.992</v>
+      </c>
+      <c r="R807">
+        <v>623.6812</v>
+      </c>
+      <c r="S807">
+        <v>5.256478718921197</v>
+      </c>
+      <c r="T807">
+        <v>1103.62998</v>
+      </c>
+      <c r="U807">
+        <v>34</v>
+      </c>
+      <c r="V807">
+        <v>35</v>
+      </c>
+      <c r="W807">
+        <v>69</v>
+      </c>
+      <c r="X807">
+        <v>118</v>
+      </c>
+      <c r="Y807">
+        <v>34</v>
+      </c>
+      <c r="Z807">
+        <v>91</v>
+      </c>
+      <c r="AA807">
+        <v>35</v>
+      </c>
+      <c r="AB807">
+        <v>40</v>
+      </c>
+      <c r="AC807">
+        <v>4.20918</v>
+      </c>
+      <c r="AD807">
+        <v>-2.15802</v>
+      </c>
+      <c r="AE807">
+        <v>0</v>
+      </c>
+      <c r="AF807">
+        <v>627.4592</v>
+      </c>
+      <c r="AG807">
+        <v>0</v>
+      </c>
+      <c r="AH807">
+        <v>3</v>
+      </c>
+      <c r="AI807">
+        <v>1871.0436</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B808" s="2">
+        <v>46231</v>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>MD-5</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Sesion 43</t>
+        </is>
+      </c>
+      <c r="E808">
+        <v>62.8</v>
+      </c>
+      <c r="F808">
+        <v>3352.12</v>
+      </c>
+      <c r="G808">
+        <v>53.37770700636943</v>
+      </c>
+      <c r="H808">
+        <v>85.23999999999999</v>
+      </c>
+      <c r="I808">
+        <v>0</v>
+      </c>
+      <c r="J808">
+        <v>0</v>
+      </c>
+      <c r="K808">
+        <v>1.357324840764331</v>
+      </c>
+      <c r="L808">
+        <v>0</v>
+      </c>
+      <c r="M808">
+        <v>0</v>
+      </c>
+      <c r="N808">
+        <v>0</v>
+      </c>
+      <c r="O808">
+        <v>23.33007</v>
+      </c>
+      <c r="P808">
+        <v>68.65015889830508</v>
+      </c>
+      <c r="Q808">
+        <v>33.984</v>
+      </c>
+      <c r="R808">
+        <v>301.84653</v>
+      </c>
+      <c r="S808">
+        <v>4.806473407643312</v>
+      </c>
+      <c r="T808">
+        <v>504.49</v>
+      </c>
+      <c r="U808">
+        <v>0</v>
+      </c>
+      <c r="V808">
+        <v>0</v>
+      </c>
+      <c r="W808">
+        <v>0</v>
+      </c>
+      <c r="X808">
+        <v>31</v>
+      </c>
+      <c r="Y808">
+        <v>0</v>
+      </c>
+      <c r="Z808">
+        <v>2</v>
+      </c>
+      <c r="AA808">
+        <v>0</v>
+      </c>
+      <c r="AB808">
+        <v>1</v>
+      </c>
+      <c r="AC808">
+        <v>2.85793</v>
+      </c>
+      <c r="AD808">
+        <v>-2.01638</v>
+      </c>
+      <c r="AE808">
+        <v>0</v>
+      </c>
+      <c r="AF808">
+        <v>253.7941</v>
+      </c>
+      <c r="AG808">
+        <v>0</v>
+      </c>
+      <c r="AH808">
+        <v>3</v>
+      </c>
+      <c r="AI808">
+        <v>905.5395900000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-30
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI808"/>
+  <dimension ref="A1:AI832"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -66775,7 +66775,7 @@
       </c>
       <c r="D589" t="inlineStr">
         <is>
-          <t>Sesión 37</t>
+          <t>Sesión 37 pelon</t>
         </is>
       </c>
       <c r="E589">
@@ -91617,6 +91617,2718 @@
       </c>
       <c r="AI808">
         <v>905.5395900000001</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B809" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E809">
+        <v>102.35</v>
+      </c>
+      <c r="F809">
+        <v>4559.509999999999</v>
+      </c>
+      <c r="G809">
+        <v>44.54821690278456</v>
+      </c>
+      <c r="H809">
+        <v>140.66</v>
+      </c>
+      <c r="I809">
+        <v>0</v>
+      </c>
+      <c r="J809">
+        <v>0</v>
+      </c>
+      <c r="K809">
+        <v>1.374303859306302</v>
+      </c>
+      <c r="L809">
+        <v>0</v>
+      </c>
+      <c r="M809">
+        <v>2</v>
+      </c>
+      <c r="N809">
+        <v>0</v>
+      </c>
+      <c r="O809">
+        <v>26.60566</v>
+      </c>
+      <c r="P809">
+        <v>73.90461111111111</v>
+      </c>
+      <c r="Q809">
+        <v>36</v>
+      </c>
+      <c r="R809">
+        <v>557.4296899999999</v>
+      </c>
+      <c r="S809">
+        <v>5.446308646800195</v>
+      </c>
+      <c r="T809">
+        <v>725.5899900000001</v>
+      </c>
+      <c r="U809">
+        <v>22</v>
+      </c>
+      <c r="V809">
+        <v>17</v>
+      </c>
+      <c r="W809">
+        <v>39</v>
+      </c>
+      <c r="X809">
+        <v>69</v>
+      </c>
+      <c r="Y809">
+        <v>22</v>
+      </c>
+      <c r="Z809">
+        <v>45</v>
+      </c>
+      <c r="AA809">
+        <v>17</v>
+      </c>
+      <c r="AB809">
+        <v>21</v>
+      </c>
+      <c r="AC809">
+        <v>4.6109</v>
+      </c>
+      <c r="AD809">
+        <v>-3.82998</v>
+      </c>
+      <c r="AE809">
+        <v>0</v>
+      </c>
+      <c r="AF809">
+        <v>1072.846</v>
+      </c>
+      <c r="AG809">
+        <v>0</v>
+      </c>
+      <c r="AH809">
+        <v>3</v>
+      </c>
+      <c r="AI809">
+        <v>1672.28907</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B810" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E810">
+        <v>102.35</v>
+      </c>
+      <c r="F810">
+        <v>4983.07</v>
+      </c>
+      <c r="G810">
+        <v>48.68656570591109</v>
+      </c>
+      <c r="H810">
+        <v>168.39</v>
+      </c>
+      <c r="I810">
+        <v>0</v>
+      </c>
+      <c r="J810">
+        <v>0</v>
+      </c>
+      <c r="K810">
+        <v>1.64523693209575</v>
+      </c>
+      <c r="L810">
+        <v>0</v>
+      </c>
+      <c r="M810">
+        <v>0</v>
+      </c>
+      <c r="N810">
+        <v>0</v>
+      </c>
+      <c r="O810">
+        <v>23.85623</v>
+      </c>
+      <c r="P810">
+        <v>73.71224199728094</v>
+      </c>
+      <c r="Q810">
+        <v>32.364</v>
+      </c>
+      <c r="R810">
+        <v>467.00157</v>
+      </c>
+      <c r="S810">
+        <v>4.562790131900343</v>
+      </c>
+      <c r="T810">
+        <v>736.99</v>
+      </c>
+      <c r="U810">
+        <v>10</v>
+      </c>
+      <c r="V810">
+        <v>9</v>
+      </c>
+      <c r="W810">
+        <v>19</v>
+      </c>
+      <c r="X810">
+        <v>51</v>
+      </c>
+      <c r="Y810">
+        <v>10</v>
+      </c>
+      <c r="Z810">
+        <v>29</v>
+      </c>
+      <c r="AA810">
+        <v>9</v>
+      </c>
+      <c r="AB810">
+        <v>17</v>
+      </c>
+      <c r="AC810">
+        <v>4.2974</v>
+      </c>
+      <c r="AD810">
+        <v>-3.25355</v>
+      </c>
+      <c r="AE810">
+        <v>0</v>
+      </c>
+      <c r="AF810">
+        <v>398.0004</v>
+      </c>
+      <c r="AG810">
+        <v>0</v>
+      </c>
+      <c r="AH810">
+        <v>3</v>
+      </c>
+      <c r="AI810">
+        <v>1401.00471</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B811" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E811">
+        <v>102.35</v>
+      </c>
+      <c r="F811">
+        <v>5308.19</v>
+      </c>
+      <c r="G811">
+        <v>51.86311675622863</v>
+      </c>
+      <c r="H811">
+        <v>155.4</v>
+      </c>
+      <c r="I811">
+        <v>0</v>
+      </c>
+      <c r="J811">
+        <v>0</v>
+      </c>
+      <c r="K811">
+        <v>1.518319491939424</v>
+      </c>
+      <c r="L811">
+        <v>0</v>
+      </c>
+      <c r="M811">
+        <v>1</v>
+      </c>
+      <c r="N811">
+        <v>0</v>
+      </c>
+      <c r="O811">
+        <v>25.92184</v>
+      </c>
+      <c r="P811">
+        <v>72.00511111111111</v>
+      </c>
+      <c r="Q811">
+        <v>36</v>
+      </c>
+      <c r="R811">
+        <v>429.30495</v>
+      </c>
+      <c r="S811">
+        <v>4.194479237909135</v>
+      </c>
+      <c r="T811">
+        <v>804.3</v>
+      </c>
+      <c r="U811">
+        <v>20</v>
+      </c>
+      <c r="V811">
+        <v>21</v>
+      </c>
+      <c r="W811">
+        <v>41</v>
+      </c>
+      <c r="X811">
+        <v>62</v>
+      </c>
+      <c r="Y811">
+        <v>20</v>
+      </c>
+      <c r="Z811">
+        <v>70</v>
+      </c>
+      <c r="AA811">
+        <v>21</v>
+      </c>
+      <c r="AB811">
+        <v>36</v>
+      </c>
+      <c r="AC811">
+        <v>4.34664</v>
+      </c>
+      <c r="AD811">
+        <v>-3.60613</v>
+      </c>
+      <c r="AE811">
+        <v>0</v>
+      </c>
+      <c r="AF811">
+        <v>1251.452</v>
+      </c>
+      <c r="AG811">
+        <v>0</v>
+      </c>
+      <c r="AH811">
+        <v>3</v>
+      </c>
+      <c r="AI811">
+        <v>1287.91485</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B812" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E812">
+        <v>102.35</v>
+      </c>
+      <c r="F812">
+        <v>5212.34</v>
+      </c>
+      <c r="G812">
+        <v>50.9266243282853</v>
+      </c>
+      <c r="H812">
+        <v>167.32</v>
+      </c>
+      <c r="I812">
+        <v>0</v>
+      </c>
+      <c r="J812">
+        <v>0</v>
+      </c>
+      <c r="K812">
+        <v>1.634782608695652</v>
+      </c>
+      <c r="L812">
+        <v>0</v>
+      </c>
+      <c r="M812">
+        <v>1</v>
+      </c>
+      <c r="N812">
+        <v>0</v>
+      </c>
+      <c r="O812">
+        <v>26.08037</v>
+      </c>
+      <c r="P812">
+        <v>80.49496913580246</v>
+      </c>
+      <c r="Q812">
+        <v>32.4</v>
+      </c>
+      <c r="R812">
+        <v>536.84333</v>
+      </c>
+      <c r="S812">
+        <v>5.245171763556424</v>
+      </c>
+      <c r="T812">
+        <v>839.09998</v>
+      </c>
+      <c r="U812">
+        <v>24</v>
+      </c>
+      <c r="V812">
+        <v>13</v>
+      </c>
+      <c r="W812">
+        <v>37</v>
+      </c>
+      <c r="X812">
+        <v>57</v>
+      </c>
+      <c r="Y812">
+        <v>24</v>
+      </c>
+      <c r="Z812">
+        <v>34</v>
+      </c>
+      <c r="AA812">
+        <v>13</v>
+      </c>
+      <c r="AB812">
+        <v>18</v>
+      </c>
+      <c r="AC812">
+        <v>3.81865</v>
+      </c>
+      <c r="AD812">
+        <v>-3.81928</v>
+      </c>
+      <c r="AE812">
+        <v>0</v>
+      </c>
+      <c r="AF812">
+        <v>422.933</v>
+      </c>
+      <c r="AG812">
+        <v>0</v>
+      </c>
+      <c r="AH812">
+        <v>3</v>
+      </c>
+      <c r="AI812">
+        <v>1610.52999</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B813" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E813">
+        <v>102.35</v>
+      </c>
+      <c r="F813">
+        <v>5043.57</v>
+      </c>
+      <c r="G813">
+        <v>49.27767464582315</v>
+      </c>
+      <c r="H813">
+        <v>400.81</v>
+      </c>
+      <c r="I813">
+        <v>0</v>
+      </c>
+      <c r="J813">
+        <v>0</v>
+      </c>
+      <c r="K813">
+        <v>3.916072300928188</v>
+      </c>
+      <c r="L813">
+        <v>6.550000000000001</v>
+      </c>
+      <c r="M813">
+        <v>10</v>
+      </c>
+      <c r="N813">
+        <v>1</v>
+      </c>
+      <c r="O813">
+        <v>30.34337</v>
+      </c>
+      <c r="P813">
+        <v>89.2872233992467</v>
+      </c>
+      <c r="Q813">
+        <v>33.984</v>
+      </c>
+      <c r="R813">
+        <v>600.54423</v>
+      </c>
+      <c r="S813">
+        <v>5.867554763067904</v>
+      </c>
+      <c r="T813">
+        <v>920.85002</v>
+      </c>
+      <c r="U813">
+        <v>12</v>
+      </c>
+      <c r="V813">
+        <v>13</v>
+      </c>
+      <c r="W813">
+        <v>25</v>
+      </c>
+      <c r="X813">
+        <v>62</v>
+      </c>
+      <c r="Y813">
+        <v>12</v>
+      </c>
+      <c r="Z813">
+        <v>43</v>
+      </c>
+      <c r="AA813">
+        <v>13</v>
+      </c>
+      <c r="AB813">
+        <v>15</v>
+      </c>
+      <c r="AC813">
+        <v>3.99439</v>
+      </c>
+      <c r="AD813">
+        <v>-3.0553</v>
+      </c>
+      <c r="AE813">
+        <v>0</v>
+      </c>
+      <c r="AF813">
+        <v>469.2568</v>
+      </c>
+      <c r="AG813">
+        <v>0</v>
+      </c>
+      <c r="AH813">
+        <v>3</v>
+      </c>
+      <c r="AI813">
+        <v>1801.63269</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B814" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E814">
+        <v>102.35</v>
+      </c>
+      <c r="F814">
+        <v>5551.160000000001</v>
+      </c>
+      <c r="G814">
+        <v>54.2370297997069</v>
+      </c>
+      <c r="H814">
+        <v>298.33</v>
+      </c>
+      <c r="I814">
+        <v>0</v>
+      </c>
+      <c r="J814">
+        <v>0</v>
+      </c>
+      <c r="K814">
+        <v>2.914802149487054</v>
+      </c>
+      <c r="L814">
+        <v>6.42</v>
+      </c>
+      <c r="M814">
+        <v>6</v>
+      </c>
+      <c r="N814">
+        <v>1</v>
+      </c>
+      <c r="O814">
+        <v>30.45017</v>
+      </c>
+      <c r="P814">
+        <v>85.61113922627081</v>
+      </c>
+      <c r="Q814">
+        <v>35.568</v>
+      </c>
+      <c r="R814">
+        <v>492.44706</v>
+      </c>
+      <c r="S814">
+        <v>4.81140263800684</v>
+      </c>
+      <c r="T814">
+        <v>957.23</v>
+      </c>
+      <c r="U814">
+        <v>32</v>
+      </c>
+      <c r="V814">
+        <v>23</v>
+      </c>
+      <c r="W814">
+        <v>55</v>
+      </c>
+      <c r="X814">
+        <v>79</v>
+      </c>
+      <c r="Y814">
+        <v>32</v>
+      </c>
+      <c r="Z814">
+        <v>61</v>
+      </c>
+      <c r="AA814">
+        <v>23</v>
+      </c>
+      <c r="AB814">
+        <v>20</v>
+      </c>
+      <c r="AC814">
+        <v>4.83191</v>
+      </c>
+      <c r="AD814">
+        <v>-4.11573</v>
+      </c>
+      <c r="AE814">
+        <v>0</v>
+      </c>
+      <c r="AF814">
+        <v>533.4296000000001</v>
+      </c>
+      <c r="AG814">
+        <v>0</v>
+      </c>
+      <c r="AH814">
+        <v>3</v>
+      </c>
+      <c r="AI814">
+        <v>1477.34118</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B815" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E815">
+        <v>102.35</v>
+      </c>
+      <c r="F815">
+        <v>5554.58</v>
+      </c>
+      <c r="G815">
+        <v>54.2704445530044</v>
+      </c>
+      <c r="H815">
+        <v>318.66</v>
+      </c>
+      <c r="I815">
+        <v>0</v>
+      </c>
+      <c r="J815">
+        <v>0</v>
+      </c>
+      <c r="K815">
+        <v>3.113434294088911</v>
+      </c>
+      <c r="L815">
+        <v>0</v>
+      </c>
+      <c r="M815">
+        <v>4</v>
+      </c>
+      <c r="N815">
+        <v>0</v>
+      </c>
+      <c r="O815">
+        <v>28.19107</v>
+      </c>
+      <c r="P815">
+        <v>78.30852777777778</v>
+      </c>
+      <c r="Q815">
+        <v>36</v>
+      </c>
+      <c r="R815">
+        <v>587.38417</v>
+      </c>
+      <c r="S815">
+        <v>5.738975769418662</v>
+      </c>
+      <c r="T815">
+        <v>885.51</v>
+      </c>
+      <c r="U815">
+        <v>21</v>
+      </c>
+      <c r="V815">
+        <v>14</v>
+      </c>
+      <c r="W815">
+        <v>35</v>
+      </c>
+      <c r="X815">
+        <v>59</v>
+      </c>
+      <c r="Y815">
+        <v>21</v>
+      </c>
+      <c r="Z815">
+        <v>41</v>
+      </c>
+      <c r="AA815">
+        <v>14</v>
+      </c>
+      <c r="AB815">
+        <v>17</v>
+      </c>
+      <c r="AC815">
+        <v>4.2665</v>
+      </c>
+      <c r="AD815">
+        <v>-3.26034</v>
+      </c>
+      <c r="AE815">
+        <v>0</v>
+      </c>
+      <c r="AF815">
+        <v>1279.044</v>
+      </c>
+      <c r="AG815">
+        <v>0</v>
+      </c>
+      <c r="AH815">
+        <v>3</v>
+      </c>
+      <c r="AI815">
+        <v>1762.15251</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B816" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E816">
+        <v>102.35</v>
+      </c>
+      <c r="F816">
+        <v>5615.93</v>
+      </c>
+      <c r="G816">
+        <v>54.86985832926234</v>
+      </c>
+      <c r="H816">
+        <v>601.41</v>
+      </c>
+      <c r="I816">
+        <v>0</v>
+      </c>
+      <c r="J816">
+        <v>0</v>
+      </c>
+      <c r="K816">
+        <v>5.876013678553981</v>
+      </c>
+      <c r="L816">
+        <v>19.95</v>
+      </c>
+      <c r="M816">
+        <v>12</v>
+      </c>
+      <c r="N816">
+        <v>2</v>
+      </c>
+      <c r="O816">
+        <v>31.29342</v>
+      </c>
+      <c r="P816">
+        <v>86.92616666666667</v>
+      </c>
+      <c r="Q816">
+        <v>36</v>
+      </c>
+      <c r="R816">
+        <v>560.62922</v>
+      </c>
+      <c r="S816">
+        <v>5.4775693209575</v>
+      </c>
+      <c r="T816">
+        <v>1181.14002</v>
+      </c>
+      <c r="U816">
+        <v>30</v>
+      </c>
+      <c r="V816">
+        <v>27</v>
+      </c>
+      <c r="W816">
+        <v>57</v>
+      </c>
+      <c r="X816">
+        <v>75</v>
+      </c>
+      <c r="Y816">
+        <v>30</v>
+      </c>
+      <c r="Z816">
+        <v>58</v>
+      </c>
+      <c r="AA816">
+        <v>27</v>
+      </c>
+      <c r="AB816">
+        <v>44</v>
+      </c>
+      <c r="AC816">
+        <v>4.6744</v>
+      </c>
+      <c r="AD816">
+        <v>-4.01649</v>
+      </c>
+      <c r="AE816">
+        <v>0</v>
+      </c>
+      <c r="AF816">
+        <v>480.7726</v>
+      </c>
+      <c r="AG816">
+        <v>0</v>
+      </c>
+      <c r="AH816">
+        <v>3</v>
+      </c>
+      <c r="AI816">
+        <v>1681.88766</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B817" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E817">
+        <v>102.35</v>
+      </c>
+      <c r="F817">
+        <v>4909.969999999999</v>
+      </c>
+      <c r="G817">
+        <v>47.97234978016609</v>
+      </c>
+      <c r="H817">
+        <v>287.03</v>
+      </c>
+      <c r="I817">
+        <v>0</v>
+      </c>
+      <c r="J817">
+        <v>0</v>
+      </c>
+      <c r="K817">
+        <v>2.804396678065462</v>
+      </c>
+      <c r="L817">
+        <v>0</v>
+      </c>
+      <c r="M817">
+        <v>7</v>
+      </c>
+      <c r="N817">
+        <v>0</v>
+      </c>
+      <c r="O817">
+        <v>28.45723</v>
+      </c>
+      <c r="P817">
+        <v>88.91772903387077</v>
+      </c>
+      <c r="Q817">
+        <v>32.004</v>
+      </c>
+      <c r="R817">
+        <v>516.07068</v>
+      </c>
+      <c r="S817">
+        <v>5.042214753297509</v>
+      </c>
+      <c r="T817">
+        <v>777.18001</v>
+      </c>
+      <c r="U817">
+        <v>30</v>
+      </c>
+      <c r="V817">
+        <v>20</v>
+      </c>
+      <c r="W817">
+        <v>50</v>
+      </c>
+      <c r="X817">
+        <v>64</v>
+      </c>
+      <c r="Y817">
+        <v>30</v>
+      </c>
+      <c r="Z817">
+        <v>46</v>
+      </c>
+      <c r="AA817">
+        <v>20</v>
+      </c>
+      <c r="AB817">
+        <v>22</v>
+      </c>
+      <c r="AC817">
+        <v>4.43845</v>
+      </c>
+      <c r="AD817">
+        <v>-4.31056</v>
+      </c>
+      <c r="AE817">
+        <v>0</v>
+      </c>
+      <c r="AF817">
+        <v>343.2228</v>
+      </c>
+      <c r="AG817">
+        <v>0</v>
+      </c>
+      <c r="AH817">
+        <v>3</v>
+      </c>
+      <c r="AI817">
+        <v>1548.21204</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B818" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E818">
+        <v>102.35</v>
+      </c>
+      <c r="F818">
+        <v>5219.15</v>
+      </c>
+      <c r="G818">
+        <v>50.99316072300928</v>
+      </c>
+      <c r="H818">
+        <v>282.36</v>
+      </c>
+      <c r="I818">
+        <v>0</v>
+      </c>
+      <c r="J818">
+        <v>0</v>
+      </c>
+      <c r="K818">
+        <v>2.758768930141671</v>
+      </c>
+      <c r="L818">
+        <v>0</v>
+      </c>
+      <c r="M818">
+        <v>4</v>
+      </c>
+      <c r="N818">
+        <v>0</v>
+      </c>
+      <c r="O818">
+        <v>26.47617</v>
+      </c>
+      <c r="P818">
+        <v>78.23927304964539</v>
+      </c>
+      <c r="Q818">
+        <v>33.84</v>
+      </c>
+      <c r="R818">
+        <v>514.7429999999999</v>
+      </c>
+      <c r="S818">
+        <v>5.02924279433317</v>
+      </c>
+      <c r="T818">
+        <v>971.5799999999999</v>
+      </c>
+      <c r="U818">
+        <v>36</v>
+      </c>
+      <c r="V818">
+        <v>22</v>
+      </c>
+      <c r="W818">
+        <v>58</v>
+      </c>
+      <c r="X818">
+        <v>89</v>
+      </c>
+      <c r="Y818">
+        <v>36</v>
+      </c>
+      <c r="Z818">
+        <v>68</v>
+      </c>
+      <c r="AA818">
+        <v>22</v>
+      </c>
+      <c r="AB818">
+        <v>35</v>
+      </c>
+      <c r="AC818">
+        <v>4.63984</v>
+      </c>
+      <c r="AD818">
+        <v>-4.25272</v>
+      </c>
+      <c r="AE818">
+        <v>0</v>
+      </c>
+      <c r="AF818">
+        <v>443.3051</v>
+      </c>
+      <c r="AG818">
+        <v>0</v>
+      </c>
+      <c r="AH818">
+        <v>3</v>
+      </c>
+      <c r="AI818">
+        <v>1544.229</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B819" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E819">
+        <v>102.35</v>
+      </c>
+      <c r="F819">
+        <v>4830.29</v>
+      </c>
+      <c r="G819">
+        <v>47.19384465070836</v>
+      </c>
+      <c r="H819">
+        <v>184.98</v>
+      </c>
+      <c r="I819">
+        <v>0</v>
+      </c>
+      <c r="J819">
+        <v>0</v>
+      </c>
+      <c r="K819">
+        <v>1.80732779677577</v>
+      </c>
+      <c r="L819">
+        <v>0</v>
+      </c>
+      <c r="M819">
+        <v>2</v>
+      </c>
+      <c r="N819">
+        <v>0</v>
+      </c>
+      <c r="O819">
+        <v>26.42095</v>
+      </c>
+      <c r="P819">
+        <v>78.40975189933525</v>
+      </c>
+      <c r="Q819">
+        <v>33.696</v>
+      </c>
+      <c r="R819">
+        <v>449.78265</v>
+      </c>
+      <c r="S819">
+        <v>4.394554469956033</v>
+      </c>
+      <c r="T819">
+        <v>664.16</v>
+      </c>
+      <c r="U819">
+        <v>18</v>
+      </c>
+      <c r="V819">
+        <v>13</v>
+      </c>
+      <c r="W819">
+        <v>31</v>
+      </c>
+      <c r="X819">
+        <v>61</v>
+      </c>
+      <c r="Y819">
+        <v>18</v>
+      </c>
+      <c r="Z819">
+        <v>41</v>
+      </c>
+      <c r="AA819">
+        <v>13</v>
+      </c>
+      <c r="AB819">
+        <v>20</v>
+      </c>
+      <c r="AC819">
+        <v>4.23993</v>
+      </c>
+      <c r="AD819">
+        <v>-2.94713</v>
+      </c>
+      <c r="AE819">
+        <v>0</v>
+      </c>
+      <c r="AF819">
+        <v>450.444</v>
+      </c>
+      <c r="AG819">
+        <v>0</v>
+      </c>
+      <c r="AH819">
+        <v>3</v>
+      </c>
+      <c r="AI819">
+        <v>1349.34795</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B820" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E820">
+        <v>102.35</v>
+      </c>
+      <c r="F820">
+        <v>5062.83</v>
+      </c>
+      <c r="G820">
+        <v>49.46585246702492</v>
+      </c>
+      <c r="H820">
+        <v>313.3</v>
+      </c>
+      <c r="I820">
+        <v>0</v>
+      </c>
+      <c r="J820">
+        <v>0</v>
+      </c>
+      <c r="K820">
+        <v>3.061064973131412</v>
+      </c>
+      <c r="L820">
+        <v>0</v>
+      </c>
+      <c r="M820">
+        <v>2</v>
+      </c>
+      <c r="N820">
+        <v>0</v>
+      </c>
+      <c r="O820">
+        <v>27.4141</v>
+      </c>
+      <c r="P820">
+        <v>76.15027777777779</v>
+      </c>
+      <c r="Q820">
+        <v>36</v>
+      </c>
+      <c r="R820">
+        <v>579.30382</v>
+      </c>
+      <c r="S820">
+        <v>5.660027552515877</v>
+      </c>
+      <c r="T820">
+        <v>962.6300100000001</v>
+      </c>
+      <c r="U820">
+        <v>20</v>
+      </c>
+      <c r="V820">
+        <v>19</v>
+      </c>
+      <c r="W820">
+        <v>39</v>
+      </c>
+      <c r="X820">
+        <v>71</v>
+      </c>
+      <c r="Y820">
+        <v>20</v>
+      </c>
+      <c r="Z820">
+        <v>51</v>
+      </c>
+      <c r="AA820">
+        <v>19</v>
+      </c>
+      <c r="AB820">
+        <v>0</v>
+      </c>
+      <c r="AC820">
+        <v>4.35074</v>
+      </c>
+      <c r="AD820">
+        <v>-3.66475</v>
+      </c>
+      <c r="AE820">
+        <v>0</v>
+      </c>
+      <c r="AF820">
+        <v>1204.82</v>
+      </c>
+      <c r="AG820">
+        <v>0</v>
+      </c>
+      <c r="AH820">
+        <v>3</v>
+      </c>
+      <c r="AI820">
+        <v>1737.91146</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B821" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E821">
+        <v>102.35</v>
+      </c>
+      <c r="F821">
+        <v>5390.31</v>
+      </c>
+      <c r="G821">
+        <v>52.66546165119688</v>
+      </c>
+      <c r="H821">
+        <v>315.36</v>
+      </c>
+      <c r="I821">
+        <v>0</v>
+      </c>
+      <c r="J821">
+        <v>0</v>
+      </c>
+      <c r="K821">
+        <v>3.081191988275525</v>
+      </c>
+      <c r="L821">
+        <v>0</v>
+      </c>
+      <c r="M821">
+        <v>4</v>
+      </c>
+      <c r="N821">
+        <v>0</v>
+      </c>
+      <c r="O821">
+        <v>26.88754</v>
+      </c>
+      <c r="P821">
+        <v>76.83910608139004</v>
+      </c>
+      <c r="Q821">
+        <v>34.992</v>
+      </c>
+      <c r="R821">
+        <v>474.38925</v>
+      </c>
+      <c r="S821">
+        <v>4.634970688812897</v>
+      </c>
+      <c r="T821">
+        <v>855.61001</v>
+      </c>
+      <c r="U821">
+        <v>22</v>
+      </c>
+      <c r="V821">
+        <v>17</v>
+      </c>
+      <c r="W821">
+        <v>39</v>
+      </c>
+      <c r="X821">
+        <v>73</v>
+      </c>
+      <c r="Y821">
+        <v>22</v>
+      </c>
+      <c r="Z821">
+        <v>52</v>
+      </c>
+      <c r="AA821">
+        <v>17</v>
+      </c>
+      <c r="AB821">
+        <v>39</v>
+      </c>
+      <c r="AC821">
+        <v>3.81192</v>
+      </c>
+      <c r="AD821">
+        <v>-3.70233</v>
+      </c>
+      <c r="AE821">
+        <v>0</v>
+      </c>
+      <c r="AF821">
+        <v>433.96239</v>
+      </c>
+      <c r="AG821">
+        <v>0</v>
+      </c>
+      <c r="AH821">
+        <v>3</v>
+      </c>
+      <c r="AI821">
+        <v>1423.16775</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B822" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E822">
+        <v>112.05</v>
+      </c>
+      <c r="F822">
+        <v>4321.120000000001</v>
+      </c>
+      <c r="G822">
+        <v>38.56421240517627</v>
+      </c>
+      <c r="H822">
+        <v>133.61</v>
+      </c>
+      <c r="I822">
+        <v>0</v>
+      </c>
+      <c r="J822">
+        <v>0</v>
+      </c>
+      <c r="K822">
+        <v>1.192414100847836</v>
+      </c>
+      <c r="L822">
+        <v>0</v>
+      </c>
+      <c r="M822">
+        <v>2</v>
+      </c>
+      <c r="N822">
+        <v>0</v>
+      </c>
+      <c r="O822">
+        <v>26.45431</v>
+      </c>
+      <c r="P822">
+        <v>75.75690148911798</v>
+      </c>
+      <c r="Q822">
+        <v>34.92</v>
+      </c>
+      <c r="R822">
+        <v>448.9175</v>
+      </c>
+      <c r="S822">
+        <v>4.00640339134315</v>
+      </c>
+      <c r="T822">
+        <v>498.96998</v>
+      </c>
+      <c r="U822">
+        <v>10</v>
+      </c>
+      <c r="V822">
+        <v>5</v>
+      </c>
+      <c r="W822">
+        <v>15</v>
+      </c>
+      <c r="X822">
+        <v>41</v>
+      </c>
+      <c r="Y822">
+        <v>10</v>
+      </c>
+      <c r="Z822">
+        <v>22</v>
+      </c>
+      <c r="AA822">
+        <v>5</v>
+      </c>
+      <c r="AB822">
+        <v>37</v>
+      </c>
+      <c r="AC822">
+        <v>3.83008</v>
+      </c>
+      <c r="AD822">
+        <v>-2.78981</v>
+      </c>
+      <c r="AE822">
+        <v>0</v>
+      </c>
+      <c r="AF822">
+        <v>389.4232</v>
+      </c>
+      <c r="AG822">
+        <v>0</v>
+      </c>
+      <c r="AH822">
+        <v>3</v>
+      </c>
+      <c r="AI822">
+        <v>1346.7525</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B823" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E823">
+        <v>102.35</v>
+      </c>
+      <c r="F823">
+        <v>5470.75</v>
+      </c>
+      <c r="G823">
+        <v>53.4513922813874</v>
+      </c>
+      <c r="H823">
+        <v>214.67</v>
+      </c>
+      <c r="I823">
+        <v>0</v>
+      </c>
+      <c r="J823">
+        <v>0</v>
+      </c>
+      <c r="K823">
+        <v>2.097410845139228</v>
+      </c>
+      <c r="L823">
+        <v>0</v>
+      </c>
+      <c r="M823">
+        <v>2</v>
+      </c>
+      <c r="N823">
+        <v>0</v>
+      </c>
+      <c r="O823">
+        <v>25.77065</v>
+      </c>
+      <c r="P823">
+        <v>73.64726223136716</v>
+      </c>
+      <c r="Q823">
+        <v>34.992</v>
+      </c>
+      <c r="R823">
+        <v>450.98856</v>
+      </c>
+      <c r="S823">
+        <v>4.406336687835858</v>
+      </c>
+      <c r="T823">
+        <v>936.83998</v>
+      </c>
+      <c r="U823">
+        <v>18</v>
+      </c>
+      <c r="V823">
+        <v>20</v>
+      </c>
+      <c r="W823">
+        <v>38</v>
+      </c>
+      <c r="X823">
+        <v>65</v>
+      </c>
+      <c r="Y823">
+        <v>18</v>
+      </c>
+      <c r="Z823">
+        <v>69</v>
+      </c>
+      <c r="AA823">
+        <v>20</v>
+      </c>
+      <c r="AB823">
+        <v>43</v>
+      </c>
+      <c r="AC823">
+        <v>4.10688</v>
+      </c>
+      <c r="AD823">
+        <v>-3.62196</v>
+      </c>
+      <c r="AE823">
+        <v>0</v>
+      </c>
+      <c r="AF823">
+        <v>444.1547</v>
+      </c>
+      <c r="AG823">
+        <v>0</v>
+      </c>
+      <c r="AH823">
+        <v>3</v>
+      </c>
+      <c r="AI823">
+        <v>1352.96568</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B824" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E824">
+        <v>112.05</v>
+      </c>
+      <c r="F824">
+        <v>5477</v>
+      </c>
+      <c r="G824">
+        <v>48.87996430165105</v>
+      </c>
+      <c r="H824">
+        <v>130.21</v>
+      </c>
+      <c r="I824">
+        <v>0</v>
+      </c>
+      <c r="J824">
+        <v>0</v>
+      </c>
+      <c r="K824">
+        <v>1.162070504239179</v>
+      </c>
+      <c r="L824">
+        <v>0</v>
+      </c>
+      <c r="M824">
+        <v>0</v>
+      </c>
+      <c r="N824">
+        <v>0</v>
+      </c>
+      <c r="O824">
+        <v>24.80714</v>
+      </c>
+      <c r="P824">
+        <v>68.90872222222222</v>
+      </c>
+      <c r="Q824">
+        <v>36</v>
+      </c>
+      <c r="R824">
+        <v>595.72014</v>
+      </c>
+      <c r="S824">
+        <v>5.316556358768407</v>
+      </c>
+      <c r="T824">
+        <v>724.37999</v>
+      </c>
+      <c r="U824">
+        <v>19</v>
+      </c>
+      <c r="V824">
+        <v>13</v>
+      </c>
+      <c r="W824">
+        <v>32</v>
+      </c>
+      <c r="X824">
+        <v>60</v>
+      </c>
+      <c r="Y824">
+        <v>19</v>
+      </c>
+      <c r="Z824">
+        <v>61</v>
+      </c>
+      <c r="AA824">
+        <v>13</v>
+      </c>
+      <c r="AB824">
+        <v>33</v>
+      </c>
+      <c r="AC824">
+        <v>3.98557</v>
+      </c>
+      <c r="AD824">
+        <v>-3.40348</v>
+      </c>
+      <c r="AE824">
+        <v>0</v>
+      </c>
+      <c r="AF824">
+        <v>1294.448</v>
+      </c>
+      <c r="AG824">
+        <v>0</v>
+      </c>
+      <c r="AH824">
+        <v>3</v>
+      </c>
+      <c r="AI824">
+        <v>1787.16042</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B825" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E825">
+        <v>102.35</v>
+      </c>
+      <c r="F825">
+        <v>4732.54</v>
+      </c>
+      <c r="G825">
+        <v>46.23878847093307</v>
+      </c>
+      <c r="H825">
+        <v>234.98</v>
+      </c>
+      <c r="I825">
+        <v>0</v>
+      </c>
+      <c r="J825">
+        <v>0</v>
+      </c>
+      <c r="K825">
+        <v>2.295847581827064</v>
+      </c>
+      <c r="L825">
+        <v>0</v>
+      </c>
+      <c r="M825">
+        <v>2</v>
+      </c>
+      <c r="N825">
+        <v>0</v>
+      </c>
+      <c r="O825">
+        <v>28.90279</v>
+      </c>
+      <c r="P825">
+        <v>85.04822857815442</v>
+      </c>
+      <c r="Q825">
+        <v>33.984</v>
+      </c>
+      <c r="R825">
+        <v>462.01016</v>
+      </c>
+      <c r="S825">
+        <v>4.514022081094285</v>
+      </c>
+      <c r="T825">
+        <v>810.34</v>
+      </c>
+      <c r="U825">
+        <v>17</v>
+      </c>
+      <c r="V825">
+        <v>19</v>
+      </c>
+      <c r="W825">
+        <v>36</v>
+      </c>
+      <c r="X825">
+        <v>59</v>
+      </c>
+      <c r="Y825">
+        <v>17</v>
+      </c>
+      <c r="Z825">
+        <v>53</v>
+      </c>
+      <c r="AA825">
+        <v>19</v>
+      </c>
+      <c r="AB825">
+        <v>24</v>
+      </c>
+      <c r="AC825">
+        <v>4.27764</v>
+      </c>
+      <c r="AD825">
+        <v>-2.83341</v>
+      </c>
+      <c r="AE825">
+        <v>0</v>
+      </c>
+      <c r="AF825">
+        <v>444.2248</v>
+      </c>
+      <c r="AG825">
+        <v>0</v>
+      </c>
+      <c r="AH825">
+        <v>3</v>
+      </c>
+      <c r="AI825">
+        <v>1386.03048</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B826" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E826">
+        <v>105.4426666666667</v>
+      </c>
+      <c r="F826">
+        <v>5856.15</v>
+      </c>
+      <c r="G826">
+        <v>55.53871298146228</v>
+      </c>
+      <c r="H826">
+        <v>676.8100000000001</v>
+      </c>
+      <c r="I826">
+        <v>0</v>
+      </c>
+      <c r="J826">
+        <v>0</v>
+      </c>
+      <c r="K826">
+        <v>6.418748893553528</v>
+      </c>
+      <c r="L826">
+        <v>0</v>
+      </c>
+      <c r="M826">
+        <v>7</v>
+      </c>
+      <c r="N826">
+        <v>0</v>
+      </c>
+      <c r="O826">
+        <v>29.7722</v>
+      </c>
+      <c r="P826">
+        <v>82.70055555555555</v>
+      </c>
+      <c r="Q826">
+        <v>36</v>
+      </c>
+      <c r="R826">
+        <v>519.62451</v>
+      </c>
+      <c r="S826">
+        <v>4.928028913026985</v>
+      </c>
+      <c r="T826">
+        <v>1046.22</v>
+      </c>
+      <c r="U826">
+        <v>20</v>
+      </c>
+      <c r="V826">
+        <v>19</v>
+      </c>
+      <c r="W826">
+        <v>39</v>
+      </c>
+      <c r="X826">
+        <v>55</v>
+      </c>
+      <c r="Y826">
+        <v>20</v>
+      </c>
+      <c r="Z826">
+        <v>43</v>
+      </c>
+      <c r="AA826">
+        <v>19</v>
+      </c>
+      <c r="AB826">
+        <v>28</v>
+      </c>
+      <c r="AC826">
+        <v>4.28832</v>
+      </c>
+      <c r="AD826">
+        <v>-2.43772</v>
+      </c>
+      <c r="AE826">
+        <v>0</v>
+      </c>
+      <c r="AF826">
+        <v>1239.112</v>
+      </c>
+      <c r="AG826">
+        <v>0</v>
+      </c>
+      <c r="AH826">
+        <v>3</v>
+      </c>
+      <c r="AI826">
+        <v>1558.87353</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B827" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E827">
+        <v>102.35</v>
+      </c>
+      <c r="F827">
+        <v>5071.49</v>
+      </c>
+      <c r="G827">
+        <v>49.5504640937958</v>
+      </c>
+      <c r="H827">
+        <v>191.92</v>
+      </c>
+      <c r="I827">
+        <v>0</v>
+      </c>
+      <c r="J827">
+        <v>0</v>
+      </c>
+      <c r="K827">
+        <v>1.875134342940889</v>
+      </c>
+      <c r="L827">
+        <v>0</v>
+      </c>
+      <c r="M827">
+        <v>1</v>
+      </c>
+      <c r="N827">
+        <v>0</v>
+      </c>
+      <c r="O827">
+        <v>25.26504</v>
+      </c>
+      <c r="P827">
+        <v>72.20233196159123</v>
+      </c>
+      <c r="Q827">
+        <v>34.992</v>
+      </c>
+      <c r="R827">
+        <v>452.81771</v>
+      </c>
+      <c r="S827">
+        <v>4.42420820713239</v>
+      </c>
+      <c r="T827">
+        <v>886.66002</v>
+      </c>
+      <c r="U827">
+        <v>21</v>
+      </c>
+      <c r="V827">
+        <v>22</v>
+      </c>
+      <c r="W827">
+        <v>43</v>
+      </c>
+      <c r="X827">
+        <v>64</v>
+      </c>
+      <c r="Y827">
+        <v>21</v>
+      </c>
+      <c r="Z827">
+        <v>63</v>
+      </c>
+      <c r="AA827">
+        <v>22</v>
+      </c>
+      <c r="AB827">
+        <v>17</v>
+      </c>
+      <c r="AC827">
+        <v>4.15261</v>
+      </c>
+      <c r="AD827">
+        <v>-3.62536</v>
+      </c>
+      <c r="AE827">
+        <v>0</v>
+      </c>
+      <c r="AF827">
+        <v>479.28</v>
+      </c>
+      <c r="AG827">
+        <v>0</v>
+      </c>
+      <c r="AH827">
+        <v>3</v>
+      </c>
+      <c r="AI827">
+        <v>1358.45313</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B828" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E828">
+        <v>102.35</v>
+      </c>
+      <c r="F828">
+        <v>4981.02</v>
+      </c>
+      <c r="G828">
+        <v>48.66653639472399</v>
+      </c>
+      <c r="H828">
+        <v>158.94</v>
+      </c>
+      <c r="I828">
+        <v>0</v>
+      </c>
+      <c r="J828">
+        <v>0</v>
+      </c>
+      <c r="K828">
+        <v>1.552906692721055</v>
+      </c>
+      <c r="L828">
+        <v>0</v>
+      </c>
+      <c r="M828">
+        <v>2</v>
+      </c>
+      <c r="N828">
+        <v>0</v>
+      </c>
+      <c r="O828">
+        <v>27.02512</v>
+      </c>
+      <c r="P828">
+        <v>81.86453410880891</v>
+      </c>
+      <c r="Q828">
+        <v>33.012</v>
+      </c>
+      <c r="R828">
+        <v>496.81937</v>
+      </c>
+      <c r="S828">
+        <v>4.854121836834392</v>
+      </c>
+      <c r="T828">
+        <v>813.14</v>
+      </c>
+      <c r="U828">
+        <v>22</v>
+      </c>
+      <c r="V828">
+        <v>16</v>
+      </c>
+      <c r="W828">
+        <v>38</v>
+      </c>
+      <c r="X828">
+        <v>80</v>
+      </c>
+      <c r="Y828">
+        <v>22</v>
+      </c>
+      <c r="Z828">
+        <v>63</v>
+      </c>
+      <c r="AA828">
+        <v>16</v>
+      </c>
+      <c r="AB828">
+        <v>22</v>
+      </c>
+      <c r="AC828">
+        <v>3.8962</v>
+      </c>
+      <c r="AD828">
+        <v>-3.82392</v>
+      </c>
+      <c r="AE828">
+        <v>0</v>
+      </c>
+      <c r="AF828">
+        <v>439.05225</v>
+      </c>
+      <c r="AG828">
+        <v>0</v>
+      </c>
+      <c r="AH828">
+        <v>3</v>
+      </c>
+      <c r="AI828">
+        <v>1490.45811</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B829" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E829">
+        <v>102.35</v>
+      </c>
+      <c r="F829">
+        <v>5695.74</v>
+      </c>
+      <c r="G829">
+        <v>55.64963361016121</v>
+      </c>
+      <c r="H829">
+        <v>145.17</v>
+      </c>
+      <c r="I829">
+        <v>0</v>
+      </c>
+      <c r="J829">
+        <v>0</v>
+      </c>
+      <c r="K829">
+        <v>1.418368343917929</v>
+      </c>
+      <c r="L829">
+        <v>0</v>
+      </c>
+      <c r="M829">
+        <v>3</v>
+      </c>
+      <c r="N829">
+        <v>0</v>
+      </c>
+      <c r="O829">
+        <v>27.6648</v>
+      </c>
+      <c r="P829">
+        <v>76.84666666666666</v>
+      </c>
+      <c r="Q829">
+        <v>36</v>
+      </c>
+      <c r="R829">
+        <v>566.63406</v>
+      </c>
+      <c r="S829">
+        <v>5.536238983878847</v>
+      </c>
+      <c r="T829">
+        <v>812.11</v>
+      </c>
+      <c r="U829">
+        <v>15</v>
+      </c>
+      <c r="V829">
+        <v>12</v>
+      </c>
+      <c r="W829">
+        <v>27</v>
+      </c>
+      <c r="X829">
+        <v>51</v>
+      </c>
+      <c r="Y829">
+        <v>15</v>
+      </c>
+      <c r="Z829">
+        <v>39</v>
+      </c>
+      <c r="AA829">
+        <v>12</v>
+      </c>
+      <c r="AB829">
+        <v>16</v>
+      </c>
+      <c r="AC829">
+        <v>4.07232</v>
+      </c>
+      <c r="AD829">
+        <v>-3.78702</v>
+      </c>
+      <c r="AE829">
+        <v>0</v>
+      </c>
+      <c r="AF829">
+        <v>1302.798</v>
+      </c>
+      <c r="AG829">
+        <v>0</v>
+      </c>
+      <c r="AH829">
+        <v>3</v>
+      </c>
+      <c r="AI829">
+        <v>1699.90218</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B830" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E830">
+        <v>102.35</v>
+      </c>
+      <c r="F830">
+        <v>4403.309999999999</v>
+      </c>
+      <c r="G830">
+        <v>43.02208109428432</v>
+      </c>
+      <c r="H830">
+        <v>132.92</v>
+      </c>
+      <c r="I830">
+        <v>0</v>
+      </c>
+      <c r="J830">
+        <v>0</v>
+      </c>
+      <c r="K830">
+        <v>1.298680996580361</v>
+      </c>
+      <c r="L830">
+        <v>0</v>
+      </c>
+      <c r="M830">
+        <v>2</v>
+      </c>
+      <c r="N830">
+        <v>0</v>
+      </c>
+      <c r="O830">
+        <v>26.19666</v>
+      </c>
+      <c r="P830">
+        <v>72.7685</v>
+      </c>
+      <c r="Q830">
+        <v>36</v>
+      </c>
+      <c r="R830">
+        <v>493.08194</v>
+      </c>
+      <c r="S830">
+        <v>4.817605666829508</v>
+      </c>
+      <c r="T830">
+        <v>668.15999</v>
+      </c>
+      <c r="U830">
+        <v>14</v>
+      </c>
+      <c r="V830">
+        <v>8</v>
+      </c>
+      <c r="W830">
+        <v>22</v>
+      </c>
+      <c r="X830">
+        <v>52</v>
+      </c>
+      <c r="Y830">
+        <v>14</v>
+      </c>
+      <c r="Z830">
+        <v>40</v>
+      </c>
+      <c r="AA830">
+        <v>8</v>
+      </c>
+      <c r="AB830">
+        <v>16</v>
+      </c>
+      <c r="AC830">
+        <v>4.1918</v>
+      </c>
+      <c r="AD830">
+        <v>-2.37487</v>
+      </c>
+      <c r="AE830">
+        <v>0</v>
+      </c>
+      <c r="AF830">
+        <v>1008.054</v>
+      </c>
+      <c r="AG830">
+        <v>0</v>
+      </c>
+      <c r="AH830">
+        <v>3</v>
+      </c>
+      <c r="AI830">
+        <v>1479.24582</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B831" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E831">
+        <v>102.35</v>
+      </c>
+      <c r="F831">
+        <v>5533.929999999999</v>
+      </c>
+      <c r="G831">
+        <v>54.06868588177821</v>
+      </c>
+      <c r="H831">
+        <v>214.6</v>
+      </c>
+      <c r="I831">
+        <v>0</v>
+      </c>
+      <c r="J831">
+        <v>0</v>
+      </c>
+      <c r="K831">
+        <v>2.096726917440157</v>
+      </c>
+      <c r="L831">
+        <v>0</v>
+      </c>
+      <c r="M831">
+        <v>3</v>
+      </c>
+      <c r="N831">
+        <v>0</v>
+      </c>
+      <c r="O831">
+        <v>28.32998</v>
+      </c>
+      <c r="P831">
+        <v>80.96130544124371</v>
+      </c>
+      <c r="Q831">
+        <v>34.992</v>
+      </c>
+      <c r="R831">
+        <v>556.35676</v>
+      </c>
+      <c r="S831">
+        <v>5.435825696140694</v>
+      </c>
+      <c r="T831">
+        <v>995.29999</v>
+      </c>
+      <c r="U831">
+        <v>34</v>
+      </c>
+      <c r="V831">
+        <v>26</v>
+      </c>
+      <c r="W831">
+        <v>60</v>
+      </c>
+      <c r="X831">
+        <v>93</v>
+      </c>
+      <c r="Y831">
+        <v>34</v>
+      </c>
+      <c r="Z831">
+        <v>78</v>
+      </c>
+      <c r="AA831">
+        <v>26</v>
+      </c>
+      <c r="AB831">
+        <v>43</v>
+      </c>
+      <c r="AC831">
+        <v>4.01664</v>
+      </c>
+      <c r="AD831">
+        <v>-4.68456</v>
+      </c>
+      <c r="AE831">
+        <v>0</v>
+      </c>
+      <c r="AF831">
+        <v>536.904</v>
+      </c>
+      <c r="AG831">
+        <v>0</v>
+      </c>
+      <c r="AH831">
+        <v>3</v>
+      </c>
+      <c r="AI831">
+        <v>1669.07028</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B832" s="2">
+        <v>46232</v>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>MD-4</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Sesión 44</t>
+        </is>
+      </c>
+      <c r="E832">
+        <v>50.61666666666667</v>
+      </c>
+      <c r="F832">
+        <v>1017.64</v>
+      </c>
+      <c r="G832">
+        <v>20.10484030293053</v>
+      </c>
+      <c r="H832">
+        <v>5.53</v>
+      </c>
+      <c r="I832">
+        <v>0</v>
+      </c>
+      <c r="J832">
+        <v>0</v>
+      </c>
+      <c r="K832">
+        <v>0.1092525518603885</v>
+      </c>
+      <c r="L832">
+        <v>0</v>
+      </c>
+      <c r="M832">
+        <v>0</v>
+      </c>
+      <c r="N832">
+        <v>0</v>
+      </c>
+      <c r="O832">
+        <v>21.42611</v>
+      </c>
+      <c r="P832">
+        <v>63.04764006591337</v>
+      </c>
+      <c r="Q832">
+        <v>33.984</v>
+      </c>
+      <c r="R832">
+        <v>119.55554</v>
+      </c>
+      <c r="S832">
+        <v>2.361979716825815</v>
+      </c>
+      <c r="T832">
+        <v>140.50999</v>
+      </c>
+      <c r="U832">
+        <v>11</v>
+      </c>
+      <c r="V832">
+        <v>0</v>
+      </c>
+      <c r="W832">
+        <v>11</v>
+      </c>
+      <c r="X832">
+        <v>19</v>
+      </c>
+      <c r="Y832">
+        <v>11</v>
+      </c>
+      <c r="Z832">
+        <v>1</v>
+      </c>
+      <c r="AA832">
+        <v>0</v>
+      </c>
+      <c r="AB832">
+        <v>2</v>
+      </c>
+      <c r="AC832">
+        <v>4.14133</v>
+      </c>
+      <c r="AD832">
+        <v>0</v>
+      </c>
+      <c r="AE832">
+        <v>0</v>
+      </c>
+      <c r="AF832">
+        <v>80.63300000000001</v>
+      </c>
+      <c r="AG832">
+        <v>0</v>
+      </c>
+      <c r="AH832">
+        <v>3</v>
+      </c>
+      <c r="AI832">
+        <v>358.66662</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-07-31
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI832"/>
+  <dimension ref="A1:AI858"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -86218,10 +86218,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F761">
-        <v>7318.84</v>
+        <v>7318.870000000001</v>
       </c>
       <c r="G761">
-        <v>67.29080918070569</v>
+        <v>67.29108500642062</v>
       </c>
       <c r="H761">
         <v>29.18</v>
@@ -86254,10 +86254,10 @@
         <v>36</v>
       </c>
       <c r="R761">
-        <v>849.05231</v>
+        <v>849.05777</v>
       </c>
       <c r="S761">
-        <v>7.806348680480428</v>
+        <v>7.806398880760544</v>
       </c>
       <c r="T761">
         <v>903.3599800000001</v>
@@ -86296,7 +86296,7 @@
         <v>0</v>
       </c>
       <c r="AF761">
-        <v>1732.338</v>
+        <v>1732.342</v>
       </c>
       <c r="AG761">
         <v>0</v>
@@ -86305,7 +86305,7 @@
         <v>3</v>
       </c>
       <c r="AI761">
-        <v>2547.15693</v>
+        <v>2547.17331</v>
       </c>
     </row>
     <row r="762">
@@ -86331,10 +86331,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F762">
-        <v>7032.9</v>
+        <v>7032.93</v>
       </c>
       <c r="G762">
-        <v>64.66182234985121</v>
+        <v>64.66209817556614</v>
       </c>
       <c r="H762">
         <v>65.52</v>
@@ -86367,10 +86367,10 @@
         <v>32.364</v>
       </c>
       <c r="R762">
-        <v>747.36132</v>
+        <v>747.36347</v>
       </c>
       <c r="S762">
-        <v>6.871382346541299</v>
+        <v>6.871402114050869</v>
       </c>
       <c r="T762">
         <v>718.58</v>
@@ -86409,7 +86409,7 @@
         <v>0</v>
       </c>
       <c r="AF762">
-        <v>565.0519</v>
+        <v>565.054</v>
       </c>
       <c r="AG762">
         <v>0</v>
@@ -86418,7 +86418,7 @@
         <v>3</v>
       </c>
       <c r="AI762">
-        <v>2242.08396</v>
+        <v>2242.09041</v>
       </c>
     </row>
     <row r="763">
@@ -86444,10 +86444,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F763">
-        <v>8279.41</v>
+        <v>8279.439999999999</v>
       </c>
       <c r="G763">
-        <v>76.122472746887</v>
+        <v>76.12274857260192</v>
       </c>
       <c r="H763">
         <v>64.83</v>
@@ -86480,10 +86480,10 @@
         <v>36</v>
       </c>
       <c r="R763">
-        <v>781.30817</v>
+        <v>781.3103599999999</v>
       </c>
       <c r="S763">
-        <v>7.183496152231277</v>
+        <v>7.183516287508466</v>
       </c>
       <c r="T763">
         <v>940.9100099999999</v>
@@ -86522,7 +86522,7 @@
         <v>0</v>
       </c>
       <c r="AF763">
-        <v>1954.78</v>
+        <v>1954.786</v>
       </c>
       <c r="AG763">
         <v>0</v>
@@ -86531,7 +86531,7 @@
         <v>3</v>
       </c>
       <c r="AI763">
-        <v>2343.92451</v>
+        <v>2343.93108</v>
       </c>
     </row>
     <row r="764">
@@ -86557,10 +86557,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F764">
-        <v>7679.98</v>
+        <v>7680.13</v>
       </c>
       <c r="G764">
-        <v>70.61119913697199</v>
+        <v>70.61257826554662</v>
       </c>
       <c r="H764">
         <v>65.08</v>
@@ -86593,10 +86593,10 @@
         <v>32.4</v>
       </c>
       <c r="R764">
-        <v>930.8503499999999</v>
+        <v>930.8576</v>
       </c>
       <c r="S764">
-        <v>8.55841544256236</v>
+        <v>8.558482100443468</v>
       </c>
       <c r="T764">
         <v>783.96998</v>
@@ -86635,7 +86635,7 @@
         <v>0</v>
       </c>
       <c r="AF764">
-        <v>629.1732999999999</v>
+        <v>629.1817</v>
       </c>
       <c r="AG764">
         <v>0</v>
@@ -86644,7 +86644,7 @@
         <v>3</v>
       </c>
       <c r="AI764">
-        <v>2792.55105</v>
+        <v>2792.5728</v>
       </c>
     </row>
     <row r="765">
@@ -86670,10 +86670,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F765">
-        <v>6686.42</v>
+        <v>6686.48</v>
       </c>
       <c r="G765">
-        <v>61.47621922627822</v>
+        <v>61.47677087770807</v>
       </c>
       <c r="H765">
         <v>72.89</v>
@@ -86706,10 +86706,10 @@
         <v>33.984</v>
       </c>
       <c r="R765">
-        <v>889.52423</v>
+        <v>889.5292400000001</v>
       </c>
       <c r="S765">
-        <v>8.178455222759913</v>
+        <v>8.178501285654306</v>
       </c>
       <c r="T765">
         <v>606.26</v>
@@ -86748,7 +86748,7 @@
         <v>0</v>
       </c>
       <c r="AF765">
-        <v>625.0384</v>
+        <v>625.0424</v>
       </c>
       <c r="AG765">
         <v>0</v>
@@ -86757,7 +86757,7 @@
         <v>3</v>
       </c>
       <c r="AI765">
-        <v>2668.57269</v>
+        <v>2668.58772</v>
       </c>
     </row>
     <row r="766">
@@ -86783,10 +86783,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F766">
-        <v>7524.65</v>
+        <v>7524.78</v>
       </c>
       <c r="G766">
-        <v>69.18306552699568</v>
+        <v>69.18426077176035</v>
       </c>
       <c r="H766">
         <v>188.68</v>
@@ -86819,10 +86819,10 @@
         <v>35.568</v>
       </c>
       <c r="R766">
-        <v>757.71576</v>
+        <v>757.7228</v>
       </c>
       <c r="S766">
-        <v>6.966583040396209</v>
+        <v>6.966647767497311</v>
       </c>
       <c r="T766">
         <v>827.38999</v>
@@ -86861,7 +86861,7 @@
         <v>0</v>
       </c>
       <c r="AF766">
-        <v>707.9608000000001</v>
+        <v>707.972</v>
       </c>
       <c r="AG766">
         <v>0</v>
@@ -86870,7 +86870,7 @@
         <v>3</v>
       </c>
       <c r="AI766">
-        <v>2273.14728</v>
+        <v>2273.1684</v>
       </c>
     </row>
     <row r="767">
@@ -86896,10 +86896,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F767">
-        <v>8296.060000000001</v>
+        <v>8296.07</v>
       </c>
       <c r="G767">
-        <v>76.27555601867036</v>
+        <v>76.27564796057531</v>
       </c>
       <c r="H767">
         <v>69.87</v>
@@ -86932,10 +86932,10 @@
         <v>36</v>
       </c>
       <c r="R767">
-        <v>871.19006</v>
+        <v>871.19346</v>
       </c>
       <c r="S767">
-        <v>8.009887371166407</v>
+        <v>8.009918631414097</v>
       </c>
       <c r="T767">
         <v>781.3399900000001</v>
@@ -86974,7 +86974,7 @@
         <v>0</v>
       </c>
       <c r="AF767">
-        <v>1919.196</v>
+        <v>1919.2</v>
       </c>
       <c r="AG767">
         <v>0</v>
@@ -86983,7 +86983,7 @@
         <v>3</v>
       </c>
       <c r="AI767">
-        <v>2613.57018</v>
+        <v>2613.58038</v>
       </c>
     </row>
     <row r="768">
@@ -87009,10 +87009,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F768">
-        <v>8034.78</v>
+        <v>8034.969999999999</v>
       </c>
       <c r="G768">
-        <v>73.87329792548415</v>
+        <v>73.87504482167867</v>
       </c>
       <c r="H768">
         <v>192.21</v>
@@ -87045,10 +87045,10 @@
         <v>36</v>
       </c>
       <c r="R768">
-        <v>890.1092199999999</v>
+        <v>890.13109</v>
       </c>
       <c r="S768">
-        <v>8.183833732259043</v>
+        <v>8.184034809205224</v>
       </c>
       <c r="T768">
         <v>1078.08001</v>
@@ -87087,7 +87087,7 @@
         <v>0</v>
       </c>
       <c r="AF768">
-        <v>665.7546</v>
+        <v>665.7637</v>
       </c>
       <c r="AG768">
         <v>0</v>
@@ -87096,7 +87096,7 @@
         <v>3</v>
       </c>
       <c r="AI768">
-        <v>2670.32766</v>
+        <v>2670.39327</v>
       </c>
     </row>
     <row r="769">
@@ -87122,10 +87122,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F769">
-        <v>6573.449999999999</v>
+        <v>6573.589999999999</v>
       </c>
       <c r="G769">
-        <v>60.43755152577591</v>
+        <v>60.43883871244556</v>
       </c>
       <c r="H769">
         <v>77.36000000000001</v>
@@ -87158,10 +87158,10 @@
         <v>32.004</v>
       </c>
       <c r="R769">
-        <v>814.15786</v>
+        <v>814.1654</v>
       </c>
       <c r="S769">
-        <v>7.485522459875021</v>
+        <v>7.485591784071372</v>
       </c>
       <c r="T769">
         <v>694.93998</v>
@@ -87200,7 +87200,7 @@
         <v>0</v>
       </c>
       <c r="AF769">
-        <v>462.3924000000001</v>
+        <v>462.3936</v>
       </c>
       <c r="AG769">
         <v>0</v>
@@ -87209,7 +87209,7 @@
         <v>3</v>
       </c>
       <c r="AI769">
-        <v>2442.47358</v>
+        <v>2442.4962</v>
       </c>
     </row>
     <row r="770">
@@ -87235,10 +87235,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F770">
-        <v>7617.879999999999</v>
+        <v>7618.12</v>
       </c>
       <c r="G770">
-        <v>70.04023990707738</v>
+        <v>70.04244651279679</v>
       </c>
       <c r="H770">
         <v>202.99</v>
@@ -87271,10 +87271,10 @@
         <v>33.84</v>
       </c>
       <c r="R770">
-        <v>814.71582</v>
+        <v>814.71937</v>
       </c>
       <c r="S770">
-        <v>7.490652450405005</v>
+        <v>7.490685089781271</v>
       </c>
       <c r="T770">
         <v>924.36001</v>
@@ -87313,7 +87313,7 @@
         <v>0</v>
       </c>
       <c r="AF770">
-        <v>634.0684</v>
+        <v>634.0712</v>
       </c>
       <c r="AG770">
         <v>0</v>
@@ -87322,7 +87322,7 @@
         <v>3</v>
       </c>
       <c r="AI770">
-        <v>2444.14746</v>
+        <v>2444.15811</v>
       </c>
     </row>
     <row r="771">
@@ -87348,10 +87348,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F771">
-        <v>6946.619999999999</v>
+        <v>6946.82</v>
       </c>
       <c r="G771">
-        <v>63.86854759372711</v>
+        <v>63.87038643182661</v>
       </c>
       <c r="H771">
         <v>29.86</v>
@@ -87384,10 +87384,10 @@
         <v>33.696</v>
       </c>
       <c r="R771">
-        <v>786.56354</v>
+        <v>786.57457</v>
       </c>
       <c r="S771">
-        <v>7.231815025146111</v>
+        <v>7.231916437067299</v>
       </c>
       <c r="T771">
         <v>688.54</v>
@@ -87426,7 +87426,7 @@
         <v>0</v>
       </c>
       <c r="AF771">
-        <v>649.8856000000001</v>
+        <v>649.9015999999999</v>
       </c>
       <c r="AG771">
         <v>0</v>
@@ -87435,7 +87435,7 @@
         <v>3</v>
       </c>
       <c r="AI771">
-        <v>2359.69062</v>
+        <v>2359.72371</v>
       </c>
     </row>
     <row r="772">
@@ -87461,10 +87461,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F772">
-        <v>7358.84</v>
+        <v>7358.849999999999</v>
       </c>
       <c r="G772">
-        <v>67.6585768006056</v>
+        <v>67.65866874251057</v>
       </c>
       <c r="H772">
         <v>110.61</v>
@@ -87497,10 +87497,10 @@
         <v>36</v>
       </c>
       <c r="R772">
-        <v>931.58859</v>
+        <v>931.58942</v>
       </c>
       <c r="S772">
-        <v>8.565202961755233</v>
+        <v>8.565210592933346</v>
       </c>
       <c r="T772">
         <v>747.41998</v>
@@ -87539,7 +87539,7 @@
         <v>0</v>
       </c>
       <c r="AF772">
-        <v>1706.154</v>
+        <v>1706.156</v>
       </c>
       <c r="AG772">
         <v>0</v>
@@ -87548,7 +87548,7 @@
         <v>3</v>
       </c>
       <c r="AI772">
-        <v>2794.76577</v>
+        <v>2794.76826</v>
       </c>
     </row>
     <row r="773">
@@ -87574,10 +87574,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F773">
-        <v>6445.15</v>
+        <v>6445.25</v>
       </c>
       <c r="G773">
-        <v>59.25793688494696</v>
+        <v>59.25885630399672</v>
       </c>
       <c r="H773">
         <v>165.19</v>
@@ -87610,10 +87610,10 @@
         <v>34.992</v>
       </c>
       <c r="R773">
-        <v>631.40715</v>
+        <v>631.41275</v>
       </c>
       <c r="S773">
-        <v>5.805277618582072</v>
+        <v>5.805329106048858</v>
       </c>
       <c r="T773">
         <v>684.11001</v>
@@ -87652,7 +87652,7 @@
         <v>0</v>
       </c>
       <c r="AF773">
-        <v>516.67269</v>
+        <v>516.68028</v>
       </c>
       <c r="AG773">
         <v>0</v>
@@ -87661,7 +87661,7 @@
         <v>3</v>
       </c>
       <c r="AI773">
-        <v>1894.22145</v>
+        <v>1894.23825</v>
       </c>
     </row>
     <row r="774">
@@ -87687,10 +87687,10 @@
         <v>126.9276666666667</v>
       </c>
       <c r="F774">
-        <v>7425.18</v>
+        <v>7425.219999999999</v>
       </c>
       <c r="G774">
-        <v>58.49930275248633</v>
+        <v>58.49961789260549</v>
       </c>
       <c r="H774">
         <v>136.17</v>
@@ -87723,10 +87723,10 @@
         <v>34.92</v>
       </c>
       <c r="R774">
-        <v>799.74793</v>
+        <v>799.74924</v>
       </c>
       <c r="S774">
-        <v>6.300816449263754</v>
+        <v>6.300826770102657</v>
       </c>
       <c r="T774">
         <v>686.6299799999999</v>
@@ -87765,7 +87765,7 @@
         <v>0</v>
       </c>
       <c r="AF774">
-        <v>674.0672</v>
+        <v>674.0712</v>
       </c>
       <c r="AG774">
         <v>0</v>
@@ -87774,7 +87774,7 @@
         <v>3</v>
       </c>
       <c r="AI774">
-        <v>2399.24379</v>
+        <v>2399.24772</v>
       </c>
     </row>
     <row r="775">
@@ -87800,10 +87800,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F775">
-        <v>7039.77</v>
+        <v>7039.9</v>
       </c>
       <c r="G775">
-        <v>64.72498643856902</v>
+        <v>64.72618168333369</v>
       </c>
       <c r="H775">
         <v>68.12</v>
@@ -87836,10 +87836,10 @@
         <v>34.992</v>
       </c>
       <c r="R775">
-        <v>671.62211</v>
+        <v>671.63045</v>
       </c>
       <c r="S775">
-        <v>6.175021621671321</v>
+        <v>6.17509830122007</v>
       </c>
       <c r="T775">
         <v>827.5</v>
@@ -87878,7 +87878,7 @@
         <v>0</v>
       </c>
       <c r="AF775">
-        <v>594.99988</v>
+        <v>595.01124</v>
       </c>
       <c r="AG775">
         <v>0</v>
@@ -87887,7 +87887,7 @@
         <v>3</v>
       </c>
       <c r="AI775">
-        <v>2014.86633</v>
+        <v>2014.89135</v>
       </c>
     </row>
     <row r="776">
@@ -87913,10 +87913,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F776">
-        <v>7697.5</v>
+        <v>7697.54</v>
       </c>
       <c r="G776">
-        <v>70.77228135448814</v>
+        <v>70.77264912210805</v>
       </c>
       <c r="H776">
         <v>54.61</v>
@@ -87949,10 +87949,10 @@
         <v>36</v>
       </c>
       <c r="R776">
-        <v>899.72492</v>
+        <v>899.72748</v>
       </c>
       <c r="S776">
-        <v>8.272242309825831</v>
+        <v>8.272265846953506</v>
       </c>
       <c r="T776">
         <v>809.26003</v>
@@ -87991,7 +87991,7 @@
         <v>0</v>
       </c>
       <c r="AF776">
-        <v>1803.476</v>
+        <v>1803.484</v>
       </c>
       <c r="AG776">
         <v>0</v>
@@ -88000,7 +88000,7 @@
         <v>3</v>
       </c>
       <c r="AI776">
-        <v>2699.17476</v>
+        <v>2699.18244</v>
       </c>
     </row>
     <row r="777">
@@ -88026,10 +88026,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F777">
-        <v>6973.5</v>
+        <v>6973.68</v>
       </c>
       <c r="G777">
-        <v>64.11568743429986</v>
+        <v>64.11734238858941</v>
       </c>
       <c r="H777">
         <v>63.22</v>
@@ -88062,10 +88062,10 @@
         <v>33.984</v>
       </c>
       <c r="R777">
-        <v>765.57813</v>
+        <v>765.5856299999999</v>
       </c>
       <c r="S777">
-        <v>7.038871167938019</v>
+        <v>7.03894012436675</v>
       </c>
       <c r="T777">
         <v>723.81999</v>
@@ -88104,7 +88104,7 @@
         <v>0</v>
       </c>
       <c r="AF777">
-        <v>649.2</v>
+        <v>649.2144</v>
       </c>
       <c r="AG777">
         <v>0</v>
@@ -88113,7 +88113,7 @@
         <v>3</v>
       </c>
       <c r="AI777">
-        <v>2296.73439</v>
+        <v>2296.75689</v>
       </c>
     </row>
     <row r="778">
@@ -88252,10 +88252,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F779">
-        <v>7577.369999999999</v>
+        <v>7577.590000000001</v>
       </c>
       <c r="G779">
-        <v>69.66778325002375</v>
+        <v>69.66980597193322</v>
       </c>
       <c r="H779">
         <v>35.31</v>
@@ -88288,10 +88288,10 @@
         <v>34.992</v>
       </c>
       <c r="R779">
-        <v>763.44659</v>
+        <v>763.45298</v>
       </c>
       <c r="S779">
-        <v>7.019273383124983</v>
+        <v>7.019332134002262</v>
       </c>
       <c r="T779">
         <v>817.3299999999999</v>
@@ -88330,7 +88330,7 @@
         <v>0</v>
       </c>
       <c r="AF779">
-        <v>714.056</v>
+        <v>714.0688</v>
       </c>
       <c r="AG779">
         <v>0</v>
@@ -88339,7 +88339,7 @@
         <v>3</v>
       </c>
       <c r="AI779">
-        <v>2290.33977</v>
+        <v>2290.35894</v>
       </c>
     </row>
     <row r="780">
@@ -88365,10 +88365,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F780">
-        <v>6818.27</v>
+        <v>6818.400000000001</v>
       </c>
       <c r="G780">
-        <v>62.68847324337329</v>
+        <v>62.68966848813797</v>
       </c>
       <c r="H780">
         <v>67.19</v>
@@ -88401,10 +88401,10 @@
         <v>33.012</v>
       </c>
       <c r="R780">
-        <v>731.84006</v>
+        <v>731.8486700000001</v>
       </c>
       <c r="S780">
-        <v>6.728676925340109</v>
+        <v>6.728756087320293</v>
       </c>
       <c r="T780">
         <v>684.40002</v>
@@ -88443,7 +88443,7 @@
         <v>0</v>
       </c>
       <c r="AF780">
-        <v>587.6745</v>
+        <v>587.68425</v>
       </c>
       <c r="AG780">
         <v>0</v>
@@ -88452,7 +88452,7 @@
         <v>3</v>
       </c>
       <c r="AI780">
-        <v>2195.52018</v>
+        <v>2195.54601</v>
       </c>
     </row>
     <row r="781">
@@ -88478,10 +88478,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F781">
-        <v>6806.549999999999</v>
+        <v>6806.599999999999</v>
       </c>
       <c r="G781">
-        <v>62.58071733074262</v>
+        <v>62.58117704026749</v>
       </c>
       <c r="H781">
         <v>26.5</v>
@@ -88514,10 +88514,10 @@
         <v>32.004</v>
       </c>
       <c r="R781">
-        <v>720.69672</v>
+        <v>720.70066</v>
       </c>
       <c r="S781">
-        <v>6.626222934601723</v>
+        <v>6.626259159712284</v>
       </c>
       <c r="T781">
         <v>564.72999</v>
@@ -88556,7 +88556,7 @@
         <v>0</v>
       </c>
       <c r="AF781">
-        <v>547.4056</v>
+        <v>547.4084</v>
       </c>
       <c r="AG781">
         <v>0</v>
@@ -88565,7 +88565,7 @@
         <v>3</v>
       </c>
       <c r="AI781">
-        <v>2162.09016</v>
+        <v>2162.10198</v>
       </c>
     </row>
     <row r="782">
@@ -88591,10 +88591,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F782">
-        <v>8414.51</v>
+        <v>8414.550000000001</v>
       </c>
       <c r="G782">
-        <v>77.36460788309894</v>
+        <v>77.36497565071885</v>
       </c>
       <c r="H782">
         <v>40.94</v>
@@ -88627,10 +88627,10 @@
         <v>36</v>
       </c>
       <c r="R782">
-        <v>955.7971500000001</v>
+        <v>955.8059500000001</v>
       </c>
       <c r="S782">
-        <v>8.787781074065336</v>
+        <v>8.787861982941713</v>
       </c>
       <c r="T782">
         <v>918.66002</v>
@@ -88669,7 +88669,7 @@
         <v>0</v>
       </c>
       <c r="AF782">
-        <v>2001.41</v>
+        <v>2001.422</v>
       </c>
       <c r="AG782">
         <v>0</v>
@@ -88678,7 +88678,7 @@
         <v>3</v>
       </c>
       <c r="AI782">
-        <v>2867.39145</v>
+        <v>2867.41785</v>
       </c>
     </row>
     <row r="783">
@@ -88704,10 +88704,10 @@
         <v>108.7643333333333</v>
       </c>
       <c r="F783">
-        <v>8064.029999999999</v>
+        <v>8064.22</v>
       </c>
       <c r="G783">
-        <v>74.14222799753595</v>
+        <v>74.14397489373049</v>
       </c>
       <c r="H783">
         <v>27.38</v>
@@ -88740,10 +88740,10 @@
         <v>36</v>
       </c>
       <c r="R783">
-        <v>921.29556</v>
+        <v>921.32139</v>
       </c>
       <c r="S783">
-        <v>8.470566883138774</v>
+        <v>8.470804369079325</v>
       </c>
       <c r="T783">
         <v>825.04002</v>
@@ -88782,7 +88782,7 @@
         <v>0</v>
       </c>
       <c r="AF783">
-        <v>1882.86</v>
+        <v>1882.898</v>
       </c>
       <c r="AG783">
         <v>0</v>
@@ -88791,7 +88791,7 @@
         <v>3</v>
       </c>
       <c r="AI783">
-        <v>2763.88668</v>
+        <v>2763.96417</v>
       </c>
     </row>
     <row r="784">
@@ -88853,10 +88853,10 @@
         <v>34.992</v>
       </c>
       <c r="R784">
-        <v>786.8002899999999</v>
+        <v>786.80397</v>
       </c>
       <c r="S784">
-        <v>7.233991749746393</v>
+        <v>7.234025584367425</v>
       </c>
       <c r="T784">
         <v>794.1700000000001</v>
@@ -88904,7 +88904,7 @@
         <v>3</v>
       </c>
       <c r="AI784">
-        <v>2360.400869999999</v>
+        <v>2360.41191</v>
       </c>
     </row>
     <row r="785">
@@ -88930,10 +88930,10 @@
         <v>84.79616666666668</v>
       </c>
       <c r="F785">
-        <v>3300</v>
+        <v>3300.08</v>
       </c>
       <c r="G785">
-        <v>38.91685355273528</v>
+        <v>38.91779699160929</v>
       </c>
       <c r="H785">
         <v>1.6</v>
@@ -88966,10 +88966,10 @@
         <v>33.984</v>
       </c>
       <c r="R785">
-        <v>328.50216</v>
+        <v>328.5051</v>
       </c>
       <c r="S785">
-        <v>3.874021349235519</v>
+        <v>3.874056020614138</v>
       </c>
       <c r="T785">
         <v>180.75</v>
@@ -89008,7 +89008,7 @@
         <v>0</v>
       </c>
       <c r="AF785">
-        <v>262.8073</v>
+        <v>262.8129</v>
       </c>
       <c r="AG785">
         <v>0</v>
@@ -89017,7 +89017,7 @@
         <v>3</v>
       </c>
       <c r="AI785">
-        <v>985.50648</v>
+        <v>985.5152999999999</v>
       </c>
     </row>
     <row r="786">
@@ -94329,6 +94329,2944 @@
       </c>
       <c r="AI832">
         <v>358.66662</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B833" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E833">
+        <v>60.1525</v>
+      </c>
+      <c r="F833">
+        <v>6817.15</v>
+      </c>
+      <c r="G833">
+        <v>113.3311167449399</v>
+      </c>
+      <c r="H833">
+        <v>97.93000000000001</v>
+      </c>
+      <c r="I833">
+        <v>0</v>
+      </c>
+      <c r="J833">
+        <v>0</v>
+      </c>
+      <c r="K833">
+        <v>1.628028760234404</v>
+      </c>
+      <c r="L833">
+        <v>0</v>
+      </c>
+      <c r="M833">
+        <v>1</v>
+      </c>
+      <c r="N833">
+        <v>0</v>
+      </c>
+      <c r="O833">
+        <v>26.38973</v>
+      </c>
+      <c r="P833">
+        <v>81.54038437770363</v>
+      </c>
+      <c r="Q833">
+        <v>32.364</v>
+      </c>
+      <c r="R833">
+        <v>679.40405</v>
+      </c>
+      <c r="S833">
+        <v>11.29469348738623</v>
+      </c>
+      <c r="T833">
+        <v>900.2800100000001</v>
+      </c>
+      <c r="U833">
+        <v>8</v>
+      </c>
+      <c r="V833">
+        <v>5</v>
+      </c>
+      <c r="W833">
+        <v>13</v>
+      </c>
+      <c r="X833">
+        <v>58</v>
+      </c>
+      <c r="Y833">
+        <v>8</v>
+      </c>
+      <c r="Z833">
+        <v>43</v>
+      </c>
+      <c r="AA833">
+        <v>5</v>
+      </c>
+      <c r="AB833">
+        <v>10</v>
+      </c>
+      <c r="AC833">
+        <v>3.61761</v>
+      </c>
+      <c r="AD833">
+        <v>-2.73828</v>
+      </c>
+      <c r="AE833">
+        <v>0</v>
+      </c>
+      <c r="AF833">
+        <v>545.6794</v>
+      </c>
+      <c r="AG833">
+        <v>0</v>
+      </c>
+      <c r="AH833">
+        <v>3</v>
+      </c>
+      <c r="AI833">
+        <v>2038.21215</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B834" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E834">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F834">
+        <v>6385.5</v>
+      </c>
+      <c r="G834">
+        <v>110.5210322565757</v>
+      </c>
+      <c r="H834">
+        <v>339.7400000000001</v>
+      </c>
+      <c r="I834">
+        <v>0</v>
+      </c>
+      <c r="J834">
+        <v>0</v>
+      </c>
+      <c r="K834">
+        <v>5.880262391175165</v>
+      </c>
+      <c r="L834">
+        <v>10.71</v>
+      </c>
+      <c r="M834">
+        <v>6</v>
+      </c>
+      <c r="N834">
+        <v>1</v>
+      </c>
+      <c r="O834">
+        <v>30.70119</v>
+      </c>
+      <c r="P834">
+        <v>85.28108333333333</v>
+      </c>
+      <c r="Q834">
+        <v>36</v>
+      </c>
+      <c r="R834">
+        <v>522.53585</v>
+      </c>
+      <c r="S834">
+        <v>9.044115814433821</v>
+      </c>
+      <c r="T834">
+        <v>1175.26001</v>
+      </c>
+      <c r="U834">
+        <v>23</v>
+      </c>
+      <c r="V834">
+        <v>32</v>
+      </c>
+      <c r="W834">
+        <v>55</v>
+      </c>
+      <c r="X834">
+        <v>95</v>
+      </c>
+      <c r="Y834">
+        <v>23</v>
+      </c>
+      <c r="Z834">
+        <v>85</v>
+      </c>
+      <c r="AA834">
+        <v>32</v>
+      </c>
+      <c r="AB834">
+        <v>24</v>
+      </c>
+      <c r="AC834">
+        <v>3.77655</v>
+      </c>
+      <c r="AD834">
+        <v>-3.73887</v>
+      </c>
+      <c r="AE834">
+        <v>0</v>
+      </c>
+      <c r="AF834">
+        <v>1541.694</v>
+      </c>
+      <c r="AG834">
+        <v>0</v>
+      </c>
+      <c r="AH834">
+        <v>3</v>
+      </c>
+      <c r="AI834">
+        <v>1567.60755</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B835" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E835">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F835">
+        <v>7312.88</v>
+      </c>
+      <c r="G835">
+        <v>126.5722412291076</v>
+      </c>
+      <c r="H835">
+        <v>149.23</v>
+      </c>
+      <c r="I835">
+        <v>0</v>
+      </c>
+      <c r="J835">
+        <v>0</v>
+      </c>
+      <c r="K835">
+        <v>2.582891495364307</v>
+      </c>
+      <c r="L835">
+        <v>0</v>
+      </c>
+      <c r="M835">
+        <v>4</v>
+      </c>
+      <c r="N835">
+        <v>0</v>
+      </c>
+      <c r="O835">
+        <v>28.41665</v>
+      </c>
+      <c r="P835">
+        <v>87.70570987654321</v>
+      </c>
+      <c r="Q835">
+        <v>32.4</v>
+      </c>
+      <c r="R835">
+        <v>790.33627</v>
+      </c>
+      <c r="S835">
+        <v>13.67923896174328</v>
+      </c>
+      <c r="T835">
+        <v>1096.50998</v>
+      </c>
+      <c r="U835">
+        <v>17</v>
+      </c>
+      <c r="V835">
+        <v>7</v>
+      </c>
+      <c r="W835">
+        <v>24</v>
+      </c>
+      <c r="X835">
+        <v>87</v>
+      </c>
+      <c r="Y835">
+        <v>17</v>
+      </c>
+      <c r="Z835">
+        <v>50</v>
+      </c>
+      <c r="AA835">
+        <v>7</v>
+      </c>
+      <c r="AB835">
+        <v>8</v>
+      </c>
+      <c r="AC835">
+        <v>4.40211</v>
+      </c>
+      <c r="AD835">
+        <v>-2.55282</v>
+      </c>
+      <c r="AE835">
+        <v>0</v>
+      </c>
+      <c r="AF835">
+        <v>598.1094000000001</v>
+      </c>
+      <c r="AG835">
+        <v>0</v>
+      </c>
+      <c r="AH835">
+        <v>3</v>
+      </c>
+      <c r="AI835">
+        <v>2371.00881</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B836" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E836">
+        <v>60.1525</v>
+      </c>
+      <c r="F836">
+        <v>5742.49</v>
+      </c>
+      <c r="G836">
+        <v>95.46552512364407</v>
+      </c>
+      <c r="H836">
+        <v>315.35</v>
+      </c>
+      <c r="I836">
+        <v>0</v>
+      </c>
+      <c r="J836">
+        <v>0</v>
+      </c>
+      <c r="K836">
+        <v>5.242508623914218</v>
+      </c>
+      <c r="L836">
+        <v>0</v>
+      </c>
+      <c r="M836">
+        <v>7</v>
+      </c>
+      <c r="N836">
+        <v>0</v>
+      </c>
+      <c r="O836">
+        <v>29.47658</v>
+      </c>
+      <c r="P836">
+        <v>86.73664077212806</v>
+      </c>
+      <c r="Q836">
+        <v>33.984</v>
+      </c>
+      <c r="R836">
+        <v>681.19969</v>
+      </c>
+      <c r="S836">
+        <v>11.32454494825652</v>
+      </c>
+      <c r="T836">
+        <v>903.48999</v>
+      </c>
+      <c r="U836">
+        <v>18</v>
+      </c>
+      <c r="V836">
+        <v>26</v>
+      </c>
+      <c r="W836">
+        <v>44</v>
+      </c>
+      <c r="X836">
+        <v>71</v>
+      </c>
+      <c r="Y836">
+        <v>18</v>
+      </c>
+      <c r="Z836">
+        <v>61</v>
+      </c>
+      <c r="AA836">
+        <v>26</v>
+      </c>
+      <c r="AB836">
+        <v>14</v>
+      </c>
+      <c r="AC836">
+        <v>4.07379</v>
+      </c>
+      <c r="AD836">
+        <v>-3.46121</v>
+      </c>
+      <c r="AE836">
+        <v>0</v>
+      </c>
+      <c r="AF836">
+        <v>543.848</v>
+      </c>
+      <c r="AG836">
+        <v>0</v>
+      </c>
+      <c r="AH836">
+        <v>3</v>
+      </c>
+      <c r="AI836">
+        <v>2043.59907</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B837" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E837">
+        <v>60.1525</v>
+      </c>
+      <c r="F837">
+        <v>6284.02</v>
+      </c>
+      <c r="G837">
+        <v>104.4681434686838</v>
+      </c>
+      <c r="H837">
+        <v>254.53</v>
+      </c>
+      <c r="I837">
+        <v>12.4</v>
+      </c>
+      <c r="J837">
+        <v>1</v>
+      </c>
+      <c r="K837">
+        <v>4.231411828269814</v>
+      </c>
+      <c r="L837">
+        <v>21.08</v>
+      </c>
+      <c r="M837">
+        <v>7</v>
+      </c>
+      <c r="N837">
+        <v>1</v>
+      </c>
+      <c r="O837">
+        <v>33.26341</v>
+      </c>
+      <c r="P837">
+        <v>93.52060841205578</v>
+      </c>
+      <c r="Q837">
+        <v>35.568</v>
+      </c>
+      <c r="R837">
+        <v>572.64649</v>
+      </c>
+      <c r="S837">
+        <v>9.519911724367233</v>
+      </c>
+      <c r="T837">
+        <v>882.21002</v>
+      </c>
+      <c r="U837">
+        <v>26</v>
+      </c>
+      <c r="V837">
+        <v>17</v>
+      </c>
+      <c r="W837">
+        <v>43</v>
+      </c>
+      <c r="X837">
+        <v>75</v>
+      </c>
+      <c r="Y837">
+        <v>26</v>
+      </c>
+      <c r="Z837">
+        <v>58</v>
+      </c>
+      <c r="AA837">
+        <v>17</v>
+      </c>
+      <c r="AB837">
+        <v>17</v>
+      </c>
+      <c r="AC837">
+        <v>4.19317</v>
+      </c>
+      <c r="AD837">
+        <v>-3.44908</v>
+      </c>
+      <c r="AE837">
+        <v>0</v>
+      </c>
+      <c r="AF837">
+        <v>594.0232000000001</v>
+      </c>
+      <c r="AG837">
+        <v>0</v>
+      </c>
+      <c r="AH837">
+        <v>3</v>
+      </c>
+      <c r="AI837">
+        <v>1717.93947</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B838" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E838">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F838">
+        <v>6903.85</v>
+      </c>
+      <c r="G838">
+        <v>101.55607966971</v>
+      </c>
+      <c r="H838">
+        <v>441.67</v>
+      </c>
+      <c r="I838">
+        <v>0</v>
+      </c>
+      <c r="J838">
+        <v>0</v>
+      </c>
+      <c r="K838">
+        <v>6.496994243461376</v>
+      </c>
+      <c r="L838">
+        <v>40.16</v>
+      </c>
+      <c r="M838">
+        <v>13</v>
+      </c>
+      <c r="N838">
+        <v>3</v>
+      </c>
+      <c r="O838">
+        <v>32.18144</v>
+      </c>
+      <c r="P838">
+        <v>89.3928888888889</v>
+      </c>
+      <c r="Q838">
+        <v>36</v>
+      </c>
+      <c r="R838">
+        <v>685.3926300000001</v>
+      </c>
+      <c r="S838">
+        <v>10.08216988163301</v>
+      </c>
+      <c r="T838">
+        <v>1070.09</v>
+      </c>
+      <c r="U838">
+        <v>12</v>
+      </c>
+      <c r="V838">
+        <v>19</v>
+      </c>
+      <c r="W838">
+        <v>31</v>
+      </c>
+      <c r="X838">
+        <v>66</v>
+      </c>
+      <c r="Y838">
+        <v>12</v>
+      </c>
+      <c r="Z838">
+        <v>70</v>
+      </c>
+      <c r="AA838">
+        <v>19</v>
+      </c>
+      <c r="AB838">
+        <v>21</v>
+      </c>
+      <c r="AC838">
+        <v>4.2151</v>
+      </c>
+      <c r="AD838">
+        <v>-3.06845</v>
+      </c>
+      <c r="AE838">
+        <v>0</v>
+      </c>
+      <c r="AF838">
+        <v>1623.068</v>
+      </c>
+      <c r="AG838">
+        <v>0</v>
+      </c>
+      <c r="AH838">
+        <v>3</v>
+      </c>
+      <c r="AI838">
+        <v>2056.17789</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B839" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E839">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F839">
+        <v>7255.26</v>
+      </c>
+      <c r="G839">
+        <v>106.725343480009</v>
+      </c>
+      <c r="H839">
+        <v>376.52</v>
+      </c>
+      <c r="I839">
+        <v>0</v>
+      </c>
+      <c r="J839">
+        <v>0</v>
+      </c>
+      <c r="K839">
+        <v>5.538633533063322</v>
+      </c>
+      <c r="L839">
+        <v>0</v>
+      </c>
+      <c r="M839">
+        <v>8</v>
+      </c>
+      <c r="N839">
+        <v>0</v>
+      </c>
+      <c r="O839">
+        <v>29.45743</v>
+      </c>
+      <c r="P839">
+        <v>81.82619444444444</v>
+      </c>
+      <c r="Q839">
+        <v>36</v>
+      </c>
+      <c r="R839">
+        <v>644.98884</v>
+      </c>
+      <c r="S839">
+        <v>9.487827519588903</v>
+      </c>
+      <c r="T839">
+        <v>1121.69</v>
+      </c>
+      <c r="U839">
+        <v>17</v>
+      </c>
+      <c r="V839">
+        <v>25</v>
+      </c>
+      <c r="W839">
+        <v>42</v>
+      </c>
+      <c r="X839">
+        <v>84</v>
+      </c>
+      <c r="Y839">
+        <v>17</v>
+      </c>
+      <c r="Z839">
+        <v>66</v>
+      </c>
+      <c r="AA839">
+        <v>25</v>
+      </c>
+      <c r="AB839">
+        <v>25</v>
+      </c>
+      <c r="AC839">
+        <v>4.36079</v>
+      </c>
+      <c r="AD839">
+        <v>-3.98068</v>
+      </c>
+      <c r="AE839">
+        <v>0</v>
+      </c>
+      <c r="AF839">
+        <v>597.9869</v>
+      </c>
+      <c r="AG839">
+        <v>0</v>
+      </c>
+      <c r="AH839">
+        <v>3</v>
+      </c>
+      <c r="AI839">
+        <v>1934.96652</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B840" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E840">
+        <v>60.1525</v>
+      </c>
+      <c r="F840">
+        <v>6415.6</v>
+      </c>
+      <c r="G840">
+        <v>106.6555837246997</v>
+      </c>
+      <c r="H840">
+        <v>182.54</v>
+      </c>
+      <c r="I840">
+        <v>0</v>
+      </c>
+      <c r="J840">
+        <v>0</v>
+      </c>
+      <c r="K840">
+        <v>3.034620339969245</v>
+      </c>
+      <c r="L840">
+        <v>0</v>
+      </c>
+      <c r="M840">
+        <v>2</v>
+      </c>
+      <c r="N840">
+        <v>0</v>
+      </c>
+      <c r="O840">
+        <v>26.12295</v>
+      </c>
+      <c r="P840">
+        <v>81.6240157480315</v>
+      </c>
+      <c r="Q840">
+        <v>32.004</v>
+      </c>
+      <c r="R840">
+        <v>668.63797</v>
+      </c>
+      <c r="S840">
+        <v>11.11571372760899</v>
+      </c>
+      <c r="T840">
+        <v>879.71</v>
+      </c>
+      <c r="U840">
+        <v>16</v>
+      </c>
+      <c r="V840">
+        <v>23</v>
+      </c>
+      <c r="W840">
+        <v>39</v>
+      </c>
+      <c r="X840">
+        <v>55</v>
+      </c>
+      <c r="Y840">
+        <v>16</v>
+      </c>
+      <c r="Z840">
+        <v>57</v>
+      </c>
+      <c r="AA840">
+        <v>23</v>
+      </c>
+      <c r="AB840">
+        <v>12</v>
+      </c>
+      <c r="AC840">
+        <v>3.91235</v>
+      </c>
+      <c r="AD840">
+        <v>-4.63424</v>
+      </c>
+      <c r="AE840">
+        <v>0</v>
+      </c>
+      <c r="AF840">
+        <v>451.9242</v>
+      </c>
+      <c r="AG840">
+        <v>0</v>
+      </c>
+      <c r="AH840">
+        <v>3</v>
+      </c>
+      <c r="AI840">
+        <v>2005.91391</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>Esteban Lozano</t>
+        </is>
+      </c>
+      <c r="B841" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E841">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F841">
+        <v>7418.43</v>
+      </c>
+      <c r="G841">
+        <v>109.1255847250689</v>
+      </c>
+      <c r="H841">
+        <v>356.9</v>
+      </c>
+      <c r="I841">
+        <v>0</v>
+      </c>
+      <c r="J841">
+        <v>0</v>
+      </c>
+      <c r="K841">
+        <v>5.25002206509694</v>
+      </c>
+      <c r="L841">
+        <v>0</v>
+      </c>
+      <c r="M841">
+        <v>9</v>
+      </c>
+      <c r="N841">
+        <v>0</v>
+      </c>
+      <c r="O841">
+        <v>29.35965</v>
+      </c>
+      <c r="P841">
+        <v>94.83091085271317</v>
+      </c>
+      <c r="Q841">
+        <v>30.96</v>
+      </c>
+      <c r="R841">
+        <v>660.77341</v>
+      </c>
+      <c r="S841">
+        <v>9.720019564385954</v>
+      </c>
+      <c r="T841">
+        <v>1039.98001</v>
+      </c>
+      <c r="U841">
+        <v>19</v>
+      </c>
+      <c r="V841">
+        <v>22</v>
+      </c>
+      <c r="W841">
+        <v>41</v>
+      </c>
+      <c r="X841">
+        <v>81</v>
+      </c>
+      <c r="Y841">
+        <v>19</v>
+      </c>
+      <c r="Z841">
+        <v>67</v>
+      </c>
+      <c r="AA841">
+        <v>22</v>
+      </c>
+      <c r="AB841">
+        <v>25</v>
+      </c>
+      <c r="AC841">
+        <v>4.2324</v>
+      </c>
+      <c r="AD841">
+        <v>-4.13212</v>
+      </c>
+      <c r="AE841">
+        <v>0</v>
+      </c>
+      <c r="AF841">
+        <v>614.1947</v>
+      </c>
+      <c r="AG841">
+        <v>0</v>
+      </c>
+      <c r="AH841">
+        <v>3</v>
+      </c>
+      <c r="AI841">
+        <v>1982.32023</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>Franco Rossano</t>
+        </is>
+      </c>
+      <c r="B842" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E842">
+        <v>60.1525</v>
+      </c>
+      <c r="F842">
+        <v>5657.17</v>
+      </c>
+      <c r="G842">
+        <v>94.04713021071444</v>
+      </c>
+      <c r="H842">
+        <v>275.4</v>
+      </c>
+      <c r="I842">
+        <v>0</v>
+      </c>
+      <c r="J842">
+        <v>0</v>
+      </c>
+      <c r="K842">
+        <v>4.578363326545031</v>
+      </c>
+      <c r="L842">
+        <v>3.95</v>
+      </c>
+      <c r="M842">
+        <v>6</v>
+      </c>
+      <c r="N842">
+        <v>0</v>
+      </c>
+      <c r="O842">
+        <v>30.23601</v>
+      </c>
+      <c r="P842">
+        <v>89.34991134751772</v>
+      </c>
+      <c r="Q842">
+        <v>33.84</v>
+      </c>
+      <c r="R842">
+        <v>496.30659</v>
+      </c>
+      <c r="S842">
+        <v>8.250805702173643</v>
+      </c>
+      <c r="T842">
+        <v>916.76999</v>
+      </c>
+      <c r="U842">
+        <v>21</v>
+      </c>
+      <c r="V842">
+        <v>25</v>
+      </c>
+      <c r="W842">
+        <v>46</v>
+      </c>
+      <c r="X842">
+        <v>82</v>
+      </c>
+      <c r="Y842">
+        <v>21</v>
+      </c>
+      <c r="Z842">
+        <v>60</v>
+      </c>
+      <c r="AA842">
+        <v>25</v>
+      </c>
+      <c r="AB842">
+        <v>25</v>
+      </c>
+      <c r="AC842">
+        <v>4.03869</v>
+      </c>
+      <c r="AD842">
+        <v>-2.65289</v>
+      </c>
+      <c r="AE842">
+        <v>0</v>
+      </c>
+      <c r="AF842">
+        <v>477.0808</v>
+      </c>
+      <c r="AG842">
+        <v>0</v>
+      </c>
+      <c r="AH842">
+        <v>3</v>
+      </c>
+      <c r="AI842">
+        <v>1488.91977</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B843" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E843">
+        <v>60.1525</v>
+      </c>
+      <c r="F843">
+        <v>5787.26</v>
+      </c>
+      <c r="G843">
+        <v>96.20980009143427</v>
+      </c>
+      <c r="H843">
+        <v>135.62</v>
+      </c>
+      <c r="I843">
+        <v>0</v>
+      </c>
+      <c r="J843">
+        <v>0</v>
+      </c>
+      <c r="K843">
+        <v>2.254602884335647</v>
+      </c>
+      <c r="L843">
+        <v>0</v>
+      </c>
+      <c r="M843">
+        <v>2</v>
+      </c>
+      <c r="N843">
+        <v>0</v>
+      </c>
+      <c r="O843">
+        <v>26.25926</v>
+      </c>
+      <c r="P843">
+        <v>77.92990265906934</v>
+      </c>
+      <c r="Q843">
+        <v>33.696</v>
+      </c>
+      <c r="R843">
+        <v>550.02054</v>
+      </c>
+      <c r="S843">
+        <v>9.14376858817173</v>
+      </c>
+      <c r="T843">
+        <v>834.86</v>
+      </c>
+      <c r="U843">
+        <v>19</v>
+      </c>
+      <c r="V843">
+        <v>27</v>
+      </c>
+      <c r="W843">
+        <v>46</v>
+      </c>
+      <c r="X843">
+        <v>87</v>
+      </c>
+      <c r="Y843">
+        <v>19</v>
+      </c>
+      <c r="Z843">
+        <v>73</v>
+      </c>
+      <c r="AA843">
+        <v>27</v>
+      </c>
+      <c r="AB843">
+        <v>11</v>
+      </c>
+      <c r="AC843">
+        <v>4.2641</v>
+      </c>
+      <c r="AD843">
+        <v>-3.99587</v>
+      </c>
+      <c r="AE843">
+        <v>0</v>
+      </c>
+      <c r="AF843">
+        <v>550.932</v>
+      </c>
+      <c r="AG843">
+        <v>0</v>
+      </c>
+      <c r="AH843">
+        <v>3</v>
+      </c>
+      <c r="AI843">
+        <v>1650.06162</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B844" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E844">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F844">
+        <v>7456.55</v>
+      </c>
+      <c r="G844">
+        <v>109.6863323886203</v>
+      </c>
+      <c r="H844">
+        <v>265.17</v>
+      </c>
+      <c r="I844">
+        <v>0</v>
+      </c>
+      <c r="J844">
+        <v>0</v>
+      </c>
+      <c r="K844">
+        <v>3.900667836934031</v>
+      </c>
+      <c r="L844">
+        <v>0</v>
+      </c>
+      <c r="M844">
+        <v>6</v>
+      </c>
+      <c r="N844">
+        <v>0</v>
+      </c>
+      <c r="O844">
+        <v>27.91021</v>
+      </c>
+      <c r="P844">
+        <v>77.52836111111111</v>
+      </c>
+      <c r="Q844">
+        <v>36</v>
+      </c>
+      <c r="R844">
+        <v>868.1239399999999</v>
+      </c>
+      <c r="S844">
+        <v>12.77015926096635</v>
+      </c>
+      <c r="T844">
+        <v>1051.32</v>
+      </c>
+      <c r="U844">
+        <v>15</v>
+      </c>
+      <c r="V844">
+        <v>22</v>
+      </c>
+      <c r="W844">
+        <v>37</v>
+      </c>
+      <c r="X844">
+        <v>78</v>
+      </c>
+      <c r="Y844">
+        <v>15</v>
+      </c>
+      <c r="Z844">
+        <v>62</v>
+      </c>
+      <c r="AA844">
+        <v>22</v>
+      </c>
+      <c r="AB844">
+        <v>12</v>
+      </c>
+      <c r="AC844">
+        <v>4.00977</v>
+      </c>
+      <c r="AD844">
+        <v>-3.89351</v>
+      </c>
+      <c r="AE844">
+        <v>0</v>
+      </c>
+      <c r="AF844">
+        <v>1739.256</v>
+      </c>
+      <c r="AG844">
+        <v>0</v>
+      </c>
+      <c r="AH844">
+        <v>3</v>
+      </c>
+      <c r="AI844">
+        <v>2604.37182</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B845" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E845">
+        <v>60.1525</v>
+      </c>
+      <c r="F845">
+        <v>5913.24</v>
+      </c>
+      <c r="G845">
+        <v>98.3041436349279</v>
+      </c>
+      <c r="H845">
+        <v>153.01</v>
+      </c>
+      <c r="I845">
+        <v>0</v>
+      </c>
+      <c r="J845">
+        <v>0</v>
+      </c>
+      <c r="K845">
+        <v>2.543701425543411</v>
+      </c>
+      <c r="L845">
+        <v>4.06</v>
+      </c>
+      <c r="M845">
+        <v>1</v>
+      </c>
+      <c r="N845">
+        <v>0</v>
+      </c>
+      <c r="O845">
+        <v>30.10568</v>
+      </c>
+      <c r="P845">
+        <v>86.03589391860997</v>
+      </c>
+      <c r="Q845">
+        <v>34.992</v>
+      </c>
+      <c r="R845">
+        <v>508.08271</v>
+      </c>
+      <c r="S845">
+        <v>8.446576784007316</v>
+      </c>
+      <c r="T845">
+        <v>690.98</v>
+      </c>
+      <c r="U845">
+        <v>13</v>
+      </c>
+      <c r="V845">
+        <v>11</v>
+      </c>
+      <c r="W845">
+        <v>24</v>
+      </c>
+      <c r="X845">
+        <v>56</v>
+      </c>
+      <c r="Y845">
+        <v>13</v>
+      </c>
+      <c r="Z845">
+        <v>40</v>
+      </c>
+      <c r="AA845">
+        <v>11</v>
+      </c>
+      <c r="AB845">
+        <v>7</v>
+      </c>
+      <c r="AC845">
+        <v>3.80151</v>
+      </c>
+      <c r="AD845">
+        <v>-3.40731</v>
+      </c>
+      <c r="AE845">
+        <v>0</v>
+      </c>
+      <c r="AF845">
+        <v>468.09186</v>
+      </c>
+      <c r="AG845">
+        <v>0</v>
+      </c>
+      <c r="AH845">
+        <v>3</v>
+      </c>
+      <c r="AI845">
+        <v>1524.24813</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B846" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E846">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F846">
+        <v>6113.27</v>
+      </c>
+      <c r="G846">
+        <v>105.8092413848808</v>
+      </c>
+      <c r="H846">
+        <v>153.19</v>
+      </c>
+      <c r="I846">
+        <v>0</v>
+      </c>
+      <c r="J846">
+        <v>0</v>
+      </c>
+      <c r="K846">
+        <v>2.651431670407145</v>
+      </c>
+      <c r="L846">
+        <v>0</v>
+      </c>
+      <c r="M846">
+        <v>1</v>
+      </c>
+      <c r="N846">
+        <v>0</v>
+      </c>
+      <c r="O846">
+        <v>26.59392</v>
+      </c>
+      <c r="P846">
+        <v>80.55834242093785</v>
+      </c>
+      <c r="Q846">
+        <v>33.012</v>
+      </c>
+      <c r="R846">
+        <v>606.68593</v>
+      </c>
+      <c r="S846">
+        <v>10.50059591874412</v>
+      </c>
+      <c r="T846">
+        <v>850.83</v>
+      </c>
+      <c r="U846">
+        <v>12</v>
+      </c>
+      <c r="V846">
+        <v>16</v>
+      </c>
+      <c r="W846">
+        <v>28</v>
+      </c>
+      <c r="X846">
+        <v>73</v>
+      </c>
+      <c r="Y846">
+        <v>12</v>
+      </c>
+      <c r="Z846">
+        <v>71</v>
+      </c>
+      <c r="AA846">
+        <v>16</v>
+      </c>
+      <c r="AB846">
+        <v>25</v>
+      </c>
+      <c r="AC846">
+        <v>3.69719</v>
+      </c>
+      <c r="AD846">
+        <v>-2.27614</v>
+      </c>
+      <c r="AE846">
+        <v>0</v>
+      </c>
+      <c r="AF846">
+        <v>560.93778</v>
+      </c>
+      <c r="AG846">
+        <v>0</v>
+      </c>
+      <c r="AH846">
+        <v>3</v>
+      </c>
+      <c r="AI846">
+        <v>1820.05779</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B847" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E847">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F847">
+        <v>6612.19</v>
+      </c>
+      <c r="G847">
+        <v>97.26574222082749</v>
+      </c>
+      <c r="H847">
+        <v>417</v>
+      </c>
+      <c r="I847">
+        <v>15.99</v>
+      </c>
+      <c r="J847">
+        <v>1</v>
+      </c>
+      <c r="K847">
+        <v>6.134096949132597</v>
+      </c>
+      <c r="L847">
+        <v>22.62</v>
+      </c>
+      <c r="M847">
+        <v>10</v>
+      </c>
+      <c r="N847">
+        <v>1</v>
+      </c>
+      <c r="O847">
+        <v>32.63664</v>
+      </c>
+      <c r="P847">
+        <v>93.46116838487973</v>
+      </c>
+      <c r="Q847">
+        <v>34.92</v>
+      </c>
+      <c r="R847">
+        <v>590.7601099999999</v>
+      </c>
+      <c r="S847">
+        <v>8.690119396691216</v>
+      </c>
+      <c r="T847">
+        <v>1006.57998</v>
+      </c>
+      <c r="U847">
+        <v>25</v>
+      </c>
+      <c r="V847">
+        <v>16</v>
+      </c>
+      <c r="W847">
+        <v>41</v>
+      </c>
+      <c r="X847">
+        <v>74</v>
+      </c>
+      <c r="Y847">
+        <v>25</v>
+      </c>
+      <c r="Z847">
+        <v>64</v>
+      </c>
+      <c r="AA847">
+        <v>16</v>
+      </c>
+      <c r="AB847">
+        <v>12</v>
+      </c>
+      <c r="AC847">
+        <v>4.49446</v>
+      </c>
+      <c r="AD847">
+        <v>-3.50322</v>
+      </c>
+      <c r="AE847">
+        <v>0</v>
+      </c>
+      <c r="AF847">
+        <v>623.4295999999999</v>
+      </c>
+      <c r="AG847">
+        <v>0</v>
+      </c>
+      <c r="AH847">
+        <v>3</v>
+      </c>
+      <c r="AI847">
+        <v>1772.28033</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B848" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E848">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F848">
+        <v>6251.820000000001</v>
+      </c>
+      <c r="G848">
+        <v>108.2072821051296</v>
+      </c>
+      <c r="H848">
+        <v>406.46</v>
+      </c>
+      <c r="I848">
+        <v>0</v>
+      </c>
+      <c r="J848">
+        <v>0</v>
+      </c>
+      <c r="K848">
+        <v>7.035060491896913</v>
+      </c>
+      <c r="L848">
+        <v>0</v>
+      </c>
+      <c r="M848">
+        <v>6</v>
+      </c>
+      <c r="N848">
+        <v>0</v>
+      </c>
+      <c r="O848">
+        <v>28.5751</v>
+      </c>
+      <c r="P848">
+        <v>81.66180841335162</v>
+      </c>
+      <c r="Q848">
+        <v>34.992</v>
+      </c>
+      <c r="R848">
+        <v>501.94179</v>
+      </c>
+      <c r="S848">
+        <v>8.687671249473544</v>
+      </c>
+      <c r="T848">
+        <v>1242.9</v>
+      </c>
+      <c r="U848">
+        <v>30</v>
+      </c>
+      <c r="V848">
+        <v>29</v>
+      </c>
+      <c r="W848">
+        <v>59</v>
+      </c>
+      <c r="X848">
+        <v>89</v>
+      </c>
+      <c r="Y848">
+        <v>30</v>
+      </c>
+      <c r="Z848">
+        <v>81</v>
+      </c>
+      <c r="AA848">
+        <v>29</v>
+      </c>
+      <c r="AB848">
+        <v>18</v>
+      </c>
+      <c r="AC848">
+        <v>4.65509</v>
+      </c>
+      <c r="AD848">
+        <v>-2.71422</v>
+      </c>
+      <c r="AE848">
+        <v>0</v>
+      </c>
+      <c r="AF848">
+        <v>538.5421</v>
+      </c>
+      <c r="AG848">
+        <v>0</v>
+      </c>
+      <c r="AH848">
+        <v>3</v>
+      </c>
+      <c r="AI848">
+        <v>1505.82537</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Marioni Araujo</t>
+        </is>
+      </c>
+      <c r="B849" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E849">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F849">
+        <v>7126.26</v>
+      </c>
+      <c r="G849">
+        <v>104.827745143227</v>
+      </c>
+      <c r="H849">
+        <v>226.4</v>
+      </c>
+      <c r="I849">
+        <v>0</v>
+      </c>
+      <c r="J849">
+        <v>0</v>
+      </c>
+      <c r="K849">
+        <v>3.330358631375587</v>
+      </c>
+      <c r="L849">
+        <v>0</v>
+      </c>
+      <c r="M849">
+        <v>3</v>
+      </c>
+      <c r="N849">
+        <v>0</v>
+      </c>
+      <c r="O849">
+        <v>26.08044</v>
+      </c>
+      <c r="P849">
+        <v>72.44566666666667</v>
+      </c>
+      <c r="Q849">
+        <v>36</v>
+      </c>
+      <c r="R849">
+        <v>702.5074</v>
+      </c>
+      <c r="S849">
+        <v>10.33392925439586</v>
+      </c>
+      <c r="T849">
+        <v>999.76999</v>
+      </c>
+      <c r="U849">
+        <v>8</v>
+      </c>
+      <c r="V849">
+        <v>17</v>
+      </c>
+      <c r="W849">
+        <v>25</v>
+      </c>
+      <c r="X849">
+        <v>62</v>
+      </c>
+      <c r="Y849">
+        <v>8</v>
+      </c>
+      <c r="Z849">
+        <v>67</v>
+      </c>
+      <c r="AA849">
+        <v>17</v>
+      </c>
+      <c r="AB849">
+        <v>11</v>
+      </c>
+      <c r="AC849">
+        <v>4.08071</v>
+      </c>
+      <c r="AD849">
+        <v>-3.63194</v>
+      </c>
+      <c r="AE849">
+        <v>0</v>
+      </c>
+      <c r="AF849">
+        <v>1656.998</v>
+      </c>
+      <c r="AG849">
+        <v>0</v>
+      </c>
+      <c r="AH849">
+        <v>3</v>
+      </c>
+      <c r="AI849">
+        <v>2107.5222</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B850" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E850">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F850">
+        <v>5860.73</v>
+      </c>
+      <c r="G850">
+        <v>101.4382474946489</v>
+      </c>
+      <c r="H850">
+        <v>224.95</v>
+      </c>
+      <c r="I850">
+        <v>0</v>
+      </c>
+      <c r="J850">
+        <v>0</v>
+      </c>
+      <c r="K850">
+        <v>3.893462721183414</v>
+      </c>
+      <c r="L850">
+        <v>0</v>
+      </c>
+      <c r="M850">
+        <v>8</v>
+      </c>
+      <c r="N850">
+        <v>0</v>
+      </c>
+      <c r="O850">
+        <v>29.51249</v>
+      </c>
+      <c r="P850">
+        <v>86.84230814500941</v>
+      </c>
+      <c r="Q850">
+        <v>33.984</v>
+      </c>
+      <c r="R850">
+        <v>591.61207</v>
+      </c>
+      <c r="S850">
+        <v>10.23969566546856</v>
+      </c>
+      <c r="T850">
+        <v>781.41998</v>
+      </c>
+      <c r="U850">
+        <v>11</v>
+      </c>
+      <c r="V850">
+        <v>22</v>
+      </c>
+      <c r="W850">
+        <v>33</v>
+      </c>
+      <c r="X850">
+        <v>56</v>
+      </c>
+      <c r="Y850">
+        <v>11</v>
+      </c>
+      <c r="Z850">
+        <v>64</v>
+      </c>
+      <c r="AA850">
+        <v>22</v>
+      </c>
+      <c r="AB850">
+        <v>18</v>
+      </c>
+      <c r="AC850">
+        <v>3.8607</v>
+      </c>
+      <c r="AD850">
+        <v>-2.70995</v>
+      </c>
+      <c r="AE850">
+        <v>0</v>
+      </c>
+      <c r="AF850">
+        <v>553.9656</v>
+      </c>
+      <c r="AG850">
+        <v>0</v>
+      </c>
+      <c r="AH850">
+        <v>3</v>
+      </c>
+      <c r="AI850">
+        <v>1774.83621</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B851" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Sesión 45 | Trabajo AM</t>
+        </is>
+      </c>
+      <c r="E851">
+        <v>121.4458333333333</v>
+      </c>
+      <c r="F851">
+        <v>6750.969999999999</v>
+      </c>
+      <c r="G851">
+        <v>55.58832126805503</v>
+      </c>
+      <c r="H851">
+        <v>246.28</v>
+      </c>
+      <c r="I851">
+        <v>5.26</v>
+      </c>
+      <c r="J851">
+        <v>1</v>
+      </c>
+      <c r="K851">
+        <v>2.027899955398497</v>
+      </c>
+      <c r="L851">
+        <v>30.61</v>
+      </c>
+      <c r="M851">
+        <v>9</v>
+      </c>
+      <c r="N851">
+        <v>2</v>
+      </c>
+      <c r="O851">
+        <v>32.75746</v>
+      </c>
+      <c r="P851">
+        <v>90.99294444444445</v>
+      </c>
+      <c r="Q851">
+        <v>36</v>
+      </c>
+      <c r="R851">
+        <v>737.3349499999999</v>
+      </c>
+      <c r="S851">
+        <v>6.071307098500703</v>
+      </c>
+      <c r="T851">
+        <v>1208.94001</v>
+      </c>
+      <c r="U851">
+        <v>75</v>
+      </c>
+      <c r="V851">
+        <v>47</v>
+      </c>
+      <c r="W851">
+        <v>122</v>
+      </c>
+      <c r="X851">
+        <v>159</v>
+      </c>
+      <c r="Y851">
+        <v>75</v>
+      </c>
+      <c r="Z851">
+        <v>144</v>
+      </c>
+      <c r="AA851">
+        <v>47</v>
+      </c>
+      <c r="AB851">
+        <v>39</v>
+      </c>
+      <c r="AC851">
+        <v>4.81876</v>
+      </c>
+      <c r="AD851">
+        <v>-3.1359</v>
+      </c>
+      <c r="AE851">
+        <v>0</v>
+      </c>
+      <c r="AF851">
+        <v>1696.406</v>
+      </c>
+      <c r="AG851">
+        <v>0</v>
+      </c>
+      <c r="AH851">
+        <v>3</v>
+      </c>
+      <c r="AI851">
+        <v>2212.00485</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B852" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E852">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F852">
+        <v>7007.799999999999</v>
+      </c>
+      <c r="G852">
+        <v>103.0851908876053</v>
+      </c>
+      <c r="H852">
+        <v>247.92</v>
+      </c>
+      <c r="I852">
+        <v>0</v>
+      </c>
+      <c r="J852">
+        <v>0</v>
+      </c>
+      <c r="K852">
+        <v>3.646919222131782</v>
+      </c>
+      <c r="L852">
+        <v>0</v>
+      </c>
+      <c r="M852">
+        <v>2</v>
+      </c>
+      <c r="N852">
+        <v>0</v>
+      </c>
+      <c r="O852">
+        <v>28.09529</v>
+      </c>
+      <c r="P852">
+        <v>80.29060928212162</v>
+      </c>
+      <c r="Q852">
+        <v>34.992</v>
+      </c>
+      <c r="R852">
+        <v>561.96806</v>
+      </c>
+      <c r="S852">
+        <v>8.266586480469938</v>
+      </c>
+      <c r="T852">
+        <v>1011.32</v>
+      </c>
+      <c r="U852">
+        <v>16</v>
+      </c>
+      <c r="V852">
+        <v>25</v>
+      </c>
+      <c r="W852">
+        <v>41</v>
+      </c>
+      <c r="X852">
+        <v>72</v>
+      </c>
+      <c r="Y852">
+        <v>16</v>
+      </c>
+      <c r="Z852">
+        <v>77</v>
+      </c>
+      <c r="AA852">
+        <v>25</v>
+      </c>
+      <c r="AB852">
+        <v>23</v>
+      </c>
+      <c r="AC852">
+        <v>4.02705</v>
+      </c>
+      <c r="AD852">
+        <v>-4.13965</v>
+      </c>
+      <c r="AE852">
+        <v>0</v>
+      </c>
+      <c r="AF852">
+        <v>656.4136</v>
+      </c>
+      <c r="AG852">
+        <v>0</v>
+      </c>
+      <c r="AH852">
+        <v>3</v>
+      </c>
+      <c r="AI852">
+        <v>1685.90418</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B853" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E853">
+        <v>60.1525</v>
+      </c>
+      <c r="F853">
+        <v>5768.549999999999</v>
+      </c>
+      <c r="G853">
+        <v>95.89875732513195</v>
+      </c>
+      <c r="H853">
+        <v>169.74</v>
+      </c>
+      <c r="I853">
+        <v>0</v>
+      </c>
+      <c r="J853">
+        <v>0</v>
+      </c>
+      <c r="K853">
+        <v>2.821827854203899</v>
+      </c>
+      <c r="L853">
+        <v>0</v>
+      </c>
+      <c r="M853">
+        <v>4</v>
+      </c>
+      <c r="N853">
+        <v>0</v>
+      </c>
+      <c r="O853">
+        <v>29.22979</v>
+      </c>
+      <c r="P853">
+        <v>88.5429237852902</v>
+      </c>
+      <c r="Q853">
+        <v>33.012</v>
+      </c>
+      <c r="R853">
+        <v>522.07118</v>
+      </c>
+      <c r="S853">
+        <v>8.679126885831845</v>
+      </c>
+      <c r="T853">
+        <v>765.32998</v>
+      </c>
+      <c r="U853">
+        <v>19</v>
+      </c>
+      <c r="V853">
+        <v>11</v>
+      </c>
+      <c r="W853">
+        <v>30</v>
+      </c>
+      <c r="X853">
+        <v>63</v>
+      </c>
+      <c r="Y853">
+        <v>19</v>
+      </c>
+      <c r="Z853">
+        <v>57</v>
+      </c>
+      <c r="AA853">
+        <v>11</v>
+      </c>
+      <c r="AB853">
+        <v>15</v>
+      </c>
+      <c r="AC853">
+        <v>3.90996</v>
+      </c>
+      <c r="AD853">
+        <v>-2.91416</v>
+      </c>
+      <c r="AE853">
+        <v>0</v>
+      </c>
+      <c r="AF853">
+        <v>505.6274999999999</v>
+      </c>
+      <c r="AG853">
+        <v>0</v>
+      </c>
+      <c r="AH853">
+        <v>3</v>
+      </c>
+      <c r="AI853">
+        <v>1566.21354</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B854" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E854">
+        <v>60.1525</v>
+      </c>
+      <c r="F854">
+        <v>6483.690000000001</v>
+      </c>
+      <c r="G854">
+        <v>107.7875400024937</v>
+      </c>
+      <c r="H854">
+        <v>296.61</v>
+      </c>
+      <c r="I854">
+        <v>0</v>
+      </c>
+      <c r="J854">
+        <v>0</v>
+      </c>
+      <c r="K854">
+        <v>4.93096712522339</v>
+      </c>
+      <c r="L854">
+        <v>0</v>
+      </c>
+      <c r="M854">
+        <v>7</v>
+      </c>
+      <c r="N854">
+        <v>0</v>
+      </c>
+      <c r="O854">
+        <v>27.85486</v>
+      </c>
+      <c r="P854">
+        <v>87.0355580552431</v>
+      </c>
+      <c r="Q854">
+        <v>32.004</v>
+      </c>
+      <c r="R854">
+        <v>618.0086700000001</v>
+      </c>
+      <c r="S854">
+        <v>10.27403133701841</v>
+      </c>
+      <c r="T854">
+        <v>956.88999</v>
+      </c>
+      <c r="U854">
+        <v>13</v>
+      </c>
+      <c r="V854">
+        <v>16</v>
+      </c>
+      <c r="W854">
+        <v>29</v>
+      </c>
+      <c r="X854">
+        <v>67</v>
+      </c>
+      <c r="Y854">
+        <v>13</v>
+      </c>
+      <c r="Z854">
+        <v>54</v>
+      </c>
+      <c r="AA854">
+        <v>16</v>
+      </c>
+      <c r="AB854">
+        <v>21</v>
+      </c>
+      <c r="AC854">
+        <v>3.91076</v>
+      </c>
+      <c r="AD854">
+        <v>-3.21788</v>
+      </c>
+      <c r="AE854">
+        <v>0</v>
+      </c>
+      <c r="AF854">
+        <v>528.7954</v>
+      </c>
+      <c r="AG854">
+        <v>0</v>
+      </c>
+      <c r="AH854">
+        <v>3</v>
+      </c>
+      <c r="AI854">
+        <v>1854.02601</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B855" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E855">
+        <v>67.98066666666666</v>
+      </c>
+      <c r="F855">
+        <v>8283.300000000001</v>
+      </c>
+      <c r="G855">
+        <v>121.8478783183454</v>
+      </c>
+      <c r="H855">
+        <v>180.73</v>
+      </c>
+      <c r="I855">
+        <v>0</v>
+      </c>
+      <c r="J855">
+        <v>0</v>
+      </c>
+      <c r="K855">
+        <v>2.658549979896245</v>
+      </c>
+      <c r="L855">
+        <v>0</v>
+      </c>
+      <c r="M855">
+        <v>3</v>
+      </c>
+      <c r="N855">
+        <v>0</v>
+      </c>
+      <c r="O855">
+        <v>27.84872</v>
+      </c>
+      <c r="P855">
+        <v>77.35755555555556</v>
+      </c>
+      <c r="Q855">
+        <v>36</v>
+      </c>
+      <c r="R855">
+        <v>833.4776300000001</v>
+      </c>
+      <c r="S855">
+        <v>12.2605098018064</v>
+      </c>
+      <c r="T855">
+        <v>1120.34</v>
+      </c>
+      <c r="U855">
+        <v>14</v>
+      </c>
+      <c r="V855">
+        <v>36</v>
+      </c>
+      <c r="W855">
+        <v>50</v>
+      </c>
+      <c r="X855">
+        <v>94</v>
+      </c>
+      <c r="Y855">
+        <v>14</v>
+      </c>
+      <c r="Z855">
+        <v>90</v>
+      </c>
+      <c r="AA855">
+        <v>36</v>
+      </c>
+      <c r="AB855">
+        <v>15</v>
+      </c>
+      <c r="AC855">
+        <v>3.46145</v>
+      </c>
+      <c r="AD855">
+        <v>-4.61165</v>
+      </c>
+      <c r="AE855">
+        <v>0</v>
+      </c>
+      <c r="AF855">
+        <v>1934.15</v>
+      </c>
+      <c r="AG855">
+        <v>0</v>
+      </c>
+      <c r="AH855">
+        <v>3</v>
+      </c>
+      <c r="AI855">
+        <v>2500.43289</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Santiago Camarena</t>
+        </is>
+      </c>
+      <c r="B856" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E856">
+        <v>57.77633333333333</v>
+      </c>
+      <c r="F856">
+        <v>7476.27</v>
+      </c>
+      <c r="G856">
+        <v>129.4002157746251</v>
+      </c>
+      <c r="H856">
+        <v>142.84</v>
+      </c>
+      <c r="I856">
+        <v>0</v>
+      </c>
+      <c r="J856">
+        <v>0</v>
+      </c>
+      <c r="K856">
+        <v>2.472292576545183</v>
+      </c>
+      <c r="L856">
+        <v>0</v>
+      </c>
+      <c r="M856">
+        <v>1</v>
+      </c>
+      <c r="N856">
+        <v>0</v>
+      </c>
+      <c r="O856">
+        <v>26.9843</v>
+      </c>
+      <c r="P856">
+        <v>74.9563888888889</v>
+      </c>
+      <c r="Q856">
+        <v>36</v>
+      </c>
+      <c r="R856">
+        <v>809.23098</v>
+      </c>
+      <c r="S856">
+        <v>14.00627096446642</v>
+      </c>
+      <c r="T856">
+        <v>1173.45998</v>
+      </c>
+      <c r="U856">
+        <v>17</v>
+      </c>
+      <c r="V856">
+        <v>19</v>
+      </c>
+      <c r="W856">
+        <v>36</v>
+      </c>
+      <c r="X856">
+        <v>84</v>
+      </c>
+      <c r="Y856">
+        <v>17</v>
+      </c>
+      <c r="Z856">
+        <v>85</v>
+      </c>
+      <c r="AA856">
+        <v>19</v>
+      </c>
+      <c r="AB856">
+        <v>13</v>
+      </c>
+      <c r="AC856">
+        <v>4.11233</v>
+      </c>
+      <c r="AD856">
+        <v>-3.24123</v>
+      </c>
+      <c r="AE856">
+        <v>0</v>
+      </c>
+      <c r="AF856">
+        <v>1749.516</v>
+      </c>
+      <c r="AG856">
+        <v>0</v>
+      </c>
+      <c r="AH856">
+        <v>3</v>
+      </c>
+      <c r="AI856">
+        <v>2427.69294</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B857" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>MD-3</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Sesión 45</t>
+        </is>
+      </c>
+      <c r="E857">
+        <v>60.1525</v>
+      </c>
+      <c r="F857">
+        <v>6086.57</v>
+      </c>
+      <c r="G857">
+        <v>101.1856531316238</v>
+      </c>
+      <c r="H857">
+        <v>242.94</v>
+      </c>
+      <c r="I857">
+        <v>1.65</v>
+      </c>
+      <c r="J857">
+        <v>0</v>
+      </c>
+      <c r="K857">
+        <v>4.038734882174474</v>
+      </c>
+      <c r="L857">
+        <v>8.25</v>
+      </c>
+      <c r="M857">
+        <v>7</v>
+      </c>
+      <c r="N857">
+        <v>1</v>
+      </c>
+      <c r="O857">
+        <v>31.40241</v>
+      </c>
+      <c r="P857">
+        <v>89.74168381344307</v>
+      </c>
+      <c r="Q857">
+        <v>34.992</v>
+      </c>
+      <c r="R857">
+        <v>576.50676</v>
+      </c>
+      <c r="S857">
+        <v>9.584086446947342</v>
+      </c>
+      <c r="T857">
+        <v>1036.98</v>
+      </c>
+      <c r="U857">
+        <v>23</v>
+      </c>
+      <c r="V857">
+        <v>29</v>
+      </c>
+      <c r="W857">
+        <v>52</v>
+      </c>
+      <c r="X857">
+        <v>101</v>
+      </c>
+      <c r="Y857">
+        <v>23</v>
+      </c>
+      <c r="Z857">
+        <v>73</v>
+      </c>
+      <c r="AA857">
+        <v>29</v>
+      </c>
+      <c r="AB857">
+        <v>18</v>
+      </c>
+      <c r="AC857">
+        <v>4.43612</v>
+      </c>
+      <c r="AD857">
+        <v>-4.52816</v>
+      </c>
+      <c r="AE857">
+        <v>0</v>
+      </c>
+      <c r="AF857">
+        <v>589.896</v>
+      </c>
+      <c r="AG857">
+        <v>0</v>
+      </c>
+      <c r="AH857">
+        <v>3</v>
+      </c>
+      <c r="AI857">
+        <v>1729.52028</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B858" s="2">
+        <v>46233</v>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Trabajo AM</t>
+        </is>
+      </c>
+      <c r="E858">
+        <v>80.08333333333333</v>
+      </c>
+      <c r="F858">
+        <v>2512.84</v>
+      </c>
+      <c r="G858">
+        <v>31.37781477627472</v>
+      </c>
+      <c r="H858">
+        <v>0</v>
+      </c>
+      <c r="I858">
+        <v>0</v>
+      </c>
+      <c r="J858">
+        <v>0</v>
+      </c>
+      <c r="K858">
+        <v>0</v>
+      </c>
+      <c r="L858">
+        <v>0</v>
+      </c>
+      <c r="M858">
+        <v>0</v>
+      </c>
+      <c r="N858">
+        <v>0</v>
+      </c>
+      <c r="O858">
+        <v>19.69679</v>
+      </c>
+      <c r="P858">
+        <v>57.95901012241055</v>
+      </c>
+      <c r="Q858">
+        <v>33.984</v>
+      </c>
+      <c r="R858">
+        <v>308.40915</v>
+      </c>
+      <c r="S858">
+        <v>3.851102809573361</v>
+      </c>
+      <c r="T858">
+        <v>452.09</v>
+      </c>
+      <c r="U858">
+        <v>21</v>
+      </c>
+      <c r="V858">
+        <v>29</v>
+      </c>
+      <c r="W858">
+        <v>50</v>
+      </c>
+      <c r="X858">
+        <v>84</v>
+      </c>
+      <c r="Y858">
+        <v>21</v>
+      </c>
+      <c r="Z858">
+        <v>83</v>
+      </c>
+      <c r="AA858">
+        <v>29</v>
+      </c>
+      <c r="AB858">
+        <v>14</v>
+      </c>
+      <c r="AC858">
+        <v>4.16473</v>
+      </c>
+      <c r="AD858">
+        <v>-3.87068</v>
+      </c>
+      <c r="AE858">
+        <v>0</v>
+      </c>
+      <c r="AF858">
+        <v>219.6859</v>
+      </c>
+      <c r="AG858">
+        <v>0</v>
+      </c>
+      <c r="AH858">
+        <v>3</v>
+      </c>
+      <c r="AI858">
+        <v>925.2274500000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-02
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI883"/>
+  <dimension ref="A1:AI905"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -100094,6 +100094,2492 @@
         <v>1533.44208</v>
       </c>
     </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B884" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E884">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F884">
+        <v>3467.920000000001</v>
+      </c>
+      <c r="G884">
+        <v>36.55457135930347</v>
+      </c>
+      <c r="H884">
+        <v>0</v>
+      </c>
+      <c r="I884">
+        <v>0</v>
+      </c>
+      <c r="J884">
+        <v>0</v>
+      </c>
+      <c r="K884">
+        <v>0</v>
+      </c>
+      <c r="L884">
+        <v>0</v>
+      </c>
+      <c r="M884">
+        <v>0</v>
+      </c>
+      <c r="N884">
+        <v>0</v>
+      </c>
+      <c r="O884">
+        <v>20.28696</v>
+      </c>
+      <c r="P884">
+        <v>62.68372265480164</v>
+      </c>
+      <c r="Q884">
+        <v>32.364</v>
+      </c>
+      <c r="R884">
+        <v>306.57404</v>
+      </c>
+      <c r="S884">
+        <v>3.231528588344009</v>
+      </c>
+      <c r="T884">
+        <v>242.37</v>
+      </c>
+      <c r="U884">
+        <v>14</v>
+      </c>
+      <c r="V884">
+        <v>3</v>
+      </c>
+      <c r="W884">
+        <v>17</v>
+      </c>
+      <c r="X884">
+        <v>41</v>
+      </c>
+      <c r="Y884">
+        <v>14</v>
+      </c>
+      <c r="Z884">
+        <v>14</v>
+      </c>
+      <c r="AA884">
+        <v>3</v>
+      </c>
+      <c r="AB884">
+        <v>7</v>
+      </c>
+      <c r="AC884">
+        <v>3.90922</v>
+      </c>
+      <c r="AD884">
+        <v>0</v>
+      </c>
+      <c r="AE884">
+        <v>0</v>
+      </c>
+      <c r="AF884">
+        <v>262.6883</v>
+      </c>
+      <c r="AG884">
+        <v>0</v>
+      </c>
+      <c r="AH884">
+        <v>3</v>
+      </c>
+      <c r="AI884">
+        <v>919.7221200000001</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B885" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E885">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F885">
+        <v>3319.19</v>
+      </c>
+      <c r="G885">
+        <v>34.9868415967169</v>
+      </c>
+      <c r="H885">
+        <v>56.32</v>
+      </c>
+      <c r="I885">
+        <v>0</v>
+      </c>
+      <c r="J885">
+        <v>0</v>
+      </c>
+      <c r="K885">
+        <v>0.5936565604039226</v>
+      </c>
+      <c r="L885">
+        <v>0</v>
+      </c>
+      <c r="M885">
+        <v>1</v>
+      </c>
+      <c r="N885">
+        <v>0</v>
+      </c>
+      <c r="O885">
+        <v>26.35544</v>
+      </c>
+      <c r="P885">
+        <v>73.20955555555557</v>
+      </c>
+      <c r="Q885">
+        <v>36</v>
+      </c>
+      <c r="R885">
+        <v>272.89099</v>
+      </c>
+      <c r="S885">
+        <v>2.876483069755348</v>
+      </c>
+      <c r="T885">
+        <v>325.97001</v>
+      </c>
+      <c r="U885">
+        <v>23</v>
+      </c>
+      <c r="V885">
+        <v>22</v>
+      </c>
+      <c r="W885">
+        <v>45</v>
+      </c>
+      <c r="X885">
+        <v>45</v>
+      </c>
+      <c r="Y885">
+        <v>23</v>
+      </c>
+      <c r="Z885">
+        <v>41</v>
+      </c>
+      <c r="AA885">
+        <v>22</v>
+      </c>
+      <c r="AB885">
+        <v>523</v>
+      </c>
+      <c r="AC885">
+        <v>4.79777</v>
+      </c>
+      <c r="AD885">
+        <v>-0.30413</v>
+      </c>
+      <c r="AE885">
+        <v>0</v>
+      </c>
+      <c r="AF885">
+        <v>765.7760000000001</v>
+      </c>
+      <c r="AG885">
+        <v>0</v>
+      </c>
+      <c r="AH885">
+        <v>3</v>
+      </c>
+      <c r="AI885">
+        <v>818.67297</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B886" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E886">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F886">
+        <v>3397.77</v>
+      </c>
+      <c r="G886">
+        <v>35.81513585304752</v>
+      </c>
+      <c r="H886">
+        <v>165.36</v>
+      </c>
+      <c r="I886">
+        <v>5.58</v>
+      </c>
+      <c r="J886">
+        <v>0</v>
+      </c>
+      <c r="K886">
+        <v>1.743022884026858</v>
+      </c>
+      <c r="L886">
+        <v>0</v>
+      </c>
+      <c r="M886">
+        <v>1</v>
+      </c>
+      <c r="N886">
+        <v>0</v>
+      </c>
+      <c r="O886">
+        <v>29.28733</v>
+      </c>
+      <c r="P886">
+        <v>90.3929938271605</v>
+      </c>
+      <c r="Q886">
+        <v>32.4</v>
+      </c>
+      <c r="R886">
+        <v>329.64203</v>
+      </c>
+      <c r="S886">
+        <v>3.474683126675544</v>
+      </c>
+      <c r="T886">
+        <v>467.40001</v>
+      </c>
+      <c r="U886">
+        <v>30</v>
+      </c>
+      <c r="V886">
+        <v>15</v>
+      </c>
+      <c r="W886">
+        <v>45</v>
+      </c>
+      <c r="X886">
+        <v>51</v>
+      </c>
+      <c r="Y886">
+        <v>30</v>
+      </c>
+      <c r="Z886">
+        <v>47</v>
+      </c>
+      <c r="AA886">
+        <v>15</v>
+      </c>
+      <c r="AB886">
+        <v>7</v>
+      </c>
+      <c r="AC886">
+        <v>4.45258</v>
+      </c>
+      <c r="AD886">
+        <v>0</v>
+      </c>
+      <c r="AE886">
+        <v>0</v>
+      </c>
+      <c r="AF886">
+        <v>277.6627</v>
+      </c>
+      <c r="AG886">
+        <v>0</v>
+      </c>
+      <c r="AH886">
+        <v>3</v>
+      </c>
+      <c r="AI886">
+        <v>988.9260899999999</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B887" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Sesión 47 | Trabajo Brian</t>
+        </is>
+      </c>
+      <c r="E887">
+        <v>145.9046666666667</v>
+      </c>
+      <c r="F887">
+        <v>6684.57</v>
+      </c>
+      <c r="G887">
+        <v>45.81464152391744</v>
+      </c>
+      <c r="H887">
+        <v>45.79000000000001</v>
+      </c>
+      <c r="I887">
+        <v>0</v>
+      </c>
+      <c r="J887">
+        <v>0</v>
+      </c>
+      <c r="K887">
+        <v>0.31383506125004</v>
+      </c>
+      <c r="L887">
+        <v>0</v>
+      </c>
+      <c r="M887">
+        <v>0</v>
+      </c>
+      <c r="N887">
+        <v>0</v>
+      </c>
+      <c r="O887">
+        <v>23.42922</v>
+      </c>
+      <c r="P887">
+        <v>65.80502190765083</v>
+      </c>
+      <c r="Q887">
+        <v>35.604</v>
+      </c>
+      <c r="R887">
+        <v>624.22518</v>
+      </c>
+      <c r="S887">
+        <v>4.2783085302275</v>
+      </c>
+      <c r="T887">
+        <v>625.56999</v>
+      </c>
+      <c r="U887">
+        <v>37</v>
+      </c>
+      <c r="V887">
+        <v>16</v>
+      </c>
+      <c r="W887">
+        <v>53</v>
+      </c>
+      <c r="X887">
+        <v>104</v>
+      </c>
+      <c r="Y887">
+        <v>37</v>
+      </c>
+      <c r="Z887">
+        <v>67</v>
+      </c>
+      <c r="AA887">
+        <v>16</v>
+      </c>
+      <c r="AB887">
+        <v>15</v>
+      </c>
+      <c r="AC887">
+        <v>4.76288</v>
+      </c>
+      <c r="AD887">
+        <v>-1.10426</v>
+      </c>
+      <c r="AE887">
+        <v>0</v>
+      </c>
+      <c r="AF887">
+        <v>541.03633</v>
+      </c>
+      <c r="AG887">
+        <v>0</v>
+      </c>
+      <c r="AH887">
+        <v>3</v>
+      </c>
+      <c r="AI887">
+        <v>1872.67554</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B888" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E888">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F888">
+        <v>3440.1</v>
+      </c>
+      <c r="G888">
+        <v>36.26132694328007</v>
+      </c>
+      <c r="H888">
+        <v>41.99999999999999</v>
+      </c>
+      <c r="I888">
+        <v>0</v>
+      </c>
+      <c r="J888">
+        <v>0</v>
+      </c>
+      <c r="K888">
+        <v>0.4427126338239478</v>
+      </c>
+      <c r="L888">
+        <v>0</v>
+      </c>
+      <c r="M888">
+        <v>2</v>
+      </c>
+      <c r="N888">
+        <v>0</v>
+      </c>
+      <c r="O888">
+        <v>26.58012</v>
+      </c>
+      <c r="P888">
+        <v>78.21362994350282</v>
+      </c>
+      <c r="Q888">
+        <v>33.984</v>
+      </c>
+      <c r="R888">
+        <v>392.22585</v>
+      </c>
+      <c r="S888">
+        <v>4.13436521684135</v>
+      </c>
+      <c r="T888">
+        <v>352.65999</v>
+      </c>
+      <c r="U888">
+        <v>17</v>
+      </c>
+      <c r="V888">
+        <v>12</v>
+      </c>
+      <c r="W888">
+        <v>29</v>
+      </c>
+      <c r="X888">
+        <v>49</v>
+      </c>
+      <c r="Y888">
+        <v>17</v>
+      </c>
+      <c r="Z888">
+        <v>44</v>
+      </c>
+      <c r="AA888">
+        <v>12</v>
+      </c>
+      <c r="AB888">
+        <v>14</v>
+      </c>
+      <c r="AC888">
+        <v>4.41907</v>
+      </c>
+      <c r="AD888">
+        <v>0</v>
+      </c>
+      <c r="AE888">
+        <v>0</v>
+      </c>
+      <c r="AF888">
+        <v>312.6808</v>
+      </c>
+      <c r="AG888">
+        <v>0</v>
+      </c>
+      <c r="AH888">
+        <v>3</v>
+      </c>
+      <c r="AI888">
+        <v>1176.67755</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B889" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E889">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F889">
+        <v>3259.31</v>
+      </c>
+      <c r="G889">
+        <v>34.35565987020789</v>
+      </c>
+      <c r="H889">
+        <v>107.03</v>
+      </c>
+      <c r="I889">
+        <v>0</v>
+      </c>
+      <c r="J889">
+        <v>0</v>
+      </c>
+      <c r="K889">
+        <v>1.128179361861361</v>
+      </c>
+      <c r="L889">
+        <v>0</v>
+      </c>
+      <c r="M889">
+        <v>1</v>
+      </c>
+      <c r="N889">
+        <v>0</v>
+      </c>
+      <c r="O889">
+        <v>25.90845</v>
+      </c>
+      <c r="P889">
+        <v>72.84202091767881</v>
+      </c>
+      <c r="Q889">
+        <v>35.568</v>
+      </c>
+      <c r="R889">
+        <v>285.72107</v>
+      </c>
+      <c r="S889">
+        <v>3.011722081873728</v>
+      </c>
+      <c r="T889">
+        <v>398.94999</v>
+      </c>
+      <c r="U889">
+        <v>32</v>
+      </c>
+      <c r="V889">
+        <v>19</v>
+      </c>
+      <c r="W889">
+        <v>51</v>
+      </c>
+      <c r="X889">
+        <v>49</v>
+      </c>
+      <c r="Y889">
+        <v>32</v>
+      </c>
+      <c r="Z889">
+        <v>43</v>
+      </c>
+      <c r="AA889">
+        <v>19</v>
+      </c>
+      <c r="AB889">
+        <v>15</v>
+      </c>
+      <c r="AC889">
+        <v>4.93329</v>
+      </c>
+      <c r="AD889">
+        <v>-0.41526</v>
+      </c>
+      <c r="AE889">
+        <v>0</v>
+      </c>
+      <c r="AF889">
+        <v>309.5728</v>
+      </c>
+      <c r="AG889">
+        <v>0</v>
+      </c>
+      <c r="AH889">
+        <v>3</v>
+      </c>
+      <c r="AI889">
+        <v>857.1632099999999</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B890" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E890">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F890">
+        <v>3161.02</v>
+      </c>
+      <c r="G890">
+        <v>33.3196068992899</v>
+      </c>
+      <c r="H890">
+        <v>66.23</v>
+      </c>
+      <c r="I890">
+        <v>0</v>
+      </c>
+      <c r="J890">
+        <v>0</v>
+      </c>
+      <c r="K890">
+        <v>0.6981156604323827</v>
+      </c>
+      <c r="L890">
+        <v>0</v>
+      </c>
+      <c r="M890">
+        <v>0</v>
+      </c>
+      <c r="N890">
+        <v>0</v>
+      </c>
+      <c r="O890">
+        <v>23.97393</v>
+      </c>
+      <c r="P890">
+        <v>66.59425</v>
+      </c>
+      <c r="Q890">
+        <v>36</v>
+      </c>
+      <c r="R890">
+        <v>274.36192</v>
+      </c>
+      <c r="S890">
+        <v>2.891987814861793</v>
+      </c>
+      <c r="T890">
+        <v>262.64999</v>
+      </c>
+      <c r="U890">
+        <v>17</v>
+      </c>
+      <c r="V890">
+        <v>11</v>
+      </c>
+      <c r="W890">
+        <v>28</v>
+      </c>
+      <c r="X890">
+        <v>32</v>
+      </c>
+      <c r="Y890">
+        <v>17</v>
+      </c>
+      <c r="Z890">
+        <v>30</v>
+      </c>
+      <c r="AA890">
+        <v>11</v>
+      </c>
+      <c r="AB890">
+        <v>14</v>
+      </c>
+      <c r="AC890">
+        <v>5.0244</v>
+      </c>
+      <c r="AD890">
+        <v>-0.49345</v>
+      </c>
+      <c r="AE890">
+        <v>0</v>
+      </c>
+      <c r="AF890">
+        <v>710.408</v>
+      </c>
+      <c r="AG890">
+        <v>0</v>
+      </c>
+      <c r="AH890">
+        <v>3</v>
+      </c>
+      <c r="AI890">
+        <v>823.0857599999999</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B891" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E891">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F891">
+        <v>3564.41</v>
+      </c>
+      <c r="G891">
+        <v>37.57158492601265</v>
+      </c>
+      <c r="H891">
+        <v>236.78</v>
+      </c>
+      <c r="I891">
+        <v>0</v>
+      </c>
+      <c r="J891">
+        <v>0</v>
+      </c>
+      <c r="K891">
+        <v>2.495840792383951</v>
+      </c>
+      <c r="L891">
+        <v>45.06</v>
+      </c>
+      <c r="M891">
+        <v>5</v>
+      </c>
+      <c r="N891">
+        <v>2</v>
+      </c>
+      <c r="O891">
+        <v>30.82795</v>
+      </c>
+      <c r="P891">
+        <v>85.63319444444446</v>
+      </c>
+      <c r="Q891">
+        <v>36</v>
+      </c>
+      <c r="R891">
+        <v>358.70023</v>
+      </c>
+      <c r="S891">
+        <v>3.780972490377166</v>
+      </c>
+      <c r="T891">
+        <v>451.40999</v>
+      </c>
+      <c r="U891">
+        <v>25</v>
+      </c>
+      <c r="V891">
+        <v>15</v>
+      </c>
+      <c r="W891">
+        <v>40</v>
+      </c>
+      <c r="X891">
+        <v>45</v>
+      </c>
+      <c r="Y891">
+        <v>25</v>
+      </c>
+      <c r="Z891">
+        <v>36</v>
+      </c>
+      <c r="AA891">
+        <v>15</v>
+      </c>
+      <c r="AB891">
+        <v>13</v>
+      </c>
+      <c r="AC891">
+        <v>4.74228</v>
+      </c>
+      <c r="AD891">
+        <v>-0.42465</v>
+      </c>
+      <c r="AE891">
+        <v>0</v>
+      </c>
+      <c r="AF891">
+        <v>285.7134</v>
+      </c>
+      <c r="AG891">
+        <v>0</v>
+      </c>
+      <c r="AH891">
+        <v>3</v>
+      </c>
+      <c r="AI891">
+        <v>1076.10069</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B892" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E892">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F892">
+        <v>3844.51</v>
+      </c>
+      <c r="G892">
+        <v>40.52405137565681</v>
+      </c>
+      <c r="H892">
+        <v>145.9</v>
+      </c>
+      <c r="I892">
+        <v>0</v>
+      </c>
+      <c r="J892">
+        <v>0</v>
+      </c>
+      <c r="K892">
+        <v>1.537896661917469</v>
+      </c>
+      <c r="L892">
+        <v>0</v>
+      </c>
+      <c r="M892">
+        <v>2</v>
+      </c>
+      <c r="N892">
+        <v>0</v>
+      </c>
+      <c r="O892">
+        <v>27.64427</v>
+      </c>
+      <c r="P892">
+        <v>86.37754655668041</v>
+      </c>
+      <c r="Q892">
+        <v>32.004</v>
+      </c>
+      <c r="R892">
+        <v>404.78742</v>
+      </c>
+      <c r="S892">
+        <v>4.266766429089682</v>
+      </c>
+      <c r="T892">
+        <v>500.06</v>
+      </c>
+      <c r="U892">
+        <v>22</v>
+      </c>
+      <c r="V892">
+        <v>17</v>
+      </c>
+      <c r="W892">
+        <v>39</v>
+      </c>
+      <c r="X892">
+        <v>49</v>
+      </c>
+      <c r="Y892">
+        <v>22</v>
+      </c>
+      <c r="Z892">
+        <v>47</v>
+      </c>
+      <c r="AA892">
+        <v>17</v>
+      </c>
+      <c r="AB892">
+        <v>12</v>
+      </c>
+      <c r="AC892">
+        <v>4.53469</v>
+      </c>
+      <c r="AD892">
+        <v>-0.18555</v>
+      </c>
+      <c r="AE892">
+        <v>0</v>
+      </c>
+      <c r="AF892">
+        <v>266.229</v>
+      </c>
+      <c r="AG892">
+        <v>0</v>
+      </c>
+      <c r="AH892">
+        <v>3</v>
+      </c>
+      <c r="AI892">
+        <v>1214.36226</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>Esteban Lozano</t>
+        </is>
+      </c>
+      <c r="B893" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Compensatorio</t>
+        </is>
+      </c>
+      <c r="E893">
+        <v>81.51666666666667</v>
+      </c>
+      <c r="F893">
+        <v>5478.51</v>
+      </c>
+      <c r="G893">
+        <v>67.20723778368432</v>
+      </c>
+      <c r="H893">
+        <v>104.91</v>
+      </c>
+      <c r="I893">
+        <v>0</v>
+      </c>
+      <c r="J893">
+        <v>0</v>
+      </c>
+      <c r="K893">
+        <v>1.286976078511552</v>
+      </c>
+      <c r="L893">
+        <v>0</v>
+      </c>
+      <c r="M893">
+        <v>0</v>
+      </c>
+      <c r="N893">
+        <v>0</v>
+      </c>
+      <c r="O893">
+        <v>24.95212</v>
+      </c>
+      <c r="P893">
+        <v>80.59470284237726</v>
+      </c>
+      <c r="Q893">
+        <v>30.96</v>
+      </c>
+      <c r="R893">
+        <v>481.49686</v>
+      </c>
+      <c r="S893">
+        <v>5.906729012471888</v>
+      </c>
+      <c r="T893">
+        <v>751.54999</v>
+      </c>
+      <c r="U893">
+        <v>17</v>
+      </c>
+      <c r="V893">
+        <v>14</v>
+      </c>
+      <c r="W893">
+        <v>31</v>
+      </c>
+      <c r="X893">
+        <v>58</v>
+      </c>
+      <c r="Y893">
+        <v>17</v>
+      </c>
+      <c r="Z893">
+        <v>48</v>
+      </c>
+      <c r="AA893">
+        <v>14</v>
+      </c>
+      <c r="AB893">
+        <v>31</v>
+      </c>
+      <c r="AC893">
+        <v>4.29399</v>
+      </c>
+      <c r="AD893">
+        <v>-4.93109</v>
+      </c>
+      <c r="AE893">
+        <v>0</v>
+      </c>
+      <c r="AF893">
+        <v>411.5027</v>
+      </c>
+      <c r="AG893">
+        <v>0</v>
+      </c>
+      <c r="AH893">
+        <v>3</v>
+      </c>
+      <c r="AI893">
+        <v>1444.49058</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B894" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E894">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F894">
+        <v>3076.21</v>
+      </c>
+      <c r="G894">
+        <v>32.4256436022754</v>
+      </c>
+      <c r="H894">
+        <v>139.23</v>
+      </c>
+      <c r="I894">
+        <v>0</v>
+      </c>
+      <c r="J894">
+        <v>0</v>
+      </c>
+      <c r="K894">
+        <v>1.467592381126387</v>
+      </c>
+      <c r="L894">
+        <v>0</v>
+      </c>
+      <c r="M894">
+        <v>1</v>
+      </c>
+      <c r="N894">
+        <v>0</v>
+      </c>
+      <c r="O894">
+        <v>26.9573</v>
+      </c>
+      <c r="P894">
+        <v>80.00148385565052</v>
+      </c>
+      <c r="Q894">
+        <v>33.696</v>
+      </c>
+      <c r="R894">
+        <v>312.16157</v>
+      </c>
+      <c r="S894">
+        <v>3.290425496031398</v>
+      </c>
+      <c r="T894">
+        <v>361.51999</v>
+      </c>
+      <c r="U894">
+        <v>22</v>
+      </c>
+      <c r="V894">
+        <v>11</v>
+      </c>
+      <c r="W894">
+        <v>33</v>
+      </c>
+      <c r="X894">
+        <v>35</v>
+      </c>
+      <c r="Y894">
+        <v>22</v>
+      </c>
+      <c r="Z894">
+        <v>29</v>
+      </c>
+      <c r="AA894">
+        <v>11</v>
+      </c>
+      <c r="AB894">
+        <v>11</v>
+      </c>
+      <c r="AC894">
+        <v>5.07985</v>
+      </c>
+      <c r="AD894">
+        <v>-0.29724</v>
+      </c>
+      <c r="AE894">
+        <v>0</v>
+      </c>
+      <c r="AF894">
+        <v>279.9192</v>
+      </c>
+      <c r="AG894">
+        <v>0</v>
+      </c>
+      <c r="AH894">
+        <v>3</v>
+      </c>
+      <c r="AI894">
+        <v>936.4847100000002</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B895" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E895">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F895">
+        <v>3123.34</v>
+      </c>
+      <c r="G895">
+        <v>32.92243042208784</v>
+      </c>
+      <c r="H895">
+        <v>10.7</v>
+      </c>
+      <c r="I895">
+        <v>0</v>
+      </c>
+      <c r="J895">
+        <v>0</v>
+      </c>
+      <c r="K895">
+        <v>0.1127863138551486</v>
+      </c>
+      <c r="L895">
+        <v>0</v>
+      </c>
+      <c r="M895">
+        <v>0</v>
+      </c>
+      <c r="N895">
+        <v>0</v>
+      </c>
+      <c r="O895">
+        <v>22.05299</v>
+      </c>
+      <c r="P895">
+        <v>61.25830555555556</v>
+      </c>
+      <c r="Q895">
+        <v>36</v>
+      </c>
+      <c r="R895">
+        <v>356.13264</v>
+      </c>
+      <c r="S895">
+        <v>3.753914739168473</v>
+      </c>
+      <c r="T895">
+        <v>295.29</v>
+      </c>
+      <c r="U895">
+        <v>14</v>
+      </c>
+      <c r="V895">
+        <v>15</v>
+      </c>
+      <c r="W895">
+        <v>29</v>
+      </c>
+      <c r="X895">
+        <v>37</v>
+      </c>
+      <c r="Y895">
+        <v>14</v>
+      </c>
+      <c r="Z895">
+        <v>35</v>
+      </c>
+      <c r="AA895">
+        <v>15</v>
+      </c>
+      <c r="AB895">
+        <v>19</v>
+      </c>
+      <c r="AC895">
+        <v>4.34822</v>
+      </c>
+      <c r="AD895">
+        <v>-0.6773400000000001</v>
+      </c>
+      <c r="AE895">
+        <v>0</v>
+      </c>
+      <c r="AF895">
+        <v>704.056</v>
+      </c>
+      <c r="AG895">
+        <v>0</v>
+      </c>
+      <c r="AH895">
+        <v>3</v>
+      </c>
+      <c r="AI895">
+        <v>1068.39792</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B896" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E896">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F896">
+        <v>3966.84</v>
+      </c>
+      <c r="G896">
+        <v>41.8135023602515</v>
+      </c>
+      <c r="H896">
+        <v>139.78</v>
+      </c>
+      <c r="I896">
+        <v>0</v>
+      </c>
+      <c r="J896">
+        <v>0</v>
+      </c>
+      <c r="K896">
+        <v>1.473387220033063</v>
+      </c>
+      <c r="L896">
+        <v>0.8</v>
+      </c>
+      <c r="M896">
+        <v>2</v>
+      </c>
+      <c r="N896">
+        <v>0</v>
+      </c>
+      <c r="O896">
+        <v>29.89208</v>
+      </c>
+      <c r="P896">
+        <v>85.42546867855511</v>
+      </c>
+      <c r="Q896">
+        <v>34.992</v>
+      </c>
+      <c r="R896">
+        <v>363.98195</v>
+      </c>
+      <c r="S896">
+        <v>3.836645825244764</v>
+      </c>
+      <c r="T896">
+        <v>467.24999</v>
+      </c>
+      <c r="U896">
+        <v>33</v>
+      </c>
+      <c r="V896">
+        <v>18</v>
+      </c>
+      <c r="W896">
+        <v>51</v>
+      </c>
+      <c r="X896">
+        <v>58</v>
+      </c>
+      <c r="Y896">
+        <v>33</v>
+      </c>
+      <c r="Z896">
+        <v>40</v>
+      </c>
+      <c r="AA896">
+        <v>18</v>
+      </c>
+      <c r="AB896">
+        <v>15</v>
+      </c>
+      <c r="AC896">
+        <v>4.65776</v>
+      </c>
+      <c r="AD896">
+        <v>-0.8310999999999999</v>
+      </c>
+      <c r="AE896">
+        <v>0</v>
+      </c>
+      <c r="AF896">
+        <v>314.90358</v>
+      </c>
+      <c r="AG896">
+        <v>0</v>
+      </c>
+      <c r="AH896">
+        <v>3</v>
+      </c>
+      <c r="AI896">
+        <v>1091.94585</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B897" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E897">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F897">
+        <v>3312.46</v>
+      </c>
+      <c r="G897">
+        <v>34.9159021675351</v>
+      </c>
+      <c r="H897">
+        <v>128.76</v>
+      </c>
+      <c r="I897">
+        <v>0</v>
+      </c>
+      <c r="J897">
+        <v>0</v>
+      </c>
+      <c r="K897">
+        <v>1.357230445980275</v>
+      </c>
+      <c r="L897">
+        <v>0</v>
+      </c>
+      <c r="M897">
+        <v>0</v>
+      </c>
+      <c r="N897">
+        <v>0</v>
+      </c>
+      <c r="O897">
+        <v>24.47603</v>
+      </c>
+      <c r="P897">
+        <v>74.14282685084213</v>
+      </c>
+      <c r="Q897">
+        <v>33.012</v>
+      </c>
+      <c r="R897">
+        <v>319.98344</v>
+      </c>
+      <c r="S897">
+        <v>3.3728740833916</v>
+      </c>
+      <c r="T897">
+        <v>329.38</v>
+      </c>
+      <c r="U897">
+        <v>17</v>
+      </c>
+      <c r="V897">
+        <v>8</v>
+      </c>
+      <c r="W897">
+        <v>25</v>
+      </c>
+      <c r="X897">
+        <v>35</v>
+      </c>
+      <c r="Y897">
+        <v>17</v>
+      </c>
+      <c r="Z897">
+        <v>27</v>
+      </c>
+      <c r="AA897">
+        <v>8</v>
+      </c>
+      <c r="AB897">
+        <v>14</v>
+      </c>
+      <c r="AC897">
+        <v>4.37002</v>
+      </c>
+      <c r="AD897">
+        <v>0</v>
+      </c>
+      <c r="AE897">
+        <v>0</v>
+      </c>
+      <c r="AF897">
+        <v>285.83646</v>
+      </c>
+      <c r="AG897">
+        <v>0</v>
+      </c>
+      <c r="AH897">
+        <v>3</v>
+      </c>
+      <c r="AI897">
+        <v>959.9503199999999</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B898" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E898">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F898">
+        <v>2940.15</v>
+      </c>
+      <c r="G898">
+        <v>30.99141103863363</v>
+      </c>
+      <c r="H898">
+        <v>122.22</v>
+      </c>
+      <c r="I898">
+        <v>0</v>
+      </c>
+      <c r="J898">
+        <v>0</v>
+      </c>
+      <c r="K898">
+        <v>1.288291501162119</v>
+      </c>
+      <c r="L898">
+        <v>0</v>
+      </c>
+      <c r="M898">
+        <v>2</v>
+      </c>
+      <c r="N898">
+        <v>0</v>
+      </c>
+      <c r="O898">
+        <v>28.30323</v>
+      </c>
+      <c r="P898">
+        <v>80.88485939643347</v>
+      </c>
+      <c r="Q898">
+        <v>34.992</v>
+      </c>
+      <c r="R898">
+        <v>239.09471</v>
+      </c>
+      <c r="S898">
+        <v>2.520239591440201</v>
+      </c>
+      <c r="T898">
+        <v>303.29999</v>
+      </c>
+      <c r="U898">
+        <v>16</v>
+      </c>
+      <c r="V898">
+        <v>15</v>
+      </c>
+      <c r="W898">
+        <v>31</v>
+      </c>
+      <c r="X898">
+        <v>32</v>
+      </c>
+      <c r="Y898">
+        <v>16</v>
+      </c>
+      <c r="Z898">
+        <v>34</v>
+      </c>
+      <c r="AA898">
+        <v>15</v>
+      </c>
+      <c r="AB898">
+        <v>17</v>
+      </c>
+      <c r="AC898">
+        <v>4.55001</v>
+      </c>
+      <c r="AD898">
+        <v>0</v>
+      </c>
+      <c r="AE898">
+        <v>0</v>
+      </c>
+      <c r="AF898">
+        <v>238.05945</v>
+      </c>
+      <c r="AG898">
+        <v>0</v>
+      </c>
+      <c r="AH898">
+        <v>3</v>
+      </c>
+      <c r="AI898">
+        <v>717.28413</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B899" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E899">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F899">
+        <v>2768.2</v>
+      </c>
+      <c r="G899">
+        <v>29.17897887979649</v>
+      </c>
+      <c r="H899">
+        <v>85.52</v>
+      </c>
+      <c r="I899">
+        <v>0</v>
+      </c>
+      <c r="J899">
+        <v>0</v>
+      </c>
+      <c r="K899">
+        <v>0.9014472486815244</v>
+      </c>
+      <c r="L899">
+        <v>0</v>
+      </c>
+      <c r="M899">
+        <v>0</v>
+      </c>
+      <c r="N899">
+        <v>0</v>
+      </c>
+      <c r="O899">
+        <v>24.60752</v>
+      </c>
+      <c r="P899">
+        <v>72.40913370998116</v>
+      </c>
+      <c r="Q899">
+        <v>33.984</v>
+      </c>
+      <c r="R899">
+        <v>257.75164</v>
+      </c>
+      <c r="S899">
+        <v>2.716902557543858</v>
+      </c>
+      <c r="T899">
+        <v>284.07001</v>
+      </c>
+      <c r="U899">
+        <v>14</v>
+      </c>
+      <c r="V899">
+        <v>11</v>
+      </c>
+      <c r="W899">
+        <v>25</v>
+      </c>
+      <c r="X899">
+        <v>30</v>
+      </c>
+      <c r="Y899">
+        <v>14</v>
+      </c>
+      <c r="Z899">
+        <v>26</v>
+      </c>
+      <c r="AA899">
+        <v>11</v>
+      </c>
+      <c r="AB899">
+        <v>11</v>
+      </c>
+      <c r="AC899">
+        <v>4.39028</v>
+      </c>
+      <c r="AD899">
+        <v>0</v>
+      </c>
+      <c r="AE899">
+        <v>0</v>
+      </c>
+      <c r="AF899">
+        <v>248.0712</v>
+      </c>
+      <c r="AG899">
+        <v>0</v>
+      </c>
+      <c r="AH899">
+        <v>3</v>
+      </c>
+      <c r="AI899">
+        <v>773.2549200000001</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B900" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Sesión 47 | Compensatorio</t>
+        </is>
+      </c>
+      <c r="E900">
+        <v>176.3863333333333</v>
+      </c>
+      <c r="F900">
+        <v>7976.429999999999</v>
+      </c>
+      <c r="G900">
+        <v>45.22136068743043</v>
+      </c>
+      <c r="H900">
+        <v>121.88</v>
+      </c>
+      <c r="I900">
+        <v>0</v>
+      </c>
+      <c r="J900">
+        <v>0</v>
+      </c>
+      <c r="K900">
+        <v>0.6909832394422092</v>
+      </c>
+      <c r="L900">
+        <v>0</v>
+      </c>
+      <c r="M900">
+        <v>1</v>
+      </c>
+      <c r="N900">
+        <v>0</v>
+      </c>
+      <c r="O900">
+        <v>25.5386</v>
+      </c>
+      <c r="P900">
+        <v>70.94055555555555</v>
+      </c>
+      <c r="Q900">
+        <v>36</v>
+      </c>
+      <c r="R900">
+        <v>812.4266700000001</v>
+      </c>
+      <c r="S900">
+        <v>4.605950215341703</v>
+      </c>
+      <c r="T900">
+        <v>895.60999</v>
+      </c>
+      <c r="U900">
+        <v>35</v>
+      </c>
+      <c r="V900">
+        <v>32</v>
+      </c>
+      <c r="W900">
+        <v>67</v>
+      </c>
+      <c r="X900">
+        <v>110</v>
+      </c>
+      <c r="Y900">
+        <v>35</v>
+      </c>
+      <c r="Z900">
+        <v>83</v>
+      </c>
+      <c r="AA900">
+        <v>32</v>
+      </c>
+      <c r="AB900">
+        <v>28</v>
+      </c>
+      <c r="AC900">
+        <v>4.77023</v>
+      </c>
+      <c r="AD900">
+        <v>-0.9101</v>
+      </c>
+      <c r="AE900">
+        <v>0</v>
+      </c>
+      <c r="AF900">
+        <v>1865.384</v>
+      </c>
+      <c r="AG900">
+        <v>0</v>
+      </c>
+      <c r="AH900">
+        <v>3</v>
+      </c>
+      <c r="AI900">
+        <v>2437.28001</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B901" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E901">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F901">
+        <v>3053.75</v>
+      </c>
+      <c r="G901">
+        <v>32.18884120171673</v>
+      </c>
+      <c r="H901">
+        <v>6.47</v>
+      </c>
+      <c r="I901">
+        <v>0</v>
+      </c>
+      <c r="J901">
+        <v>0</v>
+      </c>
+      <c r="K901">
+        <v>0.06819870735165198</v>
+      </c>
+      <c r="L901">
+        <v>0</v>
+      </c>
+      <c r="M901">
+        <v>0</v>
+      </c>
+      <c r="N901">
+        <v>0</v>
+      </c>
+      <c r="O901">
+        <v>21.24522</v>
+      </c>
+      <c r="P901">
+        <v>60.71450617283951</v>
+      </c>
+      <c r="Q901">
+        <v>34.992</v>
+      </c>
+      <c r="R901">
+        <v>248.13656</v>
+      </c>
+      <c r="S901">
+        <v>2.615547548483097</v>
+      </c>
+      <c r="T901">
+        <v>246.08</v>
+      </c>
+      <c r="U901">
+        <v>18</v>
+      </c>
+      <c r="V901">
+        <v>13</v>
+      </c>
+      <c r="W901">
+        <v>31</v>
+      </c>
+      <c r="X901">
+        <v>34</v>
+      </c>
+      <c r="Y901">
+        <v>18</v>
+      </c>
+      <c r="Z901">
+        <v>33</v>
+      </c>
+      <c r="AA901">
+        <v>13</v>
+      </c>
+      <c r="AB901">
+        <v>8</v>
+      </c>
+      <c r="AC901">
+        <v>4.41758</v>
+      </c>
+      <c r="AD901">
+        <v>-0.44839</v>
+      </c>
+      <c r="AE901">
+        <v>0</v>
+      </c>
+      <c r="AF901">
+        <v>275.6808</v>
+      </c>
+      <c r="AG901">
+        <v>0</v>
+      </c>
+      <c r="AH901">
+        <v>3</v>
+      </c>
+      <c r="AI901">
+        <v>744.40968</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B902" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E902">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F902">
+        <v>3130.07</v>
+      </c>
+      <c r="G902">
+        <v>32.99336985126963</v>
+      </c>
+      <c r="H902">
+        <v>15.98</v>
+      </c>
+      <c r="I902">
+        <v>0</v>
+      </c>
+      <c r="J902">
+        <v>0</v>
+      </c>
+      <c r="K902">
+        <v>0.1684416163930164</v>
+      </c>
+      <c r="L902">
+        <v>0</v>
+      </c>
+      <c r="M902">
+        <v>0</v>
+      </c>
+      <c r="N902">
+        <v>0</v>
+      </c>
+      <c r="O902">
+        <v>23.63277</v>
+      </c>
+      <c r="P902">
+        <v>71.58842239185751</v>
+      </c>
+      <c r="Q902">
+        <v>33.012</v>
+      </c>
+      <c r="R902">
+        <v>275.23203</v>
+      </c>
+      <c r="S902">
+        <v>2.901159450333616</v>
+      </c>
+      <c r="T902">
+        <v>286.75001</v>
+      </c>
+      <c r="U902">
+        <v>17</v>
+      </c>
+      <c r="V902">
+        <v>10</v>
+      </c>
+      <c r="W902">
+        <v>27</v>
+      </c>
+      <c r="X902">
+        <v>42</v>
+      </c>
+      <c r="Y902">
+        <v>17</v>
+      </c>
+      <c r="Z902">
+        <v>35</v>
+      </c>
+      <c r="AA902">
+        <v>10</v>
+      </c>
+      <c r="AB902">
+        <v>8</v>
+      </c>
+      <c r="AC902">
+        <v>4.57627</v>
+      </c>
+      <c r="AD902">
+        <v>-0.61265</v>
+      </c>
+      <c r="AE902">
+        <v>0</v>
+      </c>
+      <c r="AF902">
+        <v>264.00225</v>
+      </c>
+      <c r="AG902">
+        <v>0</v>
+      </c>
+      <c r="AH902">
+        <v>3</v>
+      </c>
+      <c r="AI902">
+        <v>825.69609</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B903" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E903">
+        <v>94.86983333333335</v>
+      </c>
+      <c r="F903">
+        <v>3291.23</v>
+      </c>
+      <c r="G903">
+        <v>34.69206052503517</v>
+      </c>
+      <c r="H903">
+        <v>125.55</v>
+      </c>
+      <c r="I903">
+        <v>0</v>
+      </c>
+      <c r="J903">
+        <v>0</v>
+      </c>
+      <c r="K903">
+        <v>1.32339222689334</v>
+      </c>
+      <c r="L903">
+        <v>0</v>
+      </c>
+      <c r="M903">
+        <v>3</v>
+      </c>
+      <c r="N903">
+        <v>0</v>
+      </c>
+      <c r="O903">
+        <v>28.21584</v>
+      </c>
+      <c r="P903">
+        <v>88.16347956505437</v>
+      </c>
+      <c r="Q903">
+        <v>32.004</v>
+      </c>
+      <c r="R903">
+        <v>287.43043</v>
+      </c>
+      <c r="S903">
+        <v>3.029734741812905</v>
+      </c>
+      <c r="T903">
+        <v>316.01</v>
+      </c>
+      <c r="U903">
+        <v>14</v>
+      </c>
+      <c r="V903">
+        <v>6</v>
+      </c>
+      <c r="W903">
+        <v>20</v>
+      </c>
+      <c r="X903">
+        <v>31</v>
+      </c>
+      <c r="Y903">
+        <v>14</v>
+      </c>
+      <c r="Z903">
+        <v>24</v>
+      </c>
+      <c r="AA903">
+        <v>6</v>
+      </c>
+      <c r="AB903">
+        <v>9</v>
+      </c>
+      <c r="AC903">
+        <v>4.00977</v>
+      </c>
+      <c r="AD903">
+        <v>-0.30001</v>
+      </c>
+      <c r="AE903">
+        <v>0</v>
+      </c>
+      <c r="AF903">
+        <v>253.8543</v>
+      </c>
+      <c r="AG903">
+        <v>0</v>
+      </c>
+      <c r="AH903">
+        <v>3</v>
+      </c>
+      <c r="AI903">
+        <v>862.29129</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>Santiago Naveda Lara</t>
+        </is>
+      </c>
+      <c r="B904" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Compensatorio</t>
+        </is>
+      </c>
+      <c r="E904">
+        <v>81.51666666666667</v>
+      </c>
+      <c r="F904">
+        <v>5462.570000000001</v>
+      </c>
+      <c r="G904">
+        <v>67.01169494990801</v>
+      </c>
+      <c r="H904">
+        <v>247.2</v>
+      </c>
+      <c r="I904">
+        <v>0</v>
+      </c>
+      <c r="J904">
+        <v>0</v>
+      </c>
+      <c r="K904">
+        <v>3.032508689429565</v>
+      </c>
+      <c r="L904">
+        <v>0</v>
+      </c>
+      <c r="M904">
+        <v>1</v>
+      </c>
+      <c r="N904">
+        <v>0</v>
+      </c>
+      <c r="O904">
+        <v>25.4776</v>
+      </c>
+      <c r="P904">
+        <v>79.07386716325264</v>
+      </c>
+      <c r="Q904">
+        <v>32.22</v>
+      </c>
+      <c r="R904">
+        <v>584.78235</v>
+      </c>
+      <c r="S904">
+        <v>7.173776528317317</v>
+      </c>
+      <c r="T904">
+        <v>1080.53003</v>
+      </c>
+      <c r="U904">
+        <v>20</v>
+      </c>
+      <c r="V904">
+        <v>25</v>
+      </c>
+      <c r="W904">
+        <v>45</v>
+      </c>
+      <c r="X904">
+        <v>83</v>
+      </c>
+      <c r="Y904">
+        <v>20</v>
+      </c>
+      <c r="Z904">
+        <v>59</v>
+      </c>
+      <c r="AA904">
+        <v>25</v>
+      </c>
+      <c r="AB904">
+        <v>35</v>
+      </c>
+      <c r="AC904">
+        <v>4.03275</v>
+      </c>
+      <c r="AD904">
+        <v>-4.68282</v>
+      </c>
+      <c r="AE904">
+        <v>0</v>
+      </c>
+      <c r="AF904">
+        <v>493.34054</v>
+      </c>
+      <c r="AG904">
+        <v>0</v>
+      </c>
+      <c r="AH904">
+        <v>3</v>
+      </c>
+      <c r="AI904">
+        <v>1754.34705</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B905" s="2">
+        <v>46235</v>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>MD-1</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Sesión 47</t>
+        </is>
+      </c>
+      <c r="E905">
+        <v>94.86966666666667</v>
+      </c>
+      <c r="F905">
+        <v>3557.83</v>
+      </c>
+      <c r="G905">
+        <v>37.50229261899658</v>
+      </c>
+      <c r="H905">
+        <v>86.7</v>
+      </c>
+      <c r="I905">
+        <v>0</v>
+      </c>
+      <c r="J905">
+        <v>0</v>
+      </c>
+      <c r="K905">
+        <v>0.9138853655365782</v>
+      </c>
+      <c r="L905">
+        <v>0</v>
+      </c>
+      <c r="M905">
+        <v>2</v>
+      </c>
+      <c r="N905">
+        <v>0</v>
+      </c>
+      <c r="O905">
+        <v>27.92407</v>
+      </c>
+      <c r="P905">
+        <v>79.80129743941472</v>
+      </c>
+      <c r="Q905">
+        <v>34.992</v>
+      </c>
+      <c r="R905">
+        <v>342.14862</v>
+      </c>
+      <c r="S905">
+        <v>3.60651230284355</v>
+      </c>
+      <c r="T905">
+        <v>397.44999</v>
+      </c>
+      <c r="U905">
+        <v>25</v>
+      </c>
+      <c r="V905">
+        <v>20</v>
+      </c>
+      <c r="W905">
+        <v>45</v>
+      </c>
+      <c r="X905">
+        <v>60</v>
+      </c>
+      <c r="Y905">
+        <v>25</v>
+      </c>
+      <c r="Z905">
+        <v>48</v>
+      </c>
+      <c r="AA905">
+        <v>20</v>
+      </c>
+      <c r="AB905">
+        <v>22</v>
+      </c>
+      <c r="AC905">
+        <v>5.00199</v>
+      </c>
+      <c r="AD905">
+        <v>-0.23202</v>
+      </c>
+      <c r="AE905">
+        <v>0</v>
+      </c>
+      <c r="AF905">
+        <v>331.7832</v>
+      </c>
+      <c r="AG905">
+        <v>0</v>
+      </c>
+      <c r="AH905">
+        <v>3</v>
+      </c>
+      <c r="AI905">
+        <v>1026.44586</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-03
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI905"/>
+  <dimension ref="A1:AI927"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -102580,6 +102580,2492 @@
         <v>1026.44586</v>
       </c>
     </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B906" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E906">
+        <v>121.6616666666667</v>
+      </c>
+      <c r="F906">
+        <v>14893.22</v>
+      </c>
+      <c r="G906">
+        <v>122.4150581530748</v>
+      </c>
+      <c r="H906">
+        <v>562.41</v>
+      </c>
+      <c r="I906">
+        <v>24.62</v>
+      </c>
+      <c r="J906">
+        <v>2</v>
+      </c>
+      <c r="K906">
+        <v>4.622737920736468</v>
+      </c>
+      <c r="L906">
+        <v>20.39</v>
+      </c>
+      <c r="M906">
+        <v>11</v>
+      </c>
+      <c r="N906">
+        <v>1</v>
+      </c>
+      <c r="O906">
+        <v>31.89561</v>
+      </c>
+      <c r="P906">
+        <v>98.55274378939563</v>
+      </c>
+      <c r="Q906">
+        <v>32.364</v>
+      </c>
+      <c r="R906">
+        <v>1534.35587</v>
+      </c>
+      <c r="S906">
+        <v>12.6116624244832</v>
+      </c>
+      <c r="T906">
+        <v>2190.46997</v>
+      </c>
+      <c r="U906">
+        <v>22</v>
+      </c>
+      <c r="V906">
+        <v>20</v>
+      </c>
+      <c r="W906">
+        <v>42</v>
+      </c>
+      <c r="X906">
+        <v>106</v>
+      </c>
+      <c r="Y906">
+        <v>22</v>
+      </c>
+      <c r="Z906">
+        <v>95</v>
+      </c>
+      <c r="AA906">
+        <v>20</v>
+      </c>
+      <c r="AB906">
+        <v>54</v>
+      </c>
+      <c r="AC906">
+        <v>4.26112</v>
+      </c>
+      <c r="AD906">
+        <v>-3.4913</v>
+      </c>
+      <c r="AE906">
+        <v>0</v>
+      </c>
+      <c r="AF906">
+        <v>1180.9357</v>
+      </c>
+      <c r="AG906">
+        <v>0</v>
+      </c>
+      <c r="AH906">
+        <v>3</v>
+      </c>
+      <c r="AI906">
+        <v>4603.06761</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B907" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E907">
+        <v>50.30366666666667</v>
+      </c>
+      <c r="F907">
+        <v>2490.690000000001</v>
+      </c>
+      <c r="G907">
+        <v>49.51309049704793</v>
+      </c>
+      <c r="H907">
+        <v>96.08</v>
+      </c>
+      <c r="I907">
+        <v>0</v>
+      </c>
+      <c r="J907">
+        <v>0</v>
+      </c>
+      <c r="K907">
+        <v>1.909999933735778</v>
+      </c>
+      <c r="L907">
+        <v>0</v>
+      </c>
+      <c r="M907">
+        <v>2</v>
+      </c>
+      <c r="N907">
+        <v>0</v>
+      </c>
+      <c r="O907">
+        <v>27.05993</v>
+      </c>
+      <c r="P907">
+        <v>75.16647222222223</v>
+      </c>
+      <c r="Q907">
+        <v>36</v>
+      </c>
+      <c r="R907">
+        <v>247.91613</v>
+      </c>
+      <c r="S907">
+        <v>4.928390839633956</v>
+      </c>
+      <c r="T907">
+        <v>423.52001</v>
+      </c>
+      <c r="U907">
+        <v>17</v>
+      </c>
+      <c r="V907">
+        <v>13</v>
+      </c>
+      <c r="W907">
+        <v>30</v>
+      </c>
+      <c r="X907">
+        <v>36</v>
+      </c>
+      <c r="Y907">
+        <v>17</v>
+      </c>
+      <c r="Z907">
+        <v>30</v>
+      </c>
+      <c r="AA907">
+        <v>13</v>
+      </c>
+      <c r="AB907">
+        <v>25</v>
+      </c>
+      <c r="AC907">
+        <v>4.79461</v>
+      </c>
+      <c r="AD907">
+        <v>-1.47314</v>
+      </c>
+      <c r="AE907">
+        <v>0</v>
+      </c>
+      <c r="AF907">
+        <v>585.048</v>
+      </c>
+      <c r="AG907">
+        <v>0</v>
+      </c>
+      <c r="AH907">
+        <v>3</v>
+      </c>
+      <c r="AI907">
+        <v>743.74839</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>Alexis Gutiérrez</t>
+        </is>
+      </c>
+      <c r="B908" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E908">
+        <v>98.05066666666667</v>
+      </c>
+      <c r="F908">
+        <v>11319.21</v>
+      </c>
+      <c r="G908">
+        <v>115.4424583208681</v>
+      </c>
+      <c r="H908">
+        <v>955</v>
+      </c>
+      <c r="I908">
+        <v>10.1</v>
+      </c>
+      <c r="J908">
+        <v>1</v>
+      </c>
+      <c r="K908">
+        <v>9.73986238407354</v>
+      </c>
+      <c r="L908">
+        <v>0</v>
+      </c>
+      <c r="M908">
+        <v>17</v>
+      </c>
+      <c r="N908">
+        <v>0</v>
+      </c>
+      <c r="O908">
+        <v>29.59953</v>
+      </c>
+      <c r="P908">
+        <v>91.35657407407408</v>
+      </c>
+      <c r="Q908">
+        <v>32.4</v>
+      </c>
+      <c r="R908">
+        <v>1205.5726</v>
+      </c>
+      <c r="S908">
+        <v>12.29540441676412</v>
+      </c>
+      <c r="T908">
+        <v>2523.99002</v>
+      </c>
+      <c r="U908">
+        <v>33</v>
+      </c>
+      <c r="V908">
+        <v>37</v>
+      </c>
+      <c r="W908">
+        <v>70</v>
+      </c>
+      <c r="X908">
+        <v>158</v>
+      </c>
+      <c r="Y908">
+        <v>33</v>
+      </c>
+      <c r="Z908">
+        <v>135</v>
+      </c>
+      <c r="AA908">
+        <v>37</v>
+      </c>
+      <c r="AB908">
+        <v>19</v>
+      </c>
+      <c r="AC908">
+        <v>5.18423</v>
+      </c>
+      <c r="AD908">
+        <v>-2.94727</v>
+      </c>
+      <c r="AE908">
+        <v>0</v>
+      </c>
+      <c r="AF908">
+        <v>931.217</v>
+      </c>
+      <c r="AG908">
+        <v>0</v>
+      </c>
+      <c r="AH908">
+        <v>3</v>
+      </c>
+      <c r="AI908">
+        <v>3616.7178</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B909" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E909">
+        <v>24.6735</v>
+      </c>
+      <c r="F909">
+        <v>2574.81</v>
+      </c>
+      <c r="G909">
+        <v>104.3552799562283</v>
+      </c>
+      <c r="H909">
+        <v>163.31</v>
+      </c>
+      <c r="I909">
+        <v>0</v>
+      </c>
+      <c r="J909">
+        <v>0</v>
+      </c>
+      <c r="K909">
+        <v>6.618842077532575</v>
+      </c>
+      <c r="L909">
+        <v>18.54</v>
+      </c>
+      <c r="M909">
+        <v>4</v>
+      </c>
+      <c r="N909">
+        <v>1</v>
+      </c>
+      <c r="O909">
+        <v>31.20062</v>
+      </c>
+      <c r="P909">
+        <v>87.632344680373</v>
+      </c>
+      <c r="Q909">
+        <v>35.604</v>
+      </c>
+      <c r="R909">
+        <v>198.58865</v>
+      </c>
+      <c r="S909">
+        <v>8.048661519443938</v>
+      </c>
+      <c r="T909">
+        <v>380.51001</v>
+      </c>
+      <c r="U909">
+        <v>7</v>
+      </c>
+      <c r="V909">
+        <v>6</v>
+      </c>
+      <c r="W909">
+        <v>13</v>
+      </c>
+      <c r="X909">
+        <v>30</v>
+      </c>
+      <c r="Y909">
+        <v>7</v>
+      </c>
+      <c r="Z909">
+        <v>27</v>
+      </c>
+      <c r="AA909">
+        <v>6</v>
+      </c>
+      <c r="AB909">
+        <v>7</v>
+      </c>
+      <c r="AC909">
+        <v>4.27654</v>
+      </c>
+      <c r="AD909">
+        <v>-4.30761</v>
+      </c>
+      <c r="AE909">
+        <v>0</v>
+      </c>
+      <c r="AF909">
+        <v>211.30594</v>
+      </c>
+      <c r="AG909">
+        <v>0</v>
+      </c>
+      <c r="AH909">
+        <v>3</v>
+      </c>
+      <c r="AI909">
+        <v>595.76595</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B910" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E910">
+        <v>121.6616666666667</v>
+      </c>
+      <c r="F910">
+        <v>11960.04</v>
+      </c>
+      <c r="G910">
+        <v>98.30573859199693</v>
+      </c>
+      <c r="H910">
+        <v>698.6099999999999</v>
+      </c>
+      <c r="I910">
+        <v>0</v>
+      </c>
+      <c r="J910">
+        <v>0</v>
+      </c>
+      <c r="K910">
+        <v>5.742235982300642</v>
+      </c>
+      <c r="L910">
+        <v>4.87</v>
+      </c>
+      <c r="M910">
+        <v>22</v>
+      </c>
+      <c r="N910">
+        <v>1</v>
+      </c>
+      <c r="O910">
+        <v>30.36012</v>
+      </c>
+      <c r="P910">
+        <v>89.33651129943502</v>
+      </c>
+      <c r="Q910">
+        <v>33.984</v>
+      </c>
+      <c r="R910">
+        <v>1337.45573</v>
+      </c>
+      <c r="S910">
+        <v>10.99323859884653</v>
+      </c>
+      <c r="T910">
+        <v>1839.88</v>
+      </c>
+      <c r="U910">
+        <v>27</v>
+      </c>
+      <c r="V910">
+        <v>50</v>
+      </c>
+      <c r="W910">
+        <v>77</v>
+      </c>
+      <c r="X910">
+        <v>119</v>
+      </c>
+      <c r="Y910">
+        <v>27</v>
+      </c>
+      <c r="Z910">
+        <v>126</v>
+      </c>
+      <c r="AA910">
+        <v>50</v>
+      </c>
+      <c r="AB910">
+        <v>18</v>
+      </c>
+      <c r="AC910">
+        <v>4.33724</v>
+      </c>
+      <c r="AD910">
+        <v>-4.30055</v>
+      </c>
+      <c r="AE910">
+        <v>0</v>
+      </c>
+      <c r="AF910">
+        <v>1113.9144</v>
+      </c>
+      <c r="AG910">
+        <v>0</v>
+      </c>
+      <c r="AH910">
+        <v>3</v>
+      </c>
+      <c r="AI910">
+        <v>4012.36719</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B911" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E911">
+        <v>71.64149999999999</v>
+      </c>
+      <c r="F911">
+        <v>7403.01</v>
+      </c>
+      <c r="G911">
+        <v>103.3341010447855</v>
+      </c>
+      <c r="H911">
+        <v>473.64</v>
+      </c>
+      <c r="I911">
+        <v>1.54</v>
+      </c>
+      <c r="J911">
+        <v>0</v>
+      </c>
+      <c r="K911">
+        <v>6.611251858210675</v>
+      </c>
+      <c r="L911">
+        <v>18.12</v>
+      </c>
+      <c r="M911">
+        <v>14</v>
+      </c>
+      <c r="N911">
+        <v>2</v>
+      </c>
+      <c r="O911">
+        <v>32.06335</v>
+      </c>
+      <c r="P911">
+        <v>90.14662055780477</v>
+      </c>
+      <c r="Q911">
+        <v>35.568</v>
+      </c>
+      <c r="R911">
+        <v>686.9341899999999</v>
+      </c>
+      <c r="S911">
+        <v>9.588495355345714</v>
+      </c>
+      <c r="T911">
+        <v>1211.50995</v>
+      </c>
+      <c r="U911">
+        <v>37</v>
+      </c>
+      <c r="V911">
+        <v>35</v>
+      </c>
+      <c r="W911">
+        <v>72</v>
+      </c>
+      <c r="X911">
+        <v>116</v>
+      </c>
+      <c r="Y911">
+        <v>37</v>
+      </c>
+      <c r="Z911">
+        <v>93</v>
+      </c>
+      <c r="AA911">
+        <v>35</v>
+      </c>
+      <c r="AB911">
+        <v>16</v>
+      </c>
+      <c r="AC911">
+        <v>4.77068</v>
+      </c>
+      <c r="AD911">
+        <v>-3.38774</v>
+      </c>
+      <c r="AE911">
+        <v>0</v>
+      </c>
+      <c r="AF911">
+        <v>708.6888</v>
+      </c>
+      <c r="AG911">
+        <v>0</v>
+      </c>
+      <c r="AH911">
+        <v>3</v>
+      </c>
+      <c r="AI911">
+        <v>2060.80257</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B912" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E912">
+        <v>70.64</v>
+      </c>
+      <c r="F912">
+        <v>3890.84</v>
+      </c>
+      <c r="G912">
+        <v>55.07984144960363</v>
+      </c>
+      <c r="H912">
+        <v>154.79</v>
+      </c>
+      <c r="I912">
+        <v>0</v>
+      </c>
+      <c r="J912">
+        <v>0</v>
+      </c>
+      <c r="K912">
+        <v>2.191251415628539</v>
+      </c>
+      <c r="L912">
+        <v>0</v>
+      </c>
+      <c r="M912">
+        <v>4</v>
+      </c>
+      <c r="N912">
+        <v>0</v>
+      </c>
+      <c r="O912">
+        <v>28.77054</v>
+      </c>
+      <c r="P912">
+        <v>79.91816666666666</v>
+      </c>
+      <c r="Q912">
+        <v>36</v>
+      </c>
+      <c r="R912">
+        <v>393.68292</v>
+      </c>
+      <c r="S912">
+        <v>5.573087768969422</v>
+      </c>
+      <c r="T912">
+        <v>559.14</v>
+      </c>
+      <c r="U912">
+        <v>17</v>
+      </c>
+      <c r="V912">
+        <v>19</v>
+      </c>
+      <c r="W912">
+        <v>36</v>
+      </c>
+      <c r="X912">
+        <v>44</v>
+      </c>
+      <c r="Y912">
+        <v>17</v>
+      </c>
+      <c r="Z912">
+        <v>42</v>
+      </c>
+      <c r="AA912">
+        <v>19</v>
+      </c>
+      <c r="AB912">
+        <v>17</v>
+      </c>
+      <c r="AC912">
+        <v>4.18872</v>
+      </c>
+      <c r="AD912">
+        <v>-2.35263</v>
+      </c>
+      <c r="AE912">
+        <v>0</v>
+      </c>
+      <c r="AF912">
+        <v>883.576</v>
+      </c>
+      <c r="AG912">
+        <v>0</v>
+      </c>
+      <c r="AH912">
+        <v>3</v>
+      </c>
+      <c r="AI912">
+        <v>1181.04876</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B913" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E913">
+        <v>74.93566666666668</v>
+      </c>
+      <c r="F913">
+        <v>3397.04</v>
+      </c>
+      <c r="G913">
+        <v>45.33275209401842</v>
+      </c>
+      <c r="H913">
+        <v>489.33</v>
+      </c>
+      <c r="I913">
+        <v>0</v>
+      </c>
+      <c r="J913">
+        <v>0</v>
+      </c>
+      <c r="K913">
+        <v>6.530001289995418</v>
+      </c>
+      <c r="L913">
+        <v>90.03</v>
+      </c>
+      <c r="M913">
+        <v>15</v>
+      </c>
+      <c r="N913">
+        <v>5</v>
+      </c>
+      <c r="O913">
+        <v>31.52281</v>
+      </c>
+      <c r="P913">
+        <v>87.56336111111112</v>
+      </c>
+      <c r="Q913">
+        <v>36</v>
+      </c>
+      <c r="R913">
+        <v>392.94395</v>
+      </c>
+      <c r="S913">
+        <v>5.243750639437383</v>
+      </c>
+      <c r="T913">
+        <v>727.19999</v>
+      </c>
+      <c r="U913">
+        <v>39</v>
+      </c>
+      <c r="V913">
+        <v>29</v>
+      </c>
+      <c r="W913">
+        <v>68</v>
+      </c>
+      <c r="X913">
+        <v>53</v>
+      </c>
+      <c r="Y913">
+        <v>39</v>
+      </c>
+      <c r="Z913">
+        <v>42</v>
+      </c>
+      <c r="AA913">
+        <v>29</v>
+      </c>
+      <c r="AB913">
+        <v>16</v>
+      </c>
+      <c r="AC913">
+        <v>4.49873</v>
+      </c>
+      <c r="AD913">
+        <v>-2.71442</v>
+      </c>
+      <c r="AE913">
+        <v>0</v>
+      </c>
+      <c r="AF913">
+        <v>299.4054</v>
+      </c>
+      <c r="AG913">
+        <v>0</v>
+      </c>
+      <c r="AH913">
+        <v>3</v>
+      </c>
+      <c r="AI913">
+        <v>1178.83185</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B914" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E914">
+        <v>121.6616666666667</v>
+      </c>
+      <c r="F914">
+        <v>13617.71</v>
+      </c>
+      <c r="G914">
+        <v>111.9309834650739</v>
+      </c>
+      <c r="H914">
+        <v>690.87</v>
+      </c>
+      <c r="I914">
+        <v>10.13</v>
+      </c>
+      <c r="J914">
+        <v>2</v>
+      </c>
+      <c r="K914">
+        <v>5.678616929462855</v>
+      </c>
+      <c r="L914">
+        <v>2.88</v>
+      </c>
+      <c r="M914">
+        <v>13</v>
+      </c>
+      <c r="N914">
+        <v>0</v>
+      </c>
+      <c r="O914">
+        <v>30.50045</v>
+      </c>
+      <c r="P914">
+        <v>95.30199350081242</v>
+      </c>
+      <c r="Q914">
+        <v>32.004</v>
+      </c>
+      <c r="R914">
+        <v>1402.13494</v>
+      </c>
+      <c r="S914">
+        <v>11.52487039193391</v>
+      </c>
+      <c r="T914">
+        <v>2289.38994</v>
+      </c>
+      <c r="U914">
+        <v>37</v>
+      </c>
+      <c r="V914">
+        <v>57</v>
+      </c>
+      <c r="W914">
+        <v>94</v>
+      </c>
+      <c r="X914">
+        <v>147</v>
+      </c>
+      <c r="Y914">
+        <v>37</v>
+      </c>
+      <c r="Z914">
+        <v>144</v>
+      </c>
+      <c r="AA914">
+        <v>57</v>
+      </c>
+      <c r="AB914">
+        <v>30</v>
+      </c>
+      <c r="AC914">
+        <v>4.31198</v>
+      </c>
+      <c r="AD914">
+        <v>-3.93373</v>
+      </c>
+      <c r="AE914">
+        <v>0</v>
+      </c>
+      <c r="AF914">
+        <v>946.8822</v>
+      </c>
+      <c r="AG914">
+        <v>0</v>
+      </c>
+      <c r="AH914">
+        <v>3</v>
+      </c>
+      <c r="AI914">
+        <v>4206.40482</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>Esteban Lozano</t>
+        </is>
+      </c>
+      <c r="B915" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>Futbol Complementario</t>
+        </is>
+      </c>
+      <c r="E915">
+        <v>68.36433333333333</v>
+      </c>
+      <c r="F915">
+        <v>7312.34</v>
+      </c>
+      <c r="G915">
+        <v>106.9613297382163</v>
+      </c>
+      <c r="H915">
+        <v>232.91</v>
+      </c>
+      <c r="I915">
+        <v>0</v>
+      </c>
+      <c r="J915">
+        <v>0</v>
+      </c>
+      <c r="K915">
+        <v>3.406893458089745</v>
+      </c>
+      <c r="L915">
+        <v>0</v>
+      </c>
+      <c r="M915">
+        <v>4</v>
+      </c>
+      <c r="N915">
+        <v>0</v>
+      </c>
+      <c r="O915">
+        <v>29.50576</v>
+      </c>
+      <c r="P915">
+        <v>95.30284237726097</v>
+      </c>
+      <c r="Q915">
+        <v>30.96</v>
+      </c>
+      <c r="R915">
+        <v>647.75113</v>
+      </c>
+      <c r="S915">
+        <v>9.474986420794469</v>
+      </c>
+      <c r="T915">
+        <v>978.1299799999999</v>
+      </c>
+      <c r="U915">
+        <v>27</v>
+      </c>
+      <c r="V915">
+        <v>21</v>
+      </c>
+      <c r="W915">
+        <v>48</v>
+      </c>
+      <c r="X915">
+        <v>90</v>
+      </c>
+      <c r="Y915">
+        <v>27</v>
+      </c>
+      <c r="Z915">
+        <v>67</v>
+      </c>
+      <c r="AA915">
+        <v>21</v>
+      </c>
+      <c r="AB915">
+        <v>15</v>
+      </c>
+      <c r="AC915">
+        <v>4.41093</v>
+      </c>
+      <c r="AD915">
+        <v>-2.41075</v>
+      </c>
+      <c r="AE915">
+        <v>0</v>
+      </c>
+      <c r="AF915">
+        <v>600.8877</v>
+      </c>
+      <c r="AG915">
+        <v>0</v>
+      </c>
+      <c r="AH915">
+        <v>3</v>
+      </c>
+      <c r="AI915">
+        <v>1943.25339</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B916" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E916">
+        <v>105.5075</v>
+      </c>
+      <c r="F916">
+        <v>10962.8</v>
+      </c>
+      <c r="G916">
+        <v>103.9054095680402</v>
+      </c>
+      <c r="H916">
+        <v>542.2099999999999</v>
+      </c>
+      <c r="I916">
+        <v>8.43</v>
+      </c>
+      <c r="J916">
+        <v>1</v>
+      </c>
+      <c r="K916">
+        <v>5.139065943179395</v>
+      </c>
+      <c r="L916">
+        <v>9.960000000000001</v>
+      </c>
+      <c r="M916">
+        <v>9</v>
+      </c>
+      <c r="N916">
+        <v>1</v>
+      </c>
+      <c r="O916">
+        <v>31.03054</v>
+      </c>
+      <c r="P916">
+        <v>92.08968423551757</v>
+      </c>
+      <c r="Q916">
+        <v>33.696</v>
+      </c>
+      <c r="R916">
+        <v>1261.95117</v>
+      </c>
+      <c r="S916">
+        <v>11.96077217259437</v>
+      </c>
+      <c r="T916">
+        <v>1619.23003</v>
+      </c>
+      <c r="U916">
+        <v>29</v>
+      </c>
+      <c r="V916">
+        <v>42</v>
+      </c>
+      <c r="W916">
+        <v>71</v>
+      </c>
+      <c r="X916">
+        <v>135</v>
+      </c>
+      <c r="Y916">
+        <v>29</v>
+      </c>
+      <c r="Z916">
+        <v>135</v>
+      </c>
+      <c r="AA916">
+        <v>42</v>
+      </c>
+      <c r="AB916">
+        <v>39</v>
+      </c>
+      <c r="AC916">
+        <v>4.33893</v>
+      </c>
+      <c r="AD916">
+        <v>-4.0865</v>
+      </c>
+      <c r="AE916">
+        <v>0</v>
+      </c>
+      <c r="AF916">
+        <v>1017.36</v>
+      </c>
+      <c r="AG916">
+        <v>0</v>
+      </c>
+      <c r="AH916">
+        <v>3</v>
+      </c>
+      <c r="AI916">
+        <v>3785.85351</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B917" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E917">
+        <v>54.45233333333334</v>
+      </c>
+      <c r="F917">
+        <v>1923.61</v>
+      </c>
+      <c r="G917">
+        <v>35.32649350808352</v>
+      </c>
+      <c r="H917">
+        <v>408.77</v>
+      </c>
+      <c r="I917">
+        <v>0</v>
+      </c>
+      <c r="J917">
+        <v>0</v>
+      </c>
+      <c r="K917">
+        <v>7.506932668939806</v>
+      </c>
+      <c r="L917">
+        <v>0</v>
+      </c>
+      <c r="M917">
+        <v>10</v>
+      </c>
+      <c r="N917">
+        <v>0</v>
+      </c>
+      <c r="O917">
+        <v>29.38515</v>
+      </c>
+      <c r="P917">
+        <v>81.62541666666667</v>
+      </c>
+      <c r="Q917">
+        <v>36</v>
+      </c>
+      <c r="R917">
+        <v>198.57931</v>
+      </c>
+      <c r="S917">
+        <v>3.646846660994019</v>
+      </c>
+      <c r="T917">
+        <v>525.57999</v>
+      </c>
+      <c r="U917">
+        <v>17</v>
+      </c>
+      <c r="V917">
+        <v>12</v>
+      </c>
+      <c r="W917">
+        <v>29</v>
+      </c>
+      <c r="X917">
+        <v>28</v>
+      </c>
+      <c r="Y917">
+        <v>17</v>
+      </c>
+      <c r="Z917">
+        <v>17</v>
+      </c>
+      <c r="AA917">
+        <v>12</v>
+      </c>
+      <c r="AB917">
+        <v>136</v>
+      </c>
+      <c r="AC917">
+        <v>3.95906</v>
+      </c>
+      <c r="AD917">
+        <v>-1.09773</v>
+      </c>
+      <c r="AE917">
+        <v>0</v>
+      </c>
+      <c r="AF917">
+        <v>478.56</v>
+      </c>
+      <c r="AG917">
+        <v>0</v>
+      </c>
+      <c r="AH917">
+        <v>3</v>
+      </c>
+      <c r="AI917">
+        <v>595.73793</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B918" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E918">
+        <v>105.3858333333333</v>
+      </c>
+      <c r="F918">
+        <v>11363.82</v>
+      </c>
+      <c r="G918">
+        <v>107.8306223954833</v>
+      </c>
+      <c r="H918">
+        <v>707.66</v>
+      </c>
+      <c r="I918">
+        <v>0</v>
+      </c>
+      <c r="J918">
+        <v>0</v>
+      </c>
+      <c r="K918">
+        <v>6.714944292006358</v>
+      </c>
+      <c r="L918">
+        <v>28.97</v>
+      </c>
+      <c r="M918">
+        <v>19</v>
+      </c>
+      <c r="N918">
+        <v>3</v>
+      </c>
+      <c r="O918">
+        <v>31.1439</v>
+      </c>
+      <c r="P918">
+        <v>89.00291495198903</v>
+      </c>
+      <c r="Q918">
+        <v>34.992</v>
+      </c>
+      <c r="R918">
+        <v>985.22488</v>
+      </c>
+      <c r="S918">
+        <v>9.348741181215059</v>
+      </c>
+      <c r="T918">
+        <v>1772.11</v>
+      </c>
+      <c r="U918">
+        <v>24</v>
+      </c>
+      <c r="V918">
+        <v>37</v>
+      </c>
+      <c r="W918">
+        <v>61</v>
+      </c>
+      <c r="X918">
+        <v>114</v>
+      </c>
+      <c r="Y918">
+        <v>24</v>
+      </c>
+      <c r="Z918">
+        <v>102</v>
+      </c>
+      <c r="AA918">
+        <v>37</v>
+      </c>
+      <c r="AB918">
+        <v>22</v>
+      </c>
+      <c r="AC918">
+        <v>4.70989</v>
+      </c>
+      <c r="AD918">
+        <v>-3.48292</v>
+      </c>
+      <c r="AE918">
+        <v>0</v>
+      </c>
+      <c r="AF918">
+        <v>899.8855799999999</v>
+      </c>
+      <c r="AG918">
+        <v>0</v>
+      </c>
+      <c r="AH918">
+        <v>3</v>
+      </c>
+      <c r="AI918">
+        <v>2955.67464</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B919" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E919">
+        <v>102.7058333333333</v>
+      </c>
+      <c r="F919">
+        <v>8558.889999999999</v>
+      </c>
+      <c r="G919">
+        <v>83.33402030069696</v>
+      </c>
+      <c r="H919">
+        <v>322.55</v>
+      </c>
+      <c r="I919">
+        <v>0</v>
+      </c>
+      <c r="J919">
+        <v>0</v>
+      </c>
+      <c r="K919">
+        <v>3.140522690207469</v>
+      </c>
+      <c r="L919">
+        <v>0</v>
+      </c>
+      <c r="M919">
+        <v>6</v>
+      </c>
+      <c r="N919">
+        <v>0</v>
+      </c>
+      <c r="O919">
+        <v>29.21286</v>
+      </c>
+      <c r="P919">
+        <v>88.49163940385314</v>
+      </c>
+      <c r="Q919">
+        <v>33.012</v>
+      </c>
+      <c r="R919">
+        <v>884.00162</v>
+      </c>
+      <c r="S919">
+        <v>8.607121828523209</v>
+      </c>
+      <c r="T919">
+        <v>1273.40999</v>
+      </c>
+      <c r="U919">
+        <v>17</v>
+      </c>
+      <c r="V919">
+        <v>32</v>
+      </c>
+      <c r="W919">
+        <v>49</v>
+      </c>
+      <c r="X919">
+        <v>81</v>
+      </c>
+      <c r="Y919">
+        <v>17</v>
+      </c>
+      <c r="Z919">
+        <v>93</v>
+      </c>
+      <c r="AA919">
+        <v>32</v>
+      </c>
+      <c r="AB919">
+        <v>37</v>
+      </c>
+      <c r="AC919">
+        <v>3.89414</v>
+      </c>
+      <c r="AD919">
+        <v>-2.30615</v>
+      </c>
+      <c r="AE919">
+        <v>0</v>
+      </c>
+      <c r="AF919">
+        <v>765.70026</v>
+      </c>
+      <c r="AG919">
+        <v>0</v>
+      </c>
+      <c r="AH919">
+        <v>3</v>
+      </c>
+      <c r="AI919">
+        <v>2652.00486</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B920" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E920">
+        <v>102.7058333333333</v>
+      </c>
+      <c r="F920">
+        <v>7703.779999999999</v>
+      </c>
+      <c r="G920">
+        <v>75.00820303942487</v>
+      </c>
+      <c r="H920">
+        <v>536.1800000000001</v>
+      </c>
+      <c r="I920">
+        <v>0</v>
+      </c>
+      <c r="J920">
+        <v>0</v>
+      </c>
+      <c r="K920">
+        <v>5.220540865092051</v>
+      </c>
+      <c r="L920">
+        <v>21.88</v>
+      </c>
+      <c r="M920">
+        <v>15</v>
+      </c>
+      <c r="N920">
+        <v>2</v>
+      </c>
+      <c r="O920">
+        <v>30.4357</v>
+      </c>
+      <c r="P920">
+        <v>86.9790237768633</v>
+      </c>
+      <c r="Q920">
+        <v>34.992</v>
+      </c>
+      <c r="R920">
+        <v>672.5879</v>
+      </c>
+      <c r="S920">
+        <v>6.548682564281482</v>
+      </c>
+      <c r="T920">
+        <v>1329.68995</v>
+      </c>
+      <c r="U920">
+        <v>44</v>
+      </c>
+      <c r="V920">
+        <v>40</v>
+      </c>
+      <c r="W920">
+        <v>84</v>
+      </c>
+      <c r="X920">
+        <v>102</v>
+      </c>
+      <c r="Y920">
+        <v>44</v>
+      </c>
+      <c r="Z920">
+        <v>95</v>
+      </c>
+      <c r="AA920">
+        <v>40</v>
+      </c>
+      <c r="AB920">
+        <v>34</v>
+      </c>
+      <c r="AC920">
+        <v>4.62891</v>
+      </c>
+      <c r="AD920">
+        <v>-2.004</v>
+      </c>
+      <c r="AE920">
+        <v>0</v>
+      </c>
+      <c r="AF920">
+        <v>649.5300100000001</v>
+      </c>
+      <c r="AG920">
+        <v>0</v>
+      </c>
+      <c r="AH920">
+        <v>3</v>
+      </c>
+      <c r="AI920">
+        <v>2017.7637</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B921" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E921">
+        <v>42.73333333333333</v>
+      </c>
+      <c r="F921">
+        <v>2189.89</v>
+      </c>
+      <c r="G921">
+        <v>51.24547581903277</v>
+      </c>
+      <c r="H921">
+        <v>409.4700000000001</v>
+      </c>
+      <c r="I921">
+        <v>0</v>
+      </c>
+      <c r="J921">
+        <v>0</v>
+      </c>
+      <c r="K921">
+        <v>9.581981279251172</v>
+      </c>
+      <c r="L921">
+        <v>0</v>
+      </c>
+      <c r="M921">
+        <v>10</v>
+      </c>
+      <c r="N921">
+        <v>0</v>
+      </c>
+      <c r="O921">
+        <v>29.02122</v>
+      </c>
+      <c r="P921">
+        <v>85.39671610169492</v>
+      </c>
+      <c r="Q921">
+        <v>33.984</v>
+      </c>
+      <c r="R921">
+        <v>216.56808</v>
+      </c>
+      <c r="S921">
+        <v>5.067895787831513</v>
+      </c>
+      <c r="T921">
+        <v>594.52</v>
+      </c>
+      <c r="U921">
+        <v>22</v>
+      </c>
+      <c r="V921">
+        <v>15</v>
+      </c>
+      <c r="W921">
+        <v>37</v>
+      </c>
+      <c r="X921">
+        <v>36</v>
+      </c>
+      <c r="Y921">
+        <v>22</v>
+      </c>
+      <c r="Z921">
+        <v>30</v>
+      </c>
+      <c r="AA921">
+        <v>15</v>
+      </c>
+      <c r="AB921">
+        <v>3</v>
+      </c>
+      <c r="AC921">
+        <v>4.05114</v>
+      </c>
+      <c r="AD921">
+        <v>-2.06619</v>
+      </c>
+      <c r="AE921">
+        <v>0</v>
+      </c>
+      <c r="AF921">
+        <v>202.3352</v>
+      </c>
+      <c r="AG921">
+        <v>0</v>
+      </c>
+      <c r="AH921">
+        <v>3</v>
+      </c>
+      <c r="AI921">
+        <v>649.70424</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B922" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>Futbol Complementario</t>
+        </is>
+      </c>
+      <c r="E922">
+        <v>68.36433333333333</v>
+      </c>
+      <c r="F922">
+        <v>5832.49</v>
+      </c>
+      <c r="G922">
+        <v>85.31480840399233</v>
+      </c>
+      <c r="H922">
+        <v>246.21</v>
+      </c>
+      <c r="I922">
+        <v>0</v>
+      </c>
+      <c r="J922">
+        <v>0</v>
+      </c>
+      <c r="K922">
+        <v>3.601439347027934</v>
+      </c>
+      <c r="L922">
+        <v>0</v>
+      </c>
+      <c r="M922">
+        <v>5</v>
+      </c>
+      <c r="N922">
+        <v>0</v>
+      </c>
+      <c r="O922">
+        <v>28.78942</v>
+      </c>
+      <c r="P922">
+        <v>79.97061111111111</v>
+      </c>
+      <c r="Q922">
+        <v>36</v>
+      </c>
+      <c r="R922">
+        <v>513.9080300000001</v>
+      </c>
+      <c r="S922">
+        <v>7.517195077355152</v>
+      </c>
+      <c r="T922">
+        <v>834.8099999999999</v>
+      </c>
+      <c r="U922">
+        <v>35</v>
+      </c>
+      <c r="V922">
+        <v>23</v>
+      </c>
+      <c r="W922">
+        <v>58</v>
+      </c>
+      <c r="X922">
+        <v>88</v>
+      </c>
+      <c r="Y922">
+        <v>35</v>
+      </c>
+      <c r="Z922">
+        <v>74</v>
+      </c>
+      <c r="AA922">
+        <v>23</v>
+      </c>
+      <c r="AB922">
+        <v>30</v>
+      </c>
+      <c r="AC922">
+        <v>4.45499</v>
+      </c>
+      <c r="AD922">
+        <v>-2.13012</v>
+      </c>
+      <c r="AE922">
+        <v>0</v>
+      </c>
+      <c r="AF922">
+        <v>1387.776</v>
+      </c>
+      <c r="AG922">
+        <v>0</v>
+      </c>
+      <c r="AH922">
+        <v>3</v>
+      </c>
+      <c r="AI922">
+        <v>1541.72409</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B923" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E923">
+        <v>74.93566666666668</v>
+      </c>
+      <c r="F923">
+        <v>3365.76</v>
+      </c>
+      <c r="G923">
+        <v>44.91532736969933</v>
+      </c>
+      <c r="H923">
+        <v>418.94</v>
+      </c>
+      <c r="I923">
+        <v>0</v>
+      </c>
+      <c r="J923">
+        <v>0</v>
+      </c>
+      <c r="K923">
+        <v>5.590662212475589</v>
+      </c>
+      <c r="L923">
+        <v>0</v>
+      </c>
+      <c r="M923">
+        <v>9</v>
+      </c>
+      <c r="N923">
+        <v>0</v>
+      </c>
+      <c r="O923">
+        <v>29.19003</v>
+      </c>
+      <c r="P923">
+        <v>83.41915294924554</v>
+      </c>
+      <c r="Q923">
+        <v>34.992</v>
+      </c>
+      <c r="R923">
+        <v>316.79805</v>
+      </c>
+      <c r="S923">
+        <v>4.227600341626372</v>
+      </c>
+      <c r="T923">
+        <v>688.12999</v>
+      </c>
+      <c r="U923">
+        <v>31</v>
+      </c>
+      <c r="V923">
+        <v>23</v>
+      </c>
+      <c r="W923">
+        <v>54</v>
+      </c>
+      <c r="X923">
+        <v>52</v>
+      </c>
+      <c r="Y923">
+        <v>31</v>
+      </c>
+      <c r="Z923">
+        <v>38</v>
+      </c>
+      <c r="AA923">
+        <v>23</v>
+      </c>
+      <c r="AB923">
+        <v>3</v>
+      </c>
+      <c r="AC923">
+        <v>4.13718</v>
+      </c>
+      <c r="AD923">
+        <v>-2.274</v>
+      </c>
+      <c r="AE923">
+        <v>0</v>
+      </c>
+      <c r="AF923">
+        <v>323.968</v>
+      </c>
+      <c r="AG923">
+        <v>0</v>
+      </c>
+      <c r="AH923">
+        <v>3</v>
+      </c>
+      <c r="AI923">
+        <v>950.39415</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B924" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E924">
+        <v>121.6616666666667</v>
+      </c>
+      <c r="F924">
+        <v>11730.26</v>
+      </c>
+      <c r="G924">
+        <v>96.41705823526995</v>
+      </c>
+      <c r="H924">
+        <v>503.7200000000001</v>
+      </c>
+      <c r="I924">
+        <v>0</v>
+      </c>
+      <c r="J924">
+        <v>0</v>
+      </c>
+      <c r="K924">
+        <v>4.140334534295931</v>
+      </c>
+      <c r="L924">
+        <v>0</v>
+      </c>
+      <c r="M924">
+        <v>8</v>
+      </c>
+      <c r="N924">
+        <v>0</v>
+      </c>
+      <c r="O924">
+        <v>29.05598</v>
+      </c>
+      <c r="P924">
+        <v>88.01641827214347</v>
+      </c>
+      <c r="Q924">
+        <v>33.012</v>
+      </c>
+      <c r="R924">
+        <v>1037.06381</v>
+      </c>
+      <c r="S924">
+        <v>8.524162445031989</v>
+      </c>
+      <c r="T924">
+        <v>1628.22001</v>
+      </c>
+      <c r="U924">
+        <v>21</v>
+      </c>
+      <c r="V924">
+        <v>38</v>
+      </c>
+      <c r="W924">
+        <v>59</v>
+      </c>
+      <c r="X924">
+        <v>129</v>
+      </c>
+      <c r="Y924">
+        <v>21</v>
+      </c>
+      <c r="Z924">
+        <v>121</v>
+      </c>
+      <c r="AA924">
+        <v>38</v>
+      </c>
+      <c r="AB924">
+        <v>43</v>
+      </c>
+      <c r="AC924">
+        <v>6.62846</v>
+      </c>
+      <c r="AD924">
+        <v>-3.42779</v>
+      </c>
+      <c r="AE924">
+        <v>0</v>
+      </c>
+      <c r="AF924">
+        <v>1008.6495</v>
+      </c>
+      <c r="AG924">
+        <v>0</v>
+      </c>
+      <c r="AH924">
+        <v>3</v>
+      </c>
+      <c r="AI924">
+        <v>3111.19143</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B925" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E925">
+        <v>71.64149999999999</v>
+      </c>
+      <c r="F925">
+        <v>7815.13</v>
+      </c>
+      <c r="G925">
+        <v>109.0866327477789</v>
+      </c>
+      <c r="H925">
+        <v>350.45</v>
+      </c>
+      <c r="I925">
+        <v>0</v>
+      </c>
+      <c r="J925">
+        <v>0</v>
+      </c>
+      <c r="K925">
+        <v>4.891717789270187</v>
+      </c>
+      <c r="L925">
+        <v>0</v>
+      </c>
+      <c r="M925">
+        <v>8</v>
+      </c>
+      <c r="N925">
+        <v>0</v>
+      </c>
+      <c r="O925">
+        <v>28.37255</v>
+      </c>
+      <c r="P925">
+        <v>88.65313710786153</v>
+      </c>
+      <c r="Q925">
+        <v>32.004</v>
+      </c>
+      <c r="R925">
+        <v>704.3431</v>
+      </c>
+      <c r="S925">
+        <v>9.831495711284662</v>
+      </c>
+      <c r="T925">
+        <v>1104.76999</v>
+      </c>
+      <c r="U925">
+        <v>16</v>
+      </c>
+      <c r="V925">
+        <v>23</v>
+      </c>
+      <c r="W925">
+        <v>39</v>
+      </c>
+      <c r="X925">
+        <v>84</v>
+      </c>
+      <c r="Y925">
+        <v>16</v>
+      </c>
+      <c r="Z925">
+        <v>79</v>
+      </c>
+      <c r="AA925">
+        <v>23</v>
+      </c>
+      <c r="AB925">
+        <v>21</v>
+      </c>
+      <c r="AC925">
+        <v>3.92201</v>
+      </c>
+      <c r="AD925">
+        <v>-3.90781</v>
+      </c>
+      <c r="AE925">
+        <v>0</v>
+      </c>
+      <c r="AF925">
+        <v>607.7365</v>
+      </c>
+      <c r="AG925">
+        <v>0</v>
+      </c>
+      <c r="AH925">
+        <v>3</v>
+      </c>
+      <c r="AI925">
+        <v>2113.0293</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>Santiago Naveda Lara</t>
+        </is>
+      </c>
+      <c r="B926" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Futbol Complementario</t>
+        </is>
+      </c>
+      <c r="E926">
+        <v>68.36433333333333</v>
+      </c>
+      <c r="F926">
+        <v>7695.389999999999</v>
+      </c>
+      <c r="G926">
+        <v>112.5643976147406</v>
+      </c>
+      <c r="H926">
+        <v>254.65</v>
+      </c>
+      <c r="I926">
+        <v>0</v>
+      </c>
+      <c r="J926">
+        <v>0</v>
+      </c>
+      <c r="K926">
+        <v>3.724895535196228</v>
+      </c>
+      <c r="L926">
+        <v>0</v>
+      </c>
+      <c r="M926">
+        <v>3</v>
+      </c>
+      <c r="N926">
+        <v>0</v>
+      </c>
+      <c r="O926">
+        <v>28.89912</v>
+      </c>
+      <c r="P926">
+        <v>89.69310986964618</v>
+      </c>
+      <c r="Q926">
+        <v>32.22</v>
+      </c>
+      <c r="R926">
+        <v>735.842</v>
+      </c>
+      <c r="S926">
+        <v>10.76353654195901</v>
+      </c>
+      <c r="T926">
+        <v>1159.11001</v>
+      </c>
+      <c r="U926">
+        <v>13</v>
+      </c>
+      <c r="V926">
+        <v>18</v>
+      </c>
+      <c r="W926">
+        <v>31</v>
+      </c>
+      <c r="X926">
+        <v>83</v>
+      </c>
+      <c r="Y926">
+        <v>13</v>
+      </c>
+      <c r="Z926">
+        <v>94</v>
+      </c>
+      <c r="AA926">
+        <v>18</v>
+      </c>
+      <c r="AB926">
+        <v>19</v>
+      </c>
+      <c r="AC926">
+        <v>4.0529</v>
+      </c>
+      <c r="AD926">
+        <v>-1.73636</v>
+      </c>
+      <c r="AE926">
+        <v>0</v>
+      </c>
+      <c r="AF926">
+        <v>696.6320899999999</v>
+      </c>
+      <c r="AG926">
+        <v>0</v>
+      </c>
+      <c r="AH926">
+        <v>3</v>
+      </c>
+      <c r="AI926">
+        <v>2207.526</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B927" s="2">
+        <v>46236</v>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Partido vs Santos J3</t>
+        </is>
+      </c>
+      <c r="E927">
+        <v>101.1783333333333</v>
+      </c>
+      <c r="F927">
+        <v>10684.05</v>
+      </c>
+      <c r="G927">
+        <v>105.596224488115</v>
+      </c>
+      <c r="H927">
+        <v>741.14</v>
+      </c>
+      <c r="I927">
+        <v>19.4</v>
+      </c>
+      <c r="J927">
+        <v>1</v>
+      </c>
+      <c r="K927">
+        <v>7.325086069151828</v>
+      </c>
+      <c r="L927">
+        <v>24.58</v>
+      </c>
+      <c r="M927">
+        <v>14</v>
+      </c>
+      <c r="N927">
+        <v>1</v>
+      </c>
+      <c r="O927">
+        <v>33.23449</v>
+      </c>
+      <c r="P927">
+        <v>94.97739483310473</v>
+      </c>
+      <c r="Q927">
+        <v>34.992</v>
+      </c>
+      <c r="R927">
+        <v>965.11481</v>
+      </c>
+      <c r="S927">
+        <v>9.53874983115621</v>
+      </c>
+      <c r="T927">
+        <v>1869.57</v>
+      </c>
+      <c r="U927">
+        <v>40</v>
+      </c>
+      <c r="V927">
+        <v>60</v>
+      </c>
+      <c r="W927">
+        <v>100</v>
+      </c>
+      <c r="X927">
+        <v>144</v>
+      </c>
+      <c r="Y927">
+        <v>40</v>
+      </c>
+      <c r="Z927">
+        <v>137</v>
+      </c>
+      <c r="AA927">
+        <v>60</v>
+      </c>
+      <c r="AB927">
+        <v>48</v>
+      </c>
+      <c r="AC927">
+        <v>4.52069</v>
+      </c>
+      <c r="AD927">
+        <v>-5.04864</v>
+      </c>
+      <c r="AE927">
+        <v>0</v>
+      </c>
+      <c r="AF927">
+        <v>1024.5856</v>
+      </c>
+      <c r="AG927">
+        <v>0</v>
+      </c>
+      <c r="AH927">
+        <v>3</v>
+      </c>
+      <c r="AI927">
+        <v>2895.34443</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-04
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI927"/>
+  <dimension ref="A1:AI940"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -105066,6 +105066,1470 @@
         <v>2895.34443</v>
       </c>
     </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B928" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E928">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F928">
+        <v>5894.92</v>
+      </c>
+      <c r="G928">
+        <v>81.23454294901241</v>
+      </c>
+      <c r="H928">
+        <v>226.02</v>
+      </c>
+      <c r="I928">
+        <v>0</v>
+      </c>
+      <c r="J928">
+        <v>0</v>
+      </c>
+      <c r="K928">
+        <v>3.114653192466698</v>
+      </c>
+      <c r="L928">
+        <v>0</v>
+      </c>
+      <c r="M928">
+        <v>3</v>
+      </c>
+      <c r="N928">
+        <v>0</v>
+      </c>
+      <c r="O928">
+        <v>28.66225</v>
+      </c>
+      <c r="P928">
+        <v>79.61736111111111</v>
+      </c>
+      <c r="Q928">
+        <v>36</v>
+      </c>
+      <c r="R928">
+        <v>499.57181</v>
+      </c>
+      <c r="S928">
+        <v>6.884315250344511</v>
+      </c>
+      <c r="T928">
+        <v>1087.50999</v>
+      </c>
+      <c r="U928">
+        <v>29</v>
+      </c>
+      <c r="V928">
+        <v>38</v>
+      </c>
+      <c r="W928">
+        <v>67</v>
+      </c>
+      <c r="X928">
+        <v>111</v>
+      </c>
+      <c r="Y928">
+        <v>29</v>
+      </c>
+      <c r="Z928">
+        <v>112</v>
+      </c>
+      <c r="AA928">
+        <v>38</v>
+      </c>
+      <c r="AB928">
+        <v>28</v>
+      </c>
+      <c r="AC928">
+        <v>4.19117</v>
+      </c>
+      <c r="AD928">
+        <v>-3.02728</v>
+      </c>
+      <c r="AE928">
+        <v>0</v>
+      </c>
+      <c r="AF928">
+        <v>1446.886</v>
+      </c>
+      <c r="AG928">
+        <v>0</v>
+      </c>
+      <c r="AH928">
+        <v>3</v>
+      </c>
+      <c r="AI928">
+        <v>1498.71543</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B929" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E929">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F929">
+        <v>6022.78</v>
+      </c>
+      <c r="G929">
+        <v>82.99650895728067</v>
+      </c>
+      <c r="H929">
+        <v>201.88</v>
+      </c>
+      <c r="I929">
+        <v>0</v>
+      </c>
+      <c r="J929">
+        <v>0</v>
+      </c>
+      <c r="K929">
+        <v>2.781993569131833</v>
+      </c>
+      <c r="L929">
+        <v>3.28</v>
+      </c>
+      <c r="M929">
+        <v>4</v>
+      </c>
+      <c r="N929">
+        <v>0</v>
+      </c>
+      <c r="O929">
+        <v>30.14997</v>
+      </c>
+      <c r="P929">
+        <v>84.68141220087631</v>
+      </c>
+      <c r="Q929">
+        <v>35.604</v>
+      </c>
+      <c r="R929">
+        <v>493.12993</v>
+      </c>
+      <c r="S929">
+        <v>6.795543362425357</v>
+      </c>
+      <c r="T929">
+        <v>967.62996</v>
+      </c>
+      <c r="U929">
+        <v>21</v>
+      </c>
+      <c r="V929">
+        <v>24</v>
+      </c>
+      <c r="W929">
+        <v>45</v>
+      </c>
+      <c r="X929">
+        <v>90</v>
+      </c>
+      <c r="Y929">
+        <v>21</v>
+      </c>
+      <c r="Z929">
+        <v>71</v>
+      </c>
+      <c r="AA929">
+        <v>24</v>
+      </c>
+      <c r="AB929">
+        <v>14</v>
+      </c>
+      <c r="AC929">
+        <v>4.15292</v>
+      </c>
+      <c r="AD929">
+        <v>-2.44576</v>
+      </c>
+      <c r="AE929">
+        <v>0</v>
+      </c>
+      <c r="AF929">
+        <v>512.8088600000001</v>
+      </c>
+      <c r="AG929">
+        <v>0</v>
+      </c>
+      <c r="AH929">
+        <v>3</v>
+      </c>
+      <c r="AI929">
+        <v>1479.38979</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B930" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E930">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F930">
+        <v>6319.639999999999</v>
+      </c>
+      <c r="G930">
+        <v>87.08736793752871</v>
+      </c>
+      <c r="H930">
+        <v>394.38</v>
+      </c>
+      <c r="I930">
+        <v>0</v>
+      </c>
+      <c r="J930">
+        <v>0</v>
+      </c>
+      <c r="K930">
+        <v>5.434726688102894</v>
+      </c>
+      <c r="L930">
+        <v>21.68</v>
+      </c>
+      <c r="M930">
+        <v>9</v>
+      </c>
+      <c r="N930">
+        <v>1</v>
+      </c>
+      <c r="O930">
+        <v>31.62448</v>
+      </c>
+      <c r="P930">
+        <v>88.9127305443095</v>
+      </c>
+      <c r="Q930">
+        <v>35.568</v>
+      </c>
+      <c r="R930">
+        <v>548.48961</v>
+      </c>
+      <c r="S930">
+        <v>7.558423656407901</v>
+      </c>
+      <c r="T930">
+        <v>1133.19003</v>
+      </c>
+      <c r="U930">
+        <v>30</v>
+      </c>
+      <c r="V930">
+        <v>21</v>
+      </c>
+      <c r="W930">
+        <v>51</v>
+      </c>
+      <c r="X930">
+        <v>92</v>
+      </c>
+      <c r="Y930">
+        <v>30</v>
+      </c>
+      <c r="Z930">
+        <v>66</v>
+      </c>
+      <c r="AA930">
+        <v>21</v>
+      </c>
+      <c r="AB930">
+        <v>4</v>
+      </c>
+      <c r="AC930">
+        <v>4.64556</v>
+      </c>
+      <c r="AD930">
+        <v>-2.67443</v>
+      </c>
+      <c r="AE930">
+        <v>0</v>
+      </c>
+      <c r="AF930">
+        <v>612.2776000000001</v>
+      </c>
+      <c r="AG930">
+        <v>0</v>
+      </c>
+      <c r="AH930">
+        <v>3</v>
+      </c>
+      <c r="AI930">
+        <v>1645.46883</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B931" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E931">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F931">
+        <v>6124.53</v>
+      </c>
+      <c r="G931">
+        <v>84.39866789159393</v>
+      </c>
+      <c r="H931">
+        <v>419.61</v>
+      </c>
+      <c r="I931">
+        <v>0</v>
+      </c>
+      <c r="J931">
+        <v>0</v>
+      </c>
+      <c r="K931">
+        <v>5.782406982085439</v>
+      </c>
+      <c r="L931">
+        <v>3.33</v>
+      </c>
+      <c r="M931">
+        <v>9</v>
+      </c>
+      <c r="N931">
+        <v>0</v>
+      </c>
+      <c r="O931">
+        <v>29.97624</v>
+      </c>
+      <c r="P931">
+        <v>83.26733333333334</v>
+      </c>
+      <c r="Q931">
+        <v>36</v>
+      </c>
+      <c r="R931">
+        <v>572.36513</v>
+      </c>
+      <c r="S931">
+        <v>7.887438631143777</v>
+      </c>
+      <c r="T931">
+        <v>1143.81001</v>
+      </c>
+      <c r="U931">
+        <v>15</v>
+      </c>
+      <c r="V931">
+        <v>17</v>
+      </c>
+      <c r="W931">
+        <v>32</v>
+      </c>
+      <c r="X931">
+        <v>88</v>
+      </c>
+      <c r="Y931">
+        <v>15</v>
+      </c>
+      <c r="Z931">
+        <v>72</v>
+      </c>
+      <c r="AA931">
+        <v>17</v>
+      </c>
+      <c r="AB931">
+        <v>13</v>
+      </c>
+      <c r="AC931">
+        <v>4.06989</v>
+      </c>
+      <c r="AD931">
+        <v>-2.2351</v>
+      </c>
+      <c r="AE931">
+        <v>0</v>
+      </c>
+      <c r="AF931">
+        <v>1452.798</v>
+      </c>
+      <c r="AG931">
+        <v>0</v>
+      </c>
+      <c r="AH931">
+        <v>3</v>
+      </c>
+      <c r="AI931">
+        <v>1717.09539</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B932" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E932">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F932">
+        <v>5782.129999999999</v>
+      </c>
+      <c r="G932">
+        <v>79.68024804777215</v>
+      </c>
+      <c r="H932">
+        <v>257.23</v>
+      </c>
+      <c r="I932">
+        <v>0</v>
+      </c>
+      <c r="J932">
+        <v>0</v>
+      </c>
+      <c r="K932">
+        <v>3.54474046853468</v>
+      </c>
+      <c r="L932">
+        <v>0</v>
+      </c>
+      <c r="M932">
+        <v>9</v>
+      </c>
+      <c r="N932">
+        <v>0</v>
+      </c>
+      <c r="O932">
+        <v>29.85604</v>
+      </c>
+      <c r="P932">
+        <v>82.93344444444445</v>
+      </c>
+      <c r="Q932">
+        <v>36</v>
+      </c>
+      <c r="R932">
+        <v>538.60717</v>
+      </c>
+      <c r="S932">
+        <v>7.422239366100138</v>
+      </c>
+      <c r="T932">
+        <v>894.56999</v>
+      </c>
+      <c r="U932">
+        <v>18</v>
+      </c>
+      <c r="V932">
+        <v>24</v>
+      </c>
+      <c r="W932">
+        <v>42</v>
+      </c>
+      <c r="X932">
+        <v>82</v>
+      </c>
+      <c r="Y932">
+        <v>18</v>
+      </c>
+      <c r="Z932">
+        <v>72</v>
+      </c>
+      <c r="AA932">
+        <v>24</v>
+      </c>
+      <c r="AB932">
+        <v>16</v>
+      </c>
+      <c r="AC932">
+        <v>3.78266</v>
+      </c>
+      <c r="AD932">
+        <v>-3.33537</v>
+      </c>
+      <c r="AE932">
+        <v>0</v>
+      </c>
+      <c r="AF932">
+        <v>485.275</v>
+      </c>
+      <c r="AG932">
+        <v>0</v>
+      </c>
+      <c r="AH932">
+        <v>3</v>
+      </c>
+      <c r="AI932">
+        <v>1615.82151</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>Esteban Lozano</t>
+        </is>
+      </c>
+      <c r="B933" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E933">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F933">
+        <v>6158.64</v>
+      </c>
+      <c r="G933">
+        <v>84.86871841984383</v>
+      </c>
+      <c r="H933">
+        <v>321.16</v>
+      </c>
+      <c r="I933">
+        <v>0</v>
+      </c>
+      <c r="J933">
+        <v>0</v>
+      </c>
+      <c r="K933">
+        <v>4.425723472668811</v>
+      </c>
+      <c r="L933">
+        <v>20.71</v>
+      </c>
+      <c r="M933">
+        <v>10</v>
+      </c>
+      <c r="N933">
+        <v>1</v>
+      </c>
+      <c r="O933">
+        <v>31.36859</v>
+      </c>
+      <c r="P933">
+        <v>101.3197351421189</v>
+      </c>
+      <c r="Q933">
+        <v>30.96</v>
+      </c>
+      <c r="R933">
+        <v>550.88941</v>
+      </c>
+      <c r="S933">
+        <v>7.591493936610014</v>
+      </c>
+      <c r="T933">
+        <v>765.25</v>
+      </c>
+      <c r="U933">
+        <v>14</v>
+      </c>
+      <c r="V933">
+        <v>15</v>
+      </c>
+      <c r="W933">
+        <v>29</v>
+      </c>
+      <c r="X933">
+        <v>63</v>
+      </c>
+      <c r="Y933">
+        <v>14</v>
+      </c>
+      <c r="Z933">
+        <v>54</v>
+      </c>
+      <c r="AA933">
+        <v>15</v>
+      </c>
+      <c r="AB933">
+        <v>10</v>
+      </c>
+      <c r="AC933">
+        <v>4.20574</v>
+      </c>
+      <c r="AD933">
+        <v>-2.66163</v>
+      </c>
+      <c r="AE933">
+        <v>0</v>
+      </c>
+      <c r="AF933">
+        <v>500.3369</v>
+      </c>
+      <c r="AG933">
+        <v>0</v>
+      </c>
+      <c r="AH933">
+        <v>3</v>
+      </c>
+      <c r="AI933">
+        <v>1652.66823</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B934" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E934">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F934">
+        <v>6333.809999999999</v>
+      </c>
+      <c r="G934">
+        <v>87.28263665594855</v>
+      </c>
+      <c r="H934">
+        <v>200.02</v>
+      </c>
+      <c r="I934">
+        <v>0</v>
+      </c>
+      <c r="J934">
+        <v>0</v>
+      </c>
+      <c r="K934">
+        <v>2.756361966008269</v>
+      </c>
+      <c r="L934">
+        <v>0</v>
+      </c>
+      <c r="M934">
+        <v>3</v>
+      </c>
+      <c r="N934">
+        <v>0</v>
+      </c>
+      <c r="O934">
+        <v>28.56964</v>
+      </c>
+      <c r="P934">
+        <v>79.36011111111111</v>
+      </c>
+      <c r="Q934">
+        <v>36</v>
+      </c>
+      <c r="R934">
+        <v>699.9879999999999</v>
+      </c>
+      <c r="S934">
+        <v>9.646136885622417</v>
+      </c>
+      <c r="T934">
+        <v>854.29999</v>
+      </c>
+      <c r="U934">
+        <v>15</v>
+      </c>
+      <c r="V934">
+        <v>16</v>
+      </c>
+      <c r="W934">
+        <v>31</v>
+      </c>
+      <c r="X934">
+        <v>77</v>
+      </c>
+      <c r="Y934">
+        <v>15</v>
+      </c>
+      <c r="Z934">
+        <v>55</v>
+      </c>
+      <c r="AA934">
+        <v>16</v>
+      </c>
+      <c r="AB934">
+        <v>15</v>
+      </c>
+      <c r="AC934">
+        <v>4.56755</v>
+      </c>
+      <c r="AD934">
+        <v>-2.36572</v>
+      </c>
+      <c r="AE934">
+        <v>0</v>
+      </c>
+      <c r="AF934">
+        <v>1485.374</v>
+      </c>
+      <c r="AG934">
+        <v>0</v>
+      </c>
+      <c r="AH934">
+        <v>3</v>
+      </c>
+      <c r="AI934">
+        <v>2099.964</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B935" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E935">
+        <v>39.61666666666667</v>
+      </c>
+      <c r="F935">
+        <v>2614.87</v>
+      </c>
+      <c r="G935">
+        <v>66.00429112326462</v>
+      </c>
+      <c r="H935">
+        <v>69.07000000000001</v>
+      </c>
+      <c r="I935">
+        <v>0</v>
+      </c>
+      <c r="J935">
+        <v>0</v>
+      </c>
+      <c r="K935">
+        <v>1.743458140513252</v>
+      </c>
+      <c r="L935">
+        <v>0</v>
+      </c>
+      <c r="M935">
+        <v>1</v>
+      </c>
+      <c r="N935">
+        <v>0</v>
+      </c>
+      <c r="O935">
+        <v>25.45526</v>
+      </c>
+      <c r="P935">
+        <v>77.10911183811947</v>
+      </c>
+      <c r="Q935">
+        <v>33.012</v>
+      </c>
+      <c r="R935">
+        <v>240.00802</v>
+      </c>
+      <c r="S935">
+        <v>6.058258813630626</v>
+      </c>
+      <c r="T935">
+        <v>318.17</v>
+      </c>
+      <c r="U935">
+        <v>15</v>
+      </c>
+      <c r="V935">
+        <v>11</v>
+      </c>
+      <c r="W935">
+        <v>26</v>
+      </c>
+      <c r="X935">
+        <v>38</v>
+      </c>
+      <c r="Y935">
+        <v>15</v>
+      </c>
+      <c r="Z935">
+        <v>26</v>
+      </c>
+      <c r="AA935">
+        <v>11</v>
+      </c>
+      <c r="AB935">
+        <v>2</v>
+      </c>
+      <c r="AC935">
+        <v>4.39625</v>
+      </c>
+      <c r="AD935">
+        <v>-1.72605</v>
+      </c>
+      <c r="AE935">
+        <v>0</v>
+      </c>
+      <c r="AF935">
+        <v>242.94972</v>
+      </c>
+      <c r="AG935">
+        <v>0</v>
+      </c>
+      <c r="AH935">
+        <v>3</v>
+      </c>
+      <c r="AI935">
+        <v>720.02406</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>Kevin Álvarez</t>
+        </is>
+      </c>
+      <c r="B936" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E936">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F936">
+        <v>6189.950000000001</v>
+      </c>
+      <c r="G936">
+        <v>85.3001837390905</v>
+      </c>
+      <c r="H936">
+        <v>273.77</v>
+      </c>
+      <c r="I936">
+        <v>0</v>
+      </c>
+      <c r="J936">
+        <v>0</v>
+      </c>
+      <c r="K936">
+        <v>3.772668810289389</v>
+      </c>
+      <c r="L936">
+        <v>0</v>
+      </c>
+      <c r="M936">
+        <v>3</v>
+      </c>
+      <c r="N936">
+        <v>0</v>
+      </c>
+      <c r="O936">
+        <v>27.30635</v>
+      </c>
+      <c r="P936">
+        <v>78.035979652492</v>
+      </c>
+      <c r="Q936">
+        <v>34.992</v>
+      </c>
+      <c r="R936">
+        <v>489.79407</v>
+      </c>
+      <c r="S936">
+        <v>6.749573771244832</v>
+      </c>
+      <c r="T936">
+        <v>1112.19</v>
+      </c>
+      <c r="U936">
+        <v>29</v>
+      </c>
+      <c r="V936">
+        <v>25</v>
+      </c>
+      <c r="W936">
+        <v>54</v>
+      </c>
+      <c r="X936">
+        <v>104</v>
+      </c>
+      <c r="Y936">
+        <v>29</v>
+      </c>
+      <c r="Z936">
+        <v>75</v>
+      </c>
+      <c r="AA936">
+        <v>25</v>
+      </c>
+      <c r="AB936">
+        <v>6</v>
+      </c>
+      <c r="AC936">
+        <v>4.55579</v>
+      </c>
+      <c r="AD936">
+        <v>-2.60035</v>
+      </c>
+      <c r="AE936">
+        <v>0</v>
+      </c>
+      <c r="AF936">
+        <v>537.65602</v>
+      </c>
+      <c r="AG936">
+        <v>0</v>
+      </c>
+      <c r="AH936">
+        <v>3</v>
+      </c>
+      <c r="AI936">
+        <v>1469.38221</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B937" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E937">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F937">
+        <v>6066.4</v>
+      </c>
+      <c r="G937">
+        <v>83.59761139182361</v>
+      </c>
+      <c r="H937">
+        <v>172.49</v>
+      </c>
+      <c r="I937">
+        <v>0</v>
+      </c>
+      <c r="J937">
+        <v>0</v>
+      </c>
+      <c r="K937">
+        <v>2.376986678915939</v>
+      </c>
+      <c r="L937">
+        <v>0</v>
+      </c>
+      <c r="M937">
+        <v>4</v>
+      </c>
+      <c r="N937">
+        <v>0</v>
+      </c>
+      <c r="O937">
+        <v>29.40873</v>
+      </c>
+      <c r="P937">
+        <v>86.53698799435028</v>
+      </c>
+      <c r="Q937">
+        <v>33.984</v>
+      </c>
+      <c r="R937">
+        <v>572.65943</v>
+      </c>
+      <c r="S937">
+        <v>7.89149421221865</v>
+      </c>
+      <c r="T937">
+        <v>904.98999</v>
+      </c>
+      <c r="U937">
+        <v>11</v>
+      </c>
+      <c r="V937">
+        <v>16</v>
+      </c>
+      <c r="W937">
+        <v>27</v>
+      </c>
+      <c r="X937">
+        <v>69</v>
+      </c>
+      <c r="Y937">
+        <v>11</v>
+      </c>
+      <c r="Z937">
+        <v>61</v>
+      </c>
+      <c r="AA937">
+        <v>16</v>
+      </c>
+      <c r="AB937">
+        <v>7</v>
+      </c>
+      <c r="AC937">
+        <v>4.05792</v>
+      </c>
+      <c r="AD937">
+        <v>-2.53831</v>
+      </c>
+      <c r="AE937">
+        <v>0</v>
+      </c>
+      <c r="AF937">
+        <v>570.712</v>
+      </c>
+      <c r="AG937">
+        <v>0</v>
+      </c>
+      <c r="AH937">
+        <v>3</v>
+      </c>
+      <c r="AI937">
+        <v>1717.97829</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B938" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E938">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F938">
+        <v>6022.040000000001</v>
+      </c>
+      <c r="G938">
+        <v>82.9863114377584</v>
+      </c>
+      <c r="H938">
+        <v>311.46</v>
+      </c>
+      <c r="I938">
+        <v>0</v>
+      </c>
+      <c r="J938">
+        <v>0</v>
+      </c>
+      <c r="K938">
+        <v>4.292053284336243</v>
+      </c>
+      <c r="L938">
+        <v>0</v>
+      </c>
+      <c r="M938">
+        <v>7</v>
+      </c>
+      <c r="N938">
+        <v>0</v>
+      </c>
+      <c r="O938">
+        <v>28.47937</v>
+      </c>
+      <c r="P938">
+        <v>81.38823159579333</v>
+      </c>
+      <c r="Q938">
+        <v>34.992</v>
+      </c>
+      <c r="R938">
+        <v>473.6526</v>
+      </c>
+      <c r="S938">
+        <v>6.527137344970143</v>
+      </c>
+      <c r="T938">
+        <v>1192.73997</v>
+      </c>
+      <c r="U938">
+        <v>15</v>
+      </c>
+      <c r="V938">
+        <v>19</v>
+      </c>
+      <c r="W938">
+        <v>34</v>
+      </c>
+      <c r="X938">
+        <v>90</v>
+      </c>
+      <c r="Y938">
+        <v>15</v>
+      </c>
+      <c r="Z938">
+        <v>93</v>
+      </c>
+      <c r="AA938">
+        <v>19</v>
+      </c>
+      <c r="AB938">
+        <v>12</v>
+      </c>
+      <c r="AC938">
+        <v>4.51414</v>
+      </c>
+      <c r="AD938">
+        <v>-2.60353</v>
+      </c>
+      <c r="AE938">
+        <v>0</v>
+      </c>
+      <c r="AF938">
+        <v>586.4256</v>
+      </c>
+      <c r="AG938">
+        <v>0</v>
+      </c>
+      <c r="AH938">
+        <v>3</v>
+      </c>
+      <c r="AI938">
+        <v>1420.9578</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>Santiago Naveda Lara</t>
+        </is>
+      </c>
+      <c r="B939" s="2">
+        <v>46237</v>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>MD+1</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Sesión 48</t>
+        </is>
+      </c>
+      <c r="E939">
+        <v>72.56666666666666</v>
+      </c>
+      <c r="F939">
+        <v>6571.469999999999</v>
+      </c>
+      <c r="G939">
+        <v>90.55769407441433</v>
+      </c>
+      <c r="H939">
+        <v>55.08</v>
+      </c>
+      <c r="I939">
+        <v>0</v>
+      </c>
+      <c r="J939">
+        <v>0</v>
+      </c>
+      <c r="K939">
+        <v>0.759026182820395</v>
+      </c>
+      <c r="L939">
+        <v>0</v>
+      </c>
+      <c r="M939">
+        <v>1</v>
+      </c>
+      <c r="N939">
+        <v>0</v>
+      </c>
+      <c r="O939">
+        <v>25.47779</v>
+      </c>
+      <c r="P939">
+        <v>79.07445685909373</v>
+      </c>
+      <c r="Q939">
+        <v>32.22</v>
+      </c>
+      <c r="R939">
+        <v>638.1908099999999</v>
+      </c>
+      <c r="S939">
+        <v>8.794544924207624</v>
+      </c>
+      <c r="T939">
+        <v>971.25999</v>
+      </c>
+      <c r="U939">
+        <v>20</v>
+      </c>
+      <c r="V939">
+        <v>24</v>
+      </c>
+      <c r="W939">
+        <v>44</v>
+      </c>
+      <c r="X939">
+        <v>100</v>
+      </c>
+      <c r="Y939">
+        <v>20</v>
+      </c>
+      <c r="Z939">
+        <v>69</v>
+      </c>
+      <c r="AA939">
+        <v>24</v>
+      </c>
+      <c r="AB939">
+        <v>13</v>
+      </c>
+      <c r="AC939">
+        <v>3.65665</v>
+      </c>
+      <c r="AD939">
+        <v>-2.27776</v>
+      </c>
+      <c r="AE939">
+        <v>0</v>
+      </c>
+      <c r="AF939">
+        <v>601.72343</v>
+      </c>
+      <c r="AG939">
+        <v>0</v>
+      </c>
+      <c r="AH939">
+        <v>3</v>
+      </c>
+      <c r="AI939">
+        <v>1914.57243</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B940" s="2">
+        <v>46237</v>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>RTP</t>
+        </is>
+      </c>
+      <c r="E940">
+        <v>51.51483333333333</v>
+      </c>
+      <c r="F940">
+        <v>2294.88</v>
+      </c>
+      <c r="G940">
+        <v>44.54794573731191</v>
+      </c>
+      <c r="H940">
+        <v>1.69</v>
+      </c>
+      <c r="I940">
+        <v>0</v>
+      </c>
+      <c r="J940">
+        <v>0</v>
+      </c>
+      <c r="K940">
+        <v>0.03280608497876017</v>
+      </c>
+      <c r="L940">
+        <v>0</v>
+      </c>
+      <c r="M940">
+        <v>0</v>
+      </c>
+      <c r="N940">
+        <v>0</v>
+      </c>
+      <c r="O940">
+        <v>20.91537</v>
+      </c>
+      <c r="P940">
+        <v>61.54475635593219</v>
+      </c>
+      <c r="Q940">
+        <v>33.984</v>
+      </c>
+      <c r="R940">
+        <v>313.27186</v>
+      </c>
+      <c r="S940">
+        <v>6.081197195629739</v>
+      </c>
+      <c r="T940">
+        <v>406.37001</v>
+      </c>
+      <c r="U940">
+        <v>21</v>
+      </c>
+      <c r="V940">
+        <v>24</v>
+      </c>
+      <c r="W940">
+        <v>45</v>
+      </c>
+      <c r="X940">
+        <v>51</v>
+      </c>
+      <c r="Y940">
+        <v>21</v>
+      </c>
+      <c r="Z940">
+        <v>36</v>
+      </c>
+      <c r="AA940">
+        <v>24</v>
+      </c>
+      <c r="AB940">
+        <v>13</v>
+      </c>
+      <c r="AC940">
+        <v>3.70483</v>
+      </c>
+      <c r="AD940">
+        <v>-2.23701</v>
+      </c>
+      <c r="AE940">
+        <v>0</v>
+      </c>
+      <c r="AF940">
+        <v>201.1989</v>
+      </c>
+      <c r="AG940">
+        <v>0</v>
+      </c>
+      <c r="AH940">
+        <v>3</v>
+      </c>
+      <c r="AI940">
+        <v>939.81558</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-05
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI940"/>
+  <dimension ref="A1:AI963"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
@@ -106530,6 +106530,2605 @@
         <v>939.81558</v>
       </c>
     </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>Adrian Fernandez</t>
+        </is>
+      </c>
+      <c r="B941" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E941">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F941">
+        <v>3308.85</v>
+      </c>
+      <c r="G941">
+        <v>36.18866204885162</v>
+      </c>
+      <c r="H941">
+        <v>40.21</v>
+      </c>
+      <c r="I941">
+        <v>0</v>
+      </c>
+      <c r="J941">
+        <v>0</v>
+      </c>
+      <c r="K941">
+        <v>0.4397739701057237</v>
+      </c>
+      <c r="L941">
+        <v>0</v>
+      </c>
+      <c r="M941">
+        <v>0</v>
+      </c>
+      <c r="N941">
+        <v>0</v>
+      </c>
+      <c r="O941">
+        <v>25.00356</v>
+      </c>
+      <c r="P941">
+        <v>69.45433333333332</v>
+      </c>
+      <c r="Q941">
+        <v>36</v>
+      </c>
+      <c r="R941">
+        <v>297.43755</v>
+      </c>
+      <c r="S941">
+        <v>3.253053773240977</v>
+      </c>
+      <c r="T941">
+        <v>333.76999</v>
+      </c>
+      <c r="U941">
+        <v>11</v>
+      </c>
+      <c r="V941">
+        <v>9</v>
+      </c>
+      <c r="W941">
+        <v>20</v>
+      </c>
+      <c r="X941">
+        <v>39</v>
+      </c>
+      <c r="Y941">
+        <v>11</v>
+      </c>
+      <c r="Z941">
+        <v>32</v>
+      </c>
+      <c r="AA941">
+        <v>9</v>
+      </c>
+      <c r="AB941">
+        <v>19</v>
+      </c>
+      <c r="AC941">
+        <v>4.11145</v>
+      </c>
+      <c r="AD941">
+        <v>-2.88389</v>
+      </c>
+      <c r="AE941">
+        <v>0</v>
+      </c>
+      <c r="AF941">
+        <v>747.97</v>
+      </c>
+      <c r="AG941">
+        <v>0</v>
+      </c>
+      <c r="AH941">
+        <v>3</v>
+      </c>
+      <c r="AI941">
+        <v>892.31265</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>Alan Cervantes</t>
+        </is>
+      </c>
+      <c r="B942" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E942">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F942">
+        <v>4054.53</v>
+      </c>
+      <c r="G942">
+        <v>44.34411228581844</v>
+      </c>
+      <c r="H942">
+        <v>2.81</v>
+      </c>
+      <c r="I942">
+        <v>0</v>
+      </c>
+      <c r="J942">
+        <v>0</v>
+      </c>
+      <c r="K942">
+        <v>0.03073277433467007</v>
+      </c>
+      <c r="L942">
+        <v>0</v>
+      </c>
+      <c r="M942">
+        <v>0</v>
+      </c>
+      <c r="N942">
+        <v>0</v>
+      </c>
+      <c r="O942">
+        <v>21.15754</v>
+      </c>
+      <c r="P942">
+        <v>78.15897225994352</v>
+      </c>
+      <c r="Q942">
+        <v>27.06988</v>
+      </c>
+      <c r="R942">
+        <v>413.9861</v>
+      </c>
+      <c r="S942">
+        <v>4.527737149106817</v>
+      </c>
+      <c r="T942">
+        <v>200.05</v>
+      </c>
+      <c r="U942">
+        <v>2</v>
+      </c>
+      <c r="V942">
+        <v>2</v>
+      </c>
+      <c r="W942">
+        <v>4</v>
+      </c>
+      <c r="X942">
+        <v>22</v>
+      </c>
+      <c r="Y942">
+        <v>2</v>
+      </c>
+      <c r="Z942">
+        <v>11</v>
+      </c>
+      <c r="AA942">
+        <v>2</v>
+      </c>
+      <c r="AB942">
+        <v>9</v>
+      </c>
+      <c r="AC942">
+        <v>3.41081</v>
+      </c>
+      <c r="AD942">
+        <v>-2.51202</v>
+      </c>
+      <c r="AE942">
+        <v>0</v>
+      </c>
+      <c r="AF942">
+        <v>304.5833</v>
+      </c>
+      <c r="AG942">
+        <v>0</v>
+      </c>
+      <c r="AH942">
+        <v>3</v>
+      </c>
+      <c r="AI942">
+        <v>1241.9583</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>Alejandro Cardenas</t>
+        </is>
+      </c>
+      <c r="B943" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E943">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F943">
+        <v>3741.62</v>
+      </c>
+      <c r="G943">
+        <v>40.92183740430186</v>
+      </c>
+      <c r="H943">
+        <v>28.52</v>
+      </c>
+      <c r="I943">
+        <v>0</v>
+      </c>
+      <c r="J943">
+        <v>0</v>
+      </c>
+      <c r="K943">
+        <v>0.3119212541013489</v>
+      </c>
+      <c r="L943">
+        <v>0</v>
+      </c>
+      <c r="M943">
+        <v>1</v>
+      </c>
+      <c r="N943">
+        <v>0</v>
+      </c>
+      <c r="O943">
+        <v>25.42098</v>
+      </c>
+      <c r="P943">
+        <v>70.61383333333333</v>
+      </c>
+      <c r="Q943">
+        <v>36</v>
+      </c>
+      <c r="R943">
+        <v>315.12982</v>
+      </c>
+      <c r="S943">
+        <v>3.446552898286547</v>
+      </c>
+      <c r="T943">
+        <v>340.14001</v>
+      </c>
+      <c r="U943">
+        <v>10</v>
+      </c>
+      <c r="V943">
+        <v>9</v>
+      </c>
+      <c r="W943">
+        <v>19</v>
+      </c>
+      <c r="X943">
+        <v>36</v>
+      </c>
+      <c r="Y943">
+        <v>10</v>
+      </c>
+      <c r="Z943">
+        <v>29</v>
+      </c>
+      <c r="AA943">
+        <v>9</v>
+      </c>
+      <c r="AB943">
+        <v>25</v>
+      </c>
+      <c r="AC943">
+        <v>4.23188</v>
+      </c>
+      <c r="AD943">
+        <v>-2.11111</v>
+      </c>
+      <c r="AE943">
+        <v>0</v>
+      </c>
+      <c r="AF943">
+        <v>858.5260000000001</v>
+      </c>
+      <c r="AG943">
+        <v>0</v>
+      </c>
+      <c r="AH943">
+        <v>3</v>
+      </c>
+      <c r="AI943">
+        <v>945.38946</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>Brian Rodríguez</t>
+        </is>
+      </c>
+      <c r="B944" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E944">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F944">
+        <v>3550.88</v>
+      </c>
+      <c r="G944">
+        <v>38.83572730586948</v>
+      </c>
+      <c r="H944">
+        <v>8.85</v>
+      </c>
+      <c r="I944">
+        <v>0</v>
+      </c>
+      <c r="J944">
+        <v>0</v>
+      </c>
+      <c r="K944">
+        <v>0.09679183375865839</v>
+      </c>
+      <c r="L944">
+        <v>0</v>
+      </c>
+      <c r="M944">
+        <v>0</v>
+      </c>
+      <c r="N944">
+        <v>0</v>
+      </c>
+      <c r="O944">
+        <v>22.66763</v>
+      </c>
+      <c r="P944">
+        <v>63.66596449837096</v>
+      </c>
+      <c r="Q944">
+        <v>35.604</v>
+      </c>
+      <c r="R944">
+        <v>289.7772</v>
+      </c>
+      <c r="S944">
+        <v>3.16927305869486</v>
+      </c>
+      <c r="T944">
+        <v>221.69</v>
+      </c>
+      <c r="U944">
+        <v>13</v>
+      </c>
+      <c r="V944">
+        <v>5</v>
+      </c>
+      <c r="W944">
+        <v>18</v>
+      </c>
+      <c r="X944">
+        <v>33</v>
+      </c>
+      <c r="Y944">
+        <v>13</v>
+      </c>
+      <c r="Z944">
+        <v>19</v>
+      </c>
+      <c r="AA944">
+        <v>5</v>
+      </c>
+      <c r="AB944">
+        <v>12</v>
+      </c>
+      <c r="AC944">
+        <v>4.11346</v>
+      </c>
+      <c r="AD944">
+        <v>-2.34301</v>
+      </c>
+      <c r="AE944">
+        <v>0</v>
+      </c>
+      <c r="AF944">
+        <v>278.98527</v>
+      </c>
+      <c r="AG944">
+        <v>0</v>
+      </c>
+      <c r="AH944">
+        <v>3</v>
+      </c>
+      <c r="AI944">
+        <v>869.3316</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>Cristian Borja</t>
+        </is>
+      </c>
+      <c r="B945" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E945">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F945">
+        <v>3695.69</v>
+      </c>
+      <c r="G945">
+        <v>40.41950419248997</v>
+      </c>
+      <c r="H945">
+        <v>40.62</v>
+      </c>
+      <c r="I945">
+        <v>0</v>
+      </c>
+      <c r="J945">
+        <v>0</v>
+      </c>
+      <c r="K945">
+        <v>0.4442581115566898</v>
+      </c>
+      <c r="L945">
+        <v>0</v>
+      </c>
+      <c r="M945">
+        <v>0</v>
+      </c>
+      <c r="N945">
+        <v>0</v>
+      </c>
+      <c r="O945">
+        <v>23.81357</v>
+      </c>
+      <c r="P945">
+        <v>70.0728872410546</v>
+      </c>
+      <c r="Q945">
+        <v>33.984</v>
+      </c>
+      <c r="R945">
+        <v>415.12773</v>
+      </c>
+      <c r="S945">
+        <v>4.540223076923077</v>
+      </c>
+      <c r="T945">
+        <v>265.72</v>
+      </c>
+      <c r="U945">
+        <v>8</v>
+      </c>
+      <c r="V945">
+        <v>3</v>
+      </c>
+      <c r="W945">
+        <v>11</v>
+      </c>
+      <c r="X945">
+        <v>29</v>
+      </c>
+      <c r="Y945">
+        <v>8</v>
+      </c>
+      <c r="Z945">
+        <v>16</v>
+      </c>
+      <c r="AA945">
+        <v>3</v>
+      </c>
+      <c r="AB945">
+        <v>22</v>
+      </c>
+      <c r="AC945">
+        <v>4.05656</v>
+      </c>
+      <c r="AD945">
+        <v>-1.58249</v>
+      </c>
+      <c r="AE945">
+        <v>0</v>
+      </c>
+      <c r="AF945">
+        <v>326.2888</v>
+      </c>
+      <c r="AG945">
+        <v>0</v>
+      </c>
+      <c r="AH945">
+        <v>3</v>
+      </c>
+      <c r="AI945">
+        <v>1245.38319</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>Dago Espinoza</t>
+        </is>
+      </c>
+      <c r="B946" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E946">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F946">
+        <v>3833.79</v>
+      </c>
+      <c r="G946">
+        <v>41.92989427633977</v>
+      </c>
+      <c r="H946">
+        <v>58.81</v>
+      </c>
+      <c r="I946">
+        <v>0</v>
+      </c>
+      <c r="J946">
+        <v>0</v>
+      </c>
+      <c r="K946">
+        <v>0.6432008749544295</v>
+      </c>
+      <c r="L946">
+        <v>0</v>
+      </c>
+      <c r="M946">
+        <v>0</v>
+      </c>
+      <c r="N946">
+        <v>0</v>
+      </c>
+      <c r="O946">
+        <v>24.65587</v>
+      </c>
+      <c r="P946">
+        <v>69.32037224471436</v>
+      </c>
+      <c r="Q946">
+        <v>35.568</v>
+      </c>
+      <c r="R946">
+        <v>338.949</v>
+      </c>
+      <c r="S946">
+        <v>3.707061611374407</v>
+      </c>
+      <c r="T946">
+        <v>336.99001</v>
+      </c>
+      <c r="U946">
+        <v>11</v>
+      </c>
+      <c r="V946">
+        <v>6</v>
+      </c>
+      <c r="W946">
+        <v>17</v>
+      </c>
+      <c r="X946">
+        <v>39</v>
+      </c>
+      <c r="Y946">
+        <v>11</v>
+      </c>
+      <c r="Z946">
+        <v>18</v>
+      </c>
+      <c r="AA946">
+        <v>6</v>
+      </c>
+      <c r="AB946">
+        <v>22</v>
+      </c>
+      <c r="AC946">
+        <v>4.48599</v>
+      </c>
+      <c r="AD946">
+        <v>-2.26593</v>
+      </c>
+      <c r="AE946">
+        <v>0</v>
+      </c>
+      <c r="AF946">
+        <v>342.7736</v>
+      </c>
+      <c r="AG946">
+        <v>0</v>
+      </c>
+      <c r="AH946">
+        <v>3</v>
+      </c>
+      <c r="AI946">
+        <v>1016.847</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>Diego Arriaga</t>
+        </is>
+      </c>
+      <c r="B947" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E947">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F947">
+        <v>3660.42</v>
+      </c>
+      <c r="G947">
+        <v>40.03375865840321</v>
+      </c>
+      <c r="H947">
+        <v>24.76</v>
+      </c>
+      <c r="I947">
+        <v>0</v>
+      </c>
+      <c r="J947">
+        <v>0</v>
+      </c>
+      <c r="K947">
+        <v>0.2707983959168793</v>
+      </c>
+      <c r="L947">
+        <v>0</v>
+      </c>
+      <c r="M947">
+        <v>0</v>
+      </c>
+      <c r="N947">
+        <v>0</v>
+      </c>
+      <c r="O947">
+        <v>22.41989</v>
+      </c>
+      <c r="P947">
+        <v>62.27747222222222</v>
+      </c>
+      <c r="Q947">
+        <v>36</v>
+      </c>
+      <c r="R947">
+        <v>365.62818</v>
+      </c>
+      <c r="S947">
+        <v>3.998849945315348</v>
+      </c>
+      <c r="T947">
+        <v>278.26</v>
+      </c>
+      <c r="U947">
+        <v>5</v>
+      </c>
+      <c r="V947">
+        <v>4</v>
+      </c>
+      <c r="W947">
+        <v>9</v>
+      </c>
+      <c r="X947">
+        <v>35</v>
+      </c>
+      <c r="Y947">
+        <v>5</v>
+      </c>
+      <c r="Z947">
+        <v>27</v>
+      </c>
+      <c r="AA947">
+        <v>4</v>
+      </c>
+      <c r="AB947">
+        <v>47</v>
+      </c>
+      <c r="AC947">
+        <v>3.26333</v>
+      </c>
+      <c r="AD947">
+        <v>-3.46863</v>
+      </c>
+      <c r="AE947">
+        <v>0</v>
+      </c>
+      <c r="AF947">
+        <v>877.13</v>
+      </c>
+      <c r="AG947">
+        <v>0</v>
+      </c>
+      <c r="AH947">
+        <v>3</v>
+      </c>
+      <c r="AI947">
+        <v>1096.88454</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>Emilio Lara</t>
+        </is>
+      </c>
+      <c r="B948" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E948">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F948">
+        <v>3910.23</v>
+      </c>
+      <c r="G948">
+        <v>42.76591323368574</v>
+      </c>
+      <c r="H948">
+        <v>83.15000000000001</v>
+      </c>
+      <c r="I948">
+        <v>0</v>
+      </c>
+      <c r="J948">
+        <v>0</v>
+      </c>
+      <c r="K948">
+        <v>0.9094057601166606</v>
+      </c>
+      <c r="L948">
+        <v>0</v>
+      </c>
+      <c r="M948">
+        <v>1</v>
+      </c>
+      <c r="N948">
+        <v>0</v>
+      </c>
+      <c r="O948">
+        <v>26.25454</v>
+      </c>
+      <c r="P948">
+        <v>72.92927777777778</v>
+      </c>
+      <c r="Q948">
+        <v>36</v>
+      </c>
+      <c r="R948">
+        <v>382.18976</v>
+      </c>
+      <c r="S948">
+        <v>4.179982792562887</v>
+      </c>
+      <c r="T948">
+        <v>426.64001</v>
+      </c>
+      <c r="U948">
+        <v>13</v>
+      </c>
+      <c r="V948">
+        <v>17</v>
+      </c>
+      <c r="W948">
+        <v>30</v>
+      </c>
+      <c r="X948">
+        <v>45</v>
+      </c>
+      <c r="Y948">
+        <v>13</v>
+      </c>
+      <c r="Z948">
+        <v>35</v>
+      </c>
+      <c r="AA948">
+        <v>17</v>
+      </c>
+      <c r="AB948">
+        <v>18</v>
+      </c>
+      <c r="AC948">
+        <v>4.0769</v>
+      </c>
+      <c r="AD948">
+        <v>-2.69313</v>
+      </c>
+      <c r="AE948">
+        <v>0</v>
+      </c>
+      <c r="AF948">
+        <v>314.4855</v>
+      </c>
+      <c r="AG948">
+        <v>0</v>
+      </c>
+      <c r="AH948">
+        <v>3</v>
+      </c>
+      <c r="AI948">
+        <v>1146.56928</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>Erick Sánchez</t>
+        </is>
+      </c>
+      <c r="B949" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E949">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F949">
+        <v>2949.41</v>
+      </c>
+      <c r="G949">
+        <v>32.25749179730222</v>
+      </c>
+      <c r="H949">
+        <v>4.460000000000001</v>
+      </c>
+      <c r="I949">
+        <v>0</v>
+      </c>
+      <c r="J949">
+        <v>0</v>
+      </c>
+      <c r="K949">
+        <v>0.04877870944221656</v>
+      </c>
+      <c r="L949">
+        <v>0</v>
+      </c>
+      <c r="M949">
+        <v>0</v>
+      </c>
+      <c r="N949">
+        <v>0</v>
+      </c>
+      <c r="O949">
+        <v>22.11572</v>
+      </c>
+      <c r="P949">
+        <v>69.10298712660918</v>
+      </c>
+      <c r="Q949">
+        <v>32.004</v>
+      </c>
+      <c r="R949">
+        <v>293.60213</v>
+      </c>
+      <c r="S949">
+        <v>3.211106051768137</v>
+      </c>
+      <c r="T949">
+        <v>121.97</v>
+      </c>
+      <c r="U949">
+        <v>4</v>
+      </c>
+      <c r="V949">
+        <v>5</v>
+      </c>
+      <c r="W949">
+        <v>9</v>
+      </c>
+      <c r="X949">
+        <v>24</v>
+      </c>
+      <c r="Y949">
+        <v>4</v>
+      </c>
+      <c r="Z949">
+        <v>16</v>
+      </c>
+      <c r="AA949">
+        <v>5</v>
+      </c>
+      <c r="AB949">
+        <v>11</v>
+      </c>
+      <c r="AC949">
+        <v>3.68988</v>
+      </c>
+      <c r="AD949">
+        <v>-2.32256</v>
+      </c>
+      <c r="AE949">
+        <v>0</v>
+      </c>
+      <c r="AF949">
+        <v>194.718</v>
+      </c>
+      <c r="AG949">
+        <v>0</v>
+      </c>
+      <c r="AH949">
+        <v>3</v>
+      </c>
+      <c r="AI949">
+        <v>880.80639</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>Esteban Lozano</t>
+        </is>
+      </c>
+      <c r="B950" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E950">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F950">
+        <v>4201.44</v>
+      </c>
+      <c r="G950">
+        <v>45.95085672621217</v>
+      </c>
+      <c r="H950">
+        <v>62.66</v>
+      </c>
+      <c r="I950">
+        <v>0</v>
+      </c>
+      <c r="J950">
+        <v>0</v>
+      </c>
+      <c r="K950">
+        <v>0.6853080568720379</v>
+      </c>
+      <c r="L950">
+        <v>0</v>
+      </c>
+      <c r="M950">
+        <v>0</v>
+      </c>
+      <c r="N950">
+        <v>0</v>
+      </c>
+      <c r="O950">
+        <v>24.67845</v>
+      </c>
+      <c r="P950">
+        <v>79.7107558139535</v>
+      </c>
+      <c r="Q950">
+        <v>30.96</v>
+      </c>
+      <c r="R950">
+        <v>409.4466</v>
+      </c>
+      <c r="S950">
+        <v>4.478088953700328</v>
+      </c>
+      <c r="T950">
+        <v>409.6199999999999</v>
+      </c>
+      <c r="U950">
+        <v>13</v>
+      </c>
+      <c r="V950">
+        <v>17</v>
+      </c>
+      <c r="W950">
+        <v>30</v>
+      </c>
+      <c r="X950">
+        <v>44</v>
+      </c>
+      <c r="Y950">
+        <v>13</v>
+      </c>
+      <c r="Z950">
+        <v>37</v>
+      </c>
+      <c r="AA950">
+        <v>17</v>
+      </c>
+      <c r="AB950">
+        <v>12</v>
+      </c>
+      <c r="AC950">
+        <v>4.01199</v>
+      </c>
+      <c r="AD950">
+        <v>-3.00467</v>
+      </c>
+      <c r="AE950">
+        <v>0</v>
+      </c>
+      <c r="AF950">
+        <v>336.8225</v>
+      </c>
+      <c r="AG950">
+        <v>0</v>
+      </c>
+      <c r="AH950">
+        <v>3</v>
+      </c>
+      <c r="AI950">
+        <v>1228.3398</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>Henry Martín</t>
+        </is>
+      </c>
+      <c r="B951" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E951">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F951">
+        <v>1815.05</v>
+      </c>
+      <c r="G951">
+        <v>19.85107546481954</v>
+      </c>
+      <c r="H951">
+        <v>13.77</v>
+      </c>
+      <c r="I951">
+        <v>0</v>
+      </c>
+      <c r="J951">
+        <v>0</v>
+      </c>
+      <c r="K951">
+        <v>0.1506015311702515</v>
+      </c>
+      <c r="L951">
+        <v>0</v>
+      </c>
+      <c r="M951">
+        <v>0</v>
+      </c>
+      <c r="N951">
+        <v>0</v>
+      </c>
+      <c r="O951">
+        <v>22.51363</v>
+      </c>
+      <c r="P951">
+        <v>66.81395417853751</v>
+      </c>
+      <c r="Q951">
+        <v>33.696</v>
+      </c>
+      <c r="R951">
+        <v>185.15454</v>
+      </c>
+      <c r="S951">
+        <v>2.025022311337951</v>
+      </c>
+      <c r="T951">
+        <v>106.62</v>
+      </c>
+      <c r="U951">
+        <v>3</v>
+      </c>
+      <c r="V951">
+        <v>6</v>
+      </c>
+      <c r="W951">
+        <v>9</v>
+      </c>
+      <c r="X951">
+        <v>14</v>
+      </c>
+      <c r="Y951">
+        <v>3</v>
+      </c>
+      <c r="Z951">
+        <v>11</v>
+      </c>
+      <c r="AA951">
+        <v>6</v>
+      </c>
+      <c r="AB951">
+        <v>31</v>
+      </c>
+      <c r="AC951">
+        <v>3.59614</v>
+      </c>
+      <c r="AD951">
+        <v>-1.24607</v>
+      </c>
+      <c r="AE951">
+        <v>0</v>
+      </c>
+      <c r="AF951">
+        <v>160.6328</v>
+      </c>
+      <c r="AG951">
+        <v>0</v>
+      </c>
+      <c r="AH951">
+        <v>3</v>
+      </c>
+      <c r="AI951">
+        <v>555.46362</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>Icaro Conceicao</t>
+        </is>
+      </c>
+      <c r="B952" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E952">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F952">
+        <v>3517.48</v>
+      </c>
+      <c r="G952">
+        <v>38.47043383157127</v>
+      </c>
+      <c r="H952">
+        <v>65.58</v>
+      </c>
+      <c r="I952">
+        <v>0</v>
+      </c>
+      <c r="J952">
+        <v>0</v>
+      </c>
+      <c r="K952">
+        <v>0.7172438935472111</v>
+      </c>
+      <c r="L952">
+        <v>0</v>
+      </c>
+      <c r="M952">
+        <v>1</v>
+      </c>
+      <c r="N952">
+        <v>0</v>
+      </c>
+      <c r="O952">
+        <v>25.94194</v>
+      </c>
+      <c r="P952">
+        <v>72.06094444444444</v>
+      </c>
+      <c r="Q952">
+        <v>36</v>
+      </c>
+      <c r="R952">
+        <v>383.14673</v>
+      </c>
+      <c r="S952">
+        <v>4.190449106817353</v>
+      </c>
+      <c r="T952">
+        <v>360.85999</v>
+      </c>
+      <c r="U952">
+        <v>6</v>
+      </c>
+      <c r="V952">
+        <v>9</v>
+      </c>
+      <c r="W952">
+        <v>15</v>
+      </c>
+      <c r="X952">
+        <v>37</v>
+      </c>
+      <c r="Y952">
+        <v>6</v>
+      </c>
+      <c r="Z952">
+        <v>30</v>
+      </c>
+      <c r="AA952">
+        <v>9</v>
+      </c>
+      <c r="AB952">
+        <v>16</v>
+      </c>
+      <c r="AC952">
+        <v>4.34835</v>
+      </c>
+      <c r="AD952">
+        <v>-2.22324</v>
+      </c>
+      <c r="AE952">
+        <v>0</v>
+      </c>
+      <c r="AF952">
+        <v>801.5119999999999</v>
+      </c>
+      <c r="AG952">
+        <v>0</v>
+      </c>
+      <c r="AH952">
+        <v>3</v>
+      </c>
+      <c r="AI952">
+        <v>1149.44019</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>Isaías Violante</t>
+        </is>
+      </c>
+      <c r="B953" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E953">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F953">
+        <v>3917.66</v>
+      </c>
+      <c r="G953">
+        <v>42.84717462632154</v>
+      </c>
+      <c r="H953">
+        <v>12.99</v>
+      </c>
+      <c r="I953">
+        <v>0</v>
+      </c>
+      <c r="J953">
+        <v>0</v>
+      </c>
+      <c r="K953">
+        <v>0.1420707254830477</v>
+      </c>
+      <c r="L953">
+        <v>0</v>
+      </c>
+      <c r="M953">
+        <v>0</v>
+      </c>
+      <c r="N953">
+        <v>0</v>
+      </c>
+      <c r="O953">
+        <v>22.12801</v>
+      </c>
+      <c r="P953">
+        <v>63.23733996342021</v>
+      </c>
+      <c r="Q953">
+        <v>34.992</v>
+      </c>
+      <c r="R953">
+        <v>344.32051</v>
+      </c>
+      <c r="S953">
+        <v>3.765809442216551</v>
+      </c>
+      <c r="T953">
+        <v>276.48</v>
+      </c>
+      <c r="U953">
+        <v>7</v>
+      </c>
+      <c r="V953">
+        <v>8</v>
+      </c>
+      <c r="W953">
+        <v>15</v>
+      </c>
+      <c r="X953">
+        <v>39</v>
+      </c>
+      <c r="Y953">
+        <v>7</v>
+      </c>
+      <c r="Z953">
+        <v>31</v>
+      </c>
+      <c r="AA953">
+        <v>8</v>
+      </c>
+      <c r="AB953">
+        <v>11</v>
+      </c>
+      <c r="AC953">
+        <v>3.96522</v>
+      </c>
+      <c r="AD953">
+        <v>-3.11919</v>
+      </c>
+      <c r="AE953">
+        <v>0</v>
+      </c>
+      <c r="AF953">
+        <v>302.69403</v>
+      </c>
+      <c r="AG953">
+        <v>0</v>
+      </c>
+      <c r="AH953">
+        <v>3</v>
+      </c>
+      <c r="AI953">
+        <v>1032.96153</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>Israel Reyes</t>
+        </is>
+      </c>
+      <c r="B954" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E954">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F954">
+        <v>3999.08</v>
+      </c>
+      <c r="G954">
+        <v>43.7376594969012</v>
+      </c>
+      <c r="H954">
+        <v>14.52</v>
+      </c>
+      <c r="I954">
+        <v>0</v>
+      </c>
+      <c r="J954">
+        <v>0</v>
+      </c>
+      <c r="K954">
+        <v>0.158804228946409</v>
+      </c>
+      <c r="L954">
+        <v>0</v>
+      </c>
+      <c r="M954">
+        <v>0</v>
+      </c>
+      <c r="N954">
+        <v>0</v>
+      </c>
+      <c r="O954">
+        <v>22.08458</v>
+      </c>
+      <c r="P954">
+        <v>66.89864291772687</v>
+      </c>
+      <c r="Q954">
+        <v>33.012</v>
+      </c>
+      <c r="R954">
+        <v>424.68385</v>
+      </c>
+      <c r="S954">
+        <v>4.644737695953336</v>
+      </c>
+      <c r="T954">
+        <v>296.24999</v>
+      </c>
+      <c r="U954">
+        <v>2</v>
+      </c>
+      <c r="V954">
+        <v>9</v>
+      </c>
+      <c r="W954">
+        <v>11</v>
+      </c>
+      <c r="X954">
+        <v>32</v>
+      </c>
+      <c r="Y954">
+        <v>2</v>
+      </c>
+      <c r="Z954">
+        <v>31</v>
+      </c>
+      <c r="AA954">
+        <v>9</v>
+      </c>
+      <c r="AB954">
+        <v>19</v>
+      </c>
+      <c r="AC954">
+        <v>3.35445</v>
+      </c>
+      <c r="AD954">
+        <v>-2.42126</v>
+      </c>
+      <c r="AE954">
+        <v>0</v>
+      </c>
+      <c r="AF954">
+        <v>342.97146</v>
+      </c>
+      <c r="AG954">
+        <v>0</v>
+      </c>
+      <c r="AH954">
+        <v>3</v>
+      </c>
+      <c r="AI954">
+        <v>1274.05155</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>José Raúl Zúñiga</t>
+        </is>
+      </c>
+      <c r="B955" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E955">
+        <v>25.73333333333333</v>
+      </c>
+      <c r="F955">
+        <v>1103.04</v>
+      </c>
+      <c r="G955">
+        <v>42.86424870466321</v>
+      </c>
+      <c r="H955">
+        <v>0</v>
+      </c>
+      <c r="I955">
+        <v>0</v>
+      </c>
+      <c r="J955">
+        <v>0</v>
+      </c>
+      <c r="K955">
+        <v>0</v>
+      </c>
+      <c r="L955">
+        <v>0</v>
+      </c>
+      <c r="M955">
+        <v>0</v>
+      </c>
+      <c r="N955">
+        <v>0</v>
+      </c>
+      <c r="O955">
+        <v>13.48071</v>
+      </c>
+      <c r="P955">
+        <v>38.60455326460481</v>
+      </c>
+      <c r="Q955">
+        <v>34.92</v>
+      </c>
+      <c r="R955">
+        <v>127.19788</v>
+      </c>
+      <c r="S955">
+        <v>4.942922797927461</v>
+      </c>
+      <c r="T955">
+        <v>33.4</v>
+      </c>
+      <c r="U955">
+        <v>0</v>
+      </c>
+      <c r="V955">
+        <v>0</v>
+      </c>
+      <c r="W955">
+        <v>0</v>
+      </c>
+      <c r="X955">
+        <v>5</v>
+      </c>
+      <c r="Y955">
+        <v>0</v>
+      </c>
+      <c r="Z955">
+        <v>7</v>
+      </c>
+      <c r="AA955">
+        <v>0</v>
+      </c>
+      <c r="AB955">
+        <v>9</v>
+      </c>
+      <c r="AC955">
+        <v>2.46965</v>
+      </c>
+      <c r="AD955">
+        <v>-2.56272</v>
+      </c>
+      <c r="AE955">
+        <v>0</v>
+      </c>
+      <c r="AF955">
+        <v>97.39760000000001</v>
+      </c>
+      <c r="AG955">
+        <v>0</v>
+      </c>
+      <c r="AH955">
+        <v>3</v>
+      </c>
+      <c r="AI955">
+        <v>381.59364</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>Miguel Vázquez</t>
+        </is>
+      </c>
+      <c r="B956" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E956">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F956">
+        <v>3814.47</v>
+      </c>
+      <c r="G956">
+        <v>41.71859278162596</v>
+      </c>
+      <c r="H956">
+        <v>466.71</v>
+      </c>
+      <c r="I956">
+        <v>0</v>
+      </c>
+      <c r="J956">
+        <v>0</v>
+      </c>
+      <c r="K956">
+        <v>5.104374772147284</v>
+      </c>
+      <c r="L956">
+        <v>0</v>
+      </c>
+      <c r="M956">
+        <v>5</v>
+      </c>
+      <c r="N956">
+        <v>0</v>
+      </c>
+      <c r="O956">
+        <v>26.56352</v>
+      </c>
+      <c r="P956">
+        <v>78.16478342749529</v>
+      </c>
+      <c r="Q956">
+        <v>33.984</v>
+      </c>
+      <c r="R956">
+        <v>378.93447</v>
+      </c>
+      <c r="S956">
+        <v>4.144379912504557</v>
+      </c>
+      <c r="T956">
+        <v>731.7900100000001</v>
+      </c>
+      <c r="U956">
+        <v>12</v>
+      </c>
+      <c r="V956">
+        <v>7</v>
+      </c>
+      <c r="W956">
+        <v>19</v>
+      </c>
+      <c r="X956">
+        <v>47</v>
+      </c>
+      <c r="Y956">
+        <v>12</v>
+      </c>
+      <c r="Z956">
+        <v>24</v>
+      </c>
+      <c r="AA956">
+        <v>7</v>
+      </c>
+      <c r="AB956">
+        <v>12</v>
+      </c>
+      <c r="AC956">
+        <v>3.67793</v>
+      </c>
+      <c r="AD956">
+        <v>-2.03147</v>
+      </c>
+      <c r="AE956">
+        <v>0</v>
+      </c>
+      <c r="AF956">
+        <v>344.4352</v>
+      </c>
+      <c r="AG956">
+        <v>0</v>
+      </c>
+      <c r="AH956">
+        <v>3</v>
+      </c>
+      <c r="AI956">
+        <v>1136.80341</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>Oscar Perea</t>
+        </is>
+      </c>
+      <c r="B957" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E957">
+        <v>101.8</v>
+      </c>
+      <c r="F957">
+        <v>5473.04</v>
+      </c>
+      <c r="G957">
+        <v>53.76267190569745</v>
+      </c>
+      <c r="H957">
+        <v>266.39</v>
+      </c>
+      <c r="I957">
+        <v>0</v>
+      </c>
+      <c r="J957">
+        <v>0</v>
+      </c>
+      <c r="K957">
+        <v>2.61679764243615</v>
+      </c>
+      <c r="L957">
+        <v>0</v>
+      </c>
+      <c r="M957">
+        <v>0</v>
+      </c>
+      <c r="N957">
+        <v>0</v>
+      </c>
+      <c r="O957">
+        <v>24.21205</v>
+      </c>
+      <c r="P957">
+        <v>67.25569444444444</v>
+      </c>
+      <c r="Q957">
+        <v>36</v>
+      </c>
+      <c r="R957">
+        <v>526.4396400000001</v>
+      </c>
+      <c r="S957">
+        <v>5.171312770137526</v>
+      </c>
+      <c r="T957">
+        <v>822.3899799999999</v>
+      </c>
+      <c r="U957">
+        <v>28</v>
+      </c>
+      <c r="V957">
+        <v>25</v>
+      </c>
+      <c r="W957">
+        <v>53</v>
+      </c>
+      <c r="X957">
+        <v>72</v>
+      </c>
+      <c r="Y957">
+        <v>28</v>
+      </c>
+      <c r="Z957">
+        <v>69</v>
+      </c>
+      <c r="AA957">
+        <v>25</v>
+      </c>
+      <c r="AB957">
+        <v>15</v>
+      </c>
+      <c r="AC957">
+        <v>4.44372</v>
+      </c>
+      <c r="AD957">
+        <v>-3.7997</v>
+      </c>
+      <c r="AE957">
+        <v>0</v>
+      </c>
+      <c r="AF957">
+        <v>1289.376</v>
+      </c>
+      <c r="AG957">
+        <v>0</v>
+      </c>
+      <c r="AH957">
+        <v>3</v>
+      </c>
+      <c r="AI957">
+        <v>1579.31892</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>Pato Salas</t>
+        </is>
+      </c>
+      <c r="B958" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E958">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F958">
+        <v>3010.92</v>
+      </c>
+      <c r="G958">
+        <v>32.93022238425082</v>
+      </c>
+      <c r="H958">
+        <v>19.67</v>
+      </c>
+      <c r="I958">
+        <v>0</v>
+      </c>
+      <c r="J958">
+        <v>0</v>
+      </c>
+      <c r="K958">
+        <v>0.2151294203426905</v>
+      </c>
+      <c r="L958">
+        <v>0</v>
+      </c>
+      <c r="M958">
+        <v>0</v>
+      </c>
+      <c r="N958">
+        <v>0</v>
+      </c>
+      <c r="O958">
+        <v>24.66376</v>
+      </c>
+      <c r="P958">
+        <v>70.48399634202104</v>
+      </c>
+      <c r="Q958">
+        <v>34.992</v>
+      </c>
+      <c r="R958">
+        <v>263.7265</v>
+      </c>
+      <c r="S958">
+        <v>2.884358366751731</v>
+      </c>
+      <c r="T958">
+        <v>275.1</v>
+      </c>
+      <c r="U958">
+        <v>8</v>
+      </c>
+      <c r="V958">
+        <v>7</v>
+      </c>
+      <c r="W958">
+        <v>15</v>
+      </c>
+      <c r="X958">
+        <v>44</v>
+      </c>
+      <c r="Y958">
+        <v>8</v>
+      </c>
+      <c r="Z958">
+        <v>41</v>
+      </c>
+      <c r="AA958">
+        <v>7</v>
+      </c>
+      <c r="AB958">
+        <v>12</v>
+      </c>
+      <c r="AC958">
+        <v>4.26705</v>
+      </c>
+      <c r="AD958">
+        <v>-2.14311</v>
+      </c>
+      <c r="AE958">
+        <v>0</v>
+      </c>
+      <c r="AF958">
+        <v>277.3952</v>
+      </c>
+      <c r="AG958">
+        <v>0</v>
+      </c>
+      <c r="AH958">
+        <v>3</v>
+      </c>
+      <c r="AI958">
+        <v>791.1795</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>Ramón Juárez</t>
+        </is>
+      </c>
+      <c r="B959" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E959">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F959">
+        <v>2968.69</v>
+      </c>
+      <c r="G959">
+        <v>32.46835581480131</v>
+      </c>
+      <c r="H959">
+        <v>27.31</v>
+      </c>
+      <c r="I959">
+        <v>0</v>
+      </c>
+      <c r="J959">
+        <v>0</v>
+      </c>
+      <c r="K959">
+        <v>0.2986875683558148</v>
+      </c>
+      <c r="L959">
+        <v>0</v>
+      </c>
+      <c r="M959">
+        <v>0</v>
+      </c>
+      <c r="N959">
+        <v>0</v>
+      </c>
+      <c r="O959">
+        <v>22.77811</v>
+      </c>
+      <c r="P959">
+        <v>68.99948503574458</v>
+      </c>
+      <c r="Q959">
+        <v>33.012</v>
+      </c>
+      <c r="R959">
+        <v>296.23871</v>
+      </c>
+      <c r="S959">
+        <v>3.239942143638352</v>
+      </c>
+      <c r="T959">
+        <v>256.91</v>
+      </c>
+      <c r="U959">
+        <v>12</v>
+      </c>
+      <c r="V959">
+        <v>7</v>
+      </c>
+      <c r="W959">
+        <v>19</v>
+      </c>
+      <c r="X959">
+        <v>37</v>
+      </c>
+      <c r="Y959">
+        <v>12</v>
+      </c>
+      <c r="Z959">
+        <v>23</v>
+      </c>
+      <c r="AA959">
+        <v>7</v>
+      </c>
+      <c r="AB959">
+        <v>20</v>
+      </c>
+      <c r="AC959">
+        <v>4.20693</v>
+      </c>
+      <c r="AD959">
+        <v>-3.0202</v>
+      </c>
+      <c r="AE959">
+        <v>0</v>
+      </c>
+      <c r="AF959">
+        <v>247.64325</v>
+      </c>
+      <c r="AG959">
+        <v>0</v>
+      </c>
+      <c r="AH959">
+        <v>3</v>
+      </c>
+      <c r="AI959">
+        <v>888.7161299999999</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>Raphael Veiga</t>
+        </is>
+      </c>
+      <c r="B960" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E960">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F960">
+        <v>3162.42</v>
+      </c>
+      <c r="G960">
+        <v>34.58716733503464</v>
+      </c>
+      <c r="H960">
+        <v>20.17</v>
+      </c>
+      <c r="I960">
+        <v>0</v>
+      </c>
+      <c r="J960">
+        <v>0</v>
+      </c>
+      <c r="K960">
+        <v>0.2205978855267955</v>
+      </c>
+      <c r="L960">
+        <v>0</v>
+      </c>
+      <c r="M960">
+        <v>1</v>
+      </c>
+      <c r="N960">
+        <v>0</v>
+      </c>
+      <c r="O960">
+        <v>26.2801</v>
+      </c>
+      <c r="P960">
+        <v>82.11504811898513</v>
+      </c>
+      <c r="Q960">
+        <v>32.004</v>
+      </c>
+      <c r="R960">
+        <v>267.93289</v>
+      </c>
+      <c r="S960">
+        <v>2.930363361283267</v>
+      </c>
+      <c r="T960">
+        <v>198.36</v>
+      </c>
+      <c r="U960">
+        <v>4</v>
+      </c>
+      <c r="V960">
+        <v>7</v>
+      </c>
+      <c r="W960">
+        <v>11</v>
+      </c>
+      <c r="X960">
+        <v>20</v>
+      </c>
+      <c r="Y960">
+        <v>4</v>
+      </c>
+      <c r="Z960">
+        <v>24</v>
+      </c>
+      <c r="AA960">
+        <v>7</v>
+      </c>
+      <c r="AB960">
+        <v>19</v>
+      </c>
+      <c r="AC960">
+        <v>3.71826</v>
+      </c>
+      <c r="AD960">
+        <v>-2.17651</v>
+      </c>
+      <c r="AE960">
+        <v>0</v>
+      </c>
+      <c r="AF960">
+        <v>247.4017</v>
+      </c>
+      <c r="AG960">
+        <v>0</v>
+      </c>
+      <c r="AH960">
+        <v>3</v>
+      </c>
+      <c r="AI960">
+        <v>803.7986700000001</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>Ricardo Gonzalez</t>
+        </is>
+      </c>
+      <c r="B961" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E961">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F961">
+        <v>3869.26</v>
+      </c>
+      <c r="G961">
+        <v>42.31782719650018</v>
+      </c>
+      <c r="H961">
+        <v>35.16</v>
+      </c>
+      <c r="I961">
+        <v>0</v>
+      </c>
+      <c r="J961">
+        <v>0</v>
+      </c>
+      <c r="K961">
+        <v>0.3845424717462632</v>
+      </c>
+      <c r="L961">
+        <v>0</v>
+      </c>
+      <c r="M961">
+        <v>0</v>
+      </c>
+      <c r="N961">
+        <v>0</v>
+      </c>
+      <c r="O961">
+        <v>25.22691</v>
+      </c>
+      <c r="P961">
+        <v>70.07474999999999</v>
+      </c>
+      <c r="Q961">
+        <v>36</v>
+      </c>
+      <c r="R961">
+        <v>361.16542</v>
+      </c>
+      <c r="S961">
+        <v>3.950041049945315</v>
+      </c>
+      <c r="T961">
+        <v>231.47</v>
+      </c>
+      <c r="U961">
+        <v>8</v>
+      </c>
+      <c r="V961">
+        <v>8</v>
+      </c>
+      <c r="W961">
+        <v>16</v>
+      </c>
+      <c r="X961">
+        <v>22</v>
+      </c>
+      <c r="Y961">
+        <v>8</v>
+      </c>
+      <c r="Z961">
+        <v>22</v>
+      </c>
+      <c r="AA961">
+        <v>8</v>
+      </c>
+      <c r="AB961">
+        <v>8</v>
+      </c>
+      <c r="AC961">
+        <v>3.87326</v>
+      </c>
+      <c r="AD961">
+        <v>-2.10844</v>
+      </c>
+      <c r="AE961">
+        <v>0</v>
+      </c>
+      <c r="AF961">
+        <v>853.2619999999999</v>
+      </c>
+      <c r="AG961">
+        <v>0</v>
+      </c>
+      <c r="AH961">
+        <v>3</v>
+      </c>
+      <c r="AI961">
+        <v>1083.49626</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>Sebastián Cáceres</t>
+        </is>
+      </c>
+      <c r="B962" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E962">
+        <v>91.43333333333334</v>
+      </c>
+      <c r="F962">
+        <v>4291.419999999999</v>
+      </c>
+      <c r="G962">
+        <v>46.9349617207437</v>
+      </c>
+      <c r="H962">
+        <v>112.74</v>
+      </c>
+      <c r="I962">
+        <v>0</v>
+      </c>
+      <c r="J962">
+        <v>0</v>
+      </c>
+      <c r="K962">
+        <v>1.233029529711994</v>
+      </c>
+      <c r="L962">
+        <v>4.720000000000001</v>
+      </c>
+      <c r="M962">
+        <v>3</v>
+      </c>
+      <c r="N962">
+        <v>1</v>
+      </c>
+      <c r="O962">
+        <v>30.97756</v>
+      </c>
+      <c r="P962">
+        <v>88.52754915409237</v>
+      </c>
+      <c r="Q962">
+        <v>34.992</v>
+      </c>
+      <c r="R962">
+        <v>412.82985</v>
+      </c>
+      <c r="S962">
+        <v>4.515091323368575</v>
+      </c>
+      <c r="T962">
+        <v>555.5299799999999</v>
+      </c>
+      <c r="U962">
+        <v>16</v>
+      </c>
+      <c r="V962">
+        <v>14</v>
+      </c>
+      <c r="W962">
+        <v>30</v>
+      </c>
+      <c r="X962">
+        <v>55</v>
+      </c>
+      <c r="Y962">
+        <v>16</v>
+      </c>
+      <c r="Z962">
+        <v>42</v>
+      </c>
+      <c r="AA962">
+        <v>14</v>
+      </c>
+      <c r="AB962">
+        <v>27</v>
+      </c>
+      <c r="AC962">
+        <v>3.87668</v>
+      </c>
+      <c r="AD962">
+        <v>-1.9964</v>
+      </c>
+      <c r="AE962">
+        <v>0</v>
+      </c>
+      <c r="AF962">
+        <v>398.2952</v>
+      </c>
+      <c r="AG962">
+        <v>0</v>
+      </c>
+      <c r="AH962">
+        <v>3</v>
+      </c>
+      <c r="AI962">
+        <v>1238.48955</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>Víctor Dávila</t>
+        </is>
+      </c>
+      <c r="B963" s="2">
+        <v>46238</v>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>MD-2</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Sesión 49</t>
+        </is>
+      </c>
+      <c r="E963">
+        <v>60.56666666666667</v>
+      </c>
+      <c r="F963">
+        <v>2570.54</v>
+      </c>
+      <c r="G963">
+        <v>42.44149697303248</v>
+      </c>
+      <c r="H963">
+        <v>0</v>
+      </c>
+      <c r="I963">
+        <v>0</v>
+      </c>
+      <c r="J963">
+        <v>0</v>
+      </c>
+      <c r="K963">
+        <v>0</v>
+      </c>
+      <c r="L963">
+        <v>0</v>
+      </c>
+      <c r="M963">
+        <v>0</v>
+      </c>
+      <c r="N963">
+        <v>0</v>
+      </c>
+      <c r="O963">
+        <v>19.14265</v>
+      </c>
+      <c r="P963">
+        <v>56.32841925612052</v>
+      </c>
+      <c r="Q963">
+        <v>33.984</v>
+      </c>
+      <c r="R963">
+        <v>271.42182</v>
+      </c>
+      <c r="S963">
+        <v>4.48137292239956</v>
+      </c>
+      <c r="T963">
+        <v>494.99001</v>
+      </c>
+      <c r="U963">
+        <v>55</v>
+      </c>
+      <c r="V963">
+        <v>50</v>
+      </c>
+      <c r="W963">
+        <v>105</v>
+      </c>
+      <c r="X963">
+        <v>121</v>
+      </c>
+      <c r="Y963">
+        <v>55</v>
+      </c>
+      <c r="Z963">
+        <v>96</v>
+      </c>
+      <c r="AA963">
+        <v>50</v>
+      </c>
+      <c r="AB963">
+        <v>10</v>
+      </c>
+      <c r="AC963">
+        <v>3.75403</v>
+      </c>
+      <c r="AD963">
+        <v>-1.48004</v>
+      </c>
+      <c r="AE963">
+        <v>0</v>
+      </c>
+      <c r="AF963">
+        <v>233.1938</v>
+      </c>
+      <c r="AG963">
+        <v>0</v>
+      </c>
+      <c r="AH963">
+        <v>3</v>
+      </c>
+      <c r="AI963">
+        <v>814.2654600000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-07
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="181">
   <si>
     <t>player</t>
   </si>
@@ -555,6 +555,9 @@
   <si>
     <t>Edwin Cerrillo</t>
   </si>
+  <si>
+    <t>Partido vs San Diego</t>
+  </si>
 </sst>
 </file>
 
@@ -900,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI993"/>
+  <dimension ref="A1:AI1018"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -107079,6 +107082,2681 @@
         <v>593.9558099999999</v>
       </c>
     </row>
+    <row r="994" spans="1:35">
+      <c r="A994" t="s">
+        <v>41</v>
+      </c>
+      <c r="B994" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C994" t="s">
+        <v>68</v>
+      </c>
+      <c r="D994" t="s">
+        <v>180</v>
+      </c>
+      <c r="E994">
+        <v>100.0318333333333</v>
+      </c>
+      <c r="F994">
+        <v>12538.57</v>
+      </c>
+      <c r="G994">
+        <v>125.3457982542224</v>
+      </c>
+      <c r="H994">
+        <v>547.62</v>
+      </c>
+      <c r="I994">
+        <v>103.63</v>
+      </c>
+      <c r="J994">
+        <v>13</v>
+      </c>
+      <c r="K994">
+        <v>5.474457297760214</v>
+      </c>
+      <c r="L994">
+        <v>0</v>
+      </c>
+      <c r="M994">
+        <v>8</v>
+      </c>
+      <c r="N994">
+        <v>0</v>
+      </c>
+      <c r="O994">
+        <v>28.50634</v>
+      </c>
+      <c r="P994">
+        <v>105.3064882444991</v>
+      </c>
+      <c r="Q994">
+        <v>27.06988</v>
+      </c>
+      <c r="R994">
+        <v>1301.3302</v>
+      </c>
+      <c r="S994">
+        <v>13.00916075049443</v>
+      </c>
+      <c r="T994">
+        <v>2172.29993</v>
+      </c>
+      <c r="U994">
+        <v>14</v>
+      </c>
+      <c r="V994">
+        <v>39</v>
+      </c>
+      <c r="W994">
+        <v>53</v>
+      </c>
+      <c r="X994">
+        <v>132</v>
+      </c>
+      <c r="Y994">
+        <v>14</v>
+      </c>
+      <c r="Z994">
+        <v>110</v>
+      </c>
+      <c r="AA994">
+        <v>39</v>
+      </c>
+      <c r="AB994">
+        <v>40</v>
+      </c>
+      <c r="AC994">
+        <v>4.03213</v>
+      </c>
+      <c r="AD994">
+        <v>-4.46254</v>
+      </c>
+      <c r="AE994">
+        <v>0</v>
+      </c>
+      <c r="AF994">
+        <v>1012.0663</v>
+      </c>
+      <c r="AG994">
+        <v>0</v>
+      </c>
+      <c r="AH994">
+        <v>3</v>
+      </c>
+      <c r="AI994">
+        <v>3903.9906</v>
+      </c>
+    </row>
+    <row r="995" spans="1:35">
+      <c r="A995" t="s">
+        <v>109</v>
+      </c>
+      <c r="B995" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C995" t="s">
+        <v>68</v>
+      </c>
+      <c r="D995" t="s">
+        <v>180</v>
+      </c>
+      <c r="E995">
+        <v>72.59783333333334</v>
+      </c>
+      <c r="F995">
+        <v>5145.97</v>
+      </c>
+      <c r="G995">
+        <v>70.88324490859461</v>
+      </c>
+      <c r="H995">
+        <v>133.75</v>
+      </c>
+      <c r="I995">
+        <v>0</v>
+      </c>
+      <c r="J995">
+        <v>0</v>
+      </c>
+      <c r="K995">
+        <v>1.842341484020413</v>
+      </c>
+      <c r="L995">
+        <v>0</v>
+      </c>
+      <c r="M995">
+        <v>3</v>
+      </c>
+      <c r="N995">
+        <v>0</v>
+      </c>
+      <c r="O995">
+        <v>29.64211</v>
+      </c>
+      <c r="P995">
+        <v>82.33919444444444</v>
+      </c>
+      <c r="Q995">
+        <v>36</v>
+      </c>
+      <c r="R995">
+        <v>460.0919</v>
+      </c>
+      <c r="S995">
+        <v>6.337543131452499</v>
+      </c>
+      <c r="T995">
+        <v>793.97998</v>
+      </c>
+      <c r="U995">
+        <v>19</v>
+      </c>
+      <c r="V995">
+        <v>28</v>
+      </c>
+      <c r="W995">
+        <v>47</v>
+      </c>
+      <c r="X995">
+        <v>63</v>
+      </c>
+      <c r="Y995">
+        <v>19</v>
+      </c>
+      <c r="Z995">
+        <v>74</v>
+      </c>
+      <c r="AA995">
+        <v>28</v>
+      </c>
+      <c r="AB995">
+        <v>30</v>
+      </c>
+      <c r="AC995">
+        <v>4.34755</v>
+      </c>
+      <c r="AD995">
+        <v>0</v>
+      </c>
+      <c r="AE995">
+        <v>0</v>
+      </c>
+      <c r="AF995">
+        <v>1199.362</v>
+      </c>
+      <c r="AG995">
+        <v>0</v>
+      </c>
+      <c r="AH995">
+        <v>3</v>
+      </c>
+      <c r="AI995">
+        <v>1380.2757</v>
+      </c>
+    </row>
+    <row r="996" spans="1:35">
+      <c r="A996" t="s">
+        <v>35</v>
+      </c>
+      <c r="B996" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C996" t="s">
+        <v>42</v>
+      </c>
+      <c r="D996" t="s">
+        <v>171</v>
+      </c>
+      <c r="E996">
+        <v>32.33966666666667</v>
+      </c>
+      <c r="F996">
+        <v>3064.63</v>
+      </c>
+      <c r="G996">
+        <v>94.76380915078491</v>
+      </c>
+      <c r="H996">
+        <v>0</v>
+      </c>
+      <c r="I996">
+        <v>0</v>
+      </c>
+      <c r="J996">
+        <v>0</v>
+      </c>
+      <c r="K996">
+        <v>0</v>
+      </c>
+      <c r="L996">
+        <v>0</v>
+      </c>
+      <c r="M996">
+        <v>0</v>
+      </c>
+      <c r="N996">
+        <v>0</v>
+      </c>
+      <c r="O996">
+        <v>17.19792</v>
+      </c>
+      <c r="P996">
+        <v>50.60593220338983</v>
+      </c>
+      <c r="Q996">
+        <v>33.984</v>
+      </c>
+      <c r="R996">
+        <v>278.17654</v>
+      </c>
+      <c r="S996">
+        <v>8.601713272657932</v>
+      </c>
+      <c r="T996">
+        <v>41.25</v>
+      </c>
+      <c r="U996">
+        <v>0</v>
+      </c>
+      <c r="V996">
+        <v>0</v>
+      </c>
+      <c r="W996">
+        <v>0</v>
+      </c>
+      <c r="X996">
+        <v>2</v>
+      </c>
+      <c r="Y996">
+        <v>0</v>
+      </c>
+      <c r="Z996">
+        <v>0</v>
+      </c>
+      <c r="AA996">
+        <v>0</v>
+      </c>
+      <c r="AB996">
+        <v>1</v>
+      </c>
+      <c r="AC996">
+        <v>2.01933</v>
+      </c>
+      <c r="AD996">
+        <v>-1.70708</v>
+      </c>
+      <c r="AE996">
+        <v>0</v>
+      </c>
+      <c r="AF996">
+        <v>212.75735</v>
+      </c>
+      <c r="AG996">
+        <v>0</v>
+      </c>
+      <c r="AH996">
+        <v>3</v>
+      </c>
+      <c r="AI996">
+        <v>834.52962</v>
+      </c>
+    </row>
+    <row r="997" spans="1:35">
+      <c r="A997" t="s">
+        <v>44</v>
+      </c>
+      <c r="B997" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C997" t="s">
+        <v>68</v>
+      </c>
+      <c r="D997" t="s">
+        <v>180</v>
+      </c>
+      <c r="E997">
+        <v>62.895</v>
+      </c>
+      <c r="F997">
+        <v>5376.96</v>
+      </c>
+      <c r="G997">
+        <v>85.49105652277605</v>
+      </c>
+      <c r="H997">
+        <v>261.83</v>
+      </c>
+      <c r="I997">
+        <v>0</v>
+      </c>
+      <c r="J997">
+        <v>0</v>
+      </c>
+      <c r="K997">
+        <v>4.162970029414103</v>
+      </c>
+      <c r="L997">
+        <v>0</v>
+      </c>
+      <c r="M997">
+        <v>3</v>
+      </c>
+      <c r="N997">
+        <v>0</v>
+      </c>
+      <c r="O997">
+        <v>28.56815</v>
+      </c>
+      <c r="P997">
+        <v>88.17330246913581</v>
+      </c>
+      <c r="Q997">
+        <v>32.4</v>
+      </c>
+      <c r="R997">
+        <v>586.51103</v>
+      </c>
+      <c r="S997">
+        <v>9.325240957150806</v>
+      </c>
+      <c r="T997">
+        <v>1083.58997</v>
+      </c>
+      <c r="U997">
+        <v>9</v>
+      </c>
+      <c r="V997">
+        <v>13</v>
+      </c>
+      <c r="W997">
+        <v>22</v>
+      </c>
+      <c r="X997">
+        <v>67</v>
+      </c>
+      <c r="Y997">
+        <v>9</v>
+      </c>
+      <c r="Z997">
+        <v>49</v>
+      </c>
+      <c r="AA997">
+        <v>13</v>
+      </c>
+      <c r="AB997">
+        <v>8</v>
+      </c>
+      <c r="AC997">
+        <v>3.78188</v>
+      </c>
+      <c r="AD997">
+        <v>-0.55554</v>
+      </c>
+      <c r="AE997">
+        <v>0</v>
+      </c>
+      <c r="AF997">
+        <v>424.6613</v>
+      </c>
+      <c r="AG997">
+        <v>0</v>
+      </c>
+      <c r="AH997">
+        <v>3</v>
+      </c>
+      <c r="AI997">
+        <v>1759.53309</v>
+      </c>
+    </row>
+    <row r="998" spans="1:35">
+      <c r="A998" t="s">
+        <v>126</v>
+      </c>
+      <c r="B998" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C998" t="s">
+        <v>68</v>
+      </c>
+      <c r="D998" t="s">
+        <v>180</v>
+      </c>
+      <c r="E998">
+        <v>80.54666666666667</v>
+      </c>
+      <c r="F998">
+        <v>8494.66</v>
+      </c>
+      <c r="G998">
+        <v>105.4625889753352</v>
+      </c>
+      <c r="H998">
+        <v>604.96</v>
+      </c>
+      <c r="I998">
+        <v>33.12</v>
+      </c>
+      <c r="J998">
+        <v>2</v>
+      </c>
+      <c r="K998">
+        <v>7.510677040225128</v>
+      </c>
+      <c r="L998">
+        <v>66.33999999999999</v>
+      </c>
+      <c r="M998">
+        <v>16</v>
+      </c>
+      <c r="N998">
+        <v>3</v>
+      </c>
+      <c r="O998">
+        <v>33.73538</v>
+      </c>
+      <c r="P998">
+        <v>94.75165711717784</v>
+      </c>
+      <c r="Q998">
+        <v>35.604</v>
+      </c>
+      <c r="R998">
+        <v>672.40432</v>
+      </c>
+      <c r="S998">
+        <v>8.348009269988411</v>
+      </c>
+      <c r="T998">
+        <v>1353.22003</v>
+      </c>
+      <c r="U998">
+        <v>26</v>
+      </c>
+      <c r="V998">
+        <v>29</v>
+      </c>
+      <c r="W998">
+        <v>55</v>
+      </c>
+      <c r="X998">
+        <v>88</v>
+      </c>
+      <c r="Y998">
+        <v>26</v>
+      </c>
+      <c r="Z998">
+        <v>86</v>
+      </c>
+      <c r="AA998">
+        <v>29</v>
+      </c>
+      <c r="AB998">
+        <v>18</v>
+      </c>
+      <c r="AC998">
+        <v>5.17617</v>
+      </c>
+      <c r="AD998">
+        <v>-4.79593</v>
+      </c>
+      <c r="AE998">
+        <v>0</v>
+      </c>
+      <c r="AF998">
+        <v>708.8157199999999</v>
+      </c>
+      <c r="AG998">
+        <v>0</v>
+      </c>
+      <c r="AH998">
+        <v>3</v>
+      </c>
+      <c r="AI998">
+        <v>2017.21296</v>
+      </c>
+    </row>
+    <row r="999" spans="1:35">
+      <c r="A999" t="s">
+        <v>45</v>
+      </c>
+      <c r="B999" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C999" t="s">
+        <v>68</v>
+      </c>
+      <c r="D999" t="s">
+        <v>180</v>
+      </c>
+      <c r="E999">
+        <v>124.3465</v>
+      </c>
+      <c r="F999">
+        <v>11176.24</v>
+      </c>
+      <c r="G999">
+        <v>89.87981165533408</v>
+      </c>
+      <c r="H999">
+        <v>551.5799999999999</v>
+      </c>
+      <c r="I999">
+        <v>15.89</v>
+      </c>
+      <c r="J999">
+        <v>2</v>
+      </c>
+      <c r="K999">
+        <v>4.435830521968852</v>
+      </c>
+      <c r="L999">
+        <v>18.37</v>
+      </c>
+      <c r="M999">
+        <v>12</v>
+      </c>
+      <c r="N999">
+        <v>1</v>
+      </c>
+      <c r="O999">
+        <v>33.44482</v>
+      </c>
+      <c r="P999">
+        <v>98.41342984934086</v>
+      </c>
+      <c r="Q999">
+        <v>33.984</v>
+      </c>
+      <c r="R999">
+        <v>1267.28162</v>
+      </c>
+      <c r="S999">
+        <v>10.19153430132734</v>
+      </c>
+      <c r="T999">
+        <v>1629.96001</v>
+      </c>
+      <c r="U999">
+        <v>26</v>
+      </c>
+      <c r="V999">
+        <v>38</v>
+      </c>
+      <c r="W999">
+        <v>64</v>
+      </c>
+      <c r="X999">
+        <v>123</v>
+      </c>
+      <c r="Y999">
+        <v>26</v>
+      </c>
+      <c r="Z999">
+        <v>130</v>
+      </c>
+      <c r="AA999">
+        <v>38</v>
+      </c>
+      <c r="AB999">
+        <v>28</v>
+      </c>
+      <c r="AC999">
+        <v>4.22482</v>
+      </c>
+      <c r="AD999">
+        <v>-3.33821</v>
+      </c>
+      <c r="AE999">
+        <v>0</v>
+      </c>
+      <c r="AF999">
+        <v>1036.4032</v>
+      </c>
+      <c r="AG999">
+        <v>0</v>
+      </c>
+      <c r="AH999">
+        <v>3</v>
+      </c>
+      <c r="AI999">
+        <v>3801.84486</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:35">
+      <c r="A1000" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1000" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1000" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1000" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1000">
+        <v>45.72316666666667</v>
+      </c>
+      <c r="F1000">
+        <v>3764.96</v>
+      </c>
+      <c r="G1000">
+        <v>82.34250325327423</v>
+      </c>
+      <c r="H1000">
+        <v>115.25</v>
+      </c>
+      <c r="I1000">
+        <v>0</v>
+      </c>
+      <c r="J1000">
+        <v>0</v>
+      </c>
+      <c r="K1000">
+        <v>2.520604070146789</v>
+      </c>
+      <c r="L1000">
+        <v>0</v>
+      </c>
+      <c r="M1000">
+        <v>1</v>
+      </c>
+      <c r="N1000">
+        <v>0</v>
+      </c>
+      <c r="O1000">
+        <v>28.99977</v>
+      </c>
+      <c r="P1000">
+        <v>81.53331646423753</v>
+      </c>
+      <c r="Q1000">
+        <v>35.568</v>
+      </c>
+      <c r="R1000">
+        <v>319.62571</v>
+      </c>
+      <c r="S1000">
+        <v>6.990454364855161</v>
+      </c>
+      <c r="T1000">
+        <v>605.08998</v>
+      </c>
+      <c r="U1000">
+        <v>6</v>
+      </c>
+      <c r="V1000">
+        <v>5</v>
+      </c>
+      <c r="W1000">
+        <v>11</v>
+      </c>
+      <c r="X1000">
+        <v>47</v>
+      </c>
+      <c r="Y1000">
+        <v>6</v>
+      </c>
+      <c r="Z1000">
+        <v>38</v>
+      </c>
+      <c r="AA1000">
+        <v>5</v>
+      </c>
+      <c r="AB1000">
+        <v>2</v>
+      </c>
+      <c r="AC1000">
+        <v>3.66522</v>
+      </c>
+      <c r="AD1000">
+        <v>-2.49959</v>
+      </c>
+      <c r="AE1000">
+        <v>0</v>
+      </c>
+      <c r="AF1000">
+        <v>335.62</v>
+      </c>
+      <c r="AG1000">
+        <v>0</v>
+      </c>
+      <c r="AH1000">
+        <v>3</v>
+      </c>
+      <c r="AI1000">
+        <v>958.8771300000001</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:35">
+      <c r="A1001" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1001" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1001" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1001" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1001">
+        <v>40.97466666666666</v>
+      </c>
+      <c r="F1001">
+        <v>2693.1</v>
+      </c>
+      <c r="G1001">
+        <v>65.72597702645538</v>
+      </c>
+      <c r="H1001">
+        <v>0</v>
+      </c>
+      <c r="I1001">
+        <v>0</v>
+      </c>
+      <c r="J1001">
+        <v>0</v>
+      </c>
+      <c r="K1001">
+        <v>0</v>
+      </c>
+      <c r="L1001">
+        <v>0</v>
+      </c>
+      <c r="M1001">
+        <v>0</v>
+      </c>
+      <c r="N1001">
+        <v>0</v>
+      </c>
+      <c r="O1001">
+        <v>27.66747</v>
+      </c>
+      <c r="P1001">
+        <v>76.85408333333334</v>
+      </c>
+      <c r="Q1001">
+        <v>36</v>
+      </c>
+      <c r="R1001">
+        <v>311.95239</v>
+      </c>
+      <c r="S1001">
+        <v>7.613299030295142</v>
+      </c>
+      <c r="T1001">
+        <v>12.88</v>
+      </c>
+      <c r="U1001">
+        <v>0</v>
+      </c>
+      <c r="V1001">
+        <v>0</v>
+      </c>
+      <c r="W1001">
+        <v>0</v>
+      </c>
+      <c r="X1001">
+        <v>3</v>
+      </c>
+      <c r="Y1001">
+        <v>0</v>
+      </c>
+      <c r="Z1001">
+        <v>2</v>
+      </c>
+      <c r="AA1001">
+        <v>0</v>
+      </c>
+      <c r="AB1001">
+        <v>3</v>
+      </c>
+      <c r="AC1001">
+        <v>4.3581</v>
+      </c>
+      <c r="AD1001">
+        <v>-2.73966</v>
+      </c>
+      <c r="AE1001">
+        <v>0</v>
+      </c>
+      <c r="AF1001">
+        <v>145.698</v>
+      </c>
+      <c r="AG1001">
+        <v>0</v>
+      </c>
+      <c r="AH1001">
+        <v>3</v>
+      </c>
+      <c r="AI1001">
+        <v>935.85717</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:35">
+      <c r="A1002" t="s">
+        <v>179</v>
+      </c>
+      <c r="B1002" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1002" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1002" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1002">
+        <v>92.98616666666666</v>
+      </c>
+      <c r="F1002">
+        <v>5057.97</v>
+      </c>
+      <c r="G1002">
+        <v>54.39486518604022</v>
+      </c>
+      <c r="H1002">
+        <v>42.98</v>
+      </c>
+      <c r="I1002">
+        <v>0</v>
+      </c>
+      <c r="J1002">
+        <v>0</v>
+      </c>
+      <c r="K1002">
+        <v>0.4622192906830228</v>
+      </c>
+      <c r="L1002">
+        <v>0</v>
+      </c>
+      <c r="M1002">
+        <v>0</v>
+      </c>
+      <c r="N1002">
+        <v>0</v>
+      </c>
+      <c r="O1002">
+        <v>23.81081</v>
+      </c>
+      <c r="P1002">
+        <v>66.14113888888889</v>
+      </c>
+      <c r="Q1002">
+        <v>36</v>
+      </c>
+      <c r="R1002">
+        <v>485.33963</v>
+      </c>
+      <c r="S1002">
+        <v>5.219482073498388</v>
+      </c>
+      <c r="T1002">
+        <v>737.9499900000001</v>
+      </c>
+      <c r="U1002">
+        <v>23</v>
+      </c>
+      <c r="V1002">
+        <v>15</v>
+      </c>
+      <c r="W1002">
+        <v>38</v>
+      </c>
+      <c r="X1002">
+        <v>100</v>
+      </c>
+      <c r="Y1002">
+        <v>23</v>
+      </c>
+      <c r="Z1002">
+        <v>77</v>
+      </c>
+      <c r="AA1002">
+        <v>15</v>
+      </c>
+      <c r="AB1002">
+        <v>16</v>
+      </c>
+      <c r="AC1002">
+        <v>4.34</v>
+      </c>
+      <c r="AD1002">
+        <v>0</v>
+      </c>
+      <c r="AE1002">
+        <v>0</v>
+      </c>
+      <c r="AF1002">
+        <v>1220.192</v>
+      </c>
+      <c r="AG1002">
+        <v>0</v>
+      </c>
+      <c r="AH1002">
+        <v>3</v>
+      </c>
+      <c r="AI1002">
+        <v>1456.01889</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:35">
+      <c r="A1003" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1003" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1003" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1003" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1003">
+        <v>34.18066666666667</v>
+      </c>
+      <c r="F1003">
+        <v>2560.15</v>
+      </c>
+      <c r="G1003">
+        <v>74.90052856390552</v>
+      </c>
+      <c r="H1003">
+        <v>384.24</v>
+      </c>
+      <c r="I1003">
+        <v>0</v>
+      </c>
+      <c r="J1003">
+        <v>0</v>
+      </c>
+      <c r="K1003">
+        <v>11.2414425308654</v>
+      </c>
+      <c r="L1003">
+        <v>0</v>
+      </c>
+      <c r="M1003">
+        <v>2</v>
+      </c>
+      <c r="N1003">
+        <v>0</v>
+      </c>
+      <c r="O1003">
+        <v>25.84076</v>
+      </c>
+      <c r="P1003">
+        <v>71.77988888888889</v>
+      </c>
+      <c r="Q1003">
+        <v>36</v>
+      </c>
+      <c r="R1003">
+        <v>247.41533</v>
+      </c>
+      <c r="S1003">
+        <v>7.23845829026155</v>
+      </c>
+      <c r="T1003">
+        <v>616.52001</v>
+      </c>
+      <c r="U1003">
+        <v>12</v>
+      </c>
+      <c r="V1003">
+        <v>12</v>
+      </c>
+      <c r="W1003">
+        <v>24</v>
+      </c>
+      <c r="X1003">
+        <v>24</v>
+      </c>
+      <c r="Y1003">
+        <v>12</v>
+      </c>
+      <c r="Z1003">
+        <v>24</v>
+      </c>
+      <c r="AA1003">
+        <v>12</v>
+      </c>
+      <c r="AB1003">
+        <v>14</v>
+      </c>
+      <c r="AC1003">
+        <v>3.66692</v>
+      </c>
+      <c r="AD1003">
+        <v>-2.85234</v>
+      </c>
+      <c r="AE1003">
+        <v>0</v>
+      </c>
+      <c r="AF1003">
+        <v>197.0255</v>
+      </c>
+      <c r="AG1003">
+        <v>0</v>
+      </c>
+      <c r="AH1003">
+        <v>3</v>
+      </c>
+      <c r="AI1003">
+        <v>742.2459899999999</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:35">
+      <c r="A1004" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1004" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1004" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1004" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1004">
+        <v>114.1096666666667</v>
+      </c>
+      <c r="F1004">
+        <v>11540.32</v>
+      </c>
+      <c r="G1004">
+        <v>101.133587864306</v>
+      </c>
+      <c r="H1004">
+        <v>459.2</v>
+      </c>
+      <c r="I1004">
+        <v>19.26</v>
+      </c>
+      <c r="J1004">
+        <v>2</v>
+      </c>
+      <c r="K1004">
+        <v>4.024198943121967</v>
+      </c>
+      <c r="L1004">
+        <v>14.54</v>
+      </c>
+      <c r="M1004">
+        <v>12</v>
+      </c>
+      <c r="N1004">
+        <v>1</v>
+      </c>
+      <c r="O1004">
+        <v>31.88937</v>
+      </c>
+      <c r="P1004">
+        <v>99.64182602174728</v>
+      </c>
+      <c r="Q1004">
+        <v>32.004</v>
+      </c>
+      <c r="R1004">
+        <v>1237.01928</v>
+      </c>
+      <c r="S1004">
+        <v>10.84061776828723</v>
+      </c>
+      <c r="T1004">
+        <v>1789.56996</v>
+      </c>
+      <c r="U1004">
+        <v>33</v>
+      </c>
+      <c r="V1004">
+        <v>43</v>
+      </c>
+      <c r="W1004">
+        <v>76</v>
+      </c>
+      <c r="X1004">
+        <v>133</v>
+      </c>
+      <c r="Y1004">
+        <v>33</v>
+      </c>
+      <c r="Z1004">
+        <v>141</v>
+      </c>
+      <c r="AA1004">
+        <v>43</v>
+      </c>
+      <c r="AB1004">
+        <v>36</v>
+      </c>
+      <c r="AC1004">
+        <v>4.52895</v>
+      </c>
+      <c r="AD1004">
+        <v>-3.6459</v>
+      </c>
+      <c r="AE1004">
+        <v>0</v>
+      </c>
+      <c r="AF1004">
+        <v>806.4299999999999</v>
+      </c>
+      <c r="AG1004">
+        <v>0</v>
+      </c>
+      <c r="AH1004">
+        <v>3</v>
+      </c>
+      <c r="AI1004">
+        <v>3711.05784</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:35">
+      <c r="A1005" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1005" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1005" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1005" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1005">
+        <v>87.91499999999999</v>
+      </c>
+      <c r="F1005">
+        <v>8277.6</v>
+      </c>
+      <c r="G1005">
+        <v>94.1545811295001</v>
+      </c>
+      <c r="H1005">
+        <v>298.64</v>
+      </c>
+      <c r="I1005">
+        <v>0</v>
+      </c>
+      <c r="J1005">
+        <v>0</v>
+      </c>
+      <c r="K1005">
+        <v>3.396917477108571</v>
+      </c>
+      <c r="L1005">
+        <v>0</v>
+      </c>
+      <c r="M1005">
+        <v>2</v>
+      </c>
+      <c r="N1005">
+        <v>0</v>
+      </c>
+      <c r="O1005">
+        <v>27.50443</v>
+      </c>
+      <c r="P1005">
+        <v>81.62520773979108</v>
+      </c>
+      <c r="Q1005">
+        <v>33.696</v>
+      </c>
+      <c r="R1005">
+        <v>937.9292</v>
+      </c>
+      <c r="S1005">
+        <v>10.66859125291475</v>
+      </c>
+      <c r="T1005">
+        <v>1259.97002</v>
+      </c>
+      <c r="U1005">
+        <v>33</v>
+      </c>
+      <c r="V1005">
+        <v>31</v>
+      </c>
+      <c r="W1005">
+        <v>64</v>
+      </c>
+      <c r="X1005">
+        <v>128</v>
+      </c>
+      <c r="Y1005">
+        <v>33</v>
+      </c>
+      <c r="Z1005">
+        <v>109</v>
+      </c>
+      <c r="AA1005">
+        <v>31</v>
+      </c>
+      <c r="AB1005">
+        <v>34</v>
+      </c>
+      <c r="AC1005">
+        <v>4.76975</v>
+      </c>
+      <c r="AD1005">
+        <v>-3.45546</v>
+      </c>
+      <c r="AE1005">
+        <v>0</v>
+      </c>
+      <c r="AF1005">
+        <v>763.7128</v>
+      </c>
+      <c r="AG1005">
+        <v>0</v>
+      </c>
+      <c r="AH1005">
+        <v>3</v>
+      </c>
+      <c r="AI1005">
+        <v>2813.7876</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:35">
+      <c r="A1006" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1006" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1006" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1006" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1006">
+        <v>87.235</v>
+      </c>
+      <c r="F1006">
+        <v>9076.58</v>
+      </c>
+      <c r="G1006">
+        <v>104.0474580157047</v>
+      </c>
+      <c r="H1006">
+        <v>181.55</v>
+      </c>
+      <c r="I1006">
+        <v>0</v>
+      </c>
+      <c r="J1006">
+        <v>0</v>
+      </c>
+      <c r="K1006">
+        <v>2.081160084828337</v>
+      </c>
+      <c r="L1006">
+        <v>0</v>
+      </c>
+      <c r="M1006">
+        <v>1</v>
+      </c>
+      <c r="N1006">
+        <v>0</v>
+      </c>
+      <c r="O1006">
+        <v>26.12113</v>
+      </c>
+      <c r="P1006">
+        <v>72.55869444444446</v>
+      </c>
+      <c r="Q1006">
+        <v>36</v>
+      </c>
+      <c r="R1006">
+        <v>978.02585</v>
+      </c>
+      <c r="S1006">
+        <v>11.21139278959133</v>
+      </c>
+      <c r="T1006">
+        <v>1269.35999</v>
+      </c>
+      <c r="U1006">
+        <v>26</v>
+      </c>
+      <c r="V1006">
+        <v>27</v>
+      </c>
+      <c r="W1006">
+        <v>53</v>
+      </c>
+      <c r="X1006">
+        <v>97</v>
+      </c>
+      <c r="Y1006">
+        <v>26</v>
+      </c>
+      <c r="Z1006">
+        <v>98</v>
+      </c>
+      <c r="AA1006">
+        <v>27</v>
+      </c>
+      <c r="AB1006">
+        <v>0</v>
+      </c>
+      <c r="AC1006">
+        <v>3.75782</v>
+      </c>
+      <c r="AD1006">
+        <v>-3.68744</v>
+      </c>
+      <c r="AE1006">
+        <v>0</v>
+      </c>
+      <c r="AF1006">
+        <v>2078.59</v>
+      </c>
+      <c r="AG1006">
+        <v>0</v>
+      </c>
+      <c r="AH1006">
+        <v>3</v>
+      </c>
+      <c r="AI1006">
+        <v>2934.07755</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:35">
+      <c r="A1007" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1007" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1007" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1007" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1007">
+        <v>114.1913333333333</v>
+      </c>
+      <c r="F1007">
+        <v>11636.2</v>
+      </c>
+      <c r="G1007">
+        <v>101.9009031625284</v>
+      </c>
+      <c r="H1007">
+        <v>610.0400000000001</v>
+      </c>
+      <c r="I1007">
+        <v>12.1</v>
+      </c>
+      <c r="J1007">
+        <v>1</v>
+      </c>
+      <c r="K1007">
+        <v>5.342261817884603</v>
+      </c>
+      <c r="L1007">
+        <v>31.13</v>
+      </c>
+      <c r="M1007">
+        <v>13</v>
+      </c>
+      <c r="N1007">
+        <v>2</v>
+      </c>
+      <c r="O1007">
+        <v>32.45752</v>
+      </c>
+      <c r="P1007">
+        <v>92.75697302240513</v>
+      </c>
+      <c r="Q1007">
+        <v>34.992</v>
+      </c>
+      <c r="R1007">
+        <v>964.71222</v>
+      </c>
+      <c r="S1007">
+        <v>8.448208737382288</v>
+      </c>
+      <c r="T1007">
+        <v>1757.88997</v>
+      </c>
+      <c r="U1007">
+        <v>39</v>
+      </c>
+      <c r="V1007">
+        <v>39</v>
+      </c>
+      <c r="W1007">
+        <v>78</v>
+      </c>
+      <c r="X1007">
+        <v>120</v>
+      </c>
+      <c r="Y1007">
+        <v>39</v>
+      </c>
+      <c r="Z1007">
+        <v>112</v>
+      </c>
+      <c r="AA1007">
+        <v>39</v>
+      </c>
+      <c r="AB1007">
+        <v>18</v>
+      </c>
+      <c r="AC1007">
+        <v>5.03595</v>
+      </c>
+      <c r="AD1007">
+        <v>-3.12812</v>
+      </c>
+      <c r="AE1007">
+        <v>0</v>
+      </c>
+      <c r="AF1007">
+        <v>927.1398899999999</v>
+      </c>
+      <c r="AG1007">
+        <v>0</v>
+      </c>
+      <c r="AH1007">
+        <v>3</v>
+      </c>
+      <c r="AI1007">
+        <v>2894.13666</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:35">
+      <c r="A1008" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1008" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1008" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1008" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1008">
+        <v>100.0318333333333</v>
+      </c>
+      <c r="F1008">
+        <v>11207.54</v>
+      </c>
+      <c r="G1008">
+        <v>112.0397340180043</v>
+      </c>
+      <c r="H1008">
+        <v>493.36</v>
+      </c>
+      <c r="I1008">
+        <v>0</v>
+      </c>
+      <c r="J1008">
+        <v>0</v>
+      </c>
+      <c r="K1008">
+        <v>4.932029970459404</v>
+      </c>
+      <c r="L1008">
+        <v>0</v>
+      </c>
+      <c r="M1008">
+        <v>9</v>
+      </c>
+      <c r="N1008">
+        <v>0</v>
+      </c>
+      <c r="O1008">
+        <v>29.57795</v>
+      </c>
+      <c r="P1008">
+        <v>89.59757058039501</v>
+      </c>
+      <c r="Q1008">
+        <v>33.012</v>
+      </c>
+      <c r="R1008">
+        <v>1108.77777</v>
+      </c>
+      <c r="S1008">
+        <v>11.08424921400021</v>
+      </c>
+      <c r="T1008">
+        <v>1651.88</v>
+      </c>
+      <c r="U1008">
+        <v>23</v>
+      </c>
+      <c r="V1008">
+        <v>33</v>
+      </c>
+      <c r="W1008">
+        <v>56</v>
+      </c>
+      <c r="X1008">
+        <v>101</v>
+      </c>
+      <c r="Y1008">
+        <v>23</v>
+      </c>
+      <c r="Z1008">
+        <v>101</v>
+      </c>
+      <c r="AA1008">
+        <v>33</v>
+      </c>
+      <c r="AB1008">
+        <v>32</v>
+      </c>
+      <c r="AC1008">
+        <v>4.18282</v>
+      </c>
+      <c r="AD1008">
+        <v>-4.82473</v>
+      </c>
+      <c r="AE1008">
+        <v>0</v>
+      </c>
+      <c r="AF1008">
+        <v>1009.73574</v>
+      </c>
+      <c r="AG1008">
+        <v>0</v>
+      </c>
+      <c r="AH1008">
+        <v>3</v>
+      </c>
+      <c r="AI1008">
+        <v>3326.33331</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:35">
+      <c r="A1009" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1009" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1009" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1009" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1009">
+        <v>32.33966666666667</v>
+      </c>
+      <c r="F1009">
+        <v>2380.52</v>
+      </c>
+      <c r="G1009">
+        <v>73.60991146064173</v>
+      </c>
+      <c r="H1009">
+        <v>0</v>
+      </c>
+      <c r="I1009">
+        <v>0</v>
+      </c>
+      <c r="J1009">
+        <v>0</v>
+      </c>
+      <c r="K1009">
+        <v>0</v>
+      </c>
+      <c r="L1009">
+        <v>0</v>
+      </c>
+      <c r="M1009">
+        <v>0</v>
+      </c>
+      <c r="N1009">
+        <v>0</v>
+      </c>
+      <c r="O1009">
+        <v>17.46807</v>
+      </c>
+      <c r="P1009">
+        <v>50.02310996563574</v>
+      </c>
+      <c r="Q1009">
+        <v>34.92</v>
+      </c>
+      <c r="R1009">
+        <v>193.19838</v>
+      </c>
+      <c r="S1009">
+        <v>5.974037456580669</v>
+      </c>
+      <c r="T1009">
+        <v>33.51</v>
+      </c>
+      <c r="U1009">
+        <v>0</v>
+      </c>
+      <c r="V1009">
+        <v>0</v>
+      </c>
+      <c r="W1009">
+        <v>0</v>
+      </c>
+      <c r="X1009">
+        <v>1</v>
+      </c>
+      <c r="Y1009">
+        <v>0</v>
+      </c>
+      <c r="Z1009">
+        <v>0</v>
+      </c>
+      <c r="AA1009">
+        <v>0</v>
+      </c>
+      <c r="AB1009">
+        <v>1</v>
+      </c>
+      <c r="AC1009">
+        <v>2.25376</v>
+      </c>
+      <c r="AD1009">
+        <v>-1.73932</v>
+      </c>
+      <c r="AE1009">
+        <v>0</v>
+      </c>
+      <c r="AF1009">
+        <v>204.084</v>
+      </c>
+      <c r="AG1009">
+        <v>0</v>
+      </c>
+      <c r="AH1009">
+        <v>3</v>
+      </c>
+      <c r="AI1009">
+        <v>579.5951399999999</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:35">
+      <c r="A1010" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1010" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1010" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1010" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1010">
+        <v>124.3465</v>
+      </c>
+      <c r="F1010">
+        <v>12656.18</v>
+      </c>
+      <c r="G1010">
+        <v>101.7815539641244</v>
+      </c>
+      <c r="H1010">
+        <v>988.76</v>
+      </c>
+      <c r="I1010">
+        <v>12.17</v>
+      </c>
+      <c r="J1010">
+        <v>1</v>
+      </c>
+      <c r="K1010">
+        <v>7.951651232644264</v>
+      </c>
+      <c r="L1010">
+        <v>23.93</v>
+      </c>
+      <c r="M1010">
+        <v>25</v>
+      </c>
+      <c r="N1010">
+        <v>1</v>
+      </c>
+      <c r="O1010">
+        <v>32.91493</v>
+      </c>
+      <c r="P1010">
+        <v>94.06415752171925</v>
+      </c>
+      <c r="Q1010">
+        <v>34.992</v>
+      </c>
+      <c r="R1010">
+        <v>1094.53332</v>
+      </c>
+      <c r="S1010">
+        <v>8.80228490548588</v>
+      </c>
+      <c r="T1010">
+        <v>2518.12007</v>
+      </c>
+      <c r="U1010">
+        <v>52</v>
+      </c>
+      <c r="V1010">
+        <v>83</v>
+      </c>
+      <c r="W1010">
+        <v>135</v>
+      </c>
+      <c r="X1010">
+        <v>178</v>
+      </c>
+      <c r="Y1010">
+        <v>52</v>
+      </c>
+      <c r="Z1010">
+        <v>175</v>
+      </c>
+      <c r="AA1010">
+        <v>83</v>
+      </c>
+      <c r="AB1010">
+        <v>39</v>
+      </c>
+      <c r="AC1010">
+        <v>4.81525</v>
+      </c>
+      <c r="AD1010">
+        <v>-4.57127</v>
+      </c>
+      <c r="AE1010">
+        <v>0</v>
+      </c>
+      <c r="AF1010">
+        <v>1084.81326</v>
+      </c>
+      <c r="AG1010">
+        <v>0</v>
+      </c>
+      <c r="AH1010">
+        <v>3</v>
+      </c>
+      <c r="AI1010">
+        <v>3283.59996</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:35">
+      <c r="A1011" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1011" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1011" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1011" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1011">
+        <v>34.18066666666667</v>
+      </c>
+      <c r="F1011">
+        <v>2511.38</v>
+      </c>
+      <c r="G1011">
+        <v>73.47369858204443</v>
+      </c>
+      <c r="H1011">
+        <v>122.98</v>
+      </c>
+      <c r="I1011">
+        <v>0</v>
+      </c>
+      <c r="J1011">
+        <v>0</v>
+      </c>
+      <c r="K1011">
+        <v>3.59794035614675</v>
+      </c>
+      <c r="L1011">
+        <v>0</v>
+      </c>
+      <c r="M1011">
+        <v>0</v>
+      </c>
+      <c r="N1011">
+        <v>0</v>
+      </c>
+      <c r="O1011">
+        <v>22.70767</v>
+      </c>
+      <c r="P1011">
+        <v>66.81870880414313</v>
+      </c>
+      <c r="Q1011">
+        <v>33.984</v>
+      </c>
+      <c r="R1011">
+        <v>234.1604</v>
+      </c>
+      <c r="S1011">
+        <v>6.850668018958085</v>
+      </c>
+      <c r="T1011">
+        <v>514.15999</v>
+      </c>
+      <c r="U1011">
+        <v>9</v>
+      </c>
+      <c r="V1011">
+        <v>8</v>
+      </c>
+      <c r="W1011">
+        <v>17</v>
+      </c>
+      <c r="X1011">
+        <v>24</v>
+      </c>
+      <c r="Y1011">
+        <v>9</v>
+      </c>
+      <c r="Z1011">
+        <v>25</v>
+      </c>
+      <c r="AA1011">
+        <v>8</v>
+      </c>
+      <c r="AB1011">
+        <v>2</v>
+      </c>
+      <c r="AC1011">
+        <v>3.4254</v>
+      </c>
+      <c r="AD1011">
+        <v>-2.98543</v>
+      </c>
+      <c r="AE1011">
+        <v>0</v>
+      </c>
+      <c r="AF1011">
+        <v>220.5696</v>
+      </c>
+      <c r="AG1011">
+        <v>0</v>
+      </c>
+      <c r="AH1011">
+        <v>3</v>
+      </c>
+      <c r="AI1011">
+        <v>702.4811999999999</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:35">
+      <c r="A1012" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1012" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1012" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1012" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1012">
+        <v>92.98616666666666</v>
+      </c>
+      <c r="F1012">
+        <v>5784.709999999999</v>
+      </c>
+      <c r="G1012">
+        <v>62.21043631938083</v>
+      </c>
+      <c r="H1012">
+        <v>62.99</v>
+      </c>
+      <c r="I1012">
+        <v>0</v>
+      </c>
+      <c r="J1012">
+        <v>0</v>
+      </c>
+      <c r="K1012">
+        <v>0.6774125900447558</v>
+      </c>
+      <c r="L1012">
+        <v>0</v>
+      </c>
+      <c r="M1012">
+        <v>2</v>
+      </c>
+      <c r="N1012">
+        <v>0</v>
+      </c>
+      <c r="O1012">
+        <v>25.65787</v>
+      </c>
+      <c r="P1012">
+        <v>71.27186111111111</v>
+      </c>
+      <c r="Q1012">
+        <v>36</v>
+      </c>
+      <c r="R1012">
+        <v>614.36805</v>
+      </c>
+      <c r="S1012">
+        <v>6.607090839676871</v>
+      </c>
+      <c r="T1012">
+        <v>949.75</v>
+      </c>
+      <c r="U1012">
+        <v>58</v>
+      </c>
+      <c r="V1012">
+        <v>39</v>
+      </c>
+      <c r="W1012">
+        <v>97</v>
+      </c>
+      <c r="X1012">
+        <v>156</v>
+      </c>
+      <c r="Y1012">
+        <v>58</v>
+      </c>
+      <c r="Z1012">
+        <v>126</v>
+      </c>
+      <c r="AA1012">
+        <v>39</v>
+      </c>
+      <c r="AB1012">
+        <v>35</v>
+      </c>
+      <c r="AC1012">
+        <v>4.47594</v>
+      </c>
+      <c r="AD1012">
+        <v>-3.91377</v>
+      </c>
+      <c r="AE1012">
+        <v>0</v>
+      </c>
+      <c r="AF1012">
+        <v>1460.038</v>
+      </c>
+      <c r="AG1012">
+        <v>0</v>
+      </c>
+      <c r="AH1012">
+        <v>3</v>
+      </c>
+      <c r="AI1012">
+        <v>1843.10415</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:35">
+      <c r="A1013" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1013" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1013" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1013" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1013">
+        <v>34.18066666666667</v>
+      </c>
+      <c r="F1013">
+        <v>2486.15</v>
+      </c>
+      <c r="G1013">
+        <v>72.73556201361392</v>
+      </c>
+      <c r="H1013">
+        <v>209.82</v>
+      </c>
+      <c r="I1013">
+        <v>0</v>
+      </c>
+      <c r="J1013">
+        <v>0</v>
+      </c>
+      <c r="K1013">
+        <v>6.138557859218661</v>
+      </c>
+      <c r="L1013">
+        <v>0</v>
+      </c>
+      <c r="M1013">
+        <v>0</v>
+      </c>
+      <c r="N1013">
+        <v>0</v>
+      </c>
+      <c r="O1013">
+        <v>24.09284</v>
+      </c>
+      <c r="P1013">
+        <v>68.85242341106539</v>
+      </c>
+      <c r="Q1013">
+        <v>34.992</v>
+      </c>
+      <c r="R1013">
+        <v>216.0008</v>
+      </c>
+      <c r="S1013">
+        <v>6.31938522751653</v>
+      </c>
+      <c r="T1013">
+        <v>551.6800000000001</v>
+      </c>
+      <c r="U1013">
+        <v>1</v>
+      </c>
+      <c r="V1013">
+        <v>8</v>
+      </c>
+      <c r="W1013">
+        <v>9</v>
+      </c>
+      <c r="X1013">
+        <v>18</v>
+      </c>
+      <c r="Y1013">
+        <v>1</v>
+      </c>
+      <c r="Z1013">
+        <v>24</v>
+      </c>
+      <c r="AA1013">
+        <v>8</v>
+      </c>
+      <c r="AB1013">
+        <v>1</v>
+      </c>
+      <c r="AC1013">
+        <v>3.07214</v>
+      </c>
+      <c r="AD1013">
+        <v>-1.96708</v>
+      </c>
+      <c r="AE1013">
+        <v>0</v>
+      </c>
+      <c r="AF1013">
+        <v>214.3216</v>
+      </c>
+      <c r="AG1013">
+        <v>0</v>
+      </c>
+      <c r="AH1013">
+        <v>3</v>
+      </c>
+      <c r="AI1013">
+        <v>648.0024</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:35">
+      <c r="A1014" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1014" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1014" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1014" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1014">
+        <v>34.18066666666667</v>
+      </c>
+      <c r="F1014">
+        <v>2309.43</v>
+      </c>
+      <c r="G1014">
+        <v>67.56538784107974</v>
+      </c>
+      <c r="H1014">
+        <v>2.89</v>
+      </c>
+      <c r="I1014">
+        <v>0</v>
+      </c>
+      <c r="J1014">
+        <v>0</v>
+      </c>
+      <c r="K1014">
+        <v>0.08455072068030661</v>
+      </c>
+      <c r="L1014">
+        <v>0</v>
+      </c>
+      <c r="M1014">
+        <v>0</v>
+      </c>
+      <c r="N1014">
+        <v>0</v>
+      </c>
+      <c r="O1014">
+        <v>21.35538</v>
+      </c>
+      <c r="P1014">
+        <v>64.68974918211559</v>
+      </c>
+      <c r="Q1014">
+        <v>33.012</v>
+      </c>
+      <c r="R1014">
+        <v>211.9862</v>
+      </c>
+      <c r="S1014">
+        <v>6.201932866532737</v>
+      </c>
+      <c r="T1014">
+        <v>341.40001</v>
+      </c>
+      <c r="U1014">
+        <v>3</v>
+      </c>
+      <c r="V1014">
+        <v>1</v>
+      </c>
+      <c r="W1014">
+        <v>4</v>
+      </c>
+      <c r="X1014">
+        <v>17</v>
+      </c>
+      <c r="Y1014">
+        <v>3</v>
+      </c>
+      <c r="Z1014">
+        <v>21</v>
+      </c>
+      <c r="AA1014">
+        <v>1</v>
+      </c>
+      <c r="AB1014">
+        <v>7</v>
+      </c>
+      <c r="AC1014">
+        <v>3.34768</v>
+      </c>
+      <c r="AD1014">
+        <v>-2.8058</v>
+      </c>
+      <c r="AE1014">
+        <v>0</v>
+      </c>
+      <c r="AF1014">
+        <v>184.23825</v>
+      </c>
+      <c r="AG1014">
+        <v>0</v>
+      </c>
+      <c r="AH1014">
+        <v>3</v>
+      </c>
+      <c r="AI1014">
+        <v>635.9585999999999</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:35">
+      <c r="A1015" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1015" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1015" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1015" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1015">
+        <v>45.152</v>
+      </c>
+      <c r="F1015">
+        <v>3171.99</v>
+      </c>
+      <c r="G1015">
+        <v>70.2513731396173</v>
+      </c>
+      <c r="H1015">
+        <v>153.16</v>
+      </c>
+      <c r="I1015">
+        <v>0</v>
+      </c>
+      <c r="J1015">
+        <v>0</v>
+      </c>
+      <c r="K1015">
+        <v>3.392097802976612</v>
+      </c>
+      <c r="L1015">
+        <v>0</v>
+      </c>
+      <c r="M1015">
+        <v>1</v>
+      </c>
+      <c r="N1015">
+        <v>0</v>
+      </c>
+      <c r="O1015">
+        <v>25.69283</v>
+      </c>
+      <c r="P1015">
+        <v>80.28005874265718</v>
+      </c>
+      <c r="Q1015">
+        <v>32.004</v>
+      </c>
+      <c r="R1015">
+        <v>292.30967</v>
+      </c>
+      <c r="S1015">
+        <v>6.473903038625088</v>
+      </c>
+      <c r="T1015">
+        <v>511.43999</v>
+      </c>
+      <c r="U1015">
+        <v>8</v>
+      </c>
+      <c r="V1015">
+        <v>14</v>
+      </c>
+      <c r="W1015">
+        <v>22</v>
+      </c>
+      <c r="X1015">
+        <v>30</v>
+      </c>
+      <c r="Y1015">
+        <v>8</v>
+      </c>
+      <c r="Z1015">
+        <v>26</v>
+      </c>
+      <c r="AA1015">
+        <v>14</v>
+      </c>
+      <c r="AB1015">
+        <v>11</v>
+      </c>
+      <c r="AC1015">
+        <v>4.36864</v>
+      </c>
+      <c r="AD1015">
+        <v>-2.81558</v>
+      </c>
+      <c r="AE1015">
+        <v>0</v>
+      </c>
+      <c r="AF1015">
+        <v>248.6771</v>
+      </c>
+      <c r="AG1015">
+        <v>0</v>
+      </c>
+      <c r="AH1015">
+        <v>3</v>
+      </c>
+      <c r="AI1015">
+        <v>876.9290099999999</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:35">
+      <c r="A1016" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1016" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1016" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1016" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1016">
+        <v>34.18066666666667</v>
+      </c>
+      <c r="F1016">
+        <v>2417.8</v>
+      </c>
+      <c r="G1016">
+        <v>70.73589358506759</v>
+      </c>
+      <c r="H1016">
+        <v>3.48</v>
+      </c>
+      <c r="I1016">
+        <v>0</v>
+      </c>
+      <c r="J1016">
+        <v>0</v>
+      </c>
+      <c r="K1016">
+        <v>0.101811940473172</v>
+      </c>
+      <c r="L1016">
+        <v>0</v>
+      </c>
+      <c r="M1016">
+        <v>0</v>
+      </c>
+      <c r="N1016">
+        <v>0</v>
+      </c>
+      <c r="O1016">
+        <v>20.99752</v>
+      </c>
+      <c r="P1016">
+        <v>58.32644444444445</v>
+      </c>
+      <c r="Q1016">
+        <v>36</v>
+      </c>
+      <c r="R1016">
+        <v>227.58301</v>
+      </c>
+      <c r="S1016">
+        <v>6.658237892765891</v>
+      </c>
+      <c r="T1016">
+        <v>352.77999</v>
+      </c>
+      <c r="U1016">
+        <v>3</v>
+      </c>
+      <c r="V1016">
+        <v>1</v>
+      </c>
+      <c r="W1016">
+        <v>4</v>
+      </c>
+      <c r="X1016">
+        <v>22</v>
+      </c>
+      <c r="Y1016">
+        <v>3</v>
+      </c>
+      <c r="Z1016">
+        <v>21</v>
+      </c>
+      <c r="AA1016">
+        <v>1</v>
+      </c>
+      <c r="AB1016">
+        <v>0</v>
+      </c>
+      <c r="AC1016">
+        <v>3.34237</v>
+      </c>
+      <c r="AD1016">
+        <v>-2.40826</v>
+      </c>
+      <c r="AE1016">
+        <v>0</v>
+      </c>
+      <c r="AF1016">
+        <v>520.9059999999999</v>
+      </c>
+      <c r="AG1016">
+        <v>0</v>
+      </c>
+      <c r="AH1016">
+        <v>3</v>
+      </c>
+      <c r="AI1016">
+        <v>682.7490299999999</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:35">
+      <c r="A1017" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1017" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1017" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1017" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1017">
+        <v>100.0318333333333</v>
+      </c>
+      <c r="F1017">
+        <v>10352.5</v>
+      </c>
+      <c r="G1017">
+        <v>103.4920550291491</v>
+      </c>
+      <c r="H1017">
+        <v>524.6500000000001</v>
+      </c>
+      <c r="I1017">
+        <v>19.85</v>
+      </c>
+      <c r="J1017">
+        <v>2</v>
+      </c>
+      <c r="K1017">
+        <v>5.244830395657384</v>
+      </c>
+      <c r="L1017">
+        <v>57.69</v>
+      </c>
+      <c r="M1017">
+        <v>15</v>
+      </c>
+      <c r="N1017">
+        <v>4</v>
+      </c>
+      <c r="O1017">
+        <v>32.41606</v>
+      </c>
+      <c r="P1017">
+        <v>92.63848879743942</v>
+      </c>
+      <c r="Q1017">
+        <v>34.992</v>
+      </c>
+      <c r="R1017">
+        <v>936.41797</v>
+      </c>
+      <c r="S1017">
+        <v>9.361199718089741</v>
+      </c>
+      <c r="T1017">
+        <v>1601.72003</v>
+      </c>
+      <c r="U1017">
+        <v>34</v>
+      </c>
+      <c r="V1017">
+        <v>43</v>
+      </c>
+      <c r="W1017">
+        <v>77</v>
+      </c>
+      <c r="X1017">
+        <v>120</v>
+      </c>
+      <c r="Y1017">
+        <v>34</v>
+      </c>
+      <c r="Z1017">
+        <v>128</v>
+      </c>
+      <c r="AA1017">
+        <v>43</v>
+      </c>
+      <c r="AB1017">
+        <v>38</v>
+      </c>
+      <c r="AC1017">
+        <v>4.82694</v>
+      </c>
+      <c r="AD1017">
+        <v>-5.48967</v>
+      </c>
+      <c r="AE1017">
+        <v>0</v>
+      </c>
+      <c r="AF1017">
+        <v>979.4072</v>
+      </c>
+      <c r="AG1017">
+        <v>0</v>
+      </c>
+      <c r="AH1017">
+        <v>3</v>
+      </c>
+      <c r="AI1017">
+        <v>2809.25391</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:35">
+      <c r="A1018" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1018" s="1">
+        <v>46240</v>
+      </c>
+      <c r="C1018" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1018" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1018">
+        <v>64.0505</v>
+      </c>
+      <c r="F1018">
+        <v>2620.52</v>
+      </c>
+      <c r="G1018">
+        <v>40.91334181622314</v>
+      </c>
+      <c r="H1018">
+        <v>4.48</v>
+      </c>
+      <c r="I1018">
+        <v>0</v>
+      </c>
+      <c r="J1018">
+        <v>0</v>
+      </c>
+      <c r="K1018">
+        <v>0.06994480917401112</v>
+      </c>
+      <c r="L1018">
+        <v>0</v>
+      </c>
+      <c r="M1018">
+        <v>0</v>
+      </c>
+      <c r="N1018">
+        <v>0</v>
+      </c>
+      <c r="O1018">
+        <v>21.71205</v>
+      </c>
+      <c r="P1018">
+        <v>63.88903601694915</v>
+      </c>
+      <c r="Q1018">
+        <v>33.984</v>
+      </c>
+      <c r="R1018">
+        <v>279.51062</v>
+      </c>
+      <c r="S1018">
+        <v>4.363910039734272</v>
+      </c>
+      <c r="T1018">
+        <v>361.35001</v>
+      </c>
+      <c r="U1018">
+        <v>15</v>
+      </c>
+      <c r="V1018">
+        <v>13</v>
+      </c>
+      <c r="W1018">
+        <v>28</v>
+      </c>
+      <c r="X1018">
+        <v>55</v>
+      </c>
+      <c r="Y1018">
+        <v>15</v>
+      </c>
+      <c r="Z1018">
+        <v>39</v>
+      </c>
+      <c r="AA1018">
+        <v>13</v>
+      </c>
+      <c r="AB1018">
+        <v>6</v>
+      </c>
+      <c r="AC1018">
+        <v>3.85395</v>
+      </c>
+      <c r="AD1018">
+        <v>-4.05474</v>
+      </c>
+      <c r="AE1018">
+        <v>0</v>
+      </c>
+      <c r="AF1018">
+        <v>220.4384</v>
+      </c>
+      <c r="AG1018">
+        <v>0</v>
+      </c>
+      <c r="AH1018">
+        <v>3</v>
+      </c>
+      <c r="AI1018">
+        <v>838.5318600000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update CATAPULT data 2026-08-08
</commit_message>
<xml_diff>
--- a/data/Sessions_micro01.xlsx
+++ b/data/Sessions_micro01.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="182">
   <si>
     <t>player</t>
   </si>
@@ -558,6 +558,9 @@
   <si>
     <t>Partido vs San Diego</t>
   </si>
+  <si>
+    <t>Sesión 51</t>
+  </si>
 </sst>
 </file>
 
@@ -903,7 +906,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI1018"/>
+  <dimension ref="A1:AI1030"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -109757,6 +109760,1290 @@
         <v>838.5318600000001</v>
       </c>
     </row>
+    <row r="1019" spans="1:35">
+      <c r="A1019" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1019" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1019" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1019" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1019">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1019">
+        <v>3672.71</v>
+      </c>
+      <c r="G1019">
+        <v>48.58082010582012</v>
+      </c>
+      <c r="H1019">
+        <v>69.15000000000001</v>
+      </c>
+      <c r="I1019">
+        <v>0</v>
+      </c>
+      <c r="J1019">
+        <v>0</v>
+      </c>
+      <c r="K1019">
+        <v>0.9146825396825399</v>
+      </c>
+      <c r="L1019">
+        <v>0</v>
+      </c>
+      <c r="M1019">
+        <v>1</v>
+      </c>
+      <c r="N1019">
+        <v>0</v>
+      </c>
+      <c r="O1019">
+        <v>26.0783</v>
+      </c>
+      <c r="P1019">
+        <v>72.43972222222222</v>
+      </c>
+      <c r="Q1019">
+        <v>36</v>
+      </c>
+      <c r="R1019">
+        <v>353.23447</v>
+      </c>
+      <c r="S1019">
+        <v>4.672413624338625</v>
+      </c>
+      <c r="T1019">
+        <v>527.3499899999999</v>
+      </c>
+      <c r="U1019">
+        <v>9</v>
+      </c>
+      <c r="V1019">
+        <v>12</v>
+      </c>
+      <c r="W1019">
+        <v>21</v>
+      </c>
+      <c r="X1019">
+        <v>69</v>
+      </c>
+      <c r="Y1019">
+        <v>9</v>
+      </c>
+      <c r="Z1019">
+        <v>59</v>
+      </c>
+      <c r="AA1019">
+        <v>12</v>
+      </c>
+      <c r="AB1019">
+        <v>9</v>
+      </c>
+      <c r="AC1019">
+        <v>3.80314</v>
+      </c>
+      <c r="AD1019">
+        <v>-3.58515</v>
+      </c>
+      <c r="AE1019">
+        <v>0</v>
+      </c>
+      <c r="AF1019">
+        <v>883.806</v>
+      </c>
+      <c r="AG1019">
+        <v>0</v>
+      </c>
+      <c r="AH1019">
+        <v>3</v>
+      </c>
+      <c r="AI1019">
+        <v>1059.70341</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:35">
+      <c r="A1020" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1020" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1020" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1020" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1020">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1020">
+        <v>4022.75</v>
+      </c>
+      <c r="G1020">
+        <v>53.21097883597884</v>
+      </c>
+      <c r="H1020">
+        <v>60.54</v>
+      </c>
+      <c r="I1020">
+        <v>0</v>
+      </c>
+      <c r="J1020">
+        <v>0</v>
+      </c>
+      <c r="K1020">
+        <v>0.8007936507936508</v>
+      </c>
+      <c r="L1020">
+        <v>0</v>
+      </c>
+      <c r="M1020">
+        <v>0</v>
+      </c>
+      <c r="N1020">
+        <v>0</v>
+      </c>
+      <c r="O1020">
+        <v>24.80817</v>
+      </c>
+      <c r="P1020">
+        <v>76.56842592592594</v>
+      </c>
+      <c r="Q1020">
+        <v>32.4</v>
+      </c>
+      <c r="R1020">
+        <v>465.34753</v>
+      </c>
+      <c r="S1020">
+        <v>6.155390608465609</v>
+      </c>
+      <c r="T1020">
+        <v>527.65</v>
+      </c>
+      <c r="U1020">
+        <v>9</v>
+      </c>
+      <c r="V1020">
+        <v>5</v>
+      </c>
+      <c r="W1020">
+        <v>14</v>
+      </c>
+      <c r="X1020">
+        <v>52</v>
+      </c>
+      <c r="Y1020">
+        <v>9</v>
+      </c>
+      <c r="Z1020">
+        <v>34</v>
+      </c>
+      <c r="AA1020">
+        <v>5</v>
+      </c>
+      <c r="AB1020">
+        <v>5</v>
+      </c>
+      <c r="AC1020">
+        <v>3.54675</v>
+      </c>
+      <c r="AD1020">
+        <v>-3.44386</v>
+      </c>
+      <c r="AE1020">
+        <v>0</v>
+      </c>
+      <c r="AF1020">
+        <v>325.4706</v>
+      </c>
+      <c r="AG1020">
+        <v>0</v>
+      </c>
+      <c r="AH1020">
+        <v>3</v>
+      </c>
+      <c r="AI1020">
+        <v>1396.04259</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:35">
+      <c r="A1021" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1021" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1021" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1021" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1021">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1021">
+        <v>4833.62</v>
+      </c>
+      <c r="G1021">
+        <v>63.93677248677249</v>
+      </c>
+      <c r="H1021">
+        <v>174.2</v>
+      </c>
+      <c r="I1021">
+        <v>0</v>
+      </c>
+      <c r="J1021">
+        <v>0</v>
+      </c>
+      <c r="K1021">
+        <v>2.304232804232805</v>
+      </c>
+      <c r="L1021">
+        <v>0</v>
+      </c>
+      <c r="M1021">
+        <v>4</v>
+      </c>
+      <c r="N1021">
+        <v>0</v>
+      </c>
+      <c r="O1021">
+        <v>26.81753</v>
+      </c>
+      <c r="P1021">
+        <v>75.3979138551507</v>
+      </c>
+      <c r="Q1021">
+        <v>35.568</v>
+      </c>
+      <c r="R1021">
+        <v>464.86284</v>
+      </c>
+      <c r="S1021">
+        <v>6.148979365079366</v>
+      </c>
+      <c r="T1021">
+        <v>856.0799900000001</v>
+      </c>
+      <c r="U1021">
+        <v>26</v>
+      </c>
+      <c r="V1021">
+        <v>27</v>
+      </c>
+      <c r="W1021">
+        <v>53</v>
+      </c>
+      <c r="X1021">
+        <v>89</v>
+      </c>
+      <c r="Y1021">
+        <v>26</v>
+      </c>
+      <c r="Z1021">
+        <v>78</v>
+      </c>
+      <c r="AA1021">
+        <v>27</v>
+      </c>
+      <c r="AB1021">
+        <v>4</v>
+      </c>
+      <c r="AC1021">
+        <v>4.03077</v>
+      </c>
+      <c r="AD1021">
+        <v>-4.44571</v>
+      </c>
+      <c r="AE1021">
+        <v>0</v>
+      </c>
+      <c r="AF1021">
+        <v>471.032</v>
+      </c>
+      <c r="AG1021">
+        <v>0</v>
+      </c>
+      <c r="AH1021">
+        <v>3</v>
+      </c>
+      <c r="AI1021">
+        <v>1394.58852</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:35">
+      <c r="A1022" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1022" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1022" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1022" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1022">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1022">
+        <v>4094.32</v>
+      </c>
+      <c r="G1022">
+        <v>54.15767195767196</v>
+      </c>
+      <c r="H1022">
+        <v>78.10000000000001</v>
+      </c>
+      <c r="I1022">
+        <v>0</v>
+      </c>
+      <c r="J1022">
+        <v>0</v>
+      </c>
+      <c r="K1022">
+        <v>1.033068783068783</v>
+      </c>
+      <c r="L1022">
+        <v>0</v>
+      </c>
+      <c r="M1022">
+        <v>0</v>
+      </c>
+      <c r="N1022">
+        <v>0</v>
+      </c>
+      <c r="O1022">
+        <v>24.186</v>
+      </c>
+      <c r="P1022">
+        <v>67.18333333333332</v>
+      </c>
+      <c r="Q1022">
+        <v>36</v>
+      </c>
+      <c r="R1022">
+        <v>404.13423</v>
+      </c>
+      <c r="S1022">
+        <v>5.345690873015873</v>
+      </c>
+      <c r="T1022">
+        <v>437.85999</v>
+      </c>
+      <c r="U1022">
+        <v>8</v>
+      </c>
+      <c r="V1022">
+        <v>4</v>
+      </c>
+      <c r="W1022">
+        <v>12</v>
+      </c>
+      <c r="X1022">
+        <v>46</v>
+      </c>
+      <c r="Y1022">
+        <v>8</v>
+      </c>
+      <c r="Z1022">
+        <v>29</v>
+      </c>
+      <c r="AA1022">
+        <v>4</v>
+      </c>
+      <c r="AB1022">
+        <v>8</v>
+      </c>
+      <c r="AC1022">
+        <v>3.85605</v>
+      </c>
+      <c r="AD1022">
+        <v>-2.77818</v>
+      </c>
+      <c r="AE1022">
+        <v>0</v>
+      </c>
+      <c r="AF1022">
+        <v>931</v>
+      </c>
+      <c r="AG1022">
+        <v>0</v>
+      </c>
+      <c r="AH1022">
+        <v>3</v>
+      </c>
+      <c r="AI1022">
+        <v>1212.40269</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:35">
+      <c r="A1023" t="s">
+        <v>179</v>
+      </c>
+      <c r="B1023" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1023" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1023" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1023">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="F1023">
+        <v>5090.47</v>
+      </c>
+      <c r="G1023">
+        <v>62.53648648648649</v>
+      </c>
+      <c r="H1023">
+        <v>316.87</v>
+      </c>
+      <c r="I1023">
+        <v>0</v>
+      </c>
+      <c r="J1023">
+        <v>0</v>
+      </c>
+      <c r="K1023">
+        <v>3.892751842751843</v>
+      </c>
+      <c r="L1023">
+        <v>0</v>
+      </c>
+      <c r="M1023">
+        <v>4</v>
+      </c>
+      <c r="N1023">
+        <v>0</v>
+      </c>
+      <c r="O1023">
+        <v>27.12428</v>
+      </c>
+      <c r="P1023">
+        <v>75.34522222222222</v>
+      </c>
+      <c r="Q1023">
+        <v>36</v>
+      </c>
+      <c r="R1023">
+        <v>462.32062</v>
+      </c>
+      <c r="S1023">
+        <v>5.679614496314496</v>
+      </c>
+      <c r="T1023">
+        <v>1045.88001</v>
+      </c>
+      <c r="U1023">
+        <v>19</v>
+      </c>
+      <c r="V1023">
+        <v>20</v>
+      </c>
+      <c r="W1023">
+        <v>39</v>
+      </c>
+      <c r="X1023">
+        <v>88</v>
+      </c>
+      <c r="Y1023">
+        <v>19</v>
+      </c>
+      <c r="Z1023">
+        <v>62</v>
+      </c>
+      <c r="AA1023">
+        <v>20</v>
+      </c>
+      <c r="AB1023">
+        <v>3</v>
+      </c>
+      <c r="AC1023">
+        <v>4.11674</v>
+      </c>
+      <c r="AD1023">
+        <v>-3.52999</v>
+      </c>
+      <c r="AE1023">
+        <v>0</v>
+      </c>
+      <c r="AF1023">
+        <v>1217.236</v>
+      </c>
+      <c r="AG1023">
+        <v>0</v>
+      </c>
+      <c r="AH1023">
+        <v>3</v>
+      </c>
+      <c r="AI1023">
+        <v>1386.96186</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:35">
+      <c r="A1024" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1024" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1024" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1024" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1024">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1024">
+        <v>4635.900000000001</v>
+      </c>
+      <c r="G1024">
+        <v>61.32142857142858</v>
+      </c>
+      <c r="H1024">
+        <v>192.76</v>
+      </c>
+      <c r="I1024">
+        <v>0</v>
+      </c>
+      <c r="J1024">
+        <v>0</v>
+      </c>
+      <c r="K1024">
+        <v>2.54973544973545</v>
+      </c>
+      <c r="L1024">
+        <v>0</v>
+      </c>
+      <c r="M1024">
+        <v>2</v>
+      </c>
+      <c r="N1024">
+        <v>0</v>
+      </c>
+      <c r="O1024">
+        <v>29.43785</v>
+      </c>
+      <c r="P1024">
+        <v>81.77180555555556</v>
+      </c>
+      <c r="Q1024">
+        <v>36</v>
+      </c>
+      <c r="R1024">
+        <v>504.08936</v>
+      </c>
+      <c r="S1024">
+        <v>6.667848677248678</v>
+      </c>
+      <c r="T1024">
+        <v>927.22</v>
+      </c>
+      <c r="U1024">
+        <v>41</v>
+      </c>
+      <c r="V1024">
+        <v>43</v>
+      </c>
+      <c r="W1024">
+        <v>84</v>
+      </c>
+      <c r="X1024">
+        <v>108</v>
+      </c>
+      <c r="Y1024">
+        <v>41</v>
+      </c>
+      <c r="Z1024">
+        <v>91</v>
+      </c>
+      <c r="AA1024">
+        <v>43</v>
+      </c>
+      <c r="AB1024">
+        <v>26</v>
+      </c>
+      <c r="AC1024">
+        <v>4.35032</v>
+      </c>
+      <c r="AD1024">
+        <v>-4.58155</v>
+      </c>
+      <c r="AE1024">
+        <v>0</v>
+      </c>
+      <c r="AF1024">
+        <v>416.5994</v>
+      </c>
+      <c r="AG1024">
+        <v>0</v>
+      </c>
+      <c r="AH1024">
+        <v>3</v>
+      </c>
+      <c r="AI1024">
+        <v>1512.26808</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:35">
+      <c r="A1025" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1025" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1025" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1025" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1025">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1025">
+        <v>4335.23</v>
+      </c>
+      <c r="G1025">
+        <v>57.34431216931218</v>
+      </c>
+      <c r="H1025">
+        <v>93.36</v>
+      </c>
+      <c r="I1025">
+        <v>0</v>
+      </c>
+      <c r="J1025">
+        <v>0</v>
+      </c>
+      <c r="K1025">
+        <v>1.234920634920635</v>
+      </c>
+      <c r="L1025">
+        <v>0</v>
+      </c>
+      <c r="M1025">
+        <v>2</v>
+      </c>
+      <c r="N1025">
+        <v>0</v>
+      </c>
+      <c r="O1025">
+        <v>28.83413</v>
+      </c>
+      <c r="P1025">
+        <v>84.84619232580036</v>
+      </c>
+      <c r="Q1025">
+        <v>33.984</v>
+      </c>
+      <c r="R1025">
+        <v>504.87939</v>
+      </c>
+      <c r="S1025">
+        <v>6.67829880952381</v>
+      </c>
+      <c r="T1025">
+        <v>786.38999</v>
+      </c>
+      <c r="U1025">
+        <v>13</v>
+      </c>
+      <c r="V1025">
+        <v>23</v>
+      </c>
+      <c r="W1025">
+        <v>36</v>
+      </c>
+      <c r="X1025">
+        <v>73</v>
+      </c>
+      <c r="Y1025">
+        <v>13</v>
+      </c>
+      <c r="Z1025">
+        <v>81</v>
+      </c>
+      <c r="AA1025">
+        <v>23</v>
+      </c>
+      <c r="AB1025">
+        <v>10</v>
+      </c>
+      <c r="AC1025">
+        <v>3.86714</v>
+      </c>
+      <c r="AD1025">
+        <v>-4.61169</v>
+      </c>
+      <c r="AE1025">
+        <v>0</v>
+      </c>
+      <c r="AF1025">
+        <v>421.6472</v>
+      </c>
+      <c r="AG1025">
+        <v>0</v>
+      </c>
+      <c r="AH1025">
+        <v>3</v>
+      </c>
+      <c r="AI1025">
+        <v>1514.63817</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:35">
+      <c r="A1026" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1026" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1026" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1026" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1026">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="F1026">
+        <v>4543.62</v>
+      </c>
+      <c r="G1026">
+        <v>55.81842751842751</v>
+      </c>
+      <c r="H1026">
+        <v>351.4</v>
+      </c>
+      <c r="I1026">
+        <v>0</v>
+      </c>
+      <c r="J1026">
+        <v>0</v>
+      </c>
+      <c r="K1026">
+        <v>4.316953316953317</v>
+      </c>
+      <c r="L1026">
+        <v>10.23</v>
+      </c>
+      <c r="M1026">
+        <v>9</v>
+      </c>
+      <c r="N1026">
+        <v>1</v>
+      </c>
+      <c r="O1026">
+        <v>31.227</v>
+      </c>
+      <c r="P1026">
+        <v>86.74166666666667</v>
+      </c>
+      <c r="Q1026">
+        <v>36</v>
+      </c>
+      <c r="R1026">
+        <v>480.94877</v>
+      </c>
+      <c r="S1026">
+        <v>5.908461547911548</v>
+      </c>
+      <c r="T1026">
+        <v>832.2800099999999</v>
+      </c>
+      <c r="U1026">
+        <v>30</v>
+      </c>
+      <c r="V1026">
+        <v>30</v>
+      </c>
+      <c r="W1026">
+        <v>60</v>
+      </c>
+      <c r="X1026">
+        <v>75</v>
+      </c>
+      <c r="Y1026">
+        <v>30</v>
+      </c>
+      <c r="Z1026">
+        <v>62</v>
+      </c>
+      <c r="AA1026">
+        <v>30</v>
+      </c>
+      <c r="AB1026">
+        <v>10</v>
+      </c>
+      <c r="AC1026">
+        <v>4.28861</v>
+      </c>
+      <c r="AD1026">
+        <v>-4.49523</v>
+      </c>
+      <c r="AE1026">
+        <v>0</v>
+      </c>
+      <c r="AF1026">
+        <v>1116.162</v>
+      </c>
+      <c r="AG1026">
+        <v>0</v>
+      </c>
+      <c r="AH1026">
+        <v>3</v>
+      </c>
+      <c r="AI1026">
+        <v>1442.84631</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:35">
+      <c r="A1027" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1027" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1027" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1027" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1027">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1027">
+        <v>4322.23</v>
+      </c>
+      <c r="G1027">
+        <v>57.1723544973545</v>
+      </c>
+      <c r="H1027">
+        <v>221.65</v>
+      </c>
+      <c r="I1027">
+        <v>0</v>
+      </c>
+      <c r="J1027">
+        <v>0</v>
+      </c>
+      <c r="K1027">
+        <v>2.931878306878307</v>
+      </c>
+      <c r="L1027">
+        <v>0</v>
+      </c>
+      <c r="M1027">
+        <v>6</v>
+      </c>
+      <c r="N1027">
+        <v>0</v>
+      </c>
+      <c r="O1027">
+        <v>28.88872</v>
+      </c>
+      <c r="P1027">
+        <v>82.55807041609511</v>
+      </c>
+      <c r="Q1027">
+        <v>34.992</v>
+      </c>
+      <c r="R1027">
+        <v>390.81958</v>
+      </c>
+      <c r="S1027">
+        <v>5.169571164021164</v>
+      </c>
+      <c r="T1027">
+        <v>766.0500000000001</v>
+      </c>
+      <c r="U1027">
+        <v>6</v>
+      </c>
+      <c r="V1027">
+        <v>20</v>
+      </c>
+      <c r="W1027">
+        <v>26</v>
+      </c>
+      <c r="X1027">
+        <v>71</v>
+      </c>
+      <c r="Y1027">
+        <v>6</v>
+      </c>
+      <c r="Z1027">
+        <v>66</v>
+      </c>
+      <c r="AA1027">
+        <v>20</v>
+      </c>
+      <c r="AB1027">
+        <v>7</v>
+      </c>
+      <c r="AC1027">
+        <v>3.29775</v>
+      </c>
+      <c r="AD1027">
+        <v>-3.64228</v>
+      </c>
+      <c r="AE1027">
+        <v>0</v>
+      </c>
+      <c r="AF1027">
+        <v>415.8536</v>
+      </c>
+      <c r="AG1027">
+        <v>0</v>
+      </c>
+      <c r="AH1027">
+        <v>3</v>
+      </c>
+      <c r="AI1027">
+        <v>1172.45874</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:35">
+      <c r="A1028" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1028" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1028" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1028" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1028">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1028">
+        <v>3724.1</v>
+      </c>
+      <c r="G1028">
+        <v>49.26058201058201</v>
+      </c>
+      <c r="H1028">
+        <v>91.34</v>
+      </c>
+      <c r="I1028">
+        <v>0</v>
+      </c>
+      <c r="J1028">
+        <v>0</v>
+      </c>
+      <c r="K1028">
+        <v>1.208201058201058</v>
+      </c>
+      <c r="L1028">
+        <v>0</v>
+      </c>
+      <c r="M1028">
+        <v>2</v>
+      </c>
+      <c r="N1028">
+        <v>0</v>
+      </c>
+      <c r="O1028">
+        <v>27.64826</v>
+      </c>
+      <c r="P1028">
+        <v>86.39001374828148</v>
+      </c>
+      <c r="Q1028">
+        <v>32.004</v>
+      </c>
+      <c r="R1028">
+        <v>362.84763</v>
+      </c>
+      <c r="S1028">
+        <v>4.799571825396826</v>
+      </c>
+      <c r="T1028">
+        <v>402.02001</v>
+      </c>
+      <c r="U1028">
+        <v>6</v>
+      </c>
+      <c r="V1028">
+        <v>8</v>
+      </c>
+      <c r="W1028">
+        <v>14</v>
+      </c>
+      <c r="X1028">
+        <v>37</v>
+      </c>
+      <c r="Y1028">
+        <v>6</v>
+      </c>
+      <c r="Z1028">
+        <v>28</v>
+      </c>
+      <c r="AA1028">
+        <v>8</v>
+      </c>
+      <c r="AB1028">
+        <v>6</v>
+      </c>
+      <c r="AC1028">
+        <v>3.69859</v>
+      </c>
+      <c r="AD1028">
+        <v>-3.9773</v>
+      </c>
+      <c r="AE1028">
+        <v>0</v>
+      </c>
+      <c r="AF1028">
+        <v>301.0707</v>
+      </c>
+      <c r="AG1028">
+        <v>0</v>
+      </c>
+      <c r="AH1028">
+        <v>3</v>
+      </c>
+      <c r="AI1028">
+        <v>1088.54289</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:35">
+      <c r="A1029" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1029" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1029" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1029" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1029">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="F1029">
+        <v>4990.07</v>
+      </c>
+      <c r="G1029">
+        <v>66.00621693121693</v>
+      </c>
+      <c r="H1029">
+        <v>235.33</v>
+      </c>
+      <c r="I1029">
+        <v>0</v>
+      </c>
+      <c r="J1029">
+        <v>0</v>
+      </c>
+      <c r="K1029">
+        <v>3.112830687830688</v>
+      </c>
+      <c r="L1029">
+        <v>0</v>
+      </c>
+      <c r="M1029">
+        <v>4</v>
+      </c>
+      <c r="N1029">
+        <v>0</v>
+      </c>
+      <c r="O1029">
+        <v>29.29307</v>
+      </c>
+      <c r="P1029">
+        <v>81.36963888888889</v>
+      </c>
+      <c r="Q1029">
+        <v>36</v>
+      </c>
+      <c r="R1029">
+        <v>508.82332</v>
+      </c>
+      <c r="S1029">
+        <v>6.730467195767196</v>
+      </c>
+      <c r="T1029">
+        <v>909.72996</v>
+      </c>
+      <c r="U1029">
+        <v>13</v>
+      </c>
+      <c r="V1029">
+        <v>20</v>
+      </c>
+      <c r="W1029">
+        <v>33</v>
+      </c>
+      <c r="X1029">
+        <v>86</v>
+      </c>
+      <c r="Y1029">
+        <v>13</v>
+      </c>
+      <c r="Z1029">
+        <v>61</v>
+      </c>
+      <c r="AA1029">
+        <v>20</v>
+      </c>
+      <c r="AB1029">
+        <v>10</v>
+      </c>
+      <c r="AC1029">
+        <v>3.74139</v>
+      </c>
+      <c r="AD1029">
+        <v>-3.42692</v>
+      </c>
+      <c r="AE1029">
+        <v>0</v>
+      </c>
+      <c r="AF1029">
+        <v>1182.608</v>
+      </c>
+      <c r="AG1029">
+        <v>0</v>
+      </c>
+      <c r="AH1029">
+        <v>3</v>
+      </c>
+      <c r="AI1029">
+        <v>1526.46996</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:35">
+      <c r="A1030" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1030" s="1">
+        <v>46241</v>
+      </c>
+      <c r="C1030" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1030" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1030">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="F1030">
+        <v>4650.55</v>
+      </c>
+      <c r="G1030">
+        <v>57.13206388206388</v>
+      </c>
+      <c r="H1030">
+        <v>289.03</v>
+      </c>
+      <c r="I1030">
+        <v>0</v>
+      </c>
+      <c r="J1030">
+        <v>0</v>
+      </c>
+      <c r="K1030">
+        <v>3.550737100737101</v>
+      </c>
+      <c r="L1030">
+        <v>0</v>
+      </c>
+      <c r="M1030">
+        <v>5</v>
+      </c>
+      <c r="N1030">
+        <v>0</v>
+      </c>
+      <c r="O1030">
+        <v>27.8146</v>
+      </c>
+      <c r="P1030">
+        <v>86.32712600869026</v>
+      </c>
+    